<commit_message>
Mensajero: guiones para el aire de enero 2027 (semanas 2, 3 y 4)
Agro, Prevención y Estudio de la Biblia: lunes a sábado con dato para
abrir, tres puntos con problemática y solución práctica, cierre NTV.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -19124,7 +19124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T7"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19839,6 +19839,1770 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C8" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="61" t="inlineStr">
+        <is>
+          <t>Lo que se siembra, se cosecha</t>
+        </is>
+      </c>
+      <c r="E8" s="61" t="inlineStr">
+        <is>
+          <t>Paraguay está entre los cinco mayores exportadores de soja del mundo.</t>
+        </is>
+      </c>
+      <c r="F8" s="61" t="inlineStr">
+        <is>
+          <t>Departamento de Agricultura de Estados Unidos (USDA), informes de mercado mundial de oleaginosas</t>
+        </is>
+      </c>
+      <c r="G8" s="61" t="inlineStr">
+        <is>
+          <t>La ley de la siembra</t>
+        </is>
+      </c>
+      <c r="H8" s="61" t="inlineStr">
+        <is>
+          <t>En el campo nadie espera cosechar maíz si sembró poroto. La vida funciona igual: lo que hacemos hoy con el tiempo, las palabras y el dinero es la semilla de lo que vamos a tener mañana.</t>
+        </is>
+      </c>
+      <c r="I8" s="61" t="inlineStr">
+        <is>
+          <t>La cultura de la plata fácil: apuestas, préstamos rápidos y negocios dudosos que prometen cosechar sin sembrar.</t>
+        </is>
+      </c>
+      <c r="J8" s="61" t="inlineStr">
+        <is>
+          <t>Anotá esta semana tres "semillas" concretas: un hábito, una relación y un ahorro pequeño que quieras empezar a sembrar.</t>
+        </is>
+      </c>
+      <c r="K8" s="61" t="inlineStr">
+        <is>
+          <t>Elegir buena semilla</t>
+        </is>
+      </c>
+      <c r="L8" s="61" t="inlineStr">
+        <is>
+          <t>El productor sabe que la calidad de la semilla define la cosecha. En la vida, la buena semilla son los valores: honestidad, trabajo, palabra cumplida.</t>
+        </is>
+      </c>
+      <c r="M8" s="61" t="inlineStr">
+        <is>
+          <t>Jóvenes que aprenden de las redes que el atajo vale más que el esfuerzo.</t>
+        </is>
+      </c>
+      <c r="N8" s="61" t="inlineStr">
+        <is>
+          <t>Contale a un joven de tu familia cómo conseguiste algo con trabajo y paciencia. Las historias reales siembran más que los consejos.</t>
+        </is>
+      </c>
+      <c r="O8" s="61" t="inlineStr">
+        <is>
+          <t>Sembrar con fe</t>
+        </is>
+      </c>
+      <c r="P8" s="61" t="inlineStr">
+        <is>
+          <t>Sembrar es un acto de confianza: uno pone la semilla en la tierra sin ver el resultado. La fe no reemplaza el trabajo, lo acompaña.</t>
+        </is>
+      </c>
+      <c r="Q8" s="61" t="inlineStr">
+        <is>
+          <t>El desánimo de muchos pequeños productores ante la incertidumbre del clima y los precios.</t>
+        </is>
+      </c>
+      <c r="R8" s="61" t="inlineStr">
+        <is>
+          <t>Si conocés a un productor, preguntale cómo le va y ofrecé tu ayuda o tu oración. Sembrar ánimo también cuenta.</t>
+        </is>
+      </c>
+      <c r="S8" s="61" t="inlineStr">
+        <is>
+          <t>Gálatas 6:7</t>
+        </is>
+      </c>
+      <c r="T8" s="61" t="inlineStr">
+        <is>
+          <t>No se dejen engañar: nadie puede burlarse de la justicia de Dios. Siempre se cosecha lo que se siembra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>La paciencia del agricultor</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr">
+        <is>
+          <t>Alrededor del 14 % de los alimentos que se producen en el mundo se pierde entre la cosecha y la venta.</t>
+        </is>
+      </c>
+      <c r="F9" s="61" t="inlineStr">
+        <is>
+          <t>FAO, El estado mundial de la agricultura y la alimentación, 2019</t>
+        </is>
+      </c>
+      <c r="G9" s="61" t="inlineStr">
+        <is>
+          <t>Los tiempos de la tierra</t>
+        </is>
+      </c>
+      <c r="H9" s="61" t="inlineStr">
+        <is>
+          <t>Ningún agricultor tira de la planta para que crezca más rápido. Hay procesos que no se pueden apurar: la confianza, el carácter, un emprendimiento.</t>
+        </is>
+      </c>
+      <c r="I9" s="61" t="inlineStr">
+        <is>
+          <t>La ansiedad por resultados inmediatos, que hace abandonar proyectos antes de tiempo.</t>
+        </is>
+      </c>
+      <c r="J9" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un proyecto que abandonaste por impaciencia y dale una fecha realista para retomarlo.</t>
+        </is>
+      </c>
+      <c r="K9" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar lo que ya creció</t>
+        </is>
+      </c>
+      <c r="L9" s="61" t="inlineStr">
+        <is>
+          <t>De poco sirve una buena cosecha si se pierde en el camino. Cuidar lo logrado es tan importante como lograrlo.</t>
+        </is>
+      </c>
+      <c r="M9" s="61" t="inlineStr">
+        <is>
+          <t>Pérdidas de cosecha por mal almacenamiento o transporte, que golpean el bolsillo de las familias productoras.</t>
+        </is>
+      </c>
+      <c r="N9" s="61" t="inlineStr">
+        <is>
+          <t>Revisá qué estás perdiendo por descuido: comida que se tira, herramientas sin mantenimiento, plata que se va en gastos chicos.</t>
+        </is>
+      </c>
+      <c r="O9" s="61" t="inlineStr">
+        <is>
+          <t>Esperar sin quedarse quieto</t>
+        </is>
+      </c>
+      <c r="P9" s="61" t="inlineStr">
+        <is>
+          <t>La paciencia no es pasividad. El agricultor espera la lluvia, pero mientras tanto prepara, limpia y repara.</t>
+        </is>
+      </c>
+      <c r="Q9" s="61" t="inlineStr">
+        <is>
+          <t>Personas sin trabajo que se desaniman y dejan de buscar.</t>
+        </is>
+      </c>
+      <c r="R9" s="61" t="inlineStr">
+        <is>
+          <t>Si estás esperando una oportunidad, usá el tiempo para capacitarte: hay cursos gratuitos del SNPP y otras instituciones.</t>
+        </is>
+      </c>
+      <c r="S9" s="61" t="inlineStr">
+        <is>
+          <t>Santiago 5:7</t>
+        </is>
+      </c>
+      <c r="T9" s="61" t="inlineStr">
+        <is>
+          <t>Amados hermanos, tengan paciencia mientras esperan el regreso del Señor. Piensen en los agricultores, que con paciencia esperan las lluvias en el otoño y la primavera. Con ansias esperan a que maduren los preciosos cultivos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C10" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar la tierra es una bendición</t>
+        </is>
+      </c>
+      <c r="E10" s="61" t="inlineStr">
+        <is>
+          <t>Las granjas familiares producen alrededor del 80 % de los alimentos del mundo, medido en valor.</t>
+        </is>
+      </c>
+      <c r="F10" s="61" t="inlineStr">
+        <is>
+          <t>FAO, El estado mundial de la agricultura y la alimentación, 2014</t>
+        </is>
+      </c>
+      <c r="G10" s="61" t="inlineStr">
+        <is>
+          <t>La dignidad del trabajo rural</t>
+        </is>
+      </c>
+      <c r="H10" s="61" t="inlineStr">
+        <is>
+          <t>Detrás de cada plato hay manos que trabajaron la tierra. El trabajo del campo sostiene a la ciudad, aunque muchas veces no se lo valore.</t>
+        </is>
+      </c>
+      <c r="I10" s="61" t="inlineStr">
+        <is>
+          <t>La migración del campo a la ciudad, que deja chacras abandonadas y familias separadas.</t>
+        </is>
+      </c>
+      <c r="J10" s="61" t="inlineStr">
+        <is>
+          <t>Comprale directamente a productores de tu zona en ferias y mercados: tu compra ayuda a que se queden en su tierra.</t>
+        </is>
+      </c>
+      <c r="K10" s="61" t="inlineStr">
+        <is>
+          <t>La agricultura familiar</t>
+        </is>
+      </c>
+      <c r="L10" s="61" t="inlineStr">
+        <is>
+          <t>La chacra familiar no solo produce comida: enseña a los hijos a trabajar, a cuidar y a compartir.</t>
+        </is>
+      </c>
+      <c r="M10" s="61" t="inlineStr">
+        <is>
+          <t>Niños que crecen sin saber de dónde vienen los alimentos.</t>
+        </is>
+      </c>
+      <c r="N10" s="61" t="inlineStr">
+        <is>
+          <t>Armá con tus hijos una pequeña huerta en macetas o en el patio. Un tomate cosechado por ellos enseña más que una clase.</t>
+        </is>
+      </c>
+      <c r="O10" s="61" t="inlineStr">
+        <is>
+          <t>Trabajo bien hecho</t>
+        </is>
+      </c>
+      <c r="P10" s="61" t="inlineStr">
+        <is>
+          <t>Quien trabaja la tierra con esmero ve el fruto. El esfuerzo constante rinde más que la improvisación.</t>
+        </is>
+      </c>
+      <c r="Q10" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo informal sin planificación, que deja a muchos sin ingresos estables.</t>
+        </is>
+      </c>
+      <c r="R10" s="61" t="inlineStr">
+        <is>
+          <t>Llevá un cuaderno simple de tu actividad: qué gastás, qué producís y qué vendés. Lo que se anota se puede mejorar.</t>
+        </is>
+      </c>
+      <c r="S10" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 12:11</t>
+        </is>
+      </c>
+      <c r="T10" s="61" t="inlineStr">
+        <is>
+          <t>El que trabaja con esmero su tierra tendrá abundante comida, pero el que persigue fantasías no tiene sentido común.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>Los desafíos del campo</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="inlineStr">
+        <is>
+          <t>Cerca de 1 de cada 4 trabajadores del mundo trabaja en la agricultura.</t>
+        </is>
+      </c>
+      <c r="F11" s="61" t="inlineStr">
+        <is>
+          <t>Organización Internacional del Trabajo (OIT) y Banco Mundial, estadísticas de empleo por sector</t>
+        </is>
+      </c>
+      <c r="G11" s="61" t="inlineStr">
+        <is>
+          <t>Clima que no se controla</t>
+        </is>
+      </c>
+      <c r="H11" s="61" t="inlineStr">
+        <is>
+          <t>Sequías, heladas e inundaciones recuerdan que no todo depende de nosotros. Lo que sí depende es cómo nos preparamos.</t>
+        </is>
+      </c>
+      <c r="I11" s="61" t="inlineStr">
+        <is>
+          <t>Familias productoras que lo pierden todo en una sequía por no tener ningún resguardo.</t>
+        </is>
+      </c>
+      <c r="J11" s="61" t="inlineStr">
+        <is>
+          <t>Si producís, averiguá sobre seguros agrícolas y diversificá: no pongas toda tu plata en un solo cultivo.</t>
+        </is>
+      </c>
+      <c r="K11" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar en equipo</t>
+        </is>
+      </c>
+      <c r="L11" s="61" t="inlineStr">
+        <is>
+          <t>En el campo, la minga (el trabajo comunitario) fue siempre una forma de enfrentar juntos lo que solo cuesta demasiado.</t>
+        </is>
+      </c>
+      <c r="M11" s="61" t="inlineStr">
+        <is>
+          <t>El individualismo que deja a cada productor solo frente a los intermediarios.</t>
+        </is>
+      </c>
+      <c r="N11" s="61" t="inlineStr">
+        <is>
+          <t>Sumate o creá un grupo de productores o vecinos para comprar insumos y vender juntos. Juntos se negocia mejor.</t>
+        </is>
+      </c>
+      <c r="O11" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar para algo más grande</t>
+        </is>
+      </c>
+      <c r="P11" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo duro cansa menos cuando tiene sentido. Trabajar con propósito cambia la manera de levantarse cada mañana.</t>
+        </is>
+      </c>
+      <c r="Q11" s="61" t="inlineStr">
+        <is>
+          <t>El desgaste de quienes sienten que su trabajo no vale nada.</t>
+        </is>
+      </c>
+      <c r="R11" s="61" t="inlineStr">
+        <is>
+          <t>Hoy agradecé a alguien por su trabajo: al que te vende verduras, al que maneja el colectivo, al que limpia tu calle.</t>
+        </is>
+      </c>
+      <c r="S11" s="61" t="inlineStr">
+        <is>
+          <t>Colosenses 3:23</t>
+        </is>
+      </c>
+      <c r="T11" s="61" t="inlineStr">
+        <is>
+          <t>Trabajen de buena gana en todo lo que hagan, como si fuera para el Señor y no para la gente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C12" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar la tierra que nos cuida</t>
+        </is>
+      </c>
+      <c r="E12" s="61" t="inlineStr">
+        <is>
+          <t>Un tercio de los suelos del planeta están moderada o altamente degradados.</t>
+        </is>
+      </c>
+      <c r="F12" s="61" t="inlineStr">
+        <is>
+          <t>FAO, Estado de los recursos de suelos del mundo, 2015</t>
+        </is>
+      </c>
+      <c r="G12" s="61" t="inlineStr">
+        <is>
+          <t>Administradores, no dueños</t>
+        </is>
+      </c>
+      <c r="H12" s="61" t="inlineStr">
+        <is>
+          <t>La tierra fue confiada al ser humano para cultivarla y cuidarla. Usarla bien es responsabilidad; agotarla es irresponsabilidad.</t>
+        </is>
+      </c>
+      <c r="I12" s="61" t="inlineStr">
+        <is>
+          <t>La quema de campos y la deforestación, que empobrecen la tierra y afectan la salud de todos.</t>
+        </is>
+      </c>
+      <c r="J12" s="61" t="inlineStr">
+        <is>
+          <t>Nunca quemes basura ni pastizales. Si ves una quema peligrosa, avisá a los bomberos o a la municipalidad.</t>
+        </is>
+      </c>
+      <c r="K12" s="61" t="inlineStr">
+        <is>
+          <t>El agua es vida</t>
+        </is>
+      </c>
+      <c r="L12" s="61" t="inlineStr">
+        <is>
+          <t>Ríos, arroyos y acuíferos son un tesoro. Lo que se tira al agua vuelve a nosotros.</t>
+        </is>
+      </c>
+      <c r="M12" s="61" t="inlineStr">
+        <is>
+          <t>Arroyos contaminados con basura y agroquímicos cerca de las comunidades.</t>
+        </is>
+      </c>
+      <c r="N12" s="61" t="inlineStr">
+        <is>
+          <t>Organizá con tus vecinos una limpieza del arroyo o la plaza del barrio. Una mañana de trabajo cambia el paisaje.</t>
+        </is>
+      </c>
+      <c r="O12" s="61" t="inlineStr">
+        <is>
+          <t>Pequeños gestos, gran impacto</t>
+        </is>
+      </c>
+      <c r="P12" s="61" t="inlineStr">
+        <is>
+          <t>El cuidado del ambiente empieza en casa: separar residuos, no desperdiciar agua, plantar un árbol.</t>
+        </is>
+      </c>
+      <c r="Q12" s="61" t="inlineStr">
+        <is>
+          <t>La cantidad de plástico que termina en calles y cauces.</t>
+        </is>
+      </c>
+      <c r="R12" s="61" t="inlineStr">
+        <is>
+          <t>Usá una bolsa reutilizable para las compras y separá en casa lo orgánico del resto. Con lo orgánico podés hacer abono.</t>
+        </is>
+      </c>
+      <c r="S12" s="61" t="inlineStr">
+        <is>
+          <t>Génesis 2:15</t>
+        </is>
+      </c>
+      <c r="T12" s="61" t="inlineStr">
+        <is>
+          <t>El Señor Dios puso al hombre en el jardín de Edén para que se ocupara de él y lo custodiara.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>Una herencia para los que vienen</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr">
+        <is>
+          <t>Formar apenas un centímetro de suelo fértil puede llevar hasta mil años.</t>
+        </is>
+      </c>
+      <c r="F13" s="61" t="inlineStr">
+        <is>
+          <t>FAO, Año Internacional de los Suelos, 2015</t>
+        </is>
+      </c>
+      <c r="G13" s="61" t="inlineStr">
+        <is>
+          <t>Pensar en los nietos</t>
+        </is>
+      </c>
+      <c r="H13" s="61" t="inlineStr">
+        <is>
+          <t>Las decisiones de hoy sobre la tierra son la herencia de mañana. Quien piensa solo en la cosecha de este año puede dejar un desierto a sus hijos.</t>
+        </is>
+      </c>
+      <c r="I13" s="61" t="inlineStr">
+        <is>
+          <t>La venta de tierras familiares sin planificación, que deja a las nuevas generaciones sin lugar.</t>
+        </is>
+      </c>
+      <c r="J13" s="61" t="inlineStr">
+        <is>
+          <t>Conversá en familia qué quieren dejar a la próxima generación: tierra, oficio, valores. Ponerlo en palabras ayuda a cuidarlo.</t>
+        </is>
+      </c>
+      <c r="K13" s="61" t="inlineStr">
+        <is>
+          <t>Plantar árboles</t>
+        </is>
+      </c>
+      <c r="L13" s="61" t="inlineStr">
+        <is>
+          <t>Dicen que la mejor época para plantar un árbol fue hace veinte años; la segunda mejor es hoy.</t>
+        </is>
+      </c>
+      <c r="M13" s="61" t="inlineStr">
+        <is>
+          <t>Barrios sin sombra ni árboles, más calurosos cada verano.</t>
+        </is>
+      </c>
+      <c r="N13" s="61" t="inlineStr">
+        <is>
+          <t>Plantá un árbol nativo este fin de semana: lapacho, timbó o tajy. Hacelo con los chicos y pónganle nombre.</t>
+        </is>
+      </c>
+      <c r="O13" s="61" t="inlineStr">
+        <is>
+          <t>Toda la creación es de Dios</t>
+        </is>
+      </c>
+      <c r="P13" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar la tierra es también una forma de agradecer. No somos dueños absolutos: somos parte de algo más grande.</t>
+        </is>
+      </c>
+      <c r="Q13" s="61" t="inlineStr">
+        <is>
+          <t>El consumo sin medida, que usa y tira sin pensar de dónde viene cada cosa.</t>
+        </is>
+      </c>
+      <c r="R13" s="61" t="inlineStr">
+        <is>
+          <t>Antes de comprar algo nuevo esta semana, preguntate si lo necesitás, si podés repararlo o pedirlo prestado.</t>
+        </is>
+      </c>
+      <c r="S13" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 24:1</t>
+        </is>
+      </c>
+      <c r="T13" s="61" t="inlineStr">
+        <is>
+          <t>La tierra es del Señor y todo lo que hay en ella; el mundo y todos sus habitantes le pertenecen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C14" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="61" t="inlineStr">
+        <is>
+          <t>Prevenir es amar</t>
+        </is>
+      </c>
+      <c r="E14" s="61" t="inlineStr">
+        <is>
+          <t>Las enfermedades no transmisibles (corazón, cáncer, diabetes, pulmones) causan el 74 % de las muertes en el mundo.</t>
+        </is>
+      </c>
+      <c r="F14" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, nota descriptiva sobre enfermedades no transmisibles, 2023</t>
+        </is>
+      </c>
+      <c r="G14" s="61" t="inlineStr">
+        <is>
+          <t>Mejor prevenir que curar</t>
+        </is>
+      </c>
+      <c r="H14" s="61" t="inlineStr">
+        <is>
+          <t>La prevención primaria busca que la enfermedad no aparezca: alimentación, movimiento, vacunas, no fumar. Es la medicina más barata.</t>
+        </is>
+      </c>
+      <c r="I14" s="61" t="inlineStr">
+        <is>
+          <t>Esperar a sentirse mal para recién cuidarse.</t>
+        </is>
+      </c>
+      <c r="J14" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una sola costumbre preventiva para esta semana: caminar 20 minutos, sumar una fruta al día o dejar el cigarrillo.</t>
+        </is>
+      </c>
+      <c r="K14" s="61" t="inlineStr">
+        <is>
+          <t>Las vacunas cuidan a todos</t>
+        </is>
+      </c>
+      <c r="L14" s="61" t="inlineStr">
+        <is>
+          <t>Vacunarse protege a uno mismo y a los que no pueden hacerlo, como bebés y personas enfermas.</t>
+        </is>
+      </c>
+      <c r="M14" s="61" t="inlineStr">
+        <is>
+          <t>Las dudas y la desinformación sobre las vacunas, que bajan la cobertura en los niños.</t>
+        </is>
+      </c>
+      <c r="N14" s="61" t="inlineStr">
+        <is>
+          <t>Revisá la libreta de vacunación de tus hijos y la tuya. Consultá en tu unidad de salud familiar qué vacunas te tocan.</t>
+        </is>
+      </c>
+      <c r="O14" s="61" t="inlineStr">
+        <is>
+          <t>Cuidarse por los demás</t>
+        </is>
+      </c>
+      <c r="P14" s="61" t="inlineStr">
+        <is>
+          <t>Cuando te cuidás, cuidás a quienes dependen de vos. La prevención también es una forma de amor.</t>
+        </is>
+      </c>
+      <c r="Q14" s="61" t="inlineStr">
+        <is>
+          <t>Padres y madres que se descuidan por cuidar a todos, hasta que se enferman.</t>
+        </is>
+      </c>
+      <c r="R14" s="61" t="inlineStr">
+        <is>
+          <t>Pedí a tu familia que te ayude a cumplir tu propósito de salud. Hacerlo juntos es más fácil.</t>
+        </is>
+      </c>
+      <c r="S14" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 22:3</t>
+        </is>
+      </c>
+      <c r="T14" s="61" t="inlineStr">
+        <is>
+          <t>El prudente se anticipa al peligro y toma precauciones; el simplón avanza a ciegas y sufre las consecuencias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>Hábitos que protegen</t>
+        </is>
+      </c>
+      <c r="E15" s="61" t="inlineStr">
+        <is>
+          <t>Al menos el 80 % de las enfermedades del corazón, los accidentes cerebrovasculares y la diabetes tipo 2 prematuros podrían prevenirse.</t>
+        </is>
+      </c>
+      <c r="F15" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Prevención de las enfermedades crónicas: una inversión vital, 2005</t>
+        </is>
+      </c>
+      <c r="G15" s="61" t="inlineStr">
+        <is>
+          <t>La mesa de cada día</t>
+        </is>
+      </c>
+      <c r="H15" s="61" t="inlineStr">
+        <is>
+          <t>Lo que comemos todos los días pesa más que lo que comemos en una fiesta. La sal, el azúcar y las frituras en exceso pasan factura.</t>
+        </is>
+      </c>
+      <c r="I15" s="61" t="inlineStr">
+        <is>
+          <t>El consumo diario de gaseosas y comida ultraprocesada, también en los niños.</t>
+        </is>
+      </c>
+      <c r="J15" s="61" t="inlineStr">
+        <is>
+          <t>Reducí la sal en la cocina de a poco y reemplazá la gaseosa diaria por agua o jugo natural.</t>
+        </is>
+      </c>
+      <c r="K15" s="61" t="inlineStr">
+        <is>
+          <t>Moverse para vivir</t>
+        </is>
+      </c>
+      <c r="L15" s="61" t="inlineStr">
+        <is>
+          <t>No hace falta ser deportista. Caminar, bailar o subir escaleras ya protege el corazón.</t>
+        </is>
+      </c>
+      <c r="M15" s="61" t="inlineStr">
+        <is>
+          <t>El sedentarismo de quienes pasan el día sentados y la noche frente a una pantalla.</t>
+        </is>
+      </c>
+      <c r="N15" s="61" t="inlineStr">
+        <is>
+          <t>Proponé a tu familia o a tus compañeros una caminata semanal. Ponele día y hora fijos.</t>
+        </is>
+      </c>
+      <c r="O15" s="61" t="inlineStr">
+        <is>
+          <t>Interesarse por el otro</t>
+        </is>
+      </c>
+      <c r="P15" s="61" t="inlineStr">
+        <is>
+          <t>Prevenir también es estar atento a la salud de los demás: un vecino solo, un familiar que no va al médico.</t>
+        </is>
+      </c>
+      <c r="Q15" s="61" t="inlineStr">
+        <is>
+          <t>Adultos mayores que viven solos y nadie nota cuando empiezan a decaer.</t>
+        </is>
+      </c>
+      <c r="R15" s="61" t="inlineStr">
+        <is>
+          <t>Llamá esta semana a un familiar mayor y preguntale de verdad cómo está su salud.</t>
+        </is>
+      </c>
+      <c r="S15" s="61" t="inlineStr">
+        <is>
+          <t>Filipenses 2:4</t>
+        </is>
+      </c>
+      <c r="T15" s="61" t="inlineStr">
+        <is>
+          <t>No se ocupen solo de sus propios intereses, sino también procuren interesarse en los demás.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C16" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="61" t="inlineStr">
+        <is>
+          <t>Detectar a tiempo salva vidas</t>
+        </is>
+      </c>
+      <c r="E16" s="61" t="inlineStr">
+        <is>
+          <t>Casi la mitad de las personas con presión alta no sabe que la tiene.</t>
+        </is>
+      </c>
+      <c r="F16" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Informe mundial sobre la hipertensión, 2023</t>
+        </is>
+      </c>
+      <c r="G16" s="61" t="inlineStr">
+        <is>
+          <t>Lo que no duele también importa</t>
+        </is>
+      </c>
+      <c r="H16" s="61" t="inlineStr">
+        <is>
+          <t>La presión alta, el azúcar elevada y muchos cánceres no dan síntomas al principio. Por eso se los llama enemigos silenciosos.</t>
+        </is>
+      </c>
+      <c r="I16" s="61" t="inlineStr">
+        <is>
+          <t>Personas que dicen "yo estoy sano, nunca voy al médico" hasta que aparece un problema grave.</t>
+        </is>
+      </c>
+      <c r="J16" s="61" t="inlineStr">
+        <is>
+          <t>Tomate la presión esta semana: en la farmacia, en la unidad de salud familiar o con un tensiómetro en casa.</t>
+        </is>
+      </c>
+      <c r="K16" s="61" t="inlineStr">
+        <is>
+          <t>El control anual</t>
+        </is>
+      </c>
+      <c r="L16" s="61" t="inlineStr">
+        <is>
+          <t>Un control de rutina al año (presión, glucosa, colesterol) permite actuar antes de que sea tarde.</t>
+        </is>
+      </c>
+      <c r="M16" s="61" t="inlineStr">
+        <is>
+          <t>El miedo a ir al médico por temor a lo que puedan encontrar.</t>
+        </is>
+      </c>
+      <c r="N16" s="61" t="inlineStr">
+        <is>
+          <t>Agendá tu control anual en una fecha fácil de recordar, como tu cumpleaños, y repetilo cada año.</t>
+        </is>
+      </c>
+      <c r="O16" s="61" t="inlineStr">
+        <is>
+          <t>Escuchar consejo</t>
+        </is>
+      </c>
+      <c r="P16" s="61" t="inlineStr">
+        <is>
+          <t>Pedir opinión a quien sabe no es debilidad. Los profesionales de salud están para orientarnos.</t>
+        </is>
+      </c>
+      <c r="Q16" s="61" t="inlineStr">
+        <is>
+          <t>La automedicación y los consejos de internet sin respaldo.</t>
+        </is>
+      </c>
+      <c r="R16" s="61" t="inlineStr">
+        <is>
+          <t>Antes de tomar un remedio por tu cuenta, consultá en la farmacia o en el centro de salud. Llevá la lista de lo que tomás.</t>
+        </is>
+      </c>
+      <c r="S16" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 15:22</t>
+        </is>
+      </c>
+      <c r="T16" s="61" t="inlineStr">
+        <is>
+          <t>Los planes fracasan por falta de consejo; muchos consejeros traen éxito.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C17" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="61" t="inlineStr">
+        <is>
+          <t>Animarse a hacerse los estudios</t>
+        </is>
+      </c>
+      <c r="E17" s="61" t="inlineStr">
+        <is>
+          <t>La OMS se propone que el 70 % de las mujeres se haga una prueba de detección del cáncer de cuello uterino a los 35 y a los 45 años, porque detectado a tiempo es uno de los más curables.</t>
+        </is>
+      </c>
+      <c r="F17" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Estrategia mundial para eliminar el cáncer de cuello uterino, 2020</t>
+        </is>
+      </c>
+      <c r="G17" s="61" t="inlineStr">
+        <is>
+          <t>Estudios que cuidan</t>
+        </is>
+      </c>
+      <c r="H17" s="61" t="inlineStr">
+        <is>
+          <t>El papanicolau, la mamografía y los controles de próstata son simples y pueden salvar la vida.</t>
+        </is>
+      </c>
+      <c r="I17" s="61" t="inlineStr">
+        <is>
+          <t>La vergüenza o el machismo que hacen postergar los estudios, sobre todo en los hombres.</t>
+        </is>
+      </c>
+      <c r="J17" s="61" t="inlineStr">
+        <is>
+          <t>Si sos hombre mayor de 50, pedí tu control de próstata. Si sos mujer, consultá cuándo te toca el papanicolau o la mamografía.</t>
+        </is>
+      </c>
+      <c r="K17" s="61" t="inlineStr">
+        <is>
+          <t>Acompañar al que tiene miedo</t>
+        </is>
+      </c>
+      <c r="L17" s="61" t="inlineStr">
+        <is>
+          <t>Muchos no van al médico por miedo o porque no tienen con quién ir. Un acompañante hace la diferencia.</t>
+        </is>
+      </c>
+      <c r="M17" s="61" t="inlineStr">
+        <is>
+          <t>Personas que no se atienden porque no tienen quién las lleve o cuide a los hijos.</t>
+        </is>
+      </c>
+      <c r="N17" s="61" t="inlineStr">
+        <is>
+          <t>Ofrecete a acompañar a un familiar o vecino a su próximo control.</t>
+        </is>
+      </c>
+      <c r="O17" s="61" t="inlineStr">
+        <is>
+          <t>Mejor juntos</t>
+        </is>
+      </c>
+      <c r="P17" s="61" t="inlineStr">
+        <is>
+          <t>La salud se cuida mejor en comunidad: grupos de caminata, ferias de salud, campañas del barrio.</t>
+        </is>
+      </c>
+      <c r="Q17" s="61" t="inlineStr">
+        <is>
+          <t>Campañas gratuitas de salud a las que va poca gente por falta de información.</t>
+        </is>
+      </c>
+      <c r="R17" s="61" t="inlineStr">
+        <is>
+          <t>Difundí en tus grupos de WhatsApp las campañas de salud gratuitas de tu zona.</t>
+        </is>
+      </c>
+      <c r="S17" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés 4:9-10</t>
+        </is>
+      </c>
+      <c r="T17" s="61" t="inlineStr">
+        <is>
+          <t>Es mejor ser dos que uno, porque ambos pueden ayudarse mutuamente a lograr el éxito. Si uno cae, el otro puede darle la mano y ayudarle; pero el que cae y está solo, ese sí que está en problemas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C18" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="61" t="inlineStr">
+        <is>
+          <t>Vivir bien con una enfermedad</t>
+        </is>
+      </c>
+      <c r="E18" s="61" t="inlineStr">
+        <is>
+          <t>La diabetes es una de las principales causas de ceguera, insuficiencia renal y amputación de miembros inferiores.</t>
+        </is>
+      </c>
+      <c r="F18" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, nota descriptiva sobre diabetes</t>
+        </is>
+      </c>
+      <c r="G18" s="61" t="inlineStr">
+        <is>
+          <t>Evitar que empeore</t>
+        </is>
+      </c>
+      <c r="H18" s="61" t="inlineStr">
+        <is>
+          <t>La prevención terciaria cuida a quien ya tiene una enfermedad para que no se complique: seguir el tratamiento, controlar, cuidarse.</t>
+        </is>
+      </c>
+      <c r="I18" s="61" t="inlineStr">
+        <is>
+          <t>Pacientes que dejan el tratamiento cuando se sienten mejor.</t>
+        </is>
+      </c>
+      <c r="J18" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés una enfermedad crónica, anotá tus remedios y horarios en un papel visible o en una alarma del celular.</t>
+        </is>
+      </c>
+      <c r="K18" s="61" t="inlineStr">
+        <is>
+          <t>No perder el ánimo</t>
+        </is>
+      </c>
+      <c r="L18" s="61" t="inlineStr">
+        <is>
+          <t>Un diagnóstico puede desanimar. Pero muchas personas viven años con buena calidad de vida cuidándose.</t>
+        </is>
+      </c>
+      <c r="M18" s="61" t="inlineStr">
+        <is>
+          <t>La depresión que acompaña muchas enfermedades crónicas y que pocas veces se habla.</t>
+        </is>
+      </c>
+      <c r="N18" s="61" t="inlineStr">
+        <is>
+          <t>Si te sentís sin fuerzas, contalo a tu médico y a alguien de confianza. Pedir ayuda es parte del tratamiento.</t>
+        </is>
+      </c>
+      <c r="O18" s="61" t="inlineStr">
+        <is>
+          <t>Fuerzas renovadas</t>
+        </is>
+      </c>
+      <c r="P18" s="61" t="inlineStr">
+        <is>
+          <t>La fe no reemplaza el tratamiento, pero da esperanza para sostenerlo día tras día.</t>
+        </is>
+      </c>
+      <c r="Q18" s="61" t="inlineStr">
+        <is>
+          <t>El aislamiento de quienes viven una enfermedad larga.</t>
+        </is>
+      </c>
+      <c r="R18" s="61" t="inlineStr">
+        <is>
+          <t>Buscá un grupo de apoyo de pacientes o una comunidad que te acompañe. No tenés que atravesarlo solo.</t>
+        </is>
+      </c>
+      <c r="S18" s="61" t="inlineStr">
+        <is>
+          <t>Isaías 40:31</t>
+        </is>
+      </c>
+      <c r="T18" s="61" t="inlineStr">
+        <is>
+          <t>En cambio, los que confían en el Señor encontrarán nuevas fuerzas; volarán alto, como con alas de águila. Correrán y no se cansarán; caminarán y no desmayarán.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="B19" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C19" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar al que cuida</t>
+        </is>
+      </c>
+      <c r="E19" s="61" t="inlineStr">
+        <is>
+          <t>En los países desarrollados, solo alrededor de la mitad de los pacientes con enfermedades crónicas cumple bien su tratamiento.</t>
+        </is>
+      </c>
+      <c r="F19" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Adherencia a los tratamientos a largo plazo, 2003</t>
+        </is>
+      </c>
+      <c r="G19" s="61" t="inlineStr">
+        <is>
+          <t>La familia es parte del tratamiento</t>
+        </is>
+      </c>
+      <c r="H19" s="61" t="inlineStr">
+        <is>
+          <t>Recordar un remedio, acompañar a un control o cocinar más sano son formas concretas de cuidar.</t>
+        </is>
+      </c>
+      <c r="I19" s="61" t="inlineStr">
+        <is>
+          <t>Familias que dejan toda la responsabilidad del cuidado en una sola persona.</t>
+        </is>
+      </c>
+      <c r="J19" s="61" t="inlineStr">
+        <is>
+          <t>Repartan en casa las tareas de cuidado: quién acompaña al médico, quién compra los remedios, quién cocina.</t>
+        </is>
+      </c>
+      <c r="K19" s="61" t="inlineStr">
+        <is>
+          <t>El cansancio del cuidador</t>
+        </is>
+      </c>
+      <c r="L19" s="61" t="inlineStr">
+        <is>
+          <t>Quien cuida a un enfermo también necesita descanso y apoyo.</t>
+        </is>
+      </c>
+      <c r="M19" s="61" t="inlineStr">
+        <is>
+          <t>Cuidadores, casi siempre mujeres, agotados y sin tiempo para sí mismos.</t>
+        </is>
+      </c>
+      <c r="N19" s="61" t="inlineStr">
+        <is>
+          <t>Ofrecé unas horas de relevo a alguien que cuida a un familiar enfermo: que pueda salir, dormir o descansar.</t>
+        </is>
+      </c>
+      <c r="O19" s="61" t="inlineStr">
+        <is>
+          <t>Llevar las cargas juntos</t>
+        </is>
+      </c>
+      <c r="P19" s="61" t="inlineStr">
+        <is>
+          <t>El amor se vuelve concreto cuando compartimos el peso del otro.</t>
+        </is>
+      </c>
+      <c r="Q19" s="61" t="inlineStr">
+        <is>
+          <t>La soledad de quienes enfrentan una enfermedad sin red de apoyo.</t>
+        </is>
+      </c>
+      <c r="R19" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en una persona enferma de tu entorno y llevale algo concreto esta semana: una comida, una visita, una llamada.</t>
+        </is>
+      </c>
+      <c r="S19" s="61" t="inlineStr">
+        <is>
+          <t>Gálatas 6:2</t>
+        </is>
+      </c>
+      <c r="T19" s="61" t="inlineStr">
+        <is>
+          <t>Ayúdense a llevar los unos las cargas de los otros, y obedezcan de esa manera la ley de Cristo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C20" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="61" t="inlineStr">
+        <is>
+          <t>Leer no es lo mismo que estudiar</t>
+        </is>
+      </c>
+      <c r="E20" s="61" t="inlineStr">
+        <is>
+          <t>Quienes leen la Biblia cuatro o más veces por semana muestran cambios mucho mayores en su conducta diaria que quienes la leen con menos frecuencia.</t>
+        </is>
+      </c>
+      <c r="F20" s="61" t="inlineStr">
+        <is>
+          <t>Center for Bible Engagement, Arnold Cole y Pamela Caudill Ovwigho, Understanding the Bible Engagement Challenge, 2009</t>
+        </is>
+      </c>
+      <c r="G20" s="61" t="inlineStr">
+        <is>
+          <t>Más que información</t>
+        </is>
+      </c>
+      <c r="H20" s="61" t="inlineStr">
+        <is>
+          <t>Se puede leer un capítulo sin que cambie nada. Estudiar es detenerse, preguntar y dejar que el texto nos hable.</t>
+        </is>
+      </c>
+      <c r="I20" s="61" t="inlineStr">
+        <is>
+          <t>La lectura apurada de todo: mensajes, titulares y redes, sin comprender a fondo.</t>
+        </is>
+      </c>
+      <c r="J20" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un texto corto esta semana y leelo tres veces en días distintos. Anotá qué notás de nuevo cada vez.</t>
+        </is>
+      </c>
+      <c r="K20" s="61" t="inlineStr">
+        <is>
+          <t>Un libro para la vida</t>
+        </is>
+      </c>
+      <c r="L20" s="61" t="inlineStr">
+        <is>
+          <t>La Biblia no es solo un libro religioso: habla de familia, trabajo, dinero, conflictos y esperanza.</t>
+        </is>
+      </c>
+      <c r="M20" s="61" t="inlineStr">
+        <is>
+          <t>La idea de que la Biblia no tiene nada que decir sobre los problemas de hoy.</t>
+        </is>
+      </c>
+      <c r="N20" s="61" t="inlineStr">
+        <is>
+          <t>Buscá qué dice Proverbios sobre un tema que te preocupe (dinero, trabajo, familia) y anotá un consejo práctico.</t>
+        </is>
+      </c>
+      <c r="O20" s="61" t="inlineStr">
+        <is>
+          <t>Útil para corregir y enseñar</t>
+        </is>
+      </c>
+      <c r="P20" s="61" t="inlineStr">
+        <is>
+          <t>La Escritura no está para que sepamos más, sino para que vivamos mejor.</t>
+        </is>
+      </c>
+      <c r="Q20" s="61" t="inlineStr">
+        <is>
+          <t>Personas que conocen muchos versículos pero no los aplican.</t>
+        </is>
+      </c>
+      <c r="R20" s="61" t="inlineStr">
+        <is>
+          <t>Por cada texto que estudies, escribí una acción concreta para hacer esa misma semana.</t>
+        </is>
+      </c>
+      <c r="S20" s="61" t="inlineStr">
+        <is>
+          <t>2 Timoteo 3:16-17</t>
+        </is>
+      </c>
+      <c r="T20" s="61" t="inlineStr">
+        <is>
+          <t>Toda la Escritura es inspirada por Dios y es útil para enseñarnos lo que es verdad y para hacernos ver lo que está mal en nuestra vida. Nos corrige cuando estamos equivocados y nos enseña a hacer lo correcto. Dios la usa para preparar y capacitar a su pueblo para que haga toda buena obra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B21" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C21" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="61" t="inlineStr">
+        <is>
+          <t>Del oído a la práctica</t>
+        </is>
+      </c>
+      <c r="E21" s="61" t="inlineStr">
+        <is>
+          <t>Si no repasamos lo aprendido, olvidamos más de la mitad en apenas un día.</t>
+        </is>
+      </c>
+      <c r="F21" s="61" t="inlineStr">
+        <is>
+          <t>Hermann Ebbinghaus, estudios sobre la memoria y la "curva del olvido", 1885</t>
+        </is>
+      </c>
+      <c r="G21" s="61" t="inlineStr">
+        <is>
+          <t>Repasar para recordar</t>
+        </is>
+      </c>
+      <c r="H21" s="61" t="inlineStr">
+        <is>
+          <t>Lo que se repasa se queda. Volver a un texto durante la semana lo fija en la memoria y en el corazón.</t>
+        </is>
+      </c>
+      <c r="I21" s="61" t="inlineStr">
+        <is>
+          <t>Escuchar un buen mensaje el domingo y olvidarlo el lunes.</t>
+        </is>
+      </c>
+      <c r="J21" s="61" t="inlineStr">
+        <is>
+          <t>Escribí el versículo de la semana en un papel y pegalo en la heladera o como fondo de pantalla.</t>
+        </is>
+      </c>
+      <c r="K21" s="61" t="inlineStr">
+        <is>
+          <t>Hacer, no solo escuchar</t>
+        </is>
+      </c>
+      <c r="L21" s="61" t="inlineStr">
+        <is>
+          <t>El valor de lo aprendido se ve en lo que cambia. Escuchar sin practicar es engañarse.</t>
+        </is>
+      </c>
+      <c r="M21" s="61" t="inlineStr">
+        <is>
+          <t>La distancia entre lo que se dice y lo que se vive, que aleja a muchos de la fe.</t>
+        </is>
+      </c>
+      <c r="N21" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una enseñanza y aplicala hoy mismo con alguien concreto: pedir perdón, ayudar, agradecer.</t>
+        </is>
+      </c>
+      <c r="O21" s="61" t="inlineStr">
+        <is>
+          <t>Diligencia diaria</t>
+        </is>
+      </c>
+      <c r="P21" s="61" t="inlineStr">
+        <is>
+          <t>No hace falta una hora por día. Diez minutos constantes valen más que un maratón cada tanto.</t>
+        </is>
+      </c>
+      <c r="Q21" s="61" t="inlineStr">
+        <is>
+          <t>La falta de tiempo como excusa para todo lo importante.</t>
+        </is>
+      </c>
+      <c r="R21" s="61" t="inlineStr">
+        <is>
+          <t>Fijá un horario de diez minutos para leer: al levantarte, en el colectivo o antes de dormir.</t>
+        </is>
+      </c>
+      <c r="S21" s="61" t="inlineStr">
+        <is>
+          <t>Santiago 1:22</t>
+        </is>
+      </c>
+      <c r="T21" s="61" t="inlineStr">
+        <is>
+          <t>No solo escuchen la palabra de Dios; tienen que ponerla en práctica. De lo contrario, solamente se engañan a sí mismos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C22" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="61" t="inlineStr">
+        <is>
+          <t>Métodos sencillos para estudiar</t>
+        </is>
+      </c>
+      <c r="E22" s="61" t="inlineStr">
+        <is>
+          <t>Quienes toman notas a mano comprenden mejor los conceptos que quienes escriben en una computadora.</t>
+        </is>
+      </c>
+      <c r="F22" s="61" t="inlineStr">
+        <is>
+          <t>Pam Mueller y Daniel Oppenheimer, revista Psychological Science, 2014</t>
+        </is>
+      </c>
+      <c r="G22" s="61" t="inlineStr">
+        <is>
+          <t>Observar, entender, aplicar</t>
+        </is>
+      </c>
+      <c r="H22" s="61" t="inlineStr">
+        <is>
+          <t>Un método simple: ¿qué dice el texto?, ¿qué significaba para los que lo leyeron primero?, ¿qué me dice hoy a mí?</t>
+        </is>
+      </c>
+      <c r="I22" s="61" t="inlineStr">
+        <is>
+          <t>Interpretaciones sacadas de contexto que generan confusión y división.</t>
+        </is>
+      </c>
+      <c r="J22" s="61" t="inlineStr">
+        <is>
+          <t>Antes de sacar conclusiones, leé los versículos de antes y de después. El contexto aclara casi todo.</t>
+        </is>
+      </c>
+      <c r="K22" s="61" t="inlineStr">
+        <is>
+          <t>Escribir lo que aprendés</t>
+        </is>
+      </c>
+      <c r="L22" s="61" t="inlineStr">
+        <is>
+          <t>Un cuaderno de estudio ayuda a ordenar ideas y a ver el crecimiento con el tiempo.</t>
+        </is>
+      </c>
+      <c r="M22" s="61" t="inlineStr">
+        <is>
+          <t>Mucho contenido consumido en el celular que no deja nada escrito ni recordado.</t>
+        </is>
+      </c>
+      <c r="N22" s="61" t="inlineStr">
+        <is>
+          <t>Conseguí un cuaderno solo para tu estudio bíblico y anotá la fecha, el texto y una idea por día.</t>
+        </is>
+      </c>
+      <c r="O22" s="61" t="inlineStr">
+        <is>
+          <t>Examinar con entusiasmo</t>
+        </is>
+      </c>
+      <c r="P22" s="61" t="inlineStr">
+        <is>
+          <t>Estudiar es preguntar sin miedo y comprobar lo que se escucha.</t>
+        </is>
+      </c>
+      <c r="Q22" s="61" t="inlineStr">
+        <is>
+          <t>Creer cualquier cosa que circula en cadenas y redes sin verificarla.</t>
+        </is>
+      </c>
+      <c r="R22" s="61" t="inlineStr">
+        <is>
+          <t>Cuando escuches una enseñanza, buscá vos mismo los textos citados y leelos completos.</t>
+        </is>
+      </c>
+      <c r="S22" s="61" t="inlineStr">
+        <is>
+          <t>Hechos 17:11</t>
+        </is>
+      </c>
+      <c r="T22" s="61" t="inlineStr">
+        <is>
+          <t>Ellos escucharon con entusiasmo el mensaje de Pablo. Día tras día examinaban las Escrituras para ver si Pablo y Silas enseñaban la verdad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C23" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="61" t="inlineStr">
+        <is>
+          <t>Un plan que se pueda cumplir</t>
+        </is>
+      </c>
+      <c r="E23" s="61" t="inlineStr">
+        <is>
+          <t>La Biblia completa está traducida a más de 700 idiomas.</t>
+        </is>
+      </c>
+      <c r="F23" s="61" t="inlineStr">
+        <is>
+          <t>Wycliffe Global Alliance, estadísticas de traducción de la Biblia</t>
+        </is>
+      </c>
+      <c r="G23" s="61" t="inlineStr">
+        <is>
+          <t>Un plan realista</t>
+        </is>
+      </c>
+      <c r="H23" s="61" t="inlineStr">
+        <is>
+          <t>Empezar por Génesis y abandonar en Levítico es común. Mejor un plan corto: un Evangelio, Proverbios, un salmo por día.</t>
+        </is>
+      </c>
+      <c r="I23" s="61" t="inlineStr">
+        <is>
+          <t>Las metas demasiado grandes que se abandonan rápido.</t>
+        </is>
+      </c>
+      <c r="J23" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un plan de 30 días (por ejemplo, un capítulo de Proverbios por día) y marcá cada día cumplido.</t>
+        </is>
+      </c>
+      <c r="K23" s="61" t="inlineStr">
+        <is>
+          <t>Estudiar acompañado</t>
+        </is>
+      </c>
+      <c r="L23" s="61" t="inlineStr">
+        <is>
+          <t>En grupo se aprende más: otros ven lo que uno no ve y se sostiene la constancia.</t>
+        </is>
+      </c>
+      <c r="M23" s="61" t="inlineStr">
+        <is>
+          <t>La fe vivida en soledad, que se enfría fácilmente.</t>
+        </is>
+      </c>
+      <c r="N23" s="61" t="inlineStr">
+        <is>
+          <t>Invitá a un amigo o a tu familia a leer el mismo texto durante la semana y comentarlo el sábado.</t>
+        </is>
+      </c>
+      <c r="O23" s="61" t="inlineStr">
+        <is>
+          <t>Meditar de día y de noche</t>
+        </is>
+      </c>
+      <c r="P23" s="61" t="inlineStr">
+        <is>
+          <t>Meditar es masticar despacio una idea hasta que se vuelve parte de uno.</t>
+        </is>
+      </c>
+      <c r="Q23" s="61" t="inlineStr">
+        <is>
+          <t>La mente saturada de noticias y preocupaciones, sin espacio para el silencio.</t>
+        </is>
+      </c>
+      <c r="R23" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una frase del texto del día y repetila en silencio en momentos de espera: la fila, el tránsito, la pausa del trabajo.</t>
+        </is>
+      </c>
+      <c r="S23" s="61" t="inlineStr">
+        <is>
+          <t>Josué 1:8</t>
+        </is>
+      </c>
+      <c r="T23" s="61" t="inlineStr">
+        <is>
+          <t>Estudia constantemente este libro de instrucción. Medita en él de día y de noche para asegurarte de obedecer todo lo que allí está escrito. Solamente entonces prosperarás y te irá bien en todo lo que hagas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B24" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C24" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="61" t="inlineStr">
+        <is>
+          <t>Escarbar más hondo</t>
+        </is>
+      </c>
+      <c r="E24" s="61" t="inlineStr">
+        <is>
+          <t>Quien estudia sabiendo que después va a tener que enseñarlo a otro aprende y recuerda mejor.</t>
+        </is>
+      </c>
+      <c r="F24" s="61" t="inlineStr">
+        <is>
+          <t>John Nestojko y otros, revista Memory &amp; Cognition, 2014</t>
+        </is>
+      </c>
+      <c r="G24" s="61" t="inlineStr">
+        <is>
+          <t>Descubrir el carácter de Dios</t>
+        </is>
+      </c>
+      <c r="H24" s="61" t="inlineStr">
+        <is>
+          <t>Al estudiar a fondo, la Biblia deja de ser un libro de reglas y muestra a un Dios cercano, paciente y justo.</t>
+        </is>
+      </c>
+      <c r="I24" s="61" t="inlineStr">
+        <is>
+          <t>Imágenes distorsionadas de Dios (castigador o indiferente) que alejan a muchas personas.</t>
+        </is>
+      </c>
+      <c r="J24" s="61" t="inlineStr">
+        <is>
+          <t>Mientras leés, anotá en una columna aparte qué muestra el texto sobre cómo es Dios.</t>
+        </is>
+      </c>
+      <c r="K24" s="61" t="inlineStr">
+        <is>
+          <t>Luz para decidir</t>
+        </is>
+      </c>
+      <c r="L24" s="61" t="inlineStr">
+        <is>
+          <t>La Palabra no responde todo al instante, pero ilumina el siguiente paso.</t>
+        </is>
+      </c>
+      <c r="M24" s="61" t="inlineStr">
+        <is>
+          <t>Decisiones importantes tomadas por impulso, sin reflexión ni consejo.</t>
+        </is>
+      </c>
+      <c r="N24" s="61" t="inlineStr">
+        <is>
+          <t>Antes de una decisión importante, buscá textos sobre el tema y conversalo con alguien de confianza.</t>
+        </is>
+      </c>
+      <c r="O24" s="61" t="inlineStr">
+        <is>
+          <t>Enseñar lo que aprendés</t>
+        </is>
+      </c>
+      <c r="P24" s="61" t="inlineStr">
+        <is>
+          <t>Compartir lo que descubriste fija el aprendizaje y bendice a otros.</t>
+        </is>
+      </c>
+      <c r="Q24" s="61" t="inlineStr">
+        <is>
+          <t>Padres que delegan toda la formación espiritual de sus hijos en la iglesia o la escuela.</t>
+        </is>
+      </c>
+      <c r="R24" s="61" t="inlineStr">
+        <is>
+          <t>Contá en la cena de hoy algo que aprendiste de la Biblia esta semana. Corto y sencillo.</t>
+        </is>
+      </c>
+      <c r="S24" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 119:105</t>
+        </is>
+      </c>
+      <c r="T24" s="61" t="inlineStr">
+        <is>
+          <t>Tu palabra es una lámpara que guía mis pies y una luz para mi camino.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="61" t="n">
+        <v>4</v>
+      </c>
+      <c r="B25" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C25" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="61" t="inlineStr">
+        <is>
+          <t>Buscar de todo corazón</t>
+        </is>
+      </c>
+      <c r="E25" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 119 es el capítulo más largo de la Biblia: 176 versículos dedicados casi por completo a la Palabra de Dios.</t>
+        </is>
+      </c>
+      <c r="F25" s="61" t="inlineStr">
+        <is>
+          <t>Biblia, Salmo 119</t>
+        </is>
+      </c>
+      <c r="G25" s="61" t="inlineStr">
+        <is>
+          <t>La búsqueda sincera</t>
+        </is>
+      </c>
+      <c r="H25" s="61" t="inlineStr">
+        <is>
+          <t>Dios no se esconde de quien lo busca de verdad. El estudio es una forma concreta de buscarlo.</t>
+        </is>
+      </c>
+      <c r="I25" s="61" t="inlineStr">
+        <is>
+          <t>La fe superficial, que se queda en costumbres sin una relación personal.</t>
+        </is>
+      </c>
+      <c r="J25" s="61" t="inlineStr">
+        <is>
+          <t>Este fin de semana, reservá media hora tranquila solo para leer y orar, sin celular.</t>
+        </is>
+      </c>
+      <c r="K25" s="61" t="inlineStr">
+        <is>
+          <t>Constancia en tiempos secos</t>
+        </is>
+      </c>
+      <c r="L25" s="61" t="inlineStr">
+        <is>
+          <t>Habrá días en que leer no emocione. La diligencia es seguir igual, porque el fruto llega con el tiempo.</t>
+        </is>
+      </c>
+      <c r="M25" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar todo lo valioso apenas deja de ser entretenido.</t>
+        </is>
+      </c>
+      <c r="N25" s="61" t="inlineStr">
+        <is>
+          <t>Si te cuesta, cambiá el formato: escuchá la Biblia en audio mientras caminás o viajás.</t>
+        </is>
+      </c>
+      <c r="O25" s="61" t="inlineStr">
+        <is>
+          <t>Un legado para los que vienen</t>
+        </is>
+      </c>
+      <c r="P25" s="61" t="inlineStr">
+        <is>
+          <t>Una Biblia gastada y subrayada es una herencia para hijos y nietos.</t>
+        </is>
+      </c>
+      <c r="Q25" s="61" t="inlineStr">
+        <is>
+          <t>Generaciones que crecen sin referencias de fe en casa.</t>
+        </is>
+      </c>
+      <c r="R25" s="61" t="inlineStr">
+        <is>
+          <t>Regalá una Biblia o un devocional a un joven de tu familia con una dedicatoria escrita por vos.</t>
+        </is>
+      </c>
+      <c r="S25" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías 29:13</t>
+        </is>
+      </c>
+      <c r="T25" s="61" t="inlineStr">
+        <is>
+          <t>Si me buscan de todo corazón, podrán encontrarme.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mensajero: «Día a día» une versículos y guion, con el versículo como base
- Una sola sección con pestañas de domingo a sábado y su fecha.
- Domingo: versículo de la semana e historia ilustrativa.
- Lunes a sábado: el versículo del día es la base; sus 3 puntos son los
  3 puntos del guion (desarrollo, problemática, en la práctica).
- Hoja «Guiones 2027» simplificada (sin títulos de punto ni cierre);
  guiones de enero reescritos sobre los versículos de cada día.
- El prompt de la semana incluye los versículos y puntos de cada día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -19124,29 +19124,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
-    <col width="40" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
-    <col width="40" customWidth="1" min="17" max="17"/>
-    <col width="40" customWidth="1" min="18" max="18"/>
-    <col width="40" customWidth="1" min="19" max="19"/>
-    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19162,92 +19156,62 @@
       </c>
       <c r="C1" s="60" t="inlineStr">
         <is>
-          <t>Subtema</t>
+          <t>Titulo</t>
         </is>
       </c>
       <c r="D1" s="60" t="inlineStr">
         <is>
-          <t>Titulo</t>
+          <t>Dato curioso</t>
         </is>
       </c>
       <c r="E1" s="60" t="inlineStr">
         <is>
-          <t>Dato curioso</t>
+          <t>Fuente dato</t>
         </is>
       </c>
       <c r="F1" s="60" t="inlineStr">
         <is>
-          <t>Fuente dato</t>
+          <t>Desarrollo 1</t>
         </is>
       </c>
       <c r="G1" s="60" t="inlineStr">
         <is>
-          <t>Punto 1</t>
+          <t>Problematica 1</t>
         </is>
       </c>
       <c r="H1" s="60" t="inlineStr">
         <is>
-          <t>Desarrollo 1</t>
+          <t>Solucion 1</t>
         </is>
       </c>
       <c r="I1" s="60" t="inlineStr">
         <is>
-          <t>Problematica 1</t>
+          <t>Desarrollo 2</t>
         </is>
       </c>
       <c r="J1" s="60" t="inlineStr">
         <is>
-          <t>Solucion 1</t>
+          <t>Problematica 2</t>
         </is>
       </c>
       <c r="K1" s="60" t="inlineStr">
         <is>
-          <t>Punto 2</t>
+          <t>Solucion 2</t>
         </is>
       </c>
       <c r="L1" s="60" t="inlineStr">
         <is>
-          <t>Desarrollo 2</t>
+          <t>Desarrollo 3</t>
         </is>
       </c>
       <c r="M1" s="60" t="inlineStr">
         <is>
-          <t>Problematica 2</t>
+          <t>Problematica 3</t>
         </is>
       </c>
       <c r="N1" s="60" t="inlineStr">
         <is>
-          <t>Solucion 2</t>
-        </is>
-      </c>
-      <c r="O1" s="60" t="inlineStr">
-        <is>
-          <t>Punto 3</t>
-        </is>
-      </c>
-      <c r="P1" s="60" t="inlineStr">
-        <is>
-          <t>Desarrollo 3</t>
-        </is>
-      </c>
-      <c r="Q1" s="60" t="inlineStr">
-        <is>
-          <t>Problematica 3</t>
-        </is>
-      </c>
-      <c r="R1" s="60" t="inlineStr">
-        <is>
           <t>Solucion 3</t>
-        </is>
-      </c>
-      <c r="S1" s="60" t="inlineStr">
-        <is>
-          <t>Cierre cita (NTV)</t>
-        </is>
-      </c>
-      <c r="T1" s="60" t="inlineStr">
-        <is>
-          <t>Cierre texto</t>
         </is>
       </c>
     </row>
@@ -19260,92 +19224,64 @@
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C2" s="61" t="n">
-        <v>1</v>
+      <c r="C2" s="61" t="inlineStr">
+        <is>
+          <t>Tu cuerpo no es tu enemigo</t>
+        </is>
       </c>
       <c r="D2" s="61" t="inlineStr">
         <is>
-          <t>Tu cuerpo no es tu enemigo</t>
+          <t>Casi 1 de cada 3 adultos en el mundo (31 %) no hace la actividad física mínima recomendada.</t>
         </is>
       </c>
       <c r="E2" s="61" t="inlineStr">
         <is>
-          <t>Casi 1 de cada 3 adultos en el mundo (31 %) no hace la actividad física mínima recomendada para cuidar su salud.</t>
+          <t>Organización Mundial de la Salud, 2024</t>
         </is>
       </c>
       <c r="F2" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, informe sobre actividad física, 2024</t>
+          <t>Presentar el cuerpo es ponerlo al servicio de algo más grande que la imagen o el rendimiento: cuidarlo para amar, trabajar y servir mejor.</t>
         </is>
       </c>
       <c r="G2" s="61" t="inlineStr">
         <is>
-          <t>Del maltrato al cuidado</t>
+          <t>Jornadas largas en el campo, la obra o la oficina sin pausas ni agua, que terminan en lesiones y agotamiento.</t>
         </is>
       </c>
       <c r="H2" s="61" t="inlineStr">
         <is>
-          <t>Muchos tratan al cuerpo como una máquina que debe rendir sin parar: comemos de pie, dormimos poco y solo paramos cuando algo duele. Cuidarlo no es vanidad, es administrar bien lo que se nos confió.</t>
+          <t>Programá dos pausas cortas en tu jornada: tomá agua, estirate cinco minutos y volvé. Proponelo también a tu equipo.</t>
         </is>
       </c>
       <c r="I2" s="61" t="inlineStr">
         <is>
-          <t>Jornadas largas de trabajo en el campo, la obra o la oficina sin pausas ni agua, que terminan en lesiones y agotamiento.</t>
+          <t>Adorar no es solo cantar. También es cómo vivimos lo cotidiano: cómo comemos, cómo dormimos, cómo tratamos el cuerpo que se nos confió.</t>
         </is>
       </c>
       <c r="J2" s="61" t="inlineStr">
         <is>
-          <t>Programá dos pausas cortas en tu jornada: tomá agua, estirate cinco minutos y volvé. Si trabajás con otros, proponelo para todo el equipo.</t>
+          <t>La presión de las redes por un cuerpo perfecto, que lleva a dietas extremas, sobre todo en adolescentes.</t>
         </is>
       </c>
       <c r="K2" s="61" t="inlineStr">
         <is>
-          <t>Ni ídolo ni enemigo</t>
+          <t>En casa, hablá del cuerpo por lo que hace (caminar, abrazar, trabajar) y no solo por cómo se ve.</t>
         </is>
       </c>
       <c r="L2" s="61" t="inlineStr">
         <is>
-          <t>Hay quien vive obsesionado con la imagen y quien se descuida por completo. Las dos actitudes ponen al cuerpo en el centro equivocado. El cuerpo es un medio para servir, amar y trabajar, no el fin.</t>
+          <t>Lo físico y lo espiritual no viven separados: un cuerpo agotado afecta el ánimo, la paciencia y hasta la fe.</t>
         </is>
       </c>
       <c r="M2" s="61" t="inlineStr">
         <is>
-          <t>La presión de las redes por un cuerpo perfecto, que lleva a dietas extremas, sobre todo en adolescentes.</t>
+          <t>El consumo excesivo de alcohol los fines de semana, que muchos ven como algo normal.</t>
         </is>
       </c>
       <c r="N2" s="61" t="inlineStr">
         <is>
-          <t>En casa, hablá del cuerpo por lo que hace (caminar, abrazar, trabajar) y no solo por cómo se ve. Elogiá hábitos, no medidas.</t>
-        </is>
-      </c>
-      <c r="O2" s="61" t="inlineStr">
-        <is>
-          <t>Un templo habitado</t>
-        </is>
-      </c>
-      <c r="P2" s="61" t="inlineStr">
-        <is>
-          <t>Para la fe cristiana el cuerpo tiene dignidad: es lugar donde Dios habita. Esa idea cambia la pregunta de "¿cómo me veo?" a "¿cómo lo cuido para servir mejor?".</t>
-        </is>
-      </c>
-      <c r="Q2" s="61" t="inlineStr">
-        <is>
-          <t>El consumo excesivo de alcohol los fines de semana, que muchos ven como algo normal.</t>
-        </is>
-      </c>
-      <c r="R2" s="61" t="inlineStr">
-        <is>
           <t>Elegí un cambio concreto para este fin de semana: menos alcohol, más agua y una salida al aire libre con tu familia.</t>
-        </is>
-      </c>
-      <c r="S2" s="61" t="inlineStr">
-        <is>
-          <t>1 Corintios 6:19-20</t>
-        </is>
-      </c>
-      <c r="T2" s="61" t="inlineStr">
-        <is>
-          <t>¿No se dan cuenta de que su cuerpo es el templo del Espíritu Santo, quien vive en ustedes y les fue dado por Dios? Ustedes no se pertenecen a sí mismos, porque Dios los compró a un alto precio. Por lo tanto, honren a Dios con su cuerpo.</t>
         </is>
       </c>
     </row>
@@ -19358,52 +19294,54 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C3" s="61" t="n">
-        <v>1</v>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>Cuidarte también es gratitud</t>
+        </is>
       </c>
       <c r="D3" s="61" t="inlineStr">
         <is>
-          <t>Cuidarte también es gratitud</t>
+          <t>El 85 % de las mujeres deja de participar en actividades importantes de su vida cuando no se siente bien con su aspecto.</t>
         </is>
       </c>
       <c r="E3" s="61" t="inlineStr">
         <is>
-          <t>El 85 % de las mujeres deja de participar en actividades importantes de su vida cuando no se siente bien con su aspecto.</t>
+          <t>Dove, Global Beauty and Confidence Report, 2016</t>
         </is>
       </c>
       <c r="F3" s="61" t="inlineStr">
         <is>
-          <t>Dove, Global Beauty and Confidence Report, 2016</t>
+          <t>A Dios no le es indiferente tu salud. Desear el bien de alguien incluye desear que su cuerpo esté bien.</t>
         </is>
       </c>
       <c r="G3" s="61" t="inlineStr">
         <is>
-          <t>Mirarte con otros ojos</t>
+          <t>Muchas personas postergan el control médico hasta que el problema ya es grave.</t>
         </is>
       </c>
       <c r="H3" s="61" t="inlineStr">
         <is>
-          <t>Lo que pensamos de nuestro cuerpo influye en cómo lo tratamos. Quien se desprecia se descuida; quien se sabe valioso se cuida.</t>
+          <t>Agendá hoy un control básico (presión, glucosa) en tu unidad de salud familiar más cercana.</t>
         </is>
       </c>
       <c r="I3" s="61" t="inlineStr">
         <is>
+          <t>El bienestar es integral: cuerpo, mente, relaciones y fe. Cuando una parte se descuida, las demás lo sienten.</t>
+        </is>
+      </c>
+      <c r="J3" s="61" t="inlineStr">
+        <is>
           <t>Jóvenes que se aíslan o abandonan el deporte por vergüenza de su cuerpo.</t>
         </is>
       </c>
-      <c r="J3" s="61" t="inlineStr">
+      <c r="K3" s="61" t="inlineStr">
         <is>
           <t>Si tenés hijos o sobrinos, acompañalos a una actividad física sin hablar de peso: el objetivo es disfrutar y moverse.</t>
         </is>
       </c>
-      <c r="K3" s="61" t="inlineStr">
-        <is>
-          <t>Pequeñas decisiones diarias</t>
-        </is>
-      </c>
       <c r="L3" s="61" t="inlineStr">
         <is>
-          <t>Cuidarse no exige un gimnasio caro. Exige decisiones pequeñas y repetidas: qué como, cuánto me muevo, a qué hora me acuesto.</t>
+          <t>La fe también se nota en los hábitos: en lo que ponemos en la mesa cada día.</t>
         </is>
       </c>
       <c r="M3" s="61" t="inlineStr">
@@ -19414,36 +19352,6 @@
       <c r="N3" s="61" t="inlineStr">
         <is>
           <t>Cociná una vez más por semana en casa y cambiá la gaseosa del almuerzo por agua o tereré sin azúcar.</t>
-        </is>
-      </c>
-      <c r="O3" s="61" t="inlineStr">
-        <is>
-          <t>El cuerpo como ofrenda</t>
-        </is>
-      </c>
-      <c r="P3" s="61" t="inlineStr">
-        <is>
-          <t>Agradecer por el cuerpo es también usarlo bien. Cada vez que lo cuidás, decís "gracias" con hechos.</t>
-        </is>
-      </c>
-      <c r="Q3" s="61" t="inlineStr">
-        <is>
-          <t>Muchas personas postergan el control médico hasta que el problema ya es grave.</t>
-        </is>
-      </c>
-      <c r="R3" s="61" t="inlineStr">
-        <is>
-          <t>Agendá hoy un control básico (presión, glucosa) en tu unidad de salud familiar más cercana.</t>
-        </is>
-      </c>
-      <c r="S3" s="61" t="inlineStr">
-        <is>
-          <t>Salmo 139:14</t>
-        </is>
-      </c>
-      <c r="T3" s="61" t="inlineStr">
-        <is>
-          <t>¡Gracias por hacerme tan maravillosamente complejo! Tu fino trabajo es maravilloso, lo sé muy bien.</t>
         </is>
       </c>
     </row>
@@ -19456,92 +19364,64 @@
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="C4" s="61" t="n">
-        <v>2</v>
+      <c r="C4" s="61" t="inlineStr">
+        <is>
+          <t>Hábitos pequeños, energía grande</t>
+        </is>
       </c>
       <c r="D4" s="61" t="inlineStr">
         <is>
-          <t>Hábitos pequeños, energía grande</t>
+          <t>Un hábito nuevo tarda en promedio 66 días en volverse automático; en el estudio el rango fue de 18 a 254 días.</t>
         </is>
       </c>
       <c r="E4" s="61" t="inlineStr">
         <is>
-          <t>Un hábito nuevo tarda en promedio 66 días en volverse automático; en el estudio el rango fue de 18 a 254 días.</t>
+          <t>Lally y otros, University College London, European Journal of Social Psychology, 2010</t>
         </is>
       </c>
       <c r="F4" s="61" t="inlineStr">
         <is>
-          <t>Lally y otros, University College London, European Journal of Social Psychology, 2010</t>
+          <t>Moverse cuida el cuerpo, aunque no lo es todo. Y no hace falta empezar en grande: cinco minutos de caminata ya cuentan.</t>
         </is>
       </c>
       <c r="G4" s="61" t="inlineStr">
         <is>
-          <t>Empezar chico</t>
+          <t>Los propósitos de año nuevo que se abandonan en enero: gimnasios llenos la primera semana y vacíos en febrero.</t>
         </is>
       </c>
       <c r="H4" s="61" t="inlineStr">
         <is>
-          <t>Los grandes cambios fracasan porque piden demasiado de golpe. Un hábito empieza tan pequeño que no se puede fallar: cinco minutos de caminata, un vaso de agua al despertar.</t>
+          <t>Elegí un solo hábito para esta semana y ponelo en tu agenda con hora fija. Uno solo.</t>
         </is>
       </c>
       <c r="I4" s="61" t="inlineStr">
         <is>
-          <t>Los propósitos de año nuevo que se abandonan en enero: gimnasios llenos la primera semana y vacíos en febrero.</t>
+          <t>Hay hábitos del alma que sostienen cuando el cuerpo falla: orar, agradecer, perdonar.</t>
         </is>
       </c>
       <c r="J4" s="61" t="inlineStr">
         <is>
-          <t>Elegí un solo hábito para esta semana y ponelo en tu agenda con hora fija. Uno solo.</t>
+          <t>Personas en forma por fuera pero agotadas por dentro, con ansiedad que nadie ve.</t>
         </is>
       </c>
       <c r="K4" s="61" t="inlineStr">
         <is>
-          <t>Agua, movimiento y sol</t>
+          <t>Al despertar, antes del celular, tomate cinco minutos de silencio para agradecer tres cosas.</t>
         </is>
       </c>
       <c r="L4" s="61" t="inlineStr">
         <is>
-          <t>Tres cosas simples sostienen la energía del día: tomar agua, moverse un poco y recibir luz natural por la mañana.</t>
+          <t>Ni obsesión ni descuido: cada cosa en su medida. La constancia vale más que la intensidad.</t>
         </is>
       </c>
       <c r="M4" s="61" t="inlineStr">
         <is>
-          <t>Trabajar muchas horas sentado y sin hidratarse, sobre todo con el calor del verano paraguayo.</t>
+          <t>La cultura del "todo o nada", que hace abandonar ante el primer tropiezo.</t>
         </is>
       </c>
       <c r="N4" s="61" t="inlineStr">
         <is>
-          <t>Tené una botella de agua a la vista y levantate cada hora a caminar dos minutos.</t>
-        </is>
-      </c>
-      <c r="O4" s="61" t="inlineStr">
-        <is>
-          <t>Ser constante, no perfecto</t>
-        </is>
-      </c>
-      <c r="P4" s="61" t="inlineStr">
-        <is>
-          <t>Fallar un día no arruina el hábito; abandonarlo sí. La constancia vale más que la intensidad.</t>
-        </is>
-      </c>
-      <c r="Q4" s="61" t="inlineStr">
-        <is>
-          <t>La cultura del "todo o nada", que hace que muchos abandonen ante el primer tropiezo.</t>
-        </is>
-      </c>
-      <c r="R4" s="61" t="inlineStr">
-        <is>
           <t>Si fallaste ayer, hoy hacé la versión mínima del hábito. La regla: nunca fallar dos días seguidos.</t>
-        </is>
-      </c>
-      <c r="S4" s="61" t="inlineStr">
-        <is>
-          <t>Gálatas 6:9</t>
-        </is>
-      </c>
-      <c r="T4" s="61" t="inlineStr">
-        <is>
-          <t>Así que no nos cansemos de hacer el bien. A su debido tiempo, cosecharemos numerosas bendiciones si no nos damos por vencidos.</t>
         </is>
       </c>
     </row>
@@ -19554,52 +19434,54 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C5" s="61" t="n">
-        <v>2</v>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>Una obra que merece cuidado</t>
+        </is>
       </c>
       <c r="D5" s="61" t="inlineStr">
         <is>
-          <t>El orden que da energía</t>
+          <t>El corazón late alrededor de 100.000 veces por día, sin que tengamos que pensar en ello.</t>
         </is>
       </c>
       <c r="E5" s="61" t="inlineStr">
         <is>
-          <t>Mejorar apenas un 1 % cada día durante un año te deja unas 37 veces mejor que al comienzo.</t>
+          <t>American Heart Association</t>
         </is>
       </c>
       <c r="F5" s="61" t="inlineStr">
         <is>
-          <t>James Clear, Hábitos atómicos, 2018</t>
+          <t>El cuerpo trabaja todo el día sin que se lo pidamos. Es una obra formidable, no una máquina descartable.</t>
         </is>
       </c>
       <c r="G5" s="61" t="inlineStr">
         <is>
-          <t>Ordenar el día</t>
+          <t>Trabajar muchas horas sentado y sin hidratarse, sobre todo con el calor del verano paraguayo.</t>
         </is>
       </c>
       <c r="H5" s="61" t="inlineStr">
         <is>
-          <t>La falta de energía muchas veces es falta de orden: horarios cambiados, comidas salteadas, pendientes sin anotar. Ordenar es cuidar.</t>
+          <t>Tené una botella de agua a la vista y levantate cada hora a caminar dos minutos.</t>
         </is>
       </c>
       <c r="I5" s="61" t="inlineStr">
         <is>
+          <t>Lo que valorás, lo cuidás. Ordenar el día es una forma concreta de cuidar el cuerpo.</t>
+        </is>
+      </c>
+      <c r="J5" s="61" t="inlineStr">
+        <is>
           <t>Familias sin horarios, donde se come a cualquier hora y nadie sabe qué toca hacer.</t>
         </is>
       </c>
-      <c r="J5" s="61" t="inlineStr">
+      <c r="K5" s="61" t="inlineStr">
         <is>
           <t>Fijá tres horas en casa: despertar, almuerzo y cena. Respetarlas una semana ya cambia el ánimo de todos.</t>
         </is>
       </c>
-      <c r="K5" s="61" t="inlineStr">
-        <is>
-          <t>Preparar con anticipación</t>
-        </is>
-      </c>
       <c r="L5" s="61" t="inlineStr">
         <is>
-          <t>Lo que se prepara la noche anterior (ropa, comida, agenda) ahorra estrés por la mañana.</t>
+          <t>Respetar el diseño es no abusar: ni excesos, ni desvelos, ni correr todo el día sin comer.</t>
         </is>
       </c>
       <c r="M5" s="61" t="inlineStr">
@@ -19610,36 +19492,6 @@
       <c r="N5" s="61" t="inlineStr">
         <is>
           <t>Antes de dormir, dejá listo lo de mañana: ropa, merienda y las tres tareas principales anotadas.</t>
-        </is>
-      </c>
-      <c r="O5" s="61" t="inlineStr">
-        <is>
-          <t>Fidelidad en lo pequeño</t>
-        </is>
-      </c>
-      <c r="P5" s="61" t="inlineStr">
-        <is>
-          <t>Los hábitos chicos muestran quiénes somos. Quien es fiel en lo poco aprende a ser fiel en lo mucho.</t>
-        </is>
-      </c>
-      <c r="Q5" s="61" t="inlineStr">
-        <is>
-          <t>La idea de que los cambios importantes solo llegan con grandes oportunidades.</t>
-        </is>
-      </c>
-      <c r="R5" s="61" t="inlineStr">
-        <is>
-          <t>Escribí en un papel un pequeño compromiso diario y pegalo donde lo veas. Revisalo el domingo.</t>
-        </is>
-      </c>
-      <c r="S5" s="61" t="inlineStr">
-        <is>
-          <t>Lucas 16:10</t>
-        </is>
-      </c>
-      <c r="T5" s="61" t="inlineStr">
-        <is>
-          <t>Si son fieles en las cosas pequeñas, serán fieles en las grandes; pero si son deshonestos en las cosas pequeñas, no actuarán con honradez en las responsabilidades más grandes.</t>
         </is>
       </c>
     </row>
@@ -19652,92 +19504,64 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="C6" s="61" t="n">
-        <v>3</v>
+      <c r="C6" s="61" t="inlineStr">
+        <is>
+          <t>Descansar no es perder el tiempo</t>
+        </is>
       </c>
       <c r="D6" s="61" t="inlineStr">
         <is>
-          <t>Descansar no es perder el tiempo</t>
+          <t>Uno de cada tres adultos no duerme las horas que necesita.</t>
         </is>
       </c>
       <c r="E6" s="61" t="inlineStr">
         <is>
-          <t>Uno de cada tres adultos no duerme las horas que necesita.</t>
+          <t>Centros para el Control y la Prevención de Enfermedades (CDC) de EE. UU., 2016</t>
         </is>
       </c>
       <c r="F6" s="61" t="inlineStr">
         <is>
-          <t>Centros para el Control y la Prevención de Enfermedades (CDC) de Estados Unidos, 2016</t>
+          <t>Si Dios mismo descansó, descansar no es pereza. Es parte de una vida bien ordenada.</t>
         </is>
       </c>
       <c r="G6" s="61" t="inlineStr">
         <is>
-          <t>El descanso es parte del diseño</t>
+          <t>La cultura de "estar siempre ocupado" como señal de éxito, que normaliza el agotamiento.</t>
         </is>
       </c>
       <c r="H6" s="61" t="inlineStr">
         <is>
-          <t>Dios mismo descansó al séptimo día. El descanso no es premio para los que terminan todo: es una necesidad para seguir.</t>
+          <t>Elegí un momento fijo de la semana sin trabajo ni pendientes y defendelo como una cita importante.</t>
         </is>
       </c>
       <c r="I6" s="61" t="inlineStr">
         <is>
-          <t>La cultura de "estar siempre ocupado" como señal de éxito, que normaliza el agotamiento.</t>
+          <t>El sueño repara el cuerpo y ordena la mente. Dormir poco afecta el humor, la memoria y la salud.</t>
         </is>
       </c>
       <c r="J6" s="61" t="inlineStr">
         <is>
-          <t>Elegí un momento fijo de la semana sin trabajo ni pendientes, y defendelo como una cita importante.</t>
+          <t>Adultos y jóvenes que duermen menos de seis horas por estar en el celular hasta tarde.</t>
         </is>
       </c>
       <c r="K6" s="61" t="inlineStr">
         <is>
-          <t>Dormir bien</t>
+          <t>Poné una alarma para irte a dormir, no solo para despertarte. Media hora antes, celular lejos de la cama.</t>
         </is>
       </c>
       <c r="L6" s="61" t="inlineStr">
         <is>
-          <t>El sueño repara el cuerpo y ordena la mente. Dormir poco afecta el humor, la memoria y la salud.</t>
+          <t>Trabajo y descanso se alternan. Quien nunca para, tarde o temprano se rompe.</t>
         </is>
       </c>
       <c r="M6" s="61" t="inlineStr">
         <is>
-          <t>Adultos y jóvenes que duermen menos de seis horas por estar en el celular hasta tarde.</t>
+          <t>El estrés por las deudas y el trabajo, que quita el sueño a muchas familias.</t>
         </is>
       </c>
       <c r="N6" s="61" t="inlineStr">
         <is>
-          <t>Poné una alarma para irte a dormir, no solo para despertarte. Media hora antes, celular lejos de la cama.</t>
-        </is>
-      </c>
-      <c r="O6" s="61" t="inlineStr">
-        <is>
-          <t>Descansar en confianza</t>
-        </is>
-      </c>
-      <c r="P6" s="61" t="inlineStr">
-        <is>
-          <t>Hay un cansancio que no se va durmiendo: es la ansiedad de querer controlarlo todo. Descansar también es confiar.</t>
-        </is>
-      </c>
-      <c r="Q6" s="61" t="inlineStr">
-        <is>
-          <t>El estrés por las deudas y el trabajo, que quita el sueño a muchas familias.</t>
-        </is>
-      </c>
-      <c r="R6" s="61" t="inlineStr">
-        <is>
-          <t>Antes de dormir, anotá lo que te preocupa y lo que vas a hacer mañana al respecto. Luego, entregalo en oración.</t>
-        </is>
-      </c>
-      <c r="S6" s="61" t="inlineStr">
-        <is>
-          <t>Salmo 127:2</t>
-        </is>
-      </c>
-      <c r="T6" s="61" t="inlineStr">
-        <is>
-          <t>Es inútil que te esfuerces tanto, desde temprano en la mañana hasta tarde en la noche, y te preocupes por conseguir alimento; porque Dios da descanso a sus amados.</t>
+          <t>Antes de dormir, anotá lo que te preocupa y lo que vas a hacer mañana al respecto. Después, entregalo en oración.</t>
         </is>
       </c>
     </row>
@@ -19750,92 +19574,64 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="C7" s="61" t="n">
-        <v>3</v>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>Un fin de semana que recarga</t>
+        </is>
       </c>
       <c r="D7" s="61" t="inlineStr">
         <is>
-          <t>Un fin de semana que recarga</t>
+          <t>Leer en una pantalla antes de dormir retrasa la melatonina, cuesta más dormirse y se amanece menos alerta.</t>
         </is>
       </c>
       <c r="E7" s="61" t="inlineStr">
         <is>
-          <t>Leer en una pantalla antes de dormir retrasa la liberación de melatonina, hace que cueste más conciliar el sueño y reduce el estado de alerta a la mañana siguiente.</t>
+          <t>Chang y otros, Harvard Medical School, revista PNAS, 2015</t>
         </is>
       </c>
       <c r="F7" s="61" t="inlineStr">
         <is>
-          <t>Chang y otros, Harvard Medical School, revista PNAS, 2015</t>
+          <t>La sabiduría se ve en decisiones simples: cómo usamos el tiempo libre. Pasar el sábado frente a una pantalla no siempre descansa.</t>
         </is>
       </c>
       <c r="G7" s="61" t="inlineStr">
         <is>
-          <t>Descanso real, no solo pantalla</t>
+          <t>Familias que comparten la casa pero cada uno está en su celular.</t>
         </is>
       </c>
       <c r="H7" s="61" t="inlineStr">
         <is>
-          <t>Pasar el sábado frente a una pantalla no siempre descansa. El descanso real incluye silencio, naturaleza y personas.</t>
+          <t>Proponé una hora sin pantallas este fin de semana: una caminata, un tereré en familia, un juego de mesa.</t>
         </is>
       </c>
       <c r="I7" s="61" t="inlineStr">
         <is>
-          <t>Familias que comparten la casa pero cada uno está en su celular.</t>
+          <t>Apartarse del mal también es evitar los excesos que dañan: alcohol, peleas, noches sin dormir.</t>
         </is>
       </c>
       <c r="J7" s="61" t="inlineStr">
         <is>
-          <t>Proponé una hora sin pantallas este fin de semana: una caminata, un mate o tereré en familia, un juego de mesa.</t>
+          <t>Los accidentes de tránsito de los fines de semana, muchas veces ligados al alcohol.</t>
         </is>
       </c>
       <c r="K7" s="61" t="inlineStr">
         <is>
-          <t>Descansar juntos</t>
+          <t>Si vas a tomar, no manejes. Acordá antes quién conduce o volvé en otro medio.</t>
         </is>
       </c>
       <c r="L7" s="61" t="inlineStr">
         <is>
-          <t>El descanso compartido fortalece los vínculos. Comer sin apuro, conversar y reír también es cuidar la salud.</t>
+          <t>El alma también se cansa. Soltar cargas, perdonar y reconciliarse alivia hasta el cuerpo.</t>
         </is>
       </c>
       <c r="M7" s="61" t="inlineStr">
         <is>
-          <t>La soledad de muchos adultos mayores, que pasan el fin de semana sin visitas.</t>
+          <t>El agotamiento emocional que muchos esconden detrás de una vida activa.</t>
         </is>
       </c>
       <c r="N7" s="61" t="inlineStr">
         <is>
-          <t>Visitá o llamá este fin de semana a un familiar mayor. Descansar también puede ser acompañar.</t>
-        </is>
-      </c>
-      <c r="O7" s="61" t="inlineStr">
-        <is>
-          <t>Descanso para el alma</t>
-        </is>
-      </c>
-      <c r="P7" s="61" t="inlineStr">
-        <is>
-          <t>El cuerpo descansa durmiendo; el alma descansa cuando suelta cargas que no le corresponden. Jesús invita a los cansados a encontrar descanso en él.</t>
-        </is>
-      </c>
-      <c r="Q7" s="61" t="inlineStr">
-        <is>
-          <t>El agotamiento emocional que muchos esconden detrás de una vida activa.</t>
-        </is>
-      </c>
-      <c r="R7" s="61" t="inlineStr">
-        <is>
-          <t>Tomate diez minutos para revisar la semana: qué te cansó, qué te dio vida y qué vas a cambiar la próxima.</t>
-        </is>
-      </c>
-      <c r="S7" s="61" t="inlineStr">
-        <is>
-          <t>Mateo 11:28</t>
-        </is>
-      </c>
-      <c r="T7" s="61" t="inlineStr">
-        <is>
-          <t>Luego dijo Jesús: «Vengan a mí todos los que están cansados y llevan cargas pesadas, y yo les daré descanso».</t>
+          <t>Tomate diez minutos para revisar la semana: qué te cansó, qué te dio vida y qué vas a cambiar.</t>
         </is>
       </c>
     </row>
@@ -19848,92 +19644,64 @@
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C8" s="61" t="n">
-        <v>1</v>
+      <c r="C8" s="61" t="inlineStr">
+        <is>
+          <t>Lo que se siembra, se cosecha</t>
+        </is>
       </c>
       <c r="D8" s="61" t="inlineStr">
         <is>
-          <t>Lo que se siembra, se cosecha</t>
+          <t>Paraguay está entre los cinco mayores exportadores de soja del mundo.</t>
         </is>
       </c>
       <c r="E8" s="61" t="inlineStr">
         <is>
-          <t>Paraguay está entre los cinco mayores exportadores de soja del mundo.</t>
+          <t>Departamento de Agricultura de EE. UU. (USDA), informes de oleaginosas</t>
         </is>
       </c>
       <c r="F8" s="61" t="inlineStr">
         <is>
-          <t>Departamento de Agricultura de Estados Unidos (USDA), informes de mercado mundial de oleaginosas</t>
+          <t>Nadie espera cosechar maíz si sembró poroto. Lo que hacemos hoy con el tiempo, las palabras y el dinero es la semilla de mañana.</t>
         </is>
       </c>
       <c r="G8" s="61" t="inlineStr">
         <is>
-          <t>La ley de la siembra</t>
+          <t>La cultura de la plata fácil: apuestas, préstamos rápidos y negocios dudosos que prometen cosechar sin sembrar.</t>
         </is>
       </c>
       <c r="H8" s="61" t="inlineStr">
         <is>
-          <t>En el campo nadie espera cosechar maíz si sembró poroto. La vida funciona igual: lo que hacemos hoy con el tiempo, las palabras y el dinero es la semilla de lo que vamos a tener mañana.</t>
+          <t>Anotá esta semana tres semillas concretas: un hábito, una relación y un ahorro pequeño que quieras empezar.</t>
         </is>
       </c>
       <c r="I8" s="61" t="inlineStr">
         <is>
-          <t>La cultura de la plata fácil: apuestas, préstamos rápidos y negocios dudosos que prometen cosechar sin sembrar.</t>
+          <t>La ley de la siembra vale en el campo, en la familia, en la salud y en la fe. Los valores son la mejor semilla.</t>
         </is>
       </c>
       <c r="J8" s="61" t="inlineStr">
         <is>
-          <t>Anotá esta semana tres "semillas" concretas: un hábito, una relación y un ahorro pequeño que quieras empezar a sembrar.</t>
+          <t>Jóvenes que aprenden de las redes que el atajo vale más que el esfuerzo.</t>
         </is>
       </c>
       <c r="K8" s="61" t="inlineStr">
         <is>
-          <t>Elegir buena semilla</t>
+          <t>Contale a un joven de tu familia cómo conseguiste algo con trabajo y paciencia. Las historias reales siembran más que los consejos.</t>
         </is>
       </c>
       <c r="L8" s="61" t="inlineStr">
         <is>
-          <t>El productor sabe que la calidad de la semilla define la cosecha. En la vida, la buena semilla son los valores: honestidad, trabajo, palabra cumplida.</t>
+          <t>En el campo los atajos se pagan caro: lo que se hace mal para ganar tiempo vuelve como pérdida.</t>
         </is>
       </c>
       <c r="M8" s="61" t="inlineStr">
         <is>
-          <t>Jóvenes que aprenden de las redes que el atajo vale más que el esfuerzo.</t>
+          <t>Aplicaciones de agroquímicos sin cuidado para ganar tiempo, que dañan a vecinos, al agua y al suelo.</t>
         </is>
       </c>
       <c r="N8" s="61" t="inlineStr">
         <is>
-          <t>Contale a un joven de tu familia cómo conseguiste algo con trabajo y paciencia. Las historias reales siembran más que los consejos.</t>
-        </is>
-      </c>
-      <c r="O8" s="61" t="inlineStr">
-        <is>
-          <t>Sembrar con fe</t>
-        </is>
-      </c>
-      <c r="P8" s="61" t="inlineStr">
-        <is>
-          <t>Sembrar es un acto de confianza: uno pone la semilla en la tierra sin ver el resultado. La fe no reemplaza el trabajo, lo acompaña.</t>
-        </is>
-      </c>
-      <c r="Q8" s="61" t="inlineStr">
-        <is>
-          <t>El desánimo de muchos pequeños productores ante la incertidumbre del clima y los precios.</t>
-        </is>
-      </c>
-      <c r="R8" s="61" t="inlineStr">
-        <is>
-          <t>Si conocés a un productor, preguntale cómo le va y ofrecé tu ayuda o tu oración. Sembrar ánimo también cuenta.</t>
-        </is>
-      </c>
-      <c r="S8" s="61" t="inlineStr">
-        <is>
-          <t>Gálatas 6:7</t>
-        </is>
-      </c>
-      <c r="T8" s="61" t="inlineStr">
-        <is>
-          <t>No se dejen engañar: nadie puede burlarse de la justicia de Dios. Siempre se cosecha lo que se siembra.</t>
+          <t>Si producís, respetá las franjas de protección y los horarios de aplicación, y pedí asesoramiento técnico.</t>
         </is>
       </c>
     </row>
@@ -19946,92 +19714,64 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C9" s="61" t="n">
-        <v>1</v>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>Lo que crece mientras dormís</t>
+        </is>
       </c>
       <c r="D9" s="61" t="inlineStr">
         <is>
-          <t>La paciencia del agricultor</t>
+          <t>Alrededor del 14 % de los alimentos que se producen en el mundo se pierde entre la cosecha y la venta.</t>
         </is>
       </c>
       <c r="E9" s="61" t="inlineStr">
         <is>
-          <t>Alrededor del 14 % de los alimentos que se producen en el mundo se pierde entre la cosecha y la venta.</t>
+          <t>FAO, El estado mundial de la agricultura y la alimentación, 2019</t>
         </is>
       </c>
       <c r="F9" s="61" t="inlineStr">
         <is>
-          <t>FAO, El estado mundial de la agricultura y la alimentación, 2019</t>
+          <t>La semilla crece aunque no la veamos. Hay procesos que no se pueden apurar: la confianza, el carácter, un emprendimiento.</t>
         </is>
       </c>
       <c r="G9" s="61" t="inlineStr">
         <is>
-          <t>Los tiempos de la tierra</t>
+          <t>La ansiedad por resultados inmediatos, que hace abandonar proyectos antes de tiempo.</t>
         </is>
       </c>
       <c r="H9" s="61" t="inlineStr">
         <is>
-          <t>Ningún agricultor tira de la planta para que crezca más rápido. Hay procesos que no se pueden apurar: la confianza, el carácter, un emprendimiento.</t>
+          <t>Elegí un proyecto que abandonaste por impaciencia y dale una fecha realista para retomarlo.</t>
         </is>
       </c>
       <c r="I9" s="61" t="inlineStr">
         <is>
-          <t>La ansiedad por resultados inmediatos, que hace abandonar proyectos antes de tiempo.</t>
+          <t>No controlamos el clima ni los precios, pero sí cuidamos lo que está en nuestras manos.</t>
         </is>
       </c>
       <c r="J9" s="61" t="inlineStr">
         <is>
-          <t>Elegí un proyecto que abandonaste por impaciencia y dale una fecha realista para retomarlo.</t>
+          <t>Pérdidas de cosecha por mal almacenamiento o transporte, que golpean el bolsillo de las familias productoras.</t>
         </is>
       </c>
       <c r="K9" s="61" t="inlineStr">
         <is>
-          <t>Cuidar lo que ya creció</t>
+          <t>Revisá qué estás perdiendo por descuido: comida que se tira, herramientas sin mantenimiento, plata que se va en gastos chicos.</t>
         </is>
       </c>
       <c r="L9" s="61" t="inlineStr">
         <is>
-          <t>De poco sirve una buena cosecha si se pierde en el camino. Cuidar lo logrado es tan importante como lograrlo.</t>
+          <t>Confiar no es quedarse quieto: el agricultor confía y mientras tanto prepara, limpia y repara.</t>
         </is>
       </c>
       <c r="M9" s="61" t="inlineStr">
         <is>
-          <t>Pérdidas de cosecha por mal almacenamiento o transporte, que golpean el bolsillo de las familias productoras.</t>
+          <t>Personas sin trabajo que se desaniman y dejan de buscar.</t>
         </is>
       </c>
       <c r="N9" s="61" t="inlineStr">
         <is>
-          <t>Revisá qué estás perdiendo por descuido: comida que se tira, herramientas sin mantenimiento, plata que se va en gastos chicos.</t>
-        </is>
-      </c>
-      <c r="O9" s="61" t="inlineStr">
-        <is>
-          <t>Esperar sin quedarse quieto</t>
-        </is>
-      </c>
-      <c r="P9" s="61" t="inlineStr">
-        <is>
-          <t>La paciencia no es pasividad. El agricultor espera la lluvia, pero mientras tanto prepara, limpia y repara.</t>
-        </is>
-      </c>
-      <c r="Q9" s="61" t="inlineStr">
-        <is>
-          <t>Personas sin trabajo que se desaniman y dejan de buscar.</t>
-        </is>
-      </c>
-      <c r="R9" s="61" t="inlineStr">
-        <is>
           <t>Si estás esperando una oportunidad, usá el tiempo para capacitarte: hay cursos gratuitos del SNPP y otras instituciones.</t>
-        </is>
-      </c>
-      <c r="S9" s="61" t="inlineStr">
-        <is>
-          <t>Santiago 5:7</t>
-        </is>
-      </c>
-      <c r="T9" s="61" t="inlineStr">
-        <is>
-          <t>Amados hermanos, tengan paciencia mientras esperan el regreso del Señor. Piensen en los agricultores, que con paciencia esperan las lluvias en el otoño y la primavera. Con ansias esperan a que maduren los preciosos cultivos.</t>
         </is>
       </c>
     </row>
@@ -20044,92 +19784,64 @@
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="C10" s="61" t="n">
-        <v>2</v>
+      <c r="C10" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar la tierra es una bendición</t>
+        </is>
       </c>
       <c r="D10" s="61" t="inlineStr">
         <is>
-          <t>Trabajar la tierra es una bendición</t>
+          <t>Las granjas familiares producen alrededor del 80 % de los alimentos del mundo, medido en valor.</t>
         </is>
       </c>
       <c r="E10" s="61" t="inlineStr">
         <is>
-          <t>Las granjas familiares producen alrededor del 80 % de los alimentos del mundo, medido en valor.</t>
+          <t>FAO, El estado mundial de la agricultura y la alimentación, 2014</t>
         </is>
       </c>
       <c r="F10" s="61" t="inlineStr">
         <is>
-          <t>FAO, El estado mundial de la agricultura y la alimentación, 2014</t>
+          <t>La lluvia a tiempo es un regalo. Detrás de cada plato hay agua, sol y manos que trabajaron la tierra.</t>
         </is>
       </c>
       <c r="G10" s="61" t="inlineStr">
         <is>
-          <t>La dignidad del trabajo rural</t>
+          <t>La migración del campo a la ciudad, que deja chacras abandonadas y familias separadas.</t>
         </is>
       </c>
       <c r="H10" s="61" t="inlineStr">
         <is>
-          <t>Detrás de cada plato hay manos que trabajaron la tierra. El trabajo del campo sostiene a la ciudad, aunque muchas veces no se lo valore.</t>
+          <t>Comprá directamente a productores de tu zona en ferias y mercados: tu compra ayuda a que se queden en su tierra.</t>
         </is>
       </c>
       <c r="I10" s="61" t="inlineStr">
         <is>
-          <t>La migración del campo a la ciudad, que deja chacras abandonadas y familias separadas.</t>
+          <t>No todo depende de nosotros. Reconocerlo nos hace agradecidos y generosos con lo que recibimos.</t>
         </is>
       </c>
       <c r="J10" s="61" t="inlineStr">
         <is>
-          <t>Comprale directamente a productores de tu zona en ferias y mercados: tu compra ayuda a que se queden en su tierra.</t>
+          <t>Niños que crecen sin saber de dónde vienen los alimentos.</t>
         </is>
       </c>
       <c r="K10" s="61" t="inlineStr">
         <is>
-          <t>La agricultura familiar</t>
+          <t>Armá con tus hijos una pequeña huerta en macetas o en el patio. Un tomate cosechado por ellos enseña más que una clase.</t>
         </is>
       </c>
       <c r="L10" s="61" t="inlineStr">
         <is>
-          <t>La chacra familiar no solo produce comida: enseña a los hijos a trabajar, a cuidar y a compartir.</t>
+          <t>Dios bendice el trabajo, no la improvisación. El esfuerzo ordenado rinde más.</t>
         </is>
       </c>
       <c r="M10" s="61" t="inlineStr">
         <is>
-          <t>Niños que crecen sin saber de dónde vienen los alimentos.</t>
+          <t>El trabajo informal sin planificación, que deja a muchos sin ingresos estables.</t>
         </is>
       </c>
       <c r="N10" s="61" t="inlineStr">
         <is>
-          <t>Armá con tus hijos una pequeña huerta en macetas o en el patio. Un tomate cosechado por ellos enseña más que una clase.</t>
-        </is>
-      </c>
-      <c r="O10" s="61" t="inlineStr">
-        <is>
-          <t>Trabajo bien hecho</t>
-        </is>
-      </c>
-      <c r="P10" s="61" t="inlineStr">
-        <is>
-          <t>Quien trabaja la tierra con esmero ve el fruto. El esfuerzo constante rinde más que la improvisación.</t>
-        </is>
-      </c>
-      <c r="Q10" s="61" t="inlineStr">
-        <is>
-          <t>El trabajo informal sin planificación, que deja a muchos sin ingresos estables.</t>
-        </is>
-      </c>
-      <c r="R10" s="61" t="inlineStr">
-        <is>
-          <t>Llevá un cuaderno simple de tu actividad: qué gastás, qué producís y qué vendés. Lo que se anota se puede mejorar.</t>
-        </is>
-      </c>
-      <c r="S10" s="61" t="inlineStr">
-        <is>
-          <t>Proverbios 12:11</t>
-        </is>
-      </c>
-      <c r="T10" s="61" t="inlineStr">
-        <is>
-          <t>El que trabaja con esmero su tierra tendrá abundante comida, pero el que persigue fantasías no tiene sentido común.</t>
+          <t>Llevá un cuaderno simple: qué gastás, qué producís y qué vendés. Lo que se anota se puede mejorar.</t>
         </is>
       </c>
     </row>
@@ -20142,92 +19854,64 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C11" s="61" t="n">
-        <v>2</v>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>La paciencia del agricultor</t>
+        </is>
       </c>
       <c r="D11" s="61" t="inlineStr">
         <is>
-          <t>Los desafíos del campo</t>
+          <t>Cerca de 1 de cada 4 trabajadores del mundo trabaja en la agricultura.</t>
         </is>
       </c>
       <c r="E11" s="61" t="inlineStr">
         <is>
-          <t>Cerca de 1 de cada 4 trabajadores del mundo trabaja en la agricultura.</t>
+          <t>Organización Internacional del Trabajo (OIT) y Banco Mundial</t>
         </is>
       </c>
       <c r="F11" s="61" t="inlineStr">
         <is>
-          <t>Organización Internacional del Trabajo (OIT) y Banco Mundial, estadísticas de empleo por sector</t>
+          <t>Esperar con paciencia no es resignarse: es prepararse para lo que no se controla.</t>
         </is>
       </c>
       <c r="G11" s="61" t="inlineStr">
         <is>
-          <t>Clima que no se controla</t>
+          <t>Familias productoras que lo pierden todo en una sequía por no tener ningún resguardo.</t>
         </is>
       </c>
       <c r="H11" s="61" t="inlineStr">
         <is>
-          <t>Sequías, heladas e inundaciones recuerdan que no todo depende de nosotros. Lo que sí depende es cómo nos preparamos.</t>
+          <t>Si producís, averiguá sobre seguros agrícolas y diversificá: no pongas todo en un solo cultivo.</t>
         </is>
       </c>
       <c r="I11" s="61" t="inlineStr">
         <is>
-          <t>Familias productoras que lo pierden todo en una sequía por no tener ningún resguardo.</t>
+          <t>Mientras espera, el agricultor trabaja. Y en el campo se espera mejor en comunidad: la minga siempre fue eso.</t>
         </is>
       </c>
       <c r="J11" s="61" t="inlineStr">
         <is>
-          <t>Si producís, averiguá sobre seguros agrícolas y diversificá: no pongas toda tu plata en un solo cultivo.</t>
+          <t>El individualismo que deja a cada productor solo frente a los intermediarios.</t>
         </is>
       </c>
       <c r="K11" s="61" t="inlineStr">
         <is>
-          <t>Trabajar en equipo</t>
+          <t>Sumate o creá un grupo de productores o vecinos para comprar insumos y vender juntos.</t>
         </is>
       </c>
       <c r="L11" s="61" t="inlineStr">
         <is>
-          <t>En el campo, la minga (el trabajo comunitario) fue siempre una forma de enfrentar juntos lo que solo cuesta demasiado.</t>
+          <t>Lo que se cosecha verde no sirve. Apurar los procesos suele salir más caro.</t>
         </is>
       </c>
       <c r="M11" s="61" t="inlineStr">
         <is>
-          <t>El individualismo que deja a cada productor solo frente a los intermediarios.</t>
+          <t>Endeudarse para obtener resultados rápidos, sin calcular si se va a poder pagar.</t>
         </is>
       </c>
       <c r="N11" s="61" t="inlineStr">
         <is>
-          <t>Sumate o creá un grupo de productores o vecinos para comprar insumos y vender juntos. Juntos se negocia mejor.</t>
-        </is>
-      </c>
-      <c r="O11" s="61" t="inlineStr">
-        <is>
-          <t>Trabajar para algo más grande</t>
-        </is>
-      </c>
-      <c r="P11" s="61" t="inlineStr">
-        <is>
-          <t>El trabajo duro cansa menos cuando tiene sentido. Trabajar con propósito cambia la manera de levantarse cada mañana.</t>
-        </is>
-      </c>
-      <c r="Q11" s="61" t="inlineStr">
-        <is>
-          <t>El desgaste de quienes sienten que su trabajo no vale nada.</t>
-        </is>
-      </c>
-      <c r="R11" s="61" t="inlineStr">
-        <is>
-          <t>Hoy agradecé a alguien por su trabajo: al que te vende verduras, al que maneja el colectivo, al que limpia tu calle.</t>
-        </is>
-      </c>
-      <c r="S11" s="61" t="inlineStr">
-        <is>
-          <t>Colosenses 3:23</t>
-        </is>
-      </c>
-      <c r="T11" s="61" t="inlineStr">
-        <is>
-          <t>Trabajen de buena gana en todo lo que hagan, como si fuera para el Señor y no para la gente.</t>
+          <t>Antes de tomar un crédito, hacé las cuentas por escrito y consultá en tu cooperativa o con alguien de confianza.</t>
         </is>
       </c>
     </row>
@@ -20240,92 +19924,64 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="C12" s="61" t="n">
-        <v>3</v>
+      <c r="C12" s="61" t="inlineStr">
+        <is>
+          <t>Sembrar con generosidad</t>
+        </is>
       </c>
       <c r="D12" s="61" t="inlineStr">
         <is>
-          <t>Cuidar la tierra que nos cuida</t>
+          <t>Un tercio de los suelos del planeta están moderada o altamente degradados.</t>
         </is>
       </c>
       <c r="E12" s="61" t="inlineStr">
         <is>
-          <t>Un tercio de los suelos del planeta están moderada o altamente degradados.</t>
+          <t>FAO, Estado de los recursos de suelos del mundo, 2015</t>
         </is>
       </c>
       <c r="F12" s="61" t="inlineStr">
         <is>
-          <t>FAO, Estado de los recursos de suelos del mundo, 2015</t>
+          <t>Quien siembra con generosidad cosecha con abundancia. Eso vale también para cómo tratamos la tierra que nos alimenta.</t>
         </is>
       </c>
       <c r="G12" s="61" t="inlineStr">
         <is>
-          <t>Administradores, no dueños</t>
+          <t>La quema de campos y la deforestación, que empobrecen la tierra y afectan la salud de todos.</t>
         </is>
       </c>
       <c r="H12" s="61" t="inlineStr">
         <is>
-          <t>La tierra fue confiada al ser humano para cultivarla y cuidarla. Usarla bien es responsabilidad; agotarla es irresponsabilidad.</t>
+          <t>Nunca quemes basura ni pastizales. Si ves una quema peligrosa, avisá a los bomberos o a la municipalidad.</t>
         </is>
       </c>
       <c r="I12" s="61" t="inlineStr">
         <is>
-          <t>La quema de campos y la deforestación, que empobrecen la tierra y afectan la salud de todos.</t>
+          <t>Si no invertimos en cuidar el suelo y el agua, mañana cosechamos poco.</t>
         </is>
       </c>
       <c r="J12" s="61" t="inlineStr">
         <is>
-          <t>Nunca quemes basura ni pastizales. Si ves una quema peligrosa, avisá a los bomberos o a la municipalidad.</t>
+          <t>Arroyos contaminados con basura y agroquímicos cerca de las comunidades.</t>
         </is>
       </c>
       <c r="K12" s="61" t="inlineStr">
         <is>
-          <t>El agua es vida</t>
+          <t>Organizá con tus vecinos una limpieza del arroyo o la plaza del barrio. Una mañana de trabajo cambia el paisaje.</t>
         </is>
       </c>
       <c r="L12" s="61" t="inlineStr">
         <is>
-          <t>Ríos, arroyos y acuíferos son un tesoro. Lo que se tira al agua vuelve a nosotros.</t>
+          <t>La actitud al sembrar importa: trabajar de buena gana cambia el resultado y el ánimo.</t>
         </is>
       </c>
       <c r="M12" s="61" t="inlineStr">
         <is>
-          <t>Arroyos contaminados con basura y agroquímicos cerca de las comunidades.</t>
+          <t>El desgaste de quienes sienten que su trabajo no vale nada.</t>
         </is>
       </c>
       <c r="N12" s="61" t="inlineStr">
         <is>
-          <t>Organizá con tus vecinos una limpieza del arroyo o la plaza del barrio. Una mañana de trabajo cambia el paisaje.</t>
-        </is>
-      </c>
-      <c r="O12" s="61" t="inlineStr">
-        <is>
-          <t>Pequeños gestos, gran impacto</t>
-        </is>
-      </c>
-      <c r="P12" s="61" t="inlineStr">
-        <is>
-          <t>El cuidado del ambiente empieza en casa: separar residuos, no desperdiciar agua, plantar un árbol.</t>
-        </is>
-      </c>
-      <c r="Q12" s="61" t="inlineStr">
-        <is>
-          <t>La cantidad de plástico que termina en calles y cauces.</t>
-        </is>
-      </c>
-      <c r="R12" s="61" t="inlineStr">
-        <is>
-          <t>Usá una bolsa reutilizable para las compras y separá en casa lo orgánico del resto. Con lo orgánico podés hacer abono.</t>
-        </is>
-      </c>
-      <c r="S12" s="61" t="inlineStr">
-        <is>
-          <t>Génesis 2:15</t>
-        </is>
-      </c>
-      <c r="T12" s="61" t="inlineStr">
-        <is>
-          <t>El Señor Dios puso al hombre en el jardín de Edén para que se ocupara de él y lo custodiara.</t>
+          <t>Hoy agradecé a alguien por su trabajo: al que te vende verduras, al que maneja el colectivo, al que limpia tu calle.</t>
         </is>
       </c>
     </row>
@@ -20338,52 +19994,54 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="C13" s="61" t="n">
-        <v>3</v>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>Una herencia para los que vienen</t>
+        </is>
       </c>
       <c r="D13" s="61" t="inlineStr">
         <is>
-          <t>Una herencia para los que vienen</t>
+          <t>Formar apenas un centímetro de suelo fértil puede llevar hasta mil años.</t>
         </is>
       </c>
       <c r="E13" s="61" t="inlineStr">
         <is>
-          <t>Formar apenas un centímetro de suelo fértil puede llevar hasta mil años.</t>
+          <t>FAO, Año Internacional de los Suelos, 2015</t>
         </is>
       </c>
       <c r="F13" s="61" t="inlineStr">
         <is>
-          <t>FAO, Año Internacional de los Suelos, 2015</t>
+          <t>Hay siembras que se hacen con lágrimas: una cosecha perdida, un año malo. Pero el dolor no tiene la última palabra.</t>
         </is>
       </c>
       <c r="G13" s="61" t="inlineStr">
         <is>
-          <t>Pensar en los nietos</t>
+          <t>El desánimo de muchos pequeños productores ante la incertidumbre del clima y los precios.</t>
         </is>
       </c>
       <c r="H13" s="61" t="inlineStr">
         <is>
-          <t>Las decisiones de hoy sobre la tierra son la herencia de mañana. Quien piensa solo en la cosecha de este año puede dejar un desierto a sus hijos.</t>
+          <t>Si conocés a un productor, preguntale cómo le va y ofrecé tu ayuda o tu oración.</t>
         </is>
       </c>
       <c r="I13" s="61" t="inlineStr">
         <is>
+          <t>Lo que sembramos hoy lo van a disfrutar nuestros hijos y nietos.</t>
+        </is>
+      </c>
+      <c r="J13" s="61" t="inlineStr">
+        <is>
           <t>La venta de tierras familiares sin planificación, que deja a las nuevas generaciones sin lugar.</t>
         </is>
       </c>
-      <c r="J13" s="61" t="inlineStr">
-        <is>
-          <t>Conversá en familia qué quieren dejar a la próxima generación: tierra, oficio, valores. Ponerlo en palabras ayuda a cuidarlo.</t>
-        </is>
-      </c>
       <c r="K13" s="61" t="inlineStr">
         <is>
-          <t>Plantar árboles</t>
+          <t>Conversá en familia qué quieren dejar a la próxima generación: tierra, oficio, valores.</t>
         </is>
       </c>
       <c r="L13" s="61" t="inlineStr">
         <is>
-          <t>Dicen que la mejor época para plantar un árbol fue hace veinte años; la segunda mejor es hoy.</t>
+          <t>Perseverar es seguir sembrando aunque el fruto tarde. La mejor época para plantar un árbol fue hace veinte años; la segunda es hoy.</t>
         </is>
       </c>
       <c r="M13" s="61" t="inlineStr">
@@ -20393,37 +20051,7 @@
       </c>
       <c r="N13" s="61" t="inlineStr">
         <is>
-          <t>Plantá un árbol nativo este fin de semana: lapacho, timbó o tajy. Hacelo con los chicos y pónganle nombre.</t>
-        </is>
-      </c>
-      <c r="O13" s="61" t="inlineStr">
-        <is>
-          <t>Toda la creación es de Dios</t>
-        </is>
-      </c>
-      <c r="P13" s="61" t="inlineStr">
-        <is>
-          <t>Cuidar la tierra es también una forma de agradecer. No somos dueños absolutos: somos parte de algo más grande.</t>
-        </is>
-      </c>
-      <c r="Q13" s="61" t="inlineStr">
-        <is>
-          <t>El consumo sin medida, que usa y tira sin pensar de dónde viene cada cosa.</t>
-        </is>
-      </c>
-      <c r="R13" s="61" t="inlineStr">
-        <is>
-          <t>Antes de comprar algo nuevo esta semana, preguntate si lo necesitás, si podés repararlo o pedirlo prestado.</t>
-        </is>
-      </c>
-      <c r="S13" s="61" t="inlineStr">
-        <is>
-          <t>Salmo 24:1</t>
-        </is>
-      </c>
-      <c r="T13" s="61" t="inlineStr">
-        <is>
-          <t>La tierra es del Señor y todo lo que hay en ella; el mundo y todos sus habitantes le pertenecen.</t>
+          <t>Plantá un árbol nativo este fin de semana (lapacho, timbó o tajy) con los chicos, y pónganle nombre.</t>
         </is>
       </c>
     </row>
@@ -20436,92 +20064,64 @@
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C14" s="61" t="n">
-        <v>1</v>
+      <c r="C14" s="61" t="inlineStr">
+        <is>
+          <t>Prevenir es amar</t>
+        </is>
       </c>
       <c r="D14" s="61" t="inlineStr">
         <is>
-          <t>Prevenir es amar</t>
+          <t>Las enfermedades no transmisibles (corazón, cáncer, diabetes, pulmones) causan el 74 % de las muertes en el mundo.</t>
         </is>
       </c>
       <c r="E14" s="61" t="inlineStr">
         <is>
-          <t>Las enfermedades no transmisibles (corazón, cáncer, diabetes, pulmones) causan el 74 % de las muertes en el mundo.</t>
+          <t>Organización Mundial de la Salud, 2023</t>
         </is>
       </c>
       <c r="F14" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, nota descriptiva sobre enfermedades no transmisibles, 2023</t>
+          <t>Confiar en Dios como sanador no está en contra de los médicos: Dios también cuida a través de ellos.</t>
         </is>
       </c>
       <c r="G14" s="61" t="inlineStr">
         <is>
-          <t>Mejor prevenir que curar</t>
+          <t>Personas que abandonan un tratamiento creyendo que la fe lo reemplaza.</t>
         </is>
       </c>
       <c r="H14" s="61" t="inlineStr">
         <is>
-          <t>La prevención primaria busca que la enfermedad no aparezca: alimentación, movimiento, vacunas, no fumar. Es la medicina más barata.</t>
+          <t>Orá por tu salud y, al mismo tiempo, cumplí tus controles y tratamientos. Las dos cosas van juntas.</t>
         </is>
       </c>
       <c r="I14" s="61" t="inlineStr">
         <is>
-          <t>Esperar a sentirse mal para recién cuidarse.</t>
+          <t>Escuchar y seguir buenas instrucciones protege: higiene, vacunas, cuidados básicos.</t>
         </is>
       </c>
       <c r="J14" s="61" t="inlineStr">
         <is>
-          <t>Elegí una sola costumbre preventiva para esta semana: caminar 20 minutos, sumar una fruta al día o dejar el cigarrillo.</t>
+          <t>Las dudas y la desinformación sobre las vacunas, que bajan la cobertura en los niños.</t>
         </is>
       </c>
       <c r="K14" s="61" t="inlineStr">
         <is>
-          <t>Las vacunas cuidan a todos</t>
+          <t>Revisá la libreta de vacunación de tus hijos y la tuya. Consultá en tu unidad de salud familiar qué vacunas te tocan.</t>
         </is>
       </c>
       <c r="L14" s="61" t="inlineStr">
         <is>
-          <t>Vacunarse protege a uno mismo y a los que no pueden hacerlo, como bebés y personas enfermas.</t>
+          <t>Cuidar la salud es una forma de amar a la familia: cuando te cuidás, cuidás a quienes dependen de vos.</t>
         </is>
       </c>
       <c r="M14" s="61" t="inlineStr">
         <is>
-          <t>Las dudas y la desinformación sobre las vacunas, que bajan la cobertura en los niños.</t>
+          <t>Padres y madres que se descuidan por cuidar a todos, hasta que se enferman.</t>
         </is>
       </c>
       <c r="N14" s="61" t="inlineStr">
         <is>
-          <t>Revisá la libreta de vacunación de tus hijos y la tuya. Consultá en tu unidad de salud familiar qué vacunas te tocan.</t>
-        </is>
-      </c>
-      <c r="O14" s="61" t="inlineStr">
-        <is>
-          <t>Cuidarse por los demás</t>
-        </is>
-      </c>
-      <c r="P14" s="61" t="inlineStr">
-        <is>
-          <t>Cuando te cuidás, cuidás a quienes dependen de vos. La prevención también es una forma de amor.</t>
-        </is>
-      </c>
-      <c r="Q14" s="61" t="inlineStr">
-        <is>
-          <t>Padres y madres que se descuidan por cuidar a todos, hasta que se enferman.</t>
-        </is>
-      </c>
-      <c r="R14" s="61" t="inlineStr">
-        <is>
-          <t>Pedí a tu familia que te ayude a cumplir tu propósito de salud. Hacerlo juntos es más fácil.</t>
-        </is>
-      </c>
-      <c r="S14" s="61" t="inlineStr">
-        <is>
-          <t>Proverbios 22:3</t>
-        </is>
-      </c>
-      <c r="T14" s="61" t="inlineStr">
-        <is>
-          <t>El prudente se anticipa al peligro y toma precauciones; el simplón avanza a ciegas y sufre las consecuencias.</t>
+          <t>Pedí a tu familia que te ayude a cumplir un propósito de salud. Hacerlo juntos es más fácil.</t>
         </is>
       </c>
     </row>
@@ -20534,92 +20134,64 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C15" s="61" t="n">
-        <v>1</v>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>Hábitos que protegen a la familia</t>
+        </is>
       </c>
       <c r="D15" s="61" t="inlineStr">
         <is>
-          <t>Hábitos que protegen</t>
+          <t>Al menos el 80 % de las enfermedades del corazón, los accidentes cerebrovasculares y la diabetes tipo 2 prematuros podrían prevenirse.</t>
         </is>
       </c>
       <c r="E15" s="61" t="inlineStr">
         <is>
-          <t>Al menos el 80 % de las enfermedades del corazón, los accidentes cerebrovasculares y la diabetes tipo 2 prematuros podrían prevenirse.</t>
+          <t>Organización Mundial de la Salud, Prevención de las enfermedades crónicas, 2005</t>
         </is>
       </c>
       <c r="F15" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, Prevención de las enfermedades crónicas: una inversión vital, 2005</t>
+          <t>La confianza saca el miedo: prevenir no es vivir con paranoia, es cuidarse con tranquilidad.</t>
         </is>
       </c>
       <c r="G15" s="61" t="inlineStr">
         <is>
-          <t>La mesa de cada día</t>
+          <t>El miedo a ir al médico por temor a lo que puedan encontrar.</t>
         </is>
       </c>
       <c r="H15" s="61" t="inlineStr">
         <is>
-          <t>Lo que comemos todos los días pesa más que lo que comemos en una fiesta. La sal, el azúcar y las frituras en exceso pasan factura.</t>
+          <t>Agendá tu control anual en una fecha fácil de recordar, como tu cumpleaños, y repetilo cada año.</t>
         </is>
       </c>
       <c r="I15" s="61" t="inlineStr">
         <is>
+          <t>La esperanza mueve a actuar: quien espera un futuro, se prepara para vivirlo bien.</t>
+        </is>
+      </c>
+      <c r="J15" s="61" t="inlineStr">
+        <is>
+          <t>El sedentarismo de quienes pasan el día sentados y la noche frente a una pantalla.</t>
+        </is>
+      </c>
+      <c r="K15" s="61" t="inlineStr">
+        <is>
+          <t>Proponé a tu familia una caminata semanal. Ponele día y hora fijos.</t>
+        </is>
+      </c>
+      <c r="L15" s="61" t="inlineStr">
+        <is>
+          <t>Los hijos aprenden hábitos en la mesa de casa. Lo que comemos hoy es lo que ellos van a comer mañana.</t>
+        </is>
+      </c>
+      <c r="M15" s="61" t="inlineStr">
+        <is>
           <t>El consumo diario de gaseosas y comida ultraprocesada, también en los niños.</t>
         </is>
       </c>
-      <c r="J15" s="61" t="inlineStr">
+      <c r="N15" s="61" t="inlineStr">
         <is>
           <t>Reducí la sal en la cocina de a poco y reemplazá la gaseosa diaria por agua o jugo natural.</t>
-        </is>
-      </c>
-      <c r="K15" s="61" t="inlineStr">
-        <is>
-          <t>Moverse para vivir</t>
-        </is>
-      </c>
-      <c r="L15" s="61" t="inlineStr">
-        <is>
-          <t>No hace falta ser deportista. Caminar, bailar o subir escaleras ya protege el corazón.</t>
-        </is>
-      </c>
-      <c r="M15" s="61" t="inlineStr">
-        <is>
-          <t>El sedentarismo de quienes pasan el día sentados y la noche frente a una pantalla.</t>
-        </is>
-      </c>
-      <c r="N15" s="61" t="inlineStr">
-        <is>
-          <t>Proponé a tu familia o a tus compañeros una caminata semanal. Ponele día y hora fijos.</t>
-        </is>
-      </c>
-      <c r="O15" s="61" t="inlineStr">
-        <is>
-          <t>Interesarse por el otro</t>
-        </is>
-      </c>
-      <c r="P15" s="61" t="inlineStr">
-        <is>
-          <t>Prevenir también es estar atento a la salud de los demás: un vecino solo, un familiar que no va al médico.</t>
-        </is>
-      </c>
-      <c r="Q15" s="61" t="inlineStr">
-        <is>
-          <t>Adultos mayores que viven solos y nadie nota cuando empiezan a decaer.</t>
-        </is>
-      </c>
-      <c r="R15" s="61" t="inlineStr">
-        <is>
-          <t>Llamá esta semana a un familiar mayor y preguntale de verdad cómo está su salud.</t>
-        </is>
-      </c>
-      <c r="S15" s="61" t="inlineStr">
-        <is>
-          <t>Filipenses 2:4</t>
-        </is>
-      </c>
-      <c r="T15" s="61" t="inlineStr">
-        <is>
-          <t>No se ocupen solo de sus propios intereses, sino también procuren interesarse en los demás.</t>
         </is>
       </c>
     </row>
@@ -20632,92 +20204,64 @@
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="C16" s="61" t="n">
-        <v>2</v>
+      <c r="C16" s="61" t="inlineStr">
+        <is>
+          <t>Detectar a tiempo salva vidas</t>
+        </is>
       </c>
       <c r="D16" s="61" t="inlineStr">
         <is>
-          <t>Detectar a tiempo salva vidas</t>
+          <t>Casi la mitad de las personas con presión alta no sabe que la tiene.</t>
         </is>
       </c>
       <c r="E16" s="61" t="inlineStr">
         <is>
-          <t>Casi la mitad de las personas con presión alta no sabe que la tiene.</t>
+          <t>Organización Mundial de la Salud, Informe mundial sobre la hipertensión, 2023</t>
         </is>
       </c>
       <c r="F16" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, Informe mundial sobre la hipertensión, 2023</t>
+          <t>Prestar atención a las señales a tiempo da vida. Muchas enfermedades no duelen al principio.</t>
         </is>
       </c>
       <c r="G16" s="61" t="inlineStr">
         <is>
-          <t>Lo que no duele también importa</t>
+          <t>Personas que dicen "yo estoy sano, nunca voy al médico" hasta que aparece un problema grave.</t>
         </is>
       </c>
       <c r="H16" s="61" t="inlineStr">
         <is>
-          <t>La presión alta, el azúcar elevada y muchos cánceres no dan síntomas al principio. Por eso se los llama enemigos silenciosos.</t>
+          <t>Tomate la presión esta semana: en la farmacia, en la unidad de salud familiar o con un tensiómetro en casa.</t>
         </is>
       </c>
       <c r="I16" s="61" t="inlineStr">
         <is>
-          <t>Personas que dicen "yo estoy sano, nunca voy al médico" hasta que aparece un problema grave.</t>
+          <t>Escuchar a quien sabe cuida el cuerpo. Los profesionales de salud están para orientarnos.</t>
         </is>
       </c>
       <c r="J16" s="61" t="inlineStr">
         <is>
-          <t>Tomate la presión esta semana: en la farmacia, en la unidad de salud familiar o con un tensiómetro en casa.</t>
+          <t>La automedicación y los consejos de internet sin respaldo.</t>
         </is>
       </c>
       <c r="K16" s="61" t="inlineStr">
         <is>
-          <t>El control anual</t>
+          <t>Antes de tomar un remedio por tu cuenta, consultá en la farmacia o en el centro de salud.</t>
         </is>
       </c>
       <c r="L16" s="61" t="inlineStr">
         <is>
-          <t>Un control de rutina al año (presión, glucosa, colesterol) permite actuar antes de que sea tarde.</t>
+          <t>El enojo y el estrés constante también suben la presión. Lo que pasa en el alma se nota en el cuerpo.</t>
         </is>
       </c>
       <c r="M16" s="61" t="inlineStr">
         <is>
-          <t>El miedo a ir al médico por temor a lo que puedan encontrar.</t>
+          <t>Adultos jóvenes con presión alta por estrés laboral y mala alimentación.</t>
         </is>
       </c>
       <c r="N16" s="61" t="inlineStr">
         <is>
-          <t>Agendá tu control anual en una fecha fácil de recordar, como tu cumpleaños, y repetilo cada año.</t>
-        </is>
-      </c>
-      <c r="O16" s="61" t="inlineStr">
-        <is>
-          <t>Escuchar consejo</t>
-        </is>
-      </c>
-      <c r="P16" s="61" t="inlineStr">
-        <is>
-          <t>Pedir opinión a quien sabe no es debilidad. Los profesionales de salud están para orientarnos.</t>
-        </is>
-      </c>
-      <c r="Q16" s="61" t="inlineStr">
-        <is>
-          <t>La automedicación y los consejos de internet sin respaldo.</t>
-        </is>
-      </c>
-      <c r="R16" s="61" t="inlineStr">
-        <is>
-          <t>Antes de tomar un remedio por tu cuenta, consultá en la farmacia o en el centro de salud. Llevá la lista de lo que tomás.</t>
-        </is>
-      </c>
-      <c r="S16" s="61" t="inlineStr">
-        <is>
-          <t>Proverbios 15:22</t>
-        </is>
-      </c>
-      <c r="T16" s="61" t="inlineStr">
-        <is>
-          <t>Los planes fracasan por falta de consejo; muchos consejeros traen éxito.</t>
+          <t>Cuando sientas tensión, pará un minuto: respirá hondo cinco veces y, si podés, salí a caminar.</t>
         </is>
       </c>
     </row>
@@ -20730,92 +20274,64 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C17" s="61" t="n">
-        <v>2</v>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>Animarse a hacerse los estudios</t>
+        </is>
       </c>
       <c r="D17" s="61" t="inlineStr">
         <is>
-          <t>Animarse a hacerse los estudios</t>
+          <t>La OMS se propone que el 70 % de las mujeres se haga una prueba de detección del cáncer de cuello uterino a los 35 y a los 45 años, porque detectado a tiempo es uno de los más curables.</t>
         </is>
       </c>
       <c r="E17" s="61" t="inlineStr">
         <is>
-          <t>La OMS se propone que el 70 % de las mujeres se haga una prueba de detección del cáncer de cuello uterino a los 35 y a los 45 años, porque detectado a tiempo es uno de los más curables.</t>
+          <t>Organización Mundial de la Salud, 2020</t>
         </is>
       </c>
       <c r="F17" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, Estrategia mundial para eliminar el cáncer de cuello uterino, 2020</t>
+          <t>Reconocer que no somos invencibles es sabiduría. La humildad nos lleva a cuidarnos.</t>
         </is>
       </c>
       <c r="G17" s="61" t="inlineStr">
         <is>
-          <t>Estudios que cuidan</t>
+          <t>La vergüenza o el machismo que hacen postergar los estudios, sobre todo en los hombres.</t>
         </is>
       </c>
       <c r="H17" s="61" t="inlineStr">
         <is>
-          <t>El papanicolau, la mamografía y los controles de próstata son simples y pueden salvar la vida.</t>
+          <t>Si sos hombre mayor de 50, pedí tu control de próstata. Si sos mujer, consultá cuándo te toca el papanicolau o la mamografía.</t>
         </is>
       </c>
       <c r="I17" s="61" t="inlineStr">
         <is>
-          <t>La vergüenza o el machismo que hacen postergar los estudios, sobre todo en los hombres.</t>
+          <t>Apartarse de lo que daña es prevención: el tabaco es una de las principales causas evitables de enfermedad.</t>
         </is>
       </c>
       <c r="J17" s="61" t="inlineStr">
         <is>
-          <t>Si sos hombre mayor de 50, pedí tu control de próstata. Si sos mujer, consultá cuándo te toca el papanicolau o la mamografía.</t>
+          <t>El humo del cigarrillo dentro de casa, que enferma también a los niños.</t>
         </is>
       </c>
       <c r="K17" s="61" t="inlineStr">
         <is>
-          <t>Acompañar al que tiene miedo</t>
+          <t>Si fumás, no lo hagas dentro de casa ni en el auto. Y pedí ayuda en tu centro de salud para dejarlo.</t>
         </is>
       </c>
       <c r="L17" s="61" t="inlineStr">
         <is>
-          <t>Muchos no van al médico por miedo o porque no tienen con quién ir. Un acompañante hace la diferencia.</t>
+          <t>La imprudencia dice "a mí no me va a pasar". La sabiduría se informa y actúa.</t>
         </is>
       </c>
       <c r="M17" s="61" t="inlineStr">
         <is>
-          <t>Personas que no se atienden porque no tienen quién las lleve o cuide a los hijos.</t>
+          <t>Campañas gratuitas de salud a las que va poca gente por falta de información.</t>
         </is>
       </c>
       <c r="N17" s="61" t="inlineStr">
         <is>
-          <t>Ofrecete a acompañar a un familiar o vecino a su próximo control.</t>
-        </is>
-      </c>
-      <c r="O17" s="61" t="inlineStr">
-        <is>
-          <t>Mejor juntos</t>
-        </is>
-      </c>
-      <c r="P17" s="61" t="inlineStr">
-        <is>
-          <t>La salud se cuida mejor en comunidad: grupos de caminata, ferias de salud, campañas del barrio.</t>
-        </is>
-      </c>
-      <c r="Q17" s="61" t="inlineStr">
-        <is>
-          <t>Campañas gratuitas de salud a las que va poca gente por falta de información.</t>
-        </is>
-      </c>
-      <c r="R17" s="61" t="inlineStr">
-        <is>
-          <t>Difundí en tus grupos de WhatsApp las campañas de salud gratuitas de tu zona.</t>
-        </is>
-      </c>
-      <c r="S17" s="61" t="inlineStr">
-        <is>
-          <t>Eclesiastés 4:9-10</t>
-        </is>
-      </c>
-      <c r="T17" s="61" t="inlineStr">
-        <is>
-          <t>Es mejor ser dos que uno, porque ambos pueden ayudarse mutuamente a lograr el éxito. Si uno cae, el otro puede darle la mano y ayudarle; pero el que cae y está solo, ese sí que está en problemas.</t>
+          <t>Difundí en tus grupos de WhatsApp las campañas gratuitas de tu zona y ofrecete a acompañar a alguien.</t>
         </is>
       </c>
     </row>
@@ -20828,92 +20344,64 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="C18" s="61" t="n">
-        <v>3</v>
+      <c r="C18" s="61" t="inlineStr">
+        <is>
+          <t>Vivir en paz también es salud</t>
+        </is>
       </c>
       <c r="D18" s="61" t="inlineStr">
         <is>
-          <t>Vivir bien con una enfermedad</t>
+          <t>Unos 280 millones de personas en el mundo viven con depresión.</t>
         </is>
       </c>
       <c r="E18" s="61" t="inlineStr">
         <is>
-          <t>La diabetes es una de las principales causas de ceguera, insuficiencia renal y amputación de miembros inferiores.</t>
+          <t>Organización Mundial de la Salud, 2023</t>
         </is>
       </c>
       <c r="F18" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, nota descriptiva sobre diabetes</t>
+          <t>Un corazón en paz es medicina para el cuerpo. La salud emocional también se cuida.</t>
         </is>
       </c>
       <c r="G18" s="61" t="inlineStr">
         <is>
-          <t>Evitar que empeore</t>
+          <t>La depresión que acompaña muchas enfermedades y que pocas veces se habla.</t>
         </is>
       </c>
       <c r="H18" s="61" t="inlineStr">
         <is>
-          <t>La prevención terciaria cuida a quien ya tiene una enfermedad para que no se complique: seguir el tratamiento, controlar, cuidarse.</t>
+          <t>Si te sentís sin fuerzas, contalo a tu médico y a alguien de confianza. Pedir ayuda es parte del tratamiento.</t>
         </is>
       </c>
       <c r="I18" s="61" t="inlineStr">
         <is>
+          <t>La envidia y la comparación desgastan. Mirar siempre lo que otros tienen roba la paz.</t>
+        </is>
+      </c>
+      <c r="J18" s="61" t="inlineStr">
+        <is>
+          <t>La ansiedad que generan las redes sociales al comparar nuestra vida con la de otros.</t>
+        </is>
+      </c>
+      <c r="K18" s="61" t="inlineStr">
+        <is>
+          <t>Limitá tu tiempo en redes y dejá de seguir las cuentas que te hacen sentir menos.</t>
+        </is>
+      </c>
+      <c r="L18" s="61" t="inlineStr">
+        <is>
+          <t>Lo que sentimos afecta el cuerpo, y cuidarse también afecta el ánimo. Por eso no hay que abandonar los tratamientos.</t>
+        </is>
+      </c>
+      <c r="M18" s="61" t="inlineStr">
+        <is>
           <t>Pacientes que dejan el tratamiento cuando se sienten mejor.</t>
         </is>
       </c>
-      <c r="J18" s="61" t="inlineStr">
-        <is>
-          <t>Si tenés una enfermedad crónica, anotá tus remedios y horarios en un papel visible o en una alarma del celular.</t>
-        </is>
-      </c>
-      <c r="K18" s="61" t="inlineStr">
-        <is>
-          <t>No perder el ánimo</t>
-        </is>
-      </c>
-      <c r="L18" s="61" t="inlineStr">
-        <is>
-          <t>Un diagnóstico puede desanimar. Pero muchas personas viven años con buena calidad de vida cuidándose.</t>
-        </is>
-      </c>
-      <c r="M18" s="61" t="inlineStr">
-        <is>
-          <t>La depresión que acompaña muchas enfermedades crónicas y que pocas veces se habla.</t>
-        </is>
-      </c>
       <c r="N18" s="61" t="inlineStr">
         <is>
-          <t>Si te sentís sin fuerzas, contalo a tu médico y a alguien de confianza. Pedir ayuda es parte del tratamiento.</t>
-        </is>
-      </c>
-      <c r="O18" s="61" t="inlineStr">
-        <is>
-          <t>Fuerzas renovadas</t>
-        </is>
-      </c>
-      <c r="P18" s="61" t="inlineStr">
-        <is>
-          <t>La fe no reemplaza el tratamiento, pero da esperanza para sostenerlo día tras día.</t>
-        </is>
-      </c>
-      <c r="Q18" s="61" t="inlineStr">
-        <is>
-          <t>El aislamiento de quienes viven una enfermedad larga.</t>
-        </is>
-      </c>
-      <c r="R18" s="61" t="inlineStr">
-        <is>
-          <t>Buscá un grupo de apoyo de pacientes o una comunidad que te acompañe. No tenés que atravesarlo solo.</t>
-        </is>
-      </c>
-      <c r="S18" s="61" t="inlineStr">
-        <is>
-          <t>Isaías 40:31</t>
-        </is>
-      </c>
-      <c r="T18" s="61" t="inlineStr">
-        <is>
-          <t>En cambio, los que confían en el Señor encontrarán nuevas fuerzas; volarán alto, como con alas de águila. Correrán y no se cansarán; caminarán y no desmayarán.</t>
+          <t>Si tenés una enfermedad crónica, poné tus remedios y horarios en una alarma del celular.</t>
         </is>
       </c>
     </row>
@@ -20926,52 +20414,54 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="C19" s="61" t="n">
-        <v>3</v>
+      <c r="C19" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar al que cuida</t>
+        </is>
       </c>
       <c r="D19" s="61" t="inlineStr">
         <is>
-          <t>Cuidar al que cuida</t>
+          <t>En los países desarrollados, solo alrededor de la mitad de los pacientes con enfermedades crónicas cumple bien su tratamiento.</t>
         </is>
       </c>
       <c r="E19" s="61" t="inlineStr">
         <is>
-          <t>En los países desarrollados, solo alrededor de la mitad de los pacientes con enfermedades crónicas cumple bien su tratamiento.</t>
+          <t>Organización Mundial de la Salud, Adherencia a los tratamientos a largo plazo, 2003</t>
         </is>
       </c>
       <c r="F19" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, Adherencia a los tratamientos a largo plazo, 2003</t>
+          <t>Dios sana y también nos usa para acompañar a los que están enfermos.</t>
         </is>
       </c>
       <c r="G19" s="61" t="inlineStr">
         <is>
-          <t>La familia es parte del tratamiento</t>
+          <t>La soledad de quienes enfrentan una enfermedad sin red de apoyo.</t>
         </is>
       </c>
       <c r="H19" s="61" t="inlineStr">
         <is>
-          <t>Recordar un remedio, acompañar a un control o cocinar más sano son formas concretas de cuidar.</t>
+          <t>Pensá en una persona enferma de tu entorno y llevale algo concreto esta semana: una comida, una visita, una llamada.</t>
         </is>
       </c>
       <c r="I19" s="61" t="inlineStr">
         <is>
+          <t>Agradecer la salud es también cuidarla en familia, repartiendo el peso.</t>
+        </is>
+      </c>
+      <c r="J19" s="61" t="inlineStr">
+        <is>
           <t>Familias que dejan toda la responsabilidad del cuidado en una sola persona.</t>
         </is>
       </c>
-      <c r="J19" s="61" t="inlineStr">
-        <is>
-          <t>Repartan en casa las tareas de cuidado: quién acompaña al médico, quién compra los remedios, quién cocina.</t>
-        </is>
-      </c>
       <c r="K19" s="61" t="inlineStr">
         <is>
-          <t>El cansancio del cuidador</t>
+          <t>Repartan en casa las tareas: quién acompaña al médico, quién compra los remedios, quién cocina.</t>
         </is>
       </c>
       <c r="L19" s="61" t="inlineStr">
         <is>
-          <t>Quien cuida a un enfermo también necesita descanso y apoyo.</t>
+          <t>No olvidar los beneficios de cada día incluye valorar a quien cuida.</t>
         </is>
       </c>
       <c r="M19" s="61" t="inlineStr">
@@ -20982,36 +20472,6 @@
       <c r="N19" s="61" t="inlineStr">
         <is>
           <t>Ofrecé unas horas de relevo a alguien que cuida a un familiar enfermo: que pueda salir, dormir o descansar.</t>
-        </is>
-      </c>
-      <c r="O19" s="61" t="inlineStr">
-        <is>
-          <t>Llevar las cargas juntos</t>
-        </is>
-      </c>
-      <c r="P19" s="61" t="inlineStr">
-        <is>
-          <t>El amor se vuelve concreto cuando compartimos el peso del otro.</t>
-        </is>
-      </c>
-      <c r="Q19" s="61" t="inlineStr">
-        <is>
-          <t>La soledad de quienes enfrentan una enfermedad sin red de apoyo.</t>
-        </is>
-      </c>
-      <c r="R19" s="61" t="inlineStr">
-        <is>
-          <t>Pensá en una persona enferma de tu entorno y llevale algo concreto esta semana: una comida, una visita, una llamada.</t>
-        </is>
-      </c>
-      <c r="S19" s="61" t="inlineStr">
-        <is>
-          <t>Gálatas 6:2</t>
-        </is>
-      </c>
-      <c r="T19" s="61" t="inlineStr">
-        <is>
-          <t>Ayúdense a llevar los unos las cargas de los otros, y obedezcan de esa manera la ley de Cristo.</t>
         </is>
       </c>
     </row>
@@ -21024,92 +20484,64 @@
           <t>Lunes</t>
         </is>
       </c>
-      <c r="C20" s="61" t="n">
-        <v>1</v>
+      <c r="C20" s="61" t="inlineStr">
+        <is>
+          <t>Leer no es lo mismo que estudiar</t>
+        </is>
       </c>
       <c r="D20" s="61" t="inlineStr">
         <is>
-          <t>Leer no es lo mismo que estudiar</t>
+          <t>Quienes leen la Biblia cuatro o más veces por semana muestran cambios mucho mayores en su conducta diaria que quienes la leen con menos frecuencia.</t>
         </is>
       </c>
       <c r="E20" s="61" t="inlineStr">
         <is>
-          <t>Quienes leen la Biblia cuatro o más veces por semana muestran cambios mucho mayores en su conducta diaria que quienes la leen con menos frecuencia.</t>
+          <t>Center for Bible Engagement, Cole y Ovwigho, 2009</t>
         </is>
       </c>
       <c r="F20" s="61" t="inlineStr">
         <is>
-          <t>Center for Bible Engagement, Arnold Cole y Pamela Caudill Ovwigho, Understanding the Bible Engagement Challenge, 2009</t>
+          <t>Si la Escritura viene de Dios, merece más que una lectura apurada: detenerse, preguntar y dejar que hable.</t>
         </is>
       </c>
       <c r="G20" s="61" t="inlineStr">
         <is>
-          <t>Más que información</t>
+          <t>La lectura apurada de todo: mensajes, titulares y redes, sin comprender a fondo.</t>
         </is>
       </c>
       <c r="H20" s="61" t="inlineStr">
         <is>
-          <t>Se puede leer un capítulo sin que cambie nada. Estudiar es detenerse, preguntar y dejar que el texto nos hable.</t>
+          <t>Elegí un texto corto esta semana y leelo tres veces en días distintos. Anotá qué notás de nuevo cada vez.</t>
         </is>
       </c>
       <c r="I20" s="61" t="inlineStr">
         <is>
-          <t>La lectura apurada de todo: mensajes, titulares y redes, sin comprender a fondo.</t>
+          <t>La Biblia enseña y corrige en lo concreto: familia, trabajo, dinero, conflictos.</t>
         </is>
       </c>
       <c r="J20" s="61" t="inlineStr">
         <is>
-          <t>Elegí un texto corto esta semana y leelo tres veces en días distintos. Anotá qué notás de nuevo cada vez.</t>
+          <t>La idea de que la Biblia no tiene nada que decir sobre los problemas de hoy.</t>
         </is>
       </c>
       <c r="K20" s="61" t="inlineStr">
         <is>
-          <t>Un libro para la vida</t>
+          <t>Buscá qué dice Proverbios sobre un tema que te preocupe (dinero, trabajo, familia) y anotá un consejo práctico.</t>
         </is>
       </c>
       <c r="L20" s="61" t="inlineStr">
         <is>
-          <t>La Biblia no es solo un libro religioso: habla de familia, trabajo, dinero, conflictos y esperanza.</t>
+          <t>La Escritura no está para que sepamos más, sino para que vivamos mejor.</t>
         </is>
       </c>
       <c r="M20" s="61" t="inlineStr">
         <is>
-          <t>La idea de que la Biblia no tiene nada que decir sobre los problemas de hoy.</t>
+          <t>Personas que conocen muchos versículos pero no los aplican.</t>
         </is>
       </c>
       <c r="N20" s="61" t="inlineStr">
         <is>
-          <t>Buscá qué dice Proverbios sobre un tema que te preocupe (dinero, trabajo, familia) y anotá un consejo práctico.</t>
-        </is>
-      </c>
-      <c r="O20" s="61" t="inlineStr">
-        <is>
-          <t>Útil para corregir y enseñar</t>
-        </is>
-      </c>
-      <c r="P20" s="61" t="inlineStr">
-        <is>
-          <t>La Escritura no está para que sepamos más, sino para que vivamos mejor.</t>
-        </is>
-      </c>
-      <c r="Q20" s="61" t="inlineStr">
-        <is>
-          <t>Personas que conocen muchos versículos pero no los aplican.</t>
-        </is>
-      </c>
-      <c r="R20" s="61" t="inlineStr">
-        <is>
           <t>Por cada texto que estudies, escribí una acción concreta para hacer esa misma semana.</t>
-        </is>
-      </c>
-      <c r="S20" s="61" t="inlineStr">
-        <is>
-          <t>2 Timoteo 3:16-17</t>
-        </is>
-      </c>
-      <c r="T20" s="61" t="inlineStr">
-        <is>
-          <t>Toda la Escritura es inspirada por Dios y es útil para enseñarnos lo que es verdad y para hacernos ver lo que está mal en nuestra vida. Nos corrige cuando estamos equivocados y nos enseña a hacer lo correcto. Dios la usa para preparar y capacitar a su pueblo para que haga toda buena obra.</t>
         </is>
       </c>
     </row>
@@ -21122,92 +20554,64 @@
           <t>Martes</t>
         </is>
       </c>
-      <c r="C21" s="61" t="n">
-        <v>1</v>
+      <c r="C21" s="61" t="inlineStr">
+        <is>
+          <t>Del oído a la práctica</t>
+        </is>
       </c>
       <c r="D21" s="61" t="inlineStr">
         <is>
-          <t>Del oído a la práctica</t>
+          <t>Si no repasamos lo aprendido, olvidamos más de la mitad en apenas un día.</t>
         </is>
       </c>
       <c r="E21" s="61" t="inlineStr">
         <is>
-          <t>Si no repasamos lo aprendido, olvidamos más de la mitad en apenas un día.</t>
+          <t>Hermann Ebbinghaus, estudios sobre la memoria, 1885</t>
         </is>
       </c>
       <c r="F21" s="61" t="inlineStr">
         <is>
-          <t>Hermann Ebbinghaus, estudios sobre la memoria y la "curva del olvido", 1885</t>
+          <t>Meditar es repasar: volver a un texto durante el día lo fija en la memoria y en el corazón.</t>
         </is>
       </c>
       <c r="G21" s="61" t="inlineStr">
         <is>
-          <t>Repasar para recordar</t>
+          <t>Escuchar un buen mensaje el domingo y olvidarlo el lunes.</t>
         </is>
       </c>
       <c r="H21" s="61" t="inlineStr">
         <is>
-          <t>Lo que se repasa se queda. Volver a un texto durante la semana lo fija en la memoria y en el corazón.</t>
+          <t>Escribí el versículo de la semana en un papel y pegalo en la heladera o ponelo de fondo de pantalla.</t>
         </is>
       </c>
       <c r="I21" s="61" t="inlineStr">
         <is>
-          <t>Escuchar un buen mensaje el domingo y olvidarlo el lunes.</t>
+          <t>El valor de lo aprendido se ve en lo que cambia. Guardar la Palabra es hacerla.</t>
         </is>
       </c>
       <c r="J21" s="61" t="inlineStr">
         <is>
-          <t>Escribí el versículo de la semana en un papel y pegalo en la heladera o como fondo de pantalla.</t>
+          <t>La distancia entre lo que se dice y lo que se vive, que aleja a muchos de la fe.</t>
         </is>
       </c>
       <c r="K21" s="61" t="inlineStr">
         <is>
-          <t>Hacer, no solo escuchar</t>
+          <t>Elegí una enseñanza y aplicala hoy mismo con alguien concreto: pedir perdón, ayudar, agradecer.</t>
         </is>
       </c>
       <c r="L21" s="61" t="inlineStr">
         <is>
-          <t>El valor de lo aprendido se ve en lo que cambia. Escuchar sin practicar es engañarse.</t>
+          <t>El éxito verdadero no es solo plata: es integridad, paz y relaciones sanas. Y se construye con constancia diaria.</t>
         </is>
       </c>
       <c r="M21" s="61" t="inlineStr">
         <is>
-          <t>La distancia entre lo que se dice y lo que se vive, que aleja a muchos de la fe.</t>
+          <t>La falta de tiempo como excusa para todo lo importante.</t>
         </is>
       </c>
       <c r="N21" s="61" t="inlineStr">
         <is>
-          <t>Elegí una enseñanza y aplicala hoy mismo con alguien concreto: pedir perdón, ayudar, agradecer.</t>
-        </is>
-      </c>
-      <c r="O21" s="61" t="inlineStr">
-        <is>
-          <t>Diligencia diaria</t>
-        </is>
-      </c>
-      <c r="P21" s="61" t="inlineStr">
-        <is>
-          <t>No hace falta una hora por día. Diez minutos constantes valen más que un maratón cada tanto.</t>
-        </is>
-      </c>
-      <c r="Q21" s="61" t="inlineStr">
-        <is>
-          <t>La falta de tiempo como excusa para todo lo importante.</t>
-        </is>
-      </c>
-      <c r="R21" s="61" t="inlineStr">
-        <is>
           <t>Fijá un horario de diez minutos para leer: al levantarte, en el colectivo o antes de dormir.</t>
-        </is>
-      </c>
-      <c r="S21" s="61" t="inlineStr">
-        <is>
-          <t>Santiago 1:22</t>
-        </is>
-      </c>
-      <c r="T21" s="61" t="inlineStr">
-        <is>
-          <t>No solo escuchen la palabra de Dios; tienen que ponerla en práctica. De lo contrario, solamente se engañan a sí mismos.</t>
         </is>
       </c>
     </row>
@@ -21220,92 +20624,64 @@
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="C22" s="61" t="n">
-        <v>2</v>
+      <c r="C22" s="61" t="inlineStr">
+        <is>
+          <t>Métodos sencillos para estudiar</t>
+        </is>
       </c>
       <c r="D22" s="61" t="inlineStr">
         <is>
-          <t>Métodos sencillos para estudiar</t>
+          <t>Quienes toman notas a mano comprenden mejor los conceptos que quienes escriben en una computadora.</t>
         </is>
       </c>
       <c r="E22" s="61" t="inlineStr">
         <is>
-          <t>Quienes toman notas a mano comprenden mejor los conceptos que quienes escriben en una computadora.</t>
+          <t>Mueller y Oppenheimer, revista Psychological Science, 2014</t>
         </is>
       </c>
       <c r="F22" s="61" t="inlineStr">
         <is>
-          <t>Pam Mueller y Daniel Oppenheimer, revista Psychological Science, 2014</t>
+          <t>Una Palabra viva se estudia con preguntas: ¿qué dice?, ¿qué significaba para los primeros lectores?, ¿qué me dice hoy?</t>
         </is>
       </c>
       <c r="G22" s="61" t="inlineStr">
         <is>
-          <t>Observar, entender, aplicar</t>
+          <t>Interpretaciones sacadas de contexto que generan confusión y división.</t>
         </is>
       </c>
       <c r="H22" s="61" t="inlineStr">
         <is>
-          <t>Un método simple: ¿qué dice el texto?, ¿qué significaba para los que lo leyeron primero?, ¿qué me dice hoy a mí?</t>
+          <t>Antes de sacar conclusiones, leé los versículos de antes y de después. El contexto aclara casi todo.</t>
         </is>
       </c>
       <c r="I22" s="61" t="inlineStr">
         <is>
-          <t>Interpretaciones sacadas de contexto que generan confusión y división.</t>
+          <t>Para ir más allá de lo superficial ayuda escribir: un cuaderno ordena las ideas y muestra el crecimiento.</t>
         </is>
       </c>
       <c r="J22" s="61" t="inlineStr">
         <is>
-          <t>Antes de sacar conclusiones, leé los versículos de antes y de después. El contexto aclara casi todo.</t>
+          <t>Mucho contenido consumido en el celular que no deja nada escrito ni recordado.</t>
         </is>
       </c>
       <c r="K22" s="61" t="inlineStr">
         <is>
-          <t>Escribir lo que aprendés</t>
+          <t>Conseguí un cuaderno solo para tu estudio y anotá la fecha, el texto y una idea por día.</t>
         </is>
       </c>
       <c r="L22" s="61" t="inlineStr">
         <is>
-          <t>Un cuaderno de estudio ayuda a ordenar ideas y a ver el crecimiento con el tiempo.</t>
+          <t>La Biblia es un espejo: antes de usarla para juzgar a otros, nos muestra lo que hay en nuestro corazón.</t>
         </is>
       </c>
       <c r="M22" s="61" t="inlineStr">
         <is>
-          <t>Mucho contenido consumido en el celular que no deja nada escrito ni recordado.</t>
+          <t>Personas que usan versículos para señalar a los demás y no para mirarse a sí mismas.</t>
         </is>
       </c>
       <c r="N22" s="61" t="inlineStr">
         <is>
-          <t>Conseguí un cuaderno solo para tu estudio bíblico y anotá la fecha, el texto y una idea por día.</t>
-        </is>
-      </c>
-      <c r="O22" s="61" t="inlineStr">
-        <is>
-          <t>Examinar con entusiasmo</t>
-        </is>
-      </c>
-      <c r="P22" s="61" t="inlineStr">
-        <is>
-          <t>Estudiar es preguntar sin miedo y comprobar lo que se escucha.</t>
-        </is>
-      </c>
-      <c r="Q22" s="61" t="inlineStr">
-        <is>
-          <t>Creer cualquier cosa que circula en cadenas y redes sin verificarla.</t>
-        </is>
-      </c>
-      <c r="R22" s="61" t="inlineStr">
-        <is>
-          <t>Cuando escuches una enseñanza, buscá vos mismo los textos citados y leelos completos.</t>
-        </is>
-      </c>
-      <c r="S22" s="61" t="inlineStr">
-        <is>
-          <t>Hechos 17:11</t>
-        </is>
-      </c>
-      <c r="T22" s="61" t="inlineStr">
-        <is>
-          <t>Ellos escucharon con entusiasmo el mensaje de Pablo. Día tras día examinaban las Escrituras para ver si Pablo y Silas enseñaban la verdad.</t>
+          <t>Cada vez que leas, preguntate: ¿qué tengo que cambiar yo? Y anotalo.</t>
         </is>
       </c>
     </row>
@@ -21318,92 +20694,64 @@
           <t>Jueves</t>
         </is>
       </c>
-      <c r="C23" s="61" t="n">
-        <v>2</v>
+      <c r="C23" s="61" t="inlineStr">
+        <is>
+          <t>Un plan que se pueda cumplir</t>
+        </is>
       </c>
       <c r="D23" s="61" t="inlineStr">
         <is>
-          <t>Un plan que se pueda cumplir</t>
+          <t>La Biblia completa está traducida a más de 700 idiomas.</t>
         </is>
       </c>
       <c r="E23" s="61" t="inlineStr">
         <is>
-          <t>La Biblia completa está traducida a más de 700 idiomas.</t>
+          <t>Wycliffe Global Alliance</t>
         </is>
       </c>
       <c r="F23" s="61" t="inlineStr">
         <is>
-          <t>Wycliffe Global Alliance, estadísticas de traducción de la Biblia</t>
+          <t>Disfrutar la lectura ayuda a sostenerla. Mejor un plan corto y realista que un maratón abandonado.</t>
         </is>
       </c>
       <c r="G23" s="61" t="inlineStr">
         <is>
-          <t>Un plan realista</t>
+          <t>Las metas demasiado grandes que se abandonan rápido.</t>
         </is>
       </c>
       <c r="H23" s="61" t="inlineStr">
         <is>
-          <t>Empezar por Génesis y abandonar en Levítico es común. Mejor un plan corto: un Evangelio, Proverbios, un salmo por día.</t>
+          <t>Elegí un plan de 30 días (por ejemplo, un capítulo de Proverbios por día) y marcá cada día cumplido.</t>
         </is>
       </c>
       <c r="I23" s="61" t="inlineStr">
         <is>
-          <t>Las metas demasiado grandes que se abandonan rápido.</t>
+          <t>El árbol junto al agua no se seca porque sus raíces llegan hondo. Las raíces crecen mejor en compañía.</t>
         </is>
       </c>
       <c r="J23" s="61" t="inlineStr">
         <is>
-          <t>Elegí un plan de 30 días (por ejemplo, un capítulo de Proverbios por día) y marcá cada día cumplido.</t>
+          <t>La fe vivida en soledad, que se enfría fácilmente.</t>
         </is>
       </c>
       <c r="K23" s="61" t="inlineStr">
         <is>
-          <t>Estudiar acompañado</t>
+          <t>Invitá a un amigo o a tu familia a leer el mismo texto durante la semana y comentarlo el sábado.</t>
         </is>
       </c>
       <c r="L23" s="61" t="inlineStr">
         <is>
-          <t>En grupo se aprende más: otros ven lo que uno no ve y se sostiene la constancia.</t>
+          <t>Prosperar es dar fruto a su tiempo. Meditar es masticar despacio una idea hasta que se vuelve parte de uno.</t>
         </is>
       </c>
       <c r="M23" s="61" t="inlineStr">
         <is>
-          <t>La fe vivida en soledad, que se enfría fácilmente.</t>
+          <t>La mente saturada de noticias y preocupaciones, sin espacio para el silencio.</t>
         </is>
       </c>
       <c r="N23" s="61" t="inlineStr">
         <is>
-          <t>Invitá a un amigo o a tu familia a leer el mismo texto durante la semana y comentarlo el sábado.</t>
-        </is>
-      </c>
-      <c r="O23" s="61" t="inlineStr">
-        <is>
-          <t>Meditar de día y de noche</t>
-        </is>
-      </c>
-      <c r="P23" s="61" t="inlineStr">
-        <is>
-          <t>Meditar es masticar despacio una idea hasta que se vuelve parte de uno.</t>
-        </is>
-      </c>
-      <c r="Q23" s="61" t="inlineStr">
-        <is>
-          <t>La mente saturada de noticias y preocupaciones, sin espacio para el silencio.</t>
-        </is>
-      </c>
-      <c r="R23" s="61" t="inlineStr">
-        <is>
-          <t>Elegí una frase del texto del día y repetila en silencio en momentos de espera: la fila, el tránsito, la pausa del trabajo.</t>
-        </is>
-      </c>
-      <c r="S23" s="61" t="inlineStr">
-        <is>
-          <t>Josué 1:8</t>
-        </is>
-      </c>
-      <c r="T23" s="61" t="inlineStr">
-        <is>
-          <t>Estudia constantemente este libro de instrucción. Medita en él de día y de noche para asegurarte de obedecer todo lo que allí está escrito. Solamente entonces prosperarás y te irá bien en todo lo que hagas.</t>
+          <t>Elegí una frase del texto y repetila en silencio en momentos de espera: la fila, el tránsito, la pausa del trabajo.</t>
         </is>
       </c>
     </row>
@@ -21416,92 +20764,64 @@
           <t>Viernes</t>
         </is>
       </c>
-      <c r="C24" s="61" t="n">
-        <v>3</v>
+      <c r="C24" s="61" t="inlineStr">
+        <is>
+          <t>La fe entra por el oído</t>
+        </is>
       </c>
       <c r="D24" s="61" t="inlineStr">
         <is>
-          <t>Escarbar más hondo</t>
+          <t>Quien estudia sabiendo que después va a tener que enseñarlo a otro aprende y recuerda mejor.</t>
         </is>
       </c>
       <c r="E24" s="61" t="inlineStr">
         <is>
-          <t>Quien estudia sabiendo que después va a tener que enseñarlo a otro aprende y recuerda mejor.</t>
+          <t>Nestojko y otros, revista Memory &amp; Cognition, 2014</t>
         </is>
       </c>
       <c r="F24" s="61" t="inlineStr">
         <is>
-          <t>John Nestojko y otros, revista Memory &amp; Cognition, 2014</t>
+          <t>La fe nace de escuchar. La radio, un audio o una conversación también son caminos para recibir la Palabra.</t>
         </is>
       </c>
       <c r="G24" s="61" t="inlineStr">
         <is>
-          <t>Descubrir el carácter de Dios</t>
+          <t>Personas que abandonan la lectura porque leer les cuesta o no tienen tiempo.</t>
         </is>
       </c>
       <c r="H24" s="61" t="inlineStr">
         <is>
-          <t>Al estudiar a fondo, la Biblia deja de ser un libro de reglas y muestra a un Dios cercano, paciente y justo.</t>
+          <t>Escuchá la Biblia en audio mientras caminás, cocinás o viajás.</t>
         </is>
       </c>
       <c r="I24" s="61" t="inlineStr">
         <is>
+          <t>Escuchar y compartir fortalece la fe: contar lo que aprendiste lo fija y bendice a otros.</t>
+        </is>
+      </c>
+      <c r="J24" s="61" t="inlineStr">
+        <is>
+          <t>Padres que delegan toda la formación espiritual de sus hijos en la iglesia o la escuela.</t>
+        </is>
+      </c>
+      <c r="K24" s="61" t="inlineStr">
+        <is>
+          <t>Contá en la cena de hoy algo que aprendiste de la Biblia esta semana. Corto y sencillo.</t>
+        </is>
+      </c>
+      <c r="L24" s="61" t="inlineStr">
+        <is>
+          <t>Sin alimento, la fe se debilita y aparecen ideas equivocadas sobre Dios.</t>
+        </is>
+      </c>
+      <c r="M24" s="61" t="inlineStr">
+        <is>
           <t>Imágenes distorsionadas de Dios (castigador o indiferente) que alejan a muchas personas.</t>
         </is>
       </c>
-      <c r="J24" s="61" t="inlineStr">
+      <c r="N24" s="61" t="inlineStr">
         <is>
           <t>Mientras leés, anotá en una columna aparte qué muestra el texto sobre cómo es Dios.</t>
-        </is>
-      </c>
-      <c r="K24" s="61" t="inlineStr">
-        <is>
-          <t>Luz para decidir</t>
-        </is>
-      </c>
-      <c r="L24" s="61" t="inlineStr">
-        <is>
-          <t>La Palabra no responde todo al instante, pero ilumina el siguiente paso.</t>
-        </is>
-      </c>
-      <c r="M24" s="61" t="inlineStr">
-        <is>
-          <t>Decisiones importantes tomadas por impulso, sin reflexión ni consejo.</t>
-        </is>
-      </c>
-      <c r="N24" s="61" t="inlineStr">
-        <is>
-          <t>Antes de una decisión importante, buscá textos sobre el tema y conversalo con alguien de confianza.</t>
-        </is>
-      </c>
-      <c r="O24" s="61" t="inlineStr">
-        <is>
-          <t>Enseñar lo que aprendés</t>
-        </is>
-      </c>
-      <c r="P24" s="61" t="inlineStr">
-        <is>
-          <t>Compartir lo que descubriste fija el aprendizaje y bendice a otros.</t>
-        </is>
-      </c>
-      <c r="Q24" s="61" t="inlineStr">
-        <is>
-          <t>Padres que delegan toda la formación espiritual de sus hijos en la iglesia o la escuela.</t>
-        </is>
-      </c>
-      <c r="R24" s="61" t="inlineStr">
-        <is>
-          <t>Contá en la cena de hoy algo que aprendiste de la Biblia esta semana. Corto y sencillo.</t>
-        </is>
-      </c>
-      <c r="S24" s="61" t="inlineStr">
-        <is>
-          <t>Salmo 119:105</t>
-        </is>
-      </c>
-      <c r="T24" s="61" t="inlineStr">
-        <is>
-          <t>Tu palabra es una lámpara que guía mis pies y una luz para mi camino.</t>
         </is>
       </c>
     </row>
@@ -21514,92 +20834,64 @@
           <t>Sábado</t>
         </is>
       </c>
-      <c r="C25" s="61" t="n">
-        <v>3</v>
+      <c r="C25" s="61" t="inlineStr">
+        <is>
+          <t>Una Palabra que alimenta</t>
+        </is>
       </c>
       <c r="D25" s="61" t="inlineStr">
         <is>
-          <t>Buscar de todo corazón</t>
+          <t>El Salmo 119 es el capítulo más largo de la Biblia: 176 versículos dedicados casi por completo a la Palabra de Dios.</t>
         </is>
       </c>
       <c r="E25" s="61" t="inlineStr">
         <is>
-          <t>El Salmo 119 es el capítulo más largo de la Biblia: 176 versículos dedicados casi por completo a la Palabra de Dios.</t>
+          <t>Biblia, Salmo 119</t>
         </is>
       </c>
       <c r="F25" s="61" t="inlineStr">
         <is>
-          <t>Biblia, Salmo 119</t>
+          <t>Comer la Palabra es hacerla propia: no quedarse en la costumbre, sino buscar una relación personal.</t>
         </is>
       </c>
       <c r="G25" s="61" t="inlineStr">
         <is>
-          <t>La búsqueda sincera</t>
+          <t>La fe superficial, que se queda en costumbres sin una relación personal.</t>
         </is>
       </c>
       <c r="H25" s="61" t="inlineStr">
         <is>
-          <t>Dios no se esconde de quien lo busca de verdad. El estudio es una forma concreta de buscarlo.</t>
+          <t>Este fin de semana, reservá media hora tranquila solo para leer y orar, sin celular.</t>
         </is>
       </c>
       <c r="I25" s="61" t="inlineStr">
         <is>
-          <t>La fe superficial, que se queda en costumbres sin una relación personal.</t>
+          <t>El gozo de la Palabra no depende del entusiasmo del día. La diligencia es seguir aunque no emocione.</t>
         </is>
       </c>
       <c r="J25" s="61" t="inlineStr">
         <is>
-          <t>Este fin de semana, reservá media hora tranquila solo para leer y orar, sin celular.</t>
+          <t>Abandonar todo lo valioso apenas deja de ser entretenido.</t>
         </is>
       </c>
       <c r="K25" s="61" t="inlineStr">
         <is>
-          <t>Constancia en tiempos secos</t>
+          <t>Si te cuesta, cambiá el formato: un plan nuevo, otra traducción o la Biblia en audio.</t>
         </is>
       </c>
       <c r="L25" s="61" t="inlineStr">
         <is>
-          <t>Habrá días en que leer no emocione. La diligencia es seguir igual, porque el fruto llega con el tiempo.</t>
+          <t>La alegría que da la Palabra se contagia y se hereda.</t>
         </is>
       </c>
       <c r="M25" s="61" t="inlineStr">
         <is>
-          <t>Abandonar todo lo valioso apenas deja de ser entretenido.</t>
+          <t>Generaciones que crecen sin referencias de fe en casa.</t>
         </is>
       </c>
       <c r="N25" s="61" t="inlineStr">
         <is>
-          <t>Si te cuesta, cambiá el formato: escuchá la Biblia en audio mientras caminás o viajás.</t>
-        </is>
-      </c>
-      <c r="O25" s="61" t="inlineStr">
-        <is>
-          <t>Un legado para los que vienen</t>
-        </is>
-      </c>
-      <c r="P25" s="61" t="inlineStr">
-        <is>
-          <t>Una Biblia gastada y subrayada es una herencia para hijos y nietos.</t>
-        </is>
-      </c>
-      <c r="Q25" s="61" t="inlineStr">
-        <is>
-          <t>Generaciones que crecen sin referencias de fe en casa.</t>
-        </is>
-      </c>
-      <c r="R25" s="61" t="inlineStr">
-        <is>
           <t>Regalá una Biblia o un devocional a un joven de tu familia con una dedicatoria escrita por vos.</t>
-        </is>
-      </c>
-      <c r="S25" s="61" t="inlineStr">
-        <is>
-          <t>Jeremías 29:13</t>
-        </is>
-      </c>
-      <c r="T25" s="61" t="inlineStr">
-        <is>
-          <t>Si me buscan de todo corazón, podrán encontrarme.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mensajero: lenguaje para audiencia cristiana en guiones y prompt
Sin ejemplos de alcohol, tabaco ni apuestas; ejemplos de la vida de
familias creyentes (hogar, trabajo, iglesia).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -19276,12 +19276,12 @@
       </c>
       <c r="M2" s="61" t="inlineStr">
         <is>
-          <t>El consumo excesivo de alcohol los fines de semana, que muchos ven como algo normal.</t>
+          <t>El activismo que agota: servir en el trabajo, en la casa y en la iglesia sin cuidar nunca el propio cuerpo.</t>
         </is>
       </c>
       <c r="N2" s="61" t="inlineStr">
         <is>
-          <t>Elegí un cambio concreto para este fin de semana: menos alcohol, más agua y una salida al aire libre con tu familia.</t>
+          <t>Revisá tu agenda de la semana y separá un espacio para descansar y moverte, igual que separás tiempo para servir.</t>
         </is>
       </c>
     </row>
@@ -19606,17 +19606,17 @@
       </c>
       <c r="I7" s="61" t="inlineStr">
         <is>
-          <t>Apartarse del mal también es evitar los excesos que dañan: alcohol, peleas, noches sin dormir.</t>
+          <t>Apartarse del mal también es cuidarse de lo que desgasta por dentro: el enojo guardado, los conflictos sin resolver, las noches sin dormir.</t>
         </is>
       </c>
       <c r="J7" s="61" t="inlineStr">
         <is>
-          <t>Los accidentes de tránsito de los fines de semana, muchas veces ligados al alcohol.</t>
+          <t>Discusiones familiares que se arrastran toda la semana y estallan el fin de semana.</t>
         </is>
       </c>
       <c r="K7" s="61" t="inlineStr">
         <is>
-          <t>Si vas a tomar, no manejes. Acordá antes quién conduce o volvé en otro medio.</t>
+          <t>Antes del domingo, buscá a quien tengas algo pendiente y conversá en paz. Llegar reconciliado al culto también es cuidarse.</t>
         </is>
       </c>
       <c r="L7" s="61" t="inlineStr">
@@ -19666,12 +19666,12 @@
       </c>
       <c r="G8" s="61" t="inlineStr">
         <is>
-          <t>La cultura de la plata fácil: apuestas, préstamos rápidos y negocios dudosos que prometen cosechar sin sembrar.</t>
+          <t>Las promesas de ganancia fácil (préstamos rápidos, cadenas, esquemas de inversión) que llegan incluso a los grupos de la iglesia.</t>
         </is>
       </c>
       <c r="H8" s="61" t="inlineStr">
         <is>
-          <t>Anotá esta semana tres semillas concretas: un hábito, una relación y un ahorro pequeño que quieras empezar.</t>
+          <t>Antes de entrar en cualquier negocio, consultalo con alguien de confianza y desconfiá de lo que promete mucho sin trabajo. Anotá esta semana tres semillas concretas que sí quieras sembrar.</t>
         </is>
       </c>
       <c r="I8" s="61" t="inlineStr">
@@ -20306,17 +20306,17 @@
       </c>
       <c r="I17" s="61" t="inlineStr">
         <is>
-          <t>Apartarse de lo que daña es prevención: el tabaco es una de las principales causas evitables de enfermedad.</t>
+          <t>Apartarse de lo que daña también es prevención: el exceso de azúcar, sal y frituras que en muchas mesas se ve como normal.</t>
         </is>
       </c>
       <c r="J17" s="61" t="inlineStr">
         <is>
-          <t>El humo del cigarrillo dentro de casa, que enferma también a los niños.</t>
+          <t>Las comidas de los encuentros de la familia y de la iglesia, casi siempre cargadas de frituras y gaseosas.</t>
         </is>
       </c>
       <c r="K17" s="61" t="inlineStr">
         <is>
-          <t>Si fumás, no lo hagas dentro de casa ni en el auto. Y pedí ayuda en tu centro de salud para dejarlo.</t>
+          <t>En el próximo encuentro de tu grupo o tu familia, proponé sumar frutas, ensaladas y agua fresca al menú.</t>
         </is>
       </c>
       <c r="L17" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: «Mi semana» según los días al aire de cada programa
- Domingo introducción, lun-mar subtema 1, mié-jue subtema 2, viernes
  subtema 3 completo, sábado resumen (3 ideas clave y una acción).
- Mi programa: días al aire (Dom..Sáb, atajos lun-vie y lun-sáb).
  Un solo día = guion semanal con introducción y resumen.
- Sin sección «Tres subtemas»: cada día dice su subtema y el primero
  trae «Para el locutor». Un «Al aire» y una nota por día.
- Registro y contador por días al aire; preparación según los días.
- Resúmenes de los sábados de enero.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -19576,7 +19576,7 @@
       </c>
       <c r="C7" s="61" t="inlineStr">
         <is>
-          <t>Un fin de semana que recarga</t>
+          <t>Repaso: cuidar el cuerpo que Dios nos dio</t>
         </is>
       </c>
       <c r="D7" s="61" t="inlineStr">
@@ -19591,49 +19591,29 @@
       </c>
       <c r="F7" s="61" t="inlineStr">
         <is>
-          <t>La sabiduría se ve en decisiones simples: cómo usamos el tiempo libre. Pasar el sábado frente a una pantalla no siempre descansa.</t>
-        </is>
-      </c>
-      <c r="G7" s="61" t="inlineStr">
-        <is>
-          <t>Familias que comparten la casa pero cada uno está en su celular.</t>
-        </is>
-      </c>
+          <t>Tu cuerpo no es tu enemigo ni tu ídolo: es un templo que se cuida para servir, adorar y amar mejor.</t>
+        </is>
+      </c>
+      <c r="G7" s="61" t="n"/>
       <c r="H7" s="61" t="inlineStr">
         <is>
-          <t>Proponé una hora sin pantallas este fin de semana: una caminata, un tereré en familia, un juego de mesa.</t>
+          <t>Elegí un hábito de cuidado para la próxima semana y contáselo a alguien que te ayude a cumplirlo.</t>
         </is>
       </c>
       <c r="I7" s="61" t="inlineStr">
         <is>
-          <t>Apartarse del mal también es cuidarse de lo que desgasta por dentro: el enojo guardado, los conflictos sin resolver, las noches sin dormir.</t>
-        </is>
-      </c>
-      <c r="J7" s="61" t="inlineStr">
-        <is>
-          <t>Discusiones familiares que se arrastran toda la semana y estallan el fin de semana.</t>
-        </is>
-      </c>
-      <c r="K7" s="61" t="inlineStr">
-        <is>
-          <t>Antes del domingo, buscá a quien tengas algo pendiente y conversá en paz. Llegar reconciliado al culto también es cuidarse.</t>
-        </is>
-      </c>
+          <t>Los hábitos pequeños y constantes sostienen la energía: agua, movimiento, comidas en orden y horarios claros.</t>
+        </is>
+      </c>
+      <c r="J7" s="61" t="n"/>
+      <c r="K7" s="61" t="n"/>
       <c r="L7" s="61" t="inlineStr">
         <is>
-          <t>El alma también se cansa. Soltar cargas, perdonar y reconciliarse alivia hasta el cuerpo.</t>
-        </is>
-      </c>
-      <c r="M7" s="61" t="inlineStr">
-        <is>
-          <t>El agotamiento emocional que muchos esconden detrás de una vida activa.</t>
-        </is>
-      </c>
-      <c r="N7" s="61" t="inlineStr">
-        <is>
-          <t>Tomate diez minutos para revisar la semana: qué te cansó, qué te dio vida y qué vas a cambiar.</t>
-        </is>
-      </c>
+          <t>Descansar es parte del diseño de Dios. Dormir bien y parar a tiempo también es obediencia.</t>
+        </is>
+      </c>
+      <c r="M7" s="61" t="n"/>
+      <c r="N7" s="61" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="61" t="n">
@@ -19996,7 +19976,7 @@
       </c>
       <c r="C13" s="61" t="inlineStr">
         <is>
-          <t>Una herencia para los que vienen</t>
+          <t>Repaso: sembrar, trabajar y cuidar</t>
         </is>
       </c>
       <c r="D13" s="61" t="inlineStr">
@@ -20011,49 +19991,29 @@
       </c>
       <c r="F13" s="61" t="inlineStr">
         <is>
-          <t>Hay siembras que se hacen con lágrimas: una cosecha perdida, un año malo. Pero el dolor no tiene la última palabra.</t>
-        </is>
-      </c>
-      <c r="G13" s="61" t="inlineStr">
-        <is>
-          <t>El desánimo de muchos pequeños productores ante la incertidumbre del clima y los precios.</t>
-        </is>
-      </c>
+          <t>Lo que se siembra se cosecha, y la paciencia es parte de la siembra: no hay atajos.</t>
+        </is>
+      </c>
+      <c r="G13" s="61" t="n"/>
       <c r="H13" s="61" t="inlineStr">
         <is>
-          <t>Si conocés a un productor, preguntale cómo le va y ofrecé tu ayuda o tu oración.</t>
+          <t>Esta semana comprá a un productor de tu zona y plantá o cuidá un árbol con tu familia.</t>
         </is>
       </c>
       <c r="I13" s="61" t="inlineStr">
         <is>
-          <t>Lo que sembramos hoy lo van a disfrutar nuestros hijos y nietos.</t>
-        </is>
-      </c>
-      <c r="J13" s="61" t="inlineStr">
-        <is>
-          <t>La venta de tierras familiares sin planificación, que deja a las nuevas generaciones sin lugar.</t>
-        </is>
-      </c>
-      <c r="K13" s="61" t="inlineStr">
-        <is>
-          <t>Conversá en familia qué quieren dejar a la próxima generación: tierra, oficio, valores.</t>
-        </is>
-      </c>
+          <t>El trabajo de la tierra es bendición y desafío; se enfrenta mejor en comunidad y con orden.</t>
+        </is>
+      </c>
+      <c r="J13" s="61" t="n"/>
+      <c r="K13" s="61" t="n"/>
       <c r="L13" s="61" t="inlineStr">
         <is>
-          <t>Perseverar es seguir sembrando aunque el fruto tarde. La mejor época para plantar un árbol fue hace veinte años; la segunda es hoy.</t>
-        </is>
-      </c>
-      <c r="M13" s="61" t="inlineStr">
-        <is>
-          <t>Barrios sin sombra ni árboles, más calurosos cada verano.</t>
-        </is>
-      </c>
-      <c r="N13" s="61" t="inlineStr">
-        <is>
-          <t>Plantá un árbol nativo este fin de semana (lapacho, timbó o tajy) con los chicos, y pónganle nombre.</t>
-        </is>
-      </c>
+          <t>Cuidar la tierra es una responsabilidad con los que vienen detrás: es herencia, no solo recurso.</t>
+        </is>
+      </c>
+      <c r="M13" s="61" t="n"/>
+      <c r="N13" s="61" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="61" t="n">
@@ -20416,7 +20376,7 @@
       </c>
       <c r="C19" s="61" t="inlineStr">
         <is>
-          <t>Cuidar al que cuida</t>
+          <t>Repaso: prevenir es amar</t>
         </is>
       </c>
       <c r="D19" s="61" t="inlineStr">
@@ -20431,49 +20391,29 @@
       </c>
       <c r="F19" s="61" t="inlineStr">
         <is>
-          <t>Dios sana y también nos usa para acompañar a los que están enfermos.</t>
-        </is>
-      </c>
-      <c r="G19" s="61" t="inlineStr">
-        <is>
-          <t>La soledad de quienes enfrentan una enfermedad sin red de apoyo.</t>
-        </is>
-      </c>
+          <t>Prevenir: hábitos sencillos (comer mejor, moverse, vacunarse) evitan la mayoría de las enfermedades crónicas.</t>
+        </is>
+      </c>
+      <c r="G19" s="61" t="n"/>
       <c r="H19" s="61" t="inlineStr">
         <is>
-          <t>Pensá en una persona enferma de tu entorno y llevale algo concreto esta semana: una comida, una visita, una llamada.</t>
+          <t>Agendá tu control anual y ofrecé acompañar a alguien a hacerse el suyo.</t>
         </is>
       </c>
       <c r="I19" s="61" t="inlineStr">
         <is>
-          <t>Agradecer la salud es también cuidarla en familia, repartiendo el peso.</t>
-        </is>
-      </c>
-      <c r="J19" s="61" t="inlineStr">
-        <is>
-          <t>Familias que dejan toda la responsabilidad del cuidado en una sola persona.</t>
-        </is>
-      </c>
-      <c r="K19" s="61" t="inlineStr">
-        <is>
-          <t>Repartan en casa las tareas: quién acompaña al médico, quién compra los remedios, quién cocina.</t>
-        </is>
-      </c>
+          <t>Detectar a tiempo: los controles salvan vidas aunque no haya síntomas.</t>
+        </is>
+      </c>
+      <c r="J19" s="61" t="n"/>
+      <c r="K19" s="61" t="n"/>
       <c r="L19" s="61" t="inlineStr">
         <is>
-          <t>No olvidar los beneficios de cada día incluye valorar a quien cuida.</t>
-        </is>
-      </c>
-      <c r="M19" s="61" t="inlineStr">
-        <is>
-          <t>Cuidadores, casi siempre mujeres, agotados y sin tiempo para sí mismos.</t>
-        </is>
-      </c>
-      <c r="N19" s="61" t="inlineStr">
-        <is>
-          <t>Ofrecé unas horas de relevo a alguien que cuida a un familiar enfermo: que pueda salir, dormir o descansar.</t>
-        </is>
-      </c>
+          <t>Evitar complicaciones: seguir el tratamiento y acompañar al que está enfermo y al que lo cuida.</t>
+        </is>
+      </c>
+      <c r="M19" s="61" t="n"/>
+      <c r="N19" s="61" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="61" t="n">
@@ -20836,7 +20776,7 @@
       </c>
       <c r="C25" s="61" t="inlineStr">
         <is>
-          <t>Una Palabra que alimenta</t>
+          <t>Repaso: una Palabra que se estudia y se vive</t>
         </is>
       </c>
       <c r="D25" s="61" t="inlineStr">
@@ -20851,49 +20791,29 @@
       </c>
       <c r="F25" s="61" t="inlineStr">
         <is>
-          <t>Comer la Palabra es hacerla propia: no quedarse en la costumbre, sino buscar una relación personal.</t>
-        </is>
-      </c>
-      <c r="G25" s="61" t="inlineStr">
-        <is>
-          <t>La fe superficial, que se queda en costumbres sin una relación personal.</t>
-        </is>
-      </c>
+          <t>Estudiar la Biblia es más que leerla: detenerse, preguntar y aplicar.</t>
+        </is>
+      </c>
+      <c r="G25" s="61" t="n"/>
       <c r="H25" s="61" t="inlineStr">
         <is>
-          <t>Este fin de semana, reservá media hora tranquila solo para leer y orar, sin celular.</t>
+          <t>Elegí un plan de lectura de 30 días y buscá a alguien con quien compartirlo.</t>
         </is>
       </c>
       <c r="I25" s="61" t="inlineStr">
         <is>
-          <t>El gozo de la Palabra no depende del entusiasmo del día. La diligencia es seguir aunque no emocione.</t>
-        </is>
-      </c>
-      <c r="J25" s="61" t="inlineStr">
-        <is>
-          <t>Abandonar todo lo valioso apenas deja de ser entretenido.</t>
-        </is>
-      </c>
-      <c r="K25" s="61" t="inlineStr">
-        <is>
-          <t>Si te cuesta, cambiá el formato: un plan nuevo, otra traducción o la Biblia en audio.</t>
-        </is>
-      </c>
+          <t>Métodos sencillos ayudan: leer el contexto, escribir en un cuaderno y seguir un plan realista.</t>
+        </is>
+      </c>
+      <c r="J25" s="61" t="n"/>
+      <c r="K25" s="61" t="n"/>
       <c r="L25" s="61" t="inlineStr">
         <is>
-          <t>La alegría que da la Palabra se contagia y se hereda.</t>
-        </is>
-      </c>
-      <c r="M25" s="61" t="inlineStr">
-        <is>
-          <t>Generaciones que crecen sin referencias de fe en casa.</t>
-        </is>
-      </c>
-      <c r="N25" s="61" t="inlineStr">
-        <is>
-          <t>Regalá una Biblia o un devocional a un joven de tu familia con una dedicatoria escrita por vos.</t>
-        </is>
-      </c>
+          <t>Cuanto más hondo escarbamos, más conocemos a Dios y más se nota en la vida diaria.</t>
+        </is>
+      </c>
+      <c r="M25" s="61" t="n"/>
+      <c r="N25" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: apartado «Sobre Mensajero» desde la hoja «Mensajero» de la planilla
Identidad, historia, misión, visión, valores, contacto para la audiencia y
por áreas, organigrama, programas y locutores, y frases para el aire con
botón para copiar. Lo que falta queda marcado «por completar».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historia y Marcos" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guiones 2027" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mensajero" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -20818,4 +20819,620 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>Seccion</t>
+        </is>
+      </c>
+      <c r="B1" s="60" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="C1" s="60" t="inlineStr">
+        <is>
+          <t>Texto</t>
+        </is>
+      </c>
+      <c r="D1" s="60" t="inlineStr">
+        <is>
+          <t>Para el aire</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="61" t="inlineStr">
+        <is>
+          <t>Identidad</t>
+        </is>
+      </c>
+      <c r="B2" s="61" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="C2" s="61" t="inlineStr">
+        <is>
+          <t>Mensajero 100.9 FM</t>
+        </is>
+      </c>
+      <c r="D2" s="61" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>Identidad</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>Lema</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>Suena bien, hace bien</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="61" t="inlineStr">
+        <is>
+          <t>Identidad</t>
+        </is>
+      </c>
+      <c r="B4" s="61" t="inlineStr">
+        <is>
+          <t>Ministerio</t>
+        </is>
+      </c>
+      <c r="C4" s="61" t="inlineStr">
+        <is>
+          <t>Buenas Nuevas — Comunicación Integral</t>
+        </is>
+      </c>
+      <c r="D4" s="61" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>Identidad</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>Perfil</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>Radio cristiana evangélica interdenominacional.</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="61" t="inlineStr">
+        <is>
+          <t>Identidad</t>
+        </is>
+      </c>
+      <c r="B6" s="61" t="inlineStr">
+        <is>
+          <t>Ubicación</t>
+        </is>
+      </c>
+      <c r="C6" s="61" t="inlineStr">
+        <is>
+          <t>Tres Palmas, Raúl Arsenio Oviedo, Paraguay</t>
+        </is>
+      </c>
+      <c r="D6" s="61" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>Historia</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>Historia breve</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="61" t="inlineStr">
+        <is>
+          <t>Historia</t>
+        </is>
+      </c>
+      <c r="B8" s="61" t="inlineStr">
+        <is>
+          <t>Fecha de fundación</t>
+        </is>
+      </c>
+      <c r="C8" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D8" s="61" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>Propósito</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>Misión</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="61" t="inlineStr">
+        <is>
+          <t>Propósito</t>
+        </is>
+      </c>
+      <c r="B10" s="61" t="inlineStr">
+        <is>
+          <t>Visión</t>
+        </is>
+      </c>
+      <c r="C10" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D10" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>Contacto para la audiencia</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>WhatsApp y teléfono</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>+595 974 101 200</t>
+        </is>
+      </c>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="61" t="inlineStr">
+        <is>
+          <t>Contacto para la audiencia</t>
+        </is>
+      </c>
+      <c r="B12" s="61" t="inlineStr">
+        <is>
+          <t>Correo</t>
+        </is>
+      </c>
+      <c r="C12" s="61" t="inlineStr">
+        <is>
+          <t>radio@mensajerofm.org</t>
+        </is>
+      </c>
+      <c r="D12" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>Contacto para la audiencia</t>
+        </is>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>Sitio web</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="61" t="inlineStr">
+        <is>
+          <t>Contacto para la audiencia</t>
+        </is>
+      </c>
+      <c r="B14" s="61" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C14" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D14" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="61" t="inlineStr">
+        <is>
+          <t>Contacto para la audiencia</t>
+        </is>
+      </c>
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="61" t="inlineStr">
+        <is>
+          <t>Contacto para la audiencia</t>
+        </is>
+      </c>
+      <c r="B16" s="61" t="inlineStr">
+        <is>
+          <t>Escuchar en línea</t>
+        </is>
+      </c>
+      <c r="C16" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D16" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>Contacto por áreas</t>
+        </is>
+      </c>
+      <c r="B17" s="61" t="inlineStr">
+        <is>
+          <t>Dirección</t>
+        </is>
+      </c>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D17" s="61" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="61" t="inlineStr">
+        <is>
+          <t>Contacto por áreas</t>
+        </is>
+      </c>
+      <c r="B18" s="61" t="inlineStr">
+        <is>
+          <t>Programación</t>
+        </is>
+      </c>
+      <c r="C18" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D18" s="61" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="61" t="inlineStr">
+        <is>
+          <t>Contacto por áreas</t>
+        </is>
+      </c>
+      <c r="B19" s="61" t="inlineStr">
+        <is>
+          <t>Producción</t>
+        </is>
+      </c>
+      <c r="C19" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D19" s="61" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="61" t="inlineStr">
+        <is>
+          <t>Contacto por áreas</t>
+        </is>
+      </c>
+      <c r="B20" s="61" t="inlineStr">
+        <is>
+          <t>Técnica</t>
+        </is>
+      </c>
+      <c r="C20" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D20" s="61" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="61" t="inlineStr">
+        <is>
+          <t>Contacto por áreas</t>
+        </is>
+      </c>
+      <c r="B21" s="61" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="C21" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D21" s="61" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="61" t="inlineStr">
+        <is>
+          <t>Contacto por áreas</t>
+        </is>
+      </c>
+      <c r="B22" s="61" t="inlineStr">
+        <is>
+          <t>Prensa y redes</t>
+        </is>
+      </c>
+      <c r="C22" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D22" s="61" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="61" t="inlineStr">
+        <is>
+          <t>Contacto por áreas</t>
+        </is>
+      </c>
+      <c r="B23" s="61" t="inlineStr">
+        <is>
+          <t>Oración y consejería</t>
+        </is>
+      </c>
+      <c r="C23" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D23" s="61" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="61" t="inlineStr">
+        <is>
+          <t>Organigrama</t>
+        </is>
+      </c>
+      <c r="B24" s="61" t="inlineStr">
+        <is>
+          <t>Director/a</t>
+        </is>
+      </c>
+      <c r="C24" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D24" s="61" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="61" t="inlineStr">
+        <is>
+          <t>Organigrama</t>
+        </is>
+      </c>
+      <c r="B25" s="61" t="inlineStr">
+        <is>
+          <t>Coordinación de programación</t>
+        </is>
+      </c>
+      <c r="C25" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D25" s="61" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="61" t="inlineStr">
+        <is>
+          <t>Organigrama</t>
+        </is>
+      </c>
+      <c r="B26" s="61" t="inlineStr">
+        <is>
+          <t>Coordinación técnica</t>
+        </is>
+      </c>
+      <c r="C26" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D26" s="61" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="61" t="inlineStr">
+        <is>
+          <t>Organigrama</t>
+        </is>
+      </c>
+      <c r="B27" s="61" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="C27" s="61" t="inlineStr">
+        <is>
+          <t>(por completar)</t>
+        </is>
+      </c>
+      <c r="D27" s="61" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="61" t="inlineStr">
+        <is>
+          <t>Para el aire</t>
+        </is>
+      </c>
+      <c r="B28" s="61" t="inlineStr">
+        <is>
+          <t>Identificación de la radio</t>
+        </is>
+      </c>
+      <c r="C28" s="61" t="inlineStr">
+        <is>
+          <t>Estás escuchando Mensajero 100.9 FM. Suena bien, hace bien.</t>
+        </is>
+      </c>
+      <c r="D28" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="61" t="inlineStr">
+        <is>
+          <t>Para el aire</t>
+        </is>
+      </c>
+      <c r="B29" s="61" t="inlineStr">
+        <is>
+          <t>Cómo comunicarse</t>
+        </is>
+      </c>
+      <c r="C29" s="61" t="inlineStr">
+        <is>
+          <t>Escribinos al WhatsApp +595 974 101 200 o al correo radio@mensajerofm.org.</t>
+        </is>
+      </c>
+      <c r="D29" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="61" t="inlineStr">
+        <is>
+          <t>Para el aire</t>
+        </is>
+      </c>
+      <c r="B30" s="61" t="inlineStr">
+        <is>
+          <t>Edificando una Cultura</t>
+        </is>
+      </c>
+      <c r="C30" s="61" t="inlineStr">
+        <is>
+          <t>Este año, en Mensajero estamos Edificando una Cultura: cada semana un tema para crecer en la fe, la familia, el trabajo y la comunidad.</t>
+        </is>
+      </c>
+      <c r="D30" s="61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mensajero: versículos corregidos en la planilla
- Versículos y 3 puntos tomados de la planilla corregida (272 celdas, semanas 3 a 52);
  el resto conserva las tildes ya corregidas
- Formato «Cita — texto» y puntos con viñeta en toda la planilla
- Sin números de versículo pegados al texto (111 versículos)
- Revisión: 0 repetidos, 0 avisos; los guiones de enero no cambian

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -1517,7 +1517,7 @@
       </c>
       <c r="AB4" s="57" t="inlineStr">
         <is>
-          <t>Proverbios 14:26 El temor del Señor da plena confianza,
+          <t>Proverbios 14:26 — El temor del Señor da plena confianza,
 y da esperanza a nuestros hijos.</t>
         </is>
       </c>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="AD4" s="29" t="inlineStr">
         <is>
-          <t>Proverbios 4:20-22 —  Hijo mío, presta atención a mis palabras;
+          <t>Proverbios 4:20-22 — Hijo mío, presta atención a mis palabras;
 inclina tu oído para escuchar mis razones.
 No las pierdas de vista;
 guárdalas en lo más profundo de tu corazón.
@@ -1547,7 +1547,7 @@
       </c>
       <c r="AF4" s="59" t="inlineStr">
         <is>
-          <t>Proverbios 14:16 El sabio teme a Dios y se aparta del mal,
+          <t>Proverbios 14:16 — El sabio teme a Dios y se aparta del mal,
 pero el necio se muestra temerario y engreído.</t>
         </is>
       </c>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="AJ4" s="29" t="inlineStr">
         <is>
-          <t>Salmo 103:2-3 —¡Bendice, alma mía, al Señor, y no olvides ninguna de sus bendiciones!
+          <t>Salmo 103:2-3 — ¡Bendice, alma mía, al Señor, y no olvides ninguna de sus bendiciones!
 El Señor perdona todas tus maldades,
 y sana todas tus dolencias.</t>
         </is>
@@ -1982,14 +1982,14 @@
       </c>
       <c r="AJ6" s="33" t="inlineStr">
         <is>
-          <t>Galatas 6:9 — No nos cansemos, pues, de hacer el bien; porque a su tiempo cosecharemos, si no nos desanimamos.</t>
+          <t>1 Timoteo 3:2 — Pero es necesario que el obispo sea irreprensible y que tenga una sola esposa; que sea sobrio, prudente, decoroso, hospedador, apto para enseñar;</t>
         </is>
       </c>
       <c r="AK6" s="37" t="inlineStr">
         <is>
-          <t>• No cansarse de hacer el bien
-• La cosecha llega a su tiempo
-• Perseverar aunque no se vea fruto inmediato</t>
+          <t>• Ser íntegro y prudente.
+• Tener buen testimonio y carácter.
+• Ser hospitalario y apto para enseñar.</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2122,7 @@
       </c>
       <c r="Z7" s="34" t="inlineStr">
         <is>
-          <t>Proverbios 24:3-4 —La casa se edifica con sabiduría y se afirma con inteligencia.
+          <t>Proverbios 24:3-4 — La casa se edifica con sabiduría y se afirma con inteligencia.
 Sus habitaciones se llenan con buen juicio, y con todo bien preciado y agradable.</t>
         </is>
       </c>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="AJ7" s="34" t="inlineStr">
         <is>
-          <t>Colosenses 3:15 —Que en el corazón de ustedes gobierne la paz de Cristo, a la cual fueron llamados en un solo cuerpo. Y sean agradecidos.</t>
+          <t>Colosenses 3:15 — Que en el corazón de ustedes gobierne la paz de Cristo, a la cual fueron llamados en un solo cuerpo. Y sean agradecidos.</t>
         </is>
       </c>
       <c r="AK7" s="35" t="inlineStr">
@@ -2533,14 +2533,14 @@
       </c>
       <c r="Z9" s="42" t="inlineStr">
         <is>
-          <t>Proverbios 4:23 —Cuida tu corazón más que otra cosa, porque él es la fuente de la vida.</t>
+          <t>Mateo 5:37 — Cuando ustedes digan algo, que sea “sí, sí”, o “no, no”; porque lo que es más de esto, proviene del mal.</t>
         </is>
       </c>
       <c r="AA9" s="43" t="inlineStr">
         <is>
-          <t>• El corazón es la fuente de la vida
-• Cuidarlo con diligencia
-• De el salen las decisiones y emociones</t>
+          <t>• Hablar con honestidad.
+• Cumplir nuestra palabra.
+• Ser íntegros en nuestras decisiones.</t>
         </is>
       </c>
       <c r="AB9" s="42" t="inlineStr">
@@ -2557,17 +2557,14 @@
       </c>
       <c r="AD9" s="42" t="inlineStr">
         <is>
-          <t>Salmo 42:11 — ¿Por qué te desanimas, alma mía?
-¿Por qué te inquietas dentro de mí?
-Espera en Dios, porque aún debo alabarlo.
-¡Él es mi Dios! ¡Él es mi salvador!</t>
+          <t>Juan 3:16 — »Porque de tal manera amó Dios al mundo, que ha dado a su Hijo unigénito, para que todo aquel que en él cree no se pierda, sino que tenga vida eterna.</t>
         </is>
       </c>
       <c r="AE9" s="43" t="inlineStr">
         <is>
-          <t>• El desánimo se enfrenta esperando en Dios
-• Hablarle al alma propia es valido
-• La esperanza es una decisión activa</t>
+          <t>• Dios nos ama — Su amor es inmenso e incondicional.
+• Dios dio a su Hijo — Jesús es el regalo de salvación.
+• Creer en Jesús da vida eterna — La fe en Él nos libra de la perdición.</t>
         </is>
       </c>
       <c r="AF9" s="42" t="inlineStr">
@@ -2774,7 +2771,7 @@
         <is>
           <t>Genesis 30:29-30 — Y Jacob respondió:
 «Tú bien sabes cómo he trabajado para ti, y cómo ha estado tu ganado conmigo.
-30Lo poco que tenías antes de mi llegada, ha crecido en gran número. Con mi llegada el Señor te ha bendecido, pero ¿cuándo haré algo también por mi propia casa?»</t>
+Lo poco que tenías antes de mi llegada, ha crecido en gran número. Con mi llegada el Señor te ha bendecido, pero ¿cuándo haré algo también por mi propia casa?»</t>
         </is>
       </c>
       <c r="AG10" s="47" t="inlineStr">
@@ -2926,15 +2923,14 @@
       </c>
       <c r="X11" s="49" t="inlineStr">
         <is>
-          <t>Proverbios 27:23 —Mantente atento al estado de tus ovejas;
-cuida bien a tus rebaños,</t>
+          <t>1 Pedro 5:7 — Descarguen en él todas sus angustias, porque él tiene cuidado de ustedes.</t>
         </is>
       </c>
       <c r="Y11" s="49" t="inlineStr">
         <is>
-          <t>• Conocer bien el propio estado, también el de salud
-• La vigilancia regular previene sorpresas
-• No asumir que todo esta bien sin revisar</t>
+          <t>1, Entregar nuestras angustias a Dios.
+2, Confiar en su cuidado.
+3, Descansar en Él.</t>
         </is>
       </c>
       <c r="Z11" s="49" t="inlineStr">
@@ -2963,15 +2959,14 @@
       </c>
       <c r="AD11" s="49" t="inlineStr">
         <is>
-          <t>Jeremias 17: 14 ¡Sáname, Señor, y recobraré la salud! ¡Sálvame, y quedaré a salvo! ¡Tú eres la razón de mi alabanza!</t>
+          <t>Jeremias 17:14 — ¡Sáname, Señor, y recobraré la salud! ¡Sálvame, y quedaré a salvo! ¡Tú eres la razón de mi alabanza!</t>
         </is>
       </c>
       <c r="AE11" s="49" t="inlineStr">
         <is>
-          <t>Jeremías 17:14 – 3 puntos clave
-Dios sana: “Sáname, Señor” — confiamos en su poder.
-Dios salva: “Sálvame” — Él es nuestro refugio y seguridad.
-Dios merece alabanza: “Tú eres la razón de mi alabanza” — lo adoramos en todo momento.</t>
+          <t>• Dios sana: “Sáname, Señor”. Confiamos en su poder.
+• Dios salva: “Sálvame”. Él es nuestro refugio y seguridad.
+• Dios merece alabanza: “Tú eres la razón de mi alabanza”. Lo adoramos en todo momento.</t>
         </is>
       </c>
       <c r="AF11" s="49" t="inlineStr">
@@ -2988,7 +2983,7 @@
       </c>
       <c r="AH11" s="49" t="inlineStr">
         <is>
-          <t>Proverbios 12:15 —La necedad va ligada al corazón del joven,
+          <t>Proverbios 12:15 — La necedad va ligada al corazón del joven,
 pero la vara disciplinaria le quita lo necio.</t>
         </is>
       </c>
@@ -3001,18 +2996,18 @@
       </c>
       <c r="AJ11" s="49" t="inlineStr">
         <is>
-          <t>Eclesiastes 3:1-2 — Todo tiene su tiempo. Hay un momento bajo el cielo para toda actividad:
-2El momento en que se nace,
-y el momento en que se muere;
-el momento en que se planta,
-y el momento en que se cosecha;</t>
+          <t>Salmos 18:35-36 — Tú me diste el escudo de tu salvación,
+me sostuviste con tu mano derecha,
+y con tu bondad me engrandeciste.
+Me pusiste sobre un terreno espacioso,
+para que mis pies no resbalaran,</t>
         </is>
       </c>
       <c r="AK11" s="49" t="inlineStr">
         <is>
-          <t>• Hay tiempo para nacer y tiempo para morir
-• Aceptar los ciclos de la vida con sabiduría
-• El control médico ayuda a vivir ese tiempo con cuidado</t>
+          <t>• Dios nos protege: Él es nuestro escudo y nos sostiene.
+• Dios nos fortalece: Su bondad nos ayuda a crecer.
+• Dios nos guía: Afirma nuestros pasos para no caer.</t>
         </is>
       </c>
     </row>
@@ -3133,20 +3128,19 @@
       </c>
       <c r="X12" s="51" t="inlineStr">
         <is>
-          <t>Hebreos 10:24-25 — Tengámonos en cuenta unos a otros, a fin de estimularnos al amor y a las buenas obras.
-25No dejemos de congregarnos, como es la costumbre de algunos, sino animémonos unos a otros; y con más razón ahora que vemos que aquel día se acerca.</t>
+          <t>Mateo 18:20 — Porque donde dos o tres se reúnen en mi nombre, allí estoy yo, en medio de ellos.»</t>
         </is>
       </c>
       <c r="Y12" s="51" t="inlineStr">
         <is>
-          <t>• No abandonar la congregación
-• Exhortarnos mutuamente
-• Urgencia mayor cerca del final</t>
+          <t>• Reunirnos en su nombre: Buscar a Dios juntos.  
+• Jesús está presente: Él acompaña a quienes se reúnen en su nombre.  
+• Valorar la unidad: Juntos podemos crecer y fortalecer nuestra fe.</t>
         </is>
       </c>
       <c r="Z12" s="51" t="inlineStr">
         <is>
-          <t>Hechos 2:42 — Se mantenian fieles a las ensenanzas de los apostoles y en el mutuo companerismo, en el partimiento del pan y en las oraciones</t>
+          <t>Hechos 2:42 — las cuales se mantenían fieles a las enseñanzas de los apóstoles y en el mutuo compañerismo, en el partimiento del pan y en las oraciones.</t>
         </is>
       </c>
       <c r="AA12" s="51" t="inlineStr">
@@ -3158,8 +3152,8 @@
       </c>
       <c r="AB12" s="51" t="inlineStr">
         <is>
-          <t>Eclesiastes 4:9-10 — 9Dos son mejor que uno, porque sacan más provecho de sus esfuerzos.
-10Si uno de ellos se tropieza, el otro lo levanta.
+          <t>Eclesiastes 4:9-10 — Dos son mejor que uno, porque sacan más provecho de sus esfuerzos.
+Si uno de ellos se tropieza, el otro lo levanta.
 ¡Pero ay de aquel que tropieza y no hay quien lo levante!</t>
         </is>
       </c>
@@ -3172,7 +3166,7 @@
       </c>
       <c r="AD12" s="51" t="inlineStr">
         <is>
-          <t>1 Juan 1:7 — 7 Pero si vivimos en la luz, así como él está en la luz, tenemos comunión unos con otros, y la sangre de Jesús, su Hijo, nos limpia de todo pecado.</t>
+          <t>1 Juan 1:7 — Pero si vivimos en la luz, así como él está en la luz, tenemos comunión unos con otros, y la sangre de Jesús, su Hijo, nos limpia de todo pecado.</t>
         </is>
       </c>
       <c r="AE12" s="51" t="inlineStr">
@@ -3184,8 +3178,8 @@
       </c>
       <c r="AF12" s="51" t="inlineStr">
         <is>
-          <t>Romanos 12:4-5 —4 Porque así como en un cuerpo hay muchos miembros, y no todos los miembros tienen la misma función,
-5así también nosotros, aunque somos muchos, formamos un solo cuerpo en Cristo, y cada miembro está unido a los demás.</t>
+          <t>Romanos 12:4-5 — Porque así como en un cuerpo hay muchos miembros, y no todos los miembros tienen la misma función,
+así también nosotros, aunque somos muchos, formamos un solo cuerpo en Cristo, y cada miembro está unido a los demás.</t>
         </is>
       </c>
       <c r="AG12" s="51" t="inlineStr">
@@ -3197,7 +3191,7 @@
       </c>
       <c r="AH12" s="51" t="inlineStr">
         <is>
-          <t>Proverbios 27:17 — 17El hierro se pule con el hierro,
+          <t>Proverbios 27:17 — El hierro se pule con el hierro,
 y el hombre se pule en el trato con su prójimo.</t>
         </is>
       </c>
@@ -3210,8 +3204,8 @@
       </c>
       <c r="AJ12" s="51" t="inlineStr">
         <is>
-          <t>Filipenses 2:1-2 —1 Por tanto, si hay alguna consolación en Cristo, si algún consuelo de amor, si alguna comunión del Espíritu, si algún afecto entrañable, si alguna misericordia,
-2completen mi gozo sintiendo lo mismo, teniendo el mismo amor, unánimes, sintiendo una misma cosa.</t>
+          <t>Filipenses 2:1-2 — Por tanto, si hay alguna consolación en Cristo, si algún consuelo de amor, si alguna comunión del Espíritu, si algún afecto entrañable, si alguna misericordia,
+completen mi gozo sintiendo lo mismo, teniendo el mismo amor, unánimes, sintiendo una misma cosa.</t>
         </is>
       </c>
       <c r="AK12" s="51" t="inlineStr">
@@ -3339,7 +3333,7 @@
       </c>
       <c r="X13" s="53" t="inlineStr">
         <is>
-          <t>Proverbios 15:1 — 1La respuesta amable calma la ira;
+          <t>Proverbios 15:1 — La respuesta amable calma la ira;
 la respuesta grosera aumenta el enojo.</t>
         </is>
       </c>
@@ -3352,7 +3346,7 @@
       </c>
       <c r="Z13" s="53" t="inlineStr">
         <is>
-          <t>Santiago 1:19 — 19 Por eso, amados hermanos míos, todos ustedes deben estar dispuestos a oír, pero ser lentos para hablar y para enojarse,</t>
+          <t>Santiago 1:19 — Por eso, amados hermanos míos, todos ustedes deben estar dispuestos a oír, pero ser lentos para hablar y para enojarse,</t>
         </is>
       </c>
       <c r="AA13" s="53" t="inlineStr">
@@ -3364,8 +3358,8 @@
       </c>
       <c r="AB13" s="53" t="inlineStr">
         <is>
-          <t>Exodo 18:21-22 —21 Además, escoge de entre el pueblo algunos hombres respetables y temerosos de Dios, confiables y nada ambiciosos, y ponlos al frente de grupos de mil, cien, cincuenta y diez personas.
-22Que se ocupen ellos de juzgar al pueblo en todo momento, que dicten sentencia en cuestiones menores, y que a ti te remitan todo asunto de gravedad. Así aligerarás tu carga, pues ellos la llevarán contigo.</t>
+          <t>Exodo 18:21-22 — Además, escoge de entre el pueblo algunos hombres respetables y temerosos de Dios, confiables y nada ambiciosos, y ponlos al frente de grupos de mil, cien, cincuenta y diez personas.
+Que se ocupen ellos de juzgar al pueblo en todo momento, que dicten sentencia en cuestiones menores, y que a ti te remitan todo asunto de gravedad. Así aligerarás tu carga, pues ellos la llevarán contigo.</t>
         </is>
       </c>
       <c r="AC13" s="53" t="inlineStr">
@@ -3377,7 +3371,7 @@
       </c>
       <c r="AD13" s="53" t="inlineStr">
         <is>
-          <t>Proverbios 16:9 — 9 El corazón del hombre examina su camino,
+          <t>Proverbios 16:9 — El corazón del hombre examina su camino,
 pero el Señor le corrige el rumbo.</t>
         </is>
       </c>
@@ -3390,7 +3384,7 @@
       </c>
       <c r="AF13" s="53" t="inlineStr">
         <is>
-          <t>Eclesiastes 3:1 — 1Todo tiene su tiempo. Hay un momento bajo el cielo para toda actividad:</t>
+          <t>Eclesiastes 3:1 — Todo tiene su tiempo. Hay un momento bajo el cielo para toda actividad:</t>
         </is>
       </c>
       <c r="AG13" s="53" t="inlineStr">
@@ -3402,7 +3396,7 @@
       </c>
       <c r="AH13" s="53" t="inlineStr">
         <is>
-          <t>Proverbios 29:18 — 18Cuando no hay visión, el pueblo se desvía;
+          <t>Proverbios 29:18 — Cuando no hay visión, el pueblo se desvía;
 ¡dichoso aquel que obedece la ley!</t>
         </is>
       </c>
@@ -3415,7 +3409,7 @@
       </c>
       <c r="AJ13" s="53" t="inlineStr">
         <is>
-          <t>Colosenses 4:5 — 5Compórtense sabiamente con los no creyentes, y aprovechen bien el tiempo.</t>
+          <t>Colosenses 4:5 — Compórtense sabiamente con los no creyentes, y aprovechen bien el tiempo.</t>
         </is>
       </c>
       <c r="AK13" s="53" t="inlineStr">
@@ -3543,7 +3537,7 @@
       </c>
       <c r="X14" s="35" t="inlineStr">
         <is>
-          <t>Genesis 2:24 — 24Por eso el hombre dejará a su padre y a su madre, y se unirá a su mujer, y serán un solo ser.</t>
+          <t>Genesis 2:24 — Por eso el hombre dejará a su padre y a su madre, y se unirá a su mujer, y serán un solo ser.</t>
         </is>
       </c>
       <c r="Y14" s="35" t="inlineStr">
@@ -3555,7 +3549,7 @@
       </c>
       <c r="Z14" s="35" t="inlineStr">
         <is>
-          <t>Efesios 5:25 — 25Esposos, amen a sus esposas, así como Cristo amó a la iglesia, y se entregó a sí mismo por ella,</t>
+          <t>Efesios 5:25 — Esposos, amen a sus esposas, así como Cristo amó a la iglesia, y se entregó a sí mismo por ella,</t>
         </is>
       </c>
       <c r="AA14" s="35" t="inlineStr">
@@ -3567,7 +3561,7 @@
       </c>
       <c r="AB14" s="35" t="inlineStr">
         <is>
-          <t>Efesios 5:33 — 33Por lo demás, cada uno de ustedes ame también a su esposa como a sí mismo; y ustedes, las esposas, honren a sus esposos.</t>
+          <t>Efesios 5:33 — Por lo demás, cada uno de ustedes ame también a su esposa como a sí mismo; y ustedes, las esposas, honren a sus esposos.</t>
         </is>
       </c>
       <c r="AC14" s="35" t="inlineStr">
@@ -3579,24 +3573,22 @@
       </c>
       <c r="AD14" s="35" t="inlineStr">
         <is>
-          <t>Eclesiastes 4:9-10 — 9 Dos son mejor que uno, porque sacan más provecho de sus esfuerzos.
-10Si uno de ellos se tropieza, el otro lo levanta.
-¡Pero ay de aquel que tropieza y no hay quien lo levante!</t>
+          <t>1 Samuel 12:23 — Lejos estará de mí pecar contra el Señor dejando de rogar por ustedes; al contrario, me comprometo a instruirlos en el camino bueno y recto,</t>
         </is>
       </c>
       <c r="AE14" s="35" t="inlineStr">
         <is>
-          <t>• Dos logran más que uno solo
-• Hay ayuda mutua en la pareja
-• El apoyo mutuo sostiene en la caída</t>
+          <t>• Orar por otros: Interceder es una responsabilidad.
+• Enseñar el camino: Guiar a otros hacia lo bueno y correcto.
+• Servir con compromiso: No abandonar a quienes Dios puso a nuestro cuidado.</t>
         </is>
       </c>
       <c r="AF14" s="35" t="inlineStr">
         <is>
-          <t>1 Corintios 13:4-7 — 4El amor es paciente y bondadoso; no es envidioso ni presumido, no es orgulloso;
-5no hace nada impropio; no es egoísta ni se irrita; no es rencoroso;
-6no se alegra de la injusticia, sino que se une a la alegría de la verdad.
-7Todo lo sufre, todo lo cree, todo lo espera, todo lo soporta.</t>
+          <t>1 Corintios 13:4-7 — El amor es paciente y bondadoso; no es envidioso ni presumido, no es orgulloso;
+no hace nada impropio; no es egoísta ni se irrita; no es rencoroso;
+no se alegra de la injusticia, sino que se une a la alegría de la verdad.
+Todo lo sufre, todo lo cree, todo lo espera, todo lo soporta.</t>
         </is>
       </c>
       <c r="AG14" s="35" t="inlineStr">
@@ -3608,7 +3600,8 @@
       </c>
       <c r="AH14" s="35" t="inlineStr">
         <is>
-          <t>Proverbios 18:22 — Hallaste esposa? Has hallado el bien! Has alcanzado el favor del Senor</t>
+          <t>Proverbios 18:22 — ¿Hallaste esposa? ¡Has hallado el bien!
+¡Has alcanzado el favor del Señor!</t>
         </is>
       </c>
       <c r="AI14" s="35" t="inlineStr">
@@ -3620,7 +3613,7 @@
       </c>
       <c r="AJ14" s="35" t="inlineStr">
         <is>
-          <t>Cantares 8:7 — 7Las muchas aguas no pueden apagar el amor,
+          <t>Cantares 8:7 — Las muchas aguas no pueden apagar el amor,
 ni pueden tampoco sofocarlo los ríos.
 Si por el amor diera el hombre
 todos los bienes de su casa,
@@ -3752,30 +3745,26 @@
       </c>
       <c r="X15" s="40" t="inlineStr">
         <is>
-          <t>Lucas 14:28-30 — 28Porque ¿quién de ustedes que quiera levantar una torre, no se sienta primero a calcular los costos, para ver si tiene todo lo que necesita para terminarla?
-29No sea que después de haber puesto los cimientos, se dé cuenta de que no puede terminarla, y todos los que lo sepan comiencen a burlarse de él
-30y digan: “Este hombre comenzó a construir, y no pudo terminar.”</t>
+          <t>1 Corintios 9:26 — Así que yo corro y lucho, pero no sin una meta definida; no lo hago como si estuviera golpeando el viento;</t>
         </is>
       </c>
       <c r="Y15" s="40" t="inlineStr">
         <is>
-          <t>• Terminar lo que se empieza requiere calculo
-• No tener recursos suficientes es motivo de burla
-• Planificar previene la vergüenza</t>
+          <t>• Correr con propósito.
+• Luchar con perseverancia.
+• Vivir con dirección.</t>
         </is>
       </c>
       <c r="Z15" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 24:27 — 27Comienza por preparar tus campos
-y por disponerte para la siembra,
-y después de eso construye tu casa.</t>
+          <t>1 Corintios 15:58 — Así que, amados hermanos míos, manténganse firmes y constantes, y siempre creciendo en la obra del Señor, seguros de que el trabajo de ustedes en el Señor no carece de sentido.</t>
         </is>
       </c>
       <c r="AA15" s="40" t="inlineStr">
         <is>
-          <t>• Preparar antes de construir
-• El orden en el trabajo precede al resultado
-• La preparación evita el caos</t>
+          <t>• Mantenerse firmes: No rendirse en la fe.
+• Seguir creciendo: Perseverar en la obra del Señor.
+• Confiar en Dios: Nuestro servicio nunca es en vano.</t>
         </is>
       </c>
       <c r="AB15" s="40" t="inlineStr">
@@ -3793,53 +3782,51 @@
       </c>
       <c r="AD15" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 27:23 — 23Mantente atento al estado de tus ovejas;
-cuida bien a tus rebaños,</t>
+          <t>Mateo 10:16 — »Tengan ustedes en cuenta que los estoy enviando como a ovejas en medio de lobos; así que sean prudentes como serpientes y sencillos como palomas.</t>
         </is>
       </c>
       <c r="AE15" s="40" t="inlineStr">
         <is>
-          <t>• Conocer el estado propio con diligencia
-• No asumir que todo esta bien sin revisar
-• La vigilancia regular previene sorpresas</t>
+          <t>1, Ser prudentes.
+2, Ser sencillos.
+3, Cumplir nuestra misión.</t>
         </is>
       </c>
       <c r="AF15" s="40" t="inlineStr">
         <is>
-          <t>1 Corintios 14:40 — 40siempre y cuando todo se haga decentemente y con orden.</t>
+          <t>Efesios 5:15-16 — Por tanto, ¡cuidado con su manera de vivir! No vivan ya como necios, sino como sabios.
+Aprovechen bien el tiempo, porque los días son malos.</t>
         </is>
       </c>
       <c r="AG15" s="40" t="inlineStr">
         <is>
-          <t>• El orden aplica también a las finanzas
-• La decencia en el manejo del dinero
-• Estructura clara evita el descontrol</t>
+          <t>• Vivir con sabiduría.
+• Cuidar nuestra manera de vivir.
+• Aprovechar bien el tiempo.</t>
         </is>
       </c>
       <c r="AH15" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 16:9 — 9El corazón del hombre examina su camino,
-pero el Señor le corrige el rumbo.</t>
+          <t>1 Corintios 16:2 — Cada primer día de la semana, cada uno de ustedes ponga algo aparte, según lo que haya ganado, y guárdelo, para que no se tengan que recoger las ofrendas cuando yo esté allá.</t>
         </is>
       </c>
       <c r="AI15" s="40" t="inlineStr">
         <is>
-          <t>• Planificar es humano, Dios dirige el resultado
-• Someter el presupuesto a Su voluntad
-• Flexibilidad ante los ajustes necesarios</t>
+          <t>• Dar según lo recibido.
+• Ser constantes en dar.
+• Dar con responsabilidad y propósito.</t>
         </is>
       </c>
       <c r="AJ15" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 22:3 — 3El que es astuto, ve el peligro y se esconde;
-el que es ingenuo, sigue adelante y es afectado.</t>
+          <t>1 Corintios 4:2 — Ahora bien, de los administradores se espera que demuestren ser dignos de confianza.</t>
         </is>
       </c>
       <c r="AK15" s="40" t="inlineStr">
         <is>
-          <t>• El prudente anticipa el riesgo
-• El imprudente sigue de largo y sufre
-• Ver venir el problema evita el daño</t>
+          <t>• Ser confiables.
+• Administrar bien lo recibido.
+• Ser fieles a Dios.</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3947,7 @@
       </c>
       <c r="X16" s="43" t="inlineStr">
         <is>
-          <t>Juan 15:5 — 5Yo soy la vid y ustedes las ramas; el que permanece en mí, y yo en él, este lleva mucho fruto; porque separados de mí ustedes nada pueden hacer.</t>
+          <t>Juan 15:5 — Yo soy la vid y ustedes las ramas; el que permanece en mí, y yo en él, este lleva mucho fruto; porque separados de mí ustedes nada pueden hacer.</t>
         </is>
       </c>
       <c r="Y16" s="43" t="inlineStr">
@@ -3972,8 +3959,8 @@
       </c>
       <c r="Z16" s="43" t="inlineStr">
         <is>
-          <t>Galatas 5:22-23 — 22Pero el fruto del Espíritu es amor, gozo, paz, paciencia, benignidad, bondad, fe,
-23mansedumbre, templanza. Contra tales cosas no hay ley.</t>
+          <t>Galatas 5:22-23 — Pero el fruto del Espíritu es amor, gozo, paz, paciencia, benignidad, bondad, fe,
+mansedumbre, templanza. Contra tales cosas no hay ley.</t>
         </is>
       </c>
       <c r="AA16" s="43" t="inlineStr">
@@ -3985,7 +3972,7 @@
       </c>
       <c r="AB16" s="43" t="inlineStr">
         <is>
-          <t>Salmo 63:1 — 1Dios mío, ¡tú eres mi Dios!
+          <t>Salmo 63:1 — Dios mío, ¡tú eres mi Dios!
 Yo te buscaré de madrugada.
 Mi alma tiene sed de ti;
 mi ser entero te busca con ansias,
@@ -4001,7 +3988,7 @@
       </c>
       <c r="AD16" s="43" t="inlineStr">
         <is>
-          <t>Isaias 40:31 —31pero los que confían en el Señor recobran las fuerzas y levantan el vuelo, como las águilas; corren, y no se cansan; caminan, y no se fatigan.</t>
+          <t>Isaias 40:31 — pero los que confían en el Señor recobran las fuerzas y levantan el vuelo, como las águilas; corren, y no se cansan; caminan, y no se fatigan.</t>
         </is>
       </c>
       <c r="AE16" s="43" t="inlineStr">
@@ -4013,7 +4000,7 @@
       </c>
       <c r="AF16" s="43" t="inlineStr">
         <is>
-          <t>2 Pedro 3:18 — 18Más bien, crezcan en la gracia y el conocimiento de nuestro Señor y Salvador Jesucristo, a quien sea dada la gloria ahora y hasta el día de la eternidad. Amén.</t>
+          <t>2 Pedro 3:18 — Más bien, crezcan en la gracia y el conocimiento de nuestro Señor y Salvador Jesucristo, a quien sea dada la gloria ahora y hasta el día de la eternidad. Amén.</t>
         </is>
       </c>
       <c r="AG16" s="43" t="inlineStr">
@@ -4025,7 +4012,7 @@
       </c>
       <c r="AH16" s="43" t="inlineStr">
         <is>
-          <t>Salmo 42:1 —1Como ciervo que anhela las corrientes de agua,
+          <t>Salmo 42:1 — Como ciervo que anhela las corrientes de agua,
 así mi alma clama por ti, mi Dios.</t>
         </is>
       </c>
@@ -4038,8 +4025,8 @@
       </c>
       <c r="AJ16" s="43" t="inlineStr">
         <is>
-          <t>Colosenses 2:6-7 —6Por tanto, vivan en el Señor Jesucristo de la manera que lo recibieron:
-7arraigados y sobreedificados en él, confirmados en la fe y llenos de acciones de gracias, que es como fueron enseñados.</t>
+          <t>Colosenses 2:6-7 — Por tanto, vivan en el Señor Jesucristo de la manera que lo recibieron:
+arraigados y sobreedificados en él, confirmados en la fe y llenos de acciones de gracias, que es como fueron enseñados.</t>
         </is>
       </c>
       <c r="AK16" s="43" t="inlineStr">
@@ -4167,7 +4154,7 @@
       </c>
       <c r="X17" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 16:3 —3Encomienda al Señor tus acciones,
+          <t>Proverbios 16:3 — Encomienda al Señor tus acciones,
 y tus pensamientos serán afirmados.</t>
         </is>
       </c>
@@ -4180,7 +4167,7 @@
       </c>
       <c r="Z17" s="47" t="inlineStr">
         <is>
-          <t>Deuteronomio 8:18 — 18Más bien, acuérdate del Señor tu Dios, porque él es quien te da el poder de ganar esas riquezas, a fin de confirmar el pacto que hizo con tus padres, como en este día.</t>
+          <t>Deuteronomio 8:18 — Más bien, acuérdate del Señor tu Dios, porque él es quien te da el poder de ganar esas riquezas, a fin de confirmar el pacto que hizo con tus padres, como en este día.</t>
         </is>
       </c>
       <c r="AA17" s="47" t="inlineStr">
@@ -4192,7 +4179,7 @@
       </c>
       <c r="AB17" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 22:29 — 29 Cuando veas alguien que hace bien su trabajo,
+          <t>Proverbios 22:29 — Cuando veas alguien que hace bien su trabajo,
 no lo verás entre gente de baja condición
 sino que estará en presencia de reyes.</t>
         </is>
@@ -4206,8 +4193,8 @@
       </c>
       <c r="AD17" s="47" t="inlineStr">
         <is>
-          <t>Eclesiastes 5:18-19 — 18Pero algo bueno he visto. Y es que no hay nada mejor que comer y beber y gozar, cada día de nuestra vida, del fruto del trabajo con que nos agobiamos bajo el sol. Esa es la herencia que de Dios hemos recibido.
-19A cada uno de nosotros Dios nos ha dado riquezas y bienes, y también nos ha dado el derecho de consumirlas. Tomar nuestra parte y disfrutar de nuestro trabajo es un don de Dios.</t>
+          <t>Eclesiastes 5:18-19 — Pero algo bueno he visto. Y es que no hay nada mejor que comer y beber y gozar, cada día de nuestra vida, del fruto del trabajo con que nos agobiamos bajo el sol. Esa es la herencia que de Dios hemos recibido.
+A cada uno de nosotros Dios nos ha dado riquezas y bienes, y también nos ha dado el derecho de consumirlas. Tomar nuestra parte y disfrutar de nuestro trabajo es un don de Dios.</t>
         </is>
       </c>
       <c r="AE17" s="47" t="inlineStr">
@@ -4219,23 +4206,20 @@
       </c>
       <c r="AF17" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 27:23-24 —23Mantente atento al estado de tus ovejas;
-cuida bien a tus rebaños,
-24porque las riquezas no duran para siempre
-ni la corona permanece eternamente.</t>
+          <t>Jeremías 17:7 — »Pero bendito el hombre que confía en mí, que soy el Señor, y que en mí pone su confianza.</t>
         </is>
       </c>
       <c r="AG17" s="47" t="inlineStr">
         <is>
-          <t>• Conocer bien el estado del negocio
-• Las riquezas no son permanentes sin cuidado
-• La vigilancia constante protege lo construido</t>
+          <t>• Confiar en Dios.
+• Poner nuestra confianza en Él.
+• Vivir bajo su bendición.</t>
         </is>
       </c>
       <c r="AH17" s="47" t="inlineStr">
         <is>
-          <t>Colosenses 3:23-24 — 23Y todo lo que hagan, háganlo de corazón, como para el Señor y no como para la gente,
-24porque ya saben que el Señor les dará la herencia como recompensa, pues ustedes sirven a Cristo el Señor.</t>
+          <t>Colosenses 3:23-24 — Y todo lo que hagan, háganlo de corazón, como para el Señor y no como para la gente,
+porque ya saben que el Señor les dará la herencia como recompensa, pues ustedes sirven a Cristo el Señor.</t>
         </is>
       </c>
       <c r="AI17" s="47" t="inlineStr">
@@ -4247,7 +4231,7 @@
       </c>
       <c r="AJ17" s="47" t="inlineStr">
         <is>
-          <t>Salmo 90:17 — 17Señor y Dios nuestro, ¡muéstranos tu bondad
+          <t>Salmo 90:17 — Señor y Dios nuestro, ¡muéstranos tu bondad
 y confirma la obra de nuestras manos!
 ¡Sí, confirma la obra de nuestras manos!</t>
         </is>
@@ -4377,22 +4361,21 @@
       </c>
       <c r="X18" s="56" t="inlineStr">
         <is>
-          <t>Proverbios 13:4 El perezoso desea y nada consigue,
+          <t>Proverbios 13:4 — El perezoso desea y nada consigue,
 pero el que se esfuerza será prosperado.</t>
         </is>
       </c>
       <c r="Y18" s="49" t="inlineStr">
         <is>
-          <t>Proverbios 13:4 – 3 puntos clave
-* No basta con desear: Los sueños necesitan acción y compromiso.
+          <t>* No basta con desear: Los sueños necesitan acción y compromiso.
 * El esfuerzo trae resultados: El que trabaja con dedicación puede alcanzar buenos frutos.
 * Dios bendice la perseverancia: La constancia y la responsabilidad abren camino al progreso.</t>
         </is>
       </c>
       <c r="Z18" s="49" t="inlineStr">
         <is>
-          <t>1 Corintios 9:24-25 —24¿Acaso no saben ustedes que, aunque todos corren en el estadio, solamente uno se lleva el premio? Corran, pues, de tal manera que lo obtengan.
-25Todos los que luchan, se abstienen de todo. Ellos lo hacen para recibir una corona corruptible; pero nosotros, para recibir una corona incorruptible.</t>
+          <t>1 Corintios 9:24-25 — ¿Acaso no saben ustedes que, aunque todos corren en el estadio, solamente uno se lleva el premio? Corran, pues, de tal manera que lo obtengan.
+Todos los que luchan, se abstienen de todo. Ellos lo hacen para recibir una corona corruptible; pero nosotros, para recibir una corona incorruptible.</t>
         </is>
       </c>
       <c r="AA18" s="49" t="inlineStr">
@@ -4404,7 +4387,7 @@
       </c>
       <c r="AB18" s="49" t="inlineStr">
         <is>
-          <t>1 Corintios 9:27 — 27más bien, golpeo mi cuerpo y lo someto a servidumbre, no sea que después de haber predicado a otros yo mismo quede eliminado.</t>
+          <t>1 Corintios 9:27 — más bien, golpeo mi cuerpo y lo someto a servidumbre, no sea que después de haber predicado a otros yo mismo quede eliminado.</t>
         </is>
       </c>
       <c r="AC18" s="49" t="inlineStr">
@@ -4416,7 +4399,7 @@
       </c>
       <c r="AD18" s="49" t="inlineStr">
         <is>
-          <t>Hebreos 12:1 —1Por lo tanto, también nosotros, que tenemos tan grande nube de testigos a nuestro alrededor, liberémonos de todo peso y del pecado que nos asedia, y corramos con paciencia la carrera que tenemos por delante.</t>
+          <t>Hebreos 12:1 — Por lo tanto, también nosotros, que tenemos tan grande nube de testigos a nuestro alrededor, liberémonos de todo peso y del pecado que nos asedia, y corramos con paciencia la carrera que tenemos por delante.</t>
         </is>
       </c>
       <c r="AE18" s="49" t="inlineStr">
@@ -4428,9 +4411,9 @@
       </c>
       <c r="AF18" s="49" t="inlineStr">
         <is>
-          <t>Salmo 18:32-33 — 32Dios es quien me da fuerzas;
+          <t>Salmo 18:32-33 — Dios es quien me da fuerzas;
 Dios es quien endereza mi camino;
-33Dios es quien me aligera los pies
+Dios es quien me aligera los pies
 y me hace correr como un venado;
 Dios es quien me afirma en las alturas;</t>
         </is>
@@ -4444,7 +4427,7 @@
       </c>
       <c r="AH18" s="49" t="inlineStr">
         <is>
-          <t>Genesis 2:15 — 15Dios el Señor tomó al hombre y lo puso en el huerto de Edén, para que lo cultivara y lo cuidara.</t>
+          <t>Genesis 2:15 — Dios el Señor tomó al hombre y lo puso en el huerto de Edén, para que lo cultivara y lo cuidara.</t>
         </is>
       </c>
       <c r="AI18" s="49" t="inlineStr">
@@ -4585,7 +4568,7 @@
       </c>
       <c r="X19" s="51" t="inlineStr">
         <is>
-          <t>Galatas 5:13 —Hermanos, ustedes han sido llamados a la libertad, solo que no usen la libertad como pretexto para pecar; más bien, sírvanse los unos a los otros por amor.</t>
+          <t>Galatas 5:13 — Hermanos, ustedes han sido llamados a la libertad, solo que no usen la libertad como pretexto para pecar; más bien, sírvanse los unos a los otros por amor.</t>
         </is>
       </c>
       <c r="Y19" s="51" t="inlineStr">
@@ -4621,8 +4604,8 @@
       </c>
       <c r="AD19" s="51" t="inlineStr">
         <is>
-          <t>Juan 13:14-15 — 14Pues si yo, el Señor y el Maestro, les he lavado los pies, también ustedes deben lavarse los pies unos a otros.
-15Porque les he puesto el ejemplo, para que lo mismo que yo he hecho con ustedes, también ustedes lo hagan.</t>
+          <t>Juan 13:14-15 — Pues si yo, el Señor y el Maestro, les he lavado los pies, también ustedes deben lavarse los pies unos a otros.
+Porque les he puesto el ejemplo, para que lo mismo que yo he hecho con ustedes, también ustedes lo hagan.</t>
         </is>
       </c>
       <c r="AE19" s="51" t="inlineStr">
@@ -4634,7 +4617,7 @@
       </c>
       <c r="AF19" s="51" t="inlineStr">
         <is>
-          <t>Colosenses 3:23 — 23Y todo lo que hagan, háganlo de corazón, como para el Señor y no como para la gente,</t>
+          <t>Colosenses 3:23 — Y todo lo que hagan, háganlo de corazón, como para el Señor y no como para la gente,</t>
         </is>
       </c>
       <c r="AG19" s="51" t="inlineStr">
@@ -4646,7 +4629,7 @@
       </c>
       <c r="AH19" s="51" t="inlineStr">
         <is>
-          <t>Mateo 25:40 — 40Y el Rey les responderá: “De cierto les digo que todo lo que hicieron por uno de mis hermanos más pequeños, por mí lo hicieron.”</t>
+          <t>Mateo 25:40 — Y el Rey les responderá: “De cierto les digo que todo lo que hicieron por uno de mis hermanos más pequeños, por mí lo hicieron.”</t>
         </is>
       </c>
       <c r="AI19" s="51" t="inlineStr">
@@ -4658,7 +4641,7 @@
       </c>
       <c r="AJ19" s="51" t="inlineStr">
         <is>
-          <t>Hechos 20:35 —35Siempre les enseñé, y ustedes lo aprendieron, que a los necesitados se les ayuda trabajando como he trabajado yo, y recordando las palabras del Señor Jesús, que dijo: “Hay más bendición en dar que en recibir.”»</t>
+          <t>Hechos 20:35 — Siempre les enseñé, y ustedes lo aprendieron, que a los necesitados se les ayuda trabajando como he trabajado yo, y recordando las palabras del Señor Jesús, que dijo: “Hay más bendición en dar que en recibir.”»</t>
         </is>
       </c>
       <c r="AK19" s="51" t="inlineStr">
@@ -4786,8 +4769,8 @@
       </c>
       <c r="X20" s="53" t="inlineStr">
         <is>
-          <t>2 Corintios 4:8-9 — 8que estamos en dificultades, pero no angustiados; en apuros, pero no desesperados;
-9perseguidos, pero no desamparados; derribados, pero no destruidos;</t>
+          <t>2 Corintios 4:8-9 — que estamos en dificultades, pero no angustiados; en apuros, pero no desesperados;
+perseguidos, pero no desamparados; derribados, pero no destruidos;</t>
         </is>
       </c>
       <c r="Y20" s="53" t="inlineStr">
@@ -4799,7 +4782,7 @@
       </c>
       <c r="Z20" s="53" t="inlineStr">
         <is>
-          <t>Nehemias 4:14 —14Luego, me reuní con los hombres importantes del pueblo y con los oficiales del templo, y con el pueblo en general, y les dije: “No tengan miedo de esa gente. Recuerden que el Señor es grande y temible. Luchemos por defender a nuestros hermanos, nuestros hijos, nuestras hijas y nuestras esposas; ¡luchemos por nuestros hogares!”</t>
+          <t>Nehemias 4:14 — Luego, me reuní con los hombres importantes del pueblo y con los oficiales del templo, y con el pueblo en general, y les dije: “No tengan miedo de esa gente. Recuerden que el Señor es grande y temible. Luchemos por defender a nuestros hermanos, nuestros hijos, nuestras hijas y nuestras esposas; ¡luchemos por nuestros hogares!”</t>
         </is>
       </c>
       <c r="AA20" s="53" t="inlineStr">
@@ -4811,8 +4794,8 @@
       </c>
       <c r="AB20" s="53" t="inlineStr">
         <is>
-          <t>1 Pedro 5:8-9 — 8Sean prudentes y manténganse atentos, porque su enemigo es el diablo, y él anda como un león rugiente, buscando a quien devorar.
-9Pero ustedes, manténganse firmes y háganle frente. Sepan que en todo el mundo sus hermanos están enfrentando los mismos sufrimientos,</t>
+          <t>1 Pedro 5:8-9 — Sean prudentes y manténganse atentos, porque su enemigo es el diablo, y él anda como un león rugiente, buscando a quien devorar.
+Pero ustedes, manténganse firmes y háganle frente. Sepan que en todo el mundo sus hermanos están enfrentando los mismos sufrimientos,</t>
         </is>
       </c>
       <c r="AC20" s="53" t="inlineStr">
@@ -4824,19 +4807,19 @@
       </c>
       <c r="AD20" s="53" t="inlineStr">
         <is>
-          <t>Isaias 40:31 —31pero los que confían en el Señor recobran las fuerzas y levantan el vuelo, como las águilas; corren, y no se cansan; caminan, y no se fatigan.</t>
+          <t>Hebreos 13:7 — Acuérdense de sus pastores, que les dieron a conocer la palabra de Dios. Piensen en los resultados de su conducta, e imiten su fe.</t>
         </is>
       </c>
       <c r="AE20" s="53" t="inlineStr">
         <is>
-          <t>• Esperar en Dios renueva las fuerzas
-• El cansancio no es el final
-• Correr sin fatigarse es promesa para quien espera</t>
+          <t>• Recordar a nuestros pastores — Valorar a quienes nos enseñan la Palabra.
+• Observar su ejemplo — Aprender de su conducta y testimonio.
+• Imitar su fe — Seguir su confianza y fidelidad a Dios.</t>
         </is>
       </c>
       <c r="AF20" s="53" t="inlineStr">
         <is>
-          <t>Filipenses 4:13 —13¡todo lo puedo en Cristo que me fortalece!</t>
+          <t>Filipenses 4:13 — ¡todo lo puedo en Cristo que me fortalece!</t>
         </is>
       </c>
       <c r="AG20" s="53" t="inlineStr">
@@ -4848,7 +4831,7 @@
       </c>
       <c r="AH20" s="53" t="inlineStr">
         <is>
-          <t>Josue 1:9 — 9Escucha lo que te mando: Esfuérzate y sé valiente. No temas ni desmayes, que yo soy el Señor tu Dios, y estaré contigo por dondequiera que vayas.»</t>
+          <t>Josue 1:9 — Escucha lo que te mando: Esfuérzate y sé valiente. No temas ni desmayes, que yo soy el Señor tu Dios, y estaré contigo por dondequiera que vayas.»</t>
         </is>
       </c>
       <c r="AI20" s="53" t="inlineStr">
@@ -4860,7 +4843,7 @@
       </c>
       <c r="AJ20" s="53" t="inlineStr">
         <is>
-          <t>Romanos 8:28 —28Ahora bien, sabemos que Dios dispone todas las cosas para el bien de los que lo aman, es decir, de los que él ha llamado de acuerdo a su propósito.</t>
+          <t>Romanos 8:28 — Ahora bien, sabemos que Dios dispone todas las cosas para el bien de los que lo aman, es decir, de los que él ha llamado de acuerdo a su propósito.</t>
         </is>
       </c>
       <c r="AK20" s="53" t="inlineStr">
@@ -4988,7 +4971,7 @@
       </c>
       <c r="X21" s="35" t="inlineStr">
         <is>
-          <t>Salmo 127:3 — 3Los hijos son un regalo del Señor;
+          <t>Salmo 127:3 — Los hijos son un regalo del Señor;
 los frutos del vientre son nuestra recompensa.</t>
         </is>
       </c>
@@ -5001,7 +4984,7 @@
       </c>
       <c r="Z21" s="35" t="inlineStr">
         <is>
-          <t>Proverbios 22:6 — 6Enseña al niño a seguir fielmente su camino,
+          <t>Proverbios 22:6 — Enseña al niño a seguir fielmente su camino,
 y aunque llegue a anciano no se apartará de él.</t>
         </is>
       </c>
@@ -5014,7 +4997,7 @@
       </c>
       <c r="AB21" s="35" t="inlineStr">
         <is>
-          <t>Efesios 6:4 — 4Ustedes, los padres, no hagan enojar a sus hijos, sino edúquenlos en la disciplina y la instrucción del Señor.</t>
+          <t>Efesios 6:4 — Ustedes, los padres, no hagan enojar a sus hijos, sino edúquenlos en la disciplina y la instrucción del Señor.</t>
         </is>
       </c>
       <c r="AC21" s="35" t="inlineStr">
@@ -5026,7 +5009,7 @@
       </c>
       <c r="AD21" s="35" t="inlineStr">
         <is>
-          <t>Proverbios 29:17 — 17Corrige a tu hijo, y vivirás tranquilo,
+          <t>Proverbios 29:17 — Corrige a tu hijo, y vivirás tranquilo,
 y a ti mismo te dará grandes alegrías.</t>
         </is>
       </c>
@@ -5040,7 +5023,7 @@
       <c r="AF21" s="35" t="inlineStr">
         <is>
           <t>Deuteronomio 6:6-7 — Estas palabras que hoy te mando cumplir estarán en tu corazón,
-7y se las repetirás a tus hijos, y hablarás de ellas cuando estés en tu casa, y cuando vayas por el camino, y cuando te acuestes y cuando te levantes.</t>
+y se las repetirás a tus hijos, y hablarás de ellas cuando estés en tu casa, y cuando vayas por el camino, y cuando te acuestes y cuando te levantes.</t>
         </is>
       </c>
       <c r="AG21" s="35" t="inlineStr">
@@ -5256,22 +5239,21 @@
       </c>
       <c r="AH22" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 13:11 — Las ilusorias riquezas pronto se gastan;
-el que trabaja y las guarda las hace crecer.</t>
+          <t>Santiago 3:17 — Pero la sabiduría que viene de lo alto es, ante todo, pura, y además pacífica, amable, benigna, llena de compasión y de buenos frutos, imparcial y genuina.</t>
         </is>
       </c>
       <c r="AI22" s="40" t="inlineStr">
         <is>
-          <t>• Las riquezas mal habidas disminuyen
-• Lo ganado con esfuerzo permanece
-• El origen del ingreso importa</t>
+          <t>• Sabiduría pura.
+• Actuar con amabilidad y compasión.
+• Dar buenos frutos.</t>
         </is>
       </c>
       <c r="AJ22" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 11:24-25 — 24A quienes reparten, más se les da;
+          <t>Proverbios 11:24-25 — A quienes reparten, más se les da;
 los tacaños acaban en la pobreza.
-25El que es generoso, prospera;
+El que es generoso, prospera;
 el que da a otros, también recibirá.</t>
         </is>
       </c>
@@ -5400,28 +5382,26 @@
       </c>
       <c r="X23" s="43" t="inlineStr">
         <is>
-          <t>Colosenses 3:23 — Y todo lo que hagan, háganlo de corazón, como para el Señor y no como para la gente,</t>
+          <t>1 Corintios 16:13 — Manténganse atentos y firmes en la fe; sean fuertes y valientes.</t>
         </is>
       </c>
       <c r="Y23" s="43" t="inlineStr">
         <is>
-          <t>• Trabajar de corazón, como para el Señor
-• La actitud eleva cualquier tarea
-• El trabajo tiene valor espiritual</t>
+          <t>• Manténganse atentos — Estar vigilantes espiritualmente.
+• Permanezcan firmes en la fe — No apartarse de Dios.
+• Sean fuertes y valientes — Enfrentar las dificultades con valor.</t>
         </is>
       </c>
       <c r="Z23" s="43" t="inlineStr">
         <is>
-          <t>Proverbios 22:29 — Cuando veas alguien que hace bien su trabajo,
-no lo verás entre gente de baja condición
-sino que estará en presencia de reyes.</t>
+          <t>1 Pedro 3:15 — Al contrario, honren en su corazón a Cristo, como Señor, y manténganse siempre listos para defenderse, con mansedumbre y respeto, ante aquellos que les pidan explicarles la esperanza que hay en ustedes.</t>
         </is>
       </c>
       <c r="AA23" s="43" t="inlineStr">
         <is>
-          <t>• El hombre diligente llega lejos
-• La excelencia abre puertas
-• El esfuerzo se nota y se reconoce</t>
+          <t>• Honrar a Cristo — Poner a Jesús en el centro.
+• Estar preparados — Saber explicar nuestra esperanza.
+• Responder con respeto — Hablar con mansedumbre y amor.</t>
         </is>
       </c>
       <c r="AB23" s="43" t="inlineStr">
@@ -5438,27 +5418,26 @@
       </c>
       <c r="AD23" s="43" t="inlineStr">
         <is>
-          <t>Proverbios 27:17 — El hierro se pule con el hierro,
-y el hombre se pule en el trato con su prójimo.</t>
+          <t>Esdras 7:10 — Y es que Esdras se había entregado de corazón al estudio de la ley del Señor, y a cumplirla y enseñarla a los israelitas, con todas sus normas y ordenanzas.</t>
         </is>
       </c>
       <c r="AE23" s="43" t="inlineStr">
         <is>
-          <t>• El compañero afila el carácter
-• Aprender de otros acelera el crecimiento
-• Nadie mejora completamente aislado</t>
+          <t>• Estudiar la Palabra de Dios.
+• Ponerla en práctica.
+• Enseñarla a otros.</t>
         </is>
       </c>
       <c r="AF23" s="43" t="inlineStr">
         <is>
-          <t>Filipenses 4:13 — ¡todo lo puedo en Cristo que me fortalece!</t>
+          <t>Efesios 6:6-8 — No actúen así solo cuando los estén mirando, como los que quieren agradar a la gente, sino como siervos de Cristo que de corazón hacen la voluntad de Dios.</t>
         </is>
       </c>
       <c r="AG23" s="43" t="inlineStr">
         <is>
-          <t>• La fuerza para el trabajo viene de Cristo
-• No depende solo de la capacidad propia
-• El respaldo espiritual sostiene el esfuerzo diario</t>
+          <t>• Servir de corazón — Hacer todo con sinceridad.
+• No buscar solo agradar a otros — Ser fieles aunque nadie nos vea.
+• Hacer la voluntad de Dios — Servir como verdaderos siervos de Cristo.</t>
         </is>
       </c>
       <c r="AH23" s="43" t="inlineStr">
@@ -5475,15 +5454,14 @@
       </c>
       <c r="AJ23" s="43" t="inlineStr">
         <is>
-          <t>Proverbios 16:3 —Encomienda al Señor tus acciones,
-y tus pensamientos serán afirmados.</t>
+          <t>1 Tesalonisenses 5:11 — Por lo tanto, anímense y edifíquense unos a otros, como en efecto ya lo hacen.</t>
         </is>
       </c>
       <c r="AK23" s="43" t="inlineStr">
         <is>
-          <t>• Encomendar el trabajo a Dios
-• Los planes se afirman en Su dirección
-• El desarrollo profesional también necesita oración</t>
+          <t>• Animarnos — Dar palabras de ánimo a los demás.
+• Edificarnos — Ayudarnos a crecer en la fe.
+• Hacerlo juntos — Fortalecernos mutuamente cada día.</t>
         </is>
       </c>
     </row>
@@ -5604,41 +5582,43 @@
       </c>
       <c r="X24" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 31:16 — 16Analiza el valor de un terreno, y lo compra,
-y con lo que gana planta un viñedo.</t>
+          <t>2 Reyes 4:2-4 — Eliseo le dijo:
+«¿Y en qué te puedo ayudar? Dime qué es lo que tienes en casa.»
+La viuda dijo:
+«Esta sierva tuya no tiene en casa más que una vasija de aceite.»
+Entonces Eliseo le dijo:
+«Ve y pide a tus vecinos que te presten algunas vasijas vacías. ¡Todas las que puedas conseguir!Luego, entra en tu casa y enciérrate con tus hijos. Echa aceite en todas las vasijas, y ve apartándolas conforme las vayas llenando.»</t>
         </is>
       </c>
       <c r="Y24" s="47" t="inlineStr">
         <is>
-          <t>• Evaluar antes de comprometer recursos
-• Usar el propio esfuerzo para generar fruto
-• La planificación precede a la inversión</t>
+          <t>• Dios usa lo que tienes: Aunque parezca poco, Dios puede multiplicarlo.  
+• Obedecer con fe: La viuda actuó conforme a la palabra de Eliseo.  
+• La provisión de Dios: Cuando confiamos y obedecemos, Dios abre caminos.</t>
         </is>
       </c>
       <c r="Z24" s="47" t="inlineStr">
         <is>
-          <t>Lucas 14:28 — 28Porque ¿quién de ustedes que quiera levantar una torre, no se sienta primero a calcular los costos, para ver si tiene todo lo que necesita para terminarla?</t>
+          <t>Deuteronomio 31:8 — El Señor va delante de ti. Él estará contigo, y no te dejará ni te desamparará. No temas ni te intimides.»</t>
         </is>
       </c>
       <c r="AA24" s="47" t="inlineStr">
         <is>
-          <t>• Calcular el costo antes de comenzar
-• La falta de planificación expone al fracaso
-• Todo proyecto merece evaluación previa</t>
+          <t>• Dios va delante de nosotros.
+• Dios nunca nos abandona.
+• No tener miedo ni desanimarnos.</t>
         </is>
       </c>
       <c r="AB24" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 24:27 —27Comienza por preparar tus campos
-y por disponerte para la siembra,
-y después de eso construye tu casa.</t>
+          <t>Job 8:7 — Las pocas riquezas que llegaste a poseer no podrán compararse con las que tendrás después.</t>
         </is>
       </c>
       <c r="AC24" s="47" t="inlineStr">
         <is>
-          <t>• Preparar el trabajo antes de construir la casa
-• El orden de prioridades importa
-• Primero lo esencial, después lo demás</t>
+          <t>• Dios puede restaurar: Lo poco puede convertirse en mucho.  
+• Esperar en Dios: El proceso no define el resultado.  
+• Un futuro mejor: Dios puede traer mayor bendición después.</t>
         </is>
       </c>
       <c r="AD24" s="47" t="inlineStr">
@@ -5655,39 +5635,39 @@
       </c>
       <c r="AF24" s="47" t="inlineStr">
         <is>
-          <t>Filipenses 4:13 — Todo lo puedo en Cristo que me fortalece</t>
+          <t>Proverbios 14:15 — El inexperto cree todo lo que oye;
+el que es astuto mira por dónde anda.</t>
         </is>
       </c>
       <c r="AG24" s="47" t="inlineStr">
         <is>
-          <t>• La fuerza para emprender viene de Cristo
-• No depende solo de la capacidad propia
-• El respaldo espiritual sostiene el esfuerzo</t>
+          <t>• No creer todo — Escuchar con discernimiento.
+• Ser prudentes — Examinar antes de aceptar algo.
+• Cuidar nuestro camino — Actuar con sabiduría.</t>
         </is>
       </c>
       <c r="AH24" s="47" t="inlineStr">
         <is>
-          <t>Galatas 6:9 — No nos cansemos, pues, de hacer el bien; porque a su tiempo cosecharemos, si no nos desanimamos.</t>
+          <t>Mateo 25:23 — Su señor le dijo: “Bien, buen siervo y fiel, sobre poco has sido fiel, sobre mucho te pondré. Entra en el gozo de tu señor.”</t>
         </is>
       </c>
       <c r="AI24" s="47" t="inlineStr">
         <is>
-          <t>• No desmayar en el camino del emprendimiento
-• La cosecha llega a su tiempo
-• La perseverancia es clave para el que empieza</t>
+          <t>• Ser fiel en lo poco.
+• Dios recompensa la fidelidad.
+• La fidelidad trae bendición y gozo.</t>
         </is>
       </c>
       <c r="AJ24" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 16:3 — Encomienda al Señor tus acciones,
-y tus pensamientos serán afirmados.</t>
+          <t>Juan 6:27 — Trabajen, pero no por la comida que se echa a perder, sino por la comida que permanece para vida eterna, la cual el Hijo del Hombre les dará; porque a este señaló Dios el Padre.»</t>
         </is>
       </c>
       <c r="AK24" s="47" t="inlineStr">
         <is>
-          <t>• Encomendar el proyecto a Dios desde el inicio
-• Los planes se afirman en Su dirección
-• El emprendimiento también necesita oración</t>
+          <t>• No vivir solo por lo material — Lo terrenal es pasajero.
+• Buscar lo eterno — Priorizar lo que alimenta nuestra vida espiritual.
+• Jesús da vida eterna — Él es quien satisface verdaderamente nuestra</t>
         </is>
       </c>
     </row>
@@ -5820,8 +5800,8 @@
       </c>
       <c r="Z25" s="49" t="inlineStr">
         <is>
-          <t>Daniel 1:12-13 — 12«Yo te ruego que hagas con estos siervos tuyos una prueba de diez días. Ordena que nos den de comer legumbres, y que nos den de beber agua.
-13Después de esta prueba, compara nuestra apariencia con la de los otros jóvenes que reciben la ración de la comida del rey, y haz entonces con estos siervos tuyos según lo que veas.»</t>
+          <t>Daniel 1:12-13 — «Yo te ruego que hagas con estos siervos tuyos una prueba de diez días. Ordena que nos den de comer legumbres, y que nos den de beber agua.
+Después de esta prueba, compara nuestra apariencia con la de los otros jóvenes que reciben la ración de la comida del rey, y haz entonces con estos siervos tuyos según lo que veas.»</t>
         </is>
       </c>
       <c r="AA25" s="49" t="inlineStr">
@@ -5858,9 +5838,9 @@
       </c>
       <c r="AF25" s="49" t="inlineStr">
         <is>
-          <t>Proverbios 23:20-21 — 20No te juntes con los que se hartan de vino
+          <t>Proverbios 23:20-21 — No te juntes con los que se hartan de vino
 ni con los que se atiborran de carne,
-21porque unos y otros se quedarán pobres,
+porque unos y otros se quedarán pobres,
 y por flojos acabarán cubiertos de harapos.</t>
         </is>
       </c>
@@ -5873,10 +5853,10 @@
       </c>
       <c r="AH25" s="49" t="inlineStr">
         <is>
-          <t>Salmo 104:14-15 —14Haces crecer la hierba para los ganados,
+          <t>Salmo 104:14-15 — Haces crecer la hierba para los ganados,
 y las plantas que el hombre cultiva
 para sacar de la tierra el pan que come
-15y el vino que le alegra el corazón,
+y el vino que le alegra el corazón,
 el aceite que da brillo a su rostro,
 y el pan que sostiene su vida.</t>
         </is>
@@ -6018,8 +5998,8 @@
       </c>
       <c r="X26" s="51" t="inlineStr">
         <is>
-          <t>Mateo 28:19-20 —19Por tanto, vayan y hagan discípulos en todas las naciones, y bautícenlos en el nombre del Padre, y del Hijo, y del Espíritu Santo.
-20Enséñenles a cumplir todas las cosas que les he mandado. Y yo estaré con ustedes todos los días, hasta el fin del mundo.» Amén.</t>
+          <t>Mateo 28:19-20 — Por tanto, vayan y hagan discípulos en todas las naciones, y bautícenlos en el nombre del Padre, y del Hijo, y del Espíritu Santo.
+Enséñenles a cumplir todas las cosas que les he mandado. Y yo estaré con ustedes todos los días, hasta el fin del mundo.» Amén.</t>
         </is>
       </c>
       <c r="Y26" s="51" t="inlineStr">
@@ -6031,7 +6011,7 @@
       </c>
       <c r="Z26" s="51" t="inlineStr">
         <is>
-          <t>2 Timoteo 2:2 — 2Lo que has oído de mí ante muchos testigos, encárgaselo a hombres fieles que sean idóneos para enseñar también a otros.</t>
+          <t>2 Timoteo 2:2 — Lo que has oído de mí ante muchos testigos, encárgaselo a hombres fieles que sean idóneos para enseñar también a otros.</t>
         </is>
       </c>
       <c r="AA26" s="51" t="inlineStr">
@@ -6043,7 +6023,7 @@
       </c>
       <c r="AB26" s="51" t="inlineStr">
         <is>
-          <t>Proverbios 27:19 — 19Así como en el agua se refleja el rostro,
+          <t>Proverbios 27:19 — Así como en el agua se refleja el rostro,
 también en el corazón se refleja el hombre.</t>
         </is>
       </c>
@@ -6068,20 +6048,19 @@
       </c>
       <c r="AF26" s="51" t="inlineStr">
         <is>
-          <t>Deuteronomio 6:6-7 —6Estas palabras que hoy te mando cumplir estarán en tu corazón,
-7y se las repetirás a tus hijos, y hablarás de ellas cuando estés en tu casa, y cuando vayas por el camino, y cuando te acuestes y cuando te levantes.</t>
+          <t>Juan 8:31-32 — Entonces Jesús dijo a los judíos que habían creído en él: «Si ustedes permanecen en mi palabra, serán verdaderamente mis discípulos; y conocerán la verdad, y la verdad los hará libres.»</t>
         </is>
       </c>
       <c r="AG26" s="51" t="inlineStr">
         <is>
-          <t>• Repetir las verdades en cada momento del día
-• Enseñar en lo cotidiano, no solo en lo formal
-• La constancia forma convicciones profundas</t>
+          <t>• Permanecer en la Palabra: Ser fieles a Jesús y obedecer su enseñanza.  
+• Conocer la verdad: La verdad de Cristo transforma nuestra vida.  
+• Vivir en libertad: Jesús nos libera del pecado y del engaño.</t>
         </is>
       </c>
       <c r="AH26" s="51" t="inlineStr">
         <is>
-          <t>Filipenses 4:9 — 9Lo que ustedes aprendieron y recibieron de mí; lo que de mí vieron y oyeron, pónganlo por obra, y el Dios de paz estará con ustedes.</t>
+          <t>Filipenses 4:9 — Lo que ustedes aprendieron y recibieron de mí; lo que de mí vieron y oyeron, pónganlo por obra, y el Dios de paz estará con ustedes.</t>
         </is>
       </c>
       <c r="AI26" s="51" t="inlineStr">
@@ -6093,7 +6072,7 @@
       </c>
       <c r="AJ26" s="51" t="inlineStr">
         <is>
-          <t>Daniel 12:3 —3Los entendidos resplandecerán como el resplandor del cielo; y los que instruyen a muchos en la justicia serán como las estrellas por toda la eternidad.</t>
+          <t>Daniel 12:3 — Los entendidos resplandecerán como el resplandor del cielo; y los que instruyen a muchos en la justicia serán como las estrellas por toda la eternidad.</t>
         </is>
       </c>
       <c r="AK26" s="51" t="inlineStr">
@@ -6234,20 +6213,21 @@
       </c>
       <c r="Z27" s="58" t="inlineStr">
         <is>
-          <t>1 Corintios 16: 13-14 Manténganse atentos y firmes en la fe; sean fuertes y valientes.
+          <t>1 Corintios 16:13-14 — Manténganse atentos y firmes en la fe; sean fuertes y valientes.
 Háganlo todo con amor.</t>
         </is>
       </c>
       <c r="AA27" s="53" t="inlineStr">
         <is>
-          <t>• Firmeza en la fe. 2. Fuerza y valentía. 
+          <t>• Firmeza en la fe.
+• Fuerza y valentía.
 • Hacer todo con amor.</t>
         </is>
       </c>
       <c r="AB27" s="53" t="inlineStr">
         <is>
-          <t>Efesios 4:2-3 — 2y que sean humildes y mansos, y tolerantes y pacientes unos con otros, en amor.
-3Busquen mantener la unidad del Espíritu en el vínculo de la paz.</t>
+          <t>Efesios 4:2-3 — y que sean humildes y mansos, y tolerantes y pacientes unos con otros, en amor.
+Busquen mantener la unidad del Espíritu en el vínculo de la paz.</t>
         </is>
       </c>
       <c r="AC27" s="53" t="inlineStr">
@@ -6259,7 +6239,7 @@
       </c>
       <c r="AD27" s="53" t="inlineStr">
         <is>
-          <t>Proverbios 11:14 —14Cuando no hay buen guía, la gente tropieza;
+          <t>Proverbios 11:14 — Cuando no hay buen guía, la gente tropieza;
 la seguridad depende de los muchos consejeros.</t>
         </is>
       </c>
@@ -6272,7 +6252,7 @@
       </c>
       <c r="AF27" s="53" t="inlineStr">
         <is>
-          <t>Galatas 6:2 —2Sobrelleven los unos las cargas de los otros, y cumplan así la ley de Cristo.</t>
+          <t>Galatas 6:2 — Sobrelleven los unos las cargas de los otros, y cumplan así la ley de Cristo.</t>
         </is>
       </c>
       <c r="AG27" s="53" t="inlineStr">
@@ -6284,7 +6264,7 @@
       </c>
       <c r="AH27" s="53" t="inlineStr">
         <is>
-          <t>Hebreos 10:24 — 24Tengámonos en cuenta unos a otros, a fin de estimularnos al amor y a las buenas obras.</t>
+          <t>Hebreos 10:24 — Tengámonos en cuenta unos a otros, a fin de estimularnos al amor y a las buenas obras.</t>
         </is>
       </c>
       <c r="AI27" s="53" t="inlineStr">
@@ -6296,8 +6276,8 @@
       </c>
       <c r="AJ27" s="53" t="inlineStr">
         <is>
-          <t>Filipenses 2:3-4 — 3No hagan nada por pelea o por orgullo. Al contrario, háganlo con humildad y considerando cada uno a los demás como superiores a sí mismo.
-4No busque cada uno su propio interés, sino cada cual también el de los demás.</t>
+          <t>Filipenses 2:3-4 — No hagan nada por pelea o por orgullo. Al contrario, háganlo con humildad y considerando cada uno a los demás como superiores a sí mismo.
+No busque cada uno su propio interés, sino cada cual también el de los demás.</t>
         </is>
       </c>
       <c r="AK27" s="53" t="inlineStr">
@@ -6425,9 +6405,8 @@
       </c>
       <c r="X28" s="35" t="inlineStr">
         <is>
-          <t>Mateo 5:13-14 —13»Ustedes son la sal de la tierra, pero si la sal pierde su sabor, ¿cómo volverá a ser salada? Ya no servirá para nada, sino para ser arrojada a la calle y pisoteada por la gente.
-La luz del mundo
-14»Ustedes son la luz del mundo. Una ciudad asentada sobre un monte no se puede esconder.</t>
+          <t>Mateo 5:13-14 — »Ustedes son la sal de la tierra, pero si la sal pierde su sabor, ¿cómo volverá a ser salada? Ya no servirá para nada, sino para ser arrojada a la calle y pisoteada por la gente.
+»Ustedes son la luz del mundo. Una ciudad asentada sobre un monte no se puede esconder.</t>
         </is>
       </c>
       <c r="Y28" s="35" t="inlineStr">
@@ -6439,7 +6418,7 @@
       </c>
       <c r="Z28" s="35" t="inlineStr">
         <is>
-          <t>Jeremias 29:7 —7Busquen la paz de la ciudad a la que permití que fueran llevados. Rueguen al Señor por ella, porque si ella tiene paz, también tendrán paz ustedes.”</t>
+          <t>Jeremias 29:7 — Busquen la paz de la ciudad a la que permití que fueran llevados. Rueguen al Señor por ella, porque si ella tiene paz, también tendrán paz ustedes.”</t>
         </is>
       </c>
       <c r="AA28" s="35" t="inlineStr">
@@ -6451,7 +6430,7 @@
       </c>
       <c r="AB28" s="35" t="inlineStr">
         <is>
-          <t>Romanos 13:1 — 1Todos debemos someternos a las autoridades, pues no hay autoridad que no venga de Dios. Las autoridades que hay han sido establecidas por Dios.</t>
+          <t>Romanos 13:1 — Todos debemos someternos a las autoridades, pues no hay autoridad que no venga de Dios. Las autoridades que hay han sido establecidas por Dios.</t>
         </is>
       </c>
       <c r="AC28" s="35" t="inlineStr">
@@ -6463,7 +6442,7 @@
       </c>
       <c r="AD28" s="35" t="inlineStr">
         <is>
-          <t>Miqueas 6:8 —8¡Hombre! El Señor te ha dado a conocer lo que es bueno, y lo que él espera de ti, y que no es otra cosa que hacer justicia, amar la misericordia, y humillarte ante tu Dios.</t>
+          <t>Miqueas 6:8 — ¡Hombre! El Señor te ha dado a conocer lo que es bueno, y lo que él espera de ti, y que no es otra cosa que hacer justicia, amar la misericordia, y humillarte ante tu Dios.</t>
         </is>
       </c>
       <c r="AE28" s="35" t="inlineStr">
@@ -6475,7 +6454,7 @@
       </c>
       <c r="AF28" s="35" t="inlineStr">
         <is>
-          <t>Proverbios 14:34 — 34Un pueblo justo es un gran pueblo,
+          <t>Proverbios 14:34 — Un pueblo justo es un gran pueblo,
 pero el pecado deshonra a las naciones.</t>
         </is>
       </c>
@@ -6488,7 +6467,7 @@
       </c>
       <c r="AH28" s="35" t="inlineStr">
         <is>
-          <t>Galatas 6:10 — 10Así que, según tengamos oportunidad, hagamos bien a todos, y mayormente a los de la familia de la fe.</t>
+          <t>Galatas 6:10 — Así que, según tengamos oportunidad, hagamos bien a todos, y mayormente a los de la familia de la fe.</t>
         </is>
       </c>
       <c r="AI28" s="35" t="inlineStr">
@@ -6500,8 +6479,8 @@
       </c>
       <c r="AJ28" s="35" t="inlineStr">
         <is>
-          <t>1 Timoteo 2:1-2 — 1Ante todo, animo a que se hagan ruegos, oraciones, peticiones y acciones de gracias por todos los hombres;
-2por los reyes y por todos los que ocupan altos puestos, para que vivamos con tranquilidad y reposo, y en toda piedad y honestidad.</t>
+          <t>1 Timoteo 2:1-2 — Ante todo, animo a que se hagan ruegos, oraciones, peticiones y acciones de gracias por todos los hombres;
+por los reyes y por todos los que ocupan altos puestos, para que vivamos con tranquilidad y reposo, y en toda piedad y honestidad.</t>
         </is>
       </c>
       <c r="AK28" s="35" t="inlineStr">
@@ -6629,8 +6608,8 @@
       </c>
       <c r="X29" s="40" t="inlineStr">
         <is>
-          <t>Mateo 25:14-15 — 14»Porque el reino de los cielos es como un hombre que, al irse de viaje, llamó a sus siervos y les entregó sus bienes.
-15A uno le dio cinco mil monedas de plata; a otro, dos mil; y a otro, mil, a cada uno conforme a su capacidad; y luego se marchó.</t>
+          <t>Mateo 25:14-15 — »Porque el reino de los cielos es como un hombre que, al irse de viaje, llamó a sus siervos y les entregó sus bienes.
+A uno le dio cinco mil monedas de plata; a otro, dos mil; y a otro, mil, a cada uno conforme a su capacidad; y luego se marchó.</t>
         </is>
       </c>
       <c r="Y29" s="40" t="inlineStr">
@@ -6642,8 +6621,8 @@
       </c>
       <c r="Z29" s="40" t="inlineStr">
         <is>
-          <t>Mateo 25:20-21 — 20El que había recibido las cinco mil monedas se presentó, le entregó otras cinco mil, y dijo: “Señor, tú me entregaste cinco mil monedas, y con ellas he ganado otras cinco mil; aquí las tienes.”
-21Y su señor le dijo: “Bien, buen siervo y fiel; sobre poco has sido fiel, sobre mucho te pondré. Entra en el gozo de tu señor.”</t>
+          <t>Mateo 25:20-21 — El que había recibido las cinco mil monedas se presentó, le entregó otras cinco mil, y dijo: “Señor, tú me entregaste cinco mil monedas, y con ellas he ganado otras cinco mil; aquí las tienes.”
+Y su señor le dijo: “Bien, buen siervo y fiel; sobre poco has sido fiel, sobre mucho te pondré. Entra en el gozo de tu señor.”</t>
         </is>
       </c>
       <c r="AA29" s="40" t="inlineStr">
@@ -6655,7 +6634,7 @@
       </c>
       <c r="AB29" s="40" t="inlineStr">
         <is>
-          <t>Eclesiastes 11:1 — 1Echa tu pan sobre las aguas; después de muchos días lo encontrarás.</t>
+          <t>Eclesiastes 11:1 — Echa tu pan sobre las aguas; después de muchos días lo encontrarás.</t>
         </is>
       </c>
       <c r="AC29" s="40" t="inlineStr">
@@ -6667,20 +6646,20 @@
       </c>
       <c r="AD29" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 21:5 — 5Si piensas lo que haces, tendrás abundancia;
-si te apresuras, acabarás en la pobreza.</t>
+          <t>Proverbios 1:7 — El principio de la sabiduría es el temor al Señor;
+los necios desprecian la sabiduría y la enseñanza.</t>
         </is>
       </c>
       <c r="AE29" s="40" t="inlineStr">
         <is>
-          <t>• Los planes diligentes producen abundancia
-• La prisa desordenada lleva a la pobreza
-• La constancia rinde más que el apuro</t>
+          <t>• Temer al Señor: Reconocer a Dios con reverencia.
+• Buscar sabiduría: Aprender de su Palabra y enseñanza.
+• No rechazar la corrección: Tener un corazón dispuesto a aprender.</t>
         </is>
       </c>
       <c r="AF29" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 24:16 — 16porque tal vez caiga el justo siete veces,
+          <t>Proverbios 24:16 — porque tal vez caiga el justo siete veces,
 pero otras tantas volverá a levantarse;
 en cambio, los injustos caerán en desgracia.</t>
         </is>
@@ -6694,26 +6673,28 @@
       </c>
       <c r="AH29" s="40" t="inlineStr">
         <is>
-          <t>Galatas 6:9 — No nos cansemos, pues, de hacer bien; porque a su tiempo segaremos, si no desmayamos</t>
+          <t>Mateo 6:19-21 — »No acumulen ustedes tesoros en la tierra, donde la polilla y el óxido corroen, y donde los ladrones minan y hurtan.
+Por el contrario, acumulen tesoros en el cielo, donde ni la polilla ni el óxido corroen, y donde los ladrones no minan ni hurtan.
+Pues donde esté tu tesoro, allí estará también tu corazón.</t>
         </is>
       </c>
       <c r="AI29" s="40" t="inlineStr">
         <is>
-          <t>• No desmayar en el buen camino
-• La cosecha llega a su tiempo
-• El cansancio no debe detener el esfuerzo</t>
+          <t>• No poner nuestra confianza en lo 2. material.
+• Buscar tesoros eternos en el cielo.
+Cuidar dónde está nuestro corazón.</t>
         </is>
       </c>
       <c r="AJ29" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 13:11 — Las vanas riquezas pronto se gastan; el que trabaja y las guarda las hace crecer</t>
+          <t>Hebreos 5:14 — El alimento sólido es para los que ya han alcanzado la madurez, para los que pueden diferenciar entre el bien y el mal, y han ejercitado su capacidad de tomar decisiones.</t>
         </is>
       </c>
       <c r="AK29" s="40" t="inlineStr">
         <is>
-          <t>• El esfuerzo constante aumenta el capital
-• La ganancia fácil se pierde fácil
-• La mano laboriosa es la clave</t>
+          <t>• Crecer en madurez espiritual.
+• Distinguir el bien del mal.
+3 Aprender a tomar buenas decisiones.</t>
         </is>
       </c>
     </row>
@@ -6834,21 +6815,20 @@
       </c>
       <c r="X30" s="43" t="inlineStr">
         <is>
-          <t>Proverbios 16:9 — 9El corazón del hombre examina su camino,
-pero el Señor le corrige el rumbo.</t>
+          <t>Filipenses 1:6 — Estoy persuadido de que el que comenzó en ustedes la buena obra, la perfeccionará hasta el día de Jesucristo.</t>
         </is>
       </c>
       <c r="Y30" s="43" t="inlineStr">
         <is>
-          <t>• Planificar es parte del proceso humano
-• Dios endereza el resultado final
-• La meta se somete a un propósito mayor</t>
+          <t>• Dios comienza la obra.
+• Dios la perfecciona.
+• Confiar en su proceso.</t>
         </is>
       </c>
       <c r="Z30" s="43" t="inlineStr">
         <is>
-          <t>Filipenses 3:13-14 — 13Hermanos, yo mismo no pretendo haberlo alcanzado ya; pero una cosa sí hago: me olvido ciertamente de lo que ha quedado atrás, y me extiendo hacia lo que está adelante;
-14¡prosigo a la meta, al premio del supremo llamamiento de Dios en Cristo Jesús!</t>
+          <t>Filipenses 3:13-14 — Hermanos, yo mismo no pretendo haberlo alcanzado ya; pero una cosa sí hago: me olvido ciertamente de lo que ha quedado atrás, y me extiendo hacia lo que está adelante;
+¡prosigo a la meta, al premio del supremo llamamiento de Dios en Cristo Jesús!</t>
         </is>
       </c>
       <c r="AA30" s="43" t="inlineStr">
@@ -6860,7 +6840,7 @@
       </c>
       <c r="AB30" s="43" t="inlineStr">
         <is>
-          <t>Habacuc 2:2 — 2Y el Señor me respondió, y me dijo:
+          <t>Habacuc 2:2 — Y el Señor me respondió, y me dijo:
 «Escribe esta visión. Grábala sobre unas tablillas, para que pueda leerse de corrido.</t>
         </is>
       </c>
@@ -6873,44 +6853,44 @@
       </c>
       <c r="AD30" s="43" t="inlineStr">
         <is>
-          <t>Lucas 14:28 — 28Porque ¿quién de ustedes que quiera levantar una torre, no se sienta primero a calcular los costos, para ver si tiene todo lo que necesita para terminarla?</t>
+          <t>Mateo 7:7 — »Pidan, y se les dará, busquen, y encontrarán, llamen, y se les abrirá.</t>
         </is>
       </c>
       <c r="AE30" s="43" t="inlineStr">
         <is>
-          <t>• Calcular el costo antes de empezar
-• La planificación previene el abandono
-• Toda meta requiere evaluación previa</t>
+          <t>• Pedir con fe.
+• Buscar con perseverancia.
+• Llamar con confianza.</t>
         </is>
       </c>
       <c r="AF30" s="43" t="inlineStr">
         <is>
-          <t>Proverbios 21:5 —5Si piensas lo que haces, tendrás abundancia;
-si te apresuras, acabarás en la pobreza.</t>
+          <t>Romanos 12:12 — Gocémonos en la esperanza, soportemos el sufrimiento, seamos constantes en la oración.</t>
         </is>
       </c>
       <c r="AG30" s="43" t="inlineStr">
         <is>
-          <t>• Los planes diligentes producen abundancia
-• La prisa desordenada lleva al fracaso
-• La constancia rinde mejor que el apuro</t>
+          <t>• Gozarnos en la esperanza: Confiar en las promesas de Dios.
+• Perseverar en las dificultades: No rendirnos ante el sufrimiento.
+• Ser constantes en la oración: Mantenernos siempre cerca de Dios.</t>
         </is>
       </c>
       <c r="AH30" s="43" t="inlineStr">
         <is>
-          <t>Eclesiastes 3:1 — 1Todo tiene su tiempo. Hay un momento bajo el cielo para toda actividad:</t>
+          <t>Job 22:28 — Llevarás a buen término todos tus planes,
+y en tus caminos brillará la luz.</t>
         </is>
       </c>
       <c r="AI30" s="43" t="inlineStr">
         <is>
-          <t>• Cada meta tiene su tiempo apropiado
-• Forzar el momento incorrecto trae frustración
-• Discernir el tiempo es sabiduría</t>
+          <t>• Confía en Dios: Pon tus planes en sus manos.
+• Persevera: Dios puede ayudarte a llevarlos a buen término.
+3 Camina en su luz: Busca su dirección en cada paso.</t>
         </is>
       </c>
       <c r="AJ30" s="43" t="inlineStr">
         <is>
-          <t>Santiago 4:15 —15Lo que deben decir es: «Si el Señor quiere, viviremos y haremos esto o aquello.»</t>
+          <t>Santiago 4:15 — Lo que deben decir es: «Si el Señor quiere, viviremos y haremos esto o aquello.»</t>
         </is>
       </c>
       <c r="AK30" s="43" t="inlineStr">
@@ -7038,7 +7018,7 @@
       </c>
       <c r="X31" s="47" t="inlineStr">
         <is>
-          <t>Levitico 19:36 — 36Usen balanzas, pesas y medidas justas. Yo soy el Señor su Dios, que los sacó de la tierra de Egipto.</t>
+          <t>Levitico 19:36 — Usen balanzas, pesas y medidas justas. Yo soy el Señor su Dios, que los sacó de la tierra de Egipto.</t>
         </is>
       </c>
       <c r="Y31" s="47" t="inlineStr">
@@ -7050,7 +7030,7 @@
       </c>
       <c r="Z31" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 11:1 — 1Al Señor le repugnan las pesas falsas,
+          <t>Proverbios 11:1 — Al Señor le repugnan las pesas falsas,
 pero le agradan las pesas justas.</t>
         </is>
       </c>
@@ -7063,7 +7043,7 @@
       </c>
       <c r="AB31" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 16:11 —11Las pesas y medidas justas son del Señor;
+          <t>Proverbios 16:11 — Las pesas y medidas justas son del Señor;
 todas las balanzas son su propia creación.</t>
         </is>
       </c>
@@ -7076,7 +7056,7 @@
       </c>
       <c r="AD31" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 20:14 — 14El comprador dice que lo que compra es malo,
+          <t>Proverbios 20:14 — El comprador dice que lo que compra es malo,
 pero en cuanto paga, alaba su compra.</t>
         </is>
       </c>
@@ -7089,33 +7069,31 @@
       </c>
       <c r="AF31" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 22:29 — 29Cuando veas alguien que hace bien su trabajo,
-no lo verás entre gente de baja condición
-sino que estará en presencia de reyes.</t>
+          <t>Efesios 4:25 — Por eso cada uno de ustedes debe despreciar la mentira y hablar la verdad con su prójimo; porque somos miembros los unos de los otros.</t>
         </is>
       </c>
       <c r="AG31" s="47" t="inlineStr">
         <is>
-          <t>• El diligente en su oficio es reconocido
-• La excelencia abre puertas incluso ante líderes
-• El trabajo bien hecho se distingue</t>
+          <t>• Rechazar la mentira — Vivir con integridad.
+• Hablar con verdad — Ser sinceros con los demás.
+• Cuidarnos mutuamente — Somos parte del mismo cuerpo.</t>
         </is>
       </c>
       <c r="AH31" s="47" t="inlineStr">
         <is>
-          <t>Colosenses 4:5 —5Compórtense sabiamente con los no creyentes, y aprovechen bien el tiempo.</t>
+          <t>1 Juan 3:18 — Hijitos míos, no amemos de palabra ni de lengua, sino de hecho y en verdad.</t>
         </is>
       </c>
       <c r="AI31" s="47" t="inlineStr">
         <is>
-          <t>• Actuar con sabiduría frente a los de afuera
-• Aprovechar bien las oportunidades
-• El testimonio también se juega en el comercio</t>
+          <t>• No solo palabras: El amor se demuestra con acciones.
+• De hecho: Amar es ayudar, servir y estar presentes.
+• En verdad: Amar con sinceridad y un corazón genuino.</t>
         </is>
       </c>
       <c r="AJ31" s="47" t="inlineStr">
         <is>
-          <t>Proverbios 31:24 — 24Las telas que hace, las vende,
+          <t>Proverbios 31:24 — Las telas que hace, las vende,
 y provee a los comerciantes con cinturones.</t>
         </is>
       </c>
@@ -7244,23 +7222,22 @@
       </c>
       <c r="X32" s="49" t="inlineStr">
         <is>
-          <t>Salmos 3: 5Yo me acuesto, y duermo y despierto,
+          <t>Salmos 3:5 — Yo me acuesto, y duermo y despierto,
 porque tú, Señor, me sostienes.</t>
         </is>
       </c>
       <c r="Y32" s="49" t="inlineStr">
         <is>
-          <t>Salmos 3:5 – 3 puntos clave
-Descansar en Dios: Podemos dormir tranquilos porque Él cuida de nosotros.
-Confiar en su protección: Dios nos sostiene aun en momentos difíciles.
-Despertar con esperanza: Cada nuevo día es una oportunidad porque Dios permanece a nuestro lado.</t>
+          <t>• Descansar en Dios: Podemos dormir tranquilos porque Él cuida de nosotros.
+• Confiar en su protección: Dios nos sostiene aun en momentos difíciles.
+• Despertar con esperanza: Cada nuevo día es una oportunidad porque Dios permanece a nuestro lado.</t>
         </is>
       </c>
       <c r="Z32" s="49" t="inlineStr">
         <is>
-          <t>Exodo 20:8-10 —8»Te acordarás del día de reposo, y lo santificarás.
-9Durante seis días trabajarás y harás toda tu obra,
-10pero el día séptimo es de reposo en honor del Señor tu Dios. No harás en él ningún trabajo. Ni tú, ni tu hijo, ni tu hija, ni tu siervo, ni tu criada, ni tu ganado, ni el extranjero que viva dentro de tus ciudades.</t>
+          <t>Exodo 20:8-10 — »Te acordarás del día de reposo, y lo santificarás.
+Durante seis días trabajarás y harás toda tu obra,
+pero el día séptimo es de reposo en honor del Señor tu Dios. No harás en él ningún trabajo. Ni tú, ni tu hijo, ni tu hija, ni tu siervo, ni tu criada, ni tu ganado, ni el extranjero que viva dentro de tus ciudades.</t>
         </is>
       </c>
       <c r="AA32" s="49" t="inlineStr">
@@ -7272,7 +7249,7 @@
       </c>
       <c r="AB32" s="49" t="inlineStr">
         <is>
-          <t>Salmo 4:8 — 8Por eso me acuesto y duermo en paz,
+          <t>Salmo 4:8 — Por eso me acuesto y duermo en paz,
 porque solo tú, Señor, me haces vivir confiado.</t>
         </is>
       </c>
@@ -7285,7 +7262,7 @@
       </c>
       <c r="AD32" s="49" t="inlineStr">
         <is>
-          <t>Marcos 6:31 — 31Jesús les dijo: «Vengan conmigo ustedes solos, a un lugar apartado, y descansen un poco.» Y es que tanta gente iba y venía, que ellos no tenían tiempo ni para comer.</t>
+          <t>Marcos 6:31 — Jesús les dijo: «Vengan conmigo ustedes solos, a un lugar apartado, y descansen un poco.» Y es que tanta gente iba y venía, que ellos no tenían tiempo ni para comer.</t>
         </is>
       </c>
       <c r="AE32" s="49" t="inlineStr">
@@ -7297,7 +7274,7 @@
       </c>
       <c r="AF32" s="49" t="inlineStr">
         <is>
-          <t>Salmo 127:2 — 2De nada sirve que ustedes madruguen,
+          <t>Salmo 127:2 — De nada sirve que ustedes madruguen,
 y que se acuesten muy tarde,
 si el pan que comen es pan de sufrimiento,
 y el Señor da el sueño a los que él ama.</t>
@@ -7312,7 +7289,7 @@
       </c>
       <c r="AH32" s="49" t="inlineStr">
         <is>
-          <t>Mateo 11:28 —28Vengan a mí todos ustedes, los agotados de tanto trabajar, que yo los haré descansar.</t>
+          <t>Mateo 11:28 — Vengan a mí todos ustedes, los agotados de tanto trabajar, que yo los haré descansar.</t>
         </is>
       </c>
       <c r="AI32" s="49" t="inlineStr">
@@ -7324,7 +7301,7 @@
       </c>
       <c r="AJ32" s="49" t="inlineStr">
         <is>
-          <t>Exodo 33:14 —14Y el Señor le dijo:
+          <t>Exodo 33:14 — Y el Señor le dijo:
 «Mi presencia irá contigo, y te haré descansar.»</t>
         </is>
       </c>
@@ -7453,31 +7430,33 @@
       </c>
       <c r="X33" s="8" t="inlineStr">
         <is>
-          <t>Filipenses 4:6 — Por nada esten afanosos; mas bien, presenten sus peticiones delante de Dios en toda oracion y ruego, con accion de gracias</t>
+          <t>1 Tesalonicenses 5:16-18 — Estén siempre gozosos.
+Oren sin cesar.
+Den gracias a Dios en todo, porque esta es su voluntad para ustedes en Cristo Jesús.</t>
         </is>
       </c>
       <c r="Y33" s="8" t="inlineStr">
         <is>
-          <t>• La ansiedad se combate orando, no negando
-• Todo puede llevarse a Dios en oración
-• Pedir con acción de gracias</t>
+          <t>• Vivir con gozo  — Mantener la alegría en todo momento.  
+• Orar constantemente  — Mantener una comunicación continua con Dios.  
+• Dar gracias siempre  — Agradecer a Dios aun en las dificultades.</t>
         </is>
       </c>
       <c r="Z33" s="8" t="inlineStr">
         <is>
-          <t>1 Tesalonicenses 5:17 — Oren sin cesar</t>
+          <t>Jeremías 33:3 — Clama a mí, y yo te responderé; te daré a conocer cosas grandes y maravillosas que tú no conoces.</t>
         </is>
       </c>
       <c r="AA33" s="8" t="inlineStr">
         <is>
-          <t>• Orar sin cesar es una actitud, no un maratón
-• La oración constante sostiene la fe diaria
-• No requiere ocasión especial</t>
+          <t>• Clama a Dios — Busca a Dios en oración.  
+• Confía en su respuesta — Dios escucha y responde.  
+• Espera cosas grandes — Dios puede mostrarte lo que aún no conoces.</t>
         </is>
       </c>
       <c r="AB33" s="8" t="inlineStr">
         <is>
-          <t>Mateo 6:6 — Cuando ores, entra en tu aposento, y con la puerta cerrada ora a tu Padre que esta en secreto, y tu Padre que ve en lo secreto te recompensara en publico</t>
+          <t>Mateo 6:6 — Pero tú, cuando ores, entra en tu habitación, y con la puerta cerrada ora a tu Padre que está en secreto, y tu Padre que ve en lo secreto te recompensará en público.</t>
         </is>
       </c>
       <c r="AC33" s="8" t="inlineStr">
@@ -7489,19 +7468,21 @@
       </c>
       <c r="AD33" s="8" t="inlineStr">
         <is>
-          <t>Santiago 5:16 — Confiesen sus pecados unos a otros, y oren unos por otros, para que sean sanados. La oracion del justo es muy poderosa y efectiva</t>
+          <t>1 Juan 5:14 — Y esta es la confianza que tenemos en él: si pedimos algo según su voluntad, él nos oye.</t>
         </is>
       </c>
       <c r="AE33" s="8" t="inlineStr">
         <is>
-          <t>• La oración del justo tiene poder real
-• Eficaz no significa mágica, sino con fe
-• Puede mucho cuando es sincera</t>
+          <t>• Confiar en Dios — Podemos acercarnos a Él con confianza.  
+• Pedir según su voluntad — Buscar lo que agrada a Dios.  
+• Dios nos escucha — Él oye nuestras oraciones.</t>
         </is>
       </c>
       <c r="AF33" s="8" t="inlineStr">
         <is>
-          <t>Salmo 62:8 — Confiad en el en todo tiempo, oh pueblo; derramad delante de el vuestro corazon; Dios es nuestro refugio</t>
+          <t>Salmo 62:8 — Pueblos todos, ¡confíen siempre en Dios!
+¡Vacíen delante de él su corazón!
+¡Dios es nuestro refugio!</t>
         </is>
       </c>
       <c r="AG33" s="8" t="inlineStr">
@@ -7513,7 +7494,7 @@
       </c>
       <c r="AH33" s="8" t="inlineStr">
         <is>
-          <t>Marcos 11:24 — Por tanto, les digo: todo lo que pidan en oracion, crean que lo recibiran, y se les concedera</t>
+          <t>Marcos 11:24 — Por tanto, les digo: Todo lo que pidan en oración, crean que lo recibirán, y se les concederá.</t>
         </is>
       </c>
       <c r="AI33" s="8" t="inlineStr">
@@ -7525,7 +7506,7 @@
       </c>
       <c r="AJ33" s="8" t="inlineStr">
         <is>
-          <t>Lucas 18:1 — Jesus les conto una parabola en cuanto a la necesidad de orar siempre y de no desanimarse</t>
+          <t>Lucas 18:1 — Además, Jesús les contó una parábola en cuanto a la necesidad de orar siempre y de no desanimarse.</t>
         </is>
       </c>
       <c r="AK33" s="8" t="inlineStr">
@@ -7653,31 +7634,33 @@
       </c>
       <c r="X34" s="10" t="inlineStr">
         <is>
-          <t>Proverbios 29:18 — Cuando no hay vision, el pueblo se desvia; dichoso aquel que obedece la ley</t>
+          <t>Salmos 19:14 — Tú, Señor, eres mi roca y mi redentor;
+¡agrádate de mis palabras y de mis pensamientos!</t>
         </is>
       </c>
       <c r="Y34" s="10" t="inlineStr">
         <is>
-          <t>• Sin visión el pueblo se pierde
-• La dirección clara evita el caos
-• Guardar la palabra trae bendición</t>
+          <t>• Dios es nuestra roca: En Él encontramos seguridad y firmeza.
+• Dios es nuestro redentor: Él nos rescata y transforma.
+• Cuidemos pensamientos y palabras:</t>
         </is>
       </c>
       <c r="Z34" s="10" t="inlineStr">
         <is>
-          <t>Habacuc 2:2 — El Senor me respondio, y me dijo: Escribe esta vision. Grabala sobre unas tablillas, para que pueda leerse de corrido</t>
+          <t>Hechos 20:28 — Yo les ruego que piensen en ustedes mismos, y que cuiden el rebaño sobre el cual el Espíritu Santo los ha puesto como obispos, para que cuiden de la iglesia del Señor, que él ganó por su propia sangre.28</t>
         </is>
       </c>
       <c r="AA34" s="10" t="inlineStr">
         <is>
-          <t>• Escribir la visión la hace clara
-• Declararla para que otros la sigan
-• Una visión escrita se puede correr con ella</t>
+          <t>• Cuidar de uno mismo — Velar por nuestra vida espiritual.  
+• Cuidar al rebaño — Guiar y proteger a la iglesia.  
+• Valorar la iglesia — Cristo la compró con su sangre.</t>
         </is>
       </c>
       <c r="AB34" s="10" t="inlineStr">
         <is>
-          <t>Jeremias 29:11 — Solo yo se los planes que tengo para ustedes. Son planes para su bien, y no para su mal, para que tengan un futuro lleno de esperanza</t>
+          <t>Jeremías 29:11 — Solo yo sé los planes que tengo para ustedes. Son planes para su bien, y no para su mal, para que tengan un futuro lleno de esperanza.”
+—Palabra del Señor.</t>
         </is>
       </c>
       <c r="AC34" s="10" t="inlineStr">
@@ -7689,7 +7672,7 @@
       </c>
       <c r="AD34" s="10" t="inlineStr">
         <is>
-          <t>Filipenses 3:14 — Prosigo a la meta, al premio del supremo llamamiento de Dios en Cristo Jesus</t>
+          <t>Filipenses 3:14 — ¡prosigo a la meta, al premio del supremo llamamiento de Dios en Cristo Jesús!</t>
         </is>
       </c>
       <c r="AE34" s="10" t="inlineStr">
@@ -7701,19 +7684,19 @@
       </c>
       <c r="AF34" s="10" t="inlineStr">
         <is>
-          <t>Proverbios 16:3 — Encomienda al Senor tus acciones, y tus pensamientos seran afirmados</t>
+          <t>2 Timoteo 2:15 — Intenta con esfuerzo presentarte ante Dios aprobado, como obrero que no tiene de qué avergonzarse y que usa bien la palabra de verdad.</t>
         </is>
       </c>
       <c r="AG34" s="10" t="inlineStr">
         <is>
-          <t>• Encomendar las obras a Dios
-• Los pensamientos se afirman en Su plan
-• La visión se sostiene con oración</t>
+          <t>• Estudiar la Palabra — Conocerla y comprenderla correctamente.
+• Esforzarse por agradar a Dios — Servir con dedicación y fidelidad.
+• Usar bien la verdad — Enseñar y vivir conforme a la Palabra de Dios.</t>
         </is>
       </c>
       <c r="AH34" s="10" t="inlineStr">
         <is>
-          <t>Efesios 3:20 — Aquel que es poderoso para hacer que todas las cosas excedan a lo que pedimos o entendemos, segun el poder que actua en nosotros</t>
+          <t>Efesios 3:20 — Y a Aquel que es poderoso para hacer que todas las cosas excedan a lo que pedimos o entendemos, según el poder que actúa en nosotros,</t>
         </is>
       </c>
       <c r="AI34" s="10" t="inlineStr">
@@ -7725,14 +7708,14 @@
       </c>
       <c r="AJ34" s="10" t="inlineStr">
         <is>
-          <t>Isaias 43:19 — Fijense en que yo hago algo nuevo, que pronto saldra a la luz. Volvere a abrir un camino en el desierto, y hare que corran rios en el paramo</t>
+          <t>Mateo 5:16 — De la misma manera, que la luz de ustedes alumbre delante de todos, para que todos vean sus buenas obras y glorifiquen a su Padre, que está en los cielos.</t>
         </is>
       </c>
       <c r="AK34" s="10" t="inlineStr">
         <is>
-          <t>• Dios hace cosas nuevas
-• El pasado no limita el futuro
-• Percibir lo nuevo requiere atención</t>
+          <t>• • El testimonio visible por medio de la acción
+• • La fuente de la luz es Dios, no el ser humano
+• • El propósito final es la gloria del Padre</t>
         </is>
       </c>
     </row>
@@ -7853,7 +7836,7 @@
       </c>
       <c r="X35" s="12" t="inlineStr">
         <is>
-          <t>Efesios 4:29 — No pronuncien ustedes ninguna palabra obscena, sino solo aquellas que contribuyan a la necesaria edificacion y que sean de bendicion para los oyentes</t>
+          <t>Efesios 4:29 — No pronuncien ustedes ninguna palabra obscena, sino solo aquellas que contribuyan a la necesaria edificación y que sean de bendición para los oyentes.</t>
         </is>
       </c>
       <c r="Y35" s="12" t="inlineStr">
@@ -7865,31 +7848,32 @@
       </c>
       <c r="Z35" s="12" t="inlineStr">
         <is>
-          <t>Proverbios 15:1 — La respuesta amable calma la ira; la respuesta grosera aumenta el enojo</t>
+          <t>Salmos 141:3 — Señor, pon un vigilante en mi boca;
+¡ponle un sello a mis labios!</t>
         </is>
       </c>
       <c r="AA35" s="12" t="inlineStr">
         <is>
-          <t>• La respuesta suave calma la ira
-• Las palabras duras encienden el conflicto
-• El tono decide el rumbo de la conversación</t>
+          <t>• Cuidar nuestras palabras.
+• Pedir dirección a Dios.
+• Aprender a guardar silencio.</t>
         </is>
       </c>
       <c r="AB35" s="12" t="inlineStr">
         <is>
-          <t>Santiago 1:19 — Amados hermanos mios, todos ustedes deben estar dispuestos a oir, pero ser lentos para hablar y para enojarse</t>
+          <t>1 Pedro 3:7 — De la misma manera, ustedes, los esposos, sean comprensivos con ellas en su vida matrimonial. Hónrenlas, pues como mujeres son más delicadas, y además, son coherederas con ustedes del don de la vida. Así las oraciones de ustedes no encontrarán ningún estorbo.</t>
         </is>
       </c>
       <c r="AC35" s="12" t="inlineStr">
         <is>
-          <t>• Ser pronto para oír
-• Tardío para hablar y para la ira
-• Escuchar primero evita malentendidos</t>
+          <t>1, Habrá un día de juicio.
+2, Dios hará justicia.
+3, Vivir preparados delante de Dios.</t>
         </is>
       </c>
       <c r="AD35" s="12" t="inlineStr">
         <is>
-          <t>Colosenses 4:6 — Procuren que su conversacion siempre sea agradable y de buen gusto, para que den a cada uno la respuesta debida</t>
+          <t>Colosenses 4:6 — Intenten que su conversación siempre sea agradable y de buen gusto, para que den a cada uno la respuesta debida.</t>
         </is>
       </c>
       <c r="AE35" s="12" t="inlineStr">
@@ -7901,19 +7885,20 @@
       </c>
       <c r="AF35" s="12" t="inlineStr">
         <is>
-          <t>Proverbios 25:11 — Manzana de oro con adornos de plata: eso es la palabra dicha cuando conviene</t>
+          <t>Proverbios 25:11 — Manzana de oro con adornos de plata:
+¡eso es la palabra dicha cuando conviene!</t>
         </is>
       </c>
       <c r="AG35" s="12" t="inlineStr">
         <is>
-          <t>• La palabra oportuna tiene gran valor
-• El momento importa tanto como el contenido
-• Como manzanas de oro, no se improvisa</t>
+          <t>• El momento oportuno: Decir lo correcto en el instante preciso tiene un valor extraordinario;
+• Sabiduría al hablar: Implica tacto, prudencia y discernimiento para saber cuándo es el momento de aconsejar, animar o corregir.
+• Impacto positivo: Las palabras bien expresadas edifican al oyente y traen paz o consuelo, de forma similar a como se describe en la Sociedad Bíblica a través de Bible Gateway.</t>
         </is>
       </c>
       <c r="AH35" s="12" t="inlineStr">
         <is>
-          <t>Efesios 4:32 — Desechen todo lo que sea amargura, enojo, ira, griteria, calumnias, y todo tipo de maldad. En vez de eso, sean bondadosos y misericordiosos, y perdonense unos a otros, asi como tambien Dios los perdono a ustedes en Cristo</t>
+          <t>Efesios 4:32 — En vez de eso, sean bondadosos y misericordiosos, y perdónense unos a otros, así como también Dios los perdonó a ustedes en Cristo.</t>
         </is>
       </c>
       <c r="AI35" s="12" t="inlineStr">
@@ -7925,7 +7910,8 @@
       </c>
       <c r="AJ35" s="12" t="inlineStr">
         <is>
-          <t>Proverbios 15:23 — Es muy grato dar la respuesta adecuada, y cuando es oportuna, aun es mas grato</t>
+          <t>Proverbios 15:23 — El hombre es feliz cuando sabe responder;
+¡y qué buena es una respuesta oportuna!</t>
         </is>
       </c>
       <c r="AK35" s="12" t="inlineStr">
@@ -8053,55 +8039,56 @@
       </c>
       <c r="X36" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 31:16 — Evalua un campo y lo compra; con sus ganancias planta una vina</t>
+          <t>Filipenses 4:19 — Así que mi Dios suplirá todo lo que les falte, conforme a sus riquezas en gloria en Cristo Jesús.</t>
         </is>
       </c>
       <c r="Y36" s="14" t="inlineStr">
         <is>
-          <t>• Evaluar antes de invertir
-• Usar el propio esfuerzo para producir
-• La mujer virtuosa piensa a futuro</t>
+          <t>• Provisión de Dios
+2 Necesidades vs. deseo
+3 Fuente inagotable</t>
         </is>
       </c>
       <c r="Z36" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 31:27 — Siempre atenta a la marcha de su hogar, nunca come un pan que no se haya ganado</t>
+          <t>Eclesiastes 4:10 — Si uno de ellos se tropieza, el otro lo levanta.
+¡Pero ay de aquel que tropieza y no hay quien lo levante!</t>
         </is>
       </c>
       <c r="AA36" s="14" t="inlineStr">
         <is>
-          <t>• Vigilar la administración de la casa
-• No comer el pan de la ociosidad
-• La atención constante sostiene el hogar</t>
+          <t>• Apoyarnos unos a otros.
+• Levantar al que cae.
+• No enfrentar las dificultades solos.</t>
         </is>
       </c>
       <c r="AB36" s="14" t="inlineStr">
         <is>
-          <t>1 Timoteo 5:8 — Si alguno no provee para los suyos, y especialmente para los de su casa, niega la fe y es peor que un incredulo</t>
+          <t>1 Timoteo 6:10 — porque la raíz de todos los males es el amor al dinero, el cual algunos, por codiciarlo, se extraviaron de la fe y acabaron por experimentar muchos dolores.</t>
         </is>
       </c>
       <c r="AC36" s="14" t="inlineStr">
         <is>
-          <t>• Proveer para la familia es acto de fe
-• Negarlo es negar la fe misma
-• La responsabilidad económica tiene peso espiritual</t>
+          <t>• • El amor al dinero como origen del mal: 
+• • La desviación de la fe: 
+• • Consecuencias dolorosas:</t>
         </is>
       </c>
       <c r="AD36" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 22:6 — Ensena al nino a seguir fielmente su camino, y aunque llegue a anciano no se apartara de el</t>
+          <t>Lucas 12:15 — También les dijo: «Manténganse atentos y cuídense de toda avaricia, porque la vida del hombre no depende de los muchos bienes que posea.»</t>
         </is>
       </c>
       <c r="AE36" s="14" t="inlineStr">
         <is>
-          <t>• Enseñar hábitos desde la niñez perdura
-• El ejemplo financiero forma a los hijos
-• La instrucción temprana define el futuro</t>
+          <t>• Cuidarse de la avaricia — No dejar que el deseo de tener nos domine.
+• Los bienes no lo son todo — Nuestra vida no depende de las riquezas.
+• Valorar lo verdaderamente importante — Poner a Dios y lo espiritual en</t>
         </is>
       </c>
       <c r="AF36" s="14" t="inlineStr">
         <is>
-          <t>Mateo 6:24 — Nadie puede servir a dos amos, pues odiara a uno y amara al otro, o estimara a uno y menospreciara al otro. Ustedes no pueden servir a Dios y a las riquezas</t>
+          <t>Mateo 6:24 — »Nadie puede servir a dos amos, pues odiará a uno y amará al otro, o estimará a uno y despreciará al otro. Ustedes no pueden servir a Dios y a las riquezas.</t>
         </is>
       </c>
       <c r="AG36" s="14" t="inlineStr">
@@ -8113,19 +8100,20 @@
       </c>
       <c r="AH36" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 15:16 — Es mejor lo poco, con el temor del Senor, que lo mucho, con muchos problemas</t>
+          <t>1 Corintios 1:10 — Hermanos, les ruego por el nombre de nuestro Señor Jesucristo, que se pongan de acuerdo y que no haya divisiones entre ustedes, sino que estén perfectamente unidos en un mismo sentir y en un mismo parecer.</t>
         </is>
       </c>
       <c r="AI36" s="14" t="inlineStr">
         <is>
-          <t>• Lo poco con temor de Dios es mejor
-• La paz vale más que la abundancia sin Dios
-• El contentamiento supera la ansiedad por más</t>
+          <t>• Vivir en unidad: Evitar divisiones entre nosotros.
+• Tener un mismo sentir: Buscar la armonía y el amor.
+• Caminar juntos: Estar unidos en Cristo y en propósito.</t>
         </is>
       </c>
       <c r="AJ36" s="14" t="inlineStr">
         <is>
-          <t>Filipenses 4:11-12 — No lo digo porque tenga escasez, pues he aprendido a estar contento en cualquier situacion. Se vivir con limitaciones, y tambien se tener abundancia</t>
+          <t>Filipenses 4:11-12 — No lo digo porque tenga escasez, pues he aprendido a estar contento en cualquier situación.
+Sé vivir con limitaciones, y también sé tener abundancia; en todo y por todo estoy enseñado, tanto para estar satisfecho como para tener hambre, lo mismo para tener abundancia que para sufrir necesidad;</t>
         </is>
       </c>
       <c r="AK36" s="14" t="inlineStr">
@@ -8253,19 +8241,20 @@
       </c>
       <c r="X37" s="2" t="inlineStr">
         <is>
-          <t>1 Corintios 9:27 — Mas bien, golpeo mi cuerpo y lo someto a servidumbre, no sea que despues de haber predicado a otros yo mismo quede eliminado</t>
+          <t>Filipenses 3:12 — No es que ya lo haya alcanzado, ni que ya sea perfecto, sino que sigo adelante, por ver si logro alcanzar aquello para lo cual fui también alcanzado por Cristo Jesús.</t>
         </is>
       </c>
       <c r="Y37" s="2" t="inlineStr">
         <is>
-          <t>• Disciplinar el cuerpo con propósito
-• El dominio propio evita la descalificación
-• La constancia vale más que la intensidad</t>
+          <t>• Seguir avanzando — No conformarnos con lo alcanzado.
+• Buscar crecer en Cristo — Caminar cada día más cerca de Él.
+• Vivir con propósito — Alcanzar aquello para lo cual Cristo nos llamó.</t>
         </is>
       </c>
       <c r="Z37" s="2" t="inlineStr">
         <is>
-          <t>Proverbios 25:28 — Ciudad en ruinas, sin muralla protectora: eso es el hombre que no frena sus impulsos</t>
+          <t>Proverbios 25:28 — El justo piensa bien, antes de responder;
+la boca de los injustos dice malas palabras.</t>
         </is>
       </c>
       <c r="AA37" s="2" t="inlineStr">
@@ -8277,19 +8266,20 @@
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
-          <t>Hebreos 12:11 — Claro que ninguna disciplina nos pone alegres al momento de recibirla, sino mas bien tristes; pero despues de ser ejercitados en ella, nos produce un fruto apacible de justicia</t>
+          <t>Colosenses 4:2 — Dedíquense a la oración, y sean constantes en sus acciones de gracias.</t>
         </is>
       </c>
       <c r="AC37" s="2" t="inlineStr">
         <is>
-          <t>• La disciplina no es agradable al momento
-• Después produce fruto de justicia
-• El proceso incómodo tiene recompensa</t>
+          <t>• Perseverar en la oración — Mantener una vida de oración.
+• Ser constantes — No rendirse ni dejar de buscar a Dios.
+• Dar gracias — Reconocer siempre la bondad de Dios.</t>
         </is>
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>Proverbios 12:24 — Los diligentes dominan a otros; los negligentes son dominados</t>
+          <t>Proverbios 12:24 — Al Señor le repugnan los labios mentirosos;
+pero le agradan los que dicen la verdad.</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -8301,7 +8291,7 @@
       </c>
       <c r="AF37" s="2" t="inlineStr">
         <is>
-          <t>1 Timoteo 4:7-8 — Desecha las fabulas profanas y de viejas. Ejercitate para la piedad; porque el ejercicio corporal es poco provechoso, pero la piedad es provechosa para todo</t>
+          <t>1 Timoteo 4:7-8 — Rechaza las fábulas mundanas y tontas. Ejercítate para la piedad; porque el ejercicio corporal es poco provechoso, pero la piedad es provechosa para todo, pues cuenta con promesa para esta vida presente, y para la venidera.</t>
         </is>
       </c>
       <c r="AG37" s="2" t="inlineStr">
@@ -8325,7 +8315,8 @@
       </c>
       <c r="AJ37" s="2" t="inlineStr">
         <is>
-          <t>Proverbios 20:4 — Llega el invierno y el perezoso no siembra; cuando llega el verano, no halla comida</t>
+          <t>Proverbios 20:4 — Llega el invierno y el perezoso no siembra;
+cuando llega el verano, no halla comida.</t>
         </is>
       </c>
       <c r="AK37" s="2" t="inlineStr">
@@ -8453,19 +8444,19 @@
       </c>
       <c r="X38" s="4" t="inlineStr">
         <is>
-          <t>Eclesiastes 4:9-10 — Dos son mejor que uno, porque sacan mas provecho de sus afanes. Si uno de ellos se tropieza, el otro lo levanta</t>
+          <t>Colosenses 3:14 — Y sobre todo, revístanse de amor, que es el vínculo perfecto.</t>
         </is>
       </c>
       <c r="Y38" s="4" t="inlineStr">
         <is>
-          <t>• Dos logran más que uno solo
-• El trabajo en conjunto tiene mejor recompensa
-• La ayuda mutua sostiene en la caída</t>
+          <t>1, Revestirse de amor.
+2, Mantener la unidad.
+3, Vivir en armonía.</t>
         </is>
       </c>
       <c r="Z38" s="4" t="inlineStr">
         <is>
-          <t>Hechos 4:32 — Todos los que habian creido eran de un mismo sentir y de un mismo pensar. Ninguno reclamaba como suyo nada de lo que poseia, sino que todas las cosas las tenian en comun</t>
+          <t>Hechos 4:32 — Todos los que habían creído eran de un mismo sentir y de un mismo pensar. Ninguno reclamaba como suyo nada de lo que poseía, sino que todas las cosas las tenían en común.</t>
         </is>
       </c>
       <c r="AA38" s="4" t="inlineStr">
@@ -8477,43 +8468,47 @@
       </c>
       <c r="AB38" s="4" t="inlineStr">
         <is>
-          <t>Romanos 12:4-5 — Porque asi como en un cuerpo hay muchos miembros, y no todos los miembros tienen la misma funcion, asi tambien nosotros, aunque somos muchos, formamos un solo cuerpo en Cristo</t>
+          <t>1 Pedro 4:8-10 — Por sobre todas las cosas, ámense intensamente los unos a los otros, porque el amor cubre infinidad de pecados.
+Bríndense mutuo hospedaje, pero no lo hagan a regañadientes.
+Ponga cada uno al servicio de los demás el don que haya recibido, y sea un buen administrador de la gracia de Dios en sus diferentes manifestaciones.</t>
         </is>
       </c>
       <c r="AC38" s="4" t="inlineStr">
         <is>
-          <t>• Somos un cuerpo con muchos miembros
-• Cada parte depende de las demás
-• La cooperación refleja el diseño del cuerpo</t>
+          <t>• Amarse intensamente.
+• Servir con generosidad.
+• Usar nuestros dones para Dios.</t>
         </is>
       </c>
       <c r="AD38" s="4" t="inlineStr">
         <is>
-          <t>Galatas 6:2 — Sobrelleven los unos las cargas de los otros, y cumplan asi la ley de Cristo</t>
+          <t>Salmos 133:1 — ¡Qué bueno es, y qué agradable,
+que los hermanos convivan en armonía!</t>
         </is>
       </c>
       <c r="AE38" s="4" t="inlineStr">
         <is>
-          <t>• Compartir las cargas del otro
-• Nadie debería cargar solo su carga
-• Es cumplir la ley de Cristo</t>
+          <t>• Vivir en armonía: Buscar la unidad entre hermanos.  
+• Es bueno y agradable: La unidad agrada a Dios.  
+• Cuidar las relaciones: Promover amor, respeto y paz.</t>
         </is>
       </c>
       <c r="AF38" s="4" t="inlineStr">
         <is>
-          <t>Proverbios 11:14 — Cuando no hay buen guia, la gente tropieza; la seguridad depende de los muchos consejeros</t>
+          <t>2 Corintios 13:11 — Por lo demás, hermanos, regocíjense, perfecciónense, consuélense; sean de un mismo sentir, y vivan en paz. Y el Dios de la paz y del amor estará con ustedes.</t>
         </is>
       </c>
       <c r="AG38" s="4" t="inlineStr">
         <is>
-          <t>• Muchos consejeros dan seguridad
-• Decidir en soledad es un riesgo
-• El consejo colectivo previene errores</t>
+          <t>• Vivir con gozo: Regocijarnos en el Señor.  
+• Buscar la unidad: Tener un mismo sentir y vivir en paz.  
+• Dios está con nosotros: Su presencia trae paz y amor.</t>
         </is>
       </c>
       <c r="AH38" s="4" t="inlineStr">
         <is>
-          <t>1 Corintios 12:25-26 — Para que no haya divisiones en el cuerpo, sino que todos los miembros se preocupen los unos por los otros. De manera que, si uno de los miembros padece, todos los miembros se conduelen</t>
+          <t>1 Corintios 12:25-26 — para que no haya divisiones en el cuerpo, sino que todos los miembros se preocupen los unos por los otros.
+De manera que, si uno de los miembros padece, todos los miembros se conduelen con él, y si uno de los miembros recibe honores, todos los miembros se gozan con él.</t>
         </is>
       </c>
       <c r="AI38" s="4" t="inlineStr">
@@ -8525,14 +8520,14 @@
       </c>
       <c r="AJ38" s="4" t="inlineStr">
         <is>
-          <t>Eclesiastes 4:12 — Uno solo puede ser vencido, pero dos presentan resistencia. El cordon de tres hilos no se rompe facilmente</t>
+          <t>1 Pedro 3:8-9 — En fin, únanse todos en un mismo sentir; sean compasivos, misericordiosos y amigables; ámense fraternalmente</t>
         </is>
       </c>
       <c r="AK38" s="4" t="inlineStr">
         <is>
-          <t>• El cordón triple no se rompe fácil
-• La unión da resistencia
-• Trabajar juntos multiplica la fuerza</t>
+          <t>• Vivir en unidad: Tener un mismo sentir.  
+• Practicar el amor: Ser compasivos, misericordiosos y amigables.  
+• Amarnos como hermanos: Mostrar amor con nuestras acciones.</t>
         </is>
       </c>
     </row>
@@ -8653,7 +8648,8 @@
       </c>
       <c r="X39" s="6" t="inlineStr">
         <is>
-          <t>Salmo 71:9 — No me deseches cuando llegue a la vejez; no me desampares cuando mis fuerzas se acaben</t>
+          <t>Salmo 71:9 — No me desprecies cuando llegue a la vejez;
+no me desampares cuando mis fuerzas se acaben.</t>
         </is>
       </c>
       <c r="Y39" s="6" t="inlineStr">
@@ -8677,19 +8673,24 @@
       </c>
       <c r="AB39" s="6" t="inlineStr">
         <is>
-          <t>1 Timoteo 4:12 — Ninguno tenga en poco tu juventud, sino se ejemplo de los creyentes en palabra, conducta, amor, espiritu, fe y pureza</t>
+          <t>Lucas 2:52 — Y Jesús siguió creciendo en sabiduría y en estatura, y en gracia para con Dios y con los hombres.</t>
         </is>
       </c>
       <c r="AC39" s="6" t="inlineStr">
         <is>
-          <t>• Nadie debe menospreciar la juventud
-• El ejemplo puede darse a cualquier edad
-• La madurez no depende solo de los años</t>
+          <t>• Crecer en sabiduría.
+• Crecer en lo personal.
+• Crecer en gracia ante Dios y los demás.</t>
         </is>
       </c>
       <c r="AD39" s="6" t="inlineStr">
         <is>
-          <t>Salmo 71:17-18 — Tu, mi Dios, me has ensenado desde mi juventud, y aun ahora sigo hablando de tus maravillas. No me desampares, Dios mio, aunque llegue a estar viejo y canoso</t>
+          <t>Salmo 71:17-18 — Tú, mi Dios, me has enseñado desde mi juventud,
+y aún ahora sigo hablando de tus maravillas.
+No me desampares, Dios mío,
+aunque llegue a estar viejo y canoso,
+hasta que haya anunciado tu gran poder
+a las generaciones que habrán de venir.</t>
         </is>
       </c>
       <c r="AE39" s="6" t="inlineStr">
@@ -8701,7 +8702,8 @@
       </c>
       <c r="AF39" s="6" t="inlineStr">
         <is>
-          <t>Proverbios 20:29 — Los jovenes se alegran en su fuerza; los ancianos se enorgullecen de sus canas</t>
+          <t>Proverbios 20:29 — Los jóvenes se alegran en su fuerza;
+los ancianos se enorgullecen de sus canas.</t>
         </is>
       </c>
       <c r="AG39" s="6" t="inlineStr">
@@ -8713,7 +8715,7 @@
       </c>
       <c r="AH39" s="6" t="inlineStr">
         <is>
-          <t>Isaias 46:4 — Yo mismo los seguire llevando, hasta que esten viejos y canosos. Yo los hice, yo los llevare. Yo los apoyare y los protegere</t>
+          <t>Isaías 46:4 — Yo mismo los seguiré llevando, hasta que estén viejos y canosos. Yo los hice, yo los llevaré. Yo los apoyaré y los protegeré.</t>
         </is>
       </c>
       <c r="AI39" s="6" t="inlineStr">
@@ -8725,7 +8727,7 @@
       </c>
       <c r="AJ39" s="6" t="inlineStr">
         <is>
-          <t>Salmo 92:14 — Aun en su vejez daran frutos y se mantendran sanos y vigorosos</t>
+          <t>Salmo 92:14 — Aun en su vejez darán frutos y se mantendrán sanos y fuertes</t>
         </is>
       </c>
       <c r="AK39" s="6" t="inlineStr">
@@ -8853,7 +8855,7 @@
       </c>
       <c r="X40" s="8" t="inlineStr">
         <is>
-          <t>2 Corintios 5:17 — Si alguno esta en Cristo, nueva criatura es; las cosas viejas pasaron; he aqui todas son hechas nuevas</t>
+          <t>2 Corintios 5:17 — De modo que si alguno está en Cristo, ya es una nueva creación; atrás ha quedado lo viejo: ¡ahora ya todo es nuevo!</t>
         </is>
       </c>
       <c r="Y40" s="8" t="inlineStr">
@@ -8865,7 +8867,7 @@
       </c>
       <c r="Z40" s="8" t="inlineStr">
         <is>
-          <t>Efesios 2:10 — Nosotros somos hechura suya; hemos sido creados en Cristo Jesus para realizar buenas obras, las cuales Dios preparo de antemano para que vivamos de acuerdo con ellas</t>
+          <t>Efesios 2:10 — Nosotros somos obra suya; hemos sido creados en Cristo Jesús para realizar buenas acciones, las cuales Dios preparó de antemano para que vivamos de acuerdo con ellas.</t>
         </is>
       </c>
       <c r="AA40" s="8" t="inlineStr">
@@ -8877,19 +8879,19 @@
       </c>
       <c r="AB40" s="8" t="inlineStr">
         <is>
-          <t>Galatas 2:20 — Con Cristo estoy juntamente crucificado, y ya no vivo yo, mas vive Cristo en mi; y lo que ahora vivo en la carne, lo vivo en la fe del Hijo de Dios, el cual me amo y se entrego a si mismo por mi</t>
+          <t>Gálatas 4:7 — Así que ya no eres esclavo, sino hijo; y si eres hijo, también eres heredero de Dios por medio de Cristo.</t>
         </is>
       </c>
       <c r="AC40" s="8" t="inlineStr">
         <is>
-          <t>• Cristo vive en mi, no solo yo vivo
-• La vida cristiana es una vida compartida
-• La fe en el Hijo de Dios sostiene la identidad</t>
+          <t>• • Fin de la esclavitud
+• • Adopción como hijo
+• • Herencia por medio de Cristo</t>
         </is>
       </c>
       <c r="AD40" s="8" t="inlineStr">
         <is>
-          <t>1 Pedro 2:9 — Ustedes son linaje escogido, real sacerdocio, nacion santa, pueblo adquirido por Dios, para que anuncien los hechos maravillosos de aquel que los llamo de las tinieblas a su luz admirable</t>
+          <t>1 Pedro 2:9 — Pero ustedes son linaje escogido, real sacerdocio, nación santa, pueblo perteneciente a Dios, para que anuncien los hechos maravillosos de aquel que los llamó de las tinieblas a su luz admirable.</t>
         </is>
       </c>
       <c r="AE40" s="8" t="inlineStr">
@@ -8901,15 +8903,14 @@
       </c>
       <c r="AF40" s="55" t="inlineStr">
         <is>
-          <t>Gálatas 2:20 Pero con Cristo estoy juntamente crucificado, y ya no vivo yo, sino que Cristo vive en mí; y lo que ahora vivo en la carne, lo vivo en la fe del Hijo de Dios, el cual me amó y se entregó a sí mismo por mí.</t>
+          <t>Gálatas 2:20 — Pero con Cristo estoy juntamente crucificado, y ya no vivo yo, sino que Cristo vive en mí; y lo que ahora vivo en la carne, lo vivo en la fe del Hijo de Dios, el cual me amó y se entregó a sí mismo por mí.</t>
         </is>
       </c>
       <c r="AG40" s="8" t="inlineStr">
         <is>
-          <t>Gálatas 2:20 – 3 puntos clave
-Morir al viejo yo: Ya no vivimos para nosotros mismos, sino para Cristo.
-Cristo vive en nosotros: Nuestra vida debe reflejar su amor y voluntad.
-Vivir por fe: Confiamos en Jesús porque nos amó y se entregó por nosotros.</t>
+          <t>• Morir al viejo yo: Ya no vivimos para nosotros mismos, sino para Cristo.
+• Cristo vive en nosotros: Nuestra vida debe reflejar su amor y voluntad.
+• Vivir por fe: Confiamos en Jesús porque nos amó y se entregó por nosotros.</t>
         </is>
       </c>
       <c r="AH40" s="8" t="inlineStr">
@@ -9054,7 +9055,10 @@
       </c>
       <c r="X41" s="10" t="inlineStr">
         <is>
-          <t>Exodo 3:11 — Moises le respondio a Dios: Y quien soy yo para ir ante el faraon y sacar de Egipto a los hijos de Israel</t>
+          <t>Éxodo 3:11-12 — Pero Moisés le respondió a Dios:
+«¿Y quién soy yo para ir ante el faraón y sacar de Egipto a los hijos de Israel?»
+Y Dios le respondió:
+«Ve, pues yo estaré contigo. Y esto te servirá de señal, de que yo te he enviado: Cuando tú hayas sacado de Egipto al pueblo, ustedes servirán a Dios sobre este monte.»</t>
         </is>
       </c>
       <c r="Y41" s="10" t="inlineStr">
@@ -9066,7 +9070,7 @@
       </c>
       <c r="Z41" s="10" t="inlineStr">
         <is>
-          <t>Numeros 12:3 — Moises era un hombre muy humilde. En toda la tierra no habia nadie mas humilde que el</t>
+          <t>Números 12:3 — Moisés era un hombre muy humilde. En toda la tierra no había nadie más humilde que él.</t>
         </is>
       </c>
       <c r="AA41" s="10" t="inlineStr">
@@ -9078,7 +9082,8 @@
       </c>
       <c r="AB41" s="10" t="inlineStr">
         <is>
-          <t>Nehemias 2:17-18 — Ustedes conocen bien el problema que tenemos, porque los muros de Jerusalen estan en ruinas y sus portones se quemaron. Pero vamos a reconstruirlos, para que no se burlen mas de nosotros</t>
+          <t>Nehemías 2:17-18 — »Cuando regresé, les dije: “¿Ya vieron lo mal que estamos? Jerusalén está desierta, y todas sus puertas han sido quemadas. ¡Anímense y vayamos todos a levantar las murallas de Jerusalén! ¡Basta ya de esta vergüenza!”
+»En cuanto les conté la gran ayuda que mi Dios me había brindado, y lo que el rey me había dicho, todos exclamaron: “¡Sí, comencemos a reconstruir las murallas!” Y se dispusieron a poner manos a la obra.</t>
         </is>
       </c>
       <c r="AC41" s="10" t="inlineStr">
@@ -9090,19 +9095,22 @@
       </c>
       <c r="AD41" s="10" t="inlineStr">
         <is>
-          <t>Nehemias 6:3 — No me es posible ir, porque estoy en medio de una gran obra. Si fuera yo a reunirme con ustedes, el trabajo se detendria</t>
+          <t>1 Samuel 17:45 — Pero David le respondió:
+«Tú vienes contra mí armado de espada, lanza y jabalina; pero yo vengo contra ti en el nombre del Señor de los ejércitos, el Dios de los escuadrones de Israel, a quien tú has provocado.</t>
         </is>
       </c>
       <c r="AE41" s="10" t="inlineStr">
         <is>
-          <t>• Nehemías no se distrajo de la obra
-• Rechazar interrupciones que desvían el propósito
-• La gran obra merece protección del enfoque</t>
+          <t>• El contraste de los recursos humanos frente a los divinos
+• La autoridad del respaldo divino
+• El trasfondo de la afrenta personal y nacional</t>
         </is>
       </c>
       <c r="AF41" s="10" t="inlineStr">
         <is>
-          <t>Mateo 20:26-28 — Entre ustedes no debe ser asi. Mas bien, aquel de ustedes que quiera hacerse grande sera su servidor; y aquel que quiera ser el primero, sera su esclavo. Imiten al Hijo del Hombre, que no vino para ser servido, sino para servir y dar su vida en rescate por muchos</t>
+          <t>Mateo 20:26-28 — Pero entre ustedes no debe ser así. Más bien, aquel de ustedes que quiera hacerse grande será su servidor;
+y aquel de ustedes que quiera ser el primero, será su esclavo.
+Imiten al Hijo del Hombre, que no vino para ser servido, sino para servir y para dar su vida en rescate por muchos.»</t>
         </is>
       </c>
       <c r="AG41" s="10" t="inlineStr">
@@ -9114,19 +9122,22 @@
       </c>
       <c r="AH41" s="10" t="inlineStr">
         <is>
-          <t>Juan 13:13-14 — Ustedes me llaman Maestro, y Senor; y dicen bien, porque lo soy. Pues si yo, el Senor y el Maestro, les he lavado los pies, tambien ustedes deben lavarse los pies unos a otros</t>
+          <t>Tito 1:7-9 — Porque es necesario que el obispo, como administrador de Dios, sea irreprensible, no soberbio ni enojoso, ni dado al vino, ni peleador, ni codicioso de ganancias deshonestas,
+sino hospitalario, amante de lo bueno, sobrio, justo, santo, dueño de sí mismo,
+apegado a la palabra fiel, tal y como ha sido enseñada, para que también pueda animar con sana enseñanza y convencer a los que contradicen.</t>
         </is>
       </c>
       <c r="AI41" s="10" t="inlineStr">
         <is>
-          <t>• El Maestro lavo los pies de sus discípulos
-• El ejemplo desciende, no solo asciende
-• Hacer lo que Jesús hizo</t>
+          <t>• El carácter irreprensible (no soberbio ni iracundo)
+• La virtud y el servicio (hospitalario y amante de lo bueno)
+• La fidelidad a la doctrina (apegado a la palabra fiel)</t>
         </is>
       </c>
       <c r="AJ41" s="10" t="inlineStr">
         <is>
-          <t>Lucas 22:26-27 — Entre ustedes no debe ser asi, sino que el mayor entre ustedes tiene que hacerse como el menor; y el que manda tiene que actuar como el que sirve</t>
+          <t>Lucas 22:26-27 — pero entre ustedes no debe ser así, sino que el mayor entre ustedes tiene que hacerse como el menor; y el que manda tiene que actuar como el que sirve.
+Porque, ¿quién es mayor? ¿El que se sienta a la mesa, o el que sirve? ¿Acaso no es el que se sienta a la mesa? Sin embargo, yo estoy entre ustedes como el que sirve.</t>
         </is>
       </c>
       <c r="AK41" s="10" t="inlineStr">
@@ -9254,7 +9265,7 @@
       </c>
       <c r="X42" s="12" t="inlineStr">
         <is>
-          <t>Genesis 2:18 — Despues Dios el Senor dijo: No esta bien que el hombre este solo; le hare una ayuda a su medida</t>
+          <t>Genesis 2:18 — Después Dios el Señor dijo: «No está bien que el hombre esté solo; le haré una ayuda a su medida.»</t>
         </is>
       </c>
       <c r="Y42" s="12" t="inlineStr">
@@ -9266,7 +9277,9 @@
       </c>
       <c r="Z42" s="12" t="inlineStr">
         <is>
-          <t>Proverbios 31:15 — Tambien se levanta cuando aun es de noche, y da alimento a los de su casa, y tarea a sus doncellas</t>
+          <t>Proverbios 31:15 — Aun durante la noche se levanta
+para dar de comer a su familia
+y asignar a las criadas sus deberes.</t>
         </is>
       </c>
       <c r="AA42" s="12" t="inlineStr">
@@ -9278,7 +9291,7 @@
       </c>
       <c r="AB42" s="12" t="inlineStr">
         <is>
-          <t>1 Timoteo 5:8 — Si alguno no provee para los suyos, y especialmente para los de su casa, niega la fe y es peor que un incredulo</t>
+          <t>1 Timoteo 5:8 — porque si alguno no provee para los suyos, y especialmente para los de su casa, niega la fe y es peor que un incrédulo.</t>
         </is>
       </c>
       <c r="AC42" s="12" t="inlineStr">
@@ -9290,19 +9303,20 @@
       </c>
       <c r="AD42" s="12" t="inlineStr">
         <is>
-          <t>Galatas 6:2 — Sobrelleven los unos las cargas de los otros, y cumplan asi la ley de Cristo</t>
+          <t>Colosenses 3:13 — Sean mutuamente tolerantes. Si alguno tiene una queja contra otro, perdónense de la misma manera que Cristo los perdonó.</t>
         </is>
       </c>
       <c r="AE42" s="12" t="inlineStr">
         <is>
-          <t>• Compartir las cargas del otro
-• Nadie debería llevar todo solo
-• Es cumplir la ley de Cristo</t>
+          <t>• Ser tolerantes: Tener paciencia unos con otros.  
+• Perdonar de corazón: Soltar las ofensas y las quejas.  
+• Imitar a Cristo: Perdonar como Él nos perdonó.</t>
         </is>
       </c>
       <c r="AF42" s="12" t="inlineStr">
         <is>
-          <t>Proverbios 31:28 — Sus hijos se levantan y la llaman dichosa; tambien su esposo la congratula: Muchas mujeres han hecho el bien, pero tu las sobrepasas a todas</t>
+          <t>Proverbios 31:28 — Sus hijos se levantan y la llaman dichosa;
+también su esposo la felicita:</t>
         </is>
       </c>
       <c r="AG42" s="12" t="inlineStr">
@@ -9314,7 +9328,7 @@
       </c>
       <c r="AH42" s="12" t="inlineStr">
         <is>
-          <t>Efesios 5:21 — Cultiven entre ustedes la mutua sumision, en el temor de Dios</t>
+          <t>Efesios 5:21 — Cultiven entre ustedes la mutua sumisión, en el temor de Dios.</t>
         </is>
       </c>
       <c r="AI42" s="12" t="inlineStr">
@@ -9326,7 +9340,11 @@
       </c>
       <c r="AJ42" s="12" t="inlineStr">
         <is>
-          <t>Rut 1:16 — No me pidas que te deje y me aparte de ti! A dondequiera que tu vayas, ire yo; dondequiera que tu vivas, vivire. Tu pueblo sera mi pueblo, y tu Dios sera mi Dios</t>
+          <t>Rut 1:16 — Pero Rut le respondió:
+«¡No me pidas que te deje y me aparte de ti!
+A dondequiera que tú vayas, iré yo;
+dondequiera que tú vivas, viviré.
+Tu pueblo será mi pueblo, y tu Dios será mi Dios.</t>
         </is>
       </c>
       <c r="AK42" s="12" t="inlineStr">
@@ -9454,7 +9472,7 @@
       </c>
       <c r="X43" s="14" t="inlineStr">
         <is>
-          <t>2 Corintios 9:7 — Cada uno debe dar segun se lo haya propuesto en su corazon, y no debe dar con tristeza, ni por necesidad, porque Dios ama a quien da con alegria</t>
+          <t>2 Corintios 9:7 — Cada uno debe dar según se lo haya propuesto en su corazón, y no debe dar con tristeza, ni por necesidad, porque Dios ama a quien da con alegría.</t>
         </is>
       </c>
       <c r="Y43" s="14" t="inlineStr">
@@ -9466,7 +9484,7 @@
       </c>
       <c r="Z43" s="14" t="inlineStr">
         <is>
-          <t>Malaquias 3:10 — Entreguen completos los diezmos en mi tesoreria, y habra alimento en mi templo. Con esto pueden ponerme a prueba: veran si no les abro las ventanas de los cielos y derramo sobre ustedes abundantes bendiciones</t>
+          <t>Malaquías 3:10 — Entreguen completos los diezmos en mi tesorería, y habrá alimento en mi templo. Con esto pueden ponerme a prueba: verán si no les abro las ventanas de los cielos y derramo sobre ustedes abundantes bendiciones. Lo digo yo, el Señor de los ejércitos.</t>
         </is>
       </c>
       <c r="AA43" s="14" t="inlineStr">
@@ -9478,7 +9496,9 @@
       </c>
       <c r="AB43" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 3:9-10 — Honra al Senor con tus bienes y con las primicias de tus cosechas. Tus graneros se saturaran de trigo, y tus lagares rebosaran de vino</t>
+          <t>Proverbios 3:9-10 — Honra al Señor con tus bienes y con los primeros frutos de tus cosechas.
+Tus graneros se saturarán de trigo,
+y tus lagares desbordarán de vino.</t>
         </is>
       </c>
       <c r="AC43" s="14" t="inlineStr">
@@ -9490,7 +9510,7 @@
       </c>
       <c r="AD43" s="14" t="inlineStr">
         <is>
-          <t>Lucas 6:38 — Den, y se les dara una medida buena, incluso apretada, remecida y desbordante. Porque con la misma medida con que ustedes midan, seran medidos</t>
+          <t>Lucas 6:38 — Den, y se les dará una medida buena, incluso apretada, remecida y desbordante. Porque con la misma medida con que ustedes midan, serán medidos.»</t>
         </is>
       </c>
       <c r="AE43" s="14" t="inlineStr">
@@ -9502,38 +9522,40 @@
       </c>
       <c r="AF43" s="14" t="inlineStr">
         <is>
-          <t>2 Corintios 9:6 — Recuerden esto: el que poco siembra, poco cosecha; y el que mucho siembra, mucho cosecha</t>
+          <t>1 Crónicas 29:14 — »A decir verdad, ¿quién soy yo, y quién es mi pueblo, para poder ofrecerte todo esto, y de manera voluntaria? Todo es tuyo, y lo que ahora te damos lo hemos recibido de tus manos.</t>
         </is>
       </c>
       <c r="AG43" s="14" t="inlineStr">
         <is>
-          <t>• Sembrar poco cosecha poco
-• Sembrar con generosidad cosecha con generosidad
-• La siembra determina la cosecha</t>
+          <t>• Todo le pertenece a Dios. 
+• Dar con un corazón voluntario. 
+• Reconocer que todo viene de Dios.</t>
         </is>
       </c>
       <c r="AH43" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 11:25 — El que es magnanimo, prospera; el que sacia a otros, sera saciado</t>
+          <t>Éxodo 18:24-26 — Moisés atendió a la voz de su suegro, e hizo todo lo que le dijo,
+pues de entre todo Israel escogió hombres respetables y los puso a cargo del pueblo como jefes de grupos de mil, cien, cincuenta y diez personas.
+Ellos juzgaban al pueblo en todo momento y dictaban sentencia en todo asunto menor, y remitían a Moisés las cuestiones difíciles de resolver.</t>
         </is>
       </c>
       <c r="AI43" s="14" t="inlineStr">
         <is>
-          <t>• El alma generosa prospera
-• Regar a otros también riega al que da
-• La generosidad no tiene perdida real</t>
+          <t>• La humildad y docilidad del líder.
+• La delegación de autoridad y estructura.
+• La división de funciones según la complejidad.</t>
         </is>
       </c>
       <c r="AJ43" s="14" t="inlineStr">
         <is>
-          <t>Hechos 20:35 — Hay mas bendicion en dar que en recibir</t>
+          <t>2 Corintios 9:10-11 — Y aquel que da semilla al que siembra, y pan al que come, proveerá los recursos de ustedes y los multiplicará, aumentándoles así sus frutos de justicia,para que sean ustedes enriquecidos en todo, para toda generosidad, que por medio de nosotros produce acción de gracias a Dios.</t>
         </is>
       </c>
       <c r="AK43" s="14" t="inlineStr">
         <is>
-          <t>• Dar trae mayor bienaventuranza que recibir
-• Contradice la lógica natural
-• Cambia la perspectiva sobre el dinero</t>
+          <t>• Dios provee — Él suple lo necesario.
+• Dios multiplica — Aumenta nuestros frutos para hacer el bien.
+• Ser generosos — Compartir con otros produce gratitud a Dios.</t>
         </is>
       </c>
     </row>
@@ -9654,19 +9676,23 @@
       </c>
       <c r="X44" s="2" t="inlineStr">
         <is>
-          <t>Salmo 78:4 — No las mantendremos ocultas a nuestros hijos, sino que diremos a las generaciones futuras que el Senor es digno de alabanza por su poder y por sus hechos maravillosos</t>
+          <t>Salmos 112:1-2 — Dichoso el hombre que honra al Señor
+y disfruta obedeciendo sus mandatos.
+Sus hijos tendrán poder en la tierra,
+y serán bendecidos por su rectitud.</t>
         </is>
       </c>
       <c r="Y44" s="2" t="inlineStr">
         <is>
-          <t>• Contar a la próxima generación
-• No esconder las obras de Dios
-• El legado se transmite con intención</t>
+          <t>• La fuente de la verdadera dicha
+• La bendición generacional
+• La rectitud como herencia</t>
         </is>
       </c>
       <c r="Z44" s="2" t="inlineStr">
         <is>
-          <t>Proverbios 13:22 — Es bueno dejar herencia a los nietos; las riquezas del pecador las hereda el hombre justo</t>
+          <t>Proverbios 13:22 — Es bueno dejar herencia a los nietos;
+las riquezas del pecador las hereda el hombre justo.</t>
         </is>
       </c>
       <c r="AA44" s="2" t="inlineStr">
@@ -9678,7 +9704,7 @@
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
-          <t>2 Timoteo 4:7 — He peleado la buena batalla, he acabado la carrera, he guardado la fe</t>
+          <t>2 Timoteo 4:7 — He peleado la buena batalla, he acabado la carrera, he guardado la fe.</t>
         </is>
       </c>
       <c r="AC44" s="2" t="inlineStr">
@@ -9690,7 +9716,8 @@
       </c>
       <c r="AD44" s="2" t="inlineStr">
         <is>
-          <t>Salmo 90:12 — Ensenanos a contar bien nuestros dias, para que en el corazon acumulemos sabiduria</t>
+          <t>Salmos 90:12 — ¡Enséñanos a contar bien nuestros días,
+para que en el corazón acumulemos sabiduría!</t>
         </is>
       </c>
       <c r="AE44" s="2" t="inlineStr">
@@ -9702,7 +9729,9 @@
       </c>
       <c r="AF44" s="2" t="inlineStr">
         <is>
-          <t>Eclesiastes 7:1 — Es mejor gozar de buena fama que gozar de un buen perfume. Es mejor el dia en que se muere que el dia en que se nace</t>
+          <t>Eclesiastés 7:1 — Es mejor gozar de buena fama que gozar de un buen perfume.
+Es mejor el día en que se muere
+que el día en que se nace.</t>
         </is>
       </c>
       <c r="AG44" s="2" t="inlineStr">
@@ -9714,7 +9743,7 @@
       </c>
       <c r="AH44" s="2" t="inlineStr">
         <is>
-          <t>Genesis 50:20 — Ustedes pensaron hacerme mal, pero Dios cambio todo para bien, para hacer lo que hoy vemos, que es darle vida a mucha gente</t>
+          <t>Génesis 50:20 — Ustedes pensaron hacerme mal, pero Dios cambió todo para bien, para hacer lo que hoy vemos, que es darle vida a mucha gente.</t>
         </is>
       </c>
       <c r="AI44" s="2" t="inlineStr">
@@ -9726,7 +9755,7 @@
       </c>
       <c r="AJ44" s="2" t="inlineStr">
         <is>
-          <t>Hebreos 11:4 — Por la fe, Abel ofrecio a Dios un sacrificio mas aceptable que el de Cain, y por eso fue reconocido como un hombre justo. Y aunque Abel esta muerto, todavia habla por medio de su fe</t>
+          <t>Hebreos 11:4 — Por la fe, Abel ofreció a Dios un sacrificio más aceptable que el de Caín, y por eso fue reconocido como un hombre justo, y Dios aceptó con agrado sus ofrendas. Y aunque Abel está muerto, todavía habla por medio de su fe.</t>
         </is>
       </c>
       <c r="AK44" s="2" t="inlineStr">
@@ -9854,31 +9883,31 @@
       </c>
       <c r="X45" s="4" t="inlineStr">
         <is>
-          <t>Colosenses 3:23 — Todo lo que hagan, haganlo de corazon, como para el Senor y no como para la gente</t>
+          <t>1 Tesalonicenses 5:6 — así que no durmamos como los demás, sino mantengámonos atentos y sobrios.</t>
         </is>
       </c>
       <c r="Y45" s="4" t="inlineStr">
         <is>
-          <t>• Trabajar de corazón, como para el Señor
-• La actitud eleva cualquier oficio
-• El trabajo tiene valor espiritual</t>
+          <t>• Mantenernos atentos — Estar espiritualmente despiertos.
+• Ser sobrios — Actuar con sabiduría y dominio propio.
+• No vivir distraídos — Permanecer firmes y preparados en la fe.</t>
         </is>
       </c>
       <c r="Z45" s="4" t="inlineStr">
         <is>
-          <t>Genesis 2:15 — Dios el Senor tomo al hombre y lo puso en el huerto de Eden, para que lo cultivara y lo cuidara</t>
+          <t>Romanos 13:7 — Paguen a todos lo que deban pagar, ya sea que deban pagar contribuciones, impuesto, respeto u honra.</t>
         </is>
       </c>
       <c r="AA45" s="4" t="inlineStr">
         <is>
-          <t>• El trabajo existía antes de la caída
-• Labrar y guardar es mandato original
-• El trabajo no es castigo, es propósito</t>
+          <t>• Cumplir con nuestras obligaciones — Dar a cada uno lo que corresponde.
+• Respetar a los demás — Tratar a todos con respeto.
+• Dar honra — Reconocer y valorar a quienes corresponde.</t>
         </is>
       </c>
       <c r="AB45" s="4" t="inlineStr">
         <is>
-          <t>Efesios 4:28 — El que antes robaba, que no vuelva a robar; al contrario, que trabaje y use sus manos para el bien, a fin de que pueda compartir algo con quien tenga alguna necesidad</t>
+          <t>Efesios 4:28 — El que antes robaba, que no vuelva a robar; al contrario, que trabaje y use sus manos para el bien, a fin de que pueda compartir algo con quien tenga alguna necesidad.</t>
         </is>
       </c>
       <c r="AC45" s="4" t="inlineStr">
@@ -9890,7 +9919,7 @@
       </c>
       <c r="AD45" s="4" t="inlineStr">
         <is>
-          <t>2 Tesalonicenses 3:12 — A tales personas les ordenamos y exhortamos, por nuestro Senor Jesucristo, que simplemente se pongan a trabajar y se ganen su propio pan</t>
+          <t>2 Tesalonicenses 3:12 — A tales personas les ordenamos y alentamos, por nuestro Señor Jesucristo, que simplemente se pongan a trabajar y se ganen su propio pan.</t>
         </is>
       </c>
       <c r="AE45" s="4" t="inlineStr">
@@ -9902,7 +9931,7 @@
       </c>
       <c r="AF45" s="4" t="inlineStr">
         <is>
-          <t>Proverbios 14:23 — Toda labor rinde sus frutos, pero hablar por hablar empobrece</t>
+          <t>Proverbios 14:23 — Toda labor rinde sus frutos, pero hablar por hablar empobrece.</t>
         </is>
       </c>
       <c r="AG45" s="4" t="inlineStr">
@@ -9914,7 +9943,7 @@
       </c>
       <c r="AH45" s="4" t="inlineStr">
         <is>
-          <t>Eclesiastes 3:22 — Lo que he visto es que no hay nada mejor para el hombre que disfrutar de su trabajo, porque eso es lo que le ha correspondido hacer</t>
+          <t>Eclesiastés 3:22 — Lo que he visto es que no hay nada mejor para el hombre que disfrutar de su trabajo, porque eso es lo que le ha correspondido hacer. Porque ¿quién va a traerlo a ver lo que pasará después de su muerte?</t>
         </is>
       </c>
       <c r="AI45" s="4" t="inlineStr">
@@ -9926,14 +9955,14 @@
       </c>
       <c r="AJ45" s="4" t="inlineStr">
         <is>
-          <t>Proverbios 22:29 — Cuando veas alguien que hace bien su trabajo, no lo veras entre gente de baja condicion sino que estara en presencia de reyes</t>
+          <t>1 Timoteo 5:18 — Pues la Escritura dice: «No pondrás bozal al buey que trilla», y: «Digno es el obrero de su salario.»</t>
         </is>
       </c>
       <c r="AK45" s="4" t="inlineStr">
         <is>
-          <t>• El diligente en su oficio llega lejos
-• La excelencia distingue, sin importar el rubro
-• Todo oficio hecho con esmero tiene valor</t>
+          <t>• Valorar al trabajador — Su esfuerzo merece reconocimiento.
+• Dar una justa recompensa — “Digno es el obrero de su salario”.
+• Practicar la justicia — Honrar a quienes sirven y trabajan.</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10083,7 @@
       </c>
       <c r="X46" s="6" t="inlineStr">
         <is>
-          <t>Lucas 10:33-34 — Un samaritano, que iba de camino, se acerco al hombre y, al verlo, se compadecio de el y le curo las heridas con aceite y vino, y se las vendo; luego lo puso sobre su cabalgadura y lo llevo a una posada, y cuido de el</t>
+          <t>Lucas 10:33-34 — Pero un samaritano, que iba de camino, se acercó al hombre y, al verlo, se compadeció de él y le curó las heridas con aceite y vino, y se las vendó; luego lo puso sobre su cabalgadura y lo llevó a una posada, y cuidó de él.</t>
         </is>
       </c>
       <c r="Y46" s="6" t="inlineStr">
@@ -10066,7 +10095,8 @@
       </c>
       <c r="Z46" s="6" t="inlineStr">
         <is>
-          <t>Salmo 46:1 — Dios es nuestro amparo y fortaleza, nuestro pronto auxilio en todos los problemas</t>
+          <t>Salmos 46:1 — Dios es nuestro amparo y fortaleza,
+nuestro pronto auxilio en todos los problemas.</t>
         </is>
       </c>
       <c r="AA46" s="6" t="inlineStr">
@@ -10078,7 +10108,8 @@
       </c>
       <c r="AB46" s="6" t="inlineStr">
         <is>
-          <t>Proverbios 24:11 — Libera a los que marchan a la muerte; salva a los que estan por ser ejecutados</t>
+          <t>Proverbios 24:11 — Libera a los que marchan a la muerte;
+salva a los que están por ser ejecutados.</t>
         </is>
       </c>
       <c r="AC46" s="6" t="inlineStr">
@@ -10090,7 +10121,8 @@
       </c>
       <c r="AD46" s="6" t="inlineStr">
         <is>
-          <t>Santiago 5:14-15 — Hay entre ustedes algun enfermo? Que se llame a los ancianos de la iglesia, para que oren por el y lo unjan con aceite en el nombre del Senor</t>
+          <t>Santiago 5:14-15 — ¿Hay entre ustedes algún enfermo? Que se llame a los ancianos de la iglesia, para que oren por él y lo unjan con aceite en el nombre del Señor.
+La oración de fe sanará al enfermo, y el Señor lo levantará de su lecho. Si acaso ha pecado, sus pecados le serán perdonados.</t>
         </is>
       </c>
       <c r="AE46" s="6" t="inlineStr">
@@ -10102,7 +10134,8 @@
       </c>
       <c r="AF46" s="6" t="inlineStr">
         <is>
-          <t>Salmo 34:17 — Los justos gimen, y el Senor los escucha y los libra de todas sus angustias</t>
+          <t>Salmos 34:17 — Los justos gimen, y el Señor los escucha
+y los libra de todas sus angustias.</t>
         </is>
       </c>
       <c r="AG46" s="6" t="inlineStr">
@@ -10114,7 +10147,7 @@
       </c>
       <c r="AH46" s="6" t="inlineStr">
         <is>
-          <t>Isaias 41:10 — No tengas miedo, que yo estoy contigo; no te desanimes, que yo soy tu Dios. Yo soy quien te da fuerzas, y siempre te ayudare; siempre te sostendre con mi justiciera mano derecha</t>
+          <t>Isaías 41:10 — No tengas miedo, que yo estoy contigo; no te desanimes, que yo soy tu Dios. Yo soy quien te da fuerzas, y siempre te ayudaré; siempre te sostendré con mi justiciera mano derecha.</t>
         </is>
       </c>
       <c r="AI46" s="6" t="inlineStr">
@@ -10126,14 +10159,15 @@
       </c>
       <c r="AJ46" s="6" t="inlineStr">
         <is>
-          <t>2 Timoteo 1:7 — Porque no nos ha dado Dios un espiritu de cobardia, sino de poder, de amor y de dominio propio</t>
+          <t>Salmos 50:15 — Invócame en el día de la angustia;
+yo te libraré, y tú me honrarás.»</t>
         </is>
       </c>
       <c r="AK46" s="6" t="inlineStr">
         <is>
-          <t>• El temor no viene de Dios
-• El dominio propio ayuda a actuar con claridad en emergencias
-• La calma es posible incluso bajo presión</t>
+          <t>1, Invocar a Dios en la angustia.
+2, Confiar en su liberación.
+3, Honrar a Dios por su respuesta.</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10288,8 @@
       </c>
       <c r="X47" s="8" t="inlineStr">
         <is>
-          <t>Salmo 100:2 — Sirvan al Senor con alegria! Vengan a su presencia con regocijo</t>
+          <t>Salmos 100:2 — ¡Sirvan al Señor con alegría!
+¡Vengan a su presencia felices!</t>
         </is>
       </c>
       <c r="Y47" s="8" t="inlineStr">
@@ -10266,7 +10301,7 @@
       </c>
       <c r="Z47" s="8" t="inlineStr">
         <is>
-          <t>Juan 4:24 — Dios es Espiritu; y es necesario que los que lo adoran, lo adoren en espiritu y en verdad</t>
+          <t>Juan 4:24 — Dios es Espíritu; y es necesario que los que lo adoran, lo adoren en espíritu y en verdad.»</t>
         </is>
       </c>
       <c r="AA47" s="8" t="inlineStr">
@@ -10278,7 +10313,7 @@
       </c>
       <c r="AB47" s="8" t="inlineStr">
         <is>
-          <t>Salmo 34:1 — Bendecire al Senor en todo tiempo; su alabanza estara siempre en mi boca</t>
+          <t>Salmo 34:1 — Bendeciré al Señor en todo tiempo; su alabanza estará siempre en mi boca.</t>
         </is>
       </c>
       <c r="AC47" s="8" t="inlineStr">
@@ -10290,14 +10325,14 @@
       </c>
       <c r="AD47" s="8" t="inlineStr">
         <is>
-          <t>1 Tesalonicenses 5:18 — Den gracias a Dios en todo, porque esta es su voluntad para ustedes en Cristo Jesus</t>
+          <t>Santiago 5:13 — ¿Hay alguien entre ustedes que esté sufriendo? Que ore a Dios. ¿Alguno de ustedes está de buen humor? Que cante alabanzas.</t>
         </is>
       </c>
       <c r="AE47" s="8" t="inlineStr">
         <is>
-          <t>• Dar gracias en todo, no por todo
-• Es la voluntad de Dios para nosotros
-• La gratitud transforma la perspectiva</t>
+          <t>• • La oración como respuesta al sufrimiento.
+• • La alabanza como expresión de gratitud.
+• • Una fe para todas las estaciones de la vida.</t>
         </is>
       </c>
       <c r="AF47" s="8" t="inlineStr">
@@ -10314,7 +10349,7 @@
       </c>
       <c r="AH47" s="8" t="inlineStr">
         <is>
-          <t>Hebreos 13:15 — Ofrezcamos siempre a Dios, por medio de Jesus, un sacrificio de alabanza, es decir, el fruto de labios que confiesen su nombre</t>
+          <t>Hebreos 13:15 — Por lo tanto, ofrezcamos siempre a Dios, por medio de Jesús, un sacrificio de alabanza, es decir, el fruto de labios que confiesen su nombre.</t>
         </is>
       </c>
       <c r="AI47" s="8" t="inlineStr">
@@ -10326,14 +10361,22 @@
       </c>
       <c r="AJ47" s="8" t="inlineStr">
         <is>
-          <t>Salmo 95:1-2 — Vengan y con alegria aclamemos al Senor! Cantemos con jubilo a la roca de nuestra salvacion! Lleguemos ante su presencia con alabanza! Aclamemosle con canticos</t>
+          <t>Habacuc 3:17-19 — Aunque todavía no florece la higuera,
+ni hay uvas en los viñedos,
+ni hay tampoco aceitunas en los olivos,
+ni los campos han rendido sus cosechas;
+aunque no hay ovejas en los rediles
+ni vacas en los corrales, yo me alegro por ti, Señor;
+¡me gozo en ti, Dios de mi salvación!
+Tú, Señor, eres mi Dios y fortaleza.
+Tú, Señor, me das pies ligeros, como de cierva, y me haces andar en mis alturas.</t>
         </is>
       </c>
       <c r="AK47" s="8" t="inlineStr">
         <is>
-          <t>• Aclamar con alegría, no con rutina
-• Venir con acción de gracias
-• Cantar salmos como expresión de gozo</t>
+          <t>• La pérdida material no define la relación con Dios.
+• El gozo como una decisión espiritual.
+• La fortaleza y la elevación sobrenatural.</t>
         </is>
       </c>
     </row>
@@ -10454,7 +10497,7 @@
       </c>
       <c r="X48" s="10" t="inlineStr">
         <is>
-          <t>Santiago 1:5 — Si alguno de ustedes requiere de sabiduria, pidasela a Dios, y el se la dara, pues Dios se la da a todos en abundancia y sin hacer ningun reproche</t>
+          <t>Santiago 1:5 — Si alguno de ustedes requiere de sabiduría, pídasela a Dios, y él se la dará, pues Dios se la da a todos en abundancia y sin hacer ningún reproche.</t>
         </is>
       </c>
       <c r="Y48" s="10" t="inlineStr">
@@ -10466,7 +10509,8 @@
       </c>
       <c r="Z48" s="10" t="inlineStr">
         <is>
-          <t>Proverbios 3:5-6 — Confia en el Senor de todo corazon, y no te apoyes en tu propia prudencia. Reconocelo en todos tus caminos, y el enderezara tus sendas</t>
+          <t>Proverbios 3:5-6 — Confía en el Señor de todo corazón, y no te apoyes en tu propia prudencia.
+Reconócelo en todos tus caminos, y él enderezará tus senderos.</t>
         </is>
       </c>
       <c r="AA48" s="10" t="inlineStr">
@@ -10478,19 +10522,24 @@
       </c>
       <c r="AB48" s="10" t="inlineStr">
         <is>
-          <t>Proverbios 21:5 — Si piensas lo que haces, tendras abundancia; si te apresuras, acabaras en la pobreza</t>
+          <t>Proverbios 3:21-23 — Hijo mío, preserva la ley y el consejo;
+nunca pierdas esto de vista.
+Estos darán vida a tu alma
+y adornarán tu cuello.
+Así podrás andar confiado en tu camino,
+y nunca tus pies tropezarán.</t>
         </is>
       </c>
       <c r="AC48" s="10" t="inlineStr">
         <is>
-          <t>• Los pensamientos diligentes traen abundancia
-• La prisa apresurada lleva a la pobreza
-• Planificar con cuidado rinde fruto</t>
+          <t>• Guarda la sabiduría: No pierdas de vista la enseñanza de Dios.
+• Trae vida al alma: Su consejo nos fortalece y guía.
+• Camina con confianza: Dios dirige nuestros pasos y nos ayuda a no tropezar.</t>
         </is>
       </c>
       <c r="AD48" s="10" t="inlineStr">
         <is>
-          <t>Eclesiastes 11:4 — Quien vigila al viento no siembra; quien contempla las nubes no cosecha</t>
+          <t>Eclesiastes 11:4 — El que sólo mira el viento, no siembra; el que sólo contempla las nubes, no cosecha.</t>
         </is>
       </c>
       <c r="AE48" s="10" t="inlineStr">
@@ -10502,7 +10551,7 @@
       </c>
       <c r="AF48" s="10" t="inlineStr">
         <is>
-          <t>1 Reyes 3:9 — Yo te pido que me des un corazon con mucho entendimiento para gobernar a tu pueblo y para discernir entre lo bueno y lo malo</t>
+          <t>1 Reyes 3:9 — Yo te pido que me des un corazón con mucho entendimiento para gobernar a tu pueblo y para diferenciar entre lo bueno y lo malo. Porque ¿quién es capaz de gobernar a este pueblo tan grande?»</t>
         </is>
       </c>
       <c r="AG48" s="10" t="inlineStr">
@@ -10514,7 +10563,8 @@
       </c>
       <c r="AH48" s="10" t="inlineStr">
         <is>
-          <t>Salmo 32:8 — Yo te voy a hacer que entiendas. Voy a ensenarte el camino que debes seguir, y no voy a quitarte los ojos de encima</t>
+          <t>Salmos 32:8 — «Yo te voy a hacer que entiendas.
+Voy a enseñarte el camino que debes seguir, y no voy a quitarte los ojos de encima.</t>
         </is>
       </c>
       <c r="AI48" s="10" t="inlineStr">
@@ -10526,7 +10576,8 @@
       </c>
       <c r="AJ48" s="10" t="inlineStr">
         <is>
-          <t>Proverbios 19:21 — El hombre hace muchos planes, pero solo se realiza el proposito divino</t>
+          <t>Proverbios 19:21 — Son muchas las ideas del corazón humano;
+solo el consejo del Señor permanece.</t>
         </is>
       </c>
       <c r="AK48" s="10" t="inlineStr">
@@ -10654,7 +10705,14 @@
       </c>
       <c r="X49" s="12" t="inlineStr">
         <is>
-          <t>Salmo 78:4 — No las mantendremos ocultas a nuestros hijos, sino que diremos a las generaciones futuras que el Senor es digno de alabanza por su poder y por sus hechos maravillosos</t>
+          <t>Salmos 78:2-4 — Abriré mi boca y diré proverbios;
+hablaré de los misterios de tiempos pasados,
+de cosas que ya hemos oído y que conocemos
+porque nuestros padres nos las contaron.
+No las mantendremos ocultas a nuestros hijos,
+sino que diremos a las generaciones futuras
+que el Señor es digno de alabanza
+por su poder y por sus hechos maravillosos.</t>
         </is>
       </c>
       <c r="Y49" s="12" t="inlineStr">
@@ -10666,7 +10724,7 @@
       </c>
       <c r="Z49" s="12" t="inlineStr">
         <is>
-          <t>Deuteronomio 11:19 — Ensenenselas a sus hijos, y hablen de ellas cuando te encuentres descansando en tu casa, y cuando vayas por el camino, y cuando te acuestes, y cuando te levantes</t>
+          <t>Deuteronomio 11:19 — Enséñenselas a sus hijos, y hablen de ellas cuando te encuentres descansando en tu casa, y cuando vayas por el camino, y cuando te acuestes, y cuando te levantes.</t>
         </is>
       </c>
       <c r="AA49" s="12" t="inlineStr">
@@ -10678,7 +10736,8 @@
       </c>
       <c r="AB49" s="12" t="inlineStr">
         <is>
-          <t>Josue 4:6 — Cada una de ellas sera una senal. Y el dia de manana, cuando los hijos les pregunten a sus padres que significan estas piedras, ellos les responderan</t>
+          <t>Josue 4:6-7 — Cada una de ellas será una señal. Y el día de mañana, cuando los hijos les pregunten a sus padres qué significan estas piedras,
+ellos les responderán: “Cuando el pueblo cruzó el Jordán, las aguas del río se partieron en dos delante del arca del pacto del Señor. Así que estas piedras son para que los hijos de Israel recuerden siempre lo que aquí pasó.”»</t>
         </is>
       </c>
       <c r="AC49" s="12" t="inlineStr">
@@ -10690,19 +10749,23 @@
       </c>
       <c r="AD49" s="12" t="inlineStr">
         <is>
-          <t>Proverbios 22:6 — Ensena al nino a seguir fielmente su camino, y aunque llegue a anciano no se apartara de el</t>
+          <t>1 Crónicas 16:28-29 — Ustedes, familias de los pueblos,
+¡tributen al Señor la gloria y el poder!
+¡Tributen al Señor la honra que merece su nombre!
+¡Traigan sus ofrendas, y vengan a su presencia!
+¡Adoren al Señor en la hermosura de la santidad!</t>
         </is>
       </c>
       <c r="AE49" s="12" t="inlineStr">
         <is>
-          <t>• Instruir desde niño perdura en el tiempo
-• La formación temprana no se olvida
-• El fruto llega con los años</t>
+          <t>• Dar gloria a Dios — Reconocer su grandeza y poder.
+• Entregar nuestras ofrendas — Dar con un corazón dispuesto.
+• Adorar con reverencia — Acercarnos a Dios con un corazón sincero.</t>
         </is>
       </c>
       <c r="AF49" s="12" t="inlineStr">
         <is>
-          <t>Hechos 16:31 — Ellos le dijeron: Cree en el Senor Jesucristo, y se salvaran tu y tu familia</t>
+          <t>Hechos 16:31 — Ellos le dijeron: «Cree en el Señor Jesucristo, y se salvarán tú y tu familia.»</t>
         </is>
       </c>
       <c r="AG49" s="12" t="inlineStr">
@@ -10714,7 +10777,8 @@
       </c>
       <c r="AH49" s="12" t="inlineStr">
         <is>
-          <t>Salmo 128:1 — Dichosos todos los que honran al Senor! Dichosos los que van por sus caminos</t>
+          <t>Salmos 128:1 — ¡Dichosos todos los que honran al Señor!
+¡Dichosos los que van por sus caminos!</t>
         </is>
       </c>
       <c r="AI49" s="12" t="inlineStr">
@@ -10726,7 +10790,7 @@
       </c>
       <c r="AJ49" s="12" t="inlineStr">
         <is>
-          <t>Malaquias 4:6 — El hara que el corazon de los padres se vuelva hacia los hijos, y que el corazon de los hijos se vuelva hacia los padres, para que yo no venga a destruir la tierra por completo</t>
+          <t>Malaquías 4:6 — Y él hará que el corazón de los padres se vuelva hacia los hijos, y que el corazón de los hijos se vuelva hacia los padres, para que yo no venga a destruir la tierra por completo.»</t>
         </is>
       </c>
       <c r="AK49" s="12" t="inlineStr">
@@ -10854,19 +10918,19 @@
       </c>
       <c r="X50" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 22:7 — Los ricos son los amos de los pobres; los deudores son esclavos de los prestamistas</t>
+          <t>Deuteronomio 15:6 — Puesto que el Señor tu Dios te bendecirá, como te lo ha prometido, podrás hacer préstamos a muchas naciones, pero tú no pedirás prestado nada; dominarás a muchas naciones, pero a ti nadie te dominará.</t>
         </is>
       </c>
       <c r="Y50" s="14" t="inlineStr">
         <is>
-          <t>• El deudor pierde libertad frente al acreedor
-• La deuda tiene consecuencias más allá del dinero
-• Evaluar antes de comprometerse</t>
+          <t>• Dios bendice: Él es la fuente de nuestra provisión.  
+• Prosperidad con propósito: La bendición permite ayudar y prestar a otros.  
+• Libertad financiera: No vivir bajo la esclavitud de las deudas.</t>
         </is>
       </c>
       <c r="Z50" s="14" t="inlineStr">
         <is>
-          <t>Romanos 13:8 — No tengan deudas con nadie, aparte de la deuda de amarse unos a otros; porque el que ama al projimo, ha cumplido la ley</t>
+          <t>Romanos 13:8 — No tengan deudas con nadie, aparte de la deuda de amarse unos a otros; porque el que ama al prójimo, ha cumplido la ley.</t>
         </is>
       </c>
       <c r="AA50" s="14" t="inlineStr">
@@ -10878,7 +10942,8 @@
       </c>
       <c r="AB50" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 22:26-27 — No te comprometas por otros, ni salgas fiador de nadie. Por que han de quitarte hasta la cama si resulta que no tienes con que pagar</t>
+          <t>Proverbios 22:26-27 — No te comprometas por otros, ni salgas fiador de nadie.
+¿Por qué han de quitarte hasta la cama si resulta que no tienes con qué pagar?</t>
         </is>
       </c>
       <c r="AC50" s="14" t="inlineStr">
@@ -10890,7 +10955,8 @@
       </c>
       <c r="AD50" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 6:1-5 — Se como gacela, y escapate del cazador; se como un ave, y librate del que pone trampas</t>
+          <t>Proverbios 6:5 — Sé como gacela, y escápate del cazador;
+sé como un ave, y líbrate del que pone trampas.</t>
         </is>
       </c>
       <c r="AE50" s="14" t="inlineStr">
@@ -10902,38 +10968,39 @@
       </c>
       <c r="AF50" s="14" t="inlineStr">
         <is>
-          <t>Genesis 41:34-36 — Se deben almacenar todos los alimentos de estos buenos anos que vienen, y bajo el control de Su Majestad recogerse y guardarse el trigo, para el sustento de las ciudades. Asi el pais no perecera de hambre</t>
+          <t>Deuteronomio 8:17 — No vayas a decir en tu corazón: “Mi poder y la fuerza de mi brazo me han hecho ganar estas riquezas.”</t>
         </is>
       </c>
       <c r="AG50" s="14" t="inlineStr">
         <is>
-          <t>• Guardar en tiempos buenos para los difíciles
-• La previsión evita el desastre
-• Planificar a largo plazo protege</t>
+          <t>• El peligro de la autosuficiencia
+• La raíz interior del orgullo.
+• El olvido del verdadero origen de los bienes:</t>
         </is>
       </c>
       <c r="AH50" s="14" t="inlineStr">
         <is>
-          <t>Proverbios 21:20 — Riquezas y perfumes hay en la casa del sabio; en la casa del necio solo hay despilfarro</t>
+          <t>Salmos 37:21 — El malvado pide prestado y no paga;
+el justo es bondadoso y comparte lo que tiene.</t>
         </is>
       </c>
       <c r="AI50" s="14" t="inlineStr">
         <is>
-          <t>• El sabio guarda tesoro
-• El necio lo gasta todo sin reserva
-• La reserva es signo de sabiduría</t>
+          <t>• Cumplir con nuestras deudas.
+• Ser bondadosos con los demás.
+• Compartir lo que tenemos.</t>
         </is>
       </c>
       <c r="AJ50" s="14" t="inlineStr">
         <is>
-          <t>Salmo 37:21 — El malvado pide prestado y no paga; el justo es bondadoso y comparte lo que tiene</t>
+          <t>Mateo 6:33 — Por lo tanto, busquen primeramente el reino de Dios y su justicia, y todas estas cosas les serán añadidas.</t>
         </is>
       </c>
       <c r="AK50" s="14" t="inlineStr">
         <is>
-          <t>• El impío no paga sus deudas
-• El justo tiene misericordia y da
-• El carácter se ve en como se maneja el dinero</t>
+          <t>• La prioridad máxima: buscar primero el reino de Dios.
+• El estándar de vida: y su justicia.
+• La promesa de provisión: y todas estas cosas les serán añadidas.</t>
         </is>
       </c>
     </row>
@@ -11054,31 +11121,40 @@
       </c>
       <c r="X51" s="2" t="inlineStr">
         <is>
-          <t>Filipenses 3:13 — Hermanos, yo mismo no pretendo haberlo alcanzado ya; pero una cosa si hago: me olvido ciertamente de lo que ha quedado atras, y me extiendo hacia lo que esta delante</t>
+          <t>Salmos 32:3-5 — Mientras callé, mis huesos envejecieron,
+pues todo el día me quejaba.
+De día y de noche me hiciste padecer;
+mi juventud se volvió sequedad de verano.
+Te confesé mi pecado; no oculté mi maldad.
+Me dije: «Confesaré al Señor mi rebeldía»,
+y tú perdonaste la maldad de mi pecado.</t>
         </is>
       </c>
       <c r="Y51" s="2" t="inlineStr">
         <is>
-          <t>• Olvidar lo que queda atrás
-• Extenderse a lo que esta delante
-• El progreso requiere soltar el pasado</t>
+          <t>• El peso del silencio y el pecado oculto
+• La convicción y la carga de Dios
+• La confesión sincera y el perdón inmediato</t>
         </is>
       </c>
       <c r="Z51" s="2" t="inlineStr">
         <is>
-          <t>Proverbios 24:16 — Los justos podran tropezar siete veces, pero volveran a levantarse. En cambio, basta una sola calamidad para derribar al perverso</t>
+          <t>Proverbios 28:13 — El que encubre sus pecados no prospera;
+el que los confiesa y se aparta de ellos
+alcanza la misericordia divina.</t>
         </is>
       </c>
       <c r="AA51" s="2" t="inlineStr">
         <is>
-          <t>• El justo cae, pero se levanta
-• La caída no define el resultado final
-• Levantarse es lo que distingue al sabio</t>
+          <t>• Reconocer el pecado: No esconder nuestras faltas.  
+• Confesar y apartarse: Arrepentirse y cambiar de camino.  
+• Recibir misericordia: Dios perdona al que se arrepiente sinceramente.</t>
         </is>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
-          <t>Isaias 43:18-19 — No se acuerden de las cosas pasadas, ni piensen en las cosas antiguas. Fijense en que yo hago algo nuevo, que pronto saldra a la luz. Volvere a abrir un camino en el desierto, y hare que corran rios en el paramo</t>
+          <t>Isaías 43:18-19 — «Ya no se acuerden de las cosas pasadas; no hagan memoria de las cosas antiguas.
+Fíjense en que yo hago algo nuevo, que pronto saldrá a la luz. ¿Acaso no lo saben? Volveré a abrir un camino en el desierto, y haré que corran ríos en el sequedal.</t>
         </is>
       </c>
       <c r="AC51" s="2" t="inlineStr">
@@ -11090,7 +11166,8 @@
       </c>
       <c r="AD51" s="2" t="inlineStr">
         <is>
-          <t>Romanos 5:3-4 — No solo esto, sino que tambien nos regocijamos en los sufrimientos, porque sabemos que los sufrimientos producen resistencia, la resistencia produce un caracter aprobado, y el caracter aprobado produce esperanza</t>
+          <t>Romanos 5:3-4 — Y no solo esto, sino que también nos gozamos en los sufrimientos, porque sabemos que los sufrimientos producen resistencia,
+la resistencia produce un carácter aprobado, y el carácter aprobado produce esperanza.</t>
         </is>
       </c>
       <c r="AE51" s="2" t="inlineStr">
@@ -11102,7 +11179,9 @@
       </c>
       <c r="AF51" s="2" t="inlineStr">
         <is>
-          <t>Santiago 1:2-4 — Hermanos mios, considerense muy dichosos cuando esten pasando por diversas pruebas. Bien saben que, cuando su fe es puesta a prueba, produce paciencia. Pero procuren que la paciencia complete su obra, para que sean perfectos y cabales</t>
+          <t>Santiago 1:2-4 — Hermanos míos, considérense muy dichosos cuando estén pasando por diversas pruebas.
+Bien saben que, cuando su fe es puesta a prueba, produce paciencia.
+Pero intenten que la paciencia complete su obra, para que sean perfectos e íntegros, sin que les falte nada.</t>
         </is>
       </c>
       <c r="AG51" s="2" t="inlineStr">
@@ -11114,7 +11193,7 @@
       </c>
       <c r="AH51" s="2" t="inlineStr">
         <is>
-          <t>2 Corintios 4:16 — Por lo tanto, no nos desanimamos. Y aunque por fuera nos vamos desgastando, por dentro nos vamos renovando de dia en dia</t>
+          <t>2 Corintios 4:16 — Por lo tanto, no nos desanimamos. Y aunque por fuera nos vamos desgastando, por dentro nos vamos renovando de día en día.</t>
         </is>
       </c>
       <c r="AI51" s="2" t="inlineStr">
@@ -11126,7 +11205,8 @@
       </c>
       <c r="AJ51" s="2" t="inlineStr">
         <is>
-          <t>Proverbios 4:18 — Pero la senda de los justos es como la aurora: su luz va en aumento, hasta la plenitud del dia</t>
+          <t>Proverbios 4:18 — Pero el camino de los justos es como el amanecer:
+¡su luz va en aumento, hasta la plenitud del día!</t>
         </is>
       </c>
       <c r="AK51" s="2" t="inlineStr">
@@ -11254,7 +11334,8 @@
       </c>
       <c r="X52" s="4" t="inlineStr">
         <is>
-          <t>Exodo 31:3-4 — Lo he llenado del espiritu de Dios en sabiduria, inteligencia y ciencia, y en todo arte, para crear nuevos disenos y trabajar en oro, plata y bronce</t>
+          <t>Éxodo 31:3-4 — Lo he llenado del espíritu de Dios en sabiduría, inteligencia y ciencia, y en todo arte,
+para crear nuevos diseños y trabajar en oro, plata y bronce.</t>
         </is>
       </c>
       <c r="Y52" s="4" t="inlineStr">
@@ -11266,19 +11347,20 @@
       </c>
       <c r="Z52" s="4" t="inlineStr">
         <is>
-          <t>Isaias 43:19 — Fijense en que yo hago algo nuevo, que pronto saldra a la luz. Acaso no lo saben? Volvere a abrir un camino en el desierto, y hare que corran rios en el paramo</t>
+          <t>1 Corintios 9:22-23 — Entre los débiles me comporto como débil, para ganar a los débiles; me comporto como todos ante todos, para que de todos pueda yo salvar a algunos.
+Y esto lo hago por causa del evangelio, para ser copartícipe de él.</t>
         </is>
       </c>
       <c r="AA52" s="4" t="inlineStr">
         <is>
-          <t>• Dios hace cosas nuevas
-• El pasado no limita lo que viene
-• Percibir lo nuevo requiere apertura</t>
+          <t>• Empatía y adaptabilidad cultural.
+• El propósito evangelístico (ganar y salvar).
+• Compromiso y participación con el evangelio</t>
         </is>
       </c>
       <c r="AB52" s="4" t="inlineStr">
         <is>
-          <t>1 Cronicas 12:32 — De los hijos de Isacar, doscientos jefes, cuyas palabras eran respetadas por todos sus parientes, pues sabian cuando actuar y que debia hacer Israel</t>
+          <t>1 Cronicas 12:32 — De los hijos de Isacar, doscientos jefes, cuyas palabras eran respetadas por todos sus parientes, pues sabían cuándo actuar y qué debía hacer Israel.</t>
         </is>
       </c>
       <c r="AC52" s="4" t="inlineStr">
@@ -11290,7 +11372,8 @@
       </c>
       <c r="AD52" s="4" t="inlineStr">
         <is>
-          <t>Proverbios 18:15 — La mente inteligente obtiene sabiduria, y los oidos sabios van en busca de la ciencia</t>
+          <t>Proverbios 18:15 — La mente inteligente obtiene sabiduría,
+y los oídos sabios van en busca de la ciencia.</t>
         </is>
       </c>
       <c r="AE52" s="4" t="inlineStr">
@@ -11302,7 +11385,9 @@
       </c>
       <c r="AF52" s="4" t="inlineStr">
         <is>
-          <t>Eclesiastes 10:10 — Si el filo del hacha se desafila, y no se afila, hay que golpear con mas fuerza. La sabiduria es provechosa, si se sabe dirigir</t>
+          <t>Eclesiastés 10:10 — Si el filo del hacha se desafila, y no se afila,
+hay que golpear con más fuerza.
+La sabiduría es provechosa, si se sabe dirigir.</t>
         </is>
       </c>
       <c r="AG52" s="4" t="inlineStr">
@@ -11314,7 +11399,8 @@
       </c>
       <c r="AH52" s="4" t="inlineStr">
         <is>
-          <t>Proverbios 27:12 — El astuto ve el peligro y se pone a salvo, pero los ingenuos lo ven y no lo evitan</t>
+          <t>Proverbios 27:12 — El astuto ve el peligro y se pone a salvo,
+pero los ingenuos lo ven y no lo evitan.</t>
         </is>
       </c>
       <c r="AI52" s="4" t="inlineStr">
@@ -11326,7 +11412,8 @@
       </c>
       <c r="AJ52" s="4" t="inlineStr">
         <is>
-          <t>Proverbios 1:5 — Que lo oiga el sabio, y aumente su saber, y que el entendido reciba consejo</t>
+          <t>Proverbios 1:5 — Que lo oiga el sabio, y aumente su saber,
+y que el entendido reciba consejo</t>
         </is>
       </c>
       <c r="AK52" s="4" t="inlineStr">
@@ -11454,19 +11541,19 @@
       </c>
       <c r="X53" s="56" t="inlineStr">
         <is>
-          <t>3 Juan 1:2 — Amado, deseo que seas prosperado en todo, y que tengas salud, a la vez que tu alma prospera</t>
+          <t>Éxodo 23:25 — Pero me servirán a mí, el Señor su Dios, y yo bendeciré tu pan y tus aguas, y quitaré de en medio de ti toda enfermedad.</t>
         </is>
       </c>
       <c r="Y53" s="6" t="inlineStr">
         <is>
-          <t>• La prosperidad del alma y del cuerpo están conectadas
-• Dios desea bienestar integral
-• La salud incluye más que lo físico</t>
+          <t>• La condición (Servicio exclusivo a Dios).
+• La provisión (Bendición del pan y del agua).
+• La sanidad y protección (Remoción de la enfermedad)</t>
         </is>
       </c>
       <c r="Z53" s="6" t="inlineStr">
         <is>
-          <t>Santiago 5:16 — Confiesen sus pecados unos a otros, y oren unos por otros, para que sean sanados. La oracion del justo es muy poderosa y efectiva</t>
+          <t>Santiago 5:16 — Confiesen sus pecados unos a otros, y oren unos por otros, para que sean sanados. La oración del justo es muy poderosa y efectiva.</t>
         </is>
       </c>
       <c r="AA53" s="6" t="inlineStr">
@@ -11478,7 +11565,7 @@
       </c>
       <c r="AB53" s="6" t="inlineStr">
         <is>
-          <t>Salmo 147:3 — El Senor reanima a los descorazonados, y sana sus heridas</t>
+          <t>Salmo 147:3 — El Señor reanima a los descorazonados, y sana sus heridas.</t>
         </is>
       </c>
       <c r="AC53" s="6" t="inlineStr">
@@ -11490,7 +11577,7 @@
       </c>
       <c r="AD53" s="6" t="inlineStr">
         <is>
-          <t>Mateo 9:12 — Al oir esto, Jesus les dijo: No son los sanos los que necesitan de un medico, sino los enfermos</t>
+          <t>Mateo 9:12 — Al oír esto, Jesús les dijo: «No son los sanos los que necesitan de un médico, sino los enfermos.</t>
         </is>
       </c>
       <c r="AE53" s="6" t="inlineStr">
@@ -11502,7 +11589,9 @@
       </c>
       <c r="AF53" s="6" t="inlineStr">
         <is>
-          <t>Isaias 53:5 — Pero el sera herido por nuestros pecados; molido por nuestras rebeliones! Sobre el vendra el castigo de nuestra paz, y por su llaga seremos sanados</t>
+          <t>Isaías 53:5 — Pero él será herido por nuestros pecados;
+¡molido por nuestras rebeliones!
+Sobre él vendrá el castigo de nuestra paz, y por su llaga seremos sanados.</t>
         </is>
       </c>
       <c r="AG53" s="6" t="inlineStr">
@@ -11514,7 +11603,8 @@
       </c>
       <c r="AH53" s="6" t="inlineStr">
         <is>
-          <t>Proverbios 17:22 — Un corazon alegre es la mejor medicina; un animo triste deprime a todo el cuerpo</t>
+          <t>Proverbios 17:22 — Un corazón alegre es la mejor medicina;
+un ánimo triste deprime a todo el cuerpo.</t>
         </is>
       </c>
       <c r="AI53" s="6" t="inlineStr">
@@ -11526,14 +11616,15 @@
       </c>
       <c r="AJ53" s="6" t="inlineStr">
         <is>
-          <t>Jeremias 30:17 — Aunque te han llamado la despreciada, y aunque dicen: Esta es Sion, de la que nadie se acuerda, yo te devolvere la salud y sanare tus heridas. Palabra del Senor</t>
+          <t>Proverbios 16:24 — Las palabras amables son un panal de miel;
+endulzan el alma y sanan el cuerpo.</t>
         </is>
       </c>
       <c r="AK53" s="6" t="inlineStr">
         <is>
-          <t>• Dios promete restaurar y sanar
-• La sanidad es acto de Su fidelidad
-• Confiar en Su promesa sostiene la esperanza</t>
+          <t>• El poder de la comunicación bondadosa 
+• Bienestar y alivio para el interior (el alma)
+• Salud y efecto integral (el cuerpo o los huesos)</t>
         </is>
       </c>
     </row>
@@ -15838,7 +15929,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mensajero: guiones de febrero (semanas 5 a 8)
24 guiones sobre el versículo de cada día (lunes a viernes) y el resumen
del sábado: liderazgo, hogar, ahorro y cuidado del alma. Tildes en el
Salmo 34:18 y en algunos puntos; «por qué ahorrar» en el subtema.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -1927,7 +1927,7 @@
         <is>
           <t>• El corazón es la fuente de la vida
 • Cuidarlo con diligencia es prioridad
-• De el salen las decisiones de un líder</t>
+• De él salen las decisiones de un líder</t>
         </is>
       </c>
       <c r="AB6" s="33" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="G8" s="40" t="inlineStr">
         <is>
-          <t>Principios de por que ahorrar</t>
+          <t>Principios de por qué ahorrar</t>
         </is>
       </c>
       <c r="H8" s="40" t="inlineStr">
@@ -2575,7 +2575,7 @@
       <c r="AG9" s="43" t="inlineStr">
         <is>
           <t>• El temor no viene de Dios
-• Poder, amor y dominio propio si vienen de El
+• Poder, amor y dominio propio sí vienen de Él
 • El miedo paralizante no es la identidad dada por Dios</t>
         </is>
       </c>
@@ -2593,12 +2593,12 @@
       </c>
       <c r="AJ9" s="42" t="inlineStr">
         <is>
-          <t>Salmo 34:18 — Cercano esta el Senor para salvar a los que tienen roto el corazon y el espiritu</t>
+          <t>Salmo 34:18 — Cercano está el Señor para salvar a los que tienen roto el corazón y el espíritu</t>
         </is>
       </c>
       <c r="AK9" s="43" t="inlineStr">
         <is>
-          <t>• Dios esta cerca del quebrantado
+          <t>• Dios está cerca del quebrantado
 • El dolor no aleja a Dios, lo acerca
 • Consuelo real en momentos de angustia</t>
         </is>
@@ -13444,7 +13444,7 @@
       </c>
       <c r="E23" s="16" t="inlineStr">
         <is>
-          <t>Principios de por que ahorrar</t>
+          <t>Principios de por qué ahorrar</t>
         </is>
       </c>
       <c r="F23" s="16" t="inlineStr">
@@ -19216,7 +19216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20906,6 +20906,1606 @@
       </c>
       <c r="M25" s="61" t="n"/>
       <c r="N25" s="61" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B26" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C26" s="61" t="inlineStr">
+        <is>
+          <t>El liderazgo empieza por dentro</t>
+        </is>
+      </c>
+      <c r="D26" s="61" t="inlineStr">
+        <is>
+          <t>El corazón bombea cerca de 7.500 litros de sangre por día, sin descanso.</t>
+        </is>
+      </c>
+      <c r="E26" s="61" t="inlineStr">
+        <is>
+          <t>American Heart Association</t>
+        </is>
+      </c>
+      <c r="F26" s="61" t="inlineStr">
+        <is>
+          <t>En la Biblia, el corazón es el centro de quién sos: lo que pensás, querés y decidís. Lo que hay adentro, tarde o temprano, sale afuera.</t>
+        </is>
+      </c>
+      <c r="G26" s="61" t="inlineStr">
+        <is>
+          <t>Personas muy capaces en su trabajo que pierden su lugar por un carácter que nadie trabajó: enojo, soberbia, mentira.</t>
+        </is>
+      </c>
+      <c r="H26" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en una reacción tuya que se repite y que no te gusta. Ponele nombre y pedile a Dios que te ayude a cambiarla esta semana.</t>
+        </is>
+      </c>
+      <c r="I26" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar el corazón no pasa solo: se elige todos los días qué entra, qué se guarda y qué se suelta.</t>
+        </is>
+      </c>
+      <c r="J26" s="61" t="inlineStr">
+        <is>
+          <t>Resentimientos guardados por años que terminan enfermando relaciones en la familia y en el trabajo.</t>
+        </is>
+      </c>
+      <c r="K26" s="61" t="inlineStr">
+        <is>
+          <t>Antes de dormir, repasá el día: ¿qué guardaste hoy que no te hace bien? Soltalo en oración.</t>
+        </is>
+      </c>
+      <c r="L26" s="61" t="inlineStr">
+        <is>
+          <t>Todos lideramos a alguien: hijos, compañeros, un grupo de la iglesia. Las decisiones que tomamos con ellos salen de lo que hay en el corazón.</t>
+        </is>
+      </c>
+      <c r="M26" s="61" t="inlineStr">
+        <is>
+          <t>Jefes y padres que deciden desde el enojo o el cansancio, y después tienen que pedir disculpas.</t>
+        </is>
+      </c>
+      <c r="N26" s="61" t="inlineStr">
+        <is>
+          <t>Ante una decisión importante, si estás enojado, esperá unas horas. Decidí con el corazón en calma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B27" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C27" s="61" t="inlineStr">
+        <is>
+          <t>Primero el ejemplo, después la palabra</t>
+        </is>
+      </c>
+      <c r="D27" s="61" t="inlineStr">
+        <is>
+          <t>En un experimento clásico, niños que vieron a un adulto golpear a un muñeco repitieron casi los mismos golpes al quedarse solos con él.</t>
+        </is>
+      </c>
+      <c r="E27" s="61" t="inlineStr">
+        <is>
+          <t>Bandura, Ross y Ross, Universidad de Stanford, 1961</t>
+        </is>
+      </c>
+      <c r="F27" s="61" t="inlineStr">
+        <is>
+          <t>Pablo le pide a Tito que se muestre él mismo como ejemplo. La autoridad que más pesa es la del que hace primero lo que pide.</t>
+        </is>
+      </c>
+      <c r="G27" s="61" t="inlineStr">
+        <is>
+          <t>Padres que les piden a sus hijos dejar el celular mientras ellos no lo sueltan en la mesa.</t>
+        </is>
+      </c>
+      <c r="H27" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una cosa que les pedís a otros y hacela vos primero durante toda la semana.</t>
+        </is>
+      </c>
+      <c r="I27" s="61" t="inlineStr">
+        <is>
+          <t>Las palabras abren la puerta, pero las obras hacen que la gente crea. Sin obras, el mejor discurso suena vacío.</t>
+        </is>
+      </c>
+      <c r="J27" s="61" t="inlineStr">
+        <is>
+          <t>La desconfianza hacia líderes que prometen mucho y cumplen poco, en la política, en el trabajo y también en la iglesia.</t>
+        </is>
+      </c>
+      <c r="K27" s="61" t="inlineStr">
+        <is>
+          <t>Antes de prometer algo esta semana, preguntate si lo podés cumplir. Prometé menos y cumplí todo.</t>
+        </is>
+      </c>
+      <c r="L27" s="61" t="inlineStr">
+        <is>
+          <t>Integridad y seriedad: que lo que enseñás se vea en cómo vivís. La vida diaria es la clase que más se recuerda.</t>
+        </is>
+      </c>
+      <c r="M27" s="61" t="inlineStr">
+        <is>
+          <t>Jóvenes que se alejan de la fe porque vieron incoherencia en los adultos que admiraban.</t>
+        </is>
+      </c>
+      <c r="N27" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en alguien que te mira como ejemplo. Elegí una cosa concreta que querés que aprenda de vos y vivila hoy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C28" s="61" t="inlineStr">
+        <is>
+          <t>Nadie es demasiado joven para ser ejemplo</t>
+        </is>
+      </c>
+      <c r="D28" s="61" t="inlineStr">
+        <is>
+          <t>Los jóvenes en situación de riesgo que tuvieron un mentor tuvieron 55 % más probabilidades de inscribirse en estudios superiores.</t>
+        </is>
+      </c>
+      <c r="E28" s="61" t="inlineStr">
+        <is>
+          <t>MENTOR, The Mentoring Effect, 2014</t>
+        </is>
+      </c>
+      <c r="F28" s="61" t="inlineStr">
+        <is>
+          <t>Timoteo era joven y Pablo le dice que no deje que eso lo frene. La integridad no espera a tener canas.</t>
+        </is>
+      </c>
+      <c r="G28" s="61" t="inlineStr">
+        <is>
+          <t>Jóvenes que creen que no tienen nada para aportar porque nadie los toma en serio.</t>
+        </is>
+      </c>
+      <c r="H28" s="61" t="inlineStr">
+        <is>
+          <t>Si sos joven, elegí un área donde podés dar el ejemplo ya: puntualidad, palabra, trato. Si sos adulto, dale a un joven una responsabilidad real.</t>
+        </is>
+      </c>
+      <c r="I28" s="61" t="inlineStr">
+        <is>
+          <t>La integridad no es una sola cosa: es cómo hablás, cómo actuás, cómo tratás a los demás y en quién confiás. Todo junto.</t>
+        </is>
+      </c>
+      <c r="J28" s="61" t="inlineStr">
+        <is>
+          <t>Ser muy correcto en la iglesia y otra persona en el trabajo o en las redes.</t>
+        </is>
+      </c>
+      <c r="K28" s="61" t="inlineStr">
+        <is>
+          <t>Revisá lo último que publicaste o compartiste. ¿Lo dirías igual frente a tu familia o tu pastor?</t>
+        </is>
+      </c>
+      <c r="L28" s="61" t="inlineStr">
+        <is>
+          <t>Integridad viene de «íntegro»: entero, sin partes rotas. No se negocia en lo chico, porque lo chico arrastra a lo grande.</t>
+        </is>
+      </c>
+      <c r="M28" s="61" t="inlineStr">
+        <is>
+          <t>Las mentiras pequeñas de cada día: el «estoy llegando» cuando recién salís, el «no vi tu mensaje».</t>
+        </is>
+      </c>
+      <c r="N28" s="61" t="inlineStr">
+        <is>
+          <t>Durante una semana, nada de excusas inventadas. Si llegás tarde, decí la verdad y pedí disculpas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B29" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C29" s="61" t="inlineStr">
+        <is>
+          <t>Tu nombre vale más que tu plata</t>
+        </is>
+      </c>
+      <c r="D29" s="61" t="inlineStr">
+        <is>
+          <t>«Se necesitan 20 años para construir una reputación y cinco minutos para arruinarla.»</t>
+        </is>
+      </c>
+      <c r="E29" s="61" t="inlineStr">
+        <is>
+          <t>Warren Buffett, inversor estadounidense</t>
+        </is>
+      </c>
+      <c r="F29" s="61" t="inlineStr">
+        <is>
+          <t>Hay ganancias que salen caras: cuando para ganar algo hay que mentir, el precio lo paga tu nombre.</t>
+        </is>
+      </c>
+      <c r="G29" s="61" t="inlineStr">
+        <is>
+          <t>Negocios que ganan rápido con productos de mala calidad o precios engañosos, y pierden clientes para siempre.</t>
+        </is>
+      </c>
+      <c r="H29" s="61" t="inlineStr">
+        <is>
+          <t>Si vendés o das un servicio, revisá hoy si tu precio y tu producto dicen la verdad. Corregí lo que haga falta.</t>
+        </is>
+      </c>
+      <c r="I29" s="61" t="inlineStr">
+        <is>
+          <t>La buena fama no se compra: se junta de a poco, cumpliendo una vez y otra vez.</t>
+        </is>
+      </c>
+      <c r="J29" s="61" t="inlineStr">
+        <is>
+          <t>La presión por tener éxito rápido y mostrarlo en redes, aunque no sea real.</t>
+        </is>
+      </c>
+      <c r="K29" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un compromiso pendiente (una deuda, un favor prometido, una llamada) y cumplilo esta semana.</t>
+        </is>
+      </c>
+      <c r="L29" s="61" t="inlineStr">
+        <is>
+          <t>Cuando cae el nombre, cae la confianza, y sin confianza nadie te sigue. Cuidar tu nombre es cuidar a los que dependen de vos.</t>
+        </is>
+      </c>
+      <c r="M29" s="61" t="inlineStr">
+        <is>
+          <t>Rumores y chismes que destruyen el nombre de otros en los grupos de WhatsApp.</t>
+        </is>
+      </c>
+      <c r="N29" s="61" t="inlineStr">
+        <is>
+          <t>Si te llega un comentario sobre alguien, no lo reenvíes. Si es grave, hablalo con la persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B30" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C30" s="61" t="inlineStr">
+        <is>
+          <t>Corazón íntegro y manos hábiles</t>
+        </is>
+      </c>
+      <c r="D30" s="61" t="inlineStr">
+        <is>
+          <t>Al menos el 70 % de la diferencia en el compromiso de un equipo de trabajo depende de quien lo dirige.</t>
+        </is>
+      </c>
+      <c r="E30" s="61" t="inlineStr">
+        <is>
+          <t>Gallup, State of the American Manager, 2015</t>
+        </is>
+      </c>
+      <c r="F30" s="61" t="inlineStr">
+        <is>
+          <t>David pastoreó primero ovejas en el campo, donde nadie lo veía. Ahí se formó el corazón con el que después guio a un pueblo.</t>
+        </is>
+      </c>
+      <c r="G30" s="61" t="inlineStr">
+        <is>
+          <t>Gente que solo se esfuerza cuando el jefe está mirando.</t>
+        </is>
+      </c>
+      <c r="H30" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy una tarea bien hecha que nadie va a revisar. Hacela para Dios.</t>
+        </is>
+      </c>
+      <c r="I30" s="61" t="inlineStr">
+        <is>
+          <t>Ser hábil es necesario, pero no alcanza. La habilidad sin integridad puede hacer mucho daño.</t>
+        </is>
+      </c>
+      <c r="J30" s="61" t="inlineStr">
+        <is>
+          <t>Profesionales muy capaces que usan lo que saben para aprovecharse de otros.</t>
+        </is>
+      </c>
+      <c r="K30" s="61" t="inlineStr">
+        <is>
+          <t>Usá lo que sabés para ayudar a alguien esta semana, sin cobrar ni esperar nada a cambio.</t>
+        </is>
+      </c>
+      <c r="L30" s="61" t="inlineStr">
+        <is>
+          <t>La capacidad te lleva lejos; el carácter hace que puedas quedarte. Es lo que sos cuando nadie mira.</t>
+        </is>
+      </c>
+      <c r="M30" s="61" t="inlineStr">
+        <is>
+          <t>El vuelto de más que nadie devuelve, el error de la cuenta a favor que nadie avisa.</t>
+        </is>
+      </c>
+      <c r="N30" s="61" t="inlineStr">
+        <is>
+          <t>La próxima vez que te den de más, devolvelo. Es un acto pequeño que dice mucho de quién sos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="B31" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C31" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: el líder se forma por dentro</t>
+        </is>
+      </c>
+      <c r="D31" s="61" t="inlineStr">
+        <is>
+          <t>La palabra «carácter» viene del griego y significaba la marca grabada en una moneda o en un sello.</t>
+        </is>
+      </c>
+      <c r="E31" s="61" t="inlineStr">
+        <is>
+          <t>Diccionario etimológico de la lengua castellana (Corominas)</t>
+        </is>
+      </c>
+      <c r="F31" s="61" t="inlineStr">
+        <is>
+          <t>El carácter va antes que el talento: lo que hay en el corazón sostiene lo que sabés hacer.</t>
+        </is>
+      </c>
+      <c r="G31" s="61" t="n"/>
+      <c r="H31" s="61" t="inlineStr">
+        <is>
+          <t>Elegí para la próxima semana un compromiso pequeño que nadie va a controlar, y cumplilo.</t>
+        </is>
+      </c>
+      <c r="I31" s="61" t="inlineStr">
+        <is>
+          <t>La integridad no se negocia ni en lo chico: palabra, conducta y trato van juntos, a cualquier edad.</t>
+        </is>
+      </c>
+      <c r="J31" s="61" t="n"/>
+      <c r="K31" s="61" t="n"/>
+      <c r="L31" s="61" t="inlineStr">
+        <is>
+          <t>Quién sos cuando nadie mira es quien realmente sos. Ahí se forma el líder.</t>
+        </is>
+      </c>
+      <c r="M31" s="61" t="n"/>
+      <c r="N31" s="61" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B32" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C32" s="61" t="inlineStr">
+        <is>
+          <t>Una casa se construye con sabiduría</t>
+        </is>
+      </c>
+      <c r="D32" s="61" t="inlineStr">
+        <is>
+          <t>En un estudio con familias de Los Ángeles, las mujeres que describían su casa como desordenada mostraron un nivel de cortisol, la hormona del estrés, que bajaba menos a lo largo del día: una señal de estrés sostenido.</t>
+        </is>
+      </c>
+      <c r="E32" s="61" t="inlineStr">
+        <is>
+          <t>Saxbe y Repetti, UCLA, Personality and Social Psychology Bulletin, 2010</t>
+        </is>
+      </c>
+      <c r="F32" s="61" t="inlineStr">
+        <is>
+          <t>Una casa no es solo paredes. Se edifica con decisiones sabias de todos los días: cómo hablamos, cómo nos organizamos, qué ponemos primero.</t>
+        </is>
+      </c>
+      <c r="G32" s="61" t="inlineStr">
+        <is>
+          <t>Casas donde nadie sabe qué le toca hacer y todo termina en discusiones.</t>
+        </is>
+      </c>
+      <c r="H32" s="61" t="inlineStr">
+        <is>
+          <t>Hoy en la cena, repartan entre todos tres tareas de la casa para esta semana. Cada uno sabe la suya.</t>
+        </is>
+      </c>
+      <c r="I32" s="61" t="inlineStr">
+        <is>
+          <t>Entender cómo funciona tu familia (horarios, cansancio, necesidades) afirma la casa. El orden se adapta a la familia real, no a la de la revista.</t>
+        </is>
+      </c>
+      <c r="J32" s="61" t="inlineStr">
+        <is>
+          <t>Reglas copiadas de otros que no encajan con la realidad de la familia y que nadie cumple.</t>
+        </is>
+      </c>
+      <c r="K32" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un momento del día que siempre es un caos (la mañana, la vuelta del trabajo) y pensá un cambio simple para ordenarlo.</t>
+        </is>
+      </c>
+      <c r="L32" s="61" t="inlineStr">
+        <is>
+          <t>Los bienes más preciados de una casa no son los muebles: son la paz, la confianza y el buen trato.</t>
+        </is>
+      </c>
+      <c r="M32" s="61" t="inlineStr">
+        <is>
+          <t>Familias que acumulan cosas pero tienen poco tiempo juntos.</t>
+        </is>
+      </c>
+      <c r="N32" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, antes de comprar algo para la casa, regalale a tu familia una hora juntos sin pantallas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B33" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C33" s="61" t="inlineStr">
+        <is>
+          <t>El orden también es amor</t>
+        </is>
+      </c>
+      <c r="D33" s="61" t="inlineStr">
+        <is>
+          <t>Personas que pasaron un rato en una habitación ordenada eligieron con más frecuencia una fruta en vez de un chocolate que las que estuvieron en una desordenada.</t>
+        </is>
+      </c>
+      <c r="E33" s="61" t="inlineStr">
+        <is>
+          <t>Vohs, Redden y Rahinel, Universidad de Minnesota, Psychological Science, 2013</t>
+        </is>
+      </c>
+      <c r="F33" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide orden para que la reunión edifique a todos. En casa pasa lo mismo: el orden hace lugar para que todos estén bien.</t>
+        </is>
+      </c>
+      <c r="G33" s="61" t="inlineStr">
+        <is>
+          <t>Llegar tarde, perder cosas, gritar por la mañana: el desorden roba paz todos los días.</t>
+        </is>
+      </c>
+      <c r="H33" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un lugar fijo para llaves, documentos y cargadores. Pocas cosas, siempre en el mismo lugar.</t>
+        </is>
+      </c>
+      <c r="I33" s="61" t="inlineStr">
+        <is>
+          <t>Cómo está la casa dice algo de cómo estamos por dentro. No hace falta lujo: hace falta cuidado.</t>
+        </is>
+      </c>
+      <c r="J33" s="61" t="inlineStr">
+        <is>
+          <t>Rincones que se llenan de cosas que nadie usa y nadie se anima a sacar.</t>
+        </is>
+      </c>
+      <c r="K33" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un cajón o un rincón y ordenalo hoy en quince minutos. Lo que no usás, regalalo.</t>
+        </is>
+      </c>
+      <c r="L33" s="61" t="inlineStr">
+        <is>
+          <t>Tener horarios y rutinas no es vivir como en un cuartel. Es darle a cada uno la seguridad de saber qué viene.</t>
+        </is>
+      </c>
+      <c r="M33" s="61" t="inlineStr">
+        <is>
+          <t>Niños sin horarios de sueño ni de comida, cansados e irritables.</t>
+        </is>
+      </c>
+      <c r="N33" s="61" t="inlineStr">
+        <is>
+          <t>Fijá una hora para ir a dormir en casa y respetala toda la semana, también los adultos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B34" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C34" s="61" t="inlineStr">
+        <is>
+          <t>Atentos a la marcha de la casa</t>
+        </is>
+      </c>
+      <c r="D34" s="61" t="inlineStr">
+        <is>
+          <t>Lavarse las manos con agua y jabón puede reducir entre un 23 y un 40 % las enfermedades diarreicas.</t>
+        </is>
+      </c>
+      <c r="E34" s="61" t="inlineStr">
+        <is>
+          <t>Centros para el Control y la Prevención de Enfermedades (CDC) de EE. UU.</t>
+        </is>
+      </c>
+      <c r="F34" s="61" t="inlineStr">
+        <is>
+          <t>La mujer de Proverbios 31 está atenta a lo que pasa en su casa. Estar atento es ver lo que hace falta antes de que sea un problema.</t>
+        </is>
+      </c>
+      <c r="G34" s="61" t="inlineStr">
+        <is>
+          <t>Arreglos pequeños de la casa (una pérdida de agua, un enchufe roto) que se dejan para después hasta que salen caros.</t>
+        </is>
+      </c>
+      <c r="H34" s="61" t="inlineStr">
+        <is>
+          <t>Recorré la casa hoy y anotá tres cosas que necesitan arreglo. Resolvé una esta semana.</t>
+        </is>
+      </c>
+      <c r="I34" s="61" t="inlineStr">
+        <is>
+          <t>En una casa todos comen; por eso todos colaboran. Nadie es huésped en su propia casa.</t>
+        </is>
+      </c>
+      <c r="J34" s="61" t="inlineStr">
+        <is>
+          <t>La carga de la limpieza que recae casi siempre en una sola persona, muchas veces la mamá.</t>
+        </is>
+      </c>
+      <c r="K34" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy una tarea de la casa que normalmente hace otro, sin que te lo pidan.</t>
+        </is>
+      </c>
+      <c r="L34" s="61" t="inlineStr">
+        <is>
+          <t>Limpiar, lavar, cocinar: son tareas que se notan sobre todo cuando no se hacen. Valorarlas es parte del amor en casa.</t>
+        </is>
+      </c>
+      <c r="M34" s="61" t="inlineStr">
+        <is>
+          <t>Tareas del hogar que nadie agradece porque se dan por hechas.</t>
+        </is>
+      </c>
+      <c r="N34" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy en voz alta a quien cocina, lava o limpia en tu casa. Con nombre y con detalle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B35" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C35" s="61" t="inlineStr">
+        <is>
+          <t>Lo que Dios edifica, permanece</t>
+        </is>
+      </c>
+      <c r="D35" s="61" t="inlineStr">
+        <is>
+          <t>En esponjas de cocina usadas se encontraron 362 tipos distintos de bacterias.</t>
+        </is>
+      </c>
+      <c r="E35" s="61" t="inlineStr">
+        <is>
+          <t>Cardinale y otros, Universidad de Furtwangen, Scientific Reports, 2017</t>
+        </is>
+      </c>
+      <c r="F35" s="61" t="inlineStr">
+        <is>
+          <t>Podemos tener la casa impecable y aun así vivir vacíos. Lo que sostiene un hogar es la presencia de Dios en el día a día.</t>
+        </is>
+      </c>
+      <c r="G35" s="61" t="inlineStr">
+        <is>
+          <t>Familias que se esfuerzan mucho en lo material y están agotadas y distantes entre sí.</t>
+        </is>
+      </c>
+      <c r="H35" s="61" t="inlineStr">
+        <is>
+          <t>Empezá o retomá un momento corto de oración en familia: cinco minutos antes de dormir.</t>
+        </is>
+      </c>
+      <c r="I35" s="61" t="inlineStr">
+        <is>
+          <t>Limpiar también puede ser una forma de servir a Dios: cuidar el lugar donde Él nos puso a vivir con otros.</t>
+        </is>
+      </c>
+      <c r="J35" s="61" t="inlineStr">
+        <is>
+          <t>La limpieza vista como castigo o como una tarea de segunda.</t>
+        </is>
+      </c>
+      <c r="K35" s="61" t="inlineStr">
+        <is>
+          <t>Hagan una limpieza corta en familia con música de fondo. Quince minutos todos juntos rinden más que una hora solo.</t>
+        </is>
+      </c>
+      <c r="L35" s="61" t="inlineStr">
+        <is>
+          <t>Hace falta trabajo y hace falta Dios. No es una cosa o la otra: trabajamos y confiamos.</t>
+        </is>
+      </c>
+      <c r="M35" s="61" t="inlineStr">
+        <is>
+          <t>Limpiar a fondo una vez al mes en vez de cuidar un poco cada día, y terminar con cansancio y peleas.</t>
+        </is>
+      </c>
+      <c r="N35" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una rutina de diez minutos diarios: los platos limpios antes de dormir y la mesa despejada. Constancia antes que maratón.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B36" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C36" s="61" t="inlineStr">
+        <is>
+          <t>Una casa sobre la roca</t>
+        </is>
+      </c>
+      <c r="D36" s="61" t="inlineStr">
+        <is>
+          <t>El estudio sobre la vida adulta más largo del mundo, que sigue a sus participantes desde 1938, concluye que las buenas relaciones nos mantienen más felices y más sanos.</t>
+        </is>
+      </c>
+      <c r="E36" s="61" t="inlineStr">
+        <is>
+          <t>Estudio de Desarrollo Adulto de Harvard (Robert Waldinger)</t>
+        </is>
+      </c>
+      <c r="F36" s="61" t="inlineStr">
+        <is>
+          <t>Las tormentas llegan a todas las casas: enfermedad, falta de trabajo, conflictos. La diferencia está en el fundamento.</t>
+        </is>
+      </c>
+      <c r="G36" s="61" t="inlineStr">
+        <is>
+          <t>Familias que se desarman ante la primera crisis porque no tenían a qué aferrarse.</t>
+        </is>
+      </c>
+      <c r="H36" s="61" t="inlineStr">
+        <is>
+          <t>Elegí con tu familia un versículo para esta etapa y pónganlo a la vista en la casa.</t>
+        </is>
+      </c>
+      <c r="I36" s="61" t="inlineStr">
+        <is>
+          <t>Jesús no habla del que solo oye, sino del que oye y pone en práctica. Las prioridades se ven en lo que hacemos, no en lo que decimos.</t>
+        </is>
+      </c>
+      <c r="J36" s="61" t="inlineStr">
+        <is>
+          <t>Decir que la familia es lo primero, pero darle solo el tiempo que sobra.</t>
+        </is>
+      </c>
+      <c r="K36" s="61" t="inlineStr">
+        <is>
+          <t>Mirá tu agenda de la semana y poné primero un tiempo para tu familia. Después acomodá lo demás.</t>
+        </is>
+      </c>
+      <c r="L36" s="61" t="inlineStr">
+        <is>
+          <t>Lo que va primero sostiene todo lo demás. Si Dios y la familia van primero, el trabajo y las cosas encuentran su lugar.</t>
+        </is>
+      </c>
+      <c r="M36" s="61" t="inlineStr">
+        <is>
+          <t>Padres que trabajan cada vez más para darles cosas a sus hijos, cuando los hijos solo piden tiempo.</t>
+        </is>
+      </c>
+      <c r="N36" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale hoy a tu hijo o a tu pareja qué les gustaría hacer juntos esta semana, y hacelo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="61" t="n">
+        <v>6</v>
+      </c>
+      <c r="B37" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C37" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: un hogar donde gobierna la paz</t>
+        </is>
+      </c>
+      <c r="D37" s="61" t="inlineStr">
+        <is>
+          <t>Comer en familia con frecuencia se asocia con una mejor alimentación y menos síntomas de depresión en niños y adolescentes.</t>
+        </is>
+      </c>
+      <c r="E37" s="61" t="inlineStr">
+        <is>
+          <t>Harrison y otros, Canadian Family Physician, 2015</t>
+        </is>
+      </c>
+      <c r="F37" s="61" t="inlineStr">
+        <is>
+          <t>El orden no es una casa perfecta: es que cada cosa y cada persona sepan dónde están, para vivir con más paz.</t>
+        </is>
+      </c>
+      <c r="G37" s="61" t="n"/>
+      <c r="H37" s="61" t="inlineStr">
+        <is>
+          <t>Compartan una comida en familia este fin de semana, sin pantallas, y agradezcan juntos por la casa que tienen.</t>
+        </is>
+      </c>
+      <c r="I37" s="61" t="inlineStr">
+        <is>
+          <t>Limpiar y cuidar la casa entre todos es una forma silenciosa de cuidar a los que la habitan.</t>
+        </is>
+      </c>
+      <c r="J37" s="61" t="n"/>
+      <c r="K37" s="61" t="n"/>
+      <c r="L37" s="61" t="inlineStr">
+        <is>
+          <t>Lo que va primero sostiene la casa: Dios y la familia antes que lo urgente.</t>
+        </is>
+      </c>
+      <c r="M37" s="61" t="n"/>
+      <c r="N37" s="61" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="B38" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C38" s="61" t="inlineStr">
+        <is>
+          <t>Lo que enseña la hormiga</t>
+        </is>
+      </c>
+      <c r="D38" s="61" t="inlineStr">
+        <is>
+          <t>En los países en desarrollo, solo un poco más de la mitad de los adultos (55 %) podría conseguir dinero para una emergencia en un mes sin mucha dificultad.</t>
+        </is>
+      </c>
+      <c r="E38" s="61" t="inlineStr">
+        <is>
+          <t>Banco Mundial, Global Findex, 2021</t>
+        </is>
+      </c>
+      <c r="F38" s="61" t="inlineStr">
+        <is>
+          <t>La hormiga no espera que alguien la obligue. Ahorrar es una decisión personal: nadie lo va a hacer por vos.</t>
+        </is>
+      </c>
+      <c r="G38" s="61" t="inlineStr">
+        <is>
+          <t>Esperar a que «sobre» para ahorrar, cuando a fin de mes nunca sobra.</t>
+        </is>
+      </c>
+      <c r="H38" s="61" t="inlineStr">
+        <is>
+          <t>Hoy mismo separá un monto pequeño, aunque sean diez mil guaraníes, y guardalo aparte.</t>
+        </is>
+      </c>
+      <c r="I38" s="61" t="inlineStr">
+        <is>
+          <t>Hay tiempos de cosecha y tiempos de escasez. Ahorrar es guardar en el tiempo bueno para el tiempo difícil.</t>
+        </is>
+      </c>
+      <c r="J38" s="61" t="inlineStr">
+        <is>
+          <t>Gastar todo el aguinaldo o la buena cosecha en pocos días y empezar el año con deudas.</t>
+        </is>
+      </c>
+      <c r="K38" s="61" t="inlineStr">
+        <is>
+          <t>Cuando recibas un ingreso extra, separá una parte antes de gastar nada.</t>
+        </is>
+      </c>
+      <c r="L38" s="61" t="inlineStr">
+        <is>
+          <t>Ahorrar no es desconfiar de Dios: es usar la sabiduría que Él mismo puso en la creación. Confiar y prepararse van juntos.</t>
+        </is>
+      </c>
+      <c r="M38" s="61" t="inlineStr">
+        <is>
+          <t>La idea de que ahorrar es falta de fe.</t>
+        </is>
+      </c>
+      <c r="N38" s="61" t="inlineStr">
+        <is>
+          <t>Orá por tus finanzas esta semana y, en la misma oración, pedí sabiduría para empezar a guardar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="B39" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C39" s="61" t="inlineStr">
+        <is>
+          <t>Guardar en los años buenos</t>
+        </is>
+      </c>
+      <c r="D39" s="61" t="inlineStr">
+        <is>
+          <t>Un enjambre de langostas del desierto de un kilómetro cuadrado puede comer en un día lo mismo que unas 35.000 personas.</t>
+        </is>
+      </c>
+      <c r="E39" s="61" t="inlineStr">
+        <is>
+          <t>Organización de las Naciones Unidas para la Alimentación y la Agricultura (FAO)</t>
+        </is>
+      </c>
+      <c r="F39" s="61" t="inlineStr">
+        <is>
+          <t>José no adivinó el futuro por su cuenta: Dios le mostró lo que venía, y él actuó con un plan.</t>
+        </is>
+      </c>
+      <c r="G39" s="61" t="inlineStr">
+        <is>
+          <t>Familias que viven al día, donde cualquier imprevisto (una enfermedad, un arreglo) se vuelve una crisis.</t>
+        </is>
+      </c>
+      <c r="H39" s="61" t="inlineStr">
+        <is>
+          <t>Anotá tres gastos imprevistos que tuviste el año pasado. Son la razón concreta para empezar tu fondo de emergencia.</t>
+        </is>
+      </c>
+      <c r="I39" s="61" t="inlineStr">
+        <is>
+          <t>El ahorro es el puente entre los años buenos y los malos. Lo que guardás hoy es la tranquilidad de mañana.</t>
+        </is>
+      </c>
+      <c r="J39" s="61" t="inlineStr">
+        <is>
+          <t>Ingresos que cambian mucho, como en el campo o en el trabajo por cuenta propia, sin un colchón para los meses flojos.</t>
+        </is>
+      </c>
+      <c r="K39" s="61" t="inlineStr">
+        <is>
+          <t>Si tu ingreso varía, pensá cuál es tu mes más flojo del año y empezá a guardar para cubrirlo.</t>
+        </is>
+      </c>
+      <c r="L39" s="61" t="inlineStr">
+        <is>
+          <t>José organizó, almacenó y administró. Sin un plan, la abundancia se va igual que llegó.</t>
+        </is>
+      </c>
+      <c r="M39" s="61" t="inlineStr">
+        <is>
+          <t>Compras en cuotas que se suman sin darse cuenta hasta comerse el sueldo.</t>
+        </is>
+      </c>
+      <c r="N39" s="61" t="inlineStr">
+        <is>
+          <t>Antes de sacar algo nuevo en cuotas, sumá todas las cuotas que ya pagás por mes y mirá cuánto se llevan de tu ingreso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="B40" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C40" s="61" t="inlineStr">
+        <is>
+          <t>De a poco se llega lejos</t>
+        </is>
+      </c>
+      <c r="D40" s="61" t="inlineStr">
+        <is>
+          <t>Guardar 50.000 guaraníes por semana, sin sumar intereses, da 2.600.000 en un año y 26 millones en diez años.</t>
+        </is>
+      </c>
+      <c r="E40" s="61" t="inlineStr">
+        <is>
+          <t>Cálculo simple</t>
+        </is>
+      </c>
+      <c r="F40" s="61" t="inlineStr">
+        <is>
+          <t>El que trabaja y guarda hace crecer lo que tiene. No hace falta ganar mucho para empezar a ahorrar.</t>
+        </is>
+      </c>
+      <c r="G40" s="61" t="inlineStr">
+        <is>
+          <t>Pensar «gano muy poco, no puedo ahorrar» y nunca empezar.</t>
+        </is>
+      </c>
+      <c r="H40" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un monto que puedas guardar todas las semanas sin falta, aunque sea pequeño. La constancia importa más que el monto.</t>
+        </is>
+      </c>
+      <c r="I40" s="61" t="inlineStr">
+        <is>
+          <t>Lo que llega fácil, se va fácil. Las promesas de ganancia rápida casi siempre terminan en pérdida.</t>
+        </is>
+      </c>
+      <c r="J40" s="61" t="inlineStr">
+        <is>
+          <t>Cadenas y esquemas que prometen multiplicar el dinero en poco tiempo y dejan a muchos sin nada.</t>
+        </is>
+      </c>
+      <c r="K40" s="61" t="inlineStr">
+        <is>
+          <t>Antes de poner tu plata en algo que promete mucho en poco tiempo, consultalo con alguien de confianza que sepa del tema.</t>
+        </is>
+      </c>
+      <c r="L40" s="61" t="inlineStr">
+        <is>
+          <t>El patrimonio se construye como una pared: ladrillo a ladrillo. Cada guaraní guardado cuenta.</t>
+        </is>
+      </c>
+      <c r="M40" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar el ahorro el primer mes difícil.</t>
+        </is>
+      </c>
+      <c r="N40" s="61" t="inlineStr">
+        <is>
+          <t>Si un mes no podés guardar lo que pensaste, guardá menos, pero no dejes de guardar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="B41" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C41" s="61" t="inlineStr">
+        <is>
+          <t>No pongas todo en un mismo lugar</t>
+        </is>
+      </c>
+      <c r="D41" s="61" t="inlineStr">
+        <is>
+          <t>Harry Markowitz recibió el Premio Nobel de Economía en 1990, en parte por mostrar con números que repartir el dinero en distintos lugares reduce el riesgo.</t>
+        </is>
+      </c>
+      <c r="E41" s="61" t="inlineStr">
+        <is>
+          <t>Fundación Nobel, 1990</t>
+        </is>
+      </c>
+      <c r="F41" s="61" t="inlineStr">
+        <is>
+          <t>Salomón aconseja dividir: no poner todo en una sola cosa, porque no sabemos qué puede pasar.</t>
+        </is>
+      </c>
+      <c r="G41" s="61" t="inlineStr">
+        <is>
+          <t>Tener todos los ahorros en efectivo en la casa, expuestos a robos o pérdidas.</t>
+        </is>
+      </c>
+      <c r="H41" s="61" t="inlineStr">
+        <is>
+          <t>Si guardás tus ahorros en casa, averiguá esta semana cómo abrir una cuenta de ahorro en una cooperativa o un banco.</t>
+        </is>
+      </c>
+      <c r="I41" s="61" t="inlineStr">
+        <is>
+          <t>Repartir el ahorro según para qué es (emergencias, metas, futuro) ayuda a no tocarlo todo ante el primer problema.</t>
+        </is>
+      </c>
+      <c r="J41" s="61" t="inlineStr">
+        <is>
+          <t>Usar el único ahorro para cualquier gasto y quedarse sin nada para una emergencia real.</t>
+        </is>
+      </c>
+      <c r="K41" s="61" t="inlineStr">
+        <is>
+          <t>Dividí tu ahorro en dos sobres o dos cuentas: uno para emergencias y otro para una meta concreta.</t>
+        </is>
+      </c>
+      <c r="L41" s="61" t="inlineStr">
+        <is>
+          <t>Cuánto ahorrar no tiene un número mágico: depende de cada familia. Lo sabio es empezar con lo que se puede y repartirlo bien.</t>
+        </is>
+      </c>
+      <c r="M41" s="61" t="inlineStr">
+        <is>
+          <t>Compararse con otros y desanimarse porque ellos ahorran más.</t>
+        </is>
+      </c>
+      <c r="N41" s="61" t="inlineStr">
+        <is>
+          <t>Fijá tu propio monto según tu realidad y revisalo cada tres meses para ver si podés subirlo un poco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="B42" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C42" s="61" t="inlineStr">
+        <is>
+          <t>Conocé el estado de tus ovejas</t>
+        </is>
+      </c>
+      <c r="D42" s="61" t="inlineStr">
+        <is>
+          <t>Muchas personas revisan menos sus cuentas justo cuando las cosas van mal; los investigadores lo llamaron «efecto avestruz».</t>
+        </is>
+      </c>
+      <c r="E42" s="61" t="inlineStr">
+        <is>
+          <t>Karlsson, Loewenstein y Seppi, Journal of Risk and Uncertainty, 2009</t>
+        </is>
+      </c>
+      <c r="F42" s="61" t="inlineStr">
+        <is>
+          <t>El pastor conoce a cada oveja. Para ahorrar, primero hay que saber cuánto entra y cuánto sale.</t>
+        </is>
+      </c>
+      <c r="G42" s="61" t="inlineStr">
+        <is>
+          <t>No saber en qué se va la plata: los pequeños gastos diarios que se suman sin que nadie los anote.</t>
+        </is>
+      </c>
+      <c r="H42" s="61" t="inlineStr">
+        <is>
+          <t>Durante esta semana anotá todo lo que gastás, aunque sea un chipá. Al final vas a ver dónde se te va.</t>
+        </is>
+      </c>
+      <c r="I42" s="61" t="inlineStr">
+        <is>
+          <t>Lo que hoy tenés puede no estar mañana. Por eso el ahorro se separa apenas llega el ingreso, no con lo que sobra.</t>
+        </is>
+      </c>
+      <c r="J42" s="61" t="inlineStr">
+        <is>
+          <t>Ahorrar «lo que sobra» a fin de mes, cuando casi nunca sobra nada.</t>
+        </is>
+      </c>
+      <c r="K42" s="61" t="inlineStr">
+        <is>
+          <t>Pagate primero: el día que cobrás, separá tu ahorro antes de pagar cualquier otra cosa.</t>
+        </is>
+      </c>
+      <c r="L42" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar las finanzas no es una tarea de una sola vez: es el hábito de mirar, ajustar y seguir.</t>
+        </is>
+      </c>
+      <c r="M42" s="61" t="inlineStr">
+        <is>
+          <t>Evitar mirar las cuentas cuando las cosas van mal, y dejar que el problema crezca.</t>
+        </is>
+      </c>
+      <c r="N42" s="61" t="inlineStr">
+        <is>
+          <t>Fijá un día al mes para revisar las cuentas con tu familia, con un tereré y sin pelear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="61" t="n">
+        <v>7</v>
+      </c>
+      <c r="B43" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C43" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: ahorrar es prepararse</t>
+        </is>
+      </c>
+      <c r="D43" s="61" t="inlineStr">
+        <is>
+          <t>La Torre de Pisa empezó a inclinarse en 1178, cuando iban por el segundo piso, por un suelo blando que no se había estudiado bien. Terminarla llevó casi 200 años.</t>
+        </is>
+      </c>
+      <c r="E43" s="61" t="inlineStr">
+        <is>
+          <t>Opera della Primaziale Pisana, Italia</t>
+        </is>
+      </c>
+      <c r="F43" s="61" t="inlineStr">
+        <is>
+          <t>Ahorrar no es falta de fe: es la sabiduría de la hormiga y de José, que se preparan en el tiempo bueno.</t>
+        </is>
+      </c>
+      <c r="G43" s="61" t="n"/>
+      <c r="H43" s="61" t="inlineStr">
+        <is>
+          <t>Abrí esta semana un sobre o una cuenta de ahorro y poné ahí tu primer aporte, aunque sea pequeño.</t>
+        </is>
+      </c>
+      <c r="I43" s="61" t="inlineStr">
+        <is>
+          <t>No hay un número mágico: lo importante es empezar con lo que se puede y ser constante.</t>
+        </is>
+      </c>
+      <c r="J43" s="61" t="n"/>
+      <c r="K43" s="61" t="n"/>
+      <c r="L43" s="61" t="inlineStr">
+        <is>
+          <t>El ahorro se separa apenas llega el ingreso, no con lo que sobra al final del mes.</t>
+        </is>
+      </c>
+      <c r="M43" s="61" t="n"/>
+      <c r="N43" s="61" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="B44" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C44" s="61" t="inlineStr">
+        <is>
+          <t>Decir lo que de verdad sentís</t>
+        </is>
+      </c>
+      <c r="D44" s="61" t="inlineStr">
+        <is>
+          <t>Ponerle nombre a una emoción, con una sola palabra, reduce la actividad de la amígdala, la zona del cerebro que dispara la alarma.</t>
+        </is>
+      </c>
+      <c r="E44" s="61" t="inlineStr">
+        <is>
+          <t>Lieberman y otros, UCLA, Psychological Science, 2007</t>
+        </is>
+      </c>
+      <c r="F44" s="61" t="inlineStr">
+        <is>
+          <t>Jesús pide un «sí» que sea sí y un «no» que sea no. Esa honestidad empieza por dentro: reconocer lo que de verdad sentimos.</t>
+        </is>
+      </c>
+      <c r="G44" s="61" t="inlineStr">
+        <is>
+          <t>Responder «todo bien» cuando no está todo bien, por costumbre o por vergüenza.</t>
+        </is>
+      </c>
+      <c r="H44" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, cuando alguien de confianza te pregunte cómo estás, respondé con la verdad, aunque sea en una frase.</t>
+        </is>
+      </c>
+      <c r="I44" s="61" t="inlineStr">
+        <is>
+          <t>Muchas veces decimos «sí» por presión y después cargamos enojo y cansancio. Un «no» honesto a tiempo cuida el alma y las relaciones.</t>
+        </is>
+      </c>
+      <c r="J44" s="61" t="inlineStr">
+        <is>
+          <t>Personas que no saben decir que no y terminan agotadas y resentidas.</t>
+        </is>
+      </c>
+      <c r="K44" s="61" t="inlineStr">
+        <is>
+          <t>Antes de aceptar un compromiso nuevo esta semana, tomate un momento y preguntate si de verdad podés.</t>
+        </is>
+      </c>
+      <c r="L44" s="61" t="inlineStr">
+        <is>
+          <t>Ponerle nombre a lo que sentís ayuda a decidir mejor. La tristeza, el miedo o el enojo con nombre se manejan; sin nombre, nos manejan.</t>
+        </is>
+      </c>
+      <c r="M44" s="61" t="inlineStr">
+        <is>
+          <t>Decisiones importantes tomadas en un momento de enojo o de miedo que nadie reconoció.</t>
+        </is>
+      </c>
+      <c r="N44" s="61" t="inlineStr">
+        <is>
+          <t>Cuando tengas que decidir algo, completá esta frase: «Ahora me siento…». Si es enojo o miedo, esperá antes de decidir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="B45" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C45" s="61" t="inlineStr">
+        <is>
+          <t>Una mente que se renueva</t>
+        </is>
+      </c>
+      <c r="D45" s="61" t="inlineStr">
+        <is>
+          <t>Los taxistas de Londres, que memorizan miles de calles, tienen más desarrollada una parte del hipocampo, la zona del cerebro ligada a la memoria espacial.</t>
+        </is>
+      </c>
+      <c r="E45" s="61" t="inlineStr">
+        <is>
+          <t>Maguire y otros, University College London, PNAS, 2000</t>
+        </is>
+      </c>
+      <c r="F45" s="61" t="inlineStr">
+        <is>
+          <t>Pablo dice que el cambio viene por la renovación de la mente. Lo que pensamos una y otra vez va formando lo que sentimos.</t>
+        </is>
+      </c>
+      <c r="G45" s="61" t="inlineStr">
+        <is>
+          <t>Pensamientos negativos repetidos («no sirvo», «nada me sale») que nadie cuestiona.</t>
+        </is>
+      </c>
+      <c r="H45" s="61" t="inlineStr">
+        <is>
+          <t>Cuando aparezca un pensamiento así, escribilo y, al lado, escribí lo que Dios dice de vos.</t>
+        </is>
+      </c>
+      <c r="I45" s="61" t="inlineStr">
+        <is>
+          <t>El mundo nos enseña a esconder lo que sentimos o a dejarnos llevar por todo. Dios propone otro camino: reconocerlo y llevarlo a Él.</t>
+        </is>
+      </c>
+      <c r="J45" s="61" t="inlineStr">
+        <is>
+          <t>La idea de que los hombres no lloran o de que mostrar tristeza es debilidad.</t>
+        </is>
+      </c>
+      <c r="K45" s="61" t="inlineStr">
+        <is>
+          <t>Si sos padre o madre, ayudá a tus hijos a ponerle nombre a lo que sienten: «¿Estás triste, enojado o con miedo?».</t>
+        </is>
+      </c>
+      <c r="L45" s="61" t="inlineStr">
+        <is>
+          <t>La mente puede aprender caminos nuevos a cualquier edad. Lo que practicás cada día se fortalece.</t>
+        </is>
+      </c>
+      <c r="M45" s="61" t="inlineStr">
+        <is>
+          <t>Creer que «yo soy así» y que no se puede cambiar.</t>
+        </is>
+      </c>
+      <c r="N45" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un versículo para esta semana y repetilo cada vez que sientas ansiedad o desánimo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="B46" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C46" s="61" t="inlineStr">
+        <is>
+          <t>Lo primero que tu mente necesita escuchar</t>
+        </is>
+      </c>
+      <c r="D46" s="61" t="inlineStr">
+        <is>
+          <t>Estudiantes que limitaron las redes sociales a 30 minutos por día durante tres semanas se sintieron menos solos y menos deprimidos.</t>
+        </is>
+      </c>
+      <c r="E46" s="61" t="inlineStr">
+        <is>
+          <t>Hunt y otros, Universidad de Pensilvania, Journal of Social and Clinical Psychology, 2018</t>
+        </is>
+      </c>
+      <c r="F46" s="61" t="inlineStr">
+        <is>
+          <t>Entre tantas voces que escuchamos cada día, hay una verdad que debería sonar más fuerte: Dios te ama, así como sos.</t>
+        </is>
+      </c>
+      <c r="G46" s="61" t="inlineStr">
+        <is>
+          <t>Comparaciones constantes en las redes que hacen sentir que nunca alcanza.</t>
+        </is>
+      </c>
+      <c r="H46" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, antes de abrir las redes, leé Juan 3:16 en voz alta y poné tu nombre donde dice «el mundo».</t>
+        </is>
+      </c>
+      <c r="I46" s="61" t="inlineStr">
+        <is>
+          <t>El amor de Dios no fue de palabras: dio lo más valioso. Llenar la mente de esa verdad cambia cómo nos vemos.</t>
+        </is>
+      </c>
+      <c r="J46" s="61" t="inlineStr">
+        <is>
+          <t>Contenidos que enseñan que el valor de una persona depende de lo que tiene o de cuántos «me gusta» recibe.</t>
+        </is>
+      </c>
+      <c r="K46" s="61" t="inlineStr">
+        <is>
+          <t>Dejá de seguir tres cuentas que te hacen sentir menos y seguí una que te edifique.</t>
+        </is>
+      </c>
+      <c r="L46" s="61" t="inlineStr">
+        <is>
+          <t>La fe nace de lo que escuchamos. Si lo que más escuchamos es miedo y queja, la fe se achica.</t>
+        </is>
+      </c>
+      <c r="M46" s="61" t="inlineStr">
+        <is>
+          <t>Horas frente al celular antes de dormir, que dejan la mente cargada y el sueño liviano.</t>
+        </is>
+      </c>
+      <c r="N46" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, la última media hora del día sin pantallas: una lectura, una oración o una charla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="B47" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C47" s="61" t="inlineStr">
+        <is>
+          <t>El miedo no es tu identidad</t>
+        </is>
+      </c>
+      <c r="D47" s="61" t="inlineStr">
+        <is>
+          <t>Después del atentado de Boston de 2013, quienes vieron seis horas o más de noticias por día sobre el hecho mostraron más estrés agudo que algunas personas que estuvieron en el lugar.</t>
+        </is>
+      </c>
+      <c r="E47" s="61" t="inlineStr">
+        <is>
+          <t>Holman, Garfin y Silver, Universidad de California en Irvine, PNAS, 2014</t>
+        </is>
+      </c>
+      <c r="F47" s="61" t="inlineStr">
+        <is>
+          <t>Pablo le recuerda a Timoteo que el miedo que paraliza no es lo que Dios nos dio. Mucho de ese miedo entra por lo que consumimos.</t>
+        </is>
+      </c>
+      <c r="G47" s="61" t="inlineStr">
+        <is>
+          <t>Noticias y videos de violencia vistos una y otra vez, que dejan miedo y desconfianza en todo.</t>
+        </is>
+      </c>
+      <c r="H47" s="61" t="inlineStr">
+        <is>
+          <t>Informate una o dos veces por día, en un horario fijo, y no sigas mirando lo mismo durante horas.</t>
+        </is>
+      </c>
+      <c r="I47" s="61" t="inlineStr">
+        <is>
+          <t>Dominio propio también es decidir qué entra en tu mente. No todo lo que aparece en la pantalla merece tu atención.</t>
+        </is>
+      </c>
+      <c r="J47" s="61" t="inlineStr">
+        <is>
+          <t>Abrir el celular sin un propósito y salir una hora después más cansado.</t>
+        </is>
+      </c>
+      <c r="K47" s="61" t="inlineStr">
+        <is>
+          <t>Desactivá las notificaciones que no necesitás y elegí vos cuándo mirar el teléfono.</t>
+        </is>
+      </c>
+      <c r="L47" s="61" t="inlineStr">
+        <is>
+          <t>Sos hijo de Dios, no esclavo del miedo. Cuidar tu mente es cuidar esa identidad.</t>
+        </is>
+      </c>
+      <c r="M47" s="61" t="inlineStr">
+        <is>
+          <t>La ansiedad que crece en silencio, sobre todo en los jóvenes, con miedo a todo lo que puede pasar.</t>
+        </is>
+      </c>
+      <c r="N47" s="61" t="inlineStr">
+        <is>
+          <t>Cuando aparezca el miedo, ponele nombre, respirá hondo tres veces y decí: «Dios no me dio un espíritu de cobardía».</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="B48" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C48" s="61" t="inlineStr">
+        <is>
+          <t>Pedir ayuda también es sabiduría</t>
+        </is>
+      </c>
+      <c r="D48" s="61" t="inlineStr">
+        <is>
+          <t>Se estima que unos 280 millones de personas en el mundo viven con depresión.</t>
+        </is>
+      </c>
+      <c r="E48" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud</t>
+        </is>
+      </c>
+      <c r="F48" s="61" t="inlineStr">
+        <is>
+          <t>Pensar en lo bueno no es negar lo que duele. A veces lo verdadero es reconocer que solo no podés.</t>
+        </is>
+      </c>
+      <c r="G48" s="61" t="inlineStr">
+        <is>
+          <t>Personas que cargan tristeza durante meses sin contarle a nadie.</t>
+        </is>
+      </c>
+      <c r="H48" s="61" t="inlineStr">
+        <is>
+          <t>Si algo te pesa hace tiempo, contáselo hoy a una persona de confianza.</t>
+        </is>
+      </c>
+      <c r="I48" s="61" t="inlineStr">
+        <is>
+          <t>Hay pensamientos que se vuelven un pozo del que cuesta salir solo. Buscar ayuda de un pastor, un consejero o un profesional es un acto de sabiduría.</t>
+        </is>
+      </c>
+      <c r="J48" s="61" t="inlineStr">
+        <is>
+          <t>La vergüenza de ir al psicólogo, como si fuera solo para «locos» o para gente sin fe.</t>
+        </is>
+      </c>
+      <c r="K48" s="61" t="inlineStr">
+        <is>
+          <t>Si la tristeza o la ansiedad no se van, consultá en tu unidad de salud familiar o con un profesional. Pedir ayuda no es falta de fe.</t>
+        </is>
+      </c>
+      <c r="L48" s="61" t="inlineStr">
+        <is>
+          <t>Somos responsables de cuidar lo que pensamos, y también de cuidar a los que tenemos cerca.</t>
+        </is>
+      </c>
+      <c r="M48" s="61" t="inlineStr">
+        <is>
+          <t>Amigos o familiares que dan señales de estar mal, y nadie les pregunta.</t>
+        </is>
+      </c>
+      <c r="N48" s="61" t="inlineStr">
+        <is>
+          <t>Escribile hoy a alguien que no está pasando un buen momento: «¿Cómo estás de verdad?». Y escuchá.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="61" t="n">
+        <v>8</v>
+      </c>
+      <c r="B49" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: cuidar el alma</t>
+        </is>
+      </c>
+      <c r="D49" s="61" t="inlineStr">
+        <is>
+          <t>Escribir sobre lo que nos preocupa o nos dolió, entre 15 y 20 minutos durante unos pocos días seguidos, se asoció con mejor salud en los meses siguientes.</t>
+        </is>
+      </c>
+      <c r="E49" s="61" t="inlineStr">
+        <is>
+          <t>Pennebaker y Beall, Journal of Abnormal Psychology, 1986</t>
+        </is>
+      </c>
+      <c r="F49" s="61" t="inlineStr">
+        <is>
+          <t>Ponerle nombre a lo que sentís es el primer paso para manejarlo con sabiduría y llevarlo a Dios.</t>
+        </is>
+      </c>
+      <c r="G49" s="61" t="n"/>
+      <c r="H49" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, escribí cada noche en pocas líneas qué sentiste en el día y llevalo a Dios en oración.</t>
+        </is>
+      </c>
+      <c r="I49" s="61" t="inlineStr">
+        <is>
+          <t>Lo que consumís cada día moldea tu mente: elegí con intención qué ves, qué escuchás y qué leés.</t>
+        </is>
+      </c>
+      <c r="J49" s="61" t="n"/>
+      <c r="K49" s="61" t="n"/>
+      <c r="L49" s="61" t="inlineStr">
+        <is>
+          <t>Pedir ayuda no es debilidad: Dios está cerca del que sufre y también usa a otras personas para sostenernos.</t>
+        </is>
+      </c>
+      <c r="M49" s="61" t="n"/>
+      <c r="N49" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: revisión teológica de enero y febrero, y criterios para los próximos meses
- 39 campos de guion y 4 puntos corregidos (contexto de cada versículo,
  sin prosperidad ni retribución, gracia antes que mérito, salud mental),
  con el motivo de cada cambio en tools/revision_teologica_ene_feb_2027.py
  y el informe antes/después en content/revision_teologica_2027.md
- content/criterios_teologicos.md: proceso mensual, hermenéutica,
  errores teológicos, falacias y datos
- Alarma automática de frases de riesgo en content/revision_planilla.txt
- «Copiar prompt» con los mismos criterios
- Puntos con «*» o «1,» normalizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -1110,7 +1110,7 @@
       </c>
       <c r="AC2" s="21" t="inlineStr">
         <is>
-          <t>• Dios desea prosperidad y salud
+          <t>• Juan desea a su hermano bienestar y salud
 • El bienestar integral le importa a Dios
 • No es solo espiritual, también físico</t>
         </is>
@@ -1305,7 +1305,7 @@
         <is>
           <t>• Se cosecha lo que se siembra
 • La ley de la siembra es universal
-• No hay atajos en el trabajo de la tierra</t>
+• Dios no puede ser burlado</t>
         </is>
       </c>
       <c r="AB3" s="25" t="inlineStr">
@@ -1735,7 +1735,7 @@
         <is>
           <t>• Meditar la Palabra día y noche
 • Guardar y hacer lo que dice
-• Trae éxito verdadero y prosperidad</t>
+• El verdadero éxito es andar en el camino de Dios</t>
         </is>
       </c>
       <c r="AD5" s="32" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="AG9" s="43" t="inlineStr">
         <is>
-          <t>• El temor no viene de Dios
+          <t>• La cobardía no viene de Dios
 • Poder, amor y dominio propio sí vienen de Él
 • El miedo paralizante no es la identidad dada por Dios</t>
         </is>
@@ -2928,9 +2928,9 @@
       </c>
       <c r="Y11" s="49" t="inlineStr">
         <is>
-          <t>1, Entregar nuestras angustias a Dios.
-2, Confiar en su cuidado.
-3, Descansar en Él.</t>
+          <t>• Entregar nuestras angustias a Dios.
+• Confiar en su cuidado.
+• Descansar en Él.</t>
         </is>
       </c>
       <c r="Z11" s="49" t="inlineStr">
@@ -3787,9 +3787,9 @@
       </c>
       <c r="AE15" s="40" t="inlineStr">
         <is>
-          <t>1, Ser prudentes.
-2, Ser sencillos.
-3, Cumplir nuestra misión.</t>
+          <t>• Ser prudentes.
+• Ser sencillos.
+• Cumplir nuestra misión.</t>
         </is>
       </c>
       <c r="AF15" s="40" t="inlineStr">
@@ -4367,9 +4367,9 @@
       </c>
       <c r="Y18" s="49" t="inlineStr">
         <is>
-          <t>* No basta con desear: Los sueños necesitan acción y compromiso.
-* El esfuerzo trae resultados: El que trabaja con dedicación puede alcanzar buenos frutos.
-* Dios bendice la perseverancia: La constancia y la responsabilidad abren camino al progreso.</t>
+          <t>• No basta con desear: Los sueños necesitan acción y compromiso.
+• El esfuerzo trae resultados: El que trabaja con dedicación puede alcanzar buenos frutos.
+• Dios bendice la perseverancia: La constancia y la responsabilidad abren camino al progreso.</t>
         </is>
       </c>
       <c r="Z18" s="49" t="inlineStr">
@@ -7866,9 +7866,9 @@
       </c>
       <c r="AC35" s="12" t="inlineStr">
         <is>
-          <t>1, Habrá un día de juicio.
-2, Dios hará justicia.
-3, Vivir preparados delante de Dios.</t>
+          <t>• Habrá un día de juicio.
+• Dios hará justicia.
+• Vivir preparados delante de Dios.</t>
         </is>
       </c>
       <c r="AD35" s="12" t="inlineStr">
@@ -8449,9 +8449,9 @@
       </c>
       <c r="Y38" s="4" t="inlineStr">
         <is>
-          <t>1, Revestirse de amor.
-2, Mantener la unidad.
-3, Vivir en armonía.</t>
+          <t>• Revestirse de amor.
+• Mantener la unidad.
+• Vivir en armonía.</t>
         </is>
       </c>
       <c r="Z38" s="4" t="inlineStr">
@@ -10165,9 +10165,9 @@
       </c>
       <c r="AK46" s="6" t="inlineStr">
         <is>
-          <t>1, Invocar a Dios en la angustia.
-2, Confiar en su liberación.
-3, Honrar a Dios por su respuesta.</t>
+          <t>• Invocar a Dios en la angustia.
+• Confiar en su liberación.
+• Honrar a Dios por su respuesta.</t>
         </is>
       </c>
     </row>
@@ -19333,7 +19333,7 @@
       </c>
       <c r="F2" s="61" t="inlineStr">
         <is>
-          <t>Presentar el cuerpo es ponerlo al servicio de algo más grande que la imagen o el rendimiento: cuidarlo para amar, trabajar y servir mejor.</t>
+          <t>Pablo pide presentar todo nuestro ser, cuerpo incluido, como respuesta a la misericordia de Dios: no para ganar su amor, sino porque ya lo recibimos. Cuidar el cuerpo es parte de esa ofrenda, para amar, trabajar y servir mejor.</t>
         </is>
       </c>
       <c r="G2" s="61" t="inlineStr">
@@ -19403,7 +19403,7 @@
       </c>
       <c r="F3" s="61" t="inlineStr">
         <is>
-          <t>A Dios no le es indiferente tu salud. Desear el bien de alguien incluye desear que su cuerpo esté bien.</t>
+          <t>Juan le escribe a su amigo Gayo y le desea salud y que todo le vaya bien. Es un saludo de cariño, no una promesa de que al creyente nunca le faltarán salud ni dinero. Nos enseña que desear el bien del otro incluye su cuerpo.</t>
         </is>
       </c>
       <c r="G3" s="61" t="inlineStr">
@@ -19613,7 +19613,7 @@
       </c>
       <c r="F6" s="61" t="inlineStr">
         <is>
-          <t>Si Dios mismo descansó, descansar no es pereza. Es parte de una vida bien ordenada.</t>
+          <t>Dios no se cansa (Isaías 40:28): su reposo fue terminar la obra y bendecirla, y nos dejó ese ritmo como regalo (Éxodo 20:11). Descansar no es pereza: es parte de una vida bien ordenada.</t>
         </is>
       </c>
       <c r="G6" s="61" t="inlineStr">
@@ -19733,7 +19733,7 @@
       </c>
       <c r="F8" s="61" t="inlineStr">
         <is>
-          <t>Nadie espera cosechar maíz si sembró poroto. Lo que hacemos hoy con el tiempo, las palabras y el dinero es la semilla de mañana.</t>
+          <t>Pablo habla de sembrar para la carne o para el Espíritu (Gálatas 6:8): nuestras decisiones tienen consecuencias. Lo que hacemos hoy con el tiempo, las palabras y el dinero es la semilla de mañana.</t>
         </is>
       </c>
       <c r="G8" s="61" t="inlineStr">
@@ -19748,7 +19748,7 @@
       </c>
       <c r="I8" s="61" t="inlineStr">
         <is>
-          <t>La ley de la siembra vale en el campo, en la familia, en la salud y en la fe. Los valores son la mejor semilla.</t>
+          <t>La siembra y la cosecha valen en la familia, en la salud y en la fe. Pero no es una cuenta automática: no toda dificultad es castigo por algo que hicimos (Juan 9:3). Los valores son la mejor semilla.</t>
         </is>
       </c>
       <c r="J8" s="61" t="inlineStr">
@@ -19763,7 +19763,7 @@
       </c>
       <c r="L8" s="61" t="inlineStr">
         <is>
-          <t>En el campo los atajos se pagan caro: lo que se hace mal para ganar tiempo vuelve como pérdida.</t>
+          <t>«Dios no puede ser burlado»: podemos engañar a otros por un tiempo, pero no a Dios. Lo que se hace mal para ganar tiempo, sobre todo si daña al prójimo, vuelve como pérdida.</t>
         </is>
       </c>
       <c r="M8" s="61" t="inlineStr">
@@ -19803,7 +19803,7 @@
       </c>
       <c r="F9" s="61" t="inlineStr">
         <is>
-          <t>La semilla crece aunque no la veamos. Hay procesos que no se pueden apurar: la confianza, el carácter, un emprendimiento.</t>
+          <t>Jesús habla del reino de Dios: crece por el poder de Dios, aunque no lo veamos. De esa paciencia aprendemos también en otros procesos que no se pueden apurar: la confianza, el carácter, un proyecto.</t>
         </is>
       </c>
       <c r="G9" s="61" t="inlineStr">
@@ -19833,7 +19833,7 @@
       </c>
       <c r="L9" s="61" t="inlineStr">
         <is>
-          <t>Confiar no es quedarse quieto: el agricultor confía y mientras tanto prepara, limpia y repara.</t>
+          <t>En la parábola el sembrador duerme y la semilla igual crece: el crecimiento lo da Dios. Eso no nos vuelve pasivos (él siembra y cosecha), pero nos libra de la ansiedad de controlarlo todo.</t>
         </is>
       </c>
       <c r="M9" s="61" t="inlineStr">
@@ -19903,7 +19903,7 @@
       </c>
       <c r="L10" s="61" t="inlineStr">
         <is>
-          <t>Dios bendice el trabajo, no la improvisación. El esfuerzo ordenado rinde más.</t>
+          <t>Dios da el crecimiento y nos llama a trabajar con orden y responsabilidad. El esfuerzo ordenado es buena mayordomía de lo que Él provee.</t>
         </is>
       </c>
       <c r="M10" s="61" t="inlineStr">
@@ -19943,7 +19943,7 @@
       </c>
       <c r="F11" s="61" t="inlineStr">
         <is>
-          <t>Esperar con paciencia no es resignarse: es prepararse para lo que no se controla.</t>
+          <t>Santiago anima a esperar con paciencia la venida del Señor, en medio de injusticias (5:1-6), y pone como ejemplo al labrador. Esperar con paciencia no es resignarse: es seguir firmes y prepararse para lo que no controlamos.</t>
         </is>
       </c>
       <c r="G11" s="61" t="inlineStr">
@@ -20003,57 +20003,57 @@
       </c>
       <c r="D12" s="61" t="inlineStr">
         <is>
-          <t>Un tercio de los suelos del planeta están moderada o altamente degradados.</t>
+          <t>Unos 3.100 millones de personas en el mundo no pueden pagar una alimentación saludable.</t>
         </is>
       </c>
       <c r="E12" s="61" t="inlineStr">
         <is>
-          <t>FAO, Estado de los recursos de suelos del mundo, 2015</t>
+          <t>FAO, El estado de la seguridad alimentaria y la nutrición en el mundo, 2023</t>
         </is>
       </c>
       <c r="F12" s="61" t="inlineStr">
         <is>
-          <t>Quien siembra con generosidad cosecha con abundancia. Eso vale también para cómo tratamos la tierra que nos alimenta.</t>
+          <t>Pablo habla de la ofrenda para hermanos necesitados: dar con generosidad es sembrar. La cosecha no es una ganancia asegurada, sino frutos de justicia y gratitud a Dios (2 Corintios 9:10-11).</t>
         </is>
       </c>
       <c r="G12" s="61" t="inlineStr">
         <is>
-          <t>La quema de campos y la deforestación, que empobrecen la tierra y afectan la salud de todos.</t>
+          <t>La idea de «dar para recibir más plata», que convierte la generosidad en un negocio.</t>
         </is>
       </c>
       <c r="H12" s="61" t="inlineStr">
         <is>
-          <t>Nunca quemes basura ni pastizales. Si ves una quema peligrosa, avisá a los bomberos o a la municipalidad.</t>
+          <t>Esta semana ayudá a alguien que lo necesita, sin esperar nada a cambio.</t>
         </is>
       </c>
       <c r="I12" s="61" t="inlineStr">
         <is>
-          <t>Si no invertimos en cuidar el suelo y el agua, mañana cosechamos poco.</t>
+          <t>El que guarda todo por miedo se pierde la alegría de compartir y de ver a Dios obrar a través de lo que da. Sembrar también es pensar en los que vienen detrás.</t>
         </is>
       </c>
       <c r="J12" s="61" t="inlineStr">
         <is>
-          <t>Arroyos contaminados con basura y agroquímicos cerca de las comunidades.</t>
+          <t>Vecinos y productores que no se ayudan en los tiempos difíciles, cuando una mano a tiempo cambia todo.</t>
         </is>
       </c>
       <c r="K12" s="61" t="inlineStr">
         <is>
-          <t>Organizá con tus vecinos una limpieza del arroyo o la plaza del barrio. Una mañana de trabajo cambia el paisaje.</t>
+          <t>Si tu cosecha o tu trabajo rindió, compartí una parte con una familia que pasa necesidad.</t>
         </is>
       </c>
       <c r="L12" s="61" t="inlineStr">
         <is>
-          <t>La actitud al sembrar importa: trabajar de buena gana cambia el resultado y el ánimo.</t>
+          <t>Pablo agrega que cada uno dé lo que decidió en su corazón, no con tristeza ni por obligación, porque Dios ama al que da con alegría (9:7).</t>
         </is>
       </c>
       <c r="M12" s="61" t="inlineStr">
         <is>
-          <t>El desgaste de quienes sienten que su trabajo no vale nada.</t>
+          <t>Dar por presión, por quedar bien o por culpa.</t>
         </is>
       </c>
       <c r="N12" s="61" t="inlineStr">
         <is>
-          <t>Hoy agradecé a alguien por su trabajo: al que te vende verduras, al que maneja el colectivo, al que limpia tu calle.</t>
+          <t>Antes de dar, orá y decidí en tu corazón cuánto y a quién. Después, dalo con alegría.</t>
         </is>
       </c>
     </row>
@@ -20148,7 +20148,7 @@
       </c>
       <c r="I14" s="61" t="inlineStr">
         <is>
-          <t>Escuchar y seguir buenas instrucciones protege: higiene, vacunas, cuidados básicos.</t>
+          <t>Esta promesa fue parte del pacto de Dios con Israel en el desierto, y muchas de sus leyes cuidaban la salud del pueblo. No significa que quien se enferma está en pecado: Jesús lo aclaró (Juan 9:3). Sí nos enseña que escuchar instrucciones sabias protege.</t>
         </is>
       </c>
       <c r="J14" s="61" t="inlineStr">
@@ -20203,7 +20203,7 @@
       </c>
       <c r="F15" s="61" t="inlineStr">
         <is>
-          <t>La confianza saca el miedo: prevenir no es vivir con paranoia, es cuidarse con tranquilidad.</t>
+          <t>El temor del Señor no es miedo: es reverencia y confianza. Y esa confianza saca el miedo: prevenir no es vivir con paranoia, es cuidarse con tranquilidad.</t>
         </is>
       </c>
       <c r="G15" s="61" t="inlineStr">
@@ -20273,7 +20273,7 @@
       </c>
       <c r="F16" s="61" t="inlineStr">
         <is>
-          <t>Prestar atención a las señales a tiempo da vida. Muchas enfermedades no duelen al principio.</t>
+          <t>El padre de Proverbios pide atención a sus palabras de sabiduría: son vida y salud. Esa sabiduría también nos hace atentos con el cuerpo, como escuchar sus señales a tiempo: muchas enfermedades no duelen al principio.</t>
         </is>
       </c>
       <c r="G16" s="61" t="inlineStr">
@@ -20288,7 +20288,7 @@
       </c>
       <c r="I16" s="61" t="inlineStr">
         <is>
-          <t>Escuchar a quien sabe cuida el cuerpo. Los profesionales de salud están para orientarnos.</t>
+          <t>La sabiduría se recibe escuchando. Dios nos habla en su Palabra y además pone a nuestro lado personas que saben, como los profesionales de salud, para orientarnos.</t>
         </is>
       </c>
       <c r="J16" s="61" t="inlineStr">
@@ -20633,7 +20633,7 @@
       </c>
       <c r="L21" s="61" t="inlineStr">
         <is>
-          <t>El éxito verdadero no es solo plata: es integridad, paz y relaciones sanas. Y se construye con constancia diaria.</t>
+          <t>En Josué, prosperar es cumplir con éxito la misión que Dios le dio, guiado por su Palabra. No es una promesa de riqueza: es la bendición de andar en su camino, que se ve en integridad, paz y fruto, y se construye con constancia diaria.</t>
         </is>
       </c>
       <c r="M21" s="61" t="inlineStr">
@@ -21301,7 +21301,7 @@
       <c r="K31" s="61" t="n"/>
       <c r="L31" s="61" t="inlineStr">
         <is>
-          <t>Quién sos cuando nadie mira es quien realmente sos. Ahí se forma el líder.</t>
+          <t>Quién sos cuando nadie mira es quien realmente sos. Dios forma ese carácter en nosotros cuando le abrimos el corazón (Filipenses 2:13).</t>
         </is>
       </c>
       <c r="M31" s="61" t="n"/>
@@ -21418,7 +21418,7 @@
       </c>
       <c r="I33" s="61" t="inlineStr">
         <is>
-          <t>Cómo está la casa dice algo de cómo estamos por dentro. No hace falta lujo: hace falta cuidado.</t>
+          <t>A veces el desorden de afuera refleja cansancio o cargas de adentro. No hace falta lujo ni perfección: hace falta cuidado, de a poco.</t>
         </is>
       </c>
       <c r="J33" s="61" t="inlineStr">
@@ -21643,7 +21643,7 @@
       </c>
       <c r="L36" s="61" t="inlineStr">
         <is>
-          <t>Lo que va primero sostiene todo lo demás. Si Dios y la familia van primero, el trabajo y las cosas encuentran su lugar.</t>
+          <t>Lo que va primero sostiene todo lo demás. Si Dios va primero, la familia, el trabajo y las cosas encuentran su lugar.</t>
         </is>
       </c>
       <c r="M36" s="61" t="inlineStr">
@@ -21763,7 +21763,7 @@
       </c>
       <c r="L38" s="61" t="inlineStr">
         <is>
-          <t>Ahorrar no es desconfiar de Dios: es usar la sabiduría que Él mismo puso en la creación. Confiar y prepararse van juntos.</t>
+          <t>Ahorrar no es desconfiar de Dios: es usar la sabiduría que Él puso en la creación. La diferencia está en el corazón: prepararse con confianza no es lo mismo que acumular por miedo o avaricia (Lucas 12:15-21).</t>
         </is>
       </c>
       <c r="M38" s="61" t="inlineStr">
@@ -21818,7 +21818,7 @@
       </c>
       <c r="I39" s="61" t="inlineStr">
         <is>
-          <t>El ahorro es el puente entre los años buenos y los malos. Lo que guardás hoy es la tranquilidad de mañana.</t>
+          <t>El ahorro es el puente entre los años buenos y los malos. Lo que guardás hoy puede aliviar el mañana, aunque nuestra seguridad de fondo está en Dios, no en la cuenta.</t>
         </is>
       </c>
       <c r="J39" s="61" t="inlineStr">
@@ -21943,7 +21943,7 @@
       </c>
       <c r="F41" s="61" t="inlineStr">
         <is>
-          <t>Salomón aconseja dividir: no poner todo en una sola cosa, porque no sabemos qué puede pasar.</t>
+          <t>Este consejo se lee de dos maneras: muchos lo entienden como un llamado a compartir con varios, y otros como repartir lo que uno tiene. Las dos coinciden en algo: no aferrarse a una sola seguridad, porque no sabemos qué puede pasar.</t>
         </is>
       </c>
       <c r="G41" s="61" t="inlineStr">
@@ -22089,7 +22089,7 @@
       <c r="G43" s="61" t="n"/>
       <c r="H43" s="61" t="inlineStr">
         <is>
-          <t>Abrí esta semana un sobre o una cuenta de ahorro y poné ahí tu primer aporte, aunque sea pequeño.</t>
+          <t>Jesús usó esta imagen para hablar del costo de seguirlo, y la plata también es parte de ese camino. Esta semana abrí un sobre o una cuenta de ahorro y poné tu primer aporte, aunque sea pequeño.</t>
         </is>
       </c>
       <c r="I43" s="61" t="inlineStr">
@@ -22133,7 +22133,7 @@
       </c>
       <c r="F44" s="61" t="inlineStr">
         <is>
-          <t>Jesús pide un «sí» que sea sí y un «no» que sea no. Esa honestidad empieza por dentro: reconocer lo que de verdad sentimos.</t>
+          <t>Jesús habla de los juramentos: no hace falta jurar si nuestra palabra es verdadera. Un «sí» que es sí y un «no» que es no. Esa honestidad incluye no fingir lo que sentimos.</t>
         </is>
       </c>
       <c r="G44" s="61" t="inlineStr">
@@ -22203,7 +22203,7 @@
       </c>
       <c r="F45" s="61" t="inlineStr">
         <is>
-          <t>Pablo dice que el cambio viene por la renovación de la mente. Lo que pensamos una y otra vez va formando lo que sentimos.</t>
+          <t>Pablo dice «transfórmense»: es Dios quien transforma, mientras nosotros renovamos la mente con su Palabra. Lo que pensamos una y otra vez va formando lo que sentimos.</t>
         </is>
       </c>
       <c r="G45" s="61" t="inlineStr">
@@ -22273,7 +22273,7 @@
       </c>
       <c r="F46" s="61" t="inlineStr">
         <is>
-          <t>Entre tantas voces que escuchamos cada día, hay una verdad que debería sonar más fuerte: Dios te ama, así como sos.</t>
+          <t>Entre tantas voces que escuchamos cada día, hay una verdad que debería sonar más fuerte: Dios te ama tal como sos, y por amor no te deja como estás.</t>
         </is>
       </c>
       <c r="G46" s="61" t="inlineStr">
@@ -22303,7 +22303,7 @@
       </c>
       <c r="L46" s="61" t="inlineStr">
         <is>
-          <t>La fe nace de lo que escuchamos. Si lo que más escuchamos es miedo y queja, la fe se achica.</t>
+          <t>El regalo es vida eterna para todo el que cree en Jesús. Esa fe se alimenta de lo que escuchamos: si lo que más oímos es miedo y queja, nos olvidamos de la esperanza que tenemos.</t>
         </is>
       </c>
       <c r="M46" s="61" t="inlineStr">
@@ -22343,7 +22343,7 @@
       </c>
       <c r="F47" s="61" t="inlineStr">
         <is>
-          <t>Pablo le recuerda a Timoteo que el miedo que paraliza no es lo que Dios nos dio. Mucho de ese miedo entra por lo que consumimos.</t>
+          <t>Pablo anima a Timoteo a no avergonzarse de dar testimonio: Dios no nos dio un espíritu de cobardía. Mucho del miedo que nos paraliza entra por lo que consumimos.</t>
         </is>
       </c>
       <c r="G47" s="61" t="inlineStr">
@@ -22383,7 +22383,7 @@
       </c>
       <c r="N47" s="61" t="inlineStr">
         <is>
-          <t>Cuando aparezca el miedo, ponele nombre, respirá hondo tres veces y decí: «Dios no me dio un espíritu de cobardía».</t>
+          <t>Cuando aparezca el miedo, ponele nombre, respirá hondo tres veces y decí: «Dios no me dio un espíritu de cobardía». Si la ansiedad no se va, pedí ayuda: no es falta de fe.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mensajero: guiones de marzo (semanas 9 a 13) con revisión teológica
- 30 guiones: ganadería, control médico, comunión, herramientas de
  liderazgo (Semana Santa) y matrimonio
- Revisión teológica: 2 campos, 7 puntos y tildes en 2 versículos, con motivo
  en tools/revision_teologica_mar_2027.py y en content/revision_teologica_2027.md
- content/versiculos_sugeridos.md: cambios de versículo pendientes de aprobación
  (Levítico 25:23 y otros; urgente: texto de Proverbios 12:15)
- Alarma: «jamás justifica» ya no se marca como promesa absoluta

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -2745,19 +2745,19 @@
       </c>
       <c r="AB10" s="45" t="inlineStr">
         <is>
-          <t>Salmo 23:1-2 — El Senor es mi pastor; nada me falta. En campos de verdes pastos me hace descansar; me lleva a arroyos de aguas tranquilas</t>
+          <t>Salmo 23:1-2 — El Señor es mi pastor; nada me falta. En campos de verdes pastos me hace descansar; me lleva a arroyos de aguas tranquilas</t>
         </is>
       </c>
       <c r="AC10" s="47" t="inlineStr">
         <is>
           <t>• Dios como pastor provee descanso y alimento
 • El buen cuidado refleja el carácter del pastor
-• El modelo de Dios enseña como cuidar</t>
+• El modelo de Dios enseña cómo cuidar</t>
         </is>
       </c>
       <c r="AD10" s="45" t="inlineStr">
         <is>
-          <t>Proverbios 12:10 — El justo sabe cuando su bestia tiene hambre, pero los impios son crueles de corazon</t>
+          <t>Proverbios 12:10 — El justo sabe cuando su bestia tiene hambre, pero los impíos son crueles de corazón</t>
         </is>
       </c>
       <c r="AE10" s="47" t="inlineStr">
@@ -2778,7 +2778,7 @@
         <is>
           <t>• El trabajo fiel se nota con el tiempo
 • El cuidado del ganado bendijo a Laban
-• La diligencia trae prosperidad visible</t>
+• La bendición de Dios acompañó el trabajo fiel</t>
         </is>
       </c>
       <c r="AH10" s="46" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="AG11" s="49" t="inlineStr">
         <is>
-          <t>• El uso de remedios naturales aparece en la Escritura
+          <t>• Dios usó un remedio de su tiempo
 • Dios usa medios humanos para sanar
 • La fe y el tratamiento médico no se oponen</t>
         </is>
@@ -2990,7 +2990,7 @@
       <c r="AI11" s="49" t="inlineStr">
         <is>
           <t>• El que obedece el consejo es sabio
-• Rechazar el consejo médico es necedad
+• Rechazar un buen consejo sale caro
 • Escuchar a los expertos protege la salud</t>
         </is>
       </c>
@@ -3403,7 +3403,7 @@
       <c r="AI13" s="53" t="inlineStr">
         <is>
           <t>• Sin dirección el pueblo se dispersa
-• La visión da orden y propósito
+• La Palabra de Dios da orden y propósito
 • Guardar la palabra trae bienestar</t>
         </is>
       </c>
@@ -3566,9 +3566,9 @@
       </c>
       <c r="AC14" s="35" t="inlineStr">
         <is>
-          <t>• El respeto es el lenguaje de la esposa
+          <t>• La esposa honra a su esposo
 • Ambos roles se complementan
-• No hay jerarquía de valor, si de función</t>
+• Igual valor y respeto mutuo</t>
         </is>
       </c>
       <c r="AD14" s="35" t="inlineStr">
@@ -19216,7 +19216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N49"/>
+  <dimension ref="A1:N79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22506,6 +22506,2006 @@
       </c>
       <c r="M49" s="61" t="n"/>
       <c r="N49" s="61" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="B50" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C50" s="61" t="inlineStr">
+        <is>
+          <t>Un encargo, no un permiso para abusar</t>
+        </is>
+      </c>
+      <c r="D50" s="61" t="inlineStr">
+        <is>
+          <t>Paraguay tiene más del doble de vacunos que de habitantes: unos 13 millones de cabezas de ganado y unos 6 millones de personas.</t>
+        </is>
+      </c>
+      <c r="E50" s="61" t="inlineStr">
+        <is>
+          <t>SENACSA; INE, Censo Nacional 2022</t>
+        </is>
+      </c>
+      <c r="F50" s="61" t="inlineStr">
+        <is>
+          <t>Dios crea al ser humano a su imagen y le encarga cuidar la creación. Dominar, en la Biblia, es gobernar como Dios gobierna: con cuidado, no con abuso.</t>
+        </is>
+      </c>
+      <c r="G50" s="61" t="inlineStr">
+        <is>
+          <t>Animales maltratados o abandonados, en el campo y en la ciudad.</t>
+        </is>
+      </c>
+      <c r="H50" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés animales, revisá hoy que tengan agua limpia, sombra y comida suficiente.</t>
+        </is>
+      </c>
+      <c r="I50" s="61" t="inlineStr">
+        <is>
+          <t>La autoridad viene con responsabilidad: lo que Dios pone en nuestras manos no es nuestro para hacer lo que queramos, sino para cuidarlo y rendir cuentas.</t>
+        </is>
+      </c>
+      <c r="J50" s="61" t="inlineStr">
+        <is>
+          <t>Ver el campo y los animales solo como ganancia rápida, sin pensar en el mañana.</t>
+        </is>
+      </c>
+      <c r="K50" s="61" t="inlineStr">
+        <is>
+          <t>Si trabajás con ganado, anotá esta semana una cosa que podés mejorar en el bienestar de tus animales.</t>
+        </is>
+      </c>
+      <c r="L50" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar es parte del mandato original: Dios puso al ser humano en el huerto «para que lo cultivara y lo cuidara» (Génesis 2:15). Atender a los animales todos los días es una forma de cumplirlo.</t>
+        </is>
+      </c>
+      <c r="M50" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo diario con animales, que no tiene feriados y casi nadie valora.</t>
+        </is>
+      </c>
+      <c r="N50" s="61" t="inlineStr">
+        <is>
+          <t>Si conocés a alguien que trabaja en una estancia o en un tambo, agradecele hoy su constancia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="B51" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C51" s="61" t="inlineStr">
+        <is>
+          <t>El pastor que da descanso</t>
+        </is>
+      </c>
+      <c r="D51" s="61" t="inlineStr">
+        <is>
+          <t>Las vacas lecheras necesitan pasar entre 12 y 14 horas por día echadas; cuando descansan menos, producen menos leche.</t>
+        </is>
+      </c>
+      <c r="E51" s="61" t="inlineStr">
+        <is>
+          <t>Rick Grant, W. H. Miner Agricultural Research Institute</t>
+        </is>
+      </c>
+      <c r="F51" s="61" t="inlineStr">
+        <is>
+          <t>David, que fue pastor, describe a Dios como el pastor que lleva a sus ovejas a donde hay pasto y agua tranquila. Nada falta, no porque tengamos todo, sino porque Él cuida.</t>
+        </is>
+      </c>
+      <c r="G51" s="61" t="inlineStr">
+        <is>
+          <t>Personas que viven agotadas, creyendo que todo depende de ellas.</t>
+        </is>
+      </c>
+      <c r="H51" s="61" t="inlineStr">
+        <is>
+          <t>Tomate hoy un momento de descanso real y agradecé a Dios por algo que te proveyó esta semana.</t>
+        </is>
+      </c>
+      <c r="I51" s="61" t="inlineStr">
+        <is>
+          <t>Un rebaño bien cuidado habla del pastor. Cómo cuidamos a los animales, a la familia o al equipo dice mucho de nosotros.</t>
+        </is>
+      </c>
+      <c r="J51" s="61" t="inlineStr">
+        <is>
+          <t>Trabajadores rurales que cuidan bien el ganado, pero ellos mismos no tienen descanso ni condiciones dignas.</t>
+        </is>
+      </c>
+      <c r="K51" s="61" t="inlineStr">
+        <is>
+          <t>Si sos patrón o encargado, revisá esta semana que tus trabajadores tengan su descanso y lo necesario para trabajar.</t>
+        </is>
+      </c>
+      <c r="L51" s="61" t="inlineStr">
+        <is>
+          <t>Dios no solo nos cuida: nos enseña cómo cuidar. Guía sin apurar, provee y da descanso.</t>
+        </is>
+      </c>
+      <c r="M51" s="61" t="inlineStr">
+        <is>
+          <t>Arrear a los animales y tratar a las personas con gritos y golpes.</t>
+        </is>
+      </c>
+      <c r="N51" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana probá manejar con calma: sin gritos ni golpes, con paciencia. Vas a notar la diferencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="B52" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C52" s="61" t="inlineStr">
+        <is>
+          <t>El justo cuida a sus animales</t>
+        </is>
+      </c>
+      <c r="D52" s="61" t="inlineStr">
+        <is>
+          <t>El estrés del ganado antes de la faena oscurece la carne y la vuelve más dura: el buen trato también se nota en el plato.</t>
+        </is>
+      </c>
+      <c r="E52" s="61" t="inlineStr">
+        <is>
+          <t>Temple Grandin, Universidad Estatal de Colorado</t>
+        </is>
+      </c>
+      <c r="F52" s="61" t="inlineStr">
+        <is>
+          <t>El justo conoce lo que necesitan sus animales. En la Biblia, la justicia no es solo con las personas: alcanza también a los seres que están a nuestro cargo.</t>
+        </is>
+      </c>
+      <c r="G52" s="61" t="inlineStr">
+        <is>
+          <t>Animales sin agua ni sombra en los días de calor extremo del verano.</t>
+        </is>
+      </c>
+      <c r="H52" s="61" t="inlineStr">
+        <is>
+          <t>Asegurá sombra y agua fresca para tus animales en las horas de más calor.</t>
+        </is>
+      </c>
+      <c r="I52" s="61" t="inlineStr">
+        <is>
+          <t>La crueldad con un animal no se queda ahí: muestra un corazón que se endureció. El trato a los más débiles revela quiénes somos.</t>
+        </is>
+      </c>
+      <c r="J52" s="61" t="inlineStr">
+        <is>
+          <t>Chicos que crecen viendo el maltrato a los animales como algo normal.</t>
+        </is>
+      </c>
+      <c r="K52" s="61" t="inlineStr">
+        <is>
+          <t>Enseñá a tus hijos a tratar con respeto a los animales de la casa y del campo, con tu ejemplo.</t>
+        </is>
+      </c>
+      <c r="L52" s="61" t="inlineStr">
+        <is>
+          <t>A Dios le importa toda su creación: Él alimenta a las aves del cielo (Mateo 6:26). Por eso a nosotros también nos importa.</t>
+        </is>
+      </c>
+      <c r="M52" s="61" t="inlineStr">
+        <is>
+          <t>Perros y gatos abandonados en las calles de nuestros barrios.</t>
+        </is>
+      </c>
+      <c r="N52" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés mascotas, cuidá sus vacunas y no las abandones. Adoptar un animal es un compromiso para toda su vida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="B53" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C53" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo fiel se nota con el tiempo</t>
+        </is>
+      </c>
+      <c r="D53" s="61" t="inlineStr">
+        <is>
+          <t>Paraguay vacuna a todo su ganado bovino contra la fiebre aftosa en campañas que se repiten dos veces por año.</t>
+        </is>
+      </c>
+      <c r="E53" s="61" t="inlineStr">
+        <is>
+          <t>Servicio Nacional de Calidad y Salud Animal (SENACSA)</t>
+        </is>
+      </c>
+      <c r="F53" s="61" t="inlineStr">
+        <is>
+          <t>Jacob le recuerda a Labán cuánto trabajó para él durante años. El trabajo fiel, día tras día, se nota con el tiempo, aunque al principio nadie lo vea.</t>
+        </is>
+      </c>
+      <c r="G53" s="61" t="inlineStr">
+        <is>
+          <t>Trabajadores que sienten que su esfuerzo constante no es reconocido.</t>
+        </is>
+      </c>
+      <c r="H53" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés gente a cargo, reconocé hoy, con nombre y apellido, el trabajo constante de alguien.</t>
+        </is>
+      </c>
+      <c r="I53" s="61" t="inlineStr">
+        <is>
+          <t>Jacob dice: «el Señor te ha bendecido» con mi llegada. La bendición vino de Dios, y llegó a través de un trabajo bien hecho que benefició a otro.</t>
+        </is>
+      </c>
+      <c r="J53" s="61" t="inlineStr">
+        <is>
+          <t>Hacer solo lo justo porque «total, el beneficio es del patrón».</t>
+        </is>
+      </c>
+      <c r="K53" s="61" t="inlineStr">
+        <is>
+          <t>Hacé tu trabajo de hoy de corazón, como para el Señor (Colosenses 3:23), aunque el beneficio sea de otro.</t>
+        </is>
+      </c>
+      <c r="L53" s="61" t="inlineStr">
+        <is>
+          <t>Esta historia describe lo que pasó, no es una fórmula para hacerse rico: Jacob también tuvo errores y engaños, y aun así Dios fue fiel. Y Jacob plantea algo justo: ¿cuándo voy a cuidar de mi propia casa?</t>
+        </is>
+      </c>
+      <c r="M53" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar tanto para otros que la propia familia queda descuidada.</t>
+        </is>
+      </c>
+      <c r="N53" s="61" t="inlineStr">
+        <is>
+          <t>Revisá tu semana y separá tiempo para tu propia casa, igual que lo hacés para tu trabajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="B54" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C54" s="61" t="inlineStr">
+        <is>
+          <t>El buen pastor</t>
+        </is>
+      </c>
+      <c r="D54" s="61" t="inlineStr">
+        <is>
+          <t>La carne vacuna está entre los principales productos que Paraguay vende al mundo, junto con la soja.</t>
+        </is>
+      </c>
+      <c r="E54" s="61" t="inlineStr">
+        <is>
+          <t>Banco Central del Paraguay, informes de comercio exterior</t>
+        </is>
+      </c>
+      <c r="F54" s="61" t="inlineStr">
+        <is>
+          <t>Jesús es el buen pastor: no solo cuida a las ovejas, da su vida por ellas. Lo hizo en la cruz, una vez y para siempre, para salvarnos. Eso no lo podemos imitar: lo recibimos con gratitud.</t>
+        </is>
+      </c>
+      <c r="G54" s="61" t="inlineStr">
+        <is>
+          <t>Vivir como si tuviéramos que ganarnos el amor de Dios con esfuerzo.</t>
+        </is>
+      </c>
+      <c r="H54" s="61" t="inlineStr">
+        <is>
+          <t>Hoy agradecé a Jesús, con tus propias palabras, por lo que hizo por vos.</t>
+        </is>
+      </c>
+      <c r="I54" s="61" t="inlineStr">
+        <is>
+          <t>Su entrega nos enseña lo que es un compromiso de verdad: no abandonar cuando hay peligro, como el asalariado que huye (Juan 10:12).</t>
+        </is>
+      </c>
+      <c r="J54" s="61" t="inlineStr">
+        <is>
+          <t>Compromisos que se abandonan apenas cuestan: en el trabajo, en la familia, en la iglesia.</t>
+        </is>
+      </c>
+      <c r="K54" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en un compromiso que te está costando sostener y pedile a Dios fuerzas para seguir esta semana.</t>
+        </is>
+      </c>
+      <c r="L54" s="61" t="inlineStr">
+        <is>
+          <t>La entrega de Jesús también inspira el trabajo de cada día. Detrás de cada comida hay una cadena de personas que se dedican: el que cría, el que transporta, el que vende. Cada eslabón, hecho con dedicación, es una forma de servir.</t>
+        </is>
+      </c>
+      <c r="M54" s="61" t="inlineStr">
+        <is>
+          <t>Ver la comida como algo que aparece en el supermercado, sin valorar el trabajo que hay detrás.</t>
+        </is>
+      </c>
+      <c r="N54" s="61" t="inlineStr">
+        <is>
+          <t>En la comida de hoy, agradezcan en familia a Dios y a las personas que la hicieron posible: criadores, transportistas y comerciantes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="61" t="n">
+        <v>9</v>
+      </c>
+      <c r="B55" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C55" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: cuidar como cuida Dios</t>
+        </is>
+      </c>
+      <c r="D55" s="61" t="inlineStr">
+        <is>
+          <t>Las ovejas pueden reconocer y recordar las caras de al menos 50 ovejas, y también de personas, durante más de dos años.</t>
+        </is>
+      </c>
+      <c r="E55" s="61" t="inlineStr">
+        <is>
+          <t>Kendrick y otros, revista Nature, 2001</t>
+        </is>
+      </c>
+      <c r="F55" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo con animales pide constancia todos los días: es una diligencia que sostiene la vida y la producción.</t>
+        </is>
+      </c>
+      <c r="G55" s="61" t="n"/>
+      <c r="H55" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé esta semana, en persona, a alguien de la cadena: un productor, un transportista o el carnicero de tu barrio.</t>
+        </is>
+      </c>
+      <c r="I55" s="61" t="inlineStr">
+        <is>
+          <t>Manejar el rodeo con responsabilidad es tratar bien a los animales: a Dios le importa su creación.</t>
+        </is>
+      </c>
+      <c r="J55" s="61" t="n"/>
+      <c r="K55" s="61" t="n"/>
+      <c r="L55" s="61" t="inlineStr">
+        <is>
+          <t>De la crianza a la mesa hay una cadena de trabajo: valorarla es agradecer el esfuerzo que hay detrás de cada plato.</t>
+        </is>
+      </c>
+      <c r="M55" s="61" t="n"/>
+      <c r="N55" s="61" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="B56" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C56" s="61" t="inlineStr">
+        <is>
+          <t>El médico es para el que lo necesita</t>
+        </is>
+      </c>
+      <c r="D56" s="61" t="inlineStr">
+        <is>
+          <t>Casi la mitad de los adultos con diabetes en el mundo (44 %) no sabe que la tiene.</t>
+        </is>
+      </c>
+      <c r="E56" s="61" t="inlineStr">
+        <is>
+          <t>Federación Internacional de Diabetes, Atlas de la Diabetes, 2021</t>
+        </is>
+      </c>
+      <c r="F56" s="61" t="inlineStr">
+        <is>
+          <t>Jesús responde a quienes lo criticaban por comer con pecadores: vino a buscar a los que saben que lo necesitan. Usa una imagen que todos entienden: el médico es para el que está enfermo.</t>
+        </is>
+      </c>
+      <c r="G56" s="61" t="inlineStr">
+        <is>
+          <t>Creer que estamos sanos porque no sentimos nada.</t>
+        </is>
+      </c>
+      <c r="H56" s="61" t="inlineStr">
+        <is>
+          <t>Si hace más de un año que no te hacés un control, agendalo esta semana en tu unidad de salud familiar.</t>
+        </is>
+      </c>
+      <c r="I56" s="61" t="inlineStr">
+        <is>
+          <t>El primer paso para recibir ayuda es reconocer que la necesitamos. Vale para el alma, porque Jesús llama a los que se saben necesitados de perdón, y vale también para el cuerpo.</t>
+        </is>
+      </c>
+      <c r="J56" s="61" t="inlineStr">
+        <is>
+          <t>El orgullo de decir «a mí no me pasa nada» y no consultar.</t>
+        </is>
+      </c>
+      <c r="K56" s="61" t="inlineStr">
+        <is>
+          <t>Hacé una lista honesta de los síntomas que venís ignorando y llevala a tu próxima consulta.</t>
+        </is>
+      </c>
+      <c r="L56" s="61" t="inlineStr">
+        <is>
+          <t>Buscar ayuda no es debilidad: es sabiduría. Jesús no rechazó a nadie que se le acercó a pedirle ayuda.</t>
+        </is>
+      </c>
+      <c r="M56" s="61" t="inlineStr">
+        <is>
+          <t>Hombres que no van al médico porque lo sienten como una señal de debilidad.</t>
+        </is>
+      </c>
+      <c r="N56" s="61" t="inlineStr">
+        <is>
+          <t>Si sos hombre, sacá un turno para tu control. Si tenés un padre, un esposo o un hermano que no va, acompañalo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="B57" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C57" s="61" t="inlineStr">
+        <is>
+          <t>Lucas, el médico amado</t>
+        </is>
+      </c>
+      <c r="D57" s="61" t="inlineStr">
+        <is>
+          <t>Lucas, el médico que acompañó a Pablo, escribió el Evangelio que lleva su nombre y el libro de Hechos: cerca de la cuarta parte del Nuevo Testamento.</t>
+        </is>
+      </c>
+      <c r="E57" s="61" t="inlineStr">
+        <is>
+          <t>Nuevo Testamento: Evangelio de Lucas y Hechos</t>
+        </is>
+      </c>
+      <c r="F57" s="61" t="inlineStr">
+        <is>
+          <t>Lucas, médico, acompañó a Pablo en sus viajes, y Pablo lo llama «el médico amado». Un profesional de la salud estaba en el corazón del equipo misionero.</t>
+        </is>
+      </c>
+      <c r="G57" s="61" t="inlineStr">
+        <is>
+          <t>La desconfianza hacia los médicos, alimentada por malas experiencias o por lo que circula en redes.</t>
+        </is>
+      </c>
+      <c r="H57" s="61" t="inlineStr">
+        <is>
+          <t>Si tuviste una mala experiencia, buscá una segunda opinión, pero no dejes de controlarte.</t>
+        </is>
+      </c>
+      <c r="I57" s="61" t="inlineStr">
+        <is>
+          <t>En el equipo de Pablo, la fe y la medicina estaban juntas. No hace falta elegir entre orar y consultar.</t>
+        </is>
+      </c>
+      <c r="J57" s="61" t="inlineStr">
+        <is>
+          <t>La idea de que ir al médico es no confiar en Dios.</t>
+        </is>
+      </c>
+      <c r="K57" s="61" t="inlineStr">
+        <is>
+          <t>Orá antes de tu consulta: por vos y por el profesional que te va a atender.</t>
+        </is>
+      </c>
+      <c r="L57" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar la salud de otros es un servicio valioso, y muchos profesionales de la salud viven su trabajo como un llamado.</t>
+        </is>
+      </c>
+      <c r="M57" s="61" t="inlineStr">
+        <is>
+          <t>Profesionales de la salud cansados y poco reconocidos, sobre todo en los hospitales públicos.</t>
+        </is>
+      </c>
+      <c r="N57" s="61" t="inlineStr">
+        <is>
+          <t>La próxima vez que te atiendan, agradecé al médico, a la enfermera o al personal con su nombre y una palabra amable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="B58" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C58" s="61" t="inlineStr">
+        <is>
+          <t>Sáname, Señor</t>
+        </is>
+      </c>
+      <c r="D58" s="61" t="inlineStr">
+        <is>
+          <t>Para los adultos, se recomienda medir la presión cada año desde los 40, y cada 3 a 5 años entre los 18 y los 39 si no hay factores de riesgo.</t>
+        </is>
+      </c>
+      <c r="E58" s="61" t="inlineStr">
+        <is>
+          <t>Grupo de Trabajo de Servicios Preventivos de EE. UU. (USPSTF), 2021</t>
+        </is>
+      </c>
+      <c r="F58" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías ora en medio de la persecución: «Sáname, Señor». Pedirle salud a Dios es legítimo, y nuestra confianza en Él no depende de cómo resulte.</t>
+        </is>
+      </c>
+      <c r="G58" s="61" t="inlineStr">
+        <is>
+          <t>No saber qué incluye un control y por eso no pedirlo.</t>
+        </is>
+      </c>
+      <c r="H58" s="61" t="inlineStr">
+        <is>
+          <t>Preguntá en tu unidad de salud familiar qué incluye un control completo para tu edad: presión, peso, análisis de sangre básicos y los antecedentes de tu familia.</t>
+        </is>
+      </c>
+      <c r="I58" s="61" t="inlineStr">
+        <is>
+          <t>Más que una cura, Jeremías busca a Dios mismo: Él es su refugio. Un control médico se vive distinto cuando sabemos en quién estamos seguros.</t>
+        </is>
+      </c>
+      <c r="J58" s="61" t="inlineStr">
+        <is>
+          <t>El miedo a los resultados de los análisis, que hace postergar el control.</t>
+        </is>
+      </c>
+      <c r="K58" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés miedo de ir, pedile a alguien de confianza que te acompañe, y oren juntos antes.</t>
+        </is>
+      </c>
+      <c r="L58" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías termina alabando, antes de ver la respuesta. La gratitud no depende del diagnóstico.</t>
+        </is>
+      </c>
+      <c r="M58" s="61" t="inlineStr">
+        <is>
+          <t>Vivir la salud como algo que nos corresponde, sin agradecer los días buenos.</t>
+        </is>
+      </c>
+      <c r="N58" s="61" t="inlineStr">
+        <is>
+          <t>Hoy agradecé a Dios por tres cosas que tu cuerpo puede hacer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="B59" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C59" s="61" t="inlineStr">
+        <is>
+          <t>Dios también obra a través de medios</t>
+        </is>
+      </c>
+      <c r="D59" s="61" t="inlineStr">
+        <is>
+          <t>Los errores en el uso de medicamentos cuestan en el mundo unos 42.000 millones de dólares por año.</t>
+        </is>
+      </c>
+      <c r="E59" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Medicación sin daño, 2017</t>
+        </is>
+      </c>
+      <c r="F59" s="61" t="inlineStr">
+        <is>
+          <t>Dios ya le había prometido a Ezequías que viviría (Isaías 38:5), y aun así se usó un remedio de su tiempo: una pasta de higos sobre la llaga. Dios obra también a través de medios.</t>
+        </is>
+      </c>
+      <c r="G59" s="61" t="inlineStr">
+        <is>
+          <t>Dejar un tratamiento indicado para usar solo yuyos o remedios caseros que alguien recomendó.</t>
+        </is>
+      </c>
+      <c r="H59" s="61" t="inlineStr">
+        <is>
+          <t>Si usás remedios naturales o yuyos, contáselo a tu médico: algunos pueden interferir con los medicamentos.</t>
+        </is>
+      </c>
+      <c r="I59" s="61" t="inlineStr">
+        <is>
+          <t>El remedio no reemplazó a Dios, y Dios no despreció el remedio. Los médicos, las enfermeras y los medicamentos pueden ser instrumentos de su cuidado.</t>
+        </is>
+      </c>
+      <c r="J59" s="61" t="inlineStr">
+        <is>
+          <t>Automedicarse con lo que le sirvió a un vecino.</t>
+        </is>
+      </c>
+      <c r="K59" s="61" t="inlineStr">
+        <is>
+          <t>Llevá a tu próxima consulta una lista escrita de todo lo que tomás, con dosis y horarios.</t>
+        </is>
+      </c>
+      <c r="L59" s="61" t="inlineStr">
+        <is>
+          <t>Orar y seguir el tratamiento van juntos. La fe no nos pide abandonar la medicina, sino confiar en Dios en todo el proceso.</t>
+        </is>
+      </c>
+      <c r="M59" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar el tratamiento apenas uno se siente mejor.</t>
+        </is>
+      </c>
+      <c r="N59" s="61" t="inlineStr">
+        <is>
+          <t>Si te indicaron un tratamiento, cumplilo completo, aunque te sientas bien antes de terminarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="B60" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C60" s="61" t="inlineStr">
+        <is>
+          <t>El sabio escucha el consejo</t>
+        </is>
+      </c>
+      <c r="D60" s="61" t="inlineStr">
+        <is>
+          <t>Cuando el cáncer de mama se detecta en etapa temprana y se trata a tiempo, más del 90 % de las mujeres vive al menos cinco años más.</t>
+        </is>
+      </c>
+      <c r="E60" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Iniciativa Mundial contra el Cáncer de Mama, 2023</t>
+        </is>
+      </c>
+      <c r="F60" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios compara al necio, que cree que siempre tiene razón, con el sabio, que escucha consejo. La sabiduría empieza por admitir que no lo sabemos todo.</t>
+        </is>
+      </c>
+      <c r="G60" s="61" t="inlineStr">
+        <is>
+          <t>Esperar a que algo duela para recién ir a consultar.</t>
+        </is>
+      </c>
+      <c r="H60" s="61" t="inlineStr">
+        <is>
+          <t>No esperes síntomas: si por tu edad ya te toca un control, agendalo esta semana.</t>
+        </is>
+      </c>
+      <c r="I60" s="61" t="inlineStr">
+        <is>
+          <t>Escuchar el consejo de quien sabe, como un profesional de la salud, es una forma concreta de sabiduría. Postergarlo por miedo o por orgullo suele salir caro.</t>
+        </is>
+      </c>
+      <c r="J60" s="61" t="inlineStr">
+        <is>
+          <t>Diagnósticos que llegan tarde porque se postergó la consulta, cuando el tratamiento ya es más difícil.</t>
+        </is>
+      </c>
+      <c r="K60" s="61" t="inlineStr">
+        <is>
+          <t>Si te indicaron un estudio que venís postergando, hacelo este mes.</t>
+        </is>
+      </c>
+      <c r="L60" s="61" t="inlineStr">
+        <is>
+          <t>La sabiduría también es humilde para cambiar de opinión con buena información, y prudente para no creer cualquier consejo de internet.</t>
+        </is>
+      </c>
+      <c r="M60" s="61" t="inlineStr">
+        <is>
+          <t>Consejos de salud que circulan en los grupos de WhatsApp sin ningún respaldo.</t>
+        </is>
+      </c>
+      <c r="N60" s="61" t="inlineStr">
+        <is>
+          <t>Antes de compartir un consejo de salud, preguntá: ¿quién lo dice y en qué se basa?</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="B61" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C61" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: cuidarse a tiempo</t>
+        </is>
+      </c>
+      <c r="D61" s="61" t="inlineStr">
+        <is>
+          <t>Las Unidades de Salud de la Familia (USF) ofrecen atención primaria gratuita en todo el país.</t>
+        </is>
+      </c>
+      <c r="E61" s="61" t="inlineStr">
+        <is>
+          <t>Ministerio de Salud Pública y Bienestar Social del Paraguay</t>
+        </is>
+      </c>
+      <c r="F61" s="61" t="inlineStr">
+        <is>
+          <t>Un control médico es para cuando estás bien: detecta lo que todavía no da síntomas.</t>
+        </is>
+      </c>
+      <c r="G61" s="61" t="n"/>
+      <c r="H61" s="61" t="inlineStr">
+        <is>
+          <t>Sacá esta semana un turno para tu control en la unidad de salud familiar más cercana, y animá a alguien de tu familia a hacer lo mismo.</t>
+        </is>
+      </c>
+      <c r="I61" s="61" t="inlineStr">
+        <is>
+          <t>Un control completo incluye presión, peso, análisis básicos y los antecedentes de tu familia. Orar y consultar van juntos.</t>
+        </is>
+      </c>
+      <c r="J61" s="61" t="n"/>
+      <c r="K61" s="61" t="n"/>
+      <c r="L61" s="61" t="inlineStr">
+        <is>
+          <t>No esperes a estar enfermo: lo que se detecta a tiempo es más simple de tratar.</t>
+        </is>
+      </c>
+      <c r="M61" s="61" t="n"/>
+      <c r="N61" s="61" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="B62" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C62" s="61" t="inlineStr">
+        <is>
+          <t>La fe nunca fue para vivirla solo</t>
+        </is>
+      </c>
+      <c r="D62" s="61" t="inlineStr">
+        <is>
+          <t>Las personas con vínculos sociales fuertes tuvieron un 50 % más de probabilidades de seguir con vida en el tiempo que las que tenían vínculos débiles.</t>
+        </is>
+      </c>
+      <c r="E62" s="61" t="inlineStr">
+        <is>
+          <t>Holt-Lunstad, Smith y Layton, revista PLoS Medicine, 2010</t>
+        </is>
+      </c>
+      <c r="F62" s="61" t="inlineStr">
+        <is>
+          <t>Los primeros cristianos no solo creyeron: se mantuvieron juntos, con constancia. Desde el principio, la fe se vivió en comunidad.</t>
+        </is>
+      </c>
+      <c r="G62" s="61" t="inlineStr">
+        <is>
+          <t>Personas que creen en Dios pero viven su fe completamente solas, sin nadie que las acompañe.</t>
+        </is>
+      </c>
+      <c r="H62" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, contale a alguien de tu iglesia o de tu familia algo que Dios te enseñó.</t>
+        </is>
+      </c>
+      <c r="I62" s="61" t="inlineStr">
+        <is>
+          <t>Enseñanza, compañerismo, la mesa compartida y la oración: las cuatro cosas juntas. Si falta una, la vida de fe se desequilibra.</t>
+        </is>
+      </c>
+      <c r="J62" s="61" t="inlineStr">
+        <is>
+          <t>Saber mucho de la Biblia pero no tener amigos en la fe; o tener amigos, pero no alimentarse de la Palabra.</t>
+        </is>
+      </c>
+      <c r="K62" s="61" t="inlineStr">
+        <is>
+          <t>Mirá cuál de las cuatro te falta más y da un paso pequeño esta semana.</t>
+        </is>
+      </c>
+      <c r="L62" s="61" t="inlineStr">
+        <is>
+          <t>No es un modelo de perfección: aquella iglesia también tuvo problemas (Hechos 5 y 6). Es un modelo de constancia.</t>
+        </is>
+      </c>
+      <c r="M62" s="61" t="inlineStr">
+        <is>
+          <t>Alejarse de la iglesia después de una herida o un conflicto, y quedarse solo.</t>
+        </is>
+      </c>
+      <c r="N62" s="61" t="inlineStr">
+        <is>
+          <t>Si te alejaste por una herida, orá por eso y buscá a una persona de confianza para conversarlo, sin apuro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="B63" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C63" s="61" t="inlineStr">
+        <is>
+          <t>Mejor dos que uno</t>
+        </is>
+      </c>
+      <c r="D63" s="61" t="inlineStr">
+        <is>
+          <t>En un experimento, personas que miraban una colina empinada acompañadas por un amigo la veían menos empinada que quienes estaban solas.</t>
+        </is>
+      </c>
+      <c r="E63" s="61" t="inlineStr">
+        <is>
+          <t>Schnall y otros, Journal of Experimental Social Psychology, 2008</t>
+        </is>
+      </c>
+      <c r="F63" s="61" t="inlineStr">
+        <is>
+          <t>Salomón observa la vida y concluye: dos son mejor que uno. No es un mandamiento, es sabiduría que sale de la experiencia.</t>
+        </is>
+      </c>
+      <c r="G63" s="61" t="inlineStr">
+        <is>
+          <t>El orgullo de querer arreglarlo todo solo.</t>
+        </is>
+      </c>
+      <c r="H63" s="61" t="inlineStr">
+        <is>
+          <t>Pedí ayuda hoy en algo concreto que te está costando.</t>
+        </is>
+      </c>
+      <c r="I63" s="61" t="inlineStr">
+        <is>
+          <t>Juntos sacamos más provecho del esfuerzo. Lo que uno no ve, el otro lo ve.</t>
+        </is>
+      </c>
+      <c r="J63" s="61" t="inlineStr">
+        <is>
+          <t>Grupos de la iglesia o del barrio donde cada uno hace lo suyo, sin ponerse de acuerdo.</t>
+        </is>
+      </c>
+      <c r="K63" s="61" t="inlineStr">
+        <is>
+          <t>Proponé en tu grupo una tarea para hacer juntos esta semana: visitar a alguien, preparar algo, orar.</t>
+        </is>
+      </c>
+      <c r="L63" s="61" t="inlineStr">
+        <is>
+          <t>El texto no promete que no vamos a caer: dice que, si caemos, es bueno tener quien nos levante.</t>
+        </is>
+      </c>
+      <c r="M63" s="61" t="inlineStr">
+        <is>
+          <t>Personas que pasan una crisis y nadie se entera, porque no tienen a quién contarle.</t>
+        </is>
+      </c>
+      <c r="N63" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en alguien que está pasando un mal momento y llamalo hoy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="B64" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C64" s="61" t="inlineStr">
+        <is>
+          <t>Caminar en la luz, juntos</t>
+        </is>
+      </c>
+      <c r="D64" s="61" t="inlineStr">
+        <is>
+          <t>En experimentos sobre pedir ayuda, las personas creyeron que les iban a decir que no mucho más de lo que realmente pasó: los demás estaban más dispuestos a ayudar de lo que pensaban.</t>
+        </is>
+      </c>
+      <c r="E64" s="61" t="inlineStr">
+        <is>
+          <t>Flynn y Lake, Journal of Personality and Social Psychology, 2008</t>
+        </is>
+      </c>
+      <c r="F64" s="61" t="inlineStr">
+        <is>
+          <t>Andar en la luz es vivir a la vista de Dios, sin esconder nada. De ahí nace una comunión verdadera con los demás.</t>
+        </is>
+      </c>
+      <c r="G64" s="61" t="inlineStr">
+        <is>
+          <t>Relaciones de iglesia superficiales, donde todos dicen «bien, gracias».</t>
+        </is>
+      </c>
+      <c r="H64" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, compartí con alguien de confianza una necesidad real, para que ore por vos.</t>
+        </is>
+      </c>
+      <c r="I64" s="61" t="inlineStr">
+        <is>
+          <t>La transparencia no significa contarle todo a todos, sino no vivir con máscaras. Y no depende de ser perfectos: la sangre de Jesús nos limpia de todo pecado.</t>
+        </is>
+      </c>
+      <c r="J64" s="61" t="inlineStr">
+        <is>
+          <t>El miedo a ser juzgado si los demás conocen nuestras luchas.</t>
+        </is>
+      </c>
+      <c r="K64" s="61" t="inlineStr">
+        <is>
+          <t>Elegí a una o dos personas de confianza con quienes puedas ser honesto sobre tus luchas, y orá por ellas.</t>
+        </is>
+      </c>
+      <c r="L64" s="61" t="inlineStr">
+        <is>
+          <t>La comunión con Dios y con los hermanos van juntas. Lo que se construye en comunidad, como el consuelo en el momento justo o la corrección amable, no se construye solo.</t>
+        </is>
+      </c>
+      <c r="M64" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que la relación con Dios es solo privada y que los demás no hacen falta.</t>
+        </is>
+      </c>
+      <c r="N64" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, sumate a un grupo pequeño, una célula o una reunión de oración, aunque sea una vez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="B65" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C65" s="61" t="inlineStr">
+        <is>
+          <t>Un solo cuerpo, muchos miembros</t>
+        </is>
+      </c>
+      <c r="D65" s="61" t="inlineStr">
+        <is>
+          <t>El cuerpo humano tiene más de 600 músculos, que trabajan coordinados hasta en un simple paso.</t>
+        </is>
+      </c>
+      <c r="E65" s="61" t="inlineStr">
+        <is>
+          <t>Anatomía humana</t>
+        </is>
+      </c>
+      <c r="F65" s="61" t="inlineStr">
+        <is>
+          <t>Pablo usa la imagen del cuerpo: muchos miembros, cada uno con su función, unidos en Cristo.</t>
+        </is>
+      </c>
+      <c r="G65" s="61" t="inlineStr">
+        <is>
+          <t>Personas que se sienten de más en la iglesia porque no cantan, no predican ni tocan un instrumento.</t>
+        </is>
+      </c>
+      <c r="H65" s="61" t="inlineStr">
+        <is>
+          <t>Preguntá en tu iglesia dónde hace falta ayuda y ofrecé lo que sabés hacer, aunque te parezca poco.</t>
+        </is>
+      </c>
+      <c r="I65" s="61" t="inlineStr">
+        <is>
+          <t>Ningún miembro se basta solo: todos nos necesitamos. Lo que a mí me falta, Dios lo puso en otro.</t>
+        </is>
+      </c>
+      <c r="J65" s="61" t="inlineStr">
+        <is>
+          <t>Comparar los dones y sentir envidia o menosprecio.</t>
+        </is>
+      </c>
+      <c r="K65" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy a alguien de tu comunidad por un don que vos no tenés.</t>
+        </is>
+      </c>
+      <c r="L65" s="61" t="inlineStr">
+        <is>
+          <t>Ser distintos no rompe la unidad: la enriquece. Unidad no es que todos seamos iguales.</t>
+        </is>
+      </c>
+      <c r="M65" s="61" t="inlineStr">
+        <is>
+          <t>Divisiones en las iglesias por diferencias de estilo o de opinión en cosas secundarias.</t>
+        </is>
+      </c>
+      <c r="N65" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un desacuerdo con alguien de tu comunidad, buscá hablarlo en privado y con respeto esta semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="B66" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C66" s="61" t="inlineStr">
+        <is>
+          <t>El hierro se afila con hierro</t>
+        </is>
+      </c>
+      <c r="D66" s="61" t="inlineStr">
+        <is>
+          <t>Hacer un amigo casual lleva unas 50 horas compartidas, y un amigo cercano, más de 200.</t>
+        </is>
+      </c>
+      <c r="E66" s="61" t="inlineStr">
+        <is>
+          <t>Jeffrey Hall, Universidad de Kansas, Journal of Social and Personal Relationships, 2018</t>
+        </is>
+      </c>
+      <c r="F66" s="61" t="inlineStr">
+        <is>
+          <t>El hierro se afila con hierro: hace falta contacto, y a veces roce. Las relaciones cercanas nos mejoran, también cuando incomodan.</t>
+        </is>
+      </c>
+      <c r="G66" s="61" t="inlineStr">
+        <is>
+          <t>Huir de toda relación que nos confronte.</t>
+        </is>
+      </c>
+      <c r="H66" s="61" t="inlineStr">
+        <is>
+          <t>Pedile a un amigo de confianza que te diga con sinceridad algo que podés mejorar, y escuchalo sin defenderte.</t>
+        </is>
+      </c>
+      <c r="I66" s="61" t="inlineStr">
+        <is>
+          <t>La amistad verdadera no solo acompaña: desafía. Asistir a una reunión no es lo mismo que pertenecer.</t>
+        </is>
+      </c>
+      <c r="J66" s="61" t="inlineStr">
+        <is>
+          <t>Ir a la iglesia cada domingo sin conocer de verdad a nadie.</t>
+        </is>
+      </c>
+      <c r="K66" s="61" t="inlineStr">
+        <is>
+          <t>Invitá a alguien de tu iglesia a un tereré o a comer, fuera del horario de las reuniones.</t>
+        </is>
+      </c>
+      <c r="L66" s="61" t="inlineStr">
+        <is>
+          <t>La comunidad real se construye con tiempo compartido, constancia y apertura.</t>
+        </is>
+      </c>
+      <c r="M66" s="61" t="inlineStr">
+        <is>
+          <t>Agendas tan llenas que no queda tiempo para los amigos.</t>
+        </is>
+      </c>
+      <c r="N66" s="61" t="inlineStr">
+        <is>
+          <t>Agendá esta semana un tiempo fijo, aunque sea corto, para encontrarte con alguien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="61" t="n">
+        <v>11</v>
+      </c>
+      <c r="B67" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C67" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: la fe se vive juntos</t>
+        </is>
+      </c>
+      <c r="D67" s="61" t="inlineStr">
+        <is>
+          <t>La palabra griega «koinonía», que traducimos como comunión o compañerismo, significa tener algo en común y participar juntos.</t>
+        </is>
+      </c>
+      <c r="E67" s="61" t="inlineStr">
+        <is>
+          <t>Diccionarios del griego del Nuevo Testamento</t>
+        </is>
+      </c>
+      <c r="F67" s="61" t="inlineStr">
+        <is>
+          <t>No fuimos hechos para vivir la fe solos: la comunidad nos sostiene cuando la convicción se debilita.</t>
+        </is>
+      </c>
+      <c r="G67" s="61" t="n"/>
+      <c r="H67" s="61" t="inlineStr">
+        <is>
+          <t>Llamá esta semana a alguien de tu iglesia, fuera del horario de las reuniones, solo para saber cómo está.</t>
+        </is>
+      </c>
+      <c r="I67" s="61" t="inlineStr">
+        <is>
+          <t>En comunidad aparecen cosas que no se construyen solo: el consuelo, la corrección amable y la alegría compartida.</t>
+        </is>
+      </c>
+      <c r="J67" s="61" t="n"/>
+      <c r="K67" s="61" t="n"/>
+      <c r="L67" s="61" t="inlineStr">
+        <is>
+          <t>Pertenecer no es solo asistir: la comunidad real se cultiva con tiempo, constancia y apertura.</t>
+        </is>
+      </c>
+      <c r="M67" s="61" t="n"/>
+      <c r="N67" s="61" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="B68" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C68" s="61" t="inlineStr">
+        <is>
+          <t>Escuchar antes de hablar</t>
+        </is>
+      </c>
+      <c r="D68" s="61" t="inlineStr">
+        <is>
+          <t>Cuando Google estudió qué hacía a sus mejores jefes, entre las conductas más importantes encontró ser un buen comunicador y saber escuchar.</t>
+        </is>
+      </c>
+      <c r="E68" s="61" t="inlineStr">
+        <is>
+          <t>Google, Proyecto Oxígeno</t>
+        </is>
+      </c>
+      <c r="F68" s="61" t="inlineStr">
+        <is>
+          <t>Santiago pide estar dispuestos a oír. Comunicar bien empieza por escuchar: entender al otro antes de responder.</t>
+        </is>
+      </c>
+      <c r="G68" s="61" t="inlineStr">
+        <is>
+          <t>Reuniones de trabajo o de familia donde todos hablan y nadie escucha.</t>
+        </is>
+      </c>
+      <c r="H68" s="61" t="inlineStr">
+        <is>
+          <t>En tu próxima conversación importante, antes de responder, repetí con tus palabras lo que entendiste.</t>
+        </is>
+      </c>
+      <c r="I68" s="61" t="inlineStr">
+        <is>
+          <t>Hablar rápido, sin pensar, genera malentendidos que después cuesta arreglar.</t>
+        </is>
+      </c>
+      <c r="J68" s="61" t="inlineStr">
+        <is>
+          <t>Mensajes de audio o de WhatsApp mandados en caliente, que dañan relaciones.</t>
+        </is>
+      </c>
+      <c r="K68" s="61" t="inlineStr">
+        <is>
+          <t>Antes de comunicar algo importante, resumilo en una sola frase clara. Si estás enojado, esperá antes de enviarlo.</t>
+        </is>
+      </c>
+      <c r="L68" s="61" t="inlineStr">
+        <is>
+          <t>Santiago agrega: lentos para enojarse, porque el enojo humano no produce la justicia de Dios (1:20). Un líder que controla su enojo da seguridad a su equipo.</t>
+        </is>
+      </c>
+      <c r="M68" s="61" t="inlineStr">
+        <is>
+          <t>Jefes o padres que gritan y después se preguntan por qué nadie les cuenta nada.</t>
+        </is>
+      </c>
+      <c r="N68" s="61" t="inlineStr">
+        <is>
+          <t>Si sentís que te enojás, pedí unos minutos y volvé a hablar cuando estés en calma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="B69" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C69" s="61" t="inlineStr">
+        <is>
+          <t>El consejo que salvó a Moisés</t>
+        </is>
+      </c>
+      <c r="D69" s="61" t="inlineStr">
+        <is>
+          <t>Moisés atendía al pueblo «desde la mañana hasta la tarde», y su suegro le dijo: «No está bien lo que haces».</t>
+        </is>
+      </c>
+      <c r="E69" s="61" t="inlineStr">
+        <is>
+          <t>Éxodo 18:13-17</t>
+        </is>
+      </c>
+      <c r="F69" s="61" t="inlineStr">
+        <is>
+          <t>Jetro, el suegro de Moisés, le aconseja elegir personas confiables y temerosas de Dios. Delegar empieza por elegir bien y explicar con claridad qué se espera.</t>
+        </is>
+      </c>
+      <c r="G69" s="61" t="inlineStr">
+        <is>
+          <t>Delegar en cualquiera, sin explicar bien, y después enojarse con el resultado.</t>
+        </is>
+      </c>
+      <c r="H69" s="61" t="inlineStr">
+        <is>
+          <t>Antes de delegar una tarea, explicá en una frase qué se espera, para cuándo y cómo se va a revisar.</t>
+        </is>
+      </c>
+      <c r="I69" s="61" t="inlineStr">
+        <is>
+          <t>Moisés quería hacerlo todo y se estaba agotando. Escuchar un buen consejo, aunque venga del suegro, también es humildad.</t>
+        </is>
+      </c>
+      <c r="J69" s="61" t="inlineStr">
+        <is>
+          <t>Líderes de iglesia, padres o jefes que se agotan porque creen que nadie lo hará tan bien como ellos.</t>
+        </is>
+      </c>
+      <c r="K69" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una tarea que siempre hacés vos y que otro puede aprender. Enseñala esta semana.</t>
+        </is>
+      </c>
+      <c r="L69" s="61" t="inlineStr">
+        <is>
+          <t>Delegar no es desentenderse: Moisés siguió atendiendo los casos graves. Se comparte la carga y se acompaña.</t>
+        </is>
+      </c>
+      <c r="M69" s="61" t="inlineStr">
+        <is>
+          <t>Delegar y desaparecer, sin seguimiento.</t>
+        </is>
+      </c>
+      <c r="N69" s="61" t="inlineStr">
+        <is>
+          <t>Acordá con quien te ayuda un momento corto para revisar juntos cómo va.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="B70" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C70" s="61" t="inlineStr">
+        <is>
+          <t>Planificar y soltar</t>
+        </is>
+      </c>
+      <c r="D70" s="61" t="inlineStr">
+        <is>
+          <t>Solemos subestimar el tiempo que nos lleva una tarea, aunque ya nos haya pasado antes; los psicólogos lo llaman «falacia de la planificación».</t>
+        </is>
+      </c>
+      <c r="E70" s="61" t="inlineStr">
+        <is>
+          <t>Kahneman y Tversky, 1979; Buehler y otros, 1994</t>
+        </is>
+      </c>
+      <c r="F70" s="61" t="inlineStr">
+        <is>
+          <t>Planificar es bueno y es humano. Pero el versículo nos recuerda que el rumbo final lo corrige Dios.</t>
+        </is>
+      </c>
+      <c r="G70" s="61" t="inlineStr">
+        <is>
+          <t>Planes hechos con orgullo, como si todo dependiera de nosotros.</t>
+        </is>
+      </c>
+      <c r="H70" s="61" t="inlineStr">
+        <is>
+          <t>Escribí tus planes de esta semana y orá por ellos, uno por uno.</t>
+        </is>
+      </c>
+      <c r="I70" s="61" t="inlineStr">
+        <is>
+          <t>Delegar también es soltar: no todo depende de mí. Confiar una tarea a otro, con seguimiento, es parte de reconocer que no lo controlamos todo.</t>
+        </is>
+      </c>
+      <c r="J70" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que no delegan porque necesitan controlarlo todo.</t>
+        </is>
+      </c>
+      <c r="K70" s="61" t="inlineStr">
+        <is>
+          <t>Delegá esta semana una tarea completa y, en vez de controlar cada paso, acordá un momento para revisar el resultado.</t>
+        </is>
+      </c>
+      <c r="L70" s="61" t="inlineStr">
+        <is>
+          <t>Cuando Dios corrige el rumbo, ser flexible es sabiduría, no derrota.</t>
+        </is>
+      </c>
+      <c r="M70" s="61" t="inlineStr">
+        <is>
+          <t>La frustración y el enojo cuando las cosas no salen como estaba previsto.</t>
+        </is>
+      </c>
+      <c r="N70" s="61" t="inlineStr">
+        <is>
+          <t>Cuando algo cambie tus planes esta semana, preguntate: ¿qué puedo aprender o hacer distinto?</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="B71" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C71" s="61" t="inlineStr">
+        <is>
+          <t>Un tiempo para cada cosa</t>
+        </is>
+      </c>
+      <c r="D71" s="61" t="inlineStr">
+        <is>
+          <t>En Eclesiastés 3 aparecen catorce pares de tiempos opuestos: nacer y morir, plantar y cosechar, llorar y reír, callar y hablar.</t>
+        </is>
+      </c>
+      <c r="E71" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés 3:2-8</t>
+        </is>
+      </c>
+      <c r="F71" s="61" t="inlineStr">
+        <is>
+          <t>Salomón describe la vida en tiempos. No es una técnica de organización: es reconocer que los tiempos están en las manos de Dios (Eclesiastés 3:11).</t>
+        </is>
+      </c>
+      <c r="G71" s="61" t="inlineStr">
+        <is>
+          <t>Querer hacer todo al mismo tiempo y no terminar nada.</t>
+        </is>
+      </c>
+      <c r="H71" s="61" t="inlineStr">
+        <is>
+          <t>Elegí qué es lo propio de esta etapa de tu vida y qué puede esperar.</t>
+        </is>
+      </c>
+      <c r="I71" s="61" t="inlineStr">
+        <is>
+          <t>Hay un tiempo para hacer y un tiempo para que otro haga. Saber cuándo delegar y cuándo intervenir también es discernir el tiempo.</t>
+        </is>
+      </c>
+      <c r="J71" s="61" t="inlineStr">
+        <is>
+          <t>Delegar cuando ya es tarde y todo es urgente.</t>
+        </is>
+      </c>
+      <c r="K71" s="61" t="inlineStr">
+        <is>
+          <t>Mirá las tareas del próximo mes y decidí hoy cuáles vas a delegar, antes de que sean urgentes.</t>
+        </is>
+      </c>
+      <c r="L71" s="61" t="inlineStr">
+        <is>
+          <t>Actuar a destiempo, con apuro o tarde, suele costar más. La paciencia y la oportunidad van juntas.</t>
+        </is>
+      </c>
+      <c r="M71" s="61" t="inlineStr">
+        <is>
+          <t>Decisiones importantes tomadas a último momento, bajo presión.</t>
+        </is>
+      </c>
+      <c r="N71" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés una decisión importante por delante, poné una fecha para tomarla con tiempo y consultá antes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="B72" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C72" s="61" t="inlineStr">
+        <is>
+          <t>Cuando falta la Palabra</t>
+        </is>
+      </c>
+      <c r="D72" s="61" t="inlineStr">
+        <is>
+          <t>La palabra hebrea que en este proverbio se traduce como «visión» se usa para la revelación que Dios daba a sus profetas.</t>
+        </is>
+      </c>
+      <c r="E72" s="61" t="inlineStr">
+        <is>
+          <t>Léxicos del hebreo bíblico</t>
+        </is>
+      </c>
+      <c r="F72" s="61" t="inlineStr">
+        <is>
+          <t>Este proverbio no habla de metas de empresa: la «visión» es la revelación de Dios. Cuando falta su Palabra, el pueblo se desvía.</t>
+        </is>
+      </c>
+      <c r="G72" s="61" t="inlineStr">
+        <is>
+          <t>Vivir corriendo, ocupados todo el día, sin saber hacia dónde vamos.</t>
+        </is>
+      </c>
+      <c r="H72" s="61" t="inlineStr">
+        <is>
+          <t>Al empezar el día, elegí una sola tarea importante: si se hace, el resto importa menos.</t>
+        </is>
+      </c>
+      <c r="I72" s="61" t="inlineStr">
+        <is>
+          <t>La segunda parte lo confirma: dichoso el que obedece la ley de Dios. Su Palabra ordena las prioridades, y lo urgente no siempre es lo importante.</t>
+        </is>
+      </c>
+      <c r="J72" s="61" t="inlineStr">
+        <is>
+          <t>Lo urgente que se come lo importante: el celular, los mensajes, los imprevistos.</t>
+        </is>
+      </c>
+      <c r="K72" s="61" t="inlineStr">
+        <is>
+          <t>Separá cada día un tiempo para la Palabra antes de lo urgente, aunque sean diez minutos.</t>
+        </is>
+      </c>
+      <c r="L72" s="61" t="inlineStr">
+        <is>
+          <t>La dicha de la que habla no es tener todo resuelto, sino vivir en el camino de Dios. En este Viernes Santo recordamos hasta dónde llegó su amor por nosotros.</t>
+        </is>
+      </c>
+      <c r="M72" s="61" t="inlineStr">
+        <is>
+          <t>Agendas tan llenas que no queda lugar para Dios ni para la familia.</t>
+        </is>
+      </c>
+      <c r="N72" s="61" t="inlineStr">
+        <is>
+          <t>Este fin de semana de Pascua, reservá un tiempo en familia para leer juntos lo que pasó en la cruz y en la resurrección.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="61" t="n">
+        <v>12</v>
+      </c>
+      <c r="B73" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C73" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: liderar con responsabilidad</t>
+        </is>
+      </c>
+      <c r="D73" s="61" t="inlineStr">
+        <is>
+          <t>«Lo importante rara vez es urgente, y lo urgente rara vez es importante», dijo Dwight Eisenhower; de esa idea nació un método para ordenar tareas.</t>
+        </is>
+      </c>
+      <c r="E73" s="61" t="inlineStr">
+        <is>
+          <t>Dwight D. Eisenhower, discurso de 1954</t>
+        </is>
+      </c>
+      <c r="F73" s="61" t="inlineStr">
+        <is>
+          <t>Comunicar bien empieza por escuchar: lentos para hablar y para enojarse.</t>
+        </is>
+      </c>
+      <c r="G73" s="61" t="n"/>
+      <c r="H73" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide aprovechar bien el tiempo con los que no creen. En este fin de semana de Pascua, invitá a alguien a celebrar con vos la resurrección.</t>
+        </is>
+      </c>
+      <c r="I73" s="61" t="inlineStr">
+        <is>
+          <t>Delegar no es desentenderse: es elegir bien, explicar con claridad y acompañar.</t>
+        </is>
+      </c>
+      <c r="J73" s="61" t="n"/>
+      <c r="K73" s="61" t="n"/>
+      <c r="L73" s="61" t="inlineStr">
+        <is>
+          <t>Lo urgente no siempre es lo importante: la Palabra de Dios ordena las prioridades.</t>
+        </is>
+      </c>
+      <c r="M73" s="61" t="n"/>
+      <c r="N73" s="61" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="B74" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C74" s="61" t="inlineStr">
+        <is>
+          <t>Ser cabeza es entregarse</t>
+        </is>
+      </c>
+      <c r="D74" s="61" t="inlineStr">
+        <is>
+          <t>En parejas estables se observaron unas cinco interacciones positivas por cada interacción negativa durante los conflictos.</t>
+        </is>
+      </c>
+      <c r="E74" s="61" t="inlineStr">
+        <is>
+          <t>John Gottman, Universidad de Washington</t>
+        </is>
+      </c>
+      <c r="F74" s="61" t="inlineStr">
+        <is>
+          <t>Pablo no define la cabeza por el poder, sino por la entrega: amar como Cristo, que se entregó por la iglesia. Es liderazgo de servicio, nunca de autoridad impuesta, y jamás justifica el maltrato.</t>
+        </is>
+      </c>
+      <c r="G74" s="61" t="inlineStr">
+        <is>
+          <t>La idea de que ser cabeza es mandar, decidir solo o imponerse.</t>
+        </is>
+      </c>
+      <c r="H74" s="61" t="inlineStr">
+        <is>
+          <t>Esposo: preguntale hoy a tu esposa en qué podés servirla mejor esta semana, y hacelo.</t>
+        </is>
+      </c>
+      <c r="I74" s="61" t="inlineStr">
+        <is>
+          <t>El amor de Cristo no fue un sentimiento: fue una entrega concreta. En el matrimonio, amar es una decisión de cada día.</t>
+        </is>
+      </c>
+      <c r="J74" s="61" t="inlineStr">
+        <is>
+          <t>Matrimonios que se apagan esperando volver a sentir lo del principio.</t>
+        </is>
+      </c>
+      <c r="K74" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy un gesto concreto de amor que tu pareja valore, aunque no tengas ganas.</t>
+        </is>
+      </c>
+      <c r="L74" s="61" t="inlineStr">
+        <is>
+          <t>El estándar es alto a propósito: nadie lo cumple con sus propias fuerzas. Por eso necesitamos la gracia de Cristo para amar como Él.</t>
+        </is>
+      </c>
+      <c r="M74" s="61" t="inlineStr">
+        <is>
+          <t>La culpa de sentir que nunca alcanzamos lo que deberíamos ser.</t>
+        </is>
+      </c>
+      <c r="N74" s="61" t="inlineStr">
+        <is>
+          <t>Oren juntos esta semana, aunque sea un minuto, pidiendo a Dios que los ayude a amarse como Él.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="B75" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C75" s="61" t="inlineStr">
+        <is>
+          <t>Amor y honra</t>
+        </is>
+      </c>
+      <c r="D75" s="61" t="inlineStr">
+        <is>
+          <t>Justo antes de hablar a los esposos, Pablo les pide algo a todos: «Sométanse unos a otros en el temor de Dios».</t>
+        </is>
+      </c>
+      <c r="E75" s="61" t="inlineStr">
+        <is>
+          <t>Efesios 5:21</t>
+        </is>
+      </c>
+      <c r="F75" s="61" t="inlineStr">
+        <is>
+          <t>Pablo cierra el pasaje con dos verbos: el esposo ama a su esposa como a sí mismo, y la esposa honra a su esposo. Y antes de todo pidió algo para los dos: sométanse unos a otros (5:21).</t>
+        </is>
+      </c>
+      <c r="G75" s="61" t="inlineStr">
+        <is>
+          <t>Matrimonios donde se habla con desprecio o con burla del otro, incluso delante de los hijos o en las redes.</t>
+        </is>
+      </c>
+      <c r="H75" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, hablá bien de tu pareja delante de otros, con un ejemplo concreto.</t>
+        </is>
+      </c>
+      <c r="I75" s="61" t="inlineStr">
+        <is>
+          <t>Cada uno tiene su parte, y las dos se complementan. El matrimonio es un equipo, no una competencia de quién hace más.</t>
+        </is>
+      </c>
+      <c r="J75" s="61" t="inlineStr">
+        <is>
+          <t>Llevar la cuenta de quién hizo más en la casa y usarla en las discusiones.</t>
+        </is>
+      </c>
+      <c r="K75" s="61" t="inlineStr">
+        <is>
+          <t>Repasen juntos las tareas de la casa y repártanlas de nuevo según lo que cada uno puede en esta etapa.</t>
+        </is>
+      </c>
+      <c r="L75" s="61" t="inlineStr">
+        <is>
+          <t>Varón y mujer tienen el mismo valor ante Dios y son coherederos de la gracia (1 Pedro 3:7). Las iglesias explican de distintas maneras estos roles, pero todas coinciden en el amor que se entrega y el respeto mutuo. Nada de esto justifica el maltrato.</t>
+        </is>
+      </c>
+      <c r="M75" s="61" t="inlineStr">
+        <is>
+          <t>La violencia en el hogar, a veces justificada con versículos sacados de contexto.</t>
+        </is>
+      </c>
+      <c r="N75" s="61" t="inlineStr">
+        <is>
+          <t>Si vos o alguien que conocés sufre violencia, pedí ayuda: hablá con tu pastor y llamá a la línea 137 «SOS Mujer», que atiende las 24 horas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="B76" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C76" s="61" t="inlineStr">
+        <is>
+          <t>Orar el uno por el otro</t>
+        </is>
+      </c>
+      <c r="D76" s="61" t="inlineStr">
+        <is>
+          <t>Personas que oraron por el bienestar de su pareja durante cuatro semanas mostraron más disposición a perdonar.</t>
+        </is>
+      </c>
+      <c r="E76" s="61" t="inlineStr">
+        <is>
+          <t>Lambert, Fincham y otros, Psychological Science, 2010</t>
+        </is>
+      </c>
+      <c r="F76" s="61" t="inlineStr">
+        <is>
+          <t>Samuel le dice al pueblo que sería un pecado dejar de orar por ellos. Si eso vale para un pueblo, cuánto más para la persona con quien compartimos la vida.</t>
+        </is>
+      </c>
+      <c r="G76" s="61" t="inlineStr">
+        <is>
+          <t>Parejas que oran por muchas cosas, pero casi nunca la una por la otra.</t>
+        </is>
+      </c>
+      <c r="H76" s="61" t="inlineStr">
+        <is>
+          <t>Orá cada día de esta semana por tu pareja, por su nombre y por algo concreto que esté viviendo.</t>
+        </is>
+      </c>
+      <c r="I76" s="61" t="inlineStr">
+        <is>
+          <t>Samuel no solo ora: se compromete a enseñar el camino bueno. En el matrimonio nos ayudamos a crecer, sin imponer ni sermonear.</t>
+        </is>
+      </c>
+      <c r="J76" s="61" t="inlineStr">
+        <is>
+          <t>Corregir a la pareja delante de otros o con tono de superioridad.</t>
+        </is>
+      </c>
+      <c r="K76" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés algo que decirle a tu pareja, hacelo en privado, con calma, y empezando por lo bueno.</t>
+        </is>
+      </c>
+      <c r="L76" s="61" t="inlineStr">
+        <is>
+          <t>Los deberes del matrimonio no compiten: se complementan. La pregunta no es quién hace más, sino cómo nos servimos mutuamente.</t>
+        </is>
+      </c>
+      <c r="M76" s="61" t="inlineStr">
+        <is>
+          <t>Pensar el matrimonio como un contrato de deberes y no como una entrega mutua.</t>
+        </is>
+      </c>
+      <c r="N76" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale a tu pareja: ¿qué puedo hacer esta semana para que te sientas acompañado o acompañada?</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="B77" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C77" s="61" t="inlineStr">
+        <is>
+          <t>Un amor que se ve en lo que hace</t>
+        </is>
+      </c>
+      <c r="D77" s="61" t="inlineStr">
+        <is>
+          <t>En 1 Corintios 13:4-7 el amor se describe con quince verbos: casi todo lo que dice del amor es algo que hace, no algo que siente.</t>
+        </is>
+      </c>
+      <c r="E77" s="61" t="inlineStr">
+        <is>
+          <t>Texto griego de 1 Corintios 13:4-7</t>
+        </is>
+      </c>
+      <c r="F77" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribió esto a una iglesia dividida, pero describe el amor que también sostiene un matrimonio: paciente y bondadoso en lo de todos los días.</t>
+        </is>
+      </c>
+      <c r="G77" s="61" t="inlineStr">
+        <is>
+          <t>La impaciencia del cansancio diario, que convierte cualquier detalle en pelea.</t>
+        </is>
+      </c>
+      <c r="H77" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, cuando algo de tu pareja te moleste, respondé con una palabra amable antes que con una queja.</t>
+        </is>
+      </c>
+      <c r="I77" s="61" t="inlineStr">
+        <is>
+          <t>El amor no es egoísta: piensa primero en el bien del otro. Es la actitud de servicio que hace funcionar los deberes de cada uno.</t>
+        </is>
+      </c>
+      <c r="J77" s="61" t="inlineStr">
+        <is>
+          <t>Matrimonios donde cada uno defiende su espacio y sus derechos, y nadie cede.</t>
+        </is>
+      </c>
+      <c r="K77" s="61" t="inlineStr">
+        <is>
+          <t>Elegí algo que te gusta y que esta semana podés ceder por tu pareja.</t>
+        </is>
+      </c>
+      <c r="L77" s="61" t="inlineStr">
+        <is>
+          <t>«Todo lo soporta» habla de un amor que no se rinde ante las dificultades. No significa soportar el maltrato: el amor también protege y busca ayuda.</t>
+        </is>
+      </c>
+      <c r="M77" s="61" t="inlineStr">
+        <is>
+          <t>Crisis matrimoniales que se viven en silencio, sin pedir consejo.</t>
+        </is>
+      </c>
+      <c r="N77" s="61" t="inlineStr">
+        <is>
+          <t>Si su matrimonio está en crisis, busquen juntos a un consejero o a un pastor de confianza. Pedir ayuda también es una forma de amar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="B78" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C78" s="61" t="inlineStr">
+        <is>
+          <t>Tu pareja es un regalo</t>
+        </is>
+      </c>
+      <c r="D78" s="61" t="inlineStr">
+        <is>
+          <t>En un estudio de la Universidad de Virginia, las parejas que compartían tiempo a solas al menos una vez por semana tenían más probabilidades de decir que su matrimonio era muy feliz.</t>
+        </is>
+      </c>
+      <c r="E78" s="61" t="inlineStr">
+        <is>
+          <t>National Marriage Project, Universidad de Virginia, 2012</t>
+        </is>
+      </c>
+      <c r="F78" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios celebra el matrimonio como un bien. Está escrito desde la mirada del esposo, pero vale igual para la esposa: la pareja es un regalo.</t>
+        </is>
+      </c>
+      <c r="G78" s="61" t="inlineStr">
+        <is>
+          <t>Dar por sentado al cónyuge con el paso de los años.</t>
+        </is>
+      </c>
+      <c r="H78" s="61" t="inlineStr">
+        <is>
+          <t>Decile hoy a tu pareja una razón concreta por la que agradecés a Dios por ella o por él.</t>
+        </is>
+      </c>
+      <c r="I78" s="61" t="inlineStr">
+        <is>
+          <t>No es suerte: es favor de Dios. Reconocerlo cambia cómo cuidamos ese regalo. Y quien no está casado no está fuera del favor de Dios: su valor no depende de tener pareja.</t>
+        </is>
+      </c>
+      <c r="J78" s="61" t="inlineStr">
+        <is>
+          <t>Matrimonios que se descuidan porque el trabajo, los hijos y las pantallas lo ocupan todo.</t>
+        </is>
+      </c>
+      <c r="K78" s="61" t="inlineStr">
+        <is>
+          <t>Pongan en la agenda una conversación semanal de quince minutos, sin celulares ni distracciones.</t>
+        </is>
+      </c>
+      <c r="L78" s="61" t="inlineStr">
+        <is>
+          <t>Un matrimonio bien vivido bendice a los hijos, a la familia y a la comunidad. Sostenerlo como prioridad es una decisión activa.</t>
+        </is>
+      </c>
+      <c r="M78" s="61" t="inlineStr">
+        <is>
+          <t>Parejas que solo hablan de las cuentas y de los chicos.</t>
+        </is>
+      </c>
+      <c r="N78" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, salgan a caminar o a tomar un tereré los dos solos, y hablen de ustedes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="61" t="n">
+        <v>13</v>
+      </c>
+      <c r="B79" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C79" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: un amor que no se apaga</t>
+        </is>
+      </c>
+      <c r="D79" s="61" t="inlineStr">
+        <is>
+          <t>En hebreo, el título del Cantar de los Cantares significa «el mejor de los cantos»: es un poema que celebra el amor entre esposos.</t>
+        </is>
+      </c>
+      <c r="E79" s="61" t="inlineStr">
+        <is>
+          <t>Cantar de los Cantares 1:1</t>
+        </is>
+      </c>
+      <c r="F79" s="61" t="inlineStr">
+        <is>
+          <t>Ser cabeza, según la Biblia, es amar y servir como Cristo, que se entregó; nunca es imponerse.</t>
+        </is>
+      </c>
+      <c r="G79" s="61" t="n"/>
+      <c r="H79" s="61" t="inlineStr">
+        <is>
+          <t>Este fin de semana, compartan un tiempo a solas y agradezcan juntos a Dios por su matrimonio. Si tenés un amigo con su matrimonio en crisis, ofrecele tu compañía.</t>
+        </is>
+      </c>
+      <c r="I79" s="61" t="inlineStr">
+        <is>
+          <t>Los deberes de cada uno se complementan: la clave es el servicio mutuo, no la competencia.</t>
+        </is>
+      </c>
+      <c r="J79" s="61" t="n"/>
+      <c r="K79" s="61" t="n"/>
+      <c r="L79" s="61" t="inlineStr">
+        <is>
+          <t>El matrimonio se sostiene eligiendo tiempo juntos cada semana, frente a todo lo que compite por la atención.</t>
+        </is>
+      </c>
+      <c r="M79" s="61" t="n"/>
+      <c r="N79" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de enero a marzo verificados y borrador de abril con revisión teológica
- 78 datos contrastados con su fuente: 40 confirmados, 38 ajustados
  (tools/verificacion_datos_ene_mar_2027.py, content/verificacion_datos_2027.md)
- Línea 137 «SOS Mujer» y WhatsApp verificados en el guion de matrimonio
- Textos RVC confirmados de Proverbios 12:15 y Génesis 1:26 en versiculos_sugeridos
- Abril (semanas 14 a 17): 24 guiones con revisión teológica; datos en verificación
- Scripts de revisión idempotentes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -3995,7 +3995,7 @@
         <is>
           <t>• Esperar en Dios renueva las fuerzas
 • El cansancio espiritual tiene remedio
-• Correr sin fatigarse es promesa para quien espera</t>
+• Dios da fuerzas nuevas para seguir</t>
         </is>
       </c>
       <c r="AF16" s="43" t="inlineStr">
@@ -4020,7 +4020,7 @@
         <is>
           <t>• El anhelo por Dios se compara con la sed del ciervo
 • La búsqueda intensa refleja hambre espiritual
-• Sin ese anhelo, la vida espiritual se estanca</t>
+• Aun en la sequía, el anhelo nos lleva a buscarlo</t>
         </is>
       </c>
       <c r="AJ16" s="43" t="inlineStr">
@@ -4369,7 +4369,7 @@
         <is>
           <t>• No basta con desear: Los sueños necesitan acción y compromiso.
 • El esfuerzo trae resultados: El que trabaja con dedicación puede alcanzar buenos frutos.
-• Dios bendice la perseverancia: La constancia y la responsabilidad abren camino al progreso.</t>
+• La constancia abre camino: La responsabilidad y la perseverancia suelen dar fruto.</t>
         </is>
       </c>
       <c r="Z18" s="49" t="inlineStr">
@@ -4394,7 +4394,7 @@
         <is>
           <t>• Disciplinar el cuerpo con propósito claro
 • El dominio propio evita la descalificación
-• El ejercicio también forma el carácter</t>
+• El dominio propio también se entrena</t>
         </is>
       </c>
       <c r="AD18" s="49" t="inlineStr">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="AG18" s="49" t="inlineStr">
         <is>
-          <t>• Dios cine de fuerza al que confía en El
+          <t>• Dios ciñe de fuerza al que confía en Él
 • La fortaleza física también tiene respaldo espiritual
 • Moverse con la fuerza que Dios da</t>
         </is>
@@ -19216,7 +19216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:N103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -19463,7 +19463,7 @@
       </c>
       <c r="D4" s="61" t="inlineStr">
         <is>
-          <t>Un hábito nuevo tarda en promedio 66 días en volverse automático; en el estudio el rango fue de 18 a 254 días.</t>
+          <t>Un hábito nuevo tarda una media de 66 días en volverse automático; según la persona, el rango fue de 18 a 254 días.</t>
         </is>
       </c>
       <c r="E4" s="61" t="inlineStr">
@@ -19533,12 +19533,12 @@
       </c>
       <c r="D5" s="61" t="inlineStr">
         <is>
-          <t>El corazón late alrededor de 100.000 veces por día, sin que tengamos que pensar en ello.</t>
+          <t>Con un ritmo normal de unos 70 latidos por minuto, el corazón late alrededor de 100.000 veces por día, sin que tengamos que pensar en ello.</t>
         </is>
       </c>
       <c r="E5" s="61" t="inlineStr">
         <is>
-          <t>American Heart Association</t>
+          <t>Cálculo a partir del ritmo normal en reposo (60 a 100 latidos por minuto), American Heart Association</t>
         </is>
       </c>
       <c r="F5" s="61" t="inlineStr">
@@ -19603,7 +19603,7 @@
       </c>
       <c r="D6" s="61" t="inlineStr">
         <is>
-          <t>Uno de cada tres adultos no duerme las horas que necesita.</t>
+          <t>En Estados Unidos, uno de cada tres adultos no duerme las horas que necesita.</t>
         </is>
       </c>
       <c r="E6" s="61" t="inlineStr">
@@ -19673,12 +19673,12 @@
       </c>
       <c r="D7" s="61" t="inlineStr">
         <is>
-          <t>Leer en una pantalla antes de dormir retrasa la melatonina, cuesta más dormirse y se amanece menos alerta.</t>
+          <t>Leer antes de dormir en una tableta con pantalla iluminada, en vez de un libro impreso, retrasó la melatonina, hizo más difícil dormirse y al otro día se amaneció menos alerta.</t>
         </is>
       </c>
       <c r="E7" s="61" t="inlineStr">
         <is>
-          <t>Chang y otros, Harvard Medical School, revista PNAS, 2015</t>
+          <t>Chang y otros, Brigham and Women's Hospital y Harvard Medical School, revista PNAS, 2015</t>
         </is>
       </c>
       <c r="F7" s="61" t="inlineStr">
@@ -20003,12 +20003,12 @@
       </c>
       <c r="D12" s="61" t="inlineStr">
         <is>
-          <t>Unos 3.100 millones de personas en el mundo no pueden pagar una alimentación saludable.</t>
+          <t>Unos 2.700 millones de personas en el mundo no pueden pagar una alimentación saludable.</t>
         </is>
       </c>
       <c r="E12" s="61" t="inlineStr">
         <is>
-          <t>FAO, El estado de la seguridad alimentaria y la nutrición en el mundo, 2023</t>
+          <t>FAO y otros, El estado de la seguridad alimentaria y la nutrición en el mundo (SOFI), 2026</t>
         </is>
       </c>
       <c r="F12" s="61" t="inlineStr">
@@ -20123,12 +20123,12 @@
       </c>
       <c r="D14" s="61" t="inlineStr">
         <is>
-          <t>Las enfermedades no transmisibles (corazón, cáncer, diabetes, pulmones) causan el 74 % de las muertes en el mundo.</t>
+          <t>Las enfermedades no transmisibles (corazón, cáncer, diabetes, pulmones) causan unas tres de cada cuatro muertes en el mundo, sin contar las de la pandemia.</t>
         </is>
       </c>
       <c r="E14" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, 2023</t>
+          <t>Organización Mundial de la Salud, nota descriptiva sobre enfermedades no transmisibles (datos de 2021)</t>
         </is>
       </c>
       <c r="F14" s="61" t="inlineStr">
@@ -20403,12 +20403,12 @@
       </c>
       <c r="D18" s="61" t="inlineStr">
         <is>
-          <t>Unos 280 millones de personas en el mundo viven con depresión.</t>
+          <t>Más de 300 millones de personas en el mundo viven con depresión.</t>
         </is>
       </c>
       <c r="E18" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, 2023</t>
+          <t>Organización Mundial de la Salud, nota descriptiva sobre la depresión</t>
         </is>
       </c>
       <c r="F18" s="61" t="inlineStr">
@@ -20523,12 +20523,12 @@
       </c>
       <c r="D20" s="61" t="inlineStr">
         <is>
-          <t>Quienes leen la Biblia cuatro o más veces por semana muestran cambios mucho mayores en su conducta diaria que quienes la leen con menos frecuencia.</t>
+          <t>En una encuesta del ministerio Back to the Bible, quienes leían la Biblia cuatro o más días por semana contaron hábitos de vida muy distintos de los que la leían menos.</t>
         </is>
       </c>
       <c r="E20" s="61" t="inlineStr">
         <is>
-          <t>Center for Bible Engagement, Cole y Ovwigho, 2009</t>
+          <t>Center for Bible Engagement (Back to the Bible), Cole y Ovwigho, 2009</t>
         </is>
       </c>
       <c r="F20" s="61" t="inlineStr">
@@ -20593,12 +20593,12 @@
       </c>
       <c r="D21" s="61" t="inlineStr">
         <is>
-          <t>Si no repasamos lo aprendido, olvidamos más de la mitad en apenas un día.</t>
+          <t>En sus experimentos de memoria, Hermann Ebbinghaus comprobó que, sin repasar, al día siguiente ya había olvidado cerca de dos tercios de lo aprendido.</t>
         </is>
       </c>
       <c r="E21" s="61" t="inlineStr">
         <is>
-          <t>Hermann Ebbinghaus, estudios sobre la memoria, 1885</t>
+          <t>Hermann Ebbinghaus, «Sobre la memoria», 1885; replicado por Murre y Dros, PLOS ONE, 2015</t>
         </is>
       </c>
       <c r="F21" s="61" t="inlineStr">
@@ -20663,12 +20663,12 @@
       </c>
       <c r="D22" s="61" t="inlineStr">
         <is>
-          <t>Quienes toman notas a mano comprenden mejor los conceptos que quienes escriben en una computadora.</t>
+          <t>Estudiantes que, en vez de releer, trataron de recordar lo leído retuvieron una semana después el 61 % del texto; los que solo releyeron, el 40 %.</t>
         </is>
       </c>
       <c r="E22" s="61" t="inlineStr">
         <is>
-          <t>Mueller y Oppenheimer, revista Psychological Science, 2014</t>
+          <t>Roediger y Karpicke, Washington University in St. Louis, Psychological Science, 2006</t>
         </is>
       </c>
       <c r="F22" s="61" t="inlineStr">
@@ -20993,12 +20993,12 @@
       </c>
       <c r="D27" s="61" t="inlineStr">
         <is>
-          <t>En un experimento clásico, niños que vieron a un adulto golpear a un muñeco repitieron casi los mismos golpes al quedarse solos con él.</t>
+          <t>En un experimento clásico, niños que vieron a un adulto golpear a un muñeco inflable lo imitaron después casi con los mismos golpes y gritos cuando les tocó jugar con él.</t>
         </is>
       </c>
       <c r="E27" s="61" t="inlineStr">
         <is>
-          <t>Bandura, Ross y Ross, Universidad de Stanford, 1961</t>
+          <t>Bandura, Ross y Ross, Universidad de Stanford, Journal of Abnormal and Social Psychology, 1961</t>
         </is>
       </c>
       <c r="F27" s="61" t="inlineStr">
@@ -21063,12 +21063,12 @@
       </c>
       <c r="D28" s="61" t="inlineStr">
         <is>
-          <t>Los jóvenes en situación de riesgo que tuvieron un mentor tuvieron 55 % más probabilidades de inscribirse en estudios superiores.</t>
+          <t>Los jóvenes en situación de riesgo que tuvieron un mentor estaban cursando estudios superiores con más frecuencia que los que no lo tuvieron: 45 % frente a 29 %.</t>
         </is>
       </c>
       <c r="E28" s="61" t="inlineStr">
         <is>
-          <t>MENTOR, The Mentoring Effect, 2014</t>
+          <t>MENTOR y Civic Enterprises, The Mentoring Effect, 2014</t>
         </is>
       </c>
       <c r="F28" s="61" t="inlineStr">
@@ -21133,12 +21133,12 @@
       </c>
       <c r="D29" s="61" t="inlineStr">
         <is>
-          <t>«Se necesitan 20 años para construir una reputación y cinco minutos para arruinarla.»</t>
+          <t>«Se necesitan 20 años para construir una reputación y cinco minutos para arruinarla»: la frase se le atribuye a Warren Buffett.</t>
         </is>
       </c>
       <c r="E29" s="61" t="inlineStr">
         <is>
-          <t>Warren Buffett, inversor estadounidense</t>
+          <t>Atribuida a Warren Buffett (Quote Investigator)</t>
         </is>
       </c>
       <c r="F29" s="61" t="inlineStr">
@@ -21203,7 +21203,7 @@
       </c>
       <c r="D30" s="61" t="inlineStr">
         <is>
-          <t>Al menos el 70 % de la diferencia en el compromiso de un equipo de trabajo depende de quien lo dirige.</t>
+          <t>Al menos el 70 % de la variación en el compromiso de los equipos de trabajo se explica por el jefe que los dirige.</t>
         </is>
       </c>
       <c r="E30" s="61" t="inlineStr">
@@ -21273,12 +21273,12 @@
       </c>
       <c r="D31" s="61" t="inlineStr">
         <is>
-          <t>La palabra «carácter» viene del griego y significaba la marca grabada en una moneda o en un sello.</t>
+          <t>La palabra «carácter» viene del griego, a través del latín, y significaba la marca grabada en una moneda o en un sello.</t>
         </is>
       </c>
       <c r="E31" s="61" t="inlineStr">
         <is>
-          <t>Diccionario etimológico de la lengua castellana (Corominas)</t>
+          <t>Diccionario de la lengua española (RAE), entrada «carácter»</t>
         </is>
       </c>
       <c r="F31" s="61" t="inlineStr">
@@ -21463,7 +21463,7 @@
       </c>
       <c r="D34" s="61" t="inlineStr">
         <is>
-          <t>Lavarse las manos con agua y jabón puede reducir entre un 23 y un 40 % las enfermedades diarreicas.</t>
+          <t>Enseñar en la comunidad a lavarse las manos con agua y jabón puede reducir entre un 23 y un 40 % los casos de diarrea.</t>
         </is>
       </c>
       <c r="E34" s="61" t="inlineStr">
@@ -21533,12 +21533,12 @@
       </c>
       <c r="D35" s="61" t="inlineStr">
         <is>
-          <t>En esponjas de cocina usadas se encontraron 362 tipos distintos de bacterias.</t>
+          <t>En 14 esponjas de cocina usadas se encontraron 362 tipos distintos de bacterias.</t>
         </is>
       </c>
       <c r="E35" s="61" t="inlineStr">
         <is>
-          <t>Cardinale y otros, Universidad de Furtwangen, Scientific Reports, 2017</t>
+          <t>Cardinale, Egert y otros, Universidad de Furtwangen y Universidad de Giessen, Scientific Reports, 2017</t>
         </is>
       </c>
       <c r="F35" s="61" t="inlineStr">
@@ -21673,7 +21673,7 @@
       </c>
       <c r="D37" s="61" t="inlineStr">
         <is>
-          <t>Comer en familia con frecuencia se asocia con una mejor alimentación y menos síntomas de depresión en niños y adolescentes.</t>
+          <t>Comer en familia con frecuencia se asocia con menos síntomas de depresión, menos conductas de riesgo y más autoestima en niños y adolescentes.</t>
         </is>
       </c>
       <c r="E37" s="61" t="inlineStr">
@@ -22003,7 +22003,7 @@
       </c>
       <c r="D42" s="61" t="inlineStr">
         <is>
-          <t>Muchas personas revisan menos sus cuentas justo cuando las cosas van mal; los investigadores lo llamaron «efecto avestruz».</t>
+          <t>Muchos inversores revisan sus cuentas con menos frecuencia cuando la bolsa baja que cuando sube; los investigadores lo llamaron «efecto avestruz».</t>
         </is>
       </c>
       <c r="E42" s="61" t="inlineStr">
@@ -22073,12 +22073,12 @@
       </c>
       <c r="D43" s="61" t="inlineStr">
         <is>
-          <t>La Torre de Pisa empezó a inclinarse en 1178, cuando iban por el segundo piso, por un suelo blando que no se había estudiado bien. Terminarla llevó casi 200 años.</t>
+          <t>La Torre de Pisa empezó a inclinarse hacia 1178, cuando la obra iba por el segundo piso: tenía un cimiento de apenas 3 metros sobre un suelo blando. Terminarla llevó casi 200 años, de 1173 a 1372.</t>
         </is>
       </c>
       <c r="E43" s="61" t="inlineStr">
         <is>
-          <t>Opera della Primaziale Pisana, Italia</t>
+          <t>Opera della Primaziale Pisana, historia de la Torre</t>
         </is>
       </c>
       <c r="F43" s="61" t="inlineStr">
@@ -22263,12 +22263,12 @@
       </c>
       <c r="D46" s="61" t="inlineStr">
         <is>
-          <t>Estudiantes que limitaron las redes sociales a 30 minutos por día durante tres semanas se sintieron menos solos y menos deprimidos.</t>
+          <t>Estudiantes que limitaron Facebook, Instagram y Snapchat a 10 minutos por día cada una, durante tres semanas, se sintieron menos solos y menos deprimidos que quienes siguieron igual.</t>
         </is>
       </c>
       <c r="E46" s="61" t="inlineStr">
         <is>
-          <t>Hunt y otros, Universidad de Pensilvania, Journal of Social and Clinical Psychology, 2018</t>
+          <t>Hunt, Marx, Lipson y Young, Universidad de Pensilvania, Journal of Social and Clinical Psychology, 2018</t>
         </is>
       </c>
       <c r="F46" s="61" t="inlineStr">
@@ -22403,12 +22403,12 @@
       </c>
       <c r="D48" s="61" t="inlineStr">
         <is>
-          <t>Se estima que unos 280 millones de personas en el mundo viven con depresión.</t>
+          <t>Más de 300 millones de personas en el mundo viven con depresión.</t>
         </is>
       </c>
       <c r="E48" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud</t>
+          <t>Organización Mundial de la Salud, nota descriptiva sobre la depresión</t>
         </is>
       </c>
       <c r="F48" s="61" t="inlineStr">
@@ -22473,7 +22473,7 @@
       </c>
       <c r="D49" s="61" t="inlineStr">
         <is>
-          <t>Escribir sobre lo que nos preocupa o nos dolió, entre 15 y 20 minutos durante unos pocos días seguidos, se asoció con mejor salud en los meses siguientes.</t>
+          <t>Escribir sobre algo que nos dolió, 15 minutos por día durante cuatro días seguidos, se asoció con menos visitas al médico en los meses siguientes.</t>
         </is>
       </c>
       <c r="E49" s="61" t="inlineStr">
@@ -22663,7 +22663,7 @@
       </c>
       <c r="D52" s="61" t="inlineStr">
         <is>
-          <t>El estrés del ganado antes de la faena oscurece la carne y la vuelve más dura: el buen trato también se nota en el plato.</t>
+          <t>El estrés del ganado antes de la faena puede oscurecer la carne, hacerla menos tierna y que dure menos: el buen trato también se nota en el plato.</t>
         </is>
       </c>
       <c r="E52" s="61" t="inlineStr">
@@ -22733,7 +22733,7 @@
       </c>
       <c r="D53" s="61" t="inlineStr">
         <is>
-          <t>Paraguay vacuna a todo su ganado bovino contra la fiebre aftosa en campañas que se repiten dos veces por año.</t>
+          <t>Paraguay vacuna contra la fiebre aftosa en dos períodos por año: en uno a todo el ganado bovino y en el otro a los animales jóvenes. La cobertura ronda el 99,7 %.</t>
         </is>
       </c>
       <c r="E53" s="61" t="inlineStr">
@@ -22873,12 +22873,12 @@
       </c>
       <c r="D55" s="61" t="inlineStr">
         <is>
-          <t>Las ovejas pueden reconocer y recordar las caras de al menos 50 ovejas, y también de personas, durante más de dos años.</t>
+          <t>Las ovejas pueden reconocer y recordar las caras de al menos 50 ovejas distintas durante más de dos años.</t>
         </is>
       </c>
       <c r="E55" s="61" t="inlineStr">
         <is>
-          <t>Kendrick y otros, revista Nature, 2001</t>
+          <t>Kendrick y otros, Instituto Babraham, revista Nature, 2001</t>
         </is>
       </c>
       <c r="F55" s="61" t="inlineStr">
@@ -22923,12 +22923,12 @@
       </c>
       <c r="D56" s="61" t="inlineStr">
         <is>
-          <t>Casi la mitad de los adultos con diabetes en el mundo (44 %) no sabe que la tiene.</t>
+          <t>Casi la mitad de los adultos con diabetes en el mundo (más del 40 %) no sabe que la tiene.</t>
         </is>
       </c>
       <c r="E56" s="61" t="inlineStr">
         <is>
-          <t>Federación Internacional de Diabetes, Atlas de la Diabetes, 2021</t>
+          <t>Federación Internacional de Diabetes, Atlas de la Diabetes, 2021 y 2025</t>
         </is>
       </c>
       <c r="F56" s="61" t="inlineStr">
@@ -23063,7 +23063,7 @@
       </c>
       <c r="D58" s="61" t="inlineStr">
         <is>
-          <t>Para los adultos, se recomienda medir la presión cada año desde los 40, y cada 3 a 5 años entre los 18 y los 39 si no hay factores de riesgo.</t>
+          <t>En Estados Unidos se recomienda medir la presión a todos los adultos: cada año desde los 40, y cada 3 a 5 años entre los 18 y los 39 si no hay factores de riesgo y la última medición fue normal.</t>
         </is>
       </c>
       <c r="E58" s="61" t="inlineStr">
@@ -23203,12 +23203,12 @@
       </c>
       <c r="D60" s="61" t="inlineStr">
         <is>
-          <t>Cuando el cáncer de mama se detecta en etapa temprana y se trata a tiempo, más del 90 % de las mujeres vive al menos cinco años más.</t>
+          <t>En los países donde el cáncer de mama se detecta temprano y se trata a tiempo, más del 90 % de las mujeres sigue con vida cinco años después del diagnóstico; en otros lugares, la cifra baja al 40 o 66 %.</t>
         </is>
       </c>
       <c r="E60" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, Iniciativa Mundial contra el Cáncer de Mama, 2023</t>
+          <t>Organización Mundial de la Salud, Iniciativa Mundial contra el Cáncer de Mama</t>
         </is>
       </c>
       <c r="F60" s="61" t="inlineStr">
@@ -23273,7 +23273,7 @@
       </c>
       <c r="D61" s="61" t="inlineStr">
         <is>
-          <t>Las Unidades de Salud de la Familia (USF) ofrecen atención primaria gratuita en todo el país.</t>
+          <t>Las Unidades de Salud de la Familia (USF) ofrecen atención primaria sin costo en todo el país.</t>
         </is>
       </c>
       <c r="E61" s="61" t="inlineStr">
@@ -23538,7 +23538,7 @@
       </c>
       <c r="E65" s="61" t="inlineStr">
         <is>
-          <t>Anatomía humana</t>
+          <t>Cleveland Clinic, «Muscle»</t>
         </is>
       </c>
       <c r="F65" s="61" t="inlineStr">
@@ -23678,7 +23678,7 @@
       </c>
       <c r="E67" s="61" t="inlineStr">
         <is>
-          <t>Diccionarios del griego del Nuevo Testamento</t>
+          <t>Léxico griego de Strong (G2842) y Thayer</t>
         </is>
       </c>
       <c r="F67" s="61" t="inlineStr">
@@ -23793,12 +23793,12 @@
       </c>
       <c r="D69" s="61" t="inlineStr">
         <is>
-          <t>Moisés atendía al pueblo «desde la mañana hasta la tarde», y su suegro le dijo: «No está bien lo que haces».</t>
+          <t>Moisés atendía al pueblo «desde la mañana hasta la tarde», y su suegro le advirtió que así se iba a agotar.</t>
         </is>
       </c>
       <c r="E69" s="61" t="inlineStr">
         <is>
-          <t>Éxodo 18:13-17</t>
+          <t>Éxodo 18:13-18 (RVC)</t>
         </is>
       </c>
       <c r="F69" s="61" t="inlineStr">
@@ -24008,7 +24008,7 @@
       </c>
       <c r="E72" s="61" t="inlineStr">
         <is>
-          <t>Léxicos del hebreo bíblico</t>
+          <t>Léxico hebreo de Strong (H2377) y Brown-Driver-Briggs</t>
         </is>
       </c>
       <c r="F72" s="61" t="inlineStr">
@@ -24073,12 +24073,12 @@
       </c>
       <c r="D73" s="61" t="inlineStr">
         <is>
-          <t>«Lo importante rara vez es urgente, y lo urgente rara vez es importante», dijo Dwight Eisenhower; de esa idea nació un método para ordenar tareas.</t>
+          <t>En 1954, ante el Consejo Mundial de Iglesias, Dwight Eisenhower citó a un antiguo rector: «Tengo dos clases de problemas, los urgentes y los importantes». De esa idea nació un método para ordenar tareas.</t>
         </is>
       </c>
       <c r="E73" s="61" t="inlineStr">
         <is>
-          <t>Dwight D. Eisenhower, discurso de 1954</t>
+          <t>Dwight D. Eisenhower, discurso en Evanston, 19 de agosto de 1954 (The American Presidency Project)</t>
         </is>
       </c>
       <c r="F73" s="61" t="inlineStr">
@@ -24193,17 +24193,17 @@
       </c>
       <c r="D75" s="61" t="inlineStr">
         <is>
-          <t>Justo antes de hablar a los esposos, Pablo les pide algo a todos: «Sométanse unos a otros en el temor de Dios».</t>
+          <t>Justo antes de hablar a los esposos, Pablo les pide algo a todos: «Cultiven entre ustedes la mutua sumisión, en el temor de Dios».</t>
         </is>
       </c>
       <c r="E75" s="61" t="inlineStr">
         <is>
-          <t>Efesios 5:21</t>
+          <t>Efesios 5:21 (RVC)</t>
         </is>
       </c>
       <c r="F75" s="61" t="inlineStr">
         <is>
-          <t>Pablo cierra el pasaje con dos verbos: el esposo ama a su esposa como a sí mismo, y la esposa honra a su esposo. Y antes de todo pidió algo para los dos: sométanse unos a otros (5:21).</t>
+          <t>Pablo cierra el pasaje con dos verbos: el esposo ama a su esposa como a sí mismo, y la esposa honra a su esposo. Y antes de todo pidió algo para los dos: cultivar la mutua sumisión (5:21).</t>
         </is>
       </c>
       <c r="G75" s="61" t="inlineStr">
@@ -24243,7 +24243,7 @@
       </c>
       <c r="N75" s="61" t="inlineStr">
         <is>
-          <t>Si vos o alguien que conocés sufre violencia, pedí ayuda: hablá con tu pastor y llamá a la línea 137 «SOS Mujer», que atiende las 24 horas.</t>
+          <t>Si vos o alguien que conocés sufre violencia, pedí ayuda: hablá con tu pastor y llamá a la línea 137 «SOS Mujer», gratuita y las 24 horas, o escribí al WhatsApp 0961 137 137. Si hay peligro inmediato, llamá al 911.</t>
         </is>
       </c>
     </row>
@@ -24263,7 +24263,7 @@
       </c>
       <c r="D76" s="61" t="inlineStr">
         <is>
-          <t>Personas que oraron por el bienestar de su pareja durante cuatro semanas mostraron más disposición a perdonar.</t>
+          <t>Personas que oraron cada día durante cuatro semanas por el bienestar de un amigo mostraron más disposición a perdonarlo que quienes oraron sobre otros temas o solo pensaron cosas positivas de él.</t>
         </is>
       </c>
       <c r="E76" s="61" t="inlineStr">
@@ -24408,7 +24408,7 @@
       </c>
       <c r="E78" s="61" t="inlineStr">
         <is>
-          <t>National Marriage Project, Universidad de Virginia, 2012</t>
+          <t>Wilcox y Dew, «The Date Night Opportunity», National Marriage Project, Universidad de Virginia, 2012</t>
         </is>
       </c>
       <c r="F78" s="61" t="inlineStr">
@@ -24506,6 +24506,1606 @@
       </c>
       <c r="M79" s="61" t="n"/>
       <c r="N79" s="61" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="B80" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C80" s="61" t="inlineStr">
+        <is>
+          <t>Firmes y constantes, también con la plata</t>
+        </is>
+      </c>
+      <c r="D80" s="61" t="inlineStr">
+        <is>
+          <t>Solo un tercio de los adultos del mundo entiende conceptos financieros básicos como el interés, la inflación o repartir el riesgo.</t>
+        </is>
+      </c>
+      <c r="E80" s="61" t="inlineStr">
+        <is>
+          <t>Klapper, Lusardi y van Oudheusden, Encuesta Global de Educación Financiera de S&amp;P, 2015</t>
+        </is>
+      </c>
+      <c r="F80" s="61" t="inlineStr">
+        <is>
+          <t>Pablo cierra su enseñanza sobre la resurrección con un llamado: manténganse firmes y constantes. Esa firmeza, que nace de la esperanza, también se nota en cómo administramos lo de todos los días.</t>
+        </is>
+      </c>
+      <c r="G80" s="61" t="inlineStr">
+        <is>
+          <t>Vivir con la plata «a ver qué pasa», sin saber cuánto entra ni cuánto sale.</t>
+        </is>
+      </c>
+      <c r="H80" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana anotá en una hoja tus ingresos del mes y tus gastos fijos. Ese es el comienzo de tu presupuesto.</t>
+        </is>
+      </c>
+      <c r="I80" s="61" t="inlineStr">
+        <is>
+          <t>Crecer en la obra del Señor incluye crecer en mayordomía: cuidar bien lo que Dios nos confía, sea poco o mucho.</t>
+        </is>
+      </c>
+      <c r="J80" s="61" t="inlineStr">
+        <is>
+          <t>Llegar a mitad de mes sin plata y no saber en qué se fue.</t>
+        </is>
+      </c>
+      <c r="K80" s="61" t="inlineStr">
+        <is>
+          <t>Compará lo que anotaste con lo que realmente gastaste el mes pasado: ahí aparecen las fugas.</t>
+        </is>
+      </c>
+      <c r="L80" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo hecho para el Señor no es en vano. Ordenar las finanzas no es frialdad: es cuidar a la familia y tener con qué ayudar a otros.</t>
+        </is>
+      </c>
+      <c r="M80" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que planificar la plata es cosa de ricos o de contadores.</t>
+        </is>
+      </c>
+      <c r="N80" s="61" t="inlineStr">
+        <is>
+          <t>Elegí con tu familia una meta concreta para este año y calculen cuánto deberían separar por mes para lograrla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="B81" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C81" s="61" t="inlineStr">
+        <is>
+          <t>Con calma y con plan</t>
+        </is>
+      </c>
+      <c r="D81" s="61" t="inlineStr">
+        <is>
+          <t>En una encuesta de Gallup en Estados Unidos, solo uno de cada tres hogares (32 %) dijo llevar un presupuesto detallado de sus ingresos y gastos.</t>
+        </is>
+      </c>
+      <c r="E81" s="61" t="inlineStr">
+        <is>
+          <t>Gallup, 2013</t>
+        </is>
+      </c>
+      <c r="F81" s="61" t="inlineStr">
+        <is>
+          <t>Este proverbio contrasta dos caminos: los planes del diligente llevan a la abundancia; el apuro, a la escasez. Es un principio de sabiduría, no una garantía: planificar no evita todos los problemas, pero ayuda a enfrentarlos.</t>
+        </is>
+      </c>
+      <c r="G81" s="61" t="inlineStr">
+        <is>
+          <t>Improvisar con la plata y descubrir el problema cuando ya llegó.</t>
+        </is>
+      </c>
+      <c r="H81" s="61" t="inlineStr">
+        <is>
+          <t>Así como antes de un viaje se calcula el combustible, calculá antes de que empiece el mes cuánto vas a necesitar para lo fijo.</t>
+        </is>
+      </c>
+      <c r="I81" s="61" t="inlineStr">
+        <is>
+          <t>El apuro sale caro: compras por impulso, préstamos rápidos, decisiones sin pensar.</t>
+        </is>
+      </c>
+      <c r="J81" s="61" t="inlineStr">
+        <is>
+          <t>Préstamos rápidos con intereses altísimos que se toman en un momento de apuro.</t>
+        </is>
+      </c>
+      <c r="K81" s="61" t="inlineStr">
+        <is>
+          <t>Antes de una compra grande o de un préstamo, esperá 48 horas y hacé las cuentas por escrito.</t>
+        </is>
+      </c>
+      <c r="L81" s="61" t="inlineStr">
+        <is>
+          <t>Planificar con calma no es desconfiar de Dios: es usar con sabiduría lo que Él nos da. El plan se hace orando.</t>
+        </is>
+      </c>
+      <c r="M81" s="61" t="inlineStr">
+        <is>
+          <t>Discusiones de pareja por la plata, por no planificar juntos.</t>
+        </is>
+      </c>
+      <c r="N81" s="61" t="inlineStr">
+        <is>
+          <t>Sentate con tu familia a revisar el presupuesto con calma, empezando con una oración.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="B82" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C82" s="61" t="inlineStr">
+        <is>
+          <t>Prudentes como serpientes</t>
+        </is>
+      </c>
+      <c r="D82" s="61" t="inlineStr">
+        <is>
+          <t>Un método conocido propone repartir el ingreso en 50 % para necesidades, 30 % para gustos y 20 % para ahorro o deudas; es una guía para empezar, no una ley.</t>
+        </is>
+      </c>
+      <c r="E82" s="61" t="inlineStr">
+        <is>
+          <t>Elizabeth Warren y Amelia Warren Tyagi, All Your Worth, 2005</t>
+        </is>
+      </c>
+      <c r="F82" s="61" t="inlineStr">
+        <is>
+          <t>Jesús envía a sus discípulos a una misión en medio de peligros y les pide prudencia. La prudencia sirve también en lo cotidiano: un presupuesto es una forma sencilla de prever.</t>
+        </is>
+      </c>
+      <c r="G82" s="61" t="inlineStr">
+        <is>
+          <t>Ofertas y cuotas que parecen convenientes y esconden costos.</t>
+        </is>
+      </c>
+      <c r="H82" s="61" t="inlineStr">
+        <is>
+          <t>Armá tu presupuesto en tres columnas: lo que entra, lo fijo que sale y lo variable. Con lápiz y papel alcanza.</t>
+        </is>
+      </c>
+      <c r="I82" s="61" t="inlineStr">
+        <is>
+          <t>Sencillos como palomas: sin doblez. Un presupuesto sencillo, que se entienda, funciona mejor que uno complicado que nadie sigue.</t>
+        </is>
+      </c>
+      <c r="J82" s="61" t="inlineStr">
+        <is>
+          <t>Planillas tan complicadas que se abandonan a la semana.</t>
+        </is>
+      </c>
+      <c r="K82" s="61" t="inlineStr">
+        <is>
+          <t>Empezá con pocas categorías: comida, casa, transporte, salud, iglesia y ayuda, ahorro e imprevistos.</t>
+        </is>
+      </c>
+      <c r="L82" s="61" t="inlineStr">
+        <is>
+          <t>La misión de los discípulos era anunciar el reino. Unas finanzas ordenadas también nos dejan libres para servir y para dar.</t>
+        </is>
+      </c>
+      <c r="M82" s="61" t="inlineStr">
+        <is>
+          <t>Familias tan ahogadas por las deudas que no pueden ayudar a nadie.</t>
+        </is>
+      </c>
+      <c r="N82" s="61" t="inlineStr">
+        <is>
+          <t>Dejá en tu presupuesto un margen para imprevistos y otro para ayudar a alguien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="B83" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C83" s="61" t="inlineStr">
+        <is>
+          <t>Vivir como sabios</t>
+        </is>
+      </c>
+      <c r="D83" s="61" t="inlineStr">
+        <is>
+          <t>En un experimento, las personas que pagaban con tarjeta ofrecieron pagar hasta el doble por las mismas entradas que las que pagaban en efectivo.</t>
+        </is>
+      </c>
+      <c r="E83" s="61" t="inlineStr">
+        <is>
+          <t>Prelec y Simester, MIT, Marketing Letters, 2001</t>
+        </is>
+      </c>
+      <c r="F83" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide vivir como sabios. La sabiduría bíblica es práctica: se ve en las decisiones de todos los días, también con la plata.</t>
+        </is>
+      </c>
+      <c r="G83" s="61" t="inlineStr">
+        <is>
+          <t>Usar la tarjeta sin llevar la cuenta y sorprenderse con el resumen.</t>
+        </is>
+      </c>
+      <c r="H83" s="61" t="inlineStr">
+        <is>
+          <t>Durante este mes, anotá cada gasto con tarjeta el mismo día que lo hacés.</t>
+        </is>
+      </c>
+      <c r="I83" s="61" t="inlineStr">
+        <is>
+          <t>«Cuidado con su manera de vivir»: los hábitos pequeños deciden el resultado del mes.</t>
+        </is>
+      </c>
+      <c r="J83" s="61" t="inlineStr">
+        <is>
+          <t>Gastos hormiga diarios que se comen el presupuesto sin que nadie lo note.</t>
+        </is>
+      </c>
+      <c r="K83" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un gasto diario que podés reducir esta semana y anotá cuánto ahorrás.</t>
+        </is>
+      </c>
+      <c r="L83" s="61" t="inlineStr">
+        <is>
+          <t>Aprovechar el tiempo también es revisar a tiempo: el presupuesto se mira cada semana, no cuando ya no alcanza.</t>
+        </is>
+      </c>
+      <c r="M83" s="61" t="inlineStr">
+        <is>
+          <t>Revisar las cuentas recién cuando llega el problema.</t>
+        </is>
+      </c>
+      <c r="N83" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un día fijo por semana para mirar tu presupuesto durante diez minutos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="B84" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C84" s="61" t="inlineStr">
+        <is>
+          <t>Según lo que cada uno ganó</t>
+        </is>
+      </c>
+      <c r="D84" s="61" t="inlineStr">
+        <is>
+          <t>La ofrenda que Pablo organizaba en Corinto era para los cristianos pobres de Jerusalén.</t>
+        </is>
+      </c>
+      <c r="E84" s="61" t="inlineStr">
+        <is>
+          <t>1 Corintios 16:1-3; Romanos 15:26</t>
+        </is>
+      </c>
+      <c r="F84" s="61" t="inlineStr">
+        <is>
+          <t>Pablo organiza una ofrenda para los hermanos pobres de Jerusalén y pide que cada uno aparte «según lo que haya ganado». La generosidad se ajusta a la realidad de cada uno: no es una cifra igual para todos.</t>
+        </is>
+      </c>
+      <c r="G84" s="61" t="inlineStr">
+        <is>
+          <t>Sentir culpa por no poder dar lo mismo que otros.</t>
+        </is>
+      </c>
+      <c r="H84" s="61" t="inlineStr">
+        <is>
+          <t>Incluí en tu presupuesto un monto para dar y ayudar, de acuerdo con lo que ganaste este mes.</t>
+        </is>
+      </c>
+      <c r="I84" s="61" t="inlineStr">
+        <is>
+          <t>«Cada primer día de la semana»: dar con constancia y con plan, no solo por impulso.</t>
+        </is>
+      </c>
+      <c r="J84" s="61" t="inlineStr">
+        <is>
+          <t>Ayudar solo cuando sobra, cuando casi nunca sobra.</t>
+        </is>
+      </c>
+      <c r="K84" s="61" t="inlineStr">
+        <is>
+          <t>Separá lo que vas a dar apenas cobrás, igual que separás el ahorro.</t>
+        </is>
+      </c>
+      <c r="L84" s="61" t="inlineStr">
+        <is>
+          <t>Cuando cambian los ingresos, el presupuesto se ajusta. Un presupuesto viejo que ya no refleja la realidad trae más problemas que soluciones.</t>
+        </is>
+      </c>
+      <c r="M84" s="61" t="inlineStr">
+        <is>
+          <t>Seguir gastando igual después de perder un ingreso o de sumar un gasto fijo nuevo.</t>
+        </is>
+      </c>
+      <c r="N84" s="61" t="inlineStr">
+        <is>
+          <t>Si este año cambió tu trabajo, tu familia o tus gastos, rehacé tu presupuesto esta semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="61" t="n">
+        <v>14</v>
+      </c>
+      <c r="B85" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C85" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: administradores confiables</t>
+        </is>
+      </c>
+      <c r="D85" s="61" t="inlineStr">
+        <is>
+          <t>La palabra que Pablo usa para «administrador» designaba al encargado de manejar los bienes de una casa que no era suya.</t>
+        </is>
+      </c>
+      <c r="E85" s="61" t="inlineStr">
+        <is>
+          <t>Diccionarios del griego del Nuevo Testamento (oikonómos)</t>
+        </is>
+      </c>
+      <c r="F85" s="61" t="inlineStr">
+        <is>
+          <t>Un presupuesto simple da visibilidad antes de que llegue el problema: es prudencia, no desconfianza.</t>
+        </is>
+      </c>
+      <c r="G85" s="61" t="n"/>
+      <c r="H85" s="61" t="inlineStr">
+        <is>
+          <t>Pablo habla de los que sirven administrando lo que Dios les confió: lo primero que se espera es que sean confiables. Lo mismo vale para lo que tenemos, que también es de Dios. Esta semana, sentate con tu familia y armen o ajusten su presupuesto del mes.</t>
+        </is>
+      </c>
+      <c r="I85" s="61" t="inlineStr">
+        <is>
+          <t>Para armarlo alcanza con anotar lo que entra y lo que sale, y dejar un margen para imprevistos y para dar.</t>
+        </is>
+      </c>
+      <c r="J85" s="61" t="n"/>
+      <c r="K85" s="61" t="n"/>
+      <c r="L85" s="61" t="inlineStr">
+        <is>
+          <t>El presupuesto se ajusta cuando cambia la realidad: se revisa, no se idolatra.</t>
+        </is>
+      </c>
+      <c r="M85" s="61" t="n"/>
+      <c r="N85" s="61" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="B86" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C86" s="61" t="inlineStr">
+        <is>
+          <t>Un fruto que no se fabrica</t>
+        </is>
+      </c>
+      <c r="D86" s="61" t="inlineStr">
+        <is>
+          <t>En griego, Pablo dice «el fruto» en singular: no son nueve frutos separados, sino un solo fruto con nueve rasgos.</t>
+        </is>
+      </c>
+      <c r="E86" s="61" t="inlineStr">
+        <is>
+          <t>Texto griego de Gálatas 5:22</t>
+        </is>
+      </c>
+      <c r="F86" s="61" t="inlineStr">
+        <is>
+          <t>Pablo contrasta las obras de la carne con el fruto del Espíritu. El fruto no se fabrica a fuerza de voluntad: lo produce el Espíritu en quien está unido a Cristo.</t>
+        </is>
+      </c>
+      <c r="G86" s="61" t="inlineStr">
+        <is>
+          <t>Una fe que se reduce a cumplir con actividades, sin cambios en el carácter.</t>
+        </is>
+      </c>
+      <c r="H86" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, antes de cada actividad de la iglesia, pedile a Dios que te cambie a vos, no solo que te ayude a cumplir.</t>
+        </is>
+      </c>
+      <c r="I86" s="61" t="inlineStr">
+        <is>
+          <t>Como todo fruto, necesita tiempo. No hay atajos ni fórmulas: hay permanencia en Cristo.</t>
+        </is>
+      </c>
+      <c r="J86" s="61" t="inlineStr">
+        <is>
+          <t>La frustración de no ver cambios rápidos en uno mismo.</t>
+        </is>
+      </c>
+      <c r="K86" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un rasgo del fruto (paciencia, mansedumbre…) que querés ver crecer y orá por él cada día de esta semana.</t>
+        </is>
+      </c>
+      <c r="L86" s="61" t="inlineStr">
+        <is>
+          <t>El crecimiento real se nota en cómo tratamos a los demás, no solo en cuántas reuniones asistimos.</t>
+        </is>
+      </c>
+      <c r="M86" s="61" t="inlineStr">
+        <is>
+          <t>Personas muy activas en la iglesia, pero ásperas en casa o en el trabajo.</t>
+        </is>
+      </c>
+      <c r="N86" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale a alguien de tu familia: ¿en qué notás que crecí este año? Escuchá sin defenderte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="B87" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C87" s="61" t="inlineStr">
+        <is>
+          <t>Sed de Dios</t>
+        </is>
+      </c>
+      <c r="D87" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 63 lleva como título: «Salmo de David, cuando estaba en el desierto de Judá».</t>
+        </is>
+      </c>
+      <c r="E87" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 63, título</t>
+        </is>
+      </c>
+      <c r="F87" s="61" t="inlineStr">
+        <is>
+          <t>David escribe en el desierto, lejos de todo. No busca solo bendiciones: busca a Dios mismo.</t>
+        </is>
+      </c>
+      <c r="G87" s="61" t="inlineStr">
+        <is>
+          <t>Una relación con Dios que se limita a pedir cosas.</t>
+        </is>
+      </c>
+      <c r="H87" s="61" t="inlineStr">
+        <is>
+          <t>Hoy dedicá un momento a orar sin pedir nada: solo agradecer y estar con Dios.</t>
+        </is>
+      </c>
+      <c r="I87" s="61" t="inlineStr">
+        <is>
+          <t>«Te buscaré de madrugada»: buscar a Dios temprano es una forma de decir que va primero. No es una regla de horario, es una prioridad.</t>
+        </is>
+      </c>
+      <c r="J87" s="61" t="inlineStr">
+        <is>
+          <t>Días que arrancan con el celular y las noticias, sin un minuto para Dios.</t>
+        </is>
+      </c>
+      <c r="K87" s="61" t="inlineStr">
+        <is>
+          <t>Mañana, antes de mirar el celular, dedicá cinco minutos a leer un salmo y orar.</t>
+        </is>
+      </c>
+      <c r="L87" s="61" t="inlineStr">
+        <is>
+          <t>Hay una sed que ninguna cosa llena: ni el éxito, ni la comida, ni las compras. Solo Dios sacia el alma.</t>
+        </is>
+      </c>
+      <c r="M87" s="61" t="inlineStr">
+        <is>
+          <t>Llenar el vacío con actividades, compras o pantallas.</t>
+        </is>
+      </c>
+      <c r="N87" s="61" t="inlineStr">
+        <is>
+          <t>Fijate qué usás para llenar el vacío cuando estás mal, y esta semana cambialo por un rato a solas con Dios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="B88" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C88" s="61" t="inlineStr">
+        <is>
+          <t>Los que esperan en el Señor</t>
+        </is>
+      </c>
+      <c r="D88" s="61" t="inlineStr">
+        <is>
+          <t>Las águilas aprovechan las corrientes de aire caliente para subir y planear durante largos tramos casi sin aletear, ahorrando energía.</t>
+        </is>
+      </c>
+      <c r="E88" s="61" t="inlineStr">
+        <is>
+          <t>Estudios sobre el vuelo de aves planeadoras</t>
+        </is>
+      </c>
+      <c r="F88" s="61" t="inlineStr">
+        <is>
+          <t>Isaías habla a un pueblo cansado: los que confían en el Señor recobran las fuerzas. Las disciplinas espirituales son una forma de esperar en Él: no para ganar fuerzas, sino para recibirlas.</t>
+        </is>
+      </c>
+      <c r="G88" s="61" t="inlineStr">
+        <is>
+          <t>El agotamiento espiritual de quienes sirven mucho y se alimentan poco.</t>
+        </is>
+      </c>
+      <c r="H88" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una sola disciplina para esta semana (oración, lectura o silencio) y dale un horario fijo.</t>
+        </is>
+      </c>
+      <c r="I88" s="61" t="inlineStr">
+        <is>
+          <t>El cansancio espiritual no es pecado ni fracaso: es una señal de que necesitamos volver a la fuente.</t>
+        </is>
+      </c>
+      <c r="J88" s="61" t="inlineStr">
+        <is>
+          <t>Personas que se sienten culpables por estar cansadas en la fe.</t>
+        </is>
+      </c>
+      <c r="K88" s="61" t="inlineStr">
+        <is>
+          <t>Si estás cansado, decíselo a Dios con sinceridad. Eso también es oración.</t>
+        </is>
+      </c>
+      <c r="L88" s="61" t="inlineStr">
+        <is>
+          <t>La imagen es poética: no promete que nunca nos vamos a cansar, sino que Dios da fuerzas nuevas para seguir.</t>
+        </is>
+      </c>
+      <c r="M88" s="61" t="inlineStr">
+        <is>
+          <t>Querer hacerlo todo con las propias fuerzas, sin descanso.</t>
+        </is>
+      </c>
+      <c r="N88" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, cambiá una actividad por un tiempo de descanso y oración.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="B89" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C89" s="61" t="inlineStr">
+        <is>
+          <t>Crecer en gracia y conocimiento</t>
+        </is>
+      </c>
+      <c r="D89" s="61" t="inlineStr">
+        <is>
+          <t>Repasar en sesiones cortas y repartidas en el tiempo se recuerda mejor que estudiar todo de una vez.</t>
+        </is>
+      </c>
+      <c r="E89" s="61" t="inlineStr">
+        <is>
+          <t>Cepeda y otros, Psychological Bulletin, 2006</t>
+        </is>
+      </c>
+      <c r="F89" s="61" t="inlineStr">
+        <is>
+          <t>Pedro pide crecer en dos cosas juntas: en la gracia, que recibimos sin merecerla, y en el conocimiento de Jesús. Una sin la otra se desequilibra.</t>
+        </is>
+      </c>
+      <c r="G89" s="61" t="inlineStr">
+        <is>
+          <t>Mucho conocimiento de la Biblia sin amor, o mucho sentimiento sin conocer la Palabra.</t>
+        </is>
+      </c>
+      <c r="H89" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, a lo que leas sumale una pregunta: ¿qué me muestra esto de la gracia de Jesús?</t>
+        </is>
+      </c>
+      <c r="I89" s="61" t="inlineStr">
+        <is>
+          <t>El crecimiento es un proceso de todos los días. Las disciplinas son como el riego: poco y seguido rinde más que mucho de vez en cuando.</t>
+        </is>
+      </c>
+      <c r="J89" s="61" t="inlineStr">
+        <is>
+          <t>Las rachas de entusiasmo que duran una semana y después desaparecen.</t>
+        </is>
+      </c>
+      <c r="K89" s="61" t="inlineStr">
+        <is>
+          <t>Elegí diez minutos diarios para una disciplina y mantenelos toda la semana.</t>
+        </is>
+      </c>
+      <c r="L89" s="61" t="inlineStr">
+        <is>
+          <t>Nadie llega a una madurez completa en esta vida. Eso nos libra del orgullo y también de la desesperación.</t>
+        </is>
+      </c>
+      <c r="M89" s="61" t="inlineStr">
+        <is>
+          <t>Creer que ya sabemos lo suficiente, o que nunca vamos a cambiar.</t>
+        </is>
+      </c>
+      <c r="N89" s="61" t="inlineStr">
+        <is>
+          <t>Buscá a alguien más maduro en la fe y preguntale qué lo ayudó a crecer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="B90" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C90" s="61" t="inlineStr">
+        <is>
+          <t>Cuando el alma tiene sed</t>
+        </is>
+      </c>
+      <c r="D90" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 42 se atribuye a los hijos de Coré, una familia de levitas cantores del templo.</t>
+        </is>
+      </c>
+      <c r="E90" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 42, título</t>
+        </is>
+      </c>
+      <c r="F90" s="61" t="inlineStr">
+        <is>
+          <t>El salmista tiene sed de Dios como un ciervo busca agua, y lo dice en un momento de tristeza: «¿Por qué te abates, alma mía?» (42:5).</t>
+        </is>
+      </c>
+      <c r="G90" s="61" t="inlineStr">
+        <is>
+          <t>Etapas en las que orar cuesta y Dios parece lejos.</t>
+        </is>
+      </c>
+      <c r="H90" s="61" t="inlineStr">
+        <is>
+          <t>Si estás en una etapa así, leé el Salmo 42 completo: alguien ya oró lo que vos sentís.</t>
+        </is>
+      </c>
+      <c r="I90" s="61" t="inlineStr">
+        <is>
+          <t>La sequía espiritual es normal en la vida de fe: la vivieron David, Elías y muchos creyentes. No es señal de falta de fe.</t>
+        </is>
+      </c>
+      <c r="J90" s="61" t="inlineStr">
+        <is>
+          <t>La culpa de quien siente que su fe se enfrió.</t>
+        </is>
+      </c>
+      <c r="K90" s="61" t="inlineStr">
+        <is>
+          <t>Seguí buscando a Dios aunque no sientas nada: leé, orá, cantá. La fe no depende de lo que sentimos.</t>
+        </is>
+      </c>
+      <c r="L90" s="61" t="inlineStr">
+        <is>
+          <t>El salmista termina con esperanza: «Espera en Dios, porque aún he de alabarle» (42:5). En la sequía también se construye una fe sólida.</t>
+        </is>
+      </c>
+      <c r="M90" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar la iglesia o la oración en el momento más seco.</t>
+        </is>
+      </c>
+      <c r="N90" s="61" t="inlineStr">
+        <is>
+          <t>Contale a alguien de confianza que estás en una etapa seca y pedile que ore por vos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="B91" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C91" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: crecer con raíces</t>
+        </is>
+      </c>
+      <c r="D91" s="61" t="inlineStr">
+        <is>
+          <t>En este versículo Pablo combina dos imágenes: la de una planta que echa raíces y la de un edificio que se levanta sobre cimientos.</t>
+        </is>
+      </c>
+      <c r="E91" s="61" t="inlineStr">
+        <is>
+          <t>Colosenses 2:7</t>
+        </is>
+      </c>
+      <c r="F91" s="61" t="inlineStr">
+        <is>
+          <t>Crecer no es solo cumplir con actividades: el fruto del Espíritu se nota en el carácter.</t>
+        </is>
+      </c>
+      <c r="G91" s="61" t="n"/>
+      <c r="H91" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una disciplina para la próxima semana y escribí cuándo y dónde la vas a practicar.</t>
+        </is>
+      </c>
+      <c r="I91" s="61" t="inlineStr">
+        <is>
+          <t>Las disciplinas (oración, lectura, silencio) no ganan el amor de Dios: nos ponen en el lugar para recibir su gracia.</t>
+        </is>
+      </c>
+      <c r="J91" s="61" t="n"/>
+      <c r="K91" s="61" t="n"/>
+      <c r="L91" s="61" t="inlineStr">
+        <is>
+          <t>En la sequía también se crece: seguir buscando a Dios aunque no se sienta nada es fe.</t>
+        </is>
+      </c>
+      <c r="M91" s="61" t="n"/>
+      <c r="N91" s="61" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="B92" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C92" s="61" t="inlineStr">
+        <is>
+          <t>Quién da la capacidad de producir</t>
+        </is>
+      </c>
+      <c r="D92" s="61" t="inlineStr">
+        <is>
+          <t>Las micro, pequeñas y medianas empresas son más del 90 % de las empresas de Paraguay.</t>
+        </is>
+      </c>
+      <c r="E92" s="61" t="inlineStr">
+        <is>
+          <t>Ministerio de Industria y Comercio (MIC) del Paraguay</t>
+        </is>
+      </c>
+      <c r="F92" s="61" t="inlineStr">
+        <is>
+          <t>Moisés le recuerda a Israel, antes de entrar a la tierra, que cuando le vaya bien no se olvide de Dios: es Él quien da la capacidad de producir. El texto no promete riqueza; advierte contra el orgullo.</t>
+        </is>
+      </c>
+      <c r="G92" s="61" t="inlineStr">
+        <is>
+          <t>Empresarios que creen que todo lo lograron solos y se olvidan de Dios y de su gente.</t>
+        </is>
+      </c>
+      <c r="H92" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un negocio, agradecé a Dios esta semana por lo que te permitió construir, y a la gente que trabaja con vos.</t>
+        </is>
+      </c>
+      <c r="I92" s="61" t="inlineStr">
+        <is>
+          <t>Ningún negocio se hace solo: detrás hay empleados, clientes, proveedores y una comunidad.</t>
+        </is>
+      </c>
+      <c r="J92" s="61" t="inlineStr">
+        <is>
+          <t>Ver a los empleados solo como un costo.</t>
+        </is>
+      </c>
+      <c r="K92" s="61" t="inlineStr">
+        <is>
+          <t>Reconocé esta semana, en público, el trabajo de alguien de tu equipo.</t>
+        </is>
+      </c>
+      <c r="L92" s="61" t="inlineStr">
+        <is>
+          <t>Reconocer que todo viene de Dios cambia cómo usamos lo que ganamos: generar trabajo digno es una forma de administrar ese don.</t>
+        </is>
+      </c>
+      <c r="M92" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo informal, sin seguro ni aguinaldo, que deja a familias desprotegidas.</t>
+        </is>
+      </c>
+      <c r="N92" s="61" t="inlineStr">
+        <is>
+          <t>Si das empleo, revisá que tu gente tenga lo que la ley establece: seguro social, aguinaldo y salario a tiempo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="B93" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C93" s="61" t="inlineStr">
+        <is>
+          <t>El que hace bien su trabajo</t>
+        </is>
+      </c>
+      <c r="D93" s="61" t="inlineStr">
+        <is>
+          <t>Los equipos de trabajo más comprometidos logran resultados mejores: en los análisis de Gallup, alrededor de un 23 % más de rentabilidad.</t>
+        </is>
+      </c>
+      <c r="E93" s="61" t="inlineStr">
+        <is>
+          <t>Gallup, State of the Global Workplace, 2023</t>
+        </is>
+      </c>
+      <c r="F93" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio observa que el trabajo bien hecho abre puertas, incluso ante reyes. Es un principio general, no una promesa de éxito para todos.</t>
+        </is>
+      </c>
+      <c r="G93" s="61" t="inlineStr">
+        <is>
+          <t>La cultura del «más o menos» que hace perder clientes.</t>
+        </is>
+      </c>
+      <c r="H93" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una tarea de tu trabajo y hacela esta semana con un detalle de excelencia extra.</t>
+        </is>
+      </c>
+      <c r="I93" s="61" t="inlineStr">
+        <is>
+          <t>La excelencia no es perfeccionismo: es hacer bien lo que corresponde, y a tiempo.</t>
+        </is>
+      </c>
+      <c r="J93" s="61" t="inlineStr">
+        <is>
+          <t>Jóvenes que no consiguen trabajo y no saben cómo destacarse.</t>
+        </is>
+      </c>
+      <c r="K93" s="61" t="inlineStr">
+        <is>
+          <t>Si buscás trabajo, sumá una capacitación gratuita (por ejemplo, del SNPP) y presentate siempre puntual.</t>
+        </is>
+      </c>
+      <c r="L93" s="61" t="inlineStr">
+        <is>
+          <t>Una empresa que genera trabajo digno necesita gente que trabaje bien y líderes que lo reconozcan.</t>
+        </is>
+      </c>
+      <c r="M93" s="61" t="inlineStr">
+        <is>
+          <t>Buenos trabajadores que se van porque nadie valora su esfuerzo.</t>
+        </is>
+      </c>
+      <c r="N93" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés gente a cargo, decile esta semana a un trabajador concreto qué hace bien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="B94" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C94" s="61" t="inlineStr">
+        <is>
+          <t>Disfrutar el fruto del trabajo</t>
+        </is>
+      </c>
+      <c r="D94" s="61" t="inlineStr">
+        <is>
+          <t>En un estudio con miles de empleados públicos británicos, quienes sentían que su jefe los trataba con justicia tuvieron menos enfermedades del corazón en los años siguientes.</t>
+        </is>
+      </c>
+      <c r="E94" s="61" t="inlineStr">
+        <is>
+          <t>Kivimäki y otros, estudio Whitehall II, Archives of Internal Medicine, 2005</t>
+        </is>
+      </c>
+      <c r="F94" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés, que tantas veces habla de lo pasajero, reconoce algo bueno: disfrutar del fruto del trabajo es un regalo de Dios.</t>
+        </is>
+      </c>
+      <c r="G94" s="61" t="inlineStr">
+        <is>
+          <t>Empresas que exigen tanto que nadie, ni siquiera el dueño, disfruta lo que hace.</t>
+        </is>
+      </c>
+      <c r="H94" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, festejá con tu equipo o con tu familia un logro del trabajo, aunque sea pequeño.</t>
+        </is>
+      </c>
+      <c r="I94" s="61" t="inlineStr">
+        <is>
+          <t>Si es un don, no se consigue a cualquier precio. La integridad en la gestión (pagar a tiempo, ser transparente) es parte de recibir bien ese don.</t>
+        </is>
+      </c>
+      <c r="J94" s="61" t="inlineStr">
+        <is>
+          <t>Atrasos en el pago a empleados y proveedores mientras el dueño gasta en lujos.</t>
+        </is>
+      </c>
+      <c r="K94" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un negocio, revisá esta semana que tus pagos a empleados y proveedores estén al día.</t>
+        </is>
+      </c>
+      <c r="L94" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar con gozo y honestidad es una forma de agradecer a Dios.</t>
+        </is>
+      </c>
+      <c r="M94" s="61" t="inlineStr">
+        <is>
+          <t>La queja constante sobre el trabajo, en la casa y en las redes.</t>
+        </is>
+      </c>
+      <c r="N94" s="61" t="inlineStr">
+        <is>
+          <t>Hoy agradecé a Dios por tu trabajo, aunque no sea el ideal, y nombrá una cosa buena que tiene.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="B95" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C95" s="61" t="inlineStr">
+        <is>
+          <t>La confianza que sostiene</t>
+        </is>
+      </c>
+      <c r="D95" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías 17 compara dos plantas: el que confía en el ser humano es como una zarza en el desierto; el que confía en el Señor, como un árbol junto al agua.</t>
+        </is>
+      </c>
+      <c r="E95" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías 17:5-8</t>
+        </is>
+      </c>
+      <c r="F95" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías contrasta al que confía en el ser humano con el que confía en el Señor: uno es como una zarza en el desierto; el otro, como un árbol plantado junto al agua (17:5-8).</t>
+        </is>
+      </c>
+      <c r="G95" s="61" t="inlineStr">
+        <is>
+          <t>Negocios que buscan la ganancia a cualquier costo, porque toda su seguridad está en la plata.</t>
+        </is>
+      </c>
+      <c r="H95" s="61" t="inlineStr">
+        <is>
+          <t>Antes de una decisión de trabajo difícil, preguntate: ¿esto lo haría si confiara de verdad en Dios?</t>
+        </is>
+      </c>
+      <c r="I95" s="61" t="inlineStr">
+        <is>
+          <t>Confiar en Dios libera de los atajos: no necesitamos mentir ni engañar para estar seguros.</t>
+        </is>
+      </c>
+      <c r="J95" s="61" t="inlineStr">
+        <is>
+          <t>Facturas falsas, evasión y «arreglos» que se ven como normales en algunos negocios.</t>
+        </is>
+      </c>
+      <c r="K95" s="61" t="inlineStr">
+        <is>
+          <t>Si en tu trabajo hay una práctica deshonesta que se volvió costumbre, empezá a corregirla esta semana.</t>
+        </is>
+      </c>
+      <c r="L95" s="61" t="inlineStr">
+        <is>
+          <t>La bendición del que confía no es no tener problemas: el árbol junto al agua también pasa por la sequía, pero no deja de dar fruto (17:8).</t>
+        </is>
+      </c>
+      <c r="M95" s="61" t="inlineStr">
+        <is>
+          <t>Crisis económicas que desaniman a los emprendedores.</t>
+        </is>
+      </c>
+      <c r="N95" s="61" t="inlineStr">
+        <is>
+          <t>Si tu negocio atraviesa una crisis, compartilo con alguien de confianza y oren juntos pidiendo sabiduría.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="B96" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C96" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar como para el Señor</t>
+        </is>
+      </c>
+      <c r="D96" s="61" t="inlineStr">
+        <is>
+          <t>En Paraguay, más de seis de cada diez personas ocupadas trabajan en la informalidad.</t>
+        </is>
+      </c>
+      <c r="E96" s="61" t="inlineStr">
+        <is>
+          <t>Instituto Nacional de Estadística (INE), Encuesta Permanente de Hogares Continua</t>
+        </is>
+      </c>
+      <c r="F96" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribe esto a esclavos, gente sin poder ni reconocimiento: su trabajo tenía dignidad porque lo hacían para el Señor. Ningún trabajo honesto es poca cosa.</t>
+        </is>
+      </c>
+      <c r="G96" s="61" t="inlineStr">
+        <is>
+          <t>Personas que sienten que su trabajo no vale nada.</t>
+        </is>
+      </c>
+      <c r="H96" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, al empezar a trabajar, dedicale tu trabajo a Dios con una oración corta.</t>
+        </is>
+      </c>
+      <c r="I96" s="61" t="inlineStr">
+        <is>
+          <t>Si la recompensa final viene de Dios, no hace falta buscar la aprobación de todos ni tomar atajos para destacarse.</t>
+        </is>
+      </c>
+      <c r="J96" s="61" t="inlineStr">
+        <is>
+          <t>Empresas que cumplen solo cuando hay control o inspección.</t>
+        </is>
+      </c>
+      <c r="K96" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un negocio, cumplí esta semana con algo que nadie te exige, pero que cuida a tu gente o a tus clientes.</t>
+        </is>
+      </c>
+      <c r="L96" s="61" t="inlineStr">
+        <is>
+          <t>Una empresa sana, con trabajo bien hecho y trato justo, es un motor para su comunidad: da empleo, compra a proveedores locales y es ejemplo para otros.</t>
+        </is>
+      </c>
+      <c r="M96" s="61" t="inlineStr">
+        <is>
+          <t>Comercios que cierran y dejan a familias sin ingreso.</t>
+        </is>
+      </c>
+      <c r="N96" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana comprá en un negocio pequeño y honesto de tu barrio, y decile al dueño que valorás su trabajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="61" t="n">
+        <v>16</v>
+      </c>
+      <c r="B97" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C97" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: la obra de nuestras manos</t>
+        </is>
+      </c>
+      <c r="D97" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 90 se atribuye a Moisés: es el único salmo que lleva su nombre en el título.</t>
+        </is>
+      </c>
+      <c r="E97" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 90, título</t>
+        </is>
+      </c>
+      <c r="F97" s="61" t="inlineStr">
+        <is>
+          <t>Una empresa que da trabajo digno sostiene familias enteras, y reconocer de dónde viene la capacidad de producir evita el orgullo.</t>
+        </is>
+      </c>
+      <c r="G97" s="61" t="n"/>
+      <c r="H97" s="61" t="inlineStr">
+        <is>
+          <t>Como Moisés, pidan juntos que Dios confirme la obra de sus manos, y reconozcan esta semana a un negocio local que da trabajo digno.</t>
+        </is>
+      </c>
+      <c r="I97" s="61" t="inlineStr">
+        <is>
+          <t>La integridad en la gestión (pagar a tiempo, tratar bien, ser transparente) vale más que cualquier atajo.</t>
+        </is>
+      </c>
+      <c r="J97" s="61" t="n"/>
+      <c r="K97" s="61" t="n"/>
+      <c r="L97" s="61" t="inlineStr">
+        <is>
+          <t>Un negocio sano y honesto es un motor para su comunidad.</t>
+        </is>
+      </c>
+      <c r="M97" s="61" t="n"/>
+      <c r="N97" s="61" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="61" t="n">
+        <v>17</v>
+      </c>
+      <c r="B98" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C98" s="61" t="inlineStr">
+        <is>
+          <t>Correr con propósito</t>
+        </is>
+      </c>
+      <c r="D98" s="61" t="inlineStr">
+        <is>
+          <t>La Organización Mundial de la Salud recomienda a los adultos al menos 150 minutos por semana de actividad física moderada.</t>
+        </is>
+      </c>
+      <c r="E98" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Directrices sobre actividad física, 2020</t>
+        </is>
+      </c>
+      <c r="F98" s="61" t="inlineStr">
+        <is>
+          <t>Pablo usa la imagen de los juegos atléticos, muy conocidos en Corinto, para hablar de la vida cristiana: correr con propósito. La imagen también nos recuerda que el cuerpo fue hecho para moverse.</t>
+        </is>
+      </c>
+      <c r="G98" s="61" t="inlineStr">
+        <is>
+          <t>Pasar casi todo el día sentado, en el trabajo y en la casa.</t>
+        </is>
+      </c>
+      <c r="H98" s="61" t="inlineStr">
+        <is>
+          <t>Sumá hoy una caminata de diez minutos después de una comida.</t>
+        </is>
+      </c>
+      <c r="I98" s="61" t="inlineStr">
+        <is>
+          <t>Los atletas se disciplinan por una corona que se marchita; nosotros vivimos para algo eterno. El cuidado del cuerpo es parte de una vida ordenada, no un fin en sí mismo.</t>
+        </is>
+      </c>
+      <c r="J98" s="61" t="inlineStr">
+        <is>
+          <t>La obsesión por la imagen, que lleva a dietas y ejercicios extremos.</t>
+        </is>
+      </c>
+      <c r="K98" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un movimiento que disfrutes (caminar, andar en bicicleta, jugar a la pelota con los chicos) y hacelo tres veces esta semana.</t>
+        </is>
+      </c>
+      <c r="L98" s="61" t="inlineStr">
+        <is>
+          <t>Los beneficios del movimiento se suman de a poco: más vale ser constante que intenso.</t>
+        </is>
+      </c>
+      <c r="M98" s="61" t="inlineStr">
+        <is>
+          <t>Empezar con todo y abandonar a la semana.</t>
+        </is>
+      </c>
+      <c r="N98" s="61" t="inlineStr">
+        <is>
+          <t>Proponete 15 minutos diarios de movimiento durante esta semana, sin buscar más.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="61" t="n">
+        <v>17</v>
+      </c>
+      <c r="B99" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C99" s="61" t="inlineStr">
+        <is>
+          <t>Dominio propio</t>
+        </is>
+      </c>
+      <c r="D99" s="61" t="inlineStr">
+        <is>
+          <t>Cortar los ratos largos sentado con pausas cortas de movimiento ayudó a controlar el azúcar en sangre después de comer.</t>
+        </is>
+      </c>
+      <c r="E99" s="61" t="inlineStr">
+        <is>
+          <t>Dunstan y otros, Diabetes Care, 2012</t>
+        </is>
+      </c>
+      <c r="F99" s="61" t="inlineStr">
+        <is>
+          <t>Pablo habla de su ministerio: se disciplina para no quedar descalificado después de predicar a otros. «Golpear el cuerpo» es una imagen de dominio propio, no una invitación a lastimarse.</t>
+        </is>
+      </c>
+      <c r="G99" s="61" t="inlineStr">
+        <is>
+          <t>Las buenas intenciones que nunca pasan de la intención.</t>
+        </is>
+      </c>
+      <c r="H99" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un hábito de movimiento y anotá cada día si lo cumpliste.</t>
+        </is>
+      </c>
+      <c r="I99" s="61" t="inlineStr">
+        <is>
+          <t>El dominio propio es fruto del Espíritu (Gálatas 5:23): no se logra solo con fuerza de voluntad, pero sí se ejercita.</t>
+        </is>
+      </c>
+      <c r="J99" s="61" t="inlineStr">
+        <is>
+          <t>Pasar horas frente a la pantalla sin darse cuenta.</t>
+        </is>
+      </c>
+      <c r="K99" s="61" t="inlineStr">
+        <is>
+          <t>Cada hora que estés sentado, levantate y caminá dos o tres minutos.</t>
+        </is>
+      </c>
+      <c r="L99" s="61" t="inlineStr">
+        <is>
+          <t>Así como el cuerpo se entrena, también se entrena la decisión de cuidarse: de a poco y con ayuda.</t>
+        </is>
+      </c>
+      <c r="M99" s="61" t="inlineStr">
+        <is>
+          <t>Pensar «ya es tarde para mí» y no empezar.</t>
+        </is>
+      </c>
+      <c r="N99" s="61" t="inlineStr">
+        <is>
+          <t>Si hace mucho que no hacés ejercicio, consultá antes a tu médico y empezá con caminatas cortas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="61" t="n">
+        <v>17</v>
+      </c>
+      <c r="B100" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C100" s="61" t="inlineStr">
+        <is>
+          <t>Correr con paciencia</t>
+        </is>
+      </c>
+      <c r="D100" s="61" t="inlineStr">
+        <is>
+          <t>Reemplazar tiempo sentado por 15 minutos de correr o una hora de caminata por día se asoció con un 26 % menos de riesgo de depresión.</t>
+        </is>
+      </c>
+      <c r="E100" s="61" t="inlineStr">
+        <is>
+          <t>Choi y otros, JAMA Psychiatry, 2019</t>
+        </is>
+      </c>
+      <c r="F100" s="61" t="inlineStr">
+        <is>
+          <t>La carta usa la imagen de una carrera larga, rodeados por los creyentes que nos precedieron. No es una carrera de velocidad: es de resistencia.</t>
+        </is>
+      </c>
+      <c r="G100" s="61" t="inlineStr">
+        <is>
+          <t>El estrés acumulado que no encuentra salida.</t>
+        </is>
+      </c>
+      <c r="H100" s="61" t="inlineStr">
+        <is>
+          <t>Cuando sientas tensión, salí a caminar 15 minutos: le hace bien al cuerpo y a la mente.</t>
+        </is>
+      </c>
+      <c r="I100" s="61" t="inlineStr">
+        <is>
+          <t>Para correr hay que soltar lo que pesa. En la fe, lo que nos frena es el pecado y las cargas innecesarias. En el cuidado del cuerpo, salvando las distancias, lo que más frena es la falta de movimiento.</t>
+        </is>
+      </c>
+      <c r="J100" s="61" t="inlineStr">
+        <is>
+          <t>Noches de mal sueño por la falta de actividad y el exceso de pantallas.</t>
+        </is>
+      </c>
+      <c r="K100" s="61" t="inlineStr">
+        <is>
+          <t>Hacé tu caminata por la tarde y dejá el celular lejos de la cama.</t>
+        </is>
+      </c>
+      <c r="L100" s="61" t="inlineStr">
+        <is>
+          <t>La constancia importa más que la velocidad, y la carrera se corre con los ojos puestos en Jesús (12:2), no en los demás.</t>
+        </is>
+      </c>
+      <c r="M100" s="61" t="inlineStr">
+        <is>
+          <t>Compararse con otros y desanimarse.</t>
+        </is>
+      </c>
+      <c r="N100" s="61" t="inlineStr">
+        <is>
+          <t>No te compares: medí tu avance contra vos mismo la semana pasada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="61" t="n">
+        <v>17</v>
+      </c>
+      <c r="B101" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C101" s="61" t="inlineStr">
+        <is>
+          <t>Dios da las fuerzas</t>
+        </is>
+      </c>
+      <c r="D101" s="61" t="inlineStr">
+        <is>
+          <t>Adultos que hacían al menos 150 minutos semanales de actividad física moderada o intensa contaron que dormían mucho mejor que los que se movían menos.</t>
+        </is>
+      </c>
+      <c r="E101" s="61" t="inlineStr">
+        <is>
+          <t>Loprinzi y Cardinal, Mental Health and Physical Activity, 2011</t>
+        </is>
+      </c>
+      <c r="F101" s="61" t="inlineStr">
+        <is>
+          <t>David le canta a Dios, que le dio fuerzas en la batalla. Reconocer que las fuerzas vienen de Dios nos libra del orgullo y del desánimo.</t>
+        </is>
+      </c>
+      <c r="G101" s="61" t="inlineStr">
+        <is>
+          <t>El ánimo bajo y el cansancio que se vuelven rutina.</t>
+        </is>
+      </c>
+      <c r="H101" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, al moverte, agradecé a Dios por cada parte de tu cuerpo que funciona.</t>
+        </is>
+      </c>
+      <c r="I101" s="61" t="inlineStr">
+        <is>
+          <t>Cuerpo y alma no viven separados: el movimiento mejora el ánimo y el descanso, y un alma en paz ayuda al cuerpo.</t>
+        </is>
+      </c>
+      <c r="J101" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que lo espiritual no tiene nada que ver con el cuidado del cuerpo.</t>
+        </is>
+      </c>
+      <c r="K101" s="61" t="inlineStr">
+        <is>
+          <t>Combiná tu caminata con oración o con la Biblia en audio.</t>
+        </is>
+      </c>
+      <c r="L101" s="61" t="inlineStr">
+        <is>
+          <t>No se trata de competir ni de lucirse, sino de usar bien las fuerzas que Dios da, con las capacidades que cada uno tiene.</t>
+        </is>
+      </c>
+      <c r="M101" s="61" t="inlineStr">
+        <is>
+          <t>Personas con alguna limitación física que creen que el ejercicio no es para ellas.</t>
+        </is>
+      </c>
+      <c r="N101" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés una limitación, preguntá en tu unidad de salud familiar qué movimientos podés hacer de forma segura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="61" t="n">
+        <v>17</v>
+      </c>
+      <c r="B102" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C102" s="61" t="inlineStr">
+        <is>
+          <t>Hechos para movernos</t>
+        </is>
+      </c>
+      <c r="D102" s="61" t="inlineStr">
+        <is>
+          <t>Las tareas de la casa y del jardín también cuentan como actividad física, si se hacen con ritmo.</t>
+        </is>
+      </c>
+      <c r="E102" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Directrices sobre actividad física, 2020</t>
+        </is>
+      </c>
+      <c r="F102" s="61" t="inlineStr">
+        <is>
+          <t>Antes de la caída, Dios ya le dio al ser humano un trabajo: cultivar y cuidar el huerto. Moverse y trabajar con el cuerpo es parte del diseño.</t>
+        </is>
+      </c>
+      <c r="G102" s="61" t="inlineStr">
+        <is>
+          <t>Creer que el ejercicio solo cuenta en un gimnasio.</t>
+        </is>
+      </c>
+      <c r="H102" s="61" t="inlineStr">
+        <is>
+          <t>Hoy contá como ejercicio barrer, carpir o cuidar la huerta: hacelo con ritmo durante 15 minutos.</t>
+        </is>
+      </c>
+      <c r="I102" s="61" t="inlineStr">
+        <is>
+          <t>No hace falta equipamiento: caminar, estirarse o hacer una rutina corta en casa ya suma.</t>
+        </is>
+      </c>
+      <c r="J102" s="61" t="inlineStr">
+        <is>
+          <t>La falta de tiempo o de plata como excusa para no moverse.</t>
+        </is>
+      </c>
+      <c r="K102" s="61" t="inlineStr">
+        <is>
+          <t>Probá esta rutina: 10 sentadillas, 10 flexiones con las manos apoyadas en la pared y 1 minuto de estiramiento. Repetila dos veces.</t>
+        </is>
+      </c>
+      <c r="L102" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar el cuerpo que Dios nos dio es mayordomía, no vanidad.</t>
+        </is>
+      </c>
+      <c r="M102" s="61" t="inlineStr">
+        <is>
+          <t>Niños que pasan la tarde frente a las pantallas en lugar de jugar.</t>
+        </is>
+      </c>
+      <c r="N102" s="61" t="inlineStr">
+        <is>
+          <t>Hagan en familia 15 minutos de juego activo: saltar la cuerda, la pelota o una caminata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="61" t="n">
+        <v>17</v>
+      </c>
+      <c r="B103" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C103" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: moverse es cuidar un regalo</t>
+        </is>
+      </c>
+      <c r="D103" s="61" t="inlineStr">
+        <is>
+          <t>Para niños y adolescentes, la recomendación es de al menos 60 minutos de actividad física por día, en promedio.</t>
+        </is>
+      </c>
+      <c r="E103" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Directrices sobre actividad física, 2020</t>
+        </is>
+      </c>
+      <c r="F103" s="61" t="inlineStr">
+        <is>
+          <t>El cuerpo fue diseñado para moverse: un poco cada día suma más que mucho de vez en cuando.</t>
+        </is>
+      </c>
+      <c r="G103" s="61" t="n"/>
+      <c r="H103" s="61" t="inlineStr">
+        <is>
+          <t>Hagan en familia el desafío de la semana: 15 minutos de movimiento por día. Si alguien tiene una condición de salud, que consulte antes.</t>
+        </is>
+      </c>
+      <c r="I103" s="61" t="inlineStr">
+        <is>
+          <t>El movimiento también cuida el ánimo y el sueño: cuerpo y alma no viven separados.</t>
+        </is>
+      </c>
+      <c r="J103" s="61" t="n"/>
+      <c r="K103" s="61" t="n"/>
+      <c r="L103" s="61" t="inlineStr">
+        <is>
+          <t>No hace falta gimnasio: caminar, las tareas de la casa y una rutina corta alcanzan para empezar.</t>
+        </is>
+      </c>
+      <c r="M103" s="61" t="n"/>
+      <c r="N103" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de abril verificados
24 datos contrastados: 14 confirmados, 10 ajustados (Jeremías 17:6 dice
«retama» en la RVC; informalidad del INE 60,1 % en 2025; precisiones de
estudios). Texto RVC de Proverbios 21:5 confirmado en versiculos_sugeridos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -24593,12 +24593,12 @@
       </c>
       <c r="D81" s="61" t="inlineStr">
         <is>
-          <t>En una encuesta de Gallup en Estados Unidos, solo uno de cada tres hogares (32 %) dijo llevar un presupuesto detallado de sus ingresos y gastos.</t>
+          <t>En una encuesta de Gallup en Estados Unidos, solo uno de cada tres adultos (32 %) dijo preparar cada mes un presupuesto detallado de sus ingresos y gastos.</t>
         </is>
       </c>
       <c r="E81" s="61" t="inlineStr">
         <is>
-          <t>Gallup, 2013</t>
+          <t>Gallup, abril de 2013</t>
         </is>
       </c>
       <c r="F81" s="61" t="inlineStr">
@@ -25063,12 +25063,12 @@
       </c>
       <c r="D88" s="61" t="inlineStr">
         <is>
-          <t>Las águilas aprovechan las corrientes de aire caliente para subir y planear durante largos tramos casi sin aletear, ahorrando energía.</t>
+          <t>Las águilas aprovechan las corrientes de aire caliente para subir en espiral y luego planear largos tramos casi sin aletear, ahorrando energía.</t>
         </is>
       </c>
       <c r="E88" s="61" t="inlineStr">
         <is>
-          <t>Estudios sobre el vuelo de aves planeadoras</t>
+          <t>Duerr y otros, PLoS ONE, 2012 (águilas reales seguidas con GPS)</t>
         </is>
       </c>
       <c r="F88" s="61" t="inlineStr">
@@ -25393,7 +25393,7 @@
       </c>
       <c r="D93" s="61" t="inlineStr">
         <is>
-          <t>Los equipos de trabajo más comprometidos logran resultados mejores: en los análisis de Gallup, alrededor de un 23 % más de rentabilidad.</t>
+          <t>Según los análisis de Gallup, los equipos de trabajo más comprometidos son alrededor de un 23 % más rentables que los menos comprometidos.</t>
         </is>
       </c>
       <c r="E93" s="61" t="inlineStr">
@@ -25463,7 +25463,7 @@
       </c>
       <c r="D94" s="61" t="inlineStr">
         <is>
-          <t>En un estudio con miles de empleados públicos británicos, quienes sentían que su jefe los trataba con justicia tuvieron menos enfermedades del corazón en los años siguientes.</t>
+          <t>En un estudio con más de 6.000 funcionarios públicos británicos varones, quienes sentían que en su trabajo los trataban con justicia tuvieron menos riesgo de enfermedades del corazón en los años siguientes.</t>
         </is>
       </c>
       <c r="E94" s="61" t="inlineStr">
@@ -25533,17 +25533,17 @@
       </c>
       <c r="D95" s="61" t="inlineStr">
         <is>
-          <t>Jeremías 17 compara dos plantas: el que confía en el ser humano es como una zarza en el desierto; el que confía en el Señor, como un árbol junto al agua.</t>
+          <t>Jeremías 17 compara dos plantas: el que confía en el ser humano es como una retama en el desierto; el que confía en el Señor, como un árbol junto al agua.</t>
         </is>
       </c>
       <c r="E95" s="61" t="inlineStr">
         <is>
-          <t>Jeremías 17:5-8</t>
+          <t>Jeremías 17:5-8 (RVC)</t>
         </is>
       </c>
       <c r="F95" s="61" t="inlineStr">
         <is>
-          <t>Jeremías contrasta al que confía en el ser humano con el que confía en el Señor: uno es como una zarza en el desierto; el otro, como un árbol plantado junto al agua (17:5-8).</t>
+          <t>Jeremías contrasta al que confía en el ser humano con el que confía en el Señor: uno es como una retama en el desierto; el otro, como un árbol plantado junto al agua (17:5-8).</t>
         </is>
       </c>
       <c r="G95" s="61" t="inlineStr">
@@ -25603,12 +25603,12 @@
       </c>
       <c r="D96" s="61" t="inlineStr">
         <is>
-          <t>En Paraguay, más de seis de cada diez personas ocupadas trabajan en la informalidad.</t>
+          <t>En Paraguay, seis de cada diez personas ocupadas trabajan en la informalidad: el 60,1 % en 2025.</t>
         </is>
       </c>
       <c r="E96" s="61" t="inlineStr">
         <is>
-          <t>Instituto Nacional de Estadística (INE), Encuesta Permanente de Hogares Continua</t>
+          <t>Instituto Nacional de Estadística (INE), Ocupación Informal 2025, Encuesta Permanente de Hogares Continua</t>
         </is>
       </c>
       <c r="F96" s="61" t="inlineStr">
@@ -25723,12 +25723,12 @@
       </c>
       <c r="D98" s="61" t="inlineStr">
         <is>
-          <t>La Organización Mundial de la Salud recomienda a los adultos al menos 150 minutos por semana de actividad física moderada.</t>
+          <t>La Organización Mundial de la Salud recomienda a los adultos entre 150 y 300 minutos por semana de actividad física moderada, o entre 75 y 150 de actividad intensa.</t>
         </is>
       </c>
       <c r="E98" s="61" t="inlineStr">
         <is>
-          <t>Organización Mundial de la Salud, Directrices sobre actividad física, 2020</t>
+          <t>Organización Mundial de la Salud, Directrices sobre actividad física y hábitos sedentarios, 2020</t>
         </is>
       </c>
       <c r="F98" s="61" t="inlineStr">
@@ -25863,7 +25863,7 @@
       </c>
       <c r="D100" s="61" t="inlineStr">
         <is>
-          <t>Reemplazar tiempo sentado por 15 minutos de correr o una hora de caminata por día se asoció con un 26 % menos de riesgo de depresión.</t>
+          <t>Un estudio genético estimó que sumar actividad equivalente a 15 minutos de correr o una hora de caminata rápida por día, en lugar de estar sentado, se asocia con un 26 % menos de probabilidad de depresión.</t>
         </is>
       </c>
       <c r="E100" s="61" t="inlineStr">
@@ -25933,7 +25933,7 @@
       </c>
       <c r="D101" s="61" t="inlineStr">
         <is>
-          <t>Adultos que hacían al menos 150 minutos semanales de actividad física moderada o intensa contaron que dormían mucho mejor que los que se movían menos.</t>
+          <t>Adultos que, medidos con un sensor de movimiento, sumaban al menos 150 minutos semanales de actividad física tuvieron un 65 % menos de probabilidad de sentirse muy somnolientos durante el día.</t>
         </is>
       </c>
       <c r="E101" s="61" t="inlineStr">
@@ -26073,7 +26073,7 @@
       </c>
       <c r="D103" s="61" t="inlineStr">
         <is>
-          <t>Para niños y adolescentes, la recomendación es de al menos 60 minutos de actividad física por día, en promedio.</t>
+          <t>Para niños y adolescentes de 5 a 17 años, la recomendación es de al menos 60 minutos por día, en promedio, de actividad física moderada a intensa.</t>
         </is>
       </c>
       <c r="E103" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: textos urgentes de Proverbios 12:15 y 21:5, y mayo con revisión teológica
- Aplicados los dos errores de copia aprobados (tools/versiculos_aplicados_2027.py)
- Mayo (semanas 18 a 21): 24 guiones con revisión teológica; datos en verificación
- Dos sugerencias opcionales más en versiculos_sugeridos (Mateo 6:3-4, Hageo 1:6)
- Alarma: «no garantiza» ya no se marca como promesa

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -2983,8 +2983,7 @@
       </c>
       <c r="AH11" s="49" t="inlineStr">
         <is>
-          <t>Proverbios 12:15 — La necedad va ligada al corazón del joven,
-pero la vara disciplinaria le quita lo necio.</t>
+          <t>Proverbios 12:15 — El necio piensa que va por buen camino, pero el sabio presta atención al consejo.</t>
         </is>
       </c>
       <c r="AI11" s="49" t="inlineStr">
@@ -3769,8 +3768,7 @@
       </c>
       <c r="AB15" s="40" t="inlineStr">
         <is>
-          <t>Proverbios 21:5 — 15El justo se alegra cuando se hace justicia,
-pero los malvados se ponen a temblar.</t>
+          <t>Proverbios 21:5 — Si piensas lo que haces, tendrás abundancia; si te apresuras, acabarás en la pobreza.</t>
         </is>
       </c>
       <c r="AC15" s="40" t="inlineStr">
@@ -4825,8 +4823,8 @@
       <c r="AG20" s="53" t="inlineStr">
         <is>
           <t>• La fortaleza viene de Cristo, no de uno mismo
-• Todo es posible con ese respaldo
-• No hay desafío que anule esa fuerza</t>
+• Contento en la abundancia y en la escasez
+• Su fuerza sostiene también en la derrota</t>
         </is>
       </c>
       <c r="AH20" s="53" t="inlineStr">
@@ -4848,7 +4846,7 @@
       </c>
       <c r="AK20" s="53" t="inlineStr">
         <is>
-          <t>• Todo ayuda a bien para quien ama a Dios
+          <t>• Dios obra en todo para el bien de los que lo aman
 • Incluso los desafíos tienen propósito
 • La confianza no depende de entender todo</t>
         </is>
@@ -4992,7 +4990,7 @@
         <is>
           <t>• Instruir desde temprano marca el camino
 • La formación inicial perdura
-• No se aparta cuando envejece</t>
+• La formación deja huella para toda la vida</t>
         </is>
       </c>
       <c r="AB21" s="35" t="inlineStr">
@@ -5194,7 +5192,7 @@
       </c>
       <c r="AA22" s="40" t="inlineStr">
         <is>
-          <t>• El trabajo es condición para el sustento
+          <t>• Quien puede trabajar, que trabaje
 • No fomentar la pereza
 • El esfuerzo propio antecede al ingreso</t>
         </is>
@@ -5208,7 +5206,7 @@
       <c r="AC22" s="40" t="inlineStr">
         <is>
           <t>• La mano negligente empobrece
-• La diligencia enriquece
+• La diligencia abre caminos
 • El esfuerzo constante marca la diferencia</t>
         </is>
       </c>
@@ -5261,7 +5259,7 @@
         <is>
           <t>• Repartir generosamente trae más, no menos
 • La generosidad no empobrece
-• El alma generosa prospera</t>
+• La generosidad enriquece la vida</t>
         </is>
       </c>
     </row>
@@ -19216,7 +19214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N103"/>
+  <dimension ref="A1:N127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -26106,6 +26104,1606 @@
       </c>
       <c r="M103" s="61" t="n"/>
       <c r="N103" s="61" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="B104" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C104" s="61" t="inlineStr">
+        <is>
+          <t>Vino a servir</t>
+        </is>
+      </c>
+      <c r="D104" s="61" t="inlineStr">
+        <is>
+          <t>Hacer voluntariado se asoció con menos síntomas de depresión y más satisfacción con la vida; son estudios que muestran una relación, no una causa.</t>
+        </is>
+      </c>
+      <c r="E104" s="61" t="inlineStr">
+        <is>
+          <t>Jenkinson y otros, BMC Public Health, 2013</t>
+        </is>
+      </c>
+      <c r="F104" s="61" t="inlineStr">
+        <is>
+          <t>Jesús, el Señor de todo, dice que no vino a ser servido sino a servir. Lo dice justo cuando sus discípulos discutían quién sería el más importante (10:35-44).</t>
+        </is>
+      </c>
+      <c r="G104" s="61" t="inlineStr">
+        <is>
+          <t>La búsqueda de cargos y reconocimiento, también en la iglesia.</t>
+        </is>
+      </c>
+      <c r="H104" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, ofrecete para una tarea que nadie quiere hacer en tu casa, tu trabajo o tu iglesia.</t>
+        </is>
+      </c>
+      <c r="I104" s="61" t="inlineStr">
+        <is>
+          <t>Servir nos saca de nosotros mismos: al prestar atención a la necesidad del otro, conocemos de verdad a la persona y también descubrimos nuestros propios dones.</t>
+        </is>
+      </c>
+      <c r="J104" s="61" t="inlineStr">
+        <is>
+          <t>Vivir tan concentrados en lo propio que no vemos la necesidad de quien está al lado.</t>
+        </is>
+      </c>
+      <c r="K104" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale hoy a alguien cercano: ¿en qué te puedo ayudar esta semana? Y escuchá la respuesta.</t>
+        </is>
+      </c>
+      <c r="L104" s="61" t="inlineStr">
+        <is>
+          <t>Jesús dio su vida en rescate por muchos: eso solo lo hizo Él, y lo recibimos con gratitud. Nuestro servicio no nos salva; es la respuesta a lo que Él hizo.</t>
+        </is>
+      </c>
+      <c r="M104" s="61" t="inlineStr">
+        <is>
+          <t>Servir para ganarse el favor de Dios o de los demás, y terminar agotado.</t>
+        </is>
+      </c>
+      <c r="N104" s="61" t="inlineStr">
+        <is>
+          <t>Antes de servir esta semana, agradecé a Jesús por lo que hizo por vos, y serví desde ahí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="B105" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C105" s="61" t="inlineStr">
+        <is>
+          <t>Cada uno recibió un don</t>
+        </is>
+      </c>
+      <c r="D105" s="61" t="inlineStr">
+        <is>
+          <t>La palabra griega que Pedro usa para «don», járisma, viene de járis, que significa gracia.</t>
+        </is>
+      </c>
+      <c r="E105" s="61" t="inlineStr">
+        <is>
+          <t>Léxico griego de Strong (G5486)</t>
+        </is>
+      </c>
+      <c r="F105" s="61" t="inlineStr">
+        <is>
+          <t>Pedro dice que cada uno recibió algún don. Nadie quedó afuera: todos tenemos algo para dar.</t>
+        </is>
+      </c>
+      <c r="G105" s="61" t="inlineStr">
+        <is>
+          <t>Personas que creen que no tienen nada para aportar.</t>
+        </is>
+      </c>
+      <c r="H105" s="61" t="inlineStr">
+        <is>
+          <t>Escribí tres cosas que hacés bien y que podrían servir a otros.</t>
+        </is>
+      </c>
+      <c r="I105" s="61" t="inlineStr">
+        <is>
+          <t>Somos administradores, no dueños: el don es de Dios y está para el bien de los demás.</t>
+        </is>
+      </c>
+      <c r="J105" s="61" t="inlineStr">
+        <is>
+          <t>Usar los talentos solo para destacarse o para beneficio propio.</t>
+        </is>
+      </c>
+      <c r="K105" s="61" t="inlineStr">
+        <is>
+          <t>Elegí uno de tus dones y ponelo esta semana al servicio de alguien que no te pueda devolver el favor.</t>
+        </is>
+      </c>
+      <c r="L105" s="61" t="inlineStr">
+        <is>
+          <t>Al servir, el otro deja de ser un desconocido, y nosotros descubrimos para qué Dios nos dio lo que nos dio.</t>
+        </is>
+      </c>
+      <c r="M105" s="61" t="inlineStr">
+        <is>
+          <t>Comunidades donde siempre sirven los mismos, cansados, mientras muchos miran.</t>
+        </is>
+      </c>
+      <c r="N105" s="61" t="inlineStr">
+        <is>
+          <t>Si siempre mirás, esta semana sumate a un servicio de tu iglesia o de tu barrio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="B106" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C106" s="61" t="inlineStr">
+        <is>
+          <t>El Maestro que lavó los pies</t>
+        </is>
+      </c>
+      <c r="D106" s="61" t="inlineStr">
+        <is>
+          <t>En tiempos de Jesús, lavar los pies de los invitados era una tarea que normalmente hacía un sirviente.</t>
+        </is>
+      </c>
+      <c r="E106" s="61" t="inlineStr">
+        <is>
+          <t>Juan 13:4-5; comentarios bíblicos sobre las costumbres del siglo I</t>
+        </is>
+      </c>
+      <c r="F106" s="61" t="inlineStr">
+        <is>
+          <t>Jesús se levantó de la mesa y lavó los pies de sus discípulos, una tarea de sirvientes. Lo hizo en silencio, sin discurso previo.</t>
+        </is>
+      </c>
+      <c r="G106" s="61" t="inlineStr">
+        <is>
+          <t>El servicio que solo se hace si hay fotos o reconocimiento.</t>
+        </is>
+      </c>
+      <c r="H106" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy un servicio que nadie vea: lavar, ordenar, preparar algo para otro.</t>
+        </is>
+      </c>
+      <c r="I106" s="61" t="inlineStr">
+        <is>
+          <t>El Maestro sirvió a los alumnos. En el reino de Dios, servir no tiene jerarquías.</t>
+        </is>
+      </c>
+      <c r="J106" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que ciertos trabajos son «poca cosa» para uno.</t>
+        </is>
+      </c>
+      <c r="K106" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, hacé una tarea que normalmente dejás a otros, sin comentarlo.</t>
+        </is>
+      </c>
+      <c r="L106" s="61" t="inlineStr">
+        <is>
+          <t>«Hagan lo mismo»: el ejemplo de Jesús no es para admirarlo de lejos, sino para seguirlo.</t>
+        </is>
+      </c>
+      <c r="M106" s="61" t="inlineStr">
+        <is>
+          <t>Admirar el servicio de otros sin dar nunca el paso.</t>
+        </is>
+      </c>
+      <c r="N106" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy, en privado, a alguien que sirve sin figurar en tu iglesia o en tu trabajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="B107" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C107" s="61" t="inlineStr">
+        <is>
+          <t>Para el Señor, aunque nadie aplauda</t>
+        </is>
+      </c>
+      <c r="D107" s="61" t="inlineStr">
+        <is>
+          <t>Se estima que unos 862 millones de personas mayores de 15 años hacen algún tipo de voluntariado cada mes en el mundo.</t>
+        </is>
+      </c>
+      <c r="E107" s="61" t="inlineStr">
+        <is>
+          <t>Voluntarios de las Naciones Unidas, Informe sobre el estado del voluntariado en el mundo, 2022</t>
+        </is>
+      </c>
+      <c r="F107" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribe a esclavos y trabajadores: lo que hagan, háganlo como para el Señor. Hoy lo aplicamos al servicio que nadie ve.</t>
+        </is>
+      </c>
+      <c r="G107" s="61" t="inlineStr">
+        <is>
+          <t>El cansancio de servir y sentir que nadie lo nota.</t>
+        </is>
+      </c>
+      <c r="H107" s="61" t="inlineStr">
+        <is>
+          <t>Antes de servir hoy, decí en silencio: «Esto es para vos, Señor».</t>
+        </is>
+      </c>
+      <c r="I107" s="61" t="inlineStr">
+        <is>
+          <t>La actitud del corazón importa más que la tarea: el mismo servicio puede ser ofrenda o puede ser vanidad.</t>
+        </is>
+      </c>
+      <c r="J107" s="61" t="inlineStr">
+        <is>
+          <t>Servir esperando que nos agradezcan, y enojarse cuando no pasa.</t>
+        </is>
+      </c>
+      <c r="K107" s="61" t="inlineStr">
+        <is>
+          <t>Revisá tus motivaciones: ¿qué servicio seguirías haciendo aunque nadie te lo agradezca?</t>
+        </is>
+      </c>
+      <c r="L107" s="61" t="inlineStr">
+        <is>
+          <t>Dios ve lo que nadie ve. Ese servicio silencioso es, muchas veces, el más valioso.</t>
+        </is>
+      </c>
+      <c r="M107" s="61" t="inlineStr">
+        <is>
+          <t>Comparar el propio servicio con el de otros más visibles.</t>
+        </is>
+      </c>
+      <c r="N107" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, orá por alguien sin decírselo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="B108" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C108" s="61" t="inlineStr">
+        <is>
+          <t>Lo que hicieron por el más pequeño</t>
+        </is>
+      </c>
+      <c r="D108" s="61" t="inlineStr">
+        <is>
+          <t>El psicólogo Mihaly Csikszentmihalyi llamó «flujo» al estado en que estamos tan metidos en una tarea que el tiempo se pasa volando.</t>
+        </is>
+      </c>
+      <c r="E108" s="61" t="inlineStr">
+        <is>
+          <t>Mihaly Csikszentmihalyi, «Fluir», 1990</t>
+        </is>
+      </c>
+      <c r="F108" s="61" t="inlineStr">
+        <is>
+          <t>Jesús dice que lo que hacemos por el más pequeño, se lo hacemos a Él. Servir al necesitado es servir a Cristo.</t>
+        </is>
+      </c>
+      <c r="G108" s="61" t="inlineStr">
+        <is>
+          <t>Ancianos solos, enfermos y personas en la calle que nadie visita.</t>
+        </is>
+      </c>
+      <c r="H108" s="61" t="inlineStr">
+        <is>
+          <t>Visitá esta semana a alguien que está solo o enfermo, aunque sea un rato.</t>
+        </is>
+      </c>
+      <c r="I108" s="61" t="inlineStr">
+        <is>
+          <t>Lo pequeño no pasa desapercibido para Dios: un vaso de agua, una visita, una llamada.</t>
+        </is>
+      </c>
+      <c r="J108" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que solo vale la pena el servicio grande.</t>
+        </is>
+      </c>
+      <c r="K108" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un gesto pequeño y concreto para hacer cada día de esta semana.</t>
+        </is>
+      </c>
+      <c r="L108" s="61" t="inlineStr">
+        <is>
+          <t>Para descubrir para qué servís mejor, prestá atención a qué necesidad, cuando la atendés, te da más alegría que cansancio. Ahí suele estar tu forma de servir.</t>
+        </is>
+      </c>
+      <c r="M108" s="61" t="inlineStr">
+        <is>
+          <t>Servir durante años en algo que no va con uno, hasta quemarse.</t>
+        </is>
+      </c>
+      <c r="N108" s="61" t="inlineStr">
+        <is>
+          <t>Preguntate: ¿qué tarea, cuando la hago, se me pasa el tiempo volando? Contáselo a tu pastor o a tu líder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="61" t="n">
+        <v>18</v>
+      </c>
+      <c r="B109" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C109" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: servir con amor</t>
+        </is>
+      </c>
+      <c r="D109" s="61" t="inlineStr">
+        <is>
+          <t>La frase de Jesús «Hay más bendición en dar que en recibir» no aparece en los evangelios: la conocemos porque Pablo la recordó en Hechos.</t>
+        </is>
+      </c>
+      <c r="E109" s="61" t="inlineStr">
+        <is>
+          <t>Hechos 20:35</t>
+        </is>
+      </c>
+      <c r="F109" s="61" t="inlineStr">
+        <is>
+          <t>Servir nos saca de nosotros mismos: así conocemos al otro y descubrimos nuestros dones.</t>
+        </is>
+      </c>
+      <c r="G109" s="61" t="n"/>
+      <c r="H109" s="61" t="inlineStr">
+        <is>
+          <t>Pablo recuerda las palabras de Jesús: hay más bendición en dar que en recibir. Esta semana, ofrecé tu tiempo para un servicio concreto en tu iglesia o en tu barrio.</t>
+        </is>
+      </c>
+      <c r="I109" s="61" t="inlineStr">
+        <is>
+          <t>El servicio silencioso, el que nadie aplaude, es muchas veces el más valioso: Dios lo ve.</t>
+        </is>
+      </c>
+      <c r="J109" s="61" t="n"/>
+      <c r="K109" s="61" t="n"/>
+      <c r="L109" s="61" t="inlineStr">
+        <is>
+          <t>Tu forma de servir está donde una necesidad te da más alegría que cansancio.</t>
+        </is>
+      </c>
+      <c r="M109" s="61" t="n"/>
+      <c r="N109" s="61" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="61" t="n">
+        <v>19</v>
+      </c>
+      <c r="B110" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C110" s="61" t="inlineStr">
+        <is>
+          <t>Seguir construyendo entre críticas</t>
+        </is>
+      </c>
+      <c r="D110" s="61" t="inlineStr">
+        <is>
+          <t>Las experiencias negativas nos impactan más que las positivas: una crítica suele pesar más que varios elogios.</t>
+        </is>
+      </c>
+      <c r="E110" s="61" t="inlineStr">
+        <is>
+          <t>Baumeister y otros, «Bad is stronger than good», Review of General Psychology, 2001</t>
+        </is>
+      </c>
+      <c r="F110" s="61" t="inlineStr">
+        <is>
+          <t>Nehemías reconstruía los muros de Jerusalén entre burlas y amenazas. No respondió con insultos: siguió trabajando y animó al pueblo.</t>
+        </is>
+      </c>
+      <c r="G110" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que abandonan un proyecto bueno porque algunos lo critican.</t>
+        </is>
+      </c>
+      <c r="H110" s="61" t="inlineStr">
+        <is>
+          <t>Si recibís críticas por algo bueno que estás haciendo, no respondas en caliente: orá y seguí trabajando.</t>
+        </is>
+      </c>
+      <c r="I110" s="61" t="inlineStr">
+        <is>
+          <t>«Recuerden que el Señor es grande»: mirar a Dios pone las críticas en su tamaño real.</t>
+        </is>
+      </c>
+      <c r="J110" s="61" t="inlineStr">
+        <is>
+          <t>Vivir pendiente de lo que dicen los demás, en persona o en las redes.</t>
+        </is>
+      </c>
+      <c r="K110" s="61" t="inlineStr">
+        <is>
+          <t>Cuando te llegue una crítica, hacete dos preguntas: ¿quién la dice? ¿Busca ayudar o solo desacreditar? Si ayuda, escuchala; si no, dejala pasar.</t>
+        </is>
+      </c>
+      <c r="L110" s="61" t="inlineStr">
+        <is>
+          <t>Nehemías recuerda por quién luchan: hermanos, hijos, hogares. Recordar el propósito ayuda a no rendirse.</t>
+        </is>
+      </c>
+      <c r="M110" s="61" t="inlineStr">
+        <is>
+          <t>Olvidar para qué empezamos y quedar atrapados en la discusión.</t>
+        </is>
+      </c>
+      <c r="N110" s="61" t="inlineStr">
+        <is>
+          <t>Escribí en una frase para qué hacés lo que hacés, y leela cuando te desanimes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="61" t="n">
+        <v>19</v>
+      </c>
+      <c r="B111" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C111" s="61" t="inlineStr">
+        <is>
+          <t>Atentos, sin ver enemigos en todos</t>
+        </is>
+      </c>
+      <c r="D111" s="61" t="inlineStr">
+        <is>
+          <t>El rugido de un león puede oírse a varios kilómetros de distancia.</t>
+        </is>
+      </c>
+      <c r="E111" s="61" t="inlineStr">
+        <is>
+          <t>Estudios sobre comportamiento de leones</t>
+        </is>
+      </c>
+      <c r="F111" s="61" t="inlineStr">
+        <is>
+          <t>Pedro advierte que hay un enemigo real que busca destruir. Pero eso no significa que quien nos critica sea el enemigo: la crítica, incluso la injusta, viene de personas por las que Cristo también murió.</t>
+        </is>
+      </c>
+      <c r="G111" s="61" t="inlineStr">
+        <is>
+          <t>Etiquetar como «ataque espiritual» toda crítica, para no escucharla.</t>
+        </is>
+      </c>
+      <c r="H111" s="61" t="inlineStr">
+        <is>
+          <t>Antes de descartar una crítica, preguntale a alguien de confianza si hay algo de verdad en ella.</t>
+        </is>
+      </c>
+      <c r="I111" s="61" t="inlineStr">
+        <is>
+          <t>Resistir no es atacar: es mantenerse firme en la fe, sin devolver mal por mal.</t>
+        </is>
+      </c>
+      <c r="J111" s="61" t="inlineStr">
+        <is>
+          <t>Responder a la crítica con más críticas, en grupos y redes.</t>
+        </is>
+      </c>
+      <c r="K111" s="61" t="inlineStr">
+        <is>
+          <t>Si te criticaron injustamente, no lo devuelvas: bendecí y seguí haciendo el bien (1 Pedro 3:9).</t>
+        </is>
+      </c>
+      <c r="L111" s="61" t="inlineStr">
+        <is>
+          <t>Pedro recuerda que en todo el mundo los hermanos pasan por lo mismo: no estás solo. Estar atentos juntos protege.</t>
+        </is>
+      </c>
+      <c r="M111" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que cargan solos las críticas y no se lo cuentan a nadie.</t>
+        </is>
+      </c>
+      <c r="N111" s="61" t="inlineStr">
+        <is>
+          <t>Buscá a una persona de confianza con quien hablar de lo que te pesa como líder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="61" t="n">
+        <v>19</v>
+      </c>
+      <c r="B112" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C112" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que también se equivocaron</t>
+        </is>
+      </c>
+      <c r="D112" s="61" t="inlineStr">
+        <is>
+          <t>En un estudio en hospitales, los equipos con mejores líderes reportaban más errores: no porque se equivocaran más, sino porque se animaban a decirlos.</t>
+        </is>
+      </c>
+      <c r="E112" s="61" t="inlineStr">
+        <is>
+          <t>Amy Edmondson, Universidad de Harvard, Journal of Applied Behavioral Science, 1996</t>
+        </is>
+      </c>
+      <c r="F112" s="61" t="inlineStr">
+        <is>
+          <t>La carta pide acordarse de quienes nos enseñaron la Palabra. Ellos también fallaron y se levantaron: su fe no era perfección, era confianza en Dios.</t>
+        </is>
+      </c>
+      <c r="G112" s="61" t="inlineStr">
+        <is>
+          <t>Exigir perfección a los líderes y no perdonarles ningún error.</t>
+        </is>
+      </c>
+      <c r="H112" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé esta semana a un pastor o líder que te enseñó, y orá por él.</t>
+        </is>
+      </c>
+      <c r="I112" s="61" t="inlineStr">
+        <is>
+          <t>«Piensen en los resultados de su conducta»: a un líder se lo conoce también por cómo maneja sus errores.</t>
+        </is>
+      </c>
+      <c r="J112" s="61" t="inlineStr">
+        <is>
+          <t>Ocultar los errores por miedo a perder autoridad.</t>
+        </is>
+      </c>
+      <c r="K112" s="61" t="inlineStr">
+        <is>
+          <t>Si te equivocaste en algo que afectó a otros, reconocelo con humildad y decí qué vas a corregir.</t>
+        </is>
+      </c>
+      <c r="L112" s="61" t="inlineStr">
+        <is>
+          <t>Lo que imitamos no es su éxito, sino su fe. Reconocer un error, corregir el rumbo y seguir enseña al equipo tanto como un éxito.</t>
+        </is>
+      </c>
+      <c r="M112" s="61" t="inlineStr">
+        <is>
+          <t>Quedarse paralizado después de un fracaso.</t>
+        </is>
+      </c>
+      <c r="N112" s="61" t="inlineStr">
+        <is>
+          <t>Escribí qué aprendiste de tu último error y un paso para seguir adelante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="61" t="n">
+        <v>19</v>
+      </c>
+      <c r="B113" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C113" s="61" t="inlineStr">
+        <is>
+          <t>Todo lo puedo, en el contexto correcto</t>
+        </is>
+      </c>
+      <c r="D113" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribió la carta a los Filipenses mientras estaba preso.</t>
+        </is>
+      </c>
+      <c r="E113" s="61" t="inlineStr">
+        <is>
+          <t>Filipenses 1:13</t>
+        </is>
+      </c>
+      <c r="F113" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribe desde la cárcel. Su «todo lo puedo» no es una promesa de ganar siempre: es la fuerza de Cristo para vivir contento tanto en la abundancia como en la escasez (4:11-12).</t>
+        </is>
+      </c>
+      <c r="G113" s="61" t="inlineStr">
+        <is>
+          <t>Usar este versículo como si prometiera lograr cualquier meta.</t>
+        </is>
+      </c>
+      <c r="H113" s="61" t="inlineStr">
+        <is>
+          <t>Leé Filipenses 4:10-13 completo y anotá qué te dice para tu situación de hoy.</t>
+        </is>
+      </c>
+      <c r="I113" s="61" t="inlineStr">
+        <is>
+          <t>Pablo aprendió a estar contento en cualquier situación. Esa misma fuerza sirve también cuando fracasamos.</t>
+        </is>
+      </c>
+      <c r="J113" s="61" t="inlineStr">
+        <is>
+          <t>Medir el valor propio por los éxitos y hundirse con los fracasos.</t>
+        </is>
+      </c>
+      <c r="K113" s="61" t="inlineStr">
+        <is>
+          <t>Hoy agradecé a Dios por algo, aunque las cosas no estén saliendo como querías.</t>
+        </is>
+      </c>
+      <c r="L113" s="61" t="inlineStr">
+        <is>
+          <t>Un fracaso no es el final cuando la fuerza viene de Cristo. Pedro negó a Jesús y fue restaurado (Juan 21).</t>
+        </is>
+      </c>
+      <c r="M113" s="61" t="inlineStr">
+        <is>
+          <t>Creer que un error define para siempre quiénes somos.</t>
+        </is>
+      </c>
+      <c r="N113" s="61" t="inlineStr">
+        <is>
+          <t>Si fallaste, pedí perdón a quien corresponda y recibí el perdón de Dios. Después, da el siguiente paso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="61" t="n">
+        <v>19</v>
+      </c>
+      <c r="B114" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C114" s="61" t="inlineStr">
+        <is>
+          <t>Valiente también para descansar</t>
+        </is>
+      </c>
+      <c r="D114" s="61" t="inlineStr">
+        <is>
+          <t>Dormir unas seis horas por noche durante dos semanas afectó el rendimiento casi tanto como pasar dos noches sin dormir, y los participantes no se daban cuenta.</t>
+        </is>
+      </c>
+      <c r="E114" s="61" t="inlineStr">
+        <is>
+          <t>Van Dongen y otros, revista Sleep, 2003</t>
+        </is>
+      </c>
+      <c r="F114" s="61" t="inlineStr">
+        <is>
+          <t>Dios le habla a Josué cuando asume un liderazgo enorme después de Moisés. El mandato «sé valiente» viene con una promesa: «yo estaré contigo».</t>
+        </is>
+      </c>
+      <c r="G114" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que confunden valentía con no descansar nunca.</t>
+        </is>
+      </c>
+      <c r="H114" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, defendé un tiempo de descanso como defenderías una reunión importante.</t>
+        </is>
+      </c>
+      <c r="I114" s="61" t="inlineStr">
+        <is>
+          <t>La valentía también es reconocer los propios límites y pedir ayuda. El cansancio nubla el juicio y tienta a tomar atajos.</t>
+        </is>
+      </c>
+      <c r="J114" s="61" t="inlineStr">
+        <is>
+          <t>Tomar decisiones importantes agotado, y lamentarlas después.</t>
+        </is>
+      </c>
+      <c r="K114" s="61" t="inlineStr">
+        <is>
+          <t>Si estás muy cansado, postergá las decisiones importantes hasta haber descansado.</t>
+        </is>
+      </c>
+      <c r="L114" s="61" t="inlineStr">
+        <is>
+          <t>«Dondequiera que vayas»: Dios no espera a que estemos fuertes para acompañarnos. Y el equipo también puede cuidar al líder.</t>
+        </is>
+      </c>
+      <c r="M114" s="61" t="inlineStr">
+        <is>
+          <t>Equipos que solo le piden al líder, sin preguntarle cómo está.</t>
+        </is>
+      </c>
+      <c r="N114" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un líder, preguntale esta semana cómo está y en qué lo podés ayudar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="61" t="n">
+        <v>19</v>
+      </c>
+      <c r="B115" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C115" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: liderar en medio de los desafíos</t>
+        </is>
+      </c>
+      <c r="D115" s="61" t="inlineStr">
+        <is>
+          <t>Romanos 8:28 continúa en el versículo 29: el propósito de Dios es que seamos como Jesús.</t>
+        </is>
+      </c>
+      <c r="E115" s="61" t="inlineStr">
+        <is>
+          <t>Romanos 8:28-29</t>
+        </is>
+      </c>
+      <c r="F115" s="61" t="inlineStr">
+        <is>
+          <t>La crítica se recibe con humildad y discernimiento: se escucha la que ayuda y se deja pasar la que solo desgasta.</t>
+        </is>
+      </c>
+      <c r="G115" s="61" t="n"/>
+      <c r="H115" s="61" t="inlineStr">
+        <is>
+          <t>Romanos 8:28 no dice que todo sea bueno, sino que Dios obra en todo para formarnos como Jesús (8:29). Esta semana, orá por un desafío que estás viviendo y pedile a alguien que ore con vos.</t>
+        </is>
+      </c>
+      <c r="I115" s="61" t="inlineStr">
+        <is>
+          <t>Reconocer un error con humildad genera más confianza que ocultarlo.</t>
+        </is>
+      </c>
+      <c r="J115" s="61" t="n"/>
+      <c r="K115" s="61" t="n"/>
+      <c r="L115" s="61" t="inlineStr">
+        <is>
+          <t>Descansar y pedir ayuda es parte de liderar bien.</t>
+        </is>
+      </c>
+      <c r="M115" s="61" t="n"/>
+      <c r="N115" s="61" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="B116" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C116" s="61" t="inlineStr">
+        <is>
+          <t>Formar desde temprano</t>
+        </is>
+      </c>
+      <c r="D116" s="61" t="inlineStr">
+        <is>
+          <t>En un gran estudio sobre jóvenes y religión en Estados Unidos, los padres resultaron la influencia más importante en la vida de fe de sus hijos adolescentes.</t>
+        </is>
+      </c>
+      <c r="E116" s="61" t="inlineStr">
+        <is>
+          <t>Christian Smith, Estudio Nacional sobre Juventud y Religión («Soul Searching», 2005)</t>
+        </is>
+      </c>
+      <c r="F116" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios aconseja formar a los hijos desde temprano. Es un principio de sabiduría, no una garantía automática: los hijos también eligen.</t>
+        </is>
+      </c>
+      <c r="G116" s="61" t="inlineStr">
+        <is>
+          <t>Delegar toda la formación en la escuela, la iglesia o las pantallas.</t>
+        </is>
+      </c>
+      <c r="H116" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un momento fijo de la semana para conversar con tus hijos sobre la vida y la fe.</t>
+        </is>
+      </c>
+      <c r="I116" s="61" t="inlineStr">
+        <is>
+          <t>Lo que se siembra en la infancia deja huella. No hay fórmulas: hay amor constante, límites claros y ejemplo.</t>
+        </is>
+      </c>
+      <c r="J116" s="61" t="inlineStr">
+        <is>
+          <t>Padres que buscan recetas perfectas y viven con culpa por no cumplirlas.</t>
+        </is>
+      </c>
+      <c r="K116" s="61" t="inlineStr">
+        <is>
+          <t>Hacé una lista de tres cosas que querés que tus hijos aprendan de vos, y vivilas esta semana.</t>
+        </is>
+      </c>
+      <c r="L116" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un hijo que se apartó, este versículo no es una sentencia sobre vos: es una esperanza. Dios sigue obrando y la puerta sigue abierta.</t>
+        </is>
+      </c>
+      <c r="M116" s="61" t="inlineStr">
+        <is>
+          <t>La culpa de los padres cuyos hijos se alejaron de la fe.</t>
+        </is>
+      </c>
+      <c r="N116" s="61" t="inlineStr">
+        <is>
+          <t>Si tu hijo se alejó, seguí orando por él y mostrale amor sin condiciones; no lo des por perdido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="B117" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C117" s="61" t="inlineStr">
+        <is>
+          <t>Firmeza y amor, juntos</t>
+        </is>
+      </c>
+      <c r="D117" s="61" t="inlineStr">
+        <is>
+          <t>Los hijos de padres cálidos y con límites claros suelen tener mejores resultados que los de padres muy autoritarios o muy permisivos.</t>
+        </is>
+      </c>
+      <c r="E117" s="61" t="inlineStr">
+        <is>
+          <t>Diana Baumrind, estudios sobre estilos de crianza, 1966 y 1991</t>
+        </is>
+      </c>
+      <c r="F117" s="61" t="inlineStr">
+        <is>
+          <t>Pablo habla primero a los padres: no hagan enojar a sus hijos con exigencias injustas, burlas o gritos.</t>
+        </is>
+      </c>
+      <c r="G117" s="61" t="inlineStr">
+        <is>
+          <t>Hogares donde se corrige gritando o humillando.</t>
+        </is>
+      </c>
+      <c r="H117" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, cuando tengas que corregir, bajá la voz y mirá a tu hijo a los ojos.</t>
+        </is>
+      </c>
+      <c r="I117" s="61" t="inlineStr">
+        <is>
+          <t>Educar es enseñar el camino, no solo prohibir. La instrucción del Señor incluye explicar el porqué.</t>
+        </is>
+      </c>
+      <c r="J117" s="61" t="inlineStr">
+        <is>
+          <t>Reglas sin explicación que los hijos cumplen por miedo y abandonan apenas pueden.</t>
+        </is>
+      </c>
+      <c r="K117" s="61" t="inlineStr">
+        <is>
+          <t>Explicale a tu hijo el porqué de una regla de la casa.</t>
+        </is>
+      </c>
+      <c r="L117" s="61" t="inlineStr">
+        <is>
+          <t>Amor constante y límites claros, juntos. El amor sin límites genera descontrol; los límites sin amor, resentimiento.</t>
+        </is>
+      </c>
+      <c r="M117" s="61" t="inlineStr">
+        <is>
+          <t>Padres que pasan de dejar todo a estallar de enojo.</t>
+        </is>
+      </c>
+      <c r="N117" s="61" t="inlineStr">
+        <is>
+          <t>Acordá con tu pareja dos o tres reglas claras de la casa y sosténganlas juntos, con calma.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="B118" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C118" s="61" t="inlineStr">
+        <is>
+          <t>Corregir para formar</t>
+        </is>
+      </c>
+      <c r="D118" s="61" t="inlineStr">
+        <is>
+          <t>La palabra hebrea que en Proverbios se traduce como «corregir» significa sobre todo instruir y disciplinar, no solo castigar.</t>
+        </is>
+      </c>
+      <c r="E118" s="61" t="inlineStr">
+        <is>
+          <t>Léxico hebreo de Strong (H3256, yasar)</t>
+        </is>
+      </c>
+      <c r="F118" s="61" t="inlineStr">
+        <is>
+          <t>Corregir a tiempo, con amor y sin violencia, evita problemas mayores después.</t>
+        </is>
+      </c>
+      <c r="G118" s="61" t="inlineStr">
+        <is>
+          <t>Dejar pasar todo para evitar el conflicto.</t>
+        </is>
+      </c>
+      <c r="H118" s="61" t="inlineStr">
+        <is>
+          <t>Si hay algo que venís dejando pasar con tus hijos, hablalo hoy con calma.</t>
+        </is>
+      </c>
+      <c r="I118" s="61" t="inlineStr">
+        <is>
+          <t>La corrección no es castigo por enojo ni maltrato. Nunca el golpe ni la humillación: corregir es formar.</t>
+        </is>
+      </c>
+      <c r="J118" s="61" t="inlineStr">
+        <is>
+          <t>El castigo físico y los insultos presentados como «disciplina».</t>
+        </is>
+      </c>
+      <c r="K118" s="61" t="inlineStr">
+        <is>
+          <t>Si estás enojado, esperá a calmarte antes de corregir.</t>
+        </is>
+      </c>
+      <c r="L118" s="61" t="inlineStr">
+        <is>
+          <t>Corregir con amor trae alegría a la casa. Y los hijos también tienen su parte: honrar y aportar según su edad; darles responsabilidades los hace parte activa de la familia.</t>
+        </is>
+      </c>
+      <c r="M118" s="61" t="inlineStr">
+        <is>
+          <t>Hijos a los que se les hace todo y no aprenden a colaborar.</t>
+        </is>
+      </c>
+      <c r="N118" s="61" t="inlineStr">
+        <is>
+          <t>Dale a cada hijo una tarea de la casa acorde a su edad, y agradecésela cuando la cumpla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="B119" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C119" s="61" t="inlineStr">
+        <is>
+          <t>La fe en lo de todos los días</t>
+        </is>
+      </c>
+      <c r="D119" s="61" t="inlineStr">
+        <is>
+          <t>Deuteronomio 6:4-9, el «Shemá», es la oración que el pueblo judío repite cada mañana y cada noche desde hace siglos.</t>
+        </is>
+      </c>
+      <c r="E119" s="61" t="inlineStr">
+        <is>
+          <t>Deuteronomio 6:4-9; tradición judía</t>
+        </is>
+      </c>
+      <c r="F119" s="61" t="inlineStr">
+        <is>
+          <t>Moisés pide que la Palabra esté primero en el corazón de los padres, y desde ahí se enseñe a los hijos.</t>
+        </is>
+      </c>
+      <c r="G119" s="61" t="inlineStr">
+        <is>
+          <t>Querer que los hijos tengan una fe que los padres no viven.</t>
+        </is>
+      </c>
+      <c r="H119" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, compartí con tus hijos algo que Dios te enseñó a vos.</t>
+        </is>
+      </c>
+      <c r="I119" s="61" t="inlineStr">
+        <is>
+          <t>En la casa, en el camino, al acostarse y al levantarse: la fe se enseña en lo cotidiano, no solo en un momento.</t>
+        </is>
+      </c>
+      <c r="J119" s="61" t="inlineStr">
+        <is>
+          <t>Una fe limitada al domingo.</t>
+        </is>
+      </c>
+      <c r="K119" s="61" t="inlineStr">
+        <is>
+          <t>Aprovechá un viaje o una comida para conversar con tus hijos sobre una pregunta de fe.</t>
+        </is>
+      </c>
+      <c r="L119" s="61" t="inlineStr">
+        <is>
+          <t>Los hijos aprenden a honrar cuando ven a sus padres honrar a otros. La constancia de lo que ven forma su carácter.</t>
+        </is>
+      </c>
+      <c r="M119" s="61" t="inlineStr">
+        <is>
+          <t>Hijos que no ven respeto en casa y no aprenden a darlo.</t>
+        </is>
+      </c>
+      <c r="N119" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, hablá bien de tus padres o de tus suegros delante de tus hijos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="B120" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C120" s="61" t="inlineStr">
+        <is>
+          <t>La mayor alegría</t>
+        </is>
+      </c>
+      <c r="D120" s="61" t="inlineStr">
+        <is>
+          <t>Juan llama «hijos» a los creyentes que él había guiado en la fe.</t>
+        </is>
+      </c>
+      <c r="E120" s="61" t="inlineStr">
+        <is>
+          <t>3 Juan 1:4; 1 Juan 2:1</t>
+        </is>
+      </c>
+      <c r="F120" s="61" t="inlineStr">
+        <is>
+          <t>Juan habla de sus hijos en la fe. Para cualquier padre o madre, ver a los hijos andar en la verdad es la mayor alegría.</t>
+        </is>
+      </c>
+      <c r="G120" s="61" t="inlineStr">
+        <is>
+          <t>Medir el éxito de la crianza solo por los logros académicos o económicos.</t>
+        </is>
+      </c>
+      <c r="H120" s="61" t="inlineStr">
+        <is>
+          <t>Decile hoy a tu hijo algo bueno que ves en su carácter, no en sus notas.</t>
+        </is>
+      </c>
+      <c r="I120" s="61" t="inlineStr">
+        <is>
+          <t>La alegría de ver a los hijos firmes en la fe también pasa por la disciplina: formar el carácter, no castigar. Disciplinar es corregir con propósito.</t>
+        </is>
+      </c>
+      <c r="J120" s="61" t="inlineStr">
+        <is>
+          <t>La disciplina por enojo, que deja heridas en vez de enseñanzas.</t>
+        </is>
+      </c>
+      <c r="K120" s="61" t="inlineStr">
+        <is>
+          <t>Cuando corrijas, explicá qué se espera la próxima vez y terminá con un gesto de cariño.</t>
+        </is>
+      </c>
+      <c r="L120" s="61" t="inlineStr">
+        <is>
+          <t>La fe de los hijos no se impone: se acompaña y se ora. La meta es que anden en la verdad por convicción propia.</t>
+        </is>
+      </c>
+      <c r="M120" s="61" t="inlineStr">
+        <is>
+          <t>Padres que se rinden cuando los hijos adolescentes cuestionan la fe.</t>
+        </is>
+      </c>
+      <c r="N120" s="61" t="inlineStr">
+        <is>
+          <t>Si tu hijo tiene dudas de fe, escuchalo sin enojarte y busquen juntos respuestas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="B121" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C121" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: criar con amor e integridad</t>
+        </is>
+      </c>
+      <c r="D121" s="61" t="inlineStr">
+        <is>
+          <t>En un estudio en Inglaterra y Gales, los adolescentes con abuelos más presentes en su vida tuvieron menos problemas emocionales y de conducta.</t>
+        </is>
+      </c>
+      <c r="E121" s="61" t="inlineStr">
+        <is>
+          <t>Universidad de Oxford, Buchanan y otros, 2008</t>
+        </is>
+      </c>
+      <c r="F121" s="61" t="inlineStr">
+        <is>
+          <t>No hay fórmulas para criar: amor constante, límites claros y ejemplo coherente, día a día.</t>
+        </is>
+      </c>
+      <c r="G121" s="61" t="n"/>
+      <c r="H121" s="61" t="inlineStr">
+        <is>
+          <t>Este fin de semana, compartan un tiempo en familia con abuelos, padres e hijos, y agradezcan a Dios por cada generación.</t>
+        </is>
+      </c>
+      <c r="I121" s="61" t="inlineStr">
+        <is>
+          <t>Los hijos también tienen su parte: honrar y aportar según su edad.</t>
+        </is>
+      </c>
+      <c r="J121" s="61" t="n"/>
+      <c r="K121" s="61" t="n"/>
+      <c r="L121" s="61" t="inlineStr">
+        <is>
+          <t>Disciplinar es corregir con propósito y con amor; nunca con golpes ni humillación.</t>
+        </is>
+      </c>
+      <c r="M121" s="61" t="n"/>
+      <c r="N121" s="61" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="61" t="n">
+        <v>21</v>
+      </c>
+      <c r="B122" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C122" s="61" t="inlineStr">
+        <is>
+          <t>Quien puede trabajar, que trabaje</t>
+        </is>
+      </c>
+      <c r="D122" s="61" t="inlineStr">
+        <is>
+          <t>El apóstol Pablo trabajaba fabricando carpas para sostenerse mientras anunciaba el evangelio.</t>
+        </is>
+      </c>
+      <c r="E122" s="61" t="inlineStr">
+        <is>
+          <t>Hechos 18:3</t>
+        </is>
+      </c>
+      <c r="F122" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribe a creyentes que habían dejado de trabajar esperando la venida de Cristo y vivían a costa de otros. La regla es para el que no quiere trabajar, no para el que no puede.</t>
+        </is>
+      </c>
+      <c r="G122" s="61" t="inlineStr">
+        <is>
+          <t>Juzgar a quien está sin trabajo o enfermo como si fuera perezoso.</t>
+        </is>
+      </c>
+      <c r="H122" s="61" t="inlineStr">
+        <is>
+          <t>Si conocés a alguien que busca trabajo, ayudalo con un contacto, una recomendación o compartiendo su currículum.</t>
+        </is>
+      </c>
+      <c r="I122" s="61" t="inlineStr">
+        <is>
+          <t>Pablo mismo trabajaba con sus manos para no ser una carga (3:8). El trabajo honesto da dignidad.</t>
+        </is>
+      </c>
+      <c r="J122" s="61" t="inlineStr">
+        <is>
+          <t>Depender de otros pudiendo trabajar.</t>
+        </is>
+      </c>
+      <c r="K122" s="61" t="inlineStr">
+        <is>
+          <t>Si estás sin trabajo, organizá tu búsqueda como una tarea diaria, con horario.</t>
+        </is>
+      </c>
+      <c r="L122" s="61" t="inlineStr">
+        <is>
+          <t>Tener una actividad secundaria, aunque sea pequeña, puede dar estabilidad cuando una sola fuente falla. No se trata de vivir para trabajar.</t>
+        </is>
+      </c>
+      <c r="M122" s="61" t="inlineStr">
+        <is>
+          <t>Depender de un solo ingreso y quedar sin nada si se pierde.</t>
+        </is>
+      </c>
+      <c r="N122" s="61" t="inlineStr">
+        <is>
+          <t>Pensá si tenés una habilidad que podría darte un ingreso extra pequeño, sin descuidar a tu familia ni tu descanso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="61" t="n">
+        <v>21</v>
+      </c>
+      <c r="B123" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C123" s="61" t="inlineStr">
+        <is>
+          <t>Manos dispuestas</t>
+        </is>
+      </c>
+      <c r="D123" s="61" t="inlineStr">
+        <is>
+          <t>En Paraguay, alrededor de dos de cada diez personas viven en situación de pobreza.</t>
+        </is>
+      </c>
+      <c r="E123" s="61" t="inlineStr">
+        <is>
+          <t>Instituto Nacional de Estadística (INE), Encuesta Permanente de Hogares Continua</t>
+        </is>
+      </c>
+      <c r="F123" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios observa que la pereza lleva a la escasez. Es un principio, no una explicación de toda pobreza: la Biblia también reconoce la pobreza que viene de la injusticia o de la desgracia.</t>
+        </is>
+      </c>
+      <c r="G123" s="61" t="inlineStr">
+        <is>
+          <t>Culpar a todos los pobres de su situación.</t>
+        </is>
+      </c>
+      <c r="H123" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, apoyá a un emprendimiento o a un trabajador humilde de tu zona comprándole.</t>
+        </is>
+      </c>
+      <c r="I123" s="61" t="inlineStr">
+        <is>
+          <t>Las manos dispuestas abren caminos: constancia, puntualidad, ganas de aprender. No garantizan riqueza, pero honran el trabajo.</t>
+        </is>
+      </c>
+      <c r="J123" s="61" t="inlineStr">
+        <is>
+          <t>Dejar las cosas para mañana y perder oportunidades.</t>
+        </is>
+      </c>
+      <c r="K123" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una tarea que venís postergando y hacela hoy.</t>
+        </is>
+      </c>
+      <c r="L123" s="61" t="inlineStr">
+        <is>
+          <t>Un ingreso secundario pequeño, sostenido en el tiempo, suma más de lo que parece.</t>
+        </is>
+      </c>
+      <c r="M123" s="61" t="inlineStr">
+        <is>
+          <t>Proyectos de ingreso extra que se abandonan al primer mes.</t>
+        </is>
+      </c>
+      <c r="N123" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un emprendimiento pequeño, fijá dos horas por semana para trabajarlo con constancia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="61" t="n">
+        <v>21</v>
+      </c>
+      <c r="B124" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C124" s="61" t="inlineStr">
+        <is>
+          <t>El peso de la deuda</t>
+        </is>
+      </c>
+      <c r="D124" s="61" t="inlineStr">
+        <is>
+          <t>Muchas personas subestiman cuánto crece una deuda con intereses compuestos; los economistas lo llaman «sesgo del crecimiento exponencial».</t>
+        </is>
+      </c>
+      <c r="E124" s="61" t="inlineStr">
+        <is>
+          <t>Stango y Zinman, Journal of Finance, 2009</t>
+        </is>
+      </c>
+      <c r="F124" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio describe una realidad: quien debe, pierde libertad. No prohíbe todo préstamo, pero advierte su peso.</t>
+        </is>
+      </c>
+      <c r="G124" s="61" t="inlineStr">
+        <is>
+          <t>Deudas para gastos que no son necesarios.</t>
+        </is>
+      </c>
+      <c r="H124" s="61" t="inlineStr">
+        <is>
+          <t>Clasificá tus gastos del mes pasado en dos columnas: necesario y deseable.</t>
+        </is>
+      </c>
+      <c r="I124" s="61" t="inlineStr">
+        <is>
+          <t>La deuda no cuesta solo intereses: cuesta paz, sueño y a veces relaciones.</t>
+        </is>
+      </c>
+      <c r="J124" s="61" t="inlineStr">
+        <is>
+          <t>Préstamos entre familiares que terminan en peleas.</t>
+        </is>
+      </c>
+      <c r="K124" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés una deuda con alguien cercano, hablá con esa persona y acuerden un plan de pago, aunque sea pequeño.</t>
+        </is>
+      </c>
+      <c r="L124" s="61" t="inlineStr">
+        <is>
+          <t>Distinguir lo necesario de lo deseable ayuda a decidir dónde recortar cuando no alcanza.</t>
+        </is>
+      </c>
+      <c r="M124" s="61" t="inlineStr">
+        <is>
+          <t>Recortar en lo necesario (salud, comida) para mantener los gustos.</t>
+        </is>
+      </c>
+      <c r="N124" s="61" t="inlineStr">
+        <is>
+          <t>Si este mes no alcanza, recortá primero en la columna de lo deseable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="61" t="n">
+        <v>21</v>
+      </c>
+      <c r="B125" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C125" s="61" t="inlineStr">
+        <is>
+          <t>Fieles en lo poco</t>
+        </is>
+      </c>
+      <c r="D125" s="61" t="inlineStr">
+        <is>
+          <t>Jesús dice estas palabras justo después de la parábola del administrador infiel.</t>
+        </is>
+      </c>
+      <c r="E125" s="61" t="inlineStr">
+        <is>
+          <t>Lucas 16:1-13</t>
+        </is>
+      </c>
+      <c r="F125" s="61" t="inlineStr">
+        <is>
+          <t>Jesús dice esto después de la parábola del administrador: la fidelidad se prueba en lo poco, también en el dinero.</t>
+        </is>
+      </c>
+      <c r="G125" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que los gastos chicos no importan.</t>
+        </is>
+      </c>
+      <c r="H125" s="61" t="inlineStr">
+        <is>
+          <t>Durante una semana, anotá incluso los gastos más pequeños.</t>
+        </is>
+      </c>
+      <c r="I125" s="61" t="inlineStr">
+        <is>
+          <t>Cómo manejamos poco dinero muestra cómo manejaríamos mucho.</t>
+        </is>
+      </c>
+      <c r="J125" s="61" t="inlineStr">
+        <is>
+          <t>Esperar a ganar más para empezar a ordenarse.</t>
+        </is>
+      </c>
+      <c r="K125" s="61" t="inlineStr">
+        <is>
+          <t>Ordená lo que tenés hoy: si ganás poco, empezá con poco.</t>
+        </is>
+      </c>
+      <c r="L125" s="61" t="inlineStr">
+        <is>
+          <t>Ser fiel en la base es poner primero lo primario: las necesidades, las deudas y lo que vamos a dar. Lo secundario, después.</t>
+        </is>
+      </c>
+      <c r="M125" s="61" t="inlineStr">
+        <is>
+          <t>Gastar primero en gustos y llegar a fin de mes sin lo esencial.</t>
+        </is>
+      </c>
+      <c r="N125" s="61" t="inlineStr">
+        <is>
+          <t>Al cobrar, pagá primero lo necesario y lo que vas a dar; después decidí los gustos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="61" t="n">
+        <v>21</v>
+      </c>
+      <c r="B126" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C126" s="61" t="inlineStr">
+        <is>
+          <t>Sabiduría para cerrar fugas</t>
+        </is>
+      </c>
+      <c r="D126" s="61" t="inlineStr">
+        <is>
+          <t>En varios estudios, las personas subestimaron sus gastos «excepcionales», esos que parecen únicos pero en realidad se repiten a lo largo del año.</t>
+        </is>
+      </c>
+      <c r="E126" s="61" t="inlineStr">
+        <is>
+          <t>Sussman y Alter, Journal of Consumer Research, 2012</t>
+        </is>
+      </c>
+      <c r="F126" s="61" t="inlineStr">
+        <is>
+          <t>Santiago describe la sabiduría que viene de Dios: pura, pacífica, genuina. Esa sabiduría también se pide para lo práctico (Santiago 1:5).</t>
+        </is>
+      </c>
+      <c r="G126" s="61" t="inlineStr">
+        <is>
+          <t>Decisiones de dinero tomadas sin pensar ni orar.</t>
+        </is>
+      </c>
+      <c r="H126" s="61" t="inlineStr">
+        <is>
+          <t>Antes de revisar tus gastos, pedile a Dios sabiduría con tus propias palabras.</t>
+        </is>
+      </c>
+      <c r="I126" s="61" t="inlineStr">
+        <is>
+          <t>La sabiduría de lo alto es compasiva: no se trata de ser tacaño, sino de cuidar lo que tenemos para poder cuidar a otros.</t>
+        </is>
+      </c>
+      <c r="J126" s="61" t="inlineStr">
+        <is>
+          <t>Fugas pequeñas que no dejan nada para ayudar a nadie.</t>
+        </is>
+      </c>
+      <c r="K126" s="61" t="inlineStr">
+        <is>
+          <t>Revisá los movimientos de tu cuenta o tu billetera del último mes y buscá gastos pequeños y repetidos que ya no recordás.</t>
+        </is>
+      </c>
+      <c r="L126" s="61" t="inlineStr">
+        <is>
+          <t>Una vez detectadas, las fugas se cierran de a una. Lo que se recupera puede ir al ahorro o a ayudar a alguien.</t>
+        </is>
+      </c>
+      <c r="M126" s="61" t="inlineStr">
+        <is>
+          <t>Suscripciones o servicios que se pagan y no se usan.</t>
+        </is>
+      </c>
+      <c r="N126" s="61" t="inlineStr">
+        <is>
+          <t>Cancelá esta semana un gasto repetido que no usás y destiná ese monto a tu ahorro o a ayudar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="61" t="n">
+        <v>21</v>
+      </c>
+      <c r="B127" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C127" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: orden en lo que entra y lo que sale</t>
+        </is>
+      </c>
+      <c r="D127" s="61" t="inlineStr">
+        <is>
+          <t>Personas que recibieron dinero para gastar en otros se sintieron más felices al final del día que las que lo gastaron en sí mismas, incluso con montos pequeños.</t>
+        </is>
+      </c>
+      <c r="E127" s="61" t="inlineStr">
+        <is>
+          <t>Dunn, Aknin y Norton, revista Science, 2008</t>
+        </is>
+      </c>
+      <c r="F127" s="61" t="inlineStr">
+        <is>
+          <t>Quien puede trabajar, que trabaje; tener más de una fuente de ingreso, si es posible, reduce la vulnerabilidad.</t>
+        </is>
+      </c>
+      <c r="G127" s="61" t="n"/>
+      <c r="H127" s="61" t="inlineStr">
+        <is>
+          <t>Este proverbio no promete que el que da va a recibir más plata: muestra que la generosidad enriquece la vida. Esta semana, cerrá una fuga de dinero y usá ese monto para ayudar a alguien.</t>
+        </is>
+      </c>
+      <c r="I127" s="61" t="inlineStr">
+        <is>
+          <t>Distinguir lo necesario de lo deseable ayuda a decidir dónde recortar.</t>
+        </is>
+      </c>
+      <c r="J127" s="61" t="n"/>
+      <c r="K127" s="61" t="n"/>
+      <c r="L127" s="61" t="inlineStr">
+        <is>
+          <t>Las fugas pequeñas y repetidas pesan más de lo que parece: se encuentran revisando.</t>
+        </is>
+      </c>
+      <c r="M127" s="61" t="n"/>
+      <c r="N127" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de mayo verificados
24 datos contrastados: 14 confirmados, 10 ajustados (pobreza INE 2025 16 %,
efecto de dormir 6 horas, rugido del león con fuente, precisiones de estudios).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -26261,12 +26261,12 @@
       </c>
       <c r="D106" s="61" t="inlineStr">
         <is>
-          <t>En tiempos de Jesús, lavar los pies de los invitados era una tarea que normalmente hacía un sirviente.</t>
+          <t>En tiempos de Jesús, lavar los pies de otra persona se consideraba una tarea de sirvientes: lo normal era que el anfitrión ofreciera agua o que lo hiciera un siervo de la casa.</t>
         </is>
       </c>
       <c r="E106" s="61" t="inlineStr">
         <is>
-          <t>Juan 13:4-5; comentarios bíblicos sobre las costumbres del siglo I</t>
+          <t>Juan 13:4-5; Lucas 7:44; 1 Samuel 25:41</t>
         </is>
       </c>
       <c r="F106" s="61" t="inlineStr">
@@ -26331,12 +26331,12 @@
       </c>
       <c r="D107" s="61" t="inlineStr">
         <is>
-          <t>Se estima que unos 862 millones de personas mayores de 15 años hacen algún tipo de voluntariado cada mes en el mundo.</t>
+          <t>Se estima que unos 862 millones de personas de 15 años o más hacen algún tipo de voluntariado cada mes en el mundo.</t>
         </is>
       </c>
       <c r="E107" s="61" t="inlineStr">
         <is>
-          <t>Voluntarios de las Naciones Unidas, Informe sobre el estado del voluntariado en el mundo, 2022</t>
+          <t>Voluntarios de las Naciones Unidas (VNU), Informe sobre el estado del voluntariado en el mundo, 2022</t>
         </is>
       </c>
       <c r="F107" s="61" t="inlineStr">
@@ -26406,7 +26406,7 @@
       </c>
       <c r="E108" s="61" t="inlineStr">
         <is>
-          <t>Mihaly Csikszentmihalyi, «Fluir», 1990</t>
+          <t>Mihaly Csikszentmihalyi, «Flow», 1990 (en español, «Fluir», 1997)</t>
         </is>
       </c>
       <c r="F108" s="61" t="inlineStr">
@@ -26521,12 +26521,12 @@
       </c>
       <c r="D110" s="61" t="inlineStr">
         <is>
-          <t>Las experiencias negativas nos impactan más que las positivas: una crítica suele pesar más que varios elogios.</t>
+          <t>Las experiencias negativas suelen impactarnos más que las positivas: por ejemplo, una crítica suele pesar más que un elogio.</t>
         </is>
       </c>
       <c r="E110" s="61" t="inlineStr">
         <is>
-          <t>Baumeister y otros, «Bad is stronger than good», Review of General Psychology, 2001</t>
+          <t>Baumeister, Bratslavsky, Finkenauer y Vohs, «Bad is stronger than good», Review of General Psychology, 2001</t>
         </is>
       </c>
       <c r="F110" s="61" t="inlineStr">
@@ -26591,12 +26591,12 @@
       </c>
       <c r="D111" s="61" t="inlineStr">
         <is>
-          <t>El rugido de un león puede oírse a varios kilómetros de distancia.</t>
+          <t>En la sabana abierta, el rugido de un león puede oírse hasta a unos 8 kilómetros de distancia.</t>
         </is>
       </c>
       <c r="E111" s="61" t="inlineStr">
         <is>
-          <t>Estudios sobre comportamiento de leones</t>
+          <t>IFAW (Fondo Internacional para el Bienestar Animal)</t>
         </is>
       </c>
       <c r="F111" s="61" t="inlineStr">
@@ -26661,12 +26661,12 @@
       </c>
       <c r="D112" s="61" t="inlineStr">
         <is>
-          <t>En un estudio en hospitales, los equipos con mejores líderes reportaban más errores: no porque se equivocaran más, sino porque se animaban a decirlos.</t>
+          <t>En un estudio en un hospital, los equipos de enfermería con mejor liderazgo registraban más errores de medicación; según la autora, no se equivocaban más, sino que se animaban a reportarlos.</t>
         </is>
       </c>
       <c r="E112" s="61" t="inlineStr">
         <is>
-          <t>Amy Edmondson, Universidad de Harvard, Journal of Applied Behavioral Science, 1996</t>
+          <t>Amy Edmondson, Journal of Applied Behavioral Science, 1996</t>
         </is>
       </c>
       <c r="F112" s="61" t="inlineStr">
@@ -26801,7 +26801,7 @@
       </c>
       <c r="D114" s="61" t="inlineStr">
         <is>
-          <t>Dormir unas seis horas por noche durante dos semanas afectó el rendimiento casi tanto como pasar dos noches sin dormir, y los participantes no se daban cuenta.</t>
+          <t>Dormir seis horas por noche durante dos semanas afectó la atención casi tanto como pasar una noche entera sin dormir, y los participantes apenas se sentían más somnolientos.</t>
         </is>
       </c>
       <c r="E114" s="61" t="inlineStr">
@@ -27391,12 +27391,12 @@
       </c>
       <c r="D123" s="61" t="inlineStr">
         <is>
-          <t>En Paraguay, alrededor de dos de cada diez personas viven en situación de pobreza.</t>
+          <t>En Paraguay, alrededor de 16 de cada 100 personas viven en situación de pobreza.</t>
         </is>
       </c>
       <c r="E123" s="61" t="inlineStr">
         <is>
-          <t>Instituto Nacional de Estadística (INE), Encuesta Permanente de Hogares Continua</t>
+          <t>Instituto Nacional de Estadística (INE), Encuesta Permanente de Hogares Continua 2025</t>
         </is>
       </c>
       <c r="F123" s="61" t="inlineStr">
@@ -27461,7 +27461,7 @@
       </c>
       <c r="D124" s="61" t="inlineStr">
         <is>
-          <t>Muchas personas subestiman cuánto crece una deuda con intereses compuestos; los economistas lo llaman «sesgo del crecimiento exponencial».</t>
+          <t>Muchas personas subestiman cuánto crece el dinero con intereses compuestos, tanto una deuda como un ahorro; los economistas lo llaman «sesgo del crecimiento exponencial».</t>
         </is>
       </c>
       <c r="E124" s="61" t="inlineStr">
@@ -27531,12 +27531,12 @@
       </c>
       <c r="D125" s="61" t="inlineStr">
         <is>
-          <t>Jesús dice estas palabras justo después de la parábola del administrador infiel.</t>
+          <t>Las palabras de Jesús sobre ser fiel en lo poco vienen justo después de la parábola del administrador infiel.</t>
         </is>
       </c>
       <c r="E125" s="61" t="inlineStr">
         <is>
-          <t>Lucas 16:1-13</t>
+          <t>Lucas 16:1-9 y 16:10-13</t>
         </is>
       </c>
       <c r="F125" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: junio (semanas 22 a 26) con revisión teológica; datos en verificación
- 30 guiones: desarrollo profesional, emprendimientos, nutrición, discipulado y equipo
- Job 8:7 explicado como palabras de Bildad; sugerencia recomendada: Zacarías 4:10
- 4 puntos corregidos y errata «Tesalonicenses»

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -5452,7 +5452,7 @@
       </c>
       <c r="AJ23" s="43" t="inlineStr">
         <is>
-          <t>1 Tesalonisenses 5:11 — Por lo tanto, anímense y edifíquense unos a otros, como en efecto ya lo hacen.</t>
+          <t>1 Tesalonicenses 5:11 — Por lo tanto, anímense y edifíquense unos a otros, como en efecto ya lo hacen.</t>
         </is>
       </c>
       <c r="AK23" s="43" t="inlineStr">
@@ -5614,9 +5614,9 @@
       </c>
       <c r="AC24" s="47" t="inlineStr">
         <is>
-          <t>• Dios puede restaurar: Lo poco puede convertirse en mucho.  
-• Esperar en Dios: El proceso no define el resultado.  
-• Un futuro mejor: Dios puede traer mayor bendición después.</t>
+          <t>• Quien habla es Bildad: Un amigo de Job cuya idea de Dios fue corregida (42:7).  
+• Los comienzos pequeños: No definen el final ni son una vergüenza.  
+• Dios no abandona: Restauró a Job por gracia, no como pago.</t>
         </is>
       </c>
       <c r="AD24" s="47" t="inlineStr">
@@ -5873,7 +5873,7 @@
       </c>
       <c r="AK25" s="49" t="inlineStr">
         <is>
-          <t>• La dieta sencilla mostró mejores resultados
+          <t>• Dios honró la fidelidad de Daniel
 • Lo simple puede ser más saludable
 • La fe se demuestra también en decisiones cotidianas</t>
         </is>
@@ -19214,7 +19214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N127"/>
+  <dimension ref="A1:N157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -27704,6 +27704,2006 @@
       </c>
       <c r="M127" s="61" t="n"/>
       <c r="N127" s="61" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="B128" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C128" s="61" t="inlineStr">
+        <is>
+          <t>Siempre listos</t>
+        </is>
+      </c>
+      <c r="D128" s="61" t="inlineStr">
+        <is>
+          <t>Según el Foro Económico Mundial, cerca del 39 % de las habilidades clave de los trabajadores cambiarán hacia 2030.</t>
+        </is>
+      </c>
+      <c r="E128" s="61" t="inlineStr">
+        <is>
+          <t>Foro Económico Mundial, Informe sobre el futuro del empleo, 2025</t>
+        </is>
+      </c>
+      <c r="F128" s="61" t="inlineStr">
+        <is>
+          <t>Pedro escribe a cristianos que sufrían por su fe: primero, honrar a Cristo en el corazón. Desde ahí se vive todo, también el trabajo.</t>
+        </is>
+      </c>
+      <c r="G128" s="61" t="inlineStr">
+        <is>
+          <t>Separar la fe del trabajo, como si fueran mundos aparte.</t>
+        </is>
+      </c>
+      <c r="H128" s="61" t="inlineStr">
+        <is>
+          <t>Empezá tu jornada pidiéndole a Dios que te ayude a honrarlo en tu trabajo de hoy.</t>
+        </is>
+      </c>
+      <c r="I128" s="61" t="inlineStr">
+        <is>
+          <t>«Manténganse siempre listos»: Pedro habla de saber explicar nuestra esperanza, y el principio de prepararse vale también para el oficio. Aprender más de lo que el puesto exige hoy prepara para lo que viene.</t>
+        </is>
+      </c>
+      <c r="J128" s="61" t="inlineStr">
+        <is>
+          <t>Hacer solo lo mínimo y quedarse atrás cuando cambia el trabajo.</t>
+        </is>
+      </c>
+      <c r="K128" s="61" t="inlineStr">
+        <is>
+          <t>Reservá un tiempo fijo por semana, aunque sea media hora, para aprender algo nuevo de tu oficio.</t>
+        </is>
+      </c>
+      <c r="L128" s="61" t="inlineStr">
+        <is>
+          <t>Pedro pide responder con mansedumbre y respeto. Prepararse no es para presumir, sino para servir mejor.</t>
+        </is>
+      </c>
+      <c r="M128" s="61" t="inlineStr">
+        <is>
+          <t>Personas capaces que tratan con soberbia a los que saben menos.</t>
+        </is>
+      </c>
+      <c r="N128" s="61" t="inlineStr">
+        <is>
+          <t>Si sabés algo que a un compañero le cuesta, ofrecete a explicárselo con paciencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="B129" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C129" s="61" t="inlineStr">
+        <is>
+          <t>Con todas tus fuerzas</t>
+        </is>
+      </c>
+      <c r="D129" s="61" t="inlineStr">
+        <is>
+          <t>El Servicio Nacional de Promoción Profesional (SNPP) ofrece cursos gratuitos de formación en oficios en todo el país.</t>
+        </is>
+      </c>
+      <c r="E129" s="61" t="inlineStr">
+        <is>
+          <t>Servicio Nacional de Promoción Profesional, Ministerio de Trabajo, Empleo y Seguridad Social</t>
+        </is>
+      </c>
+      <c r="F129" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés recuerda que la vida es breve: lo que hoy podés hacer, hacelo bien y con ganas. No es ansiedad, es aprovechar el regalo del tiempo.</t>
+        </is>
+      </c>
+      <c r="G129" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar desganado, contando las horas.</t>
+        </is>
+      </c>
+      <c r="H129" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una tarea de hoy y hacela con todas tus ganas, como si fuera la más importante.</t>
+        </is>
+      </c>
+      <c r="I129" s="61" t="inlineStr">
+        <is>
+          <t>La mediocridad no es falta de talento, sino de entrega. Hacer bien lo que nos toca es una forma de responsabilidad.</t>
+        </is>
+      </c>
+      <c r="J129" s="61" t="inlineStr">
+        <is>
+          <t>Excusarse en que el sueldo es bajo para trabajar mal.</t>
+        </is>
+      </c>
+      <c r="K129" s="61" t="inlineStr">
+        <is>
+          <t>Anotá una cosa de tu trabajo que podrías hacer mejor esta semana, y mejorala.</t>
+        </is>
+      </c>
+      <c r="L129" s="61" t="inlineStr">
+        <is>
+          <t>Capacitarse también es parte del esfuerzo: nadie nace sabiendo y siempre se puede aprender un poco más.</t>
+        </is>
+      </c>
+      <c r="M129" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que ya es tarde para estudiar o aprender un oficio nuevo.</t>
+        </is>
+      </c>
+      <c r="N129" s="61" t="inlineStr">
+        <is>
+          <t>Averiguá esta semana un curso gratuito del SNPP o de otra institución que te sirva para tu trabajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="B130" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C130" s="61" t="inlineStr">
+        <is>
+          <t>Estudiar, hacer y enseñar</t>
+        </is>
+      </c>
+      <c r="D130" s="61" t="inlineStr">
+        <is>
+          <t>Practicar con un objetivo concreto y con la devolución de alguien que sabe mejora mucho más que solo repetir; los investigadores lo llamaron «práctica deliberada».</t>
+        </is>
+      </c>
+      <c r="E130" s="61" t="inlineStr">
+        <is>
+          <t>Ericsson, Krampe y Tesch-Römer, Psychological Review, 1993</t>
+        </is>
+      </c>
+      <c r="F130" s="61" t="inlineStr">
+        <is>
+          <t>Esdras se entregó de corazón a estudiar la ley de Dios. Conocer bien lo que hacemos empieza por estudiar con dedicación.</t>
+        </is>
+      </c>
+      <c r="G130" s="61" t="inlineStr">
+        <is>
+          <t>Querer crecer sin dedicar tiempo a aprender.</t>
+        </is>
+      </c>
+      <c r="H130" s="61" t="inlineStr">
+        <is>
+          <t>Fijate en qué sos bueno con naturalidad y buscá un libro, un curso o un video serio para mejorarlo.</t>
+        </is>
+      </c>
+      <c r="I130" s="61" t="inlineStr">
+        <is>
+          <t>Esdras no solo estudió: la cumplió. Las habilidades crecen practicando, no solo leyendo.</t>
+        </is>
+      </c>
+      <c r="J130" s="61" t="inlineStr">
+        <is>
+          <t>Saber mucho en teoría y poco en la práctica.</t>
+        </is>
+      </c>
+      <c r="K130" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, practicá a propósito una habilidad que querés mejorar, y pedile a alguien que te diga cómo lo hiciste.</t>
+        </is>
+      </c>
+      <c r="L130" s="61" t="inlineStr">
+        <is>
+          <t>Y la enseñó a otros. Cada uno destaca en algo distinto, y en lo que sos bueno podés ayudar a otros a crecer.</t>
+        </is>
+      </c>
+      <c r="M130" s="61" t="inlineStr">
+        <is>
+          <t>Compararse con otros y querer ser bueno en todo por igual.</t>
+        </is>
+      </c>
+      <c r="N130" s="61" t="inlineStr">
+        <is>
+          <t>Preguntate: ¿qué tarea me sale con más facilidad que a la mayoría? Esa suele ser una pista de tu habilidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="B131" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C131" s="61" t="inlineStr">
+        <is>
+          <t>No solo cuando miran</t>
+        </is>
+      </c>
+      <c r="D131" s="61" t="inlineStr">
+        <is>
+          <t>La palabra griega que Pablo usa aquí significa literalmente «servicio para el ojo»: trabajar solo cuando nos ven.</t>
+        </is>
+      </c>
+      <c r="E131" s="61" t="inlineStr">
+        <is>
+          <t>Léxico griego de Strong (G3787, ofthalmodoulía)</t>
+        </is>
+      </c>
+      <c r="F131" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribe a esclavos de su tiempo: trabajen de corazón, como siervos de Cristo. Ningún trabajo honesto queda fuera de la mirada de Dios.</t>
+        </is>
+      </c>
+      <c r="G131" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar bien solo cuando hay control.</t>
+        </is>
+      </c>
+      <c r="H131" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy una tarea con la misma calidad que si te estuvieran evaluando.</t>
+        </is>
+      </c>
+      <c r="I131" s="61" t="inlineStr">
+        <is>
+          <t>Agradar a la gente no es el objetivo; hacer la voluntad de Dios sí. Eso libera de la presión por aparentar.</t>
+        </is>
+      </c>
+      <c r="J131" s="61" t="inlineStr">
+        <is>
+          <t>Vivir pendiente de la aprobación del jefe o de los compañeros.</t>
+        </is>
+      </c>
+      <c r="K131" s="61" t="inlineStr">
+        <is>
+          <t>Cuando hagas algo bien esta semana, agradecé a Dios antes de esperar el reconocimiento de otros.</t>
+        </is>
+      </c>
+      <c r="L131" s="61" t="inlineStr">
+        <is>
+          <t>Desarrollar las propias habilidades también es mayordomía: lo que Dios nos dio, lo hacemos crecer para servir mejor.</t>
+        </is>
+      </c>
+      <c r="M131" s="61" t="inlineStr">
+        <is>
+          <t>Desperdiciar un talento por miedo o por comodidad.</t>
+        </is>
+      </c>
+      <c r="N131" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una de tus habilidades y pensá cómo usarla mejor en tu trabajo este mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="B132" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C132" s="61" t="inlineStr">
+        <is>
+          <t>Un espíritu superior</t>
+        </is>
+      </c>
+      <c r="D132" s="61" t="inlineStr">
+        <is>
+          <t>Daniel sirvió en la corte de Babilonia y después en la de Persia durante más de sesenta años, bajo varios reyes.</t>
+        </is>
+      </c>
+      <c r="E132" s="61" t="inlineStr">
+        <is>
+          <t>Daniel 1:21; 6:28</t>
+        </is>
+      </c>
+      <c r="F132" s="61" t="inlineStr">
+        <is>
+          <t>Daniel se destacó por un espíritu superior, y la Biblia muestra que su sabiduría venía de Dios (Daniel 1:17). Él la cultivó con fidelidad.</t>
+        </is>
+      </c>
+      <c r="G132" s="61" t="inlineStr">
+        <is>
+          <t>Buscar destacarse a cualquier costo.</t>
+        </is>
+      </c>
+      <c r="H132" s="61" t="inlineStr">
+        <is>
+          <t>Pedile a Dios sabiduría para tu trabajo, y cultivala con constancia.</t>
+        </is>
+      </c>
+      <c r="I132" s="61" t="inlineStr">
+        <is>
+          <t>Daniel aprendió de maestros en Babilonia y sirvió a varios reyes: aprender de los que saben acelera el camino.</t>
+        </is>
+      </c>
+      <c r="J132" s="61" t="inlineStr">
+        <is>
+          <t>Querer resolverlo todo solo y repetir errores que otros ya cometieron.</t>
+        </is>
+      </c>
+      <c r="K132" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en alguien que ya recorrió el camino que estás empezando y pedile consejo esta semana.</t>
+        </is>
+      </c>
+      <c r="L132" s="61" t="inlineStr">
+        <is>
+          <t>Sus enemigos no encontraron falta en él (6:4). La integridad sostuvo su reconocimiento cuando lo quisieron hacer caer.</t>
+        </is>
+      </c>
+      <c r="M132" s="61" t="inlineStr">
+        <is>
+          <t>Ascensos logrados con atajos que después se derrumban.</t>
+        </is>
+      </c>
+      <c r="N132" s="61" t="inlineStr">
+        <is>
+          <t>Si te ofrecen un atajo deshonesto para avanzar, decí que no. Tu nombre vale más.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="61" t="n">
+        <v>22</v>
+      </c>
+      <c r="B133" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C133" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: crecer y ayudar a crecer</t>
+        </is>
+      </c>
+      <c r="D133" s="61" t="inlineStr">
+        <is>
+          <t>En una empresa tecnológica de Estados Unidos, los empleados que recibieron mentoría fueron ascendidos con mucha más frecuencia que los que no la tuvieron.</t>
+        </is>
+      </c>
+      <c r="E133" s="61" t="inlineStr">
+        <is>
+          <t>Gartner, estudio para Sun Microsystems, 2006</t>
+        </is>
+      </c>
+      <c r="F133" s="61" t="inlineStr">
+        <is>
+          <t>Capacitarse más allá de lo obligatorio prepara para las oportunidades de mañana.</t>
+        </is>
+      </c>
+      <c r="G133" s="61" t="n"/>
+      <c r="H133" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide animarse y edificarse unos a otros. Esta semana, pedí consejo a alguien con más experiencia y ofrecé el tuyo a alguien que está empezando.</t>
+        </is>
+      </c>
+      <c r="I133" s="61" t="inlineStr">
+        <is>
+          <t>Cada uno destaca en algo: identificar y pulir esa habilidad rinde más que querer ser bueno en todo.</t>
+        </is>
+      </c>
+      <c r="J133" s="61" t="n"/>
+      <c r="K133" s="61" t="n"/>
+      <c r="L133" s="61" t="inlineStr">
+        <is>
+          <t>Aprender de quienes ya recorrieron el camino evita tropiezos innecesarios.</t>
+        </is>
+      </c>
+      <c r="M133" s="61" t="n"/>
+      <c r="N133" s="61" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="61" t="n">
+        <v>23</v>
+      </c>
+      <c r="B134" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C134" s="61" t="inlineStr">
+        <is>
+          <t>Dios va delante</t>
+        </is>
+      </c>
+      <c r="D134" s="61" t="inlineStr">
+        <is>
+          <t>En muchos países, cerca de la mitad de los adultos que ven una buena oportunidad para emprender dice que el miedo a fracasar lo frenaría.</t>
+        </is>
+      </c>
+      <c r="E134" s="61" t="inlineStr">
+        <is>
+          <t>Global Entrepreneurship Monitor (GEM), informe mundial</t>
+        </is>
+      </c>
+      <c r="F134" s="61" t="inlineStr">
+        <is>
+          <t>Moisés le habla a Josué antes de entrar a una tierra nueva: el Señor va delante de ti. Empezar algo nuevo da miedo, pero no estamos solos.</t>
+        </is>
+      </c>
+      <c r="G134" s="61" t="inlineStr">
+        <is>
+          <t>El miedo a empezar, que paraliza ideas buenas durante años.</t>
+        </is>
+      </c>
+      <c r="H134" s="61" t="inlineStr">
+        <is>
+          <t>Escribí la idea de negocio o de proyecto que venís postergando, y un primer paso pequeño para esta semana.</t>
+        </is>
+      </c>
+      <c r="I134" s="61" t="inlineStr">
+        <is>
+          <t>Dios no promete que todo salga bien, sino que no nos deja. Eso da valor para dar el primer paso.</t>
+        </is>
+      </c>
+      <c r="J134" s="61" t="inlineStr">
+        <is>
+          <t>Esperar a tener todo resuelto para recién empezar, y nunca empezar.</t>
+        </is>
+      </c>
+      <c r="K134" s="61" t="inlineStr">
+        <is>
+          <t>Empezá con lo que tenés: una herramienta, un saber, un horario libre.</t>
+        </is>
+      </c>
+      <c r="L134" s="61" t="inlineStr">
+        <is>
+          <t>«No temas»: la prudencia es buena; el miedo que paraliza, no. Se puede empezar en pequeño y aprender en el camino.</t>
+        </is>
+      </c>
+      <c r="M134" s="61" t="inlineStr">
+        <is>
+          <t>Endeudarse mucho para empezar en grande.</t>
+        </is>
+      </c>
+      <c r="N134" s="61" t="inlineStr">
+        <is>
+          <t>Pensá cómo podrías probar tu idea en pequeño, sin endeudarte, durante un mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="61" t="n">
+        <v>23</v>
+      </c>
+      <c r="B135" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C135" s="61" t="inlineStr">
+        <is>
+          <t>Comienzos pequeños</t>
+        </is>
+      </c>
+      <c r="D135" s="61" t="inlineStr">
+        <is>
+          <t>Al final del libro de Job, Dios dice a los amigos de Job que no hablaron de Él con verdad.</t>
+        </is>
+      </c>
+      <c r="E135" s="61" t="inlineStr">
+        <is>
+          <t>Job 42:7</t>
+        </is>
+      </c>
+      <c r="F135" s="61" t="inlineStr">
+        <is>
+          <t>Esta frase la dice Bildad, uno de los amigos de Job. Él pensaba que a los justos siempre les va bien, y al final Dios corrige a esos amigos (42:7). Por eso no la tomamos como una promesa de riqueza.</t>
+        </is>
+      </c>
+      <c r="G135" s="61" t="inlineStr">
+        <is>
+          <t>Prometer prosperidad segura a quien emprende «si tiene fe».</t>
+        </is>
+      </c>
+      <c r="H135" s="61" t="inlineStr">
+        <is>
+          <t>Si alguien te promete ganancias seguras, desconfiá, aunque use versículos.</t>
+        </is>
+      </c>
+      <c r="I135" s="61" t="inlineStr">
+        <is>
+          <t>Lo que sí es cierto es que empezar con poco no es una vergüenza. Muchos emprendimientos sólidos empezaron con muy poco.</t>
+        </is>
+      </c>
+      <c r="J135" s="61" t="inlineStr">
+        <is>
+          <t>La vergüenza de empezar con un puesto pequeño, con ventas por WhatsApp o desde la cocina de casa.</t>
+        </is>
+      </c>
+      <c r="K135" s="61" t="inlineStr">
+        <is>
+          <t>Si empezaste en pequeño, sacale una foto a tu comienzo: algún día te va a recordar de dónde saliste.</t>
+        </is>
+      </c>
+      <c r="L135" s="61" t="inlineStr">
+        <is>
+          <t>La historia de Job enseña que Dios está presente también cuando todo se pierde. Al final restauró a Job, pero por gracia, no como pago.</t>
+        </is>
+      </c>
+      <c r="M135" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que, si un negocio fracasa, es porque Dios nos castiga.</t>
+        </is>
+      </c>
+      <c r="N135" s="61" t="inlineStr">
+        <is>
+          <t>Si tu emprendimiento pasa por un mal momento, hablalo con alguien de confianza y no lo cargues como culpa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="61" t="n">
+        <v>23</v>
+      </c>
+      <c r="B136" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C136" s="61" t="inlineStr">
+        <is>
+          <t>Sembrar sin saber</t>
+        </is>
+      </c>
+      <c r="D136" s="61" t="inlineStr">
+        <is>
+          <t>En Estados Unidos, alrededor de uno de cada cinco negocios nuevos cierra durante su primer año.</t>
+        </is>
+      </c>
+      <c r="E136" s="61" t="inlineStr">
+        <is>
+          <t>Oficina de Estadísticas Laborales de EE. UU. (BLS)</t>
+        </is>
+      </c>
+      <c r="F136" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés reconoce que no sabemos qué va a funcionar, y por eso aconseja sembrar con constancia. Emprender es trabajar sin certezas.</t>
+        </is>
+      </c>
+      <c r="G136" s="61" t="inlineStr">
+        <is>
+          <t>Poner todo en una sola idea sin probarla antes.</t>
+        </is>
+      </c>
+      <c r="H136" s="61" t="inlineStr">
+        <is>
+          <t>Antes de invertir, hacé una prueba pequeña: vendé a diez personas y escuchá lo que dicen.</t>
+        </is>
+      </c>
+      <c r="I136" s="61" t="inlineStr">
+        <is>
+          <t>La incertidumbre no es excusa para no hacer nada, pero sí es una razón para contar el costo antes. Contar el costo no apaga el entusiasmo: lo hace sostenible.</t>
+        </is>
+      </c>
+      <c r="J136" s="61" t="inlineStr">
+        <is>
+          <t>Emprender con entusiasmo sin calcular los gastos reales de tiempo, dinero y riesgo.</t>
+        </is>
+      </c>
+      <c r="K136" s="61" t="inlineStr">
+        <is>
+          <t>Escribí en una hoja todos los gastos reales previstos del primer año, no solo la idea del negocio.</t>
+        </is>
+      </c>
+      <c r="L136" s="61" t="inlineStr">
+        <is>
+          <t>La constancia, junto con un buen cálculo, es la combinación que sostiene un emprendimiento.</t>
+        </is>
+      </c>
+      <c r="M136" s="61" t="inlineStr">
+        <is>
+          <t>Mezclar la plata del negocio con la de la casa.</t>
+        </is>
+      </c>
+      <c r="N136" s="61" t="inlineStr">
+        <is>
+          <t>Separá desde el primer día la plata del emprendimiento de la de tu familia, aunque sea en dos sobres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="61" t="n">
+        <v>23</v>
+      </c>
+      <c r="B137" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C137" s="61" t="inlineStr">
+        <is>
+          <t>No creer todo lo que se oye</t>
+        </is>
+      </c>
+      <c r="D137" s="61" t="inlineStr">
+        <is>
+          <t>En Estados Unidos, las estafas de inversión fueron en 2024 la categoría con más pérdidas reportadas: unos 5.700 millones de dólares.</t>
+        </is>
+      </c>
+      <c r="E137" s="61" t="inlineStr">
+        <is>
+          <t>Comisión Federal de Comercio de EE. UU. (FTC), 2025</t>
+        </is>
+      </c>
+      <c r="F137" s="61" t="inlineStr">
+        <is>
+          <t>El inexperto cree todo lo que oye; el prudente mira por dónde anda. Emprender exige discernimiento.</t>
+        </is>
+      </c>
+      <c r="G137" s="61" t="inlineStr">
+        <is>
+          <t>Negocios «milagrosos» que se promocionan en redes y en grupos de mensajes.</t>
+        </is>
+      </c>
+      <c r="H137" s="61" t="inlineStr">
+        <is>
+          <t>Antes de entrar en un negocio que te ofrecen, preguntá: ¿cómo gana plata realmente? Si no lo entendés, no entres.</t>
+        </is>
+      </c>
+      <c r="I137" s="61" t="inlineStr">
+        <is>
+          <t>Examinar antes de aceptar: pedir números, consultar, comparar.</t>
+        </is>
+      </c>
+      <c r="J137" s="61" t="inlineStr">
+        <is>
+          <t>Contratos firmados sin leer.</t>
+        </is>
+      </c>
+      <c r="K137" s="61" t="inlineStr">
+        <is>
+          <t>No firmes nada sin leerlo completo; si hay algo que no entendés, consultalo antes.</t>
+        </is>
+      </c>
+      <c r="L137" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar el propio camino también es cuidar a la familia que depende de esa decisión.</t>
+        </is>
+      </c>
+      <c r="M137" s="61" t="inlineStr">
+        <is>
+          <t>Decisiones de negocio tomadas a escondidas de la familia.</t>
+        </is>
+      </c>
+      <c r="N137" s="61" t="inlineStr">
+        <is>
+          <t>Contale a tu familia tus planes de negocio y escuchá sus preguntas antes de decidir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="61" t="n">
+        <v>23</v>
+      </c>
+      <c r="B138" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C138" s="61" t="inlineStr">
+        <is>
+          <t>Fiel en lo poco</t>
+        </is>
+      </c>
+      <c r="D138" s="61" t="inlineStr">
+        <is>
+          <t>Un talento, en tiempos de Jesús, equivalía a unos 6.000 denarios, el salario de muchos años de trabajo de un jornalero.</t>
+        </is>
+      </c>
+      <c r="E138" s="61" t="inlineStr">
+        <is>
+          <t>Mateo 20:2; diccionarios bíblicos</t>
+        </is>
+      </c>
+      <c r="F138" s="61" t="inlineStr">
+        <is>
+          <t>En la parábola de los talentos, el señor alaba al que fue fiel con lo que se le confió. La fidelidad se prueba en lo poco y en lo cotidiano.</t>
+        </is>
+      </c>
+      <c r="G138" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar un emprendimiento en la etapa difícil, cuando el esfuerzo todavía no se ve.</t>
+        </is>
+      </c>
+      <c r="H138" s="61" t="inlineStr">
+        <is>
+          <t>Si tu emprendimiento está cuesta arriba, anotá qué ajustar sin abandonar: un precio, un horario, un producto.</t>
+        </is>
+      </c>
+      <c r="I138" s="61" t="inlineStr">
+        <is>
+          <t>La recompensa de la parábola es «el gozo de tu señor»: estar con Él. No es una promesa de ganancias, es una invitación a la fidelidad.</t>
+        </is>
+      </c>
+      <c r="J138" s="61" t="inlineStr">
+        <is>
+          <t>Medir la fidelidad a Dios por cuánto rinde el negocio.</t>
+        </is>
+      </c>
+      <c r="K138" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé a Dios por lo que hoy tenés en tus manos, sea mucho o poco.</t>
+        </is>
+      </c>
+      <c r="L138" s="61" t="inlineStr">
+        <is>
+          <t>Perseverar con fidelidad trae gozo, también cuando el camino es largo.</t>
+        </is>
+      </c>
+      <c r="M138" s="61" t="inlineStr">
+        <is>
+          <t>Emprendedores que se sienten solos en sus momentos más difíciles.</t>
+        </is>
+      </c>
+      <c r="N138" s="61" t="inlineStr">
+        <is>
+          <t>Si sos emprendedor, buscá a otro emprendedor para contarse lo que los ayudó a sostenerse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="61" t="n">
+        <v>23</v>
+      </c>
+      <c r="B139" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C139" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: emprender con fe y con cuidado</t>
+        </is>
+      </c>
+      <c r="D139" s="61" t="inlineStr">
+        <is>
+          <t>Jesús dijo estas palabras al día siguiente de multiplicar los panes para unas cinco mil personas.</t>
+        </is>
+      </c>
+      <c r="E139" s="61" t="inlineStr">
+        <is>
+          <t>Juan 6:10-27</t>
+        </is>
+      </c>
+      <c r="F139" s="61" t="inlineStr">
+        <is>
+          <t>Animarse a empezar con lo que hay: los comienzos pequeños no definen el final.</t>
+        </is>
+      </c>
+      <c r="G139" s="61" t="n"/>
+      <c r="H139" s="61" t="inlineStr">
+        <is>
+          <t>Jesús recuerda que trabajamos por algo más que el pan. Esta semana, poné tus planes de trabajo delante de Dios y separá tiempo para tu familia y tu fe.</t>
+        </is>
+      </c>
+      <c r="I139" s="61" t="inlineStr">
+        <is>
+          <t>Contar el costo antes de emprender hace sostenible el entusiasmo.</t>
+        </is>
+      </c>
+      <c r="J139" s="61" t="n"/>
+      <c r="K139" s="61" t="n"/>
+      <c r="L139" s="61" t="inlineStr">
+        <is>
+          <t>Perseverar en la etapa difícil, ajustando sin abandonar, distingue a los que siguen.</t>
+        </is>
+      </c>
+      <c r="M139" s="61" t="n"/>
+      <c r="N139" s="61" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="B140" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C140" s="61" t="inlineStr">
+        <is>
+          <t>La prueba de Daniel</t>
+        </is>
+      </c>
+      <c r="D140" s="61" t="inlineStr">
+        <is>
+          <t>La Organización Mundial de la Salud recomienda comer al menos 400 gramos de frutas y verduras por día, unas cinco porciones.</t>
+        </is>
+      </c>
+      <c r="E140" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, nota descriptiva sobre alimentación sana</t>
+        </is>
+      </c>
+      <c r="F140" s="61" t="inlineStr">
+        <is>
+          <t>Daniel no hizo una dieta para verse mejor: no quería contaminarse con la comida del rey, probablemente ligada a la idolatría (1:8). Su motivo fue la fidelidad a Dios.</t>
+        </is>
+      </c>
+      <c r="G140" s="61" t="inlineStr">
+        <is>
+          <t>Usar la Biblia para justificar dietas de moda.</t>
+        </is>
+      </c>
+      <c r="H140" s="61" t="inlineStr">
+        <is>
+          <t>Cuando escuches hablar de una «dieta bíblica» milagrosa, desconfiá y consultá a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="I140" s="61" t="inlineStr">
+        <is>
+          <t>Comer bien no es comer poco: es elegir alimentos que nutran de verdad, como legumbres, frutas y verduras.</t>
+        </is>
+      </c>
+      <c r="J140" s="61" t="inlineStr">
+        <is>
+          <t>Saltear comidas creyendo que así se come mejor.</t>
+        </is>
+      </c>
+      <c r="K140" s="61" t="inlineStr">
+        <is>
+          <t>Sumá hoy una porción de legumbres o de verduras a tu almuerzo, sin dejar de comer.</t>
+        </is>
+      </c>
+      <c r="L140" s="61" t="inlineStr">
+        <is>
+          <t>Las decisiones de cada día, también en la mesa, pueden ser una forma de honrar a Dios, sin obsesión ni culpa.</t>
+        </is>
+      </c>
+      <c r="M140" s="61" t="inlineStr">
+        <is>
+          <t>La obsesión por la comida, que ocupa la mente todo el día.</t>
+        </is>
+      </c>
+      <c r="N140" s="61" t="inlineStr">
+        <is>
+          <t>Antes de comer, agradecé a Dios por la comida: es una forma simple de recordar que es un regalo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="B141" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C141" s="61" t="inlineStr">
+        <is>
+          <t>Miel, sin hartarse</t>
+        </is>
+      </c>
+      <c r="D141" s="61" t="inlineStr">
+        <is>
+          <t>La Organización Mundial de la Salud recomienda que los azúcares libres sean menos del 10 % de la energía diaria, e idealmente menos del 5 %.</t>
+        </is>
+      </c>
+      <c r="E141" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, Directriz sobre la ingesta de azúcares, 2015</t>
+        </is>
+      </c>
+      <c r="F141" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio usa la miel, algo bueno, para enseñar medida: comer lo que basta.</t>
+        </is>
+      </c>
+      <c r="G141" s="61" t="inlineStr">
+        <is>
+          <t>Comer de más por ansiedad o por costumbre, hasta sentirse mal.</t>
+        </is>
+      </c>
+      <c r="H141" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, antes de servirte de nuevo, esperá unos minutos y preguntate si todavía tenés hambre.</t>
+        </is>
+      </c>
+      <c r="I141" s="61" t="inlineStr">
+        <is>
+          <t>Lo bueno, en exceso, también hace daño. No se trata de prohibir, sino de disfrutar con medida.</t>
+        </is>
+      </c>
+      <c r="J141" s="61" t="inlineStr">
+        <is>
+          <t>El consumo diario de gaseosas y dulces, sobre todo en los chicos.</t>
+        </is>
+      </c>
+      <c r="K141" s="61" t="inlineStr">
+        <is>
+          <t>Cambiá la gaseosa de una comida al día por agua o tereré sin azúcar.</t>
+        </is>
+      </c>
+      <c r="L141" s="61" t="inlineStr">
+        <is>
+          <t>La moderación no es castigo: es sabiduría práctica para cuidar el cuerpo.</t>
+        </is>
+      </c>
+      <c r="M141" s="61" t="inlineStr">
+        <is>
+          <t>Pasar de comer de todo a dietas extremas, y volver a empezar.</t>
+        </is>
+      </c>
+      <c r="N141" s="61" t="inlineStr">
+        <is>
+          <t>En vez de prohibirte algo, decidí cuándo y cuánto lo vas a disfrutar esta semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="B142" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C142" s="61" t="inlineStr">
+        <is>
+          <t>Para la gloria de Dios, también en la mesa</t>
+        </is>
+      </c>
+      <c r="D142" s="61" t="inlineStr">
+        <is>
+          <t>En un estudio con más de 9.000 adultos de Estados Unidos, quienes cocinaban en casa con más frecuencia comían de forma más sana.</t>
+        </is>
+      </c>
+      <c r="E142" s="61" t="inlineStr">
+        <is>
+          <t>Wolfson y Bleich, Public Health Nutrition, 2015</t>
+        </is>
+      </c>
+      <c r="F142" s="61" t="inlineStr">
+        <is>
+          <t>Pablo habla de comer con libertad y con amor al prójimo (10:23-33): todo, hasta comer, puede ser para la gloria de Dios.</t>
+        </is>
+      </c>
+      <c r="G142" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que la fe no tiene nada que ver con lo cotidiano.</t>
+        </is>
+      </c>
+      <c r="H142" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, agradezcan en voz alta antes de cada comida en familia.</t>
+        </is>
+      </c>
+      <c r="I142" s="61" t="inlineStr">
+        <is>
+          <t>Los hábitos pequeños y constantes se sostienen mejor que los cambios drásticos.</t>
+        </is>
+      </c>
+      <c r="J142" s="61" t="inlineStr">
+        <is>
+          <t>Querer cambiar toda la alimentación de golpe y abandonar a la semana.</t>
+        </is>
+      </c>
+      <c r="K142" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un solo hábito nuevo para esta semana: más agua, una fruta por día o una porción de verduras.</t>
+        </is>
+      </c>
+      <c r="L142" s="61" t="inlineStr">
+        <is>
+          <t>Cocinar y comer juntos también es cuidado y comunión.</t>
+        </is>
+      </c>
+      <c r="M142" s="61" t="inlineStr">
+        <is>
+          <t>La comida rápida que reemplaza la mesa familiar.</t>
+        </is>
+      </c>
+      <c r="N142" s="61" t="inlineStr">
+        <is>
+          <t>Cociná en casa una vez más esta semana y compartan la mesa sin pantallas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="B143" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C143" s="61" t="inlineStr">
+        <is>
+          <t>Ni exceso ni descuido</t>
+        </is>
+      </c>
+      <c r="D143" s="61" t="inlineStr">
+        <is>
+          <t>Comer frente a una pantalla, distraídos, se asoció con comer más en esa comida y también en la siguiente.</t>
+        </is>
+      </c>
+      <c r="E143" s="61" t="inlineStr">
+        <is>
+          <t>Robinson y otros, American Journal of Clinical Nutrition, 2013</t>
+        </is>
+      </c>
+      <c r="F143" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios advierte contra los excesos en la mesa, que llevan a la flojera y a la pobreza. El foco está en el descontrol, no en la comida en sí.</t>
+        </is>
+      </c>
+      <c r="G143" s="61" t="inlineStr">
+        <is>
+          <t>Reuniones donde se come de más casi por obligación.</t>
+        </is>
+      </c>
+      <c r="H143" s="61" t="inlineStr">
+        <is>
+          <t>En la próxima reunión, servite un plato y disfrutalo despacio, sin repetir por compromiso.</t>
+        </is>
+      </c>
+      <c r="I143" s="61" t="inlineStr">
+        <is>
+          <t>La moderación cuida el cuerpo y también el bolsillo: comer en exceso sale caro.</t>
+        </is>
+      </c>
+      <c r="J143" s="61" t="inlineStr">
+        <is>
+          <t>Gastar mucho en comida rápida y poco en alimentos frescos.</t>
+        </is>
+      </c>
+      <c r="K143" s="61" t="inlineStr">
+        <is>
+          <t>Hacé la lista de compras de la semana con más frutas, verduras y legumbres, y menos productos ultraprocesados.</t>
+        </is>
+      </c>
+      <c r="L143" s="61" t="inlineStr">
+        <is>
+          <t>El descontrol tiene consecuencias, pero el camino no es la culpa, sino volver a empezar con un hábito pequeño.</t>
+        </is>
+      </c>
+      <c r="M143" s="61" t="inlineStr">
+        <is>
+          <t>Comer frente al celular o la tele, sin darse cuenta de cuánto.</t>
+        </is>
+      </c>
+      <c r="N143" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, hacé al menos una comida por día sin pantallas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="B144" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C144" s="61" t="inlineStr">
+        <is>
+          <t>El pan que sostiene la vida</t>
+        </is>
+      </c>
+      <c r="D144" s="61" t="inlineStr">
+        <is>
+          <t>La mandioca, tan presente en la mesa paraguaya, es una de las principales fuentes de energía de los alimentos en las regiones tropicales del mundo.</t>
+        </is>
+      </c>
+      <c r="E144" s="61" t="inlineStr">
+        <is>
+          <t>Organización de las Naciones Unidas para la Alimentación y la Agricultura (FAO)</t>
+        </is>
+      </c>
+      <c r="F144" s="61" t="inlineStr">
+        <is>
+          <t>El salmo celebra a Dios, que hace crecer lo que comemos: el pan, el aceite, las plantas que cultivamos.</t>
+        </is>
+      </c>
+      <c r="G144" s="61" t="inlineStr">
+        <is>
+          <t>Comer apurados y sin agradecer.</t>
+        </is>
+      </c>
+      <c r="H144" s="61" t="inlineStr">
+        <is>
+          <t>Hoy comé despacio y agradecé por cada cosa que hay en tu plato.</t>
+        </is>
+      </c>
+      <c r="I144" s="61" t="inlineStr">
+        <is>
+          <t>La provisión de Dios es variada, y comer variado es una forma de aprovecharla.</t>
+        </is>
+      </c>
+      <c r="J144" s="61" t="inlineStr">
+        <is>
+          <t>Comer siempre lo mismo por costumbre.</t>
+        </is>
+      </c>
+      <c r="K144" s="61" t="inlineStr">
+        <is>
+          <t>Probá esta semana una verdura o una legumbre que casi nunca comés.</t>
+        </is>
+      </c>
+      <c r="L144" s="61" t="inlineStr">
+        <is>
+          <t>La comida es un regalo, no un enemigo. Hablar de nutrición desde la culpa hace más daño que bien: el enfoque es el cuidado, no la perfección.</t>
+        </is>
+      </c>
+      <c r="M144" s="61" t="inlineStr">
+        <is>
+          <t>Comentarios sobre el cuerpo o el plato de otros que avergüenzan, sobre todo a los adolescentes.</t>
+        </is>
+      </c>
+      <c r="N144" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, en casa, no hagan comentarios sobre el cuerpo o lo que come cada uno; hablen de lo rico y de lo que agradecen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="61" t="n">
+        <v>24</v>
+      </c>
+      <c r="B145" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C145" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: comer con gratitud y medida</t>
+        </is>
+      </c>
+      <c r="D145" s="61" t="inlineStr">
+        <is>
+          <t>Según el relato, Dios dio a Daniel y a sus amigos conocimiento y sabiduría: el texto atribuye el resultado a Dios, no solo a lo que comían.</t>
+        </is>
+      </c>
+      <c r="E145" s="61" t="inlineStr">
+        <is>
+          <t>Daniel 1:9, 17</t>
+        </is>
+      </c>
+      <c r="F145" s="61" t="inlineStr">
+        <is>
+          <t>Comer bien no es comer poco: es elegir alimentos que nutran.</t>
+        </is>
+      </c>
+      <c r="G145" s="61" t="n"/>
+      <c r="H145" s="61" t="inlineStr">
+        <is>
+          <t>Daniel fue fiel a Dios en algo tan cotidiano como la comida. Esta semana, elijan en familia un hábito sencillo para la mesa y agradezcan antes de cada comida.</t>
+        </is>
+      </c>
+      <c r="I145" s="61" t="inlineStr">
+        <is>
+          <t>Un hábito pequeño a la vez se sostiene más que un cambio drástico.</t>
+        </is>
+      </c>
+      <c r="J145" s="61" t="n"/>
+      <c r="K145" s="61" t="n"/>
+      <c r="L145" s="61" t="inlineStr">
+        <is>
+          <t>La comida es un regalo para cuidar, no una fuente de culpa.</t>
+        </is>
+      </c>
+      <c r="M145" s="61" t="n"/>
+      <c r="N145" s="61" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="B146" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C146" s="61" t="inlineStr">
+        <is>
+          <t>Una cadena de fe</t>
+        </is>
+      </c>
+      <c r="D146" s="61" t="inlineStr">
+        <is>
+          <t>En 2 Timoteo 2:2 aparecen cuatro generaciones de creyentes: Pablo, Timoteo, las personas fieles y los otros a quienes ellas van a enseñar.</t>
+        </is>
+      </c>
+      <c r="E146" s="61" t="inlineStr">
+        <is>
+          <t>2 Timoteo 2:2</t>
+        </is>
+      </c>
+      <c r="F146" s="61" t="inlineStr">
+        <is>
+          <t>Pablo, cerca del final de su vida, le pide a Timoteo que encargue lo aprendido a personas fieles. Discipular no es dar una charla: es acompañar en el tiempo.</t>
+        </is>
+      </c>
+      <c r="G146" s="61" t="inlineStr">
+        <is>
+          <t>Confundir discipular con dar un consejo una sola vez.</t>
+        </is>
+      </c>
+      <c r="H146" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en alguien más joven en la fe y proponele encontrarse una vez por semana durante un mes.</t>
+        </is>
+      </c>
+      <c r="I146" s="61" t="inlineStr">
+        <is>
+          <t>La fe pasa de persona a persona: alguien nos acompañó a nosotros.</t>
+        </is>
+      </c>
+      <c r="J146" s="61" t="inlineStr">
+        <is>
+          <t>Olvidar a quienes nos enseñaron y no pasar a otros lo recibido.</t>
+        </is>
+      </c>
+      <c r="K146" s="61" t="inlineStr">
+        <is>
+          <t>Escribile hoy a quien te acompañó en la fe para agradecerle.</t>
+        </is>
+      </c>
+      <c r="L146" s="61" t="inlineStr">
+        <is>
+          <t>El objetivo no es tener seguidores, sino formar personas que también enseñen a otros.</t>
+        </is>
+      </c>
+      <c r="M146" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que concentran todo y no forman a nadie.</t>
+        </is>
+      </c>
+      <c r="N146" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un servicio en la iglesia, enseñale a alguien a hacerlo con vos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="B147" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C147" s="61" t="inlineStr">
+        <is>
+          <t>Como el agua refleja el rostro</t>
+        </is>
+      </c>
+      <c r="D147" s="61" t="inlineStr">
+        <is>
+          <t>Antes de los espejos de vidrio, la gente se miraba en el agua quieta o en láminas de metal pulido.</t>
+        </is>
+      </c>
+      <c r="E147" s="61" t="inlineStr">
+        <is>
+          <t>Historia del espejo</t>
+        </is>
+      </c>
+      <c r="F147" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio dice que, así como el agua refleja el rostro, el corazón refleja a la persona: lo que somos por dentro se ve.</t>
+        </is>
+      </c>
+      <c r="G147" s="61" t="inlineStr">
+        <is>
+          <t>Querer enseñar a otros sin mirarse primero por dentro.</t>
+        </is>
+      </c>
+      <c r="H147" s="61" t="inlineStr">
+        <is>
+          <t>Antes de aconsejar a alguien esta semana, preguntate qué de eso necesitás vos.</t>
+        </is>
+      </c>
+      <c r="I147" s="61" t="inlineStr">
+        <is>
+          <t>Discipular no es mostrar una imagen perfecta: es dejar que el otro vea cómo vivimos la fe, también en las luchas.</t>
+        </is>
+      </c>
+      <c r="J147" s="61" t="inlineStr">
+        <is>
+          <t>Mentores que esconden sus debilidades y generan expectativas irreales.</t>
+        </is>
+      </c>
+      <c r="K147" s="61" t="inlineStr">
+        <is>
+          <t>Contale a quien acompañás una lucha tuya y cómo Dios te ayudó.</t>
+        </is>
+      </c>
+      <c r="L147" s="61" t="inlineStr">
+        <is>
+          <t>La autenticidad forma más que la perfección aparente.</t>
+        </is>
+      </c>
+      <c r="M147" s="61" t="inlineStr">
+        <is>
+          <t>Relaciones de iglesia donde nadie se muestra como es.</t>
+        </is>
+      </c>
+      <c r="N147" s="61" t="inlineStr">
+        <is>
+          <t>Compartí esta semana, con alguien de confianza, algo real de tu camino de fe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="B148" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C148" s="61" t="inlineStr">
+        <is>
+          <t>Imítenme como yo imito a Cristo</t>
+        </is>
+      </c>
+      <c r="D148" s="61" t="inlineStr">
+        <is>
+          <t>En el Nuevo Testamento, la palabra «discípulo» aparece más de 250 veces, casi siempre en los evangelios y en Hechos.</t>
+        </is>
+      </c>
+      <c r="E148" s="61" t="inlineStr">
+        <is>
+          <t>Concordancias del Nuevo Testamento</t>
+        </is>
+      </c>
+      <c r="F148" s="61" t="inlineStr">
+        <is>
+          <t>Pablo no pide que lo imiten a él sin más: pide que lo imiten en la medida en que él imita a Cristo. El modelo es Jesús.</t>
+        </is>
+      </c>
+      <c r="G148" s="61" t="inlineStr">
+        <is>
+          <t>Seguir a líderes por su carisma, sin mirar si siguen a Cristo.</t>
+        </is>
+      </c>
+      <c r="H148" s="61" t="inlineStr">
+        <is>
+          <t>Revisá a quién seguís: ¿te acerca más a Jesús?</t>
+        </is>
+      </c>
+      <c r="I148" s="61" t="inlineStr">
+        <is>
+          <t>Las palabras enseñan, pero el ejemplo confirma.</t>
+        </is>
+      </c>
+      <c r="J148" s="61" t="inlineStr">
+        <is>
+          <t>Padres y líderes que dicen una cosa y hacen otra.</t>
+        </is>
+      </c>
+      <c r="K148" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una enseñanza que das a otros y revisá si tu vida la respalda.</t>
+        </is>
+      </c>
+      <c r="L148" s="61" t="inlineStr">
+        <is>
+          <t>Discipular exige integridad: vivir lo que enseñamos, y pedir perdón cuando fallamos.</t>
+        </is>
+      </c>
+      <c r="M148" s="61" t="inlineStr">
+        <is>
+          <t>La incoherencia que aleja a los jóvenes de la fe.</t>
+        </is>
+      </c>
+      <c r="N148" s="61" t="inlineStr">
+        <is>
+          <t>Si fallaste en algo que enseñás, reconocelo delante de quien acompañás.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="B149" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C149" s="61" t="inlineStr">
+        <is>
+          <t>Permanecer en la Palabra</t>
+        </is>
+      </c>
+      <c r="D149" s="61" t="inlineStr">
+        <is>
+          <t>La frase «la verdad los hará libres» está grabada en el vestíbulo de la sede de la CIA, en Estados Unidos, sin la primera parte del versículo.</t>
+        </is>
+      </c>
+      <c r="E149" s="61" t="inlineStr">
+        <is>
+          <t>Agencia Central de Inteligencia (CIA), historia del edificio</t>
+        </is>
+      </c>
+      <c r="F149" s="61" t="inlineStr">
+        <is>
+          <t>Jesús les habla a quienes habían creído en Él: ser discípulo es permanecer en su palabra, no solo empezar.</t>
+        </is>
+      </c>
+      <c r="G149" s="61" t="inlineStr">
+        <is>
+          <t>Citar «la verdad los hará libres» sin la condición que la precede: permanecer en su palabra.</t>
+        </is>
+      </c>
+      <c r="H149" s="61" t="inlineStr">
+        <is>
+          <t>Leé esta semana Juan 8:31-36 completo.</t>
+        </is>
+      </c>
+      <c r="I149" s="61" t="inlineStr">
+        <is>
+          <t>La verdad de la que habla Jesús no es solo una idea: es Él mismo (Juan 14:6). Conocerlo transforma.</t>
+        </is>
+      </c>
+      <c r="J149" s="61" t="inlineStr">
+        <is>
+          <t>Una fe que sabe datos de Jesús, pero no lo conoce.</t>
+        </is>
+      </c>
+      <c r="K149" s="61" t="inlineStr">
+        <is>
+          <t>Orá esta semana pidiendo conocer más a Jesús, no solo saber más sobre Él.</t>
+        </is>
+      </c>
+      <c r="L149" s="61" t="inlineStr">
+        <is>
+          <t>Jesús libera del pecado (8:34-36). Un discípulo libre enseña más con su vida que con mil palabras.</t>
+        </is>
+      </c>
+      <c r="M149" s="61" t="inlineStr">
+        <is>
+          <t>Discipular con reglas que encierran en vez de liberar.</t>
+        </is>
+      </c>
+      <c r="N149" s="61" t="inlineStr">
+        <is>
+          <t>Al acompañar a alguien, hablale más de la gracia de Jesús que de reglas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="B150" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C150" s="61" t="inlineStr">
+        <is>
+          <t>Lo que vieron y oyeron</t>
+        </is>
+      </c>
+      <c r="D150" s="61" t="inlineStr">
+        <is>
+          <t>Filipos fue la primera ciudad de Europa donde Pablo fundó una iglesia, en la casa de una mujer llamada Lidia.</t>
+        </is>
+      </c>
+      <c r="E150" s="61" t="inlineStr">
+        <is>
+          <t>Hechos 16:11-15</t>
+        </is>
+      </c>
+      <c r="F150" s="61" t="inlineStr">
+        <is>
+          <t>Pablo invita a practicar lo que aprendieron, recibieron, vieron y oyeron de él. El discipulado se aprende mirando y haciendo.</t>
+        </is>
+      </c>
+      <c r="G150" s="61" t="inlineStr">
+        <is>
+          <t>Saber mucho y practicar poco.</t>
+        </is>
+      </c>
+      <c r="H150" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una enseñanza que recibiste y ponela en práctica esta semana.</t>
+        </is>
+      </c>
+      <c r="I150" s="61" t="inlineStr">
+        <is>
+          <t>La promesa es la presencia del Dios de paz. Invertir en otros deja un legado que sigue dando fruto después de nosotros.</t>
+        </is>
+      </c>
+      <c r="J150" s="61" t="inlineStr">
+        <is>
+          <t>Vivir solo para lo propio, sin pensar en lo que dejamos.</t>
+        </is>
+      </c>
+      <c r="K150" s="61" t="inlineStr">
+        <is>
+          <t>Preguntate: ¿en quién estoy invirtiendo hoy, aunque sea de manera informal?</t>
+        </is>
+      </c>
+      <c r="L150" s="61" t="inlineStr">
+        <is>
+          <t>Lo que sembramos en otro sigue creciendo cuando ya no estamos.</t>
+        </is>
+      </c>
+      <c r="M150" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que discipular es una tarea solo de pastores.</t>
+        </is>
+      </c>
+      <c r="N150" s="61" t="inlineStr">
+        <is>
+          <t>Invitá a alguien a acompañarte en un servicio esta semana, para que aprenda haciendo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="61" t="n">
+        <v>25</v>
+      </c>
+      <c r="B151" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C151" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: invertir en otros</t>
+        </is>
+      </c>
+      <c r="D151" s="61" t="inlineStr">
+        <is>
+          <t>Daniel 12 es uno de los pasajes del Antiguo Testamento que hablan claramente de la resurrección.</t>
+        </is>
+      </c>
+      <c r="E151" s="61" t="inlineStr">
+        <is>
+          <t>Daniel 12:2</t>
+        </is>
+      </c>
+      <c r="F151" s="61" t="inlineStr">
+        <is>
+          <t>Discipular es acompañar en el tiempo, no dar un consejo una sola vez.</t>
+        </is>
+      </c>
+      <c r="G151" s="61" t="n"/>
+      <c r="H151" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, elegí a una persona para acompañar en la fe durante el próximo mes, y anotá cuándo la vas a llamar.</t>
+        </is>
+      </c>
+      <c r="I151" s="61" t="inlineStr">
+        <is>
+          <t>El ejemplo confirma lo que las palabras enseñan.</t>
+        </is>
+      </c>
+      <c r="J151" s="61" t="n"/>
+      <c r="K151" s="61" t="n"/>
+      <c r="L151" s="61" t="inlineStr">
+        <is>
+          <t>Invertir en otro deja un legado que sigue dando fruto.</t>
+        </is>
+      </c>
+      <c r="M151" s="61" t="n"/>
+      <c r="N151" s="61" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="B152" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C152" s="61" t="inlineStr">
+        <is>
+          <t>Todo con amor</t>
+        </is>
+      </c>
+      <c r="D152" s="61" t="inlineStr">
+        <is>
+          <t>Un análisis de 128 experimentos encontró que los premios materiales, usados para controlar, pueden bajar el interés propio por una tarea.</t>
+        </is>
+      </c>
+      <c r="E152" s="61" t="inlineStr">
+        <is>
+          <t>Deci, Koestner y Ryan, Psychological Bulletin, 1999</t>
+        </is>
+      </c>
+      <c r="F152" s="61" t="inlineStr">
+        <is>
+          <t>Pablo cierra su carta con exhortaciones breves: firmes en la fe, fuertes, y todo con amor. La firmeza sin amor se vuelve dureza.</t>
+        </is>
+      </c>
+      <c r="G152" s="61" t="inlineStr">
+        <is>
+          <t>Líderes firmes que motivan con miedo.</t>
+        </is>
+      </c>
+      <c r="H152" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, cuando le pidas algo a tu equipo o a tu familia, explicá para qué sirve, no solo qué hay que hacer.</t>
+        </is>
+      </c>
+      <c r="I152" s="61" t="inlineStr">
+        <is>
+          <t>Motivar busca el bien del otro y de la tarea; manipular usa al otro como medio. La diferencia está en la intención y en el respeto a la libertad.</t>
+        </is>
+      </c>
+      <c r="J152" s="61" t="inlineStr">
+        <is>
+          <t>Presiones del tipo «si no lo hacés, vas a ver», en el trabajo o en la iglesia.</t>
+        </is>
+      </c>
+      <c r="K152" s="61" t="inlineStr">
+        <is>
+          <t>Una señal simple: si la persona no puede decir que no sin consecuencias, no la motivaste, la presionaste. Revisá un pedido tuyo con esa pregunta.</t>
+        </is>
+      </c>
+      <c r="L152" s="61" t="inlineStr">
+        <is>
+          <t>«Háganlo todo con amor»: el amor no manipula ni usa la culpa.</t>
+        </is>
+      </c>
+      <c r="M152" s="61" t="inlineStr">
+        <is>
+          <t>Usar la culpa o lo espiritual para que otros hagan lo que uno quiere.</t>
+        </is>
+      </c>
+      <c r="N152" s="61" t="inlineStr">
+        <is>
+          <t>Si usaste la culpa para motivar a alguien, pedile disculpas y volvé a plantear el pedido con claridad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="B153" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C153" s="61" t="inlineStr">
+        <is>
+          <t>Paciencia que une</t>
+        </is>
+      </c>
+      <c r="D153" s="61" t="inlineStr">
+        <is>
+          <t>Cuando Google estudió sus mejores equipos, encontró que lo que más los distinguía era la «seguridad psicológica»: poder opinar sin miedo.</t>
+        </is>
+      </c>
+      <c r="E153" s="61" t="inlineStr">
+        <is>
+          <t>Google, Proyecto Aristóteles, 2015</t>
+        </is>
+      </c>
+      <c r="F153" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide «buscar» mantener la unidad: no sale sola, se cuida activamente.</t>
+        </is>
+      </c>
+      <c r="G153" s="61" t="inlineStr">
+        <is>
+          <t>Equipos divididos por chismes y bandos.</t>
+        </is>
+      </c>
+      <c r="H153" s="61" t="inlineStr">
+        <is>
+          <t>Si escuchás un chisme sobre alguien del equipo, cortalo y hablá con la persona.</t>
+        </is>
+      </c>
+      <c r="I153" s="61" t="inlineStr">
+        <is>
+          <t>Humildad, mansedumbre y paciencia: un líder que motiva sin manipular tiene paciencia con los procesos de cada uno.</t>
+        </is>
+      </c>
+      <c r="J153" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que exigen resultados inmediatos y se impacientan.</t>
+        </is>
+      </c>
+      <c r="K153" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, tené paciencia con alguien del equipo que está aprendiendo, y decile qué está haciendo bien.</t>
+        </is>
+      </c>
+      <c r="L153" s="61" t="inlineStr">
+        <is>
+          <t>La unidad no es que todos piensen igual: es la que da el Espíritu, en el vínculo de la paz.</t>
+        </is>
+      </c>
+      <c r="M153" s="61" t="inlineStr">
+        <is>
+          <t>Confundir la unidad con que nadie opine distinto.</t>
+        </is>
+      </c>
+      <c r="N153" s="61" t="inlineStr">
+        <is>
+          <t>En tu próxima reunión, pedí la opinión de quien suele callar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="B154" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C154" s="61" t="inlineStr">
+        <is>
+          <t>Muchos consejeros</t>
+        </is>
+      </c>
+      <c r="D154" s="61" t="inlineStr">
+        <is>
+          <t>La confianza se pierde rápido y se recupera lento: un hecho negativo suele pesar más que varios positivos a la hora de confiar.</t>
+        </is>
+      </c>
+      <c r="E154" s="61" t="inlineStr">
+        <is>
+          <t>Paul Slovic, «Perceived risk, trust, and democracy», Risk Analysis, 1993</t>
+        </is>
+      </c>
+      <c r="F154" s="61" t="inlineStr">
+        <is>
+          <t>Cuando no hay buena guía, se tropieza; con muchos consejeros, hay seguridad. Un líder que consulta construye confianza.</t>
+        </is>
+      </c>
+      <c r="G154" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que deciden solos y después piden que todos acompañen.</t>
+        </is>
+      </c>
+      <c r="H154" s="61" t="inlineStr">
+        <is>
+          <t>Antes de una decisión que afecta al equipo, consultá a dos o tres personas.</t>
+        </is>
+      </c>
+      <c r="I154" s="61" t="inlineStr">
+        <is>
+          <t>La confianza se construye cumpliendo lo prometido y siendo transparente con los errores.</t>
+        </is>
+      </c>
+      <c r="J154" s="61" t="inlineStr">
+        <is>
+          <t>Prometer y no cumplir, aunque sea en cosas pequeñas.</t>
+        </is>
+      </c>
+      <c r="K154" s="61" t="inlineStr">
+        <is>
+          <t>Revisá qué le prometiste a tu equipo y cumplí esta semana lo que quedó pendiente.</t>
+        </is>
+      </c>
+      <c r="L154" s="61" t="inlineStr">
+        <is>
+          <t>La confianza se rompe rápido y se reconstruye lento: vale la pena cuidarla en lo pequeño.</t>
+        </is>
+      </c>
+      <c r="M154" s="61" t="inlineStr">
+        <is>
+          <t>Ocultar información al equipo «para no preocuparlo».</t>
+        </is>
+      </c>
+      <c r="N154" s="61" t="inlineStr">
+        <is>
+          <t>Compartí con tu equipo, con honestidad, cómo van las cosas, también lo que no va bien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="B155" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C155" s="61" t="inlineStr">
+        <is>
+          <t>Cargar juntos</t>
+        </is>
+      </c>
+      <c r="D155" s="61" t="inlineStr">
+        <is>
+          <t>En este capítulo Pablo usa dos palabras griegas distintas: una para la carga pesada que agobia (6:2) y otra para la carga propia de cada día (6:5).</t>
+        </is>
+      </c>
+      <c r="E155" s="61" t="inlineStr">
+        <is>
+          <t>Gálatas 6:2-5; léxico griego de Strong (G922 y G5413)</t>
+        </is>
+      </c>
+      <c r="F155" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide llevar las cargas de otros, esas que agobian. Un equipo de confianza es donde se puede decir «no doy más».</t>
+        </is>
+      </c>
+      <c r="G155" s="61" t="inlineStr">
+        <is>
+          <t>Personas del equipo que se hunden en silencio.</t>
+        </is>
+      </c>
+      <c r="H155" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale en privado a cada persona de tu equipo cómo está de verdad.</t>
+        </is>
+      </c>
+      <c r="I155" s="61" t="inlineStr">
+        <is>
+          <t>Ayudar no es hacer todo por el otro: en el versículo 5, cada uno lleva su propia carga. Se acompaña sin anular.</t>
+        </is>
+      </c>
+      <c r="J155" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que cargan con todo y no dejan crecer a nadie.</t>
+        </is>
+      </c>
+      <c r="K155" s="61" t="inlineStr">
+        <is>
+          <t>Ofrecé ayuda concreta a alguien sobrecargado, sin quitarle su responsabilidad.</t>
+        </is>
+      </c>
+      <c r="L155" s="61" t="inlineStr">
+        <is>
+          <t>Llevar las cargas cumple la ley de Cristo: amar como Él amó.</t>
+        </is>
+      </c>
+      <c r="M155" s="61" t="inlineStr">
+        <is>
+          <t>Equipos donde cada uno cuida solo lo suyo.</t>
+        </is>
+      </c>
+      <c r="N155" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, cubrí a un compañero en algo que le está costando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="B156" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C156" s="61" t="inlineStr">
+        <is>
+          <t>Estimularnos al amor</t>
+        </is>
+      </c>
+      <c r="D156" s="61" t="inlineStr">
+        <is>
+          <t>En un experimento, los comentarios críticos acompañados de la frase «te digo esto porque tengo altas expectativas y sé que podés alcanzarlas» fueron mucho mejor recibidos.</t>
+        </is>
+      </c>
+      <c r="E156" s="61" t="inlineStr">
+        <is>
+          <t>Yeager y otros, Journal of Experimental Psychology: General, 2014</t>
+        </is>
+      </c>
+      <c r="F156" s="61" t="inlineStr">
+        <is>
+          <t>La carta pide tenernos en cuenta para estimularnos al amor y a las buenas obras. Corregir también es una forma de estimular.</t>
+        </is>
+      </c>
+      <c r="G156" s="61" t="inlineStr">
+        <is>
+          <t>Corregir solo para descargar enojo.</t>
+        </is>
+      </c>
+      <c r="H156" s="61" t="inlineStr">
+        <is>
+          <t>Antes de corregir, preguntate: ¿esto ayuda a la persona a crecer?</t>
+        </is>
+      </c>
+      <c r="I156" s="61" t="inlineStr">
+        <is>
+          <t>Corregir sin amor hiere; amar sin corregir permite que el error se repita.</t>
+        </is>
+      </c>
+      <c r="J156" s="61" t="inlineStr">
+        <is>
+          <t>Evitar corregir para no generar conflicto, y que el problema crezca.</t>
+        </is>
+      </c>
+      <c r="K156" s="61" t="inlineStr">
+        <is>
+          <t>Usá esta estructura: reconocé lo bueno, señalá un punto concreto a mejorar y cerrá con confianza en la persona.</t>
+        </is>
+      </c>
+      <c r="L156" s="61" t="inlineStr">
+        <is>
+          <t>Decir la verdad con el mismo cuidado con que se le diría a alguien muy querido: eso edifica.</t>
+        </is>
+      </c>
+      <c r="M156" s="61" t="inlineStr">
+        <is>
+          <t>Correcciones en público que humillan.</t>
+        </is>
+      </c>
+      <c r="N156" s="61" t="inlineStr">
+        <is>
+          <t>Corregí siempre en privado y reconocé en público.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="61" t="n">
+        <v>26</v>
+      </c>
+      <c r="B157" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C157" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: liderar un equipo con humildad</t>
+        </is>
+      </c>
+      <c r="D157" s="61" t="inlineStr">
+        <is>
+          <t>Inmediatamente después, Pablo pone como ejemplo a Jesús, que se humilló hasta la muerte en la cruz.</t>
+        </is>
+      </c>
+      <c r="E157" s="61" t="inlineStr">
+        <is>
+          <t>Filipenses 2:5-8</t>
+        </is>
+      </c>
+      <c r="F157" s="61" t="inlineStr">
+        <is>
+          <t>Motivar busca el bien del otro; manipular lo usa. La diferencia está en la intención y en la libertad.</t>
+        </is>
+      </c>
+      <c r="G157" s="61" t="n"/>
+      <c r="H157" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pone como modelo a Jesús, que se hizo siervo. Esta semana, preguntale a tu equipo o a tu familia: ¿en qué te puedo servir mejor?</t>
+        </is>
+      </c>
+      <c r="I157" s="61" t="inlineStr">
+        <is>
+          <t>La confianza se construye cumpliendo lo prometido y siendo transparente.</t>
+        </is>
+      </c>
+      <c r="J157" s="61" t="n"/>
+      <c r="K157" s="61" t="n"/>
+      <c r="L157" s="61" t="inlineStr">
+        <is>
+          <t>Corregir con amor y firmeza: reconocer lo bueno, señalar lo concreto y confiar en la persona.</t>
+        </is>
+      </c>
+      <c r="M157" s="61" t="n"/>
+      <c r="N157" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de junio verificados
30 datos contrastados: 19 confirmados, 11 ajustados (GEM 2024 47 %,
Job 42:7 en RVC, mandioca según la FAO, inscripción de la CIA, precisiones).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -28071,12 +28071,12 @@
       </c>
       <c r="D133" s="61" t="inlineStr">
         <is>
-          <t>En una empresa tecnológica de Estados Unidos, los empleados que recibieron mentoría fueron ascendidos con mucha más frecuencia que los que no la tuvieron.</t>
+          <t>En un estudio de Sun Microsystems, los empleados que recibieron mentoría fueron ascendidos cinco veces más que los que no la tuvieron, y los mentores, seis veces más.</t>
         </is>
       </c>
       <c r="E133" s="61" t="inlineStr">
         <is>
-          <t>Gartner, estudio para Sun Microsystems, 2006</t>
+          <t>Gartner, análisis del programa de mentoría de Sun Microsystems, 2006</t>
         </is>
       </c>
       <c r="F133" s="61" t="inlineStr">
@@ -28121,12 +28121,12 @@
       </c>
       <c r="D134" s="61" t="inlineStr">
         <is>
-          <t>En muchos países, cerca de la mitad de los adultos que ven una buena oportunidad para emprender dice que el miedo a fracasar lo frenaría.</t>
+          <t>En 2024, casi la mitad (47 %) de los adultos que veían buenas oportunidades para emprender dijo que el miedo a fracasar le impediría hacerlo.</t>
         </is>
       </c>
       <c r="E134" s="61" t="inlineStr">
         <is>
-          <t>Global Entrepreneurship Monitor (GEM), informe mundial</t>
+          <t>Global Entrepreneurship Monitor (GEM), Informe mundial 2024/2025</t>
         </is>
       </c>
       <c r="F134" s="61" t="inlineStr">
@@ -28191,12 +28191,12 @@
       </c>
       <c r="D135" s="61" t="inlineStr">
         <is>
-          <t>Al final del libro de Job, Dios dice a los amigos de Job que no hablaron de Él con verdad.</t>
+          <t>Al final del libro de Job, Dios les dice a los amigos de Job que no hablaron de Él con rectitud, como sí lo hizo su siervo Job.</t>
         </is>
       </c>
       <c r="E135" s="61" t="inlineStr">
         <is>
-          <t>Job 42:7</t>
+          <t>Job 42:7 (RVC)</t>
         </is>
       </c>
       <c r="F135" s="61" t="inlineStr">
@@ -28471,12 +28471,12 @@
       </c>
       <c r="D139" s="61" t="inlineStr">
         <is>
-          <t>Jesús dijo estas palabras al día siguiente de multiplicar los panes para unas cinco mil personas.</t>
+          <t>Jesús dijo estas palabras al día siguiente de multiplicar los panes para unos cinco mil hombres, sin contar a las mujeres y a los niños.</t>
         </is>
       </c>
       <c r="E139" s="61" t="inlineStr">
         <is>
-          <t>Juan 6:10-27</t>
+          <t>Juan 6:10, 22-27; Mateo 14:21</t>
         </is>
       </c>
       <c r="F139" s="61" t="inlineStr">
@@ -28731,7 +28731,7 @@
       </c>
       <c r="D143" s="61" t="inlineStr">
         <is>
-          <t>Comer frente a una pantalla, distraídos, se asoció con comer más en esa comida y también en la siguiente.</t>
+          <t>Una revisión de 24 estudios encontró que comer distraídos, por ejemplo frente a una pantalla, se asoció con comer más en esa comida y aún más en la siguiente.</t>
         </is>
       </c>
       <c r="E143" s="61" t="inlineStr">
@@ -28801,7 +28801,7 @@
       </c>
       <c r="D144" s="61" t="inlineStr">
         <is>
-          <t>La mandioca, tan presente en la mesa paraguaya, es una de las principales fuentes de energía de los alimentos en las regiones tropicales del mundo.</t>
+          <t>La mandioca, tan presente en la mesa paraguaya, es la tercera fuente más importante de calorías en las regiones tropicales del mundo, después del arroz y el maíz.</t>
         </is>
       </c>
       <c r="E144" s="61" t="inlineStr">
@@ -28991,12 +28991,12 @@
       </c>
       <c r="D147" s="61" t="inlineStr">
         <is>
-          <t>Antes de los espejos de vidrio, la gente se miraba en el agua quieta o en láminas de metal pulido.</t>
+          <t>Antes de los espejos de vidrio, la gente se miraba en el agua quieta, en piedra volcánica pulida o en láminas de metal pulido, como cobre o bronce.</t>
         </is>
       </c>
       <c r="E147" s="61" t="inlineStr">
         <is>
-          <t>Historia del espejo</t>
+          <t>Encyclopaedia Britannica, «Mirror»</t>
         </is>
       </c>
       <c r="F147" s="61" t="inlineStr">
@@ -29061,12 +29061,12 @@
       </c>
       <c r="D148" s="61" t="inlineStr">
         <is>
-          <t>En el Nuevo Testamento, la palabra «discípulo» aparece más de 250 veces, casi siempre en los evangelios y en Hechos.</t>
+          <t>En el Nuevo Testamento, la palabra «discípulo» aparece más de 250 veces, y solo en los evangelios y en Hechos.</t>
         </is>
       </c>
       <c r="E148" s="61" t="inlineStr">
         <is>
-          <t>Concordancias del Nuevo Testamento</t>
+          <t>Mounce, Greek Dictionary (Strong G3101, mathetés)</t>
         </is>
       </c>
       <c r="F148" s="61" t="inlineStr">
@@ -29131,12 +29131,12 @@
       </c>
       <c r="D149" s="61" t="inlineStr">
         <is>
-          <t>La frase «la verdad los hará libres» está grabada en el vestíbulo de la sede de la CIA, en Estados Unidos, sin la primera parte del versículo.</t>
+          <t>En el vestíbulo de la sede de la CIA, en Estados Unidos, está grabado «conocerán la verdad, y la verdad los hará libres», pero sin la condición del versículo anterior: «si permanecen en mi palabra».</t>
         </is>
       </c>
       <c r="E149" s="61" t="inlineStr">
         <is>
-          <t>Agencia Central de Inteligencia (CIA), historia del edificio</t>
+          <t>Agencia Central de Inteligencia (CIA), «Bible Quote Carving»</t>
         </is>
       </c>
       <c r="F149" s="61" t="inlineStr">
@@ -29201,12 +29201,12 @@
       </c>
       <c r="D150" s="61" t="inlineStr">
         <is>
-          <t>Filipos fue la primera ciudad de Europa donde Pablo fundó una iglesia, en la casa de una mujer llamada Lidia.</t>
+          <t>Filipos es considerada la primera ciudad de Europa donde Pablo fundó una iglesia: allí creyó Lidia, y los creyentes se reunían en su casa.</t>
         </is>
       </c>
       <c r="E150" s="61" t="inlineStr">
         <is>
-          <t>Hechos 16:11-15</t>
+          <t>Hechos 16:11-15, 40</t>
         </is>
       </c>
       <c r="F150" s="61" t="inlineStr">
@@ -29601,7 +29601,7 @@
       </c>
       <c r="D156" s="61" t="inlineStr">
         <is>
-          <t>En un experimento, los comentarios críticos acompañados de la frase «te digo esto porque tengo altas expectativas y sé que podés alcanzarlas» fueron mucho mejor recibidos.</t>
+          <t>En un experimento con estudiantes, cuando las correcciones venían con la nota «te hago estos comentarios porque tengo altas expectativas y sé que podés alcanzarlas», muchos más decidieron corregir y mejorar su trabajo.</t>
         </is>
       </c>
       <c r="E156" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: guiones de julio con revisión teológica
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -6626,7 +6626,7 @@
       <c r="AA29" s="40" t="inlineStr">
         <is>
           <t>• La fidelidad en lo poco lleva a más responsabilidad
-• El buen manejo trae recompensa
+• La recompensa: más responsabilidad y el gozo del Señor
 • Dios celebra la fidelidad, no solo el resultado</t>
         </is>
       </c>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="AI29" s="40" t="inlineStr">
         <is>
-          <t>• No poner nuestra confianza en lo 2. material.
+          <t>• No poner nuestra confianza en lo material.
 • Buscar tesoros eternos en el cielo.
 Cuidar dónde está nuestro corazón.</t>
         </is>
@@ -6692,7 +6692,7 @@
         <is>
           <t>• Crecer en madurez espiritual.
 • Distinguir el bien del mal.
-3 Aprender a tomar buenas decisiones.</t>
+• Aprender a tomar buenas decisiones.</t>
         </is>
       </c>
     </row>
@@ -6881,9 +6881,9 @@
       </c>
       <c r="AI30" s="43" t="inlineStr">
         <is>
-          <t>• Confía en Dios: Pon tus planes en sus manos.
-• Persevera: Dios puede ayudarte a llevarlos a buen término.
-3 Camina en su luz: Busca su dirección en cada paso.</t>
+          <t>• Quien habla es Elifaz: Un amigo de Job cuya idea de Dios fue corregida (42:7).
+• Confía en Dios: Pon tus planes en sus manos.
+• Camina en su luz: Busca su dirección en cada paso.</t>
         </is>
       </c>
       <c r="AJ30" s="43" t="inlineStr">
@@ -6894,7 +6894,7 @@
       <c r="AK30" s="43" t="inlineStr">
         <is>
           <t>• Sujetar los planes a la voluntad de Dios
-• El futuro no esta garantizado por uno mismo
+• El futuro no está garantizado por uno mismo
 • La humildad reconoce los límites del control propio</t>
         </is>
       </c>
@@ -7048,7 +7048,7 @@
       <c r="AC31" s="47" t="inlineStr">
         <is>
           <t>• El peso y la balanza justos son de Dios
-• Toda medida comercial le pertenece a El
+• Toda medida comercial le pertenece a Él
 • La justicia en el negocio refleja el carácter de Dios</t>
         </is>
       </c>
@@ -7099,7 +7099,7 @@
         <is>
           <t>• La mujer virtuosa produce y vende con esfuerzo
 • El trabajo genera ingresos legítimos
-• La prAI31:AK31oduccion propia tiene valor</t>
+• La producción propia tiene valor</t>
         </is>
       </c>
     </row>
@@ -19214,7 +19214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N157"/>
+  <dimension ref="A1:N181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -29704,6 +29704,1606 @@
       </c>
       <c r="M157" s="61" t="n"/>
       <c r="N157" s="61" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="61" t="n">
+        <v>27</v>
+      </c>
+      <c r="B158" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C158" s="61" t="inlineStr">
+        <is>
+          <t>La paz de tu ciudad</t>
+        </is>
+      </c>
+      <c r="D158" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías envió esta carta a los judíos deportados a Babilonia; antes de pedirles que oraran por la ciudad, les dijo que construyeran casas, plantaran huertos y formaran familias allí.</t>
+        </is>
+      </c>
+      <c r="E158" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías 29:1-7</t>
+        </is>
+      </c>
+      <c r="F158" s="61" t="inlineStr">
+        <is>
+          <t>Dios les pidió a familias desterradas que buscaran el bien de una ciudad que no era la suya. La fe no nos aísla: nos pone a servir donde estamos.</t>
+        </is>
+      </c>
+      <c r="G158" s="61" t="inlineStr">
+        <is>
+          <t>Vivir encerrados en casa, como si lo que pasa en el barrio no nos tocara.</t>
+        </is>
+      </c>
+      <c r="H158" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, hacé algo concreto por tu cuadra: saludá al vecino nuevo, limpiá la vereda o ayudá a alguien mayor.</t>
+        </is>
+      </c>
+      <c r="I158" s="61" t="inlineStr">
+        <is>
+          <t>«Si ella tiene paz, también tendrán paz ustedes.» Lo que pasa en la casa sale a la calle, y lo que pasa en la calle entra en la casa.</t>
+        </is>
+      </c>
+      <c r="J158" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que mi familia puede estar bien aunque a mi comunidad le vaya mal.</t>
+        </is>
+      </c>
+      <c r="K158" s="61" t="inlineStr">
+        <is>
+          <t>Conversá en familia: ¿qué necesita nuestro barrio y qué podemos aportar nosotros?</t>
+        </is>
+      </c>
+      <c r="L158" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías también les pidió orar por esa ciudad. Orar por el lugar donde vivimos cambia la forma en que lo miramos.</t>
+        </is>
+      </c>
+      <c r="M158" s="61" t="inlineStr">
+        <is>
+          <t>Quejarse del barrio sin orar ni hacer nada por él.</t>
+        </is>
+      </c>
+      <c r="N158" s="61" t="inlineStr">
+        <is>
+          <t>Incluí a tu ciudad en la oración familiar de esta semana, por nombre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="61" t="n">
+        <v>27</v>
+      </c>
+      <c r="B159" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C159" s="61" t="inlineStr">
+        <is>
+          <t>Ciudadanos responsables</t>
+        </is>
+      </c>
+      <c r="D159" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribió la carta a los Romanos hacia el año 57, cuando gobernaba el emperador Nerón.</t>
+        </is>
+      </c>
+      <c r="E159" s="61" t="inlineStr">
+        <is>
+          <t>Introducciones bíblicas a Romanos; Hechos 20:2-3</t>
+        </is>
+      </c>
+      <c r="F159" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide respetar a las autoridades, que en ese tiempo eran romanas y no creyentes. Pagar lo que corresponde, cumplir las normas y tratar con respeto a quien ocupa un cargo también es parte de la fe.</t>
+        </is>
+      </c>
+      <c r="G159" s="61" t="inlineStr">
+        <is>
+          <t>Saltearse normas pequeñas porque «todos lo hacen».</t>
+        </is>
+      </c>
+      <c r="H159" s="61" t="inlineStr">
+        <is>
+          <t>Revisá si hay alguna norma que venís salteando, de tránsito, de impuestos o del barrio, y ponete al día.</t>
+        </is>
+      </c>
+      <c r="I159" s="61" t="inlineStr">
+        <is>
+          <t>Dios quiere orden y no caos. Pero ninguna autoridad humana es absoluta: cuando les ordenaron dejar de hablar de Jesús, los apóstoles respondieron que hay que obedecer a Dios antes que a los hombres (Hechos 5:29).</t>
+        </is>
+      </c>
+      <c r="J159" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que respetar a la autoridad significa aprobar todo lo que hace o callar ante una injusticia.</t>
+        </is>
+      </c>
+      <c r="K159" s="61" t="inlineStr">
+        <is>
+          <t>Cuando no estés de acuerdo con una autoridad, expresalo por los caminos correctos y con respeto.</t>
+        </is>
+      </c>
+      <c r="L159" s="61" t="inlineStr">
+        <is>
+          <t>En casa se aprende a respetar normas. Un hijo que ve a sus padres cumplir la ley aunque nadie los controle aprende más que con cualquier sermón.</t>
+        </is>
+      </c>
+      <c r="M159" s="61" t="inlineStr">
+        <is>
+          <t>Pedirles respeto a los hijos y darles el ejemplo contrario.</t>
+        </is>
+      </c>
+      <c r="N159" s="61" t="inlineStr">
+        <is>
+          <t>Que tus hijos te vean cumplir una norma esta semana, y explicales por qué lo hacés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="61" t="n">
+        <v>27</v>
+      </c>
+      <c r="B160" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C160" s="61" t="inlineStr">
+        <is>
+          <t>Lo que Dios espera</t>
+        </is>
+      </c>
+      <c r="D160" s="61" t="inlineStr">
+        <is>
+          <t>Miqueas profetizó en el siglo VIII antes de Cristo, en tiempos de los reyes Jotam, Acaz y Ezequías, igual que Isaías.</t>
+        </is>
+      </c>
+      <c r="E160" s="61" t="inlineStr">
+        <is>
+          <t>Miqueas 1:1; Isaías 1:1</t>
+        </is>
+      </c>
+      <c r="F160" s="61" t="inlineStr">
+        <is>
+          <t>Miqueas resume lo que Dios espera en tres frases. La primera es hacer justicia: tratar a cada uno como corresponde, empezando por los de casa.</t>
+        </is>
+      </c>
+      <c r="G160" s="61" t="inlineStr">
+        <is>
+          <t>Exigir justicia afuera y ser injusto con la propia familia.</t>
+        </is>
+      </c>
+      <c r="H160" s="61" t="inlineStr">
+        <is>
+          <t>Revisá si en tu casa las tareas y los permisos se reparten con justicia.</t>
+        </is>
+      </c>
+      <c r="I160" s="61" t="inlineStr">
+        <is>
+          <t>La familia forma a la persona y la sociedad le da espacio para desplegar esa formación. Lo que aprendemos en casa sobre el perdón lo llevamos al trabajo, a la escuela y a la calle.</t>
+        </is>
+      </c>
+      <c r="J160" s="61" t="inlineStr">
+        <is>
+          <t>Hogares donde nunca se pide perdón, y adultos que después no saben pedirlo.</t>
+        </is>
+      </c>
+      <c r="K160" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, pedí perdón o perdoná a alguien de tu casa por algo concreto.</t>
+        </is>
+      </c>
+      <c r="L160" s="61" t="inlineStr">
+        <is>
+          <t>Humillarse ante Dios es reconocer que no somos el centro. Una familia humilde sabe recibir ayuda de la comunidad, y también darla.</t>
+        </is>
+      </c>
+      <c r="M160" s="61" t="inlineStr">
+        <is>
+          <t>El orgullo de no pedir ayuda nunca, ni a los vecinos ni a la iglesia.</t>
+        </is>
+      </c>
+      <c r="N160" s="61" t="inlineStr">
+        <is>
+          <t>Si tu familia necesita una mano, animate a pedirla; y si podés darla, ofrecela.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="61" t="n">
+        <v>27</v>
+      </c>
+      <c r="B161" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C161" s="61" t="inlineStr">
+        <is>
+          <t>Un pueblo justo</t>
+        </is>
+      </c>
+      <c r="D161" s="61" t="inlineStr">
+        <is>
+          <t>La Asamblea General de las Naciones Unidas proclamó en 1993 el 15 de mayo como Día Internacional de las Familias.</t>
+        </is>
+      </c>
+      <c r="E161" s="61" t="inlineStr">
+        <is>
+          <t>Naciones Unidas, resolución 47/237 de la Asamblea General, 1993</t>
+        </is>
+      </c>
+      <c r="F161" s="61" t="inlineStr">
+        <is>
+          <t>Este proverbio enseña un principio: la grandeza de un pueblo no está en su riqueza, sino en su justicia. Y un pueblo está hecho de familias.</t>
+        </is>
+      </c>
+      <c r="G161" s="61" t="inlineStr">
+        <is>
+          <t>Medir el progreso del país solo por la economía.</t>
+        </is>
+      </c>
+      <c r="H161" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en una persona justa de tu comunidad y agradecele lo que hace.</t>
+        </is>
+      </c>
+      <c r="I161" s="61" t="inlineStr">
+        <is>
+          <t>La corrupción grande suele empezar con pequeñas mentiras toleradas. Lo que se permite en casa termina pareciendo normal en la sociedad.</t>
+        </is>
+      </c>
+      <c r="J161" s="61" t="inlineStr">
+        <is>
+          <t>Justificar la «viveza» y el atajo como si fueran inteligencia.</t>
+        </is>
+      </c>
+      <c r="K161" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, no aceptes un atajo deshonesto aunque sea chico, y contá en casa por qué.</t>
+        </is>
+      </c>
+      <c r="L161" s="61" t="inlineStr">
+        <is>
+          <t>Familia y sociedad se necesitan: la escuela, la iglesia y el barrio refuerzan lo que se aprende en casa, y la casa sostiene lo que ellos enseñan.</t>
+        </is>
+      </c>
+      <c r="M161" s="61" t="inlineStr">
+        <is>
+          <t>Dejar toda la formación de los hijos en manos de la escuela o de la iglesia.</t>
+        </is>
+      </c>
+      <c r="N161" s="61" t="inlineStr">
+        <is>
+          <t>Acercate a la escuela de tus hijos o a un grupo de tu comunidad y preguntá cómo podés colaborar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="61" t="n">
+        <v>27</v>
+      </c>
+      <c r="B162" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C162" s="61" t="inlineStr">
+        <is>
+          <t>Hacer el bien a todos</t>
+        </is>
+      </c>
+      <c r="D162" s="61" t="inlineStr">
+        <is>
+          <t>En guaraní, «jopói» nombra la reciprocidad: dar y recibir con las manos abiertas, una práctica central de la vida comunitaria.</t>
+        </is>
+      </c>
+      <c r="E162" s="61" t="inlineStr">
+        <is>
+          <t>Bartomeu Melià y Dominique Temple, El don, la venganza y otras formas de economía guaraní, 2004</t>
+        </is>
+      </c>
+      <c r="F162" s="61" t="inlineStr">
+        <is>
+          <t>Pablo dice «según tengamos oportunidad». No hace falta un gesto grande: el bien diario de una familia ya es un aporte a la sociedad.</t>
+        </is>
+      </c>
+      <c r="G162" s="61" t="inlineStr">
+        <is>
+          <t>Esperar a tener mucho para empezar a ayudar.</t>
+        </is>
+      </c>
+      <c r="H162" s="61" t="inlineStr">
+        <is>
+          <t>Buscá hoy una oportunidad chica de hacer el bien fuera de tu casa, y aprovechala.</t>
+        </is>
+      </c>
+      <c r="I162" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide cuidar especialmente a los hermanos en la fe. Una iglesia que se cuida muestra al barrio cómo vive una familia sana.</t>
+        </is>
+      </c>
+      <c r="J162" s="61" t="inlineStr">
+        <is>
+          <t>Ir a la iglesia sin conocer ni cuidar a los que se sientan al lado.</t>
+        </is>
+      </c>
+      <c r="K162" s="61" t="inlineStr">
+        <is>
+          <t>Llamá esta semana a alguien de tu iglesia que hace tiempo no ves.</t>
+        </is>
+      </c>
+      <c r="L162" s="61" t="inlineStr">
+        <is>
+          <t>Una familia que resuelve los conflictos dialogando y cuida a sus miembros más frágiles siembra ese mismo modelo en la sociedad.</t>
+        </is>
+      </c>
+      <c r="M162" s="61" t="inlineStr">
+        <is>
+          <t>Hogares donde se grita o se golpea, y esa violencia después se repite en la calle.</t>
+        </is>
+      </c>
+      <c r="N162" s="61" t="inlineStr">
+        <is>
+          <t>Proponé en tu casa una regla: los conflictos se hablan sentados y sin gritos. Si en tu hogar hay violencia, pedí ayuda: en Paraguay, la línea 137 atiende casos de violencia contra la mujer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="61" t="n">
+        <v>27</v>
+      </c>
+      <c r="B163" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C163" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: la familia y la sociedad</t>
+        </is>
+      </c>
+      <c r="D163" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pidió orar por los reyes y las autoridades cuando los cristianos eran una minoría sin poder en el Imperio romano.</t>
+        </is>
+      </c>
+      <c r="E163" s="61" t="inlineStr">
+        <is>
+          <t>1 Timoteo 2:1-2</t>
+        </is>
+      </c>
+      <c r="F163" s="61" t="inlineStr">
+        <is>
+          <t>Lo que pasa en una familia no se queda en casa: buscar el bien de la ciudad también es parte de la fe.</t>
+        </is>
+      </c>
+      <c r="G163" s="61" t="n"/>
+      <c r="H163" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, oren en familia por las autoridades de tu ciudad y del país, por nombre, como pide Pablo.</t>
+        </is>
+      </c>
+      <c r="I163" s="61" t="inlineStr">
+        <is>
+          <t>Familia y sociedad se necesitan: la casa forma a la persona y la comunidad le da espacio a esa formación.</t>
+        </is>
+      </c>
+      <c r="J163" s="61" t="n"/>
+      <c r="K163" s="61" t="n"/>
+      <c r="L163" s="61" t="inlineStr">
+        <is>
+          <t>El bien diario de una familia, sin gritos y cuidando al más frágil, ya es un aporte a la sociedad.</t>
+        </is>
+      </c>
+      <c r="M163" s="61" t="n"/>
+      <c r="N163" s="61" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="B164" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C164" s="61" t="inlineStr">
+        <is>
+          <t>Fiel en lo poco</t>
+        </is>
+      </c>
+      <c r="D164" s="61" t="inlineStr">
+        <is>
+          <t>En el griego original dice «cinco talentos». Un talento equivalía a unos 6.000 denarios, y un denario era el pago de un día de trabajo de un jornalero.</t>
+        </is>
+      </c>
+      <c r="E164" s="61" t="inlineStr">
+        <is>
+          <t>Mateo 25:15 y 20:2; diccionarios bíblicos</t>
+        </is>
+      </c>
+      <c r="F164" s="61" t="inlineStr">
+        <is>
+          <t>Jesús habla de todo lo que Dios nos confía, y eso incluye el dinero. El siervo fiel no enterró lo recibido: lo puso a trabajar. Ahorrar guarda el dinero quieto; invertir lo pone a producir con un riesgo calculado.</t>
+        </is>
+      </c>
+      <c r="G164" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que administrar bien o invertir es solo cosa de ricos.</t>
+        </is>
+      </c>
+      <c r="H164" s="61" t="inlineStr">
+        <is>
+          <t>Anotá qué recursos tenés hoy, aunque sean pocos: tiempo, un oficio, una herramienta, un ahorro.</t>
+        </is>
+      </c>
+      <c r="I164" s="61" t="inlineStr">
+        <is>
+          <t>El señor no le dice «ahora sos rico», sino «sobre mucho te pondré» y «entra en el gozo de tu señor». La recompensa es más confianza y comunión con él, no una ganancia asegurada.</t>
+        </is>
+      </c>
+      <c r="J164" s="61" t="inlineStr">
+        <is>
+          <t>Usar esta parábola para prometer que Dios multiplica la plata del que invierte.</t>
+        </is>
+      </c>
+      <c r="K164" s="61" t="inlineStr">
+        <is>
+          <t>Antes de buscar ganar más, preguntate: ¿estoy siendo fiel con lo que ya tengo?</t>
+        </is>
+      </c>
+      <c r="L164" s="61" t="inlineStr">
+        <is>
+          <t>El que ganó dos mil recibe exactamente el mismo elogio que el que ganó cinco mil (25:23). Dios mira la fidelidad, no el tamaño.</t>
+        </is>
+      </c>
+      <c r="M164" s="61" t="inlineStr">
+        <is>
+          <t>Compararse con quien tiene más y sentir que lo propio no vale.</t>
+        </is>
+      </c>
+      <c r="N164" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy por lo que tenés y decidí una forma concreta de cuidarlo mejor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="B165" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C165" s="61" t="inlineStr">
+        <is>
+          <t>Echá tu pan sobre las aguas</t>
+        </is>
+      </c>
+      <c r="D165" s="61" t="inlineStr">
+        <is>
+          <t>Según la «regla del 72», si dividís 72 por la tasa de interés anual, sabés en cuántos años se duplica un ahorro: al 6 % anual, en unos 12 años.</t>
+        </is>
+      </c>
+      <c r="E165" s="61" t="inlineStr">
+        <is>
+          <t>Regla del 72, aproximación del interés compuesto</t>
+        </is>
+      </c>
+      <c r="F165" s="61" t="inlineStr">
+        <is>
+          <t>El pan echado sobre las aguas se encuentra «después de muchos días». Unos lo leen como generosidad y otros como el comercio por mar; en los dos casos, lo que se suelta hoy da fruto más adelante.</t>
+        </is>
+      </c>
+      <c r="G165" s="61" t="inlineStr">
+        <is>
+          <t>Querer resultados ya y abandonar a la primera.</t>
+        </is>
+      </c>
+      <c r="H165" s="61" t="inlineStr">
+        <is>
+          <t>Separá una parte fija de lo que ganás, aunque sea pequeña, antes de empezar a gastar.</t>
+        </is>
+      </c>
+      <c r="I165" s="61" t="inlineStr">
+        <is>
+          <t>El versículo siguiente aconseja repartir entre siete y aun entre ocho, porque no sabemos qué mal vendrá (11:2). La sabiduría antigua ya enseñaba a no poner todo en un solo lugar.</t>
+        </is>
+      </c>
+      <c r="J165" s="61" t="inlineStr">
+        <is>
+          <t>Poner todos los ahorros en un solo negocio o en una promesa de ganancia rápida.</t>
+        </is>
+      </c>
+      <c r="K165" s="61" t="inlineStr">
+        <is>
+          <t>Antes de invertir, pedí consejo a alguien que sepa y que no tenga interés en venderte nada.</t>
+        </is>
+      </c>
+      <c r="L165" s="61" t="inlineStr">
+        <is>
+          <t>Invertir con sabiduría no es jugar a la suerte: es tomar decisiones informadas y dejar el resultado en manos de Dios, que es quien sostiene todo.</t>
+        </is>
+      </c>
+      <c r="M165" s="61" t="inlineStr">
+        <is>
+          <t>Contar con ganancias seguras y desesperarse cuando no llegan.</t>
+        </is>
+      </c>
+      <c r="N165" s="61" t="inlineStr">
+        <is>
+          <t>Calculá cuánto podrías perder sin poner en riesgo la comida, el alquiler o las deudas de tu casa, y no arriesgues más que eso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="B166" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C166" s="61" t="inlineStr">
+        <is>
+          <t>El principio de la sabiduría</t>
+        </is>
+      </c>
+      <c r="D166" s="61" t="inlineStr">
+        <is>
+          <t>Según una encuesta mundial de S&amp;P, solo uno de cada tres adultos entiende conceptos financieros básicos como el interés compuesto, la inflación y la diversificación del riesgo.</t>
+        </is>
+      </c>
+      <c r="E166" s="61" t="inlineStr">
+        <is>
+          <t>Klapper, Lusardi y van Oudheusden, Encuesta Global de Educación Financiera de S&amp;P, 2015</t>
+        </is>
+      </c>
+      <c r="F166" s="61" t="inlineStr">
+        <is>
+          <t>La primera decisión financiera sabia no es dónde poner la plata, sino reconocer a quién pertenece todo. Reconocer a Dios pone el dinero en su lugar: herramienta, no dueño.</t>
+        </is>
+      </c>
+      <c r="G166" s="61" t="inlineStr">
+        <is>
+          <t>Buscar la seguridad solo en el dinero.</t>
+        </is>
+      </c>
+      <c r="H166" s="61" t="inlineStr">
+        <is>
+          <t>Antes de una decisión de plata, orá y preguntate si honra a Dios y cuida a tu familia.</t>
+        </is>
+      </c>
+      <c r="I166" s="61" t="inlineStr">
+        <is>
+          <t>No hace falta ser experto ni tener grandes sumas para empezar, pero sí aprender: qué es el interés, qué es la inflación, qué es el riesgo.</t>
+        </is>
+      </c>
+      <c r="J166" s="61" t="inlineStr">
+        <is>
+          <t>Decidir por lo que dice un video o un conocido sin entender de qué se trata.</t>
+        </is>
+      </c>
+      <c r="K166" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, aprendé un concepto financiero básico con una fuente seria, como los materiales de educación financiera del Banco Central del Paraguay.</t>
+        </is>
+      </c>
+      <c r="L166" s="61" t="inlineStr">
+        <is>
+          <t>El necio desprecia la enseñanza. En finanzas, desconfiá de quien promete ganancias altas, rápidas y sin riesgo.</t>
+        </is>
+      </c>
+      <c r="M166" s="61" t="inlineStr">
+        <is>
+          <t>Caer en esquemas piramidales o en «inversiones» que piden traer a otros para ganar.</t>
+        </is>
+      </c>
+      <c r="N166" s="61" t="inlineStr">
+        <is>
+          <t>Si alguien te ofrece duplicar tu plata rápido, pedí consejo antes de poner un solo guaraní.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="B167" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C167" s="61" t="inlineStr">
+        <is>
+          <t>Volver a levantarse</t>
+        </is>
+      </c>
+      <c r="D167" s="61" t="inlineStr">
+        <is>
+          <t>Warren Buffett compró sus primeras acciones a los 11 años; cuando bajaron, las vendió apenas recuperó lo invertido, y después subieron mucho. Dijo que aprendió a tener paciencia.</t>
+        </is>
+      </c>
+      <c r="E167" s="61" t="inlineStr">
+        <is>
+          <t>Alice Schroeder, La bola de nieve (biografía de Warren Buffett), 2008</t>
+        </is>
+      </c>
+      <c r="F167" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio no dice que el justo no cae: dice que cae y se levanta. El justo es el que vive confiando en Dios, no el que nunca se equivoca.</t>
+        </is>
+      </c>
+      <c r="G167" s="61" t="inlineStr">
+        <is>
+          <t>Creer que un error con la plata te descalifica para siempre.</t>
+        </is>
+      </c>
+      <c r="H167" s="61" t="inlineStr">
+        <is>
+          <t>Si te equivocaste con plata, anotá qué aprendiste antes de volver a intentar.</t>
+        </is>
+      </c>
+      <c r="I167" s="61" t="inlineStr">
+        <is>
+          <t>Empezar con montos pequeños permite aprender sin arriesgar lo que la familia necesita.</t>
+        </is>
+      </c>
+      <c r="J167" s="61" t="inlineStr">
+        <is>
+          <t>Arriesgar de golpe todo lo ahorrado para recuperar una pérdida.</t>
+        </is>
+      </c>
+      <c r="K167" s="61" t="inlineStr">
+        <is>
+          <t>Si querés invertir, empezá con un monto chico y aprendé en el camino.</t>
+        </is>
+      </c>
+      <c r="L167" s="61" t="inlineStr">
+        <is>
+          <t>Levantarse no es repetir el mismo error, sino ajustar. La perseverancia sabia aprende y corrige.</t>
+        </is>
+      </c>
+      <c r="M167" s="61" t="inlineStr">
+        <is>
+          <t>Insistir por orgullo en algo que claramente no funciona.</t>
+        </is>
+      </c>
+      <c r="N167" s="61" t="inlineStr">
+        <is>
+          <t>Pedile a alguien de confianza que revise tus números una vez al mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="B168" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C168" s="61" t="inlineStr">
+        <is>
+          <t>Donde está tu tesoro</t>
+        </is>
+      </c>
+      <c r="D168" s="61" t="inlineStr">
+        <is>
+          <t>En tiempos bíblicos, la ropa fina era una forma de riqueza que se guardaba, y por eso la polilla era una amenaza real.</t>
+        </is>
+      </c>
+      <c r="E168" s="61" t="inlineStr">
+        <is>
+          <t>Josué 7:21; Hechos 20:33; Santiago 5:2</t>
+        </is>
+      </c>
+      <c r="F168" s="61" t="inlineStr">
+        <is>
+          <t>Jesús no condena ahorrar o invertir; advierte contra acumular para uno mismo y poner ahí la confianza. Todo lo de esta tierra se gasta.</t>
+        </is>
+      </c>
+      <c r="G168" s="61" t="inlineStr">
+        <is>
+          <t>Ahorrar o invertir por ansiedad o por codicia, queriendo siempre más.</t>
+        </is>
+      </c>
+      <c r="H168" s="61" t="inlineStr">
+        <is>
+          <t>Definí para qué querés ahorrar o invertir: la educación de tus hijos, una casa, poder ayudar a otros.</t>
+        </is>
+      </c>
+      <c r="I168" s="61" t="inlineStr">
+        <is>
+          <t>El crecimiento financiero lleva años, pero lo eterno se construye cada día: el amor, la generosidad, las personas.</t>
+        </is>
+      </c>
+      <c r="J168" s="61" t="inlineStr">
+        <is>
+          <t>Sacrificar hoy a la familia por un futuro económico que nunca termina de llegar.</t>
+        </is>
+      </c>
+      <c r="K168" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, invertí tiempo en tu familia con la misma seriedad con que cuidás tu dinero.</t>
+        </is>
+      </c>
+      <c r="L168" s="61" t="inlineStr">
+        <is>
+          <t>Donde ponemos la plata, ahí va el corazón. La paciencia financiera nace de un corazón que ya descansa en Dios.</t>
+        </is>
+      </c>
+      <c r="M168" s="61" t="inlineStr">
+        <is>
+          <t>Revisar las cuentas a cada rato y perder la paz.</t>
+        </is>
+      </c>
+      <c r="N168" s="61" t="inlineStr">
+        <is>
+          <t>Revisá tus finanzas en un momento fijo, por ejemplo una vez al mes, y el resto del tiempo descansá en Dios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="61" t="n">
+        <v>28</v>
+      </c>
+      <c r="B169" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C169" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: ahorrar, invertir y esperar</t>
+        </is>
+      </c>
+      <c r="D169" s="61" t="inlineStr">
+        <is>
+          <t>Benjamin Franklin dejó en su testamento 1.000 libras a Boston y 1.000 a Filadelfia para que crecieran durante 200 años prestándoselas a jóvenes artesanos.</t>
+        </is>
+      </c>
+      <c r="E169" s="61" t="inlineStr">
+        <is>
+          <t>Testamento de Benjamin Franklin, 1789</t>
+        </is>
+      </c>
+      <c r="F169" s="61" t="inlineStr">
+        <is>
+          <t>Ahorrar protege y invertir hace crecer; Dios mira la fidelidad con lo que nos confía, no el tamaño.</t>
+        </is>
+      </c>
+      <c r="G169" s="61" t="n"/>
+      <c r="H169" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, siéntense en familia, definan una meta de ahorro con un propósito y pidan consejo antes de cualquier inversión.</t>
+        </is>
+      </c>
+      <c r="I169" s="61" t="inlineStr">
+        <is>
+          <t>Para empezar: aprender, empezar con poco y no arriesgar lo que la familia necesita.</t>
+        </is>
+      </c>
+      <c r="J169" s="61" t="n"/>
+      <c r="K169" s="61" t="n"/>
+      <c r="L169" s="61" t="inlineStr">
+        <is>
+          <t>El crecimiento lleva tiempo, y el corazón tiene que estar en Dios y no en la plata.</t>
+        </is>
+      </c>
+      <c r="M169" s="61" t="n"/>
+      <c r="N169" s="61" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="61" t="n">
+        <v>29</v>
+      </c>
+      <c r="B170" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C170" s="61" t="inlineStr">
+        <is>
+          <t>Prosigo a la meta</t>
+        </is>
+      </c>
+      <c r="D170" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribió la carta a los Filipenses estando preso, y aun así habla de seguir avanzando hacia la meta.</t>
+        </is>
+      </c>
+      <c r="E170" s="61" t="inlineStr">
+        <is>
+          <t>Filipenses 1:13</t>
+        </is>
+      </c>
+      <c r="F170" s="61" t="inlineStr">
+        <is>
+          <t>Pablo, preso y con un pasado del que no se enorgullecía, decide no quedar atado a lo que pasó.</t>
+        </is>
+      </c>
+      <c r="G170" s="61" t="inlineStr">
+        <is>
+          <t>Repetirse «yo ya fallé antes» y no volver a intentar.</t>
+        </is>
+      </c>
+      <c r="H170" s="61" t="inlineStr">
+        <is>
+          <t>Escribí una cosa del pasado que te frena y entregásela a Dios en oración.</t>
+        </is>
+      </c>
+      <c r="I170" s="61" t="inlineStr">
+        <is>
+          <t>Pablo tiene una meta clara: el llamado de Dios en Cristo. Un deseo vago, como «quiero mejorar», no da dirección; una meta concreta, sí.</t>
+        </is>
+      </c>
+      <c r="J170" s="61" t="inlineStr">
+        <is>
+          <t>Vivir de deseos generales que nunca se concretan.</t>
+        </is>
+      </c>
+      <c r="K170" s="61" t="inlineStr">
+        <is>
+          <t>Convertí un deseo en meta: en vez de «quiero leer más», «voy a leer un capítulo cada noche».</t>
+        </is>
+      </c>
+      <c r="L170" s="61" t="inlineStr">
+        <is>
+          <t>Nuestras metas personales son pequeñas al lado del llamado de Dios, pero pueden ponerse a su servicio.</t>
+        </is>
+      </c>
+      <c r="M170" s="61" t="inlineStr">
+        <is>
+          <t>Metas que solo giran alrededor de uno mismo.</t>
+        </is>
+      </c>
+      <c r="N170" s="61" t="inlineStr">
+        <is>
+          <t>Preguntate: ¿esta meta me ayuda a amar mejor a Dios y a los demás?</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="61" t="n">
+        <v>29</v>
+      </c>
+      <c r="B171" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C171" s="61" t="inlineStr">
+        <is>
+          <t>Escribila</t>
+        </is>
+      </c>
+      <c r="D171" s="61" t="inlineStr">
+        <is>
+          <t>En un estudio de la psicóloga Gail Matthews, quienes escribieron sus metas y enviaron informes de avance a un amigo lograron más que quienes solo las pensaron. Fue un estudio pequeño.</t>
+        </is>
+      </c>
+      <c r="E171" s="61" t="inlineStr">
+        <is>
+          <t>Gail Matthews, Universidad Dominicana de California, 2015</t>
+        </is>
+      </c>
+      <c r="F171" s="61" t="inlineStr">
+        <is>
+          <t>Dios le pide a Habacuc que escriba la visión con claridad. Era una revelación de Dios, no una meta personal, pero el principio de escribir con claridad nos sirve.</t>
+        </is>
+      </c>
+      <c r="G171" s="61" t="inlineStr">
+        <is>
+          <t>Tener las metas solo en la cabeza, cambiándolas cada día.</t>
+        </is>
+      </c>
+      <c r="H171" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, escribí una meta específica y medible en un papel o en el celular.</t>
+        </is>
+      </c>
+      <c r="I171" s="61" t="inlineStr">
+        <is>
+          <t>«Para que pueda leerse de corrido»: lo escrito se puede compartir. Contarle tu meta a alguien de confianza te ayuda a sostenerla.</t>
+        </is>
+      </c>
+      <c r="J171" s="61" t="inlineStr">
+        <is>
+          <t>Esconder las metas por miedo a quedar mal si no se cumplen.</t>
+        </is>
+      </c>
+      <c r="K171" s="61" t="inlineStr">
+        <is>
+          <t>Compartí tu meta con una persona que te pueda preguntar cómo vas.</t>
+        </is>
+      </c>
+      <c r="L171" s="61" t="inlineStr">
+        <is>
+          <t>Una meta específica tiene un qué, un cuánto y un cuándo: «caminar tres veces por semana» se puede seguir y evaluar.</t>
+        </is>
+      </c>
+      <c r="M171" s="61" t="inlineStr">
+        <is>
+          <t>Metas tan grandes que asustan y nunca se empiezan.</t>
+        </is>
+      </c>
+      <c r="N171" s="61" t="inlineStr">
+        <is>
+          <t>Ponele a tu meta un número y una fecha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="61" t="n">
+        <v>29</v>
+      </c>
+      <c r="B172" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C172" s="61" t="inlineStr">
+        <is>
+          <t>Pedir, buscar y llamar</t>
+        </is>
+      </c>
+      <c r="D172" s="61" t="inlineStr">
+        <is>
+          <t>Una revisión de 94 estudios encontró que decidir de antemano cuándo, dónde y cómo se va a dar un paso aumenta mucho la probabilidad de cumplir una meta.</t>
+        </is>
+      </c>
+      <c r="E172" s="61" t="inlineStr">
+        <is>
+          <t>Gollwitzer y Sheeran, Advances in Experimental Social Psychology, 2006</t>
+        </is>
+      </c>
+      <c r="F172" s="61" t="inlineStr">
+        <is>
+          <t>Jesús invita a pedirle a un Padre bueno, que da cosas buenas a sus hijos (7:11). No es una fórmula para conseguir cualquier cosa, sino confianza en quien sabe lo que nos conviene.</t>
+        </is>
+      </c>
+      <c r="G172" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que si algo no se dio, fue porque no oramos lo suficiente.</t>
+        </is>
+      </c>
+      <c r="H172" s="61" t="inlineStr">
+        <is>
+          <t>Antes de armar tu plan, presentáselo a Dios en oración.</t>
+        </is>
+      </c>
+      <c r="I172" s="61" t="inlineStr">
+        <is>
+          <t>Buscar es poner manos a la obra. Una meta sin plan es solo una intención: hacen falta pasos concretos.</t>
+        </is>
+      </c>
+      <c r="J172" s="61" t="inlineStr">
+        <is>
+          <t>Orar por una meta y no dar ningún paso.</t>
+        </is>
+      </c>
+      <c r="K172" s="61" t="inlineStr">
+        <is>
+          <t>Escribí los tres primeros pasos de tu meta, con cuándo y dónde vas a dar cada uno.</t>
+        </is>
+      </c>
+      <c r="L172" s="61" t="inlineStr">
+        <is>
+          <t>Llamar es insistir. Revisar el avance cada semana permite ver si los pasos se están dando.</t>
+        </is>
+      </c>
+      <c r="M172" s="61" t="inlineStr">
+        <is>
+          <t>Revisar la meta solo a fin de año, cuando ya es tarde para corregir.</t>
+        </is>
+      </c>
+      <c r="N172" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un día de la semana para revisar tu avance, aunque sea cinco minutos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="61" t="n">
+        <v>29</v>
+      </c>
+      <c r="B173" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C173" s="61" t="inlineStr">
+        <is>
+          <t>Constantes</t>
+        </is>
+      </c>
+      <c r="D173" s="61" t="inlineStr">
+        <is>
+          <t>Un análisis de 138 estudios encontró que registrar el propio avance ayuda a alcanzar las metas, sobre todo cuando se anota o se cuenta a otros.</t>
+        </is>
+      </c>
+      <c r="E173" s="61" t="inlineStr">
+        <is>
+          <t>Harkin y otros, Psychological Bulletin, 2016</t>
+        </is>
+      </c>
+      <c r="F173" s="61" t="inlineStr">
+        <is>
+          <t>La esperanza de Pablo está puesta en Dios, no en el éxito de nuestros planes. Eso permite avanzar con alegría aunque el plan cambie.</t>
+        </is>
+      </c>
+      <c r="G173" s="61" t="inlineStr">
+        <is>
+          <t>Perder la alegría cuando algo no sale como se planeó.</t>
+        </is>
+      </c>
+      <c r="H173" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy por un paso que diste, aunque sea pequeño.</t>
+        </is>
+      </c>
+      <c r="I173" s="61" t="inlineStr">
+        <is>
+          <t>Todo plan encuentra obstáculos. Ajustar el plan no es fracasar: es parte del proceso.</t>
+        </is>
+      </c>
+      <c r="J173" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar la meta entera porque un paso falló.</t>
+        </is>
+      </c>
+      <c r="K173" s="61" t="inlineStr">
+        <is>
+          <t>Si un paso no funcionó esta semana, cambialo por otro más realista en vez de abandonar.</t>
+        </is>
+      </c>
+      <c r="L173" s="61" t="inlineStr">
+        <is>
+          <t>La constancia en la oración y la constancia en el plan van juntas: revisar el avance delante de Dios mantiene el rumbo.</t>
+        </is>
+      </c>
+      <c r="M173" s="61" t="inlineStr">
+        <is>
+          <t>Hacer planes sin incluir a Dios, o incluirlo solo cuando algo sale mal.</t>
+        </is>
+      </c>
+      <c r="N173" s="61" t="inlineStr">
+        <is>
+          <t>Cuando revises tu avance semanal, empezá con una breve oración.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="61" t="n">
+        <v>29</v>
+      </c>
+      <c r="B174" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C174" s="61" t="inlineStr">
+        <is>
+          <t>Mirar el camino recorrido</t>
+        </is>
+      </c>
+      <c r="D174" s="61" t="inlineStr">
+        <is>
+          <t>Job 22:28 lo dice Elifaz, uno de los amigos de Job. Al final del libro, Dios les dice a esos amigos que no hablaron de él lo recto (Job 42:7).</t>
+        </is>
+      </c>
+      <c r="E174" s="61" t="inlineStr">
+        <is>
+          <t>Job 22:1; 42:7</t>
+        </is>
+      </c>
+      <c r="F174" s="61" t="inlineStr">
+        <is>
+          <t>Elifaz le promete a Job éxito en todos sus planes si se vuelve a Dios, porque pensaba que su sufrimiento era un castigo. Dios corrigió esa idea: no todo lo que nos pasa es premio o castigo.</t>
+        </is>
+      </c>
+      <c r="G174" s="61" t="inlineStr">
+        <is>
+          <t>Evaluar la vida como si cada logro fuera un premio y cada tropiezo, un castigo.</t>
+        </is>
+      </c>
+      <c r="H174" s="61" t="inlineStr">
+        <is>
+          <t>Al evaluar tu camino, no te juzgues con la dureza de los amigos de Job: mirá con honestidad y con gracia.</t>
+        </is>
+      </c>
+      <c r="I174" s="61" t="inlineStr">
+        <is>
+          <t>Evaluar lo avanzado, y no solo lo que falta, da perspectiva y sostiene la motivación. Y nos recuerda que fue Dios quien nos sostuvo hasta acá.</t>
+        </is>
+      </c>
+      <c r="J174" s="61" t="inlineStr">
+        <is>
+          <t>Mirar solo lo que falta y sentir que nunca se avanza.</t>
+        </is>
+      </c>
+      <c r="K174" s="61" t="inlineStr">
+        <is>
+          <t>Nombrá un logro pequeño de las últimas semanas que quizás pasó desapercibido.</t>
+        </is>
+      </c>
+      <c r="L174" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios dice que el corazón del hombre traza su camino, pero el Señor dirige sus pasos (16:9). Evaluar es también preguntarle a Dios por el próximo paso.</t>
+        </is>
+      </c>
+      <c r="M174" s="61" t="inlineStr">
+        <is>
+          <t>Planificar todo sin dejar lugar a que Dios corrija el rumbo.</t>
+        </is>
+      </c>
+      <c r="N174" s="61" t="inlineStr">
+        <is>
+          <t>Después de evaluar, escribí el próximo paso y pedile a Dios su dirección.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="61" t="n">
+        <v>29</v>
+      </c>
+      <c r="B175" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C175" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: metas con propósito</t>
+        </is>
+      </c>
+      <c r="D175" s="61" t="inlineStr">
+        <is>
+          <t>La palabra «ojalá» viene del árabe hispánico y significa «si Dios quiere».</t>
+        </is>
+      </c>
+      <c r="E175" s="61" t="inlineStr">
+        <is>
+          <t>Real Academia Española, Diccionario de la lengua española, «ojalá»</t>
+        </is>
+      </c>
+      <c r="F175" s="61" t="inlineStr">
+        <is>
+          <t>Una meta clara y escrita da dirección; un deseo vago, no.</t>
+        </is>
+      </c>
+      <c r="G175" s="61" t="n"/>
+      <c r="H175" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, escribí una meta concreta, sus tres primeros pasos y el día en que vas a revisarla, y entregásela a Dios diciendo: «Si el Señor quiere».</t>
+        </is>
+      </c>
+      <c r="I175" s="61" t="inlineStr">
+        <is>
+          <t>Una meta sin plan es solo una intención: pasos concretos y revisión semanal, delante de Dios.</t>
+        </is>
+      </c>
+      <c r="J175" s="61" t="n"/>
+      <c r="K175" s="61" t="n"/>
+      <c r="L175" s="61" t="inlineStr">
+        <is>
+          <t>Evaluar lo avanzado con honestidad y con gracia sostiene la motivación.</t>
+        </is>
+      </c>
+      <c r="M175" s="61" t="n"/>
+      <c r="N175" s="61" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="B176" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C176" s="61" t="inlineStr">
+        <is>
+          <t>Pesas justas</t>
+        </is>
+      </c>
+      <c r="D176" s="61" t="inlineStr">
+        <is>
+          <t>En Paraguay, el Instituto Nacional de Tecnología, Normalización y Metrología (INTN) verifica balanzas y surtidores de combustible para que el cliente reciba lo que paga.</t>
+        </is>
+      </c>
+      <c r="E176" s="61" t="inlineStr">
+        <is>
+          <t>INTN, Metrología Legal</t>
+        </is>
+      </c>
+      <c r="F176" s="61" t="inlineStr">
+        <is>
+          <t>En los mercados antiguos todo se pesaba con balanzas y pesas de piedra, y era fácil hacer trampa. A Dios le importa ese detalle.</t>
+        </is>
+      </c>
+      <c r="G176" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que una pequeña trampa en el negocio no le importa a nadie.</t>
+        </is>
+      </c>
+      <c r="H176" s="61" t="inlineStr">
+        <is>
+          <t>Si vendés, revisá hoy tus balanzas, tus medidas y tus precios.</t>
+        </is>
+      </c>
+      <c r="I176" s="61" t="inlineStr">
+        <is>
+          <t>El precio justo, el peso correcto y la calidad prometida construyen una reputación que dura años, más que cualquier promoción.</t>
+        </is>
+      </c>
+      <c r="J176" s="61" t="inlineStr">
+        <is>
+          <t>Ganar clientes con ofertas y perderlos con engaños.</t>
+        </is>
+      </c>
+      <c r="K176" s="61" t="inlineStr">
+        <is>
+          <t>Ofrecé lo que realmente podés cumplir, ni más ni menos.</t>
+        </is>
+      </c>
+      <c r="L176" s="61" t="inlineStr">
+        <is>
+          <t>Comprar y vender también es parte de la vida de fe: el lunes en el negocio se ve lo que se cantó el domingo.</t>
+        </is>
+      </c>
+      <c r="M176" s="61" t="inlineStr">
+        <is>
+          <t>Separar la fe del bolsillo.</t>
+        </is>
+      </c>
+      <c r="N176" s="61" t="inlineStr">
+        <is>
+          <t>Si te dieron de más en el vuelto, devolvelo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="B177" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C177" s="61" t="inlineStr">
+        <is>
+          <t>Medidas que son del Señor</t>
+        </is>
+      </c>
+      <c r="D177" s="61" t="inlineStr">
+        <is>
+          <t>En excavaciones de Judá se encontraron pesas de piedra de los siglos VIII y VII antes de Cristo, marcadas con su valor en siclos.</t>
+        </is>
+      </c>
+      <c r="E177" s="61" t="inlineStr">
+        <is>
+          <t>Raz Kletter, Economic Keystones: The Weight System of the Kingdom of Judah, 1998</t>
+        </is>
+      </c>
+      <c r="F177" s="61" t="inlineStr">
+        <is>
+          <t>Las medidas justas «son del Señor»: la honestidad en el comercio refleja su carácter.</t>
+        </is>
+      </c>
+      <c r="G177" s="61" t="inlineStr">
+        <is>
+          <t>Bajar la calidad a escondidas para ganar un poco más.</t>
+        </is>
+      </c>
+      <c r="H177" s="61" t="inlineStr">
+        <is>
+          <t>Si cambiaste algo de tu producto, avisale al cliente.</t>
+        </is>
+      </c>
+      <c r="I177" s="61" t="inlineStr">
+        <is>
+          <t>Ninguna venta queda fuera de la mirada de Dios, ni la grande ni la de un kilo de mandioca.</t>
+        </is>
+      </c>
+      <c r="J177" s="61" t="inlineStr">
+        <is>
+          <t>Ser honesto con el cliente importante y descuidado con el pequeño.</t>
+        </is>
+      </c>
+      <c r="K177" s="61" t="inlineStr">
+        <is>
+          <t>Tratá con la misma honestidad al que compra mucho y al que compra poco.</t>
+        </is>
+      </c>
+      <c r="L177" s="61" t="inlineStr">
+        <is>
+          <t>El cliente también tiene su parte: pagar lo acordado, no engañar al vendedor, cumplir con las cuotas.</t>
+        </is>
+      </c>
+      <c r="M177" s="61" t="inlineStr">
+        <is>
+          <t>Exigir honestidad al comerciante y no pagar lo que se debe.</t>
+        </is>
+      </c>
+      <c r="N177" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés una deuda con un comercio del barrio, acordá hoy cómo la vas a pagar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="B178" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C178" s="61" t="inlineStr">
+        <is>
+          <t>El comercio de tu barrio</t>
+        </is>
+      </c>
+      <c r="D178" s="61" t="inlineStr">
+        <is>
+          <t>Según el Ministerio de Industria y Comercio, las micro, pequeñas y medianas empresas son la gran mayoría de las empresas del Paraguay.</t>
+        </is>
+      </c>
+      <c r="E178" s="61" t="inlineStr">
+        <is>
+          <t>Ministerio de Industria y Comercio, Viceministerio de MIPYMES</t>
+        </is>
+      </c>
+      <c r="F178" s="61" t="inlineStr">
+        <is>
+          <t>Este proverbio no da un mandato: describe con humor lo que pasa en el mercado. El comprador critica para bajar el precio y después se jacta de su compra.</t>
+        </is>
+      </c>
+      <c r="G178" s="61" t="inlineStr">
+        <is>
+          <t>Despreciar el trabajo del otro solo para pagar menos.</t>
+        </is>
+      </c>
+      <c r="H178" s="61" t="inlineStr">
+        <is>
+          <t>Si negociás un precio, hacelo con respeto, sin desmerecer el producto.</t>
+        </is>
+      </c>
+      <c r="I178" s="61" t="inlineStr">
+        <is>
+          <t>Detrás de cada comercio del barrio hay una familia. Cada compra allí sostiene un hogar de la comunidad.</t>
+        </is>
+      </c>
+      <c r="J178" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que comprar en el barrio o en otro lado da lo mismo.</t>
+        </is>
+      </c>
+      <c r="K178" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, cuando puedas, hacé tus compras en un comercio de tu zona.</t>
+        </is>
+      </c>
+      <c r="L178" s="61" t="inlineStr">
+        <is>
+          <t>Apoyar el comercio local no es aceptar cualquier precio o calidad: es una relación honesta en ambos lados.</t>
+        </is>
+      </c>
+      <c r="M178" s="61" t="inlineStr">
+        <is>
+          <t>Comercios que abusan porque «el cliente igual vuelve».</t>
+        </is>
+      </c>
+      <c r="N178" s="61" t="inlineStr">
+        <is>
+          <t>Si sos cliente fiel de un comercio, decile lo que valorás y lo que podría mejorar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="B179" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C179" s="61" t="inlineStr">
+        <is>
+          <t>Miembros los unos de los otros</t>
+        </is>
+      </c>
+      <c r="D179" s="61" t="inlineStr">
+        <is>
+          <t>Un estudio en un barrio de Chicago encontró que, de cada 100 dólares gastados en comercios locales, unos 68 seguían circulando en la economía de la zona, frente a 43 en las cadenas.</t>
+        </is>
+      </c>
+      <c r="E179" s="61" t="inlineStr">
+        <is>
+          <t>Civic Economics, Andersonville Study of Retail Economics, 2004</t>
+        </is>
+      </c>
+      <c r="F179" s="61" t="inlineStr">
+        <is>
+          <t>Pablo da la razón para no mentir: «somos miembros los unos de los otros». En el barrio, lo que le hago al otro me vuelve.</t>
+        </is>
+      </c>
+      <c r="G179" s="61" t="inlineStr">
+        <is>
+          <t>Mentir sobre un producto para cerrar una venta.</t>
+        </is>
+      </c>
+      <c r="H179" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, decí la verdad sobre lo que vendés, aunque pierdas una venta.</t>
+        </is>
+      </c>
+      <c r="I179" s="61" t="inlineStr">
+        <is>
+          <t>Cuando compramos en un comercio local, buena parte de esa plata vuelve a circular en la comunidad.</t>
+        </is>
+      </c>
+      <c r="J179" s="61" t="inlineStr">
+        <is>
+          <t>Quejarse de que el barrio no progresa y no apoyarlo nunca.</t>
+        </is>
+      </c>
+      <c r="K179" s="61" t="inlineStr">
+        <is>
+          <t>Recomendá a un amigo o en tus redes un comercio honesto de tu zona.</t>
+        </is>
+      </c>
+      <c r="L179" s="61" t="inlineStr">
+        <is>
+          <t>Comercio y comunidad se cuidan mutuamente: el comerciante sirve bien y el vecino lo sostiene.</t>
+        </is>
+      </c>
+      <c r="M179" s="61" t="inlineStr">
+        <is>
+          <t>Ver al comerciante solo como alguien que quiere sacar plata.</t>
+        </is>
+      </c>
+      <c r="N179" s="61" t="inlineStr">
+        <is>
+          <t>Saludá por su nombre al comerciante de tu barrio y agradecele su servicio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="B180" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C180" s="61" t="inlineStr">
+        <is>
+          <t>De hecho y en verdad</t>
+        </is>
+      </c>
+      <c r="D180" s="61" t="inlineStr">
+        <is>
+          <t>WhatsApp lanzó su aplicación para pequeñas empresas, WhatsApp Business, en enero de 2018.</t>
+        </is>
+      </c>
+      <c r="E180" s="61" t="inlineStr">
+        <is>
+          <t>WhatsApp, anuncio oficial, 18 de enero de 2018</t>
+        </is>
+      </c>
+      <c r="F180" s="61" t="inlineStr">
+        <is>
+          <t>Juan pide amar de hecho. Para un comercio, amar al cliente es servirlo bien también en las nuevas formas: un mensaje respondido a tiempo, un pedido entregado como se prometió.</t>
+        </is>
+      </c>
+      <c r="G180" s="61" t="inlineStr">
+        <is>
+          <t>Prometer atención por redes y no responder nunca.</t>
+        </is>
+      </c>
+      <c r="H180" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un emprendimiento, respondé hoy los mensajes pendientes de tus clientes.</t>
+        </is>
+      </c>
+      <c r="I180" s="61" t="inlineStr">
+        <is>
+          <t>Muchos comercios pequeños ya venden por WhatsApp o redes sin grandes inversiones. Adaptarse es encontrar nuevas formas de servir.</t>
+        </is>
+      </c>
+      <c r="J180" s="61" t="inlineStr">
+        <is>
+          <t>Quedarse atrás por miedo a lo nuevo.</t>
+        </is>
+      </c>
+      <c r="K180" s="61" t="inlineStr">
+        <is>
+          <t>Pedile a alguien joven de tu familia que te enseñe una herramienta simple para vender o comunicarte.</t>
+        </is>
+      </c>
+      <c r="L180" s="61" t="inlineStr">
+        <is>
+          <t>Adaptarse no significa perder la esencia: la honestidad del mostrador tiene que ser la misma en la pantalla.</t>
+        </is>
+      </c>
+      <c r="M180" s="61" t="inlineStr">
+        <is>
+          <t>Fotos que muestran algo distinto de lo que se entrega.</t>
+        </is>
+      </c>
+      <c r="N180" s="61" t="inlineStr">
+        <is>
+          <t>Publicá fotos y precios reales de lo que ofrecés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="61" t="n">
+        <v>30</v>
+      </c>
+      <c r="B181" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C181" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: comercio con integridad</t>
+        </is>
+      </c>
+      <c r="D181" s="61" t="inlineStr">
+        <is>
+          <t>Itauguá es conocida como la «ciudad del ñandutí» y cada año celebra el Festival Internacional del Ñandutí, por lo general en julio.</t>
+        </is>
+      </c>
+      <c r="E181" s="61" t="inlineStr">
+        <is>
+          <t>Secretaría Nacional de Turismo (SENATUR)</t>
+        </is>
+      </c>
+      <c r="F181" s="61" t="inlineStr">
+        <is>
+          <t>Pesas justas: la honestidad en cada venta y en cada compra refleja el carácter de Dios.</t>
+        </is>
+      </c>
+      <c r="G181" s="61" t="n"/>
+      <c r="H181" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, comprá algo hecho o vendido en tu zona y agradecele a quien lo produce.</t>
+        </is>
+      </c>
+      <c r="I181" s="61" t="inlineStr">
+        <is>
+          <t>Cada compra en el barrio sostiene a una familia; el comercio local es una relación honesta en ambos lados.</t>
+        </is>
+      </c>
+      <c r="J181" s="61" t="n"/>
+      <c r="K181" s="61" t="n"/>
+      <c r="L181" s="61" t="inlineStr">
+        <is>
+          <t>Adaptarse a nuevas formas de vender sin perder la esencia: amar al cliente de hecho y en verdad.</t>
+        </is>
+      </c>
+      <c r="M181" s="61" t="n"/>
+      <c r="N181" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de julio verificados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -7067,7 +7067,7 @@
       </c>
       <c r="AF31" s="47" t="inlineStr">
         <is>
-          <t>Efesios 4:25 — Por eso cada uno de ustedes debe despreciar la mentira y hablar la verdad con su prójimo; porque somos miembros los unos de los otros.</t>
+          <t>Efesios 4:25 — Por eso cada uno de ustedes debe desechar la mentira y hablar la verdad con su prójimo; porque somos miembros los unos de los otros.</t>
         </is>
       </c>
       <c r="AG31" s="47" t="inlineStr">
@@ -30331,12 +30331,12 @@
       </c>
       <c r="D167" s="61" t="inlineStr">
         <is>
-          <t>Warren Buffett compró sus primeras acciones a los 11 años; cuando bajaron, las vendió apenas recuperó lo invertido, y después subieron mucho. Dijo que aprendió a tener paciencia.</t>
+          <t>Warren Buffett compró sus primeras acciones a los 11 años. Cuando bajaron, se asustó y las vendió con una ganancia mínima, y después subieron muchísimo. Aprendió a no apurarse por una ganancia chica.</t>
         </is>
       </c>
       <c r="E167" s="61" t="inlineStr">
         <is>
-          <t>Alice Schroeder, La bola de nieve (biografía de Warren Buffett), 2008</t>
+          <t>Alice Schroeder, La bola de nieve: Warren Buffett y el negocio de la vida, 2008</t>
         </is>
       </c>
       <c r="F167" s="61" t="inlineStr">
@@ -30526,7 +30526,7 @@
       </c>
       <c r="E170" s="61" t="inlineStr">
         <is>
-          <t>Filipenses 1:13</t>
+          <t>Filipenses 1:13; 3:13-14</t>
         </is>
       </c>
       <c r="F170" s="61" t="inlineStr">
@@ -30661,7 +30661,7 @@
       </c>
       <c r="D172" s="61" t="inlineStr">
         <is>
-          <t>Una revisión de 94 estudios encontró que decidir de antemano cuándo, dónde y cómo se va a dar un paso aumenta mucho la probabilidad de cumplir una meta.</t>
+          <t>Una revisión de 94 pruebas, con más de 8.000 participantes, encontró que decidir de antemano cuándo, dónde y cómo se va a dar un paso aumenta bastante la probabilidad de cumplir una meta.</t>
         </is>
       </c>
       <c r="E172" s="61" t="inlineStr">
@@ -31061,12 +31061,12 @@
       </c>
       <c r="D178" s="61" t="inlineStr">
         <is>
-          <t>Según el Ministerio de Industria y Comercio, las micro, pequeñas y medianas empresas son la gran mayoría de las empresas del Paraguay.</t>
+          <t>Según el Ministerio de Industria y Comercio, cerca del 97 % de las empresas del Paraguay son micro, pequeñas o medianas, y la gran mayoría son microempresas.</t>
         </is>
       </c>
       <c r="E178" s="61" t="inlineStr">
         <is>
-          <t>Ministerio de Industria y Comercio, Viceministerio de MIPYMES</t>
+          <t>Ministerio de Industria y Comercio, Viceministerio de MIPYMES (datos del DIRGE 2019)</t>
         </is>
       </c>
       <c r="F178" s="61" t="inlineStr">
@@ -31131,7 +31131,7 @@
       </c>
       <c r="D179" s="61" t="inlineStr">
         <is>
-          <t>Un estudio en un barrio de Chicago encontró que, de cada 100 dólares gastados en comercios locales, unos 68 seguían circulando en la economía de la zona, frente a 43 en las cadenas.</t>
+          <t>Un estudio en un barrio de Chicago encontró que, de cada 100 dólares gastados en comercios locales, unos 68 seguían circulando en la economía de la ciudad, frente a 43 en las cadenas.</t>
         </is>
       </c>
       <c r="E179" s="61" t="inlineStr">
@@ -31271,12 +31271,12 @@
       </c>
       <c r="D181" s="61" t="inlineStr">
         <is>
-          <t>Itauguá es conocida como la «ciudad del ñandutí» y cada año celebra el Festival Internacional del Ñandutí, por lo general en julio.</t>
+          <t>Itauguá es conocida como la «ciudad del ñandutí», y allí se realiza desde 1970 el Festival Nacional del Ñandutí; la primera edición fue en julio.</t>
         </is>
       </c>
       <c r="E181" s="61" t="inlineStr">
         <is>
-          <t>Secretaría Nacional de Turismo (SENATUR)</t>
+          <t>Agencia de Información Paraguaya (IP), Festival Nacional del Ñandutí</t>
         </is>
       </c>
       <c r="F181" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: semana 28 sin advertencias de estafas; consejo profesional
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -6548,7 +6548,7 @@
       </c>
       <c r="M29" s="40" t="inlineStr">
         <is>
-          <t>Recordar que el mensaje es educativo, no una recomendación de producto financiero específico.</t>
+          <t>Recordar que el mensaje es educativo, no una recomendación de producto financiero específico. Tema sensible: no opinar al aire sobre empresas, productos o propuestas de inversión concretas, ni sobre si son confiables. Si la audiencia pregunta o se quiere profundizar, conviene invitar a un profesional (contador o asesor financiero) para hablar del tema.</t>
         </is>
       </c>
       <c r="N29" s="40" t="inlineStr">
@@ -30221,12 +30221,12 @@
       </c>
       <c r="J165" s="61" t="inlineStr">
         <is>
-          <t>Poner todos los ahorros en un solo negocio o en una promesa de ganancia rápida.</t>
+          <t>Poner todos los ahorros en un solo lugar.</t>
         </is>
       </c>
       <c r="K165" s="61" t="inlineStr">
         <is>
-          <t>Antes de invertir, pedí consejo a alguien que sepa y que no tenga interés en venderte nada.</t>
+          <t>Antes de invertir, pedí consejo a un profesional de confianza, como un contador o un asesor financiero.</t>
         </is>
       </c>
       <c r="L165" s="61" t="inlineStr">
@@ -30236,12 +30236,12 @@
       </c>
       <c r="M165" s="61" t="inlineStr">
         <is>
-          <t>Contar con ganancias seguras y desesperarse cuando no llegan.</t>
+          <t>Esperar resultados inmediatos y desanimarse cuando tardan.</t>
         </is>
       </c>
       <c r="N165" s="61" t="inlineStr">
         <is>
-          <t>Calculá cuánto podrías perder sin poner en riesgo la comida, el alquiler o las deudas de tu casa, y no arriesgues más que eso.</t>
+          <t>Antes de pensar en invertir, asegurate de tener cubiertos la comida, el alquiler y las deudas de tu casa.</t>
         </is>
       </c>
     </row>
@@ -30301,17 +30301,17 @@
       </c>
       <c r="L166" s="61" t="inlineStr">
         <is>
-          <t>El necio desprecia la enseñanza. En finanzas, desconfiá de quien promete ganancias altas, rápidas y sin riesgo.</t>
+          <t>El necio desprecia la enseñanza; el sabio escucha consejo. En temas de dinero nadie sabe todo, y pedir ayuda a quien sabe también es sabiduría.</t>
         </is>
       </c>
       <c r="M166" s="61" t="inlineStr">
         <is>
-          <t>Caer en esquemas piramidales o en «inversiones» que piden traer a otros para ganar.</t>
+          <t>Decidir solo, por orgullo o por apuro, sin consultar a nadie.</t>
         </is>
       </c>
       <c r="N166" s="61" t="inlineStr">
         <is>
-          <t>Si alguien te ofrece duplicar tu plata rápido, pedí consejo antes de poner un solo guaraní.</t>
+          <t>Si estás pensando en invertir, conversalo primero con un profesional de confianza.</t>
         </is>
       </c>
     </row>
@@ -30361,7 +30361,7 @@
       </c>
       <c r="J167" s="61" t="inlineStr">
         <is>
-          <t>Arriesgar de golpe todo lo ahorrado para recuperar una pérdida.</t>
+          <t>Apurarse a recuperar lo perdido sin pensar bien el siguiente paso.</t>
         </is>
       </c>
       <c r="K167" s="61" t="inlineStr">
@@ -30487,7 +30487,7 @@
       <c r="G169" s="61" t="n"/>
       <c r="H169" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, siéntense en familia, definan una meta de ahorro con un propósito y pidan consejo antes de cualquier inversión.</t>
+          <t>Esta semana, siéntense en familia, definan una meta de ahorro con un propósito y, antes de cualquier inversión, pidan consejo a un profesional.</t>
         </is>
       </c>
       <c r="I169" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: semanas 2 y 7 sin advertencias de estafas; consejo profesional
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -19736,12 +19736,12 @@
       </c>
       <c r="G8" s="61" t="inlineStr">
         <is>
-          <t>Las promesas de ganancia fácil (préstamos rápidos, cadenas, esquemas de inversión) que llegan incluso a los grupos de la iglesia.</t>
+          <t>Querer resultados sin esfuerzo y decidir sobre la plata sin pensar en el mañana.</t>
         </is>
       </c>
       <c r="H8" s="61" t="inlineStr">
         <is>
-          <t>Antes de entrar en cualquier negocio, consultalo con alguien de confianza y desconfiá de lo que promete mucho sin trabajo. Anotá esta semana tres semillas concretas que sí quieras sembrar.</t>
+          <t>Antes de una decisión importante con tu plata, consultala con un profesional de confianza. Y anotá esta semana tres semillas concretas que sí quieras sembrar.</t>
         </is>
       </c>
       <c r="I8" s="61" t="inlineStr">
@@ -21886,17 +21886,17 @@
       </c>
       <c r="I40" s="61" t="inlineStr">
         <is>
-          <t>Lo que llega fácil, se va fácil. Las promesas de ganancia rápida casi siempre terminan en pérdida.</t>
+          <t>Lo que llega fácil, se va fácil. Lo que se construye con trabajo y paciencia suele durar.</t>
         </is>
       </c>
       <c r="J40" s="61" t="inlineStr">
         <is>
-          <t>Cadenas y esquemas que prometen multiplicar el dinero en poco tiempo y dejan a muchos sin nada.</t>
+          <t>Buscar atajos para hacer crecer el dinero en poco tiempo.</t>
         </is>
       </c>
       <c r="K40" s="61" t="inlineStr">
         <is>
-          <t>Antes de poner tu plata en algo que promete mucho en poco tiempo, consultalo con alguien de confianza que sepa del tema.</t>
+          <t>Si pensás en hacer crecer tus ahorros, conversalo primero con un profesional de confianza, como un contador.</t>
         </is>
       </c>
       <c r="L40" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: guiones de agosto con revisión teológica
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -7240,7 +7240,7 @@
       </c>
       <c r="AA32" s="49" t="inlineStr">
         <is>
-          <t>• El día de reposo es mandato, no sugerencia
+          <t>• Dios estableció un ritmo de trabajo y descanso
 • Detenerse regularmente es obediencia
 • El descanso tiene valor espiritual, no solo físico</t>
         </is>
@@ -7255,7 +7255,7 @@
         <is>
           <t>• Dormir en paz es posible con confianza en Dios
 • La seguridad interior permite el descanso
-• El sueño tranquilo refleja fe, no solo cansancio</t>
+• Dios nos cuida también en las noches difíciles</t>
         </is>
       </c>
       <c r="AD32" s="49" t="inlineStr">
@@ -7265,7 +7265,7 @@
       </c>
       <c r="AE32" s="49" t="inlineStr">
         <is>
-          <t>• Jesús invito a Sus discípulos a descansar aparte
+          <t>• Jesús invitó a sus discípulos a descansar aparte
 • El descanso es necesario incluso en medio del ministerio
 • Detenerse no es debilidad, es sabiduría</t>
         </is>
@@ -7292,9 +7292,9 @@
       </c>
       <c r="AI32" s="49" t="inlineStr">
         <is>
-          <t>• Jesús invita a los cansados a descansar en El
+          <t>• Jesús invita a los cansados a descansar en Él
 • El descanso verdadero tiene origen espiritual
-• Venir a El alivia la carga</t>
+• Venir a Él alivia la carga</t>
         </is>
       </c>
       <c r="AJ32" s="49" t="inlineStr">
@@ -7498,8 +7498,8 @@
       <c r="AI33" s="8" t="inlineStr">
         <is>
           <t>• Pedir con fe, no con duda
-• Creer antes de ver la respuesta
-• La fe activa la oración</t>
+• Confiar en que Dios responde según su voluntad
+• La fe está puesta en Dios (11:22)</t>
         </is>
       </c>
       <c r="AJ33" s="8" t="inlineStr">
@@ -7640,12 +7640,12 @@
         <is>
           <t>• Dios es nuestra roca: En Él encontramos seguridad y firmeza.
 • Dios es nuestro redentor: Él nos rescata y transforma.
-• Cuidemos pensamientos y palabras:</t>
+• Cuidemos pensamientos y palabras: Que agraden a Dios. Que agraden a Dios.</t>
         </is>
       </c>
       <c r="Z34" s="10" t="inlineStr">
         <is>
-          <t>Hechos 20:28 — Yo les ruego que piensen en ustedes mismos, y que cuiden el rebaño sobre el cual el Espíritu Santo los ha puesto como obispos, para que cuiden de la iglesia del Señor, que él ganó por su propia sangre.28</t>
+          <t>Hechos 20:28 — Yo les ruego que piensen en ustedes mismos, y que cuiden el rebaño sobre el cual el Espíritu Santo los ha puesto como obispos, para que cuiden de la iglesia del Señor, que él ganó por su propia sangre.</t>
         </is>
       </c>
       <c r="AA34" s="10" t="inlineStr">
@@ -7711,9 +7711,9 @@
       </c>
       <c r="AK34" s="10" t="inlineStr">
         <is>
-          <t>• • El testimonio visible por medio de la acción
-• • La fuente de la luz es Dios, no el ser humano
-• • El propósito final es la gloria del Padre</t>
+          <t>• El testimonio visible por medio de la acción
+• La fuente de la luz es Dios, no el ser humano
+• El propósito final es la gloria del Padre</t>
         </is>
       </c>
     </row>
@@ -7864,9 +7864,9 @@
       </c>
       <c r="AC35" s="12" t="inlineStr">
         <is>
-          <t>• Habrá un día de juicio.
-• Dios hará justicia.
-• Vivir preparados delante de Dios.</t>
+          <t>• Ser comprensivos: Conocer de verdad a la esposa.
+• Honrar: Coherederos del don de la vida.
+• Cuidar la relación: Afecta también la oración.</t>
         </is>
       </c>
       <c r="AD35" s="12" t="inlineStr">
@@ -7889,9 +7889,9 @@
       </c>
       <c r="AG35" s="12" t="inlineStr">
         <is>
-          <t>• El momento oportuno: Decir lo correcto en el instante preciso tiene un valor extraordinario;
+          <t>• El momento oportuno: Decir lo correcto en el instante preciso tiene un valor extraordinario.
 • Sabiduría al hablar: Implica tacto, prudencia y discernimiento para saber cuándo es el momento de aconsejar, animar o corregir.
-• Impacto positivo: Las palabras bien expresadas edifican al oyente y traen paz o consuelo, de forma similar a como se describe en la Sociedad Bíblica a través de Bible Gateway.</t>
+• Impacto positivo: Las palabras bien expresadas edifican al oyente y traen paz o consuelo.</t>
         </is>
       </c>
       <c r="AH35" s="12" t="inlineStr">
@@ -7902,7 +7902,7 @@
       <c r="AI35" s="12" t="inlineStr">
         <is>
           <t>• Ser benignos y misericordiosos
-• Perdonar como Cristo perdono
+• Perdonar como Cristo perdonó
 • La bondad sostiene la comunicación familiar</t>
         </is>
       </c>
@@ -19214,7 +19214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N181"/>
+  <dimension ref="A1:N205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -31304,6 +31304,1606 @@
       </c>
       <c r="M181" s="61" t="n"/>
       <c r="N181" s="61" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="61" t="n">
+        <v>31</v>
+      </c>
+      <c r="B182" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C182" s="61" t="inlineStr">
+        <is>
+          <t>Un ritmo de trabajo y descanso</t>
+        </is>
+      </c>
+      <c r="D182" s="61" t="inlineStr">
+        <is>
+          <t>Los especialistas en sueño recomiendan que los adultos duerman 7 horas o más por noche de forma regular.</t>
+        </is>
+      </c>
+      <c r="E182" s="61" t="inlineStr">
+        <is>
+          <t>Watson y otros, consenso de la American Academy of Sleep Medicine y la Sleep Research Society, 2015</t>
+        </is>
+      </c>
+      <c r="F182" s="61" t="inlineStr">
+        <is>
+          <t>Dios no nos hizo para trabajar sin parar. Desde la creación, el trabajo y el descanso van juntos, y Jesús dijo que el día de reposo fue hecho para el ser humano (Marcos 2:27). Las iglesias viven este mandamiento de formas distintas, pero todas reconocen el principio: detenerse.</t>
+        </is>
+      </c>
+      <c r="G182" s="61" t="inlineStr">
+        <is>
+          <t>Sentir culpa por descansar, como si fuera pereza.</t>
+        </is>
+      </c>
+      <c r="H182" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, elegí un tiempo fijo para detenerte de verdad, sin trabajo pendiente.</t>
+        </is>
+      </c>
+      <c r="I182" s="61" t="inlineStr">
+        <is>
+          <t>El mandamiento incluía a los hijos, a los empleados, a los extranjeros y hasta a los animales. El descanso no era privilegio de unos pocos.</t>
+        </is>
+      </c>
+      <c r="J182" s="61" t="inlineStr">
+        <is>
+          <t>Descansar uno y dejar que otros carguen con todo el trabajo de la casa.</t>
+        </is>
+      </c>
+      <c r="K182" s="61" t="inlineStr">
+        <is>
+          <t>Organicen en familia las tareas para que todos, también mamá, tengan su tiempo de descanso.</t>
+        </is>
+      </c>
+      <c r="L182" s="61" t="inlineStr">
+        <is>
+          <t>El sueño es parte de ese descanso: mientras dormimos, el cuerpo se repara y el cerebro ordena la memoria. Dormir bien es cuidar el cuerpo que Dios nos dio.</t>
+        </is>
+      </c>
+      <c r="M182" s="61" t="inlineStr">
+        <is>
+          <t>Ver el sueño como tiempo perdido y quitarle horas para hacer más.</t>
+        </is>
+      </c>
+      <c r="N182" s="61" t="inlineStr">
+        <is>
+          <t>Fijate cuántas horas dormiste anoche y, si fueron pocas, adelantá hoy la hora de acostarte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="61" t="n">
+        <v>31</v>
+      </c>
+      <c r="B183" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C183" s="61" t="inlineStr">
+        <is>
+          <t>Dormir en paz</t>
+        </is>
+      </c>
+      <c r="D183" s="61" t="inlineStr">
+        <is>
+          <t>Durante el sueño, el cerebro elimina con más eficacia sustancias de desecho; así lo mostró un estudio en ratones publicado en 2013.</t>
+        </is>
+      </c>
+      <c r="E183" s="61" t="inlineStr">
+        <is>
+          <t>Xie y otros, Science, 2013</t>
+        </is>
+      </c>
+      <c r="F183" s="61" t="inlineStr">
+        <is>
+          <t>David escribe este salmo en medio de problemas y críticas (4:1-2), y aun así puede acostarse en paz, porque su seguridad está en Dios.</t>
+        </is>
+      </c>
+      <c r="G183" s="61" t="inlineStr">
+        <is>
+          <t>Llevarse a la cama todas las preocupaciones del día.</t>
+        </is>
+      </c>
+      <c r="H183" s="61" t="inlineStr">
+        <is>
+          <t>Antes de dormir, entregale a Dios en oración lo que te preocupa, por nombre.</t>
+        </is>
+      </c>
+      <c r="I183" s="61" t="inlineStr">
+        <is>
+          <t>La paz interior ayuda a descansar. Cerrar el día con orden, sin discusiones pendientes y con la conciencia tranquila, prepara el sueño.</t>
+        </is>
+      </c>
+      <c r="J183" s="61" t="inlineStr">
+        <is>
+          <t>Acostarse enojado o con una conversación pendiente.</t>
+        </is>
+      </c>
+      <c r="K183" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés algo pendiente con alguien de tu casa, intentá conversarlo antes de dormir.</t>
+        </is>
+      </c>
+      <c r="L183" s="61" t="inlineStr">
+        <is>
+          <t>Dormir mal no es falta de fe. El insomnio puede tener causas físicas o emocionales, y Dios nos acompaña también en esas noches.</t>
+        </is>
+      </c>
+      <c r="M183" s="61" t="inlineStr">
+        <is>
+          <t>Sentirse culpable o «poco espiritual» por no poder dormir.</t>
+        </is>
+      </c>
+      <c r="N183" s="61" t="inlineStr">
+        <is>
+          <t>Si hace semanas que dormís mal, consultá a un médico: pedir ayuda también es cuidar el cuerpo que Dios te dio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="61" t="n">
+        <v>31</v>
+      </c>
+      <c r="B184" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C184" s="61" t="inlineStr">
+        <is>
+          <t>Descansen un poco</t>
+        </is>
+      </c>
+      <c r="D184" s="61" t="inlineStr">
+        <is>
+          <t>Según los Centros para el Control y la Prevención de Enfermedades de Estados Unidos, cerca de uno de cada tres adultos no duerme lo suficiente de forma habitual.</t>
+        </is>
+      </c>
+      <c r="E184" s="61" t="inlineStr">
+        <is>
+          <t>Centros para el Control y la Prevención de Enfermedades (CDC), 2016</t>
+        </is>
+      </c>
+      <c r="F184" s="61" t="inlineStr">
+        <is>
+          <t>Los discípulos volvían de un viaje de servicio, entusiasmados, y Jesús les dice: vengan a descansar. Él cuida a los que trabajan.</t>
+        </is>
+      </c>
+      <c r="G184" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que mientras más ocupados, mejor estamos.</t>
+        </is>
+      </c>
+      <c r="H184" s="61" t="inlineStr">
+        <is>
+          <t>Revisá tu agenda de esta semana y anotá un tiempo de descanso como si fuera una cita.</t>
+        </is>
+      </c>
+      <c r="I184" s="61" t="inlineStr">
+        <is>
+          <t>No tenían tiempo ni para comer. La falta de descanso no siempre se nota enseguida: se acumula en cansancio, irritabilidad y malas decisiones.</t>
+        </is>
+      </c>
+      <c r="J184" s="61" t="inlineStr">
+        <is>
+          <t>Echarle la culpa del mal humor a todo, menos al cansancio.</t>
+        </is>
+      </c>
+      <c r="K184" s="61" t="inlineStr">
+        <is>
+          <t>Si estos días andás irritable, preguntate: ¿estoy durmiendo lo suficiente?</t>
+        </is>
+      </c>
+      <c r="L184" s="61" t="inlineStr">
+        <is>
+          <t>Jesús no les pidió que trabajaran más, sino que se apartaran un poco. Hasta en el servicio a Dios hace falta parar.</t>
+        </is>
+      </c>
+      <c r="M184" s="61" t="inlineStr">
+        <is>
+          <t>Servidores de la iglesia que nunca descansan y terminan agotados.</t>
+        </is>
+      </c>
+      <c r="N184" s="61" t="inlineStr">
+        <is>
+          <t>Si servís en tu iglesia, conversá con tu líder para organizar turnos y descansos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="61" t="n">
+        <v>31</v>
+      </c>
+      <c r="B185" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C185" s="61" t="inlineStr">
+        <is>
+          <t>El sueño es un regalo</t>
+        </is>
+      </c>
+      <c r="D185" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 127 se atribuye a Salomón, el rey que construyó el templo de Jerusalén.</t>
+        </is>
+      </c>
+      <c r="E185" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 127 (título); 1 Reyes 6</t>
+        </is>
+      </c>
+      <c r="F185" s="61" t="inlineStr">
+        <is>
+          <t>El salmo dice que el Señor da el sueño a los que él ama. Descansar no es robarle tiempo a la vida: es recibir un regalo.</t>
+        </is>
+      </c>
+      <c r="G185" s="61" t="inlineStr">
+        <is>
+          <t>Vivir el descanso con culpa.</t>
+        </is>
+      </c>
+      <c r="H185" s="61" t="inlineStr">
+        <is>
+          <t>Esta noche, antes de dormir, agradecele a Dios por el descanso.</t>
+        </is>
+      </c>
+      <c r="I185" s="61" t="inlineStr">
+        <is>
+          <t>Madrugar y acostarse tarde con ansiedad no asegura nada si Dios no está en la obra (127:1). El trabajo es bueno; el afán que no deja descansar, no.</t>
+        </is>
+      </c>
+      <c r="J185" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar hasta tarde todos los días creyendo que todo depende de uno.</t>
+        </is>
+      </c>
+      <c r="K185" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una hora para terminar de trabajar y respetala al menos tres días esta semana.</t>
+        </is>
+      </c>
+      <c r="L185" s="61" t="inlineStr">
+        <is>
+          <t>La falta de sueño acumulada afecta el ánimo, la concentración y la salud. Confiar en Dios incluye cuidar las horas de sueño.</t>
+        </is>
+      </c>
+      <c r="M185" s="61" t="inlineStr">
+        <is>
+          <t>Acostumbrarse a dormir poco y pensar que el cuerpo ya se adaptó.</t>
+        </is>
+      </c>
+      <c r="N185" s="61" t="inlineStr">
+        <is>
+          <t>Anotá cuántas horas dormís cada noche esta semana; los adultos necesitan unas siete o más.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="61" t="n">
+        <v>31</v>
+      </c>
+      <c r="B186" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C186" s="61" t="inlineStr">
+        <is>
+          <t>Vengan a mí</t>
+        </is>
+      </c>
+      <c r="D186" s="61" t="inlineStr">
+        <is>
+          <t>Entre los hábitos que recomiendan los especialistas están acostarse y levantarse a la misma hora, y tener el dormitorio oscuro, silencioso y fresco.</t>
+        </is>
+      </c>
+      <c r="E186" s="61" t="inlineStr">
+        <is>
+          <t>American Academy of Sleep Medicine, recomendaciones para dormir mejor</t>
+        </is>
+      </c>
+      <c r="F186" s="61" t="inlineStr">
+        <is>
+          <t>Jesús invita a los agotados, no a los que ya tienen todo resuelto. El descanso empieza por ir a él.</t>
+        </is>
+      </c>
+      <c r="G186" s="61" t="inlineStr">
+        <is>
+          <t>Buscar descanso solo en distracciones que en realidad no descansan.</t>
+        </is>
+      </c>
+      <c r="H186" s="61" t="inlineStr">
+        <is>
+          <t>Cerrá el día con unos minutos de oración en lugar de revisar el celular.</t>
+        </is>
+      </c>
+      <c r="I186" s="61" t="inlineStr">
+        <is>
+          <t>El descanso del alma viene de Jesús, y el del cuerpo también se cuida con hábitos simples: una hora fija para acostarse, un cuarto oscuro y la cena no muy tarde.</t>
+        </is>
+      </c>
+      <c r="J186" s="61" t="inlineStr">
+        <is>
+          <t>Acostarse cada día a una hora distinta.</t>
+        </is>
+      </c>
+      <c r="K186" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una hora fija para acostarte esta semana, también el fin de semana.</t>
+        </is>
+      </c>
+      <c r="L186" s="61" t="inlineStr">
+        <is>
+          <t>Jesús ofrece cambiar nuestra carga por su yugo, que es suave y liviano (11:29-30). A veces lo que no nos deja dormir es el celular en la mano.</t>
+        </is>
+      </c>
+      <c r="M186" s="61" t="inlineStr">
+        <is>
+          <t>Mirar el celular en la cama hasta quedarse dormido.</t>
+        </is>
+      </c>
+      <c r="N186" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, apagá las pantallas 30 minutos antes de dormir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="61" t="n">
+        <v>31</v>
+      </c>
+      <c r="B187" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C187" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: descansar también es cuidarse</t>
+        </is>
+      </c>
+      <c r="D187" s="61" t="inlineStr">
+        <is>
+          <t>En Génesis, Dios descansa el séptimo día de la creación, mucho antes de que existiera el mandamiento del día de reposo.</t>
+        </is>
+      </c>
+      <c r="E187" s="61" t="inlineStr">
+        <is>
+          <t>Génesis 2:2-3; Éxodo 20:11</t>
+        </is>
+      </c>
+      <c r="F187" s="61" t="inlineStr">
+        <is>
+          <t>Dormir bien es parte de cuidar el cuerpo que Dios nos dio, y el descanso es un regalo, no una culpa.</t>
+        </is>
+      </c>
+      <c r="G187" s="61" t="n"/>
+      <c r="H187" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, elegí un hábito de descanso y sostenelo siete días, y cada noche entregale a Dios tus preocupaciones.</t>
+        </is>
+      </c>
+      <c r="I187" s="61" t="inlineStr">
+        <is>
+          <t>La falta de descanso se acumula en silencio: cansancio, irritabilidad y malas decisiones.</t>
+        </is>
+      </c>
+      <c r="J187" s="61" t="n"/>
+      <c r="K187" s="61" t="n"/>
+      <c r="L187" s="61" t="inlineStr">
+        <is>
+          <t>Hábitos simples ayudan: una hora fija para dormir y las pantallas apagadas antes de acostarse.</t>
+        </is>
+      </c>
+      <c r="M187" s="61" t="n"/>
+      <c r="N187" s="61" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="61" t="n">
+        <v>32</v>
+      </c>
+      <c r="B188" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C188" s="61" t="inlineStr">
+        <is>
+          <t>Clamá a mí</t>
+        </is>
+      </c>
+      <c r="D188" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías recibió esta palabra estando preso en el patio de la guardia, mientras Jerusalén estaba sitiada.</t>
+        </is>
+      </c>
+      <c r="E188" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías 32:1-2; 33:1</t>
+        </is>
+      </c>
+      <c r="F188" s="61" t="inlineStr">
+        <is>
+          <t>Dios le habla a Jeremías, preso y con la ciudad sitiada. Orar no es un trámite: es clamar a alguien que escucha, también en el momento más difícil.</t>
+        </is>
+      </c>
+      <c r="G188" s="61" t="inlineStr">
+        <is>
+          <t>Orar con frases repetidas, sin pensar en lo que decimos.</t>
+        </is>
+      </c>
+      <c r="H188" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, hablale a Dios con tus propias palabras, como le hablarías a alguien que te escucha.</t>
+        </is>
+      </c>
+      <c r="I188" s="61" t="inlineStr">
+        <is>
+          <t>La promesa fue para Jeremías y su pueblo: Dios anunciaba que restauraría Jerusalén. De ahí aprendemos quién es Dios: alguien que escucha y responde, a su manera y a su tiempo.</t>
+        </is>
+      </c>
+      <c r="J188" s="61" t="inlineStr">
+        <is>
+          <t>Tratar a Dios como una ventanilla de pedidos.</t>
+        </is>
+      </c>
+      <c r="K188" s="61" t="inlineStr">
+        <is>
+          <t>En tu oración de hoy, antes de pedir, contale a Dios cómo estás.</t>
+        </is>
+      </c>
+      <c r="L188" s="61" t="inlineStr">
+        <is>
+          <t>Las «cosas grandes» que Dios anunció eran su plan de restauración, no lo que Jeremías imaginaba. En la oración, Dios a veces nos muestra lo que no conocíamos.</t>
+        </is>
+      </c>
+      <c r="M188" s="61" t="inlineStr">
+        <is>
+          <t>Ir a la oración solo para que Dios confirme lo que ya decidimos.</t>
+        </is>
+      </c>
+      <c r="N188" s="61" t="inlineStr">
+        <is>
+          <t>Dejá unos minutos de silencio en tu oración, para escuchar además de hablar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="61" t="n">
+        <v>32</v>
+      </c>
+      <c r="B189" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C189" s="61" t="inlineStr">
+        <is>
+          <t>En lo secreto</t>
+        </is>
+      </c>
+      <c r="D189" s="61" t="inlineStr">
+        <is>
+          <t>La palabra griega que Jesús usa para «habitación» designaba el cuarto interior o la despensa de la casa, a veces el único lugar con puerta.</t>
+        </is>
+      </c>
+      <c r="E189" s="61" t="inlineStr">
+        <is>
+          <t>Mateo 6:6; léxico griego de Strong (G5009, tameíon)</t>
+        </is>
+      </c>
+      <c r="F189" s="61" t="inlineStr">
+        <is>
+          <t>Jesús no está en contra de orar en público, sino de orar para ser visto (6:5).</t>
+        </is>
+      </c>
+      <c r="G189" s="61" t="inlineStr">
+        <is>
+          <t>Orar en público con palabras lindas y no orar nunca a solas.</t>
+        </is>
+      </c>
+      <c r="H189" s="61" t="inlineStr">
+        <is>
+          <t>Buscá hoy un momento a solas para orar, aunque sea breve.</t>
+        </is>
+      </c>
+      <c r="I189" s="61" t="inlineStr">
+        <is>
+          <t>Una relación se cuida a solas, como dos amigos que conversan sin público. Ahí la oración deja de ser rutina y se vuelve encuentro.</t>
+        </is>
+      </c>
+      <c r="J189" s="61" t="inlineStr">
+        <is>
+          <t>Orar solo cuando hay alguien mirando o cuando toca en la reunión.</t>
+        </is>
+      </c>
+      <c r="K189" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un lugar fijo de tu casa para orar esta semana.</t>
+        </is>
+      </c>
+      <c r="L189" s="61" t="inlineStr">
+        <is>
+          <t>El Padre ve en lo secreto. La recompensa es él mismo y su cuidado, no el aplauso de la gente.</t>
+        </is>
+      </c>
+      <c r="M189" s="61" t="inlineStr">
+        <is>
+          <t>Buscar reconocimiento por lo espiritual que hacemos.</t>
+        </is>
+      </c>
+      <c r="N189" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, orá por alguien sin contárselo a nadie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="61" t="n">
+        <v>32</v>
+      </c>
+      <c r="B190" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C190" s="61" t="inlineStr">
+        <is>
+          <t>Según su voluntad</t>
+        </is>
+      </c>
+      <c r="D190" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pidió tres veces que Dios le quitara un sufrimiento, y Dios le respondió que su gracia le bastaba.</t>
+        </is>
+      </c>
+      <c r="E190" s="61" t="inlineStr">
+        <is>
+          <t>2 Corintios 12:7-9</t>
+        </is>
+      </c>
+      <c r="F190" s="61" t="inlineStr">
+        <is>
+          <t>Cuando parece que Dios no responde, la carta de Juan recuerda algo firme: él nos oye.</t>
+        </is>
+      </c>
+      <c r="G190" s="61" t="inlineStr">
+        <is>
+          <t>Concluir que Dios no escucha porque no vemos la respuesta.</t>
+        </is>
+      </c>
+      <c r="H190" s="61" t="inlineStr">
+        <is>
+          <t>Si sentís que Dios no te responde, decíselo con sinceridad: él puede recibir tu frustración.</t>
+        </is>
+      </c>
+      <c r="I190" s="61" t="inlineStr">
+        <is>
+          <t>A veces la respuesta es «no» o «todavía no». Pablo pidió tres veces que le quitara un sufrimiento, y Dios le dio su gracia en lugar de quitárselo.</t>
+        </is>
+      </c>
+      <c r="J190" s="61" t="inlineStr">
+        <is>
+          <t>Creer que si algo no se dio, Dios nos falló.</t>
+        </is>
+      </c>
+      <c r="K190" s="61" t="inlineStr">
+        <is>
+          <t>Agregá a tu oración «que se haga tu voluntad», como oró Jesús.</t>
+        </is>
+      </c>
+      <c r="L190" s="61" t="inlineStr">
+        <is>
+          <t>Muchos en la Biblia oraron por un tiempo sin respuesta visible, como Ana o varios salmistas, y siguieron orando.</t>
+        </is>
+      </c>
+      <c r="M190" s="61" t="inlineStr">
+        <is>
+          <t>Dejar de orar por desánimo.</t>
+        </is>
+      </c>
+      <c r="N190" s="61" t="inlineStr">
+        <is>
+          <t>Anotá un pedido por el que estás orando, con la fecha, y volvé a mirarlo dentro de unos meses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="61" t="n">
+        <v>32</v>
+      </c>
+      <c r="B191" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C191" s="61" t="inlineStr">
+        <is>
+          <t>Vaciá tu corazón</t>
+        </is>
+      </c>
+      <c r="D191" s="61" t="inlineStr">
+        <is>
+          <t>Cerca de un tercio de los salmos son lamentos: oraciones de queja, de dolor o de pregunta a Dios.</t>
+        </is>
+      </c>
+      <c r="E191" s="61" t="inlineStr">
+        <is>
+          <t>Clasificación de los Salmos por géneros (Hermann Gunkel y estudios posteriores)</t>
+        </is>
+      </c>
+      <c r="F191" s="61" t="inlineStr">
+        <is>
+          <t>El salmista dice «confíen siempre», también cuando parece que Dios calla. La confianza no depende de tener todas las respuestas.</t>
+        </is>
+      </c>
+      <c r="G191" s="61" t="inlineStr">
+        <is>
+          <t>Confiar en Dios solo cuando las cosas salen bien.</t>
+        </is>
+      </c>
+      <c r="H191" s="61" t="inlineStr">
+        <is>
+          <t>Nombrá una situación en la que hoy te cuesta confiar, y entregásela a Dios.</t>
+        </is>
+      </c>
+      <c r="I191" s="61" t="inlineStr">
+        <is>
+          <t>La Biblia está llena de oraciones sinceras: quejas, preguntas, lágrimas. Dios no pide frases correctas, sino un corazón abierto.</t>
+        </is>
+      </c>
+      <c r="J191" s="61" t="inlineStr">
+        <is>
+          <t>Esconderle a Dios lo que sentimos porque creemos que no corresponde.</t>
+        </is>
+      </c>
+      <c r="K191" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, contale a Dios lo que sentís de verdad, sin adornarlo.</t>
+        </is>
+      </c>
+      <c r="L191" s="61" t="inlineStr">
+        <is>
+          <t>Cuando la respuesta tarda, Dios sigue siendo refugio. A veces lo primero que recibimos no es la solución, sino su compañía.</t>
+        </is>
+      </c>
+      <c r="M191" s="61" t="inlineStr">
+        <is>
+          <t>Quedarse solo con la frustración, sin hablarla con nadie.</t>
+        </is>
+      </c>
+      <c r="N191" s="61" t="inlineStr">
+        <is>
+          <t>Si estás pasando una temporada difícil, buscá a alguien de tu iglesia para orar juntos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="61" t="n">
+        <v>32</v>
+      </c>
+      <c r="B192" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C192" s="61" t="inlineStr">
+        <is>
+          <t>Orar con fe</t>
+        </is>
+      </c>
+      <c r="D192" s="61" t="inlineStr">
+        <is>
+          <t>Jesús dijo estas palabras en Jerusalén, en su última semana; pocos días después, en Getsemaní, pidió que se hiciera la voluntad del Padre y no la suya.</t>
+        </is>
+      </c>
+      <c r="E192" s="61" t="inlineStr">
+        <is>
+          <t>Marcos 11:11-24; 14:36</t>
+        </is>
+      </c>
+      <c r="F192" s="61" t="inlineStr">
+        <is>
+          <t>Jesús invita a orar con confianza, no con dudas. Pero dos versículos antes aclara que la fe es en Dios (11:22): mira a Dios, no a la fuerza de nuestro deseo.</t>
+        </is>
+      </c>
+      <c r="G192" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que si algo no se dio, fue porque no creímos lo suficiente.</t>
+        </is>
+      </c>
+      <c r="H192" s="61" t="inlineStr">
+        <is>
+          <t>Orá hoy con confianza, aunque no tengas ganas: la fe no depende del ánimo.</t>
+        </is>
+      </c>
+      <c r="I192" s="61" t="inlineStr">
+        <is>
+          <t>Jesús mismo, pocos días después, pidió que se hiciera la voluntad del Padre. Este versículo no es una fórmula: se lee junto con «si pedimos algo según su voluntad, él nos oye» (1 Juan 5:14).</t>
+        </is>
+      </c>
+      <c r="J192" s="61" t="inlineStr">
+        <is>
+          <t>Usar la oración para exigirle a Dios lo que queremos.</t>
+        </is>
+      </c>
+      <c r="K192" s="61" t="inlineStr">
+        <is>
+          <t>Cuando ores esta semana, terminá diciendo: «que se haga tu voluntad».</t>
+        </is>
+      </c>
+      <c r="L192" s="61" t="inlineStr">
+        <is>
+          <t>Los sentimientos cambian, pero la constancia sostiene la relación. Orar sin ganas, con sinceridad aunque sea breve, también es fe.</t>
+        </is>
+      </c>
+      <c r="M192" s="61" t="inlineStr">
+        <is>
+          <t>Orar solo cuando hay ganas o cuando hay una urgencia.</t>
+        </is>
+      </c>
+      <c r="N192" s="61" t="inlineStr">
+        <is>
+          <t>Comprometete esta semana a orar cinco minutos por día, sin importar el ánimo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="61" t="n">
+        <v>32</v>
+      </c>
+      <c r="B193" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C193" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: orar siempre</t>
+        </is>
+      </c>
+      <c r="D193" s="61" t="inlineStr">
+        <is>
+          <t>Después de este versículo, Jesús cuenta la parábola de una viuda que insistió ante un juez injusto; si ese juez le hizo justicia, cuánto más Dios a sus hijos.</t>
+        </is>
+      </c>
+      <c r="E193" s="61" t="inlineStr">
+        <is>
+          <t>Lucas 18:2-8</t>
+        </is>
+      </c>
+      <c r="F193" s="61" t="inlineStr">
+        <is>
+          <t>Orar no es un trámite: es hablar con alguien que escucha, también a solas y con nuestras propias palabras.</t>
+        </is>
+      </c>
+      <c r="G193" s="61" t="n"/>
+      <c r="H193" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, orá cinco minutos por día en un lugar fijo, y al final de la semana anotá cómo te fue.</t>
+        </is>
+      </c>
+      <c r="I193" s="61" t="inlineStr">
+        <is>
+          <t>Cuando parece que Dios no responde, él sigue oyendo: podemos vaciar el corazón y pedir que se haga su voluntad.</t>
+        </is>
+      </c>
+      <c r="J193" s="61" t="n"/>
+      <c r="K193" s="61" t="n"/>
+      <c r="L193" s="61" t="inlineStr">
+        <is>
+          <t>La constancia sostiene la oración aunque no haya ganas.</t>
+        </is>
+      </c>
+      <c r="M193" s="61" t="n"/>
+      <c r="N193" s="61" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="61" t="n">
+        <v>33</v>
+      </c>
+      <c r="B194" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C194" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar el rebaño</t>
+        </is>
+      </c>
+      <c r="D194" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, 16 de agosto, Paraguay celebra el Día del Niño, en memoria de los niños que combatieron en la batalla de Acosta Ñu, en 1869.</t>
+        </is>
+      </c>
+      <c r="E194" s="61" t="inlineStr">
+        <is>
+          <t>Batalla de Acosta Ñu, 16 de agosto de 1869; Día del Niño en Paraguay</t>
+        </is>
+      </c>
+      <c r="F194" s="61" t="inlineStr">
+        <is>
+          <t>Pablo habla a los líderes de la iglesia de Éfeso. Lo primero que les pide es que se cuiden a sí mismos: no se puede guiar a otros con el alma descuidada.</t>
+        </is>
+      </c>
+      <c r="G194" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que cuidan a todos menos su propia vida con Dios.</t>
+        </is>
+      </c>
+      <c r="H194" s="61" t="inlineStr">
+        <is>
+          <t>Si liderás algo, en casa, en el trabajo o en la iglesia, apartá hoy un tiempo para tu propia vida espiritual.</t>
+        </is>
+      </c>
+      <c r="I194" s="61" t="inlineStr">
+        <is>
+          <t>La visión de Pablo era clara y fácil de repetir: cuidar a las personas. Una visión que solo vive en la cabeza del líder no mueve a nadie; tiene que decirse en palabras simples.</t>
+        </is>
+      </c>
+      <c r="J194" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que hablan difícil y nadie entiende hacia dónde van.</t>
+        </is>
+      </c>
+      <c r="K194" s="61" t="inlineStr">
+        <is>
+          <t>Resumí en una sola frase la meta principal de tu familia o de tu equipo para este año, y compartila.</t>
+        </is>
+      </c>
+      <c r="L194" s="61" t="inlineStr">
+        <is>
+          <t>Las personas que lideramos valen tanto que Cristo dio su vida por ellas. Liderar con amor es recordarlo cada día, sobre todo con los más pequeños.</t>
+        </is>
+      </c>
+      <c r="M194" s="61" t="inlineStr">
+        <is>
+          <t>Ver a las personas como recursos para cumplir una meta.</t>
+        </is>
+      </c>
+      <c r="N194" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, Día del Niño, dedicale tiempo de calidad a un niño de tu familia o de tu iglesia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="61" t="n">
+        <v>33</v>
+      </c>
+      <c r="B195" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C195" s="61" t="inlineStr">
+        <is>
+          <t>Planes de bien</t>
+        </is>
+      </c>
+      <c r="D195" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías anunció que el exilio en Babilonia duraría setenta años; la promesa de Jeremías 29:11 viene justo después de ese anuncio.</t>
+        </is>
+      </c>
+      <c r="E195" s="61" t="inlineStr">
+        <is>
+          <t>Jeremías 29:10-11</t>
+        </is>
+      </c>
+      <c r="F195" s="61" t="inlineStr">
+        <is>
+          <t>Este versículo fue escrito a un pueblo en el exilio, y Dios les dijo que esperarían setenta años (29:10). Sus planes de bien no eran una salida rápida, sino fidelidad a largo plazo.</t>
+        </is>
+      </c>
+      <c r="G195" s="61" t="inlineStr">
+        <is>
+          <t>Usar este versículo como promesa de que todo va a salir como queremos, y pronto.</t>
+        </is>
+      </c>
+      <c r="H195" s="61" t="inlineStr">
+        <is>
+          <t>Si estás en una etapa difícil, leé Jeremías 29:4-14 completo y mirá cómo Dios sostuvo a su pueblo en el camino.</t>
+        </is>
+      </c>
+      <c r="I195" s="61" t="inlineStr">
+        <is>
+          <t>Una visión clara da esperanza. Dios le dio a su pueblo una dirección: buscar la paz de la ciudad, trabajar y formar familia (29:5-7). La esperanza vino con tareas concretas.</t>
+        </is>
+      </c>
+      <c r="J195" s="61" t="inlineStr">
+        <is>
+          <t>Una visión tan vaga que no dice qué hacer hoy.</t>
+        </is>
+      </c>
+      <c r="K195" s="61" t="inlineStr">
+        <is>
+          <t>Escribí tu visión y, al lado, una cosa concreta que podés hacer esta semana para acercarte a ella.</t>
+        </is>
+      </c>
+      <c r="L195" s="61" t="inlineStr">
+        <is>
+          <t>El líder no ve todo el camino, pero puede comunicar hacia dónde van y por qué vale la pena.</t>
+        </is>
+      </c>
+      <c r="M195" s="61" t="inlineStr">
+        <is>
+          <t>Esperar a tener todo claro para empezar.</t>
+        </is>
+      </c>
+      <c r="N195" s="61" t="inlineStr">
+        <is>
+          <t>Contale a tu equipo o a tu familia no solo qué hay que hacer, sino para qué.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="61" t="n">
+        <v>33</v>
+      </c>
+      <c r="B196" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C196" s="61" t="inlineStr">
+        <is>
+          <t>Una meta clara</t>
+        </is>
+      </c>
+      <c r="D196" s="61" t="inlineStr">
+        <is>
+          <t>La palabra griega que Pablo usa para «meta» (skopós) designaba la marca que el corredor miraba al final de la pista.</t>
+        </is>
+      </c>
+      <c r="E196" s="61" t="inlineStr">
+        <is>
+          <t>Filipenses 3:14; léxico griego de Strong (G4649, skopós)</t>
+        </is>
+      </c>
+      <c r="F196" s="61" t="inlineStr">
+        <is>
+          <t>Pablo usa la imagen de una carrera. Entre soñar una meta y alcanzarla hay una distancia que se recorre con pasos pequeños.</t>
+        </is>
+      </c>
+      <c r="G196" s="61" t="inlineStr">
+        <is>
+          <t>Quedarse en el sueño sin dar el primer paso.</t>
+        </is>
+      </c>
+      <c r="H196" s="61" t="inlineStr">
+        <is>
+          <t>Dividí tu meta en tres pasos pequeños y escribilos.</t>
+        </is>
+      </c>
+      <c r="I196" s="61" t="inlineStr">
+        <is>
+          <t>Para Pablo, el premio es el llamado de Dios en Cristo. Toda visión de un líder cristiano se ordena debajo de ese llamado.</t>
+        </is>
+      </c>
+      <c r="J196" s="61" t="inlineStr">
+        <is>
+          <t>Metas que nos alejan de Dios o de la familia.</t>
+        </is>
+      </c>
+      <c r="K196" s="61" t="inlineStr">
+        <is>
+          <t>Revisá tu meta: ¿te acerca o te aleja de lo que Dios te llama a ser?</t>
+        </is>
+      </c>
+      <c r="L196" s="61" t="inlineStr">
+        <is>
+          <t>Un corredor mira constantemente hacia dónde corre. Los pasos medibles permiten saber si se avanza.</t>
+        </is>
+      </c>
+      <c r="M196" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar mucho sin saber si se avanza hacia la meta.</t>
+        </is>
+      </c>
+      <c r="N196" s="61" t="inlineStr">
+        <is>
+          <t>Elegí cómo vas a medir el primer paso y cuándo lo vas a revisar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="61" t="n">
+        <v>33</v>
+      </c>
+      <c r="B197" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C197" s="61" t="inlineStr">
+        <is>
+          <t>Obrero aprobado</t>
+        </is>
+      </c>
+      <c r="D197" s="61" t="inlineStr">
+        <is>
+          <t>La segunda carta a Timoteo es considerada la última carta de Pablo, escrita desde la prisión poco antes de su muerte.</t>
+        </is>
+      </c>
+      <c r="E197" s="61" t="inlineStr">
+        <is>
+          <t>2 Timoteo 1:8; 4:6-8</t>
+        </is>
+      </c>
+      <c r="F197" s="61" t="inlineStr">
+        <is>
+          <t>Pablo le pide a Timoteo esfuerzo para usar bien la Palabra. Hacer bien las cosas requiere preparación.</t>
+        </is>
+      </c>
+      <c r="G197" s="61" t="inlineStr">
+        <is>
+          <t>Querer liderar sin prepararse.</t>
+        </is>
+      </c>
+      <c r="H197" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un tiempo fijo esta semana para leer la Biblia con calma.</t>
+        </is>
+      </c>
+      <c r="I197" s="61" t="inlineStr">
+        <is>
+          <t>Un obrero trabaja paso a paso y con orden. La visión se cumple con trabajo bien hecho cada día, no con un gran gesto.</t>
+        </is>
+      </c>
+      <c r="J197" s="61" t="inlineStr">
+        <is>
+          <t>Esperar un golpe de suerte en vez de trabajar con constancia.</t>
+        </is>
+      </c>
+      <c r="K197" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy el primer paso de tu meta, aunque sea pequeño.</t>
+        </is>
+      </c>
+      <c r="L197" s="61" t="inlineStr">
+        <is>
+          <t>Un obrero que no tiene de qué avergonzarse es honesto en los detalles. Los pasos de una visión también tienen que ser íntegros.</t>
+        </is>
+      </c>
+      <c r="M197" s="61" t="inlineStr">
+        <is>
+          <t>Tomar atajos deshonestos para llegar más rápido a la meta.</t>
+        </is>
+      </c>
+      <c r="N197" s="61" t="inlineStr">
+        <is>
+          <t>Revisá si algún paso de tu plan necesita corregirse para ser más honesto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="61" t="n">
+        <v>33</v>
+      </c>
+      <c r="B198" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C198" s="61" t="inlineStr">
+        <is>
+          <t>Más de lo que pedimos</t>
+        </is>
+      </c>
+      <c r="D198" s="61" t="inlineStr">
+        <is>
+          <t>Este versículo cierra una oración de Pablo para que los creyentes conozcan el amor de Cristo, que sobrepasa todo conocimiento.</t>
+        </is>
+      </c>
+      <c r="E198" s="61" t="inlineStr">
+        <is>
+          <t>Efesios 3:14-21</t>
+        </is>
+      </c>
+      <c r="F198" s="61" t="inlineStr">
+        <is>
+          <t>Pablo acaba de orar para que conozcamos el amor de Cristo (3:17-19). Lo que Dios hace más allá de lo que pedimos tiene que ver, ante todo, con ese amor.</t>
+        </is>
+      </c>
+      <c r="G198" s="61" t="inlineStr">
+        <is>
+          <t>Usar este versículo para prometer que nuestros proyectos van a salir más grandes de lo que soñamos.</t>
+        </is>
+      </c>
+      <c r="H198" s="61" t="inlineStr">
+        <is>
+          <t>Orá hoy por tu proyecto, y también por conocer más el amor de Cristo.</t>
+        </is>
+      </c>
+      <c r="I198" s="61" t="inlineStr">
+        <is>
+          <t>Toda visión pasa por un tramo intermedio: el entusiasmo se fue y el resultado no llega. Ahí, lo que sostiene no es nuestra fuerza, sino el poder de Dios que actúa en nosotros.</t>
+        </is>
+      </c>
+      <c r="J198" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar justo en la mitad del camino.</t>
+        </is>
+      </c>
+      <c r="K198" s="61" t="inlineStr">
+        <is>
+          <t>Identificá en qué tramo intermedio estás con algún proyecto, y no lo abandones justo ahí.</t>
+        </is>
+      </c>
+      <c r="L198" s="61" t="inlineStr">
+        <is>
+          <t>A veces Dios cambia el rumbo de nuestra visión, y lo que resulta es mejor de lo que planeamos. Sostener la visión es también estar dispuestos a ajustarla.</t>
+        </is>
+      </c>
+      <c r="M198" s="61" t="inlineStr">
+        <is>
+          <t>Aferrarse a un plan aunque esté claro que hay que cambiarlo.</t>
+        </is>
+      </c>
+      <c r="N198" s="61" t="inlineStr">
+        <is>
+          <t>Pedile a alguien de confianza su opinión sincera sobre tu proyecto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="61" t="n">
+        <v>33</v>
+      </c>
+      <c r="B199" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C199" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: visión con propósito</t>
+        </is>
+      </c>
+      <c r="D199" s="61" t="inlineStr">
+        <is>
+          <t>El 15 de agosto se recuerda la fundación de Asunción, en 1537.</t>
+        </is>
+      </c>
+      <c r="E199" s="61" t="inlineStr">
+        <is>
+          <t>Fundación de Nuestra Señora Santa María de la Asunción, 15 de agosto de 1537</t>
+        </is>
+      </c>
+      <c r="F199" s="61" t="inlineStr">
+        <is>
+          <t>Una visión clara se dice en palabras simples y pone a las personas en el centro, porque Cristo dio su vida por ellas.</t>
+        </is>
+      </c>
+      <c r="G199" s="61" t="n"/>
+      <c r="H199" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, compartí con tu familia o tu equipo la visión en una frase y los tres primeros pasos, y que el fruto apunte a la gloria de Dios.</t>
+        </is>
+      </c>
+      <c r="I199" s="61" t="inlineStr">
+        <is>
+          <t>Entre la visión y la meta hay pasos pequeños, medibles y honestos.</t>
+        </is>
+      </c>
+      <c r="J199" s="61" t="n"/>
+      <c r="K199" s="61" t="n"/>
+      <c r="L199" s="61" t="inlineStr">
+        <is>
+          <t>En el tramo difícil sostiene el poder de Dios, y a veces la visión se ajusta.</t>
+        </is>
+      </c>
+      <c r="M199" s="61" t="n"/>
+      <c r="N199" s="61" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="61" t="n">
+        <v>34</v>
+      </c>
+      <c r="B200" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C200" s="61" t="inlineStr">
+        <is>
+          <t>Un guardia en la boca</t>
+        </is>
+      </c>
+      <c r="D200" s="61" t="inlineStr">
+        <is>
+          <t>Santiago da una regla sencilla para comunicarse: ser rápidos para escuchar, lentos para hablar y lentos para enojarse.</t>
+        </is>
+      </c>
+      <c r="E200" s="61" t="inlineStr">
+        <is>
+          <t>Santiago 1:19</t>
+        </is>
+      </c>
+      <c r="F200" s="61" t="inlineStr">
+        <is>
+          <t>David le pide a Dios un guardia en la boca. En casa, la comunicación se rompe menos por lo que se dice que por cómo se dice.</t>
+        </is>
+      </c>
+      <c r="G200" s="61" t="inlineStr">
+        <is>
+          <t>Decir «yo soy así, digo lo que pienso» para justificar palabras que hieren.</t>
+        </is>
+      </c>
+      <c r="H200" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, antes de responder algo que te molestó, contá hasta diez.</t>
+        </is>
+      </c>
+      <c r="I200" s="61" t="inlineStr">
+        <is>
+          <t>Es una oración: reconocemos que solos no podemos controlar la lengua.</t>
+        </is>
+      </c>
+      <c r="J200" s="61" t="inlineStr">
+        <is>
+          <t>Prometerse no volver a gritar, sin pedirle ayuda a Dios.</t>
+        </is>
+      </c>
+      <c r="K200" s="61" t="inlineStr">
+        <is>
+          <t>Empezá el día pidiéndole a Dios que cuide tus palabras con tu familia.</t>
+        </is>
+      </c>
+      <c r="L200" s="61" t="inlineStr">
+        <is>
+          <t>Guardar silencio también es escuchar sin prepararse para contestar. Una técnica simple: repetir lo que el otro dijo antes de responder.</t>
+        </is>
+      </c>
+      <c r="M200" s="61" t="inlineStr">
+        <is>
+          <t>Escuchar solo para preparar la defensa.</t>
+        </is>
+      </c>
+      <c r="N200" s="61" t="inlineStr">
+        <is>
+          <t>En tu próxima conversación difícil en casa, repetí lo que entendiste antes de dar tu opinión.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="61" t="n">
+        <v>34</v>
+      </c>
+      <c r="B201" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C201" s="61" t="inlineStr">
+        <is>
+          <t>Comprensión y honra</t>
+        </is>
+      </c>
+      <c r="D201" s="61" t="inlineStr">
+        <is>
+          <t>Pedro escribe a creyentes dispersos por varias provincias de Asia Menor, en la actual Turquía.</t>
+        </is>
+      </c>
+      <c r="E201" s="61" t="inlineStr">
+        <is>
+          <t>1 Pedro 1:1</t>
+        </is>
+      </c>
+      <c r="F201" s="61" t="inlineStr">
+        <is>
+          <t>Pedro pide a los esposos vivir con comprensión, es decir, conocer de verdad a su esposa. Escuchar es la base de esa comprensión.</t>
+        </is>
+      </c>
+      <c r="G201" s="61" t="inlineStr">
+        <is>
+          <t>Esposos que dan órdenes pero no escuchan.</t>
+        </is>
+      </c>
+      <c r="H201" s="61" t="inlineStr">
+        <is>
+          <t>Esposo: preguntale hoy a tu esposa cómo está, y escuchá sin interrumpir.</t>
+        </is>
+      </c>
+      <c r="I201" s="61" t="inlineStr">
+        <is>
+          <t>En esa sociedad la mujer era más vulnerable, y Pedro pide honrarla. Además dice que es coheredera del don de la vida: igual ante Dios. La forma de hablar en casa muestra si honramos al otro.</t>
+        </is>
+      </c>
+      <c r="J201" s="61" t="inlineStr">
+        <is>
+          <t>Palabras que humillan o desvalorizan, aunque sea «en broma».</t>
+        </is>
+      </c>
+      <c r="K201" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, decile en voz alta a tu pareja algo que valorás de ella.</t>
+        </is>
+      </c>
+      <c r="L201" s="61" t="inlineStr">
+        <is>
+          <t>Pedro une el trato a la esposa con la vida de oración. Cómo hablamos en casa no está separado de nuestra relación con Dios.</t>
+        </is>
+      </c>
+      <c r="M201" s="61" t="inlineStr">
+        <is>
+          <t>Ser muy espiritual en la iglesia y duro con las palabras en casa.</t>
+        </is>
+      </c>
+      <c r="N201" s="61" t="inlineStr">
+        <is>
+          <t>Si heriste a alguien de tu casa con palabras, pedile perdón antes de orar esta noche.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="61" t="n">
+        <v>34</v>
+      </c>
+      <c r="B202" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C202" s="61" t="inlineStr">
+        <is>
+          <t>Con gracia y sal</t>
+        </is>
+      </c>
+      <c r="D202" s="61" t="inlineStr">
+        <is>
+          <t>En el griego, Pablo pide que la conversación sea «con gracia, sazonada con sal»: la sal daba sabor y conservaba los alimentos.</t>
+        </is>
+      </c>
+      <c r="E202" s="61" t="inlineStr">
+        <is>
+          <t>Colosenses 4:6 (texto griego; Reina-Valera 1960)</t>
+        </is>
+      </c>
+      <c r="F202" s="61" t="inlineStr">
+        <is>
+          <t>Pablo habla aquí de cómo tratar a los de afuera (4:5), y el principio vale todavía más en casa. Hablar con gracia rompe silencios que se vuelven distancia.</t>
+        </is>
+      </c>
+      <c r="G202" s="61" t="inlineStr">
+        <is>
+          <t>Ser amables con los de afuera y secos con los de casa.</t>
+        </is>
+      </c>
+      <c r="H202" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, saludá con cariño a cada uno de tu casa al llegar.</t>
+        </is>
+      </c>
+      <c r="I202" s="61" t="inlineStr">
+        <is>
+          <t>El silencio en una familia puede ser paz o distancia acumulada. La sabiduría ayuda a distinguir cuál es cuál.</t>
+        </is>
+      </c>
+      <c r="J202" s="61" t="inlineStr">
+        <is>
+          <t>Temas que nadie toca en casa y que se vuelven muros.</t>
+        </is>
+      </c>
+      <c r="K202" s="61" t="inlineStr">
+        <is>
+          <t>Pensá si hay algún silencio pendiente de romper en tu casa esta semana.</t>
+        </is>
+      </c>
+      <c r="L202" s="61" t="inlineStr">
+        <is>
+          <t>Cada persona necesita una respuesta distinta: un hijo adolescente, un padre mayor, la pareja. Responder bien empieza por conocer al otro.</t>
+        </is>
+      </c>
+      <c r="M202" s="61" t="inlineStr">
+        <is>
+          <t>Hablarles a todos de la misma manera y no entender por qué no funciona.</t>
+        </is>
+      </c>
+      <c r="N202" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale a alguien de tu casa cómo prefiere que le hables cuando está mal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="61" t="n">
+        <v>34</v>
+      </c>
+      <c r="B203" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C203" s="61" t="inlineStr">
+        <is>
+          <t>La palabra a tiempo</t>
+        </is>
+      </c>
+      <c r="D203" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 25 abre una colección de dichos de Salomón que copiaron los hombres de Ezequías, rey de Judá.</t>
+        </is>
+      </c>
+      <c r="E203" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 25:1</t>
+        </is>
+      </c>
+      <c r="F203" s="61" t="inlineStr">
+        <is>
+          <t>Una palabra justa en el momento justo vale como una joya. Romper un silencio también requiere elegir el momento.</t>
+        </is>
+      </c>
+      <c r="G203" s="61" t="inlineStr">
+        <is>
+          <t>Sacar un tema delicado en medio de una pelea o delante de otros.</t>
+        </is>
+      </c>
+      <c r="H203" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés que hablar algo difícil en casa, elegí un momento tranquilo y a solas.</t>
+        </is>
+      </c>
+      <c r="I203" s="61" t="inlineStr">
+        <is>
+          <t>Hay momentos para aconsejar, para animar y para corregir. Y a veces lo sabio es solo acompañar en silencio.</t>
+        </is>
+      </c>
+      <c r="J203" s="61" t="inlineStr">
+        <is>
+          <t>Dar consejos cuando el otro solo necesita ser escuchado.</t>
+        </is>
+      </c>
+      <c r="K203" s="61" t="inlineStr">
+        <is>
+          <t>Antes de aconsejar, preguntá: ¿querés que te dé mi opinión o preferís que solo te escuche?</t>
+        </is>
+      </c>
+      <c r="L203" s="61" t="inlineStr">
+        <is>
+          <t>Las palabras bien dichas edifican y traen paz. Una palabra de aliento a tiempo puede cambiar el día de alguien de tu casa.</t>
+        </is>
+      </c>
+      <c r="M203" s="61" t="inlineStr">
+        <is>
+          <t>Familias donde solo se habla para reclamar.</t>
+        </is>
+      </c>
+      <c r="N203" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, decile una palabra de aliento a alguien de tu familia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="61" t="n">
+        <v>34</v>
+      </c>
+      <c r="B204" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C204" s="61" t="inlineStr">
+        <is>
+          <t>Perdonar como fuimos perdonados</t>
+        </is>
+      </c>
+      <c r="D204" s="61" t="inlineStr">
+        <is>
+          <t>El investigador de parejas John Gottman señaló el desprecio como uno de los signos que más anticipan una ruptura.</t>
+        </is>
+      </c>
+      <c r="E204" s="61" t="inlineStr">
+        <is>
+          <t>John Gottman, ¿Qué hace que el amor perdure? / Why Marriages Succeed or Fail, 1994</t>
+        </is>
+      </c>
+      <c r="F204" s="61" t="inlineStr">
+        <is>
+          <t>El conflicto en sí no daña a una familia; lo que daña es no saber resolverlo. La bondad permite discutir la idea sin atacar a la persona.</t>
+        </is>
+      </c>
+      <c r="G204" s="61" t="inlineStr">
+        <is>
+          <t>Burlas, desprecio y ataques personales en medio de una discusión.</t>
+        </is>
+      </c>
+      <c r="H204" s="61" t="inlineStr">
+        <is>
+          <t>En tu próxima discusión, hablá del problema, no de la persona.</t>
+        </is>
+      </c>
+      <c r="I204" s="61" t="inlineStr">
+        <is>
+          <t>Perdonamos porque Dios nos perdonó primero. El perdón no borra el problema, pero permite resolverlo sin romper el vínculo. Perdonar no es tolerar el maltrato: si hay violencia, hace falta buscar ayuda y protección.</t>
+        </is>
+      </c>
+      <c r="J204" s="61" t="inlineStr">
+        <is>
+          <t>Guardar rencores y sacarlos en cada pelea: «siempre hacés lo mismo».</t>
+        </is>
+      </c>
+      <c r="K204" s="61" t="inlineStr">
+        <is>
+          <t>Prueben esta regla en casa: no usar el pasado para pelear el presente.</t>
+        </is>
+      </c>
+      <c r="L204" s="61" t="inlineStr">
+        <is>
+          <t>Buscar una solución en vez de ganar la discusión mantiene el vínculo, como los hermanos que descubrieron que uno quería el jugo de la naranja y el otro la cáscara.</t>
+        </is>
+      </c>
+      <c r="M204" s="61" t="inlineStr">
+        <is>
+          <t>Discutir para ganar, aunque se pierda la relación.</t>
+        </is>
+      </c>
+      <c r="N204" s="61" t="inlineStr">
+        <is>
+          <t>Cuando discutan, pregúntense: ¿qué necesita cada uno? Y busquen una solución que sirva a los dos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="61" t="n">
+        <v>34</v>
+      </c>
+      <c r="B205" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C205" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: palabras que edifican</t>
+        </is>
+      </c>
+      <c r="D205" s="61" t="inlineStr">
+        <is>
+          <t>Jesús enseñó que de lo que abunda en el corazón habla la boca.</t>
+        </is>
+      </c>
+      <c r="E205" s="61" t="inlineStr">
+        <is>
+          <t>Mateo 12:34; Lucas 6:45</t>
+        </is>
+      </c>
+      <c r="F205" s="61" t="inlineStr">
+        <is>
+          <t>Hablar sin herir y escuchar para entender, no para defenderse.</t>
+        </is>
+      </c>
+      <c r="G205" s="61" t="n"/>
+      <c r="H205" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, tengan en familia una conversación tranquila: cada uno dice algo que valora de los demás y algo que le gustaría mejorar en cómo se hablan.</t>
+        </is>
+      </c>
+      <c r="I205" s="61" t="inlineStr">
+        <is>
+          <t>El silencio puede ser paz o distancia: hay que elegir el momento para romper los silencios pendientes.</t>
+        </is>
+      </c>
+      <c r="J205" s="61" t="n"/>
+      <c r="K205" s="61" t="n"/>
+      <c r="L205" s="61" t="inlineStr">
+        <is>
+          <t>El conflicto se resuelve buscando juntos una solución, con bondad y perdón, sin atacar a la persona.</t>
+        </is>
+      </c>
+      <c r="M205" s="61" t="n"/>
+      <c r="N205" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de agosto verificados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -7645,7 +7645,7 @@
       </c>
       <c r="Z34" s="10" t="inlineStr">
         <is>
-          <t>Hechos 20:28 — Yo les ruego que piensen en ustedes mismos, y que cuiden el rebaño sobre el cual el Espíritu Santo los ha puesto como obispos, para que cuiden de la iglesia del Señor, que él ganó por su propia sangre.</t>
+          <t>Hechos 20:28 — Yo les ruego que piensen en ustedes mismos, y que velen por el rebaño sobre el cual el Espíritu Santo los ha puesto como obispos, para que cuiden de la iglesia del Señor, que él ganó por su propia sangre.</t>
         </is>
       </c>
       <c r="AA34" s="10" t="inlineStr">
@@ -31791,7 +31791,7 @@
       </c>
       <c r="D189" s="61" t="inlineStr">
         <is>
-          <t>La palabra griega que Jesús usa para «habitación» designaba el cuarto interior o la despensa de la casa, a veces el único lugar con puerta.</t>
+          <t>La palabra griega que Mateo usa para «habitación» designaba el cuarto interior o la despensa de la casa, a veces el único lugar con puerta.</t>
         </is>
       </c>
       <c r="E189" s="61" t="inlineStr">
@@ -32001,12 +32001,12 @@
       </c>
       <c r="D192" s="61" t="inlineStr">
         <is>
-          <t>Jesús dijo estas palabras en Jerusalén, en su última semana; pocos días después, en Getsemaní, pidió que se hiciera la voluntad del Padre y no la suya.</t>
+          <t>Jesús dijo estas palabras camino a Jerusalén, en su última semana; pocos días después, en Getsemaní, pidió que se hiciera la voluntad del Padre y no la suya.</t>
         </is>
       </c>
       <c r="E192" s="61" t="inlineStr">
         <is>
-          <t>Marcos 11:11-24; 14:36</t>
+          <t>Marcos 11:20-24; 14:36</t>
         </is>
       </c>
       <c r="F192" s="61" t="inlineStr">
@@ -32071,12 +32071,12 @@
       </c>
       <c r="D193" s="61" t="inlineStr">
         <is>
-          <t>Después de este versículo, Jesús cuenta la parábola de una viuda que insistió ante un juez injusto; si ese juez le hizo justicia, cuánto más Dios a sus hijos.</t>
+          <t>Después de este versículo, Jesús cuenta la parábola de una viuda que insistió ante un juez injusto; si ese juez le hizo justicia, cuánto más Dios a sus escogidos que claman a él día y noche.</t>
         </is>
       </c>
       <c r="E193" s="61" t="inlineStr">
         <is>
-          <t>Lucas 18:2-8</t>
+          <t>Lucas 18:1-8</t>
         </is>
       </c>
       <c r="F193" s="61" t="inlineStr">
@@ -32806,7 +32806,7 @@
       </c>
       <c r="E204" s="61" t="inlineStr">
         <is>
-          <t>John Gottman, ¿Qué hace que el amor perdure? / Why Marriages Succeed or Fail, 1994</t>
+          <t>John Gottman, Why Marriages Succeed or Fail, 1994</t>
         </is>
       </c>
       <c r="F204" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: guiones de septiembre con revisión teológica
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -8043,8 +8043,8 @@
       <c r="Y36" s="14" t="inlineStr">
         <is>
           <t>• Provisión de Dios
-2 Necesidades vs. deseo
-3 Fuente inagotable</t>
+• Necesidades vs. deseo
+• Fuente inagotable</t>
         </is>
       </c>
       <c r="Z36" s="14" t="inlineStr">
@@ -8067,9 +8067,9 @@
       </c>
       <c r="AC36" s="14" t="inlineStr">
         <is>
-          <t>• • El amor al dinero como origen del mal: 
-• • La desviación de la fe: 
-• • Consecuencias dolorosas:</t>
+          <t>• El amor al dinero, no el dinero, es la raíz del problema
+• La codicia aparta de la fe
+• La codicia trae muchos dolores</t>
         </is>
       </c>
       <c r="AD36" s="14" t="inlineStr">
@@ -8081,7 +8081,7 @@
         <is>
           <t>• Cuidarse de la avaricia — No dejar que el deseo de tener nos domine.
 • Los bienes no lo son todo — Nuestra vida no depende de las riquezas.
-• Valorar lo verdaderamente importante — Poner a Dios y lo espiritual en</t>
+• Valorar lo verdaderamente importante — Poner a Dios y lo espiritual en primer lugar.</t>
         </is>
       </c>
       <c r="AF36" s="14" t="inlineStr">
@@ -8283,7 +8283,7 @@
       <c r="AE37" s="2" t="inlineStr">
         <is>
           <t>• La mano diligente lidera
-• La pereza lleva a servir a otros
+• La negligencia tiene consecuencias
 • El esfuerzo constante da autoridad</t>
         </is>
       </c>
@@ -8461,7 +8461,7 @@
         <is>
           <t>• La comunidad de creyentes compartía todo
 • Un corazón y un alma en común
-• El modelo cooperativo tiene raíces bíblicas</t>
+• Compartir nace del amor, no de la obligación</t>
         </is>
       </c>
       <c r="AB38" s="4" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="Z39" s="6" t="inlineStr">
         <is>
-          <t>Eclesiastes 12:1 — Acuerdate de tu Creador ahora que eres joven. No esperes a que vengan los dias malos, y a que lleguen los anos en que digas: Vivir tanto no es motivo de regocijo</t>
+          <t>Eclesiastes 12:1 — Acuérdate de tu Creador ahora que eres joven. No esperes a que vengan los días malos, y a que lleguen los años en que digas: Vivir tanto no es motivo de regocijo</t>
         </is>
       </c>
       <c r="AA39" s="6" t="inlineStr">
@@ -8859,7 +8859,7 @@
       <c r="Y40" s="8" t="inlineStr">
         <is>
           <t>• En Cristo hay una identidad nueva
-• Lo viejo paso, lo nuevo llegó
+• Lo viejo pasó, lo nuevo llegó
 • La transformación es real, no solo simbólica</t>
         </is>
       </c>
@@ -8882,9 +8882,9 @@
       </c>
       <c r="AC40" s="8" t="inlineStr">
         <is>
-          <t>• • Fin de la esclavitud
-• • Adopción como hijo
-• • Herencia por medio de Cristo</t>
+          <t>• Fin de la esclavitud
+• Adopción como hijo
+• Herencia por medio de Cristo</t>
         </is>
       </c>
       <c r="AD40" s="8" t="inlineStr">
@@ -8913,7 +8913,7 @@
       </c>
       <c r="AH40" s="8" t="inlineStr">
         <is>
-          <t>Romanos 8:16-17 — El Espiritu mismo da testimonio a nuestro espiritu, de que somos hijos de Dios. Y si somos hijos, somos tambien herederos; herederos de Dios y coherederos con Cristo</t>
+          <t>Romanos 8:16-17 — El Espíritu mismo da testimonio a nuestro espíritu, de que somos hijos de Dios. Y si somos hijos, somos también herederos; herederos de Dios y coherederos con Cristo</t>
         </is>
       </c>
       <c r="AI40" s="8" t="inlineStr">
@@ -19214,7 +19214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N205"/>
+  <dimension ref="A1:N235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -32904,6 +32904,2006 @@
       </c>
       <c r="M205" s="61" t="n"/>
       <c r="N205" s="61" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="B206" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C206" s="61" t="inlineStr">
+        <is>
+          <t>Mejor dos que uno</t>
+        </is>
+      </c>
+      <c r="D206" s="61" t="inlineStr">
+        <is>
+          <t>El versículo anterior dice que dos rinden más que uno, porque juntos sacan más fruto de su trabajo.</t>
+        </is>
+      </c>
+      <c r="E206" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés 4:9</t>
+        </is>
+      </c>
+      <c r="F206" s="61" t="inlineStr">
+        <is>
+          <t>Salomón observa que dos rinden más que uno. En el hogar, administrar juntos no es perder autonomía: es remar hacia el mismo lado.</t>
+        </is>
+      </c>
+      <c r="G206" s="61" t="inlineStr">
+        <is>
+          <t>Que cada uno maneje su plata por su lado, sin contarle al otro.</t>
+        </is>
+      </c>
+      <c r="H206" s="61" t="inlineStr">
+        <is>
+          <t>Propongan una reunión de plata en pareja, una vez al mes, aunque sea de veinte minutos.</t>
+        </is>
+      </c>
+      <c r="I206" s="61" t="inlineStr">
+        <is>
+          <t>Cuando uno se equivoca con la plata, el otro lo levanta en vez de hundirlo con reproches.</t>
+        </is>
+      </c>
+      <c r="J206" s="61" t="inlineStr">
+        <is>
+          <t>Usar el error del otro como arma en cada discusión.</t>
+        </is>
+      </c>
+      <c r="K206" s="61" t="inlineStr">
+        <is>
+          <t>Si tu pareja se equivocó con un gasto, háblenlo para buscar una salida, no para culpar.</t>
+        </is>
+      </c>
+      <c r="L206" s="61" t="inlineStr">
+        <is>
+          <t>Las deudas y los apuros pesan menos cuando se enfrentan juntos. Y si la carga es grande, también se puede pedir consejo a un profesional de confianza.</t>
+        </is>
+      </c>
+      <c r="M206" s="61" t="inlineStr">
+        <is>
+          <t>Esconder una deuda por vergüenza hasta que ya es tarde.</t>
+        </is>
+      </c>
+      <c r="N206" s="61" t="inlineStr">
+        <is>
+          <t>Si hay una deuda que tu pareja no conoce, buscá el momento para contársela esta semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="B207" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C207" s="61" t="inlineStr">
+        <is>
+          <t>La raíz</t>
+        </is>
+      </c>
+      <c r="D207" s="61" t="inlineStr">
+        <is>
+          <t>En el griego, Pablo dice que el amor al dinero es raíz de «toda clase» de males: no la única causa de todo mal, sino una raíz que produce muchos.</t>
+        </is>
+      </c>
+      <c r="E207" s="61" t="inlineStr">
+        <is>
+          <t>1 Timoteo 6:10 (texto griego)</t>
+        </is>
+      </c>
+      <c r="F207" s="61" t="inlineStr">
+        <is>
+          <t>Pablo no dice que el dinero sea malo, sino el amor al dinero. Se puede tener poco y amarlo mucho, o tener mucho y no ponerle el corazón.</t>
+        </is>
+      </c>
+      <c r="G207" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que el problema es solo de los ricos.</t>
+        </is>
+      </c>
+      <c r="H207" s="61" t="inlineStr">
+        <is>
+          <t>Preguntate con honestidad: ¿qué lugar ocupa el dinero en mis pensamientos de cada día?</t>
+        </is>
+      </c>
+      <c r="I207" s="61" t="inlineStr">
+        <is>
+          <t>Algunos, por codiciarlo, se apartaron de la fe. En la pareja, la codicia también aparta: pone las cosas por encima de las personas.</t>
+        </is>
+      </c>
+      <c r="J207" s="61" t="inlineStr">
+        <is>
+          <t>Discusiones de pareja donde el dinero vale más que el otro.</t>
+        </is>
+      </c>
+      <c r="K207" s="61" t="inlineStr">
+        <is>
+          <t>Antes de una compra grande, consultala con tu pareja.</t>
+        </is>
+      </c>
+      <c r="L207" s="61" t="inlineStr">
+        <is>
+          <t>La codicia promete felicidad y deja dolores. La integridad en el manejo de la plata de la casa ahorra muchos dolores.</t>
+        </is>
+      </c>
+      <c r="M207" s="61" t="inlineStr">
+        <is>
+          <t>Gastos escondidos que, cuando salen a la luz, rompen la confianza.</t>
+        </is>
+      </c>
+      <c r="N207" s="61" t="inlineStr">
+        <is>
+          <t>Pongan en común los gastos fijos de la casa, a la vista de los dos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="B208" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C208" s="61" t="inlineStr">
+        <is>
+          <t>La vida vale más</t>
+        </is>
+      </c>
+      <c r="D208" s="61" t="inlineStr">
+        <is>
+          <t>Justo después, Jesús cuenta la parábola del rico que construyó graneros más grandes para guardar su cosecha, y esa misma noche murió.</t>
+        </is>
+      </c>
+      <c r="E208" s="61" t="inlineStr">
+        <is>
+          <t>Lucas 12:16-21</t>
+        </is>
+      </c>
+      <c r="F208" s="61" t="inlineStr">
+        <is>
+          <t>Jesús responde a alguien que le pedía que interviniera en una herencia. Los hijos aprenden sobre el dinero mirando cómo lo vivimos los adultos.</t>
+        </is>
+      </c>
+      <c r="G208" s="61" t="inlineStr">
+        <is>
+          <t>Decirles a los hijos que el dinero no es todo, mientras vivimos como si lo fuera.</t>
+        </is>
+      </c>
+      <c r="H208" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, que tus hijos te vean dar algo con alegría.</t>
+        </is>
+      </c>
+      <c r="I208" s="61" t="inlineStr">
+        <is>
+          <t>Enseñar a los hijos que la vida vale más que lo que tienen los protege de la comparación.</t>
+        </is>
+      </c>
+      <c r="J208" s="61" t="inlineStr">
+        <is>
+          <t>Hijos que miden su valor por la marca de su ropa o de su celular.</t>
+        </is>
+      </c>
+      <c r="K208" s="61" t="inlineStr">
+        <is>
+          <t>Conversá con tus hijos sobre algo valioso que no se compra con plata.</t>
+        </is>
+      </c>
+      <c r="L208" s="61" t="inlineStr">
+        <is>
+          <t>Una idea simple: una alcancía dividida en tres partes, ahorrar, gastar y dar. Así aprenden a ordenar prioridades desde chicos.</t>
+        </is>
+      </c>
+      <c r="M208" s="61" t="inlineStr">
+        <is>
+          <t>Darles todo lo que piden, sin enseñarles a esperar.</t>
+        </is>
+      </c>
+      <c r="N208" s="61" t="inlineStr">
+        <is>
+          <t>Armá con tus hijos una alcancía con tres partes: ahorrar, gastar y dar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="B209" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C209" s="61" t="inlineStr">
+        <is>
+          <t>Dos amos</t>
+        </is>
+      </c>
+      <c r="D209" s="61" t="inlineStr">
+        <is>
+          <t>La palabra que Jesús usa para «riquezas» es «mamón», que en arameo significa dinero o posesiones.</t>
+        </is>
+      </c>
+      <c r="E209" s="61" t="inlineStr">
+        <is>
+          <t>Mateo 6:24; léxico griego de Strong (G3126, mamonás)</t>
+        </is>
+      </c>
+      <c r="F209" s="61" t="inlineStr">
+        <is>
+          <t>Jesús no dice que el dinero sea malo, sino que no puede ser amo. Los hijos aprenden quién manda en casa viendo nuestras decisiones.</t>
+        </is>
+      </c>
+      <c r="G209" s="61" t="inlineStr">
+        <is>
+          <t>Decisiones familiares que siempre se toman solo por la plata.</t>
+        </is>
+      </c>
+      <c r="H209" s="61" t="inlineStr">
+        <is>
+          <t>Contales a tus hijos una decisión en la que pusiste a Dios o a la familia antes que el dinero.</t>
+        </is>
+      </c>
+      <c r="I209" s="61" t="inlineStr">
+        <is>
+          <t>Darles a los hijos pequeñas oportunidades de decidir con su propia plata, aunque sea poca, les enseña más que cualquier sermón.</t>
+        </is>
+      </c>
+      <c r="J209" s="61" t="inlineStr">
+        <is>
+          <t>Hijos que llegan a adultos sin haber manejado nunca un guaraní.</t>
+        </is>
+      </c>
+      <c r="K209" s="61" t="inlineStr">
+        <is>
+          <t>Dale a tu hijo una suma pequeña para que la administre esta semana, y después conversen cómo le fue.</t>
+        </is>
+      </c>
+      <c r="L209" s="61" t="inlineStr">
+        <is>
+          <t>Si se equivocan con su plata siendo chicos, aprenden barato lo que de grandes cuesta caro.</t>
+        </is>
+      </c>
+      <c r="M209" s="61" t="inlineStr">
+        <is>
+          <t>Salir al rescate cada vez, para que no sientan ninguna consecuencia.</t>
+        </is>
+      </c>
+      <c r="N209" s="61" t="inlineStr">
+        <is>
+          <t>Si tu hijo gastó todo, acompañalo sin retarlo y ayudalo a pensar qué haría distinto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="B210" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C210" s="61" t="inlineStr">
+        <is>
+          <t>De acuerdo</t>
+        </is>
+      </c>
+      <c r="D210" s="61" t="inlineStr">
+        <is>
+          <t>Un estudio con más de 4.500 parejas encontró que las discusiones por dinero predecían el divorcio mejor que otros tipos de discusiones.</t>
+        </is>
+      </c>
+      <c r="E210" s="61" t="inlineStr">
+        <is>
+          <t>Dew, Britt y Huston, Family Relations, 2012</t>
+        </is>
+      </c>
+      <c r="F210" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribe a una iglesia dividida, y el principio vale para el hogar. Muchas peleas por dinero no son por el monto, sino por la falta de acuerdo previo.</t>
+        </is>
+      </c>
+      <c r="G210" s="61" t="inlineStr">
+        <is>
+          <t>Decidir gastos grandes sin consultar.</t>
+        </is>
+      </c>
+      <c r="H210" s="61" t="inlineStr">
+        <is>
+          <t>Pónganse de acuerdo en un monto a partir del cual toda compra se consulta.</t>
+        </is>
+      </c>
+      <c r="I210" s="61" t="inlineStr">
+        <is>
+          <t>La transparencia con la plata es una forma de integridad: no hay ahorros escondidos ni cuentas secretas.</t>
+        </is>
+      </c>
+      <c r="J210" s="61" t="inlineStr">
+        <is>
+          <t>Ahorros o deudas en secreto, «para no discutir».</t>
+        </is>
+      </c>
+      <c r="K210" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés algo que tu pareja no sabe, buscá el momento para contárselo con humildad.</t>
+        </is>
+      </c>
+      <c r="L210" s="61" t="inlineStr">
+        <is>
+          <t>Unidad no es que uno decida y el otro obedezca. Ninguno de los dos debería usar la plata para dominar al otro.</t>
+        </is>
+      </c>
+      <c r="M210" s="61" t="inlineStr">
+        <is>
+          <t>Que uno controle todo el dinero y el otro tenga que pedir permiso hasta para lo mínimo.</t>
+        </is>
+      </c>
+      <c r="N210" s="61" t="inlineStr">
+        <is>
+          <t>Revisen juntos el presupuesto del mes, y que los dos tengan voz en las decisiones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="61" t="n">
+        <v>35</v>
+      </c>
+      <c r="B211" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C211" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: la plata de la casa</t>
+        </is>
+      </c>
+      <c r="D211" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribió estas palabras preso, agradeciendo una ofrenda que la iglesia de Filipos le había enviado.</t>
+        </is>
+      </c>
+      <c r="E211" s="61" t="inlineStr">
+        <is>
+          <t>Filipenses 1:13; 4:10-18</t>
+        </is>
+      </c>
+      <c r="F211" s="61" t="inlineStr">
+        <is>
+          <t>Administrar juntos, sin plata escondida, es remar hacia el mismo lado.</t>
+        </is>
+      </c>
+      <c r="G211" s="61" t="n"/>
+      <c r="H211" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, tengan en familia una conversación sobre la plata: qué tenemos, qué necesitamos y en qué estamos de acuerdo.</t>
+        </is>
+      </c>
+      <c r="I211" s="61" t="inlineStr">
+        <is>
+          <t>Los hijos aprenden sobre el dinero mirando cómo lo vivimos y decidiendo con su propia plata.</t>
+        </is>
+      </c>
+      <c r="J211" s="61" t="n"/>
+      <c r="K211" s="61" t="n"/>
+      <c r="L211" s="61" t="inlineStr">
+        <is>
+          <t>La transparencia y el acuerdo fortalecen la familia más que el monto que se gana.</t>
+        </is>
+      </c>
+      <c r="M211" s="61" t="n"/>
+      <c r="N211" s="61" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="B212" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C212" s="61" t="inlineStr">
+        <is>
+          <t>Una muralla para el alma</t>
+        </is>
+      </c>
+      <c r="D212" s="61" t="inlineStr">
+        <is>
+          <t>En la antigüedad, una ciudad sin muralla quedaba expuesta a cualquier ataque; por eso Nehemías se dedicó a reconstruir los muros de Jerusalén.</t>
+        </is>
+      </c>
+      <c r="E212" s="61" t="inlineStr">
+        <is>
+          <t>Nehemías 1:3; 2:17</t>
+        </is>
+      </c>
+      <c r="F212" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio compara a la persona sin dominio propio con una ciudad sin muralla. La motivación va y viene; el dominio propio sostiene cuando las ganas no están.</t>
+        </is>
+      </c>
+      <c r="G212" s="61" t="inlineStr">
+        <is>
+          <t>Hacer las cosas solo cuando hay ganas.</t>
+        </is>
+      </c>
+      <c r="H212" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una tarea que venís postergando y hacela hoy, aunque no tengas ganas.</t>
+        </is>
+      </c>
+      <c r="I212" s="61" t="inlineStr">
+        <is>
+          <t>El dominio propio es parte del fruto del Espíritu (Gálatas 5:22-23): no es solo fuerza de voluntad, sino obra de Dios en nosotros.</t>
+        </is>
+      </c>
+      <c r="J212" s="61" t="inlineStr">
+        <is>
+          <t>Creer que la disciplina depende solo de uno y frustrarse al fallar.</t>
+        </is>
+      </c>
+      <c r="K212" s="61" t="inlineStr">
+        <is>
+          <t>Pedile hoy a Dios ayuda en un área donde te cuesta tener dominio propio.</t>
+        </is>
+      </c>
+      <c r="L212" s="61" t="inlineStr">
+        <is>
+          <t>Está bien no tener ganas algunos días: la disciplina existe justamente para esos días.</t>
+        </is>
+      </c>
+      <c r="M212" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar todo el primer día que falta la motivación.</t>
+        </is>
+      </c>
+      <c r="N212" s="61" t="inlineStr">
+        <is>
+          <t>Decidí hoy qué vas a hacer el día que no tengas ganas, antes de que llegue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="B213" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C213" s="61" t="inlineStr">
+        <is>
+          <t>Constantes</t>
+        </is>
+      </c>
+      <c r="D213" s="61" t="inlineStr">
+        <is>
+          <t>Un estudio encontró que cerca del 43 % de lo que hacemos cada día lo hacemos por hábito, casi sin pensar.</t>
+        </is>
+      </c>
+      <c r="E213" s="61" t="inlineStr">
+        <is>
+          <t>Wood, Quinn y Kashy, Journal of Personality and Social Psychology, 2002</t>
+        </is>
+      </c>
+      <c r="F213" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide dedicarse a la oración. La constancia no nace de un sentimiento, sino de una decisión que se repite.</t>
+        </is>
+      </c>
+      <c r="G213" s="61" t="inlineStr">
+        <is>
+          <t>Orar solo cuando algo sale mal.</t>
+        </is>
+      </c>
+      <c r="H213" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una hora fija para orar cada día esta semana.</t>
+        </is>
+      </c>
+      <c r="I213" s="61" t="inlineStr">
+        <is>
+          <t>Gran parte de lo que hacemos cada día lo hacemos por hábito. Por eso vale la pena elegir bien los hábitos.</t>
+        </is>
+      </c>
+      <c r="J213" s="61" t="inlineStr">
+        <is>
+          <t>Vivir en piloto automático, con hábitos que nunca elegimos.</t>
+        </is>
+      </c>
+      <c r="K213" s="61" t="inlineStr">
+        <is>
+          <t>Anotá tres cosas que hacés todos los días sin pensar, y preguntate si te ayudan.</t>
+        </is>
+      </c>
+      <c r="L213" s="61" t="inlineStr">
+        <is>
+          <t>Pablo une la constancia con la gratitud. Agradecer cada día también es un hábito que cambia la mirada.</t>
+        </is>
+      </c>
+      <c r="M213" s="61" t="inlineStr">
+        <is>
+          <t>Fijarse solo en lo que falta.</t>
+        </is>
+      </c>
+      <c r="N213" s="61" t="inlineStr">
+        <is>
+          <t>Antes de dormir, anotá tres cosas por las que das gracias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="B214" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C214" s="61" t="inlineStr">
+        <is>
+          <t>La mano diligente</t>
+        </is>
+      </c>
+      <c r="D214" s="61" t="inlineStr">
+        <is>
+          <t>Un hábito se forma repitiendo una acción en el mismo contexto: hacerla a la misma hora o en el mismo lugar ayuda a que salga casi sin pensar.</t>
+        </is>
+      </c>
+      <c r="E214" s="61" t="inlineStr">
+        <is>
+          <t>Gardner, Lally y Wardle, British Journal of General Practice, 2012</t>
+        </is>
+      </c>
+      <c r="F214" s="61" t="inlineStr">
+        <is>
+          <t>Este proverbio enseña un principio: la diligencia suele abrir puertas. No dice que todo el que está abajo sea perezoso.</t>
+        </is>
+      </c>
+      <c r="G214" s="61" t="inlineStr">
+        <is>
+          <t>Esperar resultados sin constancia.</t>
+        </is>
+      </c>
+      <c r="H214" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un solo hábito nuevo y fijale una hora y un lugar.</t>
+        </is>
+      </c>
+      <c r="I214" s="61" t="inlineStr">
+        <is>
+          <t>La mayoría de los hábitos se abandonan en las primeras semanas, cuando se acaba la novedad. Ahí está la prueba.</t>
+        </is>
+      </c>
+      <c r="J214" s="61" t="inlineStr">
+        <is>
+          <t>Empezar con entusiasmo y dejar a la semana.</t>
+        </is>
+      </c>
+      <c r="K214" s="61" t="inlineStr">
+        <is>
+          <t>Si dejaste un hábito, retomalo hoy sin culparte: un día perdido no borra el camino.</t>
+        </is>
+      </c>
+      <c r="L214" s="61" t="inlineStr">
+        <is>
+          <t>La confianza de los demás se gana con constancia. El que cumple en lo pequeño es creíble en lo grande.</t>
+        </is>
+      </c>
+      <c r="M214" s="61" t="inlineStr">
+        <is>
+          <t>Prometer mucho y sostener poco.</t>
+        </is>
+      </c>
+      <c r="N214" s="61" t="inlineStr">
+        <is>
+          <t>Marcá en un calendario cada día que cumplís tu hábito, y mirá cómo crece la cadena.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="B215" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C215" s="61" t="inlineStr">
+        <is>
+          <t>Entrenarse</t>
+        </is>
+      </c>
+      <c r="D215" s="61" t="inlineStr">
+        <is>
+          <t>La palabra griega que Pablo usa para «ejercítate» es la raíz de nuestra palabra «gimnasio».</t>
+        </is>
+      </c>
+      <c r="E215" s="61" t="inlineStr">
+        <is>
+          <t>1 Timoteo 4:7; léxico griego de Strong (G1128, gymnázo)</t>
+        </is>
+      </c>
+      <c r="F215" s="61" t="inlineStr">
+        <is>
+          <t>Pablo usa la imagen del atleta. La vida espiritual también se entrena: lectura, oración y servicio, repetidos con paciencia.</t>
+        </is>
+      </c>
+      <c r="G215" s="61" t="inlineStr">
+        <is>
+          <t>Esperar crecer en la fe sin ningún hábito espiritual.</t>
+        </is>
+      </c>
+      <c r="H215" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un hábito espiritual pequeño, como leer un capítulo por día, y sostenelo esta semana.</t>
+        </is>
+      </c>
+      <c r="I215" s="61" t="inlineStr">
+        <is>
+          <t>Pablo no desprecia el ejercicio: dice que aprovecha poco comparado con la piedad, que vale para esta vida y para la venidera. Las dos cosas tienen su lugar.</t>
+        </is>
+      </c>
+      <c r="J215" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar mucho el cuerpo y descuidar el alma, o al revés.</t>
+        </is>
+      </c>
+      <c r="K215" s="61" t="inlineStr">
+        <is>
+          <t>Pensá cómo podés cuidar esta semana tanto tu cuerpo como tu vida con Dios.</t>
+        </is>
+      </c>
+      <c r="L215" s="61" t="inlineStr">
+        <is>
+          <t>Nadie corre una maratón el primer día. Los hábitos se construyen de a poco, sin la presión de hacerlo perfecto desde el inicio.</t>
+        </is>
+      </c>
+      <c r="M215" s="61" t="inlineStr">
+        <is>
+          <t>Querer cambiar todo de golpe y abandonar a los pocos días.</t>
+        </is>
+      </c>
+      <c r="N215" s="61" t="inlineStr">
+        <is>
+          <t>Empezá tan pequeño que no puedas fallar: cinco minutos alcanzan para empezar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="B216" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C216" s="61" t="inlineStr">
+        <is>
+          <t>A su tiempo</t>
+        </is>
+      </c>
+      <c r="D216" s="61" t="inlineStr">
+        <is>
+          <t>Leer diez páginas por día suma más de 3.600 páginas en un año: casi quince libros de 250 páginas.</t>
+        </is>
+      </c>
+      <c r="E216" s="61" t="inlineStr">
+        <is>
+          <t>Cálculo simple</t>
+        </is>
+      </c>
+      <c r="F216" s="61" t="inlineStr">
+        <is>
+          <t>Pablo anima a no cansarse. Un hábito pequeño parece insignificante hoy, pero sostenido durante años produce un cambio que ningún esfuerzo grande logra solo.</t>
+        </is>
+      </c>
+      <c r="G216" s="61" t="inlineStr">
+        <is>
+          <t>Despreciar lo pequeño porque no se nota.</t>
+        </is>
+      </c>
+      <c r="H216" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un solo hábito pequeño para sostener todo este mes.</t>
+        </is>
+      </c>
+      <c r="I216" s="61" t="inlineStr">
+        <is>
+          <t>Es un principio, no un calendario: Dios da el fruto a su tiempo, que no siempre es el nuestro.</t>
+        </is>
+      </c>
+      <c r="J216" s="61" t="inlineStr">
+        <is>
+          <t>Medir el valor de un hábito por los resultados de la primera semana.</t>
+        </is>
+      </c>
+      <c r="K216" s="61" t="inlineStr">
+        <is>
+          <t>Escribí por qué querés este hábito, para leerlo el día que no veas resultados.</t>
+        </is>
+      </c>
+      <c r="L216" s="61" t="inlineStr">
+        <is>
+          <t>Como el agua que corta la roca gota a gota, la constancia logra lo que la fuerza de un momento no puede.</t>
+        </is>
+      </c>
+      <c r="M216" s="61" t="inlineStr">
+        <is>
+          <t>Una lista larga de propósitos que no se cumple.</t>
+        </is>
+      </c>
+      <c r="N216" s="61" t="inlineStr">
+        <is>
+          <t>En vez de diez propósitos, quedate con uno solo y cumplilo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="61" t="n">
+        <v>36</v>
+      </c>
+      <c r="B217" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C217" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: pequeños hábitos, grandes cambios</t>
+        </is>
+      </c>
+      <c r="D217" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios dedica varios dichos a la hormiga y al perezoso como ejemplos de constancia y de descuido.</t>
+        </is>
+      </c>
+      <c r="E217" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 6:6-11; 24:30-34</t>
+        </is>
+      </c>
+      <c r="F217" s="61" t="inlineStr">
+        <is>
+          <t>La motivación va y viene; el dominio propio, fruto del Espíritu, sostiene cuando faltan las ganas.</t>
+        </is>
+      </c>
+      <c r="G217" s="61" t="n"/>
+      <c r="H217" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, elegí un solo hábito pequeño, fijale hora y lugar, y marcá en un calendario cada día que lo cumplas.</t>
+        </is>
+      </c>
+      <c r="I217" s="61" t="inlineStr">
+        <is>
+          <t>Los hábitos se forman repitiendo en el mismo contexto, y la prueba está en las primeras semanas.</t>
+        </is>
+      </c>
+      <c r="J217" s="61" t="n"/>
+      <c r="K217" s="61" t="n"/>
+      <c r="L217" s="61" t="inlineStr">
+        <is>
+          <t>Lo pequeño sostenido en el tiempo logra lo que ningún esfuerzo puntual puede.</t>
+        </is>
+      </c>
+      <c r="M217" s="61" t="n"/>
+      <c r="N217" s="61" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="61" t="n">
+        <v>37</v>
+      </c>
+      <c r="B218" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C218" s="61" t="inlineStr">
+        <is>
+          <t>Un mismo sentir</t>
+        </is>
+      </c>
+      <c r="D218" s="61" t="inlineStr">
+        <is>
+          <t>En Paraguay, más de un millón de personas son socias de alguna cooperativa, según el Instituto Nacional de Cooperativismo (INCOOP).</t>
+        </is>
+      </c>
+      <c r="E218" s="61" t="inlineStr">
+        <is>
+          <t>Instituto Nacional de Cooperativismo (INCOOP)</t>
+        </is>
+      </c>
+      <c r="F218" s="61" t="inlineStr">
+        <is>
+          <t>La primera iglesia compartía sus bienes para que nadie pasara necesidad (4:34). Hay metas imposibles para uno solo y alcanzables cuando varios se organizan.</t>
+        </is>
+      </c>
+      <c r="G218" s="61" t="inlineStr">
+        <is>
+          <t>Querer resolver todo solo, por orgullo o por desconfianza.</t>
+        </is>
+      </c>
+      <c r="H218" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en una necesidad de tu barrio o de tu trabajo que se podría resolver mejor entre varios.</t>
+        </is>
+      </c>
+      <c r="I218" s="61" t="inlineStr">
+        <is>
+          <t>Antes de compartir bienes, compartían un mismo sentir. Lo que sostiene a un grupo no es solo el interés económico, sino la confianza.</t>
+        </is>
+      </c>
+      <c r="J218" s="61" t="inlineStr">
+        <is>
+          <t>Grupos que se juntan solo por conveniencia y se rompen al primer problema.</t>
+        </is>
+      </c>
+      <c r="K218" s="61" t="inlineStr">
+        <is>
+          <t>Si sos parte de un grupo o de una cooperativa, conocé a alguien del grupo más allá de los negocios.</t>
+        </is>
+      </c>
+      <c r="L218" s="61" t="inlineStr">
+        <is>
+          <t>Pedro le aclara a Ananías que su propiedad era suya y podía disponer de ella (5:4): compartir era voluntario. La Biblia no impone un sistema económico, pero sí muestra el valor de cuidarnos entre todos.</t>
+        </is>
+      </c>
+      <c r="M218" s="61" t="inlineStr">
+        <is>
+          <t>Usar este pasaje para imponer o para atacar un modelo económico.</t>
+        </is>
+      </c>
+      <c r="N218" s="61" t="inlineStr">
+        <is>
+          <t>Elegí algo que tengas y puedas compartir esta semana con alguien que lo necesite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="61" t="n">
+        <v>37</v>
+      </c>
+      <c r="B219" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C219" s="61" t="inlineStr">
+        <is>
+          <t>Cada uno con su don</t>
+        </is>
+      </c>
+      <c r="D219" s="61" t="inlineStr">
+        <is>
+          <t>La primera cooperativa moderna se considera la de los Pioneros de Rochdale, en Inglaterra, fundada en 1844.</t>
+        </is>
+      </c>
+      <c r="E219" s="61" t="inlineStr">
+        <is>
+          <t>Alianza Cooperativa Internacional</t>
+        </is>
+      </c>
+      <c r="F219" s="61" t="inlineStr">
+        <is>
+          <t>Pedro pone el amor por encima de todo. En un grupo, el amor cubre las faltas pequeñas y evita que cada error se vuelva pelea.</t>
+        </is>
+      </c>
+      <c r="G219" s="61" t="inlineStr">
+        <is>
+          <t>Grupos que se desarman por roces menores.</t>
+        </is>
+      </c>
+      <c r="H219" s="61" t="inlineStr">
+        <is>
+          <t>Perdoná hoy un roce pequeño con alguien de tu grupo, sin hacer de eso un problema.</t>
+        </is>
+      </c>
+      <c r="I219" s="61" t="inlineStr">
+        <is>
+          <t>Hospedarse sin quejarse: la generosidad en lo cotidiano sostiene la vida en comunidad.</t>
+        </is>
+      </c>
+      <c r="J219" s="61" t="inlineStr">
+        <is>
+          <t>Participar solo para recibir, nunca para dar.</t>
+        </is>
+      </c>
+      <c r="K219" s="61" t="inlineStr">
+        <is>
+          <t>Ofrecé tu ayuda en la próxima actividad de tu comunidad.</t>
+        </is>
+      </c>
+      <c r="L219" s="61" t="inlineStr">
+        <is>
+          <t>Cada uno recibió un don para servir a los demás. Juntos, los dones de todos logran lo que ninguno logra solo.</t>
+        </is>
+      </c>
+      <c r="M219" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que lo que yo sé hacer no le sirve a nadie.</t>
+        </is>
+      </c>
+      <c r="N219" s="61" t="inlineStr">
+        <is>
+          <t>Anotá un don o una habilidad que tenés, y cómo podría servir a tu grupo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="61" t="n">
+        <v>37</v>
+      </c>
+      <c r="B220" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C220" s="61" t="inlineStr">
+        <is>
+          <t>Qué bueno es convivir</t>
+        </is>
+      </c>
+      <c r="D220" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 133 es uno de los «cánticos de las subidas», que los peregrinos cantaban camino a Jerusalén.</t>
+        </is>
+      </c>
+      <c r="E220" s="61" t="inlineStr">
+        <is>
+          <t>Salmos 120 a 134 (títulos)</t>
+        </is>
+      </c>
+      <c r="F220" s="61" t="inlineStr">
+        <is>
+          <t>El salmo celebra la unidad de los hermanos. Una cooperativa funciona cuando cada socio entiende que el bien de todos sostiene también el propio.</t>
+        </is>
+      </c>
+      <c r="G220" s="61" t="inlineStr">
+        <is>
+          <t>Socios que solo piensan en su beneficio inmediato.</t>
+        </is>
+      </c>
+      <c r="H220" s="61" t="inlineStr">
+        <is>
+          <t>Si sos socio de una cooperativa, participá de la próxima asamblea.</t>
+        </is>
+      </c>
+      <c r="I220" s="61" t="inlineStr">
+        <is>
+          <t>Dicho simple: en una cooperativa, los socios son a la vez dueños y usuarios, y cada socio tiene un voto, sin importar cuánto aportó.</t>
+        </is>
+      </c>
+      <c r="J220" s="61" t="inlineStr">
+        <is>
+          <t>No entender cómo funciona el grupo del que uno es parte.</t>
+        </is>
+      </c>
+      <c r="K220" s="61" t="inlineStr">
+        <is>
+          <t>Averiguá cómo se toman las decisiones en tu cooperativa o en tu grupo.</t>
+        </is>
+      </c>
+      <c r="L220" s="61" t="inlineStr">
+        <is>
+          <t>No es caridad: es reconocer que juntos se llega más lejos que compitiendo aislados. Y eso pide respeto y paz entre todos.</t>
+        </is>
+      </c>
+      <c r="M220" s="61" t="inlineStr">
+        <is>
+          <t>Hablar mal de los dirigentes sin participar nunca.</t>
+        </is>
+      </c>
+      <c r="N220" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés una crítica, llevala a la asamblea con respeto, en vez de quejarte por los pasillos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="61" t="n">
+        <v>37</v>
+      </c>
+      <c r="B221" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C221" s="61" t="inlineStr">
+        <is>
+          <t>Vivan en paz</t>
+        </is>
+      </c>
+      <c r="D221" s="61" t="inlineStr">
+        <is>
+          <t>Los principios cooperativos de la Alianza Cooperativa Internacional son siete; entre ellos, el control democrático de los socios y el compromiso con la comunidad.</t>
+        </is>
+      </c>
+      <c r="E221" s="61" t="inlineStr">
+        <is>
+          <t>Alianza Cooperativa Internacional, Declaración sobre la Identidad Cooperativa, 1995</t>
+        </is>
+      </c>
+      <c r="F221" s="61" t="inlineStr">
+        <is>
+          <t>Pablo cierra una carta difícil con alegría. Trabajar juntos tiene tensiones, pero también la alegría de lograr algo entre todos.</t>
+        </is>
+      </c>
+      <c r="G221" s="61" t="inlineStr">
+        <is>
+          <t>Ver solo los problemas del grupo y nunca celebrar los logros.</t>
+        </is>
+      </c>
+      <c r="H221" s="61" t="inlineStr">
+        <is>
+          <t>Celebrá con tu grupo un logro reciente, aunque sea pequeño.</t>
+        </is>
+      </c>
+      <c r="I221" s="61" t="inlineStr">
+        <is>
+          <t>Tener un mismo sentir no es pensar igual en todo, sino buscar juntos el bien común y vivir en paz.</t>
+        </is>
+      </c>
+      <c r="J221" s="61" t="inlineStr">
+        <is>
+          <t>Divisiones por diferencias que no son lo esencial.</t>
+        </is>
+      </c>
+      <c r="K221" s="61" t="inlineStr">
+        <is>
+          <t>En la próxima reunión, escuchá con atención a alguien que piensa distinto.</t>
+        </is>
+      </c>
+      <c r="L221" s="61" t="inlineStr">
+        <is>
+          <t>El Dios de la paz y del amor acompaña a los que buscan la paz. La unidad es un regalo que se cuida.</t>
+        </is>
+      </c>
+      <c r="M221" s="61" t="inlineStr">
+        <is>
+          <t>Creer que la unidad depende solo de nuestra habilidad para organizarnos.</t>
+        </is>
+      </c>
+      <c r="N221" s="61" t="inlineStr">
+        <is>
+          <t>Orá esta semana por tu cooperativa, tu grupo o tu comunidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="61" t="n">
+        <v>37</v>
+      </c>
+      <c r="B222" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C222" s="61" t="inlineStr">
+        <is>
+          <t>Lo que es de todos</t>
+        </is>
+      </c>
+      <c r="D222" s="61" t="inlineStr">
+        <is>
+          <t>Pablo compara a la iglesia con un cuerpo, en el que ningún miembro puede decirle a otro que no lo necesita.</t>
+        </is>
+      </c>
+      <c r="E222" s="61" t="inlineStr">
+        <is>
+          <t>1 Corintios 12:21</t>
+        </is>
+      </c>
+      <c r="F222" s="61" t="inlineStr">
+        <is>
+          <t>Pablo habla de la iglesia como un cuerpo, y el principio vale para todo grupo. Cuando un recurso es de todos, la tentación de aprovecharse existe siempre.</t>
+        </is>
+      </c>
+      <c r="G222" s="61" t="inlineStr">
+        <is>
+          <t>Usar lo que es de todos como si fuera propio.</t>
+        </is>
+      </c>
+      <c r="H222" s="61" t="inlineStr">
+        <is>
+          <t>Si manejás algo de un grupo, plata o herramientas, rendí cuentas aunque nadie te lo pida.</t>
+        </is>
+      </c>
+      <c r="I222" s="61" t="inlineStr">
+        <is>
+          <t>La honestidad en lo colectivo sostiene la confianza. La transparencia en las cuentas es la base de cualquier grupo sano.</t>
+        </is>
+      </c>
+      <c r="J222" s="61" t="inlineStr">
+        <is>
+          <t>Cuentas que nadie entiende y nadie revisa.</t>
+        </is>
+      </c>
+      <c r="K222" s="61" t="inlineStr">
+        <is>
+          <t>Pedí que las cuentas de tu grupo se presenten claras y a todos.</t>
+        </is>
+      </c>
+      <c r="L222" s="61" t="inlineStr">
+        <is>
+          <t>Si uno sufre, todos sufren; si a uno lo honran, todos se alegran. Un grupo honesto acompaña en las malas y celebra en las buenas.</t>
+        </is>
+      </c>
+      <c r="M222" s="61" t="inlineStr">
+        <is>
+          <t>Grupos que solo funcionan cuando hay ganancias.</t>
+        </is>
+      </c>
+      <c r="N222" s="61" t="inlineStr">
+        <is>
+          <t>Acercate a alguien de tu grupo que esté pasando un momento difícil.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="61" t="n">
+        <v>37</v>
+      </c>
+      <c r="B223" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C223" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: juntos llegamos más lejos</t>
+        </is>
+      </c>
+      <c r="D223" s="61" t="inlineStr">
+        <is>
+          <t>La Constitución del Paraguay establece que el Estado promoverá el cooperativismo.</t>
+        </is>
+      </c>
+      <c r="E223" s="61" t="inlineStr">
+        <is>
+          <t>Constitución Nacional del Paraguay, 1992, artículo 113</t>
+        </is>
+      </c>
+      <c r="F223" s="61" t="inlineStr">
+        <is>
+          <t>Hay metas imposibles para uno solo y alcanzables cuando varios se organizan, y lo que sostiene al grupo es la confianza.</t>
+        </is>
+      </c>
+      <c r="G223" s="61" t="n"/>
+      <c r="H223" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, participá en algo de tu cooperativa, tu iglesia o tu barrio, y ofrecé lo que sabés hacer.</t>
+        </is>
+      </c>
+      <c r="I223" s="61" t="inlineStr">
+        <is>
+          <t>Una cooperativa funciona cuando cada socio entiende que el bien de todos sostiene también el propio.</t>
+        </is>
+      </c>
+      <c r="J223" s="61" t="n"/>
+      <c r="K223" s="61" t="n"/>
+      <c r="L223" s="61" t="inlineStr">
+        <is>
+          <t>Lo que es de todos se cuida con honestidad y con cuentas claras.</t>
+        </is>
+      </c>
+      <c r="M223" s="61" t="n"/>
+      <c r="N223" s="61" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="61" t="n">
+        <v>38</v>
+      </c>
+      <c r="B224" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C224" s="61" t="inlineStr">
+        <is>
+          <t>Desde la niñez</t>
+        </is>
+      </c>
+      <c r="D224" s="61" t="inlineStr">
+        <is>
+          <t>En Paraguay, las vacunas del esquema regular son gratuitas en los servicios del Ministerio de Salud.</t>
+        </is>
+      </c>
+      <c r="E224" s="61" t="inlineStr">
+        <is>
+          <t>Ministerio de Salud Pública y Bienestar Social, Programa Ampliado de Inmunizaciones</t>
+        </is>
+      </c>
+      <c r="F224" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés invita a acordarse del Creador desde joven. Lo que se siembra en la niñez acompaña toda la vida, en la fe y en la salud.</t>
+        </is>
+      </c>
+      <c r="G224" s="61" t="inlineStr">
+        <is>
+          <t>Dejar la fe y la salud de los hijos para «cuando sean grandes».</t>
+        </is>
+      </c>
+      <c r="H224" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, compartí con tus hijos un momento de oración o una lectura bíblica corta.</t>
+        </is>
+      </c>
+      <c r="I224" s="61" t="inlineStr">
+        <is>
+          <t>Los hábitos de la niñez, la comida, el juego al aire libre y el descanso, sientan una base que dura décadas.</t>
+        </is>
+      </c>
+      <c r="J224" s="61" t="inlineStr">
+        <is>
+          <t>Niños que pasan horas frente a pantallas y poco tiempo moviéndose.</t>
+        </is>
+      </c>
+      <c r="K224" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, salgan a jugar o a caminar en familia al menos una vez.</t>
+        </is>
+      </c>
+      <c r="L224" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar la salud de los chicos no es solo ir al médico cuando se enferman: los controles regulares previenen.</t>
+        </is>
+      </c>
+      <c r="M224" s="61" t="inlineStr">
+        <is>
+          <t>Llevar a los chicos al médico solo cuando ya están enfermos.</t>
+        </is>
+      </c>
+      <c r="N224" s="61" t="inlineStr">
+        <is>
+          <t>Revisá la libreta de vacunas y controles de tus hijos y agendá lo que falte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="61" t="n">
+        <v>38</v>
+      </c>
+      <c r="B225" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C225" s="61" t="inlineStr">
+        <is>
+          <t>Crecer en todo</t>
+        </is>
+      </c>
+      <c r="D225" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, 21 de septiembre, Paraguay celebra el Día de la Juventud, junto con el inicio de la primavera.</t>
+        </is>
+      </c>
+      <c r="E225" s="61" t="inlineStr">
+        <is>
+          <t>Fechas conmemorativas del Paraguay</t>
+        </is>
+      </c>
+      <c r="F225" s="61" t="inlineStr">
+        <is>
+          <t>Lucas resume la niñez y la juventud de Jesús: creció en sabiduría, en estatura y en gracia. El crecimiento sano es integral.</t>
+        </is>
+      </c>
+      <c r="G225" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar solo las notas del colegio y no el corazón.</t>
+        </is>
+      </c>
+      <c r="H225" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale a tu hijo qué aprendió esta semana, más allá del colegio.</t>
+        </is>
+      </c>
+      <c r="I225" s="61" t="inlineStr">
+        <is>
+          <t>Crecer en estatura incluye el cuerpo: comer bien, moverse y dormir lo suficiente.</t>
+        </is>
+      </c>
+      <c r="J225" s="61" t="inlineStr">
+        <is>
+          <t>Comidas rápidas como costumbre diaria.</t>
+        </is>
+      </c>
+      <c r="K225" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, preparen en familia una comida casera con verduras.</t>
+        </is>
+      </c>
+      <c r="L225" s="61" t="inlineStr">
+        <is>
+          <t>También se crece en las relaciones, con Dios y con la gente. Un niño querido y acompañado crece más sano.</t>
+        </is>
+      </c>
+      <c r="M225" s="61" t="inlineStr">
+        <is>
+          <t>Chicos solos frente al celular mientras los adultos están ocupados.</t>
+        </is>
+      </c>
+      <c r="N225" s="61" t="inlineStr">
+        <is>
+          <t>Regalale hoy a un niño de tu familia media hora de atención sin pantallas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="61" t="n">
+        <v>38</v>
+      </c>
+      <c r="B226" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C226" s="61" t="inlineStr">
+        <is>
+          <t>Desde mi juventud</t>
+        </is>
+      </c>
+      <c r="D226" s="61" t="inlineStr">
+        <is>
+          <t>Según la Organización Mundial de la Salud, uno de cada siete adolescentes de 10 a 19 años vive con algún trastorno mental.</t>
+        </is>
+      </c>
+      <c r="E226" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, nota descriptiva sobre la salud mental de los adolescentes</t>
+        </is>
+      </c>
+      <c r="F226" s="61" t="inlineStr">
+        <is>
+          <t>El salmista recuerda que Dios lo acompañó desde la juventud. La adolescencia es una etapa de cambios rápidos, y Dios acompaña también ahí.</t>
+        </is>
+      </c>
+      <c r="G226" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que los adolescentes «están bien» solo porque tienen energía.</t>
+        </is>
+      </c>
+      <c r="H226" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale a un adolescente de tu casa cómo se siente, y escuchá sin juzgar.</t>
+        </is>
+      </c>
+      <c r="I226" s="61" t="inlineStr">
+        <is>
+          <t>El salmista quiere contar a las nuevas generaciones lo que Dios hizo. Los jóvenes necesitan adultos que los acompañen y les hablen con verdad.</t>
+        </is>
+      </c>
+      <c r="J226" s="61" t="inlineStr">
+        <is>
+          <t>Adultos que solo critican a los jóvenes.</t>
+        </is>
+      </c>
+      <c r="K226" s="61" t="inlineStr">
+        <is>
+          <t>Contale a un joven cómo Dios te acompañó cuando tenías su edad.</t>
+        </is>
+      </c>
+      <c r="L226" s="61" t="inlineStr">
+        <is>
+          <t>La salud mental en la adolescencia merece atención. La tristeza que no pasa, el aislamiento o los cambios bruscos son señales para buscar ayuda, sin vergüenza.</t>
+        </is>
+      </c>
+      <c r="M226" s="61" t="inlineStr">
+        <is>
+          <t>Minimizar lo que sienten los adolescentes: «son cosas de la edad».</t>
+        </is>
+      </c>
+      <c r="N226" s="61" t="inlineStr">
+        <is>
+          <t>Si ves señales de alarma en un adolescente, buscá ayuda profesional; en Paraguay, la línea gratuita 147 «Fono Ayuda» orienta sobre niños y adolescentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="61" t="n">
+        <v>38</v>
+      </c>
+      <c r="B227" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C227" s="61" t="inlineStr">
+        <is>
+          <t>Cada etapa tiene su valor</t>
+        </is>
+      </c>
+      <c r="D227" s="61" t="inlineStr">
+        <is>
+          <t>Los especialistas recomiendan que los adolescentes de 13 a 18 años duerman entre 8 y 10 horas por noche.</t>
+        </is>
+      </c>
+      <c r="E227" s="61" t="inlineStr">
+        <is>
+          <t>American Academy of Sleep Medicine, recomendaciones para niños y adolescentes, 2016</t>
+        </is>
+      </c>
+      <c r="F227" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio celebra la fuerza de la juventud. Esa fuerza es un regalo para cuidar, no para gastar sin medida.</t>
+        </is>
+      </c>
+      <c r="G227" s="61" t="inlineStr">
+        <is>
+          <t>Arriesgarse sin pensar porque «a mí no me va a pasar».</t>
+        </is>
+      </c>
+      <c r="H227" s="61" t="inlineStr">
+        <is>
+          <t>Si sos joven, elegí un hábito de cuidado: dormir mejor, moverte o comer más sano.</t>
+        </is>
+      </c>
+      <c r="I227" s="61" t="inlineStr">
+        <is>
+          <t>Las canas representan experiencia. Los jóvenes crecen mejor cuando escuchan a los mayores, y los mayores cuando valoran a los jóvenes.</t>
+        </is>
+      </c>
+      <c r="J227" s="61" t="inlineStr">
+        <is>
+          <t>Generaciones que no se escuchan.</t>
+        </is>
+      </c>
+      <c r="K227" s="61" t="inlineStr">
+        <is>
+          <t>Organizá una charla entre un joven y un abuelo de tu familia.</t>
+        </is>
+      </c>
+      <c r="L227" s="61" t="inlineStr">
+        <is>
+          <t>Los adolescentes necesitan dormir más de lo que creemos, y las pantallas de noche les roban descanso.</t>
+        </is>
+      </c>
+      <c r="M227" s="61" t="inlineStr">
+        <is>
+          <t>Celulares en la cama hasta la madrugada.</t>
+        </is>
+      </c>
+      <c r="N227" s="61" t="inlineStr">
+        <is>
+          <t>Acuerden en casa una hora para dejar los celulares fuera del dormitorio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="61" t="n">
+        <v>38</v>
+      </c>
+      <c r="B228" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C228" s="61" t="inlineStr">
+        <is>
+          <t>Hasta las canas</t>
+        </is>
+      </c>
+      <c r="D228" s="61" t="inlineStr">
+        <is>
+          <t>La presión alta muchas veces no da síntomas; por eso se recomienda medirla con regularidad.</t>
+        </is>
+      </c>
+      <c r="E228" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, nota descriptiva sobre la hipertensión</t>
+        </is>
+      </c>
+      <c r="F228" s="61" t="inlineStr">
+        <is>
+          <t>Dios le dice a su pueblo que lo llevó desde el nacimiento y lo llevará hasta la vejez. Él no se cansa de cuidarnos, y eso nos anima a cuidarnos también.</t>
+        </is>
+      </c>
+      <c r="G228" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que cuidar la propia salud es egoísmo.</t>
+        </is>
+      </c>
+      <c r="H228" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, hacé algo concreto por tu salud: caminá, tomá agua o comé una fruta.</t>
+        </is>
+      </c>
+      <c r="I228" s="61" t="inlineStr">
+        <is>
+          <t>En la adultez, entre el trabajo y la familia, la propia salud queda al final de la lista. Cuidarla antes de que aparezca una alarma también es amar a los tuyos.</t>
+        </is>
+      </c>
+      <c r="J228" s="61" t="inlineStr">
+        <is>
+          <t>Ir al médico solo cuando ya no se aguanta.</t>
+        </is>
+      </c>
+      <c r="K228" s="61" t="inlineStr">
+        <is>
+          <t>Agendá un control médico general si hace más de un año que no te hacés uno.</t>
+        </is>
+      </c>
+      <c r="L228" s="61" t="inlineStr">
+        <is>
+          <t>Isaías contrasta a Dios con los ídolos, que hay que cargar (46:1-2). Nuestro Dios, en cambio, nos carga a nosotros.</t>
+        </is>
+      </c>
+      <c r="M228" s="61" t="inlineStr">
+        <is>
+          <t>Cargar solos con el peso de cuidar a todos.</t>
+        </is>
+      </c>
+      <c r="N228" s="61" t="inlineStr">
+        <is>
+          <t>Pedí ayuda en casa para tener un tiempo de cuidado propio esta semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="61" t="n">
+        <v>38</v>
+      </c>
+      <c r="B229" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C229" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: la salud en cada etapa</t>
+        </is>
+      </c>
+      <c r="D229" s="61" t="inlineStr">
+        <is>
+          <t>Moisés tenía 80 años cuando habló con el faraón para sacar al pueblo de Egipto.</t>
+        </is>
+      </c>
+      <c r="E229" s="61" t="inlineStr">
+        <is>
+          <t>Éxodo 7:7</t>
+        </is>
+      </c>
+      <c r="F229" s="61" t="inlineStr">
+        <is>
+          <t>En la niñez se siembran hábitos y fe que acompañan toda la vida.</t>
+        </is>
+      </c>
+      <c r="G229" s="61" t="n"/>
+      <c r="H229" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, revisá los controles de salud de cada uno en tu casa, empezando por el tuyo, y agenden lo que falte.</t>
+        </is>
+      </c>
+      <c r="I229" s="61" t="inlineStr">
+        <is>
+          <t>En la adolescencia hay que escuchar sin minimizar y buscar ayuda cuando hace falta.</t>
+        </is>
+      </c>
+      <c r="J229" s="61" t="n"/>
+      <c r="K229" s="61" t="n"/>
+      <c r="L229" s="61" t="inlineStr">
+        <is>
+          <t>En la adultez, cuidar la propia salud también es amar a los tuyos; Dios nos lleva en cada etapa.</t>
+        </is>
+      </c>
+      <c r="M229" s="61" t="n"/>
+      <c r="N229" s="61" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="61" t="n">
+        <v>39</v>
+      </c>
+      <c r="B230" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C230" s="61" t="inlineStr">
+        <is>
+          <t>Obra de Dios</t>
+        </is>
+      </c>
+      <c r="D230" s="61" t="inlineStr">
+        <is>
+          <t>La palabra griega para «obra» en este versículo (poíema) es la raíz de nuestra palabra «poema».</t>
+        </is>
+      </c>
+      <c r="E230" s="61" t="inlineStr">
+        <is>
+          <t>Efesios 2:10; léxico griego de Strong (G4161, poíema)</t>
+        </is>
+      </c>
+      <c r="F230" s="61" t="inlineStr">
+        <is>
+          <t>Justo antes, Pablo dice que somos salvos por gracia y no por obras (2:8-9). Nuestra identidad es un regalo, no un logro.</t>
+        </is>
+      </c>
+      <c r="G230" s="61" t="inlineStr">
+        <is>
+          <t>Vivir según las etiquetas que nos pusieron: «sos un inútil», «nunca vas a cambiar».</t>
+        </is>
+      </c>
+      <c r="H230" s="61" t="inlineStr">
+        <is>
+          <t>Anotá una frase negativa que creés de vos, y al lado lo que Dios dice en Efesios 2:10.</t>
+        </is>
+      </c>
+      <c r="I230" s="61" t="inlineStr">
+        <is>
+          <t>Las buenas obras no son para ganar el amor de Dios, sino la respuesta de quien ya lo recibió.</t>
+        </is>
+      </c>
+      <c r="J230" s="61" t="inlineStr">
+        <is>
+          <t>Hacer el bien para sentirse digno de Dios.</t>
+        </is>
+      </c>
+      <c r="K230" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy una buena obra, no para demostrar nada, sino como respuesta de gratitud.</t>
+        </is>
+      </c>
+      <c r="L230" s="61" t="inlineStr">
+        <is>
+          <t>Dios preparó de antemano esas obras. Lo que vos creés de vos no es la última palabra: la última palabra es lo que Dios ya dijo.</t>
+        </is>
+      </c>
+      <c r="M230" s="61" t="inlineStr">
+        <is>
+          <t>Dejar que la opinión propia, formada por heridas, pese más que la Palabra.</t>
+        </is>
+      </c>
+      <c r="N230" s="61" t="inlineStr">
+        <is>
+          <t>Leé Efesios 2:1-10 completo y subrayá lo que Dios hizo por vos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="61" t="n">
+        <v>39</v>
+      </c>
+      <c r="B231" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C231" s="61" t="inlineStr">
+        <is>
+          <t>Hijo, no esclavo</t>
+        </is>
+      </c>
+      <c r="D231" s="61" t="inlineStr">
+        <is>
+          <t>En el derecho romano, un hijo adoptado pasaba a tener los mismos derechos de herencia que un hijo natural.</t>
+        </is>
+      </c>
+      <c r="E231" s="61" t="inlineStr">
+        <is>
+          <t>Derecho romano (adopción); comentarios a Gálatas 4 y Romanos 8</t>
+        </is>
+      </c>
+      <c r="F231" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribe a creyentes que volvían a vivir como si tuvieran que ganarse el favor de Dios. Él dice: ya no sos esclavo.</t>
+        </is>
+      </c>
+      <c r="G231" s="61" t="inlineStr">
+        <is>
+          <t>Vivir la fe con miedo, como un empleado que teme ser despedido.</t>
+        </is>
+      </c>
+      <c r="H231" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, hablale a Dios como un hijo le habla a su padre.</t>
+        </is>
+      </c>
+      <c r="I231" s="61" t="inlineStr">
+        <is>
+          <t>Como el joven adoptado que seguía escondiendo comida, muchos creyentes tardan en creer que ya son hijos. La identidad se recibe, y después se aprende a vivirla.</t>
+        </is>
+      </c>
+      <c r="J231" s="61" t="inlineStr">
+        <is>
+          <t>Esconder las dudas y los miedos en lugar de llevarlos a Dios.</t>
+        </is>
+      </c>
+      <c r="K231" s="61" t="inlineStr">
+        <is>
+          <t>Nombrá un miedo viejo que todavía te gobierna y entregáselo a Dios.</t>
+        </is>
+      </c>
+      <c r="L231" s="61" t="inlineStr">
+        <is>
+          <t>La herencia no es por mérito, sino por medio de Cristo. Eso da seguridad para vivir sin tener que probar nada.</t>
+        </is>
+      </c>
+      <c r="M231" s="61" t="inlineStr">
+        <is>
+          <t>Compararse con otros creyentes para medir cuánto vale uno.</t>
+        </is>
+      </c>
+      <c r="N231" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy a Dios por algo que recibiste sin merecerlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="61" t="n">
+        <v>39</v>
+      </c>
+      <c r="B232" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C232" s="61" t="inlineStr">
+        <is>
+          <t>Pueblo de Dios</t>
+        </is>
+      </c>
+      <c r="D232" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, 29 de septiembre, Paraguay recuerda la victoria de Boquerón, de 1932, en la Guerra del Chaco.</t>
+        </is>
+      </c>
+      <c r="E232" s="61" t="inlineStr">
+        <is>
+          <t>Batalla de Boquerón, 9 al 29 de septiembre de 1932</t>
+        </is>
+      </c>
+      <c r="F232" s="61" t="inlineStr">
+        <is>
+          <t>Pedro escribe a creyentes despreciados por su fe. Su valor no dependía de la opinión de los demás, sino de que Dios los eligió.</t>
+        </is>
+      </c>
+      <c r="G232" s="61" t="inlineStr">
+        <is>
+          <t>Cambiar de opinión según quién esté mirando.</t>
+        </is>
+      </c>
+      <c r="H232" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en una decisión de esta semana que tomaste por el «qué dirán», y cómo la tomarías hoy.</t>
+        </is>
+      </c>
+      <c r="I232" s="61" t="inlineStr">
+        <is>
+          <t>Buscar la aprobación de todos deja a la persona a merced de opiniones que cambian. La identidad recibida de Dios es una base estable.</t>
+        </is>
+      </c>
+      <c r="J232" s="61" t="inlineStr">
+        <is>
+          <t>Sentirse bien o mal según los «me gusta» de las redes.</t>
+        </is>
+      </c>
+      <c r="K232" s="61" t="inlineStr">
+        <is>
+          <t>Pasá un día sin publicar nada en redes, y fijate cómo te sentís.</t>
+        </is>
+      </c>
+      <c r="L232" s="61" t="inlineStr">
+        <is>
+          <t>El propósito no es lucirnos, sino anunciar lo que Dios hizo: nos llamó de las tinieblas a su luz.</t>
+        </is>
+      </c>
+      <c r="M232" s="61" t="inlineStr">
+        <is>
+          <t>Hacer el bien para que nos vean.</t>
+        </is>
+      </c>
+      <c r="N232" s="61" t="inlineStr">
+        <is>
+          <t>Contale a alguien algo bueno que Dios hizo en tu vida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="61" t="n">
+        <v>39</v>
+      </c>
+      <c r="B233" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C233" s="61" t="inlineStr">
+        <is>
+          <t>Cristo vive en mí</t>
+        </is>
+      </c>
+      <c r="D233" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribió Gálatas para defender que somos aceptados por Dios por la fe en Cristo, y no por cumplir la ley.</t>
+        </is>
+      </c>
+      <c r="E233" s="61" t="inlineStr">
+        <is>
+          <t>Gálatas 2:16</t>
+        </is>
+      </c>
+      <c r="F233" s="61" t="inlineStr">
+        <is>
+          <t>Pablo dice que su viejo yo fue crucificado con Cristo. Quien sabe quién es no necesita demostrarlo todo el tiempo.</t>
+        </is>
+      </c>
+      <c r="G233" s="61" t="inlineStr">
+        <is>
+          <t>Vivir para demostrarles a otros que valemos.</t>
+        </is>
+      </c>
+      <c r="H233" s="61" t="inlineStr">
+        <is>
+          <t>Identificá algo que hacés solo para que te aprueben, y soltalo esta semana.</t>
+        </is>
+      </c>
+      <c r="I233" s="61" t="inlineStr">
+        <is>
+          <t>Una identidad clara filtra las decisiones: qué aceptar, qué rechazar, en qué invertir la energía.</t>
+        </is>
+      </c>
+      <c r="J233" s="61" t="inlineStr">
+        <is>
+          <t>Decir que sí a todo por miedo a decepcionar.</t>
+        </is>
+      </c>
+      <c r="K233" s="61" t="inlineStr">
+        <is>
+          <t>Antes de aceptar un compromiso nuevo, preguntate: ¿esto refleja quién soy en Cristo?</t>
+        </is>
+      </c>
+      <c r="L233" s="61" t="inlineStr">
+        <is>
+          <t>El centro está en «me amó y se entregó a sí mismo por mí». Las decisiones nacen de ese amor, no de la ansiedad de probar algo.</t>
+        </is>
+      </c>
+      <c r="M233" s="61" t="inlineStr">
+        <is>
+          <t>Decidir desde el miedo a fallar.</t>
+        </is>
+      </c>
+      <c r="N233" s="61" t="inlineStr">
+        <is>
+          <t>Antes de una decisión importante, recordá en voz alta: «Cristo me amó y se entregó por mí».</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="61" t="n">
+        <v>39</v>
+      </c>
+      <c r="B234" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C234" s="61" t="inlineStr">
+        <is>
+          <t>Hijos y herederos</t>
+        </is>
+      </c>
+      <c r="D234" s="61" t="inlineStr">
+        <is>
+          <t>Romanos 8 empieza diciendo que ya no hay condenación para los que están en Cristo Jesús.</t>
+        </is>
+      </c>
+      <c r="E234" s="61" t="inlineStr">
+        <is>
+          <t>Romanos 8:1</t>
+        </is>
+      </c>
+      <c r="F234" s="61" t="inlineStr">
+        <is>
+          <t>La seguridad de ser hijos no depende de cómo nos sentimos hoy: el Espíritu mismo da testimonio.</t>
+        </is>
+      </c>
+      <c r="G234" s="61" t="inlineStr">
+        <is>
+          <t>Dudar de ser hijo de Dios cada vez que fallamos.</t>
+        </is>
+      </c>
+      <c r="H234" s="61" t="inlineStr">
+        <is>
+          <t>Cuando falles esta semana, recordá «sigo siendo hijo de Dios», y pedí perdón con confianza.</t>
+        </is>
+      </c>
+      <c r="I234" s="61" t="inlineStr">
+        <is>
+          <t>Ser coherederos con Cristo incluye también compartir sus sufrimientos (8:17). Ser hijo no promete una vida sin problemas, sino compañía y esperanza.</t>
+        </is>
+      </c>
+      <c r="J234" s="61" t="inlineStr">
+        <is>
+          <t>Creer que si sos hijo de Dios no deberías sufrir.</t>
+        </is>
+      </c>
+      <c r="K234" s="61" t="inlineStr">
+        <is>
+          <t>Si estás pasando un momento difícil, leé Romanos 8:28-39.</t>
+        </is>
+      </c>
+      <c r="L234" s="61" t="inlineStr">
+        <is>
+          <t>Quien se sabe hijo decide con libertad: puede decir que no, pedir perdón o empezar de nuevo sin miedo.</t>
+        </is>
+      </c>
+      <c r="M234" s="61" t="inlineStr">
+        <is>
+          <t>Decisiones tomadas por miedo al rechazo.</t>
+        </is>
+      </c>
+      <c r="N234" s="61" t="inlineStr">
+        <is>
+          <t>Tomá hoy una decisión que venías postergando por miedo al qué dirán.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="61" t="n">
+        <v>39</v>
+      </c>
+      <c r="B235" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C235" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: saber quién sos</t>
+        </is>
+      </c>
+      <c r="D235" s="61" t="inlineStr">
+        <is>
+          <t>Juan aclara que los hijos de Dios no nacen de la sangre ni de la voluntad humana, sino de Dios.</t>
+        </is>
+      </c>
+      <c r="E235" s="61" t="inlineStr">
+        <is>
+          <t>Juan 1:13</t>
+        </is>
+      </c>
+      <c r="F235" s="61" t="inlineStr">
+        <is>
+          <t>Lo que Dios dice de vos pesa más que las etiquetas y las heridas: la identidad es un regalo de gracia.</t>
+        </is>
+      </c>
+      <c r="G235" s="61" t="n"/>
+      <c r="H235" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, escribí tres cosas que Dios dice de vos en su Palabra y leelas cada mañana.</t>
+        </is>
+      </c>
+      <c r="I235" s="61" t="inlineStr">
+        <is>
+          <t>Vivir desde la identidad recibida, y no desde la aprobación de los demás, da una base estable.</t>
+        </is>
+      </c>
+      <c r="J235" s="61" t="n"/>
+      <c r="K235" s="61" t="n"/>
+      <c r="L235" s="61" t="inlineStr">
+        <is>
+          <t>Quien se sabe hijo de Dios decide con libertad, sin la ansiedad de tener que probar algo.</t>
+        </is>
+      </c>
+      <c r="M235" s="61" t="n"/>
+      <c r="N235" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de septiembre verificados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -8925,7 +8925,7 @@
       </c>
       <c r="AJ40" s="8" t="inlineStr">
         <is>
-          <t>Juan 1:12 — A todos los que recibieron la Palabra, a los que creen en su nombre, les dio la potestad de ser hechos hijos de Dios</t>
+          <t>Juan 1:12 — Pero a todos los que recibieron la Palabra, a los que creen en su nombre, les dio la potestad de ser hechos hijos de Dios</t>
         </is>
       </c>
       <c r="AK40" s="8" t="inlineStr">
@@ -32991,7 +32991,7 @@
       </c>
       <c r="D207" s="61" t="inlineStr">
         <is>
-          <t>En el griego, Pablo dice que el amor al dinero es raíz de «toda clase» de males: no la única causa de todo mal, sino una raíz que produce muchos.</t>
+          <t>En el griego, Pablo dice que el amor al dinero es raíz «de todos los males», en plural; por eso muchas versiones traducen «de toda clase de males»: no la única causa de todo mal, sino una raíz que produce muchos.</t>
         </is>
       </c>
       <c r="E207" s="61" t="inlineStr">
@@ -33061,7 +33061,7 @@
       </c>
       <c r="D208" s="61" t="inlineStr">
         <is>
-          <t>Justo después, Jesús cuenta la parábola del rico que construyó graneros más grandes para guardar su cosecha, y esa misma noche murió.</t>
+          <t>Justo después, Jesús cuenta la parábola del rico que planeaba construir graneros más grandes para guardar su cosecha, y Dios le dijo que esa misma noche le pedirían el alma.</t>
         </is>
       </c>
       <c r="E208" s="61" t="inlineStr">
@@ -33721,12 +33721,12 @@
       </c>
       <c r="D218" s="61" t="inlineStr">
         <is>
-          <t>En Paraguay, más de un millón de personas son socias de alguna cooperativa, según el Instituto Nacional de Cooperativismo (INCOOP).</t>
+          <t>En Paraguay, cerca de 1,85 millones de personas son socias de alguna cooperativa, según datos del Instituto Nacional de Cooperativismo (INCOOP).</t>
         </is>
       </c>
       <c r="E218" s="61" t="inlineStr">
         <is>
-          <t>Instituto Nacional de Cooperativismo (INCOOP)</t>
+          <t>Instituto Nacional de Cooperativismo (INCOOP), datos difundidos en julio de 2026</t>
         </is>
       </c>
       <c r="F218" s="61" t="inlineStr">
@@ -34071,7 +34071,7 @@
       </c>
       <c r="D223" s="61" t="inlineStr">
         <is>
-          <t>La Constitución del Paraguay establece que el Estado promoverá el cooperativismo.</t>
+          <t>La Constitución del Paraguay establece que el Estado fomentará la empresa cooperativa y otras formas asociativas.</t>
         </is>
       </c>
       <c r="E223" s="61" t="inlineStr">
@@ -34191,7 +34191,7 @@
       </c>
       <c r="D225" s="61" t="inlineStr">
         <is>
-          <t>Hoy, 21 de septiembre, Paraguay celebra el Día de la Juventud, junto con el inicio de la primavera.</t>
+          <t>Hoy, 21 de septiembre, Paraguay celebra el Día de la Juventud, junto con la llegada de la primavera, que tradicionalmente se festeja en esta fecha.</t>
         </is>
       </c>
       <c r="E225" s="61" t="inlineStr">
@@ -34311,7 +34311,7 @@
       </c>
       <c r="N226" s="61" t="inlineStr">
         <is>
-          <t>Si ves señales de alarma en un adolescente, buscá ayuda profesional; en Paraguay, la línea gratuita 147 «Fono Ayuda» orienta sobre niños y adolescentes.</t>
+          <t>Si ves señales de alarma en un adolescente, buscá ayuda profesional: el médico de la familia o el centro de salud pueden orientarte.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mensajero: textos urgentes de Prov 25:28 y 12:24; guiones de octubre con revisión teológica
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -8251,8 +8251,7 @@
       </c>
       <c r="Z37" s="2" t="inlineStr">
         <is>
-          <t>Proverbios 25:28 — El justo piensa bien, antes de responder;
-la boca de los injustos dice malas palabras.</t>
+          <t>Proverbios 25:28 — Ciudad en ruinas, sin muralla protectora: ¡eso es el hombre que no frena sus impulsos!</t>
         </is>
       </c>
       <c r="AA37" s="2" t="inlineStr">
@@ -8276,8 +8275,7 @@
       </c>
       <c r="AD37" s="2" t="inlineStr">
         <is>
-          <t>Proverbios 12:24 — Al Señor le repugnan los labios mentirosos;
-pero le agradan los que dicen la verdad.</t>
+          <t>Proverbios 12:24 — Los diligentes dominan a otros; los negligentes son dominados.</t>
         </is>
       </c>
       <c r="AE37" s="2" t="inlineStr">
@@ -9061,7 +9059,7 @@
       </c>
       <c r="Y41" s="10" t="inlineStr">
         <is>
-          <t>• Moisés dudo de si mismo
+          <t>• Moisés dudó de sí mismo
 • Dios llama a pesar de la inseguridad
 • El liderazgo no depende de sentirse capaz</t>
         </is>
@@ -9101,7 +9099,7 @@
         <is>
           <t>• El contraste de los recursos humanos frente a los divinos
 • La autoridad del respaldo divino
-• El trasfondo de la afrenta personal y nacional</t>
+• La batalla es del Señor (17:47)</t>
         </is>
       </c>
       <c r="AF41" s="10" t="inlineStr">
@@ -9113,7 +9111,7 @@
       </c>
       <c r="AG41" s="10" t="inlineStr">
         <is>
-          <t>• La grandeza esta en servir
+          <t>• La grandeza está en servir
 • Jesús invierte el concepto de poder
 • Ser servidor de todos es el camino</t>
         </is>
@@ -9282,7 +9280,7 @@
       </c>
       <c r="AA42" s="12" t="inlineStr">
         <is>
-          <t>• La diligencia en casa no descansa
+          <t>• La diligencia cuida a toda la familia
 • Proveer con anticipación
 • El esfuerzo cotidiano sostiene el hogar</t>
         </is>
@@ -9295,7 +9293,7 @@
       <c r="AC42" s="12" t="inlineStr">
         <is>
           <t>• Proveer para los suyos es acto de fe
-• No hacerlo niega la fe
+• Desentenderse de los suyos contradice la fe
 • La responsabilidad familiar tiene peso espiritual</t>
         </is>
       </c>
@@ -9332,7 +9330,7 @@
       <c r="AI42" s="12" t="inlineStr">
         <is>
           <t>• Someterse unos a otros con reverencia a Dios
-• No es jerarquía rígida, es humildad mutua
+• La humildad mutua sostiene la familia
 • El respeto mutuo sostiene los roles</t>
         </is>
       </c>
@@ -9489,7 +9487,7 @@
         <is>
           <t>• Traer el diezmo es acto de confianza
 • Dios invita a probarlo
-• La obediencia trae bendición prometida</t>
+• La bendición de Dios no es un pago</t>
         </is>
       </c>
       <c r="AB43" s="14" t="inlineStr">
@@ -9502,7 +9500,7 @@
       <c r="AC43" s="14" t="inlineStr">
         <is>
           <t>• Honrar a Dios con las primicias
-• Los graneros se llenan por confiar primero en El
+• Es un principio de sabiduría, no una fórmula
 • El orden correcto: Dios primero</t>
         </is>
       </c>
@@ -9513,9 +9511,9 @@
       </c>
       <c r="AE43" s="14" t="inlineStr">
         <is>
-          <t>• Dar activa el principio de recibir
+          <t>• Dar con la misma generosidad con que Dios nos trata
 • La medida que se da, se recibe
-• La generosidad no empobrece</t>
+• La generosidad nace de la gracia recibida</t>
         </is>
       </c>
       <c r="AF43" s="14" t="inlineStr">
@@ -19214,7 +19212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N235"/>
+  <dimension ref="A1:N259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -34904,6 +34902,1606 @@
       </c>
       <c r="M235" s="61" t="n"/>
       <c r="N235" s="61" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="B236" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C236" s="61" t="inlineStr">
+        <is>
+          <t>Humilde bajo presión</t>
+        </is>
+      </c>
+      <c r="D236" s="61" t="inlineStr">
+        <is>
+          <t>Números 12 cuenta que María y Aarón, los hermanos de Moisés, lo criticaron; el texto destaca su humildad justo en ese momento.</t>
+        </is>
+      </c>
+      <c r="E236" s="61" t="inlineStr">
+        <is>
+          <t>Números 12:1-3</t>
+        </is>
+      </c>
+      <c r="F236" s="61" t="inlineStr">
+        <is>
+          <t>Cuando sus propios hermanos lo criticaron, Moisés no se defendió con soberbia. El texto destaca su humildad justo en ese momento de presión.</t>
+        </is>
+      </c>
+      <c r="G236" s="61" t="inlineStr">
+        <is>
+          <t>Responder a cada crítica con enojo para defender la propia imagen.</t>
+        </is>
+      </c>
+      <c r="H236" s="61" t="inlineStr">
+        <is>
+          <t>La próxima vez que te critiquen, escuchá primero y respondé después, con calma.</t>
+        </is>
+      </c>
+      <c r="I236" s="61" t="inlineStr">
+        <is>
+          <t>Moisés guió a un pueblo que se quejaba seguido, sin manual ni experiencia. No lo sostuvo su capacidad, sino su dependencia de Dios: una y otra vez llevó los problemas delante de él.</t>
+        </is>
+      </c>
+      <c r="J236" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que creen que tienen que poder con todo solos.</t>
+        </is>
+      </c>
+      <c r="K236" s="61" t="inlineStr">
+        <is>
+          <t>Llevá hoy a Dios en oración la situación que más presión te genera.</t>
+        </is>
+      </c>
+      <c r="L236" s="61" t="inlineStr">
+        <is>
+          <t>La humildad no es dejarse pisar: Moisés también confrontó cuando hizo falta. Es fortaleza puesta al servicio de los demás.</t>
+        </is>
+      </c>
+      <c r="M236" s="61" t="inlineStr">
+        <is>
+          <t>Confundir humildad con no decir nunca nada.</t>
+        </is>
+      </c>
+      <c r="N236" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés que corregir algo en tu equipo o en tu casa, hacelo con firmeza y sin humillar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="B237" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C237" s="61" t="inlineStr">
+        <is>
+          <t>Levantemos los muros</t>
+        </is>
+      </c>
+      <c r="D237" s="61" t="inlineStr">
+        <is>
+          <t>Nehemías era copero del rey persa Artajerjes, un cargo de mucha confianza en la corte.</t>
+        </is>
+      </c>
+      <c r="E237" s="61" t="inlineStr">
+        <is>
+          <t>Nehemías 1:11; 2:1</t>
+        </is>
+      </c>
+      <c r="F237" s="61" t="inlineStr">
+        <is>
+          <t>Nehemías no tenía ejército ni recursos propios, solo un permiso del rey y una convicción. Bajo presión, no trabajó solo: convocó a todos.</t>
+        </is>
+      </c>
+      <c r="G237" s="61" t="inlineStr">
+        <is>
+          <t>Querer cargar con todo para que salga «a mi manera».</t>
+        </is>
+      </c>
+      <c r="H237" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en un proyecto atascado y en quién podría sumarse si lo invitás.</t>
+        </is>
+      </c>
+      <c r="I237" s="61" t="inlineStr">
+        <is>
+          <t>Primero mostró la realidad sin maquillarla, «¿Ya vieron lo mal que estamos?», y después invitó a actuar.</t>
+        </is>
+      </c>
+      <c r="J237" s="61" t="inlineStr">
+        <is>
+          <t>Líderes que esconden los problemas, o que solo se quejan de ellos.</t>
+        </is>
+      </c>
+      <c r="K237" s="61" t="inlineStr">
+        <is>
+          <t>Describí con honestidad un problema de tu casa o de tu equipo, y proponé un primer paso.</t>
+        </is>
+      </c>
+      <c r="L237" s="61" t="inlineStr">
+        <is>
+          <t>Nehemías contó lo que Dios había hecho, y el pueblo respondió: «¡comencemos!». La fe y el trabajo fueron juntos.</t>
+        </is>
+      </c>
+      <c r="M237" s="61" t="inlineStr">
+        <is>
+          <t>Esperar condiciones perfectas para empezar.</t>
+        </is>
+      </c>
+      <c r="N237" s="61" t="inlineStr">
+        <is>
+          <t>¿Qué muro lleva tiempo en ruinas en tu vida? Elegí un primer ladrillo y ponelo esta semana.</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="B238" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C238" s="61" t="inlineStr">
+        <is>
+          <t>En el nombre del Señor</t>
+        </is>
+      </c>
+      <c r="D238" s="61" t="inlineStr">
+        <is>
+          <t>Según el texto hebreo, Goliat medía «seis codos y un palmo», cerca de tres metros; algunos manuscritos antiguos dicen cuatro codos, unos dos metros.</t>
+        </is>
+      </c>
+      <c r="E238" s="61" t="inlineStr">
+        <is>
+          <t>1 Samuel 17:4 (texto masorético y Septuaginta)</t>
+        </is>
+      </c>
+      <c r="F238" s="61" t="inlineStr">
+        <is>
+          <t>David no tenía armadura ni experiencia militar, pero tenía un propósito claro: defender el nombre de Dios. Como Nehemías, no dependía de sus propios recursos.</t>
+        </is>
+      </c>
+      <c r="G238" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que sin recursos no se puede emprender nada que valga la pena.</t>
+        </is>
+      </c>
+      <c r="H238" s="61" t="inlineStr">
+        <is>
+          <t>Anotá qué tenés hoy, aunque sea poco, para empezar lo que Dios te puso en el corazón.</t>
+        </is>
+      </c>
+      <c r="I238" s="61" t="inlineStr">
+        <is>
+          <t>David va «en el nombre del Señor». El relato no promete que venceremos a todo «gigante»: muestra que David buscaba la gloria de Dios, no la suya.</t>
+        </is>
+      </c>
+      <c r="J238" s="61" t="inlineStr">
+        <is>
+          <t>Usar el nombre de Dios para respaldar proyectos personales.</t>
+        </is>
+      </c>
+      <c r="K238" s="61" t="inlineStr">
+        <is>
+          <t>Revisá tu proyecto: ¿busca la gloria de Dios y el bien de otros, o solo el tuyo?</t>
+        </is>
+      </c>
+      <c r="L238" s="61" t="inlineStr">
+        <is>
+          <t>David reconoce que la batalla es del Señor (17:47). Un líder con propósito hace su parte y confía el resultado a Dios.</t>
+        </is>
+      </c>
+      <c r="M238" s="61" t="inlineStr">
+        <is>
+          <t>Cargar con la ansiedad de controlar cada resultado.</t>
+        </is>
+      </c>
+      <c r="N238" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy tu parte con excelencia, y entregale el resultado a Dios en oración.</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="B239" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C239" s="61" t="inlineStr">
+        <is>
+          <t>El que quiera ser grande</t>
+        </is>
+      </c>
+      <c r="D239" s="61" t="inlineStr">
+        <is>
+          <t>Jesús dijo esto después de que la madre de Santiago y Juan le pidiera los mejores lugares para sus hijos.</t>
+        </is>
+      </c>
+      <c r="E239" s="61" t="inlineStr">
+        <is>
+          <t>Mateo 20:20-24</t>
+        </is>
+      </c>
+      <c r="F239" s="61" t="inlineStr">
+        <is>
+          <t>Los discípulos discutían por los primeros puestos. Jesús les cambia la pregunta: no quién manda, sino quién sirve.</t>
+        </is>
+      </c>
+      <c r="G239" s="61" t="inlineStr">
+        <is>
+          <t>Buscar cargos por el prestigio y no por el servicio.</t>
+        </is>
+      </c>
+      <c r="H239" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy una tarea de servicio que nadie quiere hacer en tu casa o en tu trabajo.</t>
+        </is>
+      </c>
+      <c r="I239" s="61" t="inlineStr">
+        <is>
+          <t>Nehemías también trabajó junto al pueblo y no se aprovechó de su cargo (Nehemías 5:14-15). El propósito de un buen líder es el bien de los demás.</t>
+        </is>
+      </c>
+      <c r="J239" s="61" t="inlineStr">
+        <is>
+          <t>Usar la posición para sacar ventaja.</t>
+        </is>
+      </c>
+      <c r="K239" s="61" t="inlineStr">
+        <is>
+          <t>Revisá si hay algún privilegio de tu cargo que podrías usar para servir mejor.</t>
+        </is>
+      </c>
+      <c r="L239" s="61" t="inlineStr">
+        <is>
+          <t>Jesús vino a dar su vida en rescate por muchos. Su servicio no fue una técnica de liderazgo: fue su entrega por nosotros.</t>
+        </is>
+      </c>
+      <c r="M239" s="61" t="inlineStr">
+        <is>
+          <t>Servir solo cuando conviene o cuando nos ven.</t>
+        </is>
+      </c>
+      <c r="N239" s="61" t="inlineStr">
+        <is>
+          <t>Agradecele hoy a Jesús su entrega, y servile a alguien en su nombre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="B240" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C240" s="61" t="inlineStr">
+        <is>
+          <t>Un carácter íntegro</t>
+        </is>
+      </c>
+      <c r="D240" s="61" t="inlineStr">
+        <is>
+          <t>Tito era un colaborador de Pablo que quedó en Creta para organizar las iglesias y nombrar líderes.</t>
+        </is>
+      </c>
+      <c r="E240" s="61" t="inlineStr">
+        <is>
+          <t>Tito 1:4-5</t>
+        </is>
+      </c>
+      <c r="F240" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide para los líderes un carácter íntegro antes que habilidades. Lo que hace confiable a un líder es quién es, también cuando nadie lo ve.</t>
+        </is>
+      </c>
+      <c r="G240" s="61" t="inlineStr">
+        <is>
+          <t>Elegir líderes solo por su talento o su carisma.</t>
+        </is>
+      </c>
+      <c r="H240" s="61" t="inlineStr">
+        <is>
+          <t>Revisá un área de tu vida donde lo que mostrás y lo que sos no coinciden.</t>
+        </is>
+      </c>
+      <c r="I240" s="61" t="inlineStr">
+        <is>
+          <t>Hospitalario y amante de lo bueno: el liderazgo cristiano se parece a Jesús, que lavó los pies de sus discípulos (Juan 13).</t>
+        </is>
+      </c>
+      <c r="J240" s="61" t="inlineStr">
+        <is>
+          <t>Liderar desde lejos, sin conocer a la gente.</t>
+        </is>
+      </c>
+      <c r="K240" s="61" t="inlineStr">
+        <is>
+          <t>¿A quién podrías «lavarle los pies» esta semana? Hacé un servicio concreto a alguien que liderás.</t>
+        </is>
+      </c>
+      <c r="L240" s="61" t="inlineStr">
+        <is>
+          <t>El líder se apega a la Palabra para animar y corregir con verdad. Servir no es decirles a todos lo que quieren oír.</t>
+        </is>
+      </c>
+      <c r="M240" s="61" t="inlineStr">
+        <is>
+          <t>Evitar toda corrección para quedar bien.</t>
+        </is>
+      </c>
+      <c r="N240" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés que decir una verdad difícil, decila con amor y en privado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="61" t="n">
+        <v>40</v>
+      </c>
+      <c r="B241" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C241" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: líderes según Dios</t>
+        </is>
+      </c>
+      <c r="D241" s="61" t="inlineStr">
+        <is>
+          <t>Jesús dijo estas palabras en la última cena, la misma noche en que lavó los pies de sus discípulos.</t>
+        </is>
+      </c>
+      <c r="E241" s="61" t="inlineStr">
+        <is>
+          <t>Lucas 22:14-27; Juan 13:1-15</t>
+        </is>
+      </c>
+      <c r="F241" s="61" t="inlineStr">
+        <is>
+          <t>Moisés: bajo presión, humildad y dependencia de Dios.</t>
+        </is>
+      </c>
+      <c r="G241" s="61" t="n"/>
+      <c r="H241" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, hacé un servicio concreto a alguien que liderás, en tu casa, tu trabajo o tu iglesia, sin esperar nada a cambio.</t>
+        </is>
+      </c>
+      <c r="I241" s="61" t="inlineStr">
+        <is>
+          <t>Nehemías y David: un propósito claro moviliza, y el resultado se confía a Dios.</t>
+        </is>
+      </c>
+      <c r="J241" s="61" t="n"/>
+      <c r="K241" s="61" t="n"/>
+      <c r="L241" s="61" t="inlineStr">
+        <is>
+          <t>Jesús: el líder sirve, y el carácter íntegro pesa más que el talento.</t>
+        </is>
+      </c>
+      <c r="M241" s="61" t="n"/>
+      <c r="N241" s="61" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="61" t="n">
+        <v>41</v>
+      </c>
+      <c r="B242" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C242" s="61" t="inlineStr">
+        <is>
+          <t>Una casa organizada</t>
+        </is>
+      </c>
+      <c r="D242" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 31:10-31 es un poema acróstico: en hebreo, cada versículo empieza con una letra del alfabeto, en orden.</t>
+        </is>
+      </c>
+      <c r="E242" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 31:10-31 (texto hebreo)</t>
+        </is>
+      </c>
+      <c r="F242" s="61" t="inlineStr">
+        <is>
+          <t>Este poema describe a una mujer trabajadora y sabia. No es una lista de exigencias para cada madre, sino un retrato de la sabiduría puesta en práctica.</t>
+        </is>
+      </c>
+      <c r="G242" s="61" t="inlineStr">
+        <is>
+          <t>Que todo el peso de la casa recaiga sobre una sola persona.</t>
+        </is>
+      </c>
+      <c r="H242" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale hoy a quien más trabaja en tu casa cómo podés ayudar.</t>
+        </is>
+      </c>
+      <c r="I242" s="61" t="inlineStr">
+        <is>
+          <t>Ella planifica y asigna tareas. Hacer juntos una lista real de todo lo que hay que hacer en casa muestra cuánto trabajo invisible existe.</t>
+        </is>
+      </c>
+      <c r="J242" s="61" t="inlineStr">
+        <is>
+          <t>Tareas invisibles que nadie ve hasta que dejan de hacerse.</t>
+        </is>
+      </c>
+      <c r="K242" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, hagan en familia una lista de todas las tareas de la casa, también las que no se ven.</t>
+        </is>
+      </c>
+      <c r="L242" s="61" t="inlineStr">
+        <is>
+          <t>La sensación de injusticia no siempre viene de la cantidad de tareas, sino de no haberlo hablado. Conversarlo en vez de suponerlo cambia todo.</t>
+        </is>
+      </c>
+      <c r="M242" s="61" t="inlineStr">
+        <is>
+          <t>Suponer que el otro «ya sabe» lo que le toca.</t>
+        </is>
+      </c>
+      <c r="N242" s="61" t="inlineStr">
+        <is>
+          <t>Repartan las tareas de la lista conversando, según el tiempo y las posibilidades de cada uno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="61" t="n">
+        <v>41</v>
+      </c>
+      <c r="B243" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C243" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar a los suyos</t>
+        </is>
+      </c>
+      <c r="D243" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribe este versículo en una sección sobre el cuidado de las viudas: la familia debía hacerse cargo de las suyas antes que la iglesia.</t>
+        </is>
+      </c>
+      <c r="E243" s="61" t="inlineStr">
+        <is>
+          <t>1 Timoteo 5:3-8, 16</t>
+        </is>
+      </c>
+      <c r="F243" s="61" t="inlineStr">
+        <is>
+          <t>Proveer no es solo traer plata: es cuidar. Incluye el trabajo de la casa, el tiempo y la atención a los mayores.</t>
+        </is>
+      </c>
+      <c r="G243" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que quien trae el sueldo ya cumplió con todo.</t>
+        </is>
+      </c>
+      <c r="H243" s="61" t="inlineStr">
+        <is>
+          <t>Reconocé hoy en voz alta el trabajo de casa que hace otro miembro de tu familia.</t>
+        </is>
+      </c>
+      <c r="I243" s="61" t="inlineStr">
+        <is>
+          <t>Pablo habla de quien se desentiende de su familia, no de quien no puede proveer por enfermedad o por falta de trabajo.</t>
+        </is>
+      </c>
+      <c r="J243" s="61" t="inlineStr">
+        <is>
+          <t>Culpar o avergonzar a quien hoy no tiene trabajo.</t>
+        </is>
+      </c>
+      <c r="K243" s="61" t="inlineStr">
+        <is>
+          <t>Si alguien de tu familia está sin trabajo, acompañalo y ayudalo a buscar, sin reproches.</t>
+        </is>
+      </c>
+      <c r="L243" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar a los nuestros, también a los abuelos, es parte de vivir la fe.</t>
+        </is>
+      </c>
+      <c r="M243" s="61" t="inlineStr">
+        <is>
+          <t>Dejar el cuidado de los mayores de la familia a cargo de uno solo de los hermanos.</t>
+        </is>
+      </c>
+      <c r="N243" s="61" t="inlineStr">
+        <is>
+          <t>Conversen entre hermanos cómo repartir el cuidado de sus padres o abuelos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="61" t="n">
+        <v>41</v>
+      </c>
+      <c r="B244" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C244" s="61" t="inlineStr">
+        <is>
+          <t>Paciencia mutua</t>
+        </is>
+      </c>
+      <c r="D244" s="61" t="inlineStr">
+        <is>
+          <t>Según la Organización Internacional del Trabajo, las mujeres realizan en el mundo cerca de tres cuartas partes del trabajo de cuidado no remunerado.</t>
+        </is>
+      </c>
+      <c r="E244" s="61" t="inlineStr">
+        <is>
+          <t>Organización Internacional del Trabajo, El trabajo de cuidados y los trabajadores del cuidado, 2018</t>
+        </is>
+      </c>
+      <c r="F244" s="61" t="inlineStr">
+        <is>
+          <t>Cuando los dos trabajan fuera de casa, el cansancio se nota. La paciencia mutua evita que cada tarea pendiente se vuelva pelea.</t>
+        </is>
+      </c>
+      <c r="G244" s="61" t="inlineStr">
+        <is>
+          <t>Llegar a casa y reclamar todo lo que el otro no hizo.</t>
+        </is>
+      </c>
+      <c r="H244" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, al llegar a casa, empezá con un saludo y no con un reclamo.</t>
+        </is>
+      </c>
+      <c r="I244" s="61" t="inlineStr">
+        <is>
+          <t>Si hay quejas acumuladas sobre quién hace qué, Pablo pide perdonar como Cristo nos perdonó, y después conversar.</t>
+        </is>
+      </c>
+      <c r="J244" s="61" t="inlineStr">
+        <is>
+          <t>Llevar la cuenta de todo lo que uno hace y el otro no.</t>
+        </is>
+      </c>
+      <c r="K244" s="61" t="inlineStr">
+        <is>
+          <t>Soltá una queja vieja sobre las tareas de la casa, y conversen cómo organizarse mejor.</t>
+        </is>
+      </c>
+      <c r="L244" s="61" t="inlineStr">
+        <is>
+          <t>Cristo sirvió sin llevar la cuenta. Las tareas de la casa no deberían recaer por defecto en uno solo, sino repartirse según la realidad de hoy.</t>
+        </is>
+      </c>
+      <c r="M244" s="61" t="inlineStr">
+        <is>
+          <t>Repartir las tareas por costumbre y no según la realidad actual.</t>
+        </is>
+      </c>
+      <c r="N244" s="61" t="inlineStr">
+        <is>
+          <t>Revisen el reparto de tareas según los horarios de trabajo de cada uno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="61" t="n">
+        <v>41</v>
+      </c>
+      <c r="B245" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C245" s="61" t="inlineStr">
+        <is>
+          <t>Reconocer el esfuerzo</t>
+        </is>
+      </c>
+      <c r="D245" s="61" t="inlineStr">
+        <is>
+          <t>Un estudio encontró que expresar gratitud a la pareja se asocia con una relación más satisfactoria para los dos.</t>
+        </is>
+      </c>
+      <c r="E245" s="61" t="inlineStr">
+        <is>
+          <t>Algoe, Gable y Maisel, Personal Relationships, 2010</t>
+        </is>
+      </c>
+      <c r="F245" s="61" t="inlineStr">
+        <is>
+          <t>Los hijos y el esposo reconocen en voz alta el trabajo de ella. El reconocimiento también es parte de un reparto justo.</t>
+        </is>
+      </c>
+      <c r="G245" s="61" t="inlineStr">
+        <is>
+          <t>Dar por sentado el trabajo del otro.</t>
+        </is>
+      </c>
+      <c r="H245" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, agradecé en voz alta algo concreto que hace tu pareja en casa.</t>
+        </is>
+      </c>
+      <c r="I245" s="61" t="inlineStr">
+        <is>
+          <t>Los hijos aprenden a valorar el trabajo de la casa cuando también participan.</t>
+        </is>
+      </c>
+      <c r="J245" s="61" t="inlineStr">
+        <is>
+          <t>Hijos que no colaboran porque «mamá lo hace».</t>
+        </is>
+      </c>
+      <c r="K245" s="61" t="inlineStr">
+        <is>
+          <t>Asigná a cada hijo una tarea según su edad, y explicale por qué es importante.</t>
+        </is>
+      </c>
+      <c r="L245" s="61" t="inlineStr">
+        <is>
+          <t>Cuando todos colaboran, la casa funciona mejor y queda más tiempo para estar juntos.</t>
+        </is>
+      </c>
+      <c r="M245" s="61" t="inlineStr">
+        <is>
+          <t>Casas donde todos están cansados y nadie tiene tiempo para el otro.</t>
+        </is>
+      </c>
+      <c r="N245" s="61" t="inlineStr">
+        <is>
+          <t>Planeen un momento en familia con el tiempo que ganen al repartir mejor las tareas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="61" t="n">
+        <v>41</v>
+      </c>
+      <c r="B246" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C246" s="61" t="inlineStr">
+        <is>
+          <t>Humildad mutua</t>
+        </is>
+      </c>
+      <c r="D246" s="61" t="inlineStr">
+        <is>
+          <t>Efesios 5:21 abre una sección sobre la vida en familia que habla de esposos, hijos, padres, siervos y amos.</t>
+        </is>
+      </c>
+      <c r="E246" s="61" t="inlineStr">
+        <is>
+          <t>Efesios 5:21 a 6:9</t>
+        </is>
+      </c>
+      <c r="F246" s="61" t="inlineStr">
+        <is>
+          <t>Pablo empieza la sección sobre la familia pidiendo sumisión mutua, por respeto a Cristo. Las iglesias entienden de distintas maneras los roles que siguen, pero todas reconocen este punto de partida: la humildad.</t>
+        </is>
+      </c>
+      <c r="G246" s="61" t="inlineStr">
+        <is>
+          <t>Usar la Biblia para imponerse sobre el otro.</t>
+        </is>
+      </c>
+      <c r="H246" s="61" t="inlineStr">
+        <is>
+          <t>Antes de decidir algo de la casa, preguntá: ¿qué pensás vos?</t>
+        </is>
+      </c>
+      <c r="I246" s="61" t="inlineStr">
+        <is>
+          <t>Ser flexibles en quién hace qué no es caos: es adaptarse a lo que la familia vive en cada temporada.</t>
+        </is>
+      </c>
+      <c r="J246" s="61" t="inlineStr">
+        <is>
+          <t>Roles tan rígidos que no se adaptan a una enfermedad, a un trabajo nuevo o a un bebé.</t>
+        </is>
+      </c>
+      <c r="K246" s="61" t="inlineStr">
+        <is>
+          <t>Si esta semana alguien de tu casa tiene más carga, tomá vos una de sus tareas.</t>
+        </is>
+      </c>
+      <c r="L246" s="61" t="inlineStr">
+        <is>
+          <t>La meta no es que todos hagan lo mismo, sino que el hogar funcione bien para todos.</t>
+        </is>
+      </c>
+      <c r="M246" s="61" t="inlineStr">
+        <is>
+          <t>Discutir por quién hace más en vez de buscar que la casa funcione.</t>
+        </is>
+      </c>
+      <c r="N246" s="61" t="inlineStr">
+        <is>
+          <t>Acuerden revisar el reparto una vez por mes, para ajustarlo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="61" t="n">
+        <v>41</v>
+      </c>
+      <c r="B247" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C247" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: un hogar que funciona para todos</t>
+        </is>
+      </c>
+      <c r="D247" s="61" t="inlineStr">
+        <is>
+          <t>Rut era moabita y llegó a ser bisabuela del rey David.</t>
+        </is>
+      </c>
+      <c r="E247" s="61" t="inlineStr">
+        <is>
+          <t>Rut 4:13-17</t>
+        </is>
+      </c>
+      <c r="F247" s="61" t="inlineStr">
+        <is>
+          <t>Repartir las tareas conversando, haciendo visible el trabajo invisible.</t>
+        </is>
+      </c>
+      <c r="G247" s="61" t="n"/>
+      <c r="H247" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, hagan juntos la lista de tareas de la casa, repártanla conversando y agradezcan en voz alta lo que hace cada uno.</t>
+        </is>
+      </c>
+      <c r="I247" s="61" t="inlineStr">
+        <is>
+          <t>Cuando los dos trabajan, la paciencia, el perdón y el reconocimiento hacen justo el reparto.</t>
+        </is>
+      </c>
+      <c r="J247" s="61" t="n"/>
+      <c r="K247" s="61" t="n"/>
+      <c r="L247" s="61" t="inlineStr">
+        <is>
+          <t>Flexibilidad con orden: que el hogar funcione para todos.</t>
+        </is>
+      </c>
+      <c r="M247" s="61" t="n"/>
+      <c r="N247" s="61" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="61" t="n">
+        <v>42</v>
+      </c>
+      <c r="B248" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C248" s="61" t="inlineStr">
+        <is>
+          <t>Pónganme a prueba</t>
+        </is>
+      </c>
+      <c r="D248" s="61" t="inlineStr">
+        <is>
+          <t>En la ley de Moisés, parte del diezmo se destinaba a los levitas, a los extranjeros, a los huérfanos y a las viudas.</t>
+        </is>
+      </c>
+      <c r="E248" s="61" t="inlineStr">
+        <is>
+          <t>Deuteronomio 14:28-29</t>
+        </is>
+      </c>
+      <c r="F248" s="61" t="inlineStr">
+        <is>
+          <t>Malaquías habla al pueblo de Israel, que se había apartado de Dios y descuidado su casa; el diezmo sostenía a los levitas y a los necesitados. Dar es poner a Dios primero y confiar en él.</t>
+        </is>
+      </c>
+      <c r="G248" s="61" t="inlineStr">
+        <is>
+          <t>Dar lo que sobra, si sobra.</t>
+        </is>
+      </c>
+      <c r="H248" s="61" t="inlineStr">
+        <is>
+          <t>Antes de gastar tu próximo ingreso, separá primero lo que vas a dar.</t>
+        </is>
+      </c>
+      <c r="I248" s="61" t="inlineStr">
+        <is>
+          <t>Es un caso único en la Biblia: Dios invita a su pueblo a confiar en él con sus bienes. Las iglesias enseñan el diezmo de maneras distintas; el principio que todas comparten es dar con confianza y generosidad.</t>
+        </is>
+      </c>
+      <c r="J248" s="61" t="inlineStr">
+        <is>
+          <t>Discutir el porcentaje y olvidarse del corazón.</t>
+        </is>
+      </c>
+      <c r="K248" s="61" t="inlineStr">
+        <is>
+          <t>Conversá con tu familia cómo quieren dar este mes, en tu iglesia y a quien lo necesite.</t>
+        </is>
+      </c>
+      <c r="L248" s="61" t="inlineStr">
+        <is>
+          <t>Dios promete bendecir a su pueblo, pero la bendición no es una cuenta que se cobra: dar no es una inversión para recibir más plata.</t>
+        </is>
+      </c>
+      <c r="M248" s="61" t="inlineStr">
+        <is>
+          <t>Dar para que Dios «devuelva el doble».</t>
+        </is>
+      </c>
+      <c r="N248" s="61" t="inlineStr">
+        <is>
+          <t>Cuando des esta semana, hacelo como gratitud, sin esperar nada a cambio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="61" t="n">
+        <v>42</v>
+      </c>
+      <c r="B249" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C249" s="61" t="inlineStr">
+        <is>
+          <t>Las primicias</t>
+        </is>
+      </c>
+      <c r="D249" s="61" t="inlineStr">
+        <is>
+          <t>En Israel, las primicias eran los primeros frutos de la cosecha, que se ofrecían a Dios antes de usar el resto.</t>
+        </is>
+      </c>
+      <c r="E249" s="61" t="inlineStr">
+        <is>
+          <t>Éxodo 23:19; Deuteronomio 26:1-11</t>
+        </is>
+      </c>
+      <c r="F249" s="61" t="inlineStr">
+        <is>
+          <t>Dar primero, y no lo que sobra, es una forma de decir que Dios ocupa el primer lugar.</t>
+        </is>
+      </c>
+      <c r="G249" s="61" t="inlineStr">
+        <is>
+          <t>Dejar a Dios para el final del mes.</t>
+        </is>
+      </c>
+      <c r="H249" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, poné a Dios primero también en tu presupuesto.</t>
+        </is>
+      </c>
+      <c r="I249" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios enseña principios de sabiduría, no garantías: dar no asegura graneros llenos. Hay creyentes generosos que pasan escasez.</t>
+        </is>
+      </c>
+      <c r="J249" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que si alguien pasa necesidad es porque no dio lo suficiente.</t>
+        </is>
+      </c>
+      <c r="K249" s="61" t="inlineStr">
+        <is>
+          <t>Si conocés a alguien generoso que pasa un momento difícil, acompañalo sin juzgarlo.</t>
+        </is>
+      </c>
+      <c r="L249" s="61" t="inlineStr">
+        <is>
+          <t>Dar desde la gratitud ordena el corazón: nos recuerda que todo lo recibimos de Dios.</t>
+        </is>
+      </c>
+      <c r="M249" s="61" t="inlineStr">
+        <is>
+          <t>Dar por presión o para que nos vean.</t>
+        </is>
+      </c>
+      <c r="N249" s="61" t="inlineStr">
+        <is>
+          <t>Agradecele a Dios por tres cosas concretas antes de dar tu ofrenda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="61" t="n">
+        <v>42</v>
+      </c>
+      <c r="B250" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C250" s="61" t="inlineStr">
+        <is>
+          <t>La misma medida</t>
+        </is>
+      </c>
+      <c r="D250" s="61" t="inlineStr">
+        <is>
+          <t>La imagen viene del mercado de granos: el vendedor generoso apretaba y sacudía el grano para que la medida quedara llena hasta rebalsar.</t>
+        </is>
+      </c>
+      <c r="E250" s="61" t="inlineStr">
+        <is>
+          <t>Lucas 6:38; comentarios bíblicos</t>
+        </is>
+      </c>
+      <c r="F250" s="61" t="inlineStr">
+        <is>
+          <t>Este versículo está en un pasaje sobre no juzgar, perdonar y dar (6:37). Jesús describe cómo es Dios con nosotros: generoso hasta rebalsar.</t>
+        </is>
+      </c>
+      <c r="G250" s="61" t="inlineStr">
+        <is>
+          <t>Leer este versículo como una fórmula para hacerse rico.</t>
+        </is>
+      </c>
+      <c r="H250" s="61" t="inlineStr">
+        <is>
+          <t>Leé Lucas 6:27-38 y anotá cuántas formas de dar menciona Jesús.</t>
+        </is>
+      </c>
+      <c r="I250" s="61" t="inlineStr">
+        <is>
+          <t>Quien da con generosidad suele vivir con más gratitud y más cerca de los demás: dar transforma también al que da.</t>
+        </is>
+      </c>
+      <c r="J250" s="61" t="inlineStr">
+        <is>
+          <t>Vivir con el puño cerrado por miedo a que falte.</t>
+        </is>
+      </c>
+      <c r="K250" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy un gesto generoso pequeño, y fijate qué produce en vos.</t>
+        </is>
+      </c>
+      <c r="L250" s="61" t="inlineStr">
+        <is>
+          <t>Damos porque recibimos primero: la gracia de Dios es la medida desbordante.</t>
+        </is>
+      </c>
+      <c r="M250" s="61" t="inlineStr">
+        <is>
+          <t>Contar lo que damos como un mérito.</t>
+        </is>
+      </c>
+      <c r="N250" s="61" t="inlineStr">
+        <is>
+          <t>Cuando des, no lo anotes como deuda de nadie: hacelo como respuesta a la gracia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="61" t="n">
+        <v>42</v>
+      </c>
+      <c r="B251" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C251" s="61" t="inlineStr">
+        <is>
+          <t>Todo es tuyo</t>
+        </is>
+      </c>
+      <c r="D251" s="61" t="inlineStr">
+        <is>
+          <t>David dijo estas palabras cuando el pueblo dio con generosidad para construir el templo, que edificaría su hijo Salomón.</t>
+        </is>
+      </c>
+      <c r="E251" s="61" t="inlineStr">
+        <is>
+          <t>1 Crónicas 29:1-9</t>
+        </is>
+      </c>
+      <c r="F251" s="61" t="inlineStr">
+        <is>
+          <t>David reconoce que no le da a Dios nada que no haya recibido primero. Dar es devolver con gratitud.</t>
+        </is>
+      </c>
+      <c r="G251" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que lo que tenemos es solo fruto de nuestro esfuerzo.</t>
+        </is>
+      </c>
+      <c r="H251" s="61" t="inlineStr">
+        <is>
+          <t>Anotá tres cosas que tenés y que recibiste sin haberlas ganado del todo.</t>
+        </is>
+      </c>
+      <c r="I251" s="61" t="inlineStr">
+        <is>
+          <t>El pueblo dio de manera voluntaria y con alegría (29:9). Dar con generosidad trae alegría a quien da.</t>
+        </is>
+      </c>
+      <c r="J251" s="61" t="inlineStr">
+        <is>
+          <t>Dar por obligación y con mala cara.</t>
+        </is>
+      </c>
+      <c r="K251" s="61" t="inlineStr">
+        <is>
+          <t>Si das esta semana, elegí hacerlo con alegría, aunque sea poco.</t>
+        </is>
+      </c>
+      <c r="L251" s="61" t="inlineStr">
+        <is>
+          <t>Reconocer que todo viene de Dios libera del miedo a perder y abre la mano para compartir.</t>
+        </is>
+      </c>
+      <c r="M251" s="61" t="inlineStr">
+        <is>
+          <t>Aferrarse a lo propio por miedo.</t>
+        </is>
+      </c>
+      <c r="N251" s="61" t="inlineStr">
+        <is>
+          <t>Compartí algo tuyo esta semana con alguien que lo necesite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="61" t="n">
+        <v>42</v>
+      </c>
+      <c r="B252" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C252" s="61" t="inlineStr">
+        <is>
+          <t>Dar lo que sabés</t>
+        </is>
+      </c>
+      <c r="D252" s="61" t="inlineStr">
+        <is>
+          <t>Jetró, el suegro de Moisés, era sacerdote de Madián.</t>
+        </is>
+      </c>
+      <c r="E252" s="61" t="inlineStr">
+        <is>
+          <t>Éxodo 18:1</t>
+        </is>
+      </c>
+      <c r="F252" s="61" t="inlineStr">
+        <is>
+          <t>Jetró dio algo que no era plata: su consejo y su experiencia. Dar no se limita al dinero.</t>
+        </is>
+      </c>
+      <c r="G252" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que, si no tengo plata, no tengo nada para dar.</t>
+        </is>
+      </c>
+      <c r="H252" s="61" t="inlineStr">
+        <is>
+          <t>Ofrecé esta semana tu experiencia o un consejo a alguien que está empezando.</t>
+        </is>
+      </c>
+      <c r="I252" s="61" t="inlineStr">
+        <is>
+          <t>Moisés dio responsabilidad a otros, y ellos dieron su tiempo para servir al pueblo. El tiempo es una de las ofrendas más valiosas.</t>
+        </is>
+      </c>
+      <c r="J252" s="61" t="inlineStr">
+        <is>
+          <t>Dar plata para no tener que dar tiempo.</t>
+        </is>
+      </c>
+      <c r="K252" s="61" t="inlineStr">
+        <is>
+          <t>Regalale una hora de tu tiempo a alguien que necesita compañía o ayuda.</t>
+        </is>
+      </c>
+      <c r="L252" s="61" t="inlineStr">
+        <is>
+          <t>Cada uno sirvió según su capacidad, unos con grupos de diez y otros de mil. Cada talento cuenta.</t>
+        </is>
+      </c>
+      <c r="M252" s="61" t="inlineStr">
+        <is>
+          <t>Compararse con lo que dan otros y no dar nada.</t>
+        </is>
+      </c>
+      <c r="N252" s="61" t="inlineStr">
+        <is>
+          <t>Pensá qué sabés hacer y ofrecelo esta semana en tu iglesia o en tu barrio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="61" t="n">
+        <v>42</v>
+      </c>
+      <c r="B253" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C253" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: el principio de dar</t>
+        </is>
+      </c>
+      <c r="D253" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribió 2 Corintios 8 y 9 para organizar una colecta para los creyentes pobres de Jerusalén.</t>
+        </is>
+      </c>
+      <c r="E253" s="61" t="inlineStr">
+        <is>
+          <t>2 Corintios 8:1-4; Romanos 15:25-26</t>
+        </is>
+      </c>
+      <c r="F253" s="61" t="inlineStr">
+        <is>
+          <t>Dar nace de reconocer que todo lo recibimos de Dios; no es una fórmula para recibir más.</t>
+        </is>
+      </c>
+      <c r="G253" s="61" t="n"/>
+      <c r="H253" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, da algo que no sea dinero: tu tiempo, un consejo o una habilidad, a alguien que lo necesite.</t>
+        </is>
+      </c>
+      <c r="I253" s="61" t="inlineStr">
+        <is>
+          <t>Dar con generosidad transforma también a quien da; Dios provee para que seamos generosos (2 Corintios 9:11), no para acumular.</t>
+        </is>
+      </c>
+      <c r="J253" s="61" t="n"/>
+      <c r="K253" s="61" t="n"/>
+      <c r="L253" s="61" t="inlineStr">
+        <is>
+          <t>Se da con tiempo, con talento y con recursos.</t>
+        </is>
+      </c>
+      <c r="M253" s="61" t="n"/>
+      <c r="N253" s="61" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="61" t="n">
+        <v>43</v>
+      </c>
+      <c r="B254" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C254" s="61" t="inlineStr">
+        <is>
+          <t>Una herencia para los nietos</t>
+        </is>
+      </c>
+      <c r="D254" s="61" t="inlineStr">
+        <is>
+          <t>En Israel la tierra se heredaba dentro de la familia, y la ley preveía que volviera a sus dueños en el año del jubileo.</t>
+        </is>
+      </c>
+      <c r="E254" s="61" t="inlineStr">
+        <is>
+          <t>Levítico 25:10, 23-28</t>
+        </is>
+      </c>
+      <c r="F254" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio habla de herencia, y el legado más duradero no siempre es material: es la fe, los valores y el ejemplo.</t>
+        </is>
+      </c>
+      <c r="G254" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que el legado es solo dejar bienes.</t>
+        </is>
+      </c>
+      <c r="H254" s="61" t="inlineStr">
+        <is>
+          <t>Preguntate: ¿qué valor me gustaría que mis hijos o mis nietos recuerden de mí?</t>
+        </is>
+      </c>
+      <c r="I254" s="61" t="inlineStr">
+        <is>
+          <t>Lo que vivimos hoy lo verán nuestros nietos. Una familia que ora, trabaja y perdona deja una huella de varias generaciones.</t>
+        </is>
+      </c>
+      <c r="J254" s="61" t="inlineStr">
+        <is>
+          <t>Vivir solo para el presente, sin pensar en los que vienen.</t>
+        </is>
+      </c>
+      <c r="K254" s="61" t="inlineStr">
+        <is>
+          <t>Contale a un nieto, un sobrino o un hijo una historia de cómo Dios obró en tu familia.</t>
+        </is>
+      </c>
+      <c r="L254" s="61" t="inlineStr">
+        <is>
+          <t>La segunda parte del proverbio es un principio, no una promesa de que los justos se quedarán con los bienes de otros. El centro es pensar más allá de uno mismo.</t>
+        </is>
+      </c>
+      <c r="M254" s="61" t="inlineStr">
+        <is>
+          <t>Usar la fe para esperar ganancias a costa de otros.</t>
+        </is>
+      </c>
+      <c r="N254" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en una decisión de hoy que podría beneficiar a la próxima generación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="61" t="n">
+        <v>43</v>
+      </c>
+      <c r="B255" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C255" s="61" t="inlineStr">
+        <is>
+          <t>Terminar bien</t>
+        </is>
+      </c>
+      <c r="D255" s="61" t="inlineStr">
+        <is>
+          <t>Pablo usa tres imágenes seguidas: la de un soldado, la de un corredor y la de alguien que cuida lo que se le confió.</t>
+        </is>
+      </c>
+      <c r="E255" s="61" t="inlineStr">
+        <is>
+          <t>2 Timoteo 4:7</t>
+        </is>
+      </c>
+      <c r="F255" s="61" t="inlineStr">
+        <is>
+          <t>Pablo mira hacia atrás al final de su vida. El legado espiritual se construye día a día, hasta el final.</t>
+        </is>
+      </c>
+      <c r="G255" s="61" t="inlineStr">
+        <is>
+          <t>Empezar con fuerza y abandonar a mitad de camino.</t>
+        </is>
+      </c>
+      <c r="H255" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un compromiso que dejaste a medias y retomalo esta semana.</t>
+        </is>
+      </c>
+      <c r="I255" s="61" t="inlineStr">
+        <is>
+          <t>Pablo no dice que ganó todas las batallas, sino que peleó la buena batalla. La fidelidad no es perfección.</t>
+        </is>
+      </c>
+      <c r="J255" s="61" t="inlineStr">
+        <is>
+          <t>Creer que un error descalifica todo el camino.</t>
+        </is>
+      </c>
+      <c r="K255" s="61" t="inlineStr">
+        <is>
+          <t>Si tropezaste, pedí perdón y seguí corriendo.</t>
+        </is>
+      </c>
+      <c r="L255" s="61" t="inlineStr">
+        <is>
+          <t>Guardar la fe es cuidar lo recibido para pasarlo a otros, como Pablo con Timoteo.</t>
+        </is>
+      </c>
+      <c r="M255" s="61" t="inlineStr">
+        <is>
+          <t>Guardar la fe solo para uno, sin transmitirla.</t>
+        </is>
+      </c>
+      <c r="N255" s="61" t="inlineStr">
+        <is>
+          <t>Elegí a una persona más joven para acompañarla en la fe este año.</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="61" t="n">
+        <v>43</v>
+      </c>
+      <c r="B256" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C256" s="61" t="inlineStr">
+        <is>
+          <t>Contar los días</t>
+        </is>
+      </c>
+      <c r="D256" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 90 es el único salmo atribuido a Moisés.</t>
+        </is>
+      </c>
+      <c r="E256" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 90 (título)</t>
+        </is>
+      </c>
+      <c r="F256" s="61" t="inlineStr">
+        <is>
+          <t>Saber que los días son limitados nos ayuda a no postergar lo importante: un perdón, una palabra de amor, una bendición.</t>
+        </is>
+      </c>
+      <c r="G256" s="61" t="inlineStr">
+        <is>
+          <t>Postergar una reconciliación «para más adelante».</t>
+        </is>
+      </c>
+      <c r="H256" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un perdón pendiente, dalo o pedilo esta semana.</t>
+        </is>
+      </c>
+      <c r="I256" s="61" t="inlineStr">
+        <is>
+          <t>Lo que enseñamos sobre perdonar y amar se transmite casi sin palabras a quienes nos observan, sobre todo a los más jóvenes.</t>
+        </is>
+      </c>
+      <c r="J256" s="61" t="inlineStr">
+        <is>
+          <t>Enseñar a perdonar con palabras y guardar rencores en la práctica.</t>
+        </is>
+      </c>
+      <c r="K256" s="61" t="inlineStr">
+        <is>
+          <t>Que tus hijos te vean hoy pedir perdón o perdonar.</t>
+        </is>
+      </c>
+      <c r="L256" s="61" t="inlineStr">
+        <is>
+          <t>Bendecir es decir bien del otro. Una bendición dicha a tiempo queda grabada por años.</t>
+        </is>
+      </c>
+      <c r="M256" s="61" t="inlineStr">
+        <is>
+          <t>Familias donde solo se habla para criticar.</t>
+        </is>
+      </c>
+      <c r="N256" s="61" t="inlineStr">
+        <is>
+          <t>Esta noche, bendecí a tus hijos o a tus seres queridos con una palabra o una oración en voz alta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="61" t="n">
+        <v>43</v>
+      </c>
+      <c r="B257" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C257" s="61" t="inlineStr">
+        <is>
+          <t>Un buen nombre</t>
+        </is>
+      </c>
+      <c r="D257" s="61" t="inlineStr">
+        <is>
+          <t>En hebreo hay un juego de palabras: «nombre» (shem) y «perfume» (shemen) suenan casi igual.</t>
+        </is>
+      </c>
+      <c r="E257" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés 7:1 (texto hebreo)</t>
+        </is>
+      </c>
+      <c r="F257" s="61" t="inlineStr">
+        <is>
+          <t>Un buen nombre, como un perfume, se percibe aunque no se vea. Se construye amando y perdonando cada día.</t>
+        </is>
+      </c>
+      <c r="G257" s="61" t="inlineStr">
+        <is>
+          <t>Cuidar la imagen en las redes y descuidar el carácter en casa.</t>
+        </is>
+      </c>
+      <c r="H257" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy algo bueno por alguien sin que nadie se entere.</t>
+        </is>
+      </c>
+      <c r="I257" s="61" t="inlineStr">
+        <is>
+          <t>Al final de la vida no quedan las posesiones, sino el nombre. Por eso el versículo valora el día en que una vida se cumple con buen nombre. No es un deseo de morir: si alguien piensa en la muerte como salida, que hoy mismo busque ayuda.</t>
+        </is>
+      </c>
+      <c r="J257" s="61" t="inlineStr">
+        <is>
+          <t>Callar el dolor y cargarlo solo.</t>
+        </is>
+      </c>
+      <c r="K257" s="61" t="inlineStr">
+        <is>
+          <t>Si te cuesta seguir, buscá ayuda hoy: hablá con alguien de confianza o acercate a un centro de salud.</t>
+        </is>
+      </c>
+      <c r="L257" s="61" t="inlineStr">
+        <is>
+          <t>Lo que dejamos en otros es cómo los tratamos. Amar a los de casa es la forma más segura de dejar un buen nombre.</t>
+        </is>
+      </c>
+      <c r="M257" s="61" t="inlineStr">
+        <is>
+          <t>Ser amables con todos y duros con los de casa.</t>
+        </is>
+      </c>
+      <c r="N257" s="61" t="inlineStr">
+        <is>
+          <t>Decile hoy a alguien de tu familia cuánto lo querés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="61" t="n">
+        <v>43</v>
+      </c>
+      <c r="B258" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C258" s="61" t="inlineStr">
+        <is>
+          <t>Dios lo cambió para bien</t>
+        </is>
+      </c>
+      <c r="D258" s="61" t="inlineStr">
+        <is>
+          <t>José fue vendido por sus hermanos a los 17 años, y los volvió a ver más de veinte años después.</t>
+        </is>
+      </c>
+      <c r="E258" s="61" t="inlineStr">
+        <is>
+          <t>Génesis 37:2; 41:46; 45:6</t>
+        </is>
+      </c>
+      <c r="F258" s="61" t="inlineStr">
+        <is>
+          <t>José no dice que el mal fue bueno: dice que Dios lo usó para salvar vidas. Hablar del futuro con esperanza no es negar el dolor.</t>
+        </is>
+      </c>
+      <c r="G258" s="61" t="inlineStr">
+        <is>
+          <t>Decirle a alguien que sufre «todo pasa por algo», sin acompañarlo.</t>
+        </is>
+      </c>
+      <c r="H258" s="61" t="inlineStr">
+        <is>
+          <t>Si alguien te cuenta un dolor, escuchá primero, antes de dar explicaciones.</t>
+        </is>
+      </c>
+      <c r="I258" s="61" t="inlineStr">
+        <is>
+          <t>José no sabía el final cuando estaba en la cárcel. Hablar del futuro con sabiduría es dar esperanza sin prometer certezas que no tenemos.</t>
+        </is>
+      </c>
+      <c r="J258" s="61" t="inlineStr">
+        <is>
+          <t>Prometerles a los jóvenes un futuro fácil, o asustarlos con un futuro negro.</t>
+        </is>
+      </c>
+      <c r="K258" s="61" t="inlineStr">
+        <is>
+          <t>Conversá con un joven sobre su futuro: escuchá sus planes y compartí tu esperanza en Dios.</t>
+        </is>
+      </c>
+      <c r="L258" s="61" t="inlineStr">
+        <is>
+          <t>José perdonó a sus hermanos y cuidó de sus familias (50:21). El perdón cambió la historia de toda la familia.</t>
+        </is>
+      </c>
+      <c r="M258" s="61" t="inlineStr">
+        <is>
+          <t>Heridas familiares que se heredan de generación en generación.</t>
+        </is>
+      </c>
+      <c r="N258" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en una herida familiar que no querés pasarles a tus hijos, y pedile a Dios ayuda para sanarla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="61" t="n">
+        <v>43</v>
+      </c>
+      <c r="B259" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C259" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: el legado que dejamos</t>
+        </is>
+      </c>
+      <c r="D259" s="61" t="inlineStr">
+        <is>
+          <t>Hebreos 11 menciona a Abel como el primero de una larga lista de personas que vivieron por la fe.</t>
+        </is>
+      </c>
+      <c r="E259" s="61" t="inlineStr">
+        <is>
+          <t>Hebreos 11:4-40</t>
+        </is>
+      </c>
+      <c r="F259" s="61" t="inlineStr">
+        <is>
+          <t>El legado más duradero es la fe, los valores y el ejemplo, construidos día a día hasta el final.</t>
+        </is>
+      </c>
+      <c r="G259" s="61" t="n"/>
+      <c r="H259" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, escribile una carta o un mensaje a alguien más joven contándole lo que aprendiste de Dios y lo que te gustaría que recuerde.</t>
+        </is>
+      </c>
+      <c r="I259" s="61" t="inlineStr">
+        <is>
+          <t>Perdonar, bendecir y amar se enseña con el ejemplo, sin postergarlo.</t>
+        </is>
+      </c>
+      <c r="J259" s="61" t="n"/>
+      <c r="K259" s="61" t="n"/>
+      <c r="L259" s="61" t="inlineStr">
+        <is>
+          <t>Hablar del futuro con esperanza, sin prometer certezas, prepara a quienes formamos.</t>
+        </is>
+      </c>
+      <c r="M259" s="61" t="n"/>
+      <c r="N259" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de octubre verificados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -9099,7 +9099,7 @@
         <is>
           <t>• El contraste de los recursos humanos frente a los divinos
 • La autoridad del respaldo divino
-• La batalla es del Señor (17:47)</t>
+• La victoria es del Señor (17:47)</t>
         </is>
       </c>
       <c r="AF41" s="10" t="inlineStr">
@@ -35099,7 +35099,7 @@
       </c>
       <c r="L238" s="61" t="inlineStr">
         <is>
-          <t>David reconoce que la batalla es del Señor (17:47). Un líder con propósito hace su parte y confía el resultado a Dios.</t>
+          <t>David reconoce que la victoria es del Señor (17:47). Un líder con propósito hace su parte y confía el resultado a Dios.</t>
         </is>
       </c>
       <c r="M238" s="61" t="inlineStr">
@@ -35459,12 +35459,12 @@
       </c>
       <c r="D244" s="61" t="inlineStr">
         <is>
-          <t>Según la Organización Internacional del Trabajo, las mujeres realizan en el mundo cerca de tres cuartas partes del trabajo de cuidado no remunerado.</t>
+          <t>Según la Organización Internacional del Trabajo, las mujeres realizan en el mundo el 76,2 % del trabajo de cuidado no remunerado: unas tres cuartas partes.</t>
         </is>
       </c>
       <c r="E244" s="61" t="inlineStr">
         <is>
-          <t>Organización Internacional del Trabajo, El trabajo de cuidados y los trabajadores del cuidado, 2018</t>
+          <t>Organización Internacional del Trabajo, El trabajo de cuidados y los trabajadores del cuidado para un futuro con trabajo decente, 2018</t>
         </is>
       </c>
       <c r="F244" s="61" t="inlineStr">
@@ -35529,7 +35529,7 @@
       </c>
       <c r="D245" s="61" t="inlineStr">
         <is>
-          <t>Un estudio encontró que expresar gratitud a la pareja se asocia con una relación más satisfactoria para los dos.</t>
+          <t>Un estudio con parejas encontró que sentir gratitud por los pequeños gestos del otro se asociaba, al día siguiente, con una relación más conectada y satisfactoria para los dos.</t>
         </is>
       </c>
       <c r="E245" s="61" t="inlineStr">
@@ -35719,7 +35719,7 @@
       </c>
       <c r="D248" s="61" t="inlineStr">
         <is>
-          <t>En la ley de Moisés, parte del diezmo se destinaba a los levitas, a los extranjeros, a los huérfanos y a las viudas.</t>
+          <t>En la ley de Moisés, cada tres años el diezmo de la cosecha se guardaba en cada ciudad para los levitas, los extranjeros, los huérfanos y las viudas.</t>
         </is>
       </c>
       <c r="E248" s="61" t="inlineStr">
@@ -35859,7 +35859,7 @@
       </c>
       <c r="D250" s="61" t="inlineStr">
         <is>
-          <t>La imagen viene del mercado de granos: el vendedor generoso apretaba y sacudía el grano para que la medida quedara llena hasta rebalsar.</t>
+          <t>La imagen viene de la medición del grano: se apretaba y se sacudía para que la medida quedara llena hasta rebalsar, y se volcaba en el pliegue del manto de quien la recibía.</t>
         </is>
       </c>
       <c r="E250" s="61" t="inlineStr">
@@ -36189,12 +36189,12 @@
       </c>
       <c r="D255" s="61" t="inlineStr">
         <is>
-          <t>Pablo usa tres imágenes seguidas: la de un soldado, la de un corredor y la de alguien que cuida lo que se le confió.</t>
+          <t>Pablo usa tres imágenes seguidas: la de un atleta que lucha en una competencia, la de un corredor que llega a la meta y la de alguien que cuida fielmente lo que se le confió.</t>
         </is>
       </c>
       <c r="E255" s="61" t="inlineStr">
         <is>
-          <t>2 Timoteo 4:7</t>
+          <t>2 Timoteo 4:7 (texto griego)</t>
         </is>
       </c>
       <c r="F255" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: guiones de noviembre con revisión teológica
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -10085,7 +10085,7 @@
       <c r="Y46" s="6" t="inlineStr">
         <is>
           <t>• El samaritano actuó de inmediato ante la necesidad
-• Vendar heridas es acto de compasión practica
+• Vendar heridas es acto de compasión práctica
 • La ayuda concreta refleja el amor al prójimo</t>
         </is>
       </c>
@@ -10099,7 +10099,7 @@
         <is>
           <t>• Dios es refugio y fortaleza en la angustia
 • Su auxilio llega pronto en la tribulación
-• La confianza en El calma la emergencia</t>
+• La confianza en Él calma la emergencia</t>
         </is>
       </c>
       <c r="AB46" s="6" t="inlineStr">
@@ -10110,7 +10110,7 @@
       </c>
       <c r="AC46" s="6" t="inlineStr">
         <is>
-          <t>• Actuar para librar a quien esta en peligro
+          <t>• Actuar para librar a quien está en peligro
 • No quedarse indiferente ante la necesidad ajena
 • La responsabilidad de ayudar es real</t>
         </is>
@@ -10138,7 +10138,7 @@
         <is>
           <t>• Dios oye el clamor de los justos
 • Libra de las angustias a quien clama
-• La oración en emergencia tiene respuesta</t>
+• Dios está cerca del que sufre (34:18)</t>
         </is>
       </c>
       <c r="AH46" s="6" t="inlineStr">
@@ -10148,7 +10148,7 @@
       </c>
       <c r="AI46" s="6" t="inlineStr">
         <is>
-          <t>• No temer porque Dios esta presente
+          <t>• No temer porque Dios está presente
 • Su fortaleza sostiene en el momento crítico
 • El pánico se enfrenta con esa promesa</t>
         </is>
@@ -10326,14 +10326,14 @@
       </c>
       <c r="AE47" s="8" t="inlineStr">
         <is>
-          <t>• • La oración como respuesta al sufrimiento.
-• • La alabanza como expresión de gratitud.
-• • Una fe para todas las estaciones de la vida.</t>
+          <t>• La oración como respuesta al sufrimiento.
+• La alabanza como expresión de gratitud.
+• Una fe para todas las estaciones de la vida.</t>
         </is>
       </c>
       <c r="AF47" s="8" t="inlineStr">
         <is>
-          <t>Salmo 150:6 — Que todo lo que respira alabe al Senor! Aleluya</t>
+          <t>Salmo 150:6 — ¡Que todo lo que respira alabe al Señor! ¡Aleluya!</t>
         </is>
       </c>
       <c r="AG47" s="8" t="inlineStr">
@@ -10372,7 +10372,7 @@
         <is>
           <t>• La pérdida material no define la relación con Dios.
 • El gozo como una decisión espiritual.
-• La fortaleza y la elevación sobrenatural.</t>
+• Dios da fuerza para seguir caminando.</t>
         </is>
       </c>
     </row>
@@ -10499,7 +10499,7 @@
       <c r="Y48" s="10" t="inlineStr">
         <is>
           <t>• Pedir sabiduría a Dios sin condiciones
-• El da generosamente y sin reproche
+• Él da generosamente y sin reproche
 • La falta de sabiduría no es motivo de vergüenza</t>
         </is>
       </c>
@@ -10513,7 +10513,7 @@
         <is>
           <t>• Confiar en Dios más que en el propio entendimiento
 • Reconocerlo en todos los caminos
-• El endereza las veredas</t>
+• Él endereza las veredas</t>
         </is>
       </c>
       <c r="AB48" s="10" t="inlineStr">
@@ -19212,7 +19212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N259"/>
+  <dimension ref="A1:N283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -36502,6 +36502,1606 @@
       </c>
       <c r="M259" s="61" t="n"/>
       <c r="N259" s="61" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="61" t="n">
+        <v>44</v>
+      </c>
+      <c r="B260" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C260" s="61" t="inlineStr">
+        <is>
+          <t>A cada uno lo que corresponde</t>
+        </is>
+      </c>
+      <c r="D260" s="61" t="inlineStr">
+        <is>
+          <t>En el griego, Romanos 13:7 nombra dos clases de impuestos del Imperio romano: el tributo directo (phóros) y las tasas o aduanas (télos).</t>
+        </is>
+      </c>
+      <c r="E260" s="61" t="inlineStr">
+        <is>
+          <t>Romanos 13:7 (texto griego)</t>
+        </is>
+      </c>
+      <c r="F260" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide pagar lo que corresponde, incluso a un gobierno que no era cristiano. Trabajar como para Dios incluye cumplir las obligaciones, aunque nadie controle.</t>
+        </is>
+      </c>
+      <c r="G260" s="61" t="inlineStr">
+        <is>
+          <t>Hacer solo lo que se controla y evitar lo demás.</t>
+        </is>
+      </c>
+      <c r="H260" s="61" t="inlineStr">
+        <is>
+          <t>Revisá si tenés alguna obligación de trabajo pendiente, un trámite, un aporte o una entrega, y cumplila esta semana.</t>
+        </is>
+      </c>
+      <c r="I260" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo hecho para Dios se nota en el trato: al jefe, al compañero y al cliente.</t>
+        </is>
+      </c>
+      <c r="J260" s="61" t="inlineStr">
+        <is>
+          <t>Respetar solo a quien tiene más poder.</t>
+        </is>
+      </c>
+      <c r="K260" s="61" t="inlineStr">
+        <is>
+          <t>Tratá hoy con el mismo respeto al que limpia y al que dirige.</t>
+        </is>
+      </c>
+      <c r="L260" s="61" t="inlineStr">
+        <is>
+          <t>Honrar es reconocer el valor del trabajo de otros. Cambiar la motivación, de «que no me despidan» a «lo hago para Dios», cambia la calidad del esfuerzo.</t>
+        </is>
+      </c>
+      <c r="M260" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar bien solo cuando mira el jefe.</t>
+        </is>
+      </c>
+      <c r="N260" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy una tarea que nadie va a revisar como si fuera para Dios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="61" t="n">
+        <v>44</v>
+      </c>
+      <c r="B261" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C261" s="61" t="inlineStr">
+        <is>
+          <t>Manos para el bien</t>
+        </is>
+      </c>
+      <c r="D261" s="61" t="inlineStr">
+        <is>
+          <t>En el griego, el «trabaje» de este versículo indica un esfuerzo que cansa: trabajar hasta fatigarse.</t>
+        </is>
+      </c>
+      <c r="E261" s="61" t="inlineStr">
+        <is>
+          <t>Efesios 4:28; léxico griego de Strong (G2872, kopiáo)</t>
+        </is>
+      </c>
+      <c r="F261" s="61" t="inlineStr">
+        <is>
+          <t>Pablo habla de alguien que antes robaba: el cambio no es solo dejar de robar, sino empezar a trabajar honradamente.</t>
+        </is>
+      </c>
+      <c r="G261" s="61" t="inlineStr">
+        <is>
+          <t>Ganar plata de formas que perjudican a otros.</t>
+        </is>
+      </c>
+      <c r="H261" s="61" t="inlineStr">
+        <is>
+          <t>Revisá si en tu trabajo hay algo que no es del todo honesto, y corregilo.</t>
+        </is>
+      </c>
+      <c r="I261" s="61" t="inlineStr">
+        <is>
+          <t>El propósito del trabajo va más allá del propio sustento: también sirve para ayudar a otros.</t>
+        </is>
+      </c>
+      <c r="J261" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que el sueldo es solo para uno.</t>
+        </is>
+      </c>
+      <c r="K261" s="61" t="inlineStr">
+        <is>
+          <t>Separá algo de lo que ganes esta semana para ayudar a alguien.</t>
+        </is>
+      </c>
+      <c r="L261" s="61" t="inlineStr">
+        <is>
+          <t>Todo trabajo honrado puede hacerse para Dios, también el que se hace con las manos.</t>
+        </is>
+      </c>
+      <c r="M261" s="61" t="inlineStr">
+        <is>
+          <t>Despreciar el trabajo manual.</t>
+        </is>
+      </c>
+      <c r="N261" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy el trabajo de alguien que tiene un oficio manual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="61" t="n">
+        <v>44</v>
+      </c>
+      <c r="B262" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C262" s="61" t="inlineStr">
+        <is>
+          <t>El propio pan</t>
+        </is>
+      </c>
+      <c r="D262" s="61" t="inlineStr">
+        <is>
+          <t>En Tesalónica algunos habían dejado de trabajar, quizás pensando que Jesús volvería enseguida, y vivían a costa de otros.</t>
+        </is>
+      </c>
+      <c r="E262" s="61" t="inlineStr">
+        <is>
+          <t>2 Tesalonicenses 3:6-12; comentarios bíblicos</t>
+        </is>
+      </c>
+      <c r="F262" s="61" t="inlineStr">
+        <is>
+          <t>Pablo pide a quienes no querían trabajar que trabajen con tranquilidad. No habla de quien no puede trabajar por enfermedad o por falta de empleo.</t>
+        </is>
+      </c>
+      <c r="G262" s="61" t="inlineStr">
+        <is>
+          <t>Juzgar a quien hoy no tiene trabajo.</t>
+        </is>
+      </c>
+      <c r="H262" s="61" t="inlineStr">
+        <is>
+          <t>Si conocés a alguien que busca trabajo, compartile una oportunidad o una recomendación.</t>
+        </is>
+      </c>
+      <c r="I262" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo no es solo para pagar cuentas: también es un lugar donde se vive el propósito, se sirve a otros y se usan los dones recibidos.</t>
+        </is>
+      </c>
+      <c r="J262" s="61" t="inlineStr">
+        <is>
+          <t>Vivir el trabajo solo como una carga hasta el fin de semana.</t>
+        </is>
+      </c>
+      <c r="K262" s="61" t="inlineStr">
+        <is>
+          <t>Pensá qué parte de tu trabajo conecta con algo más grande que el sueldo.</t>
+        </is>
+      </c>
+      <c r="L262" s="61" t="inlineStr">
+        <is>
+          <t>Ganarse el pan da dignidad. Y cuando hay necesidad real, recibir ayuda no quita dignidad.</t>
+        </is>
+      </c>
+      <c r="M262" s="61" t="inlineStr">
+        <is>
+          <t>Avergonzarse de pedir ayuda cuando de verdad se necesita.</t>
+        </is>
+      </c>
+      <c r="N262" s="61" t="inlineStr">
+        <is>
+          <t>Si estás en una situación difícil, animate a pedir ayuda a tu iglesia o a tu familia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="61" t="n">
+        <v>44</v>
+      </c>
+      <c r="B263" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C263" s="61" t="inlineStr">
+        <is>
+          <t>Toda labor rinde</t>
+        </is>
+      </c>
+      <c r="D263" s="61" t="inlineStr">
+        <is>
+          <t>En la Biblia, el trabajo aparece antes de la caída: Dios puso al ser humano en el huerto para que lo cultivara y lo cuidara.</t>
+        </is>
+      </c>
+      <c r="E263" s="61" t="inlineStr">
+        <is>
+          <t>Génesis 2:15</t>
+        </is>
+      </c>
+      <c r="F263" s="61" t="inlineStr">
+        <is>
+          <t>Este proverbio enseña un principio: el trabajo da fruto, aunque no siempre se vea enseguida ni sea en plata.</t>
+        </is>
+      </c>
+      <c r="G263" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que un trabajo sencillo no da ningún fruto.</t>
+        </is>
+      </c>
+      <c r="H263" s="61" t="inlineStr">
+        <is>
+          <t>Anotá un fruto de tu trabajo de esta semana que no sea el sueldo.</t>
+        </is>
+      </c>
+      <c r="I263" s="61" t="inlineStr">
+        <is>
+          <t>Hablar mucho de lo que vamos a hacer no reemplaza hacerlo. El propósito se vive en lo cotidiano.</t>
+        </is>
+      </c>
+      <c r="J263" s="61" t="inlineStr">
+        <is>
+          <t>Planes y promesas que nunca pasan a la acción.</t>
+        </is>
+      </c>
+      <c r="K263" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un plan del que venís hablando hace tiempo y da hoy el primer paso.</t>
+        </is>
+      </c>
+      <c r="L263" s="61" t="inlineStr">
+        <is>
+          <t>Dios nos dio el trabajo como parte de su diseño, no como un castigo.</t>
+        </is>
+      </c>
+      <c r="M263" s="61" t="inlineStr">
+        <is>
+          <t>Ver el trabajo como una maldición.</t>
+        </is>
+      </c>
+      <c r="N263" s="61" t="inlineStr">
+        <is>
+          <t>Empezá mañana tu jornada agradeciéndole a Dios por tu trabajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="61" t="n">
+        <v>44</v>
+      </c>
+      <c r="B264" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C264" s="61" t="inlineStr">
+        <is>
+          <t>Disfrutar del trabajo</t>
+        </is>
+      </c>
+      <c r="D264" s="61" t="inlineStr">
+        <is>
+          <t>Jesús fue conocido en Nazaret como artesano; la palabra griega (tékton) se usaba para el carpintero o el constructor.</t>
+        </is>
+      </c>
+      <c r="E264" s="61" t="inlineStr">
+        <is>
+          <t>Marcos 6:3; léxico griego de Strong (G5045, tékton)</t>
+        </is>
+      </c>
+      <c r="F264" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés ve el disfrute del trabajo como un regalo de Dios (3:13). Ningún oficio hecho con honestidad es menor.</t>
+        </is>
+      </c>
+      <c r="G264" s="61" t="inlineStr">
+        <is>
+          <t>Mirar con desprecio oficios como la limpieza, las changas o los trabajos manuales.</t>
+        </is>
+      </c>
+      <c r="H264" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy, por su nombre, a alguien que hace un trabajo que suele pasar desapercibido.</t>
+        </is>
+      </c>
+      <c r="I264" s="61" t="inlineStr">
+        <is>
+          <t>Jesús trabajó años como artesano antes de su ministerio. La dignidad del trabajo no depende del prestigio, sino de cómo se hace.</t>
+        </is>
+      </c>
+      <c r="J264" s="61" t="inlineStr">
+        <is>
+          <t>Medir el valor de una persona por su título o su cargo.</t>
+        </is>
+      </c>
+      <c r="K264" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy tu trabajo con excelencia, aunque nadie lo valore.</t>
+        </is>
+      </c>
+      <c r="L264" s="61" t="inlineStr">
+        <is>
+          <t>El sabio reconoce que no sabemos lo que vendrá; por eso invita a disfrutar con gratitud el trabajo de hoy.</t>
+        </is>
+      </c>
+      <c r="M264" s="61" t="inlineStr">
+        <is>
+          <t>Vivir esperando un trabajo «mejor» sin valorar el actual.</t>
+        </is>
+      </c>
+      <c r="N264" s="61" t="inlineStr">
+        <is>
+          <t>Encontrá hoy algo de tu trabajo que disfrutás, y agradecéselo a Dios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="61" t="n">
+        <v>44</v>
+      </c>
+      <c r="B265" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C265" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: el trabajo digno</t>
+        </is>
+      </c>
+      <c r="D265" s="61" t="inlineStr">
+        <is>
+          <t>Pablo cita aquí dos textos: uno de la ley de Moisés y otro que coincide con palabras de Jesús.</t>
+        </is>
+      </c>
+      <c r="E265" s="61" t="inlineStr">
+        <is>
+          <t>Deuteronomio 25:4; Lucas 10:7</t>
+        </is>
+      </c>
+      <c r="F265" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar como para Dios cambia la calidad del esfuerzo, también cuando nadie mira.</t>
+        </is>
+      </c>
+      <c r="G265" s="61" t="n"/>
+      <c r="H265" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, agradecé a un trabajador que suele pasar desapercibido y, si das trabajo a alguien, revisá que su pago sea justo y a tiempo.</t>
+        </is>
+      </c>
+      <c r="I265" s="61" t="inlineStr">
+        <is>
+          <t>El trabajo es parte del propósito: sirve a otros y permite compartir.</t>
+        </is>
+      </c>
+      <c r="J265" s="61" t="n"/>
+      <c r="K265" s="61" t="n"/>
+      <c r="L265" s="61" t="inlineStr">
+        <is>
+          <t>Todo oficio honesto es digno, y quien trabaja merece un salario justo.</t>
+        </is>
+      </c>
+      <c r="M265" s="61" t="n"/>
+      <c r="N265" s="61" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="61" t="n">
+        <v>45</v>
+      </c>
+      <c r="B266" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C266" s="61" t="inlineStr">
+        <is>
+          <t>Pronto auxilio</t>
+        </is>
+      </c>
+      <c r="D266" s="61" t="inlineStr">
+        <is>
+          <t>La reanimación cardiopulmonar hecha por un testigo, antes de que llegue la ambulancia, puede duplicar o triplicar las posibilidades de sobrevivir a un paro cardíaco.</t>
+        </is>
+      </c>
+      <c r="E266" s="61" t="inlineStr">
+        <is>
+          <t>American Heart Association</t>
+        </is>
+      </c>
+      <c r="F266" s="61" t="inlineStr">
+        <is>
+          <t>El salmista confía en Dios en medio de terremotos y guerras. La confianza en Dios no reemplaza la preparación: nos da calma para actuar.</t>
+        </is>
+      </c>
+      <c r="G266" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que la fe nos exime de prepararnos.</t>
+        </is>
+      </c>
+      <c r="H266" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, averiguá dónde podés hacer un curso de primeros auxilios.</t>
+        </is>
+      </c>
+      <c r="I266" s="61" t="inlineStr">
+        <is>
+          <t>Cualquier persona puede aprender lo básico: llamar a emergencias, hacer compresiones en el pecho y controlar un sangrado presionando la herida.</t>
+        </is>
+      </c>
+      <c r="J266" s="61" t="inlineStr">
+        <is>
+          <t>Creer que solo los médicos pueden ayudar.</t>
+        </is>
+      </c>
+      <c r="K266" s="61" t="inlineStr">
+        <is>
+          <t>Miren en familia un video de una fuente seria, como la Cruz Roja, sobre la RCP solo con las manos.</t>
+        </is>
+      </c>
+      <c r="L266" s="61" t="inlineStr">
+        <is>
+          <t>Saber qué hacer da tranquilidad. Y la oración acompaña la acción; no la reemplaza.</t>
+        </is>
+      </c>
+      <c r="M266" s="61" t="inlineStr">
+        <is>
+          <t>Quedarse paralizado sin saber qué hacer.</t>
+        </is>
+      </c>
+      <c r="N266" s="61" t="inlineStr">
+        <is>
+          <t>Guardá en tu celular los números de emergencia de tu zona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="61" t="n">
+        <v>45</v>
+      </c>
+      <c r="B267" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C267" s="61" t="inlineStr">
+        <is>
+          <t>Actuar a tiempo</t>
+        </is>
+      </c>
+      <c r="D267" s="61" t="inlineStr">
+        <is>
+          <t>En la RCP se recomienda comprimir el centro del pecho a un ritmo de 100 a 120 compresiones por minuto.</t>
+        </is>
+      </c>
+      <c r="E267" s="61" t="inlineStr">
+        <is>
+          <t>American Heart Association, guías de RCP, 2020</t>
+        </is>
+      </c>
+      <c r="F267" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio pide no quedarse de brazos cruzados ante quien está en peligro. En una emergencia, cada minuto cuenta.</t>
+        </is>
+      </c>
+      <c r="G267" s="61" t="inlineStr">
+        <is>
+          <t>Mirar o filmar en vez de ayudar.</t>
+        </is>
+      </c>
+      <c r="H267" s="61" t="inlineStr">
+        <is>
+          <t>Si ves una emergencia, lo primero es pedir ayuda: llamá a emergencias.</t>
+        </is>
+      </c>
+      <c r="I267" s="61" t="inlineStr">
+        <is>
+          <t>El versículo siguiente advierte que no sirve decir «no lo sabíamos» (24:12). Aprender lo básico es una forma de amar al prójimo.</t>
+        </is>
+      </c>
+      <c r="J267" s="61" t="inlineStr">
+        <is>
+          <t>Pensar «alguien más va a ayudar».</t>
+        </is>
+      </c>
+      <c r="K267" s="61" t="inlineStr">
+        <is>
+          <t>Si hay varias personas, señalá a una y pedile directamente que llame a emergencias.</t>
+        </is>
+      </c>
+      <c r="L267" s="61" t="inlineStr">
+        <is>
+          <t>Ayudar con lo que se sabe, aunque sea poco, es mejor que no hacer nada. Pero sin arriesgarse de forma imprudente: primero, que el lugar sea seguro.</t>
+        </is>
+      </c>
+      <c r="M267" s="61" t="inlineStr">
+        <is>
+          <t>Exponerse a un peligro sin pensar y terminar siendo otra víctima.</t>
+        </is>
+      </c>
+      <c r="N267" s="61" t="inlineStr">
+        <is>
+          <t>Antes de acercarte a ayudar, fijate que el lugar sea seguro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="61" t="n">
+        <v>45</v>
+      </c>
+      <c r="B268" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C268" s="61" t="inlineStr">
+        <is>
+          <t>Llamar a otros</t>
+        </is>
+      </c>
+      <c r="D268" s="61" t="inlineStr">
+        <is>
+          <t>En el mundo antiguo, el aceite de oliva también se usaba como remedio para las heridas, como hizo el buen samaritano.</t>
+        </is>
+      </c>
+      <c r="E268" s="61" t="inlineStr">
+        <is>
+          <t>Lucas 10:34; Isaías 1:6</t>
+        </is>
+      </c>
+      <c r="F268" s="61" t="inlineStr">
+        <is>
+          <t>Santiago pide al enfermo que llame a otros. En una emergencia, el primer paso es pedir ayuda: llamar al número de emergencia antes que nada.</t>
+        </is>
+      </c>
+      <c r="G268" s="61" t="inlineStr">
+        <is>
+          <t>Intentar resolver todo solo y perder minutos valiosos.</t>
+        </is>
+      </c>
+      <c r="H268" s="61" t="inlineStr">
+        <is>
+          <t>Enseñales a tus hijos cómo y a qué número llamar en una emergencia.</t>
+        </is>
+      </c>
+      <c r="I268" s="61" t="inlineStr">
+        <is>
+          <t>Orar y buscar atención médica van juntos; la Biblia no opone la oración al médico. Las iglesias practican la unción de maneras distintas, pero todas oran por los enfermos. Y Santiago no dice que toda enfermedad sea por un pecado: dice «si acaso».</t>
+        </is>
+      </c>
+      <c r="J268" s="61" t="inlineStr">
+        <is>
+          <t>Dejar de buscar atención médica por pensar que es falta de fe.</t>
+        </is>
+      </c>
+      <c r="K268" s="61" t="inlineStr">
+        <is>
+          <t>Cuando alguien esté enfermo, orá por él y acompañalo también al médico.</t>
+        </is>
+      </c>
+      <c r="L268" s="61" t="inlineStr">
+        <is>
+          <t>Respirar, mirar la situación con calma y actuar con lo que se sabe ayuda a no entrar en pánico. Tener a alguien al lado también calma.</t>
+        </is>
+      </c>
+      <c r="M268" s="61" t="inlineStr">
+        <is>
+          <t>El pánico que paraliza más que la falta de conocimiento.</t>
+        </is>
+      </c>
+      <c r="N268" s="61" t="inlineStr">
+        <is>
+          <t>Si estás en una emergencia, respirá hondo, pedí ayuda y hacé una cosa por vez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="61" t="n">
+        <v>45</v>
+      </c>
+      <c r="B269" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C269" s="61" t="inlineStr">
+        <is>
+          <t>El Señor escucha</t>
+        </is>
+      </c>
+      <c r="D269" s="61" t="inlineStr">
+        <is>
+          <t>El título del Salmo 34 lo relaciona con un momento de peligro en la vida de David, cuando huía de Saúl.</t>
+        </is>
+      </c>
+      <c r="E269" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 34 (título); 1 Samuel 21:10-15</t>
+        </is>
+      </c>
+      <c r="F269" s="61" t="inlineStr">
+        <is>
+          <t>David escribió desde el peligro. En una emergencia, clamar a Dios es natural, y él escucha.</t>
+        </is>
+      </c>
+      <c r="G269" s="61" t="inlineStr">
+        <is>
+          <t>Sentir que en el momento crítico estamos solos.</t>
+        </is>
+      </c>
+      <c r="H269" s="61" t="inlineStr">
+        <is>
+          <t>Aprendé una oración corta para los momentos de emergencia, como «Señor, ayudame».</t>
+        </is>
+      </c>
+      <c r="I269" s="61" t="inlineStr">
+        <is>
+          <t>El mismo salmo reconoce que el justo pasa muchas aflicciones (34:19). Dios no promete que no habrá emergencias, sino que estará presente en ellas.</t>
+        </is>
+      </c>
+      <c r="J269" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que si algo malo pasó es porque Dios no escuchó.</t>
+        </is>
+      </c>
+      <c r="K269" s="61" t="inlineStr">
+        <is>
+          <t>Si estás pasando una angustia, contásela hoy a Dios y a alguien de confianza.</t>
+        </is>
+      </c>
+      <c r="L269" s="61" t="inlineStr">
+        <is>
+          <t>Mantener la calma es más fácil cuando sabemos que no estamos solos. La fe sostiene mientras hacemos lo que hay que hacer.</t>
+        </is>
+      </c>
+      <c r="M269" s="61" t="inlineStr">
+        <is>
+          <t>Dejar que el miedo decida por nosotros.</t>
+        </is>
+      </c>
+      <c r="N269" s="61" t="inlineStr">
+        <is>
+          <t>Practiquen en familia qué harían ante una emergencia en casa: quién llama y quién ayuda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="61" t="n">
+        <v>45</v>
+      </c>
+      <c r="B270" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C270" s="61" t="inlineStr">
+        <is>
+          <t>No tengas miedo</t>
+        </is>
+      </c>
+      <c r="D270" s="61" t="inlineStr">
+        <is>
+          <t>En Paraguay, el 141 es el número del Servicio de Emergencias Médicas Extrahospitalarias (SEME), y el 911 el del sistema de emergencias.</t>
+        </is>
+      </c>
+      <c r="E270" s="61" t="inlineStr">
+        <is>
+          <t>Ministerio de Salud Pública y Bienestar Social; Sistema 911</t>
+        </is>
+      </c>
+      <c r="F270" s="61" t="inlineStr">
+        <is>
+          <t>Dios le habla a su pueblo en el exilio: «No tengas miedo, que yo estoy contigo». Su presencia no quita la emergencia, pero sí el pánico.</t>
+        </is>
+      </c>
+      <c r="G270" s="61" t="inlineStr">
+        <is>
+          <t>Tomar decisiones por miedo en el peor momento.</t>
+        </is>
+      </c>
+      <c r="H270" s="61" t="inlineStr">
+        <is>
+          <t>Repetí este versículo cuando sientas miedo esta semana.</t>
+        </is>
+      </c>
+      <c r="I270" s="61" t="inlineStr">
+        <is>
+          <t>Saber primeros auxilios no reemplaza la atención médica: ayuda a sostener la situación hasta que llegue.</t>
+        </is>
+      </c>
+      <c r="J270" s="61" t="inlineStr">
+        <is>
+          <t>Querer resolver con remedios caseros lo que necesita un médico.</t>
+        </is>
+      </c>
+      <c r="K270" s="61" t="inlineStr">
+        <is>
+          <t>Ante un dolor fuerte en el pecho, dificultad para respirar, desmayo o un sangrado que no para, llamá enseguida a emergencias.</t>
+        </is>
+      </c>
+      <c r="L270" s="61" t="inlineStr">
+        <is>
+          <t>Reconocer cuándo algo nos supera también es sabiduría y humildad.</t>
+        </is>
+      </c>
+      <c r="M270" s="61" t="inlineStr">
+        <is>
+          <t>Esperar a ver si «se pasa solo».</t>
+        </is>
+      </c>
+      <c r="N270" s="61" t="inlineStr">
+        <is>
+          <t>Pegá en un lugar visible de tu casa los números de emergencia y la dirección exacta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="61" t="n">
+        <v>45</v>
+      </c>
+      <c r="B271" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C271" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: preparados para ayudar</t>
+        </is>
+      </c>
+      <c r="D271" s="61" t="inlineStr">
+        <is>
+          <t>La Cruz Roja Paraguaya ofrece cursos de primeros auxilios abiertos a la comunidad.</t>
+        </is>
+      </c>
+      <c r="E271" s="61" t="inlineStr">
+        <is>
+          <t>Cruz Roja Paraguaya</t>
+        </is>
+      </c>
+      <c r="F271" s="61" t="inlineStr">
+        <is>
+          <t>Cualquiera puede aprender lo básico: pedir ayuda, hacer RCP con las manos y controlar un sangrado.</t>
+        </is>
+      </c>
+      <c r="G271" s="61" t="n"/>
+      <c r="H271" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, anoten en familia los números de emergencia, pónganlos en un lugar visible y averigüen dónde hacer un curso de primeros auxilios.</t>
+        </is>
+      </c>
+      <c r="I271" s="61" t="inlineStr">
+        <is>
+          <t>En una emergencia, primero la seguridad y pedir ayuda; la calma y la oración acompañan la acción.</t>
+        </is>
+      </c>
+      <c r="J271" s="61" t="n"/>
+      <c r="K271" s="61" t="n"/>
+      <c r="L271" s="61" t="inlineStr">
+        <is>
+          <t>Los primeros auxilios sostienen hasta que llega la ayuda profesional; reconocer los propios límites es sabiduría.</t>
+        </is>
+      </c>
+      <c r="M271" s="61" t="n"/>
+      <c r="N271" s="61" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="61" t="n">
+        <v>46</v>
+      </c>
+      <c r="B272" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C272" s="61" t="inlineStr">
+        <is>
+          <t>En espíritu y en verdad</t>
+        </is>
+      </c>
+      <c r="D272" s="61" t="inlineStr">
+        <is>
+          <t>Jesús dijo estas palabras a una mujer samaritana, junto al pozo de Jacob, en Sicar.</t>
+        </is>
+      </c>
+      <c r="E272" s="61" t="inlineStr">
+        <is>
+          <t>Juan 4:5-7</t>
+        </is>
+      </c>
+      <c r="F272" s="61" t="inlineStr">
+        <is>
+          <t>La mujer preguntaba dónde había que adorar. Jesús responde que lo importante no es el lugar, sino el corazón y la verdad.</t>
+        </is>
+      </c>
+      <c r="G272" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que solo se adora el domingo en el templo.</t>
+        </is>
+      </c>
+      <c r="H272" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, en medio de tu rutina, tomate un minuto para adorar a Dios donde estés.</t>
+        </is>
+      </c>
+      <c r="I272" s="61" t="inlineStr">
+        <is>
+          <t>Las iglesias adoran con estilos distintos, y todos pueden ser genuinos. Lo que cuenta es la sinceridad.</t>
+        </is>
+      </c>
+      <c r="J272" s="61" t="inlineStr">
+        <is>
+          <t>Criticar la forma de adorar de otras iglesias.</t>
+        </is>
+      </c>
+      <c r="K272" s="61" t="inlineStr">
+        <is>
+          <t>Agradecele a Dios por una forma de adorar distinta de la tuya.</t>
+        </is>
+      </c>
+      <c r="L272" s="61" t="inlineStr">
+        <is>
+          <t>Adorar no depende del ánimo. Está bien adorar sin sentir nada especial: la fidelidad no depende de la emoción del momento.</t>
+        </is>
+      </c>
+      <c r="M272" s="61" t="inlineStr">
+        <is>
+          <t>Dejar de adorar cuando no se siente nada.</t>
+        </is>
+      </c>
+      <c r="N272" s="61" t="inlineStr">
+        <is>
+          <t>Si hoy no tenés ganas, igual decile a Dios una frase de alabanza.</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="61" t="n">
+        <v>46</v>
+      </c>
+      <c r="B273" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C273" s="61" t="inlineStr">
+        <is>
+          <t>En todo tiempo</t>
+        </is>
+      </c>
+      <c r="D273" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 34 es un acróstico: en hebreo, cada versículo empieza con una letra distinta del alfabeto.</t>
+        </is>
+      </c>
+      <c r="E273" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 34 (texto hebreo)</t>
+        </is>
+      </c>
+      <c r="F273" s="61" t="inlineStr">
+        <is>
+          <t>David escribió este salmo después de un momento de peligro, y aun así decide bendecir a Dios en todo tiempo.</t>
+        </is>
+      </c>
+      <c r="G273" s="61" t="inlineStr">
+        <is>
+          <t>Alabar solo cuando todo sale bien.</t>
+        </is>
+      </c>
+      <c r="H273" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una situación difícil de esta semana y agradecele a Dios en medio de ella.</t>
+        </is>
+      </c>
+      <c r="I273" s="61" t="inlineStr">
+        <is>
+          <t>Alabar en todo tiempo no es negar el dolor: los salmos también tienen lamentos, y lamentarse delante de Dios también es adorar.</t>
+        </is>
+      </c>
+      <c r="J273" s="61" t="inlineStr">
+        <is>
+          <t>Fingir alegría para parecer más espiritual.</t>
+        </is>
+      </c>
+      <c r="K273" s="61" t="inlineStr">
+        <is>
+          <t>Si estás triste, contáselo a Dios con sinceridad: eso también es adoración.</t>
+        </is>
+      </c>
+      <c r="L273" s="61" t="inlineStr">
+        <is>
+          <t>La adoración no cambia las circunstancias de inmediato, pero sí la mirada sobre ellas.</t>
+        </is>
+      </c>
+      <c r="M273" s="61" t="inlineStr">
+        <is>
+          <t>Dejar que el problema ocupe todo el horizonte.</t>
+        </is>
+      </c>
+      <c r="N273" s="61" t="inlineStr">
+        <is>
+          <t>Antes de pensar hoy en tu problema, pensá en tres cosas que Dios es.</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="61" t="n">
+        <v>46</v>
+      </c>
+      <c r="B274" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C274" s="61" t="inlineStr">
+        <is>
+          <t>Orar y cantar</t>
+        </is>
+      </c>
+      <c r="D274" s="61" t="inlineStr">
+        <is>
+          <t>Un estudio encontró que, al cantar juntos, el ritmo del corazón de los integrantes de un coro tiende a sincronizarse.</t>
+        </is>
+      </c>
+      <c r="E274" s="61" t="inlineStr">
+        <is>
+          <t>Vickhoff y otros, Frontiers in Psychology, 2013</t>
+        </is>
+      </c>
+      <c r="F274" s="61" t="inlineStr">
+        <is>
+          <t>Santiago tiene una respuesta para cada estado: en el sufrimiento, orar; en la alegría, cantar. Toda la vida se puede llevar delante de Dios.</t>
+        </is>
+      </c>
+      <c r="G274" s="61" t="inlineStr">
+        <is>
+          <t>Guardarse el sufrimiento sin hablarlo con Dios.</t>
+        </is>
+      </c>
+      <c r="H274" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, orá por lo que te duele y cantá por lo que agradecés.</t>
+        </is>
+      </c>
+      <c r="I274" s="61" t="inlineStr">
+        <is>
+          <t>No hace falta un momento formal para adorar. Reconocer con gratitud lo pequeño del día es una forma accesible de adoración.</t>
+        </is>
+      </c>
+      <c r="J274" s="61" t="inlineStr">
+        <is>
+          <t>Agradecer solo por las cosas grandes.</t>
+        </is>
+      </c>
+      <c r="K274" s="61" t="inlineStr">
+        <is>
+          <t>Nombrá ahora tres cosas puntuales de hoy por las que estás agradecido.</t>
+        </is>
+      </c>
+      <c r="L274" s="61" t="inlineStr">
+        <is>
+          <t>Hay estaciones de alegría y de dolor. La gratitud diaria sostiene en las dos.</t>
+        </is>
+      </c>
+      <c r="M274" s="61" t="inlineStr">
+        <is>
+          <t>Una fe que solo funciona en la temporada buena.</t>
+        </is>
+      </c>
+      <c r="N274" s="61" t="inlineStr">
+        <is>
+          <t>Anotá cada noche de esta semana una cosa por la que das gracias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="61" t="n">
+        <v>46</v>
+      </c>
+      <c r="B275" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C275" s="61" t="inlineStr">
+        <is>
+          <t>Todo lo que respira</t>
+        </is>
+      </c>
+      <c r="D275" s="61" t="inlineStr">
+        <is>
+          <t>El libro de los Salmos tiene cinco partes, y cada una termina con una alabanza; el Salmo 150 cierra todo el libro.</t>
+        </is>
+      </c>
+      <c r="E275" s="61" t="inlineStr">
+        <is>
+          <t>Salmos 41:13; 72:19; 89:52; 106:48; 150</t>
+        </is>
+      </c>
+      <c r="F275" s="61" t="inlineStr">
+        <is>
+          <t>El último salmo invita a todo ser vivo a alabar. Cada respiración es una oportunidad de gratitud.</t>
+        </is>
+      </c>
+      <c r="G275" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que la alabanza es solo para los que cantan bien.</t>
+        </is>
+      </c>
+      <c r="H275" s="61" t="inlineStr">
+        <is>
+          <t>Respirá hondo tres veces hoy y, con cada respiración, agradecé algo.</t>
+        </is>
+      </c>
+      <c r="I275" s="61" t="inlineStr">
+        <is>
+          <t>Alabar no requiere instrumentos, voz linda ni un lugar especial: alcanza con un corazón agradecido.</t>
+        </is>
+      </c>
+      <c r="J275" s="61" t="inlineStr">
+        <is>
+          <t>Esperar el momento ideal para alabar.</t>
+        </is>
+      </c>
+      <c r="K275" s="61" t="inlineStr">
+        <is>
+          <t>Poné hoy una canción de alabanza mientras hacés tus tareas.</t>
+        </is>
+      </c>
+      <c r="L275" s="61" t="inlineStr">
+        <is>
+          <t>El libro de los Salmos empieza con la vida del justo y termina en alabanza: la vida con Dios lleva a la gratitud.</t>
+        </is>
+      </c>
+      <c r="M275" s="61" t="inlineStr">
+        <is>
+          <t>Vivir sin detenerse nunca a agradecer.</t>
+        </is>
+      </c>
+      <c r="N275" s="61" t="inlineStr">
+        <is>
+          <t>Cerrá el día con una oración de agradecimiento.</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="61" t="n">
+        <v>46</v>
+      </c>
+      <c r="B276" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C276" s="61" t="inlineStr">
+        <is>
+          <t>Sacrificio de alabanza</t>
+        </is>
+      </c>
+      <c r="D276" s="61" t="inlineStr">
+        <is>
+          <t>En la carta a los Hebreos, los sacrificios del templo dan lugar a otra ofrenda: la alabanza, hacer el bien y compartir.</t>
+        </is>
+      </c>
+      <c r="E276" s="61" t="inlineStr">
+        <is>
+          <t>Hebreos 13:15-16</t>
+        </is>
+      </c>
+      <c r="F276" s="61" t="inlineStr">
+        <is>
+          <t>Alabar cuando cuesta es ofrecerle algo a Dios. El hábito de adorar reordena la mirada: el problema se ve distinto cuando miramos primero a Dios.</t>
+        </is>
+      </c>
+      <c r="G276" s="61" t="inlineStr">
+        <is>
+          <t>Esperar sentirse bien para alabar.</t>
+        </is>
+      </c>
+      <c r="H276" s="61" t="inlineStr">
+        <is>
+          <t>Empezá cada mañana de esta semana con una frase de alabanza, antes de mirar el celular.</t>
+        </is>
+      </c>
+      <c r="I276" s="61" t="inlineStr">
+        <is>
+          <t>Un hábito simple de adoración diaria puede sostener a alguien en una semana difícil.</t>
+        </is>
+      </c>
+      <c r="J276" s="61" t="inlineStr">
+        <is>
+          <t>Dejar la adoración para cuando haya tiempo.</t>
+        </is>
+      </c>
+      <c r="K276" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un momento fijo del día para adorar, aunque sean dos minutos.</t>
+        </is>
+      </c>
+      <c r="L276" s="61" t="inlineStr">
+        <is>
+          <t>El versículo siguiente une la alabanza con hacer el bien y compartir (13:16). La adoración se nota también en cómo tratamos a los demás.</t>
+        </is>
+      </c>
+      <c r="M276" s="61" t="inlineStr">
+        <is>
+          <t>Cantar el domingo y no cambiar nada el lunes.</t>
+        </is>
+      </c>
+      <c r="N276" s="61" t="inlineStr">
+        <is>
+          <t>Hacé hoy un bien concreto como parte de tu adoración.</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="61" t="n">
+        <v>46</v>
+      </c>
+      <c r="B277" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C277" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: adorar en todo tiempo</t>
+        </is>
+      </c>
+      <c r="D277" s="61" t="inlineStr">
+        <is>
+          <t>Habacuc empieza su libro con preguntas y quejas a Dios, y lo termina con este canto de confianza.</t>
+        </is>
+      </c>
+      <c r="E277" s="61" t="inlineStr">
+        <is>
+          <t>Habacuc 1:2-4; 3:17-19</t>
+        </is>
+      </c>
+      <c r="F277" s="61" t="inlineStr">
+        <is>
+          <t>Adorar no depende del ánimo: también se adora en lo bajo, y el lamento sincero es adoración.</t>
+        </is>
+      </c>
+      <c r="G277" s="61" t="n"/>
+      <c r="H277" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, empezá cada día con una frase de alabanza y cerralo anotando tres cosas por las que das gracias.</t>
+        </is>
+      </c>
+      <c r="I277" s="61" t="inlineStr">
+        <is>
+          <t>La gratitud por lo pequeño del día es una forma diaria de adorar.</t>
+        </is>
+      </c>
+      <c r="J277" s="61" t="n"/>
+      <c r="K277" s="61" t="n"/>
+      <c r="L277" s="61" t="inlineStr">
+        <is>
+          <t>El hábito de adorar reordena la mirada y se nota en cómo tratamos a los demás.</t>
+        </is>
+      </c>
+      <c r="M277" s="61" t="n"/>
+      <c r="N277" s="61" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="61" t="n">
+        <v>47</v>
+      </c>
+      <c r="B278" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C278" s="61" t="inlineStr">
+        <is>
+          <t>Confiar de todo corazón</t>
+        </is>
+      </c>
+      <c r="D278" s="61" t="inlineStr">
+        <is>
+          <t>La palabra hebrea que se traduce «enderezará» también significa allanar un camino: quitarle los obstáculos.</t>
+        </is>
+      </c>
+      <c r="E278" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 3:6 (texto hebreo, yashar)</t>
+        </is>
+      </c>
+      <c r="F278" s="61" t="inlineStr">
+        <is>
+          <t>Nunca tenemos toda la información. Confiar en Dios no es dejar de pensar, sino reconocer que nuestro entendimiento tiene límites.</t>
+        </is>
+      </c>
+      <c r="G278" s="61" t="inlineStr">
+        <is>
+          <t>Esperar la certeza total y perder el momento.</t>
+        </is>
+      </c>
+      <c r="H278" s="61" t="inlineStr">
+        <is>
+          <t>Ante una decisión pendiente, escribí lo que sabés y lo que no sabés, y presentáselo a Dios.</t>
+        </is>
+      </c>
+      <c r="I278" s="61" t="inlineStr">
+        <is>
+          <t>Reconocer a Dios en las decisiones grandes y pequeñas es preguntarse: ¿esto lo honra?</t>
+        </is>
+      </c>
+      <c r="J278" s="61" t="inlineStr">
+        <is>
+          <t>Consultar a Dios solo en las decisiones grandes.</t>
+        </is>
+      </c>
+      <c r="K278" s="61" t="inlineStr">
+        <is>
+          <t>Antes de decidir algo hoy, hacé una oración corta pidiendo sabiduría.</t>
+        </is>
+      </c>
+      <c r="L278" s="61" t="inlineStr">
+        <is>
+          <t>Dios puede enderezar el camino aun cuando decidimos con información incompleta. Eso da paz para decidir sin miedo a equivocarse.</t>
+        </is>
+      </c>
+      <c r="M278" s="61" t="inlineStr">
+        <is>
+          <t>Quedar paralizado por miedo a equivocarse.</t>
+        </is>
+      </c>
+      <c r="N278" s="61" t="inlineStr">
+        <is>
+          <t>Tomá hoy una decisión pequeña que venías postergando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="61" t="n">
+        <v>47</v>
+      </c>
+      <c r="B279" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C279" s="61" t="inlineStr">
+        <is>
+          <t>Andar confiado</t>
+        </is>
+      </c>
+      <c r="D279" s="61" t="inlineStr">
+        <is>
+          <t>Los capítulos 1 a 9 de Proverbios están escritos como consejos de un padre a su hijo.</t>
+        </is>
+      </c>
+      <c r="E279" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 1:8; 4:1</t>
+        </is>
+      </c>
+      <c r="F279" s="61" t="inlineStr">
+        <is>
+          <t>El padre aconseja no perder de vista la sabiduría. Las buenas decisiones nacen de principios claros, no de la presión del momento.</t>
+        </is>
+      </c>
+      <c r="G279" s="61" t="inlineStr">
+        <is>
+          <t>Decidir por impulso, sin pensar.</t>
+        </is>
+      </c>
+      <c r="H279" s="61" t="inlineStr">
+        <is>
+          <t>Antes de una decisión importante, si es posible, dejala pasar una noche.</t>
+        </is>
+      </c>
+      <c r="I279" s="61" t="inlineStr">
+        <is>
+          <t>Decidir con lo que se tiene, evaluando el riesgo, es parte de la responsabilidad. El consejo de otros ayuda a ver lo que no vemos.</t>
+        </is>
+      </c>
+      <c r="J279" s="61" t="inlineStr">
+        <is>
+          <t>No pedir consejo por orgullo.</t>
+        </is>
+      </c>
+      <c r="K279" s="61" t="inlineStr">
+        <is>
+          <t>Pedile la opinión a alguien sabio sobre una decisión que tenés que tomar.</t>
+        </is>
+      </c>
+      <c r="L279" s="61" t="inlineStr">
+        <is>
+          <t>Es un principio, no una garantía de no tropezar nunca. Quien camina con sabiduría tropieza menos, y si tropieza, se levanta.</t>
+        </is>
+      </c>
+      <c r="M279" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que una mala decisión arruina todo para siempre.</t>
+        </is>
+      </c>
+      <c r="N279" s="61" t="inlineStr">
+        <is>
+          <t>Si una decisión salió mal, aprendé de ella y seguí adelante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="61" t="n">
+        <v>47</v>
+      </c>
+      <c r="B280" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C280" s="61" t="inlineStr">
+        <is>
+          <t>El que mira el viento</t>
+        </is>
+      </c>
+      <c r="D280" s="61" t="inlineStr">
+        <is>
+          <t>Una revisión de estudios sobre la postergación encontró que se asocia con peores resultados y con más estrés.</t>
+        </is>
+      </c>
+      <c r="E280" s="61" t="inlineStr">
+        <is>
+          <t>Piers Steel, Psychological Bulletin, 2007</t>
+        </is>
+      </c>
+      <c r="F280" s="61" t="inlineStr">
+        <is>
+          <t>El agricultor que espera el clima perfecto nunca siembra. No decidir también es una decisión, y suele ser la más cara.</t>
+        </is>
+      </c>
+      <c r="G280" s="61" t="inlineStr">
+        <is>
+          <t>Postergar decisiones esperando que el problema se resuelva solo.</t>
+        </is>
+      </c>
+      <c r="H280" s="61" t="inlineStr">
+        <is>
+          <t>Elegí una decisión que venís postergando y ponele una fecha.</t>
+        </is>
+      </c>
+      <c r="I280" s="61" t="inlineStr">
+        <is>
+          <t>Mientras se posterga, el problema crece o la oportunidad se cierra.</t>
+        </is>
+      </c>
+      <c r="J280" s="61" t="inlineStr">
+        <is>
+          <t>Problemas chicos que se vuelven grandes por no atenderlos a tiempo.</t>
+        </is>
+      </c>
+      <c r="K280" s="61" t="inlineStr">
+        <is>
+          <t>Atendé hoy un asunto pequeño antes de que crezca.</t>
+        </is>
+      </c>
+      <c r="L280" s="61" t="inlineStr">
+        <is>
+          <t>El versículo siguiente reconoce que no sabemos cómo obra Dios (11:5). Por eso actuamos con lo que tenemos y le confiamos el resultado.</t>
+        </is>
+      </c>
+      <c r="M280" s="61" t="inlineStr">
+        <is>
+          <t>Querer controlarlo todo antes de actuar.</t>
+        </is>
+      </c>
+      <c r="N280" s="61" t="inlineStr">
+        <is>
+          <t>Sembrá hoy algo aunque no sepas el resultado: una conversación, una solicitud, un primer paso.</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="61" t="n">
+        <v>47</v>
+      </c>
+      <c r="B281" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C281" s="61" t="inlineStr">
+        <is>
+          <t>Un corazón que entiende</t>
+        </is>
+      </c>
+      <c r="D281" s="61" t="inlineStr">
+        <is>
+          <t>Salomón hizo este pedido en Gabaón, en un sueño, al comienzo de su reinado.</t>
+        </is>
+      </c>
+      <c r="E281" s="61" t="inlineStr">
+        <is>
+          <t>1 Reyes 3:4-5</t>
+        </is>
+      </c>
+      <c r="F281" s="61" t="inlineStr">
+        <is>
+          <t>Salomón pudo pedir riquezas o una vida larga, pero pidió entendimiento para servir a su pueblo.</t>
+        </is>
+      </c>
+      <c r="G281" s="61" t="inlineStr">
+        <is>
+          <t>Pedirle a Dios solo comodidad.</t>
+        </is>
+      </c>
+      <c r="H281" s="61" t="inlineStr">
+        <is>
+          <t>Pedile hoy a Dios sabiduría para una decisión concreta.</t>
+        </is>
+      </c>
+      <c r="I281" s="61" t="inlineStr">
+        <is>
+          <t>Reconocer que no sabemos todo no es debilidad: es el comienzo de la sabiduría.</t>
+        </is>
+      </c>
+      <c r="J281" s="61" t="inlineStr">
+        <is>
+          <t>Aparentar seguridad para no mostrar dudas.</t>
+        </is>
+      </c>
+      <c r="K281" s="61" t="inlineStr">
+        <is>
+          <t>Contale a alguien de confianza una decisión en la que te sentís inseguro.</t>
+        </is>
+      </c>
+      <c r="L281" s="61" t="inlineStr">
+        <is>
+          <t>Antes de preguntar qué conviene, Salomón quiere distinguir lo bueno de lo malo. Postergar una decisión moral también tiene un costo.</t>
+        </is>
+      </c>
+      <c r="M281" s="61" t="inlineStr">
+        <is>
+          <t>Postergar lo correcto por miedo a lo que cueste.</t>
+        </is>
+      </c>
+      <c r="N281" s="61" t="inlineStr">
+        <is>
+          <t>Si sabés qué es lo correcto, decidilo hoy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="61" t="n">
+        <v>47</v>
+      </c>
+      <c r="B282" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C282" s="61" t="inlineStr">
+        <is>
+          <t>No decidir solo</t>
+        </is>
+      </c>
+      <c r="D282" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 32 empieza celebrando la dicha de quien recibe el perdón de Dios.</t>
+        </is>
+      </c>
+      <c r="E282" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 32:1-5</t>
+        </is>
+      </c>
+      <c r="F282" s="61" t="inlineStr">
+        <is>
+          <t>Dios promete enseñar el camino. Cuando una decisión afecta a otros, el peso es mayor y la guía de Dios, más necesaria.</t>
+        </is>
+      </c>
+      <c r="G282" s="61" t="inlineStr">
+        <is>
+          <t>Decidir pensando solo en lo que me conviene.</t>
+        </is>
+      </c>
+      <c r="H282" s="61" t="inlineStr">
+        <is>
+          <t>Antes de una decisión que afecta a tu familia o a tu equipo, orá por ellos.</t>
+        </is>
+      </c>
+      <c r="I282" s="61" t="inlineStr">
+        <is>
+          <t>Dios no nos quita los ojos de encima. Así también, quien decide por otros tiene que mirar cómo los afecta.</t>
+        </is>
+      </c>
+      <c r="J282" s="61" t="inlineStr">
+        <is>
+          <t>Ignorar a quienes dependen de nuestras decisiones.</t>
+        </is>
+      </c>
+      <c r="K282" s="61" t="inlineStr">
+        <is>
+          <t>Preguntales a las personas afectadas cómo ven la decisión antes de tomarla.</t>
+        </is>
+      </c>
+      <c r="L282" s="61" t="inlineStr">
+        <is>
+          <t>Consultar antes de decidir no es debilidad, sino respeto por los demás.</t>
+        </is>
+      </c>
+      <c r="M282" s="61" t="inlineStr">
+        <is>
+          <t>Decisiones familiares tomadas por uno solo, sin consultar.</t>
+        </is>
+      </c>
+      <c r="N282" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, tomá una decisión de la casa conversándola con tu familia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="61" t="n">
+        <v>47</v>
+      </c>
+      <c r="B283" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C283" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: decidir con sabiduría</t>
+        </is>
+      </c>
+      <c r="D283" s="61" t="inlineStr">
+        <is>
+          <t>Antes de elegir a los doce apóstoles, Jesús pasó la noche orando.</t>
+        </is>
+      </c>
+      <c r="E283" s="61" t="inlineStr">
+        <is>
+          <t>Lucas 6:12-13</t>
+        </is>
+      </c>
+      <c r="F283" s="61" t="inlineStr">
+        <is>
+          <t>Decidir con información incompleta es parte de la vida; confiar en Dios da paz para decidir.</t>
+        </is>
+      </c>
+      <c r="G283" s="61" t="n"/>
+      <c r="H283" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, elegí una decisión pendiente, orá por ella, pedí consejo y ponele una fecha.</t>
+        </is>
+      </c>
+      <c r="I283" s="61" t="inlineStr">
+        <is>
+          <t>No decidir también es una decisión, y suele ser la más cara.</t>
+        </is>
+      </c>
+      <c r="J283" s="61" t="n"/>
+      <c r="K283" s="61" t="n"/>
+      <c r="L283" s="61" t="inlineStr">
+        <is>
+          <t>Cuando la decisión afecta a otros, se consulta y se ora por ellos.</t>
+        </is>
+      </c>
+      <c r="M283" s="61" t="n"/>
+      <c r="N283" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de noviembre verificados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -37199,12 +37199,12 @@
       </c>
       <c r="D270" s="61" t="inlineStr">
         <is>
-          <t>En Paraguay, el 141 es el número del Servicio de Emergencias Médicas Extrahospitalarias (SEME), y el 911 el del sistema de emergencias.</t>
+          <t>En Paraguay, el 141 es el número del Servicio de Emergencias Médicas Extrahospitalarias (SEME), el 911 el del sistema de emergencias y el 132 el de los Bomberos Voluntarios.</t>
         </is>
       </c>
       <c r="E270" s="61" t="inlineStr">
         <is>
-          <t>Ministerio de Salud Pública y Bienestar Social; Sistema 911</t>
+          <t>Ministerio de Salud Pública y Bienestar Social; Sistema 911; Cuerpo de Bomberos Voluntarios del Paraguay</t>
         </is>
       </c>
       <c r="F270" s="61" t="inlineStr">
@@ -37389,7 +37389,7 @@
       </c>
       <c r="D273" s="61" t="inlineStr">
         <is>
-          <t>El Salmo 34 es un acróstico: en hebreo, cada versículo empieza con una letra distinta del alfabeto.</t>
+          <t>El Salmo 34 es un acróstico: en hebreo, sus versículos van siguiendo, uno tras otro, las letras del alfabeto.</t>
         </is>
       </c>
       <c r="E273" s="61" t="inlineStr">
@@ -37859,12 +37859,12 @@
       </c>
       <c r="D280" s="61" t="inlineStr">
         <is>
-          <t>Una revisión de estudios sobre la postergación encontró que se asocia con peores resultados y con más estrés.</t>
+          <t>Una revisión de estudios sobre la postergación encontró que se asocia con peores resultados; otros estudios la vinculan también con más estrés.</t>
         </is>
       </c>
       <c r="E280" s="61" t="inlineStr">
         <is>
-          <t>Piers Steel, Psychological Bulletin, 2007</t>
+          <t>Piers Steel, Psychological Bulletin, 2007; Tice y Baumeister, Psychological Science, 1997</t>
         </is>
       </c>
       <c r="F280" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: guiones de diciembre con revisión teológica
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -10732,7 +10732,7 @@
       </c>
       <c r="AB49" s="12" t="inlineStr">
         <is>
-          <t>Josue 4:6-7 — Cada una de ellas será una señal. Y el día de mañana, cuando los hijos les pregunten a sus padres qué significan estas piedras,
+          <t>Josué 4:6-7 — Cada una de ellas será una señal. Y el día de mañana, cuando los hijos les pregunten a sus padres qué significan estas piedras,
 ellos les responderán: “Cuando el pueblo cruzó el Jordán, las aguas del río se partieron en dos delante del arca del pacto del Señor. Así que estas piedras son para que los hijos de Israel recuerden siempre lo que aquí pasó.”»</t>
         </is>
       </c>
@@ -10766,7 +10766,7 @@
       </c>
       <c r="AG49" s="12" t="inlineStr">
         <is>
-          <t>• Creer trae salvación para la casa
+          <t>• La promesa alcanza a toda la casa que cree
 • La fe individual impacta a la familia
 • Es promesa, no automatismo sin fe propia</t>
         </is>
@@ -10793,7 +10793,7 @@
         <is>
           <t>• Restaurar el corazón de padres e hijos
 • La reconciliación familiar es obra de Dios
-• Evita la maldición del distanciamiento</t>
+• Dios restaura lo que el distanciamiento rompe</t>
         </is>
       </c>
     </row>
@@ -10920,7 +10920,7 @@
       <c r="Y50" s="14" t="inlineStr">
         <is>
           <t>• Dios bendice: Él es la fuente de nuestra provisión.  
-• Prosperidad con propósito: La bendición permite ayudar y prestar a otros.  
+• Bendición con propósito: La bendición permite ayudar y prestar a otros.  
 • Libertad financiera: No vivir bajo la esclavitud de las deudas.</t>
         </is>
       </c>
@@ -10971,7 +10971,7 @@
         <is>
           <t>• El peligro de la autosuficiencia
 • La raíz interior del orgullo.
-• El olvido del verdadero origen de los bienes:</t>
+• El olvido del verdadero origen de los bienes</t>
         </is>
       </c>
       <c r="AH50" s="14" t="inlineStr">
@@ -11356,13 +11356,13 @@
       </c>
       <c r="AB52" s="4" t="inlineStr">
         <is>
-          <t>1 Cronicas 12:32 — De los hijos de Isacar, doscientos jefes, cuyas palabras eran respetadas por todos sus parientes, pues sabían cuándo actuar y qué debía hacer Israel.</t>
+          <t>1 Crónicas 12:32 — De los hijos de Isacar, doscientos jefes, cuyas palabras eran respetadas por todos sus parientes, pues sabían cuándo actuar y qué debía hacer Israel.</t>
         </is>
       </c>
       <c r="AC52" s="4" t="inlineStr">
         <is>
-          <t>• Entender los tiempos es sabiduría practica
-• Saber que hacer en cada época
+          <t>• Entender los tiempos es sabiduría práctica
+• Saber qué hacer en cada época
 • La adaptación requiere discernimiento</t>
         </is>
       </c>
@@ -11542,9 +11542,9 @@
       </c>
       <c r="Y53" s="6" t="inlineStr">
         <is>
-          <t>• La condición (Servicio exclusivo a Dios).
-• La provisión (Bendición del pan y del agua).
-• La sanidad y protección (Remoción de la enfermedad)</t>
+          <t>• Servir solo a Dios: La fidelidad del pueblo del pacto.
+• Provisión: Dios bendice el pan y el agua.
+• Una promesa a Israel: Dios cuida la salud de su pueblo.</t>
         </is>
       </c>
       <c r="Z53" s="6" t="inlineStr">
@@ -11554,7 +11554,7 @@
       </c>
       <c r="AA53" s="6" t="inlineStr">
         <is>
-          <t>• Orar unos por otros trae sanidad
+          <t>• Orar unos por otros, también por la sanidad
 • La oración en comunidad tiene poder
 • No orar en soledad exclusivamente</t>
         </is>
@@ -19212,7 +19212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N283"/>
+  <dimension ref="A1:N313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -38102,6 +38102,2006 @@
       </c>
       <c r="M283" s="61" t="n"/>
       <c r="N283" s="61" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="61" t="n">
+        <v>48</v>
+      </c>
+      <c r="B284" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C284" s="61" t="inlineStr">
+        <is>
+          <t>En casa y en el camino</t>
+        </is>
+      </c>
+      <c r="D284" s="61" t="inlineStr">
+        <is>
+          <t>Deuteronomio 11 repite casi palabra por palabra el mandato de Deuteronomio 6: enseñar a los hijos en casa, en el camino, al acostarse y al levantarse.</t>
+        </is>
+      </c>
+      <c r="E284" s="61" t="inlineStr">
+        <is>
+          <t>Deuteronomio 6:6-9; 11:18-21</t>
+        </is>
+      </c>
+      <c r="F284" s="61" t="inlineStr">
+        <is>
+          <t>Moisés no pide una clase formal, sino hablar de Dios en la vida diaria: en casa, en el camino, al acostarse y al levantarse.</t>
+        </is>
+      </c>
+      <c r="G284" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que la fe se enseña solo en la iglesia.</t>
+        </is>
+      </c>
+      <c r="H284" s="61" t="inlineStr">
+        <is>
+          <t>Aprovechá un viaje o una comida de hoy para hablar de algo que Dios hizo.</t>
+        </is>
+      </c>
+      <c r="I284" s="61" t="inlineStr">
+        <is>
+          <t>Muchas familias empiezan un devocional con entusiasmo y lo dejan en semanas, porque buscan perfección en vez de constancia.</t>
+        </is>
+      </c>
+      <c r="J284" s="61" t="inlineStr">
+        <is>
+          <t>Devocionales largos que terminan abandonándose.</t>
+        </is>
+      </c>
+      <c r="K284" s="61" t="inlineStr">
+        <is>
+          <t>Probá un formato mínimo: un versículo corto y una pregunta, cinco minutos.</t>
+        </is>
+      </c>
+      <c r="L284" s="61" t="inlineStr">
+        <is>
+          <t>Lo que se repite con cariño queda grabado. Cinco minutos constantes valen más que una hora una vez al año.</t>
+        </is>
+      </c>
+      <c r="M284" s="61" t="inlineStr">
+        <is>
+          <t>Culparse por no hacerlo perfecto y abandonar.</t>
+        </is>
+      </c>
+      <c r="N284" s="61" t="inlineStr">
+        <is>
+          <t>Elijan un momento fijo del día, como la cena o antes de dormir, para su devocional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="61" t="n">
+        <v>48</v>
+      </c>
+      <c r="B285" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C285" s="61" t="inlineStr">
+        <is>
+          <t>Las piedras que preguntan</t>
+        </is>
+      </c>
+      <c r="D285" s="61" t="inlineStr">
+        <is>
+          <t>Las doce piedras representaban a las doce tribus de Israel, y se colocaron en Gilgal.</t>
+        </is>
+      </c>
+      <c r="E285" s="61" t="inlineStr">
+        <is>
+          <t>Josué 4:2-8, 20</t>
+        </is>
+      </c>
+      <c r="F285" s="61" t="inlineStr">
+        <is>
+          <t>Dios pensó en las preguntas de los hijos antes de que las hicieran. Un devocional también responde preguntas.</t>
+        </is>
+      </c>
+      <c r="G285" s="61" t="inlineStr">
+        <is>
+          <t>Responder «porque sí» a las preguntas de los chicos sobre Dios.</t>
+        </is>
+      </c>
+      <c r="H285" s="61" t="inlineStr">
+        <is>
+          <t>Preguntale a tu hijo qué le gustaría saber de Dios, y busquen juntos la respuesta.</t>
+        </is>
+      </c>
+      <c r="I285" s="61" t="inlineStr">
+        <is>
+          <t>Una oración antes de comer, una Biblia abierta en la mesa: las señales visibles despiertan curiosidad.</t>
+        </is>
+      </c>
+      <c r="J285" s="61" t="inlineStr">
+        <is>
+          <t>Una fe tan privada que los hijos nunca la ven.</t>
+        </is>
+      </c>
+      <c r="K285" s="61" t="inlineStr">
+        <is>
+          <t>Dejá a la vista algo que le recuerde a tu familia lo que Dios hizo: una foto, un versículo, un objeto.</t>
+        </is>
+      </c>
+      <c r="L285" s="61" t="inlineStr">
+        <is>
+          <t>Las piedras servían para contar una historia. Contar lo que Dios hizo en tu propia vida también es parte del devocional familiar.</t>
+        </is>
+      </c>
+      <c r="M285" s="61" t="inlineStr">
+        <is>
+          <t>Hablar de Dios solo con conceptos, sin historias reales.</t>
+        </is>
+      </c>
+      <c r="N285" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, contale a tu familia una historia de cómo Dios te ayudó.</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="61" t="n">
+        <v>48</v>
+      </c>
+      <c r="B286" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C286" s="61" t="inlineStr">
+        <is>
+          <t>Familias que adoran</t>
+        </is>
+      </c>
+      <c r="D286" s="61" t="inlineStr">
+        <is>
+          <t>David cantó este himno cuando llevaron el arca del pacto a Jerusalén.</t>
+        </is>
+      </c>
+      <c r="E286" s="61" t="inlineStr">
+        <is>
+          <t>1 Crónicas 16:1-7</t>
+        </is>
+      </c>
+      <c r="F286" s="61" t="inlineStr">
+        <is>
+          <t>El canto invita a todas las familias de los pueblos a adorar. La invitación es una puerta abierta, no una imposición.</t>
+        </is>
+      </c>
+      <c r="G286" s="61" t="inlineStr">
+        <is>
+          <t>Obligar a los hijos a «ser cristianos» a la fuerza.</t>
+        </is>
+      </c>
+      <c r="H286" s="61" t="inlineStr">
+        <is>
+          <t>Invitá a tus hijos a orar con vos, sin obligarlos.</t>
+        </is>
+      </c>
+      <c r="I286" s="61" t="inlineStr">
+        <is>
+          <t>Formar la fe de un hijo no es forzarla: es mostrarla con el ejemplo y dejar espacio para que se vuelva propia.</t>
+        </is>
+      </c>
+      <c r="J286" s="61" t="inlineStr">
+        <is>
+          <t>Usar la culpa o el miedo para que los hijos crean.</t>
+        </is>
+      </c>
+      <c r="K286" s="61" t="inlineStr">
+        <is>
+          <t>Contale a tu hijo por qué creés, con tus palabras y sin sermones.</t>
+        </is>
+      </c>
+      <c r="L286" s="61" t="inlineStr">
+        <is>
+          <t>Cuando un hijo cuestiona la fe, no hace falta reaccionar con miedo. Sus preguntas pueden ser el camino hacia una fe propia.</t>
+        </is>
+      </c>
+      <c r="M286" s="61" t="inlineStr">
+        <is>
+          <t>Retar o callar a un hijo que pregunta o duda.</t>
+        </is>
+      </c>
+      <c r="N286" s="61" t="inlineStr">
+        <is>
+          <t>Si tu hijo duda, agradecele que te lo cuente y busquen juntos las respuestas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="61" t="n">
+        <v>48</v>
+      </c>
+      <c r="B287" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C287" s="61" t="inlineStr">
+        <is>
+          <t>Vos y tu familia</t>
+        </is>
+      </c>
+      <c r="D287" s="61" t="inlineStr">
+        <is>
+          <t>El carcelero de Filipos creyó esa misma noche, después de un terremoto que abrió las puertas de la cárcel.</t>
+        </is>
+      </c>
+      <c r="E287" s="61" t="inlineStr">
+        <is>
+          <t>Hechos 16:25-34</t>
+        </is>
+      </c>
+      <c r="F287" s="61" t="inlineStr">
+        <is>
+          <t>Pablo y Silas les hablaron a todos los de la casa del carcelero, y todos creyeron (16:32-34). La salvación se ofrece a cada uno de la familia.</t>
+        </is>
+      </c>
+      <c r="G287" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que la fe de un padre alcanza automáticamente a los hijos.</t>
+        </is>
+      </c>
+      <c r="H287" s="61" t="inlineStr">
+        <is>
+          <t>Orá hoy por cada miembro de tu familia, uno por uno, por su nombre.</t>
+        </is>
+      </c>
+      <c r="I287" s="61" t="inlineStr">
+        <is>
+          <t>La fe de una persona puede abrirle la puerta a toda la familia. El carcelero, al creer, lavó las heridas de Pablo y les sirvió la mesa.</t>
+        </is>
+      </c>
+      <c r="J287" s="61" t="inlineStr">
+        <is>
+          <t>Una fe que no cambia el trato en casa.</t>
+        </is>
+      </c>
+      <c r="K287" s="61" t="inlineStr">
+        <is>
+          <t>Mostrá tu fe en casa con un servicio concreto hoy.</t>
+        </is>
+      </c>
+      <c r="L287" s="61" t="inlineStr">
+        <is>
+          <t>Cada hijo tiene que hacer suya la fe. Si un hijo se alejó, esa no es la última palabra: los padres siguen orando y amando, sin culpa.</t>
+        </is>
+      </c>
+      <c r="M287" s="61" t="inlineStr">
+        <is>
+          <t>Padres que se culpan porque un hijo se alejó de la fe.</t>
+        </is>
+      </c>
+      <c r="N287" s="61" t="inlineStr">
+        <is>
+          <t>Si un hijo se alejó, mantené la puerta abierta: más amor y menos reproches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="61" t="n">
+        <v>48</v>
+      </c>
+      <c r="B288" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C288" s="61" t="inlineStr">
+        <is>
+          <t>Dichosos</t>
+        </is>
+      </c>
+      <c r="D288" s="61" t="inlineStr">
+        <is>
+          <t>El Salmo 128 es otro de los «cánticos de las subidas» y describe la mesa familiar, con los hijos alrededor como plantas de olivo.</t>
+        </is>
+      </c>
+      <c r="E288" s="61" t="inlineStr">
+        <is>
+          <t>Salmo 128:1-3</t>
+        </is>
+      </c>
+      <c r="F288" s="61" t="inlineStr">
+        <is>
+          <t>Honrar al Señor es la base de un hogar dichoso. Antes de escuchar un sermón, un hijo ya ve cómo sus padres viven la fe.</t>
+        </is>
+      </c>
+      <c r="G288" s="61" t="inlineStr">
+        <is>
+          <t>Decir una cosa en la iglesia y vivir otra en casa.</t>
+        </is>
+      </c>
+      <c r="H288" s="61" t="inlineStr">
+        <is>
+          <t>Preguntate: si mis hijos aprendieran de Dios solo mirándome, ¿qué aprenderían?</t>
+        </is>
+      </c>
+      <c r="I288" s="61" t="inlineStr">
+        <is>
+          <t>Andar en los caminos de Dios se ve en lo cotidiano: cómo pedimos perdón, cómo tratamos al otro, cómo enfrentamos los problemas.</t>
+        </is>
+      </c>
+      <c r="J288" s="61" t="inlineStr">
+        <is>
+          <t>Hogares donde la fe es solo una costumbre del domingo.</t>
+        </is>
+      </c>
+      <c r="K288" s="61" t="inlineStr">
+        <is>
+          <t>Pedí perdón hoy en casa por algo concreto, delante de tus hijos.</t>
+        </is>
+      </c>
+      <c r="L288" s="61" t="inlineStr">
+        <is>
+          <t>No es una garantía de que todo saldrá bien, sino el camino de la verdadera dicha. El hogar es el primer lugar donde se ve a Cristo.</t>
+        </is>
+      </c>
+      <c r="M288" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que un hogar cristiano no tiene problemas.</t>
+        </is>
+      </c>
+      <c r="N288" s="61" t="inlineStr">
+        <is>
+          <t>Oren en familia esta noche por un problema real que estén pasando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="61" t="n">
+        <v>48</v>
+      </c>
+      <c r="B289" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C289" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: la fe en casa</t>
+        </is>
+      </c>
+      <c r="D289" s="61" t="inlineStr">
+        <is>
+          <t>El ángel aplicó esta profecía a Juan el Bautista antes de que naciera.</t>
+        </is>
+      </c>
+      <c r="E289" s="61" t="inlineStr">
+        <is>
+          <t>Lucas 1:17</t>
+        </is>
+      </c>
+      <c r="F289" s="61" t="inlineStr">
+        <is>
+          <t>La fe se transmite en la vida diaria, con una constancia simple: un versículo y una pregunta.</t>
+        </is>
+      </c>
+      <c r="G289" s="61" t="n"/>
+      <c r="H289" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, empiecen un devocional de cinco minutos en familia: un versículo, una pregunta y una oración.</t>
+        </is>
+      </c>
+      <c r="I289" s="61" t="inlineStr">
+        <is>
+          <t>Formar la fe no es forzarla: se muestra con el ejemplo y se responden las dudas sin miedo.</t>
+        </is>
+      </c>
+      <c r="J289" s="61" t="n"/>
+      <c r="K289" s="61" t="n"/>
+      <c r="L289" s="61" t="inlineStr">
+        <is>
+          <t>El hogar es el primer lugar donde los hijos ven a Cristo.</t>
+        </is>
+      </c>
+      <c r="M289" s="61" t="n"/>
+      <c r="N289" s="61" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="61" t="n">
+        <v>49</v>
+      </c>
+      <c r="B290" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C290" s="61" t="inlineStr">
+        <is>
+          <t>La única deuda</t>
+        </is>
+      </c>
+      <c r="D290" s="61" t="inlineStr">
+        <is>
+          <t>En la ley de Moisés, cada siete años se perdonaban las deudas entre israelitas, en el «año de remisión».</t>
+        </is>
+      </c>
+      <c r="E290" s="61" t="inlineStr">
+        <is>
+          <t>Deuteronomio 15:1-2</t>
+        </is>
+      </c>
+      <c r="F290" s="61" t="inlineStr">
+        <is>
+          <t>Pablo enseña a pagar lo que se debe (13:7) y a no dejar deudas pendientes. La Biblia no prohíbe todo préstamo, pero sí advierte sobre sus riesgos.</t>
+        </is>
+      </c>
+      <c r="G290" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que toda deuda es pecado, o que ninguna es peligrosa.</t>
+        </is>
+      </c>
+      <c r="H290" s="61" t="inlineStr">
+        <is>
+          <t>Anotá todas tus deudas, con su monto real y su interés.</t>
+        </is>
+      </c>
+      <c r="I290" s="61" t="inlineStr">
+        <is>
+          <t>Una deuda que financia algo que genera valor, como una herramienta de trabajo, es distinta de una deuda para sostener gastos que no se pueden pagar.</t>
+        </is>
+      </c>
+      <c r="J290" s="61" t="inlineStr">
+        <is>
+          <t>Endeudarse para gastos del día a día o para aparentar.</t>
+        </is>
+      </c>
+      <c r="K290" s="61" t="inlineStr">
+        <is>
+          <t>Antes de tomar una deuda, preguntate: ¿esto me ayuda a generar ingresos o es solo un gasto?</t>
+        </is>
+      </c>
+      <c r="L290" s="61" t="inlineStr">
+        <is>
+          <t>Pagar lo que se debe es una forma de amar al prójimo: el que prestó también tiene una familia.</t>
+        </is>
+      </c>
+      <c r="M290" s="61" t="inlineStr">
+        <is>
+          <t>Olvidarse de una deuda con un amigo o un pariente.</t>
+        </is>
+      </c>
+      <c r="N290" s="61" t="inlineStr">
+        <is>
+          <t>Si le debés algo a alguien cercano, hablale esta semana y acordá cómo pagarle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="61" t="n">
+        <v>49</v>
+      </c>
+      <c r="B291" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C291" s="61" t="inlineStr">
+        <is>
+          <t>Antes de salir de garante</t>
+        </is>
+      </c>
+      <c r="D291" s="61" t="inlineStr">
+        <is>
+          <t>En tiempos bíblicos, quien no podía pagar podía perder hasta su manto; la ley pedía devolverlo antes de la noche.</t>
+        </is>
+      </c>
+      <c r="E291" s="61" t="inlineStr">
+        <is>
+          <t>Éxodo 22:26-27; Proverbios 22:27</t>
+        </is>
+      </c>
+      <c r="F291" s="61" t="inlineStr">
+        <is>
+          <t>Ser garante es comprometerse a pagar si el otro no paga. Por eso Proverbios pide prudencia.</t>
+        </is>
+      </c>
+      <c r="G291" s="61" t="inlineStr">
+        <is>
+          <t>Firmar como garante por compromiso, sin leer ni medir el riesgo.</t>
+        </is>
+      </c>
+      <c r="H291" s="61" t="inlineStr">
+        <is>
+          <t>Antes de firmar como garante, preguntate: ¿podría pagar toda esa deuda yo solo si hiciera falta?</t>
+        </is>
+      </c>
+      <c r="I291" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio habla de perder hasta la cama. Muchas familias quedaron endeudadas por deudas ajenas.</t>
+        </is>
+      </c>
+      <c r="J291" s="61" t="inlineStr">
+        <is>
+          <t>Arriesgar lo que tu familia necesita por la deuda de otro.</t>
+        </is>
+      </c>
+      <c r="K291" s="61" t="inlineStr">
+        <is>
+          <t>Conversá con tu familia antes de comprometerte por la deuda de otro.</t>
+        </is>
+      </c>
+      <c r="L291" s="61" t="inlineStr">
+        <is>
+          <t>Ayudar a otro no siempre es firmar: a veces es mejor dar lo que se puede, sin comprometer lo que no se tiene.</t>
+        </is>
+      </c>
+      <c r="M291" s="61" t="inlineStr">
+        <is>
+          <t>Sentir culpa por decir que no a firmar.</t>
+        </is>
+      </c>
+      <c r="N291" s="61" t="inlineStr">
+        <is>
+          <t>Si querés ayudar, pensá qué podés dar sin poner en riesgo a tu familia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="61" t="n">
+        <v>49</v>
+      </c>
+      <c r="B292" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C292" s="61" t="inlineStr">
+        <is>
+          <t>Escapar de la trampa</t>
+        </is>
+      </c>
+      <c r="D292" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 6:1-5 aconseja a quien quedó comprometido por otro que vaya cuanto antes a pedir que lo liberen, sin dejar pasar el tiempo.</t>
+        </is>
+      </c>
+      <c r="E292" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 6:1-5</t>
+        </is>
+      </c>
+      <c r="F292" s="61" t="inlineStr">
+        <is>
+          <t>La imagen es la de una gacela que escapa: no hay que quedarse quieto ante una deuda que crece. Y hay salida.</t>
+        </is>
+      </c>
+      <c r="G292" s="61" t="inlineStr">
+        <is>
+          <t>No abrir las cuentas ni los mensajes del banco por miedo.</t>
+        </is>
+      </c>
+      <c r="H292" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, mirá el total real de lo que debés, sin esconderlo.</t>
+        </is>
+      </c>
+      <c r="I292" s="61" t="inlineStr">
+        <is>
+          <t>Salir de una deuda casi nunca es un salto: es un proceso de pasos ordenados. Reconocer el total, elegir qué pagar primero y sostener el plan aunque avance lento.</t>
+        </is>
+      </c>
+      <c r="J292" s="61" t="inlineStr">
+        <is>
+          <t>Desesperarse y tomar una deuda nueva para pagar la anterior.</t>
+        </is>
+      </c>
+      <c r="K292" s="61" t="inlineStr">
+        <is>
+          <t>Ordená tus deudas y elegí una para atacar primero.</t>
+        </is>
+      </c>
+      <c r="L292" s="61" t="inlineStr">
+        <is>
+          <t>Muchas veces se puede conversar con quien prestó para reorganizar los pagos. Y si la situación es complicada, conviene pedir consejo a un profesional de confianza.</t>
+        </is>
+      </c>
+      <c r="M292" s="61" t="inlineStr">
+        <is>
+          <t>Cargar solo con la deuda, por vergüenza.</t>
+        </is>
+      </c>
+      <c r="N292" s="61" t="inlineStr">
+        <is>
+          <t>Si una deuda te desborda, buscá hoy el consejo de un contador o de alguien de confianza que sepa del tema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="61" t="n">
+        <v>49</v>
+      </c>
+      <c r="B293" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C293" s="61" t="inlineStr">
+        <is>
+          <t>No fue solo mi fuerza</t>
+        </is>
+      </c>
+      <c r="D293" s="61" t="inlineStr">
+        <is>
+          <t>Moisés dijo estas palabras antes de que el pueblo entrara en la tierra prometida, cuando todavía estaban en el desierto.</t>
+        </is>
+      </c>
+      <c r="E293" s="61" t="inlineStr">
+        <is>
+          <t>Deuteronomio 1:1-5; 8:1-18</t>
+        </is>
+      </c>
+      <c r="F293" s="61" t="inlineStr">
+        <is>
+          <t>Moisés advierte que, cuando llegue la abundancia, el pueblo puede olvidarse de Dios. Salir de deudas también pide humildad: reconocer que no podemos solos.</t>
+        </is>
+      </c>
+      <c r="G293" s="61" t="inlineStr">
+        <is>
+          <t>Creer que todo depende de uno, para bien o para mal.</t>
+        </is>
+      </c>
+      <c r="H293" s="61" t="inlineStr">
+        <is>
+          <t>Presentale hoy a Dios tu situación económica, tal como está.</t>
+        </is>
+      </c>
+      <c r="I293" s="61" t="inlineStr">
+        <is>
+          <t>A veces nos endeudamos por orgullo: para aparentar lo que no tenemos.</t>
+        </is>
+      </c>
+      <c r="J293" s="61" t="inlineStr">
+        <is>
+          <t>Gastar para que otros vean.</t>
+        </is>
+      </c>
+      <c r="K293" s="61" t="inlineStr">
+        <is>
+          <t>Identificá un gasto que hacés solo para aparentar, y dejalo este mes.</t>
+        </is>
+      </c>
+      <c r="L293" s="61" t="inlineStr">
+        <is>
+          <t>Dios es quien da la fuerza para trabajar (8:18). Agradecer lo que tenemos ayuda a vivir con contentamiento y sin desesperar.</t>
+        </is>
+      </c>
+      <c r="M293" s="61" t="inlineStr">
+        <is>
+          <t>Mirar solo lo que falta y desesperarse.</t>
+        </is>
+      </c>
+      <c r="N293" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy por tres cosas que tenés, aunque estés con deudas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="61" t="n">
+        <v>49</v>
+      </c>
+      <c r="B294" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C294" s="61" t="inlineStr">
+        <is>
+          <t>Un respaldo para lo inesperado</t>
+        </is>
+      </c>
+      <c r="D294" s="61" t="inlineStr">
+        <is>
+          <t>Según una encuesta de la Reserva Federal de Estados Unidos, más de un tercio de los adultos no podría cubrir un gasto inesperado de 400 dólares con efectivo o su equivalente.</t>
+        </is>
+      </c>
+      <c r="E294" s="61" t="inlineStr">
+        <is>
+          <t>Reserva Federal, Informe sobre el bienestar económico de los hogares de EE. UU., 2024</t>
+        </is>
+      </c>
+      <c r="F294" s="61" t="inlineStr">
+        <is>
+          <t>El salmo contrasta al que no quiere pagar con el que es generoso; no habla de quien no puede pagar por una desgracia. Un pequeño fondo de emergencia ayuda a cumplir aun cuando llega un imprevisto.</t>
+        </is>
+      </c>
+      <c r="G294" s="61" t="inlineStr">
+        <is>
+          <t>Que cada imprevisto se convierta en una deuda nueva.</t>
+        </is>
+      </c>
+      <c r="H294" s="61" t="inlineStr">
+        <is>
+          <t>Empezá un fondo de emergencia con una meta pequeña y alcanzable.</t>
+        </is>
+      </c>
+      <c r="I294" s="61" t="inlineStr">
+        <is>
+          <t>El fondo de emergencia no es falta de fe, sino prudencia, como José, que guardó en los años buenos.</t>
+        </is>
+      </c>
+      <c r="J294" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que ahorrar para imprevistos es desconfiar de Dios.</t>
+        </is>
+      </c>
+      <c r="K294" s="61" t="inlineStr">
+        <is>
+          <t>Separá esta semana un monto pequeño, aunque sea mínimo, para imprevistos.</t>
+        </is>
+      </c>
+      <c r="L294" s="61" t="inlineStr">
+        <is>
+          <t>Tener un pequeño respaldo también permite ayudar a otros en su emergencia sin endeudarse.</t>
+        </is>
+      </c>
+      <c r="M294" s="61" t="inlineStr">
+        <is>
+          <t>Usar el fondo de emergencia para gastos que no son urgentes.</t>
+        </is>
+      </c>
+      <c r="N294" s="61" t="inlineStr">
+        <is>
+          <t>Definan en familia qué cuenta como emergencia y qué no.</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="61" t="n">
+        <v>49</v>
+      </c>
+      <c r="B295" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C295" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: deudas con sabiduría</t>
+        </is>
+      </c>
+      <c r="D295" s="61" t="inlineStr">
+        <is>
+          <t>Las «cosas» que Jesús promete añadir son la comida, la bebida y la ropa de las que acaba de hablar.</t>
+        </is>
+      </c>
+      <c r="E295" s="61" t="inlineStr">
+        <is>
+          <t>Mateo 6:31-33</t>
+        </is>
+      </c>
+      <c r="F295" s="61" t="inlineStr">
+        <is>
+          <t>No toda deuda es igual: hay que distinguir la que genera valor de la que es una trampa.</t>
+        </is>
+      </c>
+      <c r="G295" s="61" t="n"/>
+      <c r="H295" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, anotá todas tus deudas, elegí la primera para pagar y separá un monto pequeño para emergencias, poniendo a Dios primero.</t>
+        </is>
+      </c>
+      <c r="I295" s="61" t="inlineStr">
+        <is>
+          <t>Salir de deudas es un proceso de pasos ordenados, con esperanza y, si hace falta, con consejo profesional.</t>
+        </is>
+      </c>
+      <c r="J295" s="61" t="n"/>
+      <c r="K295" s="61" t="n"/>
+      <c r="L295" s="61" t="inlineStr">
+        <is>
+          <t>Un fondo de emergencia pequeño evita que cada imprevisto sea una deuda nueva.</t>
+        </is>
+      </c>
+      <c r="M295" s="61" t="n"/>
+      <c r="N295" s="61" t="n"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="61" t="n">
+        <v>50</v>
+      </c>
+      <c r="B296" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C296" s="61" t="inlineStr">
+        <is>
+          <t>No esconder los errores</t>
+        </is>
+      </c>
+      <c r="D296" s="61" t="inlineStr">
+        <is>
+          <t>En la aviación, los pilotos pueden reportar sus propios errores en sistemas confidenciales, y eso ayudó a que volar sea más seguro.</t>
+        </is>
+      </c>
+      <c r="E296" s="61" t="inlineStr">
+        <is>
+          <t>NASA, Sistema de Reportes de Seguridad de Aviación (ASRS)</t>
+        </is>
+      </c>
+      <c r="F296" s="61" t="inlineStr">
+        <is>
+          <t>Esconder un error por vergüenza impide aprender de él. El proverbio dice que encubrir no lleva a buen puerto.</t>
+        </is>
+      </c>
+      <c r="G296" s="61" t="inlineStr">
+        <is>
+          <t>Esconder los errores para cuidar la imagen.</t>
+        </is>
+      </c>
+      <c r="H296" s="61" t="inlineStr">
+        <is>
+          <t>Reconocé hoy un error ante quien corresponda, sin excusas.</t>
+        </is>
+      </c>
+      <c r="I296" s="61" t="inlineStr">
+        <is>
+          <t>Reconocer no alcanza: también hay que cambiar de camino. Aprender del error es la forma de no repetirlo.</t>
+        </is>
+      </c>
+      <c r="J296" s="61" t="inlineStr">
+        <is>
+          <t>Pedir perdón y repetir lo mismo.</t>
+        </is>
+      </c>
+      <c r="K296" s="61" t="inlineStr">
+        <is>
+          <t>Anotá qué vas a hacer distinto la próxima vez.</t>
+        </is>
+      </c>
+      <c r="L296" s="61" t="inlineStr">
+        <is>
+          <t>Dios no recibe con un reproche al que reconoce, sino con misericordia. Por eso podemos reconocer sin miedo.</t>
+        </is>
+      </c>
+      <c r="M296" s="61" t="inlineStr">
+        <is>
+          <t>Vivir con miedo al castigo por cada error.</t>
+        </is>
+      </c>
+      <c r="N296" s="61" t="inlineStr">
+        <is>
+          <t>Si cargás con un error del pasado, confesáselo a Dios y recibí su perdón.</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="61" t="n">
+        <v>50</v>
+      </c>
+      <c r="B297" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C297" s="61" t="inlineStr">
+        <is>
+          <t>Algo nuevo</t>
+        </is>
+      </c>
+      <c r="D297" s="61" t="inlineStr">
+        <is>
+          <t>Isaías anuncia aquí el regreso del exilio en Babilonia como un nuevo éxodo, con un camino en el desierto.</t>
+        </is>
+      </c>
+      <c r="E297" s="61" t="inlineStr">
+        <is>
+          <t>Isaías 43:14-21</t>
+        </is>
+      </c>
+      <c r="F297" s="61" t="inlineStr">
+        <is>
+          <t>Dios le pide a su pueblo que no se quede mirando atrás. Salir de la zona de confort empieza por soltar el «siempre se hizo así».</t>
+        </is>
+      </c>
+      <c r="G297" s="61" t="inlineStr">
+        <is>
+          <t>Repetir lo de siempre por miedo a lo nuevo.</t>
+        </is>
+      </c>
+      <c r="H297" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un paso pequeño e incómodo que venís postergando por miedo, y dalo esta semana.</t>
+        </is>
+      </c>
+      <c r="I297" s="61" t="inlineStr">
+        <is>
+          <t>Salir de la zona de confort no es arriesgarlo todo sin pensar: son pasos calculados hacia lo que hace crecer.</t>
+        </is>
+      </c>
+      <c r="J297" s="61" t="inlineStr">
+        <is>
+          <t>Lanzarse a cambios grandes sin evaluar el riesgo.</t>
+        </is>
+      </c>
+      <c r="K297" s="61" t="inlineStr">
+        <is>
+          <t>Antes de un cambio, preguntale a alguien de confianza qué riesgos ve.</t>
+        </is>
+      </c>
+      <c r="L297" s="61" t="inlineStr">
+        <is>
+          <t>«¿Acaso no lo saben?» A veces Dios ya está obrando y no lo vemos porque miramos hacia atrás.</t>
+        </is>
+      </c>
+      <c r="M297" s="61" t="inlineStr">
+        <is>
+          <t>Quejarse del cambio sin ver lo bueno que trae.</t>
+        </is>
+      </c>
+      <c r="N297" s="61" t="inlineStr">
+        <is>
+          <t>Anotá algo nuevo y bueno que apareció en tu vida este año.</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="61" t="n">
+        <v>50</v>
+      </c>
+      <c r="B298" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C298" s="61" t="inlineStr">
+        <is>
+          <t>Lo que forma el carácter</t>
+        </is>
+      </c>
+      <c r="D298" s="61" t="inlineStr">
+        <is>
+          <t>La palabra griega que se traduce «resistencia» (hypomoné) significa literalmente «quedarse debajo»: aguantar sin abandonar.</t>
+        </is>
+      </c>
+      <c r="E298" s="61" t="inlineStr">
+        <is>
+          <t>Romanos 5:3; léxico griego de Strong (G5281, hypomoné)</t>
+        </is>
+      </c>
+      <c r="F298" s="61" t="inlineStr">
+        <is>
+          <t>Pablo no dice que el sufrimiento sea bueno en sí, sino que Dios lo usa para formarnos. No hace falta fingir que no duele.</t>
+        </is>
+      </c>
+      <c r="G298" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que hay que estar contento con el dolor.</t>
+        </is>
+      </c>
+      <c r="H298" s="61" t="inlineStr">
+        <is>
+          <t>Si estás pasando algo difícil, contáselo a Dios con sinceridad y pedile que te forme en el proceso.</t>
+        </is>
+      </c>
+      <c r="I298" s="61" t="inlineStr">
+        <is>
+          <t>Salir de la zona de confort incomoda, y esa incomodidad, sostenida con sabiduría, forma carácter.</t>
+        </is>
+      </c>
+      <c r="J298" s="61" t="inlineStr">
+        <is>
+          <t>Huir de todo lo que incomoda.</t>
+        </is>
+      </c>
+      <c r="K298" s="61" t="inlineStr">
+        <is>
+          <t>Quedate en una tarea difícil un poco más de lo que te gustaría.</t>
+        </is>
+      </c>
+      <c r="L298" s="61" t="inlineStr">
+        <is>
+          <t>La esperanza no es optimismo: es confianza en el amor de Dios, que ya fue derramado en nosotros (5:5).</t>
+        </is>
+      </c>
+      <c r="M298" s="61" t="inlineStr">
+        <is>
+          <t>Confundir la esperanza con pensar que todo va a salir como queremos.</t>
+        </is>
+      </c>
+      <c r="N298" s="61" t="inlineStr">
+        <is>
+          <t>Leé Romanos 5:1-5 y subrayá de dónde viene la esperanza.</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="61" t="n">
+        <v>50</v>
+      </c>
+      <c r="B299" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C299" s="61" t="inlineStr">
+        <is>
+          <t>Que la paciencia complete su obra</t>
+        </is>
+      </c>
+      <c r="D299" s="61" t="inlineStr">
+        <is>
+          <t>Santiago escribe a creyentes judíos dispersos fuera de su tierra: «las doce tribus» de la dispersión.</t>
+        </is>
+      </c>
+      <c r="E299" s="61" t="inlineStr">
+        <is>
+          <t>Santiago 1:1</t>
+        </is>
+      </c>
+      <c r="F299" s="61" t="inlineStr">
+        <is>
+          <t>El gozo no niega la prueba: mira más allá, a lo que Dios forma en ella.</t>
+        </is>
+      </c>
+      <c r="G299" s="61" t="inlineStr">
+        <is>
+          <t>Ver cada prueba solo como un fracaso.</t>
+        </is>
+      </c>
+      <c r="H299" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en una prueba pasada y en lo que te enseñó.</t>
+        </is>
+      </c>
+      <c r="I299" s="61" t="inlineStr">
+        <is>
+          <t>Salir de la zona de confort con sabiduría también es una prueba: pide paciencia para no abandonar al primer obstáculo.</t>
+        </is>
+      </c>
+      <c r="J299" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar un desafío nuevo a la primera dificultad.</t>
+        </is>
+      </c>
+      <c r="K299" s="61" t="inlineStr">
+        <is>
+          <t>Si empezaste algo nuevo, comprometete a sostenerlo un mes antes de evaluarlo.</t>
+        </is>
+      </c>
+      <c r="L299" s="61" t="inlineStr">
+        <is>
+          <t>Santiago habla de madurez, no de una perfección sin errores. Crecer es un proceso.</t>
+        </is>
+      </c>
+      <c r="M299" s="61" t="inlineStr">
+        <is>
+          <t>Exigirse ser perfecto ya.</t>
+        </is>
+      </c>
+      <c r="N299" s="61" t="inlineStr">
+        <is>
+          <t>Agradecé hoy por un área en la que creciste este año, aunque te falte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="61" t="n">
+        <v>50</v>
+      </c>
+      <c r="B300" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C300" s="61" t="inlineStr">
+        <is>
+          <t>Renovados día a día</t>
+        </is>
+      </c>
+      <c r="D300" s="61" t="inlineStr">
+        <is>
+          <t>Pablo escribió esto después de sufrir persecuciones, cárceles y naufragios.</t>
+        </is>
+      </c>
+      <c r="E300" s="61" t="inlineStr">
+        <is>
+          <t>2 Corintios 11:23-27</t>
+        </is>
+      </c>
+      <c r="F300" s="61" t="inlineStr">
+        <is>
+          <t>Por fuera, el cuerpo se desgasta; por dentro, Dios renueva. El crecimiento real casi nunca se ve de un día para otro.</t>
+        </is>
+      </c>
+      <c r="G300" s="61" t="inlineStr">
+        <is>
+          <t>Desanimarse por no ver cambios inmediatos.</t>
+        </is>
+      </c>
+      <c r="H300" s="61" t="inlineStr">
+        <is>
+          <t>Compará cómo estabas hace un año con cómo estás hoy.</t>
+        </is>
+      </c>
+      <c r="I300" s="61" t="inlineStr">
+        <is>
+          <t>La edad o la salud no frenan el crecimiento interior. Siempre se puede crecer en carácter y en fe.</t>
+        </is>
+      </c>
+      <c r="J300" s="61" t="inlineStr">
+        <is>
+          <t>Pensar «ya soy grande para cambiar».</t>
+        </is>
+      </c>
+      <c r="K300" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un área en la que querés crecer el año que viene.</t>
+        </is>
+      </c>
+      <c r="L300" s="61" t="inlineStr">
+        <is>
+          <t>Pablo dice «de día en día»: la renovación es diaria, no un evento único.</t>
+        </is>
+      </c>
+      <c r="M300" s="61" t="inlineStr">
+        <is>
+          <t>Esperar un gran cambio de una sola vez.</t>
+        </is>
+      </c>
+      <c r="N300" s="61" t="inlineStr">
+        <is>
+          <t>Empezá cada día de esta semana pidiéndole a Dios que te renueve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="61" t="n">
+        <v>50</v>
+      </c>
+      <c r="B301" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C301" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: crecer sin prisa</t>
+        </is>
+      </c>
+      <c r="D301" s="61" t="inlineStr">
+        <is>
+          <t>Pablo, ya mayor y preso, todavía pedía que le llevaran sus libros y sus pergaminos.</t>
+        </is>
+      </c>
+      <c r="E301" s="61" t="inlineStr">
+        <is>
+          <t>2 Timoteo 4:13</t>
+        </is>
+      </c>
+      <c r="F301" s="61" t="inlineStr">
+        <is>
+          <t>Reconocer los errores, en vez de esconderlos, permite aprender y recibir misericordia.</t>
+        </is>
+      </c>
+      <c r="G301" s="61" t="n"/>
+      <c r="H301" s="61" t="inlineStr">
+        <is>
+          <t>Esta semana, escribí tres cosas en las que creciste este año y una en la que querés crecer el próximo, y presentáselas a Dios.</t>
+        </is>
+      </c>
+      <c r="I301" s="61" t="inlineStr">
+        <is>
+          <t>Salir de la zona de confort con pasos calculados forma carácter.</t>
+        </is>
+      </c>
+      <c r="J301" s="61" t="n"/>
+      <c r="K301" s="61" t="n"/>
+      <c r="L301" s="61" t="inlineStr">
+        <is>
+          <t>El crecimiento se nota mirando hacia atrás: Dios renueva día a día.</t>
+        </is>
+      </c>
+      <c r="M301" s="61" t="n"/>
+      <c r="N301" s="61" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="61" t="n">
+        <v>51</v>
+      </c>
+      <c r="B302" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C302" s="61" t="inlineStr">
+        <is>
+          <t>Cambiar la forma, no el mensaje</t>
+        </is>
+      </c>
+      <c r="D302" s="61" t="inlineStr">
+        <is>
+          <t>En Atenas, Pablo citó a poetas griegos para anunciar a Jesús a quienes no conocían las Escrituras.</t>
+        </is>
+      </c>
+      <c r="E302" s="61" t="inlineStr">
+        <is>
+          <t>Hechos 17:28</t>
+        </is>
+      </c>
+      <c r="F302" s="61" t="inlineStr">
+        <is>
+          <t>Pablo cambiaba la forma de comunicar según a quién le hablaba, pero nunca cambiaba el mensaje. Adoptar herramientas nuevas es parecido: cambia la forma, no la esencia.</t>
+        </is>
+      </c>
+      <c r="G302" s="61" t="inlineStr">
+        <is>
+          <t>Rechazar toda herramienta nueva solo porque es nueva.</t>
+        </is>
+      </c>
+      <c r="H302" s="61" t="inlineStr">
+        <is>
+          <t>Pensá en una herramienta que podría ayudarte en tu trabajo sin cambiar lo esencial de lo que hacés.</t>
+        </is>
+      </c>
+      <c r="I302" s="61" t="inlineStr">
+        <is>
+          <t>Pablo se adaptaba con un propósito: que más personas conocieran a Jesús. Las herramientas valen por el propósito al que sirven.</t>
+        </is>
+      </c>
+      <c r="J302" s="61" t="inlineStr">
+        <is>
+          <t>Usar la tecnología sin propósito, solo por moda.</t>
+        </is>
+      </c>
+      <c r="K302" s="61" t="inlineStr">
+        <is>
+          <t>Preguntate para qué querés usar una herramienta antes de adoptarla.</t>
+        </is>
+      </c>
+      <c r="L302" s="61" t="inlineStr">
+        <is>
+          <t>Adaptarse no es perder la identidad. Un buen oficio sigue siendo el mismo aunque se registre en una aplicación.</t>
+        </is>
+      </c>
+      <c r="M302" s="61" t="inlineStr">
+        <is>
+          <t>Perder la calidad del trabajo por buscar rapidez.</t>
+        </is>
+      </c>
+      <c r="N302" s="61" t="inlineStr">
+        <is>
+          <t>Usá una herramienta nueva para hacer mejor algo que ya hacés bien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="61" t="n">
+        <v>51</v>
+      </c>
+      <c r="B303" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C303" s="61" t="inlineStr">
+        <is>
+          <t>Entender los tiempos</t>
+        </is>
+      </c>
+      <c r="D303" s="61" t="inlineStr">
+        <is>
+          <t>Este versículo está en la lista de los hombres que se unieron a David en Hebrón para hacerlo rey.</t>
+        </is>
+      </c>
+      <c r="E303" s="61" t="inlineStr">
+        <is>
+          <t>1 Crónicas 12:23, 38</t>
+        </is>
+      </c>
+      <c r="F303" s="61" t="inlineStr">
+        <is>
+          <t>Los de Isacar sabían leer los tiempos y qué hacer. Hoy los tiempos incluyen nuevas formas de trabajar y de comunicarse.</t>
+        </is>
+      </c>
+      <c r="G303" s="61" t="inlineStr">
+        <is>
+          <t>Hacer como si nada cambiara.</t>
+        </is>
+      </c>
+      <c r="H303" s="61" t="inlineStr">
+        <is>
+          <t>Anotá un cambio en tu oficio de los últimos años y cómo podrías aprovecharlo.</t>
+        </is>
+      </c>
+      <c r="I303" s="61" t="inlineStr">
+        <is>
+          <t>Entender los tiempos no es seguir todas las modas, sino discernir qué conviene adoptar y qué no.</t>
+        </is>
+      </c>
+      <c r="J303" s="61" t="inlineStr">
+        <is>
+          <t>Adoptar todo lo nuevo sin pensar.</t>
+        </is>
+      </c>
+      <c r="K303" s="61" t="inlineStr">
+        <is>
+          <t>Antes de usar una aplicación nueva, averiguá qué datos te pide y si es confiable.</t>
+        </is>
+      </c>
+      <c r="L303" s="61" t="inlineStr">
+        <is>
+          <t>Sus palabras eran respetadas porque unían conocimiento y criterio. La tecnología no reemplaza el criterio de quien la usa.</t>
+        </is>
+      </c>
+      <c r="M303" s="61" t="inlineStr">
+        <is>
+          <t>Dejar que una herramienta decida por nosotros.</t>
+        </is>
+      </c>
+      <c r="N303" s="61" t="inlineStr">
+        <is>
+          <t>Usá la tecnología como ayuda, pero revisá vos el resultado final.</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="61" t="n">
+        <v>51</v>
+      </c>
+      <c r="B304" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C304" s="61" t="inlineStr">
+        <is>
+          <t>Buscar conocimiento</t>
+        </is>
+      </c>
+      <c r="D304" s="61" t="inlineStr">
+        <is>
+          <t>Un teléfono celular común de hoy tiene muchísima más capacidad de cálculo que la computadora de guía de las naves Apolo que llegaron a la Luna en 1969.</t>
+        </is>
+      </c>
+      <c r="E304" s="61" t="inlineStr">
+        <is>
+          <t>NASA, computadora de guía del Apolo</t>
+        </is>
+      </c>
+      <c r="F304" s="61" t="inlineStr">
+        <is>
+          <t>El sabio busca aprender. La tecnología puede facilitar tareas, pero no reemplaza el esfuerzo, el criterio ni la experiencia.</t>
+        </is>
+      </c>
+      <c r="G304" s="61" t="inlineStr">
+        <is>
+          <t>Esperar que una aplicación haga todo el trabajo por nosotros.</t>
+        </is>
+      </c>
+      <c r="H304" s="61" t="inlineStr">
+        <is>
+          <t>Pensá qué parte de tu trabajo requiere tu criterio y no la puede hacer una máquina.</t>
+        </is>
+      </c>
+      <c r="I304" s="61" t="inlineStr">
+        <is>
+          <t>Muchos temen que la tecnología les quite el trabajo. Quien aprende a usarla a su favor suele trabajar mejor.</t>
+        </is>
+      </c>
+      <c r="J304" s="61" t="inlineStr">
+        <is>
+          <t>Ver la tecnología solo como una amenaza.</t>
+        </is>
+      </c>
+      <c r="K304" s="61" t="inlineStr">
+        <is>
+          <t>Aprendé esta semana una sola función nueva de una herramienta que ya usás.</t>
+        </is>
+      </c>
+      <c r="L304" s="61" t="inlineStr">
+        <is>
+          <t>Los oídos sabios buscan: preguntar a quien sabe más, aunque sea más joven, es humildad.</t>
+        </is>
+      </c>
+      <c r="M304" s="61" t="inlineStr">
+        <is>
+          <t>Tener vergüenza de preguntar cómo se usa algo.</t>
+        </is>
+      </c>
+      <c r="N304" s="61" t="inlineStr">
+        <is>
+          <t>Pedile a alguien más joven que te enseñe algo de tecnología, y enseñale vos algo de tu oficio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="61" t="n">
+        <v>51</v>
+      </c>
+      <c r="B305" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C305" s="61" t="inlineStr">
+        <is>
+          <t>Afilar el hacha</t>
+        </is>
+      </c>
+      <c r="D305" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés observa la vida con ejemplos del trabajo de todos los días, como cavar un pozo, sacar piedras o cortar leña.</t>
+        </is>
+      </c>
+      <c r="E305" s="61" t="inlineStr">
+        <is>
+          <t>Eclesiastés 10:8-10</t>
+        </is>
+      </c>
+      <c r="F305" s="61" t="inlineStr">
+        <is>
+          <t>Con el hacha sin filo hay que golpear más fuerte. La tecnología bien usada es como afilar el hacha: el mismo esfuerzo rinde más.</t>
+        </is>
+      </c>
+      <c r="G305" s="61" t="inlineStr">
+        <is>
+          <t>Trabajar más duro en vez de trabajar mejor.</t>
+        </is>
+      </c>
+      <c r="H305" s="61" t="inlineStr">
+        <is>
+          <t>Identificá una tarea repetitiva que podrías hacer mejor con una herramienta.</t>
+        </is>
+      </c>
+      <c r="I305" s="61" t="inlineStr">
+        <is>
+          <t>Afilar lleva tiempo, pero después ahorra mucho. Capacitarse también.</t>
+        </is>
+      </c>
+      <c r="J305" s="61" t="inlineStr">
+        <is>
+          <t>Decir «no tengo tiempo para aprender» y seguir perdiendo tiempo.</t>
+        </is>
+      </c>
+      <c r="K305" s="61" t="inlineStr">
+        <is>
+          <t>Reservá media hora esta semana para aprender algo que te ahorre tiempo.</t>
+        </is>
+      </c>
+      <c r="L305" s="61" t="inlineStr">
+        <is>
+          <t>La herramienta sirve, pero la que dirige es la sabiduría.</t>
+        </is>
+      </c>
+      <c r="M305" s="61" t="inlineStr">
+        <is>
+          <t>Tener las mejores herramientas y no saber para qué usarlas.</t>
+        </is>
+      </c>
+      <c r="N305" s="61" t="inlineStr">
+        <is>
+          <t>Antes de comprar una herramienta nueva, aprendé a usar bien la que ya tenés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="61" t="n">
+        <v>51</v>
+      </c>
+      <c r="B306" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C306" s="61" t="inlineStr">
+        <is>
+          <t>Ver el peligro</t>
+        </is>
+      </c>
+      <c r="D306" s="61" t="inlineStr">
+        <is>
+          <t>Los bancos recuerdan que nunca piden por teléfono ni por mensaje las claves ni los códigos de verificación.</t>
+        </is>
+      </c>
+      <c r="E306" s="61" t="inlineStr">
+        <is>
+          <t>Recomendaciones de seguridad de los bancos y del Banco Central del Paraguay</t>
+        </is>
+      </c>
+      <c r="F306" s="61" t="inlineStr">
+        <is>
+          <t>La prudencia también vale en lo digital. Aprender lo básico de seguridad es parte de capacitarse.</t>
+        </is>
+      </c>
+      <c r="G306" s="61" t="inlineStr">
+        <is>
+          <t>Compartir códigos o claves porque alguien los pidió con urgencia.</t>
+        </is>
+      </c>
+      <c r="H306" s="61" t="inlineStr">
+        <is>
+          <t>Nunca compartas por mensaje un código de verificación o una clave, aunque parezca un conocido.</t>
+        </is>
+      </c>
+      <c r="I306" s="61" t="inlineStr">
+        <is>
+          <t>El miedo a no entender suele ser más grande que la dificultad real de aprender. Con pasos pequeños se avanza.</t>
+        </is>
+      </c>
+      <c r="J306" s="61" t="inlineStr">
+        <is>
+          <t>Quedarse atrás por miedo a lo nuevo.</t>
+        </is>
+      </c>
+      <c r="K306" s="61" t="inlineStr">
+        <is>
+          <t>Elegí un primer paso mínimo: aprender una sola función nueva esta semana.</t>
+        </is>
+      </c>
+      <c r="L306" s="61" t="inlineStr">
+        <is>
+          <t>Hoy es Nochebuena: cuidemos también el tiempo en familia, sin que las pantallas lo ocupen todo.</t>
+        </is>
+      </c>
+      <c r="M306" s="61" t="inlineStr">
+        <is>
+          <t>Pasar la Nochebuena cada uno con su celular.</t>
+        </is>
+      </c>
+      <c r="N306" s="61" t="inlineStr">
+        <is>
+          <t>Esta noche, propongan en familia un tiempo sin pantallas para conversar y agradecer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="61" t="n">
+        <v>51</v>
+      </c>
+      <c r="B307" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C307" s="61" t="inlineStr">
+        <is>
+          <t>Repaso y Navidad</t>
+        </is>
+      </c>
+      <c r="D307" s="61" t="inlineStr">
+        <is>
+          <t>Hoy celebramos el nacimiento de Jesús: el ángel les dio a los pastores un anuncio de gran alegría para todo el pueblo.</t>
+        </is>
+      </c>
+      <c r="E307" s="61" t="inlineStr">
+        <is>
+          <t>Lucas 2:10-11</t>
+        </is>
+      </c>
+      <c r="F307" s="61" t="inlineStr">
+        <is>
+          <t>Adoptar herramientas nuevas sin perder la esencia, como Pablo, que cambiaba la forma y no el mensaje.</t>
+        </is>
+      </c>
+      <c r="G307" s="61" t="n"/>
+      <c r="H307" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, Navidad, dejen las pantallas a un lado un rato, lean juntos Lucas 2:1-20 y agradezcan a Dios por el regalo de Jesús.</t>
+        </is>
+      </c>
+      <c r="I307" s="61" t="inlineStr">
+        <is>
+          <t>La tecnología es una aliada, no un reemplazo del esfuerzo ni del criterio.</t>
+        </is>
+      </c>
+      <c r="J307" s="61" t="n"/>
+      <c r="K307" s="61" t="n"/>
+      <c r="L307" s="61" t="inlineStr">
+        <is>
+          <t>Capacitarse sin miedo y con prudencia, porque el sabio nunca deja de aprender.</t>
+        </is>
+      </c>
+      <c r="M307" s="61" t="n"/>
+      <c r="N307" s="61" t="n"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="61" t="n">
+        <v>52</v>
+      </c>
+      <c r="B308" s="61" t="inlineStr">
+        <is>
+          <t>Lunes</t>
+        </is>
+      </c>
+      <c r="C308" s="61" t="inlineStr">
+        <is>
+          <t>Orar unos por otros</t>
+        </is>
+      </c>
+      <c r="D308" s="61" t="inlineStr">
+        <is>
+          <t>La Organización Mundial de la Salud define la salud como un estado de completo bienestar físico, mental y social, y no solo como la ausencia de enfermedades.</t>
+        </is>
+      </c>
+      <c r="E308" s="61" t="inlineStr">
+        <is>
+          <t>Constitución de la Organización Mundial de la Salud, 1946</t>
+        </is>
+      </c>
+      <c r="F308" s="61" t="inlineStr">
+        <is>
+          <t>Santiago une la sanidad del cuerpo con la del alma: confesarse y orar unos por otros. La salud es más que no tener una enfermedad.</t>
+        </is>
+      </c>
+      <c r="G308" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que estar sano es solo no tener un diagnóstico.</t>
+        </is>
+      </c>
+      <c r="H308" s="61" t="inlineStr">
+        <is>
+          <t>Preguntate: ¿cómo estoy de cuerpo, de ánimo y en mi relación con Dios?</t>
+        </is>
+      </c>
+      <c r="I308" s="61" t="inlineStr">
+        <is>
+          <t>Orar juntos sostiene. No sabemos cómo responderá Dios, pero sí que no estamos solos.</t>
+        </is>
+      </c>
+      <c r="J308" s="61" t="inlineStr">
+        <is>
+          <t>Enfermarse y aislarse de todos.</t>
+        </is>
+      </c>
+      <c r="K308" s="61" t="inlineStr">
+        <is>
+          <t>Pedile a alguien de confianza que ore por algo de tu salud.</t>
+        </is>
+      </c>
+      <c r="L308" s="61" t="inlineStr">
+        <is>
+          <t>Contarle a alguien de confianza lo que nos pesa alivia. Guardarse todo adentro también enferma.</t>
+        </is>
+      </c>
+      <c r="M308" s="61" t="inlineStr">
+        <is>
+          <t>Cargar culpas y preocupaciones sin hablarlas con nadie.</t>
+        </is>
+      </c>
+      <c r="N308" s="61" t="inlineStr">
+        <is>
+          <t>Contale hoy a alguien de confianza algo que te viene pesando.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="61" t="n">
+        <v>52</v>
+      </c>
+      <c r="B309" s="61" t="inlineStr">
+        <is>
+          <t>Martes</t>
+        </is>
+      </c>
+      <c r="C309" s="61" t="inlineStr">
+        <is>
+          <t>Sana las heridas</t>
+        </is>
+      </c>
+      <c r="D309" s="61" t="inlineStr">
+        <is>
+          <t>Según la Organización Mundial de la Salud, la depresión es una de las principales causas de discapacidad en el mundo.</t>
+        </is>
+      </c>
+      <c r="E309" s="61" t="inlineStr">
+        <is>
+          <t>Organización Mundial de la Salud, nota descriptiva sobre la depresión</t>
+        </is>
+      </c>
+      <c r="F309" s="61" t="inlineStr">
+        <is>
+          <t>El salmo dice que Dios reanima a los descorazonados. La salud integral incluye el corazón herido.</t>
+        </is>
+      </c>
+      <c r="G309" s="61" t="inlineStr">
+        <is>
+          <t>Ignorar las heridas emocionales porque «no se ven».</t>
+        </is>
+      </c>
+      <c r="H309" s="61" t="inlineStr">
+        <is>
+          <t>Nombrá delante de Dios una herida emocional que todavía te duele.</t>
+        </is>
+      </c>
+      <c r="I309" s="61" t="inlineStr">
+        <is>
+          <t>Dios sana de muchas maneras, también por medio de un psicólogo, un médico o un consejero. Pedir ayuda no es falta de fe.</t>
+        </is>
+      </c>
+      <c r="J309" s="61" t="inlineStr">
+        <is>
+          <t>Pensar que la tristeza profunda se cura solo con fuerza de voluntad.</t>
+        </is>
+      </c>
+      <c r="K309" s="61" t="inlineStr">
+        <is>
+          <t>Si hace semanas que estás muy triste, consultá a un profesional de la salud.</t>
+        </is>
+      </c>
+      <c r="L309" s="61" t="inlineStr">
+        <is>
+          <t>Las heridas del alma también necesitan tiempo y cuidado. Dios no se cansa de acompañar ese proceso.</t>
+        </is>
+      </c>
+      <c r="M309" s="61" t="inlineStr">
+        <is>
+          <t>Exigirse estar bien de inmediato.</t>
+        </is>
+      </c>
+      <c r="N309" s="61" t="inlineStr">
+        <is>
+          <t>Date permiso para sanar a tu ritmo, y pedí ayuda en el camino.</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="61" t="n">
+        <v>52</v>
+      </c>
+      <c r="B310" s="61" t="inlineStr">
+        <is>
+          <t>Miércoles</t>
+        </is>
+      </c>
+      <c r="C310" s="61" t="inlineStr">
+        <is>
+          <t>Los que necesitan médico</t>
+        </is>
+      </c>
+      <c r="D310" s="61" t="inlineStr">
+        <is>
+          <t>Lucas, autor del evangelio y del libro de los Hechos, era médico.</t>
+        </is>
+      </c>
+      <c r="E310" s="61" t="inlineStr">
+        <is>
+          <t>Colosenses 4:14</t>
+        </is>
+      </c>
+      <c r="F310" s="61" t="inlineStr">
+        <is>
+          <t>Jesús usa la imagen del médico para hablar de su misión con los pecadores, y la usa porque todos sabían que el enfermo necesita médico.</t>
+        </is>
+      </c>
+      <c r="G310" s="61" t="inlineStr">
+        <is>
+          <t>Rechazar la medicina en nombre de la fe.</t>
+        </is>
+      </c>
+      <c r="H310" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un control médico pendiente, agendalo esta semana.</t>
+        </is>
+      </c>
+      <c r="I310" s="61" t="inlineStr">
+        <is>
+          <t>Buscar tratamiento médico y orar no son caminos opuestos. Lucas, el médico, escribió dos libros de la Biblia.</t>
+        </is>
+      </c>
+      <c r="J310" s="61" t="inlineStr">
+        <is>
+          <t>Rechazar la fe en nombre de la ciencia, o la ciencia en nombre de la fe.</t>
+        </is>
+      </c>
+      <c r="K310" s="61" t="inlineStr">
+        <is>
+          <t>Cuando vayas al médico, orá antes y seguí sus indicaciones después.</t>
+        </is>
+      </c>
+      <c r="L310" s="61" t="inlineStr">
+        <is>
+          <t>Admitir que estamos enfermos, en el cuerpo o en el alma, es el primer paso para recibir ayuda.</t>
+        </is>
+      </c>
+      <c r="M310" s="61" t="inlineStr">
+        <is>
+          <t>Negar los síntomas por miedo.</t>
+        </is>
+      </c>
+      <c r="N310" s="61" t="inlineStr">
+        <is>
+          <t>Si venís notando un síntoma que te preocupa, consultalo sin esperar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="61" t="n">
+        <v>52</v>
+      </c>
+      <c r="B311" s="61" t="inlineStr">
+        <is>
+          <t>Jueves</t>
+        </is>
+      </c>
+      <c r="C311" s="61" t="inlineStr">
+        <is>
+          <t>Por su llaga</t>
+        </is>
+      </c>
+      <c r="D311" s="61" t="inlineStr">
+        <is>
+          <t>Isaías 53 fue escrito varios siglos antes de Jesús, y el Nuevo Testamento lo cita para explicar su muerte.</t>
+        </is>
+      </c>
+      <c r="E311" s="61" t="inlineStr">
+        <is>
+          <t>Hechos 8:32-35; 1 Pedro 2:24</t>
+        </is>
+      </c>
+      <c r="F311" s="61" t="inlineStr">
+        <is>
+          <t>Isaías anuncia al siervo que sufre por nuestros pecados. Pedro aplica este versículo al perdón: fuimos sanados para vivir para la justicia (1 Pedro 2:24).</t>
+        </is>
+      </c>
+      <c r="G311" s="61" t="inlineStr">
+        <is>
+          <t>Usar este versículo para prometer que toda enfermedad va a desaparecer si hay fe.</t>
+        </is>
+      </c>
+      <c r="H311" s="61" t="inlineStr">
+        <is>
+          <t>Agradecele hoy a Jesús su entrega por vos.</t>
+        </is>
+      </c>
+      <c r="I311" s="61" t="inlineStr">
+        <is>
+          <t>Las iglesias entienden de distintas maneras si esta promesa incluye hoy la sanidad física. Todas coinciden en que su centro es el perdón y la paz con Dios. Y nadie queda sin sanar por falta de fe.</t>
+        </is>
+      </c>
+      <c r="J311" s="61" t="inlineStr">
+        <is>
+          <t>Culpar al enfermo de «no tener fe suficiente».</t>
+        </is>
+      </c>
+      <c r="K311" s="61" t="inlineStr">
+        <is>
+          <t>Si alguien está enfermo, acompañalo sin juzgar su fe.</t>
+        </is>
+      </c>
+      <c r="L311" s="61" t="inlineStr">
+        <is>
+          <t>Dios puede sanar por un milagro o por medio de la medicina; las dos cosas vienen de él.</t>
+        </is>
+      </c>
+      <c r="M311" s="61" t="inlineStr">
+        <is>
+          <t>Despreciar la medicina como si fuera menos espiritual.</t>
+        </is>
+      </c>
+      <c r="N311" s="61" t="inlineStr">
+        <is>
+          <t>Orá hoy por los médicos y los enfermeros que cuidan a los enfermos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="61" t="n">
+        <v>52</v>
+      </c>
+      <c r="B312" s="61" t="inlineStr">
+        <is>
+          <t>Viernes</t>
+        </is>
+      </c>
+      <c r="C312" s="61" t="inlineStr">
+        <is>
+          <t>Un corazón alegre</t>
+        </is>
+      </c>
+      <c r="D312" s="61" t="inlineStr">
+        <is>
+          <t>En un estudio, reír en grupo con videos de comedia aumentó la tolerancia al dolor de los participantes.</t>
+        </is>
+      </c>
+      <c r="E312" s="61" t="inlineStr">
+        <is>
+          <t>Dunbar y otros, Proceedings of the Royal Society B, 2012</t>
+        </is>
+      </c>
+      <c r="F312" s="61" t="inlineStr">
+        <is>
+          <t>Hoy cerramos el año. El proverbio enseña que el ánimo influye en el cuerpo: la alegría, la gratitud y la buena compañía ayudan a la salud.</t>
+        </is>
+      </c>
+      <c r="G312" s="61" t="inlineStr">
+        <is>
+          <t>Terminar el año mirando solo lo que salió mal.</t>
+        </is>
+      </c>
+      <c r="H312" s="61" t="inlineStr">
+        <is>
+          <t>Esta noche, en familia, nombren tres cosas por las que agradecen este año.</t>
+        </is>
+      </c>
+      <c r="I312" s="61" t="inlineStr">
+        <is>
+          <t>El proverbio describe, no culpa: la tristeza afecta al cuerpo. Quien está triste no necesita reproches, sino compañía y, si hace falta, ayuda profesional.</t>
+        </is>
+      </c>
+      <c r="J312" s="61" t="inlineStr">
+        <is>
+          <t>Decirle a alguien triste «poné buena cara».</t>
+        </is>
+      </c>
+      <c r="K312" s="61" t="inlineStr">
+        <is>
+          <t>Llamá hoy a alguien que sabés que está pasando un fin de año difícil.</t>
+        </is>
+      </c>
+      <c r="L312" s="61" t="inlineStr">
+        <is>
+          <t>Orar por la salud y seguir el tratamiento médico no se contradicen: son formas complementarias de cuidar lo que Dios nos dio.</t>
+        </is>
+      </c>
+      <c r="M312" s="61" t="inlineStr">
+        <is>
+          <t>Abandonar un tratamiento porque «ya oramos».</t>
+        </is>
+      </c>
+      <c r="N312" s="61" t="inlineStr">
+        <is>
+          <t>Si tenés un tratamiento, seguilo con constancia y presentale cada día tu salud a Dios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="61" t="n">
+        <v>52</v>
+      </c>
+      <c r="B313" s="61" t="inlineStr">
+        <is>
+          <t>Sábado</t>
+        </is>
+      </c>
+      <c r="C313" s="61" t="inlineStr">
+        <is>
+          <t>Repaso: sanidad integral</t>
+        </is>
+      </c>
+      <c r="D313" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios compara las palabras amables con un panal: en la antigüedad, la miel también se usaba como remedio.</t>
+        </is>
+      </c>
+      <c r="E313" s="61" t="inlineStr">
+        <is>
+          <t>Proverbios 16:24; 24:13</t>
+        </is>
+      </c>
+      <c r="F313" s="61" t="inlineStr">
+        <is>
+          <t>La salud es más que no estar enfermo: incluye el cuerpo, la mente y el espíritu.</t>
+        </is>
+      </c>
+      <c r="G313" s="61" t="n"/>
+      <c r="H313" s="61" t="inlineStr">
+        <is>
+          <t>Hoy, primer día del año, decí palabras amables a los de tu casa y elegí un cuidado de salud para empezar: un control médico, una caminata o pedir ayuda donde haga falta.</t>
+        </is>
+      </c>
+      <c r="I313" s="61" t="inlineStr">
+        <is>
+          <t>La fe y la medicina caminan juntas; buscar ayuda no es falta de fe.</t>
+        </is>
+      </c>
+      <c r="J313" s="61" t="n"/>
+      <c r="K313" s="61" t="n"/>
+      <c r="L313" s="61" t="inlineStr">
+        <is>
+          <t>Orar y seguir el tratamiento son formas complementarias de cuidar la salud.</t>
+        </is>
+      </c>
+      <c r="M313" s="61" t="n"/>
+      <c r="N313" s="61" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mensajero: datos de diciembre verificados; año completo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -38259,7 +38259,7 @@
       </c>
       <c r="D286" s="61" t="inlineStr">
         <is>
-          <t>David cantó este himno cuando llevaron el arca del pacto a Jerusalén.</t>
+          <t>Cuando llevaron el arca del pacto a Jerusalén, David les encargó a Asaf y a sus hermanos que cantaran este salmo de alabanza al Señor.</t>
         </is>
       </c>
       <c r="E286" s="61" t="inlineStr">
@@ -38589,12 +38589,12 @@
       </c>
       <c r="D291" s="61" t="inlineStr">
         <is>
-          <t>En tiempos bíblicos, quien no podía pagar podía perder hasta su manto; la ley pedía devolverlo antes de la noche.</t>
+          <t>En tiempos bíblicos, quien se endeudaba podía dejar su manto en prenda; la ley pedía devolverlo antes de que se pusiera el sol, porque era su abrigo para dormir.</t>
         </is>
       </c>
       <c r="E291" s="61" t="inlineStr">
         <is>
-          <t>Éxodo 22:26-27; Proverbios 22:27</t>
+          <t>Éxodo 22:26-27; Deuteronomio 24:12-13</t>
         </is>
       </c>
       <c r="F291" s="61" t="inlineStr">
@@ -39059,7 +39059,7 @@
       </c>
       <c r="D298" s="61" t="inlineStr">
         <is>
-          <t>La palabra griega que se traduce «resistencia» (hypomoné) significa literalmente «quedarse debajo»: aguantar sin abandonar.</t>
+          <t>La palabra griega que en este versículo se traduce «resistencia» (hypomoné) se forma con «debajo» y «permanecer»: quedarse firme bajo la carga, sin abandonar.</t>
         </is>
       </c>
       <c r="E298" s="61" t="inlineStr">
@@ -39599,12 +39599,12 @@
       </c>
       <c r="D306" s="61" t="inlineStr">
         <is>
-          <t>Los bancos recuerdan que nunca piden por teléfono ni por mensaje las claves ni los códigos de verificación.</t>
+          <t>El Banco Central del Paraguay pide desconfiar de cualquier llamada o mensaje que solicite claves, PIN, token o códigos de verificación, y no compartirlos nunca, aunque quien llama diga ser del banco.</t>
         </is>
       </c>
       <c r="E306" s="61" t="inlineStr">
         <is>
-          <t>Recomendaciones de seguridad de los bancos y del Banco Central del Paraguay</t>
+          <t>Banco Central del Paraguay, campaña «Seguridad Financiera Digital», 2026</t>
         </is>
       </c>
       <c r="F306" s="61" t="inlineStr">
@@ -39669,7 +39669,7 @@
       </c>
       <c r="D307" s="61" t="inlineStr">
         <is>
-          <t>Hoy celebramos el nacimiento de Jesús: el ángel les dio a los pastores un anuncio de gran alegría para todo el pueblo.</t>
+          <t>Hoy celebramos el nacimiento de Jesús: el ángel les dio a los pastores una buena noticia, motivo de mucha alegría para todo el pueblo.</t>
         </is>
       </c>
       <c r="E307" s="61" t="inlineStr">
@@ -39859,12 +39859,12 @@
       </c>
       <c r="D310" s="61" t="inlineStr">
         <is>
-          <t>Lucas, autor del evangelio y del libro de los Hechos, era médico.</t>
+          <t>Lucas era médico, y la tradición cristiana lo reconoce como autor del evangelio que lleva su nombre y del libro de los Hechos.</t>
         </is>
       </c>
       <c r="E310" s="61" t="inlineStr">
         <is>
-          <t>Colosenses 4:14</t>
+          <t>Colosenses 4:14; Lucas 1:1-4; Hechos 1:1</t>
         </is>
       </c>
       <c r="F310" s="61" t="inlineStr">
@@ -39884,7 +39884,7 @@
       </c>
       <c r="I310" s="61" t="inlineStr">
         <is>
-          <t>Buscar tratamiento médico y orar no son caminos opuestos. Lucas, el médico, escribió dos libros de la Biblia.</t>
+          <t>Buscar tratamiento médico y orar no son caminos opuestos. Según la tradición, Lucas, el médico, escribió dos libros de la Biblia.</t>
         </is>
       </c>
       <c r="J310" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: 156 frases célebres verificadas y corregidas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -1008,7 +1008,7 @@
       </c>
       <c r="J2" s="21" t="inlineStr">
         <is>
-          <t>"Si no encuentra tiempo para hacer ejercicio, tendrá que encontrar tiempo para estar enfermo." — Ernie Zelinski</t>
+          <t>"La gloria de Dios es el hombre viviente, y la vida del hombre es la visión de Dios." — Ireneo de Lyon</t>
         </is>
       </c>
       <c r="K2" s="21" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="N2" s="21" t="inlineStr">
         <is>
-          <t>"Sé celoso de tu tiempo, porque es tu mayor tesoro." — Og Mandino</t>
+          <t>"Practicando la justicia nos hacemos justos; practicando la moderación, moderados; y practicando la valentía, valientes." — Aristóteles</t>
         </is>
       </c>
       <c r="O2" s="21" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="R2" s="21" t="inlineStr">
         <is>
-          <t>"La vida no siempre te da lo que quieres, pero si miras de cerca verás que te da lo que necesitas para tu crecimiento." — León Brown</t>
+          <t>"Toda la desgracia de los hombres viene de una sola cosa: no saber quedarse en reposo en una habitación." — Blaise Pascal</t>
         </is>
       </c>
       <c r="S2" s="21" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="J3" s="23" t="inlineStr">
         <is>
-          <t>"Siembra un carácter y cosecharás un destino." — Proverbio chino</t>
+          <t>"Con perseverancia, el caracol llegó al arca." — Charles H. Spurgeon</t>
         </is>
       </c>
       <c r="K3" s="23" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="N3" s="23" t="inlineStr">
         <is>
-          <t>"Un jardinero que cultiva su propio jardín, con sus propias manos, une en su persona los tres personajes: propietario, agricultor y obrero." — Adam Smith</t>
+          <t>"Un jardinero que cultiva su propio jardín con sus propias manos une en su persona los tres personajes: propietario, agricultor y obrero." — Adam Smith</t>
         </is>
       </c>
       <c r="O3" s="23" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="R3" s="23" t="inlineStr">
         <is>
-          <t>"Nuestra recompensa se encuentra en el esfuerzo y no en el resultado. Un esfuerzo total es una victoria completa." — Mahatma Gandhi</t>
+          <t>"La nación se comporta bien si trata sus recursos naturales como bienes que debe entregar a la próxima generación aumentados, y no disminuidos, en valor." — Theodore Roosevelt</t>
         </is>
       </c>
       <c r="S3" s="23" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="N4" s="27" t="inlineStr">
         <is>
-          <t>"La buena salud no es algo que podamos comprar. Sin embargo, puede ser una cuenta de ahorros extremadamente valiosa." — Anne Wilson Schaef</t>
+          <t>"Resistí desde el principio: tarde se prepara la medicina cuando el mal se ha fortalecido por largas demoras." — Ovidio</t>
         </is>
       </c>
       <c r="O4" s="27" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="R4" s="27" t="inlineStr">
         <is>
-          <t>"La parte nunca podrá estar bien, a menos que el todo también lo este." — Platón</t>
+          <t>"La parte nunca puede estar bien a menos que el todo esté bien." — Platón</t>
         </is>
       </c>
       <c r="S4" s="27" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="J5" s="30" t="inlineStr">
         <is>
-          <t>"El vigor de nuestra vida espiritual será en exacta proporción al lugar que la Biblia ocupa en nuestras vidas y pensamientos." — George Muller</t>
+          <t>"El vigor de nuestra vida espiritual estará en exacta proporción al lugar que la Biblia ocupe en nuestra vida y pensamientos." — atribuida a George Müller</t>
         </is>
       </c>
       <c r="K5" s="30" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="N5" s="30" t="inlineStr">
         <is>
-          <t>"Los errores más grandes de la iglesia ocurren cuando la gente honra lo que sus pastores dicen sin examinar esas enseñanzas a la luz de las Escrituras." — Bryan Chapell</t>
+          <t>"Ignorar las Escrituras es ignorar a Cristo." — Jerónimo de Estridón</t>
         </is>
       </c>
       <c r="O5" s="30" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="R5" s="30" t="inlineStr">
         <is>
-          <t>"Si no estudias teología, esto no querrá decir que no tengas ideas acerca de Dios, sino que tendrás muchas equivocadas." — C.S. Lewis</t>
+          <t>"Si no escuchás a la teología, eso no significa que no tengas ideas acerca de Dios; significa que tendrás muchas equivocadas." — C. S. Lewis</t>
         </is>
       </c>
       <c r="S5" s="30" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="J6" s="37" t="inlineStr">
         <is>
-          <t>"El liderazgo es una combinación de estrategia y carácter. Si debes prescindir de uno, prescinde de la estrategia." — Norman Schwarzkopf</t>
+          <t>"El carácter del hombre es su destino." — Heráclito</t>
         </is>
       </c>
       <c r="K6" s="37" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="N6" s="37" t="inlineStr">
         <is>
-          <t>"Hay una diferencia entre ser un líder y ser un jefe. Un jefe demanda obediencia ciega; un líder se gana su autoridad a través de conocimiento y confianza." — Klaus Balkenhol</t>
+          <t>"La integridad sin conocimiento es débil e inútil, y el conocimiento sin integridad es peligroso y temible." — Samuel Johnson</t>
         </is>
       </c>
       <c r="O6" s="37" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="R6" s="37" t="inlineStr">
         <is>
-          <t>"Un buen líder toma un poco más de su parte de la culpa, un poco menos de su parte de los elogios." — Arnold H. Glasow</t>
+          <t>"El carácter es lo que sos en la oscuridad." — Dwight L. Moody</t>
         </is>
       </c>
       <c r="S6" s="37" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="J7" s="35" t="inlineStr">
         <is>
-          <t>"Gobernar una familia es poco menos difícil que gobernar un reino." — Michel de Montaigne</t>
+          <t>"No hay mucho menos tormento en gobernar una familia que en gobernar un Estado entero." — Michel de Montaigne</t>
         </is>
       </c>
       <c r="K7" s="35" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="N7" s="35" t="inlineStr">
         <is>
-          <t>"La familia es una de las obras maestras de la naturaleza." — George Santayana</t>
+          <t>"Limpieza: no toleres falta de limpieza en el cuerpo, la ropa ni la casa." — Benjamin Franklin</t>
         </is>
       </c>
       <c r="O7" s="35" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="R7" s="35" t="inlineStr">
         <is>
-          <t>"Es imposible ganar las grandes apuestas de la vida sin correr riesgos, y las apuestas más grandes son las relacionadas con el hogar y la familia." — Teddy Roosevelt</t>
+          <t>"Quiero que encuentren a los pobres aquí, primero en su propio hogar, y que empiecen a amar allí." — Teresa de Calcuta</t>
         </is>
       </c>
       <c r="S7" s="35" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="J8" s="40" t="inlineStr">
         <is>
-          <t>"El ahorro es un ingrediente esencial del éxito." — John D. Rockefeller</t>
+          <t>"Los hombres no se hacen ricos por lo que ganan, sino por lo que ahorran." — Charles Spurgeon</t>
         </is>
       </c>
       <c r="K8" s="40" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="N8" s="40" t="inlineStr">
         <is>
-          <t>"El más rico de todos los hombres es el ahorrativo; el más pobre, el avaro." — Nicolás de Chamfort</t>
+          <t>"El más rico de todos los hombres es el ahorrativo; el más pobre, el avaro." — Nicolas de Chamfort</t>
         </is>
       </c>
       <c r="O8" s="40" t="inlineStr">
@@ -2280,7 +2280,7 @@
       </c>
       <c r="R8" s="40" t="inlineStr">
         <is>
-          <t>"Un centavo ahorrado es un centavo ganado." — Benjamin Franklin</t>
+          <t>"Tarde llega el ahorro cuando ya se ha llegado al fondo." — Séneca</t>
         </is>
       </c>
       <c r="S8" s="40" t="inlineStr">
@@ -2447,7 +2447,7 @@
       </c>
       <c r="J9" s="43" t="inlineStr">
         <is>
-          <t>"Yo no soy lo que me sucedió. Yo soy lo que elegí ser." — Carl Jung</t>
+          <t>"El corazón tiene razones que la razón no conoce." — Blaise Pascal</t>
         </is>
       </c>
       <c r="K9" s="43" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="N9" s="43" t="inlineStr">
         <is>
-          <t>"Los desafíos que enfrentamos en la vida son siempre lecciones que sirven para el crecimiento de nuestra alma." — Marianne Williamson</t>
+          <t>"Tal como sean tus pensamientos habituales, así será tu mente, porque el alma se tiñe del color de sus pensamientos." — Marco Aurelio</t>
         </is>
       </c>
       <c r="O9" s="43" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="R9" s="43" t="inlineStr">
         <is>
-          <t>"Cuando no podemos cambiar la situación a la que nos enfrentamos, el reto consiste en cambiarnos a nosotros mismos." — Viktor Frankl</t>
+          <t>"Hasta que no podamos recibir con el corazón abierto, nunca estaremos dando de verdad con el corazón abierto." — Brené Brown</t>
         </is>
       </c>
       <c r="S9" s="43" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="J10" s="47" t="inlineStr">
         <is>
-          <t>"El éxito es el resultado de la preparación, el trabajo duro y el aprendizaje continuo." — Colin Powell</t>
+          <t>"La gota horada la piedra." — Ovidio</t>
         </is>
       </c>
       <c r="K10" s="47" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="N10" s="47" t="inlineStr">
         <is>
-          <t>"Un jardinero que cultiva su propio jardín, con sus propias manos, une en su persona los tres personajes: propietario, agricultor y obrero." — Adam Smith</t>
+          <t>"Quien es cruel con los animales se vuelve duro también en su trato con los hombres." — Immanuel Kant</t>
         </is>
       </c>
       <c r="O10" s="47" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="R10" s="47" t="inlineStr">
         <is>
-          <t>"El trabajo es el único medio digno de ganarse la vida." — José Martí</t>
+          <t>"Antes de terminar de desayunar por la mañana, ya dependiste de más de la mitad del mundo." — Martin Luther King Jr.</t>
         </is>
       </c>
       <c r="S10" s="47" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="J11" s="49" t="inlineStr">
         <is>
-          <t>"La salud es la relación entre tu y tu cuerpo." — Terri Guillemets</t>
+          <t>"Más vale prevenir que curar." — Refrán castellano</t>
         </is>
       </c>
       <c r="K11" s="49" t="inlineStr">
@@ -2890,7 +2890,7 @@
       </c>
       <c r="R11" s="49" t="inlineStr">
         <is>
-          <t>"La salud no se valora hasta que llega la enfermedad." — Thomas Fuller</t>
+          <t>"Hay que pedir una mente sana en un cuerpo sano." — Juvenal</t>
         </is>
       </c>
       <c r="S11" s="49" t="inlineStr">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="J12" s="51" t="inlineStr">
         <is>
-          <t>"Usted necesita estar en una iglesia donde se predique la palabra madura de Dios. Debemos dejar el kinder si queremos crecer." — Steven Lawson</t>
+          <t>"Estás llamado a pertenecer, no solo a creer." — Rick Warren</t>
         </is>
       </c>
       <c r="K12" s="51" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="N12" s="51" t="inlineStr">
         <is>
-          <t>"No te impacientes con los demás. Recuerda que Dios trato contigo con paciencia y benignidad." — Oswald Chambers</t>
+          <t>"Cien pianos afinados con el mismo diapasón quedan automáticamente afinados entre sí." — A. W. Tozer</t>
         </is>
       </c>
       <c r="O12" s="51" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="R12" s="51" t="inlineStr">
         <is>
-          <t>"Si ves a los demás cristianos como tu enemigo, estas peleando la batalla equivocada." — Miguel Núñez</t>
+          <t>"Quien ama su sueño de comunidad más que a la comunidad cristiana misma se convierte en destructor de esta." — Dietrich Bonhoeffer</t>
         </is>
       </c>
       <c r="S12" s="51" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="J13" s="53" t="inlineStr">
         <is>
-          <t>"Los líderes que no escuchan eventualmente estarán rodeados por personas que no tienen nada que decir." — Andy Stanley</t>
+          <t>"Los líderes que no escuchan terminarán rodeados de personas que no tienen nada que decir." — atribuida a Andy Stanley</t>
         </is>
       </c>
       <c r="K13" s="53" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="N13" s="53" t="inlineStr">
         <is>
-          <t>"El liderazgo no se trata de control, se trata de servicio." — Myron Rush</t>
+          <t>"La confianza es la forma más elevada de motivación humana." — Stephen R. Covey</t>
         </is>
       </c>
       <c r="O13" s="53" t="inlineStr">
@@ -3299,7 +3299,7 @@
       </c>
       <c r="R13" s="53" t="inlineStr">
         <is>
-          <t>"El management es hacer las cosas correctamente. El liderazgo es hacer las cosas correctas." — Peter Drucker</t>
+          <t>"El tiempo es el recurso más escaso, y si no se lo administra, ninguna otra cosa podrá administrarse." — Peter Drucker</t>
         </is>
       </c>
       <c r="S13" s="53" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="J14" s="35" t="inlineStr">
         <is>
-          <t>"Gobernar una familia es poco menos difícil que gobernar un reino." — Michel de Montaigne</t>
+          <t>"No fue hecha de su cabeza para gobernarlo, ni de sus pies para ser pisoteada, sino de su costado: para ser igual, protegida y amada." — Matthew Henry</t>
         </is>
       </c>
       <c r="K14" s="35" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="N14" s="35" t="inlineStr">
         <is>
-          <t>"La fuerza de una familia, como la fuerza de un ejército, se funda en su mutua lealtad." — Mario Puzo</t>
+          <t>"Aunque sea necesario que des tu vida por ella, no lo rehúses: no haces nada que iguale lo que hizo Cristo." — Juan Crisóstomo</t>
         </is>
       </c>
       <c r="O14" s="35" t="inlineStr">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="R14" s="35" t="inlineStr">
         <is>
-          <t>"La familia no es algo importante. Lo es todo." — Michael J. Fox</t>
+          <t>"Ser amado pero no conocido es reconfortante pero superficial. Ser conocido y no amado es nuestro mayor temor." — Timothy Keller</t>
         </is>
       </c>
       <c r="S14" s="35" t="inlineStr">
@@ -3671,7 +3671,7 @@
       </c>
       <c r="J15" s="40" t="inlineStr">
         <is>
-          <t>"Un presupuesto es más que una serie de números en una página; es un reflejo de nuestros valores." — Barack Obama</t>
+          <t>"Un presupuesto es más que simples números en una página; es una medida de cuán bien cumplimos nuestras obligaciones con nosotros mismos y con los demás." — Barack Obama</t>
         </is>
       </c>
       <c r="K15" s="40" t="inlineStr">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="N15" s="40" t="inlineStr">
         <is>
-          <t>"Un presupuesto es decirle a tu dinero adonde ir, en vez de preguntarte adonde se fue." — Dave Ramsey</t>
+          <t>"Un presupuesto es decirle a tu dinero adónde ir, en vez de preguntarte adónde se fue." — Dave Ramsey</t>
         </is>
       </c>
       <c r="O15" s="40" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="R15" s="40" t="inlineStr">
         <is>
-          <t>"Gasta siempre una moneda menos de lo que ganes." — Cesare Cantú</t>
+          <t>"Ingresos anuales, veinte libras; gastos anuales, diecinueve libras, diecinueve chelines y seis peniques: resultado, felicidad. Ingresos, veinte libras; gastos, veinte libras y seis peniques: resultado, miseria." — Charles Dickens</t>
         </is>
       </c>
       <c r="S15" s="40" t="inlineStr">
@@ -3872,7 +3872,7 @@
       </c>
       <c r="J16" s="43" t="inlineStr">
         <is>
-          <t>"La vida es crecimiento. Si dejamos de crecer, estamos muertos técnica y espiritualmente." — Morihei Ueshiba</t>
+          <t>"Haber encontrado a Dios y seguir buscándolo es la paradoja del amor del alma." — A. W. Tozer</t>
         </is>
       </c>
       <c r="K16" s="43" t="inlineStr">
@@ -3892,7 +3892,7 @@
       </c>
       <c r="N16" s="43" t="inlineStr">
         <is>
-          <t>"El hombre que mueve una montaña comienza cargando pequeñas piedras." — Confucio</t>
+          <t>"La superficialidad es la maldición de nuestra época." — Richard J. Foster</t>
         </is>
       </c>
       <c r="O16" s="43" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="R16" s="43" t="inlineStr">
         <is>
-          <t>"La pequeña semilla sabia que para crecer, necesitaba ser cubierta de tierra, enterrada en la oscuridad, y luchar para alcanzar la luz." — Sandra Kring</t>
+          <t>"Cuando se te retire el consuelo, no desesperes; esperá con humildad y paciencia, porque Dios puede devolverte un consuelo mayor." — Tomás de Kempis</t>
         </is>
       </c>
       <c r="S16" s="43" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="J17" s="47" t="inlineStr">
         <is>
-          <t>"Un hombre trabajador es un hombre feliz. Un hombre con trabajo es un hombre con dignidad." — Maya Angelou</t>
+          <t>"Ningún pueblo puede prosperar hasta que aprenda que hay tanta dignidad en labrar un campo como en escribir un poema." — Booker T. Washington</t>
         </is>
       </c>
       <c r="K17" s="47" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="N17" s="47" t="inlineStr">
         <is>
-          <t>"Los planes son solamente buenas intenciones a menos que degeneren inmediatamente en trabajo duro." — Peter Drucker</t>
+          <t>"La prueba final de la sinceridad y seriedad de una gerencia es su énfasis inflexible en la integridad de carácter." — Peter Drucker</t>
         </is>
       </c>
       <c r="O17" s="47" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="R17" s="47" t="inlineStr">
         <is>
-          <t>"Las grandes cosas se hacen por una serie de pequeñas cosas reunidas." — Vincent van Gogh</t>
+          <t>"Las grandes cosas no se hacen por impulso, sino por una serie de pequeñas cosas reunidas." — Vincent van Gogh</t>
         </is>
       </c>
       <c r="S17" s="47" t="inlineStr">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="J18" s="49" t="inlineStr">
         <is>
-          <t>"Caminar es el mejor ejercicio posible. Habituate a caminar muy lejos." — Thomas Jefferson</t>
+          <t>"Caminar es el mejor ejercicio posible. Habitúate a caminar muy lejos." — Thomas Jefferson</t>
         </is>
       </c>
       <c r="K18" s="49" t="inlineStr">
@@ -4306,7 +4306,7 @@
       </c>
       <c r="N18" s="49" t="inlineStr">
         <is>
-          <t>"El ejercicio es clave para la salud física y de la mente." — Nelson Mandela</t>
+          <t>"Siempre he creído que el ejercicio es la clave no solo de la salud física, sino también de la paz mental." — Nelson Mandela</t>
         </is>
       </c>
       <c r="O18" s="49" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="R18" s="49" t="inlineStr">
         <is>
-          <t>"El secreto para tener buena salud es que el cuerpo se agite y que la mente repose." — Vincent Voiture</t>
+          <t>"Hay ejercicios fáciles y breves que fatigan pronto el cuerpo y ahorran tiempo: correr, mover las manos con algún peso, saltar." — Séneca</t>
         </is>
       </c>
       <c r="S18" s="49" t="inlineStr">
@@ -4493,7 +4493,7 @@
       </c>
       <c r="J19" s="51" t="inlineStr">
         <is>
-          <t>"La razón por la que estas aquí en la tierra es que no puedes evangelizar a nadie en el cielo." — John MacArthur</t>
+          <t>"No sé cuál será su destino, pero sé una cosa: los únicos que serán realmente felices son los que hayan buscado y encontrado cómo servir." — Albert Schweitzer</t>
         </is>
       </c>
       <c r="K19" s="51" t="inlineStr">
@@ -4513,7 +4513,7 @@
       </c>
       <c r="N19" s="51" t="inlineStr">
         <is>
-          <t>"Que el sermón principal de tu vida lo predique tu conducta." — Charles Spurgeon</t>
+          <t>"No debemos cansarnos de hacer pequeñas cosas por amor a Dios, que no mira la grandeza de la obra, sino el amor con que se hace." — Hermano Lorenzo de la Resurrección</t>
         </is>
       </c>
       <c r="O19" s="51" t="inlineStr">
@@ -4533,7 +4533,7 @@
       </c>
       <c r="R19" s="51" t="inlineStr">
         <is>
-          <t>"Creer en el evangelio no solo es el camino para conocer a Dios, sino también el camino para crecer en el." — Tim Keller</t>
+          <t>"El lugar al que Dios te llama es aquel donde tu alegría profunda y el hambre profunda del mundo se encuentran." — Frederick Buechner</t>
         </is>
       </c>
       <c r="S19" s="51" t="inlineStr">
@@ -4694,7 +4694,7 @@
       </c>
       <c r="J20" s="53" t="inlineStr">
         <is>
-          <t>"Los líderes que ofrecen sangre, sudor y lágrimas siempre obtienen más de sus seguidores que aquellos que ofrecen seguridad y diversión." — George Orwell</t>
+          <t>"No es el crítico quien cuenta. El mérito pertenece al que está realmente en la arena, con el rostro manchado de polvo, sudor y sangre." — Theodore Roosevelt</t>
         </is>
       </c>
       <c r="K20" s="53" t="inlineStr">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="N20" s="53" t="inlineStr">
         <is>
-          <t>"Si tus acciones inspiran a otros a sonar más, aprender más, hacer más y convertirse en algo más, entonces eres un líder." — John Quincy Adams</t>
+          <t>"Aprendemos sabiduría del fracaso mucho más que del éxito. A menudo descubrimos lo que sirve averiguando lo que no sirve." — Samuel Smiles</t>
         </is>
       </c>
       <c r="O20" s="53" t="inlineStr">
@@ -4734,7 +4734,7 @@
       </c>
       <c r="R20" s="53" t="inlineStr">
         <is>
-          <t>"El trabajo del líder es llevar a la gente de donde esta a donde no ha estado." — Henry Kissinger</t>
+          <t>"El tiempo de descanso no es tiempo perdido. Es economía juntar nuevas fuerzas." — Charles Spurgeon</t>
         </is>
       </c>
       <c r="S20" s="53" t="inlineStr">
@@ -4896,7 +4896,7 @@
       </c>
       <c r="J21" s="35" t="inlineStr">
         <is>
-          <t>"No le eviteis a vuestros hijos las dificultades de la vida; enseñadles más bien a superarlas." — Louis Pasteur</t>
+          <t>"El amor comienza en casa; y no importa cuánto hacemos, sino cuánto amor ponemos en lo que hacemos." — Teresa de Calcuta</t>
         </is>
       </c>
       <c r="K21" s="35" t="inlineStr">
@@ -4916,7 +4916,7 @@
       </c>
       <c r="N21" s="35" t="inlineStr">
         <is>
-          <t>"Un niño sobre los hombros de su padre: ninguna pirámide o columna de la antigüedad es más alta." — Fabrizio Caramagna</t>
+          <t>"Dios ha dado al estado de padre y madre una distinción especial por encima de todos los demás estados; manda no solo amarlos, sino honrarlos." — Martín Lutero</t>
         </is>
       </c>
       <c r="O21" s="35" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="R21" s="35" t="inlineStr">
         <is>
-          <t>"Cuando yo tenía catorce años, mi padre era tan ignorante que no podía soportarlo. Pero cuando cumplí veintiuno, me sorprendió lo mucho que había aprendido en siete años." — Mark Twain</t>
+          <t>"No es poca la diferencia entre adquirir desde jóvenes unos hábitos u otros; es muy grande, o mejor dicho, total." — Aristóteles</t>
         </is>
       </c>
       <c r="S21" s="35" t="inlineStr">
@@ -5101,7 +5101,7 @@
       </c>
       <c r="J22" s="40" t="inlineStr">
         <is>
-          <t>"El camino hacia la riqueza depende fundamentalmente de dos palabras: trabajo y ahorro." — Benjamin Franklin</t>
+          <t>"El camino hacia la riqueza depende principalmente de dos palabras: laboriosidad y frugalidad." — Benjamin Franklin</t>
         </is>
       </c>
       <c r="K22" s="40" t="inlineStr">
@@ -5121,7 +5121,7 @@
       </c>
       <c r="N22" s="40" t="inlineStr">
         <is>
-          <t>"El hombre que sabe gastar y ahorrar es el más feliz, porque disfruta de ambas cosas." — Samuel Johnson</t>
+          <t>"El costo de una cosa es la cantidad de vida que hay que entregar a cambio de ella, de inmediato o a la larga." — Henry David Thoreau</t>
         </is>
       </c>
       <c r="O22" s="40" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="R22" s="40" t="inlineStr">
         <is>
-          <t>"La manera más segura de doblar tu dinero es unir los dos extremos del billete y guardarlo en tu bolsillo." — Kin Hubbard</t>
+          <t>"La manera más segura de duplicar tu dinero es doblarlo una vez y guardarlo en el bolsillo." — atribuida a Kin Hubbard</t>
         </is>
       </c>
       <c r="S22" s="40" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="J23" s="43" t="inlineStr">
         <is>
-          <t>"Ejercita tus talentos al máximo. Al utilizarlos, desarrollas tu capacidad para enfrentarte a responsabilidades mayores." — Og Mandino</t>
+          <t>"Tené siempre presente que tu propia decisión de salir adelante es más importante que cualquier otra cosa." — Abraham Lincoln</t>
         </is>
       </c>
       <c r="K23" s="43" t="inlineStr">
@@ -5327,7 +5327,7 @@
       </c>
       <c r="N23" s="43" t="inlineStr">
         <is>
-          <t>"El crecimiento y desarrollo de las personas es el llamado más alto de liderazgo." — Harvey S. Firestone</t>
+          <t>"Si te toca ser barrendero, barré las calles como Miguel Ángel pintaba." — Martin Luther King Jr.</t>
         </is>
       </c>
       <c r="O23" s="43" t="inlineStr">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="R23" s="43" t="inlineStr">
         <is>
-          <t>"El crecimiento nunca es por mera casualidad; es el resultado de fuerzas que trabajan juntas." — James Cash Penney</t>
+          <t>"Si he visto más lejos, es porque estoy sobre los hombros de gigantes." — Isaac Newton</t>
         </is>
       </c>
       <c r="S23" s="43" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="J24" s="47" t="inlineStr">
         <is>
-          <t>"Escoge un trabajo que ames y no tendrás que trabajar ni un día de tu vida." — Confucio</t>
+          <t>"Un viaje de mil li comienza con un paso." — Lao-Tsé</t>
         </is>
       </c>
       <c r="K24" s="47" t="inlineStr">
@@ -5527,7 +5527,7 @@
       </c>
       <c r="N24" s="47" t="inlineStr">
         <is>
-          <t>"El fracaso es solo la oportunidad de empezar de nuevo, esta vez de forma más inteligente." — Henry Ford</t>
+          <t>"Hombre apercebido, medio combatido." — Miguel de Cervantes</t>
         </is>
       </c>
       <c r="O24" s="47" t="inlineStr">
@@ -5547,7 +5547,7 @@
       </c>
       <c r="R24" s="47" t="inlineStr">
         <is>
-          <t>"El éxito es la suma de pequeños esfuerzos, repetidos día tras día." — Robert Collier</t>
+          <t>"El éxito es la suma de pequeños esfuerzos, repetidos día tras día." — atribuida a Robert Collier</t>
         </is>
       </c>
       <c r="S24" s="47" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="J25" s="49" t="inlineStr">
         <is>
-          <t>"Que tu alimento sea tu medicina, y tu medicina tu alimento." — Hipócrates</t>
+          <t>"Dime lo que comes y te diré quién eres." — Jean Anthelme Brillat-Savarin</t>
         </is>
       </c>
       <c r="K25" s="49" t="inlineStr">
@@ -5733,7 +5733,7 @@
       </c>
       <c r="N25" s="49" t="inlineStr">
         <is>
-          <t>"Hoy en día, más del 95% de las enfermedades crónicas son causadas por como elegimos alimentarnos, por ingredientes tóxicos, deficiencias nutricionales y falta de actividad física." — Mike Adams</t>
+          <t>"Come poco y cena más poco, que la salud de todo el cuerpo se fragua en la oficina del estómago." — Miguel de Cervantes</t>
         </is>
       </c>
       <c r="O25" s="49" t="inlineStr">
@@ -5753,7 +5753,7 @@
       </c>
       <c r="R25" s="49" t="inlineStr">
         <is>
-          <t>"La felicidad radica, ante todo, en la salud." — George William Curtis</t>
+          <t>"Comé comida. No demasiada. Sobre todo plantas." — Michael Pollan</t>
         </is>
       </c>
       <c r="S25" s="49" t="inlineStr">
@@ -5923,7 +5923,7 @@
       </c>
       <c r="J26" s="51" t="inlineStr">
         <is>
-          <t>"Ser cristiano significa perdonar lo inexcusable en otros, porque Dios perdono lo inexcusable en ti." — C.S. Lewis</t>
+          <t>"La Iglesia no existe para ninguna otra cosa que para atraer a los hombres hacia Cristo, para hacerlos pequeños Cristos." — C. S. Lewis</t>
         </is>
       </c>
       <c r="K26" s="51" t="inlineStr">
@@ -5943,7 +5943,7 @@
       </c>
       <c r="N26" s="51" t="inlineStr">
         <is>
-          <t>"Que el sermón principal de tu vida lo predique tu conducta." — Charles Spurgeon</t>
+          <t>"Todos los hermanos prediquen con las obras." — Francisco de Asís</t>
         </is>
       </c>
       <c r="O26" s="51" t="inlineStr">
@@ -5963,7 +5963,7 @@
       </c>
       <c r="R26" s="51" t="inlineStr">
         <is>
-          <t>"Si el amor de Dios por sus hijos se midiera por nuestra salud, riqueza y comodidad en esta vida, Dios odiaba al apóstol Pablo." — John Piper</t>
+          <t>"No es ningún tonto el que da lo que no puede retener para ganar lo que no puede perder." — Jim Elliot</t>
         </is>
       </c>
       <c r="S26" s="51" t="inlineStr">
@@ -6125,7 +6125,7 @@
       </c>
       <c r="J27" s="53" t="inlineStr">
         <is>
-          <t>"Un buen objetivo del liderazgo es ayudar a aquellos que están haciendo mal las cosas para que les vaya bien, y ayudar a aquellos que lo están haciendo bien, a hacerlo aun mejor." — Jim Rohn</t>
+          <t>"El líder servidor es primero servidor. Comienza con el sentimiento natural de querer servir." — Robert K. Greenleaf</t>
         </is>
       </c>
       <c r="K27" s="53" t="inlineStr">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="N27" s="53" t="inlineStr">
         <is>
-          <t>"La autoridad no te convierte en líder. La empatía si." — Angela Ahrendts</t>
+          <t>"Ser digno de confianza es un cumplido mayor que ser amado." — George MacDonald</t>
         </is>
       </c>
       <c r="O27" s="53" t="inlineStr">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="R27" s="53" t="inlineStr">
         <is>
-          <t>"No puedes dirigir a las personas si no las amas. Y no puedes liderarlas si no te respetan." — John C. Maxwell</t>
+          <t>"Ama y haz lo que quieras: si callas, calla por amor; si gritas, grita por amor; si corriges, corrige por amor." — Agustín de Hipona</t>
         </is>
       </c>
       <c r="S27" s="53" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="J28" s="35" t="inlineStr">
         <is>
-          <t>"La familia es un complemento nuestro, mayor que nosotros, anterior a nosotros, y que nos sobrevivirá con lo mejor de nosotros." — Alphonse de Lamartine</t>
+          <t>"La familia es como un segundo nosotros mismos, más grande que nosotros, anterior a nosotros, y que nos sobrevive con lo mejor de nosotros." — Alphonse de Lamartine</t>
         </is>
       </c>
       <c r="K28" s="35" t="inlineStr">
@@ -6350,7 +6350,7 @@
       </c>
       <c r="N28" s="35" t="inlineStr">
         <is>
-          <t>"De todas las maneras concebibles, la familia es un vínculo con nuestro pasado y el puente hacia nuestro futuro." — Alex Haley</t>
+          <t>"De todas las maneras concebibles, la familia es un vínculo con nuestro pasado y un puente hacia nuestro futuro." — atribuida a Alex Haley</t>
         </is>
       </c>
       <c r="O28" s="35" t="inlineStr">
@@ -6370,7 +6370,7 @@
       </c>
       <c r="R28" s="35" t="inlineStr">
         <is>
-          <t>"Una casa será fuerte e indestructible cuando este sostenida por estas cuatro columnas: padre valiente, madre prudente, hijo obediente, hermano complaciente." — Confucio</t>
+          <t>"El futuro de la humanidad se fragua en la familia." — Juan Pablo II</t>
         </is>
       </c>
       <c r="S28" s="35" t="inlineStr">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="J29" s="40" t="inlineStr">
         <is>
-          <t>"No pongas tu interés en el dinero, pero pon tu dinero a interés." — Oliver Wendell Holmes</t>
+          <t>"No pongas tu confianza en el dinero, sino tu dinero en buen resguardo." — Oliver Wendell Holmes Sr.</t>
         </is>
       </c>
       <c r="K29" s="40" t="inlineStr">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="N29" s="40" t="inlineStr">
         <is>
-          <t>"Para invertir con éxito durante toda la vida no se necesita un cociente intelectual desorbitado, una intuición empresarial insólita, ni información privilegiada." — Warren Buffett</t>
+          <t>"Para invertir con éxito a lo largo de la vida no hace falta un coeficiente intelectual estratosférico, una intuición empresarial fuera de lo común ni información privilegiada." — Warren Buffett</t>
         </is>
       </c>
       <c r="O29" s="40" t="inlineStr">
@@ -6573,7 +6573,7 @@
       </c>
       <c r="R29" s="40" t="inlineStr">
         <is>
-          <t>"No se trata de cuanto dinero ganas, sino de cuanto dinero guardas y que tan duro trabaja para ti." — Robert Kiyosaki</t>
+          <t>"Los dos guerreros más poderosos son la paciencia y el tiempo." — León Tolstói</t>
         </is>
       </c>
       <c r="S29" s="40" t="inlineStr">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="J30" s="43" t="inlineStr">
         <is>
-          <t>"Tu tiempo es limitado, no lo desperdicies viviendo la vida de alguien más." — Steve Jobs</t>
+          <t>"Si uno no sabe a qué puerto se dirige, ningún viento le es favorable." — Séneca</t>
         </is>
       </c>
       <c r="K30" s="43" t="inlineStr">
@@ -6760,7 +6760,7 @@
       </c>
       <c r="N30" s="43" t="inlineStr">
         <is>
-          <t>"La persona que llega más lejos es normalmente la que esta dispuesta a hacer y a atreverse." — Dale Carnegie</t>
+          <t>"Bien hecho es mejor que bien dicho." — Benjamin Franklin</t>
         </is>
       </c>
       <c r="O30" s="43" t="inlineStr">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="R30" s="43" t="inlineStr">
         <is>
-          <t>"Equivocarse es parte importante del aprendizaje, pues sin equivocaciones no hay crecimiento." — Jorge Bucay</t>
+          <t>"La vida solo puede comprenderse mirando hacia atrás, pero ha de vivirse mirando hacia adelante." — Søren Kierkegaard</t>
         </is>
       </c>
       <c r="S30" s="43" t="inlineStr">
@@ -6943,7 +6943,7 @@
       </c>
       <c r="J31" s="47" t="inlineStr">
         <is>
-          <t>"Todas las personas tienen la disposición de trabajar creativamente. Lo que sucede es que la mayoría jamás lo nota." — Truman Capote</t>
+          <t>"La verdad adelgaza y no quiebra, y siempre anda sobre la mentira como el aceite sobre el agua." — Miguel de Cervantes</t>
         </is>
       </c>
       <c r="K31" s="47" t="inlineStr">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="N31" s="47" t="inlineStr">
         <is>
-          <t>"El trabajo es el único medio digno de ganarse la vida." — José Martí</t>
+          <t>"Estamos atrapados en una red ineludible de reciprocidad, atados a un mismo destino. Lo que afecta a uno directamente nos afecta a todos indirectamente." — Martin Luther King Jr.</t>
         </is>
       </c>
       <c r="O31" s="47" t="inlineStr">
@@ -6983,7 +6983,7 @@
       </c>
       <c r="R31" s="47" t="inlineStr">
         <is>
-          <t>"El genio es un uno por ciento de inspiración y un noventa y nueve por ciento de transpiración." — Thomas Edison</t>
+          <t>"No es posible bañarse dos veces en el mismo río." — Heráclito</t>
         </is>
       </c>
       <c r="S31" s="47" t="inlineStr">
@@ -7147,7 +7147,7 @@
       </c>
       <c r="J32" s="49" t="inlineStr">
         <is>
-          <t>"El descanso y el sueño de calidad son pilares de la salud, tan importantes como la alimentación y el ejercicio." — Dr. Matthew Walker</t>
+          <t>"El sueño es lo más eficaz que podemos hacer cada día para restablecer la salud de nuestro cerebro y de nuestro cuerpo." — Matthew Walker</t>
         </is>
       </c>
       <c r="K32" s="49" t="inlineStr">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="N32" s="49" t="inlineStr">
         <is>
-          <t>"Los mejores médicos del mundo son: el doctor dieta, el doctor reposo y el doctor alegría." — Jonathan Swift</t>
+          <t>"Los mejores médicos del mundo son el doctor Dieta, el doctor Reposo y el doctor Alegría." — Jonathan Swift</t>
         </is>
       </c>
       <c r="O32" s="49" t="inlineStr">
@@ -7187,7 +7187,7 @@
       </c>
       <c r="R32" s="49" t="inlineStr">
         <is>
-          <t>"El secreto para tener buena salud es que el cuerpo se agite y que la mente repose." — Vincent Voiture</t>
+          <t>"Nos hiciste, Señor, para ti, y nuestro corazón está inquieto hasta que descanse en ti." — Agustín de Hipona</t>
         </is>
       </c>
       <c r="S32" s="49" t="inlineStr">
@@ -7355,7 +7355,7 @@
       </c>
       <c r="J33" s="8" t="inlineStr">
         <is>
-          <t>"La oración no es para cambiar los planes de Dios; es para confiar y descansar en Su soberana voluntad." — Martin Lutero</t>
+          <t>"La oración no es otra cosa sino tratar de amistad, estando muchas veces tratando a solas con quien sabemos nos ama." — Teresa de Ávila</t>
         </is>
       </c>
       <c r="K33" s="8" t="inlineStr">
@@ -7375,7 +7375,7 @@
       </c>
       <c r="N33" s="8" t="inlineStr">
         <is>
-          <t>"No olvides orar hoy, porque Dios no olvido despertarte esta mañana." — Oswald Chambers</t>
+          <t>"¿Te ha confiado Dios un silencio, un silencio lleno de significado? Los silencios de Dios son sus respuestas." — Oswald Chambers</t>
         </is>
       </c>
       <c r="O33" s="8" t="inlineStr">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
-          <t>"Uno de los grandes usos de Facebook y Twitter será demostrar en el último día que la falta de oración no fue por falta de tiempo." — John Piper</t>
+          <t>"Uno de los grandes usos de Twitter y Facebook será demostrar en el último día que la falta de oración no fue por falta de tiempo." — atribuida a John Piper</t>
         </is>
       </c>
       <c r="S33" s="8" t="inlineStr">
@@ -7559,7 +7559,7 @@
       </c>
       <c r="J34" s="10" t="inlineStr">
         <is>
-          <t>"El liderazgo es la capacidad de traducir la visión en realidad." — Warren Bennis</t>
+          <t>"El liderazgo es la capacidad de convertir la visión en realidad." — atribuida a Warren Bennis</t>
         </is>
       </c>
       <c r="K34" s="10" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="N34" s="10" t="inlineStr">
         <is>
-          <t>"Liderazgo es elevar la visión de una persona, llevar su rendimiento a un mayor estándar y construir una personalidad más allá de sus límites normales." — Peter Drucker</t>
+          <t>"El liderazgo es elevar la visión de una persona a metas más altas, llevar su rendimiento a un nivel superior y formar su carácter más allá de sus límites habituales." — Peter Drucker</t>
         </is>
       </c>
       <c r="O34" s="10" t="inlineStr">
@@ -7599,7 +7599,7 @@
       </c>
       <c r="R34" s="10" t="inlineStr">
         <is>
-          <t>"Un buen líder lleva a la gente donde quiere ir. Un gran líder lleva a la gente donde debe estar." — Rosalynn Carter</t>
+          <t>"Un líder lleva a la gente adonde quiere ir. Un gran líder la lleva adonde no necesariamente quiere ir, pero adonde debe estar." — atribuida a Rosalynn Carter</t>
         </is>
       </c>
       <c r="S34" s="10" t="inlineStr">
@@ -7761,7 +7761,7 @@
       </c>
       <c r="J35" s="12" t="inlineStr">
         <is>
-          <t>"Las familias felices se parecen todas; las familias infelices son infelices cada una a su manera." — León Tolstoi</t>
+          <t>"El primer servicio que debemos al prójimo es escucharle." — Dietrich Bonhoeffer</t>
         </is>
       </c>
       <c r="K35" s="12" t="inlineStr">
@@ -7781,7 +7781,7 @@
       </c>
       <c r="N35" s="12" t="inlineStr">
         <is>
-          <t>"Jamás en la vida encontraréis ternura mejor, más profunda, ni más desinteresada que la de vuestra madre." — Honoré de Balzac</t>
+          <t>"El amigo que puede quedarse en silencio con nosotros en un momento de desesperación o confusión es un amigo que se interesa de verdad." — Henri Nouwen</t>
         </is>
       </c>
       <c r="O35" s="12" t="inlineStr">
@@ -7801,7 +7801,7 @@
       </c>
       <c r="R35" s="12" t="inlineStr">
         <is>
-          <t>"Mi familia era espiritualmente rica. Mi madre me enseñó a mantener los pies en el suelo." — Denzel Washington</t>
+          <t>"El perdón es un acto de la voluntad, y la voluntad puede actuar sin importar la temperatura del corazón." — Corrie ten Boom</t>
         </is>
       </c>
       <c r="S35" s="12" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>"La clave no es priorizar lo que esta en tu agenda, sino agendar tus prioridades." — Stephen Covey</t>
+          <t>"Amar no es mirarse el uno al otro; es mirar juntos en la misma dirección." — Antoine de Saint-Exupéry</t>
         </is>
       </c>
       <c r="K36" s="14" t="inlineStr">
@@ -8004,7 +8004,7 @@
       </c>
       <c r="R36" s="14" t="inlineStr">
         <is>
-          <t>"No ahorres lo que queda después de gastar; gasta lo que queda después de ahorrar." — Warren Buffett</t>
+          <t>"No hay otra riqueza que la vida: la vida con todos sus poderes de amor, de alegría y de admiración." — John Ruskin</t>
         </is>
       </c>
       <c r="S36" s="14" t="inlineStr">
@@ -8166,7 +8166,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>"Sé celoso de tu tiempo, porque es tu mayor tesoro." — Og Mandino</t>
+          <t>"Una larga obediencia en la misma dirección." — Eugene H. Peterson</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -8186,7 +8186,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>"Por que resistir el cambio cuando es la fuente principal de tu crecimiento?" — Robin Sharma</t>
+          <t>"Una golondrina no hace verano, ni tampoco un solo día; así tampoco un solo día ni un breve tiempo hacen a alguien dichoso." — Aristóteles</t>
         </is>
       </c>
       <c r="O37" s="2" t="inlineStr">
@@ -8206,7 +8206,7 @@
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>"El crecimiento nunca es por mera casualidad; es el resultado de fuerzas que trabajan juntas." — James Cash Penney</t>
+          <t>"Si cada año desarraigáramos un vicio, pronto seríamos perfectos." — Tomás de Kempis</t>
         </is>
       </c>
       <c r="S37" s="2" t="inlineStr">
@@ -8367,7 +8367,7 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>"Nuestra recompensa se encuentra en el esfuerzo y no en el resultado. Un esfuerzo total es una victoria completa." — Mahatma Gandhi</t>
+          <t>"Ningún hombre es una isla, completo en sí mismo; cada hombre es un pedazo del continente, una parte del todo." — John Donne</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
@@ -8387,7 +8387,7 @@
       </c>
       <c r="N38" s="4" t="inlineStr">
         <is>
-          <t>"Un jardinero que cultiva su propio jardín, con sus propias manos, une en su persona los tres personajes: propietario, agricultor y obrero." — Adam Smith</t>
+          <t>"Uno para todos y todos para uno." — Alexandre Dumas</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
@@ -8407,7 +8407,7 @@
       </c>
       <c r="R38" s="4" t="inlineStr">
         <is>
-          <t>"Un hombre trabajador es un hombre feliz. Un hombre con trabajo es un hombre con dignidad." — Maya Angelou</t>
+          <t>"Si decís la verdad, no tenés que acordarte de nada." — Mark Twain</t>
         </is>
       </c>
       <c r="S38" s="4" t="inlineStr">
@@ -8571,7 +8571,7 @@
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>"Mantener el cuerpo en buena salud es un deber, de lo contrario no seremos capaces de mantener nuestra mente fuerte y clara." — Buda</t>
+          <t>"Muchas de las cosas que necesitamos pueden esperar. El niño no puede. Su nombre es Hoy." — Gabriela Mistral</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -8591,7 +8591,7 @@
       </c>
       <c r="N39" s="6" t="inlineStr">
         <is>
-          <t>"Tu cuerpo es templo de la naturaleza y del espíritu divino. Consérvalo sano, respétalo." — Henri Frederic Amiel</t>
+          <t>"No es un cuerpo sano el que hace buena al alma, sino un alma buena la que, con su virtud, deja al cuerpo lo mejor posible." — Platón</t>
         </is>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -8611,7 +8611,7 @@
       </c>
       <c r="R39" s="6" t="inlineStr">
         <is>
-          <t>"Cuida tu cuerpo. Es el único lugar que tienes para vivir." — Jim Rohn</t>
+          <t>"Cuidá tu cuerpo. Es el único lugar que tenés para vivir." — atribuida a Jim Rohn</t>
         </is>
       </c>
       <c r="S39" s="6" t="inlineStr">
@@ -8778,7 +8778,7 @@
       </c>
       <c r="J40" s="8" t="inlineStr">
         <is>
-          <t>"Creo en el cristianismo así como creo que el sol ha salido: no solo porque lo veo, sino porque gracias a el veo todo lo demás." — C.S. Lewis</t>
+          <t>"No hay gente corriente. Nunca has hablado con un simple mortal." — C. S. Lewis</t>
         </is>
       </c>
       <c r="K40" s="8" t="inlineStr">
@@ -8798,7 +8798,7 @@
       </c>
       <c r="N40" s="8" t="inlineStr">
         <is>
-          <t>"Si el amor de Dios por sus hijos se midiera por nuestra salud, riqueza y comodidad en esta vida, Dios odiaba al apóstol Pablo." — John Piper</t>
+          <t>"Ser el Amado expresa la verdad central de nuestra existencia." — Henri Nouwen</t>
         </is>
       </c>
       <c r="O40" s="8" t="inlineStr">
@@ -8818,7 +8818,7 @@
       </c>
       <c r="R40" s="8" t="inlineStr">
         <is>
-          <t>"Creer en el evangelio no solo es el camino para conocer a Dios, sino también el camino para crecer en el." — Tim Keller</t>
+          <t>"Lo que viene a nuestra mente cuando pensamos en Dios es lo más importante acerca de nosotros." — A. W. Tozer</t>
         </is>
       </c>
       <c r="S40" s="8" t="inlineStr">
@@ -8978,7 +8978,7 @@
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>"Ser líder es tener la valentía de asumir responsabilidad, no de buscar culpables." — Simon Sinek</t>
+          <t>"Un líder es el que conoce el camino, recorre el camino y muestra el camino." — John C. Maxwell</t>
         </is>
       </c>
       <c r="K41" s="10" t="inlineStr">
@@ -8998,7 +8998,7 @@
       </c>
       <c r="N41" s="10" t="inlineStr">
         <is>
-          <t>"La función de un líder es producir más líderes, no más seguidores." — Ralph Nader</t>
+          <t>"La función del liderazgo es producir más líderes, no más seguidores." — Ralph Nader</t>
         </is>
       </c>
       <c r="O41" s="10" t="inlineStr">
@@ -9018,7 +9018,7 @@
       </c>
       <c r="R41" s="10" t="inlineStr">
         <is>
-          <t>"Un líder es mejor cuando la gente apenas sabe que existe; cuando su trabajo esta hecho y su meta cumplida, dirán: lo hicimos nosotros." — Lao Tzu</t>
+          <t>"Todos pueden ser grandes, porque todos pueden servir." — Martin Luther King Jr.</t>
         </is>
       </c>
       <c r="S41" s="10" t="inlineStr">
@@ -9188,7 +9188,7 @@
       </c>
       <c r="J42" s="12" t="inlineStr">
         <is>
-          <t>"Una casa será fuerte e indestructible cuando este sostenida por estas cuatro columnas: padre valiente, madre prudente, hijo obediente, hermano complaciente." — Confucio</t>
+          <t>"Entended que si es en la cocina, entre los pucheros anda el Señor." — Teresa de Ávila</t>
         </is>
       </c>
       <c r="K42" s="12" t="inlineStr">
@@ -9208,7 +9208,7 @@
       </c>
       <c r="N42" s="12" t="inlineStr">
         <is>
-          <t>"La fuerza de una familia, como la fuerza de un ejército, se funda en su mutua lealtad." — Mario Puzo</t>
+          <t>"Cuando un padre lava pañales o hace otra tarea humilde por su hijo, y alguien se burla, Dios, con todos sus ángeles y criaturas, sonríe." — Martín Lutero</t>
         </is>
       </c>
       <c r="O42" s="12" t="inlineStr">
@@ -9228,7 +9228,7 @@
       </c>
       <c r="R42" s="12" t="inlineStr">
         <is>
-          <t>"Gobernar una familia es poco menos difícil que gobernar un reino." — Michel de Montaigne</t>
+          <t>"En lo esencial, unidad; en lo dudoso, libertad; en todo, caridad." — Marco Antonio de Dominis</t>
         </is>
       </c>
       <c r="S42" s="12" t="inlineStr">
@@ -9395,7 +9395,7 @@
       </c>
       <c r="J43" s="14" t="inlineStr">
         <is>
-          <t>"El ahorro es una cosa muy hermosa, especialmente cuando tus padres lo han hecho por ti." — Winston Churchill</t>
+          <t>"No creo que se pueda fijar cuánto debemos dar. Me temo que la única regla segura es dar más de lo que nos sobra." — C. S. Lewis</t>
         </is>
       </c>
       <c r="K43" s="14" t="inlineStr">
@@ -9415,7 +9415,7 @@
       </c>
       <c r="N43" s="14" t="inlineStr">
         <is>
-          <t>"Compra solamente lo necesario; lo superfluo, aunque cueste solo un céntimo, es caro." — Lucio Anneo Séneca</t>
+          <t>"¡Nadie se ha empobrecido jamás por dar!" — Ana Frank</t>
         </is>
       </c>
       <c r="O43" s="14" t="inlineStr">
@@ -9435,7 +9435,7 @@
       </c>
       <c r="R43" s="14" t="inlineStr">
         <is>
-          <t>"El ahorro es un ingrediente esencial del éxito." — John D. Rockefeller</t>
+          <t>"Gana todo lo que puedas, ahorra todo lo que puedas, da todo lo que puedas." — John Wesley</t>
         </is>
       </c>
       <c r="S43" s="14" t="inlineStr">
@@ -9599,7 +9599,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>"La mayor gloria no es no caer nunca, sino levantarnos cada vez que caemos." — Nelson Mandela</t>
+          <t>"El mayor legado que podemos dejar a hijos y nietos no es el dinero, sino el legado de nuestro carácter y nuestra fe." — Billy Graham</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -9619,7 +9619,7 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>"Para aumentar nuestro grado de autoestima, primero debemos aprender a vivir conscientemente, porque este es el fundamento de todo." — Nathaniel Branden</t>
+          <t>"El débil nunca puede perdonar. El perdón es atributo de los fuertes." — Mahatma Gandhi</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
@@ -9639,7 +9639,7 @@
       </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>"La vida no siempre te da lo que quieres, pero si miras de cerca verás que te da lo que necesitas para tu crecimiento." — León Brown</t>
+          <t>"La verdad sin amor es demasiado dura; el amor sin verdad es demasiado blando." — John Stott</t>
         </is>
       </c>
       <c r="S44" s="2" t="inlineStr">
@@ -9806,7 +9806,7 @@
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>"Escoge un trabajo que ames y no tendrás que trabajar ni un día de tu vida." — Confucio</t>
+          <t>"El tiempo del trabajo no es, para mí, distinto del tiempo de la oración." — Hermano Lorenzo de la Resurrección</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
@@ -9826,7 +9826,7 @@
       </c>
       <c r="N45" s="4" t="inlineStr">
         <is>
-          <t>"El secreto de mi felicidad esta en no esforzarse por el placer, sino en encontrar el placer en el esfuerzo." — Andre Gide</t>
+          <t>"El trabajo no es, ante todo, algo que uno hace para vivir, sino aquello para lo que uno vive." — Dorothy L. Sayers</t>
         </is>
       </c>
       <c r="O45" s="4" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="R45" s="4" t="inlineStr">
         <is>
-          <t>"Las grandes cosas se hacen por una serie de pequeñas cosas reunidas." — Vincent van Gogh</t>
+          <t>"Quien barre un cuarto como para Dios hace hermoso el cuarto y la tarea." — George Herbert</t>
         </is>
       </c>
       <c r="S45" s="4" t="inlineStr">
@@ -10026,7 +10026,7 @@
       </c>
       <c r="N46" s="6" t="inlineStr">
         <is>
-          <t>"Solo la alegría es garantía de salud y longevidad." — Santiago Ramón y Cajal</t>
+          <t>"Si te aflige algo externo, no es eso lo que te perturba, sino tu juicio sobre ello." — Marco Aurelio</t>
         </is>
       </c>
       <c r="O46" s="6" t="inlineStr">
@@ -10046,7 +10046,7 @@
       </c>
       <c r="R46" s="6" t="inlineStr">
         <is>
-          <t>"La buena salud no es algo que podamos comprar. Sin embargo, puede ser una cuenta de ahorros extremadamente valiosa." — Anne Wilson Schaef</t>
+          <t>"Parte de la curación es querer ser curado." — Séneca</t>
         </is>
       </c>
       <c r="S46" s="6" t="inlineStr">
@@ -10211,7 +10211,7 @@
       </c>
       <c r="J47" s="8" t="inlineStr">
         <is>
-          <t>"Si no permanecemos en la oración, vamos a permanecer en la tentación." — John Owen</t>
+          <t>"Si no permanecemos en la oración, permaneceremos en la tentación." — John Owen</t>
         </is>
       </c>
       <c r="K47" s="8" t="inlineStr">
@@ -10231,7 +10231,7 @@
       </c>
       <c r="N47" s="8" t="inlineStr">
         <is>
-          <t>"No te impacientes con los demás. Recuerda que Dios trato contigo con paciencia y benignidad." — Oswald Chambers</t>
+          <t>"Solo quien da gracias por las cosas pequeñas recibe también las grandes." — Dietrich Bonhoeffer</t>
         </is>
       </c>
       <c r="O47" s="8" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="R47" s="8" t="inlineStr">
         <is>
-          <t>"Uno de los grandes usos de Facebook y Twitter será demostrar en el último día que la falta de oración no fue por falta de tiempo." — John Piper</t>
+          <t>"Adorar es avivar la conciencia con la santidad de Dios, alimentar la mente con su verdad, purificar la imaginación con su belleza y abrir el corazón a su amor." — William Temple</t>
         </is>
       </c>
       <c r="S47" s="8" t="inlineStr">
@@ -10420,7 +10420,7 @@
       </c>
       <c r="J48" s="10" t="inlineStr">
         <is>
-          <t>"En el siglo que viene, los líderes serán aquellos que impulsen a otros." — Bill Gates</t>
+          <t>"Los planes no valen nada, pero planificar lo es todo." — Dwight D. Eisenhower</t>
         </is>
       </c>
       <c r="K48" s="10" t="inlineStr">
@@ -10440,7 +10440,7 @@
       </c>
       <c r="N48" s="10" t="inlineStr">
         <is>
-          <t>"El liderazgo es el arte de conseguir que otra persona haga algo que tu quieres hacer, porque ella quiere hacerlo." — Dwight D. Eisenhower</t>
+          <t>"En la tardanza dicen que suele estar el peligro." — Miguel de Cervantes</t>
         </is>
       </c>
       <c r="O48" s="10" t="inlineStr">
@@ -10460,7 +10460,7 @@
       </c>
       <c r="R48" s="10" t="inlineStr">
         <is>
-          <t>"Las personas no deben sentirse obligadas. Deben ser capaces de elegir a su propio líder." — Albert Einstein</t>
+          <t>"Cada uno de nosotros es responsable ante todos, por todos y por todo." — Fiódor Dostoievski</t>
         </is>
       </c>
       <c r="S48" s="10" t="inlineStr">
@@ -10628,7 +10628,7 @@
       </c>
       <c r="J49" s="12" t="inlineStr">
         <is>
-          <t>"Mi familia era espiritualmente rica. Mi madre me enseñó a mantener los pies en el suelo." — Denzel Washington</t>
+          <t>"Vi más claramente que nunca que el primer gran asunto al que debo atender cada día es tener mi alma feliz en el Señor." — George Müller</t>
         </is>
       </c>
       <c r="K49" s="12" t="inlineStr">
@@ -10648,7 +10648,7 @@
       </c>
       <c r="N49" s="12" t="inlineStr">
         <is>
-          <t>"Cuando yo tenía catorce años, mi padre era tan ignorante que no podía soportarlo. Pero cuando cumplí veintiuno, me sorprendió lo mucho que había aprendido en siete años." — Mark Twain</t>
+          <t>"Querer poner la religión en la mente y el corazón por la fuerza y las amenazas no es poner la religión, sino el terror." — Blaise Pascal</t>
         </is>
       </c>
       <c r="O49" s="12" t="inlineStr">
@@ -10668,7 +10668,7 @@
       </c>
       <c r="R49" s="12" t="inlineStr">
         <is>
-          <t>"La familia es una de las obras maestras de la naturaleza." — George Santayana</t>
+          <t>"Toda familia cristiana debería ser como una pequeña iglesia, consagrada a Cristo y gobernada por sus reglas." — Jonathan Edwards</t>
         </is>
       </c>
       <c r="S49" s="12" t="inlineStr">
@@ -10841,7 +10841,7 @@
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>"La deuda es como cualquier otra trampa. Fácil de entrar y difícil de salir." — Josh Billings</t>
+          <t>"Mejor acostarse sin cenar que levantarse con deudas." — Benjamin Franklin</t>
         </is>
       </c>
       <c r="K50" s="14" t="inlineStr">
@@ -10861,7 +10861,7 @@
       </c>
       <c r="N50" s="14" t="inlineStr">
         <is>
-          <t>"La inflación es la madre del paro, y la ladrona invisible de quienes han ahorrado." — Margaret Thatcher</t>
+          <t>"Preocuparse no vacía el mañana de su dolor; vacía el hoy de su fuerza." — Corrie ten Boom</t>
         </is>
       </c>
       <c r="O50" s="14" t="inlineStr">
@@ -10881,7 +10881,7 @@
       </c>
       <c r="R50" s="14" t="inlineStr">
         <is>
-          <t>"A menos que se haga un compromiso, el resto son promesas y anhelos, pero no planes." — Peter F. Drucker</t>
+          <t>"Es mejor prepararse para los días de necesidad." — Esopo</t>
         </is>
       </c>
       <c r="S50" s="14" t="inlineStr">
@@ -11044,7 +11044,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>"Equivocarse es parte importante del aprendizaje, pues sin equivocaciones no hay crecimiento." — Jorge Bucay</t>
+          <t>"El fracaso es solo la oportunidad de comenzar de nuevo, esta vez con más inteligencia." — Henry Ford</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -11064,7 +11064,7 @@
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>"El éxito es la capacidad de ir de fracaso en fracaso sin perder el entusiasmo." — Winston Churchill</t>
+          <t>"Un barco en el puerto está seguro, pero no es para eso que se construyen los barcos." — John A. Shedd</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr">
@@ -11084,7 +11084,7 @@
       </c>
       <c r="R51" s="2" t="inlineStr">
         <is>
-          <t>"La pequeña semilla sabia que para crecer, necesitaba ser cubierta de tierra, enterrada en la oscuridad, y luchar para alcanzar la luz." — Sandra Kring</t>
+          <t>"Como la estrella, sin prisa, pero sin pausa, gire cada uno en torno a su propia carga." — Johann Wolfgang von Goethe</t>
         </is>
       </c>
       <c r="S51" s="2" t="inlineStr">
@@ -11257,7 +11257,7 @@
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>"El genio es un uno por ciento de inspiración y un noventa y nueve por ciento de transpiración." — Thomas Edison</t>
+          <t>"Todo buen y verdadero cristiano entienda que la verdad, dondequiera que la encuentre, pertenece a su Señor." — Agustín de Hipona</t>
         </is>
       </c>
       <c r="K52" s="4" t="inlineStr">
@@ -11277,7 +11277,7 @@
       </c>
       <c r="N52" s="4" t="inlineStr">
         <is>
-          <t>"Todas las personas tienen la disposición de trabajar creativamente. Lo que sucede es que la mayoría jamás lo nota." — Truman Capote</t>
+          <t>"La computadora es la herramienta más notable que hemos creado: es el equivalente a una bicicleta para nuestra mente." — Steve Jobs</t>
         </is>
       </c>
       <c r="O52" s="4" t="inlineStr">
@@ -11297,7 +11297,7 @@
       </c>
       <c r="R52" s="4" t="inlineStr">
         <is>
-          <t>"El éxito es el resultado de la preparación, el trabajo duro y el aprendizaje continuo." — Colin Powell</t>
+          <t>"Ser culto es el único modo de ser libre." — José Martí</t>
         </is>
       </c>
       <c r="S52" s="4" t="inlineStr">
@@ -11464,7 +11464,7 @@
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>"La parte nunca podrá estar bien, a menos que el todo también lo este." — Platón</t>
+          <t>"La salud es un estado de completo bienestar físico, mental y social, y no solamente la ausencia de afecciones o enfermedades." — Organización Mundial de la Salud</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -11484,7 +11484,7 @@
       </c>
       <c r="N53" s="6" t="inlineStr">
         <is>
-          <t>"No hay salud sin salud mental." — David Satcher</t>
+          <t>"El Dios de la Biblia es también el Dios del genoma. Se le puede adorar en la catedral o en el laboratorio." — Francis S. Collins</t>
         </is>
       </c>
       <c r="O53" s="6" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="R53" s="6" t="inlineStr">
         <is>
-          <t>"Tu cuerpo es templo de la naturaleza y del espíritu divino. Consérvalo sano, respétalo." — Henri Frederic Amiel</t>
+          <t>"Yo lo vendé, y Dios lo sanó." — Ambroise Paré</t>
         </is>
       </c>
       <c r="S53" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: pasada de estilo, 266 arranques repetidos variados en prácticas, problemáticas y acciones del sábado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -19514,7 +19514,7 @@
       </c>
       <c r="N4" s="61" t="inlineStr">
         <is>
-          <t>Si fallaste ayer, hoy hacé la versión mínima del hábito. La regla: nunca fallar dos días seguidos.</t>
+          <t>¿Fallaste ayer? Hoy hacé la versión mínima del hábito. La regla: nunca fallar dos días seguidos.</t>
         </is>
       </c>
     </row>
@@ -19624,7 +19624,7 @@
       </c>
       <c r="H6" s="61" t="inlineStr">
         <is>
-          <t>Elegí un momento fijo de la semana sin trabajo ni pendientes y defendelo como una cita importante.</t>
+          <t>Separá un momento fijo de la semana sin trabajo ni pendientes y defendelo como una cita importante.</t>
         </is>
       </c>
       <c r="I6" s="61" t="inlineStr">
@@ -19654,7 +19654,7 @@
       </c>
       <c r="N6" s="61" t="inlineStr">
         <is>
-          <t>Antes de dormir, anotá lo que te preocupa y lo que vas a hacer mañana al respecto. Después, entregalo en oración.</t>
+          <t>Hoy a la noche, anotá lo que te preocupa y lo que vas a hacer mañana al respecto. Después, entregalo en oración.</t>
         </is>
       </c>
     </row>
@@ -19744,7 +19744,7 @@
       </c>
       <c r="H8" s="61" t="inlineStr">
         <is>
-          <t>Antes de una decisión importante con tu plata, consultala con un profesional de confianza. Y anotá esta semana tres semillas concretas que sí quieras sembrar.</t>
+          <t>Consultá con un profesional de confianza cada decisión importante con tu plata. Y anotá esta semana tres semillas concretas que sí quieras sembrar.</t>
         </is>
       </c>
       <c r="I8" s="61" t="inlineStr">
@@ -19814,7 +19814,7 @@
       </c>
       <c r="H9" s="61" t="inlineStr">
         <is>
-          <t>Elegí un proyecto que abandonaste por impaciencia y dale una fecha realista para retomarlo.</t>
+          <t>Buscá un proyecto que abandonaste por impaciencia y dale una fecha realista para retomarlo.</t>
         </is>
       </c>
       <c r="I9" s="61" t="inlineStr">
@@ -19844,7 +19844,7 @@
       </c>
       <c r="N9" s="61" t="inlineStr">
         <is>
-          <t>Si estás esperando una oportunidad, usá el tiempo para capacitarte: hay cursos gratuitos del SNPP y otras instituciones.</t>
+          <t>Mientras esperás una oportunidad, usá el tiempo para capacitarte: hay cursos gratuitos del SNPP y otras instituciones.</t>
         </is>
       </c>
     </row>
@@ -20039,7 +20039,7 @@
       </c>
       <c r="K12" s="61" t="inlineStr">
         <is>
-          <t>Si tu cosecha o tu trabajo rindió, compartí una parte con una familia que pasa necesidad.</t>
+          <t>Cuando tu cosecha o tu trabajo rinda, compartí una parte con una familia que pasa necesidad.</t>
         </is>
       </c>
       <c r="L12" s="61" t="inlineStr">
@@ -20054,7 +20054,7 @@
       </c>
       <c r="N12" s="61" t="inlineStr">
         <is>
-          <t>Antes de dar, orá y decidí en tu corazón cuánto y a quién. Después, dalo con alegría.</t>
+          <t>Orá primero y decidí en tu corazón cuánto dar y a quién. Después, dalo con alegría.</t>
         </is>
       </c>
     </row>
@@ -20279,7 +20279,7 @@
       </c>
       <c r="G16" s="61" t="inlineStr">
         <is>
-          <t>Personas que dicen "yo estoy sano, nunca voy al médico" hasta que aparece un problema grave.</t>
+          <t>“Yo estoy sano, nunca voy al médico”, hasta que aparece un problema grave.</t>
         </is>
       </c>
       <c r="H16" s="61" t="inlineStr">
@@ -20299,7 +20299,7 @@
       </c>
       <c r="K16" s="61" t="inlineStr">
         <is>
-          <t>Antes de tomar un remedio por tu cuenta, consultá en la farmacia o en el centro de salud.</t>
+          <t>¿Remedio por tu cuenta? Mejor consultá primero en la farmacia o en el centro de salud.</t>
         </is>
       </c>
       <c r="L16" s="61" t="inlineStr">
@@ -20424,7 +20424,7 @@
       </c>
       <c r="H18" s="61" t="inlineStr">
         <is>
-          <t>Si te sentís sin fuerzas, contalo a tu médico y a alguien de confianza. Pedir ayuda es parte del tratamiento.</t>
+          <t>¿Te sentís sin fuerzas? Contalo a tu médico y a alguien de confianza. Pedir ayuda es parte del tratamiento.</t>
         </is>
       </c>
       <c r="I18" s="61" t="inlineStr">
@@ -20629,7 +20629,7 @@
       </c>
       <c r="K21" s="61" t="inlineStr">
         <is>
-          <t>Elegí una enseñanza y aplicala hoy mismo con alguien concreto: pedir perdón, ayudar, agradecer.</t>
+          <t>Hoy mismo, aplicá una enseñanza con alguien concreto: pedir perdón, ayudar, agradecer.</t>
         </is>
       </c>
       <c r="L21" s="61" t="inlineStr">
@@ -20709,7 +20709,7 @@
       </c>
       <c r="M22" s="61" t="inlineStr">
         <is>
-          <t>Personas que usan versículos para señalar a los demás y no para mirarse a sí mismas.</t>
+          <t>La costumbre de usar versículos para señalar a los demás y no para mirarnos a nosotros mismos.</t>
         </is>
       </c>
       <c r="N22" s="61" t="inlineStr">
@@ -20754,7 +20754,7 @@
       </c>
       <c r="H23" s="61" t="inlineStr">
         <is>
-          <t>Elegí un plan de 30 días (por ejemplo, un capítulo de Proverbios por día) y marcá cada día cumplido.</t>
+          <t>Probá un plan de 30 días (por ejemplo, un capítulo de Proverbios por día) y marcá cada día cumplido.</t>
         </is>
       </c>
       <c r="I23" s="61" t="inlineStr">
@@ -20959,7 +20959,7 @@
       </c>
       <c r="K26" s="61" t="inlineStr">
         <is>
-          <t>Antes de dormir, repasá el día: ¿qué guardaste hoy que no te hace bien? Soltalo en oración.</t>
+          <t>Al acostarte, repasá el día: ¿qué guardaste hoy que no te hace bien? Soltalo en oración.</t>
         </is>
       </c>
       <c r="L26" s="61" t="inlineStr">
@@ -21014,7 +21014,7 @@
       </c>
       <c r="H27" s="61" t="inlineStr">
         <is>
-          <t>Elegí una cosa que les pedís a otros y hacela vos primero durante toda la semana.</t>
+          <t>Eso que les pedís a otros, hacelo vos primero durante toda la semana.</t>
         </is>
       </c>
       <c r="I27" s="61" t="inlineStr">
@@ -21029,7 +21029,7 @@
       </c>
       <c r="K27" s="61" t="inlineStr">
         <is>
-          <t>Antes de prometer algo esta semana, preguntate si lo podés cumplir. Prometé menos y cumplí todo.</t>
+          <t>Prometé menos y cumplí todo: esta semana, antes de cada promesa, preguntate si la podés cumplir.</t>
         </is>
       </c>
       <c r="L27" s="61" t="inlineStr">
@@ -21044,7 +21044,7 @@
       </c>
       <c r="N27" s="61" t="inlineStr">
         <is>
-          <t>Pensá en alguien que te mira como ejemplo. Elegí una cosa concreta que querés que aprenda de vos y vivila hoy.</t>
+          <t>¿Quién te mira como ejemplo? Elegí una cosa concreta que querés que aprenda de vos y vivila hoy.</t>
         </is>
       </c>
     </row>
@@ -21084,7 +21084,7 @@
       </c>
       <c r="H28" s="61" t="inlineStr">
         <is>
-          <t>Si sos joven, elegí un área donde podés dar el ejemplo ya: puntualidad, palabra, trato. Si sos adulto, dale a un joven una responsabilidad real.</t>
+          <t>Para los jóvenes: elegí un área donde podés dar el ejemplo ya: puntualidad, palabra, trato. Para los adultos: dale a un joven una responsabilidad real.</t>
         </is>
       </c>
       <c r="I28" s="61" t="inlineStr">
@@ -21169,7 +21169,7 @@
       </c>
       <c r="K29" s="61" t="inlineStr">
         <is>
-          <t>Elegí un compromiso pendiente (una deuda, un favor prometido, una llamada) y cumplilo esta semana.</t>
+          <t>Cumplí esta semana un compromiso pendiente: una deuda, un favor prometido, una llamada.</t>
         </is>
       </c>
       <c r="L29" s="61" t="inlineStr">
@@ -21184,7 +21184,7 @@
       </c>
       <c r="N29" s="61" t="inlineStr">
         <is>
-          <t>Si te llega un comentario sobre alguien, no lo reenvíes. Si es grave, hablalo con la persona.</t>
+          <t>No reenvíes el comentario que te llega sobre alguien. Si es grave, hablalo con la persona.</t>
         </is>
       </c>
     </row>
@@ -21374,7 +21374,7 @@
       </c>
       <c r="N32" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, antes de comprar algo para la casa, regalale a tu familia una hora juntos sin pantallas.</t>
+          <t>Regalale a tu familia una hora juntos sin pantallas esta semana, antes de comprar algo para la casa.</t>
         </is>
       </c>
     </row>
@@ -21414,7 +21414,7 @@
       </c>
       <c r="H33" s="61" t="inlineStr">
         <is>
-          <t>Elegí un lugar fijo para llaves, documentos y cargadores. Pocas cosas, siempre en el mismo lugar.</t>
+          <t>Llaves, documentos y cargadores: dales un lugar fijo. Pocas cosas, siempre en el mismo lugar.</t>
         </is>
       </c>
       <c r="I33" s="61" t="inlineStr">
@@ -21429,7 +21429,7 @@
       </c>
       <c r="K33" s="61" t="inlineStr">
         <is>
-          <t>Elegí un cajón o un rincón y ordenalo hoy en quince minutos. Lo que no usás, regalalo.</t>
+          <t>Quince minutos alcanzan para ordenar hoy un cajón o un rincón. Lo que no usás, regalalo.</t>
         </is>
       </c>
       <c r="L33" s="61" t="inlineStr">
@@ -21499,7 +21499,7 @@
       </c>
       <c r="K34" s="61" t="inlineStr">
         <is>
-          <t>Hacé hoy una tarea de la casa que normalmente hace otro, sin que te lo pidan.</t>
+          <t>Sin que te lo pidan, hacé hoy una tarea de la casa que normalmente hace otro.</t>
         </is>
       </c>
       <c r="L34" s="61" t="inlineStr">
@@ -21584,7 +21584,7 @@
       </c>
       <c r="N35" s="61" t="inlineStr">
         <is>
-          <t>Elegí una rutina de diez minutos diarios: los platos limpios antes de dormir y la mesa despejada. Constancia antes que maratón.</t>
+          <t>Diez minutos diarios de rutina: los platos limpios antes de dormir y la mesa despejada. Constancia antes que maratón.</t>
         </is>
       </c>
     </row>
@@ -21884,7 +21884,7 @@
       </c>
       <c r="H40" s="61" t="inlineStr">
         <is>
-          <t>Elegí un monto que puedas guardar todas las semanas sin falta, aunque sea pequeño. La constancia importa más que el monto.</t>
+          <t>Definí un monto que puedas guardar todas las semanas sin falta, aunque sea pequeño. La constancia importa más que el monto.</t>
         </is>
       </c>
       <c r="I40" s="61" t="inlineStr">
@@ -21899,7 +21899,7 @@
       </c>
       <c r="K40" s="61" t="inlineStr">
         <is>
-          <t>Si pensás en hacer crecer tus ahorros, conversalo primero con un profesional de confianza, como un contador.</t>
+          <t>Conversá primero con un profesional de confianza, como un contador, si pensás en hacer crecer tus ahorros.</t>
         </is>
       </c>
       <c r="L40" s="61" t="inlineStr">
@@ -21954,7 +21954,7 @@
       </c>
       <c r="H41" s="61" t="inlineStr">
         <is>
-          <t>Si guardás tus ahorros en casa, averiguá esta semana cómo abrir una cuenta de ahorro en una cooperativa o un banco.</t>
+          <t>¿Guardás tus ahorros en casa? Averiguá esta semana cómo abrir una cuenta de ahorro en una cooperativa o un banco.</t>
         </is>
       </c>
       <c r="I41" s="61" t="inlineStr">
@@ -22154,12 +22154,12 @@
       </c>
       <c r="J44" s="61" t="inlineStr">
         <is>
-          <t>Personas que no saben decir que no y terminan agotadas y resentidas.</t>
+          <t>La dificultad para decir que no, que termina en agotamiento y resentimiento.</t>
         </is>
       </c>
       <c r="K44" s="61" t="inlineStr">
         <is>
-          <t>Antes de aceptar un compromiso nuevo esta semana, tomate un momento y preguntate si de verdad podés.</t>
+          <t>Cuando te pidan un compromiso nuevo esta semana, tomate un momento y preguntate si de verdad podés.</t>
         </is>
       </c>
       <c r="L44" s="61" t="inlineStr">
@@ -22244,7 +22244,7 @@
       </c>
       <c r="N45" s="61" t="inlineStr">
         <is>
-          <t>Elegí un versículo para esta semana y repetilo cada vez que sientas ansiedad o desánimo.</t>
+          <t>Anotá un versículo para esta semana y repetilo cada vez que sientas ansiedad o desánimo.</t>
         </is>
       </c>
     </row>
@@ -22314,7 +22314,7 @@
       </c>
       <c r="N46" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, la última media hora del día sin pantallas: una lectura, una oración o una charla.</t>
+          <t>La última media hora del día, sin pantallas: una lectura, una oración o una charla. Probalo esta semana.</t>
         </is>
       </c>
     </row>
@@ -22419,12 +22419,12 @@
       </c>
       <c r="G48" s="61" t="inlineStr">
         <is>
-          <t>Personas que cargan tristeza durante meses sin contarle a nadie.</t>
+          <t>La tristeza que se carga durante meses sin contársela a nadie.</t>
         </is>
       </c>
       <c r="H48" s="61" t="inlineStr">
         <is>
-          <t>Si algo te pesa hace tiempo, contáselo hoy a una persona de confianza.</t>
+          <t>Contale hoy a una persona de confianza eso que te pesa hace tiempo.</t>
         </is>
       </c>
       <c r="I48" s="61" t="inlineStr">
@@ -22490,7 +22490,7 @@
       <c r="G49" s="61" t="n"/>
       <c r="H49" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, escribí cada noche en pocas líneas qué sentiste en el día y llevalo a Dios en oración.</t>
+          <t>Durante la semana, escribí cada noche en pocas líneas qué sentiste en el día y llevalo a Dios en oración.</t>
         </is>
       </c>
       <c r="I49" s="61" t="inlineStr">
@@ -22544,7 +22544,7 @@
       </c>
       <c r="H50" s="61" t="inlineStr">
         <is>
-          <t>Si tenés animales, revisá hoy que tengan agua limpia, sombra y comida suficiente.</t>
+          <t>Revisá hoy que tus animales tengan agua limpia, sombra y comida suficiente.</t>
         </is>
       </c>
       <c r="I50" s="61" t="inlineStr">
@@ -22574,7 +22574,7 @@
       </c>
       <c r="N50" s="61" t="inlineStr">
         <is>
-          <t>Si conocés a alguien que trabaja en una estancia o en un tambo, agradecele hoy su constancia.</t>
+          <t>Agradecele hoy su constancia a alguien que trabaja en una estancia o en un tambo.</t>
         </is>
       </c>
     </row>
@@ -22714,7 +22714,7 @@
       </c>
       <c r="N52" s="61" t="inlineStr">
         <is>
-          <t>Si tenés mascotas, cuidá sus vacunas y no las abandones. Adoptar un animal es un compromiso para toda su vida.</t>
+          <t>Cuidá las vacunas de tus mascotas y no las abandones. Adoptar un animal es un compromiso para toda su vida.</t>
         </is>
       </c>
     </row>
@@ -22754,7 +22754,7 @@
       </c>
       <c r="H53" s="61" t="inlineStr">
         <is>
-          <t>Si tenés gente a cargo, reconocé hoy, con nombre y apellido, el trabajo constante de alguien.</t>
+          <t>Con nombre y apellido, reconocé hoy el trabajo constante de alguien que tenés a cargo.</t>
         </is>
       </c>
       <c r="I53" s="61" t="inlineStr">
@@ -22939,7 +22939,7 @@
       </c>
       <c r="G56" s="61" t="inlineStr">
         <is>
-          <t>Creer que estamos sanos porque no sentimos nada.</t>
+          <t>“No siento nada, así que estoy sano”.</t>
         </is>
       </c>
       <c r="H56" s="61" t="inlineStr">
@@ -22974,7 +22974,7 @@
       </c>
       <c r="N56" s="61" t="inlineStr">
         <is>
-          <t>Si sos hombre, sacá un turno para tu control. Si tenés un padre, un esposo o un hermano que no va, acompañalo.</t>
+          <t>Hombres: saquen turno para su control. Y si tu padre, tu esposo o tu hermano no va, acompañalo.</t>
         </is>
       </c>
     </row>
@@ -23099,7 +23099,7 @@
       </c>
       <c r="K58" s="61" t="inlineStr">
         <is>
-          <t>Si tenés miedo de ir, pedile a alguien de confianza que te acompañe, y oren juntos antes.</t>
+          <t>¿Te da miedo ir? Pedile a alguien de confianza que te acompañe, y oren juntos antes.</t>
         </is>
       </c>
       <c r="L58" s="61" t="inlineStr">
@@ -23184,7 +23184,7 @@
       </c>
       <c r="N59" s="61" t="inlineStr">
         <is>
-          <t>Si te indicaron un tratamiento, cumplilo completo, aunque te sientas bien antes de terminarlo.</t>
+          <t>Cumplí completo el tratamiento que te indicaron, aunque te sientas bien antes de terminarlo.</t>
         </is>
       </c>
     </row>
@@ -23254,7 +23254,7 @@
       </c>
       <c r="N60" s="61" t="inlineStr">
         <is>
-          <t>Antes de compartir un consejo de salud, preguntá: ¿quién lo dice y en qué se basa?</t>
+          <t>¿Te llegó un consejo de salud? Antes de compartirlo, preguntá quién lo dice y en qué se basa.</t>
         </is>
       </c>
     </row>
@@ -23339,12 +23339,12 @@
       </c>
       <c r="G62" s="61" t="inlineStr">
         <is>
-          <t>Personas que creen en Dios pero viven su fe completamente solas, sin nadie que las acompañe.</t>
+          <t>El creyente que vive su fe completamente solo, sin nadie que lo acompañe.</t>
         </is>
       </c>
       <c r="H62" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, contale a alguien de tu iglesia o de tu familia algo que Dios te enseñó.</t>
+          <t>Contale estos días a alguien de tu iglesia o de tu familia algo que Dios te enseñó.</t>
         </is>
       </c>
       <c r="I62" s="61" t="inlineStr">
@@ -23374,7 +23374,7 @@
       </c>
       <c r="N62" s="61" t="inlineStr">
         <is>
-          <t>Si te alejaste por una herida, orá por eso y buscá a una persona de confianza para conversarlo, sin apuro.</t>
+          <t>Orá por esa herida que te alejó y buscá a una persona de confianza para conversarlo, sin apuro.</t>
         </is>
       </c>
     </row>
@@ -23444,7 +23444,7 @@
       </c>
       <c r="N63" s="61" t="inlineStr">
         <is>
-          <t>Pensá en alguien que está pasando un mal momento y llamalo hoy.</t>
+          <t>Llamá hoy a alguien que está pasando un mal momento.</t>
         </is>
       </c>
     </row>
@@ -23484,7 +23484,7 @@
       </c>
       <c r="H64" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, compartí con alguien de confianza una necesidad real, para que ore por vos.</t>
+          <t>Compartí con alguien de confianza una necesidad real, para que ore por vos.</t>
         </is>
       </c>
       <c r="I64" s="61" t="inlineStr">
@@ -23514,7 +23514,7 @@
       </c>
       <c r="N64" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, sumate a un grupo pequeño, una célula o una reunión de oración, aunque sea una vez.</t>
+          <t>Sumate, aunque sea una vez, a un grupo pequeño, una célula o una reunión de oración.</t>
         </is>
       </c>
     </row>
@@ -23549,7 +23549,7 @@
       </c>
       <c r="G65" s="61" t="inlineStr">
         <is>
-          <t>Personas que se sienten de más en la iglesia porque no cantan, no predican ni tocan un instrumento.</t>
+          <t>La sensación de estar de más en la iglesia por no cantar, no predicar ni tocar un instrumento.</t>
         </is>
       </c>
       <c r="H65" s="61" t="inlineStr">
@@ -23759,7 +23759,7 @@
       </c>
       <c r="K68" s="61" t="inlineStr">
         <is>
-          <t>Antes de comunicar algo importante, resumilo en una sola frase clara. Si estás enojado, esperá antes de enviarlo.</t>
+          <t>Resumí en una sola frase clara eso importante que tenés que comunicar. Y si estás enojado, esperá antes de enviarlo.</t>
         </is>
       </c>
       <c r="L68" s="61" t="inlineStr">
@@ -23774,7 +23774,7 @@
       </c>
       <c r="N68" s="61" t="inlineStr">
         <is>
-          <t>Si sentís que te enojás, pedí unos minutos y volvé a hablar cuando estés en calma.</t>
+          <t>Cuando sientas que te enojás, pedí unos minutos y volvé a hablar en calma.</t>
         </is>
       </c>
     </row>
@@ -23829,7 +23829,7 @@
       </c>
       <c r="K69" s="61" t="inlineStr">
         <is>
-          <t>Elegí una tarea que siempre hacés vos y que otro puede aprender. Enseñala esta semana.</t>
+          <t>Enseñale a otro esta semana una tarea que siempre hacés vos y que puede aprender.</t>
         </is>
       </c>
       <c r="L69" s="61" t="inlineStr">
@@ -23954,7 +23954,7 @@
       </c>
       <c r="H71" s="61" t="inlineStr">
         <is>
-          <t>Elegí qué es lo propio de esta etapa de tu vida y qué puede esperar.</t>
+          <t>Distinguí qué es lo propio de esta etapa de tu vida y qué puede esperar.</t>
         </is>
       </c>
       <c r="I71" s="61" t="inlineStr">
@@ -24244,7 +24244,7 @@
       </c>
       <c r="N75" s="61" t="inlineStr">
         <is>
-          <t>Si vos o alguien que conocés sufre violencia, pedí ayuda: hablá con tu pastor y llamá a la línea 137 «SOS Mujer», gratuita y las 24 horas, o escribí al WhatsApp 0961 137 137. Si hay peligro inmediato, llamá al 911.</t>
+          <t>Ante la violencia, contra vos o contra alguien que conocés, pedí ayuda: hablá con tu pastor y llamá a la línea 137 «SOS Mujer», gratuita y las 24 horas, o escribí al WhatsApp 0961 137 137. Si hay peligro inmediato, llamá al 911.</t>
         </is>
       </c>
     </row>
@@ -24384,7 +24384,7 @@
       </c>
       <c r="N77" s="61" t="inlineStr">
         <is>
-          <t>Si su matrimonio está en crisis, busquen juntos a un consejero o a un pastor de confianza. Pedir ayuda también es una forma de amar.</t>
+          <t>Busquen juntos a un consejero o a un pastor de confianza si su matrimonio está en crisis. Pedir ayuda también es una forma de amar.</t>
         </is>
       </c>
     </row>
@@ -24454,7 +24454,7 @@
       </c>
       <c r="N78" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, salgan a caminar o a tomar un tereré los dos solos, y hablen de ustedes.</t>
+          <t>Con tu pareja, salgan a caminar o a tomar un tereré los dos solos, y hablen de ustedes.</t>
         </is>
       </c>
     </row>
@@ -24544,7 +24544,7 @@
       </c>
       <c r="H80" s="61" t="inlineStr">
         <is>
-          <t>Esta semana anotá en una hoja tus ingresos del mes y tus gastos fijos. Ese es el comienzo de tu presupuesto.</t>
+          <t>Tomá una hoja y anotá tus ingresos del mes y tus gastos fijos. Ese es el comienzo de tu presupuesto.</t>
         </is>
       </c>
       <c r="I80" s="61" t="inlineStr">
@@ -24569,12 +24569,12 @@
       </c>
       <c r="M80" s="61" t="inlineStr">
         <is>
-          <t>Pensar que planificar la plata es cosa de ricos o de contadores.</t>
+          <t>“Planificar la plata es cosa de ricos o de contadores”.</t>
         </is>
       </c>
       <c r="N80" s="61" t="inlineStr">
         <is>
-          <t>Elegí con tu familia una meta concreta para este año y calculen cuánto deberían separar por mes para lograrla.</t>
+          <t>Con tu familia, pónganse una meta concreta para este año y calculen cuánto deberían separar por mes para lograrla.</t>
         </is>
       </c>
     </row>
@@ -24629,7 +24629,7 @@
       </c>
       <c r="K81" s="61" t="inlineStr">
         <is>
-          <t>Antes de una compra grande o de un préstamo, esperá 48 horas y hacé las cuentas por escrito.</t>
+          <t>Esperá 48 horas antes de una compra grande o de un préstamo, y hacé las cuentas por escrito.</t>
         </is>
       </c>
       <c r="L81" s="61" t="inlineStr">
@@ -24769,7 +24769,7 @@
       </c>
       <c r="K83" s="61" t="inlineStr">
         <is>
-          <t>Elegí un gasto diario que podés reducir esta semana y anotá cuánto ahorrás.</t>
+          <t>Recortá esta semana un gasto diario y anotá cuánto ahorrás.</t>
         </is>
       </c>
       <c r="L83" s="61" t="inlineStr">
@@ -24944,7 +24944,7 @@
       </c>
       <c r="H86" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, antes de cada actividad de la iglesia, pedile a Dios que te cambie a vos, no solo que te ayude a cumplir.</t>
+          <t>Pedile a Dios, antes de cada actividad de la iglesia, que te cambie a vos, no solo que te ayude a cumplir.</t>
         </is>
       </c>
       <c r="I86" s="61" t="inlineStr">
@@ -24959,7 +24959,7 @@
       </c>
       <c r="K86" s="61" t="inlineStr">
         <is>
-          <t>Elegí un rasgo del fruto (paciencia, mansedumbre…) que querés ver crecer y orá por él cada día de esta semana.</t>
+          <t>Orá cada día de esta semana por un rasgo del fruto (paciencia, mansedumbre…) que querés ver crecer.</t>
         </is>
       </c>
       <c r="L86" s="61" t="inlineStr">
@@ -25084,7 +25084,7 @@
       </c>
       <c r="H88" s="61" t="inlineStr">
         <is>
-          <t>Elegí una sola disciplina para esta semana (oración, lectura o silencio) y dale un horario fijo.</t>
+          <t>Dale un horario fijo a una sola disciplina esta semana: oración, lectura o silencio.</t>
         </is>
       </c>
       <c r="I88" s="61" t="inlineStr">
@@ -25099,7 +25099,7 @@
       </c>
       <c r="K88" s="61" t="inlineStr">
         <is>
-          <t>Si estás cansado, decíselo a Dios con sinceridad. Eso también es oración.</t>
+          <t>Decile a Dios con sinceridad que estás cansado. Eso también es oración.</t>
         </is>
       </c>
       <c r="L88" s="61" t="inlineStr">
@@ -25154,7 +25154,7 @@
       </c>
       <c r="H89" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, a lo que leas sumale una pregunta: ¿qué me muestra esto de la gracia de Jesús?</t>
+          <t>A todo lo que leas estos días, sumale una pregunta: ¿qué me muestra esto de la gracia de Jesús?</t>
         </is>
       </c>
       <c r="I89" s="61" t="inlineStr">
@@ -25169,7 +25169,7 @@
       </c>
       <c r="K89" s="61" t="inlineStr">
         <is>
-          <t>Elegí diez minutos diarios para una disciplina y mantenelos toda la semana.</t>
+          <t>Dedicá diez minutos diarios a una disciplina y mantenelos toda la semana.</t>
         </is>
       </c>
       <c r="L89" s="61" t="inlineStr">
@@ -25344,7 +25344,7 @@
       </c>
       <c r="H92" s="61" t="inlineStr">
         <is>
-          <t>Si tenés un negocio, agradecé a Dios esta semana por lo que te permitió construir, y a la gente que trabaja con vos.</t>
+          <t>Agradecé a Dios esta semana por lo que te permitió construir en tu negocio, y a la gente que trabaja con vos.</t>
         </is>
       </c>
       <c r="I92" s="61" t="inlineStr">
@@ -25429,7 +25429,7 @@
       </c>
       <c r="K93" s="61" t="inlineStr">
         <is>
-          <t>Si buscás trabajo, sumá una capacitación gratuita (por ejemplo, del SNPP) y presentate siempre puntual.</t>
+          <t>Mientras buscás trabajo, sumá una capacitación gratuita (por ejemplo, del SNPP) y presentate siempre puntual.</t>
         </is>
       </c>
       <c r="L93" s="61" t="inlineStr">
@@ -25484,7 +25484,7 @@
       </c>
       <c r="H94" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, festejá con tu equipo o con tu familia un logro del trabajo, aunque sea pequeño.</t>
+          <t>Festejá con tu equipo o con tu familia un logro del trabajo, aunque sea pequeño.</t>
         </is>
       </c>
       <c r="I94" s="61" t="inlineStr">
@@ -25499,7 +25499,7 @@
       </c>
       <c r="K94" s="61" t="inlineStr">
         <is>
-          <t>Si tenés un negocio, revisá esta semana que tus pagos a empleados y proveedores estén al día.</t>
+          <t>Revisá esta semana que los pagos de tu negocio a empleados y proveedores estén al día.</t>
         </is>
       </c>
       <c r="L94" s="61" t="inlineStr">
@@ -25554,7 +25554,7 @@
       </c>
       <c r="H95" s="61" t="inlineStr">
         <is>
-          <t>Antes de una decisión de trabajo difícil, preguntate: ¿esto lo haría si confiara de verdad en Dios?</t>
+          <t>Frente a una decisión de trabajo difícil, preguntate: ¿esto lo haría si confiara de verdad en Dios?</t>
         </is>
       </c>
       <c r="I95" s="61" t="inlineStr">
@@ -25584,7 +25584,7 @@
       </c>
       <c r="N95" s="61" t="inlineStr">
         <is>
-          <t>Si tu negocio atraviesa una crisis, compartilo con alguien de confianza y oren juntos pidiendo sabiduría.</t>
+          <t>Compartí con alguien de confianza la crisis que atraviesa tu negocio, y oren juntos pidiendo sabiduría.</t>
         </is>
       </c>
     </row>
@@ -25619,7 +25619,7 @@
       </c>
       <c r="G96" s="61" t="inlineStr">
         <is>
-          <t>Personas que sienten que su trabajo no vale nada.</t>
+          <t>¿Para qué sirve mi trabajo? A veces parece que no vale nada.</t>
         </is>
       </c>
       <c r="H96" s="61" t="inlineStr">
@@ -25639,7 +25639,7 @@
       </c>
       <c r="K96" s="61" t="inlineStr">
         <is>
-          <t>Si tenés un negocio, cumplí esta semana con algo que nadie te exige, pero que cuida a tu gente o a tus clientes.</t>
+          <t>Cumplí esta semana, en tu negocio, con algo que nadie te exige pero que cuida a tu gente o a tus clientes.</t>
         </is>
       </c>
       <c r="L96" s="61" t="inlineStr">
@@ -25654,7 +25654,7 @@
       </c>
       <c r="N96" s="61" t="inlineStr">
         <is>
-          <t>Esta semana comprá en un negocio pequeño y honesto de tu barrio, y decile al dueño que valorás su trabajo.</t>
+          <t>Comprá en un negocio pequeño y honesto de tu barrio, y decile al dueño que valorás su trabajo.</t>
         </is>
       </c>
     </row>
@@ -25759,7 +25759,7 @@
       </c>
       <c r="K98" s="61" t="inlineStr">
         <is>
-          <t>Elegí un movimiento que disfrutes (caminar, andar en bicicleta, jugar a la pelota con los chicos) y hacelo tres veces esta semana.</t>
+          <t>Caminar, andar en bicicleta, jugar a la pelota con los chicos: buscá el movimiento que disfrutes y hacelo tres veces esta semana.</t>
         </is>
       </c>
       <c r="L98" s="61" t="inlineStr">
@@ -25814,7 +25814,7 @@
       </c>
       <c r="H99" s="61" t="inlineStr">
         <is>
-          <t>Elegí un hábito de movimiento y anotá cada día si lo cumpliste.</t>
+          <t>Proponete un hábito de movimiento y anotá cada día si lo cumpliste.</t>
         </is>
       </c>
       <c r="I99" s="61" t="inlineStr">
@@ -25964,7 +25964,7 @@
       </c>
       <c r="J101" s="61" t="inlineStr">
         <is>
-          <t>Pensar que lo espiritual no tiene nada que ver con el cuidado del cuerpo.</t>
+          <t>Separar lo espiritual del cuidado del cuerpo, como si no tuvieran nada que ver.</t>
         </is>
       </c>
       <c r="K101" s="61" t="inlineStr">
@@ -25984,7 +25984,7 @@
       </c>
       <c r="N101" s="61" t="inlineStr">
         <is>
-          <t>Si tenés una limitación, preguntá en tu unidad de salud familiar qué movimientos podés hacer de forma segura.</t>
+          <t>Preguntá en tu unidad de salud familiar qué movimientos podés hacer de forma segura con tu limitación.</t>
         </is>
       </c>
     </row>
@@ -26019,7 +26019,7 @@
       </c>
       <c r="G102" s="61" t="inlineStr">
         <is>
-          <t>Creer que el ejercicio solo cuenta en un gimnasio.</t>
+          <t>“Si no voy al gimnasio, no hago ejercicio”.</t>
         </is>
       </c>
       <c r="H102" s="61" t="inlineStr">
@@ -26209,7 +26209,7 @@
       </c>
       <c r="G105" s="61" t="inlineStr">
         <is>
-          <t>Personas que creen que no tienen nada para aportar.</t>
+          <t>“Yo no tengo nada para aportar”.</t>
         </is>
       </c>
       <c r="H105" s="61" t="inlineStr">
@@ -26284,7 +26284,7 @@
       </c>
       <c r="H106" s="61" t="inlineStr">
         <is>
-          <t>Hacé hoy un servicio que nadie vea: lavar, ordenar, preparar algo para otro.</t>
+          <t>Lavá, ordená o prepará algo para otro hoy, en un servicio que nadie vea.</t>
         </is>
       </c>
       <c r="I106" s="61" t="inlineStr">
@@ -26299,7 +26299,7 @@
       </c>
       <c r="K106" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, hacé una tarea que normalmente dejás a otros, sin comentarlo.</t>
+          <t>Sin comentarlo, hacé una tarea que normalmente dejás a otros.</t>
         </is>
       </c>
       <c r="L106" s="61" t="inlineStr">
@@ -26354,7 +26354,7 @@
       </c>
       <c r="H107" s="61" t="inlineStr">
         <is>
-          <t>Antes de servir hoy, decí en silencio: «Esto es para vos, Señor».</t>
+          <t>Hoy, cuando sirvas, decí en silencio: «Esto es para vos, Señor».</t>
         </is>
       </c>
       <c r="I107" s="61" t="inlineStr">
@@ -26384,7 +26384,7 @@
       </c>
       <c r="N107" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, orá por alguien sin decírselo.</t>
+          <t>Orá en silencio por alguien, sin decírselo.</t>
         </is>
       </c>
     </row>
@@ -26434,12 +26434,12 @@
       </c>
       <c r="J108" s="61" t="inlineStr">
         <is>
-          <t>Pensar que solo vale la pena el servicio grande.</t>
+          <t>La idea de que solo vale la pena el servicio grande.</t>
         </is>
       </c>
       <c r="K108" s="61" t="inlineStr">
         <is>
-          <t>Elegí un gesto pequeño y concreto para hacer cada día de esta semana.</t>
+          <t>Cada día de esta semana, hacé un gesto pequeño y concreto.</t>
         </is>
       </c>
       <c r="L108" s="61" t="inlineStr">
@@ -26544,7 +26544,7 @@
       </c>
       <c r="H110" s="61" t="inlineStr">
         <is>
-          <t>Si recibís críticas por algo bueno que estás haciendo, no respondas en caliente: orá y seguí trabajando.</t>
+          <t>Ante las críticas por algo bueno que estás haciendo, no respondas en caliente: orá y seguí trabajando.</t>
         </is>
       </c>
       <c r="I110" s="61" t="inlineStr">
@@ -26614,7 +26614,7 @@
       </c>
       <c r="H111" s="61" t="inlineStr">
         <is>
-          <t>Antes de descartar una crítica, preguntale a alguien de confianza si hay algo de verdad en ella.</t>
+          <t>¿Te criticaron? Antes de descartarlo, preguntale a alguien de confianza si hay algo de verdad en eso.</t>
         </is>
       </c>
       <c r="I111" s="61" t="inlineStr">
@@ -26699,7 +26699,7 @@
       </c>
       <c r="K112" s="61" t="inlineStr">
         <is>
-          <t>Si te equivocaste en algo que afectó a otros, reconocelo con humildad y decí qué vas a corregir.</t>
+          <t>Reconocé con humildad el error que afectó a otros, y decí qué vas a corregir.</t>
         </is>
       </c>
       <c r="L112" s="61" t="inlineStr">
@@ -26824,7 +26824,7 @@
       </c>
       <c r="H114" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, defendé un tiempo de descanso como defenderías una reunión importante.</t>
+          <t>Defendé un tiempo de descanso como defenderías una reunión importante.</t>
         </is>
       </c>
       <c r="I114" s="61" t="inlineStr">
@@ -26839,7 +26839,7 @@
       </c>
       <c r="K114" s="61" t="inlineStr">
         <is>
-          <t>Si estás muy cansado, postergá las decisiones importantes hasta haber descansado.</t>
+          <t>Con mucho cansancio encima, postergá las decisiones importantes hasta haber descansado.</t>
         </is>
       </c>
       <c r="L114" s="61" t="inlineStr">
@@ -26944,7 +26944,7 @@
       </c>
       <c r="H116" s="61" t="inlineStr">
         <is>
-          <t>Elegí un momento fijo de la semana para conversar con tus hijos sobre la vida y la fe.</t>
+          <t>Reservá un momento fijo de la semana para conversar con tus hijos sobre la vida y la fe.</t>
         </is>
       </c>
       <c r="I116" s="61" t="inlineStr">
@@ -26974,7 +26974,7 @@
       </c>
       <c r="N116" s="61" t="inlineStr">
         <is>
-          <t>Si tu hijo se alejó, seguí orando por él y mostrale amor sin condiciones; no lo des por perdido.</t>
+          <t>Seguí orando por tu hijo que se alejó y mostrale amor sin condiciones; no lo des por perdido.</t>
         </is>
       </c>
     </row>
@@ -27099,7 +27099,7 @@
       </c>
       <c r="K118" s="61" t="inlineStr">
         <is>
-          <t>Si estás enojado, esperá a calmarte antes de corregir.</t>
+          <t>Primero calmá el enojo; recién después corregí.</t>
         </is>
       </c>
       <c r="L118" s="61" t="inlineStr">
@@ -27154,7 +27154,7 @@
       </c>
       <c r="H119" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, compartí con tus hijos algo que Dios te enseñó a vos.</t>
+          <t>Junto a tus hijos, compartí algo que Dios te enseñó a vos.</t>
         </is>
       </c>
       <c r="I119" s="61" t="inlineStr">
@@ -27184,7 +27184,7 @@
       </c>
       <c r="N119" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, hablá bien de tus padres o de tus suegros delante de tus hijos.</t>
+          <t>Delante de tus hijos, hablá bien de tus padres o de tus suegros.</t>
         </is>
       </c>
     </row>
@@ -27344,7 +27344,7 @@
       </c>
       <c r="H122" s="61" t="inlineStr">
         <is>
-          <t>Si conocés a alguien que busca trabajo, ayudalo con un contacto, una recomendación o compartiendo su currículum.</t>
+          <t>Ayudá a alguien que busca trabajo con un contacto, una recomendación o compartiendo su currículum.</t>
         </is>
       </c>
       <c r="I122" s="61" t="inlineStr">
@@ -27414,7 +27414,7 @@
       </c>
       <c r="H123" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, apoyá a un emprendimiento o a un trabajador humilde de tu zona comprándole.</t>
+          <t>Apoyá a un emprendimiento o a un trabajador humilde de tu zona comprándole algo.</t>
         </is>
       </c>
       <c r="I123" s="61" t="inlineStr">
@@ -27444,7 +27444,7 @@
       </c>
       <c r="N123" s="61" t="inlineStr">
         <is>
-          <t>Si tenés un emprendimiento pequeño, fijá dos horas por semana para trabajarlo con constancia.</t>
+          <t>Dos horas por semana: fijalas para trabajar con constancia tu emprendimiento pequeño.</t>
         </is>
       </c>
     </row>
@@ -27514,7 +27514,7 @@
       </c>
       <c r="N124" s="61" t="inlineStr">
         <is>
-          <t>Si este mes no alcanza, recortá primero en la columna de lo deseable.</t>
+          <t>¿Este mes no alcanza? Recortá primero en la columna de lo deseable.</t>
         </is>
       </c>
     </row>
@@ -27549,7 +27549,7 @@
       </c>
       <c r="G125" s="61" t="inlineStr">
         <is>
-          <t>Pensar que los gastos chicos no importan.</t>
+          <t>“Total, son gastos chicos; no importan”.</t>
         </is>
       </c>
       <c r="H125" s="61" t="inlineStr">
@@ -27814,7 +27814,7 @@
       </c>
       <c r="H129" s="61" t="inlineStr">
         <is>
-          <t>Elegí una tarea de hoy y hacela con todas tus ganas, como si fuera la más importante.</t>
+          <t>Tomá una tarea de hoy y hacela con todas tus ganas, como si fuera la más importante.</t>
         </is>
       </c>
       <c r="I129" s="61" t="inlineStr">
@@ -27839,7 +27839,7 @@
       </c>
       <c r="M129" s="61" t="inlineStr">
         <is>
-          <t>Pensar que ya es tarde para estudiar o aprender un oficio nuevo.</t>
+          <t>El miedo a que ya sea tarde para estudiar o aprender un oficio nuevo.</t>
         </is>
       </c>
       <c r="N129" s="61" t="inlineStr">
@@ -27984,7 +27984,7 @@
       </c>
       <c r="N131" s="61" t="inlineStr">
         <is>
-          <t>Elegí una de tus habilidades y pensá cómo usarla mejor en tu trabajo este mes.</t>
+          <t>Este mes, mirá cuál de tus habilidades podés usar mejor en tu trabajo, y cómo.</t>
         </is>
       </c>
     </row>
@@ -28054,7 +28054,7 @@
       </c>
       <c r="N132" s="61" t="inlineStr">
         <is>
-          <t>Si te ofrecen un atajo deshonesto para avanzar, decí que no. Tu nombre vale más.</t>
+          <t>Decí que no al atajo deshonesto que te ofrezcan para avanzar. Tu nombre vale más.</t>
         </is>
       </c>
     </row>
@@ -28229,7 +28229,7 @@
       </c>
       <c r="K135" s="61" t="inlineStr">
         <is>
-          <t>Si empezaste en pequeño, sacale una foto a tu comienzo: algún día te va a recordar de dónde saliste.</t>
+          <t>Sacale una foto a tu comienzo pequeño: algún día te va a recordar de dónde saliste.</t>
         </is>
       </c>
       <c r="L135" s="61" t="inlineStr">
@@ -28244,7 +28244,7 @@
       </c>
       <c r="N135" s="61" t="inlineStr">
         <is>
-          <t>Si tu emprendimiento pasa por un mal momento, hablalo con alguien de confianza y no lo cargues como culpa.</t>
+          <t>Hablá con alguien de confianza sobre el mal momento de tu emprendimiento, y no lo cargues como culpa.</t>
         </is>
       </c>
     </row>
@@ -28284,7 +28284,7 @@
       </c>
       <c r="H136" s="61" t="inlineStr">
         <is>
-          <t>Antes de invertir, hacé una prueba pequeña: vendé a diez personas y escuchá lo que dicen.</t>
+          <t>Probá en pequeño antes de invertir: vendé a diez personas y escuchá lo que dicen.</t>
         </is>
       </c>
       <c r="I136" s="61" t="inlineStr">
@@ -28354,7 +28354,7 @@
       </c>
       <c r="H137" s="61" t="inlineStr">
         <is>
-          <t>Antes de entrar en un negocio que te ofrecen, preguntá: ¿cómo gana plata realmente? Si no lo entendés, no entres.</t>
+          <t>¿Te ofrecen un negocio? Preguntá cómo gana plata realmente. Si no lo entendés, no entres.</t>
         </is>
       </c>
       <c r="I137" s="61" t="inlineStr">
@@ -28454,7 +28454,7 @@
       </c>
       <c r="N138" s="61" t="inlineStr">
         <is>
-          <t>Si sos emprendedor, buscá a otro emprendedor para contarse lo que los ayudó a sostenerse.</t>
+          <t>Buscá a otro emprendedor y cuéntense lo que los ayudó a sostenerse.</t>
         </is>
       </c>
     </row>
@@ -28679,12 +28679,12 @@
       </c>
       <c r="G142" s="61" t="inlineStr">
         <is>
-          <t>Pensar que la fe no tiene nada que ver con lo cotidiano.</t>
+          <t>Dejar la fe para el domingo, como si no tuviera nada que ver con lo cotidiano.</t>
         </is>
       </c>
       <c r="H142" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, agradezcan en voz alta antes de cada comida en familia.</t>
+          <t>En cada comida en familia, agradezcan en voz alta antes de empezar.</t>
         </is>
       </c>
       <c r="I142" s="61" t="inlineStr">
@@ -28699,7 +28699,7 @@
       </c>
       <c r="K142" s="61" t="inlineStr">
         <is>
-          <t>Elegí un solo hábito nuevo para esta semana: más agua, una fruta por día o una porción de verduras.</t>
+          <t>Sumá un solo hábito nuevo esta semana: más agua, una fruta por día o una porción de verduras.</t>
         </is>
       </c>
       <c r="L142" s="61" t="inlineStr">
@@ -28784,7 +28784,7 @@
       </c>
       <c r="N143" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, hacé al menos una comida por día sin pantallas.</t>
+          <t>Al menos una comida por día, sin pantallas. Probalo esta semana.</t>
         </is>
       </c>
     </row>
@@ -28854,7 +28854,7 @@
       </c>
       <c r="N144" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, en casa, no hagan comentarios sobre el cuerpo o lo que come cada uno; hablen de lo rico y de lo que agradecen.</t>
+          <t>En casa, cero comentarios sobre el cuerpo o lo que come cada uno; hablen de lo rico y de lo que agradecen.</t>
         </is>
       </c>
     </row>
@@ -28944,7 +28944,7 @@
       </c>
       <c r="H146" s="61" t="inlineStr">
         <is>
-          <t>Pensá en alguien más joven en la fe y proponele encontrarse una vez por semana durante un mes.</t>
+          <t>Proponele a alguien más joven en la fe encontrarse una vez por semana durante un mes.</t>
         </is>
       </c>
       <c r="I146" s="61" t="inlineStr">
@@ -29014,7 +29014,7 @@
       </c>
       <c r="H147" s="61" t="inlineStr">
         <is>
-          <t>Antes de aconsejar a alguien esta semana, preguntate qué de eso necesitás vos.</t>
+          <t>Cuando aconsejes a alguien esta semana, preguntate qué de eso necesitás vos.</t>
         </is>
       </c>
       <c r="I147" s="61" t="inlineStr">
@@ -29114,7 +29114,7 @@
       </c>
       <c r="N148" s="61" t="inlineStr">
         <is>
-          <t>Si fallaste en algo que enseñás, reconocelo delante de quien acompañás.</t>
+          <t>Delante de quien acompañás, reconocé si fallaste en algo que enseñás.</t>
         </is>
       </c>
     </row>
@@ -29224,7 +29224,7 @@
       </c>
       <c r="H150" s="61" t="inlineStr">
         <is>
-          <t>Elegí una enseñanza que recibiste y ponela en práctica esta semana.</t>
+          <t>Poné en práctica esta semana una enseñanza que recibiste.</t>
         </is>
       </c>
       <c r="I150" s="61" t="inlineStr">
@@ -29249,7 +29249,7 @@
       </c>
       <c r="M150" s="61" t="inlineStr">
         <is>
-          <t>Pensar que discipular es una tarea solo de pastores.</t>
+          <t>“Discipular es tarea de los pastores, no mía”.</t>
         </is>
       </c>
       <c r="N150" s="61" t="inlineStr">
@@ -29290,7 +29290,7 @@
       <c r="G151" s="61" t="n"/>
       <c r="H151" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, elegí a una persona para acompañar en la fe durante el próximo mes, y anotá cuándo la vas a llamar.</t>
+          <t>Elegí a una persona para acompañar en la fe durante el próximo mes, y anotá cuándo la vas a llamar.</t>
         </is>
       </c>
       <c r="I151" s="61" t="inlineStr">
@@ -29414,7 +29414,7 @@
       </c>
       <c r="H153" s="61" t="inlineStr">
         <is>
-          <t>Si escuchás un chisme sobre alguien del equipo, cortalo y hablá con la persona.</t>
+          <t>Cortá el chisme que escuches sobre alguien del equipo, y hablá con la persona.</t>
         </is>
       </c>
       <c r="I153" s="61" t="inlineStr">
@@ -29429,7 +29429,7 @@
       </c>
       <c r="K153" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, tené paciencia con alguien del equipo que está aprendiendo, y decile qué está haciendo bien.</t>
+          <t>Con un compañero que está aprendiendo, tené paciencia y decile qué está haciendo bien.</t>
         </is>
       </c>
       <c r="L153" s="61" t="inlineStr">
@@ -29484,7 +29484,7 @@
       </c>
       <c r="H154" s="61" t="inlineStr">
         <is>
-          <t>Antes de una decisión que afecta al equipo, consultá a dos o tres personas.</t>
+          <t>Consultá a dos o tres personas cada vez que una decisión afecte al equipo.</t>
         </is>
       </c>
       <c r="I154" s="61" t="inlineStr">
@@ -29584,7 +29584,7 @@
       </c>
       <c r="N155" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, cubrí a un compañero en algo que le está costando.</t>
+          <t>Cubrí a un compañero en algo que le está costando.</t>
         </is>
       </c>
     </row>
@@ -29624,7 +29624,7 @@
       </c>
       <c r="H156" s="61" t="inlineStr">
         <is>
-          <t>Antes de corregir, preguntate: ¿esto ayuda a la persona a crecer?</t>
+          <t>Para corregir bien, primero preguntate: ¿esto ayuda a la persona a crecer?</t>
         </is>
       </c>
       <c r="I156" s="61" t="inlineStr">
@@ -29744,7 +29744,7 @@
       </c>
       <c r="H158" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, hacé algo concreto por tu cuadra: saludá al vecino nuevo, limpiá la vereda o ayudá a alguien mayor.</t>
+          <t>Por tu cuadra, algo concreto: saludá al vecino nuevo, limpiá la vereda o ayudá a alguien mayor.</t>
         </is>
       </c>
       <c r="I158" s="61" t="inlineStr">
@@ -29824,7 +29824,7 @@
       </c>
       <c r="J159" s="61" t="inlineStr">
         <is>
-          <t>Pensar que respetar a la autoridad significa aprobar todo lo que hace o callar ante una injusticia.</t>
+          <t>Confundir respetar a la autoridad con aprobar todo lo que hace o callar ante una injusticia.</t>
         </is>
       </c>
       <c r="K159" s="61" t="inlineStr">
@@ -30139,7 +30139,7 @@
       </c>
       <c r="G164" s="61" t="inlineStr">
         <is>
-          <t>Pensar que administrar bien o invertir es solo cosa de ricos.</t>
+          <t>¿Administrar bien o invertir? Parece cosa de ricos.</t>
         </is>
       </c>
       <c r="H164" s="61" t="inlineStr">
@@ -30229,7 +30229,7 @@
       </c>
       <c r="K165" s="61" t="inlineStr">
         <is>
-          <t>Antes de invertir, pedí consejo a un profesional de confianza, como un contador o un asesor financiero.</t>
+          <t>Pedí consejo a un profesional de confianza, como un contador o un asesor financiero, antes de invertir.</t>
         </is>
       </c>
       <c r="L165" s="61" t="inlineStr">
@@ -30244,7 +30244,7 @@
       </c>
       <c r="N165" s="61" t="inlineStr">
         <is>
-          <t>Antes de pensar en invertir, asegurate de tener cubiertos la comida, el alquiler y las deudas de tu casa.</t>
+          <t>Primero la comida, el alquiler y las deudas de tu casa: asegurate de tenerlos cubiertos antes de pensar en invertir.</t>
         </is>
       </c>
     </row>
@@ -30299,7 +30299,7 @@
       </c>
       <c r="K166" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, aprendé un concepto financiero básico con una fuente seria, como los materiales de educación financiera del Banco Central del Paraguay.</t>
+          <t>Aprendé un concepto financiero básico con una fuente seria, como los materiales de educación financiera del Banco Central del Paraguay.</t>
         </is>
       </c>
       <c r="L166" s="61" t="inlineStr">
@@ -30314,7 +30314,7 @@
       </c>
       <c r="N166" s="61" t="inlineStr">
         <is>
-          <t>Si estás pensando en invertir, conversalo primero con un profesional de confianza.</t>
+          <t>¿Pensás invertir? Conversalo primero con un profesional de confianza.</t>
         </is>
       </c>
     </row>
@@ -30349,7 +30349,7 @@
       </c>
       <c r="G167" s="61" t="inlineStr">
         <is>
-          <t>Creer que un error con la plata te descalifica para siempre.</t>
+          <t>La vergüenza de un error con la plata, como si te descalificara para siempre.</t>
         </is>
       </c>
       <c r="H167" s="61" t="inlineStr">
@@ -30369,7 +30369,7 @@
       </c>
       <c r="K167" s="61" t="inlineStr">
         <is>
-          <t>Si querés invertir, empezá con un monto chico y aprendé en el camino.</t>
+          <t>Empezá con un monto chico si querés invertir, y aprendé en el camino.</t>
         </is>
       </c>
       <c r="L167" s="61" t="inlineStr">
@@ -30439,7 +30439,7 @@
       </c>
       <c r="K168" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, invertí tiempo en tu familia con la misma seriedad con que cuidás tu dinero.</t>
+          <t>Invertí tiempo en tu familia con la misma seriedad con que cuidás tu dinero.</t>
         </is>
       </c>
       <c r="L168" s="61" t="inlineStr">
@@ -30490,7 +30490,7 @@
       <c r="G169" s="61" t="n"/>
       <c r="H169" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, siéntense en familia, definan una meta de ahorro con un propósito y, antes de cualquier inversión, pidan consejo a un profesional.</t>
+          <t>En familia, siéntense a definir una meta de ahorro con un propósito y, antes de cualquier inversión, pidan consejo a un profesional.</t>
         </is>
       </c>
       <c r="I169" s="61" t="inlineStr">
@@ -30679,12 +30679,12 @@
       </c>
       <c r="G172" s="61" t="inlineStr">
         <is>
-          <t>Pensar que si algo no se dio, fue porque no oramos lo suficiente.</t>
+          <t>La culpa de pensar que, si algo no se dio, fue por no orar lo suficiente.</t>
         </is>
       </c>
       <c r="H172" s="61" t="inlineStr">
         <is>
-          <t>Antes de armar tu plan, presentáselo a Dios en oración.</t>
+          <t>Presentale a Dios tu plan en oración, antes de armarlo.</t>
         </is>
       </c>
       <c r="I172" s="61" t="inlineStr">
@@ -30714,7 +30714,7 @@
       </c>
       <c r="N172" s="61" t="inlineStr">
         <is>
-          <t>Elegí un día de la semana para revisar tu avance, aunque sea cinco minutos.</t>
+          <t>Cinco minutos alcanzan: fijá un día de la semana para revisar tu avance.</t>
         </is>
       </c>
     </row>
@@ -30890,7 +30890,7 @@
       <c r="G175" s="61" t="n"/>
       <c r="H175" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, escribí una meta concreta, sus tres primeros pasos y el día en que vas a revisarla, y entregásela a Dios diciendo: «Si el Señor quiere».</t>
+          <t>El desafío: escribí una meta concreta, sus tres primeros pasos y el día en que vas a revisarla, y entregásela a Dios diciendo: «Si el Señor quiere».</t>
         </is>
       </c>
       <c r="I175" s="61" t="inlineStr">
@@ -30944,7 +30944,7 @@
       </c>
       <c r="H176" s="61" t="inlineStr">
         <is>
-          <t>Si vendés, revisá hoy tus balanzas, tus medidas y tus precios.</t>
+          <t>Balanzas, medidas y precios: si vendés, revisalos hoy.</t>
         </is>
       </c>
       <c r="I176" s="61" t="inlineStr">
@@ -31014,7 +31014,7 @@
       </c>
       <c r="H177" s="61" t="inlineStr">
         <is>
-          <t>Si cambiaste algo de tu producto, avisale al cliente.</t>
+          <t>Avisale al cliente si cambiaste algo de tu producto.</t>
         </is>
       </c>
       <c r="I177" s="61" t="inlineStr">
@@ -31084,7 +31084,7 @@
       </c>
       <c r="H178" s="61" t="inlineStr">
         <is>
-          <t>Si negociás un precio, hacelo con respeto, sin desmerecer el producto.</t>
+          <t>Al negociar un precio, hacelo con respeto, sin desmerecer el producto.</t>
         </is>
       </c>
       <c r="I178" s="61" t="inlineStr">
@@ -31094,12 +31094,12 @@
       </c>
       <c r="J178" s="61" t="inlineStr">
         <is>
-          <t>Pensar que comprar en el barrio o en otro lado da lo mismo.</t>
+          <t>“Da igual dónde compre”.</t>
         </is>
       </c>
       <c r="K178" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, cuando puedas, hacé tus compras en un comercio de tu zona.</t>
+          <t>Cuando puedas, hacé tus compras en un comercio de tu zona.</t>
         </is>
       </c>
       <c r="L178" s="61" t="inlineStr">
@@ -31224,7 +31224,7 @@
       </c>
       <c r="H180" s="61" t="inlineStr">
         <is>
-          <t>Si tenés un emprendimiento, respondé hoy los mensajes pendientes de tus clientes.</t>
+          <t>Respondé hoy los mensajes pendientes de los clientes de tu emprendimiento.</t>
         </is>
       </c>
       <c r="I180" s="61" t="inlineStr">
@@ -31414,7 +31414,7 @@
       </c>
       <c r="H183" s="61" t="inlineStr">
         <is>
-          <t>Antes de dormir, entregale a Dios en oración lo que te preocupa, por nombre.</t>
+          <t>Esta noche, al acostarte, entregale a Dios en oración lo que te preocupa, por nombre.</t>
         </is>
       </c>
       <c r="I183" s="61" t="inlineStr">
@@ -31444,7 +31444,7 @@
       </c>
       <c r="N183" s="61" t="inlineStr">
         <is>
-          <t>Si hace semanas que dormís mal, consultá a un médico: pedir ayuda también es cuidar el cuerpo que Dios te dio.</t>
+          <t>Consultá a un médico si hace semanas que dormís mal: pedir ayuda también es cuidar el cuerpo que Dios te dio.</t>
         </is>
       </c>
     </row>
@@ -31479,7 +31479,7 @@
       </c>
       <c r="G184" s="61" t="inlineStr">
         <is>
-          <t>Pensar que mientras más ocupados, mejor estamos.</t>
+          <t>La costumbre de medir el bienestar por lo ocupados que andamos.</t>
         </is>
       </c>
       <c r="H184" s="61" t="inlineStr">
@@ -31514,7 +31514,7 @@
       </c>
       <c r="N184" s="61" t="inlineStr">
         <is>
-          <t>Si servís en tu iglesia, conversá con tu líder para organizar turnos y descansos.</t>
+          <t>Junto a tu líder, organizá turnos y descansos para tu servicio en la iglesia.</t>
         </is>
       </c>
     </row>
@@ -31639,7 +31639,7 @@
       </c>
       <c r="K186" s="61" t="inlineStr">
         <is>
-          <t>Elegí una hora fija para acostarte esta semana, también el fin de semana.</t>
+          <t>Fijá una hora para acostarte esta semana, también el fin de semana.</t>
         </is>
       </c>
       <c r="L186" s="61" t="inlineStr">
@@ -31654,7 +31654,7 @@
       </c>
       <c r="N186" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, apagá las pantallas 30 minutos antes de dormir.</t>
+          <t>Treinta minutos antes de dormir, apagá las pantallas.</t>
         </is>
       </c>
     </row>
@@ -31690,7 +31690,7 @@
       <c r="G187" s="61" t="n"/>
       <c r="H187" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, elegí un hábito de descanso y sostenelo siete días, y cada noche entregale a Dios tus preocupaciones.</t>
+          <t>Para los próximos siete días: elegí un hábito de descanso, sostenelo, y cada noche entregale a Dios tus preocupaciones.</t>
         </is>
       </c>
       <c r="I187" s="61" t="inlineStr">
@@ -31829,7 +31829,7 @@
       </c>
       <c r="K189" s="61" t="inlineStr">
         <is>
-          <t>Elegí un lugar fijo de tu casa para orar esta semana.</t>
+          <t>Buscá un lugar fijo de tu casa para orar esta semana.</t>
         </is>
       </c>
       <c r="L189" s="61" t="inlineStr">
@@ -31844,7 +31844,7 @@
       </c>
       <c r="N189" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, orá por alguien sin contárselo a nadie.</t>
+          <t>En lo secreto, orá por alguien sin contárselo a nadie.</t>
         </is>
       </c>
     </row>
@@ -31984,7 +31984,7 @@
       </c>
       <c r="N191" s="61" t="inlineStr">
         <is>
-          <t>Si estás pasando una temporada difícil, buscá a alguien de tu iglesia para orar juntos.</t>
+          <t>En esta temporada difícil, buscá a alguien de tu iglesia para orar juntos.</t>
         </is>
       </c>
     </row>
@@ -32090,7 +32090,7 @@
       <c r="G193" s="61" t="n"/>
       <c r="H193" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, orá cinco minutos por día en un lugar fijo, y al final de la semana anotá cómo te fue.</t>
+          <t>Orá cinco minutos por día en un lugar fijo, y al final de la semana anotá cómo te fue.</t>
         </is>
       </c>
       <c r="I193" s="61" t="inlineStr">
@@ -32144,7 +32144,7 @@
       </c>
       <c r="H194" s="61" t="inlineStr">
         <is>
-          <t>Si liderás algo, en casa, en el trabajo o en la iglesia, apartá hoy un tiempo para tu propia vida espiritual.</t>
+          <t>Vos que liderás, en casa, en el trabajo o en la iglesia, apartá hoy un tiempo para tu propia vida espiritual.</t>
         </is>
       </c>
       <c r="I194" s="61" t="inlineStr">
@@ -32354,7 +32354,7 @@
       </c>
       <c r="H197" s="61" t="inlineStr">
         <is>
-          <t>Elegí un tiempo fijo esta semana para leer la Biblia con calma.</t>
+          <t>Apartá un tiempo fijo esta semana para leer la Biblia con calma.</t>
         </is>
       </c>
       <c r="I197" s="61" t="inlineStr">
@@ -32369,7 +32369,7 @@
       </c>
       <c r="K197" s="61" t="inlineStr">
         <is>
-          <t>Hacé hoy el primer paso de tu meta, aunque sea pequeño.</t>
+          <t>Da hoy el primer paso de tu meta, aunque sea pequeño.</t>
         </is>
       </c>
       <c r="L197" s="61" t="inlineStr">
@@ -32490,7 +32490,7 @@
       <c r="G199" s="61" t="n"/>
       <c r="H199" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, compartí con tu familia o tu equipo la visión en una frase y los tres primeros pasos, y que el fruto apunte a la gloria de Dios.</t>
+          <t>Hasta el sábado que viene, compartí con tu familia o tu equipo la visión en una frase y los tres primeros pasos, y que el fruto apunte a la gloria de Dios.</t>
         </is>
       </c>
       <c r="I199" s="61" t="inlineStr">
@@ -32644,7 +32644,7 @@
       </c>
       <c r="N201" s="61" t="inlineStr">
         <is>
-          <t>Si heriste a alguien de tu casa con palabras, pedile perdón antes de orar esta noche.</t>
+          <t>Pedile perdón a quien heriste con palabras en tu casa, antes de orar esta noche.</t>
         </is>
       </c>
     </row>
@@ -32959,7 +32959,7 @@
       </c>
       <c r="K206" s="61" t="inlineStr">
         <is>
-          <t>Si tu pareja se equivocó con un gasto, háblenlo para buscar una salida, no para culpar.</t>
+          <t>Con tu pareja, hablen del gasto equivocado para buscar una salida, no para culpar.</t>
         </is>
       </c>
       <c r="L206" s="61" t="inlineStr">
@@ -33009,7 +33009,7 @@
       </c>
       <c r="G207" s="61" t="inlineStr">
         <is>
-          <t>Pensar que el problema es solo de los ricos.</t>
+          <t>“Ese problema es solo de los ricos”.</t>
         </is>
       </c>
       <c r="H207" s="61" t="inlineStr">
@@ -33029,7 +33029,7 @@
       </c>
       <c r="K207" s="61" t="inlineStr">
         <is>
-          <t>Antes de una compra grande, consultala con tu pareja.</t>
+          <t>Hablá con tu pareja antes de una compra grande.</t>
         </is>
       </c>
       <c r="L207" s="61" t="inlineStr">
@@ -33084,7 +33084,7 @@
       </c>
       <c r="H208" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, que tus hijos te vean dar algo con alegría.</t>
+          <t>Que tus hijos te vean dar algo con alegría.</t>
         </is>
       </c>
       <c r="I208" s="61" t="inlineStr">
@@ -33184,7 +33184,7 @@
       </c>
       <c r="N209" s="61" t="inlineStr">
         <is>
-          <t>Si tu hijo gastó todo, acompañalo sin retarlo y ayudalo a pensar qué haría distinto.</t>
+          <t>Acompañá sin retos a tu hijo que gastó todo, y ayudalo a pensar qué haría distinto.</t>
         </is>
       </c>
     </row>
@@ -33290,7 +33290,7 @@
       <c r="G211" s="61" t="n"/>
       <c r="H211" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, tengan en familia una conversación sobre la plata: qué tenemos, qué necesitamos y en qué estamos de acuerdo.</t>
+          <t>Una conversación en familia sobre la plata: qué tenemos, qué necesitamos y en qué estamos de acuerdo. Ese es el desafío de esta semana.</t>
         </is>
       </c>
       <c r="I211" s="61" t="inlineStr">
@@ -33344,7 +33344,7 @@
       </c>
       <c r="H212" s="61" t="inlineStr">
         <is>
-          <t>Elegí una tarea que venís postergando y hacela hoy, aunque no tengas ganas.</t>
+          <t>Aunque no tengas ganas, hacé hoy esa tarea que venís postergando.</t>
         </is>
       </c>
       <c r="I212" s="61" t="inlineStr">
@@ -33354,7 +33354,7 @@
       </c>
       <c r="J212" s="61" t="inlineStr">
         <is>
-          <t>Creer que la disciplina depende solo de uno y frustrarse al fallar.</t>
+          <t>La frustración de fallar cuando uno cree que la disciplina depende solo de sí mismo.</t>
         </is>
       </c>
       <c r="K212" s="61" t="inlineStr">
@@ -33444,7 +33444,7 @@
       </c>
       <c r="N213" s="61" t="inlineStr">
         <is>
-          <t>Antes de dormir, anotá tres cosas por las que das gracias.</t>
+          <t>Tres cosas por las que das gracias: anotalas hoy antes de dormir.</t>
         </is>
       </c>
     </row>
@@ -33484,7 +33484,7 @@
       </c>
       <c r="H214" s="61" t="inlineStr">
         <is>
-          <t>Elegí un solo hábito nuevo y fijale una hora y un lugar.</t>
+          <t>Un solo hábito nuevo alcanza: fijale una hora y un lugar.</t>
         </is>
       </c>
       <c r="I214" s="61" t="inlineStr">
@@ -33499,7 +33499,7 @@
       </c>
       <c r="K214" s="61" t="inlineStr">
         <is>
-          <t>Si dejaste un hábito, retomalo hoy sin culparte: un día perdido no borra el camino.</t>
+          <t>Retomá hoy, sin culparte, el hábito que dejaste: un día perdido no borra el camino.</t>
         </is>
       </c>
       <c r="L214" s="61" t="inlineStr">
@@ -33554,7 +33554,7 @@
       </c>
       <c r="H215" s="61" t="inlineStr">
         <is>
-          <t>Elegí un hábito espiritual pequeño, como leer un capítulo por día, y sostenelo esta semana.</t>
+          <t>Probá un hábito espiritual pequeño, como leer un capítulo por día, y sostenelo esta semana.</t>
         </is>
       </c>
       <c r="I215" s="61" t="inlineStr">
@@ -33624,7 +33624,7 @@
       </c>
       <c r="H216" s="61" t="inlineStr">
         <is>
-          <t>Elegí un solo hábito pequeño para sostener todo este mes.</t>
+          <t>Durante todo este mes, sostené un solo hábito pequeño.</t>
         </is>
       </c>
       <c r="I216" s="61" t="inlineStr">
@@ -33690,7 +33690,7 @@
       <c r="G217" s="61" t="n"/>
       <c r="H217" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, elegí un solo hábito pequeño, fijale hora y lugar, y marcá en un calendario cada día que lo cumplas.</t>
+          <t>Un solo hábito pequeño: elegilo, fijale hora y lugar, y marcá en un calendario cada día que lo cumplas.</t>
         </is>
       </c>
       <c r="I217" s="61" t="inlineStr">
@@ -33744,7 +33744,7 @@
       </c>
       <c r="H218" s="61" t="inlineStr">
         <is>
-          <t>Pensá en una necesidad de tu barrio o de tu trabajo que se podría resolver mejor entre varios.</t>
+          <t>Mirá a tu alrededor: ¿qué necesidad de tu barrio o de tu trabajo se podría resolver mejor entre varios?</t>
         </is>
       </c>
       <c r="I218" s="61" t="inlineStr">
@@ -33839,7 +33839,7 @@
       </c>
       <c r="M219" s="61" t="inlineStr">
         <is>
-          <t>Pensar que lo que yo sé hacer no le sirve a nadie.</t>
+          <t>“Lo que yo sé hacer no le sirve a nadie”.</t>
         </is>
       </c>
       <c r="N219" s="61" t="inlineStr">
@@ -33884,7 +33884,7 @@
       </c>
       <c r="H220" s="61" t="inlineStr">
         <is>
-          <t>Si sos socio de una cooperativa, participá de la próxima asamblea.</t>
+          <t>Participá de la próxima asamblea de tu cooperativa, si sos socio.</t>
         </is>
       </c>
       <c r="I220" s="61" t="inlineStr">
@@ -34024,7 +34024,7 @@
       </c>
       <c r="H222" s="61" t="inlineStr">
         <is>
-          <t>Si manejás algo de un grupo, plata o herramientas, rendí cuentas aunque nadie te lo pida.</t>
+          <t>Rendí cuentas de lo que manejás de un grupo, plata o herramientas, aunque nadie te lo pida.</t>
         </is>
       </c>
       <c r="I222" s="61" t="inlineStr">
@@ -34229,7 +34229,7 @@
       </c>
       <c r="K225" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, preparen en familia una comida casera con verduras.</t>
+          <t>En familia, preparen una comida casera con verduras.</t>
         </is>
       </c>
       <c r="L225" s="61" t="inlineStr">
@@ -34279,7 +34279,7 @@
       </c>
       <c r="G226" s="61" t="inlineStr">
         <is>
-          <t>Pensar que los adolescentes «están bien» solo porque tienen energía.</t>
+          <t>Dar por hecho que los adolescentes «están bien» solo porque tienen energía.</t>
         </is>
       </c>
       <c r="H226" s="61" t="inlineStr">
@@ -34354,7 +34354,7 @@
       </c>
       <c r="H227" s="61" t="inlineStr">
         <is>
-          <t>Si sos joven, elegí un hábito de cuidado: dormir mejor, moverte o comer más sano.</t>
+          <t>Siendo joven, sumá un hábito de cuidado: dormir mejor, moverte o comer más sano.</t>
         </is>
       </c>
       <c r="I227" s="61" t="inlineStr">
@@ -34490,7 +34490,7 @@
       <c r="G229" s="61" t="n"/>
       <c r="H229" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, revisá los controles de salud de cada uno en tu casa, empezando por el tuyo, y agenden lo que falte.</t>
+          <t>Revisá estos días los controles de salud de cada uno en tu casa, empezando por el tuyo, y agenden lo que falte.</t>
         </is>
       </c>
       <c r="I229" s="61" t="inlineStr">
@@ -34559,7 +34559,7 @@
       </c>
       <c r="K230" s="61" t="inlineStr">
         <is>
-          <t>Hacé hoy una buena obra, no para demostrar nada, sino como respuesta de gratitud.</t>
+          <t>Como respuesta de gratitud, no para demostrar nada, hacé hoy una buena obra.</t>
         </is>
       </c>
       <c r="L230" s="61" t="inlineStr">
@@ -34784,7 +34784,7 @@
       </c>
       <c r="N233" s="61" t="inlineStr">
         <is>
-          <t>Antes de una decisión importante, recordá en voz alta: «Cristo me amó y se entregó por mí».</t>
+          <t>Recordá en voz alta, frente a una decisión importante: «Cristo me amó y se entregó por mí».</t>
         </is>
       </c>
     </row>
@@ -34834,7 +34834,7 @@
       </c>
       <c r="J234" s="61" t="inlineStr">
         <is>
-          <t>Creer que si sos hijo de Dios no deberías sufrir.</t>
+          <t>“Si soy hijo de Dios, no debería sufrir”.</t>
         </is>
       </c>
       <c r="K234" s="61" t="inlineStr">
@@ -34890,7 +34890,7 @@
       <c r="G235" s="61" t="n"/>
       <c r="H235" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, escribí tres cosas que Dios dice de vos en su Palabra y leelas cada mañana.</t>
+          <t>Escribí tres cosas que Dios dice de vos en su Palabra y leelas cada mañana de esta semana.</t>
         </is>
       </c>
       <c r="I235" s="61" t="inlineStr">
@@ -34974,7 +34974,7 @@
       </c>
       <c r="N236" s="61" t="inlineStr">
         <is>
-          <t>Si tenés que corregir algo en tu equipo o en tu casa, hacelo con firmeza y sin humillar.</t>
+          <t>Corregí con firmeza y sin humillar cuando tengas que hacerlo en tu equipo o en tu casa.</t>
         </is>
       </c>
     </row>
@@ -35014,7 +35014,7 @@
       </c>
       <c r="H237" s="61" t="inlineStr">
         <is>
-          <t>Pensá en un proyecto atascado y en quién podría sumarse si lo invitás.</t>
+          <t>Repasá un proyecto atascado: ¿quién podría sumarse si lo invitás?</t>
         </is>
       </c>
       <c r="I237" s="61" t="inlineStr">
@@ -35079,7 +35079,7 @@
       </c>
       <c r="G238" s="61" t="inlineStr">
         <is>
-          <t>Pensar que sin recursos no se puede emprender nada que valga la pena.</t>
+          <t>Creer que sin recursos es imposible emprender algo que valga la pena.</t>
         </is>
       </c>
       <c r="H238" s="61" t="inlineStr">
@@ -35154,7 +35154,7 @@
       </c>
       <c r="H239" s="61" t="inlineStr">
         <is>
-          <t>Hacé hoy una tarea de servicio que nadie quiere hacer en tu casa o en tu trabajo.</t>
+          <t>En tu casa o en tu trabajo, ocupate hoy de la tarea de servicio que nadie quiere hacer.</t>
         </is>
       </c>
       <c r="I239" s="61" t="inlineStr">
@@ -35359,7 +35359,7 @@
       </c>
       <c r="K242" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, hagan en familia una lista de todas las tareas de la casa, también las que no se ven.</t>
+          <t>Armen en familia una lista de todas las tareas de la casa, también las que no se ven.</t>
         </is>
       </c>
       <c r="L242" s="61" t="inlineStr">
@@ -35409,7 +35409,7 @@
       </c>
       <c r="G243" s="61" t="inlineStr">
         <is>
-          <t>Pensar que quien trae el sueldo ya cumplió con todo.</t>
+          <t>El que trae el sueldo y siente que ya cumplió con todo.</t>
         </is>
       </c>
       <c r="H243" s="61" t="inlineStr">
@@ -35429,7 +35429,7 @@
       </c>
       <c r="K243" s="61" t="inlineStr">
         <is>
-          <t>Si alguien de tu familia está sin trabajo, acompañalo y ayudalo a buscar, sin reproches.</t>
+          <t>Al familiar que está sin trabajo, acompañalo y ayudalo a buscar, sin reproches.</t>
         </is>
       </c>
       <c r="L243" s="61" t="inlineStr">
@@ -35624,7 +35624,7 @@
       </c>
       <c r="H246" s="61" t="inlineStr">
         <is>
-          <t>Antes de decidir algo de la casa, preguntá: ¿qué pensás vos?</t>
+          <t>En las decisiones de la casa, preguntá primero: ¿qué pensás vos?</t>
         </is>
       </c>
       <c r="I246" s="61" t="inlineStr">
@@ -35690,7 +35690,7 @@
       <c r="G247" s="61" t="n"/>
       <c r="H247" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, hagan juntos la lista de tareas de la casa, repártanla conversando y agradezcan en voz alta lo que hace cada uno.</t>
+          <t>En casa, hagan juntos la lista de tareas, repártanla conversando y agradezcan en voz alta lo que hace cada uno.</t>
         </is>
       </c>
       <c r="I247" s="61" t="inlineStr">
@@ -35744,7 +35744,7 @@
       </c>
       <c r="H248" s="61" t="inlineStr">
         <is>
-          <t>Antes de gastar tu próximo ingreso, separá primero lo que vas a dar.</t>
+          <t>Separá primero lo que vas a dar, antes de gastar tu próximo ingreso.</t>
         </is>
       </c>
       <c r="I248" s="61" t="inlineStr">
@@ -35814,7 +35814,7 @@
       </c>
       <c r="H249" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, poné a Dios primero también en tu presupuesto.</t>
+          <t>Poné a Dios primero también en tu presupuesto.</t>
         </is>
       </c>
       <c r="I249" s="61" t="inlineStr">
@@ -35824,12 +35824,12 @@
       </c>
       <c r="J249" s="61" t="inlineStr">
         <is>
-          <t>Pensar que si alguien pasa necesidad es porque no dio lo suficiente.</t>
+          <t>La sospecha de que, si alguien pasa necesidad, es porque no dio lo suficiente.</t>
         </is>
       </c>
       <c r="K249" s="61" t="inlineStr">
         <is>
-          <t>Si conocés a alguien generoso que pasa un momento difícil, acompañalo sin juzgarlo.</t>
+          <t>Acompañá sin juzgar a esa persona generosa que pasa un momento difícil.</t>
         </is>
       </c>
       <c r="L249" s="61" t="inlineStr">
@@ -36019,7 +36019,7 @@
       </c>
       <c r="G252" s="61" t="inlineStr">
         <is>
-          <t>Pensar que, si no tengo plata, no tengo nada para dar.</t>
+          <t>“No tengo plata, entonces no tengo nada para dar”.</t>
         </is>
       </c>
       <c r="H252" s="61" t="inlineStr">
@@ -36090,7 +36090,7 @@
       <c r="G253" s="61" t="n"/>
       <c r="H253" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, da algo que no sea dinero: tu tiempo, un consejo o una habilidad, a alguien que lo necesite.</t>
+          <t>Antes del próximo sábado, da algo que no sea dinero: tu tiempo, un consejo o una habilidad, a alguien que lo necesite.</t>
         </is>
       </c>
       <c r="I253" s="61" t="inlineStr">
@@ -36139,7 +36139,7 @@
       </c>
       <c r="G254" s="61" t="inlineStr">
         <is>
-          <t>Pensar que el legado es solo dejar bienes.</t>
+          <t>Reducir el legado a dejar bienes.</t>
         </is>
       </c>
       <c r="H254" s="61" t="inlineStr">
@@ -36214,7 +36214,7 @@
       </c>
       <c r="H255" s="61" t="inlineStr">
         <is>
-          <t>Elegí un compromiso que dejaste a medias y retomalo esta semana.</t>
+          <t>Retomá esta semana un compromiso que dejaste a medias.</t>
         </is>
       </c>
       <c r="I255" s="61" t="inlineStr">
@@ -36229,7 +36229,7 @@
       </c>
       <c r="K255" s="61" t="inlineStr">
         <is>
-          <t>Si tropezaste, pedí perdón y seguí corriendo.</t>
+          <t>¿Tropezaste? Pedí perdón y seguí corriendo.</t>
         </is>
       </c>
       <c r="L255" s="61" t="inlineStr">
@@ -36244,7 +36244,7 @@
       </c>
       <c r="N255" s="61" t="inlineStr">
         <is>
-          <t>Elegí a una persona más joven para acompañarla en la fe este año.</t>
+          <t>Buscá a una persona más joven para acompañarla en la fe este año.</t>
         </is>
       </c>
     </row>
@@ -36354,7 +36354,7 @@
       </c>
       <c r="H257" s="61" t="inlineStr">
         <is>
-          <t>Hacé hoy algo bueno por alguien sin que nadie se entere.</t>
+          <t>Sin que nadie se entere, hacé hoy algo bueno por alguien.</t>
         </is>
       </c>
       <c r="I257" s="61" t="inlineStr">
@@ -36369,7 +36369,7 @@
       </c>
       <c r="K257" s="61" t="inlineStr">
         <is>
-          <t>Si te cuesta seguir, buscá ayuda hoy: hablá con alguien de confianza o acercate a un centro de salud.</t>
+          <t>Buscá ayuda hoy si te cuesta seguir: hablá con alguien de confianza o acercate a un centro de salud.</t>
         </is>
       </c>
       <c r="L257" s="61" t="inlineStr">
@@ -36424,7 +36424,7 @@
       </c>
       <c r="H258" s="61" t="inlineStr">
         <is>
-          <t>Si alguien te cuenta un dolor, escuchá primero, antes de dar explicaciones.</t>
+          <t>Escuchá primero cuando alguien te cuenta un dolor, antes de dar explicaciones.</t>
         </is>
       </c>
       <c r="I258" s="61" t="inlineStr">
@@ -36454,7 +36454,7 @@
       </c>
       <c r="N258" s="61" t="inlineStr">
         <is>
-          <t>Pensá en una herida familiar que no querés pasarles a tus hijos, y pedile a Dios ayuda para sanarla.</t>
+          <t>Pedile a Dios ayuda para sanar esa herida familiar que no querés pasarles a tus hijos.</t>
         </is>
       </c>
     </row>
@@ -36490,7 +36490,7 @@
       <c r="G259" s="61" t="n"/>
       <c r="H259" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, escribile una carta o un mensaje a alguien más joven contándole lo que aprendiste de Dios y lo que te gustaría que recuerde.</t>
+          <t>Durante estos días, escribile una carta o un mensaje a alguien más joven contándole lo que aprendiste de Dios y lo que te gustaría que recuerde.</t>
         </is>
       </c>
       <c r="I259" s="61" t="inlineStr">
@@ -36714,7 +36714,7 @@
       </c>
       <c r="N262" s="61" t="inlineStr">
         <is>
-          <t>Si estás en una situación difícil, animate a pedir ayuda a tu iglesia o a tu familia.</t>
+          <t>Animate a pedir ayuda a tu iglesia o a tu familia en esta situación difícil.</t>
         </is>
       </c>
     </row>
@@ -36749,7 +36749,7 @@
       </c>
       <c r="G263" s="61" t="inlineStr">
         <is>
-          <t>Pensar que un trabajo sencillo no da ningún fruto.</t>
+          <t>La sensación de que un trabajo sencillo no da ningún fruto.</t>
         </is>
       </c>
       <c r="H263" s="61" t="inlineStr">
@@ -36839,7 +36839,7 @@
       </c>
       <c r="K264" s="61" t="inlineStr">
         <is>
-          <t>Hacé hoy tu trabajo con excelencia, aunque nadie lo valore.</t>
+          <t>Trabajá hoy con excelencia, aunque nadie lo valore.</t>
         </is>
       </c>
       <c r="L264" s="61" t="inlineStr">
@@ -36939,7 +36939,7 @@
       </c>
       <c r="G266" s="61" t="inlineStr">
         <is>
-          <t>Pensar que la fe nos exime de prepararnos.</t>
+          <t>Confundir la fe con una excusa para no prepararnos.</t>
         </is>
       </c>
       <c r="H266" s="61" t="inlineStr">
@@ -36954,7 +36954,7 @@
       </c>
       <c r="J266" s="61" t="inlineStr">
         <is>
-          <t>Creer que solo los médicos pueden ayudar.</t>
+          <t>La idea de que solo los médicos pueden ayudar.</t>
         </is>
       </c>
       <c r="K266" s="61" t="inlineStr">
@@ -37029,7 +37029,7 @@
       </c>
       <c r="K267" s="61" t="inlineStr">
         <is>
-          <t>Si hay varias personas, señalá a una y pedile directamente que llame a emergencias.</t>
+          <t>Señalá a una persona entre varias y pedile directamente que llame a emergencias.</t>
         </is>
       </c>
       <c r="L267" s="61" t="inlineStr">
@@ -37164,12 +37164,12 @@
       </c>
       <c r="J269" s="61" t="inlineStr">
         <is>
-          <t>Pensar que si algo malo pasó es porque Dios no escuchó.</t>
+          <t>“Si pasó algo malo, es porque Dios no me escuchó”.</t>
         </is>
       </c>
       <c r="K269" s="61" t="inlineStr">
         <is>
-          <t>Si estás pasando una angustia, contásela hoy a Dios y a alguien de confianza.</t>
+          <t>Hoy mismo, contale tu angustia a Dios y a alguien de confianza.</t>
         </is>
       </c>
       <c r="L269" s="61" t="inlineStr">
@@ -37290,7 +37290,7 @@
       <c r="G271" s="61" t="n"/>
       <c r="H271" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, anoten en familia los números de emergencia, pónganlos en un lugar visible y averigüen dónde hacer un curso de primeros auxilios.</t>
+          <t>En familia, anoten los números de emergencia, pónganlos en un lugar visible y averigüen dónde hacer un curso de primeros auxilios.</t>
         </is>
       </c>
       <c r="I271" s="61" t="inlineStr">
@@ -37414,7 +37414,7 @@
       </c>
       <c r="H273" s="61" t="inlineStr">
         <is>
-          <t>Elegí una situación difícil de esta semana y agradecele a Dios en medio de ella.</t>
+          <t>En medio de una situación difícil de esta semana, agradecele a Dios.</t>
         </is>
       </c>
       <c r="I273" s="61" t="inlineStr">
@@ -37429,7 +37429,7 @@
       </c>
       <c r="K273" s="61" t="inlineStr">
         <is>
-          <t>Si estás triste, contáselo a Dios con sinceridad: eso también es adoración.</t>
+          <t>Contale a Dios con sinceridad tu tristeza: eso también es adoración.</t>
         </is>
       </c>
       <c r="L273" s="61" t="inlineStr">
@@ -37444,7 +37444,7 @@
       </c>
       <c r="N273" s="61" t="inlineStr">
         <is>
-          <t>Antes de pensar hoy en tu problema, pensá en tres cosas que Dios es.</t>
+          <t>Hoy, antes de pensar en tu problema, recordá tres cosas que Dios es.</t>
         </is>
       </c>
     </row>
@@ -37549,7 +37549,7 @@
       </c>
       <c r="G275" s="61" t="inlineStr">
         <is>
-          <t>Pensar que la alabanza es solo para los que cantan bien.</t>
+          <t>¿Alabar a Dios? Eso parece solo para los que cantan bien.</t>
         </is>
       </c>
       <c r="H275" s="61" t="inlineStr">
@@ -37639,7 +37639,7 @@
       </c>
       <c r="K276" s="61" t="inlineStr">
         <is>
-          <t>Elegí un momento fijo del día para adorar, aunque sean dos minutos.</t>
+          <t>Separá un momento fijo del día para adorar, aunque sean dos minutos.</t>
         </is>
       </c>
       <c r="L276" s="61" t="inlineStr">
@@ -37654,7 +37654,7 @@
       </c>
       <c r="N276" s="61" t="inlineStr">
         <is>
-          <t>Hacé hoy un bien concreto como parte de tu adoración.</t>
+          <t>Ofrecé hoy un bien concreto como parte de tu adoración.</t>
         </is>
       </c>
     </row>
@@ -37690,7 +37690,7 @@
       <c r="G277" s="61" t="n"/>
       <c r="H277" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, empezá cada día con una frase de alabanza y cerralo anotando tres cosas por las que das gracias.</t>
+          <t>Cada día de esta semana, empezá con una frase de alabanza y cerrá anotando tres cosas por las que das gracias.</t>
         </is>
       </c>
       <c r="I277" s="61" t="inlineStr">
@@ -37759,7 +37759,7 @@
       </c>
       <c r="K278" s="61" t="inlineStr">
         <is>
-          <t>Antes de decidir algo hoy, hacé una oración corta pidiendo sabiduría.</t>
+          <t>Una oración corta pidiendo sabiduría: hacela hoy antes de decidir algo.</t>
         </is>
       </c>
       <c r="L278" s="61" t="inlineStr">
@@ -37839,7 +37839,7 @@
       </c>
       <c r="M279" s="61" t="inlineStr">
         <is>
-          <t>Pensar que una mala decisión arruina todo para siempre.</t>
+          <t>El miedo a que una mala decisión arruine todo para siempre.</t>
         </is>
       </c>
       <c r="N279" s="61" t="inlineStr">
@@ -37984,7 +37984,7 @@
       </c>
       <c r="N281" s="61" t="inlineStr">
         <is>
-          <t>Si sabés qué es lo correcto, decidilo hoy.</t>
+          <t>Si ya sabés qué es lo correcto, decidilo hoy.</t>
         </is>
       </c>
     </row>
@@ -38024,7 +38024,7 @@
       </c>
       <c r="H282" s="61" t="inlineStr">
         <is>
-          <t>Antes de una decisión que afecta a tu familia o a tu equipo, orá por ellos.</t>
+          <t>Orá por tu familia o por tu equipo antes de tomar una decisión que los afecte.</t>
         </is>
       </c>
       <c r="I282" s="61" t="inlineStr">
@@ -38054,7 +38054,7 @@
       </c>
       <c r="N282" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, tomá una decisión de la casa conversándola con tu familia.</t>
+          <t>Conversá con tu familia la próxima decisión de la casa y tómenla juntos.</t>
         </is>
       </c>
     </row>
@@ -38244,7 +38244,7 @@
       </c>
       <c r="N285" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, contale a tu familia una historia de cómo Dios te ayudó.</t>
+          <t>Contale a tu familia una historia de cómo Dios te ayudó.</t>
         </is>
       </c>
     </row>
@@ -38349,7 +38349,7 @@
       </c>
       <c r="G287" s="61" t="inlineStr">
         <is>
-          <t>Pensar que la fe de un padre alcanza automáticamente a los hijos.</t>
+          <t>Dar por sentado que la fe de un padre alcanza automáticamente a los hijos.</t>
         </is>
       </c>
       <c r="H287" s="61" t="inlineStr">
@@ -38384,7 +38384,7 @@
       </c>
       <c r="N287" s="61" t="inlineStr">
         <is>
-          <t>Si un hijo se alejó, mantené la puerta abierta: más amor y menos reproches.</t>
+          <t>Mantené la puerta abierta al hijo que se alejó: más amor y menos reproches.</t>
         </is>
       </c>
     </row>
@@ -38449,7 +38449,7 @@
       </c>
       <c r="M288" s="61" t="inlineStr">
         <is>
-          <t>Pensar que un hogar cristiano no tiene problemas.</t>
+          <t>La ilusión de que un hogar cristiano no tiene problemas.</t>
         </is>
       </c>
       <c r="N288" s="61" t="inlineStr">
@@ -38490,7 +38490,7 @@
       <c r="G289" s="61" t="n"/>
       <c r="H289" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, empiecen un devocional de cinco minutos en familia: un versículo, una pregunta y una oración.</t>
+          <t>Para los próximos siete días, un devocional de cinco minutos en familia: un versículo, una pregunta y una oración.</t>
         </is>
       </c>
       <c r="I289" s="61" t="inlineStr">
@@ -38539,7 +38539,7 @@
       </c>
       <c r="G290" s="61" t="inlineStr">
         <is>
-          <t>Pensar que toda deuda es pecado, o que ninguna es peligrosa.</t>
+          <t>Los dos extremos: creer que toda deuda es pecado, o que ninguna es peligrosa.</t>
         </is>
       </c>
       <c r="H290" s="61" t="inlineStr">
@@ -38559,7 +38559,7 @@
       </c>
       <c r="K290" s="61" t="inlineStr">
         <is>
-          <t>Antes de tomar una deuda, preguntate: ¿esto me ayuda a generar ingresos o es solo un gasto?</t>
+          <t>¿Te vas a endeudar? Preguntate primero: ¿esto me ayuda a generar ingresos o es solo un gasto?</t>
         </is>
       </c>
       <c r="L290" s="61" t="inlineStr">
@@ -38644,7 +38644,7 @@
       </c>
       <c r="N291" s="61" t="inlineStr">
         <is>
-          <t>Si querés ayudar, pensá qué podés dar sin poner en riesgo a tu familia.</t>
+          <t>Calculá qué podés dar para ayudar sin poner en riesgo a tu familia.</t>
         </is>
       </c>
     </row>
@@ -38684,7 +38684,7 @@
       </c>
       <c r="H292" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, mirá el total real de lo que debés, sin esconderlo.</t>
+          <t>Mirá el total real de lo que debés, sin esconderlo.</t>
         </is>
       </c>
       <c r="I292" s="61" t="inlineStr">
@@ -38749,7 +38749,7 @@
       </c>
       <c r="G293" s="61" t="inlineStr">
         <is>
-          <t>Creer que todo depende de uno, para bien o para mal.</t>
+          <t>“Todo depende de mí”, para bien o para mal.</t>
         </is>
       </c>
       <c r="H293" s="61" t="inlineStr">
@@ -38890,7 +38890,7 @@
       <c r="G295" s="61" t="n"/>
       <c r="H295" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, anotá todas tus deudas, elegí la primera para pagar y separá un monto pequeño para emergencias, poniendo a Dios primero.</t>
+          <t>Hasta el sábado que viene, anotá todas tus deudas, elegí la primera para pagar y separá un monto pequeño para emergencias, poniendo a Dios primero.</t>
         </is>
       </c>
       <c r="I295" s="61" t="inlineStr">
@@ -38974,7 +38974,7 @@
       </c>
       <c r="N296" s="61" t="inlineStr">
         <is>
-          <t>Si cargás con un error del pasado, confesáselo a Dios y recibí su perdón.</t>
+          <t>Confesale a Dios ese error del pasado que cargás, y recibí su perdón.</t>
         </is>
       </c>
     </row>
@@ -39014,7 +39014,7 @@
       </c>
       <c r="H297" s="61" t="inlineStr">
         <is>
-          <t>Elegí un paso pequeño e incómodo que venís postergando por miedo, y dalo esta semana.</t>
+          <t>¿Qué paso pequeño e incómodo venís postergando por miedo? Dalo esta semana.</t>
         </is>
       </c>
       <c r="I297" s="61" t="inlineStr">
@@ -39029,7 +39029,7 @@
       </c>
       <c r="K297" s="61" t="inlineStr">
         <is>
-          <t>Antes de un cambio, preguntale a alguien de confianza qué riesgos ve.</t>
+          <t>Preguntale a alguien de confianza qué riesgos ve en el cambio que estás por hacer.</t>
         </is>
       </c>
       <c r="L297" s="61" t="inlineStr">
@@ -39079,7 +39079,7 @@
       </c>
       <c r="G298" s="61" t="inlineStr">
         <is>
-          <t>Pensar que hay que estar contento con el dolor.</t>
+          <t>Confundir la fortaleza con tener que estar contento con el dolor.</t>
         </is>
       </c>
       <c r="H298" s="61" t="inlineStr">
@@ -39169,7 +39169,7 @@
       </c>
       <c r="K299" s="61" t="inlineStr">
         <is>
-          <t>Si empezaste algo nuevo, comprometete a sostenerlo un mes antes de evaluarlo.</t>
+          <t>Comprometete a sostener un mes lo nuevo que empezaste, antes de evaluarlo.</t>
         </is>
       </c>
       <c r="L299" s="61" t="inlineStr">
@@ -39239,7 +39239,7 @@
       </c>
       <c r="K300" s="61" t="inlineStr">
         <is>
-          <t>Elegí un área en la que querés crecer el año que viene.</t>
+          <t>Escribí un área en la que querés crecer el año que viene.</t>
         </is>
       </c>
       <c r="L300" s="61" t="inlineStr">
@@ -39290,7 +39290,7 @@
       <c r="G301" s="61" t="n"/>
       <c r="H301" s="61" t="inlineStr">
         <is>
-          <t>Esta semana, escribí tres cosas en las que creciste este año y una en la que querés crecer el próximo, y presentáselas a Dios.</t>
+          <t>Tomate un rato esta semana para escribir tres cosas en las que creciste este año y una en la que querés crecer el próximo, y presentáselas a Dios.</t>
         </is>
       </c>
       <c r="I301" s="61" t="inlineStr">
@@ -39344,7 +39344,7 @@
       </c>
       <c r="H302" s="61" t="inlineStr">
         <is>
-          <t>Pensá en una herramienta que podría ayudarte en tu trabajo sin cambiar lo esencial de lo que hacés.</t>
+          <t>Identificá una herramienta que podría ayudarte en tu trabajo sin cambiar lo esencial de lo que hacés.</t>
         </is>
       </c>
       <c r="I302" s="61" t="inlineStr">
@@ -39429,7 +39429,7 @@
       </c>
       <c r="K303" s="61" t="inlineStr">
         <is>
-          <t>Antes de usar una aplicación nueva, averiguá qué datos te pide y si es confiable.</t>
+          <t>Averiguá qué datos te pide una aplicación nueva y si es confiable, antes de usarla.</t>
         </is>
       </c>
       <c r="L303" s="61" t="inlineStr">
@@ -39584,7 +39584,7 @@
       </c>
       <c r="N305" s="61" t="inlineStr">
         <is>
-          <t>Antes de comprar una herramienta nueva, aprendé a usar bien la que ya tenés.</t>
+          <t>Aprendé a usar bien la herramienta que ya tenés antes de comprar una nueva.</t>
         </is>
       </c>
     </row>
@@ -39639,7 +39639,7 @@
       </c>
       <c r="K306" s="61" t="inlineStr">
         <is>
-          <t>Elegí un primer paso mínimo: aprender una sola función nueva esta semana.</t>
+          <t>Aprendé una sola función nueva esta semana: es un primer paso mínimo.</t>
         </is>
       </c>
       <c r="L306" s="61" t="inlineStr">
@@ -39739,7 +39739,7 @@
       </c>
       <c r="G308" s="61" t="inlineStr">
         <is>
-          <t>Pensar que estar sano es solo no tener un diagnóstico.</t>
+          <t>Confundir estar sano con no tener un diagnóstico.</t>
         </is>
       </c>
       <c r="H308" s="61" t="inlineStr">
@@ -39824,7 +39824,7 @@
       </c>
       <c r="J309" s="61" t="inlineStr">
         <is>
-          <t>Pensar que la tristeza profunda se cura solo con fuerza de voluntad.</t>
+          <t>La exigencia de curar la tristeza profunda solo con fuerza de voluntad.</t>
         </is>
       </c>
       <c r="K309" s="61" t="inlineStr">
@@ -39884,7 +39884,7 @@
       </c>
       <c r="H310" s="61" t="inlineStr">
         <is>
-          <t>Si tenés un control médico pendiente, agendalo esta semana.</t>
+          <t>Agendá esta semana ese control médico pendiente.</t>
         </is>
       </c>
       <c r="I310" s="61" t="inlineStr">
@@ -39969,7 +39969,7 @@
       </c>
       <c r="K311" s="61" t="inlineStr">
         <is>
-          <t>Si alguien está enfermo, acompañalo sin juzgar su fe.</t>
+          <t>Acompañá a quien está enfermo sin juzgar su fe.</t>
         </is>
       </c>
       <c r="L311" s="61" t="inlineStr">
@@ -40054,7 +40054,7 @@
       </c>
       <c r="N312" s="61" t="inlineStr">
         <is>
-          <t>Si tenés un tratamiento, seguilo con constancia y presentale cada día tu salud a Dios.</t>
+          <t>Seguí con constancia tu tratamiento y presentale cada día tu salud a Dios.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mensajero: 94 frases deportivas con arranques variados, Word actualizado y documentación de la vista liviana y la pasada de estilo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -40882,7 +40882,7 @@
       </c>
       <c r="D7" s="61" t="inlineStr">
         <is>
-          <t>En el futsal los cambios son constantes, y el que sale a descansar no abandona al equipo. Descansar no es perder el tiempo: es parte del diseño de Dios.</t>
+          <t>Cambio en el futsal: el que sale a descansar no abandona al equipo, y vuelve a entrar entero. Descansar no es perder el tiempo, es parte del diseño de Dios.</t>
         </is>
       </c>
     </row>
@@ -41002,7 +41002,7 @@
       </c>
       <c r="D13" s="61" t="inlineStr">
         <is>
-          <t>En el ajedrez, apurar una jugada suele costar caro. El agricultor espera la lluvia con paciencia; no se apura lo que necesita su tiempo.</t>
+          <t>Apurar una jugada de ajedrez suele costar caro. El agricultor espera la lluvia con paciencia: lo que necesita su tiempo no se apura.</t>
         </is>
       </c>
     </row>
@@ -41042,7 +41042,7 @@
       </c>
       <c r="D15" s="61" t="inlineStr">
         <is>
-          <t>En el remo, cada palada parece pequeña, pero sostenida lleva lejos al bote. Esta semana vimos que sembrar, aun con lágrimas, puede preceder a la alegría de la cosecha.</t>
+          <t>Cada palada parece pequeña, pero sostenida lleva lejos al bote. Lo de estos días: sembrar, aun con lágrimas, puede preceder a la alegría de la cosecha.</t>
         </is>
       </c>
     </row>
@@ -41102,7 +41102,7 @@
       </c>
       <c r="D18" s="61" t="inlineStr">
         <is>
-          <t>En el handball la defensa se arma entre todos, brazo con brazo. Los hábitos que protegen a la familia también se construyen juntos, en casa, cada día.</t>
+          <t>Brazo con brazo, la defensa de handball se arma entre todos. Los hábitos que protegen a la familia también se construyen juntos, en casa, cada día.</t>
         </is>
       </c>
     </row>
@@ -41182,7 +41182,7 @@
       </c>
       <c r="D22" s="61" t="inlineStr">
         <is>
-          <t>El utilero revisa cada botín antes del partido, sin que nadie lo aplauda. Esta semana repasamos que prevenir es amar, y bendecimos a Dios por su cuidado de cada día.</t>
+          <t>Sin que nadie lo aplauda, el utilero revisa cada botín antes del partido. Así cerramos el tema: prevenir es amar, y bendecimos a Dios por su cuidado de cada día.</t>
         </is>
       </c>
     </row>
@@ -41202,7 +41202,7 @@
       </c>
       <c r="D23" s="61" t="inlineStr">
         <is>
-          <t>En el rally, el copiloto lee la hoja de ruta curva por curva. La Palabra de Dios es esa lámpara que ilumina el camino, lo cercano y lo lejano.</t>
+          <t>Curva por curva, el copiloto de rally lee la hoja de ruta en voz alta. La Palabra de Dios es esa lámpara que ilumina el camino, lo cercano y lo lejano.</t>
         </is>
       </c>
     </row>
@@ -41362,7 +41362,7 @@
       </c>
       <c r="D31" s="61" t="inlineStr">
         <is>
-          <t>En el ciclismo, muchas veces la subida se gana o se pierde primero en la cabeza. El liderazgo empieza por dentro: cuidá tu corazón, porque de ahí salen tus decisiones.</t>
+          <t>¿Sabías que muchas subidas en bici se ganan o se pierden primero en la cabeza? El liderazgo empieza por dentro: cuidá tu corazón, porque de ahí salen tus decisiones.</t>
         </is>
       </c>
     </row>
@@ -41442,7 +41442,7 @@
       </c>
       <c r="D35" s="61" t="inlineStr">
         <is>
-          <t>En el básquet, la técnica sin compromiso no sostiene a un equipo. Corazón íntegro y manos hábiles: el carácter es el que sostiene la capacidad.</t>
+          <t>Técnica sin compromiso no sostiene a ningún equipo de básquet. Corazón íntegro y manos hábiles: el carácter es el que sostiene la capacidad.</t>
         </is>
       </c>
     </row>
@@ -41462,7 +41462,7 @@
       </c>
       <c r="D36" s="61" t="inlineStr">
         <is>
-          <t>En el tenis amateur, muchas veces el mismo jugador canta si la pelota fue afuera. Esta semana repasamos que el líder se forma por dentro, íntegro aun cuando nadie mira.</t>
+          <t>Tenis amateur: muchas veces el propio jugador canta si la pelota fue afuera. Para llevarse de la semana: el líder se forma por dentro, íntegro aun cuando nadie mira.</t>
         </is>
       </c>
     </row>
@@ -41522,7 +41522,7 @@
       </c>
       <c r="D39" s="61" t="inlineStr">
         <is>
-          <t>En el vestuario, el utilero deja cada camiseta en su lugar, y eso le da paz al plantel. El orden en casa no es rigidez: también es una forma de amar.</t>
+          <t>Cada camiseta en su lugar: así deja el vestuario el utilero, y eso le da paz al plantel. El orden en casa no es rigidez, también es una forma de amar.</t>
         </is>
       </c>
     </row>
@@ -41602,7 +41602,7 @@
       </c>
       <c r="D43" s="61" t="inlineStr">
         <is>
-          <t>En el ajedrez, la calma ayuda a ver todo el tablero. Esta semana repasamos un hogar donde la paz de Dios gobierna el corazón, con gratitud y sin imposiciones.</t>
+          <t>Con calma se ve todo el tablero de ajedrez. Así cerramos el tema: un hogar donde la paz de Dios gobierna el corazón, con gratitud y sin imposiciones.</t>
         </is>
       </c>
     </row>
@@ -41682,7 +41682,7 @@
       </c>
       <c r="D47" s="61" t="inlineStr">
         <is>
-          <t>En una vuelta ciclista se avanza etapa por etapa, no de un solo salto. Con el ahorro pasa igual: de a poco y con mano constante, se llega lejos.</t>
+          <t>Etapa por etapa, no de un solo salto: así se avanza en una vuelta ciclista. Con el ahorro pasa igual, de a poco y con mano constante se llega lejos.</t>
         </is>
       </c>
     </row>
@@ -41742,7 +41742,7 @@
       </c>
       <c r="D50" s="61" t="inlineStr">
         <is>
-          <t>El remero calcula sus fuerzas antes de largar la regata. Esta semana repasamos que ahorrar es prepararse, con la seguridad de fondo puesta en Dios y no en la plata.</t>
+          <t>Antes de largar la regata, el remero calcula sus fuerzas. Siete días después queda esto: ahorrar es prepararse, con la seguridad de fondo puesta en Dios y no en la plata.</t>
         </is>
       </c>
     </row>
@@ -41782,7 +41782,7 @@
       </c>
       <c r="D52" s="61" t="inlineStr">
         <is>
-          <t>En el vestuario, a veces lo más valiente es decir: hoy no estoy bien. Hablar con honestidad sobre lo que sentís también es parte de una vida íntegra.</t>
+          <t>A veces, en el vestuario, lo más valiente es decir: hoy no estoy bien. Hablar con honestidad sobre lo que sentís también es parte de una vida íntegra.</t>
         </is>
       </c>
     </row>
@@ -41882,7 +41882,7 @@
       </c>
       <c r="D57" s="61" t="inlineStr">
         <is>
-          <t>En una posta, nadie corre todos los tramos solo. Esta semana repasamos cómo cuidar el alma: Dios está cerca del quebrantado, y no tenés que cargar todo solo.</t>
+          <t>Nadie corre todos los tramos de una posta solo. Lo de estos días: cuidar el alma sabiendo que Dios está cerca del quebrantado, y que no tenés que cargar todo solo.</t>
         </is>
       </c>
     </row>
@@ -41962,7 +41962,7 @@
       </c>
       <c r="D61" s="61" t="inlineStr">
         <is>
-          <t>En la cancha se nota quién trata bien a los demás, aun cuando nadie mira. El justo cuida la vida de sus animales, y ese trato le importa a Dios.</t>
+          <t>Se nota en la cancha quién trata bien a los demás, aun cuando nadie mira. El justo cuida la vida de sus animales, y ese trato le importa a Dios.</t>
         </is>
       </c>
     </row>
@@ -42002,7 +42002,7 @@
       </c>
       <c r="D63" s="61" t="inlineStr">
         <is>
-          <t>En el vóley, el líbero se tira al piso para salvar la pelota de su compañero. Jesús, el buen pastor, fue mucho más lejos: dio su vida por las ovejas.</t>
+          <t>El líbero se tira al piso para salvar la pelota de su compañero. Jesús, el buen pastor, fue mucho más lejos: dio su vida por las ovejas.</t>
         </is>
       </c>
     </row>
@@ -42022,7 +42022,7 @@
       </c>
       <c r="D64" s="61" t="inlineStr">
         <is>
-          <t>En el handball, el equipo protege al compañero golpeado hasta que se recupera. Esta semana repasamos cuidar como cuida Dios: con ternura, cargando al más débil.</t>
+          <t>Compañero golpeado en el handball: el equipo lo protege hasta que se recupera. Siete días después, la idea queda clara: cuidar como cuida Dios, con ternura, cargando al más débil.</t>
         </is>
       </c>
     </row>
@@ -42162,7 +42162,7 @@
       </c>
       <c r="D71" s="61" t="inlineStr">
         <is>
-          <t>En el futsal, un pase a tiempo vale más que diez apurados al final. Esta semana repasamos cuidarse a tiempo, con Dios como escudo que afirma nuestros pasos.</t>
+          <t>Un pase a tiempo vale más que diez apurados al final del partido de futsal. Para cerrar la semana: cuidarse a tiempo, con Dios como escudo que afirma nuestros pasos.</t>
         </is>
       </c>
     </row>
@@ -42242,7 +42242,7 @@
       </c>
       <c r="D75" s="61" t="inlineStr">
         <is>
-          <t>En el rally, piloto y copiloto se dicen todo con claridad, o el auto se sale del camino. Caminar en la luz es comunión transparente con Dios y con los hermanos.</t>
+          <t>Si piloto y copiloto no se dicen todo con claridad, el auto de rally se sale del camino. Caminar en la luz es comunión transparente con Dios y con los hermanos.</t>
         </is>
       </c>
     </row>
@@ -42262,7 +42262,7 @@
       </c>
       <c r="D76" s="61" t="inlineStr">
         <is>
-          <t>En el handball cada puesto cumple su función, y ninguno sobra. Somos un solo cuerpo con muchos miembros, y cada uno depende de los demás.</t>
+          <t>Ningún puesto sobra en el handball: cada uno cumple su función. Somos un solo cuerpo con muchos miembros, y cada uno depende de los demás.</t>
         </is>
       </c>
     </row>
@@ -42302,7 +42302,7 @@
       </c>
       <c r="D78" s="61" t="inlineStr">
         <is>
-          <t>En el pelotón, los ciclistas se turnan para cortar el viento y llegan más lejos juntos. Esta semana repasamos que la fe se vive en comunidad, con un mismo amor.</t>
+          <t>Turnándose para cortar el viento, los ciclistas del pelotón llegan más lejos juntos. Así cerramos el tema: la fe se vive en comunidad, con un mismo amor.</t>
         </is>
       </c>
     </row>
@@ -42402,7 +42402,7 @@
       </c>
       <c r="D83" s="61" t="inlineStr">
         <is>
-          <t>En el básquet, un tiempo muerto pedido en el momento justo cambia el ritmo del juego. Hay un tiempo para cada cosa, y saber discernirlo es sabiduría.</t>
+          <t>Un tiempo muerto pedido en el momento justo cambia el ritmo del partido de básquet. Hay un tiempo para cada cosa, y saber discernirlo es sabiduría.</t>
         </is>
       </c>
     </row>
@@ -42442,7 +42442,7 @@
       </c>
       <c r="D85" s="61" t="inlineStr">
         <is>
-          <t>En el remo, el timonel marca el ritmo y el bote avanza parejo. Esta semana repasamos liderar con responsabilidad: con sabiduría y aprovechando bien el tiempo.</t>
+          <t>El timonel marca el ritmo y el bote avanza parejo. En una línea: liderar con responsabilidad, con sabiduría y aprovechando bien el tiempo.</t>
         </is>
       </c>
     </row>
@@ -42502,7 +42502,7 @@
       </c>
       <c r="D88" s="61" t="inlineStr">
         <is>
-          <t>En el vóley, el que arma y el que remata se necesitan y se respetan. En el matrimonio, amor y honra se complementan, con el mismo valor.</t>
+          <t>La armadora y la que remata se necesitan y se respetan. En el matrimonio, amor y honra se complementan, con el mismo valor.</t>
         </is>
       </c>
     </row>
@@ -42562,7 +42562,7 @@
       </c>
       <c r="D91" s="61" t="inlineStr">
         <is>
-          <t>En el futsal, encontrar al compañero justo para tirar la pared es una alegría. Tu pareja es un regalo, un favor de Dios y no solo cuestión de suerte.</t>
+          <t>¡Qué alegría encontrar al compañero justo para tirar la pared en el futsal! Tu pareja es un regalo, un favor de Dios y no solo cuestión de suerte.</t>
         </is>
       </c>
     </row>
@@ -42582,7 +42582,7 @@
       </c>
       <c r="D92" s="61" t="inlineStr">
         <is>
-          <t>Como la hinchada que sigue a la Albirroja en las buenas y en las malas, el amor verdadero no se apaga. Esta semana lo repasamos: ni las muchas aguas pueden extinguirlo.</t>
+          <t>Llueva o truene, la hinchada sigue a su equipo: el amor verdadero no se apaga. Para llevarse de la semana: ni las muchas aguas pueden extinguirlo.</t>
         </is>
       </c>
     </row>
@@ -42602,7 +42602,7 @@
       </c>
       <c r="D93" s="61" t="inlineStr">
         <is>
-          <t>En el Rally del Chaco nadie larga sin calcular el combustible del tramo; con la plata pasa lo mismo: el plan se hace antes de largar, no en medio del polvo.</t>
+          <t>Nadie larga en el Rally del Chaco sin calcular el combustible del tramo. Con la plata pasa lo mismo: el plan se hace antes de largar, no en medio del polvo.</t>
         </is>
       </c>
     </row>
@@ -42682,7 +42682,7 @@
       </c>
       <c r="D97" s="61" t="inlineStr">
         <is>
-          <t>En el básquet cada segundo del reloj cuenta y el buen base lo administra con cabeza; el tiempo y los recursos que Dios te da también se juegan con sabiduría.</t>
+          <t>Cada segundo del reloj cuenta, y el buen base de básquet lo administra con cabeza. El tiempo y los recursos que Dios te da también se juegan con sabiduría.</t>
         </is>
       </c>
     </row>
@@ -42702,7 +42702,7 @@
       </c>
       <c r="D98" s="61" t="inlineStr">
         <is>
-          <t>En el futsal cada uno entra a aportar lo que tiene en las piernas; dar también es eso: aportar con constancia, según lo que recibiste.</t>
+          <t>Cada jugador de futsal entra a la cancha a aportar lo que tiene en las piernas. Dar también es eso: aportar con constancia, según lo que recibiste.</t>
         </is>
       </c>
     </row>
@@ -42722,7 +42722,7 @@
       </c>
       <c r="D99" s="61" t="inlineStr">
         <is>
-          <t>El utilero no es dueño de las camisetas, pero las cuida como si lo fueran; esta semana aprendimos a ser administradores confiables de lo que Dios nos prestó.</t>
+          <t>Las camisetas no son del utilero, pero las cuida como si lo fueran. Nos llevamos esto: ser administradores confiables de lo que Dios nos prestó.</t>
         </is>
       </c>
     </row>
@@ -43002,7 +43002,7 @@
       </c>
       <c r="D113" s="61" t="inlineStr">
         <is>
-          <t>En una posta, el testimonio pasa de mano en mano y la carrera necesita a todos; esta semana pedimos como el salmista: Señor, confirmá la obra de nuestras manos.</t>
+          <t>Mano a mano pasa el testimonio, y la carrera de postas necesita a todos. Para cerrar la semana, pedimos como el salmista: Señor, confirmá la obra de nuestras manos.</t>
         </is>
       </c>
     </row>
@@ -43062,7 +43062,7 @@
       </c>
       <c r="D116" s="61" t="inlineStr">
         <is>
-          <t>En una subida larga, el ciclista que controla su ritmo llega mejor que el que se desboca al principio; el dominio propio también se entrena, de a poco.</t>
+          <t>Subida larga: el ciclista que controla su ritmo llega mejor que el que se desboca al principio. El dominio propio también se entrena, de a poco.</t>
         </is>
       </c>
     </row>
@@ -43142,7 +43142,7 @@
       </c>
       <c r="D120" s="61" t="inlineStr">
         <is>
-          <t>Como el preparador físico que cuida a sus jugadores para toda la temporada, cuidar tu cuerpo es cuidar un regalo; esa fue la invitación de esta semana.</t>
+          <t>Pensando en toda la temporada, el preparador físico cuida a sus jugadores. Así cerramos el tema: cuidar tu cuerpo es cuidar un regalo.</t>
         </is>
       </c>
     </row>
@@ -43182,7 +43182,7 @@
       </c>
       <c r="D122" s="61" t="inlineStr">
         <is>
-          <t>En el futsal, el capitán muchas veces es el primero en volver a marcar; Jesús nos mostró que la grandeza está en servir, no en ser servido.</t>
+          <t>El capitán de futsal muchas veces es el primero en volver a marcar. Jesús nos mostró que la grandeza está en servir, no en ser servido.</t>
         </is>
       </c>
     </row>
@@ -43282,7 +43282,7 @@
       </c>
       <c r="D127" s="61" t="inlineStr">
         <is>
-          <t>El atleta guía corre atado a un compañero no vidente y su alegría es que el otro llegue; esta semana aprendimos que hay más dicha en dar que en recibir.</t>
+          <t>Atado a un compañero no vidente, el atleta guía corre feliz si el otro llega. Queda de la semana: hay más dicha en dar que en recibir.</t>
         </is>
       </c>
     </row>
@@ -43302,7 +43302,7 @@
       </c>
       <c r="D128" s="61" t="inlineStr">
         <is>
-          <t>En el rally, cuando el auto se encaja en el barro, piloto y copiloto no discuten la largada: buscan la siguiente salida. Atribulados, pero no destruidos.</t>
+          <t>Auto encajado en el barro: piloto y copiloto no discuten la largada, buscan la siguiente salida. Atribulados, pero no destruidos.</t>
         </is>
       </c>
     </row>
@@ -43342,7 +43342,7 @@
       </c>
       <c r="D130" s="61" t="inlineStr">
         <is>
-          <t>En el ajedrez hay que vigilar el tablero entero sin creer que cada peón es una trampa; el buen líder está alerta y firme en la fe, sin vivir con sospecha.</t>
+          <t>Mirá el tablero de ajedrez entero, sin creer que cada peón es una trampa. El buen líder está alerta y firme en la fe, sin vivir con sospecha.</t>
         </is>
       </c>
     </row>
@@ -43442,7 +43442,7 @@
       </c>
       <c r="D135" s="61" t="inlineStr">
         <is>
-          <t>En la escuelita de fútbol, el buen profe no empuja al chico a crecer de golpe: acompaña, corrige y espera; los hijos son un regalo de Dios, no un trofeo propio.</t>
+          <t>El buen profe de la escuelita de fútbol no empuja al chico a crecer de golpe: acompaña, corrige y espera. Los hijos son un regalo de Dios, no un trofeo propio.</t>
         </is>
       </c>
     </row>
@@ -43562,7 +43562,7 @@
       </c>
       <c r="D141" s="61" t="inlineStr">
         <is>
-          <t>El abuelo que lleva al nieto a su primer partido le pasa más que una camiseta; esta semana vimos que criar con amor e integridad deja un legado de generación en generación.</t>
+          <t>Primer partido del nieto, y el abuelo le pasa mucho más que una camiseta. Lo que queda de estos días: criar con amor e integridad deja un legado de generación en generación.</t>
         </is>
       </c>
     </row>
@@ -43662,7 +43662,7 @@
       </c>
       <c r="D146" s="61" t="inlineStr">
         <is>
-          <t>En el tenis, los partidos largos se sostienen en el punto chico, el que parece no importar; la fidelidad en lo poco forma el carácter para lo mucho.</t>
+          <t>Pocas cosas sostienen tanto un partido largo de tenis como el punto chico, el que parece no importar. La fidelidad en lo poco forma el carácter para lo mucho.</t>
         </is>
       </c>
     </row>
@@ -43702,7 +43702,7 @@
       </c>
       <c r="D148" s="61" t="inlineStr">
         <is>
-          <t>El que reparte buenos pases no se empobrece: hace crecer a todo el equipo; esta semana pusimos orden en lo que entra y sale, y vimos que la generosidad enriquece la vida.</t>
+          <t>Repartir buenos pases no empobrece a nadie: hace crecer a todo el equipo. Después de ordenar lo que entra y sale, queda claro que la generosidad enriquece la vida.</t>
         </is>
       </c>
     </row>
@@ -43762,7 +43762,7 @@
       </c>
       <c r="D151" s="61" t="inlineStr">
         <is>
-          <t>En el último tramo de una regata, el remero pone toda su fuerza en cada palada; lo que tengas hoy entre manos, hacelo con todo, sin mediocridad.</t>
+          <t>Último tramo de la regata: el remero pone toda su fuerza en cada palada. Lo que tengas hoy entre manos, hacelo con todo, sin mediocridad.</t>
         </is>
       </c>
     </row>
@@ -43842,7 +43842,7 @@
       </c>
       <c r="D155" s="61" t="inlineStr">
         <is>
-          <t>En el pelotón, los ciclistas se turnan para cortar el viento y que el otro respire; esta semana aprendimos a crecer y a ayudar a crecer, animándonos unos a otros.</t>
+          <t>Uno corta el viento para que el otro respire: así se turnan en el pelotón. Crecer y ayudar a crecer, animándonos unos a otros: eso nos llevamos.</t>
         </is>
       </c>
     </row>
@@ -43882,7 +43882,7 @@
       </c>
       <c r="D157" s="61" t="inlineStr">
         <is>
-          <t>En el rally, el copiloto va leyendo el camino que viene; emprender puede dar miedo, pero Dios va delante tuyo y no te abandona.</t>
+          <t>Mientras el auto avanza, el copiloto de rally va leyendo el camino que viene. Emprender puede dar miedo, pero Dios va delante tuyo y no te abandona.</t>
         </is>
       </c>
     </row>
@@ -43962,7 +43962,7 @@
       </c>
       <c r="D161" s="61" t="inlineStr">
         <is>
-          <t>En el handball, el pase corto bien hecho, una y otra vez, sostiene al equipo; ser fiel en lo poco también es parte de emprender, y Jesús celebra esa fidelidad.</t>
+          <t>Pase corto bien hecho, una y otra vez: eso sostiene a un equipo de handball. Ser fiel en lo poco también es parte de emprender, y Jesús celebra esa fidelidad.</t>
         </is>
       </c>
     </row>
@@ -44002,7 +44002,7 @@
       </c>
       <c r="D163" s="61" t="inlineStr">
         <is>
-          <t>En la concentración, el cuerpo técnico cuida lo que come el plantel; desde el principio Dios proveyó plantas y semillas: lo que comemos también es parte de su cuidado.</t>
+          <t>Durante la concentración, el cuerpo técnico cuida lo que come el plantel. Desde el principio Dios proveyó plantas y semillas: lo que comemos también es parte de su cuidado.</t>
         </is>
       </c>
     </row>
@@ -44122,7 +44122,7 @@
       </c>
       <c r="D169" s="61" t="inlineStr">
         <is>
-          <t>Como el basquetbolista que ajusta su alimentación sin castigarse por un mal día, esta semana aprendimos a comer con gratitud y medida, como cuidado y no como culpa.</t>
+          <t>Un mal día de comidas no hace que el basquetbolista se castigue: ajusta y sigue. Para cerrar la semana: comer con gratitud y medida, como cuidado y no como culpa.</t>
         </is>
       </c>
     </row>
@@ -44162,7 +44162,7 @@
       </c>
       <c r="D171" s="61" t="inlineStr">
         <is>
-          <t>En una posta, el testimonio que no se entrega se pierde aunque hayas corrido bien; la fe también se pasa de mano en mano, a otros que la sigan llevando.</t>
+          <t>Testimonio que no se entrega se pierde, aunque hayas corrido bien tu tramo de la posta. La fe también se pasa de mano en mano, a otros que la sigan llevando.</t>
         </is>
       </c>
     </row>
@@ -44242,7 +44242,7 @@
       </c>
       <c r="D175" s="61" t="inlineStr">
         <is>
-          <t>En el tenis no alcanza con mirar videos del saque: hay que salir a la cancha y practicarlo; lo que aprendiste, ponelo en práctica, y la paz de Dios te acompaña.</t>
+          <t>Mirar videos del saque no alcanza: hay que salir a la cancha de tenis y practicarlo. Lo que aprendiste, ponelo en práctica, y la paz de Dios te acompaña.</t>
         </is>
       </c>
     </row>
@@ -44262,7 +44262,7 @@
       </c>
       <c r="D176" s="61" t="inlineStr">
         <is>
-          <t>El viejo entrenador de remo sigue presente en cada bote que avanza con los que él formó; esta semana vimos que invertir en otros deja una huella que dura.</t>
+          <t>Cada bote que avanza lleva algo del viejo entrenador de remo que formó a sus remeros. Así cerramos el tema: invertir en otros deja una huella que dura.</t>
         </is>
       </c>
     </row>
@@ -44302,7 +44302,7 @@
       </c>
       <c r="D178" s="61" t="inlineStr">
         <is>
-          <t>En el vóley hay que ser firme en el bloqueo y valiente en el ataque, pero el equipo se sostiene cuando todo se hace con amor, también la corrección.</t>
+          <t>Firme en el bloqueo y valiente en el ataque, sí; pero un equipo de vóley se sostiene cuando todo se hace con amor, también la corrección.</t>
         </is>
       </c>
     </row>
@@ -44362,7 +44362,7 @@
       </c>
       <c r="D181" s="61" t="inlineStr">
         <is>
-          <t>En el rally, cuando se pincha una goma, piloto y copiloto la cambian juntos; en un equipo nadie debería cargar solo: eso es cumplir la ley de Cristo.</t>
+          <t>¿Viste cuando se pincha una goma en pleno rally? Piloto y copiloto la cambian juntos. En un equipo nadie debería cargar solo: eso es cumplir la ley de Cristo.</t>
         </is>
       </c>
     </row>
@@ -44402,7 +44402,7 @@
       </c>
       <c r="D183" s="61" t="inlineStr">
         <is>
-          <t>En el futsal, el que da la asistencia festeja el gol como propio; esta semana vimos que un equipo se sostiene cuando cada uno busca también el bien del otro, con humildad.</t>
+          <t>El que da la asistencia en el futsal festeja el gol como propio. Así se resume la semana: el equipo se sostiene cuando cada uno busca también el bien del otro.</t>
         </is>
       </c>
     </row>
@@ -44542,7 +44542,7 @@
       </c>
       <c r="D190" s="61" t="inlineStr">
         <is>
-          <t>En el vóley el equipo se junta un segundo antes de cada saque; orar por quienes nos gobiernan es ese momento que une a la familia con su país.</t>
+          <t>Un segundo antes de cada saque, el equipo de vóley se junta. Orar por quienes nos gobiernan es ese momento que une a la familia con su país.</t>
         </is>
       </c>
     </row>
@@ -44622,7 +44622,7 @@
       </c>
       <c r="D194" s="61" t="inlineStr">
         <is>
-          <t>En el ajedrez, el que repasa sus partidas y acepta la corrección aprende más que el que solo mueve rápido; la sabiduría empieza reconociendo a Dios con reverencia.</t>
+          <t>Quien repasa sus partidas de ajedrez y acepta la corrección aprende más que el que solo mueve rápido. La sabiduría empieza reconociendo a Dios con reverencia.</t>
         </is>
       </c>
     </row>
@@ -44642,7 +44642,7 @@
       </c>
       <c r="D195" s="61" t="inlineStr">
         <is>
-          <t>En el boxeo, caer a la lona no siempre es el final de la pelea; el justo cae y se vuelve a levantar, porque un tropiezo no define toda tu historia.</t>
+          <t>Caer a la lona no siempre es el final de la pelea. El justo cae y se vuelve a levantar, porque un tropiezo no define toda tu historia.</t>
         </is>
       </c>
     </row>
@@ -44702,7 +44702,7 @@
       </c>
       <c r="D198" s="61" t="inlineStr">
         <is>
-          <t>En el tiro con arco, el arquero necesita saber hacia dónde apunta; y mientras apuntás tus metas, acordate de que Dios empezó la obra en vos y Él la va a completar.</t>
+          <t>Antes de soltar la flecha, el arquero necesita saber hacia dónde apunta. Y mientras apuntás tus metas, acordate de que Dios empezó la obra en vos y Él la va a completar.</t>
         </is>
       </c>
     </row>
@@ -44782,7 +44782,7 @@
       </c>
       <c r="D202" s="61" t="inlineStr">
         <is>
-          <t>En la subida más dura, el ciclista no se baja de la bici: sigue pedaleando con paciencia. Gozate en la esperanza, aguantá en la prueba y seguí constante en la oración.</t>
+          <t>Kilómetro final de la subida más dura: el ciclista no se baja, sigue pedaleando con paciencia. Gozate en la esperanza, aguantá en la prueba y seguí constante en la oración.</t>
         </is>
       </c>
     </row>
@@ -44802,7 +44802,7 @@
       </c>
       <c r="D203" s="61" t="inlineStr">
         <is>
-          <t>En el Rally del Chaco, el copiloto revisa el tramo recorrido antes de encarar el siguiente; mirar atrás con honestidad y poner tus planes en manos de Dios te ayuda a seguir.</t>
+          <t>Tramo terminado en el Rally del Chaco: el copiloto lo revisa antes de encarar el siguiente. Mirar atrás con honestidad y poner tus planes en manos de Dios te ayuda a seguir.</t>
         </is>
       </c>
     </row>
@@ -45042,7 +45042,7 @@
       </c>
       <c r="D215" s="61" t="inlineStr">
         <is>
-          <t>En el básquet, el entrenador pide tiempo muerto para que el equipo respire; Jesús también invitó a los suyos a descansar aparte. Parar un rato no es debilidad, es sabiduría.</t>
+          <t>Tiempo muerto: el entrenador de básquet lo pide para que el equipo respire. Jesús también invitó a los suyos a descansar aparte; parar un rato no es debilidad, es sabiduría.</t>
         </is>
       </c>
     </row>
@@ -45102,7 +45102,7 @@
       </c>
       <c r="D218" s="61" t="inlineStr">
         <is>
-          <t>En el remo hay un instante en que el bote se desliza solo entre palada y palada; descansar no es solo dejar de hacer, es saber que Dios va con vos.</t>
+          <t>Hay un instante, entre palada y palada, en que el bote de remo se desliza solo. Descansar no es solo dejar de hacer, es saber que Dios va con vos.</t>
         </is>
       </c>
     </row>
@@ -45422,7 +45422,7 @@
       </c>
       <c r="D234" s="61" t="inlineStr">
         <is>
-          <t>En el básquet, una palabra de más al árbitro puede costar una falta técnica; pedile a Dios guardia para tu boca y aprendé también el valor de callar a tiempo.</t>
+          <t>Una palabra de más al árbitro puede costar una falta técnica en el básquet. Pedile a Dios guardia para tu boca y aprendé también el valor de callar a tiempo.</t>
         </is>
       </c>
     </row>
@@ -45442,7 +45442,7 @@
       </c>
       <c r="D235" s="61" t="inlineStr">
         <is>
-          <t>En el vóley de playa son dos en la cancha y se conocen de memoria; comprender y honrar a tu esposa también es cuidar la relación que Dios les regaló.</t>
+          <t>Dos en la arena del vóley de playa, y se conocen de memoria. Comprender y honrar a tu esposa también es cuidar la relación que Dios les regaló.</t>
         </is>
       </c>
     </row>
@@ -45482,7 +45482,7 @@
       </c>
       <c r="D237" s="61" t="inlineStr">
         <is>
-          <t>En el futsal, un pase un segundo tarde ya no sirve; la palabra dicha a tiempo, con tacto y prudencia, vale como manzana de oro en la familia.</t>
+          <t>Llega un segundo tarde y el pase ya no sirve: así es el futsal. La palabra dicha a tiempo, con tacto y prudencia, vale como manzana de oro en la familia.</t>
         </is>
       </c>
     </row>
@@ -45642,7 +45642,7 @@
       </c>
       <c r="D245" s="61" t="inlineStr">
         <is>
-          <t>En el remo doble, si cada uno rema a su ritmo, el bote gira en círculos; en las finanzas del hogar, tener un mismo sentir ayuda a la familia a avanzar.</t>
+          <t>Si cada uno rema a su ritmo, el bote doble gira en círculos. En las finanzas del hogar, tener un mismo sentir ayuda a la familia a avanzar.</t>
         </is>
       </c>
     </row>
@@ -45742,7 +45742,7 @@
       </c>
       <c r="D250" s="61" t="inlineStr">
         <is>
-          <t>En el handball, el que llega primero a cada entrenamiento termina siendo referente del grupo; la mano diligente lidera, y el esfuerzo constante gana confianza.</t>
+          <t>Quien llega primero a cada entrenamiento de handball termina siendo referente del grupo. La mano diligente lidera, y el esfuerzo constante gana confianza.</t>
         </is>
       </c>
     </row>
@@ -45822,7 +45822,7 @@
       </c>
       <c r="D254" s="61" t="inlineStr">
         <is>
-          <t>En una carrera de relevos nadie llega solo: cada uno corre su tramo y pasa el testigo. Revestidos de amor, juntos llegamos donde solos no podíamos.</t>
+          <t>Cuando el testigo pasa de mano en mano, nadie llega solo: cada uno corre su tramo del relevo. Revestidos de amor, juntos llegamos donde solos no podíamos.</t>
         </is>
       </c>
     </row>
@@ -45862,7 +45862,7 @@
       </c>
       <c r="D256" s="61" t="inlineStr">
         <is>
-          <t>En el vóley, el armador, el central y el líbero cumplen funciones distintas para el mismo equipo; usá tu don con generosidad para servir a los demás.</t>
+          <t>Armador, central y líbero cumplen funciones distintas para el mismo equipo de vóley. Usá tu don con generosidad para servir a los demás.</t>
         </is>
       </c>
     </row>
@@ -45942,7 +45942,7 @@
       </c>
       <c r="D260" s="61" t="inlineStr">
         <is>
-          <t>En el pelotón, los ciclistas se turnan para cortar el viento y así llegan más lejos; un mismo sentir, compasión y amor fraternal también hacen avanzar a la comunidad.</t>
+          <t>Pocas imágenes de comunidad como el pelotón: se turnan para cortar el viento y llegan más lejos. Un mismo sentir, compasión y amor fraternal también hacen avanzar a la comunidad.</t>
         </is>
       </c>
     </row>
@@ -46182,7 +46182,7 @@
       </c>
       <c r="D272" s="61" t="inlineStr">
         <is>
-          <t>En el remo, cada remero deja su propio ritmo y sigue la palada del que marca; vivir por fe es dejar que Cristo, que vive en vos, marque tu ritmo.</t>
+          <t>Cada remero deja su propio ritmo y sigue la palada del que marca. Vivir por fe es dejar que Cristo, que vive en vos, marque tu ritmo.</t>
         </is>
       </c>
     </row>
@@ -46222,7 +46222,7 @@
       </c>
       <c r="D274" s="61" t="inlineStr">
         <is>
-          <t>En el atletismo la medalla se gana corriendo, pero ser hijo de Dios no se gana: se recibe al recibir a Cristo. Saber quién sos cambia cómo encarás cada día.</t>
+          <t>La medalla del atletismo se gana corriendo, pero ser hijo de Dios no se gana: se recibe al recibir a Cristo. Saber quién sos cambia cómo encarás cada día.</t>
         </is>
       </c>
     </row>
@@ -46262,7 +46262,7 @@
       </c>
       <c r="D276" s="61" t="inlineStr">
         <is>
-          <t>En el boxeo, el que mejor se controla no es el más débil: es el que sabe contener su fuerza. Eso es la humildad bajo presión.</t>
+          <t>Sobre el ring, el que mejor se controla no es el más débil: es el que sabe contener su fuerza. Eso es la humildad bajo presión.</t>
         </is>
       </c>
     </row>
@@ -46362,7 +46362,7 @@
       </c>
       <c r="D281" s="61" t="inlineStr">
         <is>
-          <t>En el básquet, el base que mejor dirige es el que más asistencias da. Repasamos esta semana que, con Jesús, liderar es servir.</t>
+          <t>El base que mejor dirige es el que más asistencias da. Para llevarse de la semana: con Jesús, liderar es servir.</t>
         </is>
       </c>
     </row>
@@ -46382,7 +46382,7 @@
       </c>
       <c r="D282" s="61" t="inlineStr">
         <is>
-          <t>En el vóley nadie toca la pelota dos veces seguidas: cada uno cumple su parte y el punto se construye entre todos. Un hogar funciona parecido.</t>
+          <t>Nadie toca la pelota dos veces seguidas en el vóley: cada uno cumple su parte y el punto se construye entre todos. Un hogar funciona parecido.</t>
         </is>
       </c>
     </row>
@@ -46442,7 +46442,7 @@
       </c>
       <c r="D285" s="61" t="inlineStr">
         <is>
-          <t>En el handball los roces son constantes, y el equipo sigue unido si se dan la mano después de cada choque. En casa, la paciencia y el perdón hacen lo mismo.</t>
+          <t>Roces hay todo el partido en el handball, y el equipo sigue unido si se dan la mano después de cada choque. En casa, la paciencia y el perdón hacen lo mismo.</t>
         </is>
       </c>
     </row>
@@ -46502,7 +46502,7 @@
       </c>
       <c r="D288" s="61" t="inlineStr">
         <is>
-          <t>En una maratón, quien acompaña a otro hasta la meta muestra que la lealtad pesa más que el reloj. Repasamos esta semana un hogar que camina junto, aun en lo difícil.</t>
+          <t>Kilómetro 40: alguien frena para acompañar a otro hasta la meta; la lealtad pesa más que el reloj. Siete días después, queda un hogar que camina junto, aun en lo difícil.</t>
         </is>
       </c>
     </row>
@@ -46542,7 +46542,7 @@
       </c>
       <c r="D290" s="61" t="inlineStr">
         <is>
-          <t>En la posta, el corredor suelta el testigo confiando en las manos del compañero. Dar a Dios es un acto de confianza, no un pago para recibir algo a cambio.</t>
+          <t>El relevista suelta el testigo confiando en las manos del compañero. Dar a Dios es un acto de confianza, no un pago para recibir algo a cambio.</t>
         </is>
       </c>
     </row>
@@ -46702,7 +46702,7 @@
       </c>
       <c r="D298" s="61" t="inlineStr">
         <is>
-          <t>En la maratón, el último kilómetro cuenta tanto como el primero. Pablo pudo decir «he terminado la carrera»: terminar bien también es fidelidad.</t>
+          <t>El último kilómetro de la maratón cuenta tanto como el primero. Pablo pudo decir «he terminado la carrera»: terminar bien también es fidelidad.</t>
         </is>
       </c>
     </row>
@@ -46722,7 +46722,7 @@
       </c>
       <c r="D299" s="61" t="inlineStr">
         <is>
-          <t>En el básquet, el reloj de posesión te obliga a elegir qué vale la pena. Contar nuestros días nos ayuda a ordenar las prioridades con sabiduría.</t>
+          <t>Veinticuatro segundos de posesión en el básquet te obligan a elegir qué vale la pena. Contar nuestros días nos ayuda a ordenar las prioridades con sabiduría.</t>
         </is>
       </c>
     </row>
@@ -46762,7 +46762,7 @@
       </c>
       <c r="D301" s="61" t="inlineStr">
         <is>
-          <t>En el vóley, una pelota mal recibida todavía puede terminar en un buen ataque. José lo vivió: lo que otros pensaron para mal, Dios lo encaminó para bien.</t>
+          <t>Una pelota mal recibida en el vóley todavía puede terminar en un buen ataque. José lo vivió: lo que otros pensaron para mal, Dios lo encaminó para bien.</t>
         </is>
       </c>
     </row>
@@ -46782,7 +46782,7 @@
       </c>
       <c r="D302" s="61" t="inlineStr">
         <is>
-          <t>Hay entrenadores que ya no están, y sin embargo su manera de jugar sigue viva en la cancha. Repasamos esta semana: lo que se hace por fe sigue hablando.</t>
+          <t>Algunos entrenadores ya no están, y sin embargo su manera de jugar sigue viva en la cancha. Lo que se hace por fe sigue hablando.</t>
         </is>
       </c>
     </row>
@@ -46942,7 +46942,7 @@
       </c>
       <c r="D310" s="61" t="inlineStr">
         <is>
-          <t>En un partido de barrio, cuando alguien cae lesionado, lo primero no es el resultado sino acercarse a ayudar. El buen samaritano no pasó de largo.</t>
+          <t>Partido de barrio, alguien cae lesionado, y lo primero no es el resultado sino acercarse a ayudar. El buen samaritano no pasó de largo.</t>
         </is>
       </c>
     </row>
@@ -46982,7 +46982,7 @@
       </c>
       <c r="D312" s="61" t="inlineStr">
         <is>
-          <t>En la pista, si un corredor se desploma, los jueces no esperan que termine la carrera para asistirlo. Actuar a tiempo ante el peligro ajeno es una responsabilidad real.</t>
+          <t>Si un corredor se desploma en la pista, los jueces no esperan que termine la carrera para asistirlo. Actuar a tiempo ante el peligro ajeno es una responsabilidad real.</t>
         </is>
       </c>
     </row>
@@ -47062,7 +47062,7 @@
       </c>
       <c r="D316" s="61" t="inlineStr">
         <is>
-          <t>Un equipo de vóley practica la recepción cientos de veces para estar listo cuando llega el saque difícil. Repasamos: prepararnos para ayudar e invocar a Dios en la angustia.</t>
+          <t>Cientos de recepciones en la práctica de vóley, para estar listos cuando llega el saque difícil. Queda de la semana: prepararnos para ayudar e invocar a Dios en la angustia.</t>
         </is>
       </c>
     </row>
@@ -47142,7 +47142,7 @@
       </c>
       <c r="D320" s="61" t="inlineStr">
         <is>
-          <t>En el vestuario de básquet hay noches de lágrimas y noches de canto. Santiago dice: ¿alguien sufre? que ore; ¿alguien está alegre? que cante alabanzas.</t>
+          <t>Hay noches de lágrimas y noches de canto en el vestuario de básquet. Santiago dice: ¿alguien sufre? Que ore; ¿alguien está alegre? Que cante alabanzas.</t>
         </is>
       </c>
     </row>
@@ -47202,7 +47202,7 @@
       </c>
       <c r="D323" s="61" t="inlineStr">
         <is>
-          <t>El ciclista que pinchó y quedó lejos del pelotón igual sigue pedaleando. Repasamos con Habacuc: aunque falte todo, Dios da fuerzas para seguir caminando.</t>
+          <t>Pinchó, quedó lejos del pelotón, y el ciclista igual sigue pedaleando. Con Habacuc cerramos el tema: aunque falte todo, Dios da fuerzas para seguir caminando.</t>
         </is>
       </c>
     </row>
@@ -47342,7 +47342,7 @@
       </c>
       <c r="D330" s="61" t="inlineStr">
         <is>
-          <t>Antes de un clásico, cada uno tiene su plan de juego en la cabeza. Repasamos esta semana: muchos planes hay en el corazón, pero el consejo del Señor permanece.</t>
+          <t>Minuto cero de un clásico: cada uno tiene su plan de juego en la cabeza. Siete días después, la conclusión: muchos planes hay en el corazón, pero el consejo del Señor permanece.</t>
         </is>
       </c>
     </row>
@@ -47442,7 +47442,7 @@
       </c>
       <c r="D335" s="61" t="inlineStr">
         <is>
-          <t>En una posta de natación cada nadador hace su propio tramo, aunque el equipo sea uno. La promesa alcanza a toda la casa, y cada uno está invitado a creer.</t>
+          <t>Cada nadador de la posta hace su propio tramo, aunque el equipo sea uno. La promesa alcanza a toda la casa, y cada uno está invitado a creer.</t>
         </is>
       </c>
     </row>
@@ -47462,7 +47462,7 @@
       </c>
       <c r="D336" s="61" t="inlineStr">
         <is>
-          <t>En el vóley, el equipo rota siempre en el mismo sentido y por eso no se pierde. Dichosa la familia que honra al Señor y anda en sus caminos.</t>
+          <t>Rotación en el vóley: el equipo gira siempre en el mismo sentido y por eso no se pierde. Dichosa la familia que honra al Señor y anda en sus caminos.</t>
         </is>
       </c>
     </row>
@@ -47622,7 +47622,7 @@
       </c>
       <c r="D344" s="61" t="inlineStr">
         <is>
-          <t>El atleta ordena su semana según lo más importante, y lo demás se acomoda. Repasamos: buscar primero el reino de Dios y su justicia, confiando en que Él provee lo necesario.</t>
+          <t>Primero lo más importante: así ordena el atleta su semana, y lo demás se acomoda. Para cerrar: buscar primero el reino de Dios y su justicia, confiando en que Él provee.</t>
         </is>
       </c>
     </row>
@@ -47762,7 +47762,7 @@
       </c>
       <c r="D351" s="61" t="inlineStr">
         <is>
-          <t>Ningún maratonista llega a la meta de un salto: cada kilómetro suma. Repasamos: la senda del justo es como la luz del amanecer, que va en aumento paso a paso.</t>
+          <t>Ningún maratonista llega a la meta de un salto: cada kilómetro suma. La senda del justo es como la luz del amanecer, que va en aumento paso a paso.</t>
         </is>
       </c>
     </row>
@@ -47922,7 +47922,7 @@
       </c>
       <c r="D359" s="61" t="inlineStr">
         <is>
-          <t>En el club de básquet, el kinesiólogo trata la lesión y el entrenador cuida el ánimo; el jugador necesita las dos cosas. Cuerpo, mente y espíritu sanan mejor juntos.</t>
+          <t>El kinesiólogo trata la lesión y el entrenador cuida el ánimo; el jugador de básquet necesita las dos cosas. Cuerpo, mente y espíritu sanan mejor juntos.</t>
         </is>
       </c>
     </row>
@@ -48042,7 +48042,7 @@
       </c>
       <c r="D365" s="61" t="inlineStr">
         <is>
-          <t>Una palabra amable del entrenador al que erró un penal puede levantarle el ánimo. Repasamos: las palabras bondadosas son dulces para el alma y salud para el cuerpo.</t>
+          <t>Silbato final, penal errado, y una palabra amable del entrenador levanta el ánimo del jugador. Lo de estos días: las palabras bondadosas son dulces para el alma y salud para el cuerpo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mensajero: las tres frases con fuente parcial, resueltas (Cervantes confirmada, Spurgeon como proverbio recogido, Temple con su definición completa)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -1218,7 +1218,7 @@
       </c>
       <c r="J3" s="23" t="inlineStr">
         <is>
-          <t>"Con perseverancia, el caracol llegó al arca." — Charles H. Spurgeon</t>
+          <t>"Con perseverancia, el caracol llegó al arca." — Proverbio recogido por Charles H. Spurgeon</t>
         </is>
       </c>
       <c r="K3" s="23" t="inlineStr">
@@ -10256,7 +10256,7 @@
       </c>
       <c r="R47" s="8" t="inlineStr">
         <is>
-          <t>"Adorar es avivar la conciencia con la santidad de Dios, alimentar la mente con su verdad, purificar la imaginación con su belleza y abrir el corazón a su amor." — William Temple</t>
+          <t>"Adorar es someter toda nuestra naturaleza a Dios: avivar la conciencia con su santidad, alimentar la mente con su verdad, purificar la imaginación con su belleza, abrir el corazón a su amor y rendir la voluntad a su propósito." — William Temple</t>
         </is>
       </c>
       <c r="S47" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Mensajero: 104 frases célebres nuevas verificadas (martes y jueves), una frase distinta cada día de lunes a viernes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -740,7 +740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK53"/>
+  <dimension ref="A1:AM53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7421875" defaultRowHeight="15"/>
   <cols>
     <col width="7.93359375" customWidth="1" min="1" max="1"/>
@@ -968,6 +968,16 @@
           <t>3 Puntos Sabado</t>
         </is>
       </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>Frase Celebre 1b</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Frase Celebre 2b</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="219.75" customHeight="1">
       <c r="A2" s="21" t="n">
@@ -1173,6 +1183,16 @@
 • Cuidar el alma también cuida el cuerpo</t>
         </is>
       </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>"El hombre no es ni ángel ni bestia, y la desgracia quiere que quien quiere hacer de ángel haga de bestia." — Blaise Pascal</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>"El hierro se oxida si no se usa; el agua estancada pierde su pureza y con el frío se congela; así también la inacción le quita vigor a la mente." — Leonardo da Vinci</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="219.75" customHeight="1">
       <c r="A3" s="23" t="n">
@@ -1376,6 +1396,16 @@
           <t>• Sembrar con lágrimas puede preceder al regocijo
 • El esfuerzo difícil tiene recompensa futura
 • La perseverancia en medio del dolor rinde fruto</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>"Nada te turbe, nada te espante; todo se pasa, Dios no se muda; la paciencia todo lo alcanza." — Teresa de Ávila</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>"El trabajo tenaz lo vence todo, y también la necesidad que aprieta en los tiempos duros." — Virgilio</t>
         </is>
       </c>
     </row>
@@ -1590,6 +1620,16 @@
 • No olvidar Sus beneficios cotidianos</t>
         </is>
       </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>"Hay cinco puntos esenciales para asegurar la salud de las casas: aire puro, agua pura, desagüe eficiente, limpieza y luz." — Florence Nightingale</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>"Corremos despreocupados hacia el precipicio, después de haber puesto algo delante para no verlo." — Blaise Pascal</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="219.75" customHeight="1">
       <c r="A5" s="30" t="n">
@@ -1794,6 +1834,16 @@
 • Se vuelve alegría del corazón</t>
         </is>
       </c>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>"Algunos libros son para probarlos, otros para tragarlos, y unos pocos para masticarlos y digerirlos." — Francis Bacon</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>"En la Sagrada Escritura se ha de buscar la verdad, no la elocuencia; se ha de buscar el provecho más que la sutileza de las palabras." — Tomás de Kempis</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="219.75" customHeight="1">
       <c r="A6" s="37" t="n">
@@ -1997,6 +2047,16 @@
 • Ser hospitalario y apto para enseñar.</t>
         </is>
       </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>"El talento se forma en la quietud; el carácter, en la corriente del mundo." — Johann Wolfgang von Goethe</t>
+        </is>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>"Es más fácil sostener tus principios el cien por ciento del tiempo que sostenerlos el noventa y ocho por ciento." — Clayton M. Christensen</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="219.75" customHeight="1">
       <c r="A7" s="35" t="n">
@@ -2198,6 +2258,16 @@
           <t>• La paz de Dios gobierna el corazón
 • Ser agradecido sostiene la armonía
 • El hogar necesita paz que gobierne, no que se imponga</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>"La paz de todas las cosas es la tranquilidad del orden." — Agustín de Hipona</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>"La limpieza está, ciertamente, cerca de la piedad." — John Wesley</t>
         </is>
       </c>
     </row>
@@ -2407,6 +2477,16 @@
 • Empezar sin plan expone al ridículo</t>
         </is>
       </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>"Tengas lo que tengas, gastá menos." — Samuel Johnson</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>"De sabios es guardarse hoy para mañana y no aventurarse todo en un día." — Miguel de Cervantes</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="219.75" customHeight="1">
       <c r="A9" s="43" t="n">
@@ -2608,6 +2688,16 @@
 • Consuelo real en momentos de angustia</t>
         </is>
       </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>"Dale palabras al dolor: la pena que no habla le susurra al corazón agobiado y lo empuja a romperse." — William Shakespeare</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>"Quien está en todas partes no está en ninguna." — Séneca</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="219.75" customHeight="1">
       <c r="A10" s="47" t="n">
@@ -2808,6 +2898,16 @@
           <t>• Dios apacienta como un pastor cuidadoso
 • Carga a los débiles con ternura
 • El cuidado tierno es parte del liderazgo</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>"El ojo del amo engorda al caballo." — Jenofonte</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>"La ética es responsabilidad, ampliada sin límites, hacia todo lo que vive." — Albert Schweitzer</t>
         </is>
       </c>
     </row>
@@ -3014,6 +3114,16 @@
 • Dios nos guía: Afirma nuestros pasos para no caer.</t>
         </is>
       </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>"No basta que el médico haga lo que debe; también el paciente, quienes lo asisten y las circunstancias tienen que colaborar." — Hipócrates</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>"Le pediré a Dios que en su misericordia nos proteja. Después fumigaré, ayudaré a purificar el aire, daré medicina y la tomaré." — Martín Lutero</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="219.75" customHeight="1">
       <c r="A12" s="51" t="n">
@@ -3219,6 +3329,16 @@
 • Unanimidad como meta de la comunidad</t>
         </is>
       </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>"La amistad nace en el momento en que uno le dice a otro: ¿Qué? ¿Vos también? Pensé que nadie más que yo." — C. S. Lewis</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>"El Cristo en el propio corazón es más débil que el Cristo en la palabra del hermano." — Dietrich Bonhoeffer</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="219.75" customHeight="1">
       <c r="A13" s="53" t="n">
@@ -3421,6 +3541,16 @@
           <t>• Actuar con sabiduría frente a otros
 • Aprovechar bien el tiempo
 • La prudencia en la gestión del tiempo</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>"El gran enemigo de la comunicación, descubrimos, es la ilusión de haberla logrado." — William H. Whyte</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>"Cuando su obra se completa y su tarea termina, todos dicen: lo hicimos nosotros." — Lao-Tsé</t>
         </is>
       </c>
     </row>
@@ -3631,6 +3761,16 @@
 • El amor tiene un valor que no se compra</t>
         </is>
       </c>
+      <c r="AL14" t="inlineStr">
+        <is>
+          <t>"No es su amor el que sostiene el matrimonio, sino que desde ahora es el matrimonio el que sostiene su amor." — Dietrich Bonhoeffer</t>
+        </is>
+      </c>
+      <c r="AM14" t="inlineStr">
+        <is>
+          <t>"El amor se debe poner más en las obras que en las palabras." — Ignacio de Loyola</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="219.75" customHeight="1">
       <c r="A15" s="40" t="n">
@@ -3830,6 +3970,16 @@
           <t>• Ser confiables.
 • Administrar bien lo recibido.
 • Ser fieles a Dios.</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>"Cuidado con los pequeños gastos: una pequeña vía de agua hunde un gran barco." — Benjamin Franklin</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>"¡Simplicidad, simplicidad, simplicidad! Que tus asuntos sean dos o tres, y no cien ni mil; en vez de un millón, contá media docena, y llevá tus cuentas en la uña del pulgar." — Henry David Thoreau</t>
         </is>
       </c>
     </row>
@@ -4039,6 +4189,16 @@
 • La fe se afirma con el tiempo</t>
         </is>
       </c>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>"Ciertamente, el día del juicio no nos preguntarán qué leímos, sino qué hicimos; ni cuán bien hablamos, sino cuán santamente vivimos." — Tomás de Kempis</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>"La gracia no se opone al esfuerzo; se opone a querer ganársela. Ganar es una actitud; el esfuerzo es una acción." — Dallas Willard</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="219.75" customHeight="1">
       <c r="A17" s="47" t="n">
@@ -4244,6 +4404,16 @@
           <t>• Pedir que Dios confirme la obra de las manos
 • El favor divino da estabilidad al esfuerzo
 • El éxito sostenible depende de Su bendición</t>
+        </is>
+      </c>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>"Un negocio que no produce nada más que dinero es un negocio pobre." — Henry Ford</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr">
+        <is>
+          <t>"Si pierden dinero para la empresa, seré comprensivo; si le hacen perder una pizca de reputación, seré implacable." — Warren Buffett</t>
         </is>
       </c>
     </row>
@@ -4453,6 +4623,16 @@
 • La fuerza física sostiene las tareas diarias</t>
         </is>
       </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>"Comer solo no mantiene sano a un hombre; también tiene que hacer ejercicio." — Hipócrates</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>"Sobre todo, no pierdas las ganas de caminar: cada día camino hasta llegar a un estado de bienestar, y caminando he llegado a mis mejores pensamientos." — Søren Kierkegaard</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="219.75" customHeight="1">
       <c r="A19" s="51" t="n">
@@ -4654,6 +4834,16 @@
 • Contradice la lógica del mundo</t>
         </is>
       </c>
+      <c r="AL19" t="inlineStr">
+        <is>
+          <t>"La atención es la forma más rara y más pura de la generosidad." — Simone Weil</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>"El bien creciente del mundo depende en parte de actos que la historia no registra; y que no nos vaya tan mal se debe en buena parte a los muchos que vivieron fielmente una vida oculta." — George Eliot</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="219.75" customHeight="1">
       <c r="A20" s="53" t="n">
@@ -4856,6 +5046,16 @@
 • La confianza no depende de entender todo</t>
         </is>
       </c>
+      <c r="AL20" t="inlineStr">
+        <is>
+          <t>"Si alguien puede demostrarme que pienso o actúo mal, con gusto cambiaré; porque busco la verdad, y la verdad nunca dañó a nadie." — Marco Aurelio</t>
+        </is>
+      </c>
+      <c r="AM20" t="inlineStr">
+        <is>
+          <t>"Las tropas, la aviación y la marina hicieron todo lo que la valentía y la devoción al deber podían hacer. Si hay alguna culpa o falta en este intento, es solo mía." — Dwight D. Eisenhower</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="219.75" customHeight="1">
       <c r="A21" s="35" t="n">
@@ -5061,6 +5261,16 @@
 • El legado se extiende generación tras generación</t>
         </is>
       </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>"Que los jóvenes no sean solamente amados, sino que ellos mismos se den cuenta de que son amados." — Juan Bosco</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>"Los niños saben más de lo que parece, y si les dijeran que escribiesen lo que saben, muy buenas cosas escribirían." — José Martí</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="219.75" customHeight="1">
       <c r="A22" s="40" t="n">
@@ -5267,6 +5477,16 @@
 • La generosidad enriquece la vida</t>
         </is>
       </c>
+      <c r="AL22" t="inlineStr">
+        <is>
+          <t>"La diligencia es madre de la buena ventura, y la pereza, su contraria, jamás llegó al término que pide un buen deseo." — Miguel de Cervantes</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>"Comprá lo que no necesitás y muy pronto tendrás que vender lo que sí necesitás." — Benjamin Franklin</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="219.75" customHeight="1">
       <c r="A23" s="43" t="n">
@@ -5465,6 +5685,16 @@
           <t>• Animarnos — Dar palabras de ánimo a los demás.
 • Edificarnos — Ayudarnos a crecer en la fe.
 • Hacerlo juntos — Fortalecernos mutuamente cada día.</t>
+        </is>
+      </c>
+      <c r="AL23" t="inlineStr">
+        <is>
+          <t>"Hay que seguir aprendiendo mientras haya algo que no sabemos; y, si creemos al proverbio, mientras vivamos." — Séneca</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>"Bienaventurado el que ha encontrado su trabajo; que no pida otra bienaventuranza." — Thomas Carlyle</t>
         </is>
       </c>
     </row>
@@ -5673,6 +5903,16 @@
 • Jesús da vida eterna — Él es quien satisface verdaderamente nuestra</t>
         </is>
       </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>"Hacé lo que puedas, con lo que tengas, donde estés." — Squire Bill Widener (citado por Theodore Roosevelt)</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>"Es bueno confiar el comienzo de toda gran empresa a Argos, con sus cien ojos, y el final a Briareo, con sus cien manos: primero vigilar, y después apurarse." — Francis Bacon</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="219.75" customHeight="1">
       <c r="A25" s="49" t="n">
@@ -5883,6 +6123,16 @@
 • La fe se demuestra también en decisiones cotidianas</t>
         </is>
       </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>"No se puede pensar bien, amar bien ni dormir bien si no se ha comido bien." — Virginia Woolf</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>"Un hábito es un hábito: nadie puede tirarlo por la ventana; hay que convencerlo de bajar la escalera, un escalón a la vez." — Mark Twain</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="219.75" customHeight="1">
       <c r="A26" s="51" t="n">
@@ -6085,6 +6335,16 @@
 • El discipulado tiene recompensa duradera</t>
         </is>
       </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>"Los discípulos no se pueden producir en serie. No podemos meter a la gente en un programa y esperar que salgan discípulos al final de la línea de producción. Hacer discípulos lleva tiempo y atención personal." — LeRoy Eims</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>"Es mejor callar y ser cristiano que hablar y no serlo. Bueno es enseñar, si el que habla también hace." — Ignacio de Antioquía</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="219.75" customHeight="1">
       <c r="A27" s="53" t="n">
@@ -6290,6 +6550,16 @@
 • La humildad sostiene al equipo</t>
         </is>
       </c>
+      <c r="AL27" t="inlineStr">
+        <is>
+          <t>"Obrá de tal modo que trates a la humanidad, tanto en tu persona como en la de cualquier otro, siempre al mismo tiempo como fin y nunca simplemente como medio." — Immanuel Kant</t>
+        </is>
+      </c>
+      <c r="AM27" t="inlineStr">
+        <is>
+          <t>"No sé cómo puede salir adelante un hombre en quien no se puede confiar. ¿Cómo andaría un carro sin la barra que lo une a los bueyes?" — Confucio</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="219.75" customHeight="1">
       <c r="A28" s="35" t="n">
@@ -6493,6 +6763,16 @@
 • La oración conecta la familia con la sociedad</t>
         </is>
       </c>
+      <c r="AL28" t="inlineStr">
+        <is>
+          <t>"Los antiguos que querían gobernar bien sus Estados primero ponían en orden sus familias." — Confucio (Gran Saber)</t>
+        </is>
+      </c>
+      <c r="AM28" t="inlineStr">
+        <is>
+          <t>"El ser humano está por naturaleza más inclinado a formar pareja que a formar ciudades, porque la casa es anterior y más necesaria que la ciudad." — Aristóteles</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="219.75" customHeight="1">
       <c r="A29" s="40" t="n">
@@ -6700,6 +6980,16 @@
 • Aprender a tomar buenas decisiones.</t>
         </is>
       </c>
+      <c r="AL29" t="inlineStr">
+        <is>
+          <t>"Los capitales aumentan por la frugalidad y disminuyen por la prodigalidad y la mala conducta." — Adam Smith</t>
+        </is>
+      </c>
+      <c r="AM29" t="inlineStr">
+        <is>
+          <t>"El principal problema del inversor, e incluso su peor enemigo, probablemente sea él mismo." — Benjamin Graham</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="219.75" customHeight="1">
       <c r="A30" s="43" t="n">
@@ -6903,6 +7193,16 @@
 • La humildad reconoce los límites del control propio</t>
         </is>
       </c>
+      <c r="AL30" t="inlineStr">
+        <is>
+          <t>"Primero decite a vos mismo qué querés ser; después hacé lo que tenés que hacer." — Epicteto</t>
+        </is>
+      </c>
+      <c r="AM30" t="inlineStr">
+        <is>
+          <t>"Nunca se rindan: nunca, nunca, nunca, en nada, grande o pequeño, importante o insignificante; nunca se rindan, salvo ante convicciones de honor y sensatez." — Winston Churchill</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="219.75" customHeight="1">
       <c r="A31" s="47" t="n">
@@ -7107,6 +7407,16 @@
 • La producción propia tiene valor</t>
         </is>
       </c>
+      <c r="AL31" t="inlineStr">
+        <is>
+          <t>"Vender una cosa más cara de lo que vale, o comprarla más barata de lo que vale, es en sí mismo injusto e ilícito." — Tomás de Aquino</t>
+        </is>
+      </c>
+      <c r="AM31" t="inlineStr">
+        <is>
+          <t>"Producir con recursos locales para necesidades locales es la forma más racional de vida económica." — E. F. Schumacher</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="219.75" customHeight="1">
       <c r="A32" s="49" t="n">
@@ -7315,6 +7625,16 @@
 • Su compañía es la fuente del verdadero descanso</t>
         </is>
       </c>
+      <c r="AL32" t="inlineStr">
+        <is>
+          <t>"El sueño que desenreda la madeja enmarañada de las preocupaciones, bálsamo de las mentes heridas, principal alimento en el banquete de la vida." — William Shakespeare</t>
+        </is>
+      </c>
+      <c r="AM32" t="inlineStr">
+        <is>
+          <t>"Tanto el sueño como el desvelo, cuando son desmedidos, hacen daño." — Hipócrates</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="219.75" customHeight="1">
       <c r="A33" s="8" t="n">
@@ -7519,6 +7839,16 @@
 • No rendirse aunque tarde la respuesta</t>
         </is>
       </c>
+      <c r="AL33" t="inlineStr">
+        <is>
+          <t>"La oración es, por decirlo con más audacia, una conversación con Dios." — Clemente de Alejandría</t>
+        </is>
+      </c>
+      <c r="AM33" t="inlineStr">
+        <is>
+          <t>"¿Adónde te escondiste, Amado, y me dejaste con gemido? Como el ciervo huiste, habiéndome herido; salí tras ti clamando, y eras ido." — Juan de la Cruz</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="219.75" customHeight="1">
       <c r="A34" s="10" t="n">
@@ -7721,6 +8051,16 @@
 • El propósito final es la gloria del Padre</t>
         </is>
       </c>
+      <c r="AL34" t="inlineStr">
+        <is>
+          <t>"La visión es el arte de ver lo invisible." — Jonathan Swift</t>
+        </is>
+      </c>
+      <c r="AM34" t="inlineStr">
+        <is>
+          <t>"Nuestra tarea principal no es ver lo que se vislumbra a lo lejos, sino hacer lo que está claramente al alcance de la mano." — Thomas Carlyle</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="219.75" customHeight="1">
       <c r="A35" s="12" t="n">
@@ -7924,6 +8264,16 @@
 • Comunicar bien trae satisfacción mutua</t>
         </is>
       </c>
+      <c r="AL35" t="inlineStr">
+        <is>
+          <t>"Por eso tenemos dos oídos y una sola boca: para escuchar más y hablar menos." — Zenón de Citio</t>
+        </is>
+      </c>
+      <c r="AM35" t="inlineStr">
+        <is>
+          <t>"La palabra es plata; el silencio es oro. La palabra es del tiempo; el silencio, de la eternidad." — Thomas Carlyle</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="219.75" customHeight="1">
       <c r="A36" s="14" t="n">
@@ -8126,6 +8476,16 @@
 • La estabilidad interior no depende del monto</t>
         </is>
       </c>
+      <c r="AL36" t="inlineStr">
+        <is>
+          <t>"¿Qué hay más grande para dos almas humanas que sentir que están unidas para toda la vida, para fortalecerse una a la otra en todo trabajo y apoyarse una en la otra en toda tristeza?" — George Eliot</t>
+        </is>
+      </c>
+      <c r="AM36" t="inlineStr">
+        <is>
+          <t>"La codicia, el deseo de tener más de lo que necesitamos, debe arrancarse temprano y con cuidado, y sembrarse en su lugar la disposición a compartir con los demás." — John Locke</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="219.75" customHeight="1">
       <c r="A37" s="2" t="n">
@@ -8327,6 +8687,16 @@
 • La falta de disciplina cobra factura después</t>
         </is>
       </c>
+      <c r="AL37" t="inlineStr">
+        <is>
+          <t>"La inspiración es para aficionados; los demás simplemente nos presentamos y nos ponemos a trabajar." — Chuck Close</t>
+        </is>
+      </c>
+      <c r="AM37" t="inlineStr">
+        <is>
+          <t>"No permitas que ocurra una sola excepción hasta que el nuevo hábito esté firmemente arraigado en tu vida." — William James</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="219.75" customHeight="1">
       <c r="A38" s="4" t="n">
@@ -8529,6 +8899,16 @@
           <t>• Vivir en unidad: Tener un mismo sentir.  
 • Practicar el amor: Ser compasivos, misericordiosos y amigables.  
 • Amarnos como hermanos: Mostrar amor con nuestras acciones.</t>
+        </is>
+      </c>
+      <c r="AL38" t="inlineStr">
+        <is>
+          <t>"Si vivís solo, ¿a quién le vas a lavar los pies? ¿A quién vas a cuidar?" — Basilio de Cesarea</t>
+        </is>
+      </c>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>"Solos podemos hacer muy poco; juntos podemos hacer muchísimo." — Helen Keller</t>
         </is>
       </c>
     </row>
@@ -8738,6 +9118,16 @@
 • Seguir dando fruto es posible en cualquier etapa</t>
         </is>
       </c>
+      <c r="AL39" t="inlineStr">
+        <is>
+          <t>"Amen la infancia; favorezcan sus juegos, sus placeres, su amable instinto." — Jean-Jacques Rousseau</t>
+        </is>
+      </c>
+      <c r="AM39" t="inlineStr">
+        <is>
+          <t>"Cada etapa de la vida tiene su propia sazón: la fragilidad de los niños, el ímpetu de los jóvenes, la seriedad de la edad madura y la madurez de la vejez." — Cicerón</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="219.75" customHeight="1">
       <c r="A40" s="8" t="n">
@@ -8938,6 +9328,16 @@
 • Cambia el estatus delante de Dios</t>
         </is>
       </c>
+      <c r="AL40" t="inlineStr">
+        <is>
+          <t>"Casi toda la suma de nuestra sabiduría consiste en dos puntos: el conocimiento que el hombre debe tener de Dios y el que debe tener de sí mismo." — Juan Calvino</t>
+        </is>
+      </c>
+      <c r="AM40" t="inlineStr">
+        <is>
+          <t>"Cuanto es el hombre delante de Dios, tanto es, y no más." — Francisco de Asís</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="219.75" customHeight="1">
       <c r="A41" s="10" t="n">
@@ -9146,6 +9546,16 @@
           <t>• El mayor debe ser como el más joven
 • El que sirve es el que dirige
 • El liderazgo de Jesús invierte jerarquías</t>
+        </is>
+      </c>
+      <c r="AL41" t="inlineStr">
+        <is>
+          <t>"Aprendí que el valor no era la ausencia de miedo, sino el triunfo sobre él. El valiente no es quien no siente miedo, sino quien vence ese miedo." — Nelson Mandela</t>
+        </is>
+      </c>
+      <c r="AM41" t="inlineStr">
+        <is>
+          <t>"Dios Todopoderoso ha puesto delante de mí dos grandes objetivos: la supresión del comercio de esclavos y la reforma de las costumbres." — William Wilberforce</t>
         </is>
       </c>
     </row>
@@ -9355,6 +9765,16 @@
 • Ir juntos, incluso en lo difícil</t>
         </is>
       </c>
+      <c r="AL42" t="inlineStr">
+        <is>
+          <t>"Muchas manos hacen liviano el trabajo." — John Heywood</t>
+        </is>
+      </c>
+      <c r="AM42" t="inlineStr">
+        <is>
+          <t>"El principio más profundo de la naturaleza humana es el anhelo de ser apreciado." — William James</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="219.75" customHeight="1">
       <c r="A43" s="14" t="n">
@@ -9559,6 +9979,16 @@
 • Ser generosos — Compartir con otros produce gratitud a Dios.</t>
         </is>
       </c>
+      <c r="AL43" t="inlineStr">
+        <is>
+          <t>"Toma mi plata y mi oro: ni una blanca quiero retener." — Frances Ridley Havergal</t>
+        </is>
+      </c>
+      <c r="AM43" t="inlineStr">
+        <is>
+          <t>"Hay quienes dan con alegría, y esa alegría es su recompensa." — Khalil Gibran</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="219.75" customHeight="1">
       <c r="A44" s="2" t="n">
@@ -9766,6 +10196,16 @@
 • Lo que se hizo por fe permanece</t>
         </is>
       </c>
+      <c r="AL44" t="inlineStr">
+        <is>
+          <t>"Las vidas de los grandes nos recuerdan que podemos hacer sublime la nuestra y, al partir, dejar tras nosotros huellas en las arenas del tiempo." — Henry Wadsworth Longfellow</t>
+        </is>
+      </c>
+      <c r="AM44" t="inlineStr">
+        <is>
+          <t>"Liberás a un prisionero, pero descubrís que el verdadero prisionero eras vos." — Lewis B. Smedes</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="219.75" customHeight="1">
       <c r="A45" s="4" t="n">
@@ -9966,6 +10406,16 @@
 • Practicar la justicia — Honrar a quienes sirven y trabajan.</t>
         </is>
       </c>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>"No hay un solo palmo en todo el dominio de nuestra existencia humana sobre el cual Cristo, que es soberano de todo, no clame: ¡Mío!" — Abraham Kuyper</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>"Si miramos lo de afuera, hay diferencia entre lavar los platos y predicar la Palabra de Dios; pero en cuanto a agradar a Dios, ninguna." — William Tyndale</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="219.75" customHeight="1">
       <c r="A46" s="6" t="n">
@@ -10169,6 +10619,16 @@
           <t>• Invocar a Dios en la angustia.
 • Confiar en su liberación.
 • Honrar a Dios por su respuesta.</t>
+        </is>
+      </c>
+      <c r="AL46" t="inlineStr">
+        <is>
+          <t>"Ante las enfermedades, acostumbrate a dos cosas: ayudar, o al menos no hacer daño." — Hipócrates</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>"Si podés conservar la calma cuando todos a tu alrededor la pierden y te culpan por ello… serás un hombre, hijo mío." — Rudyard Kipling</t>
         </is>
       </c>
     </row>
@@ -10380,6 +10840,16 @@
 • Dios da fuerza para seguir caminando.</t>
         </is>
       </c>
+      <c r="AL47" t="inlineStr">
+        <is>
+          <t>"Cuando la paz, como un río, acompaña mi camino, o cuando las penas ruedan como olas del mar, sea cual sea mi suerte, me enseñaste a decir: está bien con mi alma." — Horatio G. Spafford</t>
+        </is>
+      </c>
+      <c r="AM47" t="inlineStr">
+        <is>
+          <t>"Tú que tanto me has dado, dame una cosa más: un corazón agradecido." — George Herbert</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="219.75" customHeight="1">
       <c r="A48" s="10" t="n">
@@ -10586,6 +11056,16 @@
           <t>• Muchos planes hay en el corazón humano
 • El consejo de Dios prevalece
 • Someter los planes propios a Su voluntad</t>
+        </is>
+      </c>
+      <c r="AL48" t="inlineStr">
+        <is>
+          <t>"Guía mis pasos; no pido ver la escena lejana: un paso me basta." — John Henry Newman</t>
+        </is>
+      </c>
+      <c r="AM48" t="inlineStr">
+        <is>
+          <t>"Nuestras dudas son traidoras y nos hacen perder el bien que a menudo podríamos ganar, por temor a intentarlo." — William Shakespeare</t>
         </is>
       </c>
     </row>
@@ -10801,6 +11281,16 @@
 • Dios restaura lo que el distanciamiento rompe</t>
         </is>
       </c>
+      <c r="AL49" t="inlineStr">
+        <is>
+          <t>"Soy doctor y predicador, y sin embargo hago como un niño: cada mañana leo y recito, palabra por palabra, los Mandamientos, el Credo, el Padrenuestro y los Salmos." — Martín Lutero</t>
+        </is>
+      </c>
+      <c r="AM49" t="inlineStr">
+        <is>
+          <t>"Los niños nunca han sido muy buenos para escuchar a sus mayores, pero nunca han dejado de imitarlos." — James Baldwin</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="219.75" customHeight="1">
       <c r="A50" s="14" t="n">
@@ -11002,6 +11492,16 @@
           <t>• La prioridad máxima: buscar primero el reino de Dios.
 • El estándar de vida: y su justicia.
 • La promesa de provisión: y todas estas cosas les serán añadidas.</t>
+        </is>
+      </c>
+      <c r="AL50" t="inlineStr">
+        <is>
+          <t>"El préstamo a menudo se pierde a sí mismo y pierde también al amigo." — William Shakespeare</t>
+        </is>
+      </c>
+      <c r="AM50" t="inlineStr">
+        <is>
+          <t>"La esperanza significa esperar cuando las cosas son desesperadas; si no, no es ninguna virtud." — G. K. Chesterton</t>
         </is>
       </c>
     </row>
@@ -11217,6 +11717,16 @@
 • Cada paso aumenta la claridad</t>
         </is>
       </c>
+      <c r="AL51" t="inlineStr">
+        <is>
+          <t>"Nadie debería avergonzarse de reconocer que se equivocó, que no es sino decir, con otras palabras, que hoy es más sabio que ayer." — Alexander Pope</t>
+        </is>
+      </c>
+      <c r="AM51" t="inlineStr">
+        <is>
+          <t>"Respecto del miedo y la audacia, el valor es el término medio: el que se excede en audacia es temerario, y el que se excede en miedo, cobarde." — Aristóteles</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="219.75" customHeight="1">
       <c r="A52" s="4" t="n">
@@ -11424,6 +11934,16 @@
 • Nunca se deja de aprender</t>
         </is>
       </c>
+      <c r="AL52" t="inlineStr">
+        <is>
+          <t>"Damos forma a nuestras herramientas y, después, ellas nos dan forma a nosotros." — John M. Culkin</t>
+        </is>
+      </c>
+      <c r="AM52" t="inlineStr">
+        <is>
+          <t>"El artesano que quiere hacer bien su trabajo debe primero afilar sus herramientas." — Confucio</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="219.75" customHeight="1">
       <c r="A53" s="6" t="n">
@@ -11626,6 +12146,16 @@
           <t>• El poder de la comunicación bondadosa 
 • Bienestar y alivio para el interior (el alma)
 • Salud y efecto integral (el cuerpo o los huesos)</t>
+        </is>
+      </c>
+      <c r="AL53" t="inlineStr">
+        <is>
+          <t>"¡Salve, Príncipe de paz nacido del cielo! ¡Salve, Sol de justicia! Luz y vida a todos trae, y se levanta con sanidad en sus alas." — Charles Wesley</t>
+        </is>
+      </c>
+      <c r="AM53" t="inlineStr">
+        <is>
+          <t>"Un poco de filosofía inclina la mente del hombre al ateísmo; pero la profundidad en la filosofía lleva las mentes de los hombres de vuelta a la religión." — Francis Bacon</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Frases célebres: análisis de fuentes de las 260 y reemplazo de 15 dudosas o falsas
Documento de revisión en Word con el nivel de verificación de cada frase.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -1675,7 +1675,7 @@
       </c>
       <c r="J5" s="30" t="inlineStr">
         <is>
-          <t>"El vigor de nuestra vida espiritual estará en exacta proporción al lugar que la Biblia ocupe en nuestra vida y pensamientos." — atribuida a George Müller</t>
+          <t>"La lectura es el examen atento de las Escrituras con toda la aplicación del espíritu." — Guigo II el Cartujo</t>
         </is>
       </c>
       <c r="K5" s="30" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="R6" s="37" t="inlineStr">
         <is>
-          <t>"El carácter es lo que sos en la oscuridad." — Dwight L. Moody</t>
+          <t>"El perfecto valor consiste en hacer sin testigos lo que uno sería capaz de hacer delante de todo el mundo." — François de La Rochefoucauld</t>
         </is>
       </c>
       <c r="S6" s="37" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="J13" s="53" t="inlineStr">
         <is>
-          <t>"Los líderes que no escuchan terminarán rodeados de personas que no tienen nada que decir." — atribuida a Andy Stanley</t>
+          <t>"Aprendé a escuchar y sacarás provecho aun de los que hablan mal." — Plutarco</t>
         </is>
       </c>
       <c r="K13" s="53" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="N13" s="53" t="inlineStr">
         <is>
-          <t>"La confianza es la forma más elevada de motivación humana." — Stephen R. Covey</t>
+          <t>"Rodeate de las mejores personas que puedas encontrar, delegá autoridad y no interfieras." — Ronald Reagan</t>
         </is>
       </c>
       <c r="O13" s="53" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="N15" s="40" t="inlineStr">
         <is>
-          <t>"Un presupuesto es decirle a tu dinero adónde ir, en vez de preguntarte adónde se fue." — Dave Ramsey</t>
+          <t>"Un presupuesto es decirle a tu dinero adónde ir, en vez de preguntarte adónde se fue." — John C. Maxwell, citado por Dave Ramsey</t>
         </is>
       </c>
       <c r="O15" s="40" t="inlineStr">
@@ -5356,7 +5356,7 @@
       </c>
       <c r="R22" s="40" t="inlineStr">
         <is>
-          <t>"La manera más segura de duplicar tu dinero es doblarlo una vez y guardarlo en el bolsillo." — atribuida a Kin Hubbard</t>
+          <t>"Ingreso anual, veinte libras; gasto anual, diecinueve libras con diecinueve: resultado, felicidad. Ingreso anual, veinte libras; gasto anual, veinte libras con seis peniques: resultado, miseria." — Charles Dickens</t>
         </is>
       </c>
       <c r="S22" s="40" t="inlineStr">
@@ -5782,7 +5782,7 @@
       </c>
       <c r="R24" s="47" t="inlineStr">
         <is>
-          <t>"El éxito es la suma de pequeños esfuerzos, repetidos día tras día." — atribuida a Robert Collier</t>
+          <t>"Si añadís un poco a lo poco, y lo hacés seguido, pronto eso poco se hará grande." — Hesíodo</t>
         </is>
       </c>
       <c r="S24" s="47" t="inlineStr">
@@ -6625,7 +6625,7 @@
       </c>
       <c r="N28" s="35" t="inlineStr">
         <is>
-          <t>"De todas las maneras concebibles, la familia es un vínculo con nuestro pasado y un puente hacia nuestro futuro." — atribuida a Alex Haley</t>
+          <t>"El primer vínculo de la sociedad está en el matrimonio; después, en los hijos; luego, en una casa con todo en común: ese es el principio de la ciudad y el semillero de la república." — Cicerón</t>
         </is>
       </c>
       <c r="O28" s="35" t="inlineStr">
@@ -7720,7 +7720,7 @@
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
-          <t>"Uno de los grandes usos de Twitter y Facebook será demostrar en el último día que la falta de oración no fue por falta de tiempo." — atribuida a John Piper</t>
+          <t>"Tu deseo es tu oración; si tu deseo es continuo, continua es tu oración." — Agustín de Hipona</t>
         </is>
       </c>
       <c r="S33" s="8" t="inlineStr">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="J34" s="10" t="inlineStr">
         <is>
-          <t>"El liderazgo es la capacidad de convertir la visión en realidad." — atribuida a Warren Bennis</t>
+          <t>"Si pudiéramos saber primero dónde estamos y hacia dónde vamos, podríamos juzgar mejor qué hacer y cómo hacerlo." — Abraham Lincoln</t>
         </is>
       </c>
       <c r="K34" s="10" t="inlineStr">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="R34" s="10" t="inlineStr">
         <is>
-          <t>"Un líder lleva a la gente adonde quiere ir. Un gran líder la lleva adonde no necesariamente quiere ir, pero adonde debe estar." — atribuida a Rosalynn Carter</t>
+          <t>"Las grandes obras se realizan no por la fuerza, sino por la perseverancia." — Samuel Johnson</t>
         </is>
       </c>
       <c r="S34" s="10" t="inlineStr">
@@ -8956,7 +8956,7 @@
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>"Muchas de las cosas que necesitamos pueden esperar. El niño no puede. Su nombre es Hoy." — Gabriela Mistral</t>
+          <t>"Hay que pedir en oración una mente sana en un cuerpo sano." — Juvenal</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
@@ -9383,7 +9383,7 @@
       </c>
       <c r="J41" s="10" t="inlineStr">
         <is>
-          <t>"Un líder es el que conoce el camino, recorre el camino y muestra el camino." — John C. Maxwell</t>
+          <t>"La verdadera medida del liderazgo es la influencia: nada más, nada menos." — John C. Maxwell</t>
         </is>
       </c>
       <c r="K41" s="10" t="inlineStr">
@@ -10074,7 +10074,7 @@
       </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>"La verdad sin amor es demasiado dura; el amor sin verdad es demasiado blando." — John Stott</t>
+          <t>"La verdad se vuelve dura si no la suaviza el amor, y el amor se vuelve blando si no lo fortalece la verdad." — John Stott</t>
         </is>
       </c>
       <c r="S44" s="2" t="inlineStr">
@@ -11356,7 +11356,7 @@
       </c>
       <c r="N50" s="14" t="inlineStr">
         <is>
-          <t>"Preocuparse no vacía el mañana de su dolor; vacía el hoy de su fuerza." — Corrie ten Boom</t>
+          <t>"La ansiedad no le quita al mañana sus penas; solo le quita al hoy su fuerza." — Alexander Maclaren</t>
         </is>
       </c>
       <c r="O50" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Versículos: los 14 cambios decididos, con guion reescrito, y fechas especiales
Viernes Santo, Domingo de Pascua y Navidad llevan versículo propio y un aviso «Especial» en la app.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -1373,14 +1373,15 @@
       </c>
       <c r="AH3" s="25" t="inlineStr">
         <is>
-          <t>2 Corintios 9:6 — Pero recuerden esto: El que poco siembra, poco cosecha; y el que mucho siembra, mucho cosecha.</t>
+          <t>Salmos 24:1 — ¡Del Señor son la tierra y su plenitud!
+¡Del Señor son el mundo y sus habitantes!</t>
         </is>
       </c>
       <c r="AI3" s="23" t="inlineStr">
         <is>
-          <t>• Sembrar generosamente trae cosecha generosa
-• La escasez en la siembra limita el resultado
-• La actitud al sembrar importa</t>
+          <t>• No somos dueños: somos mayordomos
+• Cuidar la tierra es cuidar a los que vienen detrás
+• La plenitud de la tierra es una herencia para preservar</t>
         </is>
       </c>
       <c r="AJ3" s="25" t="inlineStr">
@@ -2618,14 +2619,17 @@
       </c>
       <c r="Z9" s="42" t="inlineStr">
         <is>
-          <t>Mateo 5:37 — Cuando ustedes digan algo, que sea “sí, sí”, o “no, no”; porque lo que es más de esto, proviene del mal.</t>
+          <t>Salmos 42:5 — ¿Por qué te desanimas, alma mía?
+¿Por qué te inquietas dentro de mí?
+Espera en Dios, porque aún debo alabarlo.
+¡Él es mi Dios! ¡Él es mi salvador!</t>
         </is>
       </c>
       <c r="AA9" s="43" t="inlineStr">
         <is>
-          <t>• Hablar con honestidad.
-• Cumplir nuestra palabra.
-• Ser íntegros en nuestras decisiones.</t>
+          <t>• Ponerle nombre a lo que sentimos, delante de Dios
+• Reconocer el desánimo sin quedarse a vivir en él
+• Volver a anclar la esperanza en Dios</t>
         </is>
       </c>
       <c r="AB9" s="42" t="inlineStr">
@@ -2642,14 +2646,15 @@
       </c>
       <c r="AD9" s="42" t="inlineStr">
         <is>
-          <t>Juan 3:16 — »Porque de tal manera amó Dios al mundo, que ha dado a su Hijo unigénito, para que todo aquel que en él cree no se pierda, sino que tenga vida eterna.</t>
+          <t>Salmos 101:2-3 — Quiero seguir el camino de la perfección. ¿Cuándo vendrás a visitarme? En mi casa quiero vivir con un corazón intachable.
+No pondré delante de mis ojos nada que sea indigno. Aborrezco la obra de los que se desvían; no quiero tener nada que ver con ellos.</t>
         </is>
       </c>
       <c r="AE9" s="43" t="inlineStr">
         <is>
-          <t>• Dios nos ama — Su amor es inmenso e incondicional.
-• Dios dio a su Hijo — Jesús es el regalo de salvación.
-• Creer en Jesús da vida eterna — La fe en Él nos libra de la perdición.</t>
+          <t>• Depender de la guía de Dios
+• La integridad empieza en lo íntimo y en el hogar
+• Filtrar lo que miramos y rechazar lo que nos daña</t>
         </is>
       </c>
       <c r="AF9" s="42" t="inlineStr">
@@ -2828,7 +2833,7 @@
       </c>
       <c r="Z10" s="45" t="inlineStr">
         <is>
-          <t>Genesis 1:26 — Entonces dijo Dios: Hagamos al hombre a nuestra imagen y semejanza! Que domine en toda la tierra sobre los peces del mar, sobre las aves de los cielos y las bestias</t>
+          <t>Génesis 1:26 — Entonces dijo Dios: «¡Hagamos al hombre a nuestra imagen y semejanza! ¡Que domine en toda la tierra sobre los peces del mar, sobre las aves de los cielos y las bestias, y sobre todo animal que repta sobre la tierra!»</t>
         </is>
       </c>
       <c r="AA10" s="47" t="inlineStr">
@@ -3520,15 +3525,14 @@
       </c>
       <c r="AH13" s="53" t="inlineStr">
         <is>
-          <t>Proverbios 29:18 — Cuando no hay visión, el pueblo se desvía;
-¡dichoso aquel que obedece la ley!</t>
+          <t>1 Pedro 2:24 — Él mismo llevó en su cuerpo nuestros pecados al madero, para que nosotros, muertos ya al pecado, vivamos para la justicia. Por sus heridas fueron ustedes sanados.</t>
         </is>
       </c>
       <c r="AI13" s="53" t="inlineStr">
         <is>
-          <t>• Sin dirección el pueblo se dispersa
-• La Palabra de Dios da orden y propósito
-• Guardar la palabra trae bienestar</t>
+          <t>• Jesús cargó en la cruz lo que no podíamos cargar
+• Murió para que vivamos para la justicia
+• Por sus heridas fuimos sanados</t>
         </is>
       </c>
       <c r="AJ13" s="53" t="inlineStr">
@@ -3671,14 +3675,14 @@
       </c>
       <c r="X14" s="35" t="inlineStr">
         <is>
-          <t>Genesis 2:24 — Por eso el hombre dejará a su padre y a su madre, y se unirá a su mujer, y serán un solo ser.</t>
+          <t>Juan 11:25 — Jesús le dijo: «Yo soy la resurrección y la vida; el que cree en mí, aunque esté muerto, vivirá.»</t>
         </is>
       </c>
       <c r="Y14" s="35" t="inlineStr">
         <is>
-          <t>• Dejar y unirse marca un nuevo inicio
-• Una sola carne implica unidad profunda
-• El matrimonio redefine las prioridades</t>
+          <t>• Jesús no solo da vida: él es la resurrección y la vida
+• La muerte no tiene la última palabra
+• Creer en él cambia cómo vivimos hoy</t>
         </is>
       </c>
       <c r="Z14" s="35" t="inlineStr">
@@ -3707,14 +3711,15 @@
       </c>
       <c r="AD14" s="35" t="inlineStr">
         <is>
-          <t>1 Samuel 12:23 — Lejos estará de mí pecar contra el Señor dejando de rogar por ustedes; al contrario, me comprometo a instruirlos en el camino bueno y recto,</t>
+          <t>Colosenses 3:18-19 — Ustedes las esposas, respeten a sus esposos, como conviene en el Señor.
+Ustedes los esposos, amen a sus esposas, y no las traten con dureza.</t>
         </is>
       </c>
       <c r="AE14" s="35" t="inlineStr">
         <is>
-          <t>• Orar por otros: Interceder es una responsabilidad.
-• Enseñar el camino: Guiar a otros hacia lo bueno y correcto.
-• Servir con compromiso: No abandonar a quienes Dios puso a nuestro cuidado.</t>
+          <t>• El respeto libre de la esposa, como conviene en el Señor
+• El amor del esposo, que se entrega como Cristo
+• Ni dureza ni aspereza en el trato</t>
         </is>
       </c>
       <c r="AF14" s="35" t="inlineStr">
@@ -4800,14 +4805,14 @@
       </c>
       <c r="AF19" s="51" t="inlineStr">
         <is>
-          <t>Colosenses 3:23 — Y todo lo que hagan, háganlo de corazón, como para el Señor y no como para la gente,</t>
+          <t>Mateo 6:3-4 — Cuando tú des limosna, que no sepa tu mano izquierda lo que hace tu mano derecha, para que tu limosna sea en secreto; y tu Padre, que ve en lo secreto, te recompensará.</t>
         </is>
       </c>
       <c r="AG19" s="51" t="inlineStr">
         <is>
-          <t>• Todo trabajo se hace para el Señor
-• La actitud del corazón importa más que la tarea
-• El servicio de corazón no busca aplausos</t>
+          <t>• La intención pura por encima del ego
+• Discreción: la mano izquierda no se entera
+• Dios ve lo secreto y recompensa</t>
         </is>
       </c>
       <c r="AH19" s="51" t="inlineStr">
@@ -5452,14 +5457,15 @@
       </c>
       <c r="AH22" s="40" t="inlineStr">
         <is>
-          <t>Santiago 3:17 — Pero la sabiduría que viene de lo alto es, ante todo, pura, y además pacífica, amable, benigna, llena de compasión y de buenos frutos, imparcial y genuina.</t>
+          <t>Hageo 1:6-7 — Ustedes siembran mucho, pero cosechan poco; comen, pero no se sacian; beben, pero no quedan satisfechos; se visten, pero no se calientan; y el que trabaja a jornal recibe su salario en saco roto.
+Así dice el Señor de los ejércitos: «Reflexionen sobre su conducta.»</t>
         </is>
       </c>
       <c r="AI22" s="40" t="inlineStr">
         <is>
-          <t>• Sabiduría pura.
-• Actuar con amabilidad y compasión.
-• Dar buenos frutos.</t>
+          <t>• Esfuerzo sin fruto: trabajar mucho y ver poco
+• Consumir sin saciarse
+• La fuga invisible: el salario en saco roto</t>
         </is>
       </c>
       <c r="AJ22" s="40" t="inlineStr">
@@ -5844,14 +5850,15 @@
       </c>
       <c r="AB24" s="47" t="inlineStr">
         <is>
-          <t>Job 8:7 — Las pocas riquezas que llegaste a poseer no podrán compararse con las que tendrás después.</t>
+          <t>Salmos 143:8 — Muéstrame tu misericordia por la mañana, porque en ti he puesto mi confianza.
+Muéstrame el camino que debo seguir, porque en tus manos he puesto mi vida.</t>
         </is>
       </c>
       <c r="AC24" s="47" t="inlineStr">
         <is>
-          <t>• Quien habla es Bildad: Un amigo de Job cuya idea de Dios fue corregida (42:7).  
-• Los comienzos pequeños: No definen el final ni son una vergüenza.  
-• Dios no abandona: Restauró a Job por gracia, no como pago.</t>
+          <t>• La renovación diaria: empezar «por la mañana»
+• La fe como capital principal: confianza antes que recursos
+• Pedir dirección en lugar de improvisar a ciegas</t>
         </is>
       </c>
       <c r="AD24" s="47" t="inlineStr">
@@ -6476,15 +6483,14 @@
       </c>
       <c r="Z27" s="58" t="inlineStr">
         <is>
-          <t>1 Corintios 16:13-14 — Manténganse atentos y firmes en la fe; sean fuertes y valientes.
-Háganlo todo con amor.</t>
+          <t>1 Tesalonicenses 2:3-4 — Nuestra exhortación no se basó en el error ni en motivos impuros, ni fue con engaño, sino que, así como Dios nos aprobó y nos confió el evangelio, así hablamos, no para agradar a los hombres sino a Dios, que examina nuestro corazón.</t>
         </is>
       </c>
       <c r="AA27" s="53" t="inlineStr">
         <is>
-          <t>• Firmeza en la fe.
-• Fuerza y valentía.
-• Hacer todo con amor.</t>
+          <t>• Intención pura y sin engaño
+• Una confianza recibida de Dios
+• Fieles al propósito por encima de la aprobación ajena</t>
         </is>
       </c>
       <c r="AB27" s="53" t="inlineStr">
@@ -7170,15 +7176,14 @@
       </c>
       <c r="AH30" s="43" t="inlineStr">
         <is>
-          <t>Job 22:28 — Llevarás a buen término todos tus planes,
-y en tus caminos brillará la luz.</t>
+          <t>Lamentaciones 3:40 — Examinemos nuestra conducta; busquemos al Señor y volvámonos a él.</t>
         </is>
       </c>
       <c r="AI30" s="43" t="inlineStr">
         <is>
-          <t>• Quien habla es Elifaz: Un amigo de Job cuya idea de Dios fue corregida (42:7).
-• Confía en Dios: Pon tus planes en sus manos.
-• Camina en su luz: Busca su dirección en cada paso.</t>
+          <t>• Examinar con sinceridad nuestra conducta
+• Volver a poner el enfoque en el Señor
+• Corregir el rumbo a propósito</t>
         </is>
       </c>
       <c r="AJ30" s="43" t="inlineStr">
@@ -8005,14 +8010,14 @@
       </c>
       <c r="AD34" s="10" t="inlineStr">
         <is>
-          <t>Filipenses 3:14 — ¡prosigo a la meta, al premio del supremo llamamiento de Dios en Cristo Jesús!</t>
+          <t>Proverbios 16:21 — Al de corazón sabio se le llama prudente; la dulzura de los labios aumenta el saber.</t>
         </is>
       </c>
       <c r="AE34" s="10" t="inlineStr">
         <is>
-          <t>• Enfocarse en la meta, no en lo pasado
-• Perseguir el premio supremo
-• La visión requiere dirección constante</t>
+          <t>• La sabiduría interior es la base de una visión clara
+• La palabra amable hace que el mensaje llegue
+• Comunicar bien multiplica el conocimiento</t>
         </is>
       </c>
       <c r="AF34" s="10" t="inlineStr">
@@ -9955,16 +9960,14 @@
       </c>
       <c r="AH43" s="14" t="inlineStr">
         <is>
-          <t>Éxodo 18:24-26 — Moisés atendió a la voz de su suegro, e hizo todo lo que le dijo,
-pues de entre todo Israel escogió hombres respetables y los puso a cargo del pueblo como jefes de grupos de mil, cien, cincuenta y diez personas.
-Ellos juzgaban al pueblo en todo momento y dictaban sentencia en todo asunto menor, y remitían a Moisés las cuestiones difíciles de resolver.</t>
+          <t>1 Corintios 13:3 — Y si repartiera todos mis bienes para dar de comer a los pobres, y si entregara mi cuerpo para ser quemado, y no tengo amor, de nada me sirve.</t>
         </is>
       </c>
       <c r="AI43" s="14" t="inlineStr">
         <is>
-          <t>• La humildad y docilidad del líder.
-• La delegación de autoridad y estructura.
-• La división de funciones según la complejidad.</t>
+          <t>• Dar bienes sin amor es solo una transacción
+• Dar el esfuerzo y el talento sin amor puede ser orgullo
+• El corazón con que damos el tiempo define su valor</t>
         </is>
       </c>
       <c r="AJ43" s="14" t="inlineStr">
@@ -11923,15 +11926,14 @@
       </c>
       <c r="AJ52" s="4" t="inlineStr">
         <is>
-          <t>Proverbios 1:5 — Que lo oiga el sabio, y aumente su saber,
-y que el entendido reciba consejo</t>
+          <t>Lucas 2:10-11 — Pero el ángel les dijo: «No teman, que les traigo una buena noticia, que será para todo el pueblo motivo de mucha alegría. Hoy, en la ciudad de David, les ha nacido un Salvador, que es Cristo el Señor.»</t>
         </is>
       </c>
       <c r="AK52" s="4" t="inlineStr">
         <is>
-          <t>• El sabio escucha y aumenta su saber
-• El aprendizaje continuo distingue al prudente
-• Nunca se deja de aprender</t>
+          <t>• No teman: Dios trae una buena noticia
+• Una alegría para todo el pueblo
+• Hoy nació el Salvador, Cristo el Señor</t>
         </is>
       </c>
       <c r="AL52" t="inlineStr">
@@ -20529,7 +20531,7 @@
       </c>
       <c r="C12" s="61" t="inlineStr">
         <is>
-          <t>Sembrar con generosidad</t>
+          <t>La tierra es del Señor</t>
         </is>
       </c>
       <c r="D12" s="61" t="inlineStr">
@@ -20544,47 +20546,47 @@
       </c>
       <c r="F12" s="61" t="inlineStr">
         <is>
-          <t>Pablo habla de la ofrenda para hermanos necesitados: dar con generosidad es sembrar. La cosecha no es una ganancia asegurada, sino frutos de justicia y gratitud a Dios (2 Corintios 9:10-11).</t>
+          <t>El salmo empieza con una afirmación que ordena todo: la tierra no es nuestra, es del Señor. Nosotros administramos lo que él nos presta.</t>
         </is>
       </c>
       <c r="G12" s="61" t="inlineStr">
         <is>
-          <t>La idea de «dar para recibir más plata», que convierte la generosidad en un negocio.</t>
+          <t>Usar la tierra como si fuera solo nuestra, sin pensar en quién viene después.</t>
         </is>
       </c>
       <c r="H12" s="61" t="inlineStr">
         <is>
-          <t>Esta semana ayudá a alguien que lo necesita, sin esperar nada a cambio.</t>
+          <t>Mirá hoy tu patio, tu chacra o tu cuadra y preguntate: ¿cómo lo cuidaría si supiera que es prestado?</t>
         </is>
       </c>
       <c r="I12" s="61" t="inlineStr">
         <is>
-          <t>El que guarda todo por miedo se pierde la alegría de compartir y de ver a Dios obrar a través de lo que da. Sembrar también es pensar en los que vienen detrás.</t>
+          <t>«El mundo y sus habitantes» también son del Señor. Cuidar la tierra es cuidar a las personas que viven de ella hoy y a las que vendrán.</t>
         </is>
       </c>
       <c r="J12" s="61" t="inlineStr">
         <is>
-          <t>Vecinos y productores que no se ayudan en los tiempos difíciles, cuando una mano a tiempo cambia todo.</t>
+          <t>Quemas, basura y arroyos contaminados que después pagan los vecinos y los hijos.</t>
         </is>
       </c>
       <c r="K12" s="61" t="inlineStr">
         <is>
-          <t>Cuando tu cosecha o tu trabajo rinda, compartí una parte con una familia que pasa necesidad.</t>
+          <t>Esta semana no quemes basura ni hojas: separá lo orgánico para abono y sacá el resto a la recolección.</t>
         </is>
       </c>
       <c r="L12" s="61" t="inlineStr">
         <is>
-          <t>Pablo agrega que cada uno dé lo que decidió en su corazón, no con tristeza ni por obligación, porque Dios ama al que da con alegría (9:7).</t>
+          <t>La plenitud de la tierra es una herencia. Lo que recibimos de nuestros padres lo dejamos, mejor o peor, a nuestros hijos.</t>
         </is>
       </c>
       <c r="M12" s="61" t="inlineStr">
         <is>
-          <t>Dar por presión, por quedar bien o por culpa.</t>
+          <t>Pensar solo en la cosecha de este año.</t>
         </is>
       </c>
       <c r="N12" s="61" t="inlineStr">
         <is>
-          <t>Orá primero y decidí en tu corazón cuánto dar y a quién. Después, dalo con alegría.</t>
+          <t>Plantá un árbol con tus hijos o tus nietos y contales por qué lo hacés.</t>
         </is>
       </c>
     </row>
@@ -22649,7 +22651,7 @@
       </c>
       <c r="C44" s="61" t="inlineStr">
         <is>
-          <t>Decir lo que de verdad sentís</t>
+          <t>¿Por qué te desanimas, alma mía?</t>
         </is>
       </c>
       <c r="D44" s="61" t="inlineStr">
@@ -22664,7 +22666,7 @@
       </c>
       <c r="F44" s="61" t="inlineStr">
         <is>
-          <t>Jesús habla de los juramentos: no hace falta jurar si nuestra palabra es verdadera. Un «sí» que es sí y un «no» que es no. Esa honestidad incluye no fingir lo que sentimos.</t>
+          <t>El salmista no esconde lo que siente: se pregunta en voz alta por qué está desanimado e inquieto. Ponerle nombre a lo que sentimos es el primer paso para salir.</t>
         </is>
       </c>
       <c r="G44" s="61" t="inlineStr">
@@ -22679,22 +22681,22 @@
       </c>
       <c r="I44" s="61" t="inlineStr">
         <is>
-          <t>Muchas veces decimos «sí» por presión y después cargamos enojo y cansancio. Un «no» honesto a tiempo cuida el alma y las relaciones.</t>
+          <t>Los salmos están llenos de lamentos: la Biblia no le tiene miedo a la tristeza. Reconocer el desánimo no es falta de fe; lo que daña es quedarse a vivir en él sin pedir ayuda.</t>
         </is>
       </c>
       <c r="J44" s="61" t="inlineStr">
         <is>
-          <t>La dificultad para decir que no, que termina en agotamiento y resentimiento.</t>
+          <t>Pensar que un creyente nunca debería sentirse triste.</t>
         </is>
       </c>
       <c r="K44" s="61" t="inlineStr">
         <is>
-          <t>Cuando te pidan un compromiso nuevo esta semana, tomate un momento y preguntate si de verdad podés.</t>
+          <t>Si la tristeza dura semanas o te quita las ganas de todo, hablalo con un profesional de la salud o con un consejero de confianza.</t>
         </is>
       </c>
       <c r="L44" s="61" t="inlineStr">
         <is>
-          <t>Ponerle nombre a lo que sentís ayuda a decidir mejor. La tristeza, el miedo o el enojo con nombre se manejan; sin nombre, nos manejan.</t>
+          <t>El salmista no se queda en la pregunta: se da una orden a sí mismo, «espera en Dios». La esperanza también se elige, todos los días.</t>
         </is>
       </c>
       <c r="M44" s="61" t="inlineStr">
@@ -22789,7 +22791,7 @@
       </c>
       <c r="C46" s="61" t="inlineStr">
         <is>
-          <t>Lo primero que tu mente necesita escuchar</t>
+          <t>Lo que ponés delante de tus ojos</t>
         </is>
       </c>
       <c r="D46" s="61" t="inlineStr">
@@ -22804,47 +22806,47 @@
       </c>
       <c r="F46" s="61" t="inlineStr">
         <is>
-          <t>Entre tantas voces que escuchamos cada día, hay una verdad que debería sonar más fuerte: Dios te ama tal como sos, y por amor no te deja como estás.</t>
+          <t>David quiere andar con integridad, pero sabe que no puede solo: le pide a Dios que venga a visitarlo.</t>
         </is>
       </c>
       <c r="G46" s="61" t="inlineStr">
         <is>
+          <t>Llenarse de contenidos todo el día sin preguntarse adónde nos llevan.</t>
+        </is>
+      </c>
+      <c r="H46" s="61" t="inlineStr">
+        <is>
+          <t>Antes de abrir el celular por la mañana, pedile a Dios sabiduría para elegir qué mirar.</t>
+        </is>
+      </c>
+      <c r="I46" s="61" t="inlineStr">
+        <is>
+          <t>«En mi casa quiero vivir con un corazón intachable»: la integridad no empieza en público, empieza puertas adentro, donde nadie nos ve.</t>
+        </is>
+      </c>
+      <c r="J46" s="61" t="inlineStr">
+        <is>
+          <t>Horas frente al celular antes de dormir, que dejan la mente cargada y el sueño liviano.</t>
+        </is>
+      </c>
+      <c r="K46" s="61" t="inlineStr">
+        <is>
+          <t>La última media hora del día, sin pantallas: una lectura, una oración o una charla. Probalo esta semana.</t>
+        </is>
+      </c>
+      <c r="L46" s="61" t="inlineStr">
+        <is>
+          <t>«No pondré delante de mis ojos nada que sea indigno»: lo que entra por los ojos va formando la mente. Elegir qué mirar es cuidar el alma.</t>
+        </is>
+      </c>
+      <c r="M46" s="61" t="inlineStr">
+        <is>
           <t>Comparaciones constantes en las redes que hacen sentir que nunca alcanza.</t>
         </is>
       </c>
-      <c r="H46" s="61" t="inlineStr">
-        <is>
-          <t>Hoy, antes de abrir las redes, leé Juan 3:16 en voz alta y poné tu nombre donde dice «el mundo».</t>
-        </is>
-      </c>
-      <c r="I46" s="61" t="inlineStr">
-        <is>
-          <t>El amor de Dios no fue de palabras: dio lo más valioso. Llenar la mente de esa verdad cambia cómo nos vemos.</t>
-        </is>
-      </c>
-      <c r="J46" s="61" t="inlineStr">
-        <is>
-          <t>Contenidos que enseñan que el valor de una persona depende de lo que tiene o de cuántos «me gusta» recibe.</t>
-        </is>
-      </c>
-      <c r="K46" s="61" t="inlineStr">
+      <c r="N46" s="61" t="inlineStr">
         <is>
           <t>Dejá de seguir tres cuentas que te hacen sentir menos y seguí una que te edifique.</t>
-        </is>
-      </c>
-      <c r="L46" s="61" t="inlineStr">
-        <is>
-          <t>El regalo es vida eterna para todo el que cree en Jesús. Esa fe se alimenta de lo que escuchamos: si lo que más oímos es miedo y queja, nos olvidamos de la esperanza que tenemos.</t>
-        </is>
-      </c>
-      <c r="M46" s="61" t="inlineStr">
-        <is>
-          <t>Horas frente al celular antes de dormir, que dejan la mente cargada y el sueño liviano.</t>
-        </is>
-      </c>
-      <c r="N46" s="61" t="inlineStr">
-        <is>
-          <t>La última media hora del día, sin pantallas: una lectura, una oración o una charla. Probalo esta semana.</t>
         </is>
       </c>
     </row>
@@ -24529,62 +24531,62 @@
       </c>
       <c r="C72" s="61" t="inlineStr">
         <is>
-          <t>Cuando falta la Palabra</t>
+          <t>Viernes Santo: por sus heridas</t>
         </is>
       </c>
       <c r="D72" s="61" t="inlineStr">
         <is>
-          <t>La palabra hebrea que en este proverbio se traduce como «visión» se usa para la revelación que Dios daba a sus profetas.</t>
+          <t>Pedro, que escribe esta carta, es el mismo discípulo que negó a Jesús tres veces la noche en que lo arrestaron.</t>
         </is>
       </c>
       <c r="E72" s="61" t="inlineStr">
         <is>
-          <t>Léxico hebreo de Strong (H2377) y Brown-Driver-Briggs</t>
+          <t>Lucas 22:54-62; 1 Pedro 1:1</t>
         </is>
       </c>
       <c r="F72" s="61" t="inlineStr">
         <is>
-          <t>Este proverbio no habla de metas de empresa: la «visión» es la revelación de Dios. Cuando falta su Palabra, el pueblo se desvía.</t>
+          <t>Hoy es Viernes Santo. Pedro, el que negó a Jesús, escribe que él llevó nuestros pecados en su cuerpo sobre la cruz. Lo que no podíamos cargar, lo cargó él.</t>
         </is>
       </c>
       <c r="G72" s="61" t="inlineStr">
         <is>
-          <t>Vivir corriendo, ocupados todo el día, sin saber hacia dónde vamos.</t>
+          <t>Vivir con culpas viejas, como si nadie las hubiera cargado.</t>
         </is>
       </c>
       <c r="H72" s="61" t="inlineStr">
         <is>
-          <t>Al empezar el día, elegí una sola tarea importante: si se hace, el resto importa menos.</t>
+          <t>Tomate hoy un momento en silencio, leé despacio 1 Pedro 2:24 y agradecé con tus palabras.</t>
         </is>
       </c>
       <c r="I72" s="61" t="inlineStr">
         <is>
-          <t>La segunda parte lo confirma: dichoso el que obedece la ley de Dios. Su Palabra ordena las prioridades, y lo urgente no siempre es lo importante.</t>
+          <t>La cruz no es solo perdón: es un cambio de rumbo. Jesús murió «para que vivamos para la justicia». Es también la mejor manera de ordenar las prioridades.</t>
         </is>
       </c>
       <c r="J72" s="61" t="inlineStr">
         <is>
-          <t>Lo urgente que se come lo importante: el celular, los mensajes, los imprevistos.</t>
+          <t>Un fin de semana largo que pasa sin recordar qué se celebra.</t>
         </is>
       </c>
       <c r="K72" s="61" t="inlineStr">
         <is>
-          <t>Separá cada día un tiempo para la Palabra antes de lo urgente, aunque sean diez minutos.</t>
+          <t>Este fin de semana, reservá un tiempo en familia para leer juntos lo que pasó en la cruz y en la resurrección (Lucas 23 y 24).</t>
         </is>
       </c>
       <c r="L72" s="61" t="inlineStr">
         <is>
-          <t>La dicha de la que habla no es tener todo resuelto, sino vivir en el camino de Dios. En este Viernes Santo recordamos hasta dónde llegó su amor por nosotros.</t>
+          <t>«Por sus heridas fueron ustedes sanados». Las heridas de Jesús sanan nuestra relación con Dios y nos enseñan a perdonar las heridas de otros.</t>
         </is>
       </c>
       <c r="M72" s="61" t="inlineStr">
         <is>
-          <t>Agendas tan llenas que no queda lugar para Dios ni para la familia.</t>
+          <t>Rencores que se arrastran años en la familia.</t>
         </is>
       </c>
       <c r="N72" s="61" t="inlineStr">
         <is>
-          <t>Este fin de semana de Pascua, reservá un tiempo en familia para leer juntos lo que pasó en la cruz y en la resurrección.</t>
+          <t>Pensá en alguien a quien te cuesta perdonar y orá hoy por esa persona. Si hubo abuso o violencia, buscá ayuda: perdonar no es quedarse en peligro.</t>
         </is>
       </c>
     </row>
@@ -24789,62 +24791,62 @@
       </c>
       <c r="C76" s="61" t="inlineStr">
         <is>
-          <t>Orar el uno por el otro</t>
+          <t>Respeto y amor en casa</t>
         </is>
       </c>
       <c r="D76" s="61" t="inlineStr">
         <is>
-          <t>Personas que oraron cada día durante cuatro semanas por el bienestar de un amigo mostraron más disposición a perdonarlo que quienes oraron sobre otros temas o solo pensaron cosas positivas de él.</t>
+          <t>Pablo escribió la carta a los Colosenses estando preso.</t>
         </is>
       </c>
       <c r="E76" s="61" t="inlineStr">
         <is>
-          <t>Lambert, Fincham y otros, Psychological Science, 2010</t>
+          <t>Colosenses 4:3 y 4:18</t>
         </is>
       </c>
       <c r="F76" s="61" t="inlineStr">
         <is>
-          <t>Samuel le dice al pueblo que sería un pecado dejar de orar por ellos. Si eso vale para un pueblo, cuánto más para la persona con quien compartimos la vida.</t>
+          <t>Pablo le habla primero a la esposa: respeto «como conviene en el Señor». No es inferioridad ni aceptar cualquier cosa: es una actitud libre, delante de Dios.</t>
         </is>
       </c>
       <c r="G76" s="61" t="inlineStr">
         <is>
-          <t>Parejas que oran por muchas cosas, pero casi nunca la una por la otra.</t>
+          <t>Hablar mal de la pareja con otros, o burlarse de ella delante de los hijos.</t>
         </is>
       </c>
       <c r="H76" s="61" t="inlineStr">
         <is>
-          <t>Orá cada día de esta semana por tu pareja, por su nombre y por algo concreto que esté viviendo.</t>
+          <t>Decí hoy algo bueno de tu pareja delante de otros.</t>
         </is>
       </c>
       <c r="I76" s="61" t="inlineStr">
         <is>
-          <t>Samuel no solo ora: se compromete a enseñar el camino bueno. En el matrimonio nos ayudamos a crecer, sin imponer ni sermonear.</t>
+          <t>Al esposo le pide amar. En la misma carta, el amor es «el vínculo perfecto» (3:14), y el modelo es Cristo, que se entregó.</t>
         </is>
       </c>
       <c r="J76" s="61" t="inlineStr">
         <is>
-          <t>Corregir a la pareja delante de otros o con tono de superioridad.</t>
+          <t>Esposos que piden respeto pero no se ocupan del hogar ni del corazón de su esposa.</t>
         </is>
       </c>
       <c r="K76" s="61" t="inlineStr">
         <is>
-          <t>Si tenés algo que decirle a tu pareja, hacelo en privado, con calma, y empezando por lo bueno.</t>
+          <t>Preguntale a tu pareja: ¿qué puedo hacer esta semana para que te sientas amada o amado y acompañada o acompañado?</t>
         </is>
       </c>
       <c r="L76" s="61" t="inlineStr">
         <is>
-          <t>Los deberes del matrimonio no compiten: se complementan. La pregunta no es quién hace más, sino cómo nos servimos mutuamente.</t>
+          <t>«No las traten con dureza». La Biblia le cierra la puerta al maltrato: ni gritos, ni humillaciones, ni violencia.</t>
         </is>
       </c>
       <c r="M76" s="61" t="inlineStr">
         <is>
-          <t>Pensar el matrimonio como un contrato de deberes y no como una entrega mutua.</t>
+          <t>Violencia que se esconde detrás de versículos sobre el matrimonio.</t>
         </is>
       </c>
       <c r="N76" s="61" t="inlineStr">
         <is>
-          <t>Preguntale a tu pareja: ¿qué puedo hacer esta semana para que te sientas acompañado o acompañada?</t>
+          <t>Si en tu casa hay violencia, no es la voluntad de Dios: llamá al 137 o buscá ayuda en alguien de confianza.</t>
         </is>
       </c>
     </row>
@@ -26859,7 +26861,7 @@
       </c>
       <c r="C107" s="61" t="inlineStr">
         <is>
-          <t>Para el Señor, aunque nadie aplauda</t>
+          <t>Que no se entere la mano izquierda</t>
         </is>
       </c>
       <c r="D107" s="61" t="inlineStr">
@@ -26874,37 +26876,37 @@
       </c>
       <c r="F107" s="61" t="inlineStr">
         <is>
-          <t>Pablo escribe a esclavos y trabajadores: lo que hagan, háganlo como para el Señor. Hoy lo aplicamos al servicio que nadie ve.</t>
+          <t>Jesús habla de los que daban limosna tocando trompeta para que todos los vieran (6:2). El problema no era dar, era dar para que los aplaudan.</t>
         </is>
       </c>
       <c r="G107" s="61" t="inlineStr">
         <is>
-          <t>El cansancio de servir y sentir que nadie lo nota.</t>
+          <t>Servir esperando que nos agradezcan, y enojarse cuando no pasa.</t>
         </is>
       </c>
       <c r="H107" s="61" t="inlineStr">
         <is>
-          <t>Hoy, cuando sirvas, decí en silencio: «Esto es para vos, Señor».</t>
+          <t>Revisá tus motivaciones: ¿qué servicio seguirías haciendo aunque nadie te lo agradezca?</t>
         </is>
       </c>
       <c r="I107" s="61" t="inlineStr">
         <is>
-          <t>La actitud del corazón importa más que la tarea: el mismo servicio puede ser ofrenda o puede ser vanidad.</t>
+          <t>La imagen de las manos es una exageración a propósito: el servicio que agrada a Dios ni siquiera se anda contando a uno mismo.</t>
         </is>
       </c>
       <c r="J107" s="61" t="inlineStr">
         <is>
-          <t>Servir esperando que nos agradezcan, y enojarse cuando no pasa.</t>
+          <t>Publicar en las redes cada ayuda que damos.</t>
         </is>
       </c>
       <c r="K107" s="61" t="inlineStr">
         <is>
-          <t>Revisá tus motivaciones: ¿qué servicio seguirías haciendo aunque nadie te lo agradezca?</t>
+          <t>Hacé hoy un favor sin contárselo a nadie y sin subirlo a las redes.</t>
         </is>
       </c>
       <c r="L107" s="61" t="inlineStr">
         <is>
-          <t>Dios ve lo que nadie ve. Ese servicio silencioso es, muchas veces, el más valioso.</t>
+          <t>«Tu Padre, que ve en lo secreto». Dios ve lo que nadie ve, y ese servicio silencioso es, muchas veces, el más valioso.</t>
         </is>
       </c>
       <c r="M107" s="61" t="inlineStr">
@@ -28129,7 +28131,7 @@
       </c>
       <c r="C126" s="61" t="inlineStr">
         <is>
-          <t>Sabiduría para cerrar fugas</t>
+          <t>El salario en saco roto</t>
         </is>
       </c>
       <c r="D126" s="61" t="inlineStr">
@@ -28144,37 +28146,37 @@
       </c>
       <c r="F126" s="61" t="inlineStr">
         <is>
-          <t>Santiago describe la sabiduría que viene de Dios: pura, pacífica, genuina. Esa sabiduría también se pide para lo práctico (Santiago 1:5).</t>
+          <t>Hageo le habla a un pueblo que había vuelto del exilio: trabajaban mucho y cosechaban poco. Dios les pide que se detengan a pensar en lo que están haciendo.</t>
         </is>
       </c>
       <c r="G126" s="61" t="inlineStr">
         <is>
-          <t>Decisiones de dinero tomadas sin pensar ni orar.</t>
+          <t>Trabajar cada vez más y no saber adónde se va el dinero.</t>
         </is>
       </c>
       <c r="H126" s="61" t="inlineStr">
         <is>
-          <t>Antes de revisar tus gastos, pedile a Dios sabiduría con tus propias palabras.</t>
+          <t>Revisá los movimientos de tu cuenta o tu billetera del último mes y buscá gastos pequeños y repetidos que ya no recordás.</t>
         </is>
       </c>
       <c r="I126" s="61" t="inlineStr">
         <is>
-          <t>La sabiduría de lo alto es compasiva: no se trata de ser tacaño, sino de cuidar lo que tenemos para poder cuidar a otros.</t>
+          <t>«Comen, pero no se sacian»: consumir más no siempre llena. A veces gastamos para tapar un vacío.</t>
         </is>
       </c>
       <c r="J126" s="61" t="inlineStr">
         <is>
-          <t>Fugas pequeñas que no dejan nada para ayudar a nadie.</t>
+          <t>Compras por impulso para levantar el ánimo.</t>
         </is>
       </c>
       <c r="K126" s="61" t="inlineStr">
         <is>
-          <t>Revisá los movimientos de tu cuenta o tu billetera del último mes y buscá gastos pequeños y repetidos que ya no recordás.</t>
+          <t>Antes de una compra que no tenías pensada, esperá un día. Si mañana la seguís necesitando, decidila con calma.</t>
         </is>
       </c>
       <c r="L126" s="61" t="inlineStr">
         <is>
-          <t>Una vez detectadas, las fugas se cierran de a una. Lo que se recupera puede ir al ahorro o a ayudar a alguien.</t>
+          <t>El saco roto es la imagen de la fuga: lo que entra se pierde sin que nos demos cuenta. En Hageo, el fondo era de prioridades: habían dejado de lado la casa de Dios. No es un castigo automático, es una invitación a ordenar el corazón.</t>
         </is>
       </c>
       <c r="M126" s="61" t="inlineStr">
@@ -28184,7 +28186,7 @@
       </c>
       <c r="N126" s="61" t="inlineStr">
         <is>
-          <t>Cancelá esta semana un gasto repetido que no usás y destiná ese monto a tu ahorro o a ayudar.</t>
+          <t>Cancelá esta semana un gasto repetido que no usás y destiná ese monto a tu ahorro o a ayudar a alguien.</t>
         </is>
       </c>
     </row>
@@ -28719,62 +28721,62 @@
       </c>
       <c r="C135" s="61" t="inlineStr">
         <is>
-          <t>Comienzos pequeños</t>
+          <t>Empezar por la mañana</t>
         </is>
       </c>
       <c r="D135" s="61" t="inlineStr">
         <is>
-          <t>Al final del libro de Job, Dios les dice a los amigos de Job que no hablaron de Él con rectitud, como sí lo hizo su siervo Job.</t>
+          <t>El Salmo 143 es uno de los siete salmos que la tradición cristiana llama «penitenciales», junto con los salmos 6, 32, 38, 51, 102 y 130.</t>
         </is>
       </c>
       <c r="E135" s="61" t="inlineStr">
         <is>
-          <t>Job 42:7 (RVC)</t>
+          <t>Casiodoro, Comentario a los Salmos (siglo VI)</t>
         </is>
       </c>
       <c r="F135" s="61" t="inlineStr">
         <is>
-          <t>Esta frase la dice Bildad, uno de los amigos de Job. Él pensaba que a los justos siempre les va bien, y al final Dios corrige a esos amigos (42:7). Por eso no la tomamos como una promesa de riqueza.</t>
+          <t>David le pide a Dios ver su misericordia «por la mañana». Cada día es un comienzo nuevo, y los comienzos pequeños también se renuevan cada mañana.</t>
         </is>
       </c>
       <c r="G135" s="61" t="inlineStr">
         <is>
+          <t>La vergüenza de empezar con un puesto pequeño, con ventas por WhatsApp o desde la cocina de casa.</t>
+        </is>
+      </c>
+      <c r="H135" s="61" t="inlineStr">
+        <is>
+          <t>Sacale una foto a tu comienzo pequeño: algún día te va a recordar de dónde saliste.</t>
+        </is>
+      </c>
+      <c r="I135" s="61" t="inlineStr">
+        <is>
+          <t>«En ti he puesto mi confianza»: antes que el capital, la fe. Empezar con poco es posible cuando la confianza no está puesta solo en los recursos.</t>
+        </is>
+      </c>
+      <c r="J135" s="61" t="inlineStr">
+        <is>
           <t>Prometer prosperidad segura a quien emprende «si tiene fe».</t>
         </is>
       </c>
-      <c r="H135" s="61" t="inlineStr">
+      <c r="K135" s="61" t="inlineStr">
         <is>
           <t>Si alguien te promete ganancias seguras, desconfiá, aunque use versículos.</t>
         </is>
       </c>
-      <c r="I135" s="61" t="inlineStr">
-        <is>
-          <t>Lo que sí es cierto es que empezar con poco no es una vergüenza. Muchos emprendimientos sólidos empezaron con muy poco.</t>
-        </is>
-      </c>
-      <c r="J135" s="61" t="inlineStr">
-        <is>
-          <t>La vergüenza de empezar con un puesto pequeño, con ventas por WhatsApp o desde la cocina de casa.</t>
-        </is>
-      </c>
-      <c r="K135" s="61" t="inlineStr">
-        <is>
-          <t>Sacale una foto a tu comienzo pequeño: algún día te va a recordar de dónde saliste.</t>
-        </is>
-      </c>
       <c r="L135" s="61" t="inlineStr">
         <is>
-          <t>La historia de Job enseña que Dios está presente también cuando todo se pierde. Al final restauró a Job, pero por gracia, no como pago.</t>
+          <t>«Muéstrame el camino que debo seguir»: pedir dirección no es improvisar a ciegas. La oración y el plan van juntos.</t>
         </is>
       </c>
       <c r="M135" s="61" t="inlineStr">
         <is>
-          <t>Pensar que, si un negocio fracasa, es porque Dios nos castiga.</t>
+          <t>Arrancar un emprendimiento sin plan y sin pedir consejo.</t>
         </is>
       </c>
       <c r="N135" s="61" t="inlineStr">
         <is>
-          <t>Hablá con alguien de confianza sobre el mal momento de tu emprendimiento, y no lo cargues como culpa.</t>
+          <t>Antes de invertir, escribí en una hoja qué vas a vender, a quién y cuánto necesitás para empezar, y orá por ese plan.</t>
         </is>
       </c>
     </row>
@@ -29849,7 +29851,7 @@
       </c>
       <c r="C152" s="61" t="inlineStr">
         <is>
-          <t>Todo con amor</t>
+          <t>Motivar sin engaño</t>
         </is>
       </c>
       <c r="D152" s="61" t="inlineStr">
@@ -29864,12 +29866,12 @@
       </c>
       <c r="F152" s="61" t="inlineStr">
         <is>
-          <t>Pablo cierra su carta con exhortaciones breves: firmes en la fe, fuertes, y todo con amor. La firmeza sin amor se vuelve dureza.</t>
+          <t>Pablo recuerda cómo animó a los tesalonicenses: sin error, sin motivos impuros y sin engaño. Motivar de verdad empieza por una intención limpia.</t>
         </is>
       </c>
       <c r="G152" s="61" t="inlineStr">
         <is>
-          <t>Líderes firmes que motivan con miedo.</t>
+          <t>Presiones del tipo «si no lo hacés, vas a ver», en el trabajo o en la iglesia.</t>
         </is>
       </c>
       <c r="H152" s="61" t="inlineStr">
@@ -29879,12 +29881,12 @@
       </c>
       <c r="I152" s="61" t="inlineStr">
         <is>
-          <t>Motivar busca el bien del otro y de la tarea; manipular usa al otro como medio. La diferencia está en la intención y en el respeto a la libertad.</t>
+          <t>Pablo dice que Dios le confió el evangelio. Quien lidera tiene una confianza prestada, y eso exige cuidar a las personas, no usarlas.</t>
         </is>
       </c>
       <c r="J152" s="61" t="inlineStr">
         <is>
-          <t>Presiones del tipo «si no lo hacés, vas a ver», en el trabajo o en la iglesia.</t>
+          <t>Usar la culpa o lo espiritual para que otros hagan lo que uno quiere.</t>
         </is>
       </c>
       <c r="K152" s="61" t="inlineStr">
@@ -29894,12 +29896,12 @@
       </c>
       <c r="L152" s="61" t="inlineStr">
         <is>
-          <t>«Háganlo todo con amor»: el amor no manipula ni usa la culpa.</t>
+          <t>«No para agradar a los hombres, sino a Dios, que examina nuestro corazón». El líder que busca aplausos termina diciendo lo que la gente quiere oír.</t>
         </is>
       </c>
       <c r="M152" s="61" t="inlineStr">
         <is>
-          <t>Usar la culpa o lo espiritual para que otros hagan lo que uno quiere.</t>
+          <t>Líderes que cambian el mensaje según quién los escucha.</t>
         </is>
       </c>
       <c r="N152" s="61" t="inlineStr">
@@ -31329,62 +31331,62 @@
       </c>
       <c r="C174" s="61" t="inlineStr">
         <is>
-          <t>Mirar el camino recorrido</t>
+          <t>Examinar el camino</t>
         </is>
       </c>
       <c r="D174" s="61" t="inlineStr">
         <is>
-          <t>Job 22:28 lo dice Elifaz, uno de los amigos de Job. Al final del libro, Dios les dice a esos amigos que no hablaron de él lo recto (Job 42:7).</t>
+          <t>Los capítulos 1 al 4 de Lamentaciones son poemas acrósticos: en el original hebreo, las estrofas siguen el orden de las letras del alfabeto.</t>
         </is>
       </c>
       <c r="E174" s="61" t="inlineStr">
         <is>
-          <t>Job 22:1; 42:7</t>
+          <t>Texto hebreo de Lamentaciones 1-4</t>
         </is>
       </c>
       <c r="F174" s="61" t="inlineStr">
         <is>
-          <t>Elifaz le promete a Job éxito en todos sus planes si se vuelve a Dios, porque pensaba que su sufrimiento era un castigo. Dios corrigió esa idea: no todo lo que nos pasa es premio o castigo.</t>
+          <t>El profeta escribe entre las ruinas de Jerusalén y aun así propone algo concreto: examinar nuestra conducta. Evaluar con honestidad es el primer paso.</t>
         </is>
       </c>
       <c r="G174" s="61" t="inlineStr">
         <is>
+          <t>Mirar solo lo que falta y sentir que nunca se avanza.</t>
+        </is>
+      </c>
+      <c r="H174" s="61" t="inlineStr">
+        <is>
+          <t>Nombrá un logro pequeño de las últimas semanas que quizás pasó desapercibido, y una cosa que podés mejorar.</t>
+        </is>
+      </c>
+      <c r="I174" s="61" t="inlineStr">
+        <is>
+          <t>«Busquemos al Señor»: evaluar no es solo contar aciertos y errores; es volver a poner a Dios en el centro de los planes.</t>
+        </is>
+      </c>
+      <c r="J174" s="61" t="inlineStr">
+        <is>
+          <t>Planificar todo sin dejar lugar a que Dios corrija el rumbo.</t>
+        </is>
+      </c>
+      <c r="K174" s="61" t="inlineStr">
+        <is>
+          <t>Separá hoy diez minutos para orar por tus planes de los próximos meses.</t>
+        </is>
+      </c>
+      <c r="L174" s="61" t="inlineStr">
+        <is>
+          <t>«Volvámonos a él»: después de evaluar, se corrige el rumbo. No con culpa, sino con la confianza de que Dios recibe al que vuelve.</t>
+        </is>
+      </c>
+      <c r="M174" s="61" t="inlineStr">
+        <is>
           <t>Evaluar la vida como si cada logro fuera un premio y cada tropiezo, un castigo.</t>
         </is>
       </c>
-      <c r="H174" s="61" t="inlineStr">
-        <is>
-          <t>Al evaluar tu camino, no te juzgues con la dureza de los amigos de Job: mirá con honestidad y con gracia.</t>
-        </is>
-      </c>
-      <c r="I174" s="61" t="inlineStr">
-        <is>
-          <t>Evaluar lo avanzado, y no solo lo que falta, da perspectiva y sostiene la motivación. Y nos recuerda que fue Dios quien nos sostuvo hasta acá.</t>
-        </is>
-      </c>
-      <c r="J174" s="61" t="inlineStr">
-        <is>
-          <t>Mirar solo lo que falta y sentir que nunca se avanza.</t>
-        </is>
-      </c>
-      <c r="K174" s="61" t="inlineStr">
-        <is>
-          <t>Nombrá un logro pequeño de las últimas semanas que quizás pasó desapercibido.</t>
-        </is>
-      </c>
-      <c r="L174" s="61" t="inlineStr">
-        <is>
-          <t>Proverbios dice que el corazón del hombre traza su camino, pero el Señor dirige sus pasos (16:9). Evaluar es también preguntarle a Dios por el próximo paso.</t>
-        </is>
-      </c>
-      <c r="M174" s="61" t="inlineStr">
-        <is>
-          <t>Planificar todo sin dejar lugar a que Dios corrija el rumbo.</t>
-        </is>
-      </c>
       <c r="N174" s="61" t="inlineStr">
         <is>
-          <t>Después de evaluar, escribí el próximo paso y pedile a Dios su dirección.</t>
+          <t>Después de evaluar, escribí el próximo paso concreto y ponele fecha.</t>
         </is>
       </c>
     </row>
@@ -32789,22 +32791,22 @@
       </c>
       <c r="C196" s="61" t="inlineStr">
         <is>
-          <t>Una meta clara</t>
+          <t>Una visión que se entiende</t>
         </is>
       </c>
       <c r="D196" s="61" t="inlineStr">
         <is>
-          <t>La palabra griega que Pablo usa para «meta» (skopós) designaba la marca que el corredor miraba al final de la pista.</t>
+          <t>En el mismo capítulo, Proverbios dice que el corazón traza su camino, pero el Señor dirige sus pasos.</t>
         </is>
       </c>
       <c r="E196" s="61" t="inlineStr">
         <is>
-          <t>Filipenses 3:14; léxico griego de Strong (G4649, skopós)</t>
+          <t>Proverbios 16:9</t>
         </is>
       </c>
       <c r="F196" s="61" t="inlineStr">
         <is>
-          <t>Pablo usa la imagen de una carrera. Entre soñar una meta y alcanzarla hay una distancia que se recorre con pasos pequeños.</t>
+          <t>«Al de corazón sabio se le llama prudente»: una visión clara nace de adentro, de pensar con calma lo que Dios pone en el corazón.</t>
         </is>
       </c>
       <c r="G196" s="61" t="inlineStr">
@@ -32819,22 +32821,22 @@
       </c>
       <c r="I196" s="61" t="inlineStr">
         <is>
-          <t>Para Pablo, el premio es el llamado de Dios en Cristo. Toda visión de un líder cristiano se ordena debajo de ese llamado.</t>
+          <t>«La dulzura de los labios aumenta el saber»: los pasos concretos casi nunca se dan solos. Hay que explicar la visión con claridad y amabilidad para que otros se sumen.</t>
         </is>
       </c>
       <c r="J196" s="61" t="inlineStr">
         <is>
-          <t>Metas que nos alejan de Dios o de la familia.</t>
+          <t>Líderes que dan órdenes sin explicar para qué.</t>
         </is>
       </c>
       <c r="K196" s="61" t="inlineStr">
         <is>
-          <t>Revisá tu meta: ¿te acerca o te aleja de lo que Dios te llama a ser?</t>
+          <t>Contale tu plan a alguien de tu equipo o de tu familia y pedile que te lo repita con sus palabras.</t>
         </is>
       </c>
       <c r="L196" s="61" t="inlineStr">
         <is>
-          <t>Un corredor mira constantemente hacia dónde corre. Los pasos medibles permiten saber si se avanza.</t>
+          <t>Cuando la visión se comunica bien, el conocimiento se multiplica: cada uno sabe qué le toca y puede aportar ideas.</t>
         </is>
       </c>
       <c r="M196" s="61" t="inlineStr">
@@ -32844,7 +32846,7 @@
       </c>
       <c r="N196" s="61" t="inlineStr">
         <is>
-          <t>Elegí cómo vas a medir el primer paso y cuándo lo vas a revisar.</t>
+          <t>Elegí cómo vas a medir el primer paso y cuándo lo vas a revisar con los demás.</t>
         </is>
       </c>
     </row>
@@ -36529,62 +36531,62 @@
       </c>
       <c r="C252" s="61" t="inlineStr">
         <is>
-          <t>Dar lo que sabés</t>
+          <t>Dar con amor</t>
         </is>
       </c>
       <c r="D252" s="61" t="inlineStr">
         <is>
-          <t>Jetró, el suegro de Moisés, era sacerdote de Madián.</t>
+          <t>El capítulo del amor, 1 Corintios 13, está en medio de la enseñanza de Pablo sobre los dones (capítulos 12 y 14).</t>
         </is>
       </c>
       <c r="E252" s="61" t="inlineStr">
         <is>
-          <t>Éxodo 18:1</t>
+          <t>1 Corintios 12-14</t>
         </is>
       </c>
       <c r="F252" s="61" t="inlineStr">
         <is>
-          <t>Jetró dio algo que no era plata: su consejo y su experiencia. Dar no se limita al dinero.</t>
+          <t>Pablo dice que se puede repartir todo lo que uno tiene y no tener amor. Sin amor, dar es solo una transacción.</t>
         </is>
       </c>
       <c r="G252" s="61" t="inlineStr">
         <is>
-          <t>“No tengo plata, entonces no tengo nada para dar”.</t>
+          <t>Dar para que después nos deban un favor.</t>
         </is>
       </c>
       <c r="H252" s="61" t="inlineStr">
         <is>
-          <t>Ofrecé esta semana tu experiencia o un consejo a alguien que está empezando.</t>
+          <t>Esta semana, ayudá a alguien que no te lo pueda devolver.</t>
         </is>
       </c>
       <c r="I252" s="61" t="inlineStr">
         <is>
-          <t>Moisés dio responsabilidad a otros, y ellos dieron su tiempo para servir al pueblo. El tiempo es una de las ofrendas más valiosas.</t>
+          <t>Entregar el cuerpo es dar el esfuerzo, el talento, hasta el sacrificio. Pero aun eso, sin amor, puede ser orgullo.</t>
         </is>
       </c>
       <c r="J252" s="61" t="inlineStr">
         <is>
+          <t>«No tengo plata, entonces no tengo nada para dar».</t>
+        </is>
+      </c>
+      <c r="K252" s="61" t="inlineStr">
+        <is>
+          <t>Pensá qué sabés hacer y ofrecelo esta semana en tu iglesia o en tu barrio.</t>
+        </is>
+      </c>
+      <c r="L252" s="61" t="inlineStr">
+        <is>
+          <t>Lo que le da valor a lo que damos no es el tamaño, sino el corazón. Una hora dada con amor vale más que mucho dinero dado de mala gana.</t>
+        </is>
+      </c>
+      <c r="M252" s="61" t="inlineStr">
+        <is>
           <t>Dar plata para no tener que dar tiempo.</t>
         </is>
       </c>
-      <c r="K252" s="61" t="inlineStr">
+      <c r="N252" s="61" t="inlineStr">
         <is>
           <t>Regalale una hora de tu tiempo a alguien que necesita compañía o ayuda.</t>
-        </is>
-      </c>
-      <c r="L252" s="61" t="inlineStr">
-        <is>
-          <t>Cada uno sirvió según su capacidad, unos con grupos de diez y otros de mil. Cada talento cuenta.</t>
-        </is>
-      </c>
-      <c r="M252" s="61" t="inlineStr">
-        <is>
-          <t>Compararse con lo que dan otros y no dar nada.</t>
-        </is>
-      </c>
-      <c r="N252" s="61" t="inlineStr">
-        <is>
-          <t>Pensá qué sabés hacer y ofrecelo esta semana en tu iglesia o en tu barrio.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Versículos: texto RVC cotejado de los seis que faltaban y guiones ajustados a esa redacción
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -2646,8 +2646,8 @@
       </c>
       <c r="AD9" s="42" t="inlineStr">
         <is>
-          <t>Salmos 101:2-3 — Quiero seguir el camino de la perfección. ¿Cuándo vendrás a visitarme? En mi casa quiero vivir con un corazón intachable.
-No pondré delante de mis ojos nada que sea indigno. Aborrezco la obra de los que se desvían; no quiero tener nada que ver con ellos.</t>
+          <t>Salmos 101:2-3 — Quiero entender tus perfectas enseñanzas. ¿Cuándo vendrás a mi encuentro? Así me conduciré con rectitud en mi hogar,
+y no pondré los ojos en la injusticia. Odio a los que actúan de manera torcida; no permito que ninguno de ellos se acerque a mí.</t>
         </is>
       </c>
       <c r="AE9" s="43" t="inlineStr">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="AF19" s="51" t="inlineStr">
         <is>
-          <t>Mateo 6:3-4 — Cuando tú des limosna, que no sepa tu mano izquierda lo que hace tu mano derecha, para que tu limosna sea en secreto; y tu Padre, que ve en lo secreto, te recompensará.</t>
+          <t>Mateo 6:3-4 — Pero cuando tú des limosna, asegúrate de que tu mano izquierda no sepa lo que hace la derecha, así tu limosna será en secreto, y tu Padre que ve en lo secreto te recompensará en público.</t>
         </is>
       </c>
       <c r="AG19" s="51" t="inlineStr">
@@ -5457,8 +5457,8 @@
       </c>
       <c r="AH22" s="40" t="inlineStr">
         <is>
-          <t>Hageo 1:6-7 — Ustedes siembran mucho, pero cosechan poco; comen, pero no se sacian; beben, pero no quedan satisfechos; se visten, pero no se calientan; y el que trabaja a jornal recibe su salario en saco roto.
-Así dice el Señor de los ejércitos: «Reflexionen sobre su conducta.»</t>
+          <t>Hageo 1:6-7 — Ustedes siembran mucho, y recogen poco; comen, y no se sacian; beben, y no quedan satisfechos; se visten, y no entran en calor; y los que trabajan por un jornal lo reciben en saco roto.
+Así ha dicho el Señor de los ejércitos: «Piensen en lo que hacen.»</t>
         </is>
       </c>
       <c r="AI22" s="40" t="inlineStr">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="Z27" s="58" t="inlineStr">
         <is>
-          <t>1 Tesalonicenses 2:3-4 — Nuestra exhortación no se basó en el error ni en motivos impuros, ni fue con engaño, sino que, así como Dios nos aprobó y nos confió el evangelio, así hablamos, no para agradar a los hombres sino a Dios, que examina nuestro corazón.</t>
+          <t>1 Tesalonicenses 2:3-4 — Porque nuestra exhortación no se basa en el error ni en malas intenciones, ni tampoco tratamos de engañar a nadie, sino que hablamos porque Dios nos aprobó y nos confió el evangelio. No buscamos agradar a los hombres, sino a Dios, que es quien examina nuestro corazón.</t>
         </is>
       </c>
       <c r="AA27" s="53" t="inlineStr">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="AD34" s="10" t="inlineStr">
         <is>
-          <t>Proverbios 16:21 — Al de corazón sabio se le llama prudente; la dulzura de los labios aumenta el saber.</t>
+          <t>Proverbios 16:21 — Al de corazón sabio se le llama prudente; los labios amables aumentan el saber.</t>
         </is>
       </c>
       <c r="AE34" s="10" t="inlineStr">
@@ -9960,7 +9960,7 @@
       </c>
       <c r="AH43" s="14" t="inlineStr">
         <is>
-          <t>1 Corintios 13:3 — Y si repartiera todos mis bienes para dar de comer a los pobres, y si entregara mi cuerpo para ser quemado, y no tengo amor, de nada me sirve.</t>
+          <t>1 Corintios 13:3 — Y si repartiera todos mis bienes para dar de comer a los pobres, y entregara mi cuerpo para ser quemado, y no tengo amor, de nada me sirve.</t>
         </is>
       </c>
       <c r="AI43" s="14" t="inlineStr">
@@ -22806,7 +22806,7 @@
       </c>
       <c r="F46" s="61" t="inlineStr">
         <is>
-          <t>David quiere andar con integridad, pero sabe que no puede solo: le pide a Dios que venga a visitarlo.</t>
+          <t>David empieza por lo de adentro: quiere entender las enseñanzas de Dios y le pregunta cuándo vendrá a su encuentro. Sabe que no puede andar derecho solo.</t>
         </is>
       </c>
       <c r="G46" s="61" t="inlineStr">
@@ -22821,7 +22821,7 @@
       </c>
       <c r="I46" s="61" t="inlineStr">
         <is>
-          <t>«En mi casa quiero vivir con un corazón intachable»: la integridad no empieza en público, empieza puertas adentro, donde nadie nos ve.</t>
+          <t>«Así me conduciré con rectitud en mi hogar»: la integridad no empieza en público, empieza puertas adentro, donde nadie nos ve.</t>
         </is>
       </c>
       <c r="J46" s="61" t="inlineStr">
@@ -22836,7 +22836,7 @@
       </c>
       <c r="L46" s="61" t="inlineStr">
         <is>
-          <t>«No pondré delante de mis ojos nada que sea indigno»: lo que entra por los ojos va formando la mente. Elegir qué mirar es cuidar el alma.</t>
+          <t>«No pondré los ojos en la injusticia»: lo que entra por los ojos va formando la mente. Elegir qué mirar es cuidar el alma.</t>
         </is>
       </c>
       <c r="M46" s="61" t="inlineStr">
@@ -26906,7 +26906,7 @@
       </c>
       <c r="L107" s="61" t="inlineStr">
         <is>
-          <t>«Tu Padre, que ve en lo secreto». Dios ve lo que nadie ve, y ese servicio silencioso es, muchas veces, el más valioso.</t>
+          <t>«Tu Padre que ve en lo secreto». Dios ve lo que nadie ve, y ese servicio silencioso es, muchas veces, el más valioso.</t>
         </is>
       </c>
       <c r="M107" s="61" t="inlineStr">
@@ -28146,7 +28146,7 @@
       </c>
       <c r="F126" s="61" t="inlineStr">
         <is>
-          <t>Hageo le habla a un pueblo que había vuelto del exilio: trabajaban mucho y cosechaban poco. Dios les pide que se detengan a pensar en lo que están haciendo.</t>
+          <t>Hageo le habla a un pueblo que había vuelto del exilio: sembraban mucho y recogían poco. Dios les dice: «Piensen en lo que hacen».</t>
         </is>
       </c>
       <c r="G126" s="61" t="inlineStr">
@@ -28161,7 +28161,7 @@
       </c>
       <c r="I126" s="61" t="inlineStr">
         <is>
-          <t>«Comen, pero no se sacian»: consumir más no siempre llena. A veces gastamos para tapar un vacío.</t>
+          <t>«Comen, y no se sacian»: consumir más no siempre llena. A veces gastamos para tapar un vacío.</t>
         </is>
       </c>
       <c r="J126" s="61" t="inlineStr">
@@ -29866,7 +29866,7 @@
       </c>
       <c r="F152" s="61" t="inlineStr">
         <is>
-          <t>Pablo recuerda cómo animó a los tesalonicenses: sin error, sin motivos impuros y sin engaño. Motivar de verdad empieza por una intención limpia.</t>
+          <t>Pablo recuerda cómo animó a los tesalonicenses: sin error, sin malas intenciones y sin tratar de engañar a nadie. Motivar de verdad empieza por una intención limpia.</t>
         </is>
       </c>
       <c r="G152" s="61" t="inlineStr">
@@ -29896,7 +29896,7 @@
       </c>
       <c r="L152" s="61" t="inlineStr">
         <is>
-          <t>«No para agradar a los hombres, sino a Dios, que examina nuestro corazón». El líder que busca aplausos termina diciendo lo que la gente quiere oír.</t>
+          <t>«No buscamos agradar a los hombres, sino a Dios, que es quien examina nuestro corazón». El líder que busca aplausos termina diciendo lo que la gente quiere oír.</t>
         </is>
       </c>
       <c r="M152" s="61" t="inlineStr">
@@ -32821,7 +32821,7 @@
       </c>
       <c r="I196" s="61" t="inlineStr">
         <is>
-          <t>«La dulzura de los labios aumenta el saber»: los pasos concretos casi nunca se dan solos. Hay que explicar la visión con claridad y amabilidad para que otros se sumen.</t>
+          <t>«Los labios amables aumentan el saber»: los pasos concretos casi nunca se dan solos. Hay que explicar la visión con claridad y amabilidad para que otros se sumen.</t>
         </is>
       </c>
       <c r="J196" s="61" t="inlineStr">

</xml_diff>

<commit_message>
Frases deportivas: alineadas con los versículos nuevos y las fechas especiales, sin muletillas de cierre los sábados
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -41329,7 +41329,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D3" s="61" t="inlineStr">
@@ -41349,7 +41349,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>natación</t>
         </is>
       </c>
       <c r="D4" s="61" t="inlineStr">
@@ -41389,7 +41389,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D6" s="61" t="inlineStr">
@@ -41429,12 +41429,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>maraton</t>
+          <t>maratón</t>
         </is>
       </c>
       <c r="D8" s="61" t="inlineStr">
         <is>
-          <t>El maratonista sabe que la carrera se corre con las piernas y con la cabeza. Esta semana vimos que cuidar el cuerpo y el alma que Dios nos dio va junto.</t>
+          <t>El maratonista sabe que la carrera se corre con las piernas y con la cabeza. Cuidar el cuerpo y el alma que Dios nos dio va junto.</t>
         </is>
       </c>
     </row>
@@ -41449,7 +41449,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D9" s="61" t="inlineStr">
@@ -41549,12 +41549,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>hinchada</t>
+          <t>canchero</t>
         </is>
       </c>
       <c r="D14" s="61" t="inlineStr">
         <is>
-          <t>La hinchada que alienta aun cuando el equipo va abajo siembra ánimo sin mezquinar. Sembrar con generosidad es dar con alegría, pensando en el hermano que necesita.</t>
+          <t>El canchero cuida el césped como si fuera suyo, aunque la cancha es del club y la van a usar otros. La tierra es del Señor: la cuidamos para los que vienen detrás.</t>
         </is>
       </c>
     </row>
@@ -41574,7 +41574,7 @@
       </c>
       <c r="D15" s="61" t="inlineStr">
         <is>
-          <t>Cada palada parece pequeña, pero sostenida lleva lejos al bote. Lo de estos días: sembrar, aun con lágrimas, puede preceder a la alegría de la cosecha.</t>
+          <t>Cada palada parece pequeña, pero sostenida lleva lejos al bote. Sembrar, aun con lágrimas, puede preceder a la alegría de la cosecha.</t>
         </is>
       </c>
     </row>
@@ -41589,7 +41589,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D16" s="61" t="inlineStr">
@@ -41609,7 +41609,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D17" s="61" t="inlineStr">
@@ -41714,7 +41714,7 @@
       </c>
       <c r="D22" s="61" t="inlineStr">
         <is>
-          <t>Sin que nadie lo aplauda, el utilero revisa cada botín antes del partido. Así cerramos el tema: prevenir es amar, y bendecimos a Dios por su cuidado de cada día.</t>
+          <t>Sin que nadie lo aplauda, el utilero revisa cada botín antes del partido. Prevenir es amar, y bendecimos a Dios por su cuidado de cada día.</t>
         </is>
       </c>
     </row>
@@ -41769,7 +41769,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D25" s="61" t="inlineStr">
@@ -41789,7 +41789,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D26" s="61" t="inlineStr">
@@ -41809,7 +41809,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>maraton</t>
+          <t>maratón</t>
         </is>
       </c>
       <c r="D27" s="61" t="inlineStr">
@@ -41849,12 +41849,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>natación</t>
         </is>
       </c>
       <c r="D29" s="61" t="inlineStr">
         <is>
-          <t>El nadador que entrena con constancia hace del agua su lugar. Esta semana vimos que la Palabra estudiada y vivida se vuelve propia y llena de gozo el corazón.</t>
+          <t>El nadador que entrena con constancia hace del agua su lugar. La Palabra estudiada y vivida se vuelve propia y llena de gozo el corazón.</t>
         </is>
       </c>
     </row>
@@ -41869,7 +41869,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D30" s="61" t="inlineStr">
@@ -41969,7 +41969,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D35" s="61" t="inlineStr">
@@ -41994,7 +41994,7 @@
       </c>
       <c r="D36" s="61" t="inlineStr">
         <is>
-          <t>Tenis amateur: muchas veces el propio jugador canta si la pelota fue afuera. Para llevarse de la semana: el líder se forma por dentro, íntegro aun cuando nadie mira.</t>
+          <t>Tenis amateur: muchas veces el propio jugador canta si la pelota fue afuera. El líder se forma por dentro, íntegro aun cuando nadie mira.</t>
         </is>
       </c>
     </row>
@@ -42009,7 +42009,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D37" s="61" t="inlineStr">
@@ -42109,7 +42109,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D42" s="61" t="inlineStr">
@@ -42134,7 +42134,7 @@
       </c>
       <c r="D43" s="61" t="inlineStr">
         <is>
-          <t>Con calma se ve todo el tablero de ajedrez. Así cerramos el tema: un hogar donde la paz de Dios gobierna el corazón, con gratitud y sin imposiciones.</t>
+          <t>Con calma se ve todo el tablero de ajedrez. Así se vive en un hogar donde la paz de Dios gobierna el corazón: con gratitud y sin imposiciones.</t>
         </is>
       </c>
     </row>
@@ -42149,7 +42149,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D44" s="61" t="inlineStr">
@@ -42169,7 +42169,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>maraton</t>
+          <t>maratón</t>
         </is>
       </c>
       <c r="D45" s="61" t="inlineStr">
@@ -42189,7 +42189,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D46" s="61" t="inlineStr">
@@ -42274,7 +42274,7 @@
       </c>
       <c r="D50" s="61" t="inlineStr">
         <is>
-          <t>Antes de largar la regata, el remero calcula sus fuerzas. Siete días después queda esto: ahorrar es prepararse, con la seguridad de fondo puesta en Dios y no en la plata.</t>
+          <t>Antes de largar la regata, el remero calcula sus fuerzas. Ahorrar es prepararse, con la seguridad de fondo puesta en Dios y no en la plata.</t>
         </is>
       </c>
     </row>
@@ -42289,7 +42289,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>natación</t>
         </is>
       </c>
       <c r="D51" s="61" t="inlineStr">
@@ -42309,12 +42309,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D52" s="61" t="inlineStr">
         <is>
-          <t>A veces, en el vestuario, lo más valiente es decir: hoy no estoy bien. Hablar con honestidad sobre lo que sentís también es parte de una vida íntegra.</t>
+          <t>A veces, en el vestuario, lo más valiente es decir: hoy no estoy bien. Como el salmista, ponerle nombre al desánimo es el primer paso para volver a esperar en Dios.</t>
         </is>
       </c>
     </row>
@@ -42349,12 +42349,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>hinchada</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D54" s="61" t="inlineStr">
         <is>
-          <t>Antes que cualquier resultado, hay algo que tu mente necesita escuchar más fuerte que una tribuna entera: Dios te ama, y dio a su Hijo para darte vida eterna.</t>
+          <t>El arquero no se distrae con todo lo que pasa en la tribuna: fija los ojos en la pelota. Elegí qué ponés delante de tus ojos; lo que mirás también forma tu mente.</t>
         </is>
       </c>
     </row>
@@ -42414,7 +42414,7 @@
       </c>
       <c r="D57" s="61" t="inlineStr">
         <is>
-          <t>Nadie corre todos los tramos de una posta solo. Lo de estos días: cuidar el alma sabiendo que Dios está cerca del quebrantado, y que no tenés que cargar todo solo.</t>
+          <t>Nadie corre todos los tramos de una posta solo. Dios está cerca del quebrantado: cuidá tu alma sabiendo que no tenés que cargar todo solo.</t>
         </is>
       </c>
     </row>
@@ -42429,7 +42429,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>preparacion fisica</t>
+          <t>preparación física</t>
         </is>
       </c>
       <c r="D58" s="61" t="inlineStr">
@@ -42489,7 +42489,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D61" s="61" t="inlineStr">
@@ -42509,7 +42509,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>maraton</t>
+          <t>maratón</t>
         </is>
       </c>
       <c r="D62" s="61" t="inlineStr">
@@ -42529,7 +42529,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D63" s="61" t="inlineStr">
@@ -42554,7 +42554,7 @@
       </c>
       <c r="D64" s="61" t="inlineStr">
         <is>
-          <t>Compañero golpeado en el handball: el equipo lo protege hasta que se recupera. Siete días después, la idea queda clara: cuidar como cuida Dios, con ternura, cargando al más débil.</t>
+          <t>Compañero golpeado en el handball: el equipo lo protege hasta que se recupera. Así cuida Dios: con ternura, cargando al más débil.</t>
         </is>
       </c>
     </row>
@@ -42589,7 +42589,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D66" s="61" t="inlineStr">
@@ -42649,7 +42649,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D69" s="61" t="inlineStr">
@@ -42669,7 +42669,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>natación</t>
         </is>
       </c>
       <c r="D70" s="61" t="inlineStr">
@@ -42694,7 +42694,7 @@
       </c>
       <c r="D71" s="61" t="inlineStr">
         <is>
-          <t>Un pase a tiempo vale más que diez apurados al final del partido de futsal. Para cerrar la semana: cuidarse a tiempo, con Dios como escudo que afirma nuestros pasos.</t>
+          <t>Un pase a tiempo vale más que diez apurados al final del partido de futsal. Cuidarse a tiempo también es sabiduría, con Dios como escudo que afirma nuestros pasos.</t>
         </is>
       </c>
     </row>
@@ -42729,7 +42729,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D73" s="61" t="inlineStr">
@@ -42749,7 +42749,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>voley de playa</t>
+          <t>vóley de playa</t>
         </is>
       </c>
       <c r="D74" s="61" t="inlineStr">
@@ -42834,7 +42834,7 @@
       </c>
       <c r="D78" s="61" t="inlineStr">
         <is>
-          <t>Turnándose para cortar el viento, los ciclistas del pelotón llegan más lejos juntos. Así cerramos el tema: la fe se vive en comunidad, con un mismo amor.</t>
+          <t>Turnándose para cortar el viento, los ciclistas del pelotón llegan más lejos juntos. La fe se vive en comunidad, con un mismo amor.</t>
         </is>
       </c>
     </row>
@@ -42869,7 +42869,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D80" s="61" t="inlineStr">
@@ -42909,7 +42909,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>maraton</t>
+          <t>maratón</t>
         </is>
       </c>
       <c r="D82" s="61" t="inlineStr">
@@ -42929,7 +42929,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D83" s="61" t="inlineStr">
@@ -42949,12 +42949,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>atletismo</t>
         </is>
       </c>
       <c r="D84" s="61" t="inlineStr">
         <is>
-          <t>Sin la línea del carril, el nadador se desvía sin darse cuenta. Cuando falta la Palabra, el pueblo se dispersa; ella nos da orden y propósito.</t>
+          <t>En la posta, uno corre el tramo más duro para que el compañero pueda llegar. En la cruz, Jesús cargó lo que no podíamos cargar: por sus heridas fuimos sanados.</t>
         </is>
       </c>
     </row>
@@ -42974,7 +42974,7 @@
       </c>
       <c r="D85" s="61" t="inlineStr">
         <is>
-          <t>El timonel marca el ritmo y el bote avanza parejo. En una línea: liderar con responsabilidad, con sabiduría y aprovechando bien el tiempo.</t>
+          <t>El timonel marca el ritmo y el bote avanza parejo. Liderar es eso: marcar el paso con responsabilidad, con sabiduría y aprovechando bien el tiempo.</t>
         </is>
       </c>
     </row>
@@ -42989,12 +42989,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>tenis</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D86" s="61" t="inlineStr">
         <is>
-          <t>En el tenis de dobles, dos estilos distintos juegan para el mismo lado de la red. En el matrimonio, dejar y unirse para ser una sola carne cambia las prioridades.</t>
+          <t>Un partido no termina hasta el silbato final, aunque muchos lo den por perdido. En Pascua celebramos que la muerte no tiene la última palabra: Jesús es la resurrección y la vida.</t>
         </is>
       </c>
     </row>
@@ -43009,7 +43009,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D87" s="61" t="inlineStr">
@@ -43029,7 +43029,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D88" s="61" t="inlineStr">
@@ -43049,12 +43049,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>atletismo</t>
+          <t>tenis</t>
         </is>
       </c>
       <c r="D89" s="61" t="inlineStr">
         <is>
-          <t>Antes de una largada, algunos atletas saben que alguien en la tribuna está orando por ellos. Orar el uno por el otro es una responsabilidad de amor en la pareja.</t>
+          <t>En el tenis de dobles, los compañeros se cubren y no se hablan con dureza en medio del partido. En el matrimonio, el respeto y el amor juegan del mismo lado de la red.</t>
         </is>
       </c>
     </row>
@@ -43114,7 +43114,7 @@
       </c>
       <c r="D92" s="61" t="inlineStr">
         <is>
-          <t>Llueva o truene, la hinchada sigue a su equipo: el amor verdadero no se apaga. Para llevarse de la semana: ni las muchas aguas pueden extinguirlo.</t>
+          <t>Llueva o truene, la hinchada sigue a su equipo: el amor verdadero no se apaga. Ni las muchas aguas pueden extinguirlo.</t>
         </is>
       </c>
     </row>
@@ -43149,7 +43149,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>maraton</t>
+          <t>maratón</t>
         </is>
       </c>
       <c r="D94" s="61" t="inlineStr">
@@ -43189,7 +43189,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D96" s="61" t="inlineStr">
@@ -43209,7 +43209,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D97" s="61" t="inlineStr">
@@ -43254,7 +43254,7 @@
       </c>
       <c r="D99" s="61" t="inlineStr">
         <is>
-          <t>Las camisetas no son del utilero, pero las cuida como si lo fueran. Nos llevamos esto: ser administradores confiables de lo que Dios nos prestó.</t>
+          <t>Las camisetas no son del utilero, pero las cuida como si lo fueran. Así somos llamados a cuidar lo que Dios nos prestó: como administradores confiables.</t>
         </is>
       </c>
     </row>
@@ -43289,7 +43289,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D101" s="61" t="inlineStr">
@@ -43329,7 +43329,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>natación</t>
         </is>
       </c>
       <c r="D103" s="61" t="inlineStr">
@@ -43369,7 +43369,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>voley de playa</t>
+          <t>vóley de playa</t>
         </is>
       </c>
       <c r="D105" s="61" t="inlineStr">
@@ -43389,12 +43389,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>futbol formativo</t>
+          <t>fútbol formativo</t>
         </is>
       </c>
       <c r="D106" s="61" t="inlineStr">
         <is>
-          <t>El jugador que se formó desde chico en el club de su barrio lleva raíces que se notan; esta semana vimos que la fe crece arraigada en Cristo, con tiempo.</t>
+          <t>El jugador que se formó desde chico en el club de su barrio lleva raíces que se notan; la fe crece arraigada en Cristo, con tiempo.</t>
         </is>
       </c>
     </row>
@@ -43409,7 +43409,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D107" s="61" t="inlineStr">
@@ -43534,7 +43534,7 @@
       </c>
       <c r="D113" s="61" t="inlineStr">
         <is>
-          <t>Mano a mano pasa el testimonio, y la carrera de postas necesita a todos. Para cerrar la semana, pedimos como el salmista: Señor, confirmá la obra de nuestras manos.</t>
+          <t>Mano a mano pasa el testimonio, y la carrera de postas necesita a todos. Por eso pedimos como el salmista: Señor, confirmá la obra de nuestras manos.</t>
         </is>
       </c>
     </row>
@@ -43549,7 +43549,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>maraton</t>
+          <t>maratón</t>
         </is>
       </c>
       <c r="D114" s="61" t="inlineStr">
@@ -43609,7 +43609,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>natación</t>
         </is>
       </c>
       <c r="D117" s="61" t="inlineStr">
@@ -43629,7 +43629,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D118" s="61" t="inlineStr">
@@ -43649,7 +43649,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D119" s="61" t="inlineStr">
@@ -43669,12 +43669,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>preparacion fisica</t>
+          <t>preparación física</t>
         </is>
       </c>
       <c r="D120" s="61" t="inlineStr">
         <is>
-          <t>Pensando en toda la temporada, el preparador físico cuida a sus jugadores. Así cerramos el tema: cuidar tu cuerpo es cuidar un regalo.</t>
+          <t>Pensando en toda la temporada, el preparador físico cuida a sus jugadores. Cuidar tu cuerpo es cuidar un regalo.</t>
         </is>
       </c>
     </row>
@@ -43729,7 +43729,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D123" s="61" t="inlineStr">
@@ -43749,7 +43749,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D124" s="61" t="inlineStr">
@@ -43774,7 +43774,7 @@
       </c>
       <c r="D125" s="61" t="inlineStr">
         <is>
-          <t>El juez de línea corre toda la banda y casi nadie sabe su nombre; trabajar de corazón para el Señor no depende de los aplausos de la tribuna.</t>
+          <t>El juez de línea corre toda la banda y casi nadie sabe su nombre. Servir sin aplausos es eso: que la mano izquierda no se entere, porque el Padre ve en lo secreto.</t>
         </is>
       </c>
     </row>
@@ -43789,7 +43789,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>futbol infantil</t>
+          <t>fútbol infantil</t>
         </is>
       </c>
       <c r="D126" s="61" t="inlineStr">
@@ -43814,7 +43814,7 @@
       </c>
       <c r="D127" s="61" t="inlineStr">
         <is>
-          <t>Atado a un compañero no vidente, el atleta guía corre feliz si el otro llega. Queda de la semana: hay más dicha en dar que en recibir.</t>
+          <t>Atado a un compañero no vidente, el atleta guía corre feliz si el otro llega. Hay más dicha en dar que en recibir.</t>
         </is>
       </c>
     </row>
@@ -43849,7 +43849,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D129" s="61" t="inlineStr">
@@ -43949,12 +43949,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D134" s="61" t="inlineStr">
         <is>
-          <t>Un set perdido no define el valor de un equipo de vóley; esta semana recordamos que Dios obra en todo, también en los desafíos, aunque no lo entendamos todo.</t>
+          <t>Un set perdido no define el valor de un equipo de vóley; Dios obra en todo, también en los desafíos, aunque no lo entendamos todo.</t>
         </is>
       </c>
     </row>
@@ -43969,7 +43969,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>futbol infantil</t>
+          <t>fútbol infantil</t>
         </is>
       </c>
       <c r="D135" s="61" t="inlineStr">
@@ -43989,7 +43989,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>natación</t>
         </is>
       </c>
       <c r="D136" s="61" t="inlineStr">
@@ -44009,7 +44009,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D137" s="61" t="inlineStr">
@@ -44094,7 +44094,7 @@
       </c>
       <c r="D141" s="61" t="inlineStr">
         <is>
-          <t>Primer partido del nieto, y el abuelo le pasa mucho más que una camiseta. Lo que queda de estos días: criar con amor e integridad deja un legado de generación en generación.</t>
+          <t>Primer partido del nieto, y el abuelo le pasa mucho más que una camiseta. Criar con amor e integridad deja un legado de generación en generación.</t>
         </is>
       </c>
     </row>
@@ -44109,7 +44109,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D142" s="61" t="inlineStr">
@@ -44129,7 +44129,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D143" s="61" t="inlineStr">
@@ -44214,7 +44214,7 @@
       </c>
       <c r="D147" s="61" t="inlineStr">
         <is>
-          <t>El buen arquero de futsal ordena a su defensa sin gritos ni humillaciones; cerrar las fugas de la casa también pide una sabiduría que habla con calma y compasión.</t>
+          <t>El equipo de futsal que corre todo el partido pero no cierra la defensa recibe goles por el mismo hueco. Antes de trabajar más, mirá por dónde se escapa tu plata.</t>
         </is>
       </c>
     </row>
@@ -44229,7 +44229,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D148" s="61" t="inlineStr">
@@ -44249,7 +44249,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D149" s="61" t="inlineStr">
@@ -44269,7 +44269,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D150" s="61" t="inlineStr">
@@ -44329,7 +44329,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>preparacion fisica</t>
+          <t>preparación física</t>
         </is>
       </c>
       <c r="D153" s="61" t="inlineStr">
@@ -44349,7 +44349,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>natación</t>
         </is>
       </c>
       <c r="D154" s="61" t="inlineStr">
@@ -44389,7 +44389,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>futbol de potrero</t>
+          <t>fútbol de potrero</t>
         </is>
       </c>
       <c r="D156" s="61" t="inlineStr">
@@ -44434,7 +44434,7 @@
       </c>
       <c r="D158" s="61" t="inlineStr">
         <is>
-          <t>Muchos jugadores de futsal empezaron en una canchita de cemento del barrio; un comienzo pequeño no es una vergüenza ni define el final.</t>
+          <t>Muchos jugadores de futsal empezaron en una canchita de cemento del barrio, entrenando temprano. Cada mañana es un comienzo nuevo: confiá en Dios y pedile que te muestre el camino.</t>
         </is>
       </c>
     </row>
@@ -44449,7 +44449,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D159" s="61" t="inlineStr">
@@ -44514,7 +44514,7 @@
       </c>
       <c r="D162" s="61" t="inlineStr">
         <is>
-          <t>Las medallas se oxidan y los trofeos juntan polvo en la vitrina; esta semana hablamos de emprender con fe y con cuidado, recordando que la vida verdadera la da Jesús.</t>
+          <t>Las medallas se oxidan y los trofeos juntan polvo en la vitrina. Emprendé con fe y con cuidado, sabiendo que la vida verdadera la da Jesús.</t>
         </is>
       </c>
     </row>
@@ -44529,7 +44529,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D163" s="61" t="inlineStr">
@@ -44569,7 +44569,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>maraton</t>
+          <t>maratón</t>
         </is>
       </c>
       <c r="D165" s="61" t="inlineStr">
@@ -44589,7 +44589,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D166" s="61" t="inlineStr">
@@ -44649,12 +44649,12 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D169" s="61" t="inlineStr">
         <is>
-          <t>Un mal día de comidas no hace que el basquetbolista se castigue: ajusta y sigue. Para cerrar la semana: comer con gratitud y medida, como cuidado y no como culpa.</t>
+          <t>Un mal día de comidas no hace que el basquetbolista se castigue: ajusta y sigue. Comer con gratitud y medida es cuidado, no culpa.</t>
         </is>
       </c>
     </row>
@@ -44669,7 +44669,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>futbol formativo</t>
+          <t>fútbol formativo</t>
         </is>
       </c>
       <c r="D170" s="61" t="inlineStr">
@@ -44709,7 +44709,7 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>natacion</t>
+          <t>natación</t>
         </is>
       </c>
       <c r="D172" s="61" t="inlineStr">
@@ -44794,7 +44794,7 @@
       </c>
       <c r="D176" s="61" t="inlineStr">
         <is>
-          <t>Cada bote que avanza lleva algo del viejo entrenador de remo que formó a sus remeros. Así cerramos el tema: invertir en otros deja una huella que dura.</t>
+          <t>Cada bote que avanza lleva algo del viejo entrenador de remo que formó a sus remeros. Invertir en otros deja una huella que dura.</t>
         </is>
       </c>
     </row>
@@ -44809,7 +44809,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D177" s="61" t="inlineStr">
@@ -44829,12 +44829,12 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>voley</t>
+          <t>vóley</t>
         </is>
       </c>
       <c r="D178" s="61" t="inlineStr">
         <is>
-          <t>Firme en el bloqueo y valiente en el ataque, sí; pero un equipo de vóley se sostiene cuando todo se hace con amor, también la corrección.</t>
+          <t>El buen capitán de vóley anima a su equipo sin engaños ni gritos que humillan. Motivar sin manipular es buscar agradar a Dios, no el aplauso de la tribuna.</t>
         </is>
       </c>
     </row>
@@ -44849,7 +44849,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>basquet</t>
+          <t>básquet</t>
         </is>
       </c>
       <c r="D179" s="61" t="inlineStr">
@@ -44869,7 +44869,7 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>futbol</t>
+          <t>fútbol</t>
         </is>
       </c>
       <c r="D180" s="61" t="inlineStr">
@@ -44934,7 +44934,7 @@
       </c>
       <c r="D183" s="61" t="inlineStr">
         <is>
-          <t>El que da la asistencia en el futsal festeja el gol como propio. Así se resume la semana: el equipo se sostiene cuando cada uno busca también el bien del otro.</t>
+          <t>El que da la asistencia en el futsal festeja el gol como propio. El equipo se sostiene cuando cada uno busca también el bien del otro.</t>
         </is>
       </c>
     </row>
@@ -45334,7 +45334,7 @@
       </c>
       <c r="D203" s="61" t="inlineStr">
         <is>
-          <t>Tramo terminado en el Rally del Chaco: el copiloto lo revisa antes de encarar el siguiente. Mirar atrás con honestidad y poner tus planes en manos de Dios te ayuda a seguir.</t>
+          <t>Tramo terminado: el copiloto de rally revisa sus notas antes de encarar el siguiente. Examinar el camino, buscar al Señor y volver a él: así se corrige el rumbo.</t>
         </is>
       </c>
     </row>
@@ -45854,7 +45854,7 @@
       </c>
       <c r="D229" s="61" t="inlineStr">
         <is>
-          <t>Un bote de remo avanza derecho cuando todos miran el mismo punto; la visión necesita una dirección clara y constante, como quien prosigue hacia la meta.</t>
+          <t>En el remo, el timonel habla claro y con calma para que todos remen al mismo ritmo. Una visión se convierte en pasos concretos cuando se comunica con palabras amables.</t>
         </is>
       </c>
     </row>
@@ -46869,7 +46869,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>árbitro</t>
+          <t>arbitraje</t>
         </is>
       </c>
       <c r="D280" s="61" t="inlineStr">
@@ -46894,7 +46894,7 @@
       </c>
       <c r="D281" s="61" t="inlineStr">
         <is>
-          <t>El base que mejor dirige es el que más asistencias da. Para llevarse de la semana: con Jesús, liderar es servir.</t>
+          <t>El base que mejor dirige es el que más asistencias da. Con Jesús, liderar es servir.</t>
         </is>
       </c>
     </row>
@@ -47034,7 +47034,7 @@
       </c>
       <c r="D288" s="61" t="inlineStr">
         <is>
-          <t>Kilómetro 40: alguien frena para acompañar a otro hasta la meta; la lealtad pesa más que el reloj. Siete días después, queda un hogar que camina junto, aun en lo difícil.</t>
+          <t>Kilómetro 40: alguien frena para acompañar a otro hasta la meta; la lealtad pesa más que el reloj. Así es un hogar que camina junto, aun en lo difícil.</t>
         </is>
       </c>
     </row>
@@ -47154,7 +47154,7 @@
       </c>
       <c r="D294" s="61" t="inlineStr">
         <is>
-          <t>El técnico veterano que comparte lo que sabe con el ayudante joven multiplica el trabajo de todos. Jetro le dio su consejo a Moisés, y Moisés tuvo la humildad de escuchar.</t>
+          <t>El técnico que regala su tiempo a los chicos del barrio, sin cobrar y sin cámaras, deja mucho más que tácticas. Dar sin amor es una transacción; dar con amor cambia vidas.</t>
         </is>
       </c>
     </row>
@@ -47449,12 +47449,12 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>árbitro</t>
+          <t>arbitraje</t>
         </is>
       </c>
       <c r="D309" s="61" t="inlineStr">
         <is>
-          <t>El árbitro, el juez de línea y quien limpia las tribunas merecen su justo pago. Repasamos esta semana: digno es el obrero de su salario.</t>
+          <t>El árbitro, el juez de línea y quien limpia las tribunas merecen su justo pago. Digno es el obrero de su salario.</t>
         </is>
       </c>
     </row>
@@ -47594,7 +47594,7 @@
       </c>
       <c r="D316" s="61" t="inlineStr">
         <is>
-          <t>Cientos de recepciones en la práctica de vóley, para estar listos cuando llega el saque difícil. Queda de la semana: prepararnos para ayudar e invocar a Dios en la angustia.</t>
+          <t>Cientos de recepciones en la práctica de vóley, para estar listos cuando llega el saque difícil. Prepararse para ayudar y clamar a Dios en la angustia también se entrena.</t>
         </is>
       </c>
     </row>
@@ -47734,7 +47734,7 @@
       </c>
       <c r="D323" s="61" t="inlineStr">
         <is>
-          <t>Pinchó, quedó lejos del pelotón, y el ciclista igual sigue pedaleando. Con Habacuc cerramos el tema: aunque falte todo, Dios da fuerzas para seguir caminando.</t>
+          <t>Pinchó, quedó lejos del pelotón, y el ciclista igual sigue pedaleando. Aunque falte todo, Dios da fuerzas para seguir caminando.</t>
         </is>
       </c>
     </row>
@@ -47874,7 +47874,7 @@
       </c>
       <c r="D330" s="61" t="inlineStr">
         <is>
-          <t>Minuto cero de un clásico: cada uno tiene su plan de juego en la cabeza. Siete días después, la conclusión: muchos planes hay en el corazón, pero el consejo del Señor permanece.</t>
+          <t>Minuto cero de un clásico: cada uno tiene su plan de juego en la cabeza. Muchos planes hay en el corazón, pero el consejo del Señor permanece.</t>
         </is>
       </c>
     </row>
@@ -48014,7 +48014,7 @@
       </c>
       <c r="D337" s="61" t="inlineStr">
         <is>
-          <t>Hay padres e hijos que se reencontraron alentando juntos a la Albirroja después de años de distancia. Repasamos: Dios puede volver el corazón de los padres hacia los hijos.</t>
+          <t>Hay padres e hijos que se reencontraron alentando juntos a la Albirroja después de años de distancia. Dios puede volver el corazón de los padres hacia los hijos.</t>
         </is>
       </c>
     </row>
@@ -48154,7 +48154,7 @@
       </c>
       <c r="D344" s="61" t="inlineStr">
         <is>
-          <t>Primero lo más importante: así ordena el atleta su semana, y lo demás se acomoda. Para cerrar: buscar primero el reino de Dios y su justicia, confiando en que Él provee.</t>
+          <t>Primero lo más importante: así ordena el atleta su semana, y lo demás se acomoda. Buscá primero el reino de Dios y su justicia, confiando en que Él provee.</t>
         </is>
       </c>
     </row>
@@ -48369,7 +48369,7 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>árbitro</t>
+          <t>arbitraje</t>
         </is>
       </c>
       <c r="D355" s="61" t="inlineStr">
@@ -48434,7 +48434,7 @@
       </c>
       <c r="D358" s="61" t="inlineStr">
         <is>
-          <t>En Navidad las canchas se aquietan y la familia se junta. El sabio nunca deja de aprender, y hoy volvemos a aprender del mayor regalo: Jesús, nacido para salvarnos.</t>
+          <t>En Navidad las canchas se aquietan y la familia se junta. No teman: hay una buena noticia para todo el pueblo. Hoy nació el Salvador, Cristo el Señor.</t>
         </is>
       </c>
     </row>
@@ -48574,7 +48574,7 @@
       </c>
       <c r="D365" s="61" t="inlineStr">
         <is>
-          <t>Silbato final, penal errado, y una palabra amable del entrenador levanta el ánimo del jugador. Lo de estos días: las palabras bondadosas son dulces para el alma y salud para el cuerpo.</t>
+          <t>Silbato final, penal errado, y una palabra amable del entrenador levanta el ánimo del jugador. Las palabras bondadosas son dulces para el alma y salud para el cuerpo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Frases deportivas: versión compacta de las 364 (de 151 a 93 caracteres en promedio)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -41314,7 +41314,7 @@
       </c>
       <c r="D2" s="61" t="inlineStr">
         <is>
-          <t>Un atleta no se prepara solo el día de la final: se cuida todos los días. Tu cuerpo es templo del Espíritu, y cuidarlo con orden también honra a Dios.</t>
+          <t>El atleta no se cuida solo el día de la final. Tu cuerpo es templo: cuidarlo honra a Dios.</t>
         </is>
       </c>
     </row>
@@ -41334,7 +41334,7 @@
       </c>
       <c r="D3" s="61" t="inlineStr">
         <is>
-          <t>Ningún técnico trata a su mejor jugador como enemigo: lo cuida y lo prepara. Tu cuerpo no es tu rival; es parte de tu adoración a Dios.</t>
+          <t>Ningún técnico trata a su mejor jugador como enemigo. Tu cuerpo no es tu rival.</t>
         </is>
       </c>
     </row>
@@ -41354,7 +41354,7 @@
       </c>
       <c r="D4" s="61" t="inlineStr">
         <is>
-          <t>El nadador que se hidrata y estira no es vanidoso, es agradecido con lo que tiene. Cuidarte también es decirle gracias a Dios por la vida.</t>
+          <t>El nadador que se hidrata no es vanidoso: es agradecido. Cuidarte también es dar gracias.</t>
         </is>
       </c>
     </row>
@@ -41374,7 +41374,7 @@
       </c>
       <c r="D5" s="61" t="inlineStr">
         <is>
-          <t>En el ciclismo, pedalear un poquito cada día rinde más que un tirón un domingo. Hábitos pequeños, energía grande; y el alma también necesita su entrenamiento.</t>
+          <t>Pedalear un poco cada día rinde más que un tirón el domingo. El alma también se entrena.</t>
         </is>
       </c>
     </row>
@@ -41394,7 +41394,7 @@
       </c>
       <c r="D6" s="61" t="inlineStr">
         <is>
-          <t>Mirá el salto de un rematador de vóley: músculos, reflejos y equilibrio en un segundo. Tu cuerpo es obra formidable de Dios; tratalo con el respeto que merece.</t>
+          <t>Un remate de vóley: fuerza, reflejos y equilibrio en un segundo. Sos obra formidable de Dios.</t>
         </is>
       </c>
     </row>
@@ -41414,7 +41414,7 @@
       </c>
       <c r="D7" s="61" t="inlineStr">
         <is>
-          <t>Cambio en el futsal: el que sale a descansar no abandona al equipo, y vuelve a entrar entero. Descansar no es perder el tiempo, es parte del diseño de Dios.</t>
+          <t>En el futsal, el que sale a descansar vuelve entero. Descansar es parte del diseño de Dios.</t>
         </is>
       </c>
     </row>
@@ -41434,7 +41434,7 @@
       </c>
       <c r="D8" s="61" t="inlineStr">
         <is>
-          <t>El maratonista sabe que la carrera se corre con las piernas y con la cabeza. Cuidar el cuerpo y el alma que Dios nos dio va junto.</t>
+          <t>La maratón se corre con las piernas y con la cabeza. Cuerpo y alma van juntos.</t>
         </is>
       </c>
     </row>
@@ -41454,7 +41454,7 @@
       </c>
       <c r="D9" s="61" t="inlineStr">
         <is>
-          <t>El canchero que deja descansar una parte del césped tiene la cancha lista por años. Así el agricultor que rota sus cultivos cuida la tierra que Dios sostiene con fidelidad.</t>
+          <t>El canchero deja descansar el césped y la cancha dura años. La tierra también necesita descanso.</t>
         </is>
       </c>
     </row>
@@ -41474,7 +41474,7 @@
       </c>
       <c r="D10" s="61" t="inlineStr">
         <is>
-          <t>Lo que entrenás en la semana es lo que aparece el domingo en la cancha. Lo que se siembra se cosecha, y con Dios no hay atajos ni trampas.</t>
+          <t>Lo que entrenás en la semana aparece el domingo. Lo que se siembra se cosecha.</t>
         </is>
       </c>
     </row>
@@ -41494,7 +41494,7 @@
       </c>
       <c r="D11" s="61" t="inlineStr">
         <is>
-          <t>El velocista no ve crecer su fuerza mientras duerme, pero ahí también se está formando. Así crece el reino de Dios: más allá de lo que vos controlás.</t>
+          <t>El velocista también se fortalece mientras duerme. El reino de Dios crece más allá de lo que controlás.</t>
         </is>
       </c>
     </row>
@@ -41514,7 +41514,7 @@
       </c>
       <c r="D12" s="61" t="inlineStr">
         <is>
-          <t>El Rally del Chaco cruza campos que alguien trabajó con sus manos. Trabajar la tierra es un desafío y también una bendición, donde el esfuerzo se une a la provisión de Dios.</t>
+          <t>El rally cruza campos que alguien trabajó con sus manos. Trabajar la tierra es esfuerzo y bendición.</t>
         </is>
       </c>
     </row>
@@ -41534,7 +41534,7 @@
       </c>
       <c r="D13" s="61" t="inlineStr">
         <is>
-          <t>Apurar una jugada de ajedrez suele costar caro. El agricultor espera la lluvia con paciencia: lo que necesita su tiempo no se apura.</t>
+          <t>Apurar una jugada de ajedrez cuesta caro. Lo que necesita su tiempo no se apura.</t>
         </is>
       </c>
     </row>
@@ -41554,7 +41554,7 @@
       </c>
       <c r="D14" s="61" t="inlineStr">
         <is>
-          <t>El canchero cuida el césped como si fuera suyo, aunque la cancha es del club y la van a usar otros. La tierra es del Señor: la cuidamos para los que vienen detrás.</t>
+          <t>El canchero cuida la cancha aunque no es suya. La tierra es del Señor: la cuidamos para los que vienen.</t>
         </is>
       </c>
     </row>
@@ -41574,7 +41574,7 @@
       </c>
       <c r="D15" s="61" t="inlineStr">
         <is>
-          <t>Cada palada parece pequeña, pero sostenida lleva lejos al bote. Sembrar, aun con lágrimas, puede preceder a la alegría de la cosecha.</t>
+          <t>Palada a palada, el bote llega lejos. Lo que se siembra con lágrimas se cosecha con alegría.</t>
         </is>
       </c>
     </row>
@@ -41594,7 +41594,7 @@
       </c>
       <c r="D16" s="61" t="inlineStr">
         <is>
-          <t>El base que lee la defensa antes del pase evita la pelota perdida. El prudente ve el peligro y se protege; en la salud, revisar antes es mejor que lamentar después.</t>
+          <t>El base que lee la defensa evita la pelota perdida. En la salud, prevenir es mejor que lamentar.</t>
         </is>
       </c>
     </row>
@@ -41614,7 +41614,7 @@
       </c>
       <c r="D17" s="61" t="inlineStr">
         <is>
-          <t>El arquero que acomoda la barrera antes del tiro libre está cuidando a todo el equipo. Prevenir también es una manera de amar a los tuyos.</t>
+          <t>El arquero que arma la barrera cuida a todo el equipo. Prevenir también es amar.</t>
         </is>
       </c>
     </row>
@@ -41634,7 +41634,7 @@
       </c>
       <c r="D18" s="61" t="inlineStr">
         <is>
-          <t>Brazo con brazo, la defensa de handball se arma entre todos. Los hábitos que protegen a la familia también se construyen juntos, en casa, cada día.</t>
+          <t>La defensa de handball se arma entre todos. Los hábitos sanos de la familia, también.</t>
         </is>
       </c>
     </row>
@@ -41654,7 +41654,7 @@
       </c>
       <c r="D19" s="61" t="inlineStr">
         <is>
-          <t>El tenista que siente una molestia y la hace revisar a tiempo puede evitar una lesión mayor. Detectar a tiempo puede salvar vidas: escuchá las señales de tu cuerpo.</t>
+          <t>El tenista que revisa a tiempo una molestia evita una lesión. Escuchá las señales de tu cuerpo.</t>
         </is>
       </c>
     </row>
@@ -41674,7 +41674,7 @@
       </c>
       <c r="D20" s="61" t="inlineStr">
         <is>
-          <t>Hasta el boxeador más valiente pasa por el control médico antes de subir al ring. Animarse a hacerse los estudios no es miedo: es prudencia y humildad.</t>
+          <t>Hasta el boxeador más valiente pasa el control médico. Hacerse los estudios es prudencia, no miedo.</t>
         </is>
       </c>
     </row>
@@ -41694,7 +41694,7 @@
       </c>
       <c r="D21" s="61" t="inlineStr">
         <is>
-          <t>El ajedrecista sabe que con la cabeza caliente no se juega bien. Un corazón en paz da vida al cuerpo; la envidia y el estrés, en cambio, desgastan.</t>
+          <t>Con la cabeza caliente no se juega bien al ajedrez. Un corazón en paz da vida al cuerpo.</t>
         </is>
       </c>
     </row>
@@ -41714,7 +41714,7 @@
       </c>
       <c r="D22" s="61" t="inlineStr">
         <is>
-          <t>Sin que nadie lo aplauda, el utilero revisa cada botín antes del partido. Prevenir es amar, y bendecimos a Dios por su cuidado de cada día.</t>
+          <t>Sin aplausos, el utilero revisa cada botín. Prevenir es amar, y Dios nos cuida cada día.</t>
         </is>
       </c>
     </row>
@@ -41734,7 +41734,7 @@
       </c>
       <c r="D23" s="61" t="inlineStr">
         <is>
-          <t>Curva por curva, el copiloto de rally lee la hoja de ruta en voz alta. La Palabra de Dios es esa lámpara que ilumina el camino, lo cercano y lo lejano.</t>
+          <t>El copiloto de rally lee la hoja de ruta curva por curva. La Palabra es lámpara para tu camino.</t>
         </is>
       </c>
     </row>
@@ -41754,7 +41754,7 @@
       </c>
       <c r="D24" s="61" t="inlineStr">
         <is>
-          <t>Leer el reglamento no es lo mismo que estudiarlo como lo hace un árbitro. Con la Biblia pasa igual: leerla es bueno, estudiarla te forma.</t>
+          <t>Leer el reglamento no es estudiarlo como un árbitro. Leer la Biblia es bueno; estudiarla te forma.</t>
         </is>
       </c>
     </row>
@@ -41774,7 +41774,7 @@
       </c>
       <c r="D25" s="61" t="inlineStr">
         <is>
-          <t>De nada sirve la charla técnica si después no se hace en la cancha. La Palabra se medita y se practica, para andar en el camino de Dios.</t>
+          <t>La charla técnica sirve si se juega en la cancha. La Palabra se medita y se practica.</t>
         </is>
       </c>
     </row>
@@ -41794,7 +41794,7 @@
       </c>
       <c r="D26" s="61" t="inlineStr">
         <is>
-          <t>El entrenador de vóley mira el video del partido una y otra vez, buscando detalles. Estudiar la Biblia con método es ir más allá de la superficie, porque la Palabra está viva.</t>
+          <t>El entrenador ve el partido una y otra vez buscando detalles. La Palabra está viva: estudiala a fondo.</t>
         </is>
       </c>
     </row>
@@ -41814,7 +41814,7 @@
       </c>
       <c r="D27" s="61" t="inlineStr">
         <is>
-          <t>Nadie corre una maratón sin un plan que se pueda cumplir, semana a semana. Con la Biblia también: mejor un plan sencillo y constante que uno enorme que se abandona.</t>
+          <t>Nadie corre una maratón sin un plan posible. Mejor un plan sencillo de lectura que uno enorme abandonado.</t>
         </is>
       </c>
     </row>
@@ -41834,7 +41834,7 @@
       </c>
       <c r="D28" s="61" t="inlineStr">
         <is>
-          <t>Cuántos vivieron un partido entero solo escuchando al relator por la radio. La fe también entra por el oído: escuchar la Palabra la fortalece.</t>
+          <t>Cuántos vivieron un partido solo por la radio. La fe también entra por el oído.</t>
         </is>
       </c>
     </row>
@@ -41854,7 +41854,7 @@
       </c>
       <c r="D29" s="61" t="inlineStr">
         <is>
-          <t>El nadador que entrena con constancia hace del agua su lugar. La Palabra estudiada y vivida se vuelve propia y llena de gozo el corazón.</t>
+          <t>Con constancia, el nadador hace del agua su lugar. La Palabra vivida se vuelve propia.</t>
         </is>
       </c>
     </row>
@@ -41874,7 +41874,7 @@
       </c>
       <c r="D30" s="61" t="inlineStr">
         <is>
-          <t>A un capitán de la Albirroja no se lo elige por el peinado, sino por lo que muestra adentro. Dios mira el corazón, y ahí empieza todo liderazgo.</t>
+          <t>Al capitán no se lo elige por el peinado. Dios mira el corazón: ahí empieza el liderazgo.</t>
         </is>
       </c>
     </row>
@@ -41894,7 +41894,7 @@
       </c>
       <c r="D31" s="61" t="inlineStr">
         <is>
-          <t>¿Sabías que muchas subidas en bici se ganan o se pierden primero en la cabeza? El liderazgo empieza por dentro: cuidá tu corazón, porque de ahí salen tus decisiones.</t>
+          <t>Muchas subidas en bici se ganan primero en la cabeza. El liderazgo empieza por dentro.</t>
         </is>
       </c>
     </row>
@@ -41914,7 +41914,7 @@
       </c>
       <c r="D32" s="61" t="inlineStr">
         <is>
-          <t>El entrenador que pide puntualidad y llega primero no necesita gritar. Primero el ejemplo, después la palabra: el líder enseña con su vida.</t>
+          <t>El técnico que pide puntualidad y llega primero no necesita gritar. Primero el ejemplo.</t>
         </is>
       </c>
     </row>
@@ -41934,7 +41934,7 @@
       </c>
       <c r="D33" s="61" t="inlineStr">
         <is>
-          <t>En el futsal de barrio, a veces el más chico es el que más corre y contagia ganas. Nadie es demasiado joven para ser ejemplo en palabra, conducta, amor y fe.</t>
+          <t>En el futsal de barrio, a veces el más chico contagia las ganas. Nadie es demasiado joven para ser ejemplo.</t>
         </is>
       </c>
     </row>
@@ -41954,7 +41954,7 @@
       </c>
       <c r="D34" s="61" t="inlineStr">
         <is>
-          <t>Un árbitro tarda años en ganarse el respeto de las canchas. Tu buen nombre vale más que tu plata, y se cuida en cada decisión.</t>
+          <t>Un árbitro tarda años en ganarse el respeto. Tu buen nombre vale más que tu plata.</t>
         </is>
       </c>
     </row>
@@ -41974,7 +41974,7 @@
       </c>
       <c r="D35" s="61" t="inlineStr">
         <is>
-          <t>Técnica sin compromiso no sostiene a ningún equipo de básquet. Corazón íntegro y manos hábiles: el carácter es el que sostiene la capacidad.</t>
+          <t>Técnica sin compromiso no sostiene a un equipo. El carácter sostiene la capacidad.</t>
         </is>
       </c>
     </row>
@@ -41994,7 +41994,7 @@
       </c>
       <c r="D36" s="61" t="inlineStr">
         <is>
-          <t>Tenis amateur: muchas veces el propio jugador canta si la pelota fue afuera. El líder se forma por dentro, íntegro aun cuando nadie mira.</t>
+          <t>En el tenis amateur, el jugador canta su propia pelota afuera. El líder es íntegro aunque nadie mire.</t>
         </is>
       </c>
     </row>
@@ -42014,7 +42014,7 @@
       </c>
       <c r="D37" s="61" t="inlineStr">
         <is>
-          <t>Antes de cada temporada, un equipo define a qué juega y con quién. En casa también hay que elegir a quién servir; esa decisión marca el rumbo de la familia.</t>
+          <t>Cada equipo define a qué juega. En casa también se elige a quién servir.</t>
         </is>
       </c>
     </row>
@@ -42034,7 +42034,7 @@
       </c>
       <c r="D38" s="61" t="inlineStr">
         <is>
-          <t>Un buen sistema de juego no se arma a los gritos, sino con sabiduría y entendimiento. Así también se edifica una casa: con sabiduría, día a día.</t>
+          <t>Un sistema de juego no se arma a los gritos. Una casa se edifica con sabiduría.</t>
         </is>
       </c>
     </row>
@@ -42054,7 +42054,7 @@
       </c>
       <c r="D39" s="61" t="inlineStr">
         <is>
-          <t>Cada camiseta en su lugar: así deja el vestuario el utilero, y eso le da paz al plantel. El orden en casa no es rigidez, también es una forma de amar.</t>
+          <t>El utilero deja cada camiseta en su lugar y el plantel juega en paz. El orden en casa también es amor.</t>
         </is>
       </c>
     </row>
@@ -42074,7 +42074,7 @@
       </c>
       <c r="D40" s="61" t="inlineStr">
         <is>
-          <t>En el remo, el timonel está atento a la marcha del bote todo el tiempo. Estar atentos a la marcha de la casa es una diligencia que, aunque nadie aplauda, se nota.</t>
+          <t>El timonel no deja de mirar la marcha del bote. Estar atentos a la casa se nota, aunque nadie aplauda.</t>
         </is>
       </c>
     </row>
@@ -42094,7 +42094,7 @@
       </c>
       <c r="D41" s="61" t="inlineStr">
         <is>
-          <t>El atleta entrena duro, pero sabe que el aliento y la vida no los fabrica él. Si Dios no edifica la casa, el esfuerzo solo no alcanza; lo que Él edifica permanece.</t>
+          <t>El atleta entrena duro, pero la vida no la fabrica él. Si Dios no edifica la casa, no alcanza.</t>
         </is>
       </c>
     </row>
@@ -42114,7 +42114,7 @@
       </c>
       <c r="D42" s="61" t="inlineStr">
         <is>
-          <t>Un estadio bien cimentado aguanta la tormenta y a la hinchada saltando. La casa sobre la roca es la que se edifica oyendo y obedeciendo la Palabra.</t>
+          <t>Un estadio bien cimentado aguanta la tormenta. Una casa sobre la roca, también.</t>
         </is>
       </c>
     </row>
@@ -42134,7 +42134,7 @@
       </c>
       <c r="D43" s="61" t="inlineStr">
         <is>
-          <t>Con calma se ve todo el tablero de ajedrez. Así se vive en un hogar donde la paz de Dios gobierna el corazón: con gratitud y sin imposiciones.</t>
+          <t>Con calma se ve todo el tablero. En casa, que la paz de Dios gobierne el corazón.</t>
         </is>
       </c>
     </row>
@@ -42154,7 +42154,7 @@
       </c>
       <c r="D44" s="61" t="inlineStr">
         <is>
-          <t>El técnico prudente guarda piernas para el segundo tiempo y no las gasta todas al principio. El sabio guarda; la prudencia con lo que tenés también habla de tu carácter.</t>
+          <t>El técnico prudente guarda piernas para el segundo tiempo. El sabio también guarda.</t>
         </is>
       </c>
     </row>
@@ -42174,7 +42174,7 @@
       </c>
       <c r="D45" s="61" t="inlineStr">
         <is>
-          <t>El que se prepara para una maratón sale a entrenar cada mañana sin que nadie lo mande. Como la hormiga, se prepara en el verano para el invierno.</t>
+          <t>El maratonista entrena sin que nadie lo mande. Como la hormiga, se prepara para el invierno.</t>
         </is>
       </c>
     </row>
@@ -42194,7 +42194,7 @@
       </c>
       <c r="D46" s="61" t="inlineStr">
         <is>
-          <t>El equipo que cuida sus tiempos muertos tiene uno guardado para el final apretado. José juntó en los años buenos para proteger a su pueblo en los años malos.</t>
+          <t>El que cuida sus tiempos muertos tiene uno para el final. José guardó en los años buenos.</t>
         </is>
       </c>
     </row>
@@ -42214,7 +42214,7 @@
       </c>
       <c r="D47" s="61" t="inlineStr">
         <is>
-          <t>Etapa por etapa, no de un solo salto: así se avanza en una vuelta ciclista. Con el ahorro pasa igual, de a poco y con mano constante se llega lejos.</t>
+          <t>Una vuelta ciclista se gana etapa por etapa. El ahorro también: de a poco y constante.</t>
         </is>
       </c>
     </row>
@@ -42234,7 +42234,7 @@
       </c>
       <c r="D48" s="61" t="inlineStr">
         <is>
-          <t>Ningún técnico arma un plantel con un solo jugador para todos los puestos. Repartir el riesgo es prudencia, y este consejo del Eclesiastés tiene más de una lectura.</t>
+          <t>Ningún técnico arma un plantel con un solo jugador. Repartir el riesgo es prudencia.</t>
         </is>
       </c>
     </row>
@@ -42254,7 +42254,7 @@
       </c>
       <c r="D49" s="61" t="inlineStr">
         <is>
-          <t>En el rally, el piloto revisa combustible y cubiertas antes de cada tramo. Conocé bien el estado de tus finanzas, porque las riquezas no duran para siempre.</t>
+          <t>El piloto revisa combustible y cubiertas antes de cada tramo. Conocé bien tus finanzas.</t>
         </is>
       </c>
     </row>
@@ -42274,7 +42274,7 @@
       </c>
       <c r="D50" s="61" t="inlineStr">
         <is>
-          <t>Antes de largar la regata, el remero calcula sus fuerzas. Ahorrar es prepararse, con la seguridad de fondo puesta en Dios y no en la plata.</t>
+          <t>El remero calcula sus fuerzas antes de largar. Ahorrar es prepararse, con la confianza puesta en Dios.</t>
         </is>
       </c>
     </row>
@@ -42294,7 +42294,7 @@
       </c>
       <c r="D51" s="61" t="inlineStr">
         <is>
-          <t>Hasta el mejor nadador sale del agua cuando el cuerpo le avisa. Escuchar las señales del alma importa, y la paz de Dios guarda tu corazón aun cuando no todo está resuelto.</t>
+          <t>Hasta el mejor nadador sale del agua cuando el cuerpo avisa. Escuchá también las señales del alma.</t>
         </is>
       </c>
     </row>
@@ -42314,7 +42314,7 @@
       </c>
       <c r="D52" s="61" t="inlineStr">
         <is>
-          <t>A veces, en el vestuario, lo más valiente es decir: hoy no estoy bien. Como el salmista, ponerle nombre al desánimo es el primer paso para volver a esperar en Dios.</t>
+          <t>En el vestuario, lo más valiente es decir: hoy no estoy bien. Nombrar el desánimo es volver a esperar en Dios.</t>
         </is>
       </c>
     </row>
@@ -42334,7 +42334,7 @@
       </c>
       <c r="D53" s="61" t="inlineStr">
         <is>
-          <t>El ajedrecista que aprende a pensar distinto el juego cambia la partida entera. La transformación empieza en la mente, y es Dios quien la va renovando.</t>
+          <t>El ajedrecista que piensa distinto cambia la partida. Dios renueva tu mente.</t>
         </is>
       </c>
     </row>
@@ -42354,7 +42354,7 @@
       </c>
       <c r="D54" s="61" t="inlineStr">
         <is>
-          <t>El arquero no se distrae con todo lo que pasa en la tribuna: fija los ojos en la pelota. Elegí qué ponés delante de tus ojos; lo que mirás también forma tu mente.</t>
+          <t>El arquero fija los ojos en la pelota, no en la tribuna. Lo que mirás forma tu mente.</t>
         </is>
       </c>
     </row>
@@ -42374,7 +42374,7 @@
       </c>
       <c r="D55" s="61" t="inlineStr">
         <is>
-          <t>Un tenista puede sentir nervios antes del saque, y eso no lo define. El miedo no es tu identidad: Dios nos da poder, amor y dominio propio.</t>
+          <t>Los nervios antes del saque no definen al tenista. Dios nos da poder, amor y dominio propio.</t>
         </is>
       </c>
     </row>
@@ -42394,7 +42394,7 @@
       </c>
       <c r="D56" s="61" t="inlineStr">
         <is>
-          <t>Hasta el boxeador más fuerte tiene a alguien en su esquina que lo cuida entre round y round. Pedir ayuda, también a un profesional, es sabiduría y no debilidad.</t>
+          <t>Hasta el boxeador más fuerte tiene a alguien en su esquina. Pedir ayuda es sabiduría.</t>
         </is>
       </c>
     </row>
@@ -42414,7 +42414,7 @@
       </c>
       <c r="D57" s="61" t="inlineStr">
         <is>
-          <t>Nadie corre todos los tramos de una posta solo. Dios está cerca del quebrantado: cuidá tu alma sabiendo que no tenés que cargar todo solo.</t>
+          <t>Nadie corre todos los tramos de una posta solo. Dios está cerca del quebrantado.</t>
         </is>
       </c>
     </row>
@@ -42434,7 +42434,7 @@
       </c>
       <c r="D58" s="61" t="inlineStr">
         <is>
-          <t>El preparador físico que conoce de cerca a cada jugador nota el cansancio antes que nadie. Conocer bien lo que tenés a cargo, cada día, es responsabilidad del que cuida.</t>
+          <t>El preparador físico nota el cansancio antes que nadie. Cuidar es conocer de cerca.</t>
         </is>
       </c>
     </row>
@@ -42454,7 +42454,7 @@
       </c>
       <c r="D59" s="61" t="inlineStr">
         <is>
-          <t>El árbitro tiene autoridad en la cancha, pero no para hacer lo que quiera. El dominio sobre los animales es un encargo de Dios, no un permiso para abusar.</t>
+          <t>El árbitro tiene autoridad, pero no para hacer lo que quiera. Dominar la creación es cuidarla.</t>
         </is>
       </c>
     </row>
@@ -42474,7 +42474,7 @@
       </c>
       <c r="D60" s="61" t="inlineStr">
         <is>
-          <t>El buen técnico sabe cuándo darle descanso al plantel. Así es Dios como pastor: provee descanso y alimento, y su cuidado nos enseña a cuidar.</t>
+          <t>El buen técnico sabe cuándo dar descanso. Así es Dios como pastor.</t>
         </is>
       </c>
     </row>
@@ -42494,7 +42494,7 @@
       </c>
       <c r="D61" s="61" t="inlineStr">
         <is>
-          <t>Se nota en la cancha quién trata bien a los demás, aun cuando nadie mira. El justo cuida la vida de sus animales, y ese trato le importa a Dios.</t>
+          <t>En la cancha se nota quién trata bien, aun sin testigos. El justo cuida a sus animales.</t>
         </is>
       </c>
     </row>
@@ -42514,7 +42514,7 @@
       </c>
       <c r="D62" s="61" t="inlineStr">
         <is>
-          <t>En la maratón, el trabajo fiel de muchos meses se nota en los últimos kilómetros. Jacob cuidó el ganado con fidelidad, y la bendición de Dios acompañó ese trabajo.</t>
+          <t>En la maratón, meses de trabajo fiel se notan al final. Jacob cuidó el ganado con fidelidad.</t>
         </is>
       </c>
     </row>
@@ -42534,7 +42534,7 @@
       </c>
       <c r="D63" s="61" t="inlineStr">
         <is>
-          <t>El líbero se tira al piso para salvar la pelota de su compañero. Jesús, el buen pastor, fue mucho más lejos: dio su vida por las ovejas.</t>
+          <t>El líbero se tira al piso por su compañero. El buen pastor dio su vida por las ovejas.</t>
         </is>
       </c>
     </row>
@@ -42554,7 +42554,7 @@
       </c>
       <c r="D64" s="61" t="inlineStr">
         <is>
-          <t>Compañero golpeado en el handball: el equipo lo protege hasta que se recupera. Así cuida Dios: con ternura, cargando al más débil.</t>
+          <t>Al compañero golpeado, el equipo lo protege. Así cuida Dios: cargando al más débil.</t>
         </is>
       </c>
     </row>
@@ -42574,7 +42574,7 @@
       </c>
       <c r="D65" s="61" t="inlineStr">
         <is>
-          <t>Entre set y set, el tenista se sienta, respira y suelta la tensión. Entregale a Dios tus angustias, también las de la salud, y descansá en su cuidado.</t>
+          <t>Entre set y set, el tenista respira. Entregale a Dios tus angustias, también las de salud.</t>
         </is>
       </c>
     </row>
@@ -42594,7 +42594,7 @@
       </c>
       <c r="D66" s="61" t="inlineStr">
         <is>
-          <t>Cuando un jugador se lesiona, nadie le reprocha que entre el médico a la cancha. Reconocer que necesitás ayuda es el primer paso, y buscarla no es debilidad.</t>
+          <t>Cuando un jugador se lesiona, entra el médico y nadie lo reprocha. Buscar ayuda no es debilidad.</t>
         </is>
       </c>
     </row>
@@ -42614,7 +42614,7 @@
       </c>
       <c r="D67" s="61" t="inlineStr">
         <is>
-          <t>Detrás de un equipo de ciclismo siempre hay un médico que acompaña la carrera. Lucas, el médico amado, fue parte del equipo de Pablo: la medicina y la fe caminan juntas.</t>
+          <t>Toda vuelta ciclista lleva un médico. Lucas fue médico y compañero de Pablo: medicina y fe caminan juntas.</t>
         </is>
       </c>
     </row>
@@ -42634,7 +42634,7 @@
       </c>
       <c r="D68" s="61" t="inlineStr">
         <is>
-          <t>Cuando un atleta cae en la pista, alguien se acerca a ayudarlo a levantarse. Sáname, Señor, es una oración humilde de quien confía en el Dios que sana y salva.</t>
+          <t>Cuando un atleta cae, alguien lo ayuda a levantarse. «Sáname, Señor» es una oración humilde.</t>
         </is>
       </c>
     </row>
@@ -42654,7 +42654,7 @@
       </c>
       <c r="D69" s="61" t="inlineStr">
         <is>
-          <t>El jugador que ora antes del partido también hace caso al kinesiólogo. Dios obra a través de medios: la fe y el tratamiento médico no se oponen.</t>
+          <t>El jugador que ora también le hace caso al kinesiólogo. La fe y el tratamiento no se oponen.</t>
         </is>
       </c>
     </row>
@@ -42674,7 +42674,7 @@
       </c>
       <c r="D70" s="61" t="inlineStr">
         <is>
-          <t>El nadador que escucha a su entrenador corrige la brazada antes de lastimarse. El sabio escucha el consejo, y en la salud eso incluye a los profesionales.</t>
+          <t>El nadador que escucha al entrenador corrige a tiempo. El sabio escucha consejo, también el médico.</t>
         </is>
       </c>
     </row>
@@ -42694,7 +42694,7 @@
       </c>
       <c r="D71" s="61" t="inlineStr">
         <is>
-          <t>Un pase a tiempo vale más que diez apurados al final del partido de futsal. Cuidarse a tiempo también es sabiduría, con Dios como escudo que afirma nuestros pasos.</t>
+          <t>Un pase a tiempo vale más que diez apurados. Cuidarse a tiempo es sabiduría.</t>
         </is>
       </c>
     </row>
@@ -42714,7 +42714,7 @@
       </c>
       <c r="D72" s="61" t="inlineStr">
         <is>
-          <t>Un hincha solo se oye poco, pero la hinchada junta llena el estadio. Como el carbón en la brasa, la fe se mantiene encendida cuando nos reunimos en el nombre de Jesús.</t>
+          <t>Un hincha solo se oye poco; la hinchada junta llena el estadio. La fe se aviva en comunidad.</t>
         </is>
       </c>
     </row>
@@ -42734,7 +42734,7 @@
       </c>
       <c r="D73" s="61" t="inlineStr">
         <is>
-          <t>Ningún equipo sale a la cancha con un solo jugador. La fe nunca fue para vivirla solo: la iglesia primitiva perseveraba unida en la enseñanza, la comunión y la oración.</t>
+          <t>Ningún equipo sale a la cancha con un solo jugador. La fe no es para vivirla solo.</t>
         </is>
       </c>
     </row>
@@ -42754,7 +42754,7 @@
       </c>
       <c r="D74" s="61" t="inlineStr">
         <is>
-          <t>En el vóley de playa son dos, y cuando uno cae, el otro lo ayuda a levantarse. Mejor dos que uno: qué bueno tener a alguien que te ponga de pie.</t>
+          <t>En el vóley de playa, cuando uno cae, el otro lo levanta. Mejor dos que uno.</t>
         </is>
       </c>
     </row>
@@ -42774,7 +42774,7 @@
       </c>
       <c r="D75" s="61" t="inlineStr">
         <is>
-          <t>Si piloto y copiloto no se dicen todo con claridad, el auto de rally se sale del camino. Caminar en la luz es comunión transparente con Dios y con los hermanos.</t>
+          <t>Si piloto y copiloto no hablan claro, el auto se sale del camino. La comunión pide transparencia.</t>
         </is>
       </c>
     </row>
@@ -42794,7 +42794,7 @@
       </c>
       <c r="D76" s="61" t="inlineStr">
         <is>
-          <t>Ningún puesto sobra en el handball: cada uno cumple su función. Somos un solo cuerpo con muchos miembros, y cada uno depende de los demás.</t>
+          <t>En el handball ningún puesto sobra. Somos un cuerpo con muchos miembros.</t>
         </is>
       </c>
     </row>
@@ -42814,7 +42814,7 @@
       </c>
       <c r="D77" s="61" t="inlineStr">
         <is>
-          <t>En el entrenamiento, el compañero que te devuelve fuerte la pelota es el que te hace mejorar. El hierro se afila con hierro: nadie crece completamente solo.</t>
+          <t>El compañero que te devuelve fuerte la pelota te hace mejor. El hierro se afila con hierro.</t>
         </is>
       </c>
     </row>
@@ -42834,7 +42834,7 @@
       </c>
       <c r="D78" s="61" t="inlineStr">
         <is>
-          <t>Turnándose para cortar el viento, los ciclistas del pelotón llegan más lejos juntos. La fe se vive en comunidad, con un mismo amor.</t>
+          <t>En el pelotón se turnan para cortar el viento y llegan más lejos. La fe se vive en comunidad.</t>
         </is>
       </c>
     </row>
@@ -42854,7 +42854,7 @@
       </c>
       <c r="D79" s="61" t="inlineStr">
         <is>
-          <t>Un árbitro que habla con calma desactiva más de una discusión en la cancha. La respuesta suave calma el enojo; el tono importa tanto como lo que decís.</t>
+          <t>El árbitro que habla con calma apaga discusiones. La respuesta suave calma el enojo.</t>
         </is>
       </c>
     </row>
@@ -42874,7 +42874,7 @@
       </c>
       <c r="D80" s="61" t="inlineStr">
         <is>
-          <t>El buen capitán escucha a sus compañeros antes de dar la indicación. Ser pronto para oír y tardo para hablar evita errores y ayuda a liderar sin enojo.</t>
+          <t>El buen capitán escucha antes de indicar. Pronto para oír, tardo para hablar.</t>
         </is>
       </c>
     </row>
@@ -42894,7 +42894,7 @@
       </c>
       <c r="D81" s="61" t="inlineStr">
         <is>
-          <t>Un director técnico no puede atajar, defender y hacer los goles a la vez. Como Moisés, el líder aprende a delegar en personas capaces y a no cargar todo solo.</t>
+          <t>Un técnico no puede atajar, defender y hacer goles. El líder aprende a delegar.</t>
         </is>
       </c>
     </row>
@@ -42914,7 +42914,7 @@
       </c>
       <c r="D82" s="61" t="inlineStr">
         <is>
-          <t>El maratonista arma su plan, pero en la ruta se adapta al viento y al calor. Planificá con cuidado y soltá, porque es Dios quien dirige tus pasos.</t>
+          <t>El maratonista planifica, pero se adapta al viento. Planificá y dejá que Dios dirija tus pasos.</t>
         </is>
       </c>
     </row>
@@ -42934,7 +42934,7 @@
       </c>
       <c r="D83" s="61" t="inlineStr">
         <is>
-          <t>Un tiempo muerto pedido en el momento justo cambia el ritmo del partido de básquet. Hay un tiempo para cada cosa, y saber discernirlo es sabiduría.</t>
+          <t>Un tiempo muerto a tiempo cambia el partido. Hay un tiempo para cada cosa.</t>
         </is>
       </c>
     </row>
@@ -42954,7 +42954,7 @@
       </c>
       <c r="D84" s="61" t="inlineStr">
         <is>
-          <t>En la posta, uno corre el tramo más duro para que el compañero pueda llegar. En la cruz, Jesús cargó lo que no podíamos cargar: por sus heridas fuimos sanados.</t>
+          <t>En la posta, uno corre el tramo más duro por el otro. En la cruz, Jesús cargó lo nuestro: por sus heridas fuimos sanados.</t>
         </is>
       </c>
     </row>
@@ -42974,7 +42974,7 @@
       </c>
       <c r="D85" s="61" t="inlineStr">
         <is>
-          <t>El timonel marca el ritmo y el bote avanza parejo. Liderar es eso: marcar el paso con responsabilidad, con sabiduría y aprovechando bien el tiempo.</t>
+          <t>El timonel marca el ritmo y el bote avanza parejo. Liderar es marcar el paso con sabiduría.</t>
         </is>
       </c>
     </row>
@@ -42994,7 +42994,7 @@
       </c>
       <c r="D86" s="61" t="inlineStr">
         <is>
-          <t>Un partido no termina hasta el silbato final, aunque muchos lo den por perdido. En Pascua celebramos que la muerte no tiene la última palabra: Jesús es la resurrección y la vida.</t>
+          <t>Un partido no termina hasta el silbato final. La muerte no tiene la última palabra: Jesús es la resurrección y la vida.</t>
         </is>
       </c>
     </row>
@@ -43014,7 +43014,7 @@
       </c>
       <c r="D87" s="61" t="inlineStr">
         <is>
-          <t>El capitán que se tira a bloquear el remate para cuidar al equipo entiende algo del amor. Ser cabeza en el hogar es entregarse, como Cristo se entregó.</t>
+          <t>El capitán que se tira a bloquear por el equipo entiende el amor. Ser cabeza es entregarse, como Cristo.</t>
         </is>
       </c>
     </row>
@@ -43034,7 +43034,7 @@
       </c>
       <c r="D88" s="61" t="inlineStr">
         <is>
-          <t>La armadora y la que remata se necesitan y se respetan. En el matrimonio, amor y honra se complementan, con el mismo valor.</t>
+          <t>La armadora y la rematadora se necesitan y se respetan. En el matrimonio, amor y honra van juntos.</t>
         </is>
       </c>
     </row>
@@ -43054,7 +43054,7 @@
       </c>
       <c r="D89" s="61" t="inlineStr">
         <is>
-          <t>En el tenis de dobles, los compañeros se cubren y no se hablan con dureza en medio del partido. En el matrimonio, el respeto y el amor juegan del mismo lado de la red.</t>
+          <t>En el tenis de dobles, nadie se habla con dureza. Respeto y amor juegan del mismo lado de la red.</t>
         </is>
       </c>
     </row>
@@ -43074,7 +43074,7 @@
       </c>
       <c r="D90" s="61" t="inlineStr">
         <is>
-          <t>El utilero no busca lo suyo: lava, ordena y sirve para que otros jueguen. Así es el amor que se ve en lo que hace: paciente, bondadoso, sin buscar lo propio.</t>
+          <t>El utilero no busca lo suyo: sirve para que otros jueguen. Así es el amor.</t>
         </is>
       </c>
     </row>
@@ -43094,7 +43094,7 @@
       </c>
       <c r="D91" s="61" t="inlineStr">
         <is>
-          <t>¡Qué alegría encontrar al compañero justo para tirar la pared en el futsal! Tu pareja es un regalo, un favor de Dios y no solo cuestión de suerte.</t>
+          <t>¡Qué alegría encontrar al compañero justo para la pared! Tu pareja es un regalo de Dios.</t>
         </is>
       </c>
     </row>
@@ -43114,7 +43114,7 @@
       </c>
       <c r="D92" s="61" t="inlineStr">
         <is>
-          <t>Llueva o truene, la hinchada sigue a su equipo: el amor verdadero no se apaga. Ni las muchas aguas pueden extinguirlo.</t>
+          <t>Llueva o truene, la hinchada sigue a su equipo. El amor verdadero no se apaga.</t>
         </is>
       </c>
     </row>
@@ -43134,7 +43134,7 @@
       </c>
       <c r="D93" s="61" t="inlineStr">
         <is>
-          <t>Nadie larga en el Rally del Chaco sin calcular el combustible del tramo. Con la plata pasa lo mismo: el plan se hace antes de largar, no en medio del polvo.</t>
+          <t>Nadie larga un rally sin calcular el combustible. Con la plata, el plan se hace antes de largar.</t>
         </is>
       </c>
     </row>
@@ -43154,7 +43154,7 @@
       </c>
       <c r="D94" s="61" t="inlineStr">
         <is>
-          <t>El maratonista no abandona cuando le pesan las piernas; sostener el presupuesto mes a mes también es cuestión de constancia, paso a paso.</t>
+          <t>El maratonista no abandona cuando le pesan las piernas. El presupuesto también se sostiene paso a paso.</t>
         </is>
       </c>
     </row>
@@ -43174,7 +43174,7 @@
       </c>
       <c r="D95" s="61" t="inlineStr">
         <is>
-          <t>En el ajedrez, la jugada apurada suele costar una pieza; pensá la siguiente movida con calma, también antes de gastar.</t>
+          <t>En el ajedrez, la jugada apurada cuesta una pieza. Pensá con calma antes de gastar.</t>
         </is>
       </c>
     </row>
@@ -43194,7 +43194,7 @@
       </c>
       <c r="D96" s="61" t="inlineStr">
         <is>
-          <t>El buen defensor lee la jugada antes de que llegue el pase, atento pero sin malicia; así se cuida la plata: prudente y con el corazón limpio.</t>
+          <t>El buen defensor lee la jugada, atento pero sin malicia. Así se cuida la plata.</t>
         </is>
       </c>
     </row>
@@ -43214,7 +43214,7 @@
       </c>
       <c r="D97" s="61" t="inlineStr">
         <is>
-          <t>Cada segundo del reloj cuenta, y el buen base de básquet lo administra con cabeza. El tiempo y los recursos que Dios te da también se juegan con sabiduría.</t>
+          <t>El base administra cada segundo del reloj. Tu tiempo y tus recursos también se juegan con sabiduría.</t>
         </is>
       </c>
     </row>
@@ -43234,7 +43234,7 @@
       </c>
       <c r="D98" s="61" t="inlineStr">
         <is>
-          <t>Cada jugador de futsal entra a la cancha a aportar lo que tiene en las piernas. Dar también es eso: aportar con constancia, según lo que recibiste.</t>
+          <t>Cada jugador aporta lo que tiene en las piernas. Dar es aportar según lo que recibiste.</t>
         </is>
       </c>
     </row>
@@ -43254,7 +43254,7 @@
       </c>
       <c r="D99" s="61" t="inlineStr">
         <is>
-          <t>Las camisetas no son del utilero, pero las cuida como si lo fueran. Así somos llamados a cuidar lo que Dios nos prestó: como administradores confiables.</t>
+          <t>Las camisetas no son del utilero, pero las cuida como propias. Somos administradores de lo que Dios presta.</t>
         </is>
       </c>
     </row>
@@ -43274,7 +43274,7 @@
       </c>
       <c r="D100" s="61" t="inlineStr">
         <is>
-          <t>El ciclista que se suelta del pelotón sigue pedaleando, pero se desgasta solo; separados de Cristo podemos seguir andando, pero el fruto viene de permanecer en Él.</t>
+          <t>El ciclista que se suelta del pelotón se desgasta solo. El fruto viene de permanecer en Cristo.</t>
         </is>
       </c>
     </row>
@@ -43294,7 +43294,7 @@
       </c>
       <c r="D101" s="61" t="inlineStr">
         <is>
-          <t>Ningún entrenador fabrica en una semana la química de un equipo; el fruto del Espíritu tampoco se fuerza: crece con el tiempo en quien permanece.</t>
+          <t>La química de un equipo no se fabrica en una semana. El fruto del Espíritu crece con el tiempo.</t>
         </is>
       </c>
     </row>
@@ -43314,7 +43314,7 @@
       </c>
       <c r="D102" s="61" t="inlineStr">
         <is>
-          <t>El atleta que sale a correr de madrugada y vuelve con sed sabe lo que es necesitar agua de verdad; así también puede tener sed el alma: sed de Dios.</t>
+          <t>El que corre de madrugada sabe lo que es tener sed. El alma también tiene sed de Dios.</t>
         </is>
       </c>
     </row>
@@ -43334,7 +43334,7 @@
       </c>
       <c r="D103" s="61" t="inlineStr">
         <is>
-          <t>El nadador cansado aprende a respirar antes de seguir braceando; esperar en el Señor no es abandonar la carrera, es recibir fuerzas nuevas.</t>
+          <t>El nadador cansado respira antes de seguir. Esperar en el Señor renueva las fuerzas.</t>
         </is>
       </c>
     </row>
@@ -43354,7 +43354,7 @@
       </c>
       <c r="D104" s="61" t="inlineStr">
         <is>
-          <t>Hasta el tenista con más años de circuito sigue puliendo su revés cada temporada; en la gracia y el conocimiento de Jesús nunca dejamos de crecer.</t>
+          <t>Hasta el tenista veterano sigue puliendo su revés. En Jesús nunca dejamos de crecer.</t>
         </is>
       </c>
     </row>
@@ -43374,7 +43374,7 @@
       </c>
       <c r="D105" s="61" t="inlineStr">
         <is>
-          <t>Después de un set bajo el sol, la sed no se disimula; cuando el alma está seca, ese mismo anhelo nos lleva a buscar a Dios como el ciervo busca el agua.</t>
+          <t>Después de un set bajo el sol, la sed no se disimula. Como el ciervo busca el agua, el alma busca a Dios.</t>
         </is>
       </c>
     </row>
@@ -43394,7 +43394,7 @@
       </c>
       <c r="D106" s="61" t="inlineStr">
         <is>
-          <t>El jugador que se formó desde chico en el club de su barrio lleva raíces que se notan; la fe crece arraigada en Cristo, con tiempo.</t>
+          <t>El que se formó desde chico en su club lleva raíces que se notan. La fe crece arraigada en Cristo.</t>
         </is>
       </c>
     </row>
@@ -43414,7 +43414,7 @@
       </c>
       <c r="D107" s="61" t="inlineStr">
         <is>
-          <t>Un club serio le paga a tiempo a su gente, gane o pierda el domingo; una empresa que encomienda sus proyectos a Dios también se nota en lo cumplidora.</t>
+          <t>Un club serio paga a tiempo, gane o pierda. Encomendar el trabajo a Dios se nota en lo cumplidor.</t>
         </is>
       </c>
     </row>
@@ -43434,7 +43434,7 @@
       </c>
       <c r="D108" s="61" t="inlineStr">
         <is>
-          <t>En el remo, ningún remero puede adjudicarse solo el avance del bote; reconocer que la capacidad de producir viene de Dios nos libra del orgullo.</t>
+          <t>Ningún remero se adjudica solo el avance del bote. La capacidad de producir viene de Dios.</t>
         </is>
       </c>
     </row>
@@ -43454,7 +43454,7 @@
       </c>
       <c r="D109" s="61" t="inlineStr">
         <is>
-          <t>El buen árbitro se prepara toda la semana para noventa minutos que casi nadie le agradece; hacer bien tu trabajo, con constancia, suele abrir puertas.</t>
+          <t>El árbitro se prepara toda la semana para noventa minutos. El trabajo constante abre puertas.</t>
         </is>
       </c>
     </row>
@@ -43474,7 +43474,7 @@
       </c>
       <c r="D110" s="61" t="inlineStr">
         <is>
-          <t>Después del último pitazo, el equipo que dejó todo disfruta el vestuario con alegría; disfrutar el fruto de tu trabajo también es un regalo de Dios.</t>
+          <t>El equipo que dejó todo disfruta el vestuario. Disfrutar el fruto del trabajo es un regalo de Dios.</t>
         </is>
       </c>
     </row>
@@ -43494,7 +43494,7 @@
       </c>
       <c r="D111" s="61" t="inlineStr">
         <is>
-          <t>El boxeador confía en su esquina entre round y round; poner la confianza en Dios es saber quién te sostiene cuando la pelea se pone dura.</t>
+          <t>Entre round y round, el boxeador confía en su esquina. Confiar en Dios es saber quién te sostiene.</t>
         </is>
       </c>
     </row>
@@ -43514,7 +43514,7 @@
       </c>
       <c r="D112" s="61" t="inlineStr">
         <is>
-          <t>El pivote se lleva los golpes para abrirle espacio al compañero, aunque el gol lo grite otro; trabajar como para el Señor cambia el porqué y el cómo de lo que hacemos.</t>
+          <t>El pivote se lleva los golpes y el gol lo grita otro. Trabajar para el Señor cambia el porqué.</t>
         </is>
       </c>
     </row>
@@ -43534,7 +43534,7 @@
       </c>
       <c r="D113" s="61" t="inlineStr">
         <is>
-          <t>Mano a mano pasa el testimonio, y la carrera de postas necesita a todos. Por eso pedimos como el salmista: Señor, confirmá la obra de nuestras manos.</t>
+          <t>En la posta, el testimonio pasa de mano en mano. Señor, confirmá la obra de nuestras manos.</t>
         </is>
       </c>
     </row>
@@ -43554,7 +43554,7 @@
       </c>
       <c r="D114" s="61" t="inlineStr">
         <is>
-          <t>Nadie termina una maratón soñándola desde el sillón; como el río que corre se mantiene limpio, el cuerpo que se mueve un poco cada día se cuida mejor.</t>
+          <t>Nadie termina una maratón desde el sillón. El cuerpo que se mueve cada día se cuida mejor.</t>
         </is>
       </c>
     </row>
@@ -43574,7 +43574,7 @@
       </c>
       <c r="D115" s="61" t="inlineStr">
         <is>
-          <t>Pablo miraba a los atletas que entrenaban con disciplina por una corona que se marchita; nosotros también corremos con propósito, por algo que dura para siempre.</t>
+          <t>Los atletas entrenan por una corona que se marchita. Nosotros corremos por algo que dura para siempre.</t>
         </is>
       </c>
     </row>
@@ -43594,7 +43594,7 @@
       </c>
       <c r="D116" s="61" t="inlineStr">
         <is>
-          <t>Subida larga: el ciclista que controla su ritmo llega mejor que el que se desboca al principio. El dominio propio también se entrena, de a poco.</t>
+          <t>En la subida, el ciclista que controla su ritmo llega mejor. El dominio propio se entrena.</t>
         </is>
       </c>
     </row>
@@ -43614,7 +43614,7 @@
       </c>
       <c r="D117" s="61" t="inlineStr">
         <is>
-          <t>Ningún nadador compite con la ropa puesta: se saca lo que pesa para avanzar; correr con paciencia la carrera también es soltar lo que nos estorba.</t>
+          <t>Nadie nada con la ropa puesta. Soltá lo que pesa para correr con paciencia.</t>
         </is>
       </c>
     </row>
@@ -43634,7 +43634,7 @@
       </c>
       <c r="D118" s="61" t="inlineStr">
         <is>
-          <t>Para saltar al bloqueo una y otra vez hace falta fuerza en las piernas; el salmista reconocía que hasta esa fuerza viene de Dios.</t>
+          <t>Saltar al bloqueo una y otra vez pide piernas fuertes. Hasta esa fuerza viene de Dios.</t>
         </is>
       </c>
     </row>
@@ -43654,7 +43654,7 @@
       </c>
       <c r="D119" s="61" t="inlineStr">
         <is>
-          <t>Un partidito con amigos en la canchita del barrio ya es movimiento; desde el principio, Dios diseñó el cuerpo para la actividad, para labrar y cuidar.</t>
+          <t>Un partidito en la canchita del barrio ya es movimiento. Dios diseñó el cuerpo para la actividad.</t>
         </is>
       </c>
     </row>
@@ -43674,7 +43674,7 @@
       </c>
       <c r="D120" s="61" t="inlineStr">
         <is>
-          <t>Pensando en toda la temporada, el preparador físico cuida a sus jugadores. Cuidar tu cuerpo es cuidar un regalo.</t>
+          <t>El preparador físico piensa en toda la temporada. Cuidar tu cuerpo es cuidar un regalo.</t>
         </is>
       </c>
     </row>
@@ -43694,7 +43694,7 @@
       </c>
       <c r="D121" s="61" t="inlineStr">
         <is>
-          <t>Antes de que llegue el primer hincha, alguien ya marcó la cancha y colgó las redes; servir por amor muchas veces es trabajar donde no llegan las cámaras.</t>
+          <t>Antes del primer hincha, alguien ya marcó la cancha. Servir por amor es trabajar donde no hay cámaras.</t>
         </is>
       </c>
     </row>
@@ -43714,7 +43714,7 @@
       </c>
       <c r="D122" s="61" t="inlineStr">
         <is>
-          <t>El capitán de futsal muchas veces es el primero en volver a marcar. Jesús nos mostró que la grandeza está en servir, no en ser servido.</t>
+          <t>El capitán de futsal es el primero en volver a marcar. La grandeza está en servir.</t>
         </is>
       </c>
     </row>
@@ -43734,7 +43734,7 @@
       </c>
       <c r="D123" s="61" t="inlineStr">
         <is>
-          <t>En el básquet hay quien rebotea, quien asiste y quien tira de tres; cada uno recibió un don, y se activa cuando lo ponés al servicio del equipo.</t>
+          <t>En el básquet uno rebotea, otro asiste, otro tira. Cada don sirve cuando se pone al servicio del equipo.</t>
         </is>
       </c>
     </row>
@@ -43754,7 +43754,7 @@
       </c>
       <c r="D124" s="61" t="inlineStr">
         <is>
-          <t>Imaginá al técnico juntando los botines embarrados de sus jugadores después de la práctica; eso hizo el Maestro al lavar los pies: en el servicio no hay jerarquías.</t>
+          <t>Imaginá al técnico limpiando los botines de sus jugadores. Jesús lavó los pies: en el servicio no hay jerarquías.</t>
         </is>
       </c>
     </row>
@@ -43774,7 +43774,7 @@
       </c>
       <c r="D125" s="61" t="inlineStr">
         <is>
-          <t>El juez de línea corre toda la banda y casi nadie sabe su nombre. Servir sin aplausos es eso: que la mano izquierda no se entere, porque el Padre ve en lo secreto.</t>
+          <t>El juez de línea corre toda la banda y nadie sabe su nombre. El Padre ve en lo secreto.</t>
         </is>
       </c>
     </row>
@@ -43794,7 +43794,7 @@
       </c>
       <c r="D126" s="61" t="inlineStr">
         <is>
-          <t>El profe que se queda con el chico que casi no juega hace algo que Jesús no pasa por alto: lo que hacemos por el más pequeño, a Él se lo hacemos.</t>
+          <t>El profe que se queda con el chico que casi no juega lo hace para Jesús: lo hecho al más pequeño, a Él se lo hacemos.</t>
         </is>
       </c>
     </row>
@@ -43814,7 +43814,7 @@
       </c>
       <c r="D127" s="61" t="inlineStr">
         <is>
-          <t>Atado a un compañero no vidente, el atleta guía corre feliz si el otro llega. Hay más dicha en dar que en recibir.</t>
+          <t>El atleta guía corre feliz si su compañero no vidente llega. Hay más dicha en dar que en recibir.</t>
         </is>
       </c>
     </row>
@@ -43834,7 +43834,7 @@
       </c>
       <c r="D128" s="61" t="inlineStr">
         <is>
-          <t>Auto encajado en el barro: piloto y copiloto no discuten la largada, buscan la siguiente salida. Atribulados, pero no destruidos.</t>
+          <t>Auto encajado en el barro: piloto y copiloto buscan la salida. Atribulados, pero no destruidos.</t>
         </is>
       </c>
     </row>
@@ -43854,7 +43854,7 @@
       </c>
       <c r="D129" s="61" t="inlineStr">
         <is>
-          <t>El arquero que escucha silbidos de la tribuna y sigue atajando entiende a Nehemías: frente a la oposición, acordarse de Dios vence el temor y deja seguir construyendo.</t>
+          <t>El arquero sigue atajando entre silbidos. Frente a la oposición, acordarse de Dios vence el temor.</t>
         </is>
       </c>
     </row>
@@ -43874,7 +43874,7 @@
       </c>
       <c r="D130" s="61" t="inlineStr">
         <is>
-          <t>Mirá el tablero de ajedrez entero, sin creer que cada peón es una trampa. El buen líder está alerta y firme en la fe, sin vivir con sospecha.</t>
+          <t>Mirá el tablero entero sin ver trampas en cada peón. El buen líder está alerta, no con sospecha.</t>
         </is>
       </c>
     </row>
@@ -43894,7 +43894,7 @@
       </c>
       <c r="D131" s="61" t="inlineStr">
         <is>
-          <t>Los buenos entrenadores también perdieron partidos y aprendieron de eso; recordá a quienes te enseñaron la Palabra, mirá su ejemplo e imitá su fe.</t>
+          <t>Los buenos entrenadores también perdieron y aprendieron. Mirá el ejemplo de quienes te enseñaron e imitá su fe.</t>
         </is>
       </c>
     </row>
@@ -43914,7 +43914,7 @@
       </c>
       <c r="D132" s="61" t="inlineStr">
         <is>
-          <t>«Todo lo puedo» no es un grito para ganar un partido de tenis: Pablo hablaba de estar contento en la abundancia y en la escasez; Cristo sostiene también cuando perdemos.</t>
+          <t>«Todo lo puedo» no es para ganar un partido. Cristo sostiene en la abundancia y en la escasez, también al perder.</t>
         </is>
       </c>
     </row>
@@ -43934,7 +43934,7 @@
       </c>
       <c r="D133" s="61" t="inlineStr">
         <is>
-          <t>Hasta en las grandes vueltas ciclistas hay días de descanso, y nadie los llama cobardía; ser valiente también es parar a tiempo, sabiendo que Dios te acompaña.</t>
+          <t>Las grandes vueltas ciclistas tienen días de descanso. Parar a tiempo también es valentía.</t>
         </is>
       </c>
     </row>
@@ -43954,7 +43954,7 @@
       </c>
       <c r="D134" s="61" t="inlineStr">
         <is>
-          <t>Un set perdido no define el valor de un equipo de vóley; Dios obra en todo, también en los desafíos, aunque no lo entendamos todo.</t>
+          <t>Un set perdido no define a un equipo. Dios obra en todo, aunque no lo entendamos.</t>
         </is>
       </c>
     </row>
@@ -43974,7 +43974,7 @@
       </c>
       <c r="D135" s="61" t="inlineStr">
         <is>
-          <t>El buen profe de la escuelita de fútbol no empuja al chico a crecer de golpe: acompaña, corrige y espera. Los hijos son un regalo de Dios, no un trofeo propio.</t>
+          <t>El buen profe de la escuelita acompaña y espera. Los hijos son un regalo, no un trofeo.</t>
         </is>
       </c>
     </row>
@@ -43994,7 +43994,7 @@
       </c>
       <c r="D136" s="61" t="inlineStr">
         <is>
-          <t>Lo que un chico aprende de pequeño en la pileta, a flotar y a no tenerle miedo al agua, lo acompaña toda la vida; la formación temprana deja huella.</t>
+          <t>Lo que un chico aprende de pequeño en la pileta lo acompaña toda la vida. La formación temprana deja huella.</t>
         </is>
       </c>
     </row>
@@ -44014,7 +44014,7 @@
       </c>
       <c r="D137" s="61" t="inlineStr">
         <is>
-          <t>El buen entrenador de formativas es firme con la disciplina sin humillar a nadie; Pablo pide eso a los padres: criar sin provocar a ira, con firmeza y amor juntos.</t>
+          <t>El buen entrenador es firme sin humillar. Criar sin provocar a ira: firmeza y amor juntos.</t>
         </is>
       </c>
     </row>
@@ -44034,7 +44034,7 @@
       </c>
       <c r="D138" s="61" t="inlineStr">
         <is>
-          <t>El árbitro que cobra a tiempo evita que el partido se descontrole; corregir a los hijos a tiempo, con amor, no es crueldad: es cuidarlos.</t>
+          <t>El árbitro que cobra a tiempo evita el descontrol. Corregir a tiempo, con amor, es cuidar.</t>
         </is>
       </c>
     </row>
@@ -44054,7 +44054,7 @@
       </c>
       <c r="D139" s="61" t="inlineStr">
         <is>
-          <t>A andar en bici no se enseña con un discurso, sino caminando al lado, una tarde y otra; la fe también se enseña así, en lo de todos los días.</t>
+          <t>A andar en bici se enseña caminando al lado. La fe también se enseña en lo de todos los días.</t>
         </is>
       </c>
     </row>
@@ -44074,7 +44074,7 @@
       </c>
       <c r="D140" s="61" t="inlineStr">
         <is>
-          <t>Ninguna medalla se compara con ver a un hijo caminar en la verdad; para muchos padres esa es la alegría más profunda.</t>
+          <t>Ninguna medalla se compara con ver a un hijo caminar en la verdad.</t>
         </is>
       </c>
     </row>
@@ -44094,7 +44094,7 @@
       </c>
       <c r="D141" s="61" t="inlineStr">
         <is>
-          <t>Primer partido del nieto, y el abuelo le pasa mucho más que una camiseta. Criar con amor e integridad deja un legado de generación en generación.</t>
+          <t>El abuelo le pasa al nieto mucho más que una camiseta. El amor y la integridad dejan legado.</t>
         </is>
       </c>
     </row>
@@ -44114,7 +44114,7 @@
       </c>
       <c r="D142" s="61" t="inlineStr">
         <is>
-          <t>Una red de arco con un agujerito deja pasar la pelota igual que una rota; las pequeñas fugas de plata, si nadie las repara, también vacían el bolsillo.</t>
+          <t>Una red con un agujerito deja pasar la pelota igual. Las pequeñas fugas también vacían el bolsillo.</t>
         </is>
       </c>
     </row>
@@ -44134,7 +44134,7 @@
       </c>
       <c r="D143" s="61" t="inlineStr">
         <is>
-          <t>En el vóley nadie puede quedarse mirando cuando la pelota cae en su zona; quien puede trabajar, que trabaje: el esfuerzo propio va antes del ingreso.</t>
+          <t>En el vóley, nadie se queda mirando la pelota en su zona. El esfuerzo propio va antes del ingreso.</t>
         </is>
       </c>
     </row>
@@ -44154,7 +44154,7 @@
       </c>
       <c r="D144" s="61" t="inlineStr">
         <is>
-          <t>El fondista no gana metros con un sprint de un día, sino con kilómetros constantes; la mano diligente suele abrir caminos que la desidia cierra.</t>
+          <t>El fondista gana metros con kilómetros constantes. La mano diligente abre caminos.</t>
         </is>
       </c>
     </row>
@@ -44174,7 +44174,7 @@
       </c>
       <c r="D145" s="61" t="inlineStr">
         <is>
-          <t>Estar contra las cuerdas por una deuda quita libertad, como al boxeador acorralado; si hoy estás ahí, no estás solo: pedí consejo y avanzá de a un paso.</t>
+          <t>Una deuda te deja contra las cuerdas, como al boxeador. No estás solo: pedí consejo y avanzá de a un paso.</t>
         </is>
       </c>
     </row>
@@ -44194,7 +44194,7 @@
       </c>
       <c r="D146" s="61" t="inlineStr">
         <is>
-          <t>Pocas cosas sostienen tanto un partido largo de tenis como el punto chico, el que parece no importar. La fidelidad en lo poco forma el carácter para lo mucho.</t>
+          <t>El punto chico sostiene un partido largo. La fidelidad en lo poco forma para lo mucho.</t>
         </is>
       </c>
     </row>
@@ -44214,7 +44214,7 @@
       </c>
       <c r="D147" s="61" t="inlineStr">
         <is>
-          <t>El equipo de futsal que corre todo el partido pero no cierra la defensa recibe goles por el mismo hueco. Antes de trabajar más, mirá por dónde se escapa tu plata.</t>
+          <t>El que no cierra la defensa recibe goles por el mismo hueco. Antes de trabajar más, mirá por dónde se escapa tu plata.</t>
         </is>
       </c>
     </row>
@@ -44234,7 +44234,7 @@
       </c>
       <c r="D148" s="61" t="inlineStr">
         <is>
-          <t>Repartir buenos pases no empobrece a nadie: hace crecer a todo el equipo. Después de ordenar lo que entra y sale, queda claro que la generosidad enriquece la vida.</t>
+          <t>Repartir buenos pases hace crecer a todo el equipo. La generosidad enriquece la vida.</t>
         </is>
       </c>
     </row>
@@ -44254,7 +44254,7 @@
       </c>
       <c r="D149" s="61" t="inlineStr">
         <is>
-          <t>El jugador que se queda practicando tiros libres no pierde tiempo, lo invierte; como el carpintero que se detiene a afilar la sierra, capacitarte también es estar atento y firme.</t>
+          <t>El que se queda practicando tiros libres invierte tiempo. Capacitarte es afilar la sierra.</t>
         </is>
       </c>
     </row>
@@ -44274,7 +44274,7 @@
       </c>
       <c r="D150" s="61" t="inlineStr">
         <is>
-          <t>El suplente que está siempre listo entra y responde con lo que entrenó; estar preparados es también saber explicar, con respeto, la esperanza que tenemos en Cristo.</t>
+          <t>El suplente siempre listo responde con lo que entrenó. Estemos listos para explicar nuestra esperanza.</t>
         </is>
       </c>
     </row>
@@ -44294,7 +44294,7 @@
       </c>
       <c r="D151" s="61" t="inlineStr">
         <is>
-          <t>Último tramo de la regata: el remero pone toda su fuerza en cada palada. Lo que tengas hoy entre manos, hacelo con todo, sin mediocridad.</t>
+          <t>En el último tramo, el remero pone todo en cada palada. Lo que hagas hoy, hacelo con todo.</t>
         </is>
       </c>
     </row>
@@ -44314,7 +44314,7 @@
       </c>
       <c r="D152" s="61" t="inlineStr">
         <is>
-          <t>El ajedrecista estudia partidas, las juega y después enseña a los nuevos del club; Esdras hizo lo mismo con la Palabra: estudiarla, vivirla y enseñarla.</t>
+          <t>El ajedrecista estudia, juega y enseña a los nuevos. Como Esdras con la Palabra.</t>
         </is>
       </c>
     </row>
@@ -44334,7 +44334,7 @@
       </c>
       <c r="D153" s="61" t="inlineStr">
         <is>
-          <t>Los abdominales que nadie ve en la pretemporada se notan en el segundo tiempo; servir de corazón es ser fiel aunque nadie esté mirando.</t>
+          <t>Los abdominales de pretemporada se notan en el segundo tiempo. Servir de corazón es ser fiel sin testigos.</t>
         </is>
       </c>
     </row>
@@ -44354,7 +44354,7 @@
       </c>
       <c r="D154" s="61" t="inlineStr">
         <is>
-          <t>El nadador que respeta cada viraje, aunque nadie lo controle, se gana algo más valioso que un récord: la confianza; Daniel se distinguió por esa integridad constante.</t>
+          <t>El nadador que respeta cada viraje sin control gana confianza. Como Daniel: integridad constante.</t>
         </is>
       </c>
     </row>
@@ -44374,7 +44374,7 @@
       </c>
       <c r="D155" s="61" t="inlineStr">
         <is>
-          <t>Uno corta el viento para que el otro respire: así se turnan en el pelotón. Crecer y ayudar a crecer, animándonos unos a otros: eso nos llevamos.</t>
+          <t>En el pelotón, uno corta el viento para que el otro respire. Crecer es ayudar a crecer.</t>
         </is>
       </c>
     </row>
@@ -44394,7 +44394,7 @@
       </c>
       <c r="D156" s="61" t="inlineStr">
         <is>
-          <t>Muchos empezaron a jugar con una pelota de trapo en un baldío; la viuda tenía apenas una vasija de aceite, y Dios usó lo poco que había en su casa.</t>
+          <t>Muchos empezaron con una pelota de trapo. Dios usó la vasija de aceite que la viuda tenía en casa.</t>
         </is>
       </c>
     </row>
@@ -44414,7 +44414,7 @@
       </c>
       <c r="D157" s="61" t="inlineStr">
         <is>
-          <t>Mientras el auto avanza, el copiloto de rally va leyendo el camino que viene. Emprender puede dar miedo, pero Dios va delante tuyo y no te abandona.</t>
+          <t>El copiloto va leyendo el camino que viene. Emprender da miedo, pero Dios va delante tuyo.</t>
         </is>
       </c>
     </row>
@@ -44434,7 +44434,7 @@
       </c>
       <c r="D158" s="61" t="inlineStr">
         <is>
-          <t>Muchos jugadores de futsal empezaron en una canchita de cemento del barrio, entrenando temprano. Cada mañana es un comienzo nuevo: confiá en Dios y pedile que te muestre el camino.</t>
+          <t>Muchos cracks empezaron en una canchita de cemento, entrenando temprano. Cada mañana, confiá en Dios y pedile el camino.</t>
         </is>
       </c>
     </row>
@@ -44454,7 +44454,7 @@
       </c>
       <c r="D159" s="61" t="inlineStr">
         <is>
-          <t>El sacador no sabe si su saque va a ser punto, pero saca igual, con su mejor técnica; sembrá en la mañana y en la tarde, aunque no sepas qué va a dar fruto.</t>
+          <t>El sacador no sabe si será punto, pero saca igual. Sembrá aunque no sepas qué va a dar fruto.</t>
         </is>
       </c>
     </row>
@@ -44474,7 +44474,7 @@
       </c>
       <c r="D160" s="61" t="inlineStr">
         <is>
-          <t>Antes de cobrar, el buen árbitro mira bien la jugada y no se deja llevar por el griterío; antes de decidir, examiná con calma: no todo lo que se oye es cierto.</t>
+          <t>El buen árbitro mira bien antes de cobrar. No todo lo que se oye es cierto.</t>
         </is>
       </c>
     </row>
@@ -44494,7 +44494,7 @@
       </c>
       <c r="D161" s="61" t="inlineStr">
         <is>
-          <t>Pase corto bien hecho, una y otra vez: eso sostiene a un equipo de handball. Ser fiel en lo poco también es parte de emprender, y Jesús celebra esa fidelidad.</t>
+          <t>El pase corto bien hecho sostiene al equipo. Jesús celebra la fidelidad en lo poco.</t>
         </is>
       </c>
     </row>
@@ -44514,7 +44514,7 @@
       </c>
       <c r="D162" s="61" t="inlineStr">
         <is>
-          <t>Las medallas se oxidan y los trofeos juntan polvo en la vitrina. Emprendé con fe y con cuidado, sabiendo que la vida verdadera la da Jesús.</t>
+          <t>Las medallas se oxidan en la vitrina. Emprendé con fe: la vida verdadera la da Jesús.</t>
         </is>
       </c>
     </row>
@@ -44534,7 +44534,7 @@
       </c>
       <c r="D163" s="61" t="inlineStr">
         <is>
-          <t>Durante la concentración, el cuerpo técnico cuida lo que come el plantel. Desde el principio Dios proveyó plantas y semillas: lo que comemos también es parte de su cuidado.</t>
+          <t>En la concentración se cuida lo que come el plantel. Lo que comemos también es parte del cuidado de Dios.</t>
         </is>
       </c>
     </row>
@@ -44554,7 +44554,7 @@
       </c>
       <c r="D164" s="61" t="inlineStr">
         <is>
-          <t>Daniel pidió diez días de prueba con comida sencilla, como el atleta que ajusta lo que come y mira cómo responde; una decisión en la mesa también puede ser un acto de fe.</t>
+          <t>Daniel probó diez días con comida sencilla, como el atleta que ajusta su dieta. La mesa también puede ser un acto de fe.</t>
         </is>
       </c>
     </row>
@@ -44574,7 +44574,7 @@
       </c>
       <c r="D165" s="61" t="inlineStr">
         <is>
-          <t>En la maratón, tomar demasiado de golpe hace tanto daño como no tomar nada; hasta lo bueno, en exceso, cae mal: la medida es sabiduría práctica.</t>
+          <t>En la maratón, tomar de más hace tanto daño como no tomar. Hasta lo bueno pide medida.</t>
         </is>
       </c>
     </row>
@@ -44594,7 +44594,7 @@
       </c>
       <c r="D166" s="61" t="inlineStr">
         <is>
-          <t>El equipo de vóley que comparte la merienda después del entrenamiento también vive algo valioso; comer y beber, hasta lo más cotidiano, puede ser para la gloria de Dios.</t>
+          <t>La merienda compartida después del entrenamiento también vale. Hasta comer puede ser para la gloria de Dios.</t>
         </is>
       </c>
     </row>
@@ -44614,7 +44614,7 @@
       </c>
       <c r="D167" s="61" t="inlineStr">
         <is>
-          <t>El ciclista que no come en la etapa se queda sin piernas, y el que come de más pedalea pesado; ni exceso ni descuido: la medida cuida el cuerpo y el bolsillo.</t>
+          <t>El ciclista que no come se queda sin piernas; el que come de más, pedalea pesado. La medida cuida el cuerpo.</t>
         </is>
       </c>
     </row>
@@ -44634,7 +44634,7 @@
       </c>
       <c r="D168" s="61" t="inlineStr">
         <is>
-          <t>El tereré y la chipa compartidos en la tribuna también son regalos; el salmista reconocía que el pan que sostiene la vida sale de la mano de Dios.</t>
+          <t>El tereré y la chipa en la tribuna también son regalos. El pan de cada día sale de la mano de Dios.</t>
         </is>
       </c>
     </row>
@@ -44654,7 +44654,7 @@
       </c>
       <c r="D169" s="61" t="inlineStr">
         <is>
-          <t>Un mal día de comidas no hace que el basquetbolista se castigue: ajusta y sigue. Comer con gratitud y medida es cuidado, no culpa.</t>
+          <t>Un mal día de comidas no hace que el atleta se castigue: ajusta y sigue. Comer con medida es cuidado, no culpa.</t>
         </is>
       </c>
     </row>
@@ -44674,7 +44674,7 @@
       </c>
       <c r="D170" s="61" t="inlineStr">
         <is>
-          <t>Un buen técnico de formativas no se conforma con que el chico sepa el reglamento: lo acompaña hasta que juega; así nos mandó Jesús hacer discípulos, prometiendo estar con nosotros.</t>
+          <t>El buen técnico acompaña al chico hasta que juega. Así nos mandó Jesús a hacer discípulos.</t>
         </is>
       </c>
     </row>
@@ -44694,7 +44694,7 @@
       </c>
       <c r="D171" s="61" t="inlineStr">
         <is>
-          <t>Testimonio que no se entrega se pierde, aunque hayas corrido bien tu tramo de la posta. La fe también se pasa de mano en mano, a otros que la sigan llevando.</t>
+          <t>El testimonio que no se entrega se pierde. La fe se pasa de mano en mano.</t>
         </is>
       </c>
     </row>
@@ -44714,7 +44714,7 @@
       </c>
       <c r="D172" s="61" t="inlineStr">
         <is>
-          <t>Como el agua quieta de la pileta refleja al nadador antes de tirarse, el corazón se refleja en el del otro; discipular es mostrarse tal cual uno es.</t>
+          <t>El agua quieta refleja al nadador. Discipular es mostrarse tal cual uno es.</t>
         </is>
       </c>
     </row>
@@ -44734,7 +44734,7 @@
       </c>
       <c r="D173" s="61" t="inlineStr">
         <is>
-          <t>Los chicos del futsal copian hasta cómo festeja su referente; por eso Pablo decía: imítenme como yo imito a Cristo. El ejemplo enseña más que el discurso.</t>
+          <t>Los chicos copian hasta cómo festeja su referente. El ejemplo enseña más que el discurso.</t>
         </is>
       </c>
     </row>
@@ -44754,7 +44754,7 @@
       </c>
       <c r="D174" s="61" t="inlineStr">
         <is>
-          <t>El ajedrecista que conoce bien los principios juega con libertad, sin miedo a cada movimiento; permanecer en la Palabra de Jesús nos hace conocer la verdad que libera.</t>
+          <t>El ajedrecista que conoce los principios juega con libertad. La verdad de Jesús nos hace libres.</t>
         </is>
       </c>
     </row>
@@ -44774,7 +44774,7 @@
       </c>
       <c r="D175" s="61" t="inlineStr">
         <is>
-          <t>Mirar videos del saque no alcanza: hay que salir a la cancha de tenis y practicarlo. Lo que aprendiste, ponelo en práctica, y la paz de Dios te acompaña.</t>
+          <t>Mirar videos del saque no alcanza: hay que practicarlo. Lo que aprendiste, ponelo en práctica.</t>
         </is>
       </c>
     </row>
@@ -44794,7 +44794,7 @@
       </c>
       <c r="D176" s="61" t="inlineStr">
         <is>
-          <t>Cada bote que avanza lleva algo del viejo entrenador de remo que formó a sus remeros. Invertir en otros deja una huella que dura.</t>
+          <t>Cada bote lleva algo del viejo entrenador que formó a sus remeros. Invertir en otros deja huella.</t>
         </is>
       </c>
     </row>
@@ -44814,7 +44814,7 @@
       </c>
       <c r="D177" s="61" t="inlineStr">
         <is>
-          <t>Como el entrenador que, en vez de presionar a su jugador, lo rodeó de confianza, un equipo unido resiste más: el cordón de tres dobleces no se rompe fácil.</t>
+          <t>Un equipo unido resiste más. El cordón de tres dobleces no se rompe fácil.</t>
         </is>
       </c>
     </row>
@@ -44834,7 +44834,7 @@
       </c>
       <c r="D178" s="61" t="inlineStr">
         <is>
-          <t>El buen capitán de vóley anima a su equipo sin engaños ni gritos que humillan. Motivar sin manipular es buscar agradar a Dios, no el aplauso de la tribuna.</t>
+          <t>El buen capitán anima sin engaños ni gritos que humillan. Motivar es buscar agradar a Dios, no a la tribuna.</t>
         </is>
       </c>
     </row>
@@ -44854,7 +44854,7 @@
       </c>
       <c r="D179" s="61" t="inlineStr">
         <is>
-          <t>En el básquet, el base paciente que espera a que todos se acomoden arma mejores jugadas; la unidad del equipo se cuida con paciencia y esfuerzo.</t>
+          <t>El base paciente espera que todos se acomoden. La unidad se cuida con paciencia.</t>
         </is>
       </c>
     </row>
@@ -44874,7 +44874,7 @@
       </c>
       <c r="D180" s="61" t="inlineStr">
         <is>
-          <t>Un buen técnico escucha a sus ayudantes, al preparador físico y al médico antes de decidir; en los muchos consejeros hay seguridad, y decidir solo es un riesgo.</t>
+          <t>El buen técnico escucha a su cuerpo técnico antes de decidir. En los muchos consejeros hay seguridad.</t>
         </is>
       </c>
     </row>
@@ -44894,7 +44894,7 @@
       </c>
       <c r="D181" s="61" t="inlineStr">
         <is>
-          <t>¿Viste cuando se pincha una goma en pleno rally? Piloto y copiloto la cambian juntos. En un equipo nadie debería cargar solo: eso es cumplir la ley de Cristo.</t>
+          <t>Pinchazo en pleno rally: piloto y copiloto cambian la goma juntos. Llevar las cargas unos de otros.</t>
         </is>
       </c>
     </row>
@@ -44914,7 +44914,7 @@
       </c>
       <c r="D182" s="61" t="inlineStr">
         <is>
-          <t>La hinchada que alienta cuando el equipo va abajo no lo hace por casualidad, lo hace a propósito; considerémonos unos a otros para estimularnos al amor y a las buenas obras.</t>
+          <t>La hinchada alienta cuando el equipo va abajo, a propósito. Animémonos al amor y a las buenas obras.</t>
         </is>
       </c>
     </row>
@@ -44934,7 +44934,7 @@
       </c>
       <c r="D183" s="61" t="inlineStr">
         <is>
-          <t>El que da la asistencia en el futsal festeja el gol como propio. El equipo se sostiene cuando cada uno busca también el bien del otro.</t>
+          <t>El que da la asistencia festeja el gol como propio. El equipo se sostiene buscando el bien del otro.</t>
         </is>
       </c>
     </row>
@@ -44954,7 +44954,7 @@
       </c>
       <c r="D184" s="61" t="inlineStr">
         <is>
-          <t>Lo que un equipo vive en el vestuario se nota en la cancha; lo que una familia vive puertas adentro sale al barrio, como sal y luz que no se esconden.</t>
+          <t>Lo que se vive en el vestuario se nota en la cancha. Lo que vive una familia sale al barrio, como sal y luz.</t>
         </is>
       </c>
     </row>
@@ -44974,7 +44974,7 @@
       </c>
       <c r="D185" s="61" t="inlineStr">
         <is>
-          <t>La hinchada que cuida su estadio disfruta mejor cada partido; buscar el bien de tu ciudad también es cuidar la casa donde vive tu familia.</t>
+          <t>La hinchada que cuida su estadio disfruta mejor el partido. Buscar el bien de tu ciudad es cuidar tu casa.</t>
         </is>
       </c>
     </row>
@@ -44994,7 +44994,7 @@
       </c>
       <c r="D186" s="61" t="inlineStr">
         <is>
-          <t>Ningún partido se juega sin reglas ni sin árbitro; respetar la autoridad y cumplir tu parte también es jugar limpio como familia dentro de la sociedad.</t>
+          <t>Ningún partido se juega sin reglas. Respetar la autoridad también es jugar limpio.</t>
         </is>
       </c>
     </row>
@@ -45014,7 +45014,7 @@
       </c>
       <c r="D187" s="61" t="inlineStr">
         <is>
-          <t>El tenista que canta con honestidad una pelota dudosa muestra su carácter; hacer justicia, amar la misericordia y caminar humilde se juega en cada punto.</t>
+          <t>El tenista que canta con honestidad una pelota dudosa muestra su carácter. Justicia, misericordia y humildad, punto a punto.</t>
         </is>
       </c>
     </row>
@@ -45034,7 +45034,7 @@
       </c>
       <c r="D188" s="61" t="inlineStr">
         <is>
-          <t>El entrenador de inferiores siembra hoy el juego limpio que mañana se ve en primera; la justicia que se aprende en casa también engrandece a una nación.</t>
+          <t>Lo que se siembra en inferiores se ve en primera. La justicia aprendida en casa engrandece a una nación.</t>
         </is>
       </c>
     </row>
@@ -45054,7 +45054,7 @@
       </c>
       <c r="D189" s="61" t="inlineStr">
         <is>
-          <t>En el futsal el pase va al que está libre, no solo al amigo; hacer el bien a todos empieza por mirar más allá de tu propio círculo.</t>
+          <t>En el futsal, el pase va al que está libre, no solo al amigo. Hacer el bien a todos es mirar más allá de tu círculo.</t>
         </is>
       </c>
     </row>
@@ -45074,7 +45074,7 @@
       </c>
       <c r="D190" s="61" t="inlineStr">
         <is>
-          <t>Un segundo antes de cada saque, el equipo de vóley se junta. Orar por quienes nos gobiernan es ese momento que une a la familia con su país.</t>
+          <t>Antes de cada saque, el equipo de vóley se junta. Orar por quienes gobiernan une a la familia con su país.</t>
         </is>
       </c>
     </row>
@@ -45094,7 +45094,7 @@
       </c>
       <c r="D191" s="61" t="inlineStr">
         <is>
-          <t>El entrenador no le da a todos la misma posición, pero a cada uno le confía algo; lo que Dios puso en tus manos es para administrarlo con propósito.</t>
+          <t>El técnico confía a cada jugador algo distinto. Lo que Dios puso en tus manos es para administrarlo bien.</t>
         </is>
       </c>
     </row>
@@ -45114,7 +45114,7 @@
       </c>
       <c r="D192" s="61" t="inlineStr">
         <is>
-          <t>El suplente de básquet que da todo en sus dos minutos en cancha muestra su corazón; Dios celebra la fidelidad en lo poco, no solo el resultado.</t>
+          <t>El suplente que da todo en dos minutos muestra su corazón. Dios celebra la fidelidad en lo poco.</t>
         </is>
       </c>
     </row>
@@ -45134,7 +45134,7 @@
       </c>
       <c r="D193" s="61" t="inlineStr">
         <is>
-          <t>El maratonista no ve la meta en el primer kilómetro, pero corre con paciencia; sembrar con sabiduría también pide esperar sin ver todavía la cosecha.</t>
+          <t>El maratonista no ve la meta en el primer kilómetro. Sembrar con sabiduría pide paciencia.</t>
         </is>
       </c>
     </row>
@@ -45154,7 +45154,7 @@
       </c>
       <c r="D194" s="61" t="inlineStr">
         <is>
-          <t>Quien repasa sus partidas de ajedrez y acepta la corrección aprende más que el que solo mueve rápido. La sabiduría empieza reconociendo a Dios con reverencia.</t>
+          <t>El ajedrecista que acepta la corrección aprende más. La sabiduría empieza reverenciando a Dios.</t>
         </is>
       </c>
     </row>
@@ -45174,7 +45174,7 @@
       </c>
       <c r="D195" s="61" t="inlineStr">
         <is>
-          <t>Caer a la lona no siempre es el final de la pelea. El justo cae y se vuelve a levantar, porque un tropiezo no define toda tu historia.</t>
+          <t>Caer a la lona no siempre es el final. El justo cae y se vuelve a levantar.</t>
         </is>
       </c>
     </row>
@@ -45194,7 +45194,7 @@
       </c>
       <c r="D196" s="61" t="inlineStr">
         <is>
-          <t>Las copas juntan polvo en la vitrina del club; mirá bien dónde ponés tu corazón, porque el tesoro que dura de verdad está en las manos de Dios.</t>
+          <t>Las copas juntan polvo en la vitrina. El tesoro que dura está en las manos de Dios.</t>
         </is>
       </c>
     </row>
@@ -45214,7 +45214,7 @@
       </c>
       <c r="D197" s="61" t="inlineStr">
         <is>
-          <t>En el remo, el que aprendió a leer el río sabe cuándo apurar y cuándo esperar; madurar es aprender, con Dios, a decidir bien qué hacer con lo que tenés.</t>
+          <t>El remero que lee el río sabe cuándo apurar y cuándo esperar. Madurar es decidir bien, con Dios.</t>
         </is>
       </c>
     </row>
@@ -45234,7 +45234,7 @@
       </c>
       <c r="D198" s="61" t="inlineStr">
         <is>
-          <t>Antes de soltar la flecha, el arquero necesita saber hacia dónde apunta. Y mientras apuntás tus metas, acordate de que Dios empezó la obra en vos y Él la va a completar.</t>
+          <t>El arquero necesita saber adónde apunta. Y Dios, que empezó la obra en vos, la va a completar.</t>
         </is>
       </c>
     </row>
@@ -45254,7 +45254,7 @@
       </c>
       <c r="D199" s="61" t="inlineStr">
         <is>
-          <t>El corredor que mira para atrás pierde el ritmo; olvidá lo que quedó atrás y seguí hacia la meta, que el pasado no tiene por qué frenarte.</t>
+          <t>El corredor que mira atrás pierde el ritmo. Olvidá lo que quedó atrás y seguí hacia la meta.</t>
         </is>
       </c>
     </row>
@@ -45274,7 +45274,7 @@
       </c>
       <c r="D200" s="61" t="inlineStr">
         <is>
-          <t>Antes del partido de handball, el entrenador dibuja la jugada en la pizarra para que todos la vean clara; escribí tu meta y vas a saber mejor cómo ir tras ella.</t>
+          <t>El técnico dibuja la jugada en la pizarra para que todos la vean. Escribí tu meta.</t>
         </is>
       </c>
     </row>
@@ -45294,7 +45294,7 @@
       </c>
       <c r="D201" s="61" t="inlineStr">
         <is>
-          <t>El delantero que pide la pelota, busca el espacio y no deja de moverse muestra hambre; con Dios es parecido: pedí, buscá y llamá con perseverancia y confianza.</t>
+          <t>El delantero pide la pelota y busca el espacio. Con Dios: pedí, buscá y llamá con confianza.</t>
         </is>
       </c>
     </row>
@@ -45314,7 +45314,7 @@
       </c>
       <c r="D202" s="61" t="inlineStr">
         <is>
-          <t>Kilómetro final de la subida más dura: el ciclista no se baja, sigue pedaleando con paciencia. Gozate en la esperanza, aguantá en la prueba y seguí constante en la oración.</t>
+          <t>En el kilómetro final de la subida, el ciclista no se baja. Constantes en la oración, firmes en la prueba.</t>
         </is>
       </c>
     </row>
@@ -45334,7 +45334,7 @@
       </c>
       <c r="D203" s="61" t="inlineStr">
         <is>
-          <t>Tramo terminado: el copiloto de rally revisa sus notas antes de encarar el siguiente. Examinar el camino, buscar al Señor y volver a él: así se corrige el rumbo.</t>
+          <t>El copiloto revisa sus notas antes del siguiente tramo. Examinar el camino y volver a Dios corrige el rumbo.</t>
         </is>
       </c>
     </row>
@@ -45354,7 +45354,7 @@
       </c>
       <c r="D204" s="61" t="inlineStr">
         <is>
-          <t>El nadador planifica cada largo, pero no controla el agua; hacé tus planes con ganas y con humildad, diciendo: si el Señor quiere, haremos esto o aquello.</t>
+          <t>El nadador planifica cada largo, pero no controla el agua. Planificá diciendo: si el Señor quiere.</t>
         </is>
       </c>
     </row>
@@ -45374,7 +45374,7 @@
       </c>
       <c r="D205" s="61" t="inlineStr">
         <is>
-          <t>El árbitro que cobra parejo para los dos equipos se gana el respeto de todos; en el comercio pasa igual: la balanza justa también le importa a Dios.</t>
+          <t>El árbitro que cobra parejo se gana el respeto. La balanza justa también le importa a Dios.</t>
         </is>
       </c>
     </row>
@@ -45394,7 +45394,7 @@
       </c>
       <c r="D206" s="61" t="inlineStr">
         <is>
-          <t>Antes de una pelea de boxeo, el peso se controla en una balanza que no puede mentir; en tu negocio, la pesa cabal agrada a Dios y la trampa le desagrada.</t>
+          <t>En el boxeo, la balanza no puede mentir. En tu negocio, la pesa cabal agrada a Dios.</t>
         </is>
       </c>
     </row>
@@ -45414,7 +45414,7 @@
       </c>
       <c r="D207" s="61" t="inlineStr">
         <is>
-          <t>Una pista de atletismo tiene que medir lo que dice, ni un metro menos; el peso y la medida justos en tu negocio reflejan el carácter de Dios.</t>
+          <t>Una pista mide lo que dice, ni un metro menos. La medida justa refleja el carácter de Dios.</t>
         </is>
       </c>
     </row>
@@ -45434,7 +45434,7 @@
       </c>
       <c r="D208" s="61" t="inlineStr">
         <is>
-          <t>El torneo de futsal del barrio se sostiene con el kiosco y el vecino que pone la red; comprar en tu zona y negociar con honestidad también es jugar en equipo.</t>
+          <t>El torneo del barrio se sostiene con el kiosco de la esquina. Comprar en tu zona también es jugar en equipo.</t>
         </is>
       </c>
     </row>
@@ -45454,7 +45454,7 @@
       </c>
       <c r="D209" s="61" t="inlineStr">
         <is>
-          <t>En el vóley, si alguien grita «mía» y no va, la pelota cae; decirle la verdad a tu compañero sostiene al equipo, porque somos parte del mismo cuerpo.</t>
+          <t>En el vóley, si alguien grita «mía» y no va, la pelota cae. Decir la verdad sostiene al equipo.</t>
         </is>
       </c>
     </row>
@@ -45474,7 +45474,7 @@
       </c>
       <c r="D210" s="61" t="inlineStr">
         <is>
-          <t>El utilero casi no habla, pero cada camiseta lista y cada botín limpio dicen cuánto le importa el equipo; el amor se demuestra con hechos y con un corazón sincero.</t>
+          <t>El utilero casi no habla, pero cada camiseta lista lo dice todo. El amor se demuestra con hechos.</t>
         </is>
       </c>
     </row>
@@ -45494,7 +45494,7 @@
       </c>
       <c r="D211" s="61" t="inlineStr">
         <is>
-          <t>Como el equipo de básquet que suma sus puntos jugando limpio, el trabajo honesto de tus manos tiene valor; producir y vender con integridad también honra a Dios.</t>
+          <t>Un equipo que suma jugando limpio vale más. Producir y vender con integridad honra a Dios.</t>
         </is>
       </c>
     </row>
@@ -45514,7 +45514,7 @@
       </c>
       <c r="D212" s="61" t="inlineStr">
         <is>
-          <t>La noche antes de una final, el mejor entrenamiento es dormir; podés acostarte en paz, porque no sos vos quien sostiene todo: es Dios quien te cuida.</t>
+          <t>La noche antes de la final, lo mejor es dormir. Acostate en paz: Dios te cuida.</t>
         </is>
       </c>
     </row>
@@ -45534,7 +45534,7 @@
       </c>
       <c r="D213" s="61" t="inlineStr">
         <is>
-          <t>Todo preparador físico planifica días de recuperación, porque sin descanso no hay temporada; Dios mismo nos dio un ritmo de trabajo y descanso.</t>
+          <t>Todo preparador físico planifica la recuperación. Dios nos dio un ritmo de trabajo y descanso.</t>
         </is>
       </c>
     </row>
@@ -45554,7 +45554,7 @@
       </c>
       <c r="D214" s="61" t="inlineStr">
         <is>
-          <t>Después de un partido difícil cuesta dormir, dando vueltas a cada punto; aun en esas noches, Dios te cuida y te invita a descansar en paz.</t>
+          <t>Después de un partido difícil cuesta dormir. Aun en esas noches, Dios te invita a descansar.</t>
         </is>
       </c>
     </row>
@@ -45574,7 +45574,7 @@
       </c>
       <c r="D215" s="61" t="inlineStr">
         <is>
-          <t>Tiempo muerto: el entrenador de básquet lo pide para que el equipo respire. Jesús también invitó a los suyos a descansar aparte; parar un rato no es debilidad, es sabiduría.</t>
+          <t>El tiempo muerto es para que el equipo respire. Jesús invitó a los suyos a descansar aparte.</t>
         </is>
       </c>
     </row>
@@ -45594,7 +45594,7 @@
       </c>
       <c r="D216" s="61" t="inlineStr">
         <is>
-          <t>El nadador que entrena hasta el agotamiento no siempre nada mejor; el afán sin descanso no asegura resultados, y el sueño es un regalo que Dios da a los que ama.</t>
+          <t>Entrenar hasta el agotamiento no siempre mejora. El sueño es un regalo de Dios.</t>
         </is>
       </c>
     </row>
@@ -45614,7 +45614,7 @@
       </c>
       <c r="D217" s="61" t="inlineStr">
         <is>
-          <t>Al cruzar la meta de una maratón, alguien te alcanza agua y una manta; Jesús invita a los cansados a venir a Él, y en su presencia la carga se alivia.</t>
+          <t>Al cruzar la meta, alguien te alcanza agua y una manta. Jesús invita a los cansados a venir a Él.</t>
         </is>
       </c>
     </row>
@@ -45634,7 +45634,7 @@
       </c>
       <c r="D218" s="61" t="inlineStr">
         <is>
-          <t>Hay un instante, entre palada y palada, en que el bote de remo se desliza solo. Descansar no es solo dejar de hacer, es saber que Dios va con vos.</t>
+          <t>Entre palada y palada, el bote se desliza solo. Descansar es saber que Dios va con vos.</t>
         </is>
       </c>
     </row>
@@ -45654,7 +45654,7 @@
       </c>
       <c r="D219" s="61" t="inlineStr">
         <is>
-          <t>Un buen arquero habla con su defensa todo el partido, no solo cuando hay peligro; así es orar sin cesar: hablar con Dios siempre, con gozo y gratitud.</t>
+          <t>El buen arquero habla con su defensa todo el partido. Orar sin cesar es hablar con Dios siempre.</t>
         </is>
       </c>
     </row>
@@ -45674,7 +45674,7 @@
       </c>
       <c r="D220" s="61" t="inlineStr">
         <is>
-          <t>En una carrera de ciclismo, el corredor que pide ayuda por radio recibe respuesta de su equipo; clamá a Dios, que escucha y puede mostrarte cosas que todavía no conocés.</t>
+          <t>El ciclista pide ayuda por radio y su equipo responde. Clamá a Dios, que escucha.</t>
         </is>
       </c>
     </row>
@@ -45694,7 +45694,7 @@
       </c>
       <c r="D221" s="61" t="inlineStr">
         <is>
-          <t>Lo que el atleta entrena a solas, sin tribuna ni cámaras, es lo que más lo forma; la oración en lo secreto también profundiza tu relación con Dios.</t>
+          <t>Lo que el atleta entrena a solas es lo que más lo forma. La oración en lo secreto también.</t>
         </is>
       </c>
     </row>
@@ -45714,7 +45714,7 @@
       </c>
       <c r="D222" s="61" t="inlineStr">
         <is>
-          <t>El jugador que conoce a su técnico entiende lo que le pide antes de que lo diga; acercate a Dios con confianza y pedí buscando lo que a Él le agrada.</t>
+          <t>El jugador que conoce a su técnico entiende lo que pide. Acercate a Dios con confianza.</t>
         </is>
       </c>
     </row>
@@ -45734,7 +45734,7 @@
       </c>
       <c r="D223" s="61" t="inlineStr">
         <is>
-          <t>Entre round y round, el boxeador vuelve a su rincón y dice cómo está de verdad; con Dios podés hacer lo mismo: derramá tu corazón, que Él es refugio seguro.</t>
+          <t>Entre round y round, el boxeador dice cómo está de verdad. Derramá tu corazón ante Dios.</t>
         </is>
       </c>
     </row>
@@ -45754,7 +45754,7 @@
       </c>
       <c r="D224" s="61" t="inlineStr">
         <is>
-          <t>Pedir con fe no es reclamar un resultado como quien discute un punto en el vóley; es confiar en Dios, que escucha y responde según su voluntad.</t>
+          <t>Orar no es discutir un punto con el árbitro. Es confiar en Dios, que responde según su voluntad.</t>
         </is>
       </c>
     </row>
@@ -45774,7 +45774,7 @@
       </c>
       <c r="D225" s="61" t="inlineStr">
         <is>
-          <t>La hinchada que alienta aunque el partido venga difícil no se va antes del final; orar siempre es eso: no desmayar aunque la respuesta tarde.</t>
+          <t>La hinchada no se va antes del final. Orar siempre es no desmayar aunque la respuesta tarde.</t>
         </is>
       </c>
     </row>
@@ -45794,7 +45794,7 @@
       </c>
       <c r="D226" s="61" t="inlineStr">
         <is>
-          <t>Dos jugadores pueden hacer el mismo ejercicio en la práctica: uno cumple una rutina, el otro se prepara para una final. La visión le da sentido a lo que hacés.</t>
+          <t>Dos jugadores, el mismo ejercicio: uno cumple, el otro se prepara para la final. La visión da sentido.</t>
         </is>
       </c>
     </row>
@@ -45814,7 +45814,7 @@
       </c>
       <c r="D227" s="61" t="inlineStr">
         <is>
-          <t>Un buen capitán de handball se cuida a sí mismo y cuida a sus compañeros; liderar es velar por tu propia vida y por quienes Dios te confió.</t>
+          <t>El buen capitán se cuida y cuida a su equipo. Liderar es velar por tu vida y por los que Dios te confió.</t>
         </is>
       </c>
     </row>
@@ -45834,7 +45834,7 @@
       </c>
       <c r="D228" s="61" t="inlineStr">
         <is>
-          <t>El ajedrecista no ve todo el plan desde la primera jugada; aunque hoy no veas el cuadro completo, Dios tiene pensamientos de bien y de esperanza.</t>
+          <t>El ajedrecista no ve todo el plan en la primera jugada. Dios tiene planes de bien y de esperanza.</t>
         </is>
       </c>
     </row>
@@ -45854,7 +45854,7 @@
       </c>
       <c r="D229" s="61" t="inlineStr">
         <is>
-          <t>En el remo, el timonel habla claro y con calma para que todos remen al mismo ritmo. Una visión se convierte en pasos concretos cuando se comunica con palabras amables.</t>
+          <t>El timonel habla claro y con calma, y todos reman al mismo ritmo. La visión avanza con palabras amables.</t>
         </is>
       </c>
     </row>
@@ -45874,7 +45874,7 @@
       </c>
       <c r="D230" s="61" t="inlineStr">
         <is>
-          <t>El árbitro que estudia el reglamento a fondo cobra con seguridad; conocer bien la Palabra te ayuda a usarla con cuidado y a servir a Dios con dedicación.</t>
+          <t>El árbitro que estudia el reglamento cobra con seguridad. Conocer la Palabra te ayuda a usarla bien.</t>
         </is>
       </c>
     </row>
@@ -45894,7 +45894,7 @@
       </c>
       <c r="D231" s="61" t="inlineStr">
         <is>
-          <t>Un entrenador de futsal ve en un chico más de lo que el chico ve en sí mismo; Dios puede hacer mucho más de lo que pedimos o imaginamos.</t>
+          <t>El entrenador ve en un chico más de lo que él ve en sí mismo. Dios puede hacer más de lo que imaginás.</t>
         </is>
       </c>
     </row>
@@ -45914,7 +45914,7 @@
       </c>
       <c r="D232" s="61" t="inlineStr">
         <is>
-          <t>Cuando un tenista juega limpio y saluda a su rival, todos lo notan; que tus obras se vean, pero que la gloria sea para el Padre, la verdadera fuente de la luz.</t>
+          <t>Todos notan al tenista que saluda a su rival. Que tus obras se vean y la gloria sea para el Padre.</t>
         </is>
       </c>
     </row>
@@ -45934,7 +45934,7 @@
       </c>
       <c r="D233" s="61" t="inlineStr">
         <is>
-          <t>Antes de reclamar un pase, conviene preguntar qué vio el compañero; en casa, una pregunta a tiempo y una palabra que edifica evitan muchas peleas.</t>
+          <t>Antes de reclamar un pase, preguntá qué vio tu compañero. En casa, una pregunta a tiempo evita peleas.</t>
         </is>
       </c>
     </row>
@@ -45954,7 +45954,7 @@
       </c>
       <c r="D234" s="61" t="inlineStr">
         <is>
-          <t>Una palabra de más al árbitro puede costar una falta técnica en el básquet. Pedile a Dios guardia para tu boca y aprendé también el valor de callar a tiempo.</t>
+          <t>Una palabra de más al árbitro cuesta una técnica. Pedile a Dios guardia para tu boca.</t>
         </is>
       </c>
     </row>
@@ -45974,7 +45974,7 @@
       </c>
       <c r="D235" s="61" t="inlineStr">
         <is>
-          <t>Dos en la arena del vóley de playa, y se conocen de memoria. Comprender y honrar a tu esposa también es cuidar la relación que Dios les regaló.</t>
+          <t>En el vóley de playa, la dupla se conoce de memoria. Comprender y honrar a tu pareja cuida la relación.</t>
         </is>
       </c>
     </row>
@@ -45994,7 +45994,7 @@
       </c>
       <c r="D236" s="61" t="inlineStr">
         <is>
-          <t>Un buen entrenador de handball corrige sin humillar y sabe qué decirle a cada jugador; que tu palabra en casa sea siempre con gracia, sazonada con sabiduría.</t>
+          <t>El buen entrenador corrige sin humillar. Que tu palabra en casa sea con gracia.</t>
         </is>
       </c>
     </row>
@@ -46014,7 +46014,7 @@
       </c>
       <c r="D237" s="61" t="inlineStr">
         <is>
-          <t>Llega un segundo tarde y el pase ya no sirve: así es el futsal. La palabra dicha a tiempo, con tacto y prudencia, vale como manzana de oro en la familia.</t>
+          <t>Un segundo tarde y el pase ya no sirve. La palabra a tiempo vale oro en la familia.</t>
         </is>
       </c>
     </row>
@@ -46034,7 +46034,7 @@
       </c>
       <c r="D238" s="61" t="inlineStr">
         <is>
-          <t>Al final del clásico, los que se chocaron todo el partido se dan la mano; en la familia, ser bondadosos y perdonar como Cristo nos perdonó sostiene el vínculo.</t>
+          <t>Al final del clásico, los rivales se dan la mano. En casa, perdonar como Cristo sostiene el vínculo.</t>
         </is>
       </c>
     </row>
@@ -46054,7 +46054,7 @@
       </c>
       <c r="D239" s="61" t="inlineStr">
         <is>
-          <t>Un buen relator sabe qué decir en el momento justo, y la tribuna lo disfruta; en casa, la respuesta acertada y la palabra a tiempo también traen alegría.</t>
+          <t>El buen relator dice lo justo en el momento justo. En casa, la palabra a tiempo trae alegría.</t>
         </is>
       </c>
     </row>
@@ -46074,7 +46074,7 @@
       </c>
       <c r="D240" s="61" t="inlineStr">
         <is>
-          <t>Una dupla de tenis donde cada uno juega su propio plan, sin hablar, se desordena; en casa, administrar juntos y confiar en el Dios que provee lo necesario une a la familia.</t>
+          <t>Una dupla que no habla se desordena. En casa, administrar juntos une a la familia.</t>
         </is>
       </c>
     </row>
@@ -46094,7 +46094,7 @@
       </c>
       <c r="D241" s="61" t="inlineStr">
         <is>
-          <t>En el rally, piloto y copiloto se necesitan: si uno se pierde, el otro lo orienta; mejor dos que uno, también para enfrentar juntos las cuentas de la casa.</t>
+          <t>En el rally, si uno se pierde, el otro lo orienta. Las cuentas de la casa se enfrentan de a dos.</t>
         </is>
       </c>
     </row>
@@ -46114,7 +46114,7 @@
       </c>
       <c r="D242" s="61" t="inlineStr">
         <is>
-          <t>Cuando el amor a la camiseta se cambia por el amor a la plata, algo puede romperse; no es el dinero, es el amor al dinero el que trae muchos dolores.</t>
+          <t>Cuando el amor a la camiseta se cambia por el amor a la plata, algo se rompe. El problema es el amor al dinero.</t>
         </is>
       </c>
     </row>
@@ -46134,7 +46134,7 @@
       </c>
       <c r="D243" s="61" t="inlineStr">
         <is>
-          <t>El ciclista que carga demasiado peso en la bici se cansa antes; cuidate de la avaricia, porque tu vida no depende de la cantidad de cosas que tenés.</t>
+          <t>Demasiado peso cansa al ciclista. Tu vida no depende de la cantidad de cosas que tenés.</t>
         </is>
       </c>
     </row>
@@ -46154,7 +46154,7 @@
       </c>
       <c r="D244" s="61" t="inlineStr">
         <is>
-          <t>Nadie puede defender dos camisetas en el mismo partido; tampoco se puede servir a Dios y al dinero: que la plata no gobierne tu corazón.</t>
+          <t>Nadie defiende dos camisetas en un partido. No se puede servir a Dios y al dinero.</t>
         </is>
       </c>
     </row>
@@ -46174,7 +46174,7 @@
       </c>
       <c r="D245" s="61" t="inlineStr">
         <is>
-          <t>Si cada uno rema a su ritmo, el bote doble gira en círculos. En las finanzas del hogar, tener un mismo sentir ayuda a la familia a avanzar.</t>
+          <t>Si cada uno rema a su ritmo, el bote gira en círculos. En las finanzas de casa, un mismo sentir.</t>
         </is>
       </c>
     </row>
@@ -46194,7 +46194,7 @@
       </c>
       <c r="D246" s="61" t="inlineStr">
         <is>
-          <t>El hincha de un club humilde aprende a disfrutar cada partido, con poco o con mucho; el contentamiento también se aprende, y la paz no depende del monto de tu cuenta.</t>
+          <t>El hincha de un club humilde disfruta cada partido. El contentamiento se aprende.</t>
         </is>
       </c>
     </row>
@@ -46214,7 +46214,7 @@
       </c>
       <c r="D247" s="61" t="inlineStr">
         <is>
-          <t>Nadie aprende a recibir en el vóley en un día: es el pase repetido miles de veces. Como la gota en la roca, los hábitos pequeños te ayudan a avanzar en Cristo.</t>
+          <t>Recibir bien en el vóley es un pase repetido miles de veces. Los hábitos pequeños te hacen avanzar.</t>
         </is>
       </c>
     </row>
@@ -46234,7 +46234,7 @@
       </c>
       <c r="D248" s="61" t="inlineStr">
         <is>
-          <t>El jugador que pierde el control y se hace expulsar deja a su equipo con uno menos; el dominio propio protege tu vida como una muralla protege la ciudad.</t>
+          <t>El expulsado deja al equipo con uno menos. El dominio propio es muralla para tu vida.</t>
         </is>
       </c>
     </row>
@@ -46254,7 +46254,7 @@
       </c>
       <c r="D249" s="61" t="inlineStr">
         <is>
-          <t>El nadador vuelve a la pileta cada mañana, aunque a veces no tenga ganas; perseverar en la oración y dar gracias también se vuelve hábito con constancia.</t>
+          <t>El nadador vuelve a la pileta aunque no tenga ganas. La oración también se vuelve hábito.</t>
         </is>
       </c>
     </row>
@@ -46274,7 +46274,7 @@
       </c>
       <c r="D250" s="61" t="inlineStr">
         <is>
-          <t>Quien llega primero a cada entrenamiento de handball termina siendo referente del grupo. La mano diligente lidera, y el esfuerzo constante gana confianza.</t>
+          <t>El que llega primero a cada entrenamiento termina siendo referente. La mano diligente lidera.</t>
         </is>
       </c>
     </row>
@@ -46294,7 +46294,7 @@
       </c>
       <c r="D251" s="61" t="inlineStr">
         <is>
-          <t>El atleta entrena el cuerpo con disciplina, y eso vale; pero ejercitarse en la piedad vale para todo, aquí y en la eternidad. Las dos cosas piden constancia.</t>
+          <t>El atleta entrena el cuerpo, y eso vale. Ejercitarse en la fe vale para siempre.</t>
         </is>
       </c>
     </row>
@@ -46314,7 +46314,7 @@
       </c>
       <c r="D252" s="61" t="inlineStr">
         <is>
-          <t>Las inferiores no muestran sus frutos en una sola temporada; no te canses de hacer el bien, que la cosecha llega a su tiempo, aunque hoy no la veas.</t>
+          <t>Las inferiores no dan frutos en una temporada. No te canses de hacer el bien.</t>
         </is>
       </c>
     </row>
@@ -46334,7 +46334,7 @@
       </c>
       <c r="D253" s="61" t="inlineStr">
         <is>
-          <t>El ciclista que no sale a rodar porque hace frío lo nota después en la ruta; la pereza pospone lo necesario, y los pequeños hábitos de hoy preparan lo que viene.</t>
+          <t>El ciclista que no sale por el frío lo nota en la ruta. Los hábitos de hoy preparan lo que viene.</t>
         </is>
       </c>
     </row>
@@ -46354,7 +46354,7 @@
       </c>
       <c r="D254" s="61" t="inlineStr">
         <is>
-          <t>Cuando el testigo pasa de mano en mano, nadie llega solo: cada uno corre su tramo del relevo. Revestidos de amor, juntos llegamos donde solos no podíamos.</t>
+          <t>En el relevo, nadie llega solo. Revestidos de amor, juntos llegamos más lejos.</t>
         </is>
       </c>
     </row>
@@ -46374,7 +46374,7 @@
       </c>
       <c r="D255" s="61" t="inlineStr">
         <is>
-          <t>En el fútbol de barrio, uno presta la pelota, otro el arco y otro marca la cancha; compartir nace del amor, no de la obligación, y así se arma un solo corazón.</t>
+          <t>En el fútbol de barrio, uno presta la pelota y otro el arco. Compartir nace del amor.</t>
         </is>
       </c>
     </row>
@@ -46394,7 +46394,7 @@
       </c>
       <c r="D256" s="61" t="inlineStr">
         <is>
-          <t>Armador, central y líbero cumplen funciones distintas para el mismo equipo de vóley. Usá tu don con generosidad para servir a los demás.</t>
+          <t>Armador, central y líbero cumplen funciones distintas. Usá tu don para servir.</t>
         </is>
       </c>
     </row>
@@ -46414,7 +46414,7 @@
       </c>
       <c r="D257" s="61" t="inlineStr">
         <is>
-          <t>Un equipo de básquet en armonía se nota en cada pase; qué bueno y agradable es que los hermanos convivan en unidad, cuidándose con respeto y paz.</t>
+          <t>Un equipo en armonía se nota en cada pase. Qué bueno es convivir en unidad.</t>
         </is>
       </c>
     </row>
@@ -46434,7 +46434,7 @@
       </c>
       <c r="D258" s="61" t="inlineStr">
         <is>
-          <t>Cuando juega la Albirroja, en el barrio se juntan vecinos que piensan distinto en todo; vivir en paz y en unidad es posible, y el Dios de paz está con nosotros.</t>
+          <t>Cuando juega la Albirroja, se juntan vecinos que piensan distinto. La unidad es posible.</t>
         </is>
       </c>
     </row>
@@ -46454,7 +46454,7 @@
       </c>
       <c r="D259" s="61" t="inlineStr">
         <is>
-          <t>Cuando un compañero se lesiona, todo el equipo de handball lo siente; así funciona el cuerpo: cuidarnos mutuamente, sufrir juntos y alegrarnos juntos.</t>
+          <t>Cuando un compañero se lesiona, todo el equipo lo siente. Así funciona el cuerpo de Cristo.</t>
         </is>
       </c>
     </row>
@@ -46474,7 +46474,7 @@
       </c>
       <c r="D260" s="61" t="inlineStr">
         <is>
-          <t>Pocas imágenes de comunidad como el pelotón: se turnan para cortar el viento y llegan más lejos. Un mismo sentir, compasión y amor fraternal también hacen avanzar a la comunidad.</t>
+          <t>En el pelotón se turnan para cortar el viento. Compasión y amor fraternal hacen avanzar a la comunidad.</t>
         </is>
       </c>
     </row>
@@ -46494,7 +46494,7 @@
       </c>
       <c r="D261" s="61" t="inlineStr">
         <is>
-          <t>El veterano del plantel ya no corre como antes, pero su voz ordena al equipo; una persona mayor no pierde valor con los años, y cuidarla es una forma de amar.</t>
+          <t>El veterano ya no corre como antes, pero su voz ordena al equipo. Los años no le quitan valor a nadie.</t>
         </is>
       </c>
     </row>
@@ -46514,7 +46514,7 @@
       </c>
       <c r="D262" s="61" t="inlineStr">
         <is>
-          <t>El chico que aprende a nadar de pequeño lleva esa habilidad toda la vida; acordarse de Dios desde la niñez también deja raíces que sostienen después.</t>
+          <t>Lo que se aprende de chico en la pileta dura toda la vida. Acordarse de Dios desde la niñez, también.</t>
         </is>
       </c>
     </row>
@@ -46534,7 +46534,7 @@
       </c>
       <c r="D263" s="61" t="inlineStr">
         <is>
-          <t>Un juvenil de básquet no crece solo en altura: también aprende a pensar el juego y a convivir; como Jesús, crecer es en sabiduría, en estatura y en gracia.</t>
+          <t>El juvenil no crece solo en altura. Como Jesús: en sabiduría, en estatura y en gracia.</t>
         </is>
       </c>
     </row>
@@ -46554,7 +46554,7 @@
       </c>
       <c r="D264" s="61" t="inlineStr">
         <is>
-          <t>Hay ajedrecistas que siguen jugando con pasión a los ochenta; la fe que nos acompañó desde jóvenes sigue con nosotros en cada etapa, también en la vejez.</t>
+          <t>Hay ajedrecistas que juegan con pasión a los ochenta. La fe nos acompaña en cada etapa.</t>
         </is>
       </c>
     </row>
@@ -46574,7 +46574,7 @@
       </c>
       <c r="D265" s="61" t="inlineStr">
         <is>
-          <t>En un equipo de futsal, el joven pone las piernas y el veterano pone la lectura del partido; la fuerza y las canas tienen su honra, y cada etapa tiene su valor.</t>
+          <t>El joven pone las piernas; el veterano, la lectura del partido. Cada etapa tiene su honra.</t>
         </is>
       </c>
     </row>
@@ -46594,7 +46594,7 @@
       </c>
       <c r="D266" s="61" t="inlineStr">
         <is>
-          <t>En las maratones también corren abuelos a su propio ritmo, y siempre hay alguien que los alienta; Dios te sostiene hasta las canas, y su cuidado no se achica con la edad.</t>
+          <t>En la maratón también corren abuelos, y siempre hay alguien que los alienta. Dios te sostiene hasta las canas.</t>
         </is>
       </c>
     </row>
@@ -46614,7 +46614,7 @@
       </c>
       <c r="D267" s="61" t="inlineStr">
         <is>
-          <t>El entrenador veterano de vóley ya no salta, pero sigue formando jugadores; aun en la vejez se puede dar fruto, y los años no le quitan valor a tu vida.</t>
+          <t>El entrenador veterano ya no salta, pero sigue formando. Aun en la vejez se da fruto.</t>
         </is>
       </c>
     </row>
@@ -46634,7 +46634,7 @@
       </c>
       <c r="D268" s="61" t="inlineStr">
         <is>
-          <t>Al jugador que llega a un club nuevo le cuesta sentir que la camiseta ya es suya; en Cristo sos nueva criatura: lo viejo pasó y tu identidad nueva es real.</t>
+          <t>Al recién llegado le cuesta sentir suya la camiseta. En Cristo sos nueva criatura.</t>
         </is>
       </c>
     </row>
@@ -46654,7 +46654,7 @@
       </c>
       <c r="D269" s="61" t="inlineStr">
         <is>
-          <t>Una raqueta hecha a mano tiene un diseño pensado para su uso; vos sos obra de Dios, no un accidente, creado para las buenas obras que Él preparó.</t>
+          <t>Una raqueta hecha a mano tiene un diseño pensado. Sos obra de Dios, no un accidente.</t>
         </is>
       </c>
     </row>
@@ -46674,7 +46674,7 @@
       </c>
       <c r="D270" s="61" t="inlineStr">
         <is>
-          <t>El juvenil que sube a primera a veces juega con miedo a que lo devuelvan; en Cristo ya no sos esclavo sino hijo, y tu lugar no depende de tu rendimiento.</t>
+          <t>El juvenil juega con miedo a que lo devuelvan. En Cristo sos hijo: tu lugar no depende del rendimiento.</t>
         </is>
       </c>
     </row>
@@ -46694,7 +46694,7 @@
       </c>
       <c r="D271" s="61" t="inlineStr">
         <is>
-          <t>Cuando suena el himno antes de un partido de la Albirroja, los jugadores saben a quién representan; vos sos pueblo escogido por Dios, llamado a anunciar sus virtudes.</t>
+          <t>Con el himno, los jugadores saben a quién representan. Vos sos pueblo de Dios.</t>
         </is>
       </c>
     </row>
@@ -46714,7 +46714,7 @@
       </c>
       <c r="D272" s="61" t="inlineStr">
         <is>
-          <t>Cada remero deja su propio ritmo y sigue la palada del que marca. Vivir por fe es dejar que Cristo, que vive en vos, marque tu ritmo.</t>
+          <t>Cada remero sigue la palada del que marca. Vivir por fe es dejar que Cristo marque tu ritmo.</t>
         </is>
       </c>
     </row>
@@ -46734,7 +46734,7 @@
       </c>
       <c r="D273" s="61" t="inlineStr">
         <is>
-          <t>El chico que entra a la cancha de la mano de su papá no pide permiso: sabe que es hijo. El Espíritu te confirma que sos hijo de Dios y heredero.</t>
+          <t>El chico que entra a la cancha de la mano de su papá sabe que es hijo. Vos sos hijo de Dios.</t>
         </is>
       </c>
     </row>
@@ -46754,7 +46754,7 @@
       </c>
       <c r="D274" s="61" t="inlineStr">
         <is>
-          <t>La medalla del atletismo se gana corriendo, pero ser hijo de Dios no se gana: se recibe al recibir a Cristo. Saber quién sos cambia cómo encarás cada día.</t>
+          <t>Una medalla se gana corriendo; ser hijo de Dios se recibe. Saber quién sos cambia tu día.</t>
         </is>
       </c>
     </row>
@@ -46774,7 +46774,7 @@
       </c>
       <c r="D275" s="61" t="inlineStr">
         <is>
-          <t>El capitán de futsal no siempre se siente listo para llevar la cinta; a veces el llamado llega antes que la seguridad. Moisés también dudó, y Dios igual lo llamó.</t>
+          <t>El capitán no siempre se siente listo para la cinta. Moisés también dudó, y Dios igual lo llamó.</t>
         </is>
       </c>
     </row>
@@ -46794,7 +46794,7 @@
       </c>
       <c r="D276" s="61" t="inlineStr">
         <is>
-          <t>Sobre el ring, el que mejor se controla no es el más débil: es el que sabe contener su fuerza. Eso es la humildad bajo presión.</t>
+          <t>En el ring, el que mejor se controla sabe contener su fuerza. Eso es humildad bajo presión.</t>
         </is>
       </c>
     </row>
@@ -46814,7 +46814,7 @@
       </c>
       <c r="D277" s="61" t="inlineStr">
         <is>
-          <t>En el remo nadie avanza solo: alguien tiene que decir «¡vamos!» y todos reman juntos. Nehemías invitó al pueblo a levantar los muros codo a codo.</t>
+          <t>En el remo, alguien dice «¡vamos!» y todos reman juntos. Nehemías levantó los muros codo a codo.</t>
         </is>
       </c>
     </row>
@@ -46834,7 +46834,7 @@
       </c>
       <c r="D278" s="61" t="inlineStr">
         <is>
-          <t>Frente a un rival más grande, el equipo chico sabe de dónde saca el ánimo. David no salió confiado en la armadura, sino en el nombre del Señor.</t>
+          <t>El equipo chico sabe de dónde saca el ánimo. David salió en el nombre del Señor, no en la armadura.</t>
         </is>
       </c>
     </row>
@@ -46854,7 +46854,7 @@
       </c>
       <c r="D279" s="61" t="inlineStr">
         <is>
-          <t>El utilero llega primero y se va último, y sin él no sale nadie a la cancha. Jesús enseñó que el grande es el que sirve.</t>
+          <t>El utilero llega primero y se va último. Jesús enseñó que el grande es el que sirve.</t>
         </is>
       </c>
     </row>
@@ -46874,7 +46874,7 @@
       </c>
       <c r="D280" s="61" t="inlineStr">
         <is>
-          <t>Un buen árbitro no se gana el respeto por el silbato, sino por su carácter dentro y fuera de la cancha. Así se mide también un líder íntegro.</t>
+          <t>Al árbitro se lo respeta por su carácter, no por el silbato. Así se mide un líder íntegro.</t>
         </is>
       </c>
     </row>
@@ -46914,7 +46914,7 @@
       </c>
       <c r="D282" s="61" t="inlineStr">
         <is>
-          <t>Nadie toca la pelota dos veces seguidas en el vóley: cada uno cumple su parte y el punto se construye entre todos. Un hogar funciona parecido.</t>
+          <t>En el vóley, cada uno cumple su parte y el punto se arma entre todos. Un hogar funciona parecido.</t>
         </is>
       </c>
     </row>
@@ -46934,7 +46934,7 @@
       </c>
       <c r="D283" s="61" t="inlineStr">
         <is>
-          <t>El entrenador que prepara la semana antes del partido le ahorra apuros a todo el plantel. Una casa organizada también se cuida con anticipación.</t>
+          <t>El técnico que prepara la semana le ahorra apuros al plantel. Una casa organizada se cuida con tiempo.</t>
         </is>
       </c>
     </row>
@@ -46954,7 +46954,7 @@
       </c>
       <c r="D284" s="61" t="inlineStr">
         <is>
-          <t>Un buen defensor no abandona a su compañero cuando el rival ataca por su lado: lo cubre. Cuidar a los nuestros también es parte de vivir la fe.</t>
+          <t>El buen defensor cubre a su compañero. Cuidar a los nuestros también es vivir la fe.</t>
         </is>
       </c>
     </row>
@@ -46974,7 +46974,7 @@
       </c>
       <c r="D285" s="61" t="inlineStr">
         <is>
-          <t>Roces hay todo el partido en el handball, y el equipo sigue unido si se dan la mano después de cada choque. En casa, la paciencia y el perdón hacen lo mismo.</t>
+          <t>En el handball hay roces, y el equipo se da la mano después. En casa, paciencia y perdón.</t>
         </is>
       </c>
     </row>
@@ -46994,7 +46994,7 @@
       </c>
       <c r="D286" s="61" t="inlineStr">
         <is>
-          <t>El aplauso de la hinchada al que corrió todo el partido vale mucho. En casa también hace falta reconocer el esfuerzo de quien sostiene el día a día.</t>
+          <t>La hinchada aplaude al que corrió todo el partido. En casa, reconocé a quien sostiene el día a día.</t>
         </is>
       </c>
     </row>
@@ -47014,7 +47014,7 @@
       </c>
       <c r="D287" s="61" t="inlineStr">
         <is>
-          <t>En el pelotón, los ciclistas se turnan para ir adelante cortando el viento: hoy tirás vos, mañana yo. Así se vive la humildad mutua en familia.</t>
+          <t>En el pelotón, hoy tirás vos y mañana yo. Así se vive la humildad en familia.</t>
         </is>
       </c>
     </row>
@@ -47034,7 +47034,7 @@
       </c>
       <c r="D288" s="61" t="inlineStr">
         <is>
-          <t>Kilómetro 40: alguien frena para acompañar a otro hasta la meta; la lealtad pesa más que el reloj. Así es un hogar que camina junto, aun en lo difícil.</t>
+          <t>En el kilómetro 40, alguien frena para acompañar a otro. Un hogar camina junto, aun en lo difícil.</t>
         </is>
       </c>
     </row>
@@ -47054,7 +47054,7 @@
       </c>
       <c r="D289" s="61" t="inlineStr">
         <is>
-          <t>El que regala un pase de gol con alegría lo disfruta tanto como el que la empuja. Dios ama al dador alegre, no al que da con tristeza u obligación.</t>
+          <t>Quien regala un pase de gol lo disfruta como el que la empuja. Dios ama al dador alegre.</t>
         </is>
       </c>
     </row>
@@ -47074,7 +47074,7 @@
       </c>
       <c r="D290" s="61" t="inlineStr">
         <is>
-          <t>El relevista suelta el testigo confiando en las manos del compañero. Dar a Dios es un acto de confianza, no un pago para recibir algo a cambio.</t>
+          <t>El relevista suelta el testigo confiando en su compañero. Dar a Dios es confianza, no un pago.</t>
         </is>
       </c>
     </row>
@@ -47094,7 +47094,7 @@
       </c>
       <c r="D291" s="61" t="inlineStr">
         <is>
-          <t>Antes del partido, muchos equipos se juntan en ronda para orar. Honrar a Dios con lo primero es poner las cosas en orden, no una cábala.</t>
+          <t>Muchos equipos oran en ronda antes del partido. Honrar a Dios con lo primero no es una cábala.</t>
         </is>
       </c>
     </row>
@@ -47114,7 +47114,7 @@
       </c>
       <c r="D292" s="61" t="inlineStr">
         <is>
-          <t>El veterano que de chico tuvo quien le enseñara a tirar al aro hoy regala sus sábados a los chicos del barrio. La generosidad nace de la gracia que primero recibimos.</t>
+          <t>Al que de chico le enseñaron a tirar al aro, hoy enseña a otros. La generosidad nace de la gracia recibida.</t>
         </is>
       </c>
     </row>
@@ -47134,7 +47134,7 @@
       </c>
       <c r="D293" s="61" t="inlineStr">
         <is>
-          <t>Los brazos para nadar, el aire en los pulmones, el talento para competir: nada de eso lo fabricamos. Todo viene de Dios, y de lo suyo le damos.</t>
+          <t>Los brazos, el aire, el talento: nada lo fabricamos. De lo que Dios nos da, le damos.</t>
         </is>
       </c>
     </row>
@@ -47154,7 +47154,7 @@
       </c>
       <c r="D294" s="61" t="inlineStr">
         <is>
-          <t>El técnico que regala su tiempo a los chicos del barrio, sin cobrar y sin cámaras, deja mucho más que tácticas. Dar sin amor es una transacción; dar con amor cambia vidas.</t>
+          <t>El técnico que regala su tiempo a los chicos del barrio deja más que tácticas. Dar con amor cambia vidas.</t>
         </is>
       </c>
     </row>
@@ -47174,7 +47174,7 @@
       </c>
       <c r="D295" s="61" t="inlineStr">
         <is>
-          <t>En el Rally del Chaco el navegante no maneja, pero da lo que sabe en cada curva. Dar es eso: tiempo, talento y recursos que Dios mismo nos provee.</t>
+          <t>El navegante no maneja, pero da lo que sabe en cada curva. Dar es tiempo, talento y recursos.</t>
         </is>
       </c>
     </row>
@@ -47194,7 +47194,7 @@
       </c>
       <c r="D296" s="61" t="inlineStr">
         <is>
-          <t>El que abre una escuelita de fútbol en el barrio quizá nunca vea a esos chicos jugar en primera. Como el abuelo que planta un árbol, el legado se siembra sin garantías.</t>
+          <t>El que abre una escuelita quizá nunca vea a esos chicos en primera. El legado se siembra sin garantías.</t>
         </is>
       </c>
     </row>
@@ -47214,7 +47214,7 @@
       </c>
       <c r="D297" s="61" t="inlineStr">
         <is>
-          <t>El abuelo que enseña a sus nietos a mover las piezas del ajedrez deja algo que dura más que una partida ganada. Una buena herencia piensa en varias generaciones.</t>
+          <t>El abuelo que enseña ajedrez a sus nietos deja más que una partida ganada. Una buena herencia piensa en generaciones.</t>
         </is>
       </c>
     </row>
@@ -47234,7 +47234,7 @@
       </c>
       <c r="D298" s="61" t="inlineStr">
         <is>
-          <t>El último kilómetro de la maratón cuenta tanto como el primero. Pablo pudo decir «he terminado la carrera»: terminar bien también es fidelidad.</t>
+          <t>El último kilómetro cuenta tanto como el primero. Terminar bien la carrera también es fidelidad.</t>
         </is>
       </c>
     </row>
@@ -47254,7 +47254,7 @@
       </c>
       <c r="D299" s="61" t="inlineStr">
         <is>
-          <t>Veinticuatro segundos de posesión en el básquet te obligan a elegir qué vale la pena. Contar nuestros días nos ayuda a ordenar las prioridades con sabiduría.</t>
+          <t>Veinticuatro segundos te obligan a elegir. Contar nuestros días ordena las prioridades.</t>
         </is>
       </c>
     </row>
@@ -47274,7 +47274,7 @@
       </c>
       <c r="D300" s="61" t="inlineStr">
         <is>
-          <t>El barrio puede olvidar los goles de un jugador, pero recuerda si fue leal y respetuoso. Un buen nombre vale más que cualquier trofeo.</t>
+          <t>El barrio olvida los goles, pero recuerda si fuiste leal. Un buen nombre vale más que un trofeo.</t>
         </is>
       </c>
     </row>
@@ -47294,7 +47294,7 @@
       </c>
       <c r="D301" s="61" t="inlineStr">
         <is>
-          <t>Una pelota mal recibida en el vóley todavía puede terminar en un buen ataque. José lo vivió: lo que otros pensaron para mal, Dios lo encaminó para bien.</t>
+          <t>Una pelota mal recibida todavía puede terminar en punto. Lo que otros pensaron para mal, Dios lo encamina para bien.</t>
         </is>
       </c>
     </row>
@@ -47314,7 +47314,7 @@
       </c>
       <c r="D302" s="61" t="inlineStr">
         <is>
-          <t>Algunos entrenadores ya no están, y sin embargo su manera de jugar sigue viva en la cancha. Lo que se hace por fe sigue hablando.</t>
+          <t>Hay entrenadores que ya no están, pero su juego sigue vivo en la cancha. Lo que se hace por fe sigue hablando.</t>
         </is>
       </c>
     </row>
@@ -47334,7 +47334,7 @@
       </c>
       <c r="D303" s="61" t="inlineStr">
         <is>
-          <t>El canchero que marca las líneas con cuidado, aunque nadie lo aplauda, trabaja como para Dios. Todo oficio tiene dignidad cuando se hace con el corazón despierto.</t>
+          <t>El canchero marca las líneas con cuidado aunque nadie aplauda. Todo oficio tiene dignidad.</t>
         </is>
       </c>
     </row>
@@ -47354,7 +47354,7 @@
       </c>
       <c r="D304" s="61" t="inlineStr">
         <is>
-          <t>Saludar al árbitro, al rival y al aguatero por igual es dar a cada uno el respeto que le corresponde. Eso también es vivir nuestra fe.</t>
+          <t>Saludar al árbitro, al rival y al aguatero por igual. Dar a cada uno el respeto que le corresponde.</t>
         </is>
       </c>
     </row>
@@ -47374,7 +47374,7 @@
       </c>
       <c r="D305" s="61" t="inlineStr">
         <is>
-          <t>El ciclista que tira del grupo no pedalea solo para su llegada: su esfuerzo sostiene a otros. El fruto de nuestro trabajo también puede bendecir al necesitado.</t>
+          <t>El ciclista que tira del grupo sostiene a otros. Tu trabajo también puede bendecir al necesitado.</t>
         </is>
       </c>
     </row>
@@ -47394,7 +47394,7 @@
       </c>
       <c r="D306" s="61" t="inlineStr">
         <is>
-          <t>El maratonista no llega con un pique, sino con un ritmo constante. Trabajar con sosiego, día a día, para comer el propio pan es parte de una vida digna.</t>
+          <t>El maratonista llega con ritmo constante, no con un pique. Trabajar con sosiego es parte de una vida digna.</t>
         </is>
       </c>
     </row>
@@ -47414,7 +47414,7 @@
       </c>
       <c r="D307" s="61" t="inlineStr">
         <is>
-          <t>En el vestuario se puede hablar mucho, pero el partido de futsal se juega en la cancha. En toda labor hay fruto; el puro discurso no construye nada.</t>
+          <t>En el vestuario se habla mucho, pero el partido se juega en la cancha. El puro discurso no construye.</t>
         </is>
       </c>
     </row>
@@ -47434,7 +47434,7 @@
       </c>
       <c r="D308" s="61" t="inlineStr">
         <is>
-          <t>Mirá a los chicos que juegan al vóley en la playa del lago hasta que cae el sol: disfrutan cada pelota. Alegrarse en el propio trabajo también es un regalo de Dios.</t>
+          <t>Los chicos juegan al vóley en la playa hasta que cae el sol. Alegrarse en el trabajo es un regalo de Dios.</t>
         </is>
       </c>
     </row>
@@ -47454,7 +47454,7 @@
       </c>
       <c r="D309" s="61" t="inlineStr">
         <is>
-          <t>El árbitro, el juez de línea y quien limpia las tribunas merecen su justo pago. Digno es el obrero de su salario.</t>
+          <t>El árbitro, el juez de línea y quien limpia las tribunas merecen su pago. Digno es el obrero de su salario.</t>
         </is>
       </c>
     </row>
@@ -47474,7 +47474,7 @@
       </c>
       <c r="D310" s="61" t="inlineStr">
         <is>
-          <t>Partido de barrio, alguien cae lesionado, y lo primero no es el resultado sino acercarse a ayudar. El buen samaritano no pasó de largo.</t>
+          <t>En el partido de barrio, si alguien cae, lo primero es ayudar. El buen samaritano no pasó de largo.</t>
         </is>
       </c>
     </row>
@@ -47494,7 +47494,7 @@
       </c>
       <c r="D311" s="61" t="inlineStr">
         <is>
-          <t>Cuando al nadador se le acaban las fuerzas, saber que hay un guardavidas atento le devuelve la calma. Dios es nuestro pronto auxilio en la angustia.</t>
+          <t>Al nadador sin fuerzas lo calma saber que hay un guardavidas. Dios es pronto auxilio en la angustia.</t>
         </is>
       </c>
     </row>
@@ -47514,7 +47514,7 @@
       </c>
       <c r="D312" s="61" t="inlineStr">
         <is>
-          <t>Si un corredor se desploma en la pista, los jueces no esperan que termine la carrera para asistirlo. Actuar a tiempo ante el peligro ajeno es una responsabilidad real.</t>
+          <t>Si un corredor se desploma, nadie espera que termine la carrera. Ayudar a tiempo es responsabilidad.</t>
         </is>
       </c>
     </row>
@@ -47534,7 +47534,7 @@
       </c>
       <c r="D313" s="61" t="inlineStr">
         <is>
-          <t>Ningún entrenador atiende solo una lesión seria: pide camilla, médico y ayuda. En la enfermedad tampoco tenemos que estar solos; llamamos a otros y oramos juntos.</t>
+          <t>Ante una lesión seria, el entrenador pide ayuda. En la enfermedad no estamos solos: oramos juntos.</t>
         </is>
       </c>
     </row>
@@ -47554,7 +47554,7 @@
       </c>
       <c r="D314" s="61" t="inlineStr">
         <is>
-          <t>En medio del ruido de un estadio lleno, una madre reconoce la voz de su hijo en la cancha. Así de cerca está Dios del que clama en su angustia.</t>
+          <t>En un estadio lleno, una madre reconoce la voz de su hijo. Así de cerca está Dios del que clama.</t>
         </is>
       </c>
     </row>
@@ -47574,7 +47574,7 @@
       </c>
       <c r="D315" s="61" t="inlineStr">
         <is>
-          <t>El equipo de rescate de un rally entrena para mantener la calma cuando todo se complica. El pánico se enfrenta con la promesa de Dios: «No tengas miedo, yo estoy contigo».</t>
+          <t>El rescate del rally entrena para mantener la calma. «No tengas miedo, yo estoy contigo».</t>
         </is>
       </c>
     </row>
@@ -47594,7 +47594,7 @@
       </c>
       <c r="D316" s="61" t="inlineStr">
         <is>
-          <t>Cientos de recepciones en la práctica de vóley, para estar listos cuando llega el saque difícil. Prepararse para ayudar y clamar a Dios en la angustia también se entrena.</t>
+          <t>Cientos de recepciones para el saque difícil. Prepararse para ayudar también se entrena.</t>
         </is>
       </c>
     </row>
@@ -47614,7 +47614,7 @@
       </c>
       <c r="D317" s="61" t="inlineStr">
         <is>
-          <t>La hinchada canta con el alma aunque el marcador no acompañe. Venir ante Dios con alegría no depende del resultado, sino del corazón.</t>
+          <t>La hinchada canta aunque el marcador no acompañe. Alabar a Dios no depende del resultado.</t>
         </is>
       </c>
     </row>
@@ -47634,7 +47634,7 @@
       </c>
       <c r="D318" s="61" t="inlineStr">
         <is>
-          <t>Una cosa es ponerse la camiseta para la foto y otra es llevarla en el corazón. Dios busca adoradores en espíritu y en verdad, no solo de forma.</t>
+          <t>No es lo mismo ponerse la camiseta para la foto que llevarla en el corazón. Dios busca adoradores en verdad.</t>
         </is>
       </c>
     </row>
@@ -47654,7 +47654,7 @@
       </c>
       <c r="D319" s="61" t="inlineStr">
         <is>
-          <t>El remero sale al río con frío, con calor o con lluvia, tenga ganas o no. Bendecir a Dios en todo tiempo es parecido: no depende de las circunstancias.</t>
+          <t>El remero sale con frío, calor o lluvia. Bendecir a Dios no depende de las circunstancias.</t>
         </is>
       </c>
     </row>
@@ -47674,7 +47674,7 @@
       </c>
       <c r="D320" s="61" t="inlineStr">
         <is>
-          <t>Hay noches de lágrimas y noches de canto en el vestuario de básquet. Santiago dice: ¿alguien sufre? Que ore; ¿alguien está alegre? Que cante alabanzas.</t>
+          <t>En el vestuario hay noches de lágrimas y noches de canto. ¿Alguien sufre? Que ore. ¿Está alegre? Que cante.</t>
         </is>
       </c>
     </row>
@@ -47694,7 +47694,7 @@
       </c>
       <c r="D321" s="61" t="inlineStr">
         <is>
-          <t>Desde el corredor de maratón hasta el abuelo que camina despacito por la costanera, todos respiran. Y todo lo que respira puede alabar al Señor.</t>
+          <t>Del maratonista al abuelo que camina por la costanera, todos respiran. Todo lo que respira alabe al Señor.</t>
         </is>
       </c>
     </row>
@@ -47714,7 +47714,7 @@
       </c>
       <c r="D322" s="61" t="inlineStr">
         <is>
-          <t>El boxeador que se levanta de madrugada a entrenar sabe que cuesta. La alabanza también es un sacrificio: se ofrece aun cuando no es fácil.</t>
+          <t>Entrenar de madrugada cuesta. La alabanza también se ofrece cuando no es fácil.</t>
         </is>
       </c>
     </row>
@@ -47734,7 +47734,7 @@
       </c>
       <c r="D323" s="61" t="inlineStr">
         <is>
-          <t>Pinchó, quedó lejos del pelotón, y el ciclista igual sigue pedaleando. Aunque falte todo, Dios da fuerzas para seguir caminando.</t>
+          <t>Pinchó y quedó lejos del pelotón, pero sigue pedaleando. Dios da fuerzas aunque falte todo.</t>
         </is>
       </c>
     </row>
@@ -47754,7 +47754,7 @@
       </c>
       <c r="D324" s="61" t="inlineStr">
         <is>
-          <t>El arquero tiene un segundo para decidir hacia dónde tirarse, sin toda la información. Por eso necesitamos pedirle sabiduría a Dios, que la da sin reproche.</t>
+          <t>El arquero decide en un segundo, sin toda la información. Pedile sabiduría a Dios: la da sin reproche.</t>
         </is>
       </c>
     </row>
@@ -47774,7 +47774,7 @@
       </c>
       <c r="D325" s="61" t="inlineStr">
         <is>
-          <t>El piloto de rally confía en las notas de su navegante aunque todavía no vea la próxima curva. Confiar en Dios más que en nuestro propio entendimiento se parece a eso.</t>
+          <t>El piloto confía en las notas del navegante antes de ver la curva. Confiá en Dios más que en tu entendimiento.</t>
         </is>
       </c>
     </row>
@@ -47794,7 +47794,7 @@
       </c>
       <c r="D326" s="61" t="inlineStr">
         <is>
-          <t>El ajedrecista que estudió bien sus aperturas mueve con calma, sin que le tiemble la mano. Guardar la sabiduría de Dios nos deja caminar con confianza.</t>
+          <t>El ajedrecista que estudió sus aperturas mueve con calma. La sabiduría de Dios da confianza.</t>
         </is>
       </c>
     </row>
@@ -47814,7 +47814,7 @@
       </c>
       <c r="D327" s="61" t="inlineStr">
         <is>
-          <t>El tenista que espera el viento perfecto para sacar se queda con la pelota en la mano. El que mira el viento no siembra: hay que actuar con lo que se tiene.</t>
+          <t>El que espera el viento perfecto se queda con la pelota en la mano. Actuá con lo que tenés.</t>
         </is>
       </c>
     </row>
@@ -47834,7 +47834,7 @@
       </c>
       <c r="D328" s="61" t="inlineStr">
         <is>
-          <t>Un buen capitán de handball no pide la mejor camiseta, pide entender a su equipo. Salomón pidió un corazón que sepa discernir, y eso le agradó a Dios.</t>
+          <t>El buen capitán pide entender a su equipo. Salomón pidió un corazón que sepa discernir.</t>
         </is>
       </c>
     </row>
@@ -47854,7 +47854,7 @@
       </c>
       <c r="D329" s="61" t="inlineStr">
         <is>
-          <t>En el futsal, el técnico guía desde el costado con la mirada y la voz. Dios promete enseñarnos el camino; no tenemos que decidir solos.</t>
+          <t>Desde el costado, el técnico guía con la mirada y la voz. Dios promete enseñarte el camino.</t>
         </is>
       </c>
     </row>
@@ -47874,7 +47874,7 @@
       </c>
       <c r="D330" s="61" t="inlineStr">
         <is>
-          <t>Minuto cero de un clásico: cada uno tiene su plan de juego en la cabeza. Muchos planes hay en el corazón, pero el consejo del Señor permanece.</t>
+          <t>Antes del clásico, cada uno tiene su plan. Muchos planes hay en el corazón, pero el consejo del Señor permanece.</t>
         </is>
       </c>
     </row>
@@ -47894,7 +47894,7 @@
       </c>
       <c r="D331" s="61" t="inlineStr">
         <is>
-          <t>Los chicos aprenden a tirar al aro mirando a papá en el patio. La fe también se transmite así: contando y mostrando las obras de Dios a la próxima generación.</t>
+          <t>Los chicos aprenden a tirar al aro mirando a papá. La fe también se transmite mostrando.</t>
         </is>
       </c>
     </row>
@@ -47914,7 +47914,7 @@
       </c>
       <c r="D332" s="61" t="inlineStr">
         <is>
-          <t>Camino al entrenamiento, en el colectivo o en la moto, hay charlas que valen oro. Deuteronomio nos invita a hablar de Dios en casa y en el camino.</t>
+          <t>Camino al entrenamiento hay charlas que valen oro. Hablá de Dios en casa y en el camino.</t>
         </is>
       </c>
     </row>
@@ -47934,7 +47934,7 @@
       </c>
       <c r="D333" s="61" t="inlineStr">
         <is>
-          <t>Una medalla colgada en la pared hace que los nietos pregunten: ¿y esto de dónde salió? Las señales de fe en casa también abren la puerta para contar la historia de Dios.</t>
+          <t>Una medalla en la pared hace preguntar a los nietos. Las señales de fe en casa abren la charla.</t>
         </is>
       </c>
     </row>
@@ -47954,7 +47954,7 @@
       </c>
       <c r="D334" s="61" t="inlineStr">
         <is>
-          <t>Como la familia que va junta a alentar con los mismos colores, hay hogares que se juntan para dar gloria a Dios. Adorar en familia también se aprende.</t>
+          <t>La familia va junta a alentar con los mismos colores. Adorar en familia también se aprende.</t>
         </is>
       </c>
     </row>
@@ -47974,7 +47974,7 @@
       </c>
       <c r="D335" s="61" t="inlineStr">
         <is>
-          <t>Cada nadador de la posta hace su propio tramo, aunque el equipo sea uno. La promesa alcanza a toda la casa, y cada uno está invitado a creer.</t>
+          <t>En la posta, cada nadador hace su tramo. La promesa alcanza a toda la casa.</t>
         </is>
       </c>
     </row>
@@ -47994,7 +47994,7 @@
       </c>
       <c r="D336" s="61" t="inlineStr">
         <is>
-          <t>Rotación en el vóley: el equipo gira siempre en el mismo sentido y por eso no se pierde. Dichosa la familia que honra al Señor y anda en sus caminos.</t>
+          <t>En el vóley, el equipo rota siempre en el mismo sentido. Dichosa la familia que anda en los caminos de Dios.</t>
         </is>
       </c>
     </row>
@@ -48014,7 +48014,7 @@
       </c>
       <c r="D337" s="61" t="inlineStr">
         <is>
-          <t>Hay padres e hijos que se reencontraron alentando juntos a la Albirroja después de años de distancia. Dios puede volver el corazón de los padres hacia los hijos.</t>
+          <t>Padres e hijos se reencontraron alentando a la Albirroja. Dios vuelve el corazón de los padres hacia los hijos.</t>
         </is>
       </c>
     </row>
@@ -48034,7 +48034,7 @@
       </c>
       <c r="D338" s="61" t="inlineStr">
         <is>
-          <t>El ciclista que carga más peso del que puede llevar no llega lejos en la subida. Una deuda mal medida también hunde más de lo que ayuda; medir bien es sabiduría.</t>
+          <t>El ciclista con demasiado peso no llega lejos en la subida. Una deuda mal medida hunde.</t>
         </is>
       </c>
     </row>
@@ -48054,7 +48054,7 @@
       </c>
       <c r="D339" s="61" t="inlineStr">
         <is>
-          <t>Al terminar el torneo del barrio, el equipo arregla cuentas con el transporte y la cancha, pero el cariño entre compañeros sigue. La única deuda que siempre queda es el amor.</t>
+          <t>Las cuentas del torneo se arreglan; el cariño sigue. La única deuda que siempre queda es el amor.</t>
         </is>
       </c>
     </row>
@@ -48074,7 +48074,7 @@
       </c>
       <c r="D340" s="61" t="inlineStr">
         <is>
-          <t>Antes de entrar a la cancha, el jugador de futsal mide si está para jugar. Antes de salir de garante, también conviene medir el riesgo con prudencia y buen consejo.</t>
+          <t>El jugador mide si está para jugar. Antes de salir de garante, medí el riesgo.</t>
         </is>
       </c>
     </row>
@@ -48094,7 +48094,7 @@
       </c>
       <c r="D341" s="61" t="inlineStr">
         <is>
-          <t>Cuando el boxeador queda contra las cuerdas, lo sabio es salir pronto, sin desesperar. Con un compromiso financiero riesgoso pasa igual: no postergues buscar la salida, y pedí ayuda.</t>
+          <t>Contra las cuerdas, lo sabio es salir pronto. Ante una deuda riesgosa, buscá la salida y pedí ayuda.</t>
         </is>
       </c>
     </row>
@@ -48114,7 +48114,7 @@
       </c>
       <c r="D342" s="61" t="inlineStr">
         <is>
-          <t>El goleador que dice «lo hice solo» se olvida del pase, del entrenador y de quien le dio las piernas. No fue solo nuestra fuerza: todo viene de Dios.</t>
+          <t>El goleador que dice «lo hice solo» se olvida del pase. Todo viene de Dios.</t>
         </is>
       </c>
     </row>
@@ -48134,7 +48134,7 @@
       </c>
       <c r="D343" s="61" t="inlineStr">
         <is>
-          <t>Un buen equipo de vóley siempre tiene a alguien en el banco para lo inesperado. Un pequeño respaldo ayuda a cumplir lo que debemos y a seguir siendo generosos.</t>
+          <t>Un buen equipo tiene a alguien en el banco para lo inesperado. Un pequeño respaldo te ayuda a cumplir.</t>
         </is>
       </c>
     </row>
@@ -48154,7 +48154,7 @@
       </c>
       <c r="D344" s="61" t="inlineStr">
         <is>
-          <t>Primero lo más importante: así ordena el atleta su semana, y lo demás se acomoda. Buscá primero el reino de Dios y su justicia, confiando en que Él provee.</t>
+          <t>El atleta ordena su semana por lo más importante. Buscá primero el reino de Dios.</t>
         </is>
       </c>
     </row>
@@ -48174,7 +48174,7 @@
       </c>
       <c r="D345" s="61" t="inlineStr">
         <is>
-          <t>El jugador que esconde una lesión la empeora; el que la cuenta empieza a sanar. Con el pecado pasa igual: callarlo pesa, confesarlo nos lleva al perdón de Dios.</t>
+          <t>El que esconde una lesión la empeora; el que la cuenta empieza a sanar. Confesar nos lleva al perdón.</t>
         </is>
       </c>
     </row>
@@ -48194,7 +48194,7 @@
       </c>
       <c r="D346" s="61" t="inlineStr">
         <is>
-          <t>El tenista que mira su error en el video, en lugar de esconderlo, puede corregirlo. El que confiesa sus faltas y se aparta de ellas alcanza misericordia.</t>
+          <t>El tenista que mira su error en el video lo puede corregir. El que confiesa sus faltas alcanza misericordia.</t>
         </is>
       </c>
     </row>
@@ -48214,7 +48214,7 @@
       </c>
       <c r="D347" s="61" t="inlineStr">
         <is>
-          <t>El equipo que perdió la final no puede quedarse mirando la repetición para siempre. Dios dice: no te aferres a lo pasado, mirá que yo hago algo nuevo.</t>
+          <t>No se puede mirar la repetición de la final perdida para siempre. Dios hace algo nuevo.</t>
         </is>
       </c>
     </row>
@@ -48234,7 +48234,7 @@
       </c>
       <c r="D348" s="61" t="inlineStr">
         <is>
-          <t>Las horas incómodas en la pileta forman la resistencia del nadador. Pablo dice que la tribulación produce paciencia, y la paciencia, carácter probado y esperanza.</t>
+          <t>Las horas incómodas en la pileta forman resistencia. La prueba produce paciencia y esperanza.</t>
         </is>
       </c>
     </row>
@@ -48254,7 +48254,7 @@
       </c>
       <c r="D349" s="61" t="inlineStr">
         <is>
-          <t>Un ajedrecista no madura en una sola partida, sino en cientos, perdiendo y aprendiendo. Que la paciencia complete su obra, para que seamos maduros en la fe.</t>
+          <t>El ajedrecista madura en cientos de partidas. La paciencia completa su obra.</t>
         </is>
       </c>
     </row>
@@ -48274,7 +48274,7 @@
       </c>
       <c r="D350" s="61" t="inlineStr">
         <is>
-          <t>Con los años, el veterano ya no corre como antes, pero juega con más sabiduría. Aunque lo de afuera se desgaste, por dentro Dios nos renueva día a día.</t>
+          <t>El veterano corre menos, pero juega con más sabiduría. Por dentro, Dios nos renueva cada día.</t>
         </is>
       </c>
     </row>
@@ -48294,7 +48294,7 @@
       </c>
       <c r="D351" s="61" t="inlineStr">
         <is>
-          <t>Ningún maratonista llega a la meta de un salto: cada kilómetro suma. La senda del justo es como la luz del amanecer, que va en aumento paso a paso.</t>
+          <t>Ningún maratonista llega de un salto. La senda del justo crece como la luz del amanecer.</t>
         </is>
       </c>
     </row>
@@ -48314,7 +48314,7 @@
       </c>
       <c r="D352" s="61" t="inlineStr">
         <is>
-          <t>El entrenador que inventa una jugada nueva usa una creatividad que tiene su origen en Dios. Como a Bezalel, Dios también hoy da sabiduría para crear con excelencia.</t>
+          <t>El técnico que inventa una jugada usa una creatividad que viene de Dios. Él da sabiduría para crear.</t>
         </is>
       </c>
     </row>
@@ -48334,7 +48334,7 @@
       </c>
       <c r="D353" s="61" t="inlineStr">
         <is>
-          <t>Las pelotas y los botines cambiaron muchísimo, pero el juego sigue siendo el mismo. Pablo cambiaba la forma para alcanzar a otros, sin cambiar nunca el evangelio.</t>
+          <t>Los botines cambiaron, pero el juego es el mismo. Se cambia la forma, nunca el evangelio.</t>
         </is>
       </c>
     </row>
@@ -48354,7 +48354,7 @@
       </c>
       <c r="D354" s="61" t="inlineStr">
         <is>
-          <t>El técnico de vóley que estudia al rival sabe qué hacer en cada set. Los hijos de Isacar entendían los tiempos y sabían lo que había que hacer.</t>
+          <t>El técnico que estudia al rival sabe qué hacer en cada set. Entender los tiempos es sabiduría.</t>
         </is>
       </c>
     </row>
@@ -48374,7 +48374,7 @@
       </c>
       <c r="D355" s="61" t="inlineStr">
         <is>
-          <t>El árbitro que estudia cada cambio del reglamento sigue aprendiendo aunque tenga años de carrera. El corazón entendido nunca deja de buscar conocimiento.</t>
+          <t>El árbitro veterano sigue estudiando el reglamento. El corazón entendido nunca deja de aprender.</t>
         </is>
       </c>
     </row>
@@ -48394,7 +48394,7 @@
       </c>
       <c r="D356" s="61" t="inlineStr">
         <is>
-          <t>El ciclista que ajusta su bici antes de la carrera rinde mejor que el que sale apurado. Afilar el hacha antes de cortar es sabiduría práctica.</t>
+          <t>El ciclista que ajusta su bici rinde más. Afilar el hacha antes de cortar es sabiduría.</t>
         </is>
       </c>
     </row>
@@ -48414,7 +48414,7 @@
       </c>
       <c r="D357" s="61" t="inlineStr">
         <is>
-          <t>El piloto de rally baja la velocidad cuando su navegante le avisa del peligro. Con la tecnología también: el prudente ve el riesgo y se protege.</t>
+          <t>El piloto baja la velocidad cuando el navegante avisa. Con la tecnología, el prudente ve el riesgo.</t>
         </is>
       </c>
     </row>
@@ -48434,7 +48434,7 @@
       </c>
       <c r="D358" s="61" t="inlineStr">
         <is>
-          <t>En Navidad las canchas se aquietan y la familia se junta. No teman: hay una buena noticia para todo el pueblo. Hoy nació el Salvador, Cristo el Señor.</t>
+          <t>En Navidad las canchas se aquietan. No teman: hoy nació el Salvador, Cristo el Señor.</t>
         </is>
       </c>
     </row>
@@ -48454,7 +48454,7 @@
       </c>
       <c r="D359" s="61" t="inlineStr">
         <is>
-          <t>El kinesiólogo trata la lesión y el entrenador cuida el ánimo; el jugador de básquet necesita las dos cosas. Cuerpo, mente y espíritu sanan mejor juntos.</t>
+          <t>El kinesiólogo trata la lesión y el entrenador cuida el ánimo. Cuerpo, mente y espíritu sanan juntos.</t>
         </is>
       </c>
     </row>
@@ -48474,7 +48474,7 @@
       </c>
       <c r="D360" s="61" t="inlineStr">
         <is>
-          <t>Cuando un jugador de handball se lesiona, en muchos equipos el plantel lo rodea y ora por él. Orar unos por otros, también por la sanidad, es una invitación de Dios.</t>
+          <t>Cuando uno se lesiona, el plantel lo rodea y ora. Oren unos por otros.</t>
         </is>
       </c>
     </row>
@@ -48494,7 +48494,7 @@
       </c>
       <c r="D361" s="61" t="inlineStr">
         <is>
-          <t>Hay heridas que no aparecen en la radiografía, como la del tenista después de una derrota dura. Dios sana a los quebrantados de corazón y venda también esas heridas.</t>
+          <t>Hay heridas que no salen en la radiografía. Dios sana a los quebrantados de corazón.</t>
         </is>
       </c>
     </row>
@@ -48514,7 +48514,7 @@
       </c>
       <c r="D362" s="61" t="inlineStr">
         <is>
-          <t>El atleta que avisa a tiempo que algo le duele no es débil: es sabio. Reconocer que necesitamos médico, o ayuda, es el primer paso para sanar.</t>
+          <t>El atleta que avisa que le duele no es débil: es sabio. Reconocer que necesitás ayuda es empezar a sanar.</t>
         </is>
       </c>
     </row>
@@ -48534,7 +48534,7 @@
       </c>
       <c r="D363" s="61" t="inlineStr">
         <is>
-          <t>Un defensor que se tira a bloquear un remate recibe el golpe por su equipo: apenas una sombra de lo que hizo Jesús, por cuyas llagas fuimos curados.</t>
+          <t>El defensor que se tira a bloquear recibe el golpe por el equipo. Jesús cargó con nuestras heridas.</t>
         </is>
       </c>
     </row>
@@ -48554,7 +48554,7 @@
       </c>
       <c r="D364" s="61" t="inlineStr">
         <is>
-          <t>Las risas en el vestuario después del entrenamiento le hacen bien al equipo. El corazón alegre es buen remedio; y si la tristeza pesa mucho, pedir ayuda también es cuidarse.</t>
+          <t>Las risas en el vestuario le hacen bien al equipo. El corazón alegre es buen remedio.</t>
         </is>
       </c>
     </row>
@@ -48574,7 +48574,7 @@
       </c>
       <c r="D365" s="61" t="inlineStr">
         <is>
-          <t>Silbato final, penal errado, y una palabra amable del entrenador levanta el ánimo del jugador. Las palabras bondadosas son dulces para el alma y salud para el cuerpo.</t>
+          <t>Penal errado, y una palabra amable del entrenador levanta el ánimo. Las palabras bondadosas sanan.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Planilla de versículos para los diseñadores de flyers y tres correcciones de tildes en los textos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012sZjyYY9ZpXrog9pNGjXta
</commit_message>
<xml_diff>
--- a/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
+++ b/mensajero/content/planillas/Mensajero_TemasMacro_2027.xlsx
@@ -1096,7 +1096,7 @@
       </c>
       <c r="X2" s="21" t="inlineStr">
         <is>
-          <t>1 Corintios 6:19-20 — ¿Acaso ignoran que el cuerpo de ustedes es templo del Espiritu Santo, que esta en ustedes, y que recibieron de parte de Dios, y que ustedes no son dueños de si mismos? Porque ustedes han sido comprados; el precio de ustedes ya ha sido pagado. Por lo tanto, den gloria a Dios en su cuerpo y en su espíritu, los cuales son de Dios.</t>
+          <t>1 Corintios 6:19-20 — ¿Acaso ignoran que el cuerpo de ustedes es templo del Espíritu Santo, que está en ustedes, y que recibieron de parte de Dios, y que ustedes no son dueños de si mismos? Porque ustedes han sido comprados; el precio de ustedes ya ha sido pagado. Por lo tanto, den gloria a Dios en su cuerpo y en su espíritu, los cuales son de Dios.</t>
         </is>
       </c>
       <c r="Y2" s="21" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="X10" s="45" t="inlineStr">
         <is>
-          <t>Proverbios 27:23 — Mantente atento al estado de tus ovejas; cuida bien a tus rebanos</t>
+          <t>Proverbios 27:23 — Mantente atento al estado de tus ovejas; cuida bien a tus rebaños</t>
         </is>
       </c>
       <c r="Y10" s="47" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="AD10" s="45" t="inlineStr">
         <is>
-          <t>Proverbios 12:10 — El justo sabe cuando su bestia tiene hambre, pero los impíos son crueles de corazón</t>
+          <t>Proverbios 12:10 — El justo sabe cuándo su bestia tiene hambre, pero los impíos son crueles de corazón</t>
         </is>
       </c>
       <c r="AE10" s="47" t="inlineStr">

</xml_diff>